<commit_message>
docs(compliance): re-score GL-05/AC-08/AC-09 to Implemented in RCM
These controls are implemented in code and now carry automated
operating-effectiveness evidence (cutover/compliance.ts), so the Risk &
Control Matrix is updated to match reality:

- build_rcm.py: status Gap -> Implemented for ITGC-AC-08, ITGC-AC-09, GL-05,
  with references pointing at the real code paths + the test harness; removed
  their now-closed rows from the Gap Remediation tab.
- Regenerated Oshinei_ERP_SOX_RCM_v1.xlsx (66 controls: 39 Implemented /
  12 Partial / 15 Gap; Summary tab COUNTIFs update automatically).
- Readiness plan: corrected the control tally and marked the three controls
  closed in the remediation tables and roadmap.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HfE3vEKQxTc7LnYTH8xvRG
</commit_message>
<xml_diff>
--- a/compliance/Oshinei_ERP_SOX_RCM_v1.xlsx
+++ b/compliance/Oshinei_ERP_SOX_RCM_v1.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RCM" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gap Remediation" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COSO Mapping" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Cover" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="RCM" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Gap Remediation" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="COSO Mapping" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Summary" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'RCM'!$A$1:$Q$67</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Gap Remediation'!$A$2:$H$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Gap Remediation'!$A$2:$H$28</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -2158,7 +2158,7 @@
       </c>
       <c r="M15" s="16" t="inlineStr">
         <is>
-          <t>admin-users (export to build)</t>
+          <t>admin-users.service.ts (access-review / export CSV / certify); admin-users.controller.ts; cutover/compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N15" s="16" t="inlineStr">
@@ -2168,7 +2168,7 @@
       </c>
       <c r="O15" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: each quarter reviewed &amp; exceptions remediated.</t>
+          <t>Re-perform: each quarter reviewed &amp; exceptions remediated (automated harness re-performs report/export/certify).</t>
         </is>
       </c>
       <c r="P15" s="16" t="inlineStr">
@@ -2176,9 +2176,9 @@
           <t>UAR sign-off</t>
         </is>
       </c>
-      <c r="Q15" s="14" t="inlineStr">
-        <is>
-          <t>Gap</t>
+      <c r="Q15" s="19" t="inlineStr">
+        <is>
+          <t>Implemented</t>
         </is>
       </c>
     </row>
@@ -2245,7 +2245,7 @@
       </c>
       <c r="M16" s="12" t="inlineStr">
         <is>
-          <t>/sod (web); workflow/approvals (to extend)</t>
+          <t>permissions.ts (SOD_RULES, 13 rules); admin-users.service.ts (assertNoSodConflict preventive block); sod.service.ts (detective report); cutover/compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N16" s="12" t="inlineStr">
@@ -2255,7 +2255,7 @@
       </c>
       <c r="O16" s="12" t="inlineStr">
         <is>
-          <t>Run conflict report; evidence conflicts cleared/approved.</t>
+          <t>Run conflict report; assigning a conflicting set is blocked (422) unless justified-override+reason — re-performed by the harness.</t>
         </is>
       </c>
       <c r="P16" s="12" t="inlineStr">
@@ -2263,9 +2263,9 @@
           <t>SoD report</t>
         </is>
       </c>
-      <c r="Q16" s="14" t="inlineStr">
-        <is>
-          <t>Gap</t>
+      <c r="Q16" s="19" t="inlineStr">
+        <is>
+          <t>Implemented</t>
         </is>
       </c>
     </row>
@@ -5725,7 +5725,7 @@
       </c>
       <c r="M56" s="12" t="inlineStr">
         <is>
-          <t>workflow / approvals (to extend to JE)</t>
+          <t>ledger.service.ts (postEntry pendingApproval→Draft; approveEntry preparer≠approver; rejectEntry); ledger.controller.ts (gl_post posts / gl_close approves); cutover/compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N56" s="12" t="inlineStr">
@@ -5735,7 +5735,7 @@
       </c>
       <c r="O56" s="12" t="inlineStr">
         <is>
-          <t>Sample manual JEs: approver ≠ preparer.</t>
+          <t>Sample manual JEs: approver ≠ preparer; Draft excluded from balances until approved (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P56" s="12" t="inlineStr">
@@ -5743,9 +5743,9 @@
           <t>JE approvals</t>
         </is>
       </c>
-      <c r="Q56" s="14" t="inlineStr">
-        <is>
-          <t>Gap</t>
+      <c r="Q56" s="19" t="inlineStr">
+        <is>
+          <t>Implemented</t>
         </is>
       </c>
     </row>
@@ -6718,7 +6718,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H31"/>
+  <dimension ref="A1:H28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -7035,7 +7035,7 @@
     <row r="9">
       <c r="A9" s="11" t="inlineStr">
         <is>
-          <t>ITGC-AC-08</t>
+          <t>ITGC-AC-13</t>
         </is>
       </c>
       <c r="B9" s="13" t="inlineStr">
@@ -7045,17 +7045,17 @@
       </c>
       <c r="C9" s="12" t="inlineStr">
         <is>
-          <t>No periodic user access review.</t>
+          <t>DB access controls / named users not formalized.</t>
         </is>
       </c>
       <c r="D9" s="12" t="inlineStr">
         <is>
-          <t>Build user×permission export + quarterly recertification workflow.</t>
+          <t>Restrict DB roles to least privilege; named users; log DBA access.</t>
         </is>
       </c>
       <c r="E9" s="13" t="inlineStr">
         <is>
-          <t>Controller / IT</t>
+          <t>DBA / DevOps</t>
         </is>
       </c>
       <c r="F9" s="13" t="inlineStr">
@@ -7068,46 +7068,46 @@
           <t>Month 2-3</t>
         </is>
       </c>
-      <c r="H9" s="22" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="H9" s="23" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="15" t="inlineStr">
         <is>
-          <t>ITGC-AC-09</t>
+          <t>ITGC-OP-01</t>
         </is>
       </c>
       <c r="B10" s="17" t="inlineStr">
         <is>
-          <t>ITGC · Access</t>
+          <t>ITGC · Operations</t>
         </is>
       </c>
       <c r="C10" s="16" t="inlineStr">
         <is>
-          <t>SoD only a UI page; no enforced ruleset.</t>
+          <t>Backup/restore not proven by test.</t>
         </is>
       </c>
       <c r="D10" s="16" t="inlineStr">
         <is>
-          <t>Define SoD conflict matrix vs 37 perms/5 roles; preventive blocks + detective report.</t>
+          <t>Automate backups; perform + evidence a quarterly restore test.</t>
         </is>
       </c>
       <c r="E10" s="17" t="inlineStr">
         <is>
-          <t>Controller / IT</t>
+          <t>DevOps</t>
         </is>
       </c>
       <c r="F10" s="17" t="inlineStr">
         <is>
-          <t>Phase 2</t>
+          <t>Phase 1</t>
         </is>
       </c>
       <c r="G10" s="17" t="inlineStr">
         <is>
-          <t>Month 3-4</t>
+          <t>Month 1-2</t>
         </is>
       </c>
       <c r="H10" s="22" t="inlineStr">
@@ -7119,37 +7119,37 @@
     <row r="11">
       <c r="A11" s="11" t="inlineStr">
         <is>
-          <t>ITGC-AC-13</t>
+          <t>ITGC-OP-02</t>
         </is>
       </c>
       <c r="B11" s="13" t="inlineStr">
         <is>
-          <t>ITGC · Access</t>
+          <t>ITGC · Operations</t>
         </is>
       </c>
       <c r="C11" s="12" t="inlineStr">
         <is>
-          <t>DB access controls / named users not formalized.</t>
+          <t>No DR/BCP plan.</t>
         </is>
       </c>
       <c r="D11" s="12" t="inlineStr">
         <is>
-          <t>Restrict DB roles to least privilege; named users; log DBA access.</t>
+          <t>Author DR/BCP with RTO/RPO; schedule annual test.</t>
         </is>
       </c>
       <c r="E11" s="13" t="inlineStr">
         <is>
-          <t>DBA / DevOps</t>
+          <t>CTO / DevOps</t>
         </is>
       </c>
       <c r="F11" s="13" t="inlineStr">
         <is>
-          <t>Phase 1-2</t>
+          <t>Phase 2</t>
         </is>
       </c>
       <c r="G11" s="13" t="inlineStr">
         <is>
-          <t>Month 2-3</t>
+          <t>Month 3-5</t>
         </is>
       </c>
       <c r="H11" s="23" t="inlineStr">
@@ -7161,7 +7161,7 @@
     <row r="12">
       <c r="A12" s="15" t="inlineStr">
         <is>
-          <t>ITGC-OP-01</t>
+          <t>ITGC-OP-04</t>
         </is>
       </c>
       <c r="B12" s="17" t="inlineStr">
@@ -7171,59 +7171,59 @@
       </c>
       <c r="C12" s="16" t="inlineStr">
         <is>
-          <t>Backup/restore not proven by test.</t>
+          <t>Scheduled financial jobs not monitored.</t>
         </is>
       </c>
       <c r="D12" s="16" t="inlineStr">
         <is>
-          <t>Automate backups; perform + evidence a quarterly restore test.</t>
+          <t>Inventory batch jobs; add failure alerting + review evidence.</t>
         </is>
       </c>
       <c r="E12" s="17" t="inlineStr">
         <is>
-          <t>DevOps</t>
+          <t>DevOps / Controller</t>
         </is>
       </c>
       <c r="F12" s="17" t="inlineStr">
         <is>
-          <t>Phase 1</t>
+          <t>Phase 2</t>
         </is>
       </c>
       <c r="G12" s="17" t="inlineStr">
         <is>
-          <t>Month 1-2</t>
-        </is>
-      </c>
-      <c r="H12" s="22" t="inlineStr">
-        <is>
-          <t>High</t>
+          <t>Month 3</t>
+        </is>
+      </c>
+      <c r="H12" s="23" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="11" t="inlineStr">
         <is>
-          <t>ITGC-OP-02</t>
+          <t>ITGC-SD-01</t>
         </is>
       </c>
       <c r="B13" s="13" t="inlineStr">
         <is>
-          <t>ITGC · Operations</t>
+          <t>ITGC · SDLC</t>
         </is>
       </c>
       <c r="C13" s="12" t="inlineStr">
         <is>
-          <t>No DR/BCP plan.</t>
+          <t>No formal SDLC policy.</t>
         </is>
       </c>
       <c r="D13" s="12" t="inlineStr">
         <is>
-          <t>Author DR/BCP with RTO/RPO; schedule annual test.</t>
+          <t>Author SDLC policy with design/test/UAT/go-live sign-offs.</t>
         </is>
       </c>
       <c r="E13" s="13" t="inlineStr">
         <is>
-          <t>CTO / DevOps</t>
+          <t>Head of Eng / Product</t>
         </is>
       </c>
       <c r="F13" s="13" t="inlineStr">
@@ -7233,7 +7233,7 @@
       </c>
       <c r="G13" s="13" t="inlineStr">
         <is>
-          <t>Month 3-5</t>
+          <t>Month 3-4</t>
         </is>
       </c>
       <c r="H13" s="23" t="inlineStr">
@@ -7245,27 +7245,27 @@
     <row r="14">
       <c r="A14" s="15" t="inlineStr">
         <is>
-          <t>ITGC-OP-04</t>
+          <t>ITGC-SD-02</t>
         </is>
       </c>
       <c r="B14" s="17" t="inlineStr">
         <is>
-          <t>ITGC · Operations</t>
+          <t>ITGC · SDLC</t>
         </is>
       </c>
       <c r="C14" s="16" t="inlineStr">
         <is>
-          <t>Scheduled financial jobs not monitored.</t>
+          <t>Cutover reconciliation not documented.</t>
         </is>
       </c>
       <c r="D14" s="16" t="inlineStr">
         <is>
-          <t>Inventory batch jobs; add failure alerting + review evidence.</t>
+          <t>Document source→target balance tie-out + sign-off for any migration.</t>
         </is>
       </c>
       <c r="E14" s="17" t="inlineStr">
         <is>
-          <t>DevOps / Controller</t>
+          <t>Controller / Eng</t>
         </is>
       </c>
       <c r="F14" s="17" t="inlineStr">
@@ -7275,7 +7275,7 @@
       </c>
       <c r="G14" s="17" t="inlineStr">
         <is>
-          <t>Month 3</t>
+          <t>Month 4</t>
         </is>
       </c>
       <c r="H14" s="23" t="inlineStr">
@@ -7287,7 +7287,7 @@
     <row r="15">
       <c r="A15" s="11" t="inlineStr">
         <is>
-          <t>ITGC-SD-01</t>
+          <t>ITGC-SD-03</t>
         </is>
       </c>
       <c r="B15" s="13" t="inlineStr">
@@ -7297,17 +7297,17 @@
       </c>
       <c r="C15" s="12" t="inlineStr">
         <is>
-          <t>No formal SDLC policy.</t>
+          <t>Test coverage of key controls partial.</t>
         </is>
       </c>
       <c r="D15" s="12" t="inlineStr">
         <is>
-          <t>Author SDLC policy with design/test/UAT/go-live sign-offs.</t>
+          <t>Expand key-control regression tests; CI archives dated evidence.</t>
         </is>
       </c>
       <c r="E15" s="13" t="inlineStr">
         <is>
-          <t>Head of Eng / Product</t>
+          <t>Head of Eng</t>
         </is>
       </c>
       <c r="F15" s="13" t="inlineStr">
@@ -7317,7 +7317,7 @@
       </c>
       <c r="G15" s="13" t="inlineStr">
         <is>
-          <t>Month 3-4</t>
+          <t>Month 3-5</t>
         </is>
       </c>
       <c r="H15" s="23" t="inlineStr">
@@ -7329,27 +7329,27 @@
     <row r="16">
       <c r="A16" s="15" t="inlineStr">
         <is>
-          <t>ITGC-SD-02</t>
+          <t>EXP-03</t>
         </is>
       </c>
       <c r="B16" s="17" t="inlineStr">
         <is>
-          <t>ITGC · SDLC</t>
+          <t>Expenditure</t>
         </is>
       </c>
       <c r="C16" s="16" t="inlineStr">
         <is>
-          <t>Cutover reconciliation not documented.</t>
+          <t>PR/PO approval workflow partial.</t>
         </is>
       </c>
       <c r="D16" s="16" t="inlineStr">
         <is>
-          <t>Document source→target balance tie-out + sign-off for any migration.</t>
+          <t>Finalize PR/PO maker-checker against DoA thresholds.</t>
         </is>
       </c>
       <c r="E16" s="17" t="inlineStr">
         <is>
-          <t>Controller / Eng</t>
+          <t>Procurement Mgr</t>
         </is>
       </c>
       <c r="F16" s="17" t="inlineStr">
@@ -7359,7 +7359,7 @@
       </c>
       <c r="G16" s="17" t="inlineStr">
         <is>
-          <t>Month 4</t>
+          <t>Month 3-4</t>
         </is>
       </c>
       <c r="H16" s="23" t="inlineStr">
@@ -7371,27 +7371,27 @@
     <row r="17">
       <c r="A17" s="11" t="inlineStr">
         <is>
-          <t>ITGC-SD-03</t>
+          <t>INV-04</t>
         </is>
       </c>
       <c r="B17" s="13" t="inlineStr">
         <is>
-          <t>ITGC · SDLC</t>
+          <t>Inventory &amp; COGS</t>
         </is>
       </c>
       <c r="C17" s="12" t="inlineStr">
         <is>
-          <t>Test coverage of key controls partial.</t>
+          <t>Stocktake variance review informal.</t>
         </is>
       </c>
       <c r="D17" s="12" t="inlineStr">
         <is>
-          <t>Expand key-control regression tests; CI archives dated evidence.</t>
+          <t>Formalize count cadence + variance review/approval sign-off.</t>
         </is>
       </c>
       <c r="E17" s="13" t="inlineStr">
         <is>
-          <t>Head of Eng</t>
+          <t>Warehouse Mgr</t>
         </is>
       </c>
       <c r="F17" s="13" t="inlineStr">
@@ -7401,7 +7401,7 @@
       </c>
       <c r="G17" s="13" t="inlineStr">
         <is>
-          <t>Month 3-5</t>
+          <t>Month 4</t>
         </is>
       </c>
       <c r="H17" s="23" t="inlineStr">
@@ -7413,79 +7413,79 @@
     <row r="18">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>GL-05</t>
+          <t>REC-03</t>
         </is>
       </c>
       <c r="B18" s="17" t="inlineStr">
         <is>
-          <t>General Ledger</t>
+          <t>Reconciliation</t>
         </is>
       </c>
       <c r="C18" s="16" t="inlineStr">
         <is>
-          <t>Manual JE has no maker-checker.</t>
+          <t>Intercompany recon partial.</t>
         </is>
       </c>
       <c r="D18" s="16" t="inlineStr">
         <is>
-          <t>Extend approvals engine to require approver ≠ preparer for manual JEs.</t>
+          <t>Formalize IC matching + elimination sign-off each period.</t>
         </is>
       </c>
       <c r="E18" s="17" t="inlineStr">
         <is>
-          <t>Controller / Eng</t>
+          <t>Group Controller</t>
         </is>
       </c>
       <c r="F18" s="17" t="inlineStr">
         <is>
-          <t>Phase 2</t>
+          <t>Phase 2-3</t>
         </is>
       </c>
       <c r="G18" s="17" t="inlineStr">
         <is>
-          <t>Month 3-4</t>
-        </is>
-      </c>
-      <c r="H18" s="22" t="inlineStr">
-        <is>
-          <t>High</t>
+          <t>Month 4-6</t>
+        </is>
+      </c>
+      <c r="H18" s="23" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="11" t="inlineStr">
         <is>
-          <t>EXP-03</t>
+          <t>ITGC-AC-07</t>
         </is>
       </c>
       <c r="B19" s="13" t="inlineStr">
         <is>
-          <t>Expenditure</t>
+          <t>ITGC · Access</t>
         </is>
       </c>
       <c r="C19" s="12" t="inlineStr">
         <is>
-          <t>PR/PO approval workflow partial.</t>
+          <t>Password/session policy partial.</t>
         </is>
       </c>
       <c r="D19" s="12" t="inlineStr">
         <is>
-          <t>Finalize PR/PO maker-checker against DoA thresholds.</t>
+          <t>Document + enforce password policy, lockout, session expiry.</t>
         </is>
       </c>
       <c r="E19" s="13" t="inlineStr">
         <is>
-          <t>Procurement Mgr</t>
+          <t>IT Security</t>
         </is>
       </c>
       <c r="F19" s="13" t="inlineStr">
         <is>
-          <t>Phase 2</t>
+          <t>Phase 1</t>
         </is>
       </c>
       <c r="G19" s="13" t="inlineStr">
         <is>
-          <t>Month 3-4</t>
+          <t>Month 2</t>
         </is>
       </c>
       <c r="H19" s="23" t="inlineStr">
@@ -7497,37 +7497,37 @@
     <row r="20">
       <c r="A20" s="15" t="inlineStr">
         <is>
-          <t>INV-04</t>
+          <t>ITGC-CM-02</t>
         </is>
       </c>
       <c r="B20" s="17" t="inlineStr">
         <is>
-          <t>Inventory &amp; COGS</t>
+          <t>ITGC · Change</t>
         </is>
       </c>
       <c r="C20" s="16" t="inlineStr">
         <is>
-          <t>Stocktake variance review informal.</t>
+          <t>Migration-only DDL not strictly enforced.</t>
         </is>
       </c>
       <c r="D20" s="16" t="inlineStr">
         <is>
-          <t>Formalize count cadence + variance review/approval sign-off.</t>
+          <t>Block direct prod DDL; gate migrations behind review + pipeline.</t>
         </is>
       </c>
       <c r="E20" s="17" t="inlineStr">
         <is>
-          <t>Warehouse Mgr</t>
+          <t>Head of Eng / DBA</t>
         </is>
       </c>
       <c r="F20" s="17" t="inlineStr">
         <is>
-          <t>Phase 2</t>
+          <t>Phase 1</t>
         </is>
       </c>
       <c r="G20" s="17" t="inlineStr">
         <is>
-          <t>Month 4</t>
+          <t>Month 2</t>
         </is>
       </c>
       <c r="H20" s="23" t="inlineStr">
@@ -7539,37 +7539,37 @@
     <row r="21">
       <c r="A21" s="11" t="inlineStr">
         <is>
-          <t>REC-03</t>
+          <t>ITGC-OP-03</t>
         </is>
       </c>
       <c r="B21" s="13" t="inlineStr">
         <is>
-          <t>Reconciliation</t>
+          <t>ITGC · Operations</t>
         </is>
       </c>
       <c r="C21" s="12" t="inlineStr">
         <is>
-          <t>Intercompany recon partial.</t>
+          <t>Alerting/incident process partial.</t>
         </is>
       </c>
       <c r="D21" s="12" t="inlineStr">
         <is>
-          <t>Formalize IC matching + elimination sign-off each period.</t>
+          <t>Formalize alert routing, on-call, incident log + post-mortems.</t>
         </is>
       </c>
       <c r="E21" s="13" t="inlineStr">
         <is>
-          <t>Group Controller</t>
+          <t>DevOps</t>
         </is>
       </c>
       <c r="F21" s="13" t="inlineStr">
         <is>
-          <t>Phase 2-3</t>
+          <t>Phase 2</t>
         </is>
       </c>
       <c r="G21" s="13" t="inlineStr">
         <is>
-          <t>Month 4-6</t>
+          <t>Month 3</t>
         </is>
       </c>
       <c r="H21" s="23" t="inlineStr">
@@ -7581,37 +7581,37 @@
     <row r="22">
       <c r="A22" s="15" t="inlineStr">
         <is>
-          <t>ITGC-AC-07</t>
+          <t>TAX-03</t>
         </is>
       </c>
       <c r="B22" s="17" t="inlineStr">
         <is>
-          <t>ITGC · Access</t>
+          <t>Tax</t>
         </is>
       </c>
       <c r="C22" s="16" t="inlineStr">
         <is>
-          <t>Password/session policy partial.</t>
+          <t>WHT reporting partial.</t>
         </is>
       </c>
       <c r="D22" s="16" t="inlineStr">
         <is>
-          <t>Document + enforce password policy, lockout, session expiry.</t>
+          <t>Complete WHT calc coverage + monthly ภ.ง.ด. tie-out.</t>
         </is>
       </c>
       <c r="E22" s="17" t="inlineStr">
         <is>
-          <t>IT Security</t>
+          <t>Tax</t>
         </is>
       </c>
       <c r="F22" s="17" t="inlineStr">
         <is>
-          <t>Phase 1</t>
+          <t>Phase 2-3</t>
         </is>
       </c>
       <c r="G22" s="17" t="inlineStr">
         <is>
-          <t>Month 2</t>
+          <t>Month 4-6</t>
         </is>
       </c>
       <c r="H22" s="23" t="inlineStr">
@@ -7623,37 +7623,37 @@
     <row r="23">
       <c r="A23" s="11" t="inlineStr">
         <is>
-          <t>ITGC-CM-02</t>
+          <t>PAY-02</t>
         </is>
       </c>
       <c r="B23" s="13" t="inlineStr">
         <is>
-          <t>ITGC · Change</t>
+          <t>Payroll</t>
         </is>
       </c>
       <c r="C23" s="12" t="inlineStr">
         <is>
-          <t>Migration-only DDL not strictly enforced.</t>
+          <t>Statutory payroll items partial.</t>
         </is>
       </c>
       <c r="D23" s="12" t="inlineStr">
         <is>
-          <t>Block direct prod DDL; gate migrations behind review + pipeline.</t>
+          <t>Complete PF/OT/leave + ภ.ง.ด.1ก reconciliation to filings.</t>
         </is>
       </c>
       <c r="E23" s="13" t="inlineStr">
         <is>
-          <t>Head of Eng / DBA</t>
+          <t>HR / Payroll</t>
         </is>
       </c>
       <c r="F23" s="13" t="inlineStr">
         <is>
-          <t>Phase 1</t>
+          <t>Phase 2-3</t>
         </is>
       </c>
       <c r="G23" s="13" t="inlineStr">
         <is>
-          <t>Month 2</t>
+          <t>Month 4-6</t>
         </is>
       </c>
       <c r="H23" s="23" t="inlineStr">
@@ -7665,133 +7665,133 @@
     <row r="24">
       <c r="A24" s="15" t="inlineStr">
         <is>
-          <t>ITGC-OP-03</t>
+          <t>ELC-01</t>
         </is>
       </c>
       <c r="B24" s="17" t="inlineStr">
         <is>
-          <t>ITGC · Operations</t>
+          <t>Entity-Level</t>
         </is>
       </c>
       <c r="C24" s="16" t="inlineStr">
         <is>
-          <t>Alerting/incident process partial.</t>
+          <t>No ethics policy / acknowledgements.</t>
         </is>
       </c>
       <c r="D24" s="16" t="inlineStr">
         <is>
-          <t>Formalize alert routing, on-call, incident log + post-mortems.</t>
+          <t>Issue code of conduct; annual acknowledgement register.</t>
         </is>
       </c>
       <c r="E24" s="17" t="inlineStr">
         <is>
-          <t>DevOps</t>
+          <t>CEO / HR</t>
         </is>
       </c>
       <c r="F24" s="17" t="inlineStr">
         <is>
-          <t>Phase 2</t>
+          <t>Phase 1</t>
         </is>
       </c>
       <c r="G24" s="17" t="inlineStr">
         <is>
-          <t>Month 3</t>
-        </is>
-      </c>
-      <c r="H24" s="23" t="inlineStr">
-        <is>
-          <t>Medium</t>
+          <t>Month 1-2</t>
+        </is>
+      </c>
+      <c r="H24" s="22" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="11" t="inlineStr">
         <is>
-          <t>TAX-03</t>
+          <t>ELC-02</t>
         </is>
       </c>
       <c r="B25" s="13" t="inlineStr">
         <is>
-          <t>Tax</t>
+          <t>Entity-Level</t>
         </is>
       </c>
       <c r="C25" s="12" t="inlineStr">
         <is>
-          <t>WHT reporting partial.</t>
+          <t>No audit-committee ICFR oversight.</t>
         </is>
       </c>
       <c r="D25" s="12" t="inlineStr">
         <is>
-          <t>Complete WHT calc coverage + monthly ภ.ง.ด. tie-out.</t>
+          <t>Charter audit committee; quarterly ICFR review minutes.</t>
         </is>
       </c>
       <c r="E25" s="13" t="inlineStr">
         <is>
-          <t>Tax</t>
+          <t>Board</t>
         </is>
       </c>
       <c r="F25" s="13" t="inlineStr">
         <is>
-          <t>Phase 2-3</t>
+          <t>Phase 1</t>
         </is>
       </c>
       <c r="G25" s="13" t="inlineStr">
         <is>
-          <t>Month 4-6</t>
-        </is>
-      </c>
-      <c r="H25" s="23" t="inlineStr">
-        <is>
-          <t>Medium</t>
+          <t>Month 1-2</t>
+        </is>
+      </c>
+      <c r="H25" s="22" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="15" t="inlineStr">
         <is>
-          <t>PAY-02</t>
+          <t>ELC-03</t>
         </is>
       </c>
       <c r="B26" s="17" t="inlineStr">
         <is>
-          <t>Payroll</t>
+          <t>Entity-Level</t>
         </is>
       </c>
       <c r="C26" s="16" t="inlineStr">
         <is>
-          <t>Statutory payroll items partial.</t>
+          <t>No documented delegation of authority.</t>
         </is>
       </c>
       <c r="D26" s="16" t="inlineStr">
         <is>
-          <t>Complete PF/OT/leave + ภ.ง.ด.1ก reconciliation to filings.</t>
+          <t>Author DoA/approval matrix; reconcile to RBAC roles.</t>
         </is>
       </c>
       <c r="E26" s="17" t="inlineStr">
         <is>
-          <t>HR / Payroll</t>
+          <t>CFO</t>
         </is>
       </c>
       <c r="F26" s="17" t="inlineStr">
         <is>
-          <t>Phase 2-3</t>
+          <t>Phase 1</t>
         </is>
       </c>
       <c r="G26" s="17" t="inlineStr">
         <is>
-          <t>Month 4-6</t>
-        </is>
-      </c>
-      <c r="H26" s="23" t="inlineStr">
-        <is>
-          <t>Medium</t>
+          <t>Month 2</t>
+        </is>
+      </c>
+      <c r="H26" s="22" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="11" t="inlineStr">
         <is>
-          <t>ELC-01</t>
+          <t>ELC-04</t>
         </is>
       </c>
       <c r="B27" s="13" t="inlineStr">
@@ -7801,17 +7801,17 @@
       </c>
       <c r="C27" s="12" t="inlineStr">
         <is>
-          <t>No ethics policy / acknowledgements.</t>
+          <t>No whistleblower channel.</t>
         </is>
       </c>
       <c r="D27" s="12" t="inlineStr">
         <is>
-          <t>Issue code of conduct; annual acknowledgement register.</t>
+          <t>Stand up anonymous hotline + non-retaliation policy.</t>
         </is>
       </c>
       <c r="E27" s="13" t="inlineStr">
         <is>
-          <t>CEO / HR</t>
+          <t>Audit Cttee</t>
         </is>
       </c>
       <c r="F27" s="13" t="inlineStr">
@@ -7821,19 +7821,19 @@
       </c>
       <c r="G27" s="13" t="inlineStr">
         <is>
-          <t>Month 1-2</t>
-        </is>
-      </c>
-      <c r="H27" s="22" t="inlineStr">
-        <is>
-          <t>High</t>
+          <t>Month 2</t>
+        </is>
+      </c>
+      <c r="H27" s="23" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="15" t="inlineStr">
         <is>
-          <t>ELC-02</t>
+          <t>ELC-05</t>
         </is>
       </c>
       <c r="B28" s="17" t="inlineStr">
@@ -7843,163 +7843,37 @@
       </c>
       <c r="C28" s="16" t="inlineStr">
         <is>
-          <t>No audit-committee ICFR oversight.</t>
+          <t>No fraud risk assessment.</t>
         </is>
       </c>
       <c r="D28" s="16" t="inlineStr">
         <is>
-          <t>Charter audit committee; quarterly ICFR review minutes.</t>
+          <t>Perform annual fraud risk assessment; map to controls.</t>
         </is>
       </c>
       <c r="E28" s="17" t="inlineStr">
         <is>
-          <t>Board</t>
+          <t>CFO / IA</t>
         </is>
       </c>
       <c r="F28" s="17" t="inlineStr">
         <is>
-          <t>Phase 1</t>
+          <t>Phase 2</t>
         </is>
       </c>
       <c r="G28" s="17" t="inlineStr">
         <is>
-          <t>Month 1-2</t>
-        </is>
-      </c>
-      <c r="H28" s="22" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="11" t="inlineStr">
-        <is>
-          <t>ELC-03</t>
-        </is>
-      </c>
-      <c r="B29" s="13" t="inlineStr">
-        <is>
-          <t>Entity-Level</t>
-        </is>
-      </c>
-      <c r="C29" s="12" t="inlineStr">
-        <is>
-          <t>No documented delegation of authority.</t>
-        </is>
-      </c>
-      <c r="D29" s="12" t="inlineStr">
-        <is>
-          <t>Author DoA/approval matrix; reconcile to RBAC roles.</t>
-        </is>
-      </c>
-      <c r="E29" s="13" t="inlineStr">
-        <is>
-          <t>CFO</t>
-        </is>
-      </c>
-      <c r="F29" s="13" t="inlineStr">
-        <is>
-          <t>Phase 1</t>
-        </is>
-      </c>
-      <c r="G29" s="13" t="inlineStr">
-        <is>
-          <t>Month 2</t>
-        </is>
-      </c>
-      <c r="H29" s="22" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="15" t="inlineStr">
-        <is>
-          <t>ELC-04</t>
-        </is>
-      </c>
-      <c r="B30" s="17" t="inlineStr">
-        <is>
-          <t>Entity-Level</t>
-        </is>
-      </c>
-      <c r="C30" s="16" t="inlineStr">
-        <is>
-          <t>No whistleblower channel.</t>
-        </is>
-      </c>
-      <c r="D30" s="16" t="inlineStr">
-        <is>
-          <t>Stand up anonymous hotline + non-retaliation policy.</t>
-        </is>
-      </c>
-      <c r="E30" s="17" t="inlineStr">
-        <is>
-          <t>Audit Cttee</t>
-        </is>
-      </c>
-      <c r="F30" s="17" t="inlineStr">
-        <is>
-          <t>Phase 1</t>
-        </is>
-      </c>
-      <c r="G30" s="17" t="inlineStr">
-        <is>
-          <t>Month 2</t>
-        </is>
-      </c>
-      <c r="H30" s="23" t="inlineStr">
+          <t>Month 3</t>
+        </is>
+      </c>
+      <c r="H28" s="23" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="11" t="inlineStr">
-        <is>
-          <t>ELC-05</t>
-        </is>
-      </c>
-      <c r="B31" s="13" t="inlineStr">
-        <is>
-          <t>Entity-Level</t>
-        </is>
-      </c>
-      <c r="C31" s="12" t="inlineStr">
-        <is>
-          <t>No fraud risk assessment.</t>
-        </is>
-      </c>
-      <c r="D31" s="12" t="inlineStr">
-        <is>
-          <t>Perform annual fraud risk assessment; map to controls.</t>
-        </is>
-      </c>
-      <c r="E31" s="13" t="inlineStr">
-        <is>
-          <t>CFO / IA</t>
-        </is>
-      </c>
-      <c r="F31" s="13" t="inlineStr">
-        <is>
-          <t>Phase 2</t>
-        </is>
-      </c>
-      <c r="G31" s="13" t="inlineStr">
-        <is>
-          <t>Month 3</t>
-        </is>
-      </c>
-      <c r="H31" s="23" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A2:H31"/>
+  <autoFilter ref="A2:H28"/>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>

</xml_diff>

<commit_message>
feat(compliance): REV-08 credit-limit ToE test + entity-level policy templates
- Adds REV-08 credit-limit / credit-hold operating-effectiveness test to the
  control harness (outstanding AR + order > limit -> CREDIT_LIMIT; credit hold
  -> CREDIT_HOLD). Harness now 30 checks, all green. RCM ToE reference updated.
- Adds a full entity-level + ITGC policy template suite under compliance/policies/
  (13 DRAFT documents + register), each mapped to RCM control IDs and the
  implemented system controls. Closes the documentation side of ELC-01..05 and
  anchors the ITGC policies (infosec, access control, change/SDLC, backup/DR,
  incident response, financial close, third-party/sub-service orgs).
- Readiness plan section 6 now references the templates; next-actions updated.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HfE3vEKQxTc7LnYTH8xvRG
</commit_message>
<xml_diff>
--- a/compliance/Oshinei_ERP_SOX_RCM_v1.xlsx
+++ b/compliance/Oshinei_ERP_SOX_RCM_v1.xlsx
@@ -4333,7 +4333,7 @@
       </c>
       <c r="M40" s="12" t="inlineStr">
         <is>
-          <t>pos.service.ts (createOrder)</t>
+          <t>pos.service.ts (createOrder, FOR UPDATE); cutover/compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N40" s="12" t="inlineStr">
@@ -4343,7 +4343,7 @@
       </c>
       <c r="O40" s="12" t="inlineStr">
         <is>
-          <t>Concurrent orders cannot jointly breach limit.</t>
+          <t>Sample: outstanding+order ≤ limit allowed, &gt; limit → CREDIT_LIMIT, credit-hold → CREDIT_HOLD (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P40" s="12" t="inlineStr">

</xml_diff>

<commit_message>
Pre-production gate-keeping audit: integrity, performance, SOX controls & UX hardening (#73)
Four-pillar NASDAQ-readiness audit. Pillar 1: AR/AP lost-update row locks + diner error surfacing. Pillar 2: 24 hot-path indexes + maintenance plan + N+1 elimination. Pillar 3: AP disbursement maker-checker (EXP-06) + field-level change log (ITGC-AC-14); RCM 72 controls. Pillar 4: double-submit guards on money-movement + ~35 table-row mutations. All CI green (75 checks).
</commit_message>
<xml_diff>
--- a/compliance/Oshinei_ERP_SOX_RCM_v1.xlsx
+++ b/compliance/Oshinei_ERP_SOX_RCM_v1.xlsx
@@ -14,7 +14,7 @@
     <sheet name="Summary" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'RCM'!$A$1:$Q$71</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'RCM'!$A$1:$Q$73</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Gap Remediation'!$A$2:$H$18</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -855,7 +855,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q71"/>
+  <dimension ref="A1:Q73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -2302,7 +2302,7 @@
       </c>
       <c r="G17" s="16" t="inlineStr">
         <is>
-          <t>Audit trail — financially-relevant create/update/delete logged with user, timestamp, before/after.</t>
+          <t>Audit trail — every mutating request logged with user, timestamp, IP, action, status (field-level before/after is ITGC-AC-14).</t>
         </is>
       </c>
       <c r="H17" s="17" t="inlineStr">
@@ -2620,12 +2620,12 @@
     <row r="21">
       <c r="A21" s="15" t="inlineStr">
         <is>
-          <t>ITGC-CM-01</t>
+          <t>ITGC-AC-14</t>
         </is>
       </c>
       <c r="B21" s="16" t="inlineStr">
         <is>
-          <t>ITGC · Change</t>
+          <t>ITGC · Access</t>
         </is>
       </c>
       <c r="C21" s="17" t="inlineStr">
@@ -2635,67 +2635,67 @@
       </c>
       <c r="D21" s="16" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Revenue / Cash; Expenditure</t>
         </is>
       </c>
       <c r="E21" s="16" t="inlineStr">
         <is>
-          <t>Unauthorized/untested code reaches production.</t>
+          <t>Financial data changed without a field-level record of WHAT changed (old→new).</t>
         </is>
       </c>
       <c r="F21" s="16" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Completeness/Integrity</t>
         </is>
       </c>
       <c r="G21" s="16" t="inlineStr">
         <is>
-          <t>All code changes via peer-reviewed PR; branch protection on main; no self-merge; CI must pass before merge.</t>
+          <t>Field-level change log — DB triggers capture OLD/NEW row images + changed columns + actor on every INSERT/UPDATE/DELETE of the core financial tables (GL header, AP/AR sub-ledgers, AP payments, tenders); append-only.</t>
         </is>
       </c>
       <c r="H21" s="17" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I21" s="17" t="inlineStr">
         <is>
-          <t>Auto+Manual</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J21" s="17" t="inlineStr">
         <is>
-          <t>Per change</t>
+          <t>Continuous</t>
         </is>
       </c>
       <c r="K21" s="16" t="inlineStr">
         <is>
-          <t>Head of Eng</t>
+          <t>Eng Lead</t>
         </is>
       </c>
       <c r="L21" s="17" t="inlineStr">
         <is>
-          <t>P11</t>
+          <t>P13/P16</t>
         </is>
       </c>
       <c r="M21" s="16" t="inlineStr">
         <is>
-          <t>.github/rulesets/main-branch-protection.json; .github/CODEOWNERS</t>
+          <t>drizzle/0116_field_change_log.sql (log_data_change triggers; data_change_log append-only); tenant-tx.interceptor.ts (app.actor GUC); audit-viewer.service.ts (changes / GET /api/admin/audit/changes); cutover/compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N21" s="16" t="inlineStr">
         <is>
-          <t>Inspect branch protection + required-review settings.</t>
+          <t>Inspect trigger coverage + actor capture; verify append-only trigger.</t>
         </is>
       </c>
       <c r="O21" s="16" t="inlineStr">
         <is>
-          <t>Sample merges: independent + code-owner approval + green CI; no force-push.</t>
+          <t>Sample a financial update → change log holds old/new + changed columns + actor; UPDATE/DELETE on data_change_log rejected (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P21" s="16" t="inlineStr">
         <is>
-          <t>PR approvals</t>
+          <t>Field change log</t>
         </is>
       </c>
       <c r="Q21" s="19" t="inlineStr">
@@ -2707,7 +2707,7 @@
     <row r="22">
       <c r="A22" s="11" t="inlineStr">
         <is>
-          <t>ITGC-CM-02</t>
+          <t>ITGC-CM-01</t>
         </is>
       </c>
       <c r="B22" s="12" t="inlineStr">
@@ -2727,7 +2727,7 @@
       </c>
       <c r="E22" s="12" t="inlineStr">
         <is>
-          <t>Ad-hoc prod schema change corrupts data.</t>
+          <t>Unauthorized/untested code reaches production.</t>
         </is>
       </c>
       <c r="F22" s="12" t="inlineStr">
@@ -2737,7 +2737,7 @@
       </c>
       <c r="G22" s="12" t="inlineStr">
         <is>
-          <t>Schema changes only via reviewed Drizzle migrations; no direct prod DDL; migration journal maintained.</t>
+          <t>All code changes via peer-reviewed PR; branch protection on main; no self-merge; CI must pass before merge.</t>
         </is>
       </c>
       <c r="H22" s="13" t="inlineStr">
@@ -2757,7 +2757,7 @@
       </c>
       <c r="K22" s="12" t="inlineStr">
         <is>
-          <t>Head of Eng / DBA</t>
+          <t>Head of Eng</t>
         </is>
       </c>
       <c r="L22" s="13" t="inlineStr">
@@ -2767,22 +2767,22 @@
       </c>
       <c r="M22" s="12" t="inlineStr">
         <is>
-          <t>apps/api/drizzle/*; meta/_journal.json; CODEOWNERS on drizzle/</t>
+          <t>.github/rulesets/main-branch-protection.json; .github/CODEOWNERS</t>
         </is>
       </c>
       <c r="N22" s="12" t="inlineStr">
         <is>
-          <t>Inspect migration process + journal.</t>
+          <t>Inspect branch protection + required-review settings.</t>
         </is>
       </c>
       <c r="O22" s="12" t="inlineStr">
         <is>
-          <t>Sample migrations: code-owner reviewed + applied via pipeline only.</t>
+          <t>Sample merges: independent + code-owner approval + green CI; no force-push.</t>
         </is>
       </c>
       <c r="P22" s="12" t="inlineStr">
         <is>
-          <t>Migration log</t>
+          <t>PR approvals</t>
         </is>
       </c>
       <c r="Q22" s="19" t="inlineStr">
@@ -2794,7 +2794,7 @@
     <row r="23">
       <c r="A23" s="15" t="inlineStr">
         <is>
-          <t>ITGC-CM-03</t>
+          <t>ITGC-CM-02</t>
         </is>
       </c>
       <c r="B23" s="16" t="inlineStr">
@@ -2814,7 +2814,7 @@
       </c>
       <c r="E23" s="16" t="inlineStr">
         <is>
-          <t>Developer self-deploys unreviewed change to prod.</t>
+          <t>Ad-hoc prod schema change corrupts data.</t>
         </is>
       </c>
       <c r="F23" s="16" t="inlineStr">
@@ -2824,7 +2824,7 @@
       </c>
       <c r="G23" s="16" t="inlineStr">
         <is>
-          <t>Segregation: developer ≠ prod deployer; production deploy requires separate approval.</t>
+          <t>Schema changes only via reviewed Drizzle migrations; no direct prod DDL; migration journal maintained.</t>
         </is>
       </c>
       <c r="H23" s="17" t="inlineStr">
@@ -2834,7 +2834,7 @@
       </c>
       <c r="I23" s="17" t="inlineStr">
         <is>
-          <t>Manual</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="J23" s="17" t="inlineStr">
@@ -2844,7 +2844,7 @@
       </c>
       <c r="K23" s="16" t="inlineStr">
         <is>
-          <t>Head of Eng</t>
+          <t>Head of Eng / DBA</t>
         </is>
       </c>
       <c r="L23" s="17" t="inlineStr">
@@ -2854,22 +2854,22 @@
       </c>
       <c r="M23" s="16" t="inlineStr">
         <is>
-          <t>.github/workflows/deploy.yml (production environment required reviewers)</t>
+          <t>apps/api/drizzle/*; meta/_journal.json; CODEOWNERS on drizzle/</t>
         </is>
       </c>
       <c r="N23" s="16" t="inlineStr">
         <is>
-          <t>Inspect deploy approval gate + role separation.</t>
+          <t>Inspect migration process + journal.</t>
         </is>
       </c>
       <c r="O23" s="16" t="inlineStr">
         <is>
-          <t>Sample deploys: approver ≠ author.</t>
+          <t>Sample migrations: code-owner reviewed + applied via pipeline only.</t>
         </is>
       </c>
       <c r="P23" s="16" t="inlineStr">
         <is>
-          <t>Deploy approvals</t>
+          <t>Migration log</t>
         </is>
       </c>
       <c r="Q23" s="19" t="inlineStr">
@@ -2881,7 +2881,7 @@
     <row r="24">
       <c r="A24" s="11" t="inlineStr">
         <is>
-          <t>ITGC-CM-04</t>
+          <t>ITGC-CM-03</t>
         </is>
       </c>
       <c r="B24" s="12" t="inlineStr">
@@ -2901,7 +2901,7 @@
       </c>
       <c r="E24" s="12" t="inlineStr">
         <is>
-          <t>Changes not traceable to an authorized request.</t>
+          <t>Developer self-deploys unreviewed change to prod.</t>
         </is>
       </c>
       <c r="F24" s="12" t="inlineStr">
@@ -2911,12 +2911,12 @@
       </c>
       <c r="G24" s="12" t="inlineStr">
         <is>
-          <t>Change traceability: ticket → PR → test → deploy linkage retained for every change.</t>
+          <t>Segregation: developer ≠ prod deployer; production deploy requires separate approval.</t>
         </is>
       </c>
       <c r="H24" s="13" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I24" s="13" t="inlineStr">
@@ -2941,22 +2941,22 @@
       </c>
       <c r="M24" s="12" t="inlineStr">
         <is>
-          <t>.github/pull_request_template.md (required linked ticket)</t>
+          <t>.github/workflows/deploy.yml (production environment required reviewers)</t>
         </is>
       </c>
       <c r="N24" s="12" t="inlineStr">
         <is>
-          <t>Inspect linkage convention.</t>
+          <t>Inspect deploy approval gate + role separation.</t>
         </is>
       </c>
       <c r="O24" s="12" t="inlineStr">
         <is>
-          <t>Sample changes traced ticket→PR→deploy.</t>
+          <t>Sample deploys: approver ≠ author.</t>
         </is>
       </c>
       <c r="P24" s="12" t="inlineStr">
         <is>
-          <t>Traceability</t>
+          <t>Deploy approvals</t>
         </is>
       </c>
       <c r="Q24" s="19" t="inlineStr">
@@ -2968,7 +2968,7 @@
     <row r="25">
       <c r="A25" s="15" t="inlineStr">
         <is>
-          <t>ITGC-CM-05</t>
+          <t>ITGC-CM-04</t>
         </is>
       </c>
       <c r="B25" s="16" t="inlineStr">
@@ -2988,7 +2988,7 @@
       </c>
       <c r="E25" s="16" t="inlineStr">
         <is>
-          <t>Emergency fixes bypass controls permanently.</t>
+          <t>Changes not traceable to an authorized request.</t>
         </is>
       </c>
       <c r="F25" s="16" t="inlineStr">
@@ -2998,12 +2998,12 @@
       </c>
       <c r="G25" s="16" t="inlineStr">
         <is>
-          <t>Emergency-change procedure with retroactive review/approval within defined SLA.</t>
+          <t>Change traceability: ticket → PR → test → deploy linkage retained for every change.</t>
         </is>
       </c>
       <c r="H25" s="17" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I25" s="17" t="inlineStr">
@@ -3013,7 +3013,7 @@
       </c>
       <c r="J25" s="17" t="inlineStr">
         <is>
-          <t>As needed</t>
+          <t>Per change</t>
         </is>
       </c>
       <c r="K25" s="16" t="inlineStr">
@@ -3028,22 +3028,22 @@
       </c>
       <c r="M25" s="16" t="inlineStr">
         <is>
-          <t>docs/ops/change-management.md (emergency-change procedure)</t>
+          <t>.github/pull_request_template.md (required linked ticket)</t>
         </is>
       </c>
       <c r="N25" s="16" t="inlineStr">
         <is>
-          <t>Inspect emergency procedure.</t>
+          <t>Inspect linkage convention.</t>
         </is>
       </c>
       <c r="O25" s="16" t="inlineStr">
         <is>
-          <t>Sample emergency changes had expedited review + 1-day retro.</t>
+          <t>Sample changes traced ticket→PR→deploy.</t>
         </is>
       </c>
       <c r="P25" s="16" t="inlineStr">
         <is>
-          <t>Emergency log</t>
+          <t>Traceability</t>
         </is>
       </c>
       <c r="Q25" s="19" t="inlineStr">
@@ -3055,12 +3055,12 @@
     <row r="26">
       <c r="A26" s="11" t="inlineStr">
         <is>
-          <t>ITGC-SD-01</t>
+          <t>ITGC-CM-05</t>
         </is>
       </c>
       <c r="B26" s="12" t="inlineStr">
         <is>
-          <t>ITGC · SDLC</t>
+          <t>ITGC · Change</t>
         </is>
       </c>
       <c r="C26" s="13" t="inlineStr">
@@ -3075,7 +3075,7 @@
       </c>
       <c r="E26" s="12" t="inlineStr">
         <is>
-          <t>New functionality goes live without design/test sign-off.</t>
+          <t>Emergency fixes bypass controls permanently.</t>
         </is>
       </c>
       <c r="F26" s="12" t="inlineStr">
@@ -3085,7 +3085,7 @@
       </c>
       <c r="G26" s="12" t="inlineStr">
         <is>
-          <t>SDLC policy: requirements, design, test and UAT sign-off prior to go-live.</t>
+          <t>Emergency-change procedure with retroactive review/approval within defined SLA.</t>
         </is>
       </c>
       <c r="H26" s="13" t="inlineStr">
@@ -3100,12 +3100,12 @@
       </c>
       <c r="J26" s="13" t="inlineStr">
         <is>
-          <t>Per project</t>
+          <t>As needed</t>
         </is>
       </c>
       <c r="K26" s="12" t="inlineStr">
         <is>
-          <t>Head of Eng / Product</t>
+          <t>Head of Eng</t>
         </is>
       </c>
       <c r="L26" s="13" t="inlineStr">
@@ -3115,34 +3115,34 @@
       </c>
       <c r="M26" s="12" t="inlineStr">
         <is>
-          <t>SDLC policy (to author)</t>
+          <t>docs/ops/change-management.md (emergency-change procedure)</t>
         </is>
       </c>
       <c r="N26" s="12" t="inlineStr">
         <is>
-          <t>Inspect SDLC policy + a project's artefacts.</t>
+          <t>Inspect emergency procedure.</t>
         </is>
       </c>
       <c r="O26" s="12" t="inlineStr">
         <is>
-          <t>Sample releases: UAT + go-live sign-off present.</t>
+          <t>Sample emergency changes had expedited review + 1-day retro.</t>
         </is>
       </c>
       <c r="P26" s="12" t="inlineStr">
         <is>
-          <t>SDLC artefacts</t>
-        </is>
-      </c>
-      <c r="Q26" s="14" t="inlineStr">
-        <is>
-          <t>Gap</t>
+          <t>Emergency log</t>
+        </is>
+      </c>
+      <c r="Q26" s="19" t="inlineStr">
+        <is>
+          <t>Implemented</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="15" t="inlineStr">
         <is>
-          <t>ITGC-SD-02</t>
+          <t>ITGC-SD-01</t>
         </is>
       </c>
       <c r="B27" s="16" t="inlineStr">
@@ -3162,74 +3162,74 @@
       </c>
       <c r="E27" s="16" t="inlineStr">
         <is>
-          <t>Migrated opening balances incomplete/inaccurate.</t>
+          <t>New functionality goes live without design/test sign-off.</t>
         </is>
       </c>
       <c r="F27" s="16" t="inlineStr">
         <is>
-          <t>Completeness/Accuracy</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G27" s="16" t="inlineStr">
         <is>
-          <t>Cutover data-migration controls: source→target balance reconciliation + sign-off; opening balances idempotent.</t>
+          <t>SDLC policy: requirements, design, test and UAT sign-off prior to go-live.</t>
         </is>
       </c>
       <c r="H27" s="17" t="inlineStr">
         <is>
-          <t>Prev/Det</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I27" s="17" t="inlineStr">
         <is>
-          <t>Auto+Manual</t>
+          <t>Manual</t>
         </is>
       </c>
       <c r="J27" s="17" t="inlineStr">
         <is>
-          <t>At cutover</t>
+          <t>Per project</t>
         </is>
       </c>
       <c r="K27" s="16" t="inlineStr">
         <is>
-          <t>Controller / Eng</t>
+          <t>Head of Eng / Product</t>
         </is>
       </c>
       <c r="L27" s="17" t="inlineStr">
         <is>
-          <t>P11/P13</t>
+          <t>P11</t>
         </is>
       </c>
       <c r="M27" s="16" t="inlineStr">
         <is>
-          <t>tools/etl; tools/cutover; ledger opening-balances (idempotent on batch_ref)</t>
+          <t>SDLC policy (to author)</t>
         </is>
       </c>
       <c r="N27" s="16" t="inlineStr">
         <is>
-          <t>Inspect migration reconciliation + sign-off.</t>
+          <t>Inspect SDLC policy + a project's artefacts.</t>
         </is>
       </c>
       <c r="O27" s="16" t="inlineStr">
         <is>
-          <t>Re-perform migrated trial-balance tie-out.</t>
+          <t>Sample releases: UAT + go-live sign-off present.</t>
         </is>
       </c>
       <c r="P27" s="16" t="inlineStr">
         <is>
-          <t>Migration recon</t>
-        </is>
-      </c>
-      <c r="Q27" s="18" t="inlineStr">
-        <is>
-          <t>Partial</t>
+          <t>SDLC artefacts</t>
+        </is>
+      </c>
+      <c r="Q27" s="14" t="inlineStr">
+        <is>
+          <t>Gap</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="11" t="inlineStr">
         <is>
-          <t>ITGC-SD-03</t>
+          <t>ITGC-SD-02</t>
         </is>
       </c>
       <c r="B28" s="12" t="inlineStr">
@@ -3249,62 +3249,62 @@
       </c>
       <c r="E28" s="12" t="inlineStr">
         <is>
-          <t>Control logic regresses unnoticed.</t>
+          <t>Migrated opening balances incomplete/inaccurate.</t>
         </is>
       </c>
       <c r="F28" s="12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Completeness/Accuracy</t>
         </is>
       </c>
       <c r="G28" s="12" t="inlineStr">
         <is>
-          <t>Automated test suite is control evidence; CI archives dated results; key-control assertions covered.</t>
+          <t>Cutover data-migration controls: source→target balance reconciliation + sign-off; opening balances idempotent.</t>
         </is>
       </c>
       <c r="H28" s="13" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Prev/Det</t>
         </is>
       </c>
       <c r="I28" s="13" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="J28" s="13" t="inlineStr">
         <is>
-          <t>Per change</t>
+          <t>At cutover</t>
         </is>
       </c>
       <c r="K28" s="12" t="inlineStr">
         <is>
-          <t>Head of Eng</t>
+          <t>Controller / Eng</t>
         </is>
       </c>
       <c r="L28" s="13" t="inlineStr">
         <is>
-          <t>P11/P16</t>
+          <t>P11/P13</t>
         </is>
       </c>
       <c r="M28" s="12" t="inlineStr">
         <is>
-          <t>apps/api/test/unit.test.ts; vitest</t>
+          <t>tools/etl; tools/cutover; ledger opening-balances (idempotent on batch_ref)</t>
         </is>
       </c>
       <c r="N28" s="12" t="inlineStr">
         <is>
-          <t>Inspect tests map to key controls.</t>
+          <t>Inspect migration reconciliation + sign-off.</t>
         </is>
       </c>
       <c r="O28" s="12" t="inlineStr">
         <is>
-          <t>Review archived CI runs over period; all green.</t>
+          <t>Re-perform migrated trial-balance tie-out.</t>
         </is>
       </c>
       <c r="P28" s="12" t="inlineStr">
         <is>
-          <t>CI reports</t>
+          <t>Migration recon</t>
         </is>
       </c>
       <c r="Q28" s="18" t="inlineStr">
@@ -3316,12 +3316,12 @@
     <row r="29">
       <c r="A29" s="15" t="inlineStr">
         <is>
-          <t>ITGC-OP-01</t>
+          <t>ITGC-SD-03</t>
         </is>
       </c>
       <c r="B29" s="16" t="inlineStr">
         <is>
-          <t>ITGC · Operations</t>
+          <t>ITGC · SDLC</t>
         </is>
       </c>
       <c r="C29" s="17" t="inlineStr">
@@ -3336,7 +3336,7 @@
       </c>
       <c r="E29" s="16" t="inlineStr">
         <is>
-          <t>Data loss with no recovery.</t>
+          <t>Control logic regresses unnoticed.</t>
         </is>
       </c>
       <c r="F29" s="16" t="inlineStr">
@@ -3346,64 +3346,64 @@
       </c>
       <c r="G29" s="16" t="inlineStr">
         <is>
-          <t>Automated DB backups + a TESTED quarterly restore (recovery proven, not just scheduled).</t>
+          <t>Automated test suite is control evidence; CI archives dated results; key-control assertions covered.</t>
         </is>
       </c>
       <c r="H29" s="17" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I29" s="17" t="inlineStr">
         <is>
-          <t>Auto+Manual</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J29" s="17" t="inlineStr">
         <is>
-          <t>Daily / Qtrly test</t>
+          <t>Per change</t>
         </is>
       </c>
       <c r="K29" s="16" t="inlineStr">
         <is>
-          <t>DevOps</t>
+          <t>Head of Eng</t>
         </is>
       </c>
       <c r="L29" s="17" t="inlineStr">
         <is>
-          <t>P11</t>
+          <t>P11/P16</t>
         </is>
       </c>
       <c r="M29" s="16" t="inlineStr">
         <is>
-          <t>tools/ops/pg-backup.sh, restore.sh, verify-restore.sh; BACKUP-RUNBOOK.md</t>
+          <t>apps/api/test/unit.test.ts; vitest</t>
         </is>
       </c>
       <c r="N29" s="16" t="inlineStr">
         <is>
-          <t>Inspect backup schedule + scripted restore-drill procedure.</t>
+          <t>Inspect tests map to key controls.</t>
         </is>
       </c>
       <c r="O29" s="16" t="inlineStr">
         <is>
-          <t>Inspect a successful restore-drill record each quarter.</t>
+          <t>Review archived CI runs over period; all green.</t>
         </is>
       </c>
       <c r="P29" s="16" t="inlineStr">
         <is>
-          <t>Restore test</t>
-        </is>
-      </c>
-      <c r="Q29" s="19" t="inlineStr">
-        <is>
-          <t>Implemented</t>
+          <t>CI reports</t>
+        </is>
+      </c>
+      <c r="Q29" s="18" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="11" t="inlineStr">
         <is>
-          <t>ITGC-OP-02</t>
+          <t>ITGC-OP-01</t>
         </is>
       </c>
       <c r="B30" s="12" t="inlineStr">
@@ -3423,7 +3423,7 @@
       </c>
       <c r="E30" s="12" t="inlineStr">
         <is>
-          <t>Prolonged outage; no continuity plan.</t>
+          <t>Data loss with no recovery.</t>
         </is>
       </c>
       <c r="F30" s="12" t="inlineStr">
@@ -3433,7 +3433,7 @@
       </c>
       <c r="G30" s="12" t="inlineStr">
         <is>
-          <t>DR / BCP plan with defined RTO/RPO and periodic test.</t>
+          <t>Automated DB backups + a TESTED quarterly restore (recovery proven, not just scheduled).</t>
         </is>
       </c>
       <c r="H30" s="13" t="inlineStr">
@@ -3443,17 +3443,17 @@
       </c>
       <c r="I30" s="13" t="inlineStr">
         <is>
-          <t>Manual</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="J30" s="13" t="inlineStr">
         <is>
-          <t>Annual test</t>
+          <t>Daily / Qtrly test</t>
         </is>
       </c>
       <c r="K30" s="12" t="inlineStr">
         <is>
-          <t>CTO / DevOps</t>
+          <t>DevOps</t>
         </is>
       </c>
       <c r="L30" s="13" t="inlineStr">
@@ -3463,34 +3463,34 @@
       </c>
       <c r="M30" s="12" t="inlineStr">
         <is>
-          <t>RTO/RPO in tools/ops/BACKUP-RUNBOOK.md; full DR/BCP to author</t>
+          <t>tools/ops/pg-backup.sh, restore.sh, verify-restore.sh; BACKUP-RUNBOOK.md</t>
         </is>
       </c>
       <c r="N30" s="12" t="inlineStr">
         <is>
-          <t>Inspect DR plan + RTO/RPO.</t>
+          <t>Inspect backup schedule + scripted restore-drill procedure.</t>
         </is>
       </c>
       <c r="O30" s="12" t="inlineStr">
         <is>
-          <t>Inspect DR test results.</t>
+          <t>Inspect a successful restore-drill record each quarter.</t>
         </is>
       </c>
       <c r="P30" s="12" t="inlineStr">
         <is>
-          <t>DR test</t>
-        </is>
-      </c>
-      <c r="Q30" s="18" t="inlineStr">
-        <is>
-          <t>Partial</t>
+          <t>Restore test</t>
+        </is>
+      </c>
+      <c r="Q30" s="19" t="inlineStr">
+        <is>
+          <t>Implemented</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="15" t="inlineStr">
         <is>
-          <t>ITGC-OP-03</t>
+          <t>ITGC-OP-02</t>
         </is>
       </c>
       <c r="B31" s="16" t="inlineStr">
@@ -3510,7 +3510,7 @@
       </c>
       <c r="E31" s="16" t="inlineStr">
         <is>
-          <t>Failures/incidents undetected.</t>
+          <t>Prolonged outage; no continuity plan.</t>
         </is>
       </c>
       <c r="F31" s="16" t="inlineStr">
@@ -3520,64 +3520,64 @@
       </c>
       <c r="G31" s="16" t="inlineStr">
         <is>
-          <t>Monitoring + alerting (APM/errors) with on-call and an incident-management log.</t>
+          <t>DR / BCP plan with defined RTO/RPO and periodic test.</t>
         </is>
       </c>
       <c r="H31" s="17" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I31" s="17" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Manual</t>
         </is>
       </c>
       <c r="J31" s="17" t="inlineStr">
         <is>
-          <t>Continuous</t>
+          <t>Annual test</t>
         </is>
       </c>
       <c r="K31" s="16" t="inlineStr">
         <is>
-          <t>DevOps</t>
+          <t>CTO / DevOps</t>
         </is>
       </c>
       <c r="L31" s="17" t="inlineStr">
         <is>
-          <t>P11/P16</t>
+          <t>P11</t>
         </is>
       </c>
       <c r="M31" s="16" t="inlineStr">
         <is>
-          <t>observability/instrumentation.ts (OTel); Sentry; docs/ops/observability-incident.md; /healthz+/readyz probes</t>
+          <t>RTO/RPO in tools/ops/BACKUP-RUNBOOK.md; full DR/BCP to author</t>
         </is>
       </c>
       <c r="N31" s="16" t="inlineStr">
         <is>
-          <t>Inspect alerting config + incident process.</t>
+          <t>Inspect DR plan + RTO/RPO.</t>
         </is>
       </c>
       <c r="O31" s="16" t="inlineStr">
         <is>
-          <t>Sample alerts → incident tickets resolved.</t>
+          <t>Inspect DR test results.</t>
         </is>
       </c>
       <c r="P31" s="16" t="inlineStr">
         <is>
-          <t>Incident log</t>
-        </is>
-      </c>
-      <c r="Q31" s="19" t="inlineStr">
-        <is>
-          <t>Implemented</t>
+          <t>DR test</t>
+        </is>
+      </c>
+      <c r="Q31" s="18" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="11" t="inlineStr">
         <is>
-          <t>ITGC-OP-04</t>
+          <t>ITGC-OP-03</t>
         </is>
       </c>
       <c r="B32" s="12" t="inlineStr">
@@ -3592,22 +3592,22 @@
       </c>
       <c r="D32" s="12" t="inlineStr">
         <is>
-          <t>Revenue / GL</t>
+          <t>All</t>
         </is>
       </c>
       <c r="E32" s="12" t="inlineStr">
         <is>
-          <t>Scheduled financial jobs fail silently (missed billing/postings).</t>
+          <t>Failures/incidents undetected.</t>
         </is>
       </c>
       <c r="F32" s="12" t="inlineStr">
         <is>
-          <t>Completeness</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G32" s="12" t="inlineStr">
         <is>
-          <t>Batch-job monitoring (recurring billing, FX revaluation, subscriptions) with failure alerting + review.</t>
+          <t>Monitoring + alerting (APM/errors) with on-call and an incident-management log.</t>
         </is>
       </c>
       <c r="H32" s="13" t="inlineStr">
@@ -3622,84 +3622,84 @@
       </c>
       <c r="J32" s="13" t="inlineStr">
         <is>
-          <t>Per run</t>
+          <t>Continuous</t>
         </is>
       </c>
       <c r="K32" s="12" t="inlineStr">
         <is>
-          <t>DevOps / Controller</t>
+          <t>DevOps</t>
         </is>
       </c>
       <c r="L32" s="13" t="inlineStr">
         <is>
-          <t>P11</t>
+          <t>P11/P16</t>
         </is>
       </c>
       <c r="M32" s="12" t="inlineStr">
         <is>
-          <t>billing; fx; service modules; alert spec in docs/ops/observability-incident.md</t>
+          <t>observability/instrumentation.ts (OTel); Sentry; docs/ops/observability-incident.md; /healthz+/readyz probes</t>
         </is>
       </c>
       <c r="N32" s="12" t="inlineStr">
         <is>
-          <t>Inspect job inventory + alerting.</t>
+          <t>Inspect alerting config + incident process.</t>
         </is>
       </c>
       <c r="O32" s="12" t="inlineStr">
         <is>
-          <t>Sample runs: success logged; failures investigated.</t>
+          <t>Sample alerts → incident tickets resolved.</t>
         </is>
       </c>
       <c r="P32" s="12" t="inlineStr">
         <is>
-          <t>Job logs</t>
-        </is>
-      </c>
-      <c r="Q32" s="18" t="inlineStr">
-        <is>
-          <t>Partial</t>
+          <t>Incident log</t>
+        </is>
+      </c>
+      <c r="Q32" s="19" t="inlineStr">
+        <is>
+          <t>Implemented</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="15" t="inlineStr">
         <is>
-          <t>REV-01</t>
+          <t>ITGC-OP-04</t>
         </is>
       </c>
       <c r="B33" s="16" t="inlineStr">
         <is>
-          <t>Revenue &amp; Cash</t>
+          <t>ITGC · Operations</t>
         </is>
       </c>
       <c r="C33" s="17" t="inlineStr">
         <is>
-          <t>Application</t>
+          <t>ITGC</t>
         </is>
       </c>
       <c r="D33" s="16" t="inlineStr">
         <is>
-          <t>Revenue; Cash</t>
+          <t>Revenue / GL</t>
         </is>
       </c>
       <c r="E33" s="16" t="inlineStr">
         <is>
-          <t>Invalid/garbage data posted (negatives, wrong types).</t>
+          <t>Scheduled financial jobs fail silently (missed billing/postings).</t>
         </is>
       </c>
       <c r="F33" s="16" t="inlineStr">
         <is>
-          <t>Accuracy/Validity</t>
+          <t>Completeness</t>
         </is>
       </c>
       <c r="G33" s="16" t="inlineStr">
         <is>
-          <t>Zod schema validation on all sales/tender inputs (qty&gt;0, price&gt;=0, amount&gt;0); standard error envelope.</t>
+          <t>Batch-job monitoring (recurring billing, FX revaluation, subscriptions) with failure alerting + review.</t>
         </is>
       </c>
       <c r="H33" s="17" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I33" s="17" t="inlineStr">
@@ -3709,49 +3709,49 @@
       </c>
       <c r="J33" s="17" t="inlineStr">
         <is>
-          <t>Per txn</t>
+          <t>Per run</t>
         </is>
       </c>
       <c r="K33" s="16" t="inlineStr">
         <is>
-          <t>Eng Lead</t>
+          <t>DevOps / Controller</t>
         </is>
       </c>
       <c r="L33" s="17" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P11</t>
         </is>
       </c>
       <c r="M33" s="16" t="inlineStr">
         <is>
-          <t>pos.controller.ts; payments.controller.ts; common/zod-validation.pipe.ts</t>
+          <t>billing; fx; service modules; alert spec in docs/ops/observability-incident.md</t>
         </is>
       </c>
       <c r="N33" s="16" t="inlineStr">
         <is>
-          <t>Inspect schemas; submit invalid payload → 400.</t>
+          <t>Inspect job inventory + alerting.</t>
         </is>
       </c>
       <c r="O33" s="16" t="inlineStr">
         <is>
-          <t>Re-perform invalid-input sample → rejected.</t>
+          <t>Sample runs: success logged; failures investigated.</t>
         </is>
       </c>
       <c r="P33" s="16" t="inlineStr">
         <is>
-          <t>Validation tests</t>
-        </is>
-      </c>
-      <c r="Q33" s="19" t="inlineStr">
-        <is>
-          <t>Implemented</t>
+          <t>Job logs</t>
+        </is>
+      </c>
+      <c r="Q33" s="18" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="11" t="inlineStr">
         <is>
-          <t>REV-02</t>
+          <t>REV-01</t>
         </is>
       </c>
       <c r="B34" s="12" t="inlineStr">
@@ -3766,22 +3766,22 @@
       </c>
       <c r="D34" s="12" t="inlineStr">
         <is>
-          <t>Cash</t>
+          <t>Revenue; Cash</t>
         </is>
       </c>
       <c r="E34" s="12" t="inlineStr">
         <is>
-          <t>Retried/double-submitted tender charges customer twice.</t>
+          <t>Invalid/garbage data posted (negatives, wrong types).</t>
         </is>
       </c>
       <c r="F34" s="12" t="inlineStr">
         <is>
-          <t>Occurrence/Completeness</t>
+          <t>Accuracy/Validity</t>
         </is>
       </c>
       <c r="G34" s="12" t="inlineStr">
         <is>
-          <t>Payment idempotency — same idempotency_key returns the original tender; unique index backstops the race.</t>
+          <t>Zod schema validation on all sales/tender inputs (qty&gt;0, price&gt;=0, amount&gt;0); standard error envelope.</t>
         </is>
       </c>
       <c r="H34" s="13" t="inlineStr">
@@ -3811,22 +3811,22 @@
       </c>
       <c r="M34" s="12" t="inlineStr">
         <is>
-          <t>payments.service.ts (recordTender); schema/payments.ts (ux_payments_idem); migration 0057</t>
+          <t>pos.controller.ts; payments.controller.ts; common/zod-validation.pipe.ts</t>
         </is>
       </c>
       <c r="N34" s="12" t="inlineStr">
         <is>
-          <t>Inspect key handling + unique index.</t>
+          <t>Inspect schemas; submit invalid payload → 400.</t>
         </is>
       </c>
       <c r="O34" s="12" t="inlineStr">
         <is>
-          <t>Re-submit same key → single charge; concurrent test.</t>
+          <t>Re-perform invalid-input sample → rejected.</t>
         </is>
       </c>
       <c r="P34" s="12" t="inlineStr">
         <is>
-          <t>Idempotency test</t>
+          <t>Validation tests</t>
         </is>
       </c>
       <c r="Q34" s="19" t="inlineStr">
@@ -3838,7 +3838,7 @@
     <row r="35">
       <c r="A35" s="15" t="inlineStr">
         <is>
-          <t>REV-03</t>
+          <t>REV-02</t>
         </is>
       </c>
       <c r="B35" s="16" t="inlineStr">
@@ -3858,17 +3858,17 @@
       </c>
       <c r="E35" s="16" t="inlineStr">
         <is>
-          <t>Funds captured at gateway but no record (orphaned charge).</t>
+          <t>Retried/double-submitted tender charges customer twice.</t>
         </is>
       </c>
       <c r="F35" s="16" t="inlineStr">
         <is>
-          <t>Completeness</t>
+          <t>Occurrence/Completeness</t>
         </is>
       </c>
       <c r="G35" s="16" t="inlineStr">
         <is>
-          <t>Row persisted Pending BEFORE gateway capture; flipped Failed on error — no unrecorded captured funds.</t>
+          <t>Payment idempotency — same idempotency_key returns the original tender; unique index backstops the race.</t>
         </is>
       </c>
       <c r="H35" s="17" t="inlineStr">
@@ -3898,22 +3898,22 @@
       </c>
       <c r="M35" s="16" t="inlineStr">
         <is>
-          <t>payments.service.ts (recordTender)</t>
+          <t>payments.service.ts (recordTender); schema/payments.ts (ux_payments_idem); migration 0057</t>
         </is>
       </c>
       <c r="N35" s="16" t="inlineStr">
         <is>
-          <t>Inspect pre-persist + error path.</t>
+          <t>Inspect key handling + unique index.</t>
         </is>
       </c>
       <c r="O35" s="16" t="inlineStr">
         <is>
-          <t>Simulate capture/persist failure → no orphan.</t>
+          <t>Re-submit same key → single charge; concurrent test.</t>
         </is>
       </c>
       <c r="P35" s="16" t="inlineStr">
         <is>
-          <t>Negative test</t>
+          <t>Idempotency test</t>
         </is>
       </c>
       <c r="Q35" s="19" t="inlineStr">
@@ -3925,7 +3925,7 @@
     <row r="36">
       <c r="A36" s="11" t="inlineStr">
         <is>
-          <t>REV-04</t>
+          <t>REV-03</t>
         </is>
       </c>
       <c r="B36" s="12" t="inlineStr">
@@ -3940,12 +3940,12 @@
       </c>
       <c r="D36" s="12" t="inlineStr">
         <is>
-          <t>Revenue</t>
+          <t>Cash</t>
         </is>
       </c>
       <c r="E36" s="12" t="inlineStr">
         <is>
-          <t>Missing/duplicate sales not detected (completeness).</t>
+          <t>Funds captured at gateway but no record (orphaned charge).</t>
         </is>
       </c>
       <c r="F36" s="12" t="inlineStr">
@@ -3955,7 +3955,7 @@
       </c>
       <c r="G36" s="12" t="inlineStr">
         <is>
-          <t>Sequential, gapless document numbering for sales/payments (per type/day).</t>
+          <t>Row persisted Pending BEFORE gateway capture; flipped Failed on error — no unrecorded captured funds.</t>
         </is>
       </c>
       <c r="H36" s="13" t="inlineStr">
@@ -3980,27 +3980,27 @@
       </c>
       <c r="L36" s="13" t="inlineStr">
         <is>
-          <t>P13</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="M36" s="12" t="inlineStr">
         <is>
-          <t>common/doc-number.service.ts</t>
+          <t>payments.service.ts (recordTender)</t>
         </is>
       </c>
       <c r="N36" s="12" t="inlineStr">
         <is>
-          <t>Inspect numbering scheme.</t>
+          <t>Inspect pre-persist + error path.</t>
         </is>
       </c>
       <c r="O36" s="12" t="inlineStr">
         <is>
-          <t>Sample sequence for gaps/duplicates.</t>
+          <t>Simulate capture/persist failure → no orphan.</t>
         </is>
       </c>
       <c r="P36" s="12" t="inlineStr">
         <is>
-          <t>Doc-no sequence</t>
+          <t>Negative test</t>
         </is>
       </c>
       <c r="Q36" s="19" t="inlineStr">
@@ -4012,7 +4012,7 @@
     <row r="37">
       <c r="A37" s="15" t="inlineStr">
         <is>
-          <t>REV-05</t>
+          <t>REV-04</t>
         </is>
       </c>
       <c r="B37" s="16" t="inlineStr">
@@ -4027,67 +4027,67 @@
       </c>
       <c r="D37" s="16" t="inlineStr">
         <is>
-          <t>Cash</t>
+          <t>Revenue</t>
         </is>
       </c>
       <c r="E37" s="16" t="inlineStr">
         <is>
-          <t>Cash drawer shortages/skimming undetected.</t>
+          <t>Missing/duplicate sales not detected (completeness).</t>
         </is>
       </c>
       <c r="F37" s="16" t="inlineStr">
         <is>
-          <t>Existence/Accuracy</t>
+          <t>Completeness</t>
         </is>
       </c>
       <c r="G37" s="16" t="inlineStr">
         <is>
-          <t>Till reconciliation: opening float, counted vs expected cash, variance + X/Z shift reports.</t>
+          <t>Sequential, gapless document numbering for sales/payments (per type/day).</t>
         </is>
       </c>
       <c r="H37" s="17" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I37" s="17" t="inlineStr">
         <is>
-          <t>Auto+Manual</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J37" s="17" t="inlineStr">
         <is>
-          <t>Per shift</t>
+          <t>Per txn</t>
         </is>
       </c>
       <c r="K37" s="16" t="inlineStr">
         <is>
-          <t>Store Ops Mgr</t>
+          <t>Eng Lead</t>
         </is>
       </c>
       <c r="L37" s="17" t="inlineStr">
         <is>
-          <t>P10/P16</t>
+          <t>P13</t>
         </is>
       </c>
       <c r="M37" s="16" t="inlineStr">
         <is>
-          <t>payments.service.ts (openTill/closeTill/aggregateTill)</t>
+          <t>common/doc-number.service.ts</t>
         </is>
       </c>
       <c r="N37" s="16" t="inlineStr">
         <is>
-          <t>Inspect variance computation.</t>
+          <t>Inspect numbering scheme.</t>
         </is>
       </c>
       <c r="O37" s="16" t="inlineStr">
         <is>
-          <t>Sample shifts: Z-report variance reviewed &amp; signed.</t>
+          <t>Sample sequence for gaps/duplicates.</t>
         </is>
       </c>
       <c r="P37" s="16" t="inlineStr">
         <is>
-          <t>Z-reports</t>
+          <t>Doc-no sequence</t>
         </is>
       </c>
       <c r="Q37" s="19" t="inlineStr">
@@ -4099,7 +4099,7 @@
     <row r="38">
       <c r="A38" s="11" t="inlineStr">
         <is>
-          <t>REV-06</t>
+          <t>REV-05</t>
         </is>
       </c>
       <c r="B38" s="12" t="inlineStr">
@@ -4114,67 +4114,67 @@
       </c>
       <c r="D38" s="12" t="inlineStr">
         <is>
-          <t>Cash; Revenue</t>
+          <t>Cash</t>
         </is>
       </c>
       <c r="E38" s="12" t="inlineStr">
         <is>
-          <t>Refunds exceed original payment (leakage/fraud).</t>
+          <t>Cash drawer shortages/skimming undetected.</t>
         </is>
       </c>
       <c r="F38" s="12" t="inlineStr">
         <is>
-          <t>Validity</t>
+          <t>Existence/Accuracy</t>
         </is>
       </c>
       <c r="G38" s="12" t="inlineStr">
         <is>
-          <t>Over-refund prevention — refund + prior refunds ≤ captured, evaluated under a payment-row lock.</t>
+          <t>Till reconciliation: opening float, counted vs expected cash, variance + X/Z shift reports.</t>
         </is>
       </c>
       <c r="H38" s="13" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I38" s="13" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="J38" s="13" t="inlineStr">
         <is>
-          <t>Per txn</t>
+          <t>Per shift</t>
         </is>
       </c>
       <c r="K38" s="12" t="inlineStr">
         <is>
-          <t>Eng Lead</t>
+          <t>Store Ops Mgr</t>
         </is>
       </c>
       <c r="L38" s="13" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P10/P16</t>
         </is>
       </c>
       <c r="M38" s="12" t="inlineStr">
         <is>
-          <t>payments.service.ts (refund, FOR UPDATE)</t>
+          <t>payments.service.ts (openTill/closeTill/aggregateTill)</t>
         </is>
       </c>
       <c r="N38" s="12" t="inlineStr">
         <is>
-          <t>Inspect lock + cumulative check.</t>
+          <t>Inspect variance computation.</t>
         </is>
       </c>
       <c r="O38" s="12" t="inlineStr">
         <is>
-          <t>Concurrent-refund test cannot exceed captured.</t>
+          <t>Sample shifts: Z-report variance reviewed &amp; signed.</t>
         </is>
       </c>
       <c r="P38" s="12" t="inlineStr">
         <is>
-          <t>Refund test</t>
+          <t>Z-reports</t>
         </is>
       </c>
       <c r="Q38" s="19" t="inlineStr">
@@ -4186,7 +4186,7 @@
     <row r="39">
       <c r="A39" s="15" t="inlineStr">
         <is>
-          <t>REV-07</t>
+          <t>REV-06</t>
         </is>
       </c>
       <c r="B39" s="16" t="inlineStr">
@@ -4201,22 +4201,22 @@
       </c>
       <c r="D39" s="16" t="inlineStr">
         <is>
-          <t>Revenue; Inventory</t>
+          <t>Cash; Revenue</t>
         </is>
       </c>
       <c r="E39" s="16" t="inlineStr">
         <is>
-          <t>Refund posts but stock/GL not reversed (partial state).</t>
+          <t>Refunds exceed original payment (leakage/fraud).</t>
         </is>
       </c>
       <c r="F39" s="16" t="inlineStr">
         <is>
-          <t>Completeness/Accuracy</t>
+          <t>Validity</t>
         </is>
       </c>
       <c r="G39" s="16" t="inlineStr">
         <is>
-          <t>Returns processed atomically — refund + restock + return record + GL reversal in one transaction.</t>
+          <t>Over-refund prevention — refund + prior refunds ≤ captured, evaluated under a payment-row lock.</t>
         </is>
       </c>
       <c r="H39" s="17" t="inlineStr">
@@ -4246,22 +4246,22 @@
       </c>
       <c r="M39" s="16" t="inlineStr">
         <is>
-          <t>returns.service.ts (createReturn)</t>
+          <t>payments.service.ts (refund, FOR UPDATE)</t>
         </is>
       </c>
       <c r="N39" s="16" t="inlineStr">
         <is>
-          <t>Inspect single-transaction boundary.</t>
+          <t>Inspect lock + cumulative check.</t>
         </is>
       </c>
       <c r="O39" s="16" t="inlineStr">
         <is>
-          <t>Inject mid-flow failure → full rollback.</t>
+          <t>Concurrent-refund test cannot exceed captured.</t>
         </is>
       </c>
       <c r="P39" s="16" t="inlineStr">
         <is>
-          <t>Atomicity test</t>
+          <t>Refund test</t>
         </is>
       </c>
       <c r="Q39" s="19" t="inlineStr">
@@ -4273,7 +4273,7 @@
     <row r="40">
       <c r="A40" s="11" t="inlineStr">
         <is>
-          <t>REV-08</t>
+          <t>REV-07</t>
         </is>
       </c>
       <c r="B40" s="12" t="inlineStr">
@@ -4288,22 +4288,22 @@
       </c>
       <c r="D40" s="12" t="inlineStr">
         <is>
-          <t>Accounts Receivable</t>
+          <t>Revenue; Inventory</t>
         </is>
       </c>
       <c r="E40" s="12" t="inlineStr">
         <is>
-          <t>Orders accepted beyond customer credit limit.</t>
+          <t>Refund posts but stock/GL not reversed (partial state).</t>
         </is>
       </c>
       <c r="F40" s="12" t="inlineStr">
         <is>
-          <t>Valuation</t>
+          <t>Completeness/Accuracy</t>
         </is>
       </c>
       <c r="G40" s="12" t="inlineStr">
         <is>
-          <t>Credit-limit check at order — outstanding AR + order ≤ limit, under tenant-row lock; credit-hold block.</t>
+          <t>Returns processed atomically — refund + restock + return record + GL reversal in one transaction.</t>
         </is>
       </c>
       <c r="H40" s="13" t="inlineStr">
@@ -4318,12 +4318,12 @@
       </c>
       <c r="J40" s="13" t="inlineStr">
         <is>
-          <t>Per order</t>
+          <t>Per txn</t>
         </is>
       </c>
       <c r="K40" s="12" t="inlineStr">
         <is>
-          <t>Controller</t>
+          <t>Eng Lead</t>
         </is>
       </c>
       <c r="L40" s="13" t="inlineStr">
@@ -4333,22 +4333,22 @@
       </c>
       <c r="M40" s="12" t="inlineStr">
         <is>
-          <t>pos.service.ts (createOrder, FOR UPDATE); cutover/compliance.ts (ToE)</t>
+          <t>returns.service.ts (createReturn)</t>
         </is>
       </c>
       <c r="N40" s="12" t="inlineStr">
         <is>
-          <t>Inspect AR sum + lock + limit logic.</t>
+          <t>Inspect single-transaction boundary.</t>
         </is>
       </c>
       <c r="O40" s="12" t="inlineStr">
         <is>
-          <t>Sample: outstanding+order ≤ limit allowed, &gt; limit → CREDIT_LIMIT, credit-hold → CREDIT_HOLD (re-performed by the harness).</t>
+          <t>Inject mid-flow failure → full rollback.</t>
         </is>
       </c>
       <c r="P40" s="12" t="inlineStr">
         <is>
-          <t>Credit test</t>
+          <t>Atomicity test</t>
         </is>
       </c>
       <c r="Q40" s="19" t="inlineStr">
@@ -4360,7 +4360,7 @@
     <row r="41">
       <c r="A41" s="15" t="inlineStr">
         <is>
-          <t>REV-09</t>
+          <t>REV-08</t>
         </is>
       </c>
       <c r="B41" s="16" t="inlineStr">
@@ -4375,22 +4375,22 @@
       </c>
       <c r="D41" s="16" t="inlineStr">
         <is>
-          <t>Cash</t>
+          <t>Accounts Receivable</t>
         </is>
       </c>
       <c r="E41" s="16" t="inlineStr">
         <is>
-          <t>Forged payment-gateway callback flips a payment to captured.</t>
+          <t>Orders accepted beyond customer credit limit.</t>
         </is>
       </c>
       <c r="F41" s="16" t="inlineStr">
         <is>
-          <t>Occurrence</t>
+          <t>Valuation</t>
         </is>
       </c>
       <c r="G41" s="16" t="inlineStr">
         <is>
-          <t>PSP webhook HMAC-SHA256 signature over raw body; fail-closed in production; out-of-band status re-verify.</t>
+          <t>Credit-limit check at order — outstanding AR + order ≤ limit, under tenant-row lock; credit-hold block.</t>
         </is>
       </c>
       <c r="H41" s="17" t="inlineStr">
@@ -4405,37 +4405,37 @@
       </c>
       <c r="J41" s="17" t="inlineStr">
         <is>
-          <t>Per callback</t>
+          <t>Per order</t>
         </is>
       </c>
       <c r="K41" s="16" t="inlineStr">
         <is>
-          <t>Eng Lead</t>
+          <t>Controller</t>
         </is>
       </c>
       <c r="L41" s="17" t="inlineStr">
         <is>
-          <t>P10/P11</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="M41" s="16" t="inlineStr">
         <is>
-          <t>pos-terminal.controller.ts (PspWebhookController); crypto.verifyWebhookSignature</t>
+          <t>pos.service.ts (createOrder, FOR UPDATE); cutover/compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N41" s="16" t="inlineStr">
         <is>
-          <t>Inspect signature check + prod gate.</t>
+          <t>Inspect AR sum + lock + limit logic.</t>
         </is>
       </c>
       <c r="O41" s="16" t="inlineStr">
         <is>
-          <t>Replay/forged signature → 401; valid → accepted.</t>
+          <t>Sample: outstanding+order ≤ limit allowed, &gt; limit → CREDIT_LIMIT, credit-hold → CREDIT_HOLD (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P41" s="16" t="inlineStr">
         <is>
-          <t>Webhook tests</t>
+          <t>Credit test</t>
         </is>
       </c>
       <c r="Q41" s="19" t="inlineStr">
@@ -4447,7 +4447,7 @@
     <row r="42">
       <c r="A42" s="11" t="inlineStr">
         <is>
-          <t>REV-10</t>
+          <t>REV-09</t>
         </is>
       </c>
       <c r="B42" s="12" t="inlineStr">
@@ -4462,27 +4462,27 @@
       </c>
       <c r="D42" s="12" t="inlineStr">
         <is>
-          <t>Revenue; Tax</t>
+          <t>Cash</t>
         </is>
       </c>
       <c r="E42" s="12" t="inlineStr">
         <is>
-          <t>Sales not posted to GL or posted unbalanced.</t>
+          <t>Forged payment-gateway callback flips a payment to captured.</t>
         </is>
       </c>
       <c r="F42" s="12" t="inlineStr">
         <is>
-          <t>Completeness/Accuracy</t>
+          <t>Occurrence</t>
         </is>
       </c>
       <c r="G42" s="12" t="inlineStr">
         <is>
-          <t>Sale/accept posts a balanced revenue + VAT journal entry to the GL automatically.</t>
+          <t>PSP webhook HMAC-SHA256 signature over raw body; fail-closed in production; out-of-band status re-verify.</t>
         </is>
       </c>
       <c r="H42" s="13" t="inlineStr">
         <is>
-          <t>Auto</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I42" s="13" t="inlineStr">
@@ -4492,37 +4492,37 @@
       </c>
       <c r="J42" s="13" t="inlineStr">
         <is>
-          <t>Per txn</t>
+          <t>Per callback</t>
         </is>
       </c>
       <c r="K42" s="12" t="inlineStr">
         <is>
-          <t>Controller</t>
+          <t>Eng Lead</t>
         </is>
       </c>
       <c r="L42" s="13" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P10/P11</t>
         </is>
       </c>
       <c r="M42" s="12" t="inlineStr">
         <is>
-          <t>ledger.service.ts (postEntry) from POS/CPQ flows</t>
+          <t>pos-terminal.controller.ts (PspWebhookController); crypto.verifyWebhookSignature</t>
         </is>
       </c>
       <c r="N42" s="12" t="inlineStr">
         <is>
-          <t>Walkthrough sale → JE.</t>
+          <t>Inspect signature check + prod gate.</t>
         </is>
       </c>
       <c r="O42" s="12" t="inlineStr">
         <is>
-          <t>Tie sample sales to GL postings.</t>
+          <t>Replay/forged signature → 401; valid → accepted.</t>
         </is>
       </c>
       <c r="P42" s="12" t="inlineStr">
         <is>
-          <t>Sale→GL tie-out</t>
+          <t>Webhook tests</t>
         </is>
       </c>
       <c r="Q42" s="19" t="inlineStr">
@@ -4534,7 +4534,7 @@
     <row r="43">
       <c r="A43" s="15" t="inlineStr">
         <is>
-          <t>REV-11</t>
+          <t>REV-10</t>
         </is>
       </c>
       <c r="B43" s="16" t="inlineStr">
@@ -4549,37 +4549,37 @@
       </c>
       <c r="D43" s="16" t="inlineStr">
         <is>
-          <t>Cash</t>
+          <t>Revenue; Tax</t>
         </is>
       </c>
       <c r="E43" s="16" t="inlineStr">
         <is>
-          <t>Card settlements not reconciled to PSP payouts.</t>
+          <t>Sales not posted to GL or posted unbalanced.</t>
         </is>
       </c>
       <c r="F43" s="16" t="inlineStr">
         <is>
-          <t>Existence/Accuracy</t>
+          <t>Completeness/Accuracy</t>
         </is>
       </c>
       <c r="G43" s="16" t="inlineStr">
         <is>
-          <t>Payment intents batched into settlement; settlement reconcile step.</t>
+          <t>Sale/accept posts a balanced revenue + VAT journal entry to the GL automatically.</t>
         </is>
       </c>
       <c r="H43" s="17" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Auto</t>
         </is>
       </c>
       <c r="I43" s="17" t="inlineStr">
         <is>
-          <t>Auto+Manual</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J43" s="17" t="inlineStr">
         <is>
-          <t>Daily</t>
+          <t>Per txn</t>
         </is>
       </c>
       <c r="K43" s="16" t="inlineStr">
@@ -4589,27 +4589,27 @@
       </c>
       <c r="L43" s="17" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="M43" s="16" t="inlineStr">
         <is>
-          <t>pos-terminal.service.ts (settle / reconcile)</t>
+          <t>ledger.service.ts (postEntry) from POS/CPQ flows</t>
         </is>
       </c>
       <c r="N43" s="16" t="inlineStr">
         <is>
-          <t>Inspect settlement batching.</t>
+          <t>Walkthrough sale → JE.</t>
         </is>
       </c>
       <c r="O43" s="16" t="inlineStr">
         <is>
-          <t>Sample batch reconciled to PSP statement.</t>
+          <t>Tie sample sales to GL postings.</t>
         </is>
       </c>
       <c r="P43" s="16" t="inlineStr">
         <is>
-          <t>Settlement recon</t>
+          <t>Sale→GL tie-out</t>
         </is>
       </c>
       <c r="Q43" s="19" t="inlineStr">
@@ -4621,7 +4621,7 @@
     <row r="44">
       <c r="A44" s="11" t="inlineStr">
         <is>
-          <t>REV-12</t>
+          <t>REV-11</t>
         </is>
       </c>
       <c r="B44" s="12" t="inlineStr">
@@ -4636,27 +4636,27 @@
       </c>
       <c r="D44" s="12" t="inlineStr">
         <is>
-          <t>Accounts Receivable</t>
+          <t>Cash</t>
         </is>
       </c>
       <c r="E44" s="12" t="inlineStr">
         <is>
-          <t>Overdue receivables not pursued; collection lapses; further credit extended to a defaulting customer.</t>
+          <t>Card settlements not reconciled to PSP payouts.</t>
         </is>
       </c>
       <c r="F44" s="12" t="inlineStr">
         <is>
-          <t>Valuation/Authorization</t>
+          <t>Existence/Accuracy</t>
         </is>
       </c>
       <c r="G44" s="12" t="inlineStr">
         <is>
-          <t>AR collections worklist + escalating dunning ladder (reminder→legal) recorded per invoice (DUN-), with the per-stage notice DISPATCHED to the customer (email/SMS/LINE via the messaging gateway; delivery outcome + recipient logged); credit-status / credit-check hold (over-limit OR 90+ days overdue). The serious-overdue hold is ENFORCED at POS/portal order entry (CREDIT_OVERDUE) under the FOR-UPDATE tenant lock, single-sourced with the collections on_hold threshold so the two never drift.</t>
+          <t>Payment intents batched into settlement; settlement reconcile step.</t>
         </is>
       </c>
       <c r="H44" s="13" t="inlineStr">
         <is>
-          <t>Det/Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I44" s="13" t="inlineStr">
@@ -4666,37 +4666,37 @@
       </c>
       <c r="J44" s="13" t="inlineStr">
         <is>
-          <t>Per overdue invoice / per order</t>
+          <t>Daily</t>
         </is>
       </c>
       <c r="K44" s="12" t="inlineStr">
         <is>
-          <t>AR / Controller</t>
+          <t>Controller</t>
         </is>
       </c>
       <c r="L44" s="13" t="inlineStr">
         <is>
-          <t>P10/P16</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="M44" s="12" t="inlineStr">
         <is>
-          <t>collections.service.ts (worklist, recordDunning+dispatch, runDunningSweep, creditStatus, creditCheck, SERIOUS_OVERDUE_DAYS); messaging.service.ts (notice delivery); pos.service.ts (createOrder CREDIT_OVERDUE); collections.controller.ts (incl. cron-callable /collections/sweep); bi.service.ts (ar_collections_dunning scheduled job, daily via runDue); /finance Collections UI; cutover/basics.ts (ToE)</t>
+          <t>pos-terminal.service.ts (settle / reconcile)</t>
         </is>
       </c>
       <c r="N44" s="12" t="inlineStr">
         <is>
-          <t>Inspect aging→stage logic, notice dispatch, hold decision, automated+scheduled sweep + order-entry gate.</t>
+          <t>Inspect settlement batching.</t>
         </is>
       </c>
       <c r="O44" s="12" t="inlineStr">
         <is>
-          <t>Worklist ages open AR; manual + automated (idempotent) + daily-scheduled dunning recorded AND the notice delivered (message_log, channel auto-picked from contact); held customer's credit-check denied; a 90+ defaulter is blocked at order entry while a good-standing customer orders (re-performed by the harness).</t>
+          <t>Sample batch reconciled to PSP statement.</t>
         </is>
       </c>
       <c r="P44" s="12" t="inlineStr">
         <is>
-          <t>Dunning log + message_log; sweep/scheduler run log; credit-hold report; CREDIT_OVERDUE rejections</t>
+          <t>Settlement recon</t>
         </is>
       </c>
       <c r="Q44" s="19" t="inlineStr">
@@ -4708,12 +4708,12 @@
     <row r="45">
       <c r="A45" s="15" t="inlineStr">
         <is>
-          <t>EXP-01</t>
+          <t>REV-12</t>
         </is>
       </c>
       <c r="B45" s="16" t="inlineStr">
         <is>
-          <t>Expenditure</t>
+          <t>Revenue &amp; Cash</t>
         </is>
       </c>
       <c r="C45" s="17" t="inlineStr">
@@ -4723,67 +4723,67 @@
       </c>
       <c r="D45" s="16" t="inlineStr">
         <is>
-          <t>Accounts Payable; Inventory</t>
+          <t>Accounts Receivable</t>
         </is>
       </c>
       <c r="E45" s="16" t="inlineStr">
         <is>
-          <t>Pay supplier for goods not ordered/received or wrong price.</t>
+          <t>Overdue receivables not pursued; collection lapses; further credit extended to a defaulting customer.</t>
         </is>
       </c>
       <c r="F45" s="16" t="inlineStr">
         <is>
-          <t>Occurrence/Accuracy</t>
+          <t>Valuation/Authorization</t>
         </is>
       </c>
       <c r="G45" s="16" t="inlineStr">
         <is>
-          <t>3-way match (PO ↔ GR ↔ Invoice) within tolerance gates AP payment.</t>
+          <t>AR collections worklist + escalating dunning ladder (reminder→legal) recorded per invoice (DUN-), with the per-stage notice DISPATCHED to the customer (email/SMS/LINE via the messaging gateway; delivery outcome + recipient logged); credit-status / credit-check hold (over-limit OR 90+ days overdue). The serious-overdue hold is ENFORCED at POS/portal order entry (CREDIT_OVERDUE) under the FOR-UPDATE tenant lock, single-sourced with the collections on_hold threshold so the two never drift.</t>
         </is>
       </c>
       <c r="H45" s="17" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det/Prev</t>
         </is>
       </c>
       <c r="I45" s="17" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="J45" s="17" t="inlineStr">
         <is>
-          <t>Per invoice</t>
+          <t>Per overdue invoice / per order</t>
         </is>
       </c>
       <c r="K45" s="16" t="inlineStr">
         <is>
-          <t>AP / Controller</t>
+          <t>AR / Controller</t>
         </is>
       </c>
       <c r="L45" s="17" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P10/P16</t>
         </is>
       </c>
       <c r="M45" s="16" t="inlineStr">
         <is>
-          <t>match/three-way-match.service.ts</t>
+          <t>collections.service.ts (worklist, recordDunning+dispatch, runDunningSweep, creditStatus, creditCheck, SERIOUS_OVERDUE_DAYS); messaging.service.ts (notice delivery); pos.service.ts (createOrder CREDIT_OVERDUE); collections.controller.ts (incl. cron-callable /collections/sweep); bi.service.ts (ar_collections_dunning scheduled job, daily via runDue); /finance Collections UI; cutover/basics.ts (ToE)</t>
         </is>
       </c>
       <c r="N45" s="16" t="inlineStr">
         <is>
-          <t>Inspect match + tolerance + payment gate.</t>
+          <t>Inspect aging→stage logic, notice dispatch, hold decision, automated+scheduled sweep + order-entry gate.</t>
         </is>
       </c>
       <c r="O45" s="16" t="inlineStr">
         <is>
-          <t>Sample invoices: payment blocked until matched.</t>
+          <t>Worklist ages open AR; manual + automated (idempotent) + daily-scheduled dunning recorded AND the notice delivered (message_log, channel auto-picked from contact); held customer's credit-check denied; a 90+ defaulter is blocked at order entry while a good-standing customer orders (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P45" s="16" t="inlineStr">
         <is>
-          <t>Match results</t>
+          <t>Dunning log + message_log; sweep/scheduler run log; credit-hold report; CREDIT_OVERDUE rejections</t>
         </is>
       </c>
       <c r="Q45" s="19" t="inlineStr">
@@ -4795,7 +4795,7 @@
     <row r="46">
       <c r="A46" s="11" t="inlineStr">
         <is>
-          <t>EXP-02</t>
+          <t>EXP-01</t>
         </is>
       </c>
       <c r="B46" s="12" t="inlineStr">
@@ -4810,22 +4810,22 @@
       </c>
       <c r="D46" s="12" t="inlineStr">
         <is>
-          <t>Accounts Payable</t>
+          <t>Accounts Payable; Inventory</t>
         </is>
       </c>
       <c r="E46" s="12" t="inlineStr">
         <is>
-          <t>Payment to blocklisted/unapproved vendor.</t>
+          <t>Pay supplier for goods not ordered/received or wrong price.</t>
         </is>
       </c>
       <c r="F46" s="12" t="inlineStr">
         <is>
-          <t>Validity</t>
+          <t>Occurrence/Accuracy</t>
         </is>
       </c>
       <c r="G46" s="12" t="inlineStr">
         <is>
-          <t>Supplier approval-status / blocklist check blocks PO &amp; payment to blocked vendors.</t>
+          <t>3-way match (PO ↔ GR ↔ Invoice) within tolerance gates AP payment.</t>
         </is>
       </c>
       <c r="H46" s="13" t="inlineStr">
@@ -4840,12 +4840,12 @@
       </c>
       <c r="J46" s="13" t="inlineStr">
         <is>
-          <t>Per txn</t>
+          <t>Per invoice</t>
         </is>
       </c>
       <c r="K46" s="12" t="inlineStr">
         <is>
-          <t>Procurement / AP</t>
+          <t>AP / Controller</t>
         </is>
       </c>
       <c r="L46" s="13" t="inlineStr">
@@ -4855,22 +4855,22 @@
       </c>
       <c r="M46" s="12" t="inlineStr">
         <is>
-          <t>procurement.service.ts (SUPPLIER_BLOCKED)</t>
+          <t>match/three-way-match.service.ts</t>
         </is>
       </c>
       <c r="N46" s="12" t="inlineStr">
         <is>
-          <t>Inspect vendor-status gate.</t>
+          <t>Inspect match + tolerance + payment gate.</t>
         </is>
       </c>
       <c r="O46" s="12" t="inlineStr">
         <is>
-          <t>Attempt PO to blocked vendor → 422.</t>
+          <t>Sample invoices: payment blocked until matched.</t>
         </is>
       </c>
       <c r="P46" s="12" t="inlineStr">
         <is>
-          <t>Vendor gate test</t>
+          <t>Match results</t>
         </is>
       </c>
       <c r="Q46" s="19" t="inlineStr">
@@ -4882,7 +4882,7 @@
     <row r="47">
       <c r="A47" s="15" t="inlineStr">
         <is>
-          <t>EXP-03</t>
+          <t>EXP-02</t>
         </is>
       </c>
       <c r="B47" s="16" t="inlineStr">
@@ -4902,17 +4902,17 @@
       </c>
       <c r="E47" s="16" t="inlineStr">
         <is>
-          <t>PR/PO raised without authorization.</t>
+          <t>Payment to blocklisted/unapproved vendor.</t>
         </is>
       </c>
       <c r="F47" s="16" t="inlineStr">
         <is>
-          <t>Authorization</t>
+          <t>Validity</t>
         </is>
       </c>
       <c r="G47" s="16" t="inlineStr">
         <is>
-          <t>Purchase requisition / PO approval workflow (maker-checker) per approval matrix.</t>
+          <t>Supplier approval-status / blocklist check blocks PO &amp; payment to blocked vendors.</t>
         </is>
       </c>
       <c r="H47" s="17" t="inlineStr">
@@ -4922,17 +4922,17 @@
       </c>
       <c r="I47" s="17" t="inlineStr">
         <is>
-          <t>Auto+Manual</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J47" s="17" t="inlineStr">
         <is>
-          <t>Per PR/PO</t>
+          <t>Per txn</t>
         </is>
       </c>
       <c r="K47" s="16" t="inlineStr">
         <is>
-          <t>Procurement Mgr</t>
+          <t>Procurement / AP</t>
         </is>
       </c>
       <c r="L47" s="17" t="inlineStr">
@@ -4942,34 +4942,34 @@
       </c>
       <c r="M47" s="16" t="inlineStr">
         <is>
-          <t>workflow / approvals; procurement.service.ts</t>
+          <t>procurement.service.ts (SUPPLIER_BLOCKED)</t>
         </is>
       </c>
       <c r="N47" s="16" t="inlineStr">
         <is>
-          <t>Inspect approval routing + thresholds.</t>
+          <t>Inspect vendor-status gate.</t>
         </is>
       </c>
       <c r="O47" s="16" t="inlineStr">
         <is>
-          <t>Sample PRs: approved by authorized approver ≠ requester.</t>
+          <t>Attempt PO to blocked vendor → 422.</t>
         </is>
       </c>
       <c r="P47" s="16" t="inlineStr">
         <is>
-          <t>Approval trail</t>
-        </is>
-      </c>
-      <c r="Q47" s="18" t="inlineStr">
-        <is>
-          <t>Partial</t>
+          <t>Vendor gate test</t>
+        </is>
+      </c>
+      <c r="Q47" s="19" t="inlineStr">
+        <is>
+          <t>Implemented</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="11" t="inlineStr">
         <is>
-          <t>EXP-04</t>
+          <t>EXP-03</t>
         </is>
       </c>
       <c r="B48" s="12" t="inlineStr">
@@ -4989,17 +4989,17 @@
       </c>
       <c r="E48" s="12" t="inlineStr">
         <is>
-          <t>Match tolerance loosened to force payment.</t>
+          <t>PR/PO raised without authorization.</t>
         </is>
       </c>
       <c r="F48" s="12" t="inlineStr">
         <is>
-          <t>Validity</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="G48" s="12" t="inlineStr">
         <is>
-          <t>Match-tolerance configuration change restricted to 'creditors' permission.</t>
+          <t>Purchase requisition / PO approval workflow (maker-checker) per approval matrix.</t>
         </is>
       </c>
       <c r="H48" s="13" t="inlineStr">
@@ -5009,54 +5009,54 @@
       </c>
       <c r="I48" s="13" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="J48" s="13" t="inlineStr">
         <is>
-          <t>Per change</t>
+          <t>Per PR/PO</t>
         </is>
       </c>
       <c r="K48" s="12" t="inlineStr">
         <is>
-          <t>Controller</t>
+          <t>Procurement Mgr</t>
         </is>
       </c>
       <c r="L48" s="13" t="inlineStr">
         <is>
-          <t>P10/P11</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="M48" s="12" t="inlineStr">
         <is>
-          <t>match.controller.ts (PUT tolerance @Permissions creditors)</t>
+          <t>workflow / approvals; procurement.service.ts</t>
         </is>
       </c>
       <c r="N48" s="12" t="inlineStr">
         <is>
-          <t>Inspect permission on tolerance change.</t>
+          <t>Inspect approval routing + thresholds.</t>
         </is>
       </c>
       <c r="O48" s="12" t="inlineStr">
         <is>
-          <t>Attempt change w/o perm → 403; log changes.</t>
+          <t>Sample PRs: approved by authorized approver ≠ requester.</t>
         </is>
       </c>
       <c r="P48" s="12" t="inlineStr">
         <is>
-          <t>Config-change log</t>
-        </is>
-      </c>
-      <c r="Q48" s="19" t="inlineStr">
-        <is>
-          <t>Implemented</t>
+          <t>Approval trail</t>
+        </is>
+      </c>
+      <c r="Q48" s="18" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="15" t="inlineStr">
         <is>
-          <t>EXP-05</t>
+          <t>EXP-04</t>
         </is>
       </c>
       <c r="B49" s="16" t="inlineStr">
@@ -5071,22 +5071,22 @@
       </c>
       <c r="D49" s="16" t="inlineStr">
         <is>
-          <t>Operating Expense; Accounts Payable</t>
+          <t>Accounts Payable</t>
         </is>
       </c>
       <c r="E49" s="16" t="inlineStr">
         <is>
-          <t>Employee/maintenance spend recorded in GL but not as a payable (escapes AP aging; AP sub-ledger ≠ GL control).</t>
+          <t>Match tolerance loosened to force payment.</t>
         </is>
       </c>
       <c r="F49" s="16" t="inlineStr">
         <is>
-          <t>Completeness/Accuracy</t>
+          <t>Validity</t>
         </is>
       </c>
       <c r="G49" s="16" t="inlineStr">
         <is>
-          <t>ESS expense approval and EAM work-order completion raise an AP payable via createApTxn (Dr 5100/5710 / Cr 2000) — not a bare GL post — so the liability appears in AP aging, settles through the AP pay flow, and keeps the AP sub-ledger ↔ GL 2000 reconciled (REC-01). Reimbursements vat-exempt; SoD approver ≠ claimant retained.</t>
+          <t>Match-tolerance configuration change restricted to 'creditors' permission.</t>
         </is>
       </c>
       <c r="H49" s="17" t="inlineStr">
@@ -5101,37 +5101,37 @@
       </c>
       <c r="J49" s="17" t="inlineStr">
         <is>
-          <t>Per claim/WO</t>
+          <t>Per change</t>
         </is>
       </c>
       <c r="K49" s="16" t="inlineStr">
         <is>
-          <t>AP / Controller</t>
+          <t>Controller</t>
         </is>
       </c>
       <c r="L49" s="17" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P10/P11</t>
         </is>
       </c>
       <c r="M49" s="16" t="inlineStr">
         <is>
-          <t>ess.service.ts (approveExpense → createApTxn); eam.service.ts (updateWorkOrderStatus → createApTxn, acct 5710); finance.service.ts (createApTxn expense_account/tenant_id); cutover/ess.ts + basics.ts (ToE)</t>
+          <t>match.controller.ts (PUT tolerance @Permissions creditors)</t>
         </is>
       </c>
       <c r="N49" s="16" t="inlineStr">
         <is>
-          <t>Inspect approval→AP routing + reconciliation.</t>
+          <t>Inspect permission on tolerance change.</t>
         </is>
       </c>
       <c r="O49" s="16" t="inlineStr">
         <is>
-          <t>Approve a claim / complete a WO → AP payable raised, paid via AP, sub-ledger ties to GL 2000 (re-performed by the harness).</t>
+          <t>Attempt change w/o perm → 403; log changes.</t>
         </is>
       </c>
       <c r="P49" s="16" t="inlineStr">
         <is>
-          <t>AP sub-ledger; reimbursement/maintenance payables</t>
+          <t>Config-change log</t>
         </is>
       </c>
       <c r="Q49" s="19" t="inlineStr">
@@ -5143,12 +5143,12 @@
     <row r="50">
       <c r="A50" s="11" t="inlineStr">
         <is>
-          <t>FA-06</t>
+          <t>EXP-05</t>
         </is>
       </c>
       <c r="B50" s="12" t="inlineStr">
         <is>
-          <t>Fixed Assets</t>
+          <t>Expenditure</t>
         </is>
       </c>
       <c r="C50" s="13" t="inlineStr">
@@ -5158,27 +5158,27 @@
       </c>
       <c r="D50" s="12" t="inlineStr">
         <is>
-          <t>Property, Plant &amp; Equipment</t>
+          <t>Operating Expense; Accounts Payable</t>
         </is>
       </c>
       <c r="E50" s="12" t="inlineStr">
         <is>
-          <t>Equipment not maintained; maintenance uncontrolled; preventive maintenance missed.</t>
+          <t>Employee/maintenance spend recorded in GL but not as a payable (escapes AP aging; AP sub-ledger ≠ GL control).</t>
         </is>
       </c>
       <c r="F50" s="12" t="inlineStr">
         <is>
-          <t>Existence/Valuation</t>
+          <t>Completeness/Accuracy</t>
         </is>
       </c>
       <c r="G50" s="12" t="inlineStr">
         <is>
-          <t>EAM maintenance work orders against the asset register with a guarded lifecycle (open→in_progress→completed/cancelled; BAD_TRANSITION); preventive-maintenance schedules (time/meter) with an idempotent due-generation sweep (cron / daily scheduled job eam_pm_generate).</t>
+          <t>ESS expense approval and EAM work-order completion raise an AP payable via createApTxn (Dr 5100/5710 / Cr 2000) — not a bare GL post — so the liability appears in AP aging, settles through the AP pay flow, and keeps the AP sub-ledger ↔ GL 2000 reconciled (REC-01). Reimbursements vat-exempt; SoD approver ≠ claimant retained.</t>
         </is>
       </c>
       <c r="H50" s="13" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I50" s="13" t="inlineStr">
@@ -5188,37 +5188,37 @@
       </c>
       <c r="J50" s="13" t="inlineStr">
         <is>
-          <t>Per WO / per sweep</t>
+          <t>Per claim/WO</t>
         </is>
       </c>
       <c r="K50" s="12" t="inlineStr">
         <is>
-          <t>Maintenance / FaAccountant</t>
+          <t>AP / Controller</t>
         </is>
       </c>
       <c r="L50" s="13" t="inlineStr">
         <is>
-          <t>P13/P16</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="M50" s="12" t="inlineStr">
         <is>
-          <t>eam.service.ts (work orders, PM schedules, runPmDue, meters); eam.controller.ts; bi.service.ts (eam_pm_generate); cutover/basics.ts (ToE)</t>
+          <t>ess.service.ts (approveExpense → createApTxn); eam.service.ts (updateWorkOrderStatus → createApTxn, acct 5710); finance.service.ts (createApTxn expense_account/tenant_id); cutover/ess.ts + basics.ts (ToE)</t>
         </is>
       </c>
       <c r="N50" s="12" t="inlineStr">
         <is>
-          <t>Inspect WO lifecycle guard + PM due logic.</t>
+          <t>Inspect approval→AP routing + reconciliation.</t>
         </is>
       </c>
       <c r="O50" s="12" t="inlineStr">
         <is>
-          <t>Raise/complete a WO; PM sweep raises due preventive WOs (time + meter) and is idempotent (re-performed by the harness).</t>
+          <t>Approve a claim / complete a WO → AP payable raised, paid via AP, sub-ledger ties to GL 2000 (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P50" s="12" t="inlineStr">
         <is>
-          <t>Work-order log; PM schedule + sweep run log</t>
+          <t>AP sub-ledger; reimbursement/maintenance payables</t>
         </is>
       </c>
       <c r="Q50" s="19" t="inlineStr">
@@ -5230,12 +5230,12 @@
     <row r="51">
       <c r="A51" s="15" t="inlineStr">
         <is>
-          <t>INV-01</t>
+          <t>EXP-06</t>
         </is>
       </c>
       <c r="B51" s="16" t="inlineStr">
         <is>
-          <t>Inventory &amp; COGS</t>
+          <t>Expenditure</t>
         </is>
       </c>
       <c r="C51" s="17" t="inlineStr">
@@ -5245,22 +5245,22 @@
       </c>
       <c r="D51" s="16" t="inlineStr">
         <is>
-          <t>Inventory; COGS</t>
+          <t>Accounts Payable; Cash</t>
         </is>
       </c>
       <c r="E51" s="16" t="inlineStr">
         <is>
-          <t>Two terminals sell last unit → negative/oversold stock.</t>
+          <t>Vendor payment disbursed without independent approval — one person both books and pays a bill.</t>
         </is>
       </c>
       <c r="F51" s="16" t="inlineStr">
         <is>
-          <t>Existence/Valuation</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="G51" s="16" t="inlineStr">
         <is>
-          <t>Bin-stock decrement under FOR UPDATE inside a transaction — concurrent picks serialize (no oversell).</t>
+          <t>AP disbursement maker-checker — a payment is REQUESTED by a 'creditors' holder and APPROVED by a DIFFERENT user (approvals/gl_close); the bill's paid_amount and the cash-disbursement GL move only on approval. Booking a bill pre-paid in one call is blocked.</t>
         </is>
       </c>
       <c r="H51" s="17" t="inlineStr">
@@ -5270,17 +5270,17 @@
       </c>
       <c r="I51" s="17" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="J51" s="17" t="inlineStr">
         <is>
-          <t>Per txn</t>
+          <t>Per payment</t>
         </is>
       </c>
       <c r="K51" s="16" t="inlineStr">
         <is>
-          <t>Eng Lead / Warehouse</t>
+          <t>AP / Controller</t>
         </is>
       </c>
       <c r="L51" s="17" t="inlineStr">
@@ -5290,22 +5290,22 @@
       </c>
       <c r="M51" s="16" t="inlineStr">
         <is>
-          <t>wms.service.ts (pick)</t>
+          <t>finance.service.ts (requestApPayment / approveApPayment requester≠approver / rejectApPayment); finance.controller.ts (creditors requests, approvals|gl_close approves); schema/finance.ts (ap_payments) + migration 0115; cutover/compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N51" s="16" t="inlineStr">
         <is>
-          <t>Inspect lock + sufficiency check in tx.</t>
+          <t>Inspect AP payment approval routing + SoD guard.</t>
         </is>
       </c>
       <c r="O51" s="16" t="inlineStr">
         <is>
-          <t>Concurrent last-unit test → one PICK_SHORT.</t>
+          <t>Sample payments: approver ≠ requester; no cash/GL effect until approved; self-approval → 403 SOD_VIOLATION; pre-paid creation → 400 (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P51" s="16" t="inlineStr">
         <is>
-          <t>Concurrency test</t>
+          <t>AP payment approvals</t>
         </is>
       </c>
       <c r="Q51" s="19" t="inlineStr">
@@ -5317,12 +5317,12 @@
     <row r="52">
       <c r="A52" s="11" t="inlineStr">
         <is>
-          <t>INV-02</t>
+          <t>FA-06</t>
         </is>
       </c>
       <c r="B52" s="12" t="inlineStr">
         <is>
-          <t>Inventory &amp; COGS</t>
+          <t>Fixed Assets</t>
         </is>
       </c>
       <c r="C52" s="13" t="inlineStr">
@@ -5332,22 +5332,22 @@
       </c>
       <c r="D52" s="12" t="inlineStr">
         <is>
-          <t>Inventory</t>
+          <t>Property, Plant &amp; Equipment</t>
         </is>
       </c>
       <c r="E52" s="12" t="inlineStr">
         <is>
-          <t>Stock movements not recorded (completeness of perpetual stock).</t>
+          <t>Equipment not maintained; maintenance uncontrolled; preventive maintenance missed.</t>
         </is>
       </c>
       <c r="F52" s="12" t="inlineStr">
         <is>
-          <t>Completeness</t>
+          <t>Existence/Valuation</t>
         </is>
       </c>
       <c r="G52" s="12" t="inlineStr">
         <is>
-          <t>Perpetual stock-movement + lot ledger logging on every issue/receipt/return.</t>
+          <t>EAM maintenance work orders against the asset register with a guarded lifecycle (open→in_progress→completed/cancelled; BAD_TRANSITION); preventive-maintenance schedules (time/meter) with an idempotent due-generation sweep (cron / daily scheduled job eam_pm_generate).</t>
         </is>
       </c>
       <c r="H52" s="13" t="inlineStr">
@@ -5362,37 +5362,37 @@
       </c>
       <c r="J52" s="13" t="inlineStr">
         <is>
-          <t>Per txn</t>
+          <t>Per WO / per sweep</t>
         </is>
       </c>
       <c r="K52" s="12" t="inlineStr">
         <is>
-          <t>Warehouse</t>
+          <t>Maintenance / FaAccountant</t>
         </is>
       </c>
       <c r="L52" s="13" t="inlineStr">
         <is>
-          <t>P13</t>
+          <t>P13/P16</t>
         </is>
       </c>
       <c r="M52" s="12" t="inlineStr">
         <is>
-          <t>stock-ops; custStockLog; lotLedger</t>
+          <t>eam.service.ts (work orders, PM schedules, runPmDue, meters); eam.controller.ts; bi.service.ts (eam_pm_generate); cutover/basics.ts (ToE)</t>
         </is>
       </c>
       <c r="N52" s="12" t="inlineStr">
         <is>
-          <t>Inspect movement logging.</t>
+          <t>Inspect WO lifecycle guard + PM due logic.</t>
         </is>
       </c>
       <c r="O52" s="12" t="inlineStr">
         <is>
-          <t>Tie sample movements to balances.</t>
+          <t>Raise/complete a WO; PM sweep raises due preventive WOs (time + meter) and is idempotent (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P52" s="12" t="inlineStr">
         <is>
-          <t>Stock ledger</t>
+          <t>Work-order log; PM schedule + sweep run log</t>
         </is>
       </c>
       <c r="Q52" s="19" t="inlineStr">
@@ -5404,7 +5404,7 @@
     <row r="53">
       <c r="A53" s="15" t="inlineStr">
         <is>
-          <t>INV-03</t>
+          <t>INV-01</t>
         </is>
       </c>
       <c r="B53" s="16" t="inlineStr">
@@ -5419,27 +5419,27 @@
       </c>
       <c r="D53" s="16" t="inlineStr">
         <is>
-          <t>COGS</t>
+          <t>Inventory; COGS</t>
         </is>
       </c>
       <c r="E53" s="16" t="inlineStr">
         <is>
-          <t>COGS misstated; consumption not costed.</t>
+          <t>Two terminals sell last unit → negative/oversold stock.</t>
         </is>
       </c>
       <c r="F53" s="16" t="inlineStr">
         <is>
-          <t>Accuracy</t>
+          <t>Existence/Valuation</t>
         </is>
       </c>
       <c r="G53" s="16" t="inlineStr">
         <is>
-          <t>Inventory costing → COGS posting on consumption; recipe/BOM deduction + reversal on return.</t>
+          <t>Bin-stock decrement under FOR UPDATE inside a transaction — concurrent picks serialize (no oversell).</t>
         </is>
       </c>
       <c r="H53" s="17" t="inlineStr">
         <is>
-          <t>Auto</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I53" s="17" t="inlineStr">
@@ -5454,7 +5454,7 @@
       </c>
       <c r="K53" s="16" t="inlineStr">
         <is>
-          <t>Controller</t>
+          <t>Eng Lead / Warehouse</t>
         </is>
       </c>
       <c r="L53" s="17" t="inlineStr">
@@ -5464,22 +5464,22 @@
       </c>
       <c r="M53" s="16" t="inlineStr">
         <is>
-          <t>costing; menu/recipe.service.ts</t>
+          <t>wms.service.ts (pick)</t>
         </is>
       </c>
       <c r="N53" s="16" t="inlineStr">
         <is>
-          <t>Walkthrough consumption → COGS JE.</t>
+          <t>Inspect lock + sufficiency check in tx.</t>
         </is>
       </c>
       <c r="O53" s="16" t="inlineStr">
         <is>
-          <t>Tie sample consumption to COGS.</t>
+          <t>Concurrent last-unit test → one PICK_SHORT.</t>
         </is>
       </c>
       <c r="P53" s="16" t="inlineStr">
         <is>
-          <t>COGS tie-out</t>
+          <t>Concurrency test</t>
         </is>
       </c>
       <c r="Q53" s="19" t="inlineStr">
@@ -5491,7 +5491,7 @@
     <row r="54">
       <c r="A54" s="11" t="inlineStr">
         <is>
-          <t>INV-04</t>
+          <t>INV-02</t>
         </is>
       </c>
       <c r="B54" s="12" t="inlineStr">
@@ -5511,17 +5511,17 @@
       </c>
       <c r="E54" s="12" t="inlineStr">
         <is>
-          <t>Book vs physical stock diverges; no count control.</t>
+          <t>Stock movements not recorded (completeness of perpetual stock).</t>
         </is>
       </c>
       <c r="F54" s="12" t="inlineStr">
         <is>
-          <t>Existence</t>
+          <t>Completeness</t>
         </is>
       </c>
       <c r="G54" s="12" t="inlineStr">
         <is>
-          <t>Periodic stocktake / cycle count; variance posted with review &amp; approval.</t>
+          <t>Perpetual stock-movement + lot ledger logging on every issue/receipt/return.</t>
         </is>
       </c>
       <c r="H54" s="13" t="inlineStr">
@@ -5531,59 +5531,59 @@
       </c>
       <c r="I54" s="13" t="inlineStr">
         <is>
-          <t>Auto+Manual</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J54" s="13" t="inlineStr">
         <is>
-          <t>Periodic</t>
+          <t>Per txn</t>
         </is>
       </c>
       <c r="K54" s="12" t="inlineStr">
         <is>
-          <t>Warehouse Mgr</t>
+          <t>Warehouse</t>
         </is>
       </c>
       <c r="L54" s="13" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>P13</t>
         </is>
       </c>
       <c r="M54" s="12" t="inlineStr">
         <is>
-          <t>stocktake (web); stock-ops</t>
+          <t>stock-ops; custStockLog; lotLedger</t>
         </is>
       </c>
       <c r="N54" s="12" t="inlineStr">
         <is>
-          <t>Inspect count + variance process.</t>
+          <t>Inspect movement logging.</t>
         </is>
       </c>
       <c r="O54" s="12" t="inlineStr">
         <is>
-          <t>Sample counts: variance reviewed &amp; approved.</t>
+          <t>Tie sample movements to balances.</t>
         </is>
       </c>
       <c r="P54" s="12" t="inlineStr">
         <is>
-          <t>Count sheets</t>
-        </is>
-      </c>
-      <c r="Q54" s="18" t="inlineStr">
-        <is>
-          <t>Partial</t>
+          <t>Stock ledger</t>
+        </is>
+      </c>
+      <c r="Q54" s="19" t="inlineStr">
+        <is>
+          <t>Implemented</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="15" t="inlineStr">
         <is>
-          <t>GL-01</t>
+          <t>INV-03</t>
         </is>
       </c>
       <c r="B55" s="16" t="inlineStr">
         <is>
-          <t>General Ledger</t>
+          <t>Inventory &amp; COGS</t>
         </is>
       </c>
       <c r="C55" s="17" t="inlineStr">
@@ -5593,12 +5593,12 @@
       </c>
       <c r="D55" s="16" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>COGS</t>
         </is>
       </c>
       <c r="E55" s="16" t="inlineStr">
         <is>
-          <t>Unbalanced / one-sided journal entries.</t>
+          <t>COGS misstated; consumption not costed.</t>
         </is>
       </c>
       <c r="F55" s="16" t="inlineStr">
@@ -5608,12 +5608,12 @@
       </c>
       <c r="G55" s="16" t="inlineStr">
         <is>
-          <t>Double-entry balanced-by-construction — Σdebit=Σcredit enforced; each line single-sided &amp; non-negative.</t>
+          <t>Inventory costing → COGS posting on consumption; recipe/BOM deduction + reversal on return.</t>
         </is>
       </c>
       <c r="H55" s="17" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Auto</t>
         </is>
       </c>
       <c r="I55" s="17" t="inlineStr">
@@ -5623,7 +5623,7 @@
       </c>
       <c r="J55" s="17" t="inlineStr">
         <is>
-          <t>Per JE</t>
+          <t>Per txn</t>
         </is>
       </c>
       <c r="K55" s="16" t="inlineStr">
@@ -5638,22 +5638,22 @@
       </c>
       <c r="M55" s="16" t="inlineStr">
         <is>
-          <t>ledger.service.ts (postEntry — UNBALANCED / INVALID_LINE)</t>
+          <t>costing; menu/recipe.service.ts</t>
         </is>
       </c>
       <c r="N55" s="16" t="inlineStr">
         <is>
-          <t>Inspect balance + line invariants.</t>
+          <t>Walkthrough consumption → COGS JE.</t>
         </is>
       </c>
       <c r="O55" s="16" t="inlineStr">
         <is>
-          <t>Attempt unbalanced JE → rejected.</t>
+          <t>Tie sample consumption to COGS.</t>
         </is>
       </c>
       <c r="P55" s="16" t="inlineStr">
         <is>
-          <t>Invariant test</t>
+          <t>COGS tie-out</t>
         </is>
       </c>
       <c r="Q55" s="19" t="inlineStr">
@@ -5665,12 +5665,12 @@
     <row r="56">
       <c r="A56" s="11" t="inlineStr">
         <is>
-          <t>GL-02</t>
+          <t>INV-04</t>
         </is>
       </c>
       <c r="B56" s="12" t="inlineStr">
         <is>
-          <t>General Ledger</t>
+          <t>Inventory &amp; COGS</t>
         </is>
       </c>
       <c r="C56" s="13" t="inlineStr">
@@ -5680,79 +5680,79 @@
       </c>
       <c r="D56" s="12" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Inventory</t>
         </is>
       </c>
       <c r="E56" s="12" t="inlineStr">
         <is>
-          <t>Postings to a closed period distort reported results.</t>
+          <t>Book vs physical stock diverges; no count control.</t>
         </is>
       </c>
       <c r="F56" s="12" t="inlineStr">
         <is>
-          <t>Cutoff</t>
+          <t>Existence</t>
         </is>
       </c>
       <c r="G56" s="12" t="inlineStr">
         <is>
-          <t>Period-close lockout — postings to a CLOSED fiscal period are rejected (per-tenant calendar).</t>
+          <t>Periodic stocktake / cycle count; variance posted with review &amp; approval.</t>
         </is>
       </c>
       <c r="H56" s="13" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I56" s="13" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="J56" s="13" t="inlineStr">
         <is>
-          <t>Per JE</t>
+          <t>Periodic</t>
         </is>
       </c>
       <c r="K56" s="12" t="inlineStr">
         <is>
-          <t>Controller</t>
+          <t>Warehouse Mgr</t>
         </is>
       </c>
       <c r="L56" s="13" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="M56" s="12" t="inlineStr">
         <is>
-          <t>ledger.service.ts (postEntry PERIOD_CLOSED); fiscal_periods</t>
+          <t>stocktake (web); stock-ops</t>
         </is>
       </c>
       <c r="N56" s="12" t="inlineStr">
         <is>
-          <t>Inspect close check.</t>
+          <t>Inspect count + variance process.</t>
         </is>
       </c>
       <c r="O56" s="12" t="inlineStr">
         <is>
-          <t>Post to closed period → rejected; review exceptions.</t>
+          <t>Sample counts: variance reviewed &amp; approved.</t>
         </is>
       </c>
       <c r="P56" s="12" t="inlineStr">
         <is>
-          <t>Close-lock test</t>
-        </is>
-      </c>
-      <c r="Q56" s="19" t="inlineStr">
-        <is>
-          <t>Implemented</t>
+          <t>Count sheets</t>
+        </is>
+      </c>
+      <c r="Q56" s="18" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="15" t="inlineStr">
         <is>
-          <t>GL-03</t>
+          <t>GL-01</t>
         </is>
       </c>
       <c r="B57" s="16" t="inlineStr">
@@ -5767,22 +5767,22 @@
       </c>
       <c r="D57" s="16" t="inlineStr">
         <is>
-          <t>Equity</t>
+          <t>All</t>
         </is>
       </c>
       <c r="E57" s="16" t="inlineStr">
         <is>
-          <t>Unauthorized year-end close / RE roll.</t>
+          <t>Unbalanced / one-sided journal entries.</t>
         </is>
       </c>
       <c r="F57" s="16" t="inlineStr">
         <is>
-          <t>Cutoff/Authorization</t>
+          <t>Accuracy</t>
         </is>
       </c>
       <c r="G57" s="16" t="inlineStr">
         <is>
-          <t>Year-end close restricted to 'exec'; closing entries roll to retained earnings.</t>
+          <t>Double-entry balanced-by-construction — Σdebit=Σcredit enforced; each line single-sided &amp; non-negative.</t>
         </is>
       </c>
       <c r="H57" s="17" t="inlineStr">
@@ -5792,42 +5792,42 @@
       </c>
       <c r="I57" s="17" t="inlineStr">
         <is>
-          <t>Auto+Manual</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J57" s="17" t="inlineStr">
         <is>
-          <t>Annual</t>
+          <t>Per JE</t>
         </is>
       </c>
       <c r="K57" s="16" t="inlineStr">
         <is>
-          <t>CFO / Controller</t>
+          <t>Controller</t>
         </is>
       </c>
       <c r="L57" s="17" t="inlineStr">
         <is>
-          <t>P10/P11</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="M57" s="16" t="inlineStr">
         <is>
-          <t>ledger.controller.ts (close-year @Permissions exec); closeYear</t>
+          <t>ledger.service.ts (postEntry — UNBALANCED / INVALID_LINE)</t>
         </is>
       </c>
       <c r="N57" s="16" t="inlineStr">
         <is>
-          <t>Inspect permission + closing logic.</t>
+          <t>Inspect balance + line invariants.</t>
         </is>
       </c>
       <c r="O57" s="16" t="inlineStr">
         <is>
-          <t>Attempt close w/o exec → 403; review annual close.</t>
+          <t>Attempt unbalanced JE → rejected.</t>
         </is>
       </c>
       <c r="P57" s="16" t="inlineStr">
         <is>
-          <t>Close package</t>
+          <t>Invariant test</t>
         </is>
       </c>
       <c r="Q57" s="19" t="inlineStr">
@@ -5839,7 +5839,7 @@
     <row r="58">
       <c r="A58" s="11" t="inlineStr">
         <is>
-          <t>GL-04</t>
+          <t>GL-02</t>
         </is>
       </c>
       <c r="B58" s="12" t="inlineStr">
@@ -5859,17 +5859,17 @@
       </c>
       <c r="E58" s="12" t="inlineStr">
         <is>
-          <t>Concurrent posting double-books the same source doc.</t>
+          <t>Postings to a closed period distort reported results.</t>
         </is>
       </c>
       <c r="F58" s="12" t="inlineStr">
         <is>
-          <t>Completeness/Accuracy</t>
+          <t>Cutoff</t>
         </is>
       </c>
       <c r="G58" s="12" t="inlineStr">
         <is>
-          <t>Ledger idempotency — UNIQUE (tenant,source,source_ref,ledger) + ON CONFLICT DO NOTHING in postEntry.</t>
+          <t>Period-close lockout — postings to a CLOSED fiscal period are rejected (per-tenant calendar).</t>
         </is>
       </c>
       <c r="H58" s="13" t="inlineStr">
@@ -5889,7 +5889,7 @@
       </c>
       <c r="K58" s="12" t="inlineStr">
         <is>
-          <t>Eng Lead / Controller</t>
+          <t>Controller</t>
         </is>
       </c>
       <c r="L58" s="13" t="inlineStr">
@@ -5899,22 +5899,22 @@
       </c>
       <c r="M58" s="12" t="inlineStr">
         <is>
-          <t>schema/ledger.ts (ux_je_idem); ledger.service.ts; migration 0058</t>
+          <t>ledger.service.ts (postEntry PERIOD_CLOSED); fiscal_periods</t>
         </is>
       </c>
       <c r="N58" s="12" t="inlineStr">
         <is>
-          <t>Inspect unique index + conflict handling.</t>
+          <t>Inspect close check.</t>
         </is>
       </c>
       <c r="O58" s="12" t="inlineStr">
         <is>
-          <t>Concurrent identical post → single entry.</t>
+          <t>Post to closed period → rejected; review exceptions.</t>
         </is>
       </c>
       <c r="P58" s="12" t="inlineStr">
         <is>
-          <t>Dedup test</t>
+          <t>Close-lock test</t>
         </is>
       </c>
       <c r="Q58" s="19" t="inlineStr">
@@ -5926,7 +5926,7 @@
     <row r="59">
       <c r="A59" s="15" t="inlineStr">
         <is>
-          <t>GL-05</t>
+          <t>GL-03</t>
         </is>
       </c>
       <c r="B59" s="16" t="inlineStr">
@@ -5941,22 +5941,22 @@
       </c>
       <c r="D59" s="16" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Equity</t>
         </is>
       </c>
       <c r="E59" s="16" t="inlineStr">
         <is>
-          <t>Manual JE posted without independent review (override risk).</t>
+          <t>Unauthorized year-end close / RE roll.</t>
         </is>
       </c>
       <c r="F59" s="16" t="inlineStr">
         <is>
-          <t>Authorization</t>
+          <t>Cutoff/Authorization</t>
         </is>
       </c>
       <c r="G59" s="16" t="inlineStr">
         <is>
-          <t>Manual journal-entry maker-checker — preparer ≠ approver before a manual JE posts.</t>
+          <t>Year-end close restricted to 'exec'; closing entries roll to retained earnings.</t>
         </is>
       </c>
       <c r="H59" s="17" t="inlineStr">
@@ -5971,37 +5971,37 @@
       </c>
       <c r="J59" s="17" t="inlineStr">
         <is>
-          <t>Per manual JE</t>
+          <t>Annual</t>
         </is>
       </c>
       <c r="K59" s="16" t="inlineStr">
         <is>
-          <t>Controller</t>
+          <t>CFO / Controller</t>
         </is>
       </c>
       <c r="L59" s="17" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P10/P11</t>
         </is>
       </c>
       <c r="M59" s="16" t="inlineStr">
         <is>
-          <t>ledger.service.ts (postEntry pendingApproval→Draft; approveEntry preparer≠approver; rejectEntry); ledger.controller.ts (gl_post posts / gl_close approves); cutover/compliance.ts (ToE)</t>
+          <t>ledger.controller.ts (close-year @Permissions exec); closeYear</t>
         </is>
       </c>
       <c r="N59" s="16" t="inlineStr">
         <is>
-          <t>Inspect JE approval routing.</t>
+          <t>Inspect permission + closing logic.</t>
         </is>
       </c>
       <c r="O59" s="16" t="inlineStr">
         <is>
-          <t>Sample manual JEs: approver ≠ preparer; Draft excluded from balances until approved (re-performed by the harness).</t>
+          <t>Attempt close w/o exec → 403; review annual close.</t>
         </is>
       </c>
       <c r="P59" s="16" t="inlineStr">
         <is>
-          <t>JE approvals</t>
+          <t>Close package</t>
         </is>
       </c>
       <c r="Q59" s="19" t="inlineStr">
@@ -6013,7 +6013,7 @@
     <row r="60">
       <c r="A60" s="11" t="inlineStr">
         <is>
-          <t>GL-06</t>
+          <t>GL-04</t>
         </is>
       </c>
       <c r="B60" s="12" t="inlineStr">
@@ -6033,17 +6033,17 @@
       </c>
       <c r="E60" s="12" t="inlineStr">
         <is>
-          <t>Operator mis-posts to another tenant's books.</t>
+          <t>Concurrent posting double-books the same source doc.</t>
         </is>
       </c>
       <c r="F60" s="12" t="inlineStr">
         <is>
-          <t>Validity</t>
+          <t>Completeness/Accuracy</t>
         </is>
       </c>
       <c r="G60" s="12" t="inlineStr">
         <is>
-          <t>HQ cross-tenant posting gated to Admin (explicit tenant override); others pinned to context (also RLS).</t>
+          <t>Ledger idempotency — UNIQUE (tenant,source,source_ref,ledger) + ON CONFLICT DO NOTHING in postEntry.</t>
         </is>
       </c>
       <c r="H60" s="13" t="inlineStr">
@@ -6063,32 +6063,32 @@
       </c>
       <c r="K60" s="12" t="inlineStr">
         <is>
-          <t>Eng Lead</t>
+          <t>Eng Lead / Controller</t>
         </is>
       </c>
       <c r="L60" s="13" t="inlineStr">
         <is>
-          <t>P10/P11</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="M60" s="12" t="inlineStr">
         <is>
-          <t>ledger.controller.ts (hqTenant)</t>
+          <t>schema/ledger.ts (ux_je_idem); ledger.service.ts; migration 0058</t>
         </is>
       </c>
       <c r="N60" s="12" t="inlineStr">
         <is>
-          <t>Inspect Admin gating of tenant_id.</t>
+          <t>Inspect unique index + conflict handling.</t>
         </is>
       </c>
       <c r="O60" s="12" t="inlineStr">
         <is>
-          <t>Non-Admin tenant override ignored; Admin audited.</t>
+          <t>Concurrent identical post → single entry.</t>
         </is>
       </c>
       <c r="P60" s="12" t="inlineStr">
         <is>
-          <t>Override test</t>
+          <t>Dedup test</t>
         </is>
       </c>
       <c r="Q60" s="19" t="inlineStr">
@@ -6100,7 +6100,7 @@
     <row r="61">
       <c r="A61" s="15" t="inlineStr">
         <is>
-          <t>GL-07</t>
+          <t>GL-05</t>
         </is>
       </c>
       <c r="B61" s="16" t="inlineStr">
@@ -6115,37 +6115,37 @@
       </c>
       <c r="D61" s="16" t="inlineStr">
         <is>
-          <t>Cash</t>
+          <t>All</t>
         </is>
       </c>
       <c r="E61" s="16" t="inlineStr">
         <is>
-          <t>Statement of cash flows mis-stated or doesn't tie to the change in cash.</t>
+          <t>Manual JE posted without independent review (override risk).</t>
         </is>
       </c>
       <c r="F61" s="16" t="inlineStr">
         <is>
-          <t>Accuracy/Completeness</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="G61" s="16" t="inlineStr">
         <is>
-          <t>Statement of Cash Flows (indirect) reconstructed from the GL: net income + non-cash add-backs + working-capital + investing + financing; year-end CLOSE entries excluded; reconciles to Δcash (1000/1010/1020) by construction with a `reconciled` tie-out flag.</t>
+          <t>Manual journal-entry maker-checker — preparer ≠ approver before a manual JE posts.</t>
         </is>
       </c>
       <c r="H61" s="17" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I61" s="17" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="J61" s="17" t="inlineStr">
         <is>
-          <t>Per period</t>
+          <t>Per manual JE</t>
         </is>
       </c>
       <c r="K61" s="16" t="inlineStr">
@@ -6160,22 +6160,22 @@
       </c>
       <c r="M61" s="16" t="inlineStr">
         <is>
-          <t>ledger.service.ts (cashFlowStatement); ledger.controller.ts (GET cash-flow); cutover/basics.ts (ToE)</t>
+          <t>ledger.service.ts (postEntry pendingApproval→Draft; approveEntry preparer≠approver; rejectEntry); ledger.controller.ts (gl_post posts / gl_close approves); cutover/compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N61" s="16" t="inlineStr">
         <is>
-          <t>Inspect SCF derivation + reconciliation flag.</t>
+          <t>Inspect JE approval routing.</t>
         </is>
       </c>
       <c r="O61" s="16" t="inlineStr">
         <is>
-          <t>Run cash-flow over a seeded period — activities tie to the movement in cash; CLOSE excluded (re-performed by the harness).</t>
+          <t>Sample manual JEs: approver ≠ preparer; Draft excluded from balances until approved (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P61" s="16" t="inlineStr">
         <is>
-          <t>Cash-flow reconciliation</t>
+          <t>JE approvals</t>
         </is>
       </c>
       <c r="Q61" s="19" t="inlineStr">
@@ -6187,12 +6187,12 @@
     <row r="62">
       <c r="A62" s="11" t="inlineStr">
         <is>
-          <t>REC-01</t>
+          <t>GL-06</t>
         </is>
       </c>
       <c r="B62" s="12" t="inlineStr">
         <is>
-          <t>Reconciliation</t>
+          <t>General Ledger</t>
         </is>
       </c>
       <c r="C62" s="13" t="inlineStr">
@@ -6207,62 +6207,62 @@
       </c>
       <c r="E62" s="12" t="inlineStr">
         <is>
-          <t>Subledgers diverge from GL undetected.</t>
+          <t>Operator mis-posts to another tenant's books.</t>
         </is>
       </c>
       <c r="F62" s="12" t="inlineStr">
         <is>
-          <t>Completeness/Accuracy</t>
+          <t>Validity</t>
         </is>
       </c>
       <c r="G62" s="12" t="inlineStr">
         <is>
-          <t>Subledger-to-GL reconciliation per period: import GL, auto-match, certify (sign-off via 'approvals').</t>
+          <t>HQ cross-tenant posting gated to Admin (explicit tenant override); others pinned to context (also RLS).</t>
         </is>
       </c>
       <c r="H62" s="13" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I62" s="13" t="inlineStr">
         <is>
-          <t>Auto+Manual</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J62" s="13" t="inlineStr">
         <is>
-          <t>Monthly</t>
+          <t>Per JE</t>
         </is>
       </c>
       <c r="K62" s="12" t="inlineStr">
         <is>
-          <t>Controller</t>
+          <t>Eng Lead</t>
         </is>
       </c>
       <c r="L62" s="13" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>P10/P11</t>
         </is>
       </c>
       <c r="M62" s="12" t="inlineStr">
         <is>
-          <t>reconciliation.service.ts (importGlItems/autoMatch/certify)</t>
+          <t>ledger.controller.ts (hqTenant)</t>
         </is>
       </c>
       <c r="N62" s="12" t="inlineStr">
         <is>
-          <t>Inspect recon + certify gate.</t>
+          <t>Inspect Admin gating of tenant_id.</t>
         </is>
       </c>
       <c r="O62" s="12" t="inlineStr">
         <is>
-          <t>Sample periods: reconciled, unmatched cleared, certified.</t>
+          <t>Non-Admin tenant override ignored; Admin audited.</t>
         </is>
       </c>
       <c r="P62" s="12" t="inlineStr">
         <is>
-          <t>Certified recon</t>
+          <t>Override test</t>
         </is>
       </c>
       <c r="Q62" s="19" t="inlineStr">
@@ -6274,12 +6274,12 @@
     <row r="63">
       <c r="A63" s="15" t="inlineStr">
         <is>
-          <t>REC-02</t>
+          <t>GL-07</t>
         </is>
       </c>
       <c r="B63" s="16" t="inlineStr">
         <is>
-          <t>Reconciliation</t>
+          <t>General Ledger</t>
         </is>
       </c>
       <c r="C63" s="17" t="inlineStr">
@@ -6294,17 +6294,17 @@
       </c>
       <c r="E63" s="16" t="inlineStr">
         <is>
-          <t>Bank balance not reconciled to GL.</t>
+          <t>Statement of cash flows mis-stated or doesn't tie to the change in cash.</t>
         </is>
       </c>
       <c r="F63" s="16" t="inlineStr">
         <is>
-          <t>Existence/Completeness</t>
+          <t>Accuracy/Completeness</t>
         </is>
       </c>
       <c r="G63" s="16" t="inlineStr">
         <is>
-          <t>Bank reconciliation against statements.</t>
+          <t>Statement of Cash Flows (indirect) reconstructed from the GL: net income + non-cash add-backs + working-capital + investing + financing; year-end CLOSE entries excluded; reconciles to Δcash (1000/1010/1020) by construction with a `reconciled` tie-out flag.</t>
         </is>
       </c>
       <c r="H63" s="17" t="inlineStr">
@@ -6314,12 +6314,12 @@
       </c>
       <c r="I63" s="17" t="inlineStr">
         <is>
-          <t>Auto+Manual</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J63" s="17" t="inlineStr">
         <is>
-          <t>Monthly</t>
+          <t>Per period</t>
         </is>
       </c>
       <c r="K63" s="16" t="inlineStr">
@@ -6329,27 +6329,27 @@
       </c>
       <c r="L63" s="17" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="M63" s="16" t="inlineStr">
         <is>
-          <t>bank module; drizzle/0015_bank_reconciliation</t>
+          <t>ledger.service.ts (cashFlowStatement); ledger.controller.ts (GET cash-flow); cutover/basics.ts (ToE)</t>
         </is>
       </c>
       <c r="N63" s="16" t="inlineStr">
         <is>
-          <t>Inspect bank-rec process.</t>
+          <t>Inspect SCF derivation + reconciliation flag.</t>
         </is>
       </c>
       <c r="O63" s="16" t="inlineStr">
         <is>
-          <t>Sample months reconciled &amp; reviewed.</t>
+          <t>Run cash-flow over a seeded period — activities tie to the movement in cash; CLOSE excluded (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P63" s="16" t="inlineStr">
         <is>
-          <t>Bank rec</t>
+          <t>Cash-flow reconciliation</t>
         </is>
       </c>
       <c r="Q63" s="19" t="inlineStr">
@@ -6361,7 +6361,7 @@
     <row r="64">
       <c r="A64" s="11" t="inlineStr">
         <is>
-          <t>REC-03</t>
+          <t>REC-01</t>
         </is>
       </c>
       <c r="B64" s="12" t="inlineStr">
@@ -6376,22 +6376,22 @@
       </c>
       <c r="D64" s="12" t="inlineStr">
         <is>
-          <t>Consolidation</t>
+          <t>All</t>
         </is>
       </c>
       <c r="E64" s="12" t="inlineStr">
         <is>
-          <t>Intercompany balances not eliminated/agreed.</t>
+          <t>Subledgers diverge from GL undetected.</t>
         </is>
       </c>
       <c r="F64" s="12" t="inlineStr">
         <is>
-          <t>Accuracy</t>
+          <t>Completeness/Accuracy</t>
         </is>
       </c>
       <c r="G64" s="12" t="inlineStr">
         <is>
-          <t>Intercompany reconciliation &amp; elimination on consolidation.</t>
+          <t>Subledger-to-GL reconciliation per period: import GL, auto-match, certify (sign-off via 'approvals').</t>
         </is>
       </c>
       <c r="H64" s="13" t="inlineStr">
@@ -6406,12 +6406,12 @@
       </c>
       <c r="J64" s="13" t="inlineStr">
         <is>
-          <t>Period</t>
+          <t>Monthly</t>
         </is>
       </c>
       <c r="K64" s="12" t="inlineStr">
         <is>
-          <t>Group Controller</t>
+          <t>Controller</t>
         </is>
       </c>
       <c r="L64" s="13" t="inlineStr">
@@ -6421,39 +6421,39 @@
       </c>
       <c r="M64" s="12" t="inlineStr">
         <is>
-          <t>intercompany; consolidation</t>
+          <t>reconciliation.service.ts (importGlItems/autoMatch/certify)</t>
         </is>
       </c>
       <c r="N64" s="12" t="inlineStr">
         <is>
-          <t>Inspect IC matching + elimination.</t>
+          <t>Inspect recon + certify gate.</t>
         </is>
       </c>
       <c r="O64" s="12" t="inlineStr">
         <is>
-          <t>Sample IC pairs agree &amp; eliminate.</t>
+          <t>Sample periods: reconciled, unmatched cleared, certified.</t>
         </is>
       </c>
       <c r="P64" s="12" t="inlineStr">
         <is>
-          <t>IC recon</t>
-        </is>
-      </c>
-      <c r="Q64" s="18" t="inlineStr">
-        <is>
-          <t>Partial</t>
+          <t>Certified recon</t>
+        </is>
+      </c>
+      <c r="Q64" s="19" t="inlineStr">
+        <is>
+          <t>Implemented</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="15" t="inlineStr">
         <is>
-          <t>TAX-01</t>
+          <t>REC-02</t>
         </is>
       </c>
       <c r="B65" s="16" t="inlineStr">
         <is>
-          <t>Tax</t>
+          <t>Reconciliation</t>
         </is>
       </c>
       <c r="C65" s="17" t="inlineStr">
@@ -6463,67 +6463,67 @@
       </c>
       <c r="D65" s="16" t="inlineStr">
         <is>
-          <t>Tax (VAT)</t>
+          <t>Cash</t>
         </is>
       </c>
       <c r="E65" s="16" t="inlineStr">
         <is>
-          <t>VAT computed incorrectly → filing/penalty risk.</t>
+          <t>Bank balance not reconciled to GL.</t>
         </is>
       </c>
       <c r="F65" s="16" t="inlineStr">
         <is>
-          <t>Accuracy</t>
+          <t>Existence/Completeness</t>
         </is>
       </c>
       <c r="G65" s="16" t="inlineStr">
         <is>
-          <t>VAT via pluggable provider (TH 7%); unit-tested; no hard-coded rate.</t>
+          <t>Bank reconciliation against statements.</t>
         </is>
       </c>
       <c r="H65" s="17" t="inlineStr">
         <is>
-          <t>Auto</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I65" s="17" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="J65" s="17" t="inlineStr">
         <is>
-          <t>Per txn</t>
+          <t>Monthly</t>
         </is>
       </c>
       <c r="K65" s="16" t="inlineStr">
         <is>
-          <t>Tax / Controller</t>
+          <t>Controller</t>
         </is>
       </c>
       <c r="L65" s="17" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="M65" s="16" t="inlineStr">
         <is>
-          <t>tax/tax-providers.ts; tax.service.ts; test/unit.test.ts</t>
+          <t>bank module; drizzle/0015_bank_reconciliation</t>
         </is>
       </c>
       <c r="N65" s="16" t="inlineStr">
         <is>
-          <t>Inspect rate provider + tests.</t>
+          <t>Inspect bank-rec process.</t>
         </is>
       </c>
       <c r="O65" s="16" t="inlineStr">
         <is>
-          <t>Re-perform VAT on sample; tie to return.</t>
+          <t>Sample months reconciled &amp; reviewed.</t>
         </is>
       </c>
       <c r="P65" s="16" t="inlineStr">
         <is>
-          <t>VAT tests</t>
+          <t>Bank rec</t>
         </is>
       </c>
       <c r="Q65" s="19" t="inlineStr">
@@ -6535,12 +6535,12 @@
     <row r="66">
       <c r="A66" s="11" t="inlineStr">
         <is>
-          <t>TAX-02</t>
+          <t>REC-03</t>
         </is>
       </c>
       <c r="B66" s="12" t="inlineStr">
         <is>
-          <t>Tax</t>
+          <t>Reconciliation</t>
         </is>
       </c>
       <c r="C66" s="13" t="inlineStr">
@@ -6550,79 +6550,79 @@
       </c>
       <c r="D66" s="12" t="inlineStr">
         <is>
-          <t>Tax; Revenue</t>
+          <t>Consolidation</t>
         </is>
       </c>
       <c r="E66" s="12" t="inlineStr">
         <is>
-          <t>Non-compliant e-Tax invoice / not transmitted to ETDA.</t>
+          <t>Intercompany balances not eliminated/agreed.</t>
         </is>
       </c>
       <c r="F66" s="12" t="inlineStr">
         <is>
-          <t>Accuracy/Compliance</t>
+          <t>Accuracy</t>
         </is>
       </c>
       <c r="G66" s="12" t="inlineStr">
         <is>
-          <t>e-Tax invoice (ETDA UBL 2.1 XML) generation + email with CC to ETDA timestamp mailbox.</t>
+          <t>Intercompany reconciliation &amp; elimination on consolidation.</t>
         </is>
       </c>
       <c r="H66" s="13" t="inlineStr">
         <is>
-          <t>Auto</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I66" s="13" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="J66" s="13" t="inlineStr">
         <is>
-          <t>Per invoice</t>
+          <t>Period</t>
         </is>
       </c>
       <c r="K66" s="12" t="inlineStr">
         <is>
-          <t>Tax</t>
+          <t>Group Controller</t>
         </is>
       </c>
       <c r="L66" s="13" t="inlineStr">
         <is>
-          <t>P10/P13</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="M66" s="12" t="inlineStr">
         <is>
-          <t>tax-docs/etax-xml.ts; etax-email.service.ts (tested)</t>
+          <t>intercompany; consolidation</t>
         </is>
       </c>
       <c r="N66" s="12" t="inlineStr">
         <is>
-          <t>Inspect XML schema + email composer.</t>
+          <t>Inspect IC matching + elimination.</t>
         </is>
       </c>
       <c r="O66" s="12" t="inlineStr">
         <is>
-          <t>Sample invoices: valid XML, correct CC/escaping.</t>
+          <t>Sample IC pairs agree &amp; eliminate.</t>
         </is>
       </c>
       <c r="P66" s="12" t="inlineStr">
         <is>
-          <t>e-Tax samples</t>
-        </is>
-      </c>
-      <c r="Q66" s="19" t="inlineStr">
-        <is>
-          <t>Implemented</t>
+          <t>IC recon</t>
+        </is>
+      </c>
+      <c r="Q66" s="18" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="15" t="inlineStr">
         <is>
-          <t>TAX-03</t>
+          <t>TAX-01</t>
         </is>
       </c>
       <c r="B67" s="16" t="inlineStr">
@@ -6637,12 +6637,12 @@
       </c>
       <c r="D67" s="16" t="inlineStr">
         <is>
-          <t>Tax (WHT)</t>
+          <t>Tax (VAT)</t>
         </is>
       </c>
       <c r="E67" s="16" t="inlineStr">
         <is>
-          <t>Withholding tax mis-computed / not reported.</t>
+          <t>VAT computed incorrectly → filing/penalty risk.</t>
         </is>
       </c>
       <c r="F67" s="16" t="inlineStr">
@@ -6652,7 +6652,7 @@
       </c>
       <c r="G67" s="16" t="inlineStr">
         <is>
-          <t>WHT computation and ภ.ง.ด. reporting.</t>
+          <t>VAT via pluggable provider (TH 7%); unit-tested; no hard-coded rate.</t>
         </is>
       </c>
       <c r="H67" s="17" t="inlineStr">
@@ -6667,12 +6667,12 @@
       </c>
       <c r="J67" s="17" t="inlineStr">
         <is>
-          <t>Per txn / monthly</t>
+          <t>Per txn</t>
         </is>
       </c>
       <c r="K67" s="16" t="inlineStr">
         <is>
-          <t>Tax</t>
+          <t>Tax / Controller</t>
         </is>
       </c>
       <c r="L67" s="17" t="inlineStr">
@@ -6682,39 +6682,39 @@
       </c>
       <c r="M67" s="16" t="inlineStr">
         <is>
-          <t>tax-reports; payroll</t>
+          <t>tax/tax-providers.ts; tax.service.ts; test/unit.test.ts</t>
         </is>
       </c>
       <c r="N67" s="16" t="inlineStr">
         <is>
-          <t>Inspect WHT logic + report.</t>
+          <t>Inspect rate provider + tests.</t>
         </is>
       </c>
       <c r="O67" s="16" t="inlineStr">
         <is>
-          <t>Re-perform WHT on sample; tie to filing.</t>
+          <t>Re-perform VAT on sample; tie to return.</t>
         </is>
       </c>
       <c r="P67" s="16" t="inlineStr">
         <is>
-          <t>WHT report</t>
-        </is>
-      </c>
-      <c r="Q67" s="18" t="inlineStr">
-        <is>
-          <t>Partial</t>
+          <t>VAT tests</t>
+        </is>
+      </c>
+      <c r="Q67" s="19" t="inlineStr">
+        <is>
+          <t>Implemented</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="11" t="inlineStr">
         <is>
-          <t>PAY-01</t>
+          <t>TAX-02</t>
         </is>
       </c>
       <c r="B68" s="12" t="inlineStr">
         <is>
-          <t>Payroll</t>
+          <t>Tax</t>
         </is>
       </c>
       <c r="C68" s="13" t="inlineStr">
@@ -6724,22 +6724,22 @@
       </c>
       <c r="D68" s="12" t="inlineStr">
         <is>
-          <t>Payroll expense/liability</t>
+          <t>Tax; Revenue</t>
         </is>
       </c>
       <c r="E68" s="12" t="inlineStr">
         <is>
-          <t>Payroll, SSO and PIT mis-computed.</t>
+          <t>Non-compliant e-Tax invoice / not transmitted to ETDA.</t>
         </is>
       </c>
       <c r="F68" s="12" t="inlineStr">
         <is>
-          <t>Accuracy</t>
+          <t>Accuracy/Compliance</t>
         </is>
       </c>
       <c r="G68" s="12" t="inlineStr">
         <is>
-          <t>Payroll engine — SSO 5% (cap 750), progressive PIT, payslip net; unit-tested.</t>
+          <t>e-Tax invoice (ETDA UBL 2.1 XML) generation + email with CC to ETDA timestamp mailbox.</t>
         </is>
       </c>
       <c r="H68" s="13" t="inlineStr">
@@ -6754,37 +6754,37 @@
       </c>
       <c r="J68" s="13" t="inlineStr">
         <is>
-          <t>Per run</t>
+          <t>Per invoice</t>
         </is>
       </c>
       <c r="K68" s="12" t="inlineStr">
         <is>
-          <t>HR / Payroll</t>
+          <t>Tax</t>
         </is>
       </c>
       <c r="L68" s="13" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P10/P13</t>
         </is>
       </c>
       <c r="M68" s="12" t="inlineStr">
         <is>
-          <t>payroll/payroll-calc.ts; test/unit.test.ts</t>
+          <t>tax-docs/etax-xml.ts; etax-email.service.ts (tested)</t>
         </is>
       </c>
       <c r="N68" s="12" t="inlineStr">
         <is>
-          <t>Inspect calc + tests.</t>
+          <t>Inspect XML schema + email composer.</t>
         </is>
       </c>
       <c r="O68" s="12" t="inlineStr">
         <is>
-          <t>Re-perform sample payslips.</t>
+          <t>Sample invoices: valid XML, correct CC/escaping.</t>
         </is>
       </c>
       <c r="P68" s="12" t="inlineStr">
         <is>
-          <t>Payslip tests</t>
+          <t>e-Tax samples</t>
         </is>
       </c>
       <c r="Q68" s="19" t="inlineStr">
@@ -6796,12 +6796,12 @@
     <row r="69">
       <c r="A69" s="15" t="inlineStr">
         <is>
-          <t>PAY-02</t>
+          <t>TAX-03</t>
         </is>
       </c>
       <c r="B69" s="16" t="inlineStr">
         <is>
-          <t>Payroll</t>
+          <t>Tax</t>
         </is>
       </c>
       <c r="C69" s="17" t="inlineStr">
@@ -6811,22 +6811,22 @@
       </c>
       <c r="D69" s="16" t="inlineStr">
         <is>
-          <t>Payroll liability</t>
+          <t>Tax (WHT)</t>
         </is>
       </c>
       <c r="E69" s="16" t="inlineStr">
         <is>
-          <t>Statutory items (PF/OT/leave/ภ.ง.ด.1ก) wrong.</t>
+          <t>Withholding tax mis-computed / not reported.</t>
         </is>
       </c>
       <c r="F69" s="16" t="inlineStr">
         <is>
-          <t>Accuracy/Compliance</t>
+          <t>Accuracy</t>
         </is>
       </c>
       <c r="G69" s="16" t="inlineStr">
         <is>
-          <t>Provident fund, overtime, leave accrual and ภ.ง.ด.1ก reporting.</t>
+          <t>WHT computation and ภ.ง.ด. reporting.</t>
         </is>
       </c>
       <c r="H69" s="17" t="inlineStr">
@@ -6841,12 +6841,12 @@
       </c>
       <c r="J69" s="17" t="inlineStr">
         <is>
-          <t>Per run / monthly</t>
+          <t>Per txn / monthly</t>
         </is>
       </c>
       <c r="K69" s="16" t="inlineStr">
         <is>
-          <t>HR / Payroll</t>
+          <t>Tax</t>
         </is>
       </c>
       <c r="L69" s="17" t="inlineStr">
@@ -6856,22 +6856,22 @@
       </c>
       <c r="M69" s="16" t="inlineStr">
         <is>
-          <t>hcm; payroll (Phase 19)</t>
+          <t>tax-reports; payroll</t>
         </is>
       </c>
       <c r="N69" s="16" t="inlineStr">
         <is>
-          <t>Inspect statutory logic.</t>
+          <t>Inspect WHT logic + report.</t>
         </is>
       </c>
       <c r="O69" s="16" t="inlineStr">
         <is>
-          <t>Sample run tied to statutory filings.</t>
+          <t>Re-perform WHT on sample; tie to filing.</t>
         </is>
       </c>
       <c r="P69" s="16" t="inlineStr">
         <is>
-          <t>Filings</t>
+          <t>WHT report</t>
         </is>
       </c>
       <c r="Q69" s="18" t="inlineStr">
@@ -6883,12 +6883,12 @@
     <row r="70">
       <c r="A70" s="11" t="inlineStr">
         <is>
-          <t>CON-01</t>
+          <t>PAY-01</t>
         </is>
       </c>
       <c r="B70" s="12" t="inlineStr">
         <is>
-          <t>Consolidation &amp; FX</t>
+          <t>Payroll</t>
         </is>
       </c>
       <c r="C70" s="13" t="inlineStr">
@@ -6898,12 +6898,12 @@
       </c>
       <c r="D70" s="12" t="inlineStr">
         <is>
-          <t>Consolidation</t>
+          <t>Payroll expense/liability</t>
         </is>
       </c>
       <c r="E70" s="12" t="inlineStr">
         <is>
-          <t>Group consolidation mis-stated (ownership/currency).</t>
+          <t>Payroll, SSO and PIT mis-computed.</t>
         </is>
       </c>
       <c r="F70" s="12" t="inlineStr">
@@ -6913,27 +6913,27 @@
       </c>
       <c r="G70" s="12" t="inlineStr">
         <is>
-          <t>Consolidation run (ownership %, entity currency) gated by 'approvals'.</t>
+          <t>Payroll engine — SSO 5% (cap 750), progressive PIT, payslip net; unit-tested.</t>
         </is>
       </c>
       <c r="H70" s="13" t="inlineStr">
         <is>
-          <t>Auto+Manual</t>
+          <t>Auto</t>
         </is>
       </c>
       <c r="I70" s="13" t="inlineStr">
         <is>
-          <t>Period</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J70" s="13" t="inlineStr">
         <is>
-          <t>Period</t>
+          <t>Per run</t>
         </is>
       </c>
       <c r="K70" s="12" t="inlineStr">
         <is>
-          <t>Group Controller</t>
+          <t>HR / Payroll</t>
         </is>
       </c>
       <c r="L70" s="13" t="inlineStr">
@@ -6943,22 +6943,22 @@
       </c>
       <c r="M70" s="12" t="inlineStr">
         <is>
-          <t>consolidation.service.ts (runConsolidation @Permissions approvals)</t>
+          <t>payroll/payroll-calc.ts; test/unit.test.ts</t>
         </is>
       </c>
       <c r="N70" s="12" t="inlineStr">
         <is>
-          <t>Inspect consolidation logic + gate.</t>
+          <t>Inspect calc + tests.</t>
         </is>
       </c>
       <c r="O70" s="12" t="inlineStr">
         <is>
-          <t>Sample period: consolidated TB ties to entities.</t>
+          <t>Re-perform sample payslips.</t>
         </is>
       </c>
       <c r="P70" s="12" t="inlineStr">
         <is>
-          <t>Consol TB</t>
+          <t>Payslip tests</t>
         </is>
       </c>
       <c r="Q70" s="19" t="inlineStr">
@@ -6970,92 +6970,266 @@
     <row r="71">
       <c r="A71" s="15" t="inlineStr">
         <is>
+          <t>PAY-02</t>
+        </is>
+      </c>
+      <c r="B71" s="16" t="inlineStr">
+        <is>
+          <t>Payroll</t>
+        </is>
+      </c>
+      <c r="C71" s="17" t="inlineStr">
+        <is>
+          <t>Application</t>
+        </is>
+      </c>
+      <c r="D71" s="16" t="inlineStr">
+        <is>
+          <t>Payroll liability</t>
+        </is>
+      </c>
+      <c r="E71" s="16" t="inlineStr">
+        <is>
+          <t>Statutory items (PF/OT/leave/ภ.ง.ด.1ก) wrong.</t>
+        </is>
+      </c>
+      <c r="F71" s="16" t="inlineStr">
+        <is>
+          <t>Accuracy/Compliance</t>
+        </is>
+      </c>
+      <c r="G71" s="16" t="inlineStr">
+        <is>
+          <t>Provident fund, overtime, leave accrual and ภ.ง.ด.1ก reporting.</t>
+        </is>
+      </c>
+      <c r="H71" s="17" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="I71" s="17" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="J71" s="17" t="inlineStr">
+        <is>
+          <t>Per run / monthly</t>
+        </is>
+      </c>
+      <c r="K71" s="16" t="inlineStr">
+        <is>
+          <t>HR / Payroll</t>
+        </is>
+      </c>
+      <c r="L71" s="17" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="M71" s="16" t="inlineStr">
+        <is>
+          <t>hcm; payroll (Phase 19)</t>
+        </is>
+      </c>
+      <c r="N71" s="16" t="inlineStr">
+        <is>
+          <t>Inspect statutory logic.</t>
+        </is>
+      </c>
+      <c r="O71" s="16" t="inlineStr">
+        <is>
+          <t>Sample run tied to statutory filings.</t>
+        </is>
+      </c>
+      <c r="P71" s="16" t="inlineStr">
+        <is>
+          <t>Filings</t>
+        </is>
+      </c>
+      <c r="Q71" s="18" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="11" t="inlineStr">
+        <is>
+          <t>CON-01</t>
+        </is>
+      </c>
+      <c r="B72" s="12" t="inlineStr">
+        <is>
+          <t>Consolidation &amp; FX</t>
+        </is>
+      </c>
+      <c r="C72" s="13" t="inlineStr">
+        <is>
+          <t>Application</t>
+        </is>
+      </c>
+      <c r="D72" s="12" t="inlineStr">
+        <is>
+          <t>Consolidation</t>
+        </is>
+      </c>
+      <c r="E72" s="12" t="inlineStr">
+        <is>
+          <t>Group consolidation mis-stated (ownership/currency).</t>
+        </is>
+      </c>
+      <c r="F72" s="12" t="inlineStr">
+        <is>
+          <t>Accuracy</t>
+        </is>
+      </c>
+      <c r="G72" s="12" t="inlineStr">
+        <is>
+          <t>Consolidation run (ownership %, entity currency) gated by 'approvals'.</t>
+        </is>
+      </c>
+      <c r="H72" s="13" t="inlineStr">
+        <is>
+          <t>Auto+Manual</t>
+        </is>
+      </c>
+      <c r="I72" s="13" t="inlineStr">
+        <is>
+          <t>Period</t>
+        </is>
+      </c>
+      <c r="J72" s="13" t="inlineStr">
+        <is>
+          <t>Period</t>
+        </is>
+      </c>
+      <c r="K72" s="12" t="inlineStr">
+        <is>
+          <t>Group Controller</t>
+        </is>
+      </c>
+      <c r="L72" s="13" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="M72" s="12" t="inlineStr">
+        <is>
+          <t>consolidation.service.ts (runConsolidation @Permissions approvals)</t>
+        </is>
+      </c>
+      <c r="N72" s="12" t="inlineStr">
+        <is>
+          <t>Inspect consolidation logic + gate.</t>
+        </is>
+      </c>
+      <c r="O72" s="12" t="inlineStr">
+        <is>
+          <t>Sample period: consolidated TB ties to entities.</t>
+        </is>
+      </c>
+      <c r="P72" s="12" t="inlineStr">
+        <is>
+          <t>Consol TB</t>
+        </is>
+      </c>
+      <c r="Q72" s="19" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="15" t="inlineStr">
+        <is>
           <t>CON-02</t>
         </is>
       </c>
-      <c r="B71" s="16" t="inlineStr">
+      <c r="B73" s="16" t="inlineStr">
         <is>
           <t>Consolidation &amp; FX</t>
         </is>
       </c>
-      <c r="C71" s="17" t="inlineStr">
+      <c r="C73" s="17" t="inlineStr">
         <is>
           <t>Application</t>
         </is>
       </c>
-      <c r="D71" s="16" t="inlineStr">
+      <c r="D73" s="16" t="inlineStr">
         <is>
           <t>FX gain/loss</t>
         </is>
       </c>
-      <c r="E71" s="16" t="inlineStr">
+      <c r="E73" s="16" t="inlineStr">
         <is>
           <t>FX exposures not revalued at period-end.</t>
         </is>
       </c>
-      <c r="F71" s="16" t="inlineStr">
+      <c r="F73" s="16" t="inlineStr">
         <is>
           <t>Valuation</t>
         </is>
       </c>
-      <c r="G71" s="16" t="inlineStr">
+      <c r="G73" s="16" t="inlineStr">
         <is>
           <t>FX revaluation at period-end rates; unrealized FX posted (acct 5400).</t>
         </is>
       </c>
-      <c r="H71" s="17" t="inlineStr">
+      <c r="H73" s="17" t="inlineStr">
         <is>
           <t>Auto+Manual</t>
         </is>
       </c>
-      <c r="I71" s="17" t="inlineStr">
+      <c r="I73" s="17" t="inlineStr">
         <is>
           <t>Period-end</t>
         </is>
       </c>
-      <c r="J71" s="17" t="inlineStr">
+      <c r="J73" s="17" t="inlineStr">
         <is>
           <t>Period</t>
         </is>
       </c>
-      <c r="K71" s="16" t="inlineStr">
+      <c r="K73" s="16" t="inlineStr">
         <is>
           <t>Controller</t>
         </is>
       </c>
-      <c r="L71" s="17" t="inlineStr">
+      <c r="L73" s="17" t="inlineStr">
         <is>
           <t>P10</t>
         </is>
       </c>
-      <c r="M71" s="16" t="inlineStr">
+      <c r="M73" s="16" t="inlineStr">
         <is>
           <t>fx.service.ts (revalue / unrealized report)</t>
         </is>
       </c>
-      <c r="N71" s="16" t="inlineStr">
+      <c r="N73" s="16" t="inlineStr">
         <is>
           <t>Inspect reval logic + rates.</t>
         </is>
       </c>
-      <c r="O71" s="16" t="inlineStr">
+      <c r="O73" s="16" t="inlineStr">
         <is>
           <t>Recompute reval on sample balances.</t>
         </is>
       </c>
-      <c r="P71" s="16" t="inlineStr">
+      <c r="P73" s="16" t="inlineStr">
         <is>
           <t>FX reval JE</t>
         </is>
       </c>
-      <c r="Q71" s="19" t="inlineStr">
+      <c r="Q73" s="19" t="inlineStr">
         <is>
           <t>Implemented</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q71"/>
+  <autoFilter ref="A1:Q73"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -8238,7 +8412,7 @@
         </is>
       </c>
       <c r="C5" s="28">
-        <f>COUNTIF(RCM!$Q$2:$Q$71,B5)</f>
+        <f>COUNTIF(RCM!$Q$2:$Q$73,B5)</f>
         <v/>
       </c>
     </row>
@@ -8249,7 +8423,7 @@
         </is>
       </c>
       <c r="C6" s="28">
-        <f>COUNTIF(RCM!$Q$2:$Q$71,B6)</f>
+        <f>COUNTIF(RCM!$Q$2:$Q$73,B6)</f>
         <v/>
       </c>
     </row>
@@ -8260,7 +8434,7 @@
         </is>
       </c>
       <c r="C7" s="28">
-        <f>COUNTIF(RCM!$Q$2:$Q$71,B7)</f>
+        <f>COUNTIF(RCM!$Q$2:$Q$73,B7)</f>
         <v/>
       </c>
     </row>
@@ -8271,7 +8445,7 @@
         </is>
       </c>
       <c r="C8" s="31">
-        <f>COUNTA(RCM!$A$2:$A$71)</f>
+        <f>COUNTA(RCM!$A$2:$A$73)</f>
         <v/>
       </c>
     </row>
@@ -8289,7 +8463,7 @@
         </is>
       </c>
       <c r="C11" s="28">
-        <f>COUNTIF(RCM!$C$2:$C$71,B11)</f>
+        <f>COUNTIF(RCM!$C$2:$C$73,B11)</f>
         <v/>
       </c>
     </row>
@@ -8300,7 +8474,7 @@
         </is>
       </c>
       <c r="C12" s="28">
-        <f>COUNTIF(RCM!$C$2:$C$71,B12)</f>
+        <f>COUNTIF(RCM!$C$2:$C$73,B12)</f>
         <v/>
       </c>
     </row>
@@ -8311,7 +8485,7 @@
         </is>
       </c>
       <c r="C13" s="28">
-        <f>COUNTIF(RCM!$C$2:$C$71,B13)</f>
+        <f>COUNTIF(RCM!$C$2:$C$73,B13)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(budget): budget maker-checker (BUD-01) — pending & excluded from variance until independent approval
Budgets were fire-and-forget; one person upserted any amount and it drove budget-vs-actual. BUD-01 makes an upserted budget PendingApproval and EXCLUDED from budget-vs-actual until a DIFFERENT user approves (self-approve -> SOD_VIOLATION, binds Admin; reject -> Rejected). status DEFAULT 'Approved' keeps existing rows + direct planning seeds usable. Pending budgets surfaced/aged by MON-01.

migration 0138 (journaled); budget.service upsert/approve/reject/budgetVsActual(Approved-only); budget.controller approve|reject|pending (approvals/gl_close); finance.service MON-01 budget queue; web /budget badges + approve/reject; RCM BUD-01 (88); docs PN 13/04 + manual 10 + UAT 09 + matrix. ToE budget.ts. budget 16, epm-planning 16, compliance 88.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/compliance/Oshinei_ERP_SOX_RCM_v1.xlsx
+++ b/compliance/Oshinei_ERP_SOX_RCM_v1.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'RCM'!$A$1:$Q$88</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'RCM'!$A$1:$Q$89</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Gap Remediation'!$A$2:$H$18</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -858,7 +858,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q88"/>
+  <dimension ref="A1:Q89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -7612,7 +7612,7 @@
       </c>
       <c r="G78" s="12" t="inlineStr">
         <is>
-          <t>Pending-approvals aging monitor (GET /api/finance/approvals/aging): ONE read across every maker-checker queue, aged by how long each item has waited for its second signature. Scans every Draft journal entry — so it AUTO-COVERS any control that posts a Draft JE via ledger.postEntry pendingApproval (GL-05 manual JE, PAY-03 payroll, FA-08 revaluation, FA-09 disposal, BANK-02 bank adjustment) — PLUS the queues that post nothing until approval (INV-07 inventory write-offs, AP-PAY vendor payments, FX-04 manual FX rates). Each item is control-tagged, attributed to its requester, valued, and aged; items past the SLA (default 7 days, ?stale_days overrides) are surfaced as exceptions with an all_clear flag and per-control roll-up. The supervisory 'is anything stuck in approval?' view over the whole control environment.</t>
+          <t>Pending-approvals aging monitor (GET /api/finance/approvals/aging): ONE read across every maker-checker queue, aged by how long each item has waited for its second signature. Scans every Draft journal entry — so it AUTO-COVERS any control that posts a Draft JE via ledger.postEntry pendingApproval (GL-05 manual JE, PAY-03 payroll, FA-08 revaluation, FA-09 disposal, BANK-02 bank adjustment) — PLUS the queues that post nothing until approval (INV-07 inventory write-offs, AP-PAY vendor payments, FX-04 manual FX rates, BUD-01 budgets). Each item is control-tagged, attributed to its requester, valued, and aged; items past the SLA (default 7 days, ?stale_days overrides) are surfaced as exceptions with an all_clear flag and per-control roll-up. The supervisory 'is anything stuck in approval?' view over the whole control environment.</t>
         </is>
       </c>
       <c r="H78" s="13" t="inlineStr">
@@ -8536,8 +8536,95 @@
         </is>
       </c>
     </row>
+    <row r="89">
+      <c r="A89" s="15" t="inlineStr">
+        <is>
+          <t>BUD-01</t>
+        </is>
+      </c>
+      <c r="B89" s="16" t="inlineStr">
+        <is>
+          <t>Budgeting &amp; Planning</t>
+        </is>
+      </c>
+      <c r="C89" s="17" t="inlineStr">
+        <is>
+          <t>Application</t>
+        </is>
+      </c>
+      <c r="D89" s="16" t="inlineStr">
+        <is>
+          <t>Budget; All (variance reporting)</t>
+        </is>
+      </c>
+      <c r="E89" s="16" t="inlineStr">
+        <is>
+          <t>A budget figure is entered/changed by one person and immediately drives the budget-vs-actual variance report — the basis for spend authorization and performance review — with no independent approval; a wrong or self-serving budget makes overspending look 'on budget'.</t>
+        </is>
+      </c>
+      <c r="F89" s="16" t="inlineStr">
+        <is>
+          <t>Authorization/Accuracy</t>
+        </is>
+      </c>
+      <c r="G89" s="16" t="inlineStr">
+        <is>
+          <t>Budget maker-checker (SoD): an upserted budget (POST /api/ledger/budgets) lands as PendingApproval and is EXCLUDED from budget-vs-actual until a DIFFERENT user approves it (POST /api/ledger/budgets/approve for the fiscal_year/account/cost-centre[/period]). Self-approval → SOD_VIOLATION (binds even Admin); reject marks it Rejected (excluded). DEFAULT 'Approved' keeps existing rows + direct planning seeds usable. Pending budgets are also surfaced, aged, by the pending-approvals monitor (MON-01).</t>
+        </is>
+      </c>
+      <c r="H89" s="17" t="inlineStr">
+        <is>
+          <t>Prev</t>
+        </is>
+      </c>
+      <c r="I89" s="17" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="J89" s="17" t="inlineStr">
+        <is>
+          <t>Per budget</t>
+        </is>
+      </c>
+      <c r="K89" s="16" t="inlineStr">
+        <is>
+          <t>Controller / FP&amp;A</t>
+        </is>
+      </c>
+      <c r="L89" s="17" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="M89" s="16" t="inlineStr">
+        <is>
+          <t>budget.service.ts upsertBudget(→PendingApproval)/approveBudget/rejectBudget/budgetVsActual(Approved only); budget.controller.ts (budgets/approve|reject|pending gated approvals/gl_close); schema/budgets.ts budgets.status + migration 0138; cutover/budget.ts (ToE)</t>
+        </is>
+      </c>
+      <c r="N89" s="16" t="inlineStr">
+        <is>
+          <t>Inspect the request→approve flow + the approver≠requester check + that budget-vs-actual counts Approved budgets only.</t>
+        </is>
+      </c>
+      <c r="O89" s="16" t="inlineStr">
+        <is>
+          <t>Re-perform: upsert a budget (PendingApproval, excluded from variance), attempt self-approve (SOD_VIOLATION), approve as a different user, confirm it then appears in budget-vs-actual (re-performed by the budget harness).</t>
+        </is>
+      </c>
+      <c r="P89" s="16" t="inlineStr">
+        <is>
+          <t>Budget approval log + SoD test</t>
+        </is>
+      </c>
+      <c r="Q89" s="19" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Q88"/>
+  <autoFilter ref="A1:Q89"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -9720,7 +9807,7 @@
         </is>
       </c>
       <c r="C5" s="29">
-        <f>COUNTIF(RCM!$Q$2:$Q$88,B5)</f>
+        <f>COUNTIF(RCM!$Q$2:$Q$89,B5)</f>
         <v/>
       </c>
     </row>
@@ -9731,7 +9818,7 @@
         </is>
       </c>
       <c r="C6" s="29">
-        <f>COUNTIF(RCM!$Q$2:$Q$88,B6)</f>
+        <f>COUNTIF(RCM!$Q$2:$Q$89,B6)</f>
         <v/>
       </c>
     </row>
@@ -9742,7 +9829,7 @@
         </is>
       </c>
       <c r="C7" s="29">
-        <f>COUNTIF(RCM!$Q$2:$Q$88,B7)</f>
+        <f>COUNTIF(RCM!$Q$2:$Q$89,B7)</f>
         <v/>
       </c>
     </row>
@@ -9753,7 +9840,7 @@
         </is>
       </c>
       <c r="C8" s="32">
-        <f>COUNTA(RCM!$A$2:$A$88)</f>
+        <f>COUNTA(RCM!$A$2:$A$89)</f>
         <v/>
       </c>
     </row>
@@ -9771,7 +9858,7 @@
         </is>
       </c>
       <c r="C11" s="29">
-        <f>COUNTIF(RCM!$C$2:$C$88,B11)</f>
+        <f>COUNTIF(RCM!$C$2:$C$89,B11)</f>
         <v/>
       </c>
     </row>
@@ -9782,7 +9869,7 @@
         </is>
       </c>
       <c r="C12" s="29">
-        <f>COUNTIF(RCM!$C$2:$C$88,B12)</f>
+        <f>COUNTIF(RCM!$C$2:$C$89,B12)</f>
         <v/>
       </c>
     </row>
@@ -9793,7 +9880,7 @@
         </is>
       </c>
       <c r="C13" s="29">
-        <f>COUNTIF(RCM!$C$2:$C$88,B13)</f>
+        <f>COUNTIF(RCM!$C$2:$C$89,B13)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(gl): WS1.2 — posting/account-determination engine (GL-12)
- New posting_event_types + posting_rules tables (migration 0156)
  with RLS; seeds 28 event types + 44 global-default rule legs
  matching all existing inline account_code literals exactly
- PostingService: post(eventType, ctx) resolves rules → calls
  postEntry; preview() dry-run; tenant rules shadow global defaults
- PostingRulesController: GET event-types, GET rules, POST preview,
  POST upsert (perm gl_posting_rules)
- basics harness: 4 golden-snapshot parity checks (157/157 green)
- GL-12 RCM control; process-narrative + UAT TC-GL-12-01..04
- RCM xlsx regenerated to 115 controls

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/compliance/Oshinei_ERP_SOX_RCM_v1.xlsx
+++ b/compliance/Oshinei_ERP_SOX_RCM_v1.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'RCM'!$A$1:$Q$114</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'RCM'!$A$1:$Q$116</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Gap Remediation'!$A$2:$H$18</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -858,7 +858,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q114"/>
+  <dimension ref="A1:Q116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -8626,12 +8626,12 @@
     <row r="90">
       <c r="A90" s="11" t="inlineStr">
         <is>
-          <t>EXP-07</t>
+          <t>GL-11</t>
         </is>
       </c>
       <c r="B90" s="12" t="inlineStr">
         <is>
-          <t>Expenditure</t>
+          <t>General Ledger</t>
         </is>
       </c>
       <c r="C90" s="13" t="inlineStr">
@@ -8641,27 +8641,27 @@
       </c>
       <c r="D90" s="12" t="inlineStr">
         <is>
-          <t>Cash; Operating expense</t>
+          <t>All</t>
         </is>
       </c>
       <c r="E90" s="12" t="inlineStr">
         <is>
-          <t>Petty-cash / employee advance issued but never accounted for — cash leakage, expense unrecorded.</t>
+          <t>Chart of Accounts changed without authorisation; account code changed after postings exist; account deactivated while carrying a non-zero balance; manual JE posted directly to a control account (AR/AP/INV/FA), bypassing the sub-ledger and hiding a sub-ledger discrepancy.</t>
         </is>
       </c>
       <c r="F90" s="12" t="inlineStr">
         <is>
-          <t>Existence/Completeness</t>
+          <t>Authorization/Completeness/Accuracy</t>
         </is>
       </c>
       <c r="G90" s="12" t="inlineStr">
         <is>
-          <t>Employee cash advances: issuing an advance debits the 1180 Employee Advances control (Dr 1180 / Cr 1000); settlement clears it against actual spend + returned cash (Dr expense + Dr 1000 / Cr 1180), enforced to reconcile (settled_expense + returned_cash must equal the advance → SETTLE_MISMATCH). The 1180 balance is the outstanding float subject to review.</t>
+          <t>CoA Change Control: account creation/update/deactivation requires the gl_coa permission (held by FinancialController, not GlAccountant — separated from gl_post per SoD). Disabling postability on an account that already has posted entries is rejected (CODE_HAS_POSTINGS). Deactivation is rejected if the account carries a non-zero net balance (ACCOUNT_HAS_BALANCE) — prevents orphaning a balance in a closed account. Four accounts are flagged is_control=true at setup: 1100 (AR), 2000 (AP), 1200 (INV), 1500 (FA); a direct manual JE that touches any of these without viaSubledger:true is rejected (CONTROL_ACCOUNT), ensuring AR/AP/INV/FA balances are exclusively maintained by their respective sub-ledger service methods.</t>
         </is>
       </c>
       <c r="H90" s="13" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I90" s="13" t="inlineStr">
@@ -8671,12 +8671,12 @@
       </c>
       <c r="J90" s="13" t="inlineStr">
         <is>
-          <t>Per advance</t>
+          <t>Event-driven</t>
         </is>
       </c>
       <c r="K90" s="12" t="inlineStr">
         <is>
-          <t>AP / Controller</t>
+          <t>Financial Controller</t>
         </is>
       </c>
       <c r="L90" s="13" t="inlineStr">
@@ -8686,22 +8686,22 @@
       </c>
       <c r="M90" s="12" t="inlineStr">
         <is>
-          <t>finance.service.ts (issueAdvance, settleAdvance reconcile-or-reject, listAdvances outstanding); finance.controller.ts (creditors/exec); schema/finance.ts (employee_advances) + migration 0120; cutover/basics.ts (ToE)</t>
+          <t>coa.service.ts (createAccount DUPLICATE_ACCOUNT, updateAccount CODE_HAS_POSTINGS, deactivateAccount ACCOUNT_HAS_BALANCE); coa.controller.ts (gl_coa permission gate); ledger.service.ts postEntry control-account guard (CONTROL_ACCOUNT, viaSubledger flag); schema/ledger.ts (account_groups table, accounts.is_control/control_subledger/is_postable/normal_balance + migration 0155); packages/shared/src/permissions.ts (gl_coa sub-permission, FinancialController default)</t>
         </is>
       </c>
       <c r="N90" s="12" t="inlineStr">
         <is>
-          <t>Inspect issue/settle GL + settlement reconciliation guard.</t>
+          <t>Inspect gl_coa permission gate + CODE_HAS_POSTINGS guard + ACCOUNT_HAS_BALANCE guard + CONTROL_ACCOUNT guard + viaSubledger bypass.</t>
         </is>
       </c>
       <c r="O90" s="12" t="inlineStr">
         <is>
-          <t>Issue an advance (1180 up); settle 700+300 clears 1180; mismatched settle → SETTLE_MISMATCH (re-performed by the harness).</t>
+          <t>Re-perform: create an account with gl_coa → 201; attempt to deactivate an account with balance → ACCOUNT_HAS_BALANCE; post directly to account 1100 without viaSubledger → CONTROL_ACCOUNT (re-performed by TC-GL-11-01/02/03 UAT cases).</t>
         </is>
       </c>
       <c r="P90" s="12" t="inlineStr">
         <is>
-          <t>Advance register; outstanding float</t>
+          <t>CoA change log (audit_log); permission test; control-account guard test</t>
         </is>
       </c>
       <c r="Q90" s="18" t="inlineStr">
@@ -8713,12 +8713,12 @@
     <row r="91">
       <c r="A91" s="15" t="inlineStr">
         <is>
-          <t>EXP-08</t>
+          <t>GL-12</t>
         </is>
       </c>
       <c r="B91" s="16" t="inlineStr">
         <is>
-          <t>Expenditure</t>
+          <t>General Ledger</t>
         </is>
       </c>
       <c r="C91" s="17" t="inlineStr">
@@ -8728,22 +8728,22 @@
       </c>
       <c r="D91" s="16" t="inlineStr">
         <is>
-          <t>Cash; Operating expense</t>
+          <t>All</t>
         </is>
       </c>
       <c r="E91" s="16" t="inlineStr">
         <is>
-          <t>Petty-cash disbursed beyond authority / without independent review, or drawn past the fund's limit — cash leakage, unauthorised or unrecorded expense, over-extended float.</t>
+          <t>Account-assignment errors introduced by scattered inline account-code literals in service code; a tenant needing a different account for a given business event has no mechanism to override without a code change.</t>
         </is>
       </c>
       <c r="F91" s="16" t="inlineStr">
         <is>
-          <t>Authorization; Completeness</t>
+          <t>Authorization/Accuracy</t>
         </is>
       </c>
       <c r="G91" s="16" t="inlineStr">
         <is>
-          <t>Petty-cash imprest float + maker-checker on disbursement (SoD): a fund holds cash capped at a credit limit/วงเงิน (1015 Petty Cash, a cash account); each direct EXPENSE or ADVANCE is a REQUEST that posts NOTHING and a DIFFERENT user must approve before the GL posts (expense Dr &lt;expense&gt; / Cr 1015; advance Dr 1180 / Cr 1015) and the fund balance is decremented. Self-approval → SOD_VIOLATION (binds even Admin). A draw beyond the fund balance → INSUFFICIENT_FLOAT; establishing/replenishing above the float limit → OVER_FLOAT. Advances settle (Dr expense + Dr 1015 returned / Cr 1180), returning unused cash to the fund. Every request carries a document reference + receipt key + a status trail (StatusLog) and surfaces in the GOV-01 pending-approvals monitor.</t>
+          <t>Posting / Account-Determination Engine: two tables — posting_event_types (28 seeded event types, e.g. SALE.FOOD, GR.INVENTORY, DEPRECIATION.FA) and posting_rules (maps event × leg-order to semantic role → account_code + DR/CR side) — drive account assignment instead of hard-coded literals. PostingService.post(eventType, ctx) resolves the applicable rules (global defaults, or shadowed by tenant-specific overrides for the same leg_order), translates role-keyed amounts into DR/CR lines, and delegates to LedgerService.postEntry. If no active rules exist for an event the call fails with NO_POSTING_RULE. Tenant-specific rules require gl_posting_rules permission to create/update. PostingService.preview() provides a dry-run for audit.</t>
         </is>
       </c>
       <c r="H91" s="17" t="inlineStr">
@@ -8758,12 +8758,12 @@
       </c>
       <c r="J91" s="17" t="inlineStr">
         <is>
-          <t>Per disbursement</t>
+          <t>Event-driven</t>
         </is>
       </c>
       <c r="K91" s="16" t="inlineStr">
         <is>
-          <t>AP / Controller</t>
+          <t>Financial Controller</t>
         </is>
       </c>
       <c r="L91" s="17" t="inlineStr">
@@ -8773,22 +8773,22 @@
       </c>
       <c r="M91" s="16" t="inlineStr">
         <is>
-          <t>petty-cash.service.ts (establishFund/replenishFund float guards, createRequest INSUFFICIENT_FLOAT, approveRequest SoD+GL, rejectRequest, settleRequest); petty-cash.controller.ts (creditors/exec); schema/petty-cash.ts (petty_cash_funds, expense_requests) + migration 0139; finance.service.ts pendingApprovals (GOV-01 source 7); cutover/basics.ts + compliance.ts (ToE)</t>
+          <t>posting.service.ts (resolveRules, post, preview, listEventTypes, listRules, upsertRule); posting-rules.controller.ts (gl_posting_rules permission gate); schema/posting-rules.ts (posting_event_types, posting_rules tables); migration 0156 (tables + 28 event types + global-default rules); ledger.module.ts (PostingService exported); packages/shared/src/permissions.ts (gl_posting_rules sub-permission); cutover/basics.ts (golden-snapshot ToE)</t>
         </is>
       </c>
       <c r="N91" s="16" t="inlineStr">
         <is>
-          <t>Inspect the float ceiling + the request→approve flow + the approver≠requester check + that the request posts nothing until approval.</t>
+          <t>Inspect the rule-resolution logic + NO_POSTING_RULE fast-fail + tenant-shadow logic + gl_posting_rules permission gate.</t>
         </is>
       </c>
       <c r="O91" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: establish a fund (Dr 1015), request an expense (no GL), self-approve → SOD_VIOLATION, approve as a different user → Dr expense/Cr 1015 + fund down; over-balance draw → INSUFFICIENT_FLOAT; advance approve→settle clears 1180; replenish past float → OVER_FLOAT (re-performed by the harnesses).</t>
+          <t>Re-perform: preview DEPRECIATION.FA with dep_expense:1000 → DR 5200 / CR 1590; preview GR.INVENTORY with inventory:500 → DR 1200 / CR 2000; preview UNKNOWN_EVENT → NO_POSTING_RULE (400); event-type catalogue returns ≥20 entries (re-performed by TC-GL-12-01/02/03/04 UAT cases + basics.ts harness).</t>
         </is>
       </c>
       <c r="P91" s="16" t="inlineStr">
         <is>
-          <t>Fund register + disbursement approval log + SoD test</t>
+          <t>Posting-rule change log; preview dry-run; harness golden snapshot</t>
         </is>
       </c>
       <c r="Q91" s="18" t="inlineStr">
@@ -8800,12 +8800,12 @@
     <row r="92">
       <c r="A92" s="11" t="inlineStr">
         <is>
-          <t>FA-07</t>
+          <t>EXP-07</t>
         </is>
       </c>
       <c r="B92" s="12" t="inlineStr">
         <is>
-          <t>Fixed Assets</t>
+          <t>Expenditure</t>
         </is>
       </c>
       <c r="C92" s="13" t="inlineStr">
@@ -8815,22 +8815,22 @@
       </c>
       <c r="D92" s="12" t="inlineStr">
         <is>
-          <t>Property, Plant &amp; Equipment; Equity</t>
+          <t>Cash; Operating expense</t>
         </is>
       </c>
       <c r="E92" s="12" t="inlineStr">
         <is>
-          <t>Carrying amount not adjusted for revaluation/impairment — asset over/understated.</t>
+          <t>Petty-cash / employee advance issued but never accounted for — cash leakage, expense unrecorded.</t>
         </is>
       </c>
       <c r="F92" s="12" t="inlineStr">
         <is>
-          <t>Valuation</t>
+          <t>Existence/Completeness</t>
         </is>
       </c>
       <c r="G92" s="12" t="inlineStr">
         <is>
-          <t>Asset revaluation / impairment: an upward revaluation credits the revaluation surplus in equity (Dr 1500 / Cr 3200); a downward revaluation (impairment) debits impairment loss (Dr 5820 / Cr 1500). The gross 1500 moves by the delta so the register stays tied to the GL; a no-op revaluation is rejected (NO_CHANGE). Every event is logged for the audit trail.</t>
+          <t>Employee cash advances: issuing an advance debits the 1180 Employee Advances control (Dr 1180 / Cr 1000); settlement clears it against actual spend + returned cash (Dr expense + Dr 1000 / Cr 1180), enforced to reconcile (settled_expense + returned_cash must equal the advance → SETTLE_MISMATCH). The 1180 balance is the outstanding float subject to review.</t>
         </is>
       </c>
       <c r="H92" s="13" t="inlineStr">
@@ -8845,12 +8845,12 @@
       </c>
       <c r="J92" s="13" t="inlineStr">
         <is>
-          <t>Per event</t>
+          <t>Per advance</t>
         </is>
       </c>
       <c r="K92" s="12" t="inlineStr">
         <is>
-          <t>FaAccountant / Controller</t>
+          <t>AP / Controller</t>
         </is>
       </c>
       <c r="L92" s="13" t="inlineStr">
@@ -8860,22 +8860,22 @@
       </c>
       <c r="M92" s="12" t="inlineStr">
         <is>
-          <t>assets.service.ts (revalue up→3200 / down→5820, listRevaluations; dispose recycles surplus 3200→3100); assets.controller.ts (exec/creditors); schema/assets.ts (asset_revaluations) + migration 0120; cutover/basics.ts (ToE)</t>
+          <t>finance.service.ts (issueAdvance, settleAdvance reconcile-or-reject, listAdvances outstanding); finance.controller.ts (creditors/exec); schema/finance.ts (employee_advances) + migration 0120; cutover/basics.ts (ToE)</t>
         </is>
       </c>
       <c r="N92" s="12" t="inlineStr">
         <is>
-          <t>Inspect revaluation/impairment routing + audit log + disposal recycling.</t>
+          <t>Inspect issue/settle GL + settlement reconciliation guard.</t>
         </is>
       </c>
       <c r="O92" s="12" t="inlineStr">
         <is>
-          <t>Upward revaluation credits 3200; impairment debits 5820; no-change → NO_CHANGE; both events logged; on disposal the revaluation surplus is recycled to retained earnings (Dr 3200 / Cr 3100), not through P&amp;L (re-performed by the harness).</t>
+          <t>Issue an advance (1180 up); settle 700+300 clears 1180; mismatched settle → SETTLE_MISMATCH (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P92" s="12" t="inlineStr">
         <is>
-          <t>Revaluation log; disposal recycling JE</t>
+          <t>Advance register; outstanding float</t>
         </is>
       </c>
       <c r="Q92" s="18" t="inlineStr">
@@ -8887,12 +8887,12 @@
     <row r="93">
       <c r="A93" s="15" t="inlineStr">
         <is>
-          <t>FA-08</t>
+          <t>EXP-08</t>
         </is>
       </c>
       <c r="B93" s="16" t="inlineStr">
         <is>
-          <t>Fixed Assets</t>
+          <t>Expenditure</t>
         </is>
       </c>
       <c r="C93" s="17" t="inlineStr">
@@ -8902,22 +8902,22 @@
       </c>
       <c r="D93" s="16" t="inlineStr">
         <is>
-          <t>Property, Plant &amp; Equipment; Equity</t>
+          <t>Cash; Operating expense</t>
         </is>
       </c>
       <c r="E93" s="16" t="inlineStr">
         <is>
-          <t>Carrying amount changed by fair-value revaluation/impairment without independent review — the preparer revalues the asset and posts to equity/P&amp;L on their own (earnings/equity management).</t>
+          <t>Petty-cash disbursed beyond authority / without independent review, or drawn past the fund's limit — cash leakage, unauthorised or unrecorded expense, over-extended float.</t>
         </is>
       </c>
       <c r="F93" s="16" t="inlineStr">
         <is>
-          <t>Authorization</t>
+          <t>Authorization; Completeness</t>
         </is>
       </c>
       <c r="G93" s="16" t="inlineStr">
         <is>
-          <t>Asset-revaluation maker-checker (SoD): a revalue/impairment request posts its GL entry as a DRAFT (excluded from balances) and records status 'PendingApproval' WITHOUT moving the carrying value; a DIFFERENT user must approve before the JE is effective and the register is re-valued (approver ≠ preparer enforced regardless of permissions, reusing the GL-05 ledger approval). Reject voids the draft; only one revaluation may be pending per asset; the disposal surplus recycle counts only approved revaluations.</t>
+          <t>Petty-cash imprest float + maker-checker on disbursement (SoD): a fund holds cash capped at a credit limit/วงเงิน (1015 Petty Cash, a cash account); each direct EXPENSE or ADVANCE is a REQUEST that posts NOTHING and a DIFFERENT user must approve before the GL posts (expense Dr &lt;expense&gt; / Cr 1015; advance Dr 1180 / Cr 1015) and the fund balance is decremented. Self-approval → SOD_VIOLATION (binds even Admin). A draw beyond the fund balance → INSUFFICIENT_FLOAT; establishing/replenishing above the float limit → OVER_FLOAT. Advances settle (Dr expense + Dr 1015 returned / Cr 1180), returning unused cash to the fund. Every request carries a document reference + receipt key + a status trail (StatusLog) and surfaces in the GOV-01 pending-approvals monitor.</t>
         </is>
       </c>
       <c r="H93" s="17" t="inlineStr">
@@ -8932,12 +8932,12 @@
       </c>
       <c r="J93" s="17" t="inlineStr">
         <is>
-          <t>Per event</t>
+          <t>Per disbursement</t>
         </is>
       </c>
       <c r="K93" s="16" t="inlineStr">
         <is>
-          <t>FaAccountant / Controller</t>
+          <t>AP / Controller</t>
         </is>
       </c>
       <c r="L93" s="17" t="inlineStr">
@@ -8947,22 +8947,22 @@
       </c>
       <c r="M93" s="16" t="inlineStr">
         <is>
-          <t>assets.service.ts revalue(pendingApproval Draft)/approveRevaluation/rejectRevaluation; assets.controller.ts (:assetNo/revalue/approve|reject); schema/assets.ts asset_revaluations.status + migration 0134; cutover/basics.ts + compliance.ts (ToE)</t>
+          <t>petty-cash.service.ts (establishFund/replenishFund float guards, createRequest INSUFFICIENT_FLOAT, approveRequest SoD+GL, rejectRequest, settleRequest); petty-cash.controller.ts (creditors/exec); schema/petty-cash.ts (petty_cash_funds, expense_requests) + migration 0139; finance.service.ts pendingApprovals (GOV-01 source 7); cutover/basics.ts + compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N93" s="16" t="inlineStr">
         <is>
-          <t>Inspect Draft→approve flow + the approver≠preparer check + deferred carrying-value update.</t>
+          <t>Inspect the float ceiling + the request→approve flow + the approver≠requester check + that the request posts nothing until approval.</t>
         </is>
       </c>
       <c r="O93" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: request a revaluation (Draft JE excluded from 3200), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm the surplus/impairment + carrying value move only after approval (re-performed by the harnesses).</t>
+          <t>Re-perform: establish a fund (Dr 1015), request an expense (no GL), self-approve → SOD_VIOLATION, approve as a different user → Dr expense/Cr 1015 + fund down; over-balance draw → INSUFFICIENT_FLOAT; advance approve→settle clears 1180; replenish past float → OVER_FLOAT (re-performed by the harnesses).</t>
         </is>
       </c>
       <c r="P93" s="16" t="inlineStr">
         <is>
-          <t>Revaluation approval log + SoD test</t>
+          <t>Fund register + disbursement approval log + SoD test</t>
         </is>
       </c>
       <c r="Q93" s="18" t="inlineStr">
@@ -8974,12 +8974,12 @@
     <row r="94">
       <c r="A94" s="11" t="inlineStr">
         <is>
-          <t>LSE-01</t>
+          <t>FA-07</t>
         </is>
       </c>
       <c r="B94" s="12" t="inlineStr">
         <is>
-          <t>Leases</t>
+          <t>Fixed Assets</t>
         </is>
       </c>
       <c r="C94" s="13" t="inlineStr">
@@ -8989,22 +8989,22 @@
       </c>
       <c r="D94" s="12" t="inlineStr">
         <is>
-          <t>Right-of-use assets; Lease liabilities</t>
+          <t>Property, Plant &amp; Equipment; Equity</t>
         </is>
       </c>
       <c r="E94" s="12" t="inlineStr">
         <is>
-          <t>Lease not capitalised (IFRS 16 / TFRS 16) — ROU asset + lease liability omitted; interest/depreciation mis-stated.</t>
+          <t>Carrying amount not adjusted for revaluation/impairment — asset over/understated.</t>
         </is>
       </c>
       <c r="F94" s="12" t="inlineStr">
         <is>
-          <t>Completeness/Accuracy/Valuation</t>
+          <t>Valuation</t>
         </is>
       </c>
       <c r="G94" s="12" t="inlineStr">
         <is>
-          <t>Lease accounting: at commencement a right-of-use asset and lease liability are recognised at the present value of the lease payments (Dr 1600 / Cr 2600). The scheduled job lease_periodic_run posts each period — interest unwinding on the liability (Dr 5900), the cash payment reducing the liability (Dr 2600 / Cr 1000), and straight-line ROU depreciation (Dr 5210 / Cr 1690) — the last period clearing the liability + ROU exactly. Idempotent per (lease, period).</t>
+          <t>Asset revaluation / impairment: an upward revaluation credits the revaluation surplus in equity (Dr 1500 / Cr 3200); a downward revaluation (impairment) debits impairment loss (Dr 5820 / Cr 1500). The gross 1500 moves by the delta so the register stays tied to the GL; a no-op revaluation is rejected (NO_CHANGE). Every event is logged for the audit trail.</t>
         </is>
       </c>
       <c r="H94" s="13" t="inlineStr">
@@ -9019,12 +9019,12 @@
       </c>
       <c r="J94" s="13" t="inlineStr">
         <is>
-          <t>Per period / per lease</t>
+          <t>Per event</t>
         </is>
       </c>
       <c r="K94" s="12" t="inlineStr">
         <is>
-          <t>Controller</t>
+          <t>FaAccountant / Controller</t>
         </is>
       </c>
       <c r="L94" s="13" t="inlineStr">
@@ -9034,22 +9034,22 @@
       </c>
       <c r="M94" s="12" t="inlineStr">
         <is>
-          <t>leases.service.ts (createLease PV recognition, runDueLeases interest+payment+depreciation, modifyLease remeasurement); leases.controller.ts (gl_post); bi.service.ts (lease_periodic_run); schema/leases.ts (leases, rou_nbv) + migration 0120/0121; cutover/basics.ts (ToE)</t>
+          <t>assets.service.ts (revalue up→3200 / down→5820, listRevaluations; dispose recycles surplus 3200→3100); assets.controller.ts (exec/creditors); schema/assets.ts (asset_revaluations) + migration 0120; cutover/basics.ts (ToE)</t>
         </is>
       </c>
       <c r="N94" s="12" t="inlineStr">
         <is>
-          <t>Inspect PV recognition + periodic interest/payment/depreciation + final-period clearing + modification remeasurement.</t>
+          <t>Inspect revaluation/impairment routing + audit log + disposal recycling.</t>
         </is>
       </c>
       <c r="O94" s="12" t="inlineStr">
         <is>
-          <t>Commencement recognises ROU=liability=PV; periodic run posts interest+principal(=payment)+ROU depreciation; liability + ROU reduce; a modification remeasures the liability at the revised PV and adjusts the ROU by the same delta (Dr/Cr 1600↔2600), then depreciates over the remaining term (re-performed by the harness).</t>
+          <t>Upward revaluation credits 3200; impairment debits 5820; no-change → NO_CHANGE; both events logged; on disposal the revaluation surplus is recycled to retained earnings (Dr 3200 / Cr 3100), not through P&amp;L (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P94" s="12" t="inlineStr">
         <is>
-          <t>Lease register; periodic run log; modification remeasurement</t>
+          <t>Revaluation log; disposal recycling JE</t>
         </is>
       </c>
       <c r="Q94" s="18" t="inlineStr">
@@ -9061,12 +9061,12 @@
     <row r="95">
       <c r="A95" s="15" t="inlineStr">
         <is>
-          <t>REC-01</t>
+          <t>FA-08</t>
         </is>
       </c>
       <c r="B95" s="16" t="inlineStr">
         <is>
-          <t>Reconciliation</t>
+          <t>Fixed Assets</t>
         </is>
       </c>
       <c r="C95" s="17" t="inlineStr">
@@ -9076,67 +9076,67 @@
       </c>
       <c r="D95" s="16" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Property, Plant &amp; Equipment; Equity</t>
         </is>
       </c>
       <c r="E95" s="16" t="inlineStr">
         <is>
-          <t>Subledgers diverge from GL undetected.</t>
+          <t>Carrying amount changed by fair-value revaluation/impairment without independent review — the preparer revalues the asset and posts to equity/P&amp;L on their own (earnings/equity management).</t>
         </is>
       </c>
       <c r="F95" s="16" t="inlineStr">
         <is>
-          <t>Completeness/Accuracy</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="G95" s="16" t="inlineStr">
         <is>
-          <t>Subledger-to-GL reconciliation per period: import GL, auto-match, certify (sign-off via 'approvals').</t>
+          <t>Asset-revaluation maker-checker (SoD): a revalue/impairment request posts its GL entry as a DRAFT (excluded from balances) and records status 'PendingApproval' WITHOUT moving the carrying value; a DIFFERENT user must approve before the JE is effective and the register is re-valued (approver ≠ preparer enforced regardless of permissions, reusing the GL-05 ledger approval). Reject voids the draft; only one revaluation may be pending per asset; the disposal surplus recycle counts only approved revaluations.</t>
         </is>
       </c>
       <c r="H95" s="17" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I95" s="17" t="inlineStr">
         <is>
-          <t>Auto+Manual</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J95" s="17" t="inlineStr">
         <is>
-          <t>Monthly</t>
+          <t>Per event</t>
         </is>
       </c>
       <c r="K95" s="16" t="inlineStr">
         <is>
-          <t>Controller</t>
+          <t>FaAccountant / Controller</t>
         </is>
       </c>
       <c r="L95" s="17" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="M95" s="16" t="inlineStr">
         <is>
-          <t>reconciliation.service.ts (importGlItems/autoMatch/certify)</t>
+          <t>assets.service.ts revalue(pendingApproval Draft)/approveRevaluation/rejectRevaluation; assets.controller.ts (:assetNo/revalue/approve|reject); schema/assets.ts asset_revaluations.status + migration 0134; cutover/basics.ts + compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N95" s="16" t="inlineStr">
         <is>
-          <t>Inspect recon + certify gate.</t>
+          <t>Inspect Draft→approve flow + the approver≠preparer check + deferred carrying-value update.</t>
         </is>
       </c>
       <c r="O95" s="16" t="inlineStr">
         <is>
-          <t>Sample periods: reconciled, unmatched cleared, certified.</t>
+          <t>Re-perform: request a revaluation (Draft JE excluded from 3200), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm the surplus/impairment + carrying value move only after approval (re-performed by the harnesses).</t>
         </is>
       </c>
       <c r="P95" s="16" t="inlineStr">
         <is>
-          <t>Certified recon</t>
+          <t>Revaluation approval log + SoD test</t>
         </is>
       </c>
       <c r="Q95" s="18" t="inlineStr">
@@ -9148,12 +9148,12 @@
     <row r="96">
       <c r="A96" s="11" t="inlineStr">
         <is>
-          <t>REC-02</t>
+          <t>LSE-01</t>
         </is>
       </c>
       <c r="B96" s="12" t="inlineStr">
         <is>
-          <t>Reconciliation</t>
+          <t>Leases</t>
         </is>
       </c>
       <c r="C96" s="13" t="inlineStr">
@@ -9163,22 +9163,22 @@
       </c>
       <c r="D96" s="12" t="inlineStr">
         <is>
-          <t>Cash</t>
+          <t>Right-of-use assets; Lease liabilities</t>
         </is>
       </c>
       <c r="E96" s="12" t="inlineStr">
         <is>
-          <t>Bank balance not reconciled to GL.</t>
+          <t>Lease not capitalised (IFRS 16 / TFRS 16) — ROU asset + lease liability omitted; interest/depreciation mis-stated.</t>
         </is>
       </c>
       <c r="F96" s="12" t="inlineStr">
         <is>
-          <t>Existence/Completeness</t>
+          <t>Completeness/Accuracy/Valuation</t>
         </is>
       </c>
       <c r="G96" s="12" t="inlineStr">
         <is>
-          <t>Bank reconciliation against statements.</t>
+          <t>Lease accounting: at commencement a right-of-use asset and lease liability are recognised at the present value of the lease payments (Dr 1600 / Cr 2600). The scheduled job lease_periodic_run posts each period — interest unwinding on the liability (Dr 5900), the cash payment reducing the liability (Dr 2600 / Cr 1000), and straight-line ROU depreciation (Dr 5210 / Cr 1690) — the last period clearing the liability + ROU exactly. Idempotent per (lease, period).</t>
         </is>
       </c>
       <c r="H96" s="13" t="inlineStr">
@@ -9188,12 +9188,12 @@
       </c>
       <c r="I96" s="13" t="inlineStr">
         <is>
-          <t>Auto+Manual</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J96" s="13" t="inlineStr">
         <is>
-          <t>Monthly</t>
+          <t>Per period / per lease</t>
         </is>
       </c>
       <c r="K96" s="12" t="inlineStr">
@@ -9203,27 +9203,27 @@
       </c>
       <c r="L96" s="13" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="M96" s="12" t="inlineStr">
         <is>
-          <t>bank module; drizzle/0015_bank_reconciliation</t>
+          <t>leases.service.ts (createLease PV recognition, runDueLeases interest+payment+depreciation, modifyLease remeasurement); leases.controller.ts (gl_post); bi.service.ts (lease_periodic_run); schema/leases.ts (leases, rou_nbv) + migration 0120/0121; cutover/basics.ts (ToE)</t>
         </is>
       </c>
       <c r="N96" s="12" t="inlineStr">
         <is>
-          <t>Inspect bank-rec process.</t>
+          <t>Inspect PV recognition + periodic interest/payment/depreciation + final-period clearing + modification remeasurement.</t>
         </is>
       </c>
       <c r="O96" s="12" t="inlineStr">
         <is>
-          <t>Sample months reconciled &amp; reviewed.</t>
+          <t>Commencement recognises ROU=liability=PV; periodic run posts interest+principal(=payment)+ROU depreciation; liability + ROU reduce; a modification remeasures the liability at the revised PV and adjusts the ROU by the same delta (Dr/Cr 1600↔2600), then depreciates over the remaining term (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P96" s="12" t="inlineStr">
         <is>
-          <t>Bank rec</t>
+          <t>Lease register; periodic run log; modification remeasurement</t>
         </is>
       </c>
       <c r="Q96" s="18" t="inlineStr">
@@ -9235,12 +9235,12 @@
     <row r="97">
       <c r="A97" s="15" t="inlineStr">
         <is>
-          <t>BANK-02</t>
+          <t>REC-01</t>
         </is>
       </c>
       <c r="B97" s="16" t="inlineStr">
         <is>
-          <t>Cash &amp; Treasury</t>
+          <t>Reconciliation</t>
         </is>
       </c>
       <c r="C97" s="17" t="inlineStr">
@@ -9250,37 +9250,37 @@
       </c>
       <c r="D97" s="16" t="inlineStr">
         <is>
-          <t>Cash; Operating expense; Interest income</t>
+          <t>All</t>
         </is>
       </c>
       <c r="E97" s="16" t="inlineStr">
         <is>
-          <t>A bank fee/interest adjustment is posted straight to the GL by one person during reconciliation — a cash outflow mis-booked as interest income, or a fictitious fee posted, with no independent review (single-person posting to the cash account).</t>
+          <t>Subledgers diverge from GL undetected.</t>
         </is>
       </c>
       <c r="F97" s="16" t="inlineStr">
         <is>
-          <t>Authorization/Accuracy</t>
+          <t>Completeness/Accuracy</t>
         </is>
       </c>
       <c r="G97" s="16" t="inlineStr">
         <is>
-          <t>Bank adjustment maker-checker (SoD): a fee/interest adjustment on a statement line is a REQUEST that posts a DRAFT JE (no balance/GL effect; the line stays unreconciled) until a DIFFERENT user with approval authority approves (POST /api/bank/lines/:id/adjustment/approve). Self-approval → SOD_VIOLATION (binds even Admin); approval flips the line to reconciled and the JE to Posted; reject voids the Draft and frees the line. The Draft JE (source BANKADJ) is also surfaced, aged, by the pending-approvals monitor (GOV-01).</t>
+          <t>Subledger-to-GL reconciliation per period: import GL, auto-match, certify (sign-off via 'approvals').</t>
         </is>
       </c>
       <c r="H97" s="17" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I97" s="17" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="J97" s="17" t="inlineStr">
         <is>
-          <t>Per adjustment</t>
+          <t>Monthly</t>
         </is>
       </c>
       <c r="K97" s="16" t="inlineStr">
@@ -9290,27 +9290,27 @@
       </c>
       <c r="L97" s="17" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="M97" s="16" t="inlineStr">
         <is>
-          <t>bank.service.ts requestAdjustment/approveAdjustment/rejectAdjustment/listPendingAdjustments (reuses ledger.approveEntry SoD); bank.controller.ts (lines/:id/adjustment requests; adjustment/approve|reject gated approvals/gl_close); cutover/bankrec.ts (ToE)</t>
+          <t>reconciliation.service.ts (importGlItems/autoMatch/certify)</t>
         </is>
       </c>
       <c r="N97" s="16" t="inlineStr">
         <is>
-          <t>Inspect the request→approve flow + the approver≠requester check + that the Draft posts nothing until approval.</t>
+          <t>Inspect recon + certify gate.</t>
         </is>
       </c>
       <c r="O97" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: request a fee adjustment (line unreconciled, GL difference unchanged), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm the difference closes to 0 only after approval (re-performed by the bankrec harness).</t>
+          <t>Sample periods: reconciled, unmatched cleared, certified.</t>
         </is>
       </c>
       <c r="P97" s="16" t="inlineStr">
         <is>
-          <t>Bank adjustment queue + SoD test</t>
+          <t>Certified recon</t>
         </is>
       </c>
       <c r="Q97" s="18" t="inlineStr">
@@ -9322,7 +9322,7 @@
     <row r="98">
       <c r="A98" s="11" t="inlineStr">
         <is>
-          <t>REC-03</t>
+          <t>REC-02</t>
         </is>
       </c>
       <c r="B98" s="12" t="inlineStr">
@@ -9337,22 +9337,22 @@
       </c>
       <c r="D98" s="12" t="inlineStr">
         <is>
-          <t>Consolidation</t>
+          <t>Cash</t>
         </is>
       </c>
       <c r="E98" s="12" t="inlineStr">
         <is>
-          <t>Intercompany balances not eliminated/agreed.</t>
+          <t>Bank balance not reconciled to GL.</t>
         </is>
       </c>
       <c r="F98" s="12" t="inlineStr">
         <is>
-          <t>Accuracy</t>
+          <t>Existence/Completeness</t>
         </is>
       </c>
       <c r="G98" s="12" t="inlineStr">
         <is>
-          <t>Intercompany reconciliation &amp; elimination on consolidation.</t>
+          <t>Bank reconciliation against statements.</t>
         </is>
       </c>
       <c r="H98" s="13" t="inlineStr">
@@ -9367,12 +9367,12 @@
       </c>
       <c r="J98" s="13" t="inlineStr">
         <is>
-          <t>Period</t>
+          <t>Monthly</t>
         </is>
       </c>
       <c r="K98" s="12" t="inlineStr">
         <is>
-          <t>Group Controller</t>
+          <t>Controller</t>
         </is>
       </c>
       <c r="L98" s="13" t="inlineStr">
@@ -9382,39 +9382,39 @@
       </c>
       <c r="M98" s="12" t="inlineStr">
         <is>
-          <t>intercompany; consolidation</t>
+          <t>bank module; drizzle/0015_bank_reconciliation</t>
         </is>
       </c>
       <c r="N98" s="12" t="inlineStr">
         <is>
-          <t>Inspect IC matching + elimination.</t>
+          <t>Inspect bank-rec process.</t>
         </is>
       </c>
       <c r="O98" s="12" t="inlineStr">
         <is>
-          <t>Sample IC pairs agree &amp; eliminate.</t>
+          <t>Sample months reconciled &amp; reviewed.</t>
         </is>
       </c>
       <c r="P98" s="12" t="inlineStr">
         <is>
-          <t>IC recon</t>
-        </is>
-      </c>
-      <c r="Q98" s="19" t="inlineStr">
-        <is>
-          <t>Partial</t>
+          <t>Bank rec</t>
+        </is>
+      </c>
+      <c r="Q98" s="18" t="inlineStr">
+        <is>
+          <t>Implemented</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="15" t="inlineStr">
         <is>
-          <t>REC-04</t>
+          <t>BANK-02</t>
         </is>
       </c>
       <c r="B99" s="16" t="inlineStr">
         <is>
-          <t>Reconciliation</t>
+          <t>Cash &amp; Treasury</t>
         </is>
       </c>
       <c r="C99" s="17" t="inlineStr">
@@ -9424,27 +9424,27 @@
       </c>
       <c r="D99" s="16" t="inlineStr">
         <is>
-          <t>All control accounts</t>
+          <t>Cash; Operating expense; Interest income</t>
         </is>
       </c>
       <c r="E99" s="16" t="inlineStr">
         <is>
-          <t>A sub-ledger silently drifts from its GL control account at period-end and no single review catches it (incomplete/inaccurate balances reach the financial statements).</t>
+          <t>A bank fee/interest adjustment is posted straight to the GL by one person during reconciliation — a cash outflow mis-booked as interest income, or a fictitious fee posted, with no independent review (single-person posting to the cash account).</t>
         </is>
       </c>
       <c r="F99" s="16" t="inlineStr">
         <is>
-          <t>Completeness/Accuracy</t>
+          <t>Authorization/Accuracy</t>
         </is>
       </c>
       <c r="G99" s="16" t="inlineStr">
         <is>
-          <t>Period-end control-account reconciliation PACK: one read (GET /api/finance/reconciliation/controls) ties every major sub-ledger to its GL control account and FLAGS any out-of-balance — AR↔1100, AP↔2000, Inventory↔1200, Gift cards/Customer-deposits↔2200, Deferred revenue↔2400 — reporting per line {sub_ledger, gl_control, variance, reconciled} plus an overall all_reconciled flag and an exceptions count. Liability controls are sign-flipped before comparison. The controller's single 'are the books reconciled?' close view; an exception is a control finding to investigate before sign-off.</t>
+          <t>Bank adjustment maker-checker (SoD): a fee/interest adjustment on a statement line is a REQUEST that posts a DRAFT JE (no balance/GL effect; the line stays unreconciled) until a DIFFERENT user with approval authority approves (POST /api/bank/lines/:id/adjustment/approve). Self-approval → SOD_VIOLATION (binds even Admin); approval flips the line to reconciled and the JE to Posted; reject voids the Draft and frees the line. The Draft JE (source BANKADJ) is also surfaced, aged, by the pending-approvals monitor (GOV-01).</t>
         </is>
       </c>
       <c r="H99" s="17" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I99" s="17" t="inlineStr">
@@ -9454,37 +9454,37 @@
       </c>
       <c r="J99" s="17" t="inlineStr">
         <is>
-          <t>Period / on demand</t>
+          <t>Per adjustment</t>
         </is>
       </c>
       <c r="K99" s="16" t="inlineStr">
         <is>
-          <t>Controller / CFO</t>
+          <t>Controller</t>
         </is>
       </c>
       <c r="L99" s="17" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="M99" s="16" t="inlineStr">
         <is>
-          <t>finance.service.ts reconcileControls; finance.controller.ts GET reconciliation/controls (exec/ar/creditors); reuses ledger.trialBalance + the AR/AP/inventory/gift-card/deferred sub-ledgers; cutover/giftcards.ts + compliance.ts (ToE)</t>
+          <t>bank.service.ts requestAdjustment/approveAdjustment/rejectAdjustment/listPendingAdjustments (reuses ledger.approveEntry SoD); bank.controller.ts (lines/:id/adjustment requests; adjustment/approve|reject gated approvals/gl_close); cutover/bankrec.ts (ToE)</t>
         </is>
       </c>
       <c r="N99" s="16" t="inlineStr">
         <is>
-          <t>Inspect the pack: each control account's sub-ledger query + the GL tie + the exceptions roll-up.</t>
+          <t>Inspect the request→approve flow + the approver≠requester check + that the Draft posts nothing until approval.</t>
         </is>
       </c>
       <c r="O99" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: with a clean set, every line reconciled + all_reconciled=true; introduce a known sub-ledger/GL difference and confirm it surfaces as an exception (re-performed: gift-card 2200 + inventory 1200 ties asserted by the harnesses).</t>
+          <t>Re-perform: request a fee adjustment (line unreconciled, GL difference unchanged), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm the difference closes to 0 only after approval (re-performed by the bankrec harness).</t>
         </is>
       </c>
       <c r="P99" s="16" t="inlineStr">
         <is>
-          <t>Reconciliation pack; exceptions list</t>
+          <t>Bank adjustment queue + SoD test</t>
         </is>
       </c>
       <c r="Q99" s="18" t="inlineStr">
@@ -9496,7 +9496,7 @@
     <row r="100">
       <c r="A100" s="11" t="inlineStr">
         <is>
-          <t>REC-05</t>
+          <t>REC-03</t>
         </is>
       </c>
       <c r="B100" s="12" t="inlineStr">
@@ -9511,27 +9511,27 @@
       </c>
       <c r="D100" s="12" t="inlineStr">
         <is>
-          <t>Cash; Bank</t>
+          <t>Consolidation</t>
         </is>
       </c>
       <c r="E100" s="12" t="inlineStr">
         <is>
-          <t>Till cash dropped to the safe never reaches the bank, or a deposit isn't matched to the statement — cash sits unbanked (theft/loss exposure) or the bank balance can't be tied to the books.</t>
+          <t>Intercompany balances not eliminated/agreed.</t>
         </is>
       </c>
       <c r="F100" s="12" t="inlineStr">
         <is>
-          <t>Completeness/Existence/Authorization</t>
+          <t>Accuracy</t>
         </is>
       </c>
       <c r="G100" s="12" t="inlineStr">
         <is>
-          <t>Cash banking — safe-drop → bank deposit → reconciliation: till 'drop's move cash from the drawer to the safe (drawer-only, no GL). Banking BATCHES the undeposited drops into a deposit and posts the GL (Dr &lt;bank account, e.g. 1010&gt; / Cr 1000 Cash), stamping each drop with the deposit id; the deposit is then RECONCILED to the bank statement (status Deposited→Reconciled). A detective read (GET /api/bank/deposits/undeposited-drops) surfaces the CASH STILL IN THE SAFE (drops with deposit_id NULL) — the unbanked exposure to chase. SoD: banking is a treasury duty (exec/ar) — segregated from the cashier (pos_till) who drops the cash, so the person who removes cash from the drawer is not the one who banks it.</t>
+          <t>Intercompany reconciliation &amp; elimination on consolidation.</t>
         </is>
       </c>
       <c r="H100" s="13" t="inlineStr">
         <is>
-          <t>Det/Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I100" s="13" t="inlineStr">
@@ -9541,12 +9541,12 @@
       </c>
       <c r="J100" s="13" t="inlineStr">
         <is>
-          <t>Per banking run</t>
+          <t>Period</t>
         </is>
       </c>
       <c r="K100" s="12" t="inlineStr">
         <is>
-          <t>FinancialController / Treasury</t>
+          <t>Group Controller</t>
         </is>
       </c>
       <c r="L100" s="13" t="inlineStr">
@@ -9556,39 +9556,39 @@
       </c>
       <c r="M100" s="12" t="inlineStr">
         <is>
-          <t>bank.service.ts undepositedDrops/createDeposit (Dr bank/Cr 1000, stamps deposit_id)/reconcileDeposit/listDeposits; bank.controller.ts (deposits, deposits/undeposited-drops, deposits/:id/reconcile; exec/ar); schema/cash.ts bank_deposits + cash_movements.deposit_id + migration 0152; /cash-banking UI; cutover/cash-banking.ts (ToE)</t>
+          <t>intercompany; consolidation</t>
         </is>
       </c>
       <c r="N100" s="12" t="inlineStr">
         <is>
-          <t>Inspect the undeposited-drop exposure read + the deposit GL (bank↔1000) + the reconcile step + the SoD (cashier vs treasury).</t>
+          <t>Inspect IC matching + elimination.</t>
         </is>
       </c>
       <c r="O100" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: two till drops → cash-in-safe shows the total; a cashier (pos_till) cannot bank (403); treasury banks → Dr bank / Cr 1000, cash-in-safe back to 0; reconcile the deposit; trial balance balanced (re-performed by the cash-banking harness).</t>
+          <t>Sample IC pairs agree &amp; eliminate.</t>
         </is>
       </c>
       <c r="P100" s="12" t="inlineStr">
         <is>
-          <t>Bank-deposit register; undeposited-drop (cash-in-safe) exposure</t>
-        </is>
-      </c>
-      <c r="Q100" s="18" t="inlineStr">
-        <is>
-          <t>Implemented</t>
+          <t>IC recon</t>
+        </is>
+      </c>
+      <c r="Q100" s="19" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="15" t="inlineStr">
         <is>
-          <t>GOV-01</t>
+          <t>REC-04</t>
         </is>
       </c>
       <c r="B101" s="16" t="inlineStr">
         <is>
-          <t>Monitoring</t>
+          <t>Reconciliation</t>
         </is>
       </c>
       <c r="C101" s="17" t="inlineStr">
@@ -9598,22 +9598,22 @@
       </c>
       <c r="D101" s="16" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>All control accounts</t>
         </is>
       </c>
       <c r="E101" s="16" t="inlineStr">
         <is>
-          <t>A maker-checker approval sits un-actioned and is forgotten — a transaction stalls before it is effective, or (worse) a control is quietly bypassed and no one notices an item never got its independent review.</t>
+          <t>A sub-ledger silently drifts from its GL control account at period-end and no single review catches it (incomplete/inaccurate balances reach the financial statements).</t>
         </is>
       </c>
       <c r="F101" s="16" t="inlineStr">
         <is>
-          <t>Authorization/Completeness</t>
+          <t>Completeness/Accuracy</t>
         </is>
       </c>
       <c r="G101" s="16" t="inlineStr">
         <is>
-          <t>Pending-approvals MONITOR (COSO monitoring): a single worklist of EVERY item awaiting independent approval across the system, each with its AGE in days and an overdue roll-up — spanning the manual-JE (GL-05), bank-adjustment (BANK-02), AP-disbursement (EXP-06), payroll (PAY-03), asset-revaluation (FA-08), asset-disposal (FA-09), inventory-write-off (INV-07), till-close cash over/short (REV-13), FX-rate (FX-04), budget (BUD-01) and large-refund (REV-16) maker-checkers. The controller reviews it before close; a stale item (age beyond the threshold) is a control finding to chase or escalate. The /approvals screen also lets a manager approve/reject a material till variance or a large refund inline (the pending types with no dedicated module screen). Read-only worklist; tenant-scoped via the caller's RLS.</t>
+          <t>Period-end control-account reconciliation PACK: one read (GET /api/finance/reconciliation/controls) ties every major sub-ledger to its GL control account and FLAGS any out-of-balance — AR↔1100, AP↔2000, Inventory↔1200, Gift cards/Customer-deposits↔2200, Deferred revenue↔2400 — reporting per line {sub_ledger, gl_control, variance, reconciled} plus an overall all_reconciled flag and an exceptions count. Liability controls are sign-flipped before comparison. The controller's single 'are the books reconciled?' close view; an exception is a control finding to investigate before sign-off.</t>
         </is>
       </c>
       <c r="H101" s="17" t="inlineStr">
@@ -9628,7 +9628,7 @@
       </c>
       <c r="J101" s="17" t="inlineStr">
         <is>
-          <t>Continuous / pre-close</t>
+          <t>Period / on demand</t>
         </is>
       </c>
       <c r="K101" s="16" t="inlineStr">
@@ -9643,22 +9643,22 @@
       </c>
       <c r="M101" s="16" t="inlineStr">
         <is>
-          <t>finance.service.ts pendingApprovals; finance.controller.ts GET approvals/pending (exec/approvals/creditors); aggregates journalEntries(Draft incl. BANKADJ→BANK-02)/apPayments/payruns/asset_revaluations/fixed_assets(disposal_pending)/inv_writeoff_requests/till_sessions(PendingApproval)/fx_rates(PendingApproval)/budgets(PendingApproval); cutover/compliance.ts (ToE)</t>
+          <t>finance.service.ts reconcileControls; finance.controller.ts GET reconciliation/controls (exec/ar/creditors); reuses ledger.trialBalance + the AR/AP/inventory/gift-card/deferred sub-ledgers; cutover/giftcards.ts + compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N101" s="16" t="inlineStr">
         <is>
-          <t>Inspect the aggregation across all pending sources + the age/overdue roll-up.</t>
+          <t>Inspect the pack: each control account's sub-ledger query + the GL tie + the exceptions roll-up.</t>
         </is>
       </c>
       <c r="O101" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: create a pending item (e.g. a Draft JE) and confirm it appears in the worklist with its control ID, amount and age; the overdue count flags items past the threshold (re-performed by the harness).</t>
+          <t>Re-perform: with a clean set, every line reconciled + all_reconciled=true; introduce a known sub-ledger/GL difference and confirm it surfaces as an exception (re-performed: gift-card 2200 + inventory 1200 ties asserted by the harnesses).</t>
         </is>
       </c>
       <c r="P101" s="16" t="inlineStr">
         <is>
-          <t>Pending-approvals worklist</t>
+          <t>Reconciliation pack; exceptions list</t>
         </is>
       </c>
       <c r="Q101" s="18" t="inlineStr">
@@ -9670,12 +9670,12 @@
     <row r="102">
       <c r="A102" s="11" t="inlineStr">
         <is>
-          <t>TAX-01</t>
+          <t>REC-05</t>
         </is>
       </c>
       <c r="B102" s="12" t="inlineStr">
         <is>
-          <t>Tax</t>
+          <t>Reconciliation</t>
         </is>
       </c>
       <c r="C102" s="13" t="inlineStr">
@@ -9685,67 +9685,67 @@
       </c>
       <c r="D102" s="12" t="inlineStr">
         <is>
-          <t>Tax (VAT)</t>
+          <t>Cash; Bank</t>
         </is>
       </c>
       <c r="E102" s="12" t="inlineStr">
         <is>
-          <t>VAT computed incorrectly → filing/penalty risk.</t>
+          <t>Till cash dropped to the safe never reaches the bank, or a deposit isn't matched to the statement — cash sits unbanked (theft/loss exposure) or the bank balance can't be tied to the books.</t>
         </is>
       </c>
       <c r="F102" s="12" t="inlineStr">
         <is>
-          <t>Accuracy</t>
+          <t>Completeness/Existence/Authorization</t>
         </is>
       </c>
       <c r="G102" s="12" t="inlineStr">
         <is>
-          <t>VAT via pluggable provider (TH 7%); unit-tested; no hard-coded rate.</t>
+          <t>Cash banking — safe-drop → bank deposit → reconciliation: till 'drop's move cash from the drawer to the safe (drawer-only, no GL). Banking BATCHES the undeposited drops into a deposit and posts the GL (Dr &lt;bank account, e.g. 1010&gt; / Cr 1000 Cash), stamping each drop with the deposit id; the deposit is then RECONCILED to the bank statement (status Deposited→Reconciled). A detective read (GET /api/bank/deposits/undeposited-drops) surfaces the CASH STILL IN THE SAFE (drops with deposit_id NULL) — the unbanked exposure to chase. SoD: banking is a treasury duty (exec/ar) — segregated from the cashier (pos_till) who drops the cash, so the person who removes cash from the drawer is not the one who banks it.</t>
         </is>
       </c>
       <c r="H102" s="13" t="inlineStr">
         <is>
-          <t>Auto</t>
+          <t>Det/Prev</t>
         </is>
       </c>
       <c r="I102" s="13" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="J102" s="13" t="inlineStr">
         <is>
-          <t>Per txn</t>
+          <t>Per banking run</t>
         </is>
       </c>
       <c r="K102" s="12" t="inlineStr">
         <is>
-          <t>Tax / Controller</t>
+          <t>FinancialController / Treasury</t>
         </is>
       </c>
       <c r="L102" s="13" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="M102" s="12" t="inlineStr">
         <is>
-          <t>tax/tax-providers.ts; tax.service.ts; test/unit.test.ts</t>
+          <t>bank.service.ts undepositedDrops/createDeposit (Dr bank/Cr 1000, stamps deposit_id)/reconcileDeposit/listDeposits; bank.controller.ts (deposits, deposits/undeposited-drops, deposits/:id/reconcile; exec/ar); schema/cash.ts bank_deposits + cash_movements.deposit_id + migration 0152; /cash-banking UI; cutover/cash-banking.ts (ToE)</t>
         </is>
       </c>
       <c r="N102" s="12" t="inlineStr">
         <is>
-          <t>Inspect rate provider + tests.</t>
+          <t>Inspect the undeposited-drop exposure read + the deposit GL (bank↔1000) + the reconcile step + the SoD (cashier vs treasury).</t>
         </is>
       </c>
       <c r="O102" s="12" t="inlineStr">
         <is>
-          <t>Re-perform VAT on sample; tie to return.</t>
+          <t>Re-perform: two till drops → cash-in-safe shows the total; a cashier (pos_till) cannot bank (403); treasury banks → Dr bank / Cr 1000, cash-in-safe back to 0; reconcile the deposit; trial balance balanced (re-performed by the cash-banking harness).</t>
         </is>
       </c>
       <c r="P102" s="12" t="inlineStr">
         <is>
-          <t>VAT tests</t>
+          <t>Bank-deposit register; undeposited-drop (cash-in-safe) exposure</t>
         </is>
       </c>
       <c r="Q102" s="18" t="inlineStr">
@@ -9757,12 +9757,12 @@
     <row r="103">
       <c r="A103" s="15" t="inlineStr">
         <is>
-          <t>TAX-02</t>
+          <t>GOV-01</t>
         </is>
       </c>
       <c r="B103" s="16" t="inlineStr">
         <is>
-          <t>Tax</t>
+          <t>Monitoring</t>
         </is>
       </c>
       <c r="C103" s="17" t="inlineStr">
@@ -9772,27 +9772,27 @@
       </c>
       <c r="D103" s="16" t="inlineStr">
         <is>
-          <t>Tax; Revenue</t>
+          <t>All</t>
         </is>
       </c>
       <c r="E103" s="16" t="inlineStr">
         <is>
-          <t>Non-compliant e-Tax invoice / not transmitted to ETDA.</t>
+          <t>A maker-checker approval sits un-actioned and is forgotten — a transaction stalls before it is effective, or (worse) a control is quietly bypassed and no one notices an item never got its independent review.</t>
         </is>
       </c>
       <c r="F103" s="16" t="inlineStr">
         <is>
-          <t>Accuracy/Compliance</t>
+          <t>Authorization/Completeness</t>
         </is>
       </c>
       <c r="G103" s="16" t="inlineStr">
         <is>
-          <t>e-Tax invoice (ETDA UBL 2.1 XML) generation + email with CC to ETDA timestamp mailbox.</t>
+          <t>Pending-approvals MONITOR (COSO monitoring): a single worklist of EVERY item awaiting independent approval across the system, each with its AGE in days and an overdue roll-up — spanning the manual-JE (GL-05), bank-adjustment (BANK-02), AP-disbursement (EXP-06), payroll (PAY-03), asset-revaluation (FA-08), asset-disposal (FA-09), inventory-write-off (INV-07), till-close cash over/short (REV-13), FX-rate (FX-04), budget (BUD-01) and large-refund (REV-16) maker-checkers. The controller reviews it before close; a stale item (age beyond the threshold) is a control finding to chase or escalate. The /approvals screen also lets a manager approve/reject a material till variance or a large refund inline (the pending types with no dedicated module screen). Read-only worklist; tenant-scoped via the caller's RLS.</t>
         </is>
       </c>
       <c r="H103" s="17" t="inlineStr">
         <is>
-          <t>Auto</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I103" s="17" t="inlineStr">
@@ -9802,37 +9802,37 @@
       </c>
       <c r="J103" s="17" t="inlineStr">
         <is>
-          <t>Per invoice</t>
+          <t>Continuous / pre-close</t>
         </is>
       </c>
       <c r="K103" s="16" t="inlineStr">
         <is>
-          <t>Tax</t>
+          <t>Controller / CFO</t>
         </is>
       </c>
       <c r="L103" s="17" t="inlineStr">
         <is>
-          <t>P10/P13</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="M103" s="16" t="inlineStr">
         <is>
-          <t>tax-docs/etax-xml.ts; etax-email.service.ts (tested)</t>
+          <t>finance.service.ts pendingApprovals; finance.controller.ts GET approvals/pending (exec/approvals/creditors); aggregates journalEntries(Draft incl. BANKADJ→BANK-02)/apPayments/payruns/asset_revaluations/fixed_assets(disposal_pending)/inv_writeoff_requests/till_sessions(PendingApproval)/fx_rates(PendingApproval)/budgets(PendingApproval); cutover/compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N103" s="16" t="inlineStr">
         <is>
-          <t>Inspect XML schema + email composer.</t>
+          <t>Inspect the aggregation across all pending sources + the age/overdue roll-up.</t>
         </is>
       </c>
       <c r="O103" s="16" t="inlineStr">
         <is>
-          <t>Sample invoices: valid XML, correct CC/escaping.</t>
+          <t>Re-perform: create a pending item (e.g. a Draft JE) and confirm it appears in the worklist with its control ID, amount and age; the overdue count flags items past the threshold (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P103" s="16" t="inlineStr">
         <is>
-          <t>e-Tax samples</t>
+          <t>Pending-approvals worklist</t>
         </is>
       </c>
       <c r="Q103" s="18" t="inlineStr">
@@ -9844,7 +9844,7 @@
     <row r="104">
       <c r="A104" s="11" t="inlineStr">
         <is>
-          <t>TAX-03</t>
+          <t>TAX-01</t>
         </is>
       </c>
       <c r="B104" s="12" t="inlineStr">
@@ -9859,12 +9859,12 @@
       </c>
       <c r="D104" s="12" t="inlineStr">
         <is>
-          <t>Tax (WHT)</t>
+          <t>Tax (VAT)</t>
         </is>
       </c>
       <c r="E104" s="12" t="inlineStr">
         <is>
-          <t>Withholding tax mis-computed / not reported.</t>
+          <t>VAT computed incorrectly → filing/penalty risk.</t>
         </is>
       </c>
       <c r="F104" s="12" t="inlineStr">
@@ -9874,7 +9874,7 @@
       </c>
       <c r="G104" s="12" t="inlineStr">
         <is>
-          <t>WHT computation and ภ.ง.ด. reporting.</t>
+          <t>VAT via pluggable provider (TH 7%); unit-tested; no hard-coded rate.</t>
         </is>
       </c>
       <c r="H104" s="13" t="inlineStr">
@@ -9889,12 +9889,12 @@
       </c>
       <c r="J104" s="13" t="inlineStr">
         <is>
-          <t>Per txn / monthly</t>
+          <t>Per txn</t>
         </is>
       </c>
       <c r="K104" s="12" t="inlineStr">
         <is>
-          <t>Tax</t>
+          <t>Tax / Controller</t>
         </is>
       </c>
       <c r="L104" s="13" t="inlineStr">
@@ -9904,34 +9904,34 @@
       </c>
       <c r="M104" s="12" t="inlineStr">
         <is>
-          <t>tax-reports; payroll</t>
+          <t>tax/tax-providers.ts; tax.service.ts; test/unit.test.ts</t>
         </is>
       </c>
       <c r="N104" s="12" t="inlineStr">
         <is>
-          <t>Inspect WHT logic + report.</t>
+          <t>Inspect rate provider + tests.</t>
         </is>
       </c>
       <c r="O104" s="12" t="inlineStr">
         <is>
-          <t>Re-perform WHT on sample; tie to filing.</t>
+          <t>Re-perform VAT on sample; tie to return.</t>
         </is>
       </c>
       <c r="P104" s="12" t="inlineStr">
         <is>
-          <t>WHT report</t>
-        </is>
-      </c>
-      <c r="Q104" s="19" t="inlineStr">
-        <is>
-          <t>Partial</t>
+          <t>VAT tests</t>
+        </is>
+      </c>
+      <c r="Q104" s="18" t="inlineStr">
+        <is>
+          <t>Implemented</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="15" t="inlineStr">
         <is>
-          <t>TAX-04</t>
+          <t>TAX-02</t>
         </is>
       </c>
       <c r="B105" s="16" t="inlineStr">
@@ -9946,27 +9946,27 @@
       </c>
       <c r="D105" s="16" t="inlineStr">
         <is>
-          <t>Tax (VAT); Tax Payable (2100)</t>
+          <t>Tax; Revenue</t>
         </is>
       </c>
       <c r="E105" s="16" t="inlineStr">
         <is>
-          <t>Output/input VAT on the filed ภ.พ.30 return does not agree to the GL — VAT liability mis-stated, a filing/penalty exposure, or a posting omission goes undetected before submission.</t>
+          <t>Non-compliant e-Tax invoice / not transmitted to ETDA.</t>
         </is>
       </c>
       <c r="F105" s="16" t="inlineStr">
         <is>
-          <t>Completeness/Accuracy</t>
+          <t>Accuracy/Compliance</t>
         </is>
       </c>
       <c r="G105" s="16" t="inlineStr">
         <is>
-          <t>Periodic VAT-return ↔ GL reconciliation (ภ.พ.30): the monthly return (GET /api/tax-reports/pp30) is built from the sales/output-VAT and purchase/input-VAT sub-reports, computes net VAT = output − input, and RECONCILES it to the **GL account 2100 (Tax Payable) net movement** for the same period (Σ credit − Σ debit over Posted entries) — returning `reconciliation.tied` = true only when the two agree within rounding. A non-tie is a detective finding to investigate and clear BEFORE filing (the form also carries the ม.157 deadline = the 15th of the next month). Output VAT is posted to 2100 on every sale (Cr) and reversed on returns (Dr); input VAT is posted on AP bills (Dr) — so 2100's net is the period's VAT payable. Read-only report; exportable to a ภ.พ.30 PDF/HTML.</t>
+          <t>e-Tax invoice (ETDA UBL 2.1 XML) generation + email with CC to ETDA timestamp mailbox.</t>
         </is>
       </c>
       <c r="H105" s="17" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Auto</t>
         </is>
       </c>
       <c r="I105" s="17" t="inlineStr">
@@ -9976,37 +9976,37 @@
       </c>
       <c r="J105" s="17" t="inlineStr">
         <is>
-          <t>Monthly / pre-filing</t>
+          <t>Per invoice</t>
         </is>
       </c>
       <c r="K105" s="16" t="inlineStr">
         <is>
-          <t>Tax / FinancialController</t>
+          <t>Tax</t>
         </is>
       </c>
       <c r="L105" s="17" t="inlineStr">
         <is>
-          <t>P10/P16</t>
+          <t>P10/P13</t>
         </is>
       </c>
       <c r="M105" s="16" t="inlineStr">
         <is>
-          <t>tax-reports.service.ts pp30 (outputVat/inputVat + 2100 net-movement tie); tax-reports.controller.ts (GET pp30, pp30/export, exec); tax-reports-pdf.ts; dine-in.service.ts/returns.service.ts/finance.service.ts post 2100 on sale/return/AP; /tax/reports UI; cutover/taxdocs.ts (ToE)</t>
+          <t>tax-docs/etax-xml.ts; etax-email.service.ts (tested)</t>
         </is>
       </c>
       <c r="N105" s="16" t="inlineStr">
         <is>
-          <t>Inspect the pp30 build + the 2100 net-movement query + the tie flag + the filing deadline.</t>
+          <t>Inspect XML schema + email composer.</t>
         </is>
       </c>
       <c r="O105" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: the pp30 return computes net VAT (output − input), the GL 2100 net movement reflects the posted input VAT, and the reconciliation block exposes the gl_account (2100), the report net VAT and a boolean tie verdict (tied iff the two agree within rounding); the ภ.พ.30 export renders (re-performed by the taxdocs harness).</t>
+          <t>Sample invoices: valid XML, correct CC/escaping.</t>
         </is>
       </c>
       <c r="P105" s="16" t="inlineStr">
         <is>
-          <t>ภ.พ.30 return + GL-2100 reconciliation tie</t>
+          <t>e-Tax samples</t>
         </is>
       </c>
       <c r="Q105" s="18" t="inlineStr">
@@ -10018,12 +10018,12 @@
     <row r="106">
       <c r="A106" s="11" t="inlineStr">
         <is>
-          <t>PAY-01</t>
+          <t>TAX-03</t>
         </is>
       </c>
       <c r="B106" s="12" t="inlineStr">
         <is>
-          <t>Payroll</t>
+          <t>Tax</t>
         </is>
       </c>
       <c r="C106" s="13" t="inlineStr">
@@ -10033,12 +10033,12 @@
       </c>
       <c r="D106" s="12" t="inlineStr">
         <is>
-          <t>Payroll expense/liability</t>
+          <t>Tax (WHT)</t>
         </is>
       </c>
       <c r="E106" s="12" t="inlineStr">
         <is>
-          <t>Payroll, SSO and PIT mis-computed.</t>
+          <t>Withholding tax mis-computed / not reported.</t>
         </is>
       </c>
       <c r="F106" s="12" t="inlineStr">
@@ -10048,7 +10048,7 @@
       </c>
       <c r="G106" s="12" t="inlineStr">
         <is>
-          <t>Payroll engine — SSO 5% (cap 750), progressive PIT, payslip net; unit-tested.</t>
+          <t>WHT computation and ภ.ง.ด. reporting.</t>
         </is>
       </c>
       <c r="H106" s="13" t="inlineStr">
@@ -10063,12 +10063,12 @@
       </c>
       <c r="J106" s="13" t="inlineStr">
         <is>
-          <t>Per run</t>
+          <t>Per txn / monthly</t>
         </is>
       </c>
       <c r="K106" s="12" t="inlineStr">
         <is>
-          <t>HR / Payroll</t>
+          <t>Tax</t>
         </is>
       </c>
       <c r="L106" s="13" t="inlineStr">
@@ -10078,39 +10078,39 @@
       </c>
       <c r="M106" s="12" t="inlineStr">
         <is>
-          <t>payroll/payroll-calc.ts; test/unit.test.ts</t>
+          <t>tax-reports; payroll</t>
         </is>
       </c>
       <c r="N106" s="12" t="inlineStr">
         <is>
-          <t>Inspect calc + tests.</t>
+          <t>Inspect WHT logic + report.</t>
         </is>
       </c>
       <c r="O106" s="12" t="inlineStr">
         <is>
-          <t>Re-perform sample payslips.</t>
+          <t>Re-perform WHT on sample; tie to filing.</t>
         </is>
       </c>
       <c r="P106" s="12" t="inlineStr">
         <is>
-          <t>Payslip tests</t>
-        </is>
-      </c>
-      <c r="Q106" s="18" t="inlineStr">
-        <is>
-          <t>Implemented</t>
+          <t>WHT report</t>
+        </is>
+      </c>
+      <c r="Q106" s="19" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="15" t="inlineStr">
         <is>
-          <t>PAY-02</t>
+          <t>TAX-04</t>
         </is>
       </c>
       <c r="B107" s="16" t="inlineStr">
         <is>
-          <t>Payroll</t>
+          <t>Tax</t>
         </is>
       </c>
       <c r="C107" s="17" t="inlineStr">
@@ -10120,22 +10120,22 @@
       </c>
       <c r="D107" s="16" t="inlineStr">
         <is>
-          <t>Payroll liability</t>
+          <t>Tax (VAT); Tax Payable (2100)</t>
         </is>
       </c>
       <c r="E107" s="16" t="inlineStr">
         <is>
-          <t>Statutory withholdings (SSO/WHT/PF) mis-stated or not remitted, so the liability owed to the authorities diverges from the books.</t>
+          <t>Output/input VAT on the filed ภ.พ.30 return does not agree to the GL — VAT liability mis-stated, a filing/penalty exposure, or a posting omission goes undetected before submission.</t>
         </is>
       </c>
       <c r="F107" s="16" t="inlineStr">
         <is>
-          <t>Accuracy/Compliance</t>
+          <t>Completeness/Accuracy</t>
         </is>
       </c>
       <c r="G107" s="16" t="inlineStr">
         <is>
-          <t>Payroll-liability schedule (GET /api/payroll/liabilities): each statutory account — SSO 2350, WHT/PND1 2360, PF 2370 — shows accrued (GL credits) − remitted (GL debits) = outstanding, tied back to the INDEPENDENT payrun accrual with a `reconciled` flag (a divergence flags a manual JE that touched a payroll-liability account outside the payroll process). Treasury remits the cash (POST .../remit → Dr liability / Cr 1000) which clears the outstanding and keeps the books reconciled to the statutory filings; a remittance beyond the outstanding is blocked (REMIT_EXCEEDS_OUTSTANDING).</t>
+          <t>Periodic VAT-return ↔ GL reconciliation (ภ.พ.30): the monthly return (GET /api/tax-reports/pp30) is built from the sales/output-VAT and purchase/input-VAT sub-reports, computes net VAT = output − input, and RECONCILES it to the **GL account 2100 (Tax Payable) net movement** for the same period (Σ credit − Σ debit over Posted entries) — returning `reconciliation.tied` = true only when the two agree within rounding. A non-tie is a detective finding to investigate and clear BEFORE filing (the form also carries the ม.157 deadline = the 15th of the next month). Output VAT is posted to 2100 on every sale (Cr) and reversed on returns (Dr); input VAT is posted on AP bills (Dr) — so 2100's net is the period's VAT payable. Read-only report; exportable to a ภ.พ.30 PDF/HTML.</t>
         </is>
       </c>
       <c r="H107" s="17" t="inlineStr">
@@ -10150,37 +10150,37 @@
       </c>
       <c r="J107" s="17" t="inlineStr">
         <is>
-          <t>Per run / monthly</t>
+          <t>Monthly / pre-filing</t>
         </is>
       </c>
       <c r="K107" s="16" t="inlineStr">
         <is>
-          <t>HR / Payroll / Treasury</t>
+          <t>Tax / FinancialController</t>
         </is>
       </c>
       <c r="L107" s="17" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P10/P16</t>
         </is>
       </c>
       <c r="M107" s="16" t="inlineStr">
         <is>
-          <t>payroll/payroll.service.ts liabilities/remitLiability</t>
+          <t>tax-reports.service.ts pp30 (outputVat/inputVat + 2100 net-movement tie); tax-reports.controller.ts (GET pp30, pp30/export, exec); tax-reports-pdf.ts; dine-in.service.ts/returns.service.ts/finance.service.ts post 2100 on sale/return/AP; /tax/reports UI; cutover/taxdocs.ts (ToE)</t>
         </is>
       </c>
       <c r="N107" s="16" t="inlineStr">
         <is>
-          <t>Inspect the schedule + the accrued/remitted/outstanding tie-out and the reconciled flag.</t>
+          <t>Inspect the pp30 build + the 2100 net-movement query + the tie flag + the filing deadline.</t>
         </is>
       </c>
       <c r="O107" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: run a payroll, confirm the SSO/WHT outstanding equals the payrun accrual; remit part and confirm the outstanding falls and the TB stays balanced; attempt an over-remit (REMIT_EXCEEDS_OUTSTANDING).</t>
+          <t>Re-perform: the pp30 return computes net VAT (output − input), the GL 2100 net movement reflects the posted input VAT, and the reconciliation block exposes the gl_account (2100), the report net VAT and a boolean tie verdict (tied iff the two agree within rounding); the ภ.พ.30 export renders (re-performed by the taxdocs harness).</t>
         </is>
       </c>
       <c r="P107" s="16" t="inlineStr">
         <is>
-          <t>Liability schedule + remittance JEs tied to filings</t>
+          <t>ภ.พ.30 return + GL-2100 reconciliation tie</t>
         </is>
       </c>
       <c r="Q107" s="18" t="inlineStr">
@@ -10192,7 +10192,7 @@
     <row r="108">
       <c r="A108" s="11" t="inlineStr">
         <is>
-          <t>PAY-03</t>
+          <t>PAY-01</t>
         </is>
       </c>
       <c r="B108" s="12" t="inlineStr">
@@ -10207,27 +10207,27 @@
       </c>
       <c r="D108" s="12" t="inlineStr">
         <is>
-          <t>Payroll expense/liability; Cash</t>
+          <t>Payroll expense/liability</t>
         </is>
       </c>
       <c r="E108" s="12" t="inlineStr">
         <is>
-          <t>Payroll run posted to the GL without independent review — the preparer both computes and posts their own payroll (ghost employees, inflated rate/hours).</t>
+          <t>Payroll, SSO and PIT mis-computed.</t>
         </is>
       </c>
       <c r="F108" s="12" t="inlineStr">
         <is>
-          <t>Authorization</t>
+          <t>Accuracy</t>
         </is>
       </c>
       <c r="G108" s="12" t="inlineStr">
         <is>
-          <t>Payroll maker-checker (SoD): a run posts its GL entry as a DRAFT (excluded from balances) with the run record 'PendingApproval'; a DIFFERENT user must approve before it becomes effective (approver ≠ preparer enforced regardless of permissions, reusing the GL-05 ledger approval). Reject voids the draft; idempotent per (tenant, period).</t>
+          <t>Payroll engine — SSO 5% (cap 750), progressive PIT, payslip net; unit-tested.</t>
         </is>
       </c>
       <c r="H108" s="13" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Auto</t>
         </is>
       </c>
       <c r="I108" s="13" t="inlineStr">
@@ -10242,7 +10242,7 @@
       </c>
       <c r="K108" s="12" t="inlineStr">
         <is>
-          <t>HR / Payroll; Controller</t>
+          <t>HR / Payroll</t>
         </is>
       </c>
       <c r="L108" s="13" t="inlineStr">
@@ -10252,22 +10252,22 @@
       </c>
       <c r="M108" s="12" t="inlineStr">
         <is>
-          <t>payroll/payroll.service.ts approvePayroll/rejectPayroll; migration 0133</t>
+          <t>payroll/payroll-calc.ts; test/unit.test.ts</t>
         </is>
       </c>
       <c r="N108" s="12" t="inlineStr">
         <is>
-          <t>Inspect Draft→approve flow + the approver≠preparer check.</t>
+          <t>Inspect calc + tests.</t>
         </is>
       </c>
       <c r="O108" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: run as A, attempt self-approve (SOD_VIOLATION), approve as B; confirm the JE hits balances only after approval.</t>
+          <t>Re-perform sample payslips.</t>
         </is>
       </c>
       <c r="P108" s="12" t="inlineStr">
         <is>
-          <t>Approval log + SoD test</t>
+          <t>Payslip tests</t>
         </is>
       </c>
       <c r="Q108" s="18" t="inlineStr">
@@ -10279,12 +10279,12 @@
     <row r="109">
       <c r="A109" s="15" t="inlineStr">
         <is>
-          <t>FA-09</t>
+          <t>PAY-02</t>
         </is>
       </c>
       <c r="B109" s="16" t="inlineStr">
         <is>
-          <t>Fixed Assets</t>
+          <t>Payroll</t>
         </is>
       </c>
       <c r="C109" s="17" t="inlineStr">
@@ -10294,27 +10294,27 @@
       </c>
       <c r="D109" s="16" t="inlineStr">
         <is>
-          <t>Property, Plant &amp; Equipment; Cash</t>
+          <t>Payroll liability</t>
         </is>
       </c>
       <c r="E109" s="16" t="inlineStr">
         <is>
-          <t>Asset disposed without independent review — one person writes an asset off the books and records the proceeds (asset-stripping / theft: dispose a still-held asset, or to a related party below value).</t>
+          <t>Statutory withholdings (SSO/WHT/PF) mis-stated or not remitted, so the liability owed to the authorities diverges from the books.</t>
         </is>
       </c>
       <c r="F109" s="16" t="inlineStr">
         <is>
-          <t>Authorization</t>
+          <t>Accuracy/Compliance</t>
         </is>
       </c>
       <c r="G109" s="16" t="inlineStr">
         <is>
-          <t>Asset-disposal maker-checker (SoD): a disposal REQUEST posts its GL entry as a DRAFT (excluded from balances) and flags the asset disposal_pending WITHOUT marking it disposed or moving the register; a DIFFERENT user must approve before it is effective (status→disposed, revaluation surplus recycled 3200→3100) (approver ≠ requester enforced regardless of permissions, reusing the GL-05 ledger approval). Reject voids the draft and the asset stays in service; only one disposal may be pending per asset; a disposal-pending asset is frozen from depreciation.</t>
+          <t>Payroll-liability schedule (GET /api/payroll/liabilities): each statutory account — SSO 2350, WHT/PND1 2360, PF 2370 — shows accrued (GL credits) − remitted (GL debits) = outstanding, tied back to the INDEPENDENT payrun accrual with a `reconciled` flag (a divergence flags a manual JE that touched a payroll-liability account outside the payroll process). Treasury remits the cash (POST .../remit → Dr liability / Cr 1000) which clears the outstanding and keeps the books reconciled to the statutory filings; a remittance beyond the outstanding is blocked (REMIT_EXCEEDS_OUTSTANDING).</t>
         </is>
       </c>
       <c r="H109" s="17" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I109" s="17" t="inlineStr">
@@ -10324,12 +10324,12 @@
       </c>
       <c r="J109" s="17" t="inlineStr">
         <is>
-          <t>Per disposal</t>
+          <t>Per run / monthly</t>
         </is>
       </c>
       <c r="K109" s="16" t="inlineStr">
         <is>
-          <t>FaAccountant / Controller</t>
+          <t>HR / Payroll / Treasury</t>
         </is>
       </c>
       <c r="L109" s="17" t="inlineStr">
@@ -10339,22 +10339,22 @@
       </c>
       <c r="M109" s="16" t="inlineStr">
         <is>
-          <t>assets.service.ts dispose(pendingApproval Draft)/approveDisposal/rejectDisposal; assets.controller.ts (:assetNo/dispose/approve|reject); schema/assets.ts fixed_assets.disposal_pending + migration 0135; cutover/basics.ts + worldclass.ts + compliance.ts (ToE)</t>
+          <t>payroll/payroll.service.ts liabilities/remitLiability</t>
         </is>
       </c>
       <c r="N109" s="16" t="inlineStr">
         <is>
-          <t>Inspect Draft→approve flow + the approver≠requester check + deferred status/recycle.</t>
+          <t>Inspect the schedule + the accrued/remitted/outstanding tie-out and the reconciled flag.</t>
         </is>
       </c>
       <c r="O109" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: request a disposal (Draft JE excluded), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm status→disposed + surplus recycled only after approval (re-performed by the harnesses).</t>
+          <t>Re-perform: run a payroll, confirm the SSO/WHT outstanding equals the payrun accrual; remit part and confirm the outstanding falls and the TB stays balanced; attempt an over-remit (REMIT_EXCEEDS_OUTSTANDING).</t>
         </is>
       </c>
       <c r="P109" s="16" t="inlineStr">
         <is>
-          <t>Disposal approval log + SoD test</t>
+          <t>Liability schedule + remittance JEs tied to filings</t>
         </is>
       </c>
       <c r="Q109" s="18" t="inlineStr">
@@ -10366,12 +10366,12 @@
     <row r="110">
       <c r="A110" s="11" t="inlineStr">
         <is>
-          <t>FA-10</t>
+          <t>PAY-03</t>
         </is>
       </c>
       <c r="B110" s="12" t="inlineStr">
         <is>
-          <t>Fixed Assets</t>
+          <t>Payroll</t>
         </is>
       </c>
       <c r="C110" s="13" t="inlineStr">
@@ -10381,22 +10381,22 @@
       </c>
       <c r="D110" s="12" t="inlineStr">
         <is>
-          <t>Property, Plant &amp; Equipment; Accounts Payable</t>
+          <t>Payroll expense/liability; Cash</t>
         </is>
       </c>
       <c r="E110" s="12" t="inlineStr">
         <is>
-          <t>Capital purchases mis-capitalised or capitalised without independent review — the person who receives the goods also decides what enters the asset register and at what cost/useful life (fictitious or over-valued assets; capex/opex mis-classification).</t>
+          <t>Payroll run posted to the GL without independent review — the preparer both computes and posts their own payroll (ghost employees, inflated rate/hours).</t>
         </is>
       </c>
       <c r="F110" s="12" t="inlineStr">
         <is>
-          <t>Authorization; Accuracy</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="G110" s="12" t="inlineStr">
         <is>
-          <t>Procure-to-Capitalize maker-checker (SoD): a goods-receipt line flagged capital (item-master is_fixed_asset or per-PO-line override) is excluded from inventory capitalisation (1200) at receipt and instead becomes ELIGIBLE for the asset register. Capitalisation is a REQUEST that posts NOTHING to the GL; a DIFFERENT user must approve before the fixed_assets row + acquisition JE (Dr 1500 / Cr 2000) are created (approver ≠ requester enforced regardless of permissions). The created asset carries its source GR/PO for end-to-end PR→PO→GR→FA traceability; a GR line cannot be capitalised twice.</t>
+          <t>Payroll maker-checker (SoD): a run posts its GL entry as a DRAFT (excluded from balances) with the run record 'PendingApproval'; a DIFFERENT user must approve before it becomes effective (approver ≠ preparer enforced regardless of permissions, reusing the GL-05 ledger approval). Reject voids the draft; idempotent per (tenant, period).</t>
         </is>
       </c>
       <c r="H110" s="13" t="inlineStr">
@@ -10411,12 +10411,12 @@
       </c>
       <c r="J110" s="13" t="inlineStr">
         <is>
-          <t>Per capital receipt</t>
+          <t>Per run</t>
         </is>
       </c>
       <c r="K110" s="12" t="inlineStr">
         <is>
-          <t>FaAccountant / Controller</t>
+          <t>HR / Payroll; Controller</t>
         </is>
       </c>
       <c r="L110" s="13" t="inlineStr">
@@ -10426,22 +10426,22 @@
       </c>
       <c r="M110" s="12" t="inlineStr">
         <is>
-          <t>assets.service.ts registerFromGr/approveRegistration/rejectRegistration/eligibleFromGr; assets.controller.ts (registrations*); procurement.service.ts createGr (is_capital routing, costing excluded); schema/assets.ts asset_registration_requests + fixed_assets.source_gr_no/po_no + migration 0137; cutover/basics.ts + compliance.ts (ToE)</t>
+          <t>payroll/payroll.service.ts approvePayroll/rejectPayroll; migration 0133</t>
         </is>
       </c>
       <c r="N110" s="12" t="inlineStr">
         <is>
-          <t>Inspect the eligible→request→approve flow + approver≠requester check + the inventory-vs-asset routing of capital lines.</t>
+          <t>Inspect Draft→approve flow + the approver≠preparer check.</t>
         </is>
       </c>
       <c r="O110" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: receive a capital line, raise a registration (no GL), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm the asset + Dr 1500/Cr 2000 post only after approval and the line cannot be re-registered (re-performed by the harnesses).</t>
+          <t>Re-perform: run as A, attempt self-approve (SOD_VIOLATION), approve as B; confirm the JE hits balances only after approval.</t>
         </is>
       </c>
       <c r="P110" s="12" t="inlineStr">
         <is>
-          <t>Capitalization approval log + SoD test</t>
+          <t>Approval log + SoD test</t>
         </is>
       </c>
       <c r="Q110" s="18" t="inlineStr">
@@ -10453,12 +10453,12 @@
     <row r="111">
       <c r="A111" s="15" t="inlineStr">
         <is>
-          <t>CON-01</t>
+          <t>FA-09</t>
         </is>
       </c>
       <c r="B111" s="16" t="inlineStr">
         <is>
-          <t>Consolidation &amp; FX</t>
+          <t>Fixed Assets</t>
         </is>
       </c>
       <c r="C111" s="17" t="inlineStr">
@@ -10468,42 +10468,42 @@
       </c>
       <c r="D111" s="16" t="inlineStr">
         <is>
-          <t>Consolidation</t>
+          <t>Property, Plant &amp; Equipment; Cash</t>
         </is>
       </c>
       <c r="E111" s="16" t="inlineStr">
         <is>
-          <t>Group consolidation mis-stated (ownership/currency).</t>
+          <t>Asset disposed without independent review — one person writes an asset off the books and records the proceeds (asset-stripping / theft: dispose a still-held asset, or to a related party below value).</t>
         </is>
       </c>
       <c r="F111" s="16" t="inlineStr">
         <is>
-          <t>Accuracy</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="G111" s="16" t="inlineStr">
         <is>
-          <t>Consolidation run (ownership %, entity currency) gated by 'approvals'.</t>
+          <t>Asset-disposal maker-checker (SoD): a disposal REQUEST posts its GL entry as a DRAFT (excluded from balances) and flags the asset disposal_pending WITHOUT marking it disposed or moving the register; a DIFFERENT user must approve before it is effective (status→disposed, revaluation surplus recycled 3200→3100) (approver ≠ requester enforced regardless of permissions, reusing the GL-05 ledger approval). Reject voids the draft and the asset stays in service; only one disposal may be pending per asset; a disposal-pending asset is frozen from depreciation.</t>
         </is>
       </c>
       <c r="H111" s="17" t="inlineStr">
         <is>
-          <t>Auto+Manual</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I111" s="17" t="inlineStr">
         <is>
-          <t>Period</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J111" s="17" t="inlineStr">
         <is>
-          <t>Period</t>
+          <t>Per disposal</t>
         </is>
       </c>
       <c r="K111" s="16" t="inlineStr">
         <is>
-          <t>Group Controller</t>
+          <t>FaAccountant / Controller</t>
         </is>
       </c>
       <c r="L111" s="17" t="inlineStr">
@@ -10513,22 +10513,22 @@
       </c>
       <c r="M111" s="16" t="inlineStr">
         <is>
-          <t>consolidation.service.ts (runConsolidation @Permissions approvals)</t>
+          <t>assets.service.ts dispose(pendingApproval Draft)/approveDisposal/rejectDisposal; assets.controller.ts (:assetNo/dispose/approve|reject); schema/assets.ts fixed_assets.disposal_pending + migration 0135; cutover/basics.ts + worldclass.ts + compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N111" s="16" t="inlineStr">
         <is>
-          <t>Inspect consolidation logic + gate.</t>
+          <t>Inspect Draft→approve flow + the approver≠requester check + deferred status/recycle.</t>
         </is>
       </c>
       <c r="O111" s="16" t="inlineStr">
         <is>
-          <t>Sample period: consolidated TB ties to entities.</t>
+          <t>Re-perform: request a disposal (Draft JE excluded), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm status→disposed + surplus recycled only after approval (re-performed by the harnesses).</t>
         </is>
       </c>
       <c r="P111" s="16" t="inlineStr">
         <is>
-          <t>Consol TB</t>
+          <t>Disposal approval log + SoD test</t>
         </is>
       </c>
       <c r="Q111" s="18" t="inlineStr">
@@ -10540,12 +10540,12 @@
     <row r="112">
       <c r="A112" s="11" t="inlineStr">
         <is>
-          <t>CON-02</t>
+          <t>FA-10</t>
         </is>
       </c>
       <c r="B112" s="12" t="inlineStr">
         <is>
-          <t>Consolidation &amp; FX</t>
+          <t>Fixed Assets</t>
         </is>
       </c>
       <c r="C112" s="13" t="inlineStr">
@@ -10555,42 +10555,42 @@
       </c>
       <c r="D112" s="12" t="inlineStr">
         <is>
-          <t>FX gain/loss</t>
+          <t>Property, Plant &amp; Equipment; Accounts Payable</t>
         </is>
       </c>
       <c r="E112" s="12" t="inlineStr">
         <is>
-          <t>FX exposures not revalued at period-end.</t>
+          <t>Capital purchases mis-capitalised or capitalised without independent review — the person who receives the goods also decides what enters the asset register and at what cost/useful life (fictitious or over-valued assets; capex/opex mis-classification).</t>
         </is>
       </c>
       <c r="F112" s="12" t="inlineStr">
         <is>
-          <t>Valuation</t>
+          <t>Authorization; Accuracy</t>
         </is>
       </c>
       <c r="G112" s="12" t="inlineStr">
         <is>
-          <t>FX revaluation at period-end rates; unrealized FX posted (acct 5400).</t>
+          <t>Procure-to-Capitalize maker-checker (SoD): a goods-receipt line flagged capital (item-master is_fixed_asset or per-PO-line override) is excluded from inventory capitalisation (1200) at receipt and instead becomes ELIGIBLE for the asset register. Capitalisation is a REQUEST that posts NOTHING to the GL; a DIFFERENT user must approve before the fixed_assets row + acquisition JE (Dr 1500 / Cr 2000) are created (approver ≠ requester enforced regardless of permissions). The created asset carries its source GR/PO for end-to-end PR→PO→GR→FA traceability; a GR line cannot be capitalised twice.</t>
         </is>
       </c>
       <c r="H112" s="13" t="inlineStr">
         <is>
-          <t>Auto+Manual</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I112" s="13" t="inlineStr">
         <is>
-          <t>Period-end</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J112" s="13" t="inlineStr">
         <is>
-          <t>Period</t>
+          <t>Per capital receipt</t>
         </is>
       </c>
       <c r="K112" s="12" t="inlineStr">
         <is>
-          <t>Controller</t>
+          <t>FaAccountant / Controller</t>
         </is>
       </c>
       <c r="L112" s="13" t="inlineStr">
@@ -10600,22 +10600,22 @@
       </c>
       <c r="M112" s="12" t="inlineStr">
         <is>
-          <t>fx.service.ts (revalue / unrealized report)</t>
+          <t>assets.service.ts registerFromGr/approveRegistration/rejectRegistration/eligibleFromGr; assets.controller.ts (registrations*); procurement.service.ts createGr (is_capital routing, costing excluded); schema/assets.ts asset_registration_requests + fixed_assets.source_gr_no/po_no + migration 0137; cutover/basics.ts + compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N112" s="12" t="inlineStr">
         <is>
-          <t>Inspect reval logic + rates.</t>
+          <t>Inspect the eligible→request→approve flow + approver≠requester check + the inventory-vs-asset routing of capital lines.</t>
         </is>
       </c>
       <c r="O112" s="12" t="inlineStr">
         <is>
-          <t>Recompute reval on sample balances.</t>
+          <t>Re-perform: receive a capital line, raise a registration (no GL), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm the asset + Dr 1500/Cr 2000 post only after approval and the line cannot be re-registered (re-performed by the harnesses).</t>
         </is>
       </c>
       <c r="P112" s="12" t="inlineStr">
         <is>
-          <t>FX reval JE</t>
+          <t>Capitalization approval log + SoD test</t>
         </is>
       </c>
       <c r="Q112" s="18" t="inlineStr">
@@ -10627,7 +10627,7 @@
     <row r="113">
       <c r="A113" s="15" t="inlineStr">
         <is>
-          <t>FX-04</t>
+          <t>CON-01</t>
         </is>
       </c>
       <c r="B113" s="16" t="inlineStr">
@@ -10642,42 +10642,42 @@
       </c>
       <c r="D113" s="16" t="inlineStr">
         <is>
-          <t>FX gain/loss; Revenue; AR/AP</t>
+          <t>Consolidation</t>
         </is>
       </c>
       <c r="E113" s="16" t="inlineStr">
         <is>
-          <t>A wrong manually-entered FX rate (fat-fingered, e.g. USD 36 keyed as 63) flows straight into a period-end revaluation JE and the unrealized-FX report with no independent review — mis-stating earnings/equity and FX-translated balances.</t>
+          <t>Group consolidation mis-stated (ownership/currency).</t>
         </is>
       </c>
       <c r="F113" s="16" t="inlineStr">
         <is>
-          <t>Accuracy/Valuation</t>
+          <t>Accuracy</t>
         </is>
       </c>
       <c r="G113" s="16" t="inlineStr">
         <is>
-          <t>FX rate maker-checker (SoD): a MANUALLY-entered rate lands as PendingApproval and is EXCLUDED from rate resolution — revaluation, the unrealized-FX report, and consolidation translation all use APPROVED rates only — until a DIFFERENT user approves it (POST /api/fx/rates/approve). Self-approval → SOD_VIOLATION (binds even Admin); reject marks the rate Rejected (never usable); re-entering a rate sends it back to PendingApproval. Externally-sourced (feed) rates carrying an explicit non-manual source are auto-approved. Pending rates are also surfaced, aged, by the pending-approvals monitor (GOV-01).</t>
+          <t>Consolidation run (ownership %, entity currency) gated by 'approvals'.</t>
         </is>
       </c>
       <c r="H113" s="17" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="I113" s="17" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Period</t>
         </is>
       </c>
       <c r="J113" s="17" t="inlineStr">
         <is>
-          <t>Per rate</t>
+          <t>Period</t>
         </is>
       </c>
       <c r="K113" s="16" t="inlineStr">
         <is>
-          <t>Controller / Treasury</t>
+          <t>Group Controller</t>
         </is>
       </c>
       <c r="L113" s="17" t="inlineStr">
@@ -10687,22 +10687,22 @@
       </c>
       <c r="M113" s="16" t="inlineStr">
         <is>
-          <t>fx.service.ts setRate(manual→PendingApproval)/approveRate/rejectRate/rateAsOf(Approved only); fx.controller.ts (rates/approve|reject|pending gated approvals/gl_close); consolidation.service.ts (translation reads Approved rates); schema/fx.ts fx_rates.status + migration 0141; cutover/fxreval.ts (ToE)</t>
+          <t>consolidation.service.ts (runConsolidation @Permissions approvals)</t>
         </is>
       </c>
       <c r="N113" s="16" t="inlineStr">
         <is>
-          <t>Inspect the request→approve flow + the approver≠requester check + that revaluation/reporting resolve Approved rates only.</t>
+          <t>Inspect consolidation logic + gate.</t>
         </is>
       </c>
       <c r="O113" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: enter a manual rate (PendingApproval), confirm revalue is blocked NO_RATE while pending, attempt self-approve (SOD_VIOLATION), approve as a different user, then revalue succeeds (re-performed by the fxreval harness).</t>
+          <t>Sample period: consolidated TB ties to entities.</t>
         </is>
       </c>
       <c r="P113" s="16" t="inlineStr">
         <is>
-          <t>FX rate approval log + SoD test</t>
+          <t>Consol TB</t>
         </is>
       </c>
       <c r="Q113" s="18" t="inlineStr">
@@ -10714,92 +10714,266 @@
     <row r="114">
       <c r="A114" s="11" t="inlineStr">
         <is>
+          <t>CON-02</t>
+        </is>
+      </c>
+      <c r="B114" s="12" t="inlineStr">
+        <is>
+          <t>Consolidation &amp; FX</t>
+        </is>
+      </c>
+      <c r="C114" s="13" t="inlineStr">
+        <is>
+          <t>Application</t>
+        </is>
+      </c>
+      <c r="D114" s="12" t="inlineStr">
+        <is>
+          <t>FX gain/loss</t>
+        </is>
+      </c>
+      <c r="E114" s="12" t="inlineStr">
+        <is>
+          <t>FX exposures not revalued at period-end.</t>
+        </is>
+      </c>
+      <c r="F114" s="12" t="inlineStr">
+        <is>
+          <t>Valuation</t>
+        </is>
+      </c>
+      <c r="G114" s="12" t="inlineStr">
+        <is>
+          <t>FX revaluation at period-end rates; unrealized FX posted (acct 5400).</t>
+        </is>
+      </c>
+      <c r="H114" s="13" t="inlineStr">
+        <is>
+          <t>Auto+Manual</t>
+        </is>
+      </c>
+      <c r="I114" s="13" t="inlineStr">
+        <is>
+          <t>Period-end</t>
+        </is>
+      </c>
+      <c r="J114" s="13" t="inlineStr">
+        <is>
+          <t>Period</t>
+        </is>
+      </c>
+      <c r="K114" s="12" t="inlineStr">
+        <is>
+          <t>Controller</t>
+        </is>
+      </c>
+      <c r="L114" s="13" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="M114" s="12" t="inlineStr">
+        <is>
+          <t>fx.service.ts (revalue / unrealized report)</t>
+        </is>
+      </c>
+      <c r="N114" s="12" t="inlineStr">
+        <is>
+          <t>Inspect reval logic + rates.</t>
+        </is>
+      </c>
+      <c r="O114" s="12" t="inlineStr">
+        <is>
+          <t>Recompute reval on sample balances.</t>
+        </is>
+      </c>
+      <c r="P114" s="12" t="inlineStr">
+        <is>
+          <t>FX reval JE</t>
+        </is>
+      </c>
+      <c r="Q114" s="18" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="15" t="inlineStr">
+        <is>
+          <t>FX-04</t>
+        </is>
+      </c>
+      <c r="B115" s="16" t="inlineStr">
+        <is>
+          <t>Consolidation &amp; FX</t>
+        </is>
+      </c>
+      <c r="C115" s="17" t="inlineStr">
+        <is>
+          <t>Application</t>
+        </is>
+      </c>
+      <c r="D115" s="16" t="inlineStr">
+        <is>
+          <t>FX gain/loss; Revenue; AR/AP</t>
+        </is>
+      </c>
+      <c r="E115" s="16" t="inlineStr">
+        <is>
+          <t>A wrong manually-entered FX rate (fat-fingered, e.g. USD 36 keyed as 63) flows straight into a period-end revaluation JE and the unrealized-FX report with no independent review — mis-stating earnings/equity and FX-translated balances.</t>
+        </is>
+      </c>
+      <c r="F115" s="16" t="inlineStr">
+        <is>
+          <t>Accuracy/Valuation</t>
+        </is>
+      </c>
+      <c r="G115" s="16" t="inlineStr">
+        <is>
+          <t>FX rate maker-checker (SoD): a MANUALLY-entered rate lands as PendingApproval and is EXCLUDED from rate resolution — revaluation, the unrealized-FX report, and consolidation translation all use APPROVED rates only — until a DIFFERENT user approves it (POST /api/fx/rates/approve). Self-approval → SOD_VIOLATION (binds even Admin); reject marks the rate Rejected (never usable); re-entering a rate sends it back to PendingApproval. Externally-sourced (feed) rates carrying an explicit non-manual source are auto-approved. Pending rates are also surfaced, aged, by the pending-approvals monitor (GOV-01).</t>
+        </is>
+      </c>
+      <c r="H115" s="17" t="inlineStr">
+        <is>
+          <t>Prev</t>
+        </is>
+      </c>
+      <c r="I115" s="17" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="J115" s="17" t="inlineStr">
+        <is>
+          <t>Per rate</t>
+        </is>
+      </c>
+      <c r="K115" s="16" t="inlineStr">
+        <is>
+          <t>Controller / Treasury</t>
+        </is>
+      </c>
+      <c r="L115" s="17" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="M115" s="16" t="inlineStr">
+        <is>
+          <t>fx.service.ts setRate(manual→PendingApproval)/approveRate/rejectRate/rateAsOf(Approved only); fx.controller.ts (rates/approve|reject|pending gated approvals/gl_close); consolidation.service.ts (translation reads Approved rates); schema/fx.ts fx_rates.status + migration 0141; cutover/fxreval.ts (ToE)</t>
+        </is>
+      </c>
+      <c r="N115" s="16" t="inlineStr">
+        <is>
+          <t>Inspect the request→approve flow + the approver≠requester check + that revaluation/reporting resolve Approved rates only.</t>
+        </is>
+      </c>
+      <c r="O115" s="16" t="inlineStr">
+        <is>
+          <t>Re-perform: enter a manual rate (PendingApproval), confirm revalue is blocked NO_RATE while pending, attempt self-approve (SOD_VIOLATION), approve as a different user, then revalue succeeds (re-performed by the fxreval harness).</t>
+        </is>
+      </c>
+      <c r="P115" s="16" t="inlineStr">
+        <is>
+          <t>FX rate approval log + SoD test</t>
+        </is>
+      </c>
+      <c r="Q115" s="18" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="11" t="inlineStr">
+        <is>
           <t>BUD-01</t>
         </is>
       </c>
-      <c r="B114" s="12" t="inlineStr">
+      <c r="B116" s="12" t="inlineStr">
         <is>
           <t>Budgeting &amp; Planning</t>
         </is>
       </c>
-      <c r="C114" s="13" t="inlineStr">
+      <c r="C116" s="13" t="inlineStr">
         <is>
           <t>Application</t>
         </is>
       </c>
-      <c r="D114" s="12" t="inlineStr">
+      <c r="D116" s="12" t="inlineStr">
         <is>
           <t>Budget; All (variance reporting)</t>
         </is>
       </c>
-      <c r="E114" s="12" t="inlineStr">
+      <c r="E116" s="12" t="inlineStr">
         <is>
           <t>A budget figure is entered/changed by one person and immediately drives the budget-vs-actual variance report — the basis for spend authorization and performance review — with no independent approval; a wrong or self-serving budget makes overspending look 'on budget'.</t>
         </is>
       </c>
-      <c r="F114" s="12" t="inlineStr">
+      <c r="F116" s="12" t="inlineStr">
         <is>
           <t>Authorization/Accuracy</t>
         </is>
       </c>
-      <c r="G114" s="12" t="inlineStr">
+      <c r="G116" s="12" t="inlineStr">
         <is>
           <t>Budget maker-checker (SoD): an upserted budget (POST /api/ledger/budgets) lands as PendingApproval and is EXCLUDED from budget-vs-actual until a DIFFERENT user approves it (POST /api/ledger/budgets/approve for the fiscal_year/account/cost-centre[/period]). Self-approval → SOD_VIOLATION (binds even Admin); reject marks it Rejected (excluded). DEFAULT 'Approved' keeps existing rows + direct planning seeds usable. Pending budgets are also surfaced, aged, by the pending-approvals monitor (GOV-01).</t>
         </is>
       </c>
-      <c r="H114" s="13" t="inlineStr">
+      <c r="H116" s="13" t="inlineStr">
         <is>
           <t>Prev</t>
         </is>
       </c>
-      <c r="I114" s="13" t="inlineStr">
+      <c r="I116" s="13" t="inlineStr">
         <is>
           <t>Automated</t>
         </is>
       </c>
-      <c r="J114" s="13" t="inlineStr">
+      <c r="J116" s="13" t="inlineStr">
         <is>
           <t>Per budget</t>
         </is>
       </c>
-      <c r="K114" s="12" t="inlineStr">
+      <c r="K116" s="12" t="inlineStr">
         <is>
           <t>Controller / FP&amp;A</t>
         </is>
       </c>
-      <c r="L114" s="13" t="inlineStr">
+      <c r="L116" s="13" t="inlineStr">
         <is>
           <t>P10</t>
         </is>
       </c>
-      <c r="M114" s="12" t="inlineStr">
+      <c r="M116" s="12" t="inlineStr">
         <is>
           <t>budget.service.ts upsertBudget(→PendingApproval)/approveBudget/rejectBudget/budgetVsActual(Approved only); budget.controller.ts (budgets/approve|reject|pending gated approvals/gl_close); schema/budgets.ts budgets.status + migration 0142; cutover/budget.ts (ToE)</t>
         </is>
       </c>
-      <c r="N114" s="12" t="inlineStr">
+      <c r="N116" s="12" t="inlineStr">
         <is>
           <t>Inspect the request→approve flow + the approver≠requester check + that budget-vs-actual counts Approved budgets only.</t>
         </is>
       </c>
-      <c r="O114" s="12" t="inlineStr">
+      <c r="O116" s="12" t="inlineStr">
         <is>
           <t>Re-perform: upsert a budget (PendingApproval, excluded from variance), attempt self-approve (SOD_VIOLATION), approve as a different user, confirm it then appears in budget-vs-actual (re-performed by the budget harness).</t>
         </is>
       </c>
-      <c r="P114" s="12" t="inlineStr">
+      <c r="P116" s="12" t="inlineStr">
         <is>
           <t>Budget approval log + SoD test</t>
         </is>
       </c>
-      <c r="Q114" s="18" t="inlineStr">
+      <c r="Q116" s="18" t="inlineStr">
         <is>
           <t>Implemented</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q114"/>
+  <autoFilter ref="A1:Q116"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -11982,7 +12156,7 @@
         </is>
       </c>
       <c r="C5" s="29">
-        <f>COUNTIF(RCM!$Q$2:$Q$114,B5)</f>
+        <f>COUNTIF(RCM!$Q$2:$Q$116,B5)</f>
         <v/>
       </c>
     </row>
@@ -11993,7 +12167,7 @@
         </is>
       </c>
       <c r="C6" s="29">
-        <f>COUNTIF(RCM!$Q$2:$Q$114,B6)</f>
+        <f>COUNTIF(RCM!$Q$2:$Q$116,B6)</f>
         <v/>
       </c>
     </row>
@@ -12004,7 +12178,7 @@
         </is>
       </c>
       <c r="C7" s="29">
-        <f>COUNTIF(RCM!$Q$2:$Q$114,B7)</f>
+        <f>COUNTIF(RCM!$Q$2:$Q$116,B7)</f>
         <v/>
       </c>
     </row>
@@ -12015,7 +12189,7 @@
         </is>
       </c>
       <c r="C8" s="32">
-        <f>COUNTA(RCM!$A$2:$A$114)</f>
+        <f>COUNTA(RCM!$A$2:$A$116)</f>
         <v/>
       </c>
     </row>
@@ -12033,7 +12207,7 @@
         </is>
       </c>
       <c r="C11" s="29">
-        <f>COUNTIF(RCM!$C$2:$C$114,B11)</f>
+        <f>COUNTIF(RCM!$C$2:$C$116,B11)</f>
         <v/>
       </c>
     </row>
@@ -12044,7 +12218,7 @@
         </is>
       </c>
       <c r="C12" s="29">
-        <f>COUNTIF(RCM!$C$2:$C$114,B12)</f>
+        <f>COUNTIF(RCM!$C$2:$C$116,B12)</f>
         <v/>
       </c>
     </row>
@@ -12055,7 +12229,7 @@
         </is>
       </c>
       <c r="C13" s="29">
-        <f>COUNTIF(RCM!$C$2:$C$114,B13)</f>
+        <f>COUNTIF(RCM!$C$2:$C$116,B13)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(gl): WS1.4 — sub-ledger tie-out + maker-checker certify (GL-14)
- subledger_tieout_runs table (migration 0160) + RLS
- SubledgerTieoutService.runTieOut: compares GL control-account balance
  vs sub-ledger sum (AR/AP from invoice tables, INV from inv_balances,
  FA from fixed_assets NBV); flags Matched/Variance
- certify(): maker-checker, blocks SELF_CERTIFY
- Controller GET/POST run/certify (perms gl_close, gl_post)
- basics harness: 4 GL-14 checks (164/164 green)
- GL-14 RCM control (Detective/Monthly, SoD certifier≠runner); RCM 118
- process-narrative §1.4 + UAT TC-GL-14-01..03

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/compliance/Oshinei_ERP_SOX_RCM_v1.xlsx
+++ b/compliance/Oshinei_ERP_SOX_RCM_v1.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'RCM'!$A$1:$Q$118</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'RCM'!$A$1:$Q$119</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Gap Remediation'!$A$2:$H$18</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -858,7 +858,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q118"/>
+  <dimension ref="A1:Q119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -8974,12 +8974,12 @@
     <row r="94">
       <c r="A94" s="11" t="inlineStr">
         <is>
-          <t>EXP-07</t>
+          <t>GL-14</t>
         </is>
       </c>
       <c r="B94" s="12" t="inlineStr">
         <is>
-          <t>Expenditure</t>
+          <t>General Ledger</t>
         </is>
       </c>
       <c r="C94" s="13" t="inlineStr">
@@ -8989,22 +8989,22 @@
       </c>
       <c r="D94" s="12" t="inlineStr">
         <is>
-          <t>Cash; Operating expense</t>
+          <t>All</t>
         </is>
       </c>
       <c r="E94" s="12" t="inlineStr">
         <is>
-          <t>Petty-cash / employee advance issued but never accounted for — cash leakage, expense unrecorded.</t>
+          <t>GL control-account balances (AR/AP/INV/FA) drift from the underlying sub-ledger detail without detection — the control account no longer represents the sum of its sub-ledger, masking posting errors, unrecorded items, or fraud.</t>
         </is>
       </c>
       <c r="F94" s="12" t="inlineStr">
         <is>
-          <t>Existence/Completeness</t>
+          <t>Completeness/Accuracy/Valuation</t>
         </is>
       </c>
       <c r="G94" s="12" t="inlineStr">
         <is>
-          <t>Employee cash advances: issuing an advance debits the 1180 Employee Advances control (Dr 1180 / Cr 1000); settlement clears it against actual spend + returned cash (Dr expense + Dr 1000 / Cr 1180), enforced to reconcile (settled_expense + returned_cash must equal the advance → SETTLE_MISMATCH). The 1180 balance is the outstanding float subject to review.</t>
+          <t>Sub-ledger tie-out / reconciliation: POST /api/ledger/tie-out/run computes, per control account, the GL balance (Σ debit−credit of posted journal_lines on the control account up to the as-of date, tenant-scoped) and the sub-ledger detail balance (AR = Σ outstanding ar_invoices; AP = Σ outstanding ap_transactions; INV = Σ inv_balances.total_value perpetual valuation; FA = Σ acquire_cost − accumulated_depreciation of non-disposed fixed_assets), records the variance (gl − subledger) and a status (Matched if |variance|&lt;0.01 else Variance). Runs upsert per (tenant, subledger, as-of). Certification is maker-checker: POST /api/ledger/tie-out/:id/certify sets status=Certified and records certifier + timestamp, and REJECTS a certifier equal to the runner (SELF_CERTIFY) — the gl_close certifier must differ from the gl_post/gl_close runner (SoD).</t>
         </is>
       </c>
       <c r="H94" s="13" t="inlineStr">
@@ -9019,12 +9019,12 @@
       </c>
       <c r="J94" s="13" t="inlineStr">
         <is>
-          <t>Per advance</t>
+          <t>Monthly</t>
         </is>
       </c>
       <c r="K94" s="12" t="inlineStr">
         <is>
-          <t>AP / Controller</t>
+          <t>Financial Controller</t>
         </is>
       </c>
       <c r="L94" s="13" t="inlineStr">
@@ -9034,22 +9034,22 @@
       </c>
       <c r="M94" s="12" t="inlineStr">
         <is>
-          <t>finance.service.ts (issueAdvance, settleAdvance reconcile-or-reject, listAdvances outstanding); finance.controller.ts (creditors/exec); schema/finance.ts (employee_advances) + migration 0120; cutover/basics.ts (ToE)</t>
+          <t>subledger-tieout.service.ts (runTieOut GL/sub-ledger balance computation + variance/status, certify SELF_CERTIFY maker-checker, list/get); subledger-tieout.controller.ts (gl_close/gl_post run, gl_close certify, gl_close/gl_post/exec/creditors/ar read); schema/subledger-tieout.ts (subledger_tieout_runs table, uq on tenant/subledger/as-of); migration 0160 (table + RLS); ledger.module.ts (service+controller wired); cutover/basics.ts (GL-14 ToE)</t>
         </is>
       </c>
       <c r="N94" s="12" t="inlineStr">
         <is>
-          <t>Inspect issue/settle GL + settlement reconciliation guard.</t>
+          <t>Inspect the GL-vs-sub-ledger balance computation + variance/status + SELF_CERTIFY maker-checker gate + gl_close certify permission.</t>
         </is>
       </c>
       <c r="O94" s="12" t="inlineStr">
         <is>
-          <t>Issue an advance (1180 up); settle 700+300 clears 1180; mismatched settle → SETTLE_MISMATCH (re-performed by the harness).</t>
+          <t>TC-GL-14-01: run AR tie-out → balances + Matched/Variance; TC-GL-14-02: self-certify by the runner → SELF_CERTIFY (400); TC-GL-14-03: certify by a different gl_close user → Certified (re-performed by the basics.ts harness).</t>
         </is>
       </c>
       <c r="P94" s="12" t="inlineStr">
         <is>
-          <t>Advance register; outstanding float</t>
+          <t>Tie-out run log (subledger_tieout_runs) with variance + certification trail; monthly reconciliation sign-off</t>
         </is>
       </c>
       <c r="Q94" s="18" t="inlineStr">
@@ -9061,7 +9061,7 @@
     <row r="95">
       <c r="A95" s="15" t="inlineStr">
         <is>
-          <t>EXP-08</t>
+          <t>EXP-07</t>
         </is>
       </c>
       <c r="B95" s="16" t="inlineStr">
@@ -9081,22 +9081,22 @@
       </c>
       <c r="E95" s="16" t="inlineStr">
         <is>
-          <t>Petty-cash disbursed beyond authority / without independent review, or drawn past the fund's limit — cash leakage, unauthorised or unrecorded expense, over-extended float.</t>
+          <t>Petty-cash / employee advance issued but never accounted for — cash leakage, expense unrecorded.</t>
         </is>
       </c>
       <c r="F95" s="16" t="inlineStr">
         <is>
-          <t>Authorization; Completeness</t>
+          <t>Existence/Completeness</t>
         </is>
       </c>
       <c r="G95" s="16" t="inlineStr">
         <is>
-          <t>Petty-cash imprest float + maker-checker on disbursement (SoD): a fund holds cash capped at a credit limit/วงเงิน (1015 Petty Cash, a cash account); each direct EXPENSE or ADVANCE is a REQUEST that posts NOTHING and a DIFFERENT user must approve before the GL posts (expense Dr &lt;expense&gt; / Cr 1015; advance Dr 1180 / Cr 1015) and the fund balance is decremented. Self-approval → SOD_VIOLATION (binds even Admin). A draw beyond the fund balance → INSUFFICIENT_FLOAT; establishing/replenishing above the float limit → OVER_FLOAT. Advances settle (Dr expense + Dr 1015 returned / Cr 1180), returning unused cash to the fund. Every request carries a document reference + receipt key + a status trail (StatusLog) and surfaces in the GOV-01 pending-approvals monitor.</t>
+          <t>Employee cash advances: issuing an advance debits the 1180 Employee Advances control (Dr 1180 / Cr 1000); settlement clears it against actual spend + returned cash (Dr expense + Dr 1000 / Cr 1180), enforced to reconcile (settled_expense + returned_cash must equal the advance → SETTLE_MISMATCH). The 1180 balance is the outstanding float subject to review.</t>
         </is>
       </c>
       <c r="H95" s="17" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I95" s="17" t="inlineStr">
@@ -9106,7 +9106,7 @@
       </c>
       <c r="J95" s="17" t="inlineStr">
         <is>
-          <t>Per disbursement</t>
+          <t>Per advance</t>
         </is>
       </c>
       <c r="K95" s="16" t="inlineStr">
@@ -9121,22 +9121,22 @@
       </c>
       <c r="M95" s="16" t="inlineStr">
         <is>
-          <t>petty-cash.service.ts (establishFund/replenishFund float guards, createRequest INSUFFICIENT_FLOAT, approveRequest SoD+GL, rejectRequest, settleRequest); petty-cash.controller.ts (creditors/exec); schema/petty-cash.ts (petty_cash_funds, expense_requests) + migration 0139; finance.service.ts pendingApprovals (GOV-01 source 7); cutover/basics.ts + compliance.ts (ToE)</t>
+          <t>finance.service.ts (issueAdvance, settleAdvance reconcile-or-reject, listAdvances outstanding); finance.controller.ts (creditors/exec); schema/finance.ts (employee_advances) + migration 0120; cutover/basics.ts (ToE)</t>
         </is>
       </c>
       <c r="N95" s="16" t="inlineStr">
         <is>
-          <t>Inspect the float ceiling + the request→approve flow + the approver≠requester check + that the request posts nothing until approval.</t>
+          <t>Inspect issue/settle GL + settlement reconciliation guard.</t>
         </is>
       </c>
       <c r="O95" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: establish a fund (Dr 1015), request an expense (no GL), self-approve → SOD_VIOLATION, approve as a different user → Dr expense/Cr 1015 + fund down; over-balance draw → INSUFFICIENT_FLOAT; advance approve→settle clears 1180; replenish past float → OVER_FLOAT (re-performed by the harnesses).</t>
+          <t>Issue an advance (1180 up); settle 700+300 clears 1180; mismatched settle → SETTLE_MISMATCH (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P95" s="16" t="inlineStr">
         <is>
-          <t>Fund register + disbursement approval log + SoD test</t>
+          <t>Advance register; outstanding float</t>
         </is>
       </c>
       <c r="Q95" s="18" t="inlineStr">
@@ -9148,12 +9148,12 @@
     <row r="96">
       <c r="A96" s="11" t="inlineStr">
         <is>
-          <t>FA-07</t>
+          <t>EXP-08</t>
         </is>
       </c>
       <c r="B96" s="12" t="inlineStr">
         <is>
-          <t>Fixed Assets</t>
+          <t>Expenditure</t>
         </is>
       </c>
       <c r="C96" s="13" t="inlineStr">
@@ -9163,27 +9163,27 @@
       </c>
       <c r="D96" s="12" t="inlineStr">
         <is>
-          <t>Property, Plant &amp; Equipment; Equity</t>
+          <t>Cash; Operating expense</t>
         </is>
       </c>
       <c r="E96" s="12" t="inlineStr">
         <is>
-          <t>Carrying amount not adjusted for revaluation/impairment — asset over/understated.</t>
+          <t>Petty-cash disbursed beyond authority / without independent review, or drawn past the fund's limit — cash leakage, unauthorised or unrecorded expense, over-extended float.</t>
         </is>
       </c>
       <c r="F96" s="12" t="inlineStr">
         <is>
-          <t>Valuation</t>
+          <t>Authorization; Completeness</t>
         </is>
       </c>
       <c r="G96" s="12" t="inlineStr">
         <is>
-          <t>Asset revaluation / impairment: an upward revaluation credits the revaluation surplus in equity (Dr 1500 / Cr 3200); a downward revaluation (impairment) debits impairment loss (Dr 5820 / Cr 1500). The gross 1500 moves by the delta so the register stays tied to the GL; a no-op revaluation is rejected (NO_CHANGE). Every event is logged for the audit trail.</t>
+          <t>Petty-cash imprest float + maker-checker on disbursement (SoD): a fund holds cash capped at a credit limit/วงเงิน (1015 Petty Cash, a cash account); each direct EXPENSE or ADVANCE is a REQUEST that posts NOTHING and a DIFFERENT user must approve before the GL posts (expense Dr &lt;expense&gt; / Cr 1015; advance Dr 1180 / Cr 1015) and the fund balance is decremented. Self-approval → SOD_VIOLATION (binds even Admin). A draw beyond the fund balance → INSUFFICIENT_FLOAT; establishing/replenishing above the float limit → OVER_FLOAT. Advances settle (Dr expense + Dr 1015 returned / Cr 1180), returning unused cash to the fund. Every request carries a document reference + receipt key + a status trail (StatusLog) and surfaces in the GOV-01 pending-approvals monitor.</t>
         </is>
       </c>
       <c r="H96" s="13" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I96" s="13" t="inlineStr">
@@ -9193,12 +9193,12 @@
       </c>
       <c r="J96" s="13" t="inlineStr">
         <is>
-          <t>Per event</t>
+          <t>Per disbursement</t>
         </is>
       </c>
       <c r="K96" s="12" t="inlineStr">
         <is>
-          <t>FaAccountant / Controller</t>
+          <t>AP / Controller</t>
         </is>
       </c>
       <c r="L96" s="13" t="inlineStr">
@@ -9208,22 +9208,22 @@
       </c>
       <c r="M96" s="12" t="inlineStr">
         <is>
-          <t>assets.service.ts (revalue up→3200 / down→5820, listRevaluations; dispose recycles surplus 3200→3100); assets.controller.ts (exec/creditors); schema/assets.ts (asset_revaluations) + migration 0120; cutover/basics.ts (ToE)</t>
+          <t>petty-cash.service.ts (establishFund/replenishFund float guards, createRequest INSUFFICIENT_FLOAT, approveRequest SoD+GL, rejectRequest, settleRequest); petty-cash.controller.ts (creditors/exec); schema/petty-cash.ts (petty_cash_funds, expense_requests) + migration 0139; finance.service.ts pendingApprovals (GOV-01 source 7); cutover/basics.ts + compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N96" s="12" t="inlineStr">
         <is>
-          <t>Inspect revaluation/impairment routing + audit log + disposal recycling.</t>
+          <t>Inspect the float ceiling + the request→approve flow + the approver≠requester check + that the request posts nothing until approval.</t>
         </is>
       </c>
       <c r="O96" s="12" t="inlineStr">
         <is>
-          <t>Upward revaluation credits 3200; impairment debits 5820; no-change → NO_CHANGE; both events logged; on disposal the revaluation surplus is recycled to retained earnings (Dr 3200 / Cr 3100), not through P&amp;L (re-performed by the harness).</t>
+          <t>Re-perform: establish a fund (Dr 1015), request an expense (no GL), self-approve → SOD_VIOLATION, approve as a different user → Dr expense/Cr 1015 + fund down; over-balance draw → INSUFFICIENT_FLOAT; advance approve→settle clears 1180; replenish past float → OVER_FLOAT (re-performed by the harnesses).</t>
         </is>
       </c>
       <c r="P96" s="12" t="inlineStr">
         <is>
-          <t>Revaluation log; disposal recycling JE</t>
+          <t>Fund register + disbursement approval log + SoD test</t>
         </is>
       </c>
       <c r="Q96" s="18" t="inlineStr">
@@ -9235,7 +9235,7 @@
     <row r="97">
       <c r="A97" s="15" t="inlineStr">
         <is>
-          <t>FA-08</t>
+          <t>FA-07</t>
         </is>
       </c>
       <c r="B97" s="16" t="inlineStr">
@@ -9255,22 +9255,22 @@
       </c>
       <c r="E97" s="16" t="inlineStr">
         <is>
-          <t>Carrying amount changed by fair-value revaluation/impairment without independent review — the preparer revalues the asset and posts to equity/P&amp;L on their own (earnings/equity management).</t>
+          <t>Carrying amount not adjusted for revaluation/impairment — asset over/understated.</t>
         </is>
       </c>
       <c r="F97" s="16" t="inlineStr">
         <is>
-          <t>Authorization</t>
+          <t>Valuation</t>
         </is>
       </c>
       <c r="G97" s="16" t="inlineStr">
         <is>
-          <t>Asset-revaluation maker-checker (SoD): a revalue/impairment request posts its GL entry as a DRAFT (excluded from balances) and records status 'PendingApproval' WITHOUT moving the carrying value; a DIFFERENT user must approve before the JE is effective and the register is re-valued (approver ≠ preparer enforced regardless of permissions, reusing the GL-05 ledger approval). Reject voids the draft; only one revaluation may be pending per asset; the disposal surplus recycle counts only approved revaluations.</t>
+          <t>Asset revaluation / impairment: an upward revaluation credits the revaluation surplus in equity (Dr 1500 / Cr 3200); a downward revaluation (impairment) debits impairment loss (Dr 5820 / Cr 1500). The gross 1500 moves by the delta so the register stays tied to the GL; a no-op revaluation is rejected (NO_CHANGE). Every event is logged for the audit trail.</t>
         </is>
       </c>
       <c r="H97" s="17" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I97" s="17" t="inlineStr">
@@ -9295,22 +9295,22 @@
       </c>
       <c r="M97" s="16" t="inlineStr">
         <is>
-          <t>assets.service.ts revalue(pendingApproval Draft)/approveRevaluation/rejectRevaluation; assets.controller.ts (:assetNo/revalue/approve|reject); schema/assets.ts asset_revaluations.status + migration 0134; cutover/basics.ts + compliance.ts (ToE)</t>
+          <t>assets.service.ts (revalue up→3200 / down→5820, listRevaluations; dispose recycles surplus 3200→3100); assets.controller.ts (exec/creditors); schema/assets.ts (asset_revaluations) + migration 0120; cutover/basics.ts (ToE)</t>
         </is>
       </c>
       <c r="N97" s="16" t="inlineStr">
         <is>
-          <t>Inspect Draft→approve flow + the approver≠preparer check + deferred carrying-value update.</t>
+          <t>Inspect revaluation/impairment routing + audit log + disposal recycling.</t>
         </is>
       </c>
       <c r="O97" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: request a revaluation (Draft JE excluded from 3200), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm the surplus/impairment + carrying value move only after approval (re-performed by the harnesses).</t>
+          <t>Upward revaluation credits 3200; impairment debits 5820; no-change → NO_CHANGE; both events logged; on disposal the revaluation surplus is recycled to retained earnings (Dr 3200 / Cr 3100), not through P&amp;L (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P97" s="16" t="inlineStr">
         <is>
-          <t>Revaluation approval log + SoD test</t>
+          <t>Revaluation log; disposal recycling JE</t>
         </is>
       </c>
       <c r="Q97" s="18" t="inlineStr">
@@ -9322,12 +9322,12 @@
     <row r="98">
       <c r="A98" s="11" t="inlineStr">
         <is>
-          <t>LSE-01</t>
+          <t>FA-08</t>
         </is>
       </c>
       <c r="B98" s="12" t="inlineStr">
         <is>
-          <t>Leases</t>
+          <t>Fixed Assets</t>
         </is>
       </c>
       <c r="C98" s="13" t="inlineStr">
@@ -9337,27 +9337,27 @@
       </c>
       <c r="D98" s="12" t="inlineStr">
         <is>
-          <t>Right-of-use assets; Lease liabilities</t>
+          <t>Property, Plant &amp; Equipment; Equity</t>
         </is>
       </c>
       <c r="E98" s="12" t="inlineStr">
         <is>
-          <t>Lease not capitalised (IFRS 16 / TFRS 16) — ROU asset + lease liability omitted; interest/depreciation mis-stated.</t>
+          <t>Carrying amount changed by fair-value revaluation/impairment without independent review — the preparer revalues the asset and posts to equity/P&amp;L on their own (earnings/equity management).</t>
         </is>
       </c>
       <c r="F98" s="12" t="inlineStr">
         <is>
-          <t>Completeness/Accuracy/Valuation</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="G98" s="12" t="inlineStr">
         <is>
-          <t>Lease accounting: at commencement a right-of-use asset and lease liability are recognised at the present value of the lease payments (Dr 1600 / Cr 2600). The scheduled job lease_periodic_run posts each period — interest unwinding on the liability (Dr 5900), the cash payment reducing the liability (Dr 2600 / Cr 1000), and straight-line ROU depreciation (Dr 5210 / Cr 1690) — the last period clearing the liability + ROU exactly. Idempotent per (lease, period).</t>
+          <t>Asset-revaluation maker-checker (SoD): a revalue/impairment request posts its GL entry as a DRAFT (excluded from balances) and records status 'PendingApproval' WITHOUT moving the carrying value; a DIFFERENT user must approve before the JE is effective and the register is re-valued (approver ≠ preparer enforced regardless of permissions, reusing the GL-05 ledger approval). Reject voids the draft; only one revaluation may be pending per asset; the disposal surplus recycle counts only approved revaluations.</t>
         </is>
       </c>
       <c r="H98" s="13" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I98" s="13" t="inlineStr">
@@ -9367,12 +9367,12 @@
       </c>
       <c r="J98" s="13" t="inlineStr">
         <is>
-          <t>Per period / per lease</t>
+          <t>Per event</t>
         </is>
       </c>
       <c r="K98" s="12" t="inlineStr">
         <is>
-          <t>Controller</t>
+          <t>FaAccountant / Controller</t>
         </is>
       </c>
       <c r="L98" s="13" t="inlineStr">
@@ -9382,22 +9382,22 @@
       </c>
       <c r="M98" s="12" t="inlineStr">
         <is>
-          <t>leases.service.ts (createLease PV recognition, runDueLeases interest+payment+depreciation, modifyLease remeasurement); leases.controller.ts (gl_post); bi.service.ts (lease_periodic_run); schema/leases.ts (leases, rou_nbv) + migration 0120/0121; cutover/basics.ts (ToE)</t>
+          <t>assets.service.ts revalue(pendingApproval Draft)/approveRevaluation/rejectRevaluation; assets.controller.ts (:assetNo/revalue/approve|reject); schema/assets.ts asset_revaluations.status + migration 0134; cutover/basics.ts + compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N98" s="12" t="inlineStr">
         <is>
-          <t>Inspect PV recognition + periodic interest/payment/depreciation + final-period clearing + modification remeasurement.</t>
+          <t>Inspect Draft→approve flow + the approver≠preparer check + deferred carrying-value update.</t>
         </is>
       </c>
       <c r="O98" s="12" t="inlineStr">
         <is>
-          <t>Commencement recognises ROU=liability=PV; periodic run posts interest+principal(=payment)+ROU depreciation; liability + ROU reduce; a modification remeasures the liability at the revised PV and adjusts the ROU by the same delta (Dr/Cr 1600↔2600), then depreciates over the remaining term (re-performed by the harness).</t>
+          <t>Re-perform: request a revaluation (Draft JE excluded from 3200), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm the surplus/impairment + carrying value move only after approval (re-performed by the harnesses).</t>
         </is>
       </c>
       <c r="P98" s="12" t="inlineStr">
         <is>
-          <t>Lease register; periodic run log; modification remeasurement</t>
+          <t>Revaluation approval log + SoD test</t>
         </is>
       </c>
       <c r="Q98" s="18" t="inlineStr">
@@ -9409,12 +9409,12 @@
     <row r="99">
       <c r="A99" s="15" t="inlineStr">
         <is>
-          <t>REC-01</t>
+          <t>LSE-01</t>
         </is>
       </c>
       <c r="B99" s="16" t="inlineStr">
         <is>
-          <t>Reconciliation</t>
+          <t>Leases</t>
         </is>
       </c>
       <c r="C99" s="17" t="inlineStr">
@@ -9424,22 +9424,22 @@
       </c>
       <c r="D99" s="16" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Right-of-use assets; Lease liabilities</t>
         </is>
       </c>
       <c r="E99" s="16" t="inlineStr">
         <is>
-          <t>Subledgers diverge from GL undetected.</t>
+          <t>Lease not capitalised (IFRS 16 / TFRS 16) — ROU asset + lease liability omitted; interest/depreciation mis-stated.</t>
         </is>
       </c>
       <c r="F99" s="16" t="inlineStr">
         <is>
-          <t>Completeness/Accuracy</t>
+          <t>Completeness/Accuracy/Valuation</t>
         </is>
       </c>
       <c r="G99" s="16" t="inlineStr">
         <is>
-          <t>Subledger-to-GL reconciliation per period: import GL, auto-match, certify (sign-off via 'approvals').</t>
+          <t>Lease accounting: at commencement a right-of-use asset and lease liability are recognised at the present value of the lease payments (Dr 1600 / Cr 2600). The scheduled job lease_periodic_run posts each period — interest unwinding on the liability (Dr 5900), the cash payment reducing the liability (Dr 2600 / Cr 1000), and straight-line ROU depreciation (Dr 5210 / Cr 1690) — the last period clearing the liability + ROU exactly. Idempotent per (lease, period).</t>
         </is>
       </c>
       <c r="H99" s="17" t="inlineStr">
@@ -9449,12 +9449,12 @@
       </c>
       <c r="I99" s="17" t="inlineStr">
         <is>
-          <t>Auto+Manual</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J99" s="17" t="inlineStr">
         <is>
-          <t>Monthly</t>
+          <t>Per period / per lease</t>
         </is>
       </c>
       <c r="K99" s="16" t="inlineStr">
@@ -9464,27 +9464,27 @@
       </c>
       <c r="L99" s="17" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="M99" s="16" t="inlineStr">
         <is>
-          <t>reconciliation.service.ts (importGlItems/autoMatch/certify)</t>
+          <t>leases.service.ts (createLease PV recognition, runDueLeases interest+payment+depreciation, modifyLease remeasurement); leases.controller.ts (gl_post); bi.service.ts (lease_periodic_run); schema/leases.ts (leases, rou_nbv) + migration 0120/0121; cutover/basics.ts (ToE)</t>
         </is>
       </c>
       <c r="N99" s="16" t="inlineStr">
         <is>
-          <t>Inspect recon + certify gate.</t>
+          <t>Inspect PV recognition + periodic interest/payment/depreciation + final-period clearing + modification remeasurement.</t>
         </is>
       </c>
       <c r="O99" s="16" t="inlineStr">
         <is>
-          <t>Sample periods: reconciled, unmatched cleared, certified.</t>
+          <t>Commencement recognises ROU=liability=PV; periodic run posts interest+principal(=payment)+ROU depreciation; liability + ROU reduce; a modification remeasures the liability at the revised PV and adjusts the ROU by the same delta (Dr/Cr 1600↔2600), then depreciates over the remaining term (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P99" s="16" t="inlineStr">
         <is>
-          <t>Certified recon</t>
+          <t>Lease register; periodic run log; modification remeasurement</t>
         </is>
       </c>
       <c r="Q99" s="18" t="inlineStr">
@@ -9496,7 +9496,7 @@
     <row r="100">
       <c r="A100" s="11" t="inlineStr">
         <is>
-          <t>REC-02</t>
+          <t>REC-01</t>
         </is>
       </c>
       <c r="B100" s="12" t="inlineStr">
@@ -9511,22 +9511,22 @@
       </c>
       <c r="D100" s="12" t="inlineStr">
         <is>
-          <t>Cash</t>
+          <t>All</t>
         </is>
       </c>
       <c r="E100" s="12" t="inlineStr">
         <is>
-          <t>Bank balance not reconciled to GL.</t>
+          <t>Subledgers diverge from GL undetected.</t>
         </is>
       </c>
       <c r="F100" s="12" t="inlineStr">
         <is>
-          <t>Existence/Completeness</t>
+          <t>Completeness/Accuracy</t>
         </is>
       </c>
       <c r="G100" s="12" t="inlineStr">
         <is>
-          <t>Bank reconciliation against statements.</t>
+          <t>Subledger-to-GL reconciliation per period: import GL, auto-match, certify (sign-off via 'approvals').</t>
         </is>
       </c>
       <c r="H100" s="13" t="inlineStr">
@@ -9556,22 +9556,22 @@
       </c>
       <c r="M100" s="12" t="inlineStr">
         <is>
-          <t>bank module; drizzle/0015_bank_reconciliation</t>
+          <t>reconciliation.service.ts (importGlItems/autoMatch/certify)</t>
         </is>
       </c>
       <c r="N100" s="12" t="inlineStr">
         <is>
-          <t>Inspect bank-rec process.</t>
+          <t>Inspect recon + certify gate.</t>
         </is>
       </c>
       <c r="O100" s="12" t="inlineStr">
         <is>
-          <t>Sample months reconciled &amp; reviewed.</t>
+          <t>Sample periods: reconciled, unmatched cleared, certified.</t>
         </is>
       </c>
       <c r="P100" s="12" t="inlineStr">
         <is>
-          <t>Bank rec</t>
+          <t>Certified recon</t>
         </is>
       </c>
       <c r="Q100" s="18" t="inlineStr">
@@ -9583,12 +9583,12 @@
     <row r="101">
       <c r="A101" s="15" t="inlineStr">
         <is>
-          <t>BANK-02</t>
+          <t>REC-02</t>
         </is>
       </c>
       <c r="B101" s="16" t="inlineStr">
         <is>
-          <t>Cash &amp; Treasury</t>
+          <t>Reconciliation</t>
         </is>
       </c>
       <c r="C101" s="17" t="inlineStr">
@@ -9598,37 +9598,37 @@
       </c>
       <c r="D101" s="16" t="inlineStr">
         <is>
-          <t>Cash; Operating expense; Interest income</t>
+          <t>Cash</t>
         </is>
       </c>
       <c r="E101" s="16" t="inlineStr">
         <is>
-          <t>A bank fee/interest adjustment is posted straight to the GL by one person during reconciliation — a cash outflow mis-booked as interest income, or a fictitious fee posted, with no independent review (single-person posting to the cash account).</t>
+          <t>Bank balance not reconciled to GL.</t>
         </is>
       </c>
       <c r="F101" s="16" t="inlineStr">
         <is>
-          <t>Authorization/Accuracy</t>
+          <t>Existence/Completeness</t>
         </is>
       </c>
       <c r="G101" s="16" t="inlineStr">
         <is>
-          <t>Bank adjustment maker-checker (SoD): a fee/interest adjustment on a statement line is a REQUEST that posts a DRAFT JE (no balance/GL effect; the line stays unreconciled) until a DIFFERENT user with approval authority approves (POST /api/bank/lines/:id/adjustment/approve). Self-approval → SOD_VIOLATION (binds even Admin); approval flips the line to reconciled and the JE to Posted; reject voids the Draft and frees the line. The Draft JE (source BANKADJ) is also surfaced, aged, by the pending-approvals monitor (GOV-01).</t>
+          <t>Bank reconciliation against statements.</t>
         </is>
       </c>
       <c r="H101" s="17" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I101" s="17" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="J101" s="17" t="inlineStr">
         <is>
-          <t>Per adjustment</t>
+          <t>Monthly</t>
         </is>
       </c>
       <c r="K101" s="16" t="inlineStr">
@@ -9638,27 +9638,27 @@
       </c>
       <c r="L101" s="17" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="M101" s="16" t="inlineStr">
         <is>
-          <t>bank.service.ts requestAdjustment/approveAdjustment/rejectAdjustment/listPendingAdjustments (reuses ledger.approveEntry SoD); bank.controller.ts (lines/:id/adjustment requests; adjustment/approve|reject gated approvals/gl_close); cutover/bankrec.ts (ToE)</t>
+          <t>bank module; drizzle/0015_bank_reconciliation</t>
         </is>
       </c>
       <c r="N101" s="16" t="inlineStr">
         <is>
-          <t>Inspect the request→approve flow + the approver≠requester check + that the Draft posts nothing until approval.</t>
+          <t>Inspect bank-rec process.</t>
         </is>
       </c>
       <c r="O101" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: request a fee adjustment (line unreconciled, GL difference unchanged), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm the difference closes to 0 only after approval (re-performed by the bankrec harness).</t>
+          <t>Sample months reconciled &amp; reviewed.</t>
         </is>
       </c>
       <c r="P101" s="16" t="inlineStr">
         <is>
-          <t>Bank adjustment queue + SoD test</t>
+          <t>Bank rec</t>
         </is>
       </c>
       <c r="Q101" s="18" t="inlineStr">
@@ -9670,12 +9670,12 @@
     <row r="102">
       <c r="A102" s="11" t="inlineStr">
         <is>
-          <t>REC-03</t>
+          <t>BANK-02</t>
         </is>
       </c>
       <c r="B102" s="12" t="inlineStr">
         <is>
-          <t>Reconciliation</t>
+          <t>Cash &amp; Treasury</t>
         </is>
       </c>
       <c r="C102" s="13" t="inlineStr">
@@ -9685,79 +9685,79 @@
       </c>
       <c r="D102" s="12" t="inlineStr">
         <is>
-          <t>Consolidation</t>
+          <t>Cash; Operating expense; Interest income</t>
         </is>
       </c>
       <c r="E102" s="12" t="inlineStr">
         <is>
-          <t>Intercompany balances not eliminated/agreed.</t>
+          <t>A bank fee/interest adjustment is posted straight to the GL by one person during reconciliation — a cash outflow mis-booked as interest income, or a fictitious fee posted, with no independent review (single-person posting to the cash account).</t>
         </is>
       </c>
       <c r="F102" s="12" t="inlineStr">
         <is>
-          <t>Accuracy</t>
+          <t>Authorization/Accuracy</t>
         </is>
       </c>
       <c r="G102" s="12" t="inlineStr">
         <is>
-          <t>Intercompany reconciliation &amp; elimination on consolidation.</t>
+          <t>Bank adjustment maker-checker (SoD): a fee/interest adjustment on a statement line is a REQUEST that posts a DRAFT JE (no balance/GL effect; the line stays unreconciled) until a DIFFERENT user with approval authority approves (POST /api/bank/lines/:id/adjustment/approve). Self-approval → SOD_VIOLATION (binds even Admin); approval flips the line to reconciled and the JE to Posted; reject voids the Draft and frees the line. The Draft JE (source BANKADJ) is also surfaced, aged, by the pending-approvals monitor (GOV-01).</t>
         </is>
       </c>
       <c r="H102" s="13" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I102" s="13" t="inlineStr">
         <is>
-          <t>Auto+Manual</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J102" s="13" t="inlineStr">
         <is>
-          <t>Period</t>
+          <t>Per adjustment</t>
         </is>
       </c>
       <c r="K102" s="12" t="inlineStr">
         <is>
-          <t>Group Controller</t>
+          <t>Controller</t>
         </is>
       </c>
       <c r="L102" s="13" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="M102" s="12" t="inlineStr">
         <is>
-          <t>intercompany; consolidation</t>
+          <t>bank.service.ts requestAdjustment/approveAdjustment/rejectAdjustment/listPendingAdjustments (reuses ledger.approveEntry SoD); bank.controller.ts (lines/:id/adjustment requests; adjustment/approve|reject gated approvals/gl_close); cutover/bankrec.ts (ToE)</t>
         </is>
       </c>
       <c r="N102" s="12" t="inlineStr">
         <is>
-          <t>Inspect IC matching + elimination.</t>
+          <t>Inspect the request→approve flow + the approver≠requester check + that the Draft posts nothing until approval.</t>
         </is>
       </c>
       <c r="O102" s="12" t="inlineStr">
         <is>
-          <t>Sample IC pairs agree &amp; eliminate.</t>
+          <t>Re-perform: request a fee adjustment (line unreconciled, GL difference unchanged), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm the difference closes to 0 only after approval (re-performed by the bankrec harness).</t>
         </is>
       </c>
       <c r="P102" s="12" t="inlineStr">
         <is>
-          <t>IC recon</t>
-        </is>
-      </c>
-      <c r="Q102" s="19" t="inlineStr">
-        <is>
-          <t>Partial</t>
+          <t>Bank adjustment queue + SoD test</t>
+        </is>
+      </c>
+      <c r="Q102" s="18" t="inlineStr">
+        <is>
+          <t>Implemented</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="15" t="inlineStr">
         <is>
-          <t>REC-04</t>
+          <t>REC-03</t>
         </is>
       </c>
       <c r="B103" s="16" t="inlineStr">
@@ -9772,22 +9772,22 @@
       </c>
       <c r="D103" s="16" t="inlineStr">
         <is>
-          <t>All control accounts</t>
+          <t>Consolidation</t>
         </is>
       </c>
       <c r="E103" s="16" t="inlineStr">
         <is>
-          <t>A sub-ledger silently drifts from its GL control account at period-end and no single review catches it (incomplete/inaccurate balances reach the financial statements).</t>
+          <t>Intercompany balances not eliminated/agreed.</t>
         </is>
       </c>
       <c r="F103" s="16" t="inlineStr">
         <is>
-          <t>Completeness/Accuracy</t>
+          <t>Accuracy</t>
         </is>
       </c>
       <c r="G103" s="16" t="inlineStr">
         <is>
-          <t>Period-end control-account reconciliation PACK: one read (GET /api/finance/reconciliation/controls) ties every major sub-ledger to its GL control account and FLAGS any out-of-balance — AR↔1100, AP↔2000, Inventory↔1200, Gift cards/Customer-deposits↔2200, Deferred revenue↔2400 — reporting per line {sub_ledger, gl_control, variance, reconciled} plus an overall all_reconciled flag and an exceptions count. Liability controls are sign-flipped before comparison. The controller's single 'are the books reconciled?' close view; an exception is a control finding to investigate before sign-off.</t>
+          <t>Intercompany reconciliation &amp; elimination on consolidation.</t>
         </is>
       </c>
       <c r="H103" s="17" t="inlineStr">
@@ -9797,17 +9797,17 @@
       </c>
       <c r="I103" s="17" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="J103" s="17" t="inlineStr">
         <is>
-          <t>Period / on demand</t>
+          <t>Period</t>
         </is>
       </c>
       <c r="K103" s="16" t="inlineStr">
         <is>
-          <t>Controller / CFO</t>
+          <t>Group Controller</t>
         </is>
       </c>
       <c r="L103" s="17" t="inlineStr">
@@ -9817,34 +9817,34 @@
       </c>
       <c r="M103" s="16" t="inlineStr">
         <is>
-          <t>finance.service.ts reconcileControls; finance.controller.ts GET reconciliation/controls (exec/ar/creditors); reuses ledger.trialBalance + the AR/AP/inventory/gift-card/deferred sub-ledgers; cutover/giftcards.ts + compliance.ts (ToE)</t>
+          <t>intercompany; consolidation</t>
         </is>
       </c>
       <c r="N103" s="16" t="inlineStr">
         <is>
-          <t>Inspect the pack: each control account's sub-ledger query + the GL tie + the exceptions roll-up.</t>
+          <t>Inspect IC matching + elimination.</t>
         </is>
       </c>
       <c r="O103" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: with a clean set, every line reconciled + all_reconciled=true; introduce a known sub-ledger/GL difference and confirm it surfaces as an exception (re-performed: gift-card 2200 + inventory 1200 ties asserted by the harnesses).</t>
+          <t>Sample IC pairs agree &amp; eliminate.</t>
         </is>
       </c>
       <c r="P103" s="16" t="inlineStr">
         <is>
-          <t>Reconciliation pack; exceptions list</t>
-        </is>
-      </c>
-      <c r="Q103" s="18" t="inlineStr">
-        <is>
-          <t>Implemented</t>
+          <t>IC recon</t>
+        </is>
+      </c>
+      <c r="Q103" s="19" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="11" t="inlineStr">
         <is>
-          <t>REC-05</t>
+          <t>REC-04</t>
         </is>
       </c>
       <c r="B104" s="12" t="inlineStr">
@@ -9859,42 +9859,42 @@
       </c>
       <c r="D104" s="12" t="inlineStr">
         <is>
-          <t>Cash; Bank</t>
+          <t>All control accounts</t>
         </is>
       </c>
       <c r="E104" s="12" t="inlineStr">
         <is>
-          <t>Till cash dropped to the safe never reaches the bank, or a deposit isn't matched to the statement — cash sits unbanked (theft/loss exposure) or the bank balance can't be tied to the books.</t>
+          <t>A sub-ledger silently drifts from its GL control account at period-end and no single review catches it (incomplete/inaccurate balances reach the financial statements).</t>
         </is>
       </c>
       <c r="F104" s="12" t="inlineStr">
         <is>
-          <t>Completeness/Existence/Authorization</t>
+          <t>Completeness/Accuracy</t>
         </is>
       </c>
       <c r="G104" s="12" t="inlineStr">
         <is>
-          <t>Cash banking — safe-drop → bank deposit → reconciliation: till 'drop's move cash from the drawer to the safe (drawer-only, no GL). Banking BATCHES the undeposited drops into a deposit and posts the GL (Dr &lt;bank account, e.g. 1010&gt; / Cr 1000 Cash), stamping each drop with the deposit id; the deposit is then RECONCILED to the bank statement (status Deposited→Reconciled). A detective read (GET /api/bank/deposits/undeposited-drops) surfaces the CASH STILL IN THE SAFE (drops with deposit_id NULL) — the unbanked exposure to chase. SoD: banking is a treasury duty (exec/ar) — segregated from the cashier (pos_till) who drops the cash, so the person who removes cash from the drawer is not the one who banks it.</t>
+          <t>Period-end control-account reconciliation PACK: one read (GET /api/finance/reconciliation/controls) ties every major sub-ledger to its GL control account and FLAGS any out-of-balance — AR↔1100, AP↔2000, Inventory↔1200, Gift cards/Customer-deposits↔2200, Deferred revenue↔2400 — reporting per line {sub_ledger, gl_control, variance, reconciled} plus an overall all_reconciled flag and an exceptions count. Liability controls are sign-flipped before comparison. The controller's single 'are the books reconciled?' close view; an exception is a control finding to investigate before sign-off.</t>
         </is>
       </c>
       <c r="H104" s="13" t="inlineStr">
         <is>
-          <t>Det/Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I104" s="13" t="inlineStr">
         <is>
-          <t>Auto+Manual</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J104" s="13" t="inlineStr">
         <is>
-          <t>Per banking run</t>
+          <t>Period / on demand</t>
         </is>
       </c>
       <c r="K104" s="12" t="inlineStr">
         <is>
-          <t>FinancialController / Treasury</t>
+          <t>Controller / CFO</t>
         </is>
       </c>
       <c r="L104" s="13" t="inlineStr">
@@ -9904,22 +9904,22 @@
       </c>
       <c r="M104" s="12" t="inlineStr">
         <is>
-          <t>bank.service.ts undepositedDrops/createDeposit (Dr bank/Cr 1000, stamps deposit_id)/reconcileDeposit/listDeposits; bank.controller.ts (deposits, deposits/undeposited-drops, deposits/:id/reconcile; exec/ar); schema/cash.ts bank_deposits + cash_movements.deposit_id + migration 0152; /cash-banking UI; cutover/cash-banking.ts (ToE)</t>
+          <t>finance.service.ts reconcileControls; finance.controller.ts GET reconciliation/controls (exec/ar/creditors); reuses ledger.trialBalance + the AR/AP/inventory/gift-card/deferred sub-ledgers; cutover/giftcards.ts + compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N104" s="12" t="inlineStr">
         <is>
-          <t>Inspect the undeposited-drop exposure read + the deposit GL (bank↔1000) + the reconcile step + the SoD (cashier vs treasury).</t>
+          <t>Inspect the pack: each control account's sub-ledger query + the GL tie + the exceptions roll-up.</t>
         </is>
       </c>
       <c r="O104" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: two till drops → cash-in-safe shows the total; a cashier (pos_till) cannot bank (403); treasury banks → Dr bank / Cr 1000, cash-in-safe back to 0; reconcile the deposit; trial balance balanced (re-performed by the cash-banking harness).</t>
+          <t>Re-perform: with a clean set, every line reconciled + all_reconciled=true; introduce a known sub-ledger/GL difference and confirm it surfaces as an exception (re-performed: gift-card 2200 + inventory 1200 ties asserted by the harnesses).</t>
         </is>
       </c>
       <c r="P104" s="12" t="inlineStr">
         <is>
-          <t>Bank-deposit register; undeposited-drop (cash-in-safe) exposure</t>
+          <t>Reconciliation pack; exceptions list</t>
         </is>
       </c>
       <c r="Q104" s="18" t="inlineStr">
@@ -9931,12 +9931,12 @@
     <row r="105">
       <c r="A105" s="15" t="inlineStr">
         <is>
-          <t>GOV-01</t>
+          <t>REC-05</t>
         </is>
       </c>
       <c r="B105" s="16" t="inlineStr">
         <is>
-          <t>Monitoring</t>
+          <t>Reconciliation</t>
         </is>
       </c>
       <c r="C105" s="17" t="inlineStr">
@@ -9946,42 +9946,42 @@
       </c>
       <c r="D105" s="16" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Cash; Bank</t>
         </is>
       </c>
       <c r="E105" s="16" t="inlineStr">
         <is>
-          <t>A maker-checker approval sits un-actioned and is forgotten — a transaction stalls before it is effective, or (worse) a control is quietly bypassed and no one notices an item never got its independent review.</t>
+          <t>Till cash dropped to the safe never reaches the bank, or a deposit isn't matched to the statement — cash sits unbanked (theft/loss exposure) or the bank balance can't be tied to the books.</t>
         </is>
       </c>
       <c r="F105" s="16" t="inlineStr">
         <is>
-          <t>Authorization/Completeness</t>
+          <t>Completeness/Existence/Authorization</t>
         </is>
       </c>
       <c r="G105" s="16" t="inlineStr">
         <is>
-          <t>Pending-approvals MONITOR (COSO monitoring): a single worklist of EVERY item awaiting independent approval across the system, each with its AGE in days and an overdue roll-up — spanning the manual-JE (GL-05), bank-adjustment (BANK-02), AP-disbursement (EXP-06), payroll (PAY-03), asset-revaluation (FA-08), asset-disposal (FA-09), inventory-write-off (INV-07), till-close cash over/short (REV-13), FX-rate (FX-04), budget (BUD-01) and large-refund (REV-16) maker-checkers. The controller reviews it before close; a stale item (age beyond the threshold) is a control finding to chase or escalate. The /approvals screen also lets a manager approve/reject a material till variance or a large refund inline (the pending types with no dedicated module screen). Read-only worklist; tenant-scoped via the caller's RLS.</t>
+          <t>Cash banking — safe-drop → bank deposit → reconciliation: till 'drop's move cash from the drawer to the safe (drawer-only, no GL). Banking BATCHES the undeposited drops into a deposit and posts the GL (Dr &lt;bank account, e.g. 1010&gt; / Cr 1000 Cash), stamping each drop with the deposit id; the deposit is then RECONCILED to the bank statement (status Deposited→Reconciled). A detective read (GET /api/bank/deposits/undeposited-drops) surfaces the CASH STILL IN THE SAFE (drops with deposit_id NULL) — the unbanked exposure to chase. SoD: banking is a treasury duty (exec/ar) — segregated from the cashier (pos_till) who drops the cash, so the person who removes cash from the drawer is not the one who banks it.</t>
         </is>
       </c>
       <c r="H105" s="17" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Det/Prev</t>
         </is>
       </c>
       <c r="I105" s="17" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="J105" s="17" t="inlineStr">
         <is>
-          <t>Continuous / pre-close</t>
+          <t>Per banking run</t>
         </is>
       </c>
       <c r="K105" s="16" t="inlineStr">
         <is>
-          <t>Controller / CFO</t>
+          <t>FinancialController / Treasury</t>
         </is>
       </c>
       <c r="L105" s="17" t="inlineStr">
@@ -9991,22 +9991,22 @@
       </c>
       <c r="M105" s="16" t="inlineStr">
         <is>
-          <t>finance.service.ts pendingApprovals; finance.controller.ts GET approvals/pending (exec/approvals/creditors); aggregates journalEntries(Draft incl. BANKADJ→BANK-02)/apPayments/payruns/asset_revaluations/fixed_assets(disposal_pending)/inv_writeoff_requests/till_sessions(PendingApproval)/fx_rates(PendingApproval)/budgets(PendingApproval); cutover/compliance.ts (ToE)</t>
+          <t>bank.service.ts undepositedDrops/createDeposit (Dr bank/Cr 1000, stamps deposit_id)/reconcileDeposit/listDeposits; bank.controller.ts (deposits, deposits/undeposited-drops, deposits/:id/reconcile; exec/ar); schema/cash.ts bank_deposits + cash_movements.deposit_id + migration 0152; /cash-banking UI; cutover/cash-banking.ts (ToE)</t>
         </is>
       </c>
       <c r="N105" s="16" t="inlineStr">
         <is>
-          <t>Inspect the aggregation across all pending sources + the age/overdue roll-up.</t>
+          <t>Inspect the undeposited-drop exposure read + the deposit GL (bank↔1000) + the reconcile step + the SoD (cashier vs treasury).</t>
         </is>
       </c>
       <c r="O105" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: create a pending item (e.g. a Draft JE) and confirm it appears in the worklist with its control ID, amount and age; the overdue count flags items past the threshold (re-performed by the harness).</t>
+          <t>Re-perform: two till drops → cash-in-safe shows the total; a cashier (pos_till) cannot bank (403); treasury banks → Dr bank / Cr 1000, cash-in-safe back to 0; reconcile the deposit; trial balance balanced (re-performed by the cash-banking harness).</t>
         </is>
       </c>
       <c r="P105" s="16" t="inlineStr">
         <is>
-          <t>Pending-approvals worklist</t>
+          <t>Bank-deposit register; undeposited-drop (cash-in-safe) exposure</t>
         </is>
       </c>
       <c r="Q105" s="18" t="inlineStr">
@@ -10018,12 +10018,12 @@
     <row r="106">
       <c r="A106" s="11" t="inlineStr">
         <is>
-          <t>TAX-01</t>
+          <t>GOV-01</t>
         </is>
       </c>
       <c r="B106" s="12" t="inlineStr">
         <is>
-          <t>Tax</t>
+          <t>Monitoring</t>
         </is>
       </c>
       <c r="C106" s="13" t="inlineStr">
@@ -10033,27 +10033,27 @@
       </c>
       <c r="D106" s="12" t="inlineStr">
         <is>
-          <t>Tax (VAT)</t>
+          <t>All</t>
         </is>
       </c>
       <c r="E106" s="12" t="inlineStr">
         <is>
-          <t>VAT computed incorrectly → filing/penalty risk.</t>
+          <t>A maker-checker approval sits un-actioned and is forgotten — a transaction stalls before it is effective, or (worse) a control is quietly bypassed and no one notices an item never got its independent review.</t>
         </is>
       </c>
       <c r="F106" s="12" t="inlineStr">
         <is>
-          <t>Accuracy</t>
+          <t>Authorization/Completeness</t>
         </is>
       </c>
       <c r="G106" s="12" t="inlineStr">
         <is>
-          <t>VAT via pluggable provider (TH 7%); unit-tested; no hard-coded rate.</t>
+          <t>Pending-approvals MONITOR (COSO monitoring): a single worklist of EVERY item awaiting independent approval across the system, each with its AGE in days and an overdue roll-up — spanning the manual-JE (GL-05), bank-adjustment (BANK-02), AP-disbursement (EXP-06), payroll (PAY-03), asset-revaluation (FA-08), asset-disposal (FA-09), inventory-write-off (INV-07), till-close cash over/short (REV-13), FX-rate (FX-04), budget (BUD-01) and large-refund (REV-16) maker-checkers. The controller reviews it before close; a stale item (age beyond the threshold) is a control finding to chase or escalate. The /approvals screen also lets a manager approve/reject a material till variance or a large refund inline (the pending types with no dedicated module screen). Read-only worklist; tenant-scoped via the caller's RLS.</t>
         </is>
       </c>
       <c r="H106" s="13" t="inlineStr">
         <is>
-          <t>Auto</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I106" s="13" t="inlineStr">
@@ -10063,37 +10063,37 @@
       </c>
       <c r="J106" s="13" t="inlineStr">
         <is>
-          <t>Per txn</t>
+          <t>Continuous / pre-close</t>
         </is>
       </c>
       <c r="K106" s="12" t="inlineStr">
         <is>
-          <t>Tax / Controller</t>
+          <t>Controller / CFO</t>
         </is>
       </c>
       <c r="L106" s="13" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="M106" s="12" t="inlineStr">
         <is>
-          <t>tax/tax-providers.ts; tax.service.ts; test/unit.test.ts</t>
+          <t>finance.service.ts pendingApprovals; finance.controller.ts GET approvals/pending (exec/approvals/creditors); aggregates journalEntries(Draft incl. BANKADJ→BANK-02)/apPayments/payruns/asset_revaluations/fixed_assets(disposal_pending)/inv_writeoff_requests/till_sessions(PendingApproval)/fx_rates(PendingApproval)/budgets(PendingApproval); cutover/compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N106" s="12" t="inlineStr">
         <is>
-          <t>Inspect rate provider + tests.</t>
+          <t>Inspect the aggregation across all pending sources + the age/overdue roll-up.</t>
         </is>
       </c>
       <c r="O106" s="12" t="inlineStr">
         <is>
-          <t>Re-perform VAT on sample; tie to return.</t>
+          <t>Re-perform: create a pending item (e.g. a Draft JE) and confirm it appears in the worklist with its control ID, amount and age; the overdue count flags items past the threshold (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P106" s="12" t="inlineStr">
         <is>
-          <t>VAT tests</t>
+          <t>Pending-approvals worklist</t>
         </is>
       </c>
       <c r="Q106" s="18" t="inlineStr">
@@ -10105,7 +10105,7 @@
     <row r="107">
       <c r="A107" s="15" t="inlineStr">
         <is>
-          <t>TAX-02</t>
+          <t>TAX-01</t>
         </is>
       </c>
       <c r="B107" s="16" t="inlineStr">
@@ -10120,22 +10120,22 @@
       </c>
       <c r="D107" s="16" t="inlineStr">
         <is>
-          <t>Tax; Revenue</t>
+          <t>Tax (VAT)</t>
         </is>
       </c>
       <c r="E107" s="16" t="inlineStr">
         <is>
-          <t>Non-compliant e-Tax invoice / not transmitted to ETDA.</t>
+          <t>VAT computed incorrectly → filing/penalty risk.</t>
         </is>
       </c>
       <c r="F107" s="16" t="inlineStr">
         <is>
-          <t>Accuracy/Compliance</t>
+          <t>Accuracy</t>
         </is>
       </c>
       <c r="G107" s="16" t="inlineStr">
         <is>
-          <t>e-Tax invoice (ETDA UBL 2.1 XML) generation + email with CC to ETDA timestamp mailbox.</t>
+          <t>VAT via pluggable provider (TH 7%); unit-tested; no hard-coded rate.</t>
         </is>
       </c>
       <c r="H107" s="17" t="inlineStr">
@@ -10150,37 +10150,37 @@
       </c>
       <c r="J107" s="17" t="inlineStr">
         <is>
-          <t>Per invoice</t>
+          <t>Per txn</t>
         </is>
       </c>
       <c r="K107" s="16" t="inlineStr">
         <is>
-          <t>Tax</t>
+          <t>Tax / Controller</t>
         </is>
       </c>
       <c r="L107" s="17" t="inlineStr">
         <is>
-          <t>P10/P13</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="M107" s="16" t="inlineStr">
         <is>
-          <t>tax-docs/etax-xml.ts; etax-email.service.ts (tested)</t>
+          <t>tax/tax-providers.ts; tax.service.ts; test/unit.test.ts</t>
         </is>
       </c>
       <c r="N107" s="16" t="inlineStr">
         <is>
-          <t>Inspect XML schema + email composer.</t>
+          <t>Inspect rate provider + tests.</t>
         </is>
       </c>
       <c r="O107" s="16" t="inlineStr">
         <is>
-          <t>Sample invoices: valid XML, correct CC/escaping.</t>
+          <t>Re-perform VAT on sample; tie to return.</t>
         </is>
       </c>
       <c r="P107" s="16" t="inlineStr">
         <is>
-          <t>e-Tax samples</t>
+          <t>VAT tests</t>
         </is>
       </c>
       <c r="Q107" s="18" t="inlineStr">
@@ -10192,7 +10192,7 @@
     <row r="108">
       <c r="A108" s="11" t="inlineStr">
         <is>
-          <t>TAX-03</t>
+          <t>TAX-02</t>
         </is>
       </c>
       <c r="B108" s="12" t="inlineStr">
@@ -10207,22 +10207,22 @@
       </c>
       <c r="D108" s="12" t="inlineStr">
         <is>
-          <t>Tax (WHT)</t>
+          <t>Tax; Revenue</t>
         </is>
       </c>
       <c r="E108" s="12" t="inlineStr">
         <is>
-          <t>Withholding tax mis-computed / not reported.</t>
+          <t>Non-compliant e-Tax invoice / not transmitted to ETDA.</t>
         </is>
       </c>
       <c r="F108" s="12" t="inlineStr">
         <is>
-          <t>Accuracy</t>
+          <t>Accuracy/Compliance</t>
         </is>
       </c>
       <c r="G108" s="12" t="inlineStr">
         <is>
-          <t>WHT computation and ภ.ง.ด. reporting.</t>
+          <t>e-Tax invoice (ETDA UBL 2.1 XML) generation + email with CC to ETDA timestamp mailbox.</t>
         </is>
       </c>
       <c r="H108" s="13" t="inlineStr">
@@ -10237,7 +10237,7 @@
       </c>
       <c r="J108" s="13" t="inlineStr">
         <is>
-          <t>Per txn / monthly</t>
+          <t>Per invoice</t>
         </is>
       </c>
       <c r="K108" s="12" t="inlineStr">
@@ -10247,39 +10247,39 @@
       </c>
       <c r="L108" s="13" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P10/P13</t>
         </is>
       </c>
       <c r="M108" s="12" t="inlineStr">
         <is>
-          <t>tax-reports; payroll</t>
+          <t>tax-docs/etax-xml.ts; etax-email.service.ts (tested)</t>
         </is>
       </c>
       <c r="N108" s="12" t="inlineStr">
         <is>
-          <t>Inspect WHT logic + report.</t>
+          <t>Inspect XML schema + email composer.</t>
         </is>
       </c>
       <c r="O108" s="12" t="inlineStr">
         <is>
-          <t>Re-perform WHT on sample; tie to filing.</t>
+          <t>Sample invoices: valid XML, correct CC/escaping.</t>
         </is>
       </c>
       <c r="P108" s="12" t="inlineStr">
         <is>
-          <t>WHT report</t>
-        </is>
-      </c>
-      <c r="Q108" s="19" t="inlineStr">
-        <is>
-          <t>Partial</t>
+          <t>e-Tax samples</t>
+        </is>
+      </c>
+      <c r="Q108" s="18" t="inlineStr">
+        <is>
+          <t>Implemented</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="15" t="inlineStr">
         <is>
-          <t>TAX-04</t>
+          <t>TAX-03</t>
         </is>
       </c>
       <c r="B109" s="16" t="inlineStr">
@@ -10294,27 +10294,27 @@
       </c>
       <c r="D109" s="16" t="inlineStr">
         <is>
-          <t>Tax (VAT); Tax Payable (2100)</t>
+          <t>Tax (WHT)</t>
         </is>
       </c>
       <c r="E109" s="16" t="inlineStr">
         <is>
-          <t>Output/input VAT on the filed ภ.พ.30 return does not agree to the GL — VAT liability mis-stated, a filing/penalty exposure, or a posting omission goes undetected before submission.</t>
+          <t>Withholding tax mis-computed / not reported.</t>
         </is>
       </c>
       <c r="F109" s="16" t="inlineStr">
         <is>
-          <t>Completeness/Accuracy</t>
+          <t>Accuracy</t>
         </is>
       </c>
       <c r="G109" s="16" t="inlineStr">
         <is>
-          <t>Periodic VAT-return ↔ GL reconciliation (ภ.พ.30): the monthly return (GET /api/tax-reports/pp30) is built from the sales/output-VAT and purchase/input-VAT sub-reports, computes net VAT = output − input, and RECONCILES it to the **GL account 2100 (Tax Payable) net movement** for the same period (Σ credit − Σ debit over Posted entries) — returning `reconciliation.tied` = true only when the two agree within rounding. A non-tie is a detective finding to investigate and clear BEFORE filing (the form also carries the ม.157 deadline = the 15th of the next month). Output VAT is posted to 2100 on every sale (Cr) and reversed on returns (Dr); input VAT is posted on AP bills (Dr) — so 2100's net is the period's VAT payable. Read-only report; exportable to a ภ.พ.30 PDF/HTML.</t>
+          <t>WHT computation and ภ.ง.ด. reporting.</t>
         </is>
       </c>
       <c r="H109" s="17" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Auto</t>
         </is>
       </c>
       <c r="I109" s="17" t="inlineStr">
@@ -10324,54 +10324,54 @@
       </c>
       <c r="J109" s="17" t="inlineStr">
         <is>
-          <t>Monthly / pre-filing</t>
+          <t>Per txn / monthly</t>
         </is>
       </c>
       <c r="K109" s="16" t="inlineStr">
         <is>
-          <t>Tax / FinancialController</t>
+          <t>Tax</t>
         </is>
       </c>
       <c r="L109" s="17" t="inlineStr">
         <is>
-          <t>P10/P16</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="M109" s="16" t="inlineStr">
         <is>
-          <t>tax-reports.service.ts pp30 (outputVat/inputVat + 2100 net-movement tie); tax-reports.controller.ts (GET pp30, pp30/export, exec); tax-reports-pdf.ts; dine-in.service.ts/returns.service.ts/finance.service.ts post 2100 on sale/return/AP; /tax/reports UI; cutover/taxdocs.ts (ToE)</t>
+          <t>tax-reports; payroll</t>
         </is>
       </c>
       <c r="N109" s="16" t="inlineStr">
         <is>
-          <t>Inspect the pp30 build + the 2100 net-movement query + the tie flag + the filing deadline.</t>
+          <t>Inspect WHT logic + report.</t>
         </is>
       </c>
       <c r="O109" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: the pp30 return computes net VAT (output − input), the GL 2100 net movement reflects the posted input VAT, and the reconciliation block exposes the gl_account (2100), the report net VAT and a boolean tie verdict (tied iff the two agree within rounding); the ภ.พ.30 export renders (re-performed by the taxdocs harness).</t>
+          <t>Re-perform WHT on sample; tie to filing.</t>
         </is>
       </c>
       <c r="P109" s="16" t="inlineStr">
         <is>
-          <t>ภ.พ.30 return + GL-2100 reconciliation tie</t>
-        </is>
-      </c>
-      <c r="Q109" s="18" t="inlineStr">
-        <is>
-          <t>Implemented</t>
+          <t>WHT report</t>
+        </is>
+      </c>
+      <c r="Q109" s="19" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="11" t="inlineStr">
         <is>
-          <t>PAY-01</t>
+          <t>TAX-04</t>
         </is>
       </c>
       <c r="B110" s="12" t="inlineStr">
         <is>
-          <t>Payroll</t>
+          <t>Tax</t>
         </is>
       </c>
       <c r="C110" s="13" t="inlineStr">
@@ -10381,27 +10381,27 @@
       </c>
       <c r="D110" s="12" t="inlineStr">
         <is>
-          <t>Payroll expense/liability</t>
+          <t>Tax (VAT); Tax Payable (2100)</t>
         </is>
       </c>
       <c r="E110" s="12" t="inlineStr">
         <is>
-          <t>Payroll, SSO and PIT mis-computed.</t>
+          <t>Output/input VAT on the filed ภ.พ.30 return does not agree to the GL — VAT liability mis-stated, a filing/penalty exposure, or a posting omission goes undetected before submission.</t>
         </is>
       </c>
       <c r="F110" s="12" t="inlineStr">
         <is>
-          <t>Accuracy</t>
+          <t>Completeness/Accuracy</t>
         </is>
       </c>
       <c r="G110" s="12" t="inlineStr">
         <is>
-          <t>Payroll engine — SSO 5% (cap 750), progressive PIT, payslip net; unit-tested.</t>
+          <t>Periodic VAT-return ↔ GL reconciliation (ภ.พ.30): the monthly return (GET /api/tax-reports/pp30) is built from the sales/output-VAT and purchase/input-VAT sub-reports, computes net VAT = output − input, and RECONCILES it to the **GL account 2100 (Tax Payable) net movement** for the same period (Σ credit − Σ debit over Posted entries) — returning `reconciliation.tied` = true only when the two agree within rounding. A non-tie is a detective finding to investigate and clear BEFORE filing (the form also carries the ม.157 deadline = the 15th of the next month). Output VAT is posted to 2100 on every sale (Cr) and reversed on returns (Dr); input VAT is posted on AP bills (Dr) — so 2100's net is the period's VAT payable. Read-only report; exportable to a ภ.พ.30 PDF/HTML.</t>
         </is>
       </c>
       <c r="H110" s="13" t="inlineStr">
         <is>
-          <t>Auto</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I110" s="13" t="inlineStr">
@@ -10411,37 +10411,37 @@
       </c>
       <c r="J110" s="13" t="inlineStr">
         <is>
-          <t>Per run</t>
+          <t>Monthly / pre-filing</t>
         </is>
       </c>
       <c r="K110" s="12" t="inlineStr">
         <is>
-          <t>HR / Payroll</t>
+          <t>Tax / FinancialController</t>
         </is>
       </c>
       <c r="L110" s="13" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P10/P16</t>
         </is>
       </c>
       <c r="M110" s="12" t="inlineStr">
         <is>
-          <t>payroll/payroll-calc.ts; test/unit.test.ts</t>
+          <t>tax-reports.service.ts pp30 (outputVat/inputVat + 2100 net-movement tie); tax-reports.controller.ts (GET pp30, pp30/export, exec); tax-reports-pdf.ts; dine-in.service.ts/returns.service.ts/finance.service.ts post 2100 on sale/return/AP; /tax/reports UI; cutover/taxdocs.ts (ToE)</t>
         </is>
       </c>
       <c r="N110" s="12" t="inlineStr">
         <is>
-          <t>Inspect calc + tests.</t>
+          <t>Inspect the pp30 build + the 2100 net-movement query + the tie flag + the filing deadline.</t>
         </is>
       </c>
       <c r="O110" s="12" t="inlineStr">
         <is>
-          <t>Re-perform sample payslips.</t>
+          <t>Re-perform: the pp30 return computes net VAT (output − input), the GL 2100 net movement reflects the posted input VAT, and the reconciliation block exposes the gl_account (2100), the report net VAT and a boolean tie verdict (tied iff the two agree within rounding); the ภ.พ.30 export renders (re-performed by the taxdocs harness).</t>
         </is>
       </c>
       <c r="P110" s="12" t="inlineStr">
         <is>
-          <t>Payslip tests</t>
+          <t>ภ.พ.30 return + GL-2100 reconciliation tie</t>
         </is>
       </c>
       <c r="Q110" s="18" t="inlineStr">
@@ -10453,7 +10453,7 @@
     <row r="111">
       <c r="A111" s="15" t="inlineStr">
         <is>
-          <t>PAY-02</t>
+          <t>PAY-01</t>
         </is>
       </c>
       <c r="B111" s="16" t="inlineStr">
@@ -10468,27 +10468,27 @@
       </c>
       <c r="D111" s="16" t="inlineStr">
         <is>
-          <t>Payroll liability</t>
+          <t>Payroll expense/liability</t>
         </is>
       </c>
       <c r="E111" s="16" t="inlineStr">
         <is>
-          <t>Statutory withholdings (SSO/WHT/PF) mis-stated or not remitted, so the liability owed to the authorities diverges from the books.</t>
+          <t>Payroll, SSO and PIT mis-computed.</t>
         </is>
       </c>
       <c r="F111" s="16" t="inlineStr">
         <is>
-          <t>Accuracy/Compliance</t>
+          <t>Accuracy</t>
         </is>
       </c>
       <c r="G111" s="16" t="inlineStr">
         <is>
-          <t>Payroll-liability schedule (GET /api/payroll/liabilities): each statutory account — SSO 2350, WHT/PND1 2360, PF 2370 — shows accrued (GL credits) − remitted (GL debits) = outstanding, tied back to the INDEPENDENT payrun accrual with a `reconciled` flag (a divergence flags a manual JE that touched a payroll-liability account outside the payroll process). Treasury remits the cash (POST .../remit → Dr liability / Cr 1000) which clears the outstanding and keeps the books reconciled to the statutory filings; a remittance beyond the outstanding is blocked (REMIT_EXCEEDS_OUTSTANDING).</t>
+          <t>Payroll engine — SSO 5% (cap 750), progressive PIT, payslip net; unit-tested.</t>
         </is>
       </c>
       <c r="H111" s="17" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Auto</t>
         </is>
       </c>
       <c r="I111" s="17" t="inlineStr">
@@ -10498,12 +10498,12 @@
       </c>
       <c r="J111" s="17" t="inlineStr">
         <is>
-          <t>Per run / monthly</t>
+          <t>Per run</t>
         </is>
       </c>
       <c r="K111" s="16" t="inlineStr">
         <is>
-          <t>HR / Payroll / Treasury</t>
+          <t>HR / Payroll</t>
         </is>
       </c>
       <c r="L111" s="17" t="inlineStr">
@@ -10513,22 +10513,22 @@
       </c>
       <c r="M111" s="16" t="inlineStr">
         <is>
-          <t>payroll/payroll.service.ts liabilities/remitLiability</t>
+          <t>payroll/payroll-calc.ts; test/unit.test.ts</t>
         </is>
       </c>
       <c r="N111" s="16" t="inlineStr">
         <is>
-          <t>Inspect the schedule + the accrued/remitted/outstanding tie-out and the reconciled flag.</t>
+          <t>Inspect calc + tests.</t>
         </is>
       </c>
       <c r="O111" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: run a payroll, confirm the SSO/WHT outstanding equals the payrun accrual; remit part and confirm the outstanding falls and the TB stays balanced; attempt an over-remit (REMIT_EXCEEDS_OUTSTANDING).</t>
+          <t>Re-perform sample payslips.</t>
         </is>
       </c>
       <c r="P111" s="16" t="inlineStr">
         <is>
-          <t>Liability schedule + remittance JEs tied to filings</t>
+          <t>Payslip tests</t>
         </is>
       </c>
       <c r="Q111" s="18" t="inlineStr">
@@ -10540,7 +10540,7 @@
     <row r="112">
       <c r="A112" s="11" t="inlineStr">
         <is>
-          <t>PAY-03</t>
+          <t>PAY-02</t>
         </is>
       </c>
       <c r="B112" s="12" t="inlineStr">
@@ -10555,27 +10555,27 @@
       </c>
       <c r="D112" s="12" t="inlineStr">
         <is>
-          <t>Payroll expense/liability; Cash</t>
+          <t>Payroll liability</t>
         </is>
       </c>
       <c r="E112" s="12" t="inlineStr">
         <is>
-          <t>Payroll run posted to the GL without independent review — the preparer both computes and posts their own payroll (ghost employees, inflated rate/hours).</t>
+          <t>Statutory withholdings (SSO/WHT/PF) mis-stated or not remitted, so the liability owed to the authorities diverges from the books.</t>
         </is>
       </c>
       <c r="F112" s="12" t="inlineStr">
         <is>
-          <t>Authorization</t>
+          <t>Accuracy/Compliance</t>
         </is>
       </c>
       <c r="G112" s="12" t="inlineStr">
         <is>
-          <t>Payroll maker-checker (SoD): a run posts its GL entry as a DRAFT (excluded from balances) with the run record 'PendingApproval'; a DIFFERENT user must approve before it becomes effective (approver ≠ preparer enforced regardless of permissions, reusing the GL-05 ledger approval). Reject voids the draft; idempotent per (tenant, period).</t>
+          <t>Payroll-liability schedule (GET /api/payroll/liabilities): each statutory account — SSO 2350, WHT/PND1 2360, PF 2370 — shows accrued (GL credits) − remitted (GL debits) = outstanding, tied back to the INDEPENDENT payrun accrual with a `reconciled` flag (a divergence flags a manual JE that touched a payroll-liability account outside the payroll process). Treasury remits the cash (POST .../remit → Dr liability / Cr 1000) which clears the outstanding and keeps the books reconciled to the statutory filings; a remittance beyond the outstanding is blocked (REMIT_EXCEEDS_OUTSTANDING).</t>
         </is>
       </c>
       <c r="H112" s="13" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I112" s="13" t="inlineStr">
@@ -10585,12 +10585,12 @@
       </c>
       <c r="J112" s="13" t="inlineStr">
         <is>
-          <t>Per run</t>
+          <t>Per run / monthly</t>
         </is>
       </c>
       <c r="K112" s="12" t="inlineStr">
         <is>
-          <t>HR / Payroll; Controller</t>
+          <t>HR / Payroll / Treasury</t>
         </is>
       </c>
       <c r="L112" s="13" t="inlineStr">
@@ -10600,22 +10600,22 @@
       </c>
       <c r="M112" s="12" t="inlineStr">
         <is>
-          <t>payroll/payroll.service.ts approvePayroll/rejectPayroll; migration 0133</t>
+          <t>payroll/payroll.service.ts liabilities/remitLiability</t>
         </is>
       </c>
       <c r="N112" s="12" t="inlineStr">
         <is>
-          <t>Inspect Draft→approve flow + the approver≠preparer check.</t>
+          <t>Inspect the schedule + the accrued/remitted/outstanding tie-out and the reconciled flag.</t>
         </is>
       </c>
       <c r="O112" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: run as A, attempt self-approve (SOD_VIOLATION), approve as B; confirm the JE hits balances only after approval.</t>
+          <t>Re-perform: run a payroll, confirm the SSO/WHT outstanding equals the payrun accrual; remit part and confirm the outstanding falls and the TB stays balanced; attempt an over-remit (REMIT_EXCEEDS_OUTSTANDING).</t>
         </is>
       </c>
       <c r="P112" s="12" t="inlineStr">
         <is>
-          <t>Approval log + SoD test</t>
+          <t>Liability schedule + remittance JEs tied to filings</t>
         </is>
       </c>
       <c r="Q112" s="18" t="inlineStr">
@@ -10627,12 +10627,12 @@
     <row r="113">
       <c r="A113" s="15" t="inlineStr">
         <is>
-          <t>FA-09</t>
+          <t>PAY-03</t>
         </is>
       </c>
       <c r="B113" s="16" t="inlineStr">
         <is>
-          <t>Fixed Assets</t>
+          <t>Payroll</t>
         </is>
       </c>
       <c r="C113" s="17" t="inlineStr">
@@ -10642,12 +10642,12 @@
       </c>
       <c r="D113" s="16" t="inlineStr">
         <is>
-          <t>Property, Plant &amp; Equipment; Cash</t>
+          <t>Payroll expense/liability; Cash</t>
         </is>
       </c>
       <c r="E113" s="16" t="inlineStr">
         <is>
-          <t>Asset disposed without independent review — one person writes an asset off the books and records the proceeds (asset-stripping / theft: dispose a still-held asset, or to a related party below value).</t>
+          <t>Payroll run posted to the GL without independent review — the preparer both computes and posts their own payroll (ghost employees, inflated rate/hours).</t>
         </is>
       </c>
       <c r="F113" s="16" t="inlineStr">
@@ -10657,7 +10657,7 @@
       </c>
       <c r="G113" s="16" t="inlineStr">
         <is>
-          <t>Asset-disposal maker-checker (SoD): a disposal REQUEST posts its GL entry as a DRAFT (excluded from balances) and flags the asset disposal_pending WITHOUT marking it disposed or moving the register; a DIFFERENT user must approve before it is effective (status→disposed, revaluation surplus recycled 3200→3100) (approver ≠ requester enforced regardless of permissions, reusing the GL-05 ledger approval). Reject voids the draft and the asset stays in service; only one disposal may be pending per asset; a disposal-pending asset is frozen from depreciation.</t>
+          <t>Payroll maker-checker (SoD): a run posts its GL entry as a DRAFT (excluded from balances) with the run record 'PendingApproval'; a DIFFERENT user must approve before it becomes effective (approver ≠ preparer enforced regardless of permissions, reusing the GL-05 ledger approval). Reject voids the draft; idempotent per (tenant, period).</t>
         </is>
       </c>
       <c r="H113" s="17" t="inlineStr">
@@ -10672,12 +10672,12 @@
       </c>
       <c r="J113" s="17" t="inlineStr">
         <is>
-          <t>Per disposal</t>
+          <t>Per run</t>
         </is>
       </c>
       <c r="K113" s="16" t="inlineStr">
         <is>
-          <t>FaAccountant / Controller</t>
+          <t>HR / Payroll; Controller</t>
         </is>
       </c>
       <c r="L113" s="17" t="inlineStr">
@@ -10687,22 +10687,22 @@
       </c>
       <c r="M113" s="16" t="inlineStr">
         <is>
-          <t>assets.service.ts dispose(pendingApproval Draft)/approveDisposal/rejectDisposal; assets.controller.ts (:assetNo/dispose/approve|reject); schema/assets.ts fixed_assets.disposal_pending + migration 0135; cutover/basics.ts + worldclass.ts + compliance.ts (ToE)</t>
+          <t>payroll/payroll.service.ts approvePayroll/rejectPayroll; migration 0133</t>
         </is>
       </c>
       <c r="N113" s="16" t="inlineStr">
         <is>
-          <t>Inspect Draft→approve flow + the approver≠requester check + deferred status/recycle.</t>
+          <t>Inspect Draft→approve flow + the approver≠preparer check.</t>
         </is>
       </c>
       <c r="O113" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: request a disposal (Draft JE excluded), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm status→disposed + surplus recycled only after approval (re-performed by the harnesses).</t>
+          <t>Re-perform: run as A, attempt self-approve (SOD_VIOLATION), approve as B; confirm the JE hits balances only after approval.</t>
         </is>
       </c>
       <c r="P113" s="16" t="inlineStr">
         <is>
-          <t>Disposal approval log + SoD test</t>
+          <t>Approval log + SoD test</t>
         </is>
       </c>
       <c r="Q113" s="18" t="inlineStr">
@@ -10714,7 +10714,7 @@
     <row r="114">
       <c r="A114" s="11" t="inlineStr">
         <is>
-          <t>FA-10</t>
+          <t>FA-09</t>
         </is>
       </c>
       <c r="B114" s="12" t="inlineStr">
@@ -10729,22 +10729,22 @@
       </c>
       <c r="D114" s="12" t="inlineStr">
         <is>
-          <t>Property, Plant &amp; Equipment; Accounts Payable</t>
+          <t>Property, Plant &amp; Equipment; Cash</t>
         </is>
       </c>
       <c r="E114" s="12" t="inlineStr">
         <is>
-          <t>Capital purchases mis-capitalised or capitalised without independent review — the person who receives the goods also decides what enters the asset register and at what cost/useful life (fictitious or over-valued assets; capex/opex mis-classification).</t>
+          <t>Asset disposed without independent review — one person writes an asset off the books and records the proceeds (asset-stripping / theft: dispose a still-held asset, or to a related party below value).</t>
         </is>
       </c>
       <c r="F114" s="12" t="inlineStr">
         <is>
-          <t>Authorization; Accuracy</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="G114" s="12" t="inlineStr">
         <is>
-          <t>Procure-to-Capitalize maker-checker (SoD): a goods-receipt line flagged capital (item-master is_fixed_asset or per-PO-line override) is excluded from inventory capitalisation (1200) at receipt and instead becomes ELIGIBLE for the asset register. Capitalisation is a REQUEST that posts NOTHING to the GL; a DIFFERENT user must approve before the fixed_assets row + acquisition JE (Dr 1500 / Cr 2000) are created (approver ≠ requester enforced regardless of permissions). The created asset carries its source GR/PO for end-to-end PR→PO→GR→FA traceability; a GR line cannot be capitalised twice.</t>
+          <t>Asset-disposal maker-checker (SoD): a disposal REQUEST posts its GL entry as a DRAFT (excluded from balances) and flags the asset disposal_pending WITHOUT marking it disposed or moving the register; a DIFFERENT user must approve before it is effective (status→disposed, revaluation surplus recycled 3200→3100) (approver ≠ requester enforced regardless of permissions, reusing the GL-05 ledger approval). Reject voids the draft and the asset stays in service; only one disposal may be pending per asset; a disposal-pending asset is frozen from depreciation.</t>
         </is>
       </c>
       <c r="H114" s="13" t="inlineStr">
@@ -10759,7 +10759,7 @@
       </c>
       <c r="J114" s="13" t="inlineStr">
         <is>
-          <t>Per capital receipt</t>
+          <t>Per disposal</t>
         </is>
       </c>
       <c r="K114" s="12" t="inlineStr">
@@ -10774,22 +10774,22 @@
       </c>
       <c r="M114" s="12" t="inlineStr">
         <is>
-          <t>assets.service.ts registerFromGr/approveRegistration/rejectRegistration/eligibleFromGr; assets.controller.ts (registrations*); procurement.service.ts createGr (is_capital routing, costing excluded); schema/assets.ts asset_registration_requests + fixed_assets.source_gr_no/po_no + migration 0137; cutover/basics.ts + compliance.ts (ToE)</t>
+          <t>assets.service.ts dispose(pendingApproval Draft)/approveDisposal/rejectDisposal; assets.controller.ts (:assetNo/dispose/approve|reject); schema/assets.ts fixed_assets.disposal_pending + migration 0135; cutover/basics.ts + worldclass.ts + compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N114" s="12" t="inlineStr">
         <is>
-          <t>Inspect the eligible→request→approve flow + approver≠requester check + the inventory-vs-asset routing of capital lines.</t>
+          <t>Inspect Draft→approve flow + the approver≠requester check + deferred status/recycle.</t>
         </is>
       </c>
       <c r="O114" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: receive a capital line, raise a registration (no GL), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm the asset + Dr 1500/Cr 2000 post only after approval and the line cannot be re-registered (re-performed by the harnesses).</t>
+          <t>Re-perform: request a disposal (Draft JE excluded), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm status→disposed + surplus recycled only after approval (re-performed by the harnesses).</t>
         </is>
       </c>
       <c r="P114" s="12" t="inlineStr">
         <is>
-          <t>Capitalization approval log + SoD test</t>
+          <t>Disposal approval log + SoD test</t>
         </is>
       </c>
       <c r="Q114" s="18" t="inlineStr">
@@ -10801,12 +10801,12 @@
     <row r="115">
       <c r="A115" s="15" t="inlineStr">
         <is>
-          <t>CON-01</t>
+          <t>FA-10</t>
         </is>
       </c>
       <c r="B115" s="16" t="inlineStr">
         <is>
-          <t>Consolidation &amp; FX</t>
+          <t>Fixed Assets</t>
         </is>
       </c>
       <c r="C115" s="17" t="inlineStr">
@@ -10816,42 +10816,42 @@
       </c>
       <c r="D115" s="16" t="inlineStr">
         <is>
-          <t>Consolidation</t>
+          <t>Property, Plant &amp; Equipment; Accounts Payable</t>
         </is>
       </c>
       <c r="E115" s="16" t="inlineStr">
         <is>
-          <t>Group consolidation mis-stated (ownership/currency).</t>
+          <t>Capital purchases mis-capitalised or capitalised without independent review — the person who receives the goods also decides what enters the asset register and at what cost/useful life (fictitious or over-valued assets; capex/opex mis-classification).</t>
         </is>
       </c>
       <c r="F115" s="16" t="inlineStr">
         <is>
-          <t>Accuracy</t>
+          <t>Authorization; Accuracy</t>
         </is>
       </c>
       <c r="G115" s="16" t="inlineStr">
         <is>
-          <t>Consolidation run (ownership %, entity currency) gated by 'approvals'.</t>
+          <t>Procure-to-Capitalize maker-checker (SoD): a goods-receipt line flagged capital (item-master is_fixed_asset or per-PO-line override) is excluded from inventory capitalisation (1200) at receipt and instead becomes ELIGIBLE for the asset register. Capitalisation is a REQUEST that posts NOTHING to the GL; a DIFFERENT user must approve before the fixed_assets row + acquisition JE (Dr 1500 / Cr 2000) are created (approver ≠ requester enforced regardless of permissions). The created asset carries its source GR/PO for end-to-end PR→PO→GR→FA traceability; a GR line cannot be capitalised twice.</t>
         </is>
       </c>
       <c r="H115" s="17" t="inlineStr">
         <is>
-          <t>Auto+Manual</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I115" s="17" t="inlineStr">
         <is>
-          <t>Period</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J115" s="17" t="inlineStr">
         <is>
-          <t>Period</t>
+          <t>Per capital receipt</t>
         </is>
       </c>
       <c r="K115" s="16" t="inlineStr">
         <is>
-          <t>Group Controller</t>
+          <t>FaAccountant / Controller</t>
         </is>
       </c>
       <c r="L115" s="17" t="inlineStr">
@@ -10861,22 +10861,22 @@
       </c>
       <c r="M115" s="16" t="inlineStr">
         <is>
-          <t>consolidation.service.ts (runConsolidation @Permissions approvals)</t>
+          <t>assets.service.ts registerFromGr/approveRegistration/rejectRegistration/eligibleFromGr; assets.controller.ts (registrations*); procurement.service.ts createGr (is_capital routing, costing excluded); schema/assets.ts asset_registration_requests + fixed_assets.source_gr_no/po_no + migration 0137; cutover/basics.ts + compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N115" s="16" t="inlineStr">
         <is>
-          <t>Inspect consolidation logic + gate.</t>
+          <t>Inspect the eligible→request→approve flow + approver≠requester check + the inventory-vs-asset routing of capital lines.</t>
         </is>
       </c>
       <c r="O115" s="16" t="inlineStr">
         <is>
-          <t>Sample period: consolidated TB ties to entities.</t>
+          <t>Re-perform: receive a capital line, raise a registration (no GL), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm the asset + Dr 1500/Cr 2000 post only after approval and the line cannot be re-registered (re-performed by the harnesses).</t>
         </is>
       </c>
       <c r="P115" s="16" t="inlineStr">
         <is>
-          <t>Consol TB</t>
+          <t>Capitalization approval log + SoD test</t>
         </is>
       </c>
       <c r="Q115" s="18" t="inlineStr">
@@ -10888,7 +10888,7 @@
     <row r="116">
       <c r="A116" s="11" t="inlineStr">
         <is>
-          <t>CON-02</t>
+          <t>CON-01</t>
         </is>
       </c>
       <c r="B116" s="12" t="inlineStr">
@@ -10903,22 +10903,22 @@
       </c>
       <c r="D116" s="12" t="inlineStr">
         <is>
-          <t>FX gain/loss</t>
+          <t>Consolidation</t>
         </is>
       </c>
       <c r="E116" s="12" t="inlineStr">
         <is>
-          <t>FX exposures not revalued at period-end.</t>
+          <t>Group consolidation mis-stated (ownership/currency).</t>
         </is>
       </c>
       <c r="F116" s="12" t="inlineStr">
         <is>
-          <t>Valuation</t>
+          <t>Accuracy</t>
         </is>
       </c>
       <c r="G116" s="12" t="inlineStr">
         <is>
-          <t>FX revaluation at period-end rates; unrealized FX posted (acct 5400).</t>
+          <t>Consolidation run (ownership %, entity currency) gated by 'approvals'.</t>
         </is>
       </c>
       <c r="H116" s="13" t="inlineStr">
@@ -10928,7 +10928,7 @@
       </c>
       <c r="I116" s="13" t="inlineStr">
         <is>
-          <t>Period-end</t>
+          <t>Period</t>
         </is>
       </c>
       <c r="J116" s="13" t="inlineStr">
@@ -10938,7 +10938,7 @@
       </c>
       <c r="K116" s="12" t="inlineStr">
         <is>
-          <t>Controller</t>
+          <t>Group Controller</t>
         </is>
       </c>
       <c r="L116" s="13" t="inlineStr">
@@ -10948,22 +10948,22 @@
       </c>
       <c r="M116" s="12" t="inlineStr">
         <is>
-          <t>fx.service.ts (revalue / unrealized report)</t>
+          <t>consolidation.service.ts (runConsolidation @Permissions approvals)</t>
         </is>
       </c>
       <c r="N116" s="12" t="inlineStr">
         <is>
-          <t>Inspect reval logic + rates.</t>
+          <t>Inspect consolidation logic + gate.</t>
         </is>
       </c>
       <c r="O116" s="12" t="inlineStr">
         <is>
-          <t>Recompute reval on sample balances.</t>
+          <t>Sample period: consolidated TB ties to entities.</t>
         </is>
       </c>
       <c r="P116" s="12" t="inlineStr">
         <is>
-          <t>FX reval JE</t>
+          <t>Consol TB</t>
         </is>
       </c>
       <c r="Q116" s="18" t="inlineStr">
@@ -10975,7 +10975,7 @@
     <row r="117">
       <c r="A117" s="15" t="inlineStr">
         <is>
-          <t>FX-04</t>
+          <t>CON-02</t>
         </is>
       </c>
       <c r="B117" s="16" t="inlineStr">
@@ -10990,42 +10990,42 @@
       </c>
       <c r="D117" s="16" t="inlineStr">
         <is>
-          <t>FX gain/loss; Revenue; AR/AP</t>
+          <t>FX gain/loss</t>
         </is>
       </c>
       <c r="E117" s="16" t="inlineStr">
         <is>
-          <t>A wrong manually-entered FX rate (fat-fingered, e.g. USD 36 keyed as 63) flows straight into a period-end revaluation JE and the unrealized-FX report with no independent review — mis-stating earnings/equity and FX-translated balances.</t>
+          <t>FX exposures not revalued at period-end.</t>
         </is>
       </c>
       <c r="F117" s="16" t="inlineStr">
         <is>
-          <t>Accuracy/Valuation</t>
+          <t>Valuation</t>
         </is>
       </c>
       <c r="G117" s="16" t="inlineStr">
         <is>
-          <t>FX rate maker-checker (SoD): a MANUALLY-entered rate lands as PendingApproval and is EXCLUDED from rate resolution — revaluation, the unrealized-FX report, and consolidation translation all use APPROVED rates only — until a DIFFERENT user approves it (POST /api/fx/rates/approve). Self-approval → SOD_VIOLATION (binds even Admin); reject marks the rate Rejected (never usable); re-entering a rate sends it back to PendingApproval. Externally-sourced (feed) rates carrying an explicit non-manual source are auto-approved. Pending rates are also surfaced, aged, by the pending-approvals monitor (GOV-01).</t>
+          <t>FX revaluation at period-end rates; unrealized FX posted (acct 5400).</t>
         </is>
       </c>
       <c r="H117" s="17" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="I117" s="17" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Period-end</t>
         </is>
       </c>
       <c r="J117" s="17" t="inlineStr">
         <is>
-          <t>Per rate</t>
+          <t>Period</t>
         </is>
       </c>
       <c r="K117" s="16" t="inlineStr">
         <is>
-          <t>Controller / Treasury</t>
+          <t>Controller</t>
         </is>
       </c>
       <c r="L117" s="17" t="inlineStr">
@@ -11035,22 +11035,22 @@
       </c>
       <c r="M117" s="16" t="inlineStr">
         <is>
-          <t>fx.service.ts setRate(manual→PendingApproval)/approveRate/rejectRate/rateAsOf(Approved only); fx.controller.ts (rates/approve|reject|pending gated approvals/gl_close); consolidation.service.ts (translation reads Approved rates); schema/fx.ts fx_rates.status + migration 0141; cutover/fxreval.ts (ToE)</t>
+          <t>fx.service.ts (revalue / unrealized report)</t>
         </is>
       </c>
       <c r="N117" s="16" t="inlineStr">
         <is>
-          <t>Inspect the request→approve flow + the approver≠requester check + that revaluation/reporting resolve Approved rates only.</t>
+          <t>Inspect reval logic + rates.</t>
         </is>
       </c>
       <c r="O117" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: enter a manual rate (PendingApproval), confirm revalue is blocked NO_RATE while pending, attempt self-approve (SOD_VIOLATION), approve as a different user, then revalue succeeds (re-performed by the fxreval harness).</t>
+          <t>Recompute reval on sample balances.</t>
         </is>
       </c>
       <c r="P117" s="16" t="inlineStr">
         <is>
-          <t>FX rate approval log + SoD test</t>
+          <t>FX reval JE</t>
         </is>
       </c>
       <c r="Q117" s="18" t="inlineStr">
@@ -11062,92 +11062,179 @@
     <row r="118">
       <c r="A118" s="11" t="inlineStr">
         <is>
+          <t>FX-04</t>
+        </is>
+      </c>
+      <c r="B118" s="12" t="inlineStr">
+        <is>
+          <t>Consolidation &amp; FX</t>
+        </is>
+      </c>
+      <c r="C118" s="13" t="inlineStr">
+        <is>
+          <t>Application</t>
+        </is>
+      </c>
+      <c r="D118" s="12" t="inlineStr">
+        <is>
+          <t>FX gain/loss; Revenue; AR/AP</t>
+        </is>
+      </c>
+      <c r="E118" s="12" t="inlineStr">
+        <is>
+          <t>A wrong manually-entered FX rate (fat-fingered, e.g. USD 36 keyed as 63) flows straight into a period-end revaluation JE and the unrealized-FX report with no independent review — mis-stating earnings/equity and FX-translated balances.</t>
+        </is>
+      </c>
+      <c r="F118" s="12" t="inlineStr">
+        <is>
+          <t>Accuracy/Valuation</t>
+        </is>
+      </c>
+      <c r="G118" s="12" t="inlineStr">
+        <is>
+          <t>FX rate maker-checker (SoD): a MANUALLY-entered rate lands as PendingApproval and is EXCLUDED from rate resolution — revaluation, the unrealized-FX report, and consolidation translation all use APPROVED rates only — until a DIFFERENT user approves it (POST /api/fx/rates/approve). Self-approval → SOD_VIOLATION (binds even Admin); reject marks the rate Rejected (never usable); re-entering a rate sends it back to PendingApproval. Externally-sourced (feed) rates carrying an explicit non-manual source are auto-approved. Pending rates are also surfaced, aged, by the pending-approvals monitor (GOV-01).</t>
+        </is>
+      </c>
+      <c r="H118" s="13" t="inlineStr">
+        <is>
+          <t>Prev</t>
+        </is>
+      </c>
+      <c r="I118" s="13" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="J118" s="13" t="inlineStr">
+        <is>
+          <t>Per rate</t>
+        </is>
+      </c>
+      <c r="K118" s="12" t="inlineStr">
+        <is>
+          <t>Controller / Treasury</t>
+        </is>
+      </c>
+      <c r="L118" s="13" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="M118" s="12" t="inlineStr">
+        <is>
+          <t>fx.service.ts setRate(manual→PendingApproval)/approveRate/rejectRate/rateAsOf(Approved only); fx.controller.ts (rates/approve|reject|pending gated approvals/gl_close); consolidation.service.ts (translation reads Approved rates); schema/fx.ts fx_rates.status + migration 0141; cutover/fxreval.ts (ToE)</t>
+        </is>
+      </c>
+      <c r="N118" s="12" t="inlineStr">
+        <is>
+          <t>Inspect the request→approve flow + the approver≠requester check + that revaluation/reporting resolve Approved rates only.</t>
+        </is>
+      </c>
+      <c r="O118" s="12" t="inlineStr">
+        <is>
+          <t>Re-perform: enter a manual rate (PendingApproval), confirm revalue is blocked NO_RATE while pending, attempt self-approve (SOD_VIOLATION), approve as a different user, then revalue succeeds (re-performed by the fxreval harness).</t>
+        </is>
+      </c>
+      <c r="P118" s="12" t="inlineStr">
+        <is>
+          <t>FX rate approval log + SoD test</t>
+        </is>
+      </c>
+      <c r="Q118" s="18" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="15" t="inlineStr">
+        <is>
           <t>BUD-01</t>
         </is>
       </c>
-      <c r="B118" s="12" t="inlineStr">
+      <c r="B119" s="16" t="inlineStr">
         <is>
           <t>Budgeting &amp; Planning</t>
         </is>
       </c>
-      <c r="C118" s="13" t="inlineStr">
+      <c r="C119" s="17" t="inlineStr">
         <is>
           <t>Application</t>
         </is>
       </c>
-      <c r="D118" s="12" t="inlineStr">
+      <c r="D119" s="16" t="inlineStr">
         <is>
           <t>Budget; All (variance reporting)</t>
         </is>
       </c>
-      <c r="E118" s="12" t="inlineStr">
+      <c r="E119" s="16" t="inlineStr">
         <is>
           <t>A budget figure is entered/changed by one person and immediately drives the budget-vs-actual variance report — the basis for spend authorization and performance review — with no independent approval; a wrong or self-serving budget makes overspending look 'on budget'.</t>
         </is>
       </c>
-      <c r="F118" s="12" t="inlineStr">
+      <c r="F119" s="16" t="inlineStr">
         <is>
           <t>Authorization/Accuracy</t>
         </is>
       </c>
-      <c r="G118" s="12" t="inlineStr">
+      <c r="G119" s="16" t="inlineStr">
         <is>
           <t>Budget maker-checker (SoD): an upserted budget (POST /api/ledger/budgets) lands as PendingApproval and is EXCLUDED from budget-vs-actual until a DIFFERENT user approves it (POST /api/ledger/budgets/approve for the fiscal_year/account/cost-centre[/period]). Self-approval → SOD_VIOLATION (binds even Admin); reject marks it Rejected (excluded). DEFAULT 'Approved' keeps existing rows + direct planning seeds usable. Pending budgets are also surfaced, aged, by the pending-approvals monitor (GOV-01).</t>
         </is>
       </c>
-      <c r="H118" s="13" t="inlineStr">
+      <c r="H119" s="17" t="inlineStr">
         <is>
           <t>Prev</t>
         </is>
       </c>
-      <c r="I118" s="13" t="inlineStr">
+      <c r="I119" s="17" t="inlineStr">
         <is>
           <t>Automated</t>
         </is>
       </c>
-      <c r="J118" s="13" t="inlineStr">
+      <c r="J119" s="17" t="inlineStr">
         <is>
           <t>Per budget</t>
         </is>
       </c>
-      <c r="K118" s="12" t="inlineStr">
+      <c r="K119" s="16" t="inlineStr">
         <is>
           <t>Controller / FP&amp;A</t>
         </is>
       </c>
-      <c r="L118" s="13" t="inlineStr">
+      <c r="L119" s="17" t="inlineStr">
         <is>
           <t>P10</t>
         </is>
       </c>
-      <c r="M118" s="12" t="inlineStr">
+      <c r="M119" s="16" t="inlineStr">
         <is>
           <t>budget.service.ts upsertBudget(→PendingApproval)/approveBudget/rejectBudget/budgetVsActual(Approved only); budget.controller.ts (budgets/approve|reject|pending gated approvals/gl_close); schema/budgets.ts budgets.status + migration 0142; cutover/budget.ts (ToE)</t>
         </is>
       </c>
-      <c r="N118" s="12" t="inlineStr">
+      <c r="N119" s="16" t="inlineStr">
         <is>
           <t>Inspect the request→approve flow + the approver≠requester check + that budget-vs-actual counts Approved budgets only.</t>
         </is>
       </c>
-      <c r="O118" s="12" t="inlineStr">
+      <c r="O119" s="16" t="inlineStr">
         <is>
           <t>Re-perform: upsert a budget (PendingApproval, excluded from variance), attempt self-approve (SOD_VIOLATION), approve as a different user, confirm it then appears in budget-vs-actual (re-performed by the budget harness).</t>
         </is>
       </c>
-      <c r="P118" s="12" t="inlineStr">
+      <c r="P119" s="16" t="inlineStr">
         <is>
           <t>Budget approval log + SoD test</t>
         </is>
       </c>
-      <c r="Q118" s="18" t="inlineStr">
+      <c r="Q119" s="18" t="inlineStr">
         <is>
           <t>Implemented</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q118"/>
+  <autoFilter ref="A1:Q119"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -12330,7 +12417,7 @@
         </is>
       </c>
       <c r="C5" s="29">
-        <f>COUNTIF(RCM!$Q$2:$Q$118,B5)</f>
+        <f>COUNTIF(RCM!$Q$2:$Q$119,B5)</f>
         <v/>
       </c>
     </row>
@@ -12341,7 +12428,7 @@
         </is>
       </c>
       <c r="C6" s="29">
-        <f>COUNTIF(RCM!$Q$2:$Q$118,B6)</f>
+        <f>COUNTIF(RCM!$Q$2:$Q$119,B6)</f>
         <v/>
       </c>
     </row>
@@ -12352,7 +12439,7 @@
         </is>
       </c>
       <c r="C7" s="29">
-        <f>COUNTIF(RCM!$Q$2:$Q$118,B7)</f>
+        <f>COUNTIF(RCM!$Q$2:$Q$119,B7)</f>
         <v/>
       </c>
     </row>
@@ -12363,7 +12450,7 @@
         </is>
       </c>
       <c r="C8" s="32">
-        <f>COUNTA(RCM!$A$2:$A$118)</f>
+        <f>COUNTA(RCM!$A$2:$A$119)</f>
         <v/>
       </c>
     </row>
@@ -12381,7 +12468,7 @@
         </is>
       </c>
       <c r="C11" s="29">
-        <f>COUNTIF(RCM!$C$2:$C$118,B11)</f>
+        <f>COUNTIF(RCM!$C$2:$C$119,B11)</f>
         <v/>
       </c>
     </row>
@@ -12392,7 +12479,7 @@
         </is>
       </c>
       <c r="C12" s="29">
-        <f>COUNTIF(RCM!$C$2:$C$118,B12)</f>
+        <f>COUNTIF(RCM!$C$2:$C$119,B12)</f>
         <v/>
       </c>
     </row>
@@ -12403,7 +12490,7 @@
         </is>
       </c>
       <c r="C13" s="29">
-        <f>COUNTIF(RCM!$C$2:$C$118,B13)</f>
+        <f>COUNTIF(RCM!$C$2:$C$119,B13)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(gl): WS1.4 — sub-ledger tie-out + maker-checker certify (GL-14) (#162)
* feat(gl): WS1.4 — sub-ledger tie-out + maker-checker certify (GL-14)

- subledger_tieout_runs table (migration 0160) + RLS
- SubledgerTieoutService.runTieOut: compares GL control-account balance
  vs sub-ledger sum (AR/AP from invoice tables, INV from inv_balances,
  FA from fixed_assets NBV); flags Matched/Variance
- certify(): maker-checker, blocks SELF_CERTIFY
- Controller GET/POST run/certify (perms gl_close, gl_post)
- basics harness: 4 GL-14 checks (164/164 green)
- GL-14 RCM control (Detective/Monthly, SoD certifier≠runner); RCM 118
- process-narrative §1.4 + UAT TC-GL-14-01..03

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>

* chore: merge main, renumber subledger-tieout 0160→0161 (bom_yield took 0160)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>

---------

Co-authored-by: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/compliance/Oshinei_ERP_SOX_RCM_v1.xlsx
+++ b/compliance/Oshinei_ERP_SOX_RCM_v1.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'RCM'!$A$1:$Q$118</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'RCM'!$A$1:$Q$119</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Gap Remediation'!$A$2:$H$18</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -858,7 +858,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q118"/>
+  <dimension ref="A1:Q119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -8974,12 +8974,12 @@
     <row r="94">
       <c r="A94" s="11" t="inlineStr">
         <is>
-          <t>EXP-07</t>
+          <t>GL-14</t>
         </is>
       </c>
       <c r="B94" s="12" t="inlineStr">
         <is>
-          <t>Expenditure</t>
+          <t>General Ledger</t>
         </is>
       </c>
       <c r="C94" s="13" t="inlineStr">
@@ -8989,22 +8989,22 @@
       </c>
       <c r="D94" s="12" t="inlineStr">
         <is>
-          <t>Cash; Operating expense</t>
+          <t>All</t>
         </is>
       </c>
       <c r="E94" s="12" t="inlineStr">
         <is>
-          <t>Petty-cash / employee advance issued but never accounted for — cash leakage, expense unrecorded.</t>
+          <t>GL control-account balances (AR/AP/INV/FA) drift from the underlying sub-ledger detail without detection — the control account no longer represents the sum of its sub-ledger, masking posting errors, unrecorded items, or fraud.</t>
         </is>
       </c>
       <c r="F94" s="12" t="inlineStr">
         <is>
-          <t>Existence/Completeness</t>
+          <t>Completeness/Accuracy/Valuation</t>
         </is>
       </c>
       <c r="G94" s="12" t="inlineStr">
         <is>
-          <t>Employee cash advances: issuing an advance debits the 1180 Employee Advances control (Dr 1180 / Cr 1000); settlement clears it against actual spend + returned cash (Dr expense + Dr 1000 / Cr 1180), enforced to reconcile (settled_expense + returned_cash must equal the advance → SETTLE_MISMATCH). The 1180 balance is the outstanding float subject to review.</t>
+          <t>Sub-ledger tie-out / reconciliation: POST /api/ledger/tie-out/run computes, per control account, the GL balance (Σ debit−credit of posted journal_lines on the control account up to the as-of date, tenant-scoped) and the sub-ledger detail balance (AR = Σ outstanding ar_invoices; AP = Σ outstanding ap_transactions; INV = Σ inv_balances.total_value perpetual valuation; FA = Σ acquire_cost − accumulated_depreciation of non-disposed fixed_assets), records the variance (gl − subledger) and a status (Matched if |variance|&lt;0.01 else Variance). Runs upsert per (tenant, subledger, as-of). Certification is maker-checker: POST /api/ledger/tie-out/:id/certify sets status=Certified and records certifier + timestamp, and REJECTS a certifier equal to the runner (SELF_CERTIFY) — the gl_close certifier must differ from the gl_post/gl_close runner (SoD).</t>
         </is>
       </c>
       <c r="H94" s="13" t="inlineStr">
@@ -9019,12 +9019,12 @@
       </c>
       <c r="J94" s="13" t="inlineStr">
         <is>
-          <t>Per advance</t>
+          <t>Monthly</t>
         </is>
       </c>
       <c r="K94" s="12" t="inlineStr">
         <is>
-          <t>AP / Controller</t>
+          <t>Financial Controller</t>
         </is>
       </c>
       <c r="L94" s="13" t="inlineStr">
@@ -9034,22 +9034,22 @@
       </c>
       <c r="M94" s="12" t="inlineStr">
         <is>
-          <t>finance.service.ts (issueAdvance, settleAdvance reconcile-or-reject, listAdvances outstanding); finance.controller.ts (creditors/exec); schema/finance.ts (employee_advances) + migration 0120; cutover/basics.ts (ToE)</t>
+          <t>subledger-tieout.service.ts (runTieOut GL/sub-ledger balance computation + variance/status, certify SELF_CERTIFY maker-checker, list/get); subledger-tieout.controller.ts (gl_close/gl_post run, gl_close certify, gl_close/gl_post/exec/creditors/ar read); schema/subledger-tieout.ts (subledger_tieout_runs table, uq on tenant/subledger/as-of); migration 0160 (table + RLS); ledger.module.ts (service+controller wired); cutover/basics.ts (GL-14 ToE)</t>
         </is>
       </c>
       <c r="N94" s="12" t="inlineStr">
         <is>
-          <t>Inspect issue/settle GL + settlement reconciliation guard.</t>
+          <t>Inspect the GL-vs-sub-ledger balance computation + variance/status + SELF_CERTIFY maker-checker gate + gl_close certify permission.</t>
         </is>
       </c>
       <c r="O94" s="12" t="inlineStr">
         <is>
-          <t>Issue an advance (1180 up); settle 700+300 clears 1180; mismatched settle → SETTLE_MISMATCH (re-performed by the harness).</t>
+          <t>TC-GL-14-01: run AR tie-out → balances + Matched/Variance; TC-GL-14-02: self-certify by the runner → SELF_CERTIFY (400); TC-GL-14-03: certify by a different gl_close user → Certified (re-performed by the basics.ts harness).</t>
         </is>
       </c>
       <c r="P94" s="12" t="inlineStr">
         <is>
-          <t>Advance register; outstanding float</t>
+          <t>Tie-out run log (subledger_tieout_runs) with variance + certification trail; monthly reconciliation sign-off</t>
         </is>
       </c>
       <c r="Q94" s="18" t="inlineStr">
@@ -9061,7 +9061,7 @@
     <row r="95">
       <c r="A95" s="15" t="inlineStr">
         <is>
-          <t>EXP-08</t>
+          <t>EXP-07</t>
         </is>
       </c>
       <c r="B95" s="16" t="inlineStr">
@@ -9081,22 +9081,22 @@
       </c>
       <c r="E95" s="16" t="inlineStr">
         <is>
-          <t>Petty-cash disbursed beyond authority / without independent review, or drawn past the fund's limit — cash leakage, unauthorised or unrecorded expense, over-extended float.</t>
+          <t>Petty-cash / employee advance issued but never accounted for — cash leakage, expense unrecorded.</t>
         </is>
       </c>
       <c r="F95" s="16" t="inlineStr">
         <is>
-          <t>Authorization; Completeness</t>
+          <t>Existence/Completeness</t>
         </is>
       </c>
       <c r="G95" s="16" t="inlineStr">
         <is>
-          <t>Petty-cash imprest float + maker-checker on disbursement (SoD): a fund holds cash capped at a credit limit/วงเงิน (1015 Petty Cash, a cash account); each direct EXPENSE or ADVANCE is a REQUEST that posts NOTHING and a DIFFERENT user must approve before the GL posts (expense Dr &lt;expense&gt; / Cr 1015; advance Dr 1180 / Cr 1015) and the fund balance is decremented. Self-approval → SOD_VIOLATION (binds even Admin). A draw beyond the fund balance → INSUFFICIENT_FLOAT; establishing/replenishing above the float limit → OVER_FLOAT. Advances settle (Dr expense + Dr 1015 returned / Cr 1180), returning unused cash to the fund. Every request carries a document reference + receipt key + a status trail (StatusLog) and surfaces in the GOV-01 pending-approvals monitor.</t>
+          <t>Employee cash advances: issuing an advance debits the 1180 Employee Advances control (Dr 1180 / Cr 1000); settlement clears it against actual spend + returned cash (Dr expense + Dr 1000 / Cr 1180), enforced to reconcile (settled_expense + returned_cash must equal the advance → SETTLE_MISMATCH). The 1180 balance is the outstanding float subject to review.</t>
         </is>
       </c>
       <c r="H95" s="17" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I95" s="17" t="inlineStr">
@@ -9106,7 +9106,7 @@
       </c>
       <c r="J95" s="17" t="inlineStr">
         <is>
-          <t>Per disbursement</t>
+          <t>Per advance</t>
         </is>
       </c>
       <c r="K95" s="16" t="inlineStr">
@@ -9121,22 +9121,22 @@
       </c>
       <c r="M95" s="16" t="inlineStr">
         <is>
-          <t>petty-cash.service.ts (establishFund/replenishFund float guards, createRequest INSUFFICIENT_FLOAT, approveRequest SoD+GL, rejectRequest, settleRequest); petty-cash.controller.ts (creditors/exec); schema/petty-cash.ts (petty_cash_funds, expense_requests) + migration 0139; finance.service.ts pendingApprovals (GOV-01 source 7); cutover/basics.ts + compliance.ts (ToE)</t>
+          <t>finance.service.ts (issueAdvance, settleAdvance reconcile-or-reject, listAdvances outstanding); finance.controller.ts (creditors/exec); schema/finance.ts (employee_advances) + migration 0120; cutover/basics.ts (ToE)</t>
         </is>
       </c>
       <c r="N95" s="16" t="inlineStr">
         <is>
-          <t>Inspect the float ceiling + the request→approve flow + the approver≠requester check + that the request posts nothing until approval.</t>
+          <t>Inspect issue/settle GL + settlement reconciliation guard.</t>
         </is>
       </c>
       <c r="O95" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: establish a fund (Dr 1015), request an expense (no GL), self-approve → SOD_VIOLATION, approve as a different user → Dr expense/Cr 1015 + fund down; over-balance draw → INSUFFICIENT_FLOAT; advance approve→settle clears 1180; replenish past float → OVER_FLOAT (re-performed by the harnesses).</t>
+          <t>Issue an advance (1180 up); settle 700+300 clears 1180; mismatched settle → SETTLE_MISMATCH (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P95" s="16" t="inlineStr">
         <is>
-          <t>Fund register + disbursement approval log + SoD test</t>
+          <t>Advance register; outstanding float</t>
         </is>
       </c>
       <c r="Q95" s="18" t="inlineStr">
@@ -9148,12 +9148,12 @@
     <row r="96">
       <c r="A96" s="11" t="inlineStr">
         <is>
-          <t>FA-07</t>
+          <t>EXP-08</t>
         </is>
       </c>
       <c r="B96" s="12" t="inlineStr">
         <is>
-          <t>Fixed Assets</t>
+          <t>Expenditure</t>
         </is>
       </c>
       <c r="C96" s="13" t="inlineStr">
@@ -9163,27 +9163,27 @@
       </c>
       <c r="D96" s="12" t="inlineStr">
         <is>
-          <t>Property, Plant &amp; Equipment; Equity</t>
+          <t>Cash; Operating expense</t>
         </is>
       </c>
       <c r="E96" s="12" t="inlineStr">
         <is>
-          <t>Carrying amount not adjusted for revaluation/impairment — asset over/understated.</t>
+          <t>Petty-cash disbursed beyond authority / without independent review, or drawn past the fund's limit — cash leakage, unauthorised or unrecorded expense, over-extended float.</t>
         </is>
       </c>
       <c r="F96" s="12" t="inlineStr">
         <is>
-          <t>Valuation</t>
+          <t>Authorization; Completeness</t>
         </is>
       </c>
       <c r="G96" s="12" t="inlineStr">
         <is>
-          <t>Asset revaluation / impairment: an upward revaluation credits the revaluation surplus in equity (Dr 1500 / Cr 3200); a downward revaluation (impairment) debits impairment loss (Dr 5820 / Cr 1500). The gross 1500 moves by the delta so the register stays tied to the GL; a no-op revaluation is rejected (NO_CHANGE). Every event is logged for the audit trail.</t>
+          <t>Petty-cash imprest float + maker-checker on disbursement (SoD): a fund holds cash capped at a credit limit/วงเงิน (1015 Petty Cash, a cash account); each direct EXPENSE or ADVANCE is a REQUEST that posts NOTHING and a DIFFERENT user must approve before the GL posts (expense Dr &lt;expense&gt; / Cr 1015; advance Dr 1180 / Cr 1015) and the fund balance is decremented. Self-approval → SOD_VIOLATION (binds even Admin). A draw beyond the fund balance → INSUFFICIENT_FLOAT; establishing/replenishing above the float limit → OVER_FLOAT. Advances settle (Dr expense + Dr 1015 returned / Cr 1180), returning unused cash to the fund. Every request carries a document reference + receipt key + a status trail (StatusLog) and surfaces in the GOV-01 pending-approvals monitor.</t>
         </is>
       </c>
       <c r="H96" s="13" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I96" s="13" t="inlineStr">
@@ -9193,12 +9193,12 @@
       </c>
       <c r="J96" s="13" t="inlineStr">
         <is>
-          <t>Per event</t>
+          <t>Per disbursement</t>
         </is>
       </c>
       <c r="K96" s="12" t="inlineStr">
         <is>
-          <t>FaAccountant / Controller</t>
+          <t>AP / Controller</t>
         </is>
       </c>
       <c r="L96" s="13" t="inlineStr">
@@ -9208,22 +9208,22 @@
       </c>
       <c r="M96" s="12" t="inlineStr">
         <is>
-          <t>assets.service.ts (revalue up→3200 / down→5820, listRevaluations; dispose recycles surplus 3200→3100); assets.controller.ts (exec/creditors); schema/assets.ts (asset_revaluations) + migration 0120; cutover/basics.ts (ToE)</t>
+          <t>petty-cash.service.ts (establishFund/replenishFund float guards, createRequest INSUFFICIENT_FLOAT, approveRequest SoD+GL, rejectRequest, settleRequest); petty-cash.controller.ts (creditors/exec); schema/petty-cash.ts (petty_cash_funds, expense_requests) + migration 0139; finance.service.ts pendingApprovals (GOV-01 source 7); cutover/basics.ts + compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N96" s="12" t="inlineStr">
         <is>
-          <t>Inspect revaluation/impairment routing + audit log + disposal recycling.</t>
+          <t>Inspect the float ceiling + the request→approve flow + the approver≠requester check + that the request posts nothing until approval.</t>
         </is>
       </c>
       <c r="O96" s="12" t="inlineStr">
         <is>
-          <t>Upward revaluation credits 3200; impairment debits 5820; no-change → NO_CHANGE; both events logged; on disposal the revaluation surplus is recycled to retained earnings (Dr 3200 / Cr 3100), not through P&amp;L (re-performed by the harness).</t>
+          <t>Re-perform: establish a fund (Dr 1015), request an expense (no GL), self-approve → SOD_VIOLATION, approve as a different user → Dr expense/Cr 1015 + fund down; over-balance draw → INSUFFICIENT_FLOAT; advance approve→settle clears 1180; replenish past float → OVER_FLOAT (re-performed by the harnesses).</t>
         </is>
       </c>
       <c r="P96" s="12" t="inlineStr">
         <is>
-          <t>Revaluation log; disposal recycling JE</t>
+          <t>Fund register + disbursement approval log + SoD test</t>
         </is>
       </c>
       <c r="Q96" s="18" t="inlineStr">
@@ -9235,7 +9235,7 @@
     <row r="97">
       <c r="A97" s="15" t="inlineStr">
         <is>
-          <t>FA-08</t>
+          <t>FA-07</t>
         </is>
       </c>
       <c r="B97" s="16" t="inlineStr">
@@ -9255,22 +9255,22 @@
       </c>
       <c r="E97" s="16" t="inlineStr">
         <is>
-          <t>Carrying amount changed by fair-value revaluation/impairment without independent review — the preparer revalues the asset and posts to equity/P&amp;L on their own (earnings/equity management).</t>
+          <t>Carrying amount not adjusted for revaluation/impairment — asset over/understated.</t>
         </is>
       </c>
       <c r="F97" s="16" t="inlineStr">
         <is>
-          <t>Authorization</t>
+          <t>Valuation</t>
         </is>
       </c>
       <c r="G97" s="16" t="inlineStr">
         <is>
-          <t>Asset-revaluation maker-checker (SoD): a revalue/impairment request posts its GL entry as a DRAFT (excluded from balances) and records status 'PendingApproval' WITHOUT moving the carrying value; a DIFFERENT user must approve before the JE is effective and the register is re-valued (approver ≠ preparer enforced regardless of permissions, reusing the GL-05 ledger approval). Reject voids the draft; only one revaluation may be pending per asset; the disposal surplus recycle counts only approved revaluations.</t>
+          <t>Asset revaluation / impairment: an upward revaluation credits the revaluation surplus in equity (Dr 1500 / Cr 3200); a downward revaluation (impairment) debits impairment loss (Dr 5820 / Cr 1500). The gross 1500 moves by the delta so the register stays tied to the GL; a no-op revaluation is rejected (NO_CHANGE). Every event is logged for the audit trail.</t>
         </is>
       </c>
       <c r="H97" s="17" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I97" s="17" t="inlineStr">
@@ -9295,22 +9295,22 @@
       </c>
       <c r="M97" s="16" t="inlineStr">
         <is>
-          <t>assets.service.ts revalue(pendingApproval Draft)/approveRevaluation/rejectRevaluation; assets.controller.ts (:assetNo/revalue/approve|reject); schema/assets.ts asset_revaluations.status + migration 0134; cutover/basics.ts + compliance.ts (ToE)</t>
+          <t>assets.service.ts (revalue up→3200 / down→5820, listRevaluations; dispose recycles surplus 3200→3100); assets.controller.ts (exec/creditors); schema/assets.ts (asset_revaluations) + migration 0120; cutover/basics.ts (ToE)</t>
         </is>
       </c>
       <c r="N97" s="16" t="inlineStr">
         <is>
-          <t>Inspect Draft→approve flow + the approver≠preparer check + deferred carrying-value update.</t>
+          <t>Inspect revaluation/impairment routing + audit log + disposal recycling.</t>
         </is>
       </c>
       <c r="O97" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: request a revaluation (Draft JE excluded from 3200), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm the surplus/impairment + carrying value move only after approval (re-performed by the harnesses).</t>
+          <t>Upward revaluation credits 3200; impairment debits 5820; no-change → NO_CHANGE; both events logged; on disposal the revaluation surplus is recycled to retained earnings (Dr 3200 / Cr 3100), not through P&amp;L (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P97" s="16" t="inlineStr">
         <is>
-          <t>Revaluation approval log + SoD test</t>
+          <t>Revaluation log; disposal recycling JE</t>
         </is>
       </c>
       <c r="Q97" s="18" t="inlineStr">
@@ -9322,12 +9322,12 @@
     <row r="98">
       <c r="A98" s="11" t="inlineStr">
         <is>
-          <t>LSE-01</t>
+          <t>FA-08</t>
         </is>
       </c>
       <c r="B98" s="12" t="inlineStr">
         <is>
-          <t>Leases</t>
+          <t>Fixed Assets</t>
         </is>
       </c>
       <c r="C98" s="13" t="inlineStr">
@@ -9337,27 +9337,27 @@
       </c>
       <c r="D98" s="12" t="inlineStr">
         <is>
-          <t>Right-of-use assets; Lease liabilities</t>
+          <t>Property, Plant &amp; Equipment; Equity</t>
         </is>
       </c>
       <c r="E98" s="12" t="inlineStr">
         <is>
-          <t>Lease not capitalised (IFRS 16 / TFRS 16) — ROU asset + lease liability omitted; interest/depreciation mis-stated.</t>
+          <t>Carrying amount changed by fair-value revaluation/impairment without independent review — the preparer revalues the asset and posts to equity/P&amp;L on their own (earnings/equity management).</t>
         </is>
       </c>
       <c r="F98" s="12" t="inlineStr">
         <is>
-          <t>Completeness/Accuracy/Valuation</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="G98" s="12" t="inlineStr">
         <is>
-          <t>Lease accounting: at commencement a right-of-use asset and lease liability are recognised at the present value of the lease payments (Dr 1600 / Cr 2600). The scheduled job lease_periodic_run posts each period — interest unwinding on the liability (Dr 5900), the cash payment reducing the liability (Dr 2600 / Cr 1000), and straight-line ROU depreciation (Dr 5210 / Cr 1690) — the last period clearing the liability + ROU exactly. Idempotent per (lease, period).</t>
+          <t>Asset-revaluation maker-checker (SoD): a revalue/impairment request posts its GL entry as a DRAFT (excluded from balances) and records status 'PendingApproval' WITHOUT moving the carrying value; a DIFFERENT user must approve before the JE is effective and the register is re-valued (approver ≠ preparer enforced regardless of permissions, reusing the GL-05 ledger approval). Reject voids the draft; only one revaluation may be pending per asset; the disposal surplus recycle counts only approved revaluations.</t>
         </is>
       </c>
       <c r="H98" s="13" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I98" s="13" t="inlineStr">
@@ -9367,12 +9367,12 @@
       </c>
       <c r="J98" s="13" t="inlineStr">
         <is>
-          <t>Per period / per lease</t>
+          <t>Per event</t>
         </is>
       </c>
       <c r="K98" s="12" t="inlineStr">
         <is>
-          <t>Controller</t>
+          <t>FaAccountant / Controller</t>
         </is>
       </c>
       <c r="L98" s="13" t="inlineStr">
@@ -9382,22 +9382,22 @@
       </c>
       <c r="M98" s="12" t="inlineStr">
         <is>
-          <t>leases.service.ts (createLease PV recognition, runDueLeases interest+payment+depreciation, modifyLease remeasurement); leases.controller.ts (gl_post); bi.service.ts (lease_periodic_run); schema/leases.ts (leases, rou_nbv) + migration 0120/0121; cutover/basics.ts (ToE)</t>
+          <t>assets.service.ts revalue(pendingApproval Draft)/approveRevaluation/rejectRevaluation; assets.controller.ts (:assetNo/revalue/approve|reject); schema/assets.ts asset_revaluations.status + migration 0134; cutover/basics.ts + compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N98" s="12" t="inlineStr">
         <is>
-          <t>Inspect PV recognition + periodic interest/payment/depreciation + final-period clearing + modification remeasurement.</t>
+          <t>Inspect Draft→approve flow + the approver≠preparer check + deferred carrying-value update.</t>
         </is>
       </c>
       <c r="O98" s="12" t="inlineStr">
         <is>
-          <t>Commencement recognises ROU=liability=PV; periodic run posts interest+principal(=payment)+ROU depreciation; liability + ROU reduce; a modification remeasures the liability at the revised PV and adjusts the ROU by the same delta (Dr/Cr 1600↔2600), then depreciates over the remaining term (re-performed by the harness).</t>
+          <t>Re-perform: request a revaluation (Draft JE excluded from 3200), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm the surplus/impairment + carrying value move only after approval (re-performed by the harnesses).</t>
         </is>
       </c>
       <c r="P98" s="12" t="inlineStr">
         <is>
-          <t>Lease register; periodic run log; modification remeasurement</t>
+          <t>Revaluation approval log + SoD test</t>
         </is>
       </c>
       <c r="Q98" s="18" t="inlineStr">
@@ -9409,12 +9409,12 @@
     <row r="99">
       <c r="A99" s="15" t="inlineStr">
         <is>
-          <t>REC-01</t>
+          <t>LSE-01</t>
         </is>
       </c>
       <c r="B99" s="16" t="inlineStr">
         <is>
-          <t>Reconciliation</t>
+          <t>Leases</t>
         </is>
       </c>
       <c r="C99" s="17" t="inlineStr">
@@ -9424,22 +9424,22 @@
       </c>
       <c r="D99" s="16" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Right-of-use assets; Lease liabilities</t>
         </is>
       </c>
       <c r="E99" s="16" t="inlineStr">
         <is>
-          <t>Subledgers diverge from GL undetected.</t>
+          <t>Lease not capitalised (IFRS 16 / TFRS 16) — ROU asset + lease liability omitted; interest/depreciation mis-stated.</t>
         </is>
       </c>
       <c r="F99" s="16" t="inlineStr">
         <is>
-          <t>Completeness/Accuracy</t>
+          <t>Completeness/Accuracy/Valuation</t>
         </is>
       </c>
       <c r="G99" s="16" t="inlineStr">
         <is>
-          <t>Subledger-to-GL reconciliation per period: import GL, auto-match, certify (sign-off via 'approvals').</t>
+          <t>Lease accounting: at commencement a right-of-use asset and lease liability are recognised at the present value of the lease payments (Dr 1600 / Cr 2600). The scheduled job lease_periodic_run posts each period — interest unwinding on the liability (Dr 5900), the cash payment reducing the liability (Dr 2600 / Cr 1000), and straight-line ROU depreciation (Dr 5210 / Cr 1690) — the last period clearing the liability + ROU exactly. Idempotent per (lease, period).</t>
         </is>
       </c>
       <c r="H99" s="17" t="inlineStr">
@@ -9449,12 +9449,12 @@
       </c>
       <c r="I99" s="17" t="inlineStr">
         <is>
-          <t>Auto+Manual</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J99" s="17" t="inlineStr">
         <is>
-          <t>Monthly</t>
+          <t>Per period / per lease</t>
         </is>
       </c>
       <c r="K99" s="16" t="inlineStr">
@@ -9464,27 +9464,27 @@
       </c>
       <c r="L99" s="17" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="M99" s="16" t="inlineStr">
         <is>
-          <t>reconciliation.service.ts (importGlItems/autoMatch/certify)</t>
+          <t>leases.service.ts (createLease PV recognition, runDueLeases interest+payment+depreciation, modifyLease remeasurement); leases.controller.ts (gl_post); bi.service.ts (lease_periodic_run); schema/leases.ts (leases, rou_nbv) + migration 0120/0121; cutover/basics.ts (ToE)</t>
         </is>
       </c>
       <c r="N99" s="16" t="inlineStr">
         <is>
-          <t>Inspect recon + certify gate.</t>
+          <t>Inspect PV recognition + periodic interest/payment/depreciation + final-period clearing + modification remeasurement.</t>
         </is>
       </c>
       <c r="O99" s="16" t="inlineStr">
         <is>
-          <t>Sample periods: reconciled, unmatched cleared, certified.</t>
+          <t>Commencement recognises ROU=liability=PV; periodic run posts interest+principal(=payment)+ROU depreciation; liability + ROU reduce; a modification remeasures the liability at the revised PV and adjusts the ROU by the same delta (Dr/Cr 1600↔2600), then depreciates over the remaining term (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P99" s="16" t="inlineStr">
         <is>
-          <t>Certified recon</t>
+          <t>Lease register; periodic run log; modification remeasurement</t>
         </is>
       </c>
       <c r="Q99" s="18" t="inlineStr">
@@ -9496,7 +9496,7 @@
     <row r="100">
       <c r="A100" s="11" t="inlineStr">
         <is>
-          <t>REC-02</t>
+          <t>REC-01</t>
         </is>
       </c>
       <c r="B100" s="12" t="inlineStr">
@@ -9511,22 +9511,22 @@
       </c>
       <c r="D100" s="12" t="inlineStr">
         <is>
-          <t>Cash</t>
+          <t>All</t>
         </is>
       </c>
       <c r="E100" s="12" t="inlineStr">
         <is>
-          <t>Bank balance not reconciled to GL.</t>
+          <t>Subledgers diverge from GL undetected.</t>
         </is>
       </c>
       <c r="F100" s="12" t="inlineStr">
         <is>
-          <t>Existence/Completeness</t>
+          <t>Completeness/Accuracy</t>
         </is>
       </c>
       <c r="G100" s="12" t="inlineStr">
         <is>
-          <t>Bank reconciliation against statements.</t>
+          <t>Subledger-to-GL reconciliation per period: import GL, auto-match, certify (sign-off via 'approvals').</t>
         </is>
       </c>
       <c r="H100" s="13" t="inlineStr">
@@ -9556,22 +9556,22 @@
       </c>
       <c r="M100" s="12" t="inlineStr">
         <is>
-          <t>bank module; drizzle/0015_bank_reconciliation</t>
+          <t>reconciliation.service.ts (importGlItems/autoMatch/certify)</t>
         </is>
       </c>
       <c r="N100" s="12" t="inlineStr">
         <is>
-          <t>Inspect bank-rec process.</t>
+          <t>Inspect recon + certify gate.</t>
         </is>
       </c>
       <c r="O100" s="12" t="inlineStr">
         <is>
-          <t>Sample months reconciled &amp; reviewed.</t>
+          <t>Sample periods: reconciled, unmatched cleared, certified.</t>
         </is>
       </c>
       <c r="P100" s="12" t="inlineStr">
         <is>
-          <t>Bank rec</t>
+          <t>Certified recon</t>
         </is>
       </c>
       <c r="Q100" s="18" t="inlineStr">
@@ -9583,12 +9583,12 @@
     <row r="101">
       <c r="A101" s="15" t="inlineStr">
         <is>
-          <t>BANK-02</t>
+          <t>REC-02</t>
         </is>
       </c>
       <c r="B101" s="16" t="inlineStr">
         <is>
-          <t>Cash &amp; Treasury</t>
+          <t>Reconciliation</t>
         </is>
       </c>
       <c r="C101" s="17" t="inlineStr">
@@ -9598,37 +9598,37 @@
       </c>
       <c r="D101" s="16" t="inlineStr">
         <is>
-          <t>Cash; Operating expense; Interest income</t>
+          <t>Cash</t>
         </is>
       </c>
       <c r="E101" s="16" t="inlineStr">
         <is>
-          <t>A bank fee/interest adjustment is posted straight to the GL by one person during reconciliation — a cash outflow mis-booked as interest income, or a fictitious fee posted, with no independent review (single-person posting to the cash account).</t>
+          <t>Bank balance not reconciled to GL.</t>
         </is>
       </c>
       <c r="F101" s="16" t="inlineStr">
         <is>
-          <t>Authorization/Accuracy</t>
+          <t>Existence/Completeness</t>
         </is>
       </c>
       <c r="G101" s="16" t="inlineStr">
         <is>
-          <t>Bank adjustment maker-checker (SoD): a fee/interest adjustment on a statement line is a REQUEST that posts a DRAFT JE (no balance/GL effect; the line stays unreconciled) until a DIFFERENT user with approval authority approves (POST /api/bank/lines/:id/adjustment/approve). Self-approval → SOD_VIOLATION (binds even Admin); approval flips the line to reconciled and the JE to Posted; reject voids the Draft and frees the line. The Draft JE (source BANKADJ) is also surfaced, aged, by the pending-approvals monitor (GOV-01).</t>
+          <t>Bank reconciliation against statements.</t>
         </is>
       </c>
       <c r="H101" s="17" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I101" s="17" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="J101" s="17" t="inlineStr">
         <is>
-          <t>Per adjustment</t>
+          <t>Monthly</t>
         </is>
       </c>
       <c r="K101" s="16" t="inlineStr">
@@ -9638,27 +9638,27 @@
       </c>
       <c r="L101" s="17" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="M101" s="16" t="inlineStr">
         <is>
-          <t>bank.service.ts requestAdjustment/approveAdjustment/rejectAdjustment/listPendingAdjustments (reuses ledger.approveEntry SoD); bank.controller.ts (lines/:id/adjustment requests; adjustment/approve|reject gated approvals/gl_close); cutover/bankrec.ts (ToE)</t>
+          <t>bank module; drizzle/0015_bank_reconciliation</t>
         </is>
       </c>
       <c r="N101" s="16" t="inlineStr">
         <is>
-          <t>Inspect the request→approve flow + the approver≠requester check + that the Draft posts nothing until approval.</t>
+          <t>Inspect bank-rec process.</t>
         </is>
       </c>
       <c r="O101" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: request a fee adjustment (line unreconciled, GL difference unchanged), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm the difference closes to 0 only after approval (re-performed by the bankrec harness).</t>
+          <t>Sample months reconciled &amp; reviewed.</t>
         </is>
       </c>
       <c r="P101" s="16" t="inlineStr">
         <is>
-          <t>Bank adjustment queue + SoD test</t>
+          <t>Bank rec</t>
         </is>
       </c>
       <c r="Q101" s="18" t="inlineStr">
@@ -9670,12 +9670,12 @@
     <row r="102">
       <c r="A102" s="11" t="inlineStr">
         <is>
-          <t>REC-03</t>
+          <t>BANK-02</t>
         </is>
       </c>
       <c r="B102" s="12" t="inlineStr">
         <is>
-          <t>Reconciliation</t>
+          <t>Cash &amp; Treasury</t>
         </is>
       </c>
       <c r="C102" s="13" t="inlineStr">
@@ -9685,79 +9685,79 @@
       </c>
       <c r="D102" s="12" t="inlineStr">
         <is>
-          <t>Consolidation</t>
+          <t>Cash; Operating expense; Interest income</t>
         </is>
       </c>
       <c r="E102" s="12" t="inlineStr">
         <is>
-          <t>Intercompany balances not eliminated/agreed.</t>
+          <t>A bank fee/interest adjustment is posted straight to the GL by one person during reconciliation — a cash outflow mis-booked as interest income, or a fictitious fee posted, with no independent review (single-person posting to the cash account).</t>
         </is>
       </c>
       <c r="F102" s="12" t="inlineStr">
         <is>
-          <t>Accuracy</t>
+          <t>Authorization/Accuracy</t>
         </is>
       </c>
       <c r="G102" s="12" t="inlineStr">
         <is>
-          <t>Intercompany reconciliation &amp; elimination on consolidation.</t>
+          <t>Bank adjustment maker-checker (SoD): a fee/interest adjustment on a statement line is a REQUEST that posts a DRAFT JE (no balance/GL effect; the line stays unreconciled) until a DIFFERENT user with approval authority approves (POST /api/bank/lines/:id/adjustment/approve). Self-approval → SOD_VIOLATION (binds even Admin); approval flips the line to reconciled and the JE to Posted; reject voids the Draft and frees the line. The Draft JE (source BANKADJ) is also surfaced, aged, by the pending-approvals monitor (GOV-01).</t>
         </is>
       </c>
       <c r="H102" s="13" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I102" s="13" t="inlineStr">
         <is>
-          <t>Auto+Manual</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J102" s="13" t="inlineStr">
         <is>
-          <t>Period</t>
+          <t>Per adjustment</t>
         </is>
       </c>
       <c r="K102" s="12" t="inlineStr">
         <is>
-          <t>Group Controller</t>
+          <t>Controller</t>
         </is>
       </c>
       <c r="L102" s="13" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="M102" s="12" t="inlineStr">
         <is>
-          <t>intercompany; consolidation</t>
+          <t>bank.service.ts requestAdjustment/approveAdjustment/rejectAdjustment/listPendingAdjustments (reuses ledger.approveEntry SoD); bank.controller.ts (lines/:id/adjustment requests; adjustment/approve|reject gated approvals/gl_close); cutover/bankrec.ts (ToE)</t>
         </is>
       </c>
       <c r="N102" s="12" t="inlineStr">
         <is>
-          <t>Inspect IC matching + elimination.</t>
+          <t>Inspect the request→approve flow + the approver≠requester check + that the Draft posts nothing until approval.</t>
         </is>
       </c>
       <c r="O102" s="12" t="inlineStr">
         <is>
-          <t>Sample IC pairs agree &amp; eliminate.</t>
+          <t>Re-perform: request a fee adjustment (line unreconciled, GL difference unchanged), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm the difference closes to 0 only after approval (re-performed by the bankrec harness).</t>
         </is>
       </c>
       <c r="P102" s="12" t="inlineStr">
         <is>
-          <t>IC recon</t>
-        </is>
-      </c>
-      <c r="Q102" s="19" t="inlineStr">
-        <is>
-          <t>Partial</t>
+          <t>Bank adjustment queue + SoD test</t>
+        </is>
+      </c>
+      <c r="Q102" s="18" t="inlineStr">
+        <is>
+          <t>Implemented</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="15" t="inlineStr">
         <is>
-          <t>REC-04</t>
+          <t>REC-03</t>
         </is>
       </c>
       <c r="B103" s="16" t="inlineStr">
@@ -9772,22 +9772,22 @@
       </c>
       <c r="D103" s="16" t="inlineStr">
         <is>
-          <t>All control accounts</t>
+          <t>Consolidation</t>
         </is>
       </c>
       <c r="E103" s="16" t="inlineStr">
         <is>
-          <t>A sub-ledger silently drifts from its GL control account at period-end and no single review catches it (incomplete/inaccurate balances reach the financial statements).</t>
+          <t>Intercompany balances not eliminated/agreed.</t>
         </is>
       </c>
       <c r="F103" s="16" t="inlineStr">
         <is>
-          <t>Completeness/Accuracy</t>
+          <t>Accuracy</t>
         </is>
       </c>
       <c r="G103" s="16" t="inlineStr">
         <is>
-          <t>Period-end control-account reconciliation PACK: one read (GET /api/finance/reconciliation/controls) ties every major sub-ledger to its GL control account and FLAGS any out-of-balance — AR↔1100, AP↔2000, Inventory↔1200, Gift cards/Customer-deposits↔2200, Deferred revenue↔2400 — reporting per line {sub_ledger, gl_control, variance, reconciled} plus an overall all_reconciled flag and an exceptions count. Liability controls are sign-flipped before comparison. The controller's single 'are the books reconciled?' close view; an exception is a control finding to investigate before sign-off.</t>
+          <t>Intercompany reconciliation &amp; elimination on consolidation.</t>
         </is>
       </c>
       <c r="H103" s="17" t="inlineStr">
@@ -9797,17 +9797,17 @@
       </c>
       <c r="I103" s="17" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="J103" s="17" t="inlineStr">
         <is>
-          <t>Period / on demand</t>
+          <t>Period</t>
         </is>
       </c>
       <c r="K103" s="16" t="inlineStr">
         <is>
-          <t>Controller / CFO</t>
+          <t>Group Controller</t>
         </is>
       </c>
       <c r="L103" s="17" t="inlineStr">
@@ -9817,34 +9817,34 @@
       </c>
       <c r="M103" s="16" t="inlineStr">
         <is>
-          <t>finance.service.ts reconcileControls; finance.controller.ts GET reconciliation/controls (exec/ar/creditors); reuses ledger.trialBalance + the AR/AP/inventory/gift-card/deferred sub-ledgers; cutover/giftcards.ts + compliance.ts (ToE)</t>
+          <t>intercompany; consolidation</t>
         </is>
       </c>
       <c r="N103" s="16" t="inlineStr">
         <is>
-          <t>Inspect the pack: each control account's sub-ledger query + the GL tie + the exceptions roll-up.</t>
+          <t>Inspect IC matching + elimination.</t>
         </is>
       </c>
       <c r="O103" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: with a clean set, every line reconciled + all_reconciled=true; introduce a known sub-ledger/GL difference and confirm it surfaces as an exception (re-performed: gift-card 2200 + inventory 1200 ties asserted by the harnesses).</t>
+          <t>Sample IC pairs agree &amp; eliminate.</t>
         </is>
       </c>
       <c r="P103" s="16" t="inlineStr">
         <is>
-          <t>Reconciliation pack; exceptions list</t>
-        </is>
-      </c>
-      <c r="Q103" s="18" t="inlineStr">
-        <is>
-          <t>Implemented</t>
+          <t>IC recon</t>
+        </is>
+      </c>
+      <c r="Q103" s="19" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="11" t="inlineStr">
         <is>
-          <t>REC-05</t>
+          <t>REC-04</t>
         </is>
       </c>
       <c r="B104" s="12" t="inlineStr">
@@ -9859,42 +9859,42 @@
       </c>
       <c r="D104" s="12" t="inlineStr">
         <is>
-          <t>Cash; Bank</t>
+          <t>All control accounts</t>
         </is>
       </c>
       <c r="E104" s="12" t="inlineStr">
         <is>
-          <t>Till cash dropped to the safe never reaches the bank, or a deposit isn't matched to the statement — cash sits unbanked (theft/loss exposure) or the bank balance can't be tied to the books.</t>
+          <t>A sub-ledger silently drifts from its GL control account at period-end and no single review catches it (incomplete/inaccurate balances reach the financial statements).</t>
         </is>
       </c>
       <c r="F104" s="12" t="inlineStr">
         <is>
-          <t>Completeness/Existence/Authorization</t>
+          <t>Completeness/Accuracy</t>
         </is>
       </c>
       <c r="G104" s="12" t="inlineStr">
         <is>
-          <t>Cash banking — safe-drop → bank deposit → reconciliation: till 'drop's move cash from the drawer to the safe (drawer-only, no GL). Banking BATCHES the undeposited drops into a deposit and posts the GL (Dr &lt;bank account, e.g. 1010&gt; / Cr 1000 Cash), stamping each drop with the deposit id; the deposit is then RECONCILED to the bank statement (status Deposited→Reconciled). A detective read (GET /api/bank/deposits/undeposited-drops) surfaces the CASH STILL IN THE SAFE (drops with deposit_id NULL) — the unbanked exposure to chase. SoD: banking is a treasury duty (exec/ar) — segregated from the cashier (pos_till) who drops the cash, so the person who removes cash from the drawer is not the one who banks it.</t>
+          <t>Period-end control-account reconciliation PACK: one read (GET /api/finance/reconciliation/controls) ties every major sub-ledger to its GL control account and FLAGS any out-of-balance — AR↔1100, AP↔2000, Inventory↔1200, Gift cards/Customer-deposits↔2200, Deferred revenue↔2400 — reporting per line {sub_ledger, gl_control, variance, reconciled} plus an overall all_reconciled flag and an exceptions count. Liability controls are sign-flipped before comparison. The controller's single 'are the books reconciled?' close view; an exception is a control finding to investigate before sign-off.</t>
         </is>
       </c>
       <c r="H104" s="13" t="inlineStr">
         <is>
-          <t>Det/Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I104" s="13" t="inlineStr">
         <is>
-          <t>Auto+Manual</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J104" s="13" t="inlineStr">
         <is>
-          <t>Per banking run</t>
+          <t>Period / on demand</t>
         </is>
       </c>
       <c r="K104" s="12" t="inlineStr">
         <is>
-          <t>FinancialController / Treasury</t>
+          <t>Controller / CFO</t>
         </is>
       </c>
       <c r="L104" s="13" t="inlineStr">
@@ -9904,22 +9904,22 @@
       </c>
       <c r="M104" s="12" t="inlineStr">
         <is>
-          <t>bank.service.ts undepositedDrops/createDeposit (Dr bank/Cr 1000, stamps deposit_id)/reconcileDeposit/listDeposits; bank.controller.ts (deposits, deposits/undeposited-drops, deposits/:id/reconcile; exec/ar); schema/cash.ts bank_deposits + cash_movements.deposit_id + migration 0152; /cash-banking UI; cutover/cash-banking.ts (ToE)</t>
+          <t>finance.service.ts reconcileControls; finance.controller.ts GET reconciliation/controls (exec/ar/creditors); reuses ledger.trialBalance + the AR/AP/inventory/gift-card/deferred sub-ledgers; cutover/giftcards.ts + compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N104" s="12" t="inlineStr">
         <is>
-          <t>Inspect the undeposited-drop exposure read + the deposit GL (bank↔1000) + the reconcile step + the SoD (cashier vs treasury).</t>
+          <t>Inspect the pack: each control account's sub-ledger query + the GL tie + the exceptions roll-up.</t>
         </is>
       </c>
       <c r="O104" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: two till drops → cash-in-safe shows the total; a cashier (pos_till) cannot bank (403); treasury banks → Dr bank / Cr 1000, cash-in-safe back to 0; reconcile the deposit; trial balance balanced (re-performed by the cash-banking harness).</t>
+          <t>Re-perform: with a clean set, every line reconciled + all_reconciled=true; introduce a known sub-ledger/GL difference and confirm it surfaces as an exception (re-performed: gift-card 2200 + inventory 1200 ties asserted by the harnesses).</t>
         </is>
       </c>
       <c r="P104" s="12" t="inlineStr">
         <is>
-          <t>Bank-deposit register; undeposited-drop (cash-in-safe) exposure</t>
+          <t>Reconciliation pack; exceptions list</t>
         </is>
       </c>
       <c r="Q104" s="18" t="inlineStr">
@@ -9931,12 +9931,12 @@
     <row r="105">
       <c r="A105" s="15" t="inlineStr">
         <is>
-          <t>GOV-01</t>
+          <t>REC-05</t>
         </is>
       </c>
       <c r="B105" s="16" t="inlineStr">
         <is>
-          <t>Monitoring</t>
+          <t>Reconciliation</t>
         </is>
       </c>
       <c r="C105" s="17" t="inlineStr">
@@ -9946,42 +9946,42 @@
       </c>
       <c r="D105" s="16" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Cash; Bank</t>
         </is>
       </c>
       <c r="E105" s="16" t="inlineStr">
         <is>
-          <t>A maker-checker approval sits un-actioned and is forgotten — a transaction stalls before it is effective, or (worse) a control is quietly bypassed and no one notices an item never got its independent review.</t>
+          <t>Till cash dropped to the safe never reaches the bank, or a deposit isn't matched to the statement — cash sits unbanked (theft/loss exposure) or the bank balance can't be tied to the books.</t>
         </is>
       </c>
       <c r="F105" s="16" t="inlineStr">
         <is>
-          <t>Authorization/Completeness</t>
+          <t>Completeness/Existence/Authorization</t>
         </is>
       </c>
       <c r="G105" s="16" t="inlineStr">
         <is>
-          <t>Pending-approvals MONITOR (COSO monitoring): a single worklist of EVERY item awaiting independent approval across the system, each with its AGE in days and an overdue roll-up — spanning the manual-JE (GL-05), bank-adjustment (BANK-02), AP-disbursement (EXP-06), payroll (PAY-03), asset-revaluation (FA-08), asset-disposal (FA-09), inventory-write-off (INV-07), till-close cash over/short (REV-13), FX-rate (FX-04), budget (BUD-01) and large-refund (REV-16) maker-checkers. The controller reviews it before close; a stale item (age beyond the threshold) is a control finding to chase or escalate. The /approvals screen also lets a manager approve/reject a material till variance or a large refund inline (the pending types with no dedicated module screen). Read-only worklist; tenant-scoped via the caller's RLS.</t>
+          <t>Cash banking — safe-drop → bank deposit → reconciliation: till 'drop's move cash from the drawer to the safe (drawer-only, no GL). Banking BATCHES the undeposited drops into a deposit and posts the GL (Dr &lt;bank account, e.g. 1010&gt; / Cr 1000 Cash), stamping each drop with the deposit id; the deposit is then RECONCILED to the bank statement (status Deposited→Reconciled). A detective read (GET /api/bank/deposits/undeposited-drops) surfaces the CASH STILL IN THE SAFE (drops with deposit_id NULL) — the unbanked exposure to chase. SoD: banking is a treasury duty (exec/ar) — segregated from the cashier (pos_till) who drops the cash, so the person who removes cash from the drawer is not the one who banks it.</t>
         </is>
       </c>
       <c r="H105" s="17" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Det/Prev</t>
         </is>
       </c>
       <c r="I105" s="17" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="J105" s="17" t="inlineStr">
         <is>
-          <t>Continuous / pre-close</t>
+          <t>Per banking run</t>
         </is>
       </c>
       <c r="K105" s="16" t="inlineStr">
         <is>
-          <t>Controller / CFO</t>
+          <t>FinancialController / Treasury</t>
         </is>
       </c>
       <c r="L105" s="17" t="inlineStr">
@@ -9991,22 +9991,22 @@
       </c>
       <c r="M105" s="16" t="inlineStr">
         <is>
-          <t>finance.service.ts pendingApprovals; finance.controller.ts GET approvals/pending (exec/approvals/creditors); aggregates journalEntries(Draft incl. BANKADJ→BANK-02)/apPayments/payruns/asset_revaluations/fixed_assets(disposal_pending)/inv_writeoff_requests/till_sessions(PendingApproval)/fx_rates(PendingApproval)/budgets(PendingApproval); cutover/compliance.ts (ToE)</t>
+          <t>bank.service.ts undepositedDrops/createDeposit (Dr bank/Cr 1000, stamps deposit_id)/reconcileDeposit/listDeposits; bank.controller.ts (deposits, deposits/undeposited-drops, deposits/:id/reconcile; exec/ar); schema/cash.ts bank_deposits + cash_movements.deposit_id + migration 0152; /cash-banking UI; cutover/cash-banking.ts (ToE)</t>
         </is>
       </c>
       <c r="N105" s="16" t="inlineStr">
         <is>
-          <t>Inspect the aggregation across all pending sources + the age/overdue roll-up.</t>
+          <t>Inspect the undeposited-drop exposure read + the deposit GL (bank↔1000) + the reconcile step + the SoD (cashier vs treasury).</t>
         </is>
       </c>
       <c r="O105" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: create a pending item (e.g. a Draft JE) and confirm it appears in the worklist with its control ID, amount and age; the overdue count flags items past the threshold (re-performed by the harness).</t>
+          <t>Re-perform: two till drops → cash-in-safe shows the total; a cashier (pos_till) cannot bank (403); treasury banks → Dr bank / Cr 1000, cash-in-safe back to 0; reconcile the deposit; trial balance balanced (re-performed by the cash-banking harness).</t>
         </is>
       </c>
       <c r="P105" s="16" t="inlineStr">
         <is>
-          <t>Pending-approvals worklist</t>
+          <t>Bank-deposit register; undeposited-drop (cash-in-safe) exposure</t>
         </is>
       </c>
       <c r="Q105" s="18" t="inlineStr">
@@ -10018,12 +10018,12 @@
     <row r="106">
       <c r="A106" s="11" t="inlineStr">
         <is>
-          <t>TAX-01</t>
+          <t>GOV-01</t>
         </is>
       </c>
       <c r="B106" s="12" t="inlineStr">
         <is>
-          <t>Tax</t>
+          <t>Monitoring</t>
         </is>
       </c>
       <c r="C106" s="13" t="inlineStr">
@@ -10033,27 +10033,27 @@
       </c>
       <c r="D106" s="12" t="inlineStr">
         <is>
-          <t>Tax (VAT)</t>
+          <t>All</t>
         </is>
       </c>
       <c r="E106" s="12" t="inlineStr">
         <is>
-          <t>VAT computed incorrectly → filing/penalty risk.</t>
+          <t>A maker-checker approval sits un-actioned and is forgotten — a transaction stalls before it is effective, or (worse) a control is quietly bypassed and no one notices an item never got its independent review.</t>
         </is>
       </c>
       <c r="F106" s="12" t="inlineStr">
         <is>
-          <t>Accuracy</t>
+          <t>Authorization/Completeness</t>
         </is>
       </c>
       <c r="G106" s="12" t="inlineStr">
         <is>
-          <t>VAT via pluggable provider (TH 7%); unit-tested; no hard-coded rate.</t>
+          <t>Pending-approvals MONITOR (COSO monitoring): a single worklist of EVERY item awaiting independent approval across the system, each with its AGE in days and an overdue roll-up — spanning the manual-JE (GL-05), bank-adjustment (BANK-02), AP-disbursement (EXP-06), payroll (PAY-03), asset-revaluation (FA-08), asset-disposal (FA-09), inventory-write-off (INV-07), till-close cash over/short (REV-13), FX-rate (FX-04), budget (BUD-01) and large-refund (REV-16) maker-checkers. The controller reviews it before close; a stale item (age beyond the threshold) is a control finding to chase or escalate. The /approvals screen also lets a manager approve/reject a material till variance or a large refund inline (the pending types with no dedicated module screen). Read-only worklist; tenant-scoped via the caller's RLS.</t>
         </is>
       </c>
       <c r="H106" s="13" t="inlineStr">
         <is>
-          <t>Auto</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I106" s="13" t="inlineStr">
@@ -10063,37 +10063,37 @@
       </c>
       <c r="J106" s="13" t="inlineStr">
         <is>
-          <t>Per txn</t>
+          <t>Continuous / pre-close</t>
         </is>
       </c>
       <c r="K106" s="12" t="inlineStr">
         <is>
-          <t>Tax / Controller</t>
+          <t>Controller / CFO</t>
         </is>
       </c>
       <c r="L106" s="13" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="M106" s="12" t="inlineStr">
         <is>
-          <t>tax/tax-providers.ts; tax.service.ts; test/unit.test.ts</t>
+          <t>finance.service.ts pendingApprovals; finance.controller.ts GET approvals/pending (exec/approvals/creditors); aggregates journalEntries(Draft incl. BANKADJ→BANK-02)/apPayments/payruns/asset_revaluations/fixed_assets(disposal_pending)/inv_writeoff_requests/till_sessions(PendingApproval)/fx_rates(PendingApproval)/budgets(PendingApproval); cutover/compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N106" s="12" t="inlineStr">
         <is>
-          <t>Inspect rate provider + tests.</t>
+          <t>Inspect the aggregation across all pending sources + the age/overdue roll-up.</t>
         </is>
       </c>
       <c r="O106" s="12" t="inlineStr">
         <is>
-          <t>Re-perform VAT on sample; tie to return.</t>
+          <t>Re-perform: create a pending item (e.g. a Draft JE) and confirm it appears in the worklist with its control ID, amount and age; the overdue count flags items past the threshold (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P106" s="12" t="inlineStr">
         <is>
-          <t>VAT tests</t>
+          <t>Pending-approvals worklist</t>
         </is>
       </c>
       <c r="Q106" s="18" t="inlineStr">
@@ -10105,7 +10105,7 @@
     <row r="107">
       <c r="A107" s="15" t="inlineStr">
         <is>
-          <t>TAX-02</t>
+          <t>TAX-01</t>
         </is>
       </c>
       <c r="B107" s="16" t="inlineStr">
@@ -10120,22 +10120,22 @@
       </c>
       <c r="D107" s="16" t="inlineStr">
         <is>
-          <t>Tax; Revenue</t>
+          <t>Tax (VAT)</t>
         </is>
       </c>
       <c r="E107" s="16" t="inlineStr">
         <is>
-          <t>Non-compliant e-Tax invoice / not transmitted to ETDA.</t>
+          <t>VAT computed incorrectly → filing/penalty risk.</t>
         </is>
       </c>
       <c r="F107" s="16" t="inlineStr">
         <is>
-          <t>Accuracy/Compliance</t>
+          <t>Accuracy</t>
         </is>
       </c>
       <c r="G107" s="16" t="inlineStr">
         <is>
-          <t>e-Tax invoice (ETDA UBL 2.1 XML) generation + email with CC to ETDA timestamp mailbox.</t>
+          <t>VAT via pluggable provider (TH 7%); unit-tested; no hard-coded rate.</t>
         </is>
       </c>
       <c r="H107" s="17" t="inlineStr">
@@ -10150,37 +10150,37 @@
       </c>
       <c r="J107" s="17" t="inlineStr">
         <is>
-          <t>Per invoice</t>
+          <t>Per txn</t>
         </is>
       </c>
       <c r="K107" s="16" t="inlineStr">
         <is>
-          <t>Tax</t>
+          <t>Tax / Controller</t>
         </is>
       </c>
       <c r="L107" s="17" t="inlineStr">
         <is>
-          <t>P10/P13</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="M107" s="16" t="inlineStr">
         <is>
-          <t>tax-docs/etax-xml.ts; etax-email.service.ts (tested)</t>
+          <t>tax/tax-providers.ts; tax.service.ts; test/unit.test.ts</t>
         </is>
       </c>
       <c r="N107" s="16" t="inlineStr">
         <is>
-          <t>Inspect XML schema + email composer.</t>
+          <t>Inspect rate provider + tests.</t>
         </is>
       </c>
       <c r="O107" s="16" t="inlineStr">
         <is>
-          <t>Sample invoices: valid XML, correct CC/escaping.</t>
+          <t>Re-perform VAT on sample; tie to return.</t>
         </is>
       </c>
       <c r="P107" s="16" t="inlineStr">
         <is>
-          <t>e-Tax samples</t>
+          <t>VAT tests</t>
         </is>
       </c>
       <c r="Q107" s="18" t="inlineStr">
@@ -10192,7 +10192,7 @@
     <row r="108">
       <c r="A108" s="11" t="inlineStr">
         <is>
-          <t>TAX-03</t>
+          <t>TAX-02</t>
         </is>
       </c>
       <c r="B108" s="12" t="inlineStr">
@@ -10207,22 +10207,22 @@
       </c>
       <c r="D108" s="12" t="inlineStr">
         <is>
-          <t>Tax (WHT)</t>
+          <t>Tax; Revenue</t>
         </is>
       </c>
       <c r="E108" s="12" t="inlineStr">
         <is>
-          <t>Withholding tax mis-computed / not reported.</t>
+          <t>Non-compliant e-Tax invoice / not transmitted to ETDA.</t>
         </is>
       </c>
       <c r="F108" s="12" t="inlineStr">
         <is>
-          <t>Accuracy</t>
+          <t>Accuracy/Compliance</t>
         </is>
       </c>
       <c r="G108" s="12" t="inlineStr">
         <is>
-          <t>WHT computation and ภ.ง.ด. reporting.</t>
+          <t>e-Tax invoice (ETDA UBL 2.1 XML) generation + email with CC to ETDA timestamp mailbox.</t>
         </is>
       </c>
       <c r="H108" s="13" t="inlineStr">
@@ -10237,7 +10237,7 @@
       </c>
       <c r="J108" s="13" t="inlineStr">
         <is>
-          <t>Per txn / monthly</t>
+          <t>Per invoice</t>
         </is>
       </c>
       <c r="K108" s="12" t="inlineStr">
@@ -10247,39 +10247,39 @@
       </c>
       <c r="L108" s="13" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P10/P13</t>
         </is>
       </c>
       <c r="M108" s="12" t="inlineStr">
         <is>
-          <t>tax-reports; payroll</t>
+          <t>tax-docs/etax-xml.ts; etax-email.service.ts (tested)</t>
         </is>
       </c>
       <c r="N108" s="12" t="inlineStr">
         <is>
-          <t>Inspect WHT logic + report.</t>
+          <t>Inspect XML schema + email composer.</t>
         </is>
       </c>
       <c r="O108" s="12" t="inlineStr">
         <is>
-          <t>Re-perform WHT on sample; tie to filing.</t>
+          <t>Sample invoices: valid XML, correct CC/escaping.</t>
         </is>
       </c>
       <c r="P108" s="12" t="inlineStr">
         <is>
-          <t>WHT report</t>
-        </is>
-      </c>
-      <c r="Q108" s="19" t="inlineStr">
-        <is>
-          <t>Partial</t>
+          <t>e-Tax samples</t>
+        </is>
+      </c>
+      <c r="Q108" s="18" t="inlineStr">
+        <is>
+          <t>Implemented</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="15" t="inlineStr">
         <is>
-          <t>TAX-04</t>
+          <t>TAX-03</t>
         </is>
       </c>
       <c r="B109" s="16" t="inlineStr">
@@ -10294,27 +10294,27 @@
       </c>
       <c r="D109" s="16" t="inlineStr">
         <is>
-          <t>Tax (VAT); Tax Payable (2100)</t>
+          <t>Tax (WHT)</t>
         </is>
       </c>
       <c r="E109" s="16" t="inlineStr">
         <is>
-          <t>Output/input VAT on the filed ภ.พ.30 return does not agree to the GL — VAT liability mis-stated, a filing/penalty exposure, or a posting omission goes undetected before submission.</t>
+          <t>Withholding tax mis-computed / not reported.</t>
         </is>
       </c>
       <c r="F109" s="16" t="inlineStr">
         <is>
-          <t>Completeness/Accuracy</t>
+          <t>Accuracy</t>
         </is>
       </c>
       <c r="G109" s="16" t="inlineStr">
         <is>
-          <t>Periodic VAT-return ↔ GL reconciliation (ภ.พ.30): the monthly return (GET /api/tax-reports/pp30) is built from the sales/output-VAT and purchase/input-VAT sub-reports, computes net VAT = output − input, and RECONCILES it to the **GL account 2100 (Tax Payable) net movement** for the same period (Σ credit − Σ debit over Posted entries) — returning `reconciliation.tied` = true only when the two agree within rounding. A non-tie is a detective finding to investigate and clear BEFORE filing (the form also carries the ม.157 deadline = the 15th of the next month). Output VAT is posted to 2100 on every sale (Cr) and reversed on returns (Dr); input VAT is posted on AP bills (Dr) — so 2100's net is the period's VAT payable. Read-only report; exportable to a ภ.พ.30 PDF/HTML.</t>
+          <t>WHT computation and ภ.ง.ด. reporting.</t>
         </is>
       </c>
       <c r="H109" s="17" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Auto</t>
         </is>
       </c>
       <c r="I109" s="17" t="inlineStr">
@@ -10324,54 +10324,54 @@
       </c>
       <c r="J109" s="17" t="inlineStr">
         <is>
-          <t>Monthly / pre-filing</t>
+          <t>Per txn / monthly</t>
         </is>
       </c>
       <c r="K109" s="16" t="inlineStr">
         <is>
-          <t>Tax / FinancialController</t>
+          <t>Tax</t>
         </is>
       </c>
       <c r="L109" s="17" t="inlineStr">
         <is>
-          <t>P10/P16</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="M109" s="16" t="inlineStr">
         <is>
-          <t>tax-reports.service.ts pp30 (outputVat/inputVat + 2100 net-movement tie); tax-reports.controller.ts (GET pp30, pp30/export, exec); tax-reports-pdf.ts; dine-in.service.ts/returns.service.ts/finance.service.ts post 2100 on sale/return/AP; /tax/reports UI; cutover/taxdocs.ts (ToE)</t>
+          <t>tax-reports; payroll</t>
         </is>
       </c>
       <c r="N109" s="16" t="inlineStr">
         <is>
-          <t>Inspect the pp30 build + the 2100 net-movement query + the tie flag + the filing deadline.</t>
+          <t>Inspect WHT logic + report.</t>
         </is>
       </c>
       <c r="O109" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: the pp30 return computes net VAT (output − input), the GL 2100 net movement reflects the posted input VAT, and the reconciliation block exposes the gl_account (2100), the report net VAT and a boolean tie verdict (tied iff the two agree within rounding); the ภ.พ.30 export renders (re-performed by the taxdocs harness).</t>
+          <t>Re-perform WHT on sample; tie to filing.</t>
         </is>
       </c>
       <c r="P109" s="16" t="inlineStr">
         <is>
-          <t>ภ.พ.30 return + GL-2100 reconciliation tie</t>
-        </is>
-      </c>
-      <c r="Q109" s="18" t="inlineStr">
-        <is>
-          <t>Implemented</t>
+          <t>WHT report</t>
+        </is>
+      </c>
+      <c r="Q109" s="19" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="11" t="inlineStr">
         <is>
-          <t>PAY-01</t>
+          <t>TAX-04</t>
         </is>
       </c>
       <c r="B110" s="12" t="inlineStr">
         <is>
-          <t>Payroll</t>
+          <t>Tax</t>
         </is>
       </c>
       <c r="C110" s="13" t="inlineStr">
@@ -10381,27 +10381,27 @@
       </c>
       <c r="D110" s="12" t="inlineStr">
         <is>
-          <t>Payroll expense/liability</t>
+          <t>Tax (VAT); Tax Payable (2100)</t>
         </is>
       </c>
       <c r="E110" s="12" t="inlineStr">
         <is>
-          <t>Payroll, SSO and PIT mis-computed.</t>
+          <t>Output/input VAT on the filed ภ.พ.30 return does not agree to the GL — VAT liability mis-stated, a filing/penalty exposure, or a posting omission goes undetected before submission.</t>
         </is>
       </c>
       <c r="F110" s="12" t="inlineStr">
         <is>
-          <t>Accuracy</t>
+          <t>Completeness/Accuracy</t>
         </is>
       </c>
       <c r="G110" s="12" t="inlineStr">
         <is>
-          <t>Payroll engine — SSO 5% (cap 750), progressive PIT, payslip net; unit-tested.</t>
+          <t>Periodic VAT-return ↔ GL reconciliation (ภ.พ.30): the monthly return (GET /api/tax-reports/pp30) is built from the sales/output-VAT and purchase/input-VAT sub-reports, computes net VAT = output − input, and RECONCILES it to the **GL account 2100 (Tax Payable) net movement** for the same period (Σ credit − Σ debit over Posted entries) — returning `reconciliation.tied` = true only when the two agree within rounding. A non-tie is a detective finding to investigate and clear BEFORE filing (the form also carries the ม.157 deadline = the 15th of the next month). Output VAT is posted to 2100 on every sale (Cr) and reversed on returns (Dr); input VAT is posted on AP bills (Dr) — so 2100's net is the period's VAT payable. Read-only report; exportable to a ภ.พ.30 PDF/HTML.</t>
         </is>
       </c>
       <c r="H110" s="13" t="inlineStr">
         <is>
-          <t>Auto</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I110" s="13" t="inlineStr">
@@ -10411,37 +10411,37 @@
       </c>
       <c r="J110" s="13" t="inlineStr">
         <is>
-          <t>Per run</t>
+          <t>Monthly / pre-filing</t>
         </is>
       </c>
       <c r="K110" s="12" t="inlineStr">
         <is>
-          <t>HR / Payroll</t>
+          <t>Tax / FinancialController</t>
         </is>
       </c>
       <c r="L110" s="13" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P10/P16</t>
         </is>
       </c>
       <c r="M110" s="12" t="inlineStr">
         <is>
-          <t>payroll/payroll-calc.ts; test/unit.test.ts</t>
+          <t>tax-reports.service.ts pp30 (outputVat/inputVat + 2100 net-movement tie); tax-reports.controller.ts (GET pp30, pp30/export, exec); tax-reports-pdf.ts; dine-in.service.ts/returns.service.ts/finance.service.ts post 2100 on sale/return/AP; /tax/reports UI; cutover/taxdocs.ts (ToE)</t>
         </is>
       </c>
       <c r="N110" s="12" t="inlineStr">
         <is>
-          <t>Inspect calc + tests.</t>
+          <t>Inspect the pp30 build + the 2100 net-movement query + the tie flag + the filing deadline.</t>
         </is>
       </c>
       <c r="O110" s="12" t="inlineStr">
         <is>
-          <t>Re-perform sample payslips.</t>
+          <t>Re-perform: the pp30 return computes net VAT (output − input), the GL 2100 net movement reflects the posted input VAT, and the reconciliation block exposes the gl_account (2100), the report net VAT and a boolean tie verdict (tied iff the two agree within rounding); the ภ.พ.30 export renders (re-performed by the taxdocs harness).</t>
         </is>
       </c>
       <c r="P110" s="12" t="inlineStr">
         <is>
-          <t>Payslip tests</t>
+          <t>ภ.พ.30 return + GL-2100 reconciliation tie</t>
         </is>
       </c>
       <c r="Q110" s="18" t="inlineStr">
@@ -10453,7 +10453,7 @@
     <row r="111">
       <c r="A111" s="15" t="inlineStr">
         <is>
-          <t>PAY-02</t>
+          <t>PAY-01</t>
         </is>
       </c>
       <c r="B111" s="16" t="inlineStr">
@@ -10468,27 +10468,27 @@
       </c>
       <c r="D111" s="16" t="inlineStr">
         <is>
-          <t>Payroll liability</t>
+          <t>Payroll expense/liability</t>
         </is>
       </c>
       <c r="E111" s="16" t="inlineStr">
         <is>
-          <t>Statutory withholdings (SSO/WHT/PF) mis-stated or not remitted, so the liability owed to the authorities diverges from the books.</t>
+          <t>Payroll, SSO and PIT mis-computed.</t>
         </is>
       </c>
       <c r="F111" s="16" t="inlineStr">
         <is>
-          <t>Accuracy/Compliance</t>
+          <t>Accuracy</t>
         </is>
       </c>
       <c r="G111" s="16" t="inlineStr">
         <is>
-          <t>Payroll-liability schedule (GET /api/payroll/liabilities): each statutory account — SSO 2350, WHT/PND1 2360, PF 2370 — shows accrued (GL credits) − remitted (GL debits) = outstanding, tied back to the INDEPENDENT payrun accrual with a `reconciled` flag (a divergence flags a manual JE that touched a payroll-liability account outside the payroll process). Treasury remits the cash (POST .../remit → Dr liability / Cr 1000) which clears the outstanding and keeps the books reconciled to the statutory filings; a remittance beyond the outstanding is blocked (REMIT_EXCEEDS_OUTSTANDING).</t>
+          <t>Payroll engine — SSO 5% (cap 750), progressive PIT, payslip net; unit-tested.</t>
         </is>
       </c>
       <c r="H111" s="17" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Auto</t>
         </is>
       </c>
       <c r="I111" s="17" t="inlineStr">
@@ -10498,12 +10498,12 @@
       </c>
       <c r="J111" s="17" t="inlineStr">
         <is>
-          <t>Per run / monthly</t>
+          <t>Per run</t>
         </is>
       </c>
       <c r="K111" s="16" t="inlineStr">
         <is>
-          <t>HR / Payroll / Treasury</t>
+          <t>HR / Payroll</t>
         </is>
       </c>
       <c r="L111" s="17" t="inlineStr">
@@ -10513,22 +10513,22 @@
       </c>
       <c r="M111" s="16" t="inlineStr">
         <is>
-          <t>payroll/payroll.service.ts liabilities/remitLiability</t>
+          <t>payroll/payroll-calc.ts; test/unit.test.ts</t>
         </is>
       </c>
       <c r="N111" s="16" t="inlineStr">
         <is>
-          <t>Inspect the schedule + the accrued/remitted/outstanding tie-out and the reconciled flag.</t>
+          <t>Inspect calc + tests.</t>
         </is>
       </c>
       <c r="O111" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: run a payroll, confirm the SSO/WHT outstanding equals the payrun accrual; remit part and confirm the outstanding falls and the TB stays balanced; attempt an over-remit (REMIT_EXCEEDS_OUTSTANDING).</t>
+          <t>Re-perform sample payslips.</t>
         </is>
       </c>
       <c r="P111" s="16" t="inlineStr">
         <is>
-          <t>Liability schedule + remittance JEs tied to filings</t>
+          <t>Payslip tests</t>
         </is>
       </c>
       <c r="Q111" s="18" t="inlineStr">
@@ -10540,7 +10540,7 @@
     <row r="112">
       <c r="A112" s="11" t="inlineStr">
         <is>
-          <t>PAY-03</t>
+          <t>PAY-02</t>
         </is>
       </c>
       <c r="B112" s="12" t="inlineStr">
@@ -10555,27 +10555,27 @@
       </c>
       <c r="D112" s="12" t="inlineStr">
         <is>
-          <t>Payroll expense/liability; Cash</t>
+          <t>Payroll liability</t>
         </is>
       </c>
       <c r="E112" s="12" t="inlineStr">
         <is>
-          <t>Payroll run posted to the GL without independent review — the preparer both computes and posts their own payroll (ghost employees, inflated rate/hours).</t>
+          <t>Statutory withholdings (SSO/WHT/PF) mis-stated or not remitted, so the liability owed to the authorities diverges from the books.</t>
         </is>
       </c>
       <c r="F112" s="12" t="inlineStr">
         <is>
-          <t>Authorization</t>
+          <t>Accuracy/Compliance</t>
         </is>
       </c>
       <c r="G112" s="12" t="inlineStr">
         <is>
-          <t>Payroll maker-checker (SoD): a run posts its GL entry as a DRAFT (excluded from balances) with the run record 'PendingApproval'; a DIFFERENT user must approve before it becomes effective (approver ≠ preparer enforced regardless of permissions, reusing the GL-05 ledger approval). Reject voids the draft; idempotent per (tenant, period).</t>
+          <t>Payroll-liability schedule (GET /api/payroll/liabilities): each statutory account — SSO 2350, WHT/PND1 2360, PF 2370 — shows accrued (GL credits) − remitted (GL debits) = outstanding, tied back to the INDEPENDENT payrun accrual with a `reconciled` flag (a divergence flags a manual JE that touched a payroll-liability account outside the payroll process). Treasury remits the cash (POST .../remit → Dr liability / Cr 1000) which clears the outstanding and keeps the books reconciled to the statutory filings; a remittance beyond the outstanding is blocked (REMIT_EXCEEDS_OUTSTANDING).</t>
         </is>
       </c>
       <c r="H112" s="13" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I112" s="13" t="inlineStr">
@@ -10585,12 +10585,12 @@
       </c>
       <c r="J112" s="13" t="inlineStr">
         <is>
-          <t>Per run</t>
+          <t>Per run / monthly</t>
         </is>
       </c>
       <c r="K112" s="12" t="inlineStr">
         <is>
-          <t>HR / Payroll; Controller</t>
+          <t>HR / Payroll / Treasury</t>
         </is>
       </c>
       <c r="L112" s="13" t="inlineStr">
@@ -10600,22 +10600,22 @@
       </c>
       <c r="M112" s="12" t="inlineStr">
         <is>
-          <t>payroll/payroll.service.ts approvePayroll/rejectPayroll; migration 0133</t>
+          <t>payroll/payroll.service.ts liabilities/remitLiability</t>
         </is>
       </c>
       <c r="N112" s="12" t="inlineStr">
         <is>
-          <t>Inspect Draft→approve flow + the approver≠preparer check.</t>
+          <t>Inspect the schedule + the accrued/remitted/outstanding tie-out and the reconciled flag.</t>
         </is>
       </c>
       <c r="O112" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: run as A, attempt self-approve (SOD_VIOLATION), approve as B; confirm the JE hits balances only after approval.</t>
+          <t>Re-perform: run a payroll, confirm the SSO/WHT outstanding equals the payrun accrual; remit part and confirm the outstanding falls and the TB stays balanced; attempt an over-remit (REMIT_EXCEEDS_OUTSTANDING).</t>
         </is>
       </c>
       <c r="P112" s="12" t="inlineStr">
         <is>
-          <t>Approval log + SoD test</t>
+          <t>Liability schedule + remittance JEs tied to filings</t>
         </is>
       </c>
       <c r="Q112" s="18" t="inlineStr">
@@ -10627,12 +10627,12 @@
     <row r="113">
       <c r="A113" s="15" t="inlineStr">
         <is>
-          <t>FA-09</t>
+          <t>PAY-03</t>
         </is>
       </c>
       <c r="B113" s="16" t="inlineStr">
         <is>
-          <t>Fixed Assets</t>
+          <t>Payroll</t>
         </is>
       </c>
       <c r="C113" s="17" t="inlineStr">
@@ -10642,12 +10642,12 @@
       </c>
       <c r="D113" s="16" t="inlineStr">
         <is>
-          <t>Property, Plant &amp; Equipment; Cash</t>
+          <t>Payroll expense/liability; Cash</t>
         </is>
       </c>
       <c r="E113" s="16" t="inlineStr">
         <is>
-          <t>Asset disposed without independent review — one person writes an asset off the books and records the proceeds (asset-stripping / theft: dispose a still-held asset, or to a related party below value).</t>
+          <t>Payroll run posted to the GL without independent review — the preparer both computes and posts their own payroll (ghost employees, inflated rate/hours).</t>
         </is>
       </c>
       <c r="F113" s="16" t="inlineStr">
@@ -10657,7 +10657,7 @@
       </c>
       <c r="G113" s="16" t="inlineStr">
         <is>
-          <t>Asset-disposal maker-checker (SoD): a disposal REQUEST posts its GL entry as a DRAFT (excluded from balances) and flags the asset disposal_pending WITHOUT marking it disposed or moving the register; a DIFFERENT user must approve before it is effective (status→disposed, revaluation surplus recycled 3200→3100) (approver ≠ requester enforced regardless of permissions, reusing the GL-05 ledger approval). Reject voids the draft and the asset stays in service; only one disposal may be pending per asset; a disposal-pending asset is frozen from depreciation.</t>
+          <t>Payroll maker-checker (SoD): a run posts its GL entry as a DRAFT (excluded from balances) with the run record 'PendingApproval'; a DIFFERENT user must approve before it becomes effective (approver ≠ preparer enforced regardless of permissions, reusing the GL-05 ledger approval). Reject voids the draft; idempotent per (tenant, period).</t>
         </is>
       </c>
       <c r="H113" s="17" t="inlineStr">
@@ -10672,12 +10672,12 @@
       </c>
       <c r="J113" s="17" t="inlineStr">
         <is>
-          <t>Per disposal</t>
+          <t>Per run</t>
         </is>
       </c>
       <c r="K113" s="16" t="inlineStr">
         <is>
-          <t>FaAccountant / Controller</t>
+          <t>HR / Payroll; Controller</t>
         </is>
       </c>
       <c r="L113" s="17" t="inlineStr">
@@ -10687,22 +10687,22 @@
       </c>
       <c r="M113" s="16" t="inlineStr">
         <is>
-          <t>assets.service.ts dispose(pendingApproval Draft)/approveDisposal/rejectDisposal; assets.controller.ts (:assetNo/dispose/approve|reject); schema/assets.ts fixed_assets.disposal_pending + migration 0135; cutover/basics.ts + worldclass.ts + compliance.ts (ToE)</t>
+          <t>payroll/payroll.service.ts approvePayroll/rejectPayroll; migration 0133</t>
         </is>
       </c>
       <c r="N113" s="16" t="inlineStr">
         <is>
-          <t>Inspect Draft→approve flow + the approver≠requester check + deferred status/recycle.</t>
+          <t>Inspect Draft→approve flow + the approver≠preparer check.</t>
         </is>
       </c>
       <c r="O113" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: request a disposal (Draft JE excluded), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm status→disposed + surplus recycled only after approval (re-performed by the harnesses).</t>
+          <t>Re-perform: run as A, attempt self-approve (SOD_VIOLATION), approve as B; confirm the JE hits balances only after approval.</t>
         </is>
       </c>
       <c r="P113" s="16" t="inlineStr">
         <is>
-          <t>Disposal approval log + SoD test</t>
+          <t>Approval log + SoD test</t>
         </is>
       </c>
       <c r="Q113" s="18" t="inlineStr">
@@ -10714,7 +10714,7 @@
     <row r="114">
       <c r="A114" s="11" t="inlineStr">
         <is>
-          <t>FA-10</t>
+          <t>FA-09</t>
         </is>
       </c>
       <c r="B114" s="12" t="inlineStr">
@@ -10729,22 +10729,22 @@
       </c>
       <c r="D114" s="12" t="inlineStr">
         <is>
-          <t>Property, Plant &amp; Equipment; Accounts Payable</t>
+          <t>Property, Plant &amp; Equipment; Cash</t>
         </is>
       </c>
       <c r="E114" s="12" t="inlineStr">
         <is>
-          <t>Capital purchases mis-capitalised or capitalised without independent review — the person who receives the goods also decides what enters the asset register and at what cost/useful life (fictitious or over-valued assets; capex/opex mis-classification).</t>
+          <t>Asset disposed without independent review — one person writes an asset off the books and records the proceeds (asset-stripping / theft: dispose a still-held asset, or to a related party below value).</t>
         </is>
       </c>
       <c r="F114" s="12" t="inlineStr">
         <is>
-          <t>Authorization; Accuracy</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="G114" s="12" t="inlineStr">
         <is>
-          <t>Procure-to-Capitalize maker-checker (SoD): a goods-receipt line flagged capital (item-master is_fixed_asset or per-PO-line override) is excluded from inventory capitalisation (1200) at receipt and instead becomes ELIGIBLE for the asset register. Capitalisation is a REQUEST that posts NOTHING to the GL; a DIFFERENT user must approve before the fixed_assets row + acquisition JE (Dr 1500 / Cr 2000) are created (approver ≠ requester enforced regardless of permissions). The created asset carries its source GR/PO for end-to-end PR→PO→GR→FA traceability; a GR line cannot be capitalised twice.</t>
+          <t>Asset-disposal maker-checker (SoD): a disposal REQUEST posts its GL entry as a DRAFT (excluded from balances) and flags the asset disposal_pending WITHOUT marking it disposed or moving the register; a DIFFERENT user must approve before it is effective (status→disposed, revaluation surplus recycled 3200→3100) (approver ≠ requester enforced regardless of permissions, reusing the GL-05 ledger approval). Reject voids the draft and the asset stays in service; only one disposal may be pending per asset; a disposal-pending asset is frozen from depreciation.</t>
         </is>
       </c>
       <c r="H114" s="13" t="inlineStr">
@@ -10759,7 +10759,7 @@
       </c>
       <c r="J114" s="13" t="inlineStr">
         <is>
-          <t>Per capital receipt</t>
+          <t>Per disposal</t>
         </is>
       </c>
       <c r="K114" s="12" t="inlineStr">
@@ -10774,22 +10774,22 @@
       </c>
       <c r="M114" s="12" t="inlineStr">
         <is>
-          <t>assets.service.ts registerFromGr/approveRegistration/rejectRegistration/eligibleFromGr; assets.controller.ts (registrations*); procurement.service.ts createGr (is_capital routing, costing excluded); schema/assets.ts asset_registration_requests + fixed_assets.source_gr_no/po_no + migration 0137; cutover/basics.ts + compliance.ts (ToE)</t>
+          <t>assets.service.ts dispose(pendingApproval Draft)/approveDisposal/rejectDisposal; assets.controller.ts (:assetNo/dispose/approve|reject); schema/assets.ts fixed_assets.disposal_pending + migration 0135; cutover/basics.ts + worldclass.ts + compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N114" s="12" t="inlineStr">
         <is>
-          <t>Inspect the eligible→request→approve flow + approver≠requester check + the inventory-vs-asset routing of capital lines.</t>
+          <t>Inspect Draft→approve flow + the approver≠requester check + deferred status/recycle.</t>
         </is>
       </c>
       <c r="O114" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: receive a capital line, raise a registration (no GL), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm the asset + Dr 1500/Cr 2000 post only after approval and the line cannot be re-registered (re-performed by the harnesses).</t>
+          <t>Re-perform: request a disposal (Draft JE excluded), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm status→disposed + surplus recycled only after approval (re-performed by the harnesses).</t>
         </is>
       </c>
       <c r="P114" s="12" t="inlineStr">
         <is>
-          <t>Capitalization approval log + SoD test</t>
+          <t>Disposal approval log + SoD test</t>
         </is>
       </c>
       <c r="Q114" s="18" t="inlineStr">
@@ -10801,12 +10801,12 @@
     <row r="115">
       <c r="A115" s="15" t="inlineStr">
         <is>
-          <t>CON-01</t>
+          <t>FA-10</t>
         </is>
       </c>
       <c r="B115" s="16" t="inlineStr">
         <is>
-          <t>Consolidation &amp; FX</t>
+          <t>Fixed Assets</t>
         </is>
       </c>
       <c r="C115" s="17" t="inlineStr">
@@ -10816,42 +10816,42 @@
       </c>
       <c r="D115" s="16" t="inlineStr">
         <is>
-          <t>Consolidation</t>
+          <t>Property, Plant &amp; Equipment; Accounts Payable</t>
         </is>
       </c>
       <c r="E115" s="16" t="inlineStr">
         <is>
-          <t>Group consolidation mis-stated (ownership/currency).</t>
+          <t>Capital purchases mis-capitalised or capitalised without independent review — the person who receives the goods also decides what enters the asset register and at what cost/useful life (fictitious or over-valued assets; capex/opex mis-classification).</t>
         </is>
       </c>
       <c r="F115" s="16" t="inlineStr">
         <is>
-          <t>Accuracy</t>
+          <t>Authorization; Accuracy</t>
         </is>
       </c>
       <c r="G115" s="16" t="inlineStr">
         <is>
-          <t>Consolidation run (ownership %, entity currency) gated by 'approvals'.</t>
+          <t>Procure-to-Capitalize maker-checker (SoD): a goods-receipt line flagged capital (item-master is_fixed_asset or per-PO-line override) is excluded from inventory capitalisation (1200) at receipt and instead becomes ELIGIBLE for the asset register. Capitalisation is a REQUEST that posts NOTHING to the GL; a DIFFERENT user must approve before the fixed_assets row + acquisition JE (Dr 1500 / Cr 2000) are created (approver ≠ requester enforced regardless of permissions). The created asset carries its source GR/PO for end-to-end PR→PO→GR→FA traceability; a GR line cannot be capitalised twice.</t>
         </is>
       </c>
       <c r="H115" s="17" t="inlineStr">
         <is>
-          <t>Auto+Manual</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I115" s="17" t="inlineStr">
         <is>
-          <t>Period</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J115" s="17" t="inlineStr">
         <is>
-          <t>Period</t>
+          <t>Per capital receipt</t>
         </is>
       </c>
       <c r="K115" s="16" t="inlineStr">
         <is>
-          <t>Group Controller</t>
+          <t>FaAccountant / Controller</t>
         </is>
       </c>
       <c r="L115" s="17" t="inlineStr">
@@ -10861,22 +10861,22 @@
       </c>
       <c r="M115" s="16" t="inlineStr">
         <is>
-          <t>consolidation.service.ts (runConsolidation @Permissions approvals)</t>
+          <t>assets.service.ts registerFromGr/approveRegistration/rejectRegistration/eligibleFromGr; assets.controller.ts (registrations*); procurement.service.ts createGr (is_capital routing, costing excluded); schema/assets.ts asset_registration_requests + fixed_assets.source_gr_no/po_no + migration 0137; cutover/basics.ts + compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N115" s="16" t="inlineStr">
         <is>
-          <t>Inspect consolidation logic + gate.</t>
+          <t>Inspect the eligible→request→approve flow + approver≠requester check + the inventory-vs-asset routing of capital lines.</t>
         </is>
       </c>
       <c r="O115" s="16" t="inlineStr">
         <is>
-          <t>Sample period: consolidated TB ties to entities.</t>
+          <t>Re-perform: receive a capital line, raise a registration (no GL), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm the asset + Dr 1500/Cr 2000 post only after approval and the line cannot be re-registered (re-performed by the harnesses).</t>
         </is>
       </c>
       <c r="P115" s="16" t="inlineStr">
         <is>
-          <t>Consol TB</t>
+          <t>Capitalization approval log + SoD test</t>
         </is>
       </c>
       <c r="Q115" s="18" t="inlineStr">
@@ -10888,7 +10888,7 @@
     <row r="116">
       <c r="A116" s="11" t="inlineStr">
         <is>
-          <t>CON-02</t>
+          <t>CON-01</t>
         </is>
       </c>
       <c r="B116" s="12" t="inlineStr">
@@ -10903,22 +10903,22 @@
       </c>
       <c r="D116" s="12" t="inlineStr">
         <is>
-          <t>FX gain/loss</t>
+          <t>Consolidation</t>
         </is>
       </c>
       <c r="E116" s="12" t="inlineStr">
         <is>
-          <t>FX exposures not revalued at period-end.</t>
+          <t>Group consolidation mis-stated (ownership/currency).</t>
         </is>
       </c>
       <c r="F116" s="12" t="inlineStr">
         <is>
-          <t>Valuation</t>
+          <t>Accuracy</t>
         </is>
       </c>
       <c r="G116" s="12" t="inlineStr">
         <is>
-          <t>FX revaluation at period-end rates; unrealized FX posted (acct 5400).</t>
+          <t>Consolidation run (ownership %, entity currency) gated by 'approvals'.</t>
         </is>
       </c>
       <c r="H116" s="13" t="inlineStr">
@@ -10928,7 +10928,7 @@
       </c>
       <c r="I116" s="13" t="inlineStr">
         <is>
-          <t>Period-end</t>
+          <t>Period</t>
         </is>
       </c>
       <c r="J116" s="13" t="inlineStr">
@@ -10938,7 +10938,7 @@
       </c>
       <c r="K116" s="12" t="inlineStr">
         <is>
-          <t>Controller</t>
+          <t>Group Controller</t>
         </is>
       </c>
       <c r="L116" s="13" t="inlineStr">
@@ -10948,22 +10948,22 @@
       </c>
       <c r="M116" s="12" t="inlineStr">
         <is>
-          <t>fx.service.ts (revalue / unrealized report)</t>
+          <t>consolidation.service.ts (runConsolidation @Permissions approvals)</t>
         </is>
       </c>
       <c r="N116" s="12" t="inlineStr">
         <is>
-          <t>Inspect reval logic + rates.</t>
+          <t>Inspect consolidation logic + gate.</t>
         </is>
       </c>
       <c r="O116" s="12" t="inlineStr">
         <is>
-          <t>Recompute reval on sample balances.</t>
+          <t>Sample period: consolidated TB ties to entities.</t>
         </is>
       </c>
       <c r="P116" s="12" t="inlineStr">
         <is>
-          <t>FX reval JE</t>
+          <t>Consol TB</t>
         </is>
       </c>
       <c r="Q116" s="18" t="inlineStr">
@@ -10975,7 +10975,7 @@
     <row r="117">
       <c r="A117" s="15" t="inlineStr">
         <is>
-          <t>FX-04</t>
+          <t>CON-02</t>
         </is>
       </c>
       <c r="B117" s="16" t="inlineStr">
@@ -10990,42 +10990,42 @@
       </c>
       <c r="D117" s="16" t="inlineStr">
         <is>
-          <t>FX gain/loss; Revenue; AR/AP</t>
+          <t>FX gain/loss</t>
         </is>
       </c>
       <c r="E117" s="16" t="inlineStr">
         <is>
-          <t>A wrong manually-entered FX rate (fat-fingered, e.g. USD 36 keyed as 63) flows straight into a period-end revaluation JE and the unrealized-FX report with no independent review — mis-stating earnings/equity and FX-translated balances.</t>
+          <t>FX exposures not revalued at period-end.</t>
         </is>
       </c>
       <c r="F117" s="16" t="inlineStr">
         <is>
-          <t>Accuracy/Valuation</t>
+          <t>Valuation</t>
         </is>
       </c>
       <c r="G117" s="16" t="inlineStr">
         <is>
-          <t>FX rate maker-checker (SoD): a MANUALLY-entered rate lands as PendingApproval and is EXCLUDED from rate resolution — revaluation, the unrealized-FX report, and consolidation translation all use APPROVED rates only — until a DIFFERENT user approves it (POST /api/fx/rates/approve). Self-approval → SOD_VIOLATION (binds even Admin); reject marks the rate Rejected (never usable); re-entering a rate sends it back to PendingApproval. Externally-sourced (feed) rates carrying an explicit non-manual source are auto-approved. Pending rates are also surfaced, aged, by the pending-approvals monitor (GOV-01).</t>
+          <t>FX revaluation at period-end rates; unrealized FX posted (acct 5400).</t>
         </is>
       </c>
       <c r="H117" s="17" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="I117" s="17" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Period-end</t>
         </is>
       </c>
       <c r="J117" s="17" t="inlineStr">
         <is>
-          <t>Per rate</t>
+          <t>Period</t>
         </is>
       </c>
       <c r="K117" s="16" t="inlineStr">
         <is>
-          <t>Controller / Treasury</t>
+          <t>Controller</t>
         </is>
       </c>
       <c r="L117" s="17" t="inlineStr">
@@ -11035,22 +11035,22 @@
       </c>
       <c r="M117" s="16" t="inlineStr">
         <is>
-          <t>fx.service.ts setRate(manual→PendingApproval)/approveRate/rejectRate/rateAsOf(Approved only); fx.controller.ts (rates/approve|reject|pending gated approvals/gl_close); consolidation.service.ts (translation reads Approved rates); schema/fx.ts fx_rates.status + migration 0141; cutover/fxreval.ts (ToE)</t>
+          <t>fx.service.ts (revalue / unrealized report)</t>
         </is>
       </c>
       <c r="N117" s="16" t="inlineStr">
         <is>
-          <t>Inspect the request→approve flow + the approver≠requester check + that revaluation/reporting resolve Approved rates only.</t>
+          <t>Inspect reval logic + rates.</t>
         </is>
       </c>
       <c r="O117" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: enter a manual rate (PendingApproval), confirm revalue is blocked NO_RATE while pending, attempt self-approve (SOD_VIOLATION), approve as a different user, then revalue succeeds (re-performed by the fxreval harness).</t>
+          <t>Recompute reval on sample balances.</t>
         </is>
       </c>
       <c r="P117" s="16" t="inlineStr">
         <is>
-          <t>FX rate approval log + SoD test</t>
+          <t>FX reval JE</t>
         </is>
       </c>
       <c r="Q117" s="18" t="inlineStr">
@@ -11062,92 +11062,179 @@
     <row r="118">
       <c r="A118" s="11" t="inlineStr">
         <is>
+          <t>FX-04</t>
+        </is>
+      </c>
+      <c r="B118" s="12" t="inlineStr">
+        <is>
+          <t>Consolidation &amp; FX</t>
+        </is>
+      </c>
+      <c r="C118" s="13" t="inlineStr">
+        <is>
+          <t>Application</t>
+        </is>
+      </c>
+      <c r="D118" s="12" t="inlineStr">
+        <is>
+          <t>FX gain/loss; Revenue; AR/AP</t>
+        </is>
+      </c>
+      <c r="E118" s="12" t="inlineStr">
+        <is>
+          <t>A wrong manually-entered FX rate (fat-fingered, e.g. USD 36 keyed as 63) flows straight into a period-end revaluation JE and the unrealized-FX report with no independent review — mis-stating earnings/equity and FX-translated balances.</t>
+        </is>
+      </c>
+      <c r="F118" s="12" t="inlineStr">
+        <is>
+          <t>Accuracy/Valuation</t>
+        </is>
+      </c>
+      <c r="G118" s="12" t="inlineStr">
+        <is>
+          <t>FX rate maker-checker (SoD): a MANUALLY-entered rate lands as PendingApproval and is EXCLUDED from rate resolution — revaluation, the unrealized-FX report, and consolidation translation all use APPROVED rates only — until a DIFFERENT user approves it (POST /api/fx/rates/approve). Self-approval → SOD_VIOLATION (binds even Admin); reject marks the rate Rejected (never usable); re-entering a rate sends it back to PendingApproval. Externally-sourced (feed) rates carrying an explicit non-manual source are auto-approved. Pending rates are also surfaced, aged, by the pending-approvals monitor (GOV-01).</t>
+        </is>
+      </c>
+      <c r="H118" s="13" t="inlineStr">
+        <is>
+          <t>Prev</t>
+        </is>
+      </c>
+      <c r="I118" s="13" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="J118" s="13" t="inlineStr">
+        <is>
+          <t>Per rate</t>
+        </is>
+      </c>
+      <c r="K118" s="12" t="inlineStr">
+        <is>
+          <t>Controller / Treasury</t>
+        </is>
+      </c>
+      <c r="L118" s="13" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="M118" s="12" t="inlineStr">
+        <is>
+          <t>fx.service.ts setRate(manual→PendingApproval)/approveRate/rejectRate/rateAsOf(Approved only); fx.controller.ts (rates/approve|reject|pending gated approvals/gl_close); consolidation.service.ts (translation reads Approved rates); schema/fx.ts fx_rates.status + migration 0141; cutover/fxreval.ts (ToE)</t>
+        </is>
+      </c>
+      <c r="N118" s="12" t="inlineStr">
+        <is>
+          <t>Inspect the request→approve flow + the approver≠requester check + that revaluation/reporting resolve Approved rates only.</t>
+        </is>
+      </c>
+      <c r="O118" s="12" t="inlineStr">
+        <is>
+          <t>Re-perform: enter a manual rate (PendingApproval), confirm revalue is blocked NO_RATE while pending, attempt self-approve (SOD_VIOLATION), approve as a different user, then revalue succeeds (re-performed by the fxreval harness).</t>
+        </is>
+      </c>
+      <c r="P118" s="12" t="inlineStr">
+        <is>
+          <t>FX rate approval log + SoD test</t>
+        </is>
+      </c>
+      <c r="Q118" s="18" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="15" t="inlineStr">
+        <is>
           <t>BUD-01</t>
         </is>
       </c>
-      <c r="B118" s="12" t="inlineStr">
+      <c r="B119" s="16" t="inlineStr">
         <is>
           <t>Budgeting &amp; Planning</t>
         </is>
       </c>
-      <c r="C118" s="13" t="inlineStr">
+      <c r="C119" s="17" t="inlineStr">
         <is>
           <t>Application</t>
         </is>
       </c>
-      <c r="D118" s="12" t="inlineStr">
+      <c r="D119" s="16" t="inlineStr">
         <is>
           <t>Budget; All (variance reporting)</t>
         </is>
       </c>
-      <c r="E118" s="12" t="inlineStr">
+      <c r="E119" s="16" t="inlineStr">
         <is>
           <t>A budget figure is entered/changed by one person and immediately drives the budget-vs-actual variance report — the basis for spend authorization and performance review — with no independent approval; a wrong or self-serving budget makes overspending look 'on budget'.</t>
         </is>
       </c>
-      <c r="F118" s="12" t="inlineStr">
+      <c r="F119" s="16" t="inlineStr">
         <is>
           <t>Authorization/Accuracy</t>
         </is>
       </c>
-      <c r="G118" s="12" t="inlineStr">
+      <c r="G119" s="16" t="inlineStr">
         <is>
           <t>Budget maker-checker (SoD): an upserted budget (POST /api/ledger/budgets) lands as PendingApproval and is EXCLUDED from budget-vs-actual until a DIFFERENT user approves it (POST /api/ledger/budgets/approve for the fiscal_year/account/cost-centre[/period]). Self-approval → SOD_VIOLATION (binds even Admin); reject marks it Rejected (excluded). DEFAULT 'Approved' keeps existing rows + direct planning seeds usable. Pending budgets are also surfaced, aged, by the pending-approvals monitor (GOV-01).</t>
         </is>
       </c>
-      <c r="H118" s="13" t="inlineStr">
+      <c r="H119" s="17" t="inlineStr">
         <is>
           <t>Prev</t>
         </is>
       </c>
-      <c r="I118" s="13" t="inlineStr">
+      <c r="I119" s="17" t="inlineStr">
         <is>
           <t>Automated</t>
         </is>
       </c>
-      <c r="J118" s="13" t="inlineStr">
+      <c r="J119" s="17" t="inlineStr">
         <is>
           <t>Per budget</t>
         </is>
       </c>
-      <c r="K118" s="12" t="inlineStr">
+      <c r="K119" s="16" t="inlineStr">
         <is>
           <t>Controller / FP&amp;A</t>
         </is>
       </c>
-      <c r="L118" s="13" t="inlineStr">
+      <c r="L119" s="17" t="inlineStr">
         <is>
           <t>P10</t>
         </is>
       </c>
-      <c r="M118" s="12" t="inlineStr">
+      <c r="M119" s="16" t="inlineStr">
         <is>
           <t>budget.service.ts upsertBudget(→PendingApproval)/approveBudget/rejectBudget/budgetVsActual(Approved only); budget.controller.ts (budgets/approve|reject|pending gated approvals/gl_close); schema/budgets.ts budgets.status + migration 0142; cutover/budget.ts (ToE)</t>
         </is>
       </c>
-      <c r="N118" s="12" t="inlineStr">
+      <c r="N119" s="16" t="inlineStr">
         <is>
           <t>Inspect the request→approve flow + the approver≠requester check + that budget-vs-actual counts Approved budgets only.</t>
         </is>
       </c>
-      <c r="O118" s="12" t="inlineStr">
+      <c r="O119" s="16" t="inlineStr">
         <is>
           <t>Re-perform: upsert a budget (PendingApproval, excluded from variance), attempt self-approve (SOD_VIOLATION), approve as a different user, confirm it then appears in budget-vs-actual (re-performed by the budget harness).</t>
         </is>
       </c>
-      <c r="P118" s="12" t="inlineStr">
+      <c r="P119" s="16" t="inlineStr">
         <is>
           <t>Budget approval log + SoD test</t>
         </is>
       </c>
-      <c r="Q118" s="18" t="inlineStr">
+      <c r="Q119" s="18" t="inlineStr">
         <is>
           <t>Implemented</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q118"/>
+  <autoFilter ref="A1:Q119"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -12330,7 +12417,7 @@
         </is>
       </c>
       <c r="C5" s="29">
-        <f>COUNTIF(RCM!$Q$2:$Q$118,B5)</f>
+        <f>COUNTIF(RCM!$Q$2:$Q$119,B5)</f>
         <v/>
       </c>
     </row>
@@ -12341,7 +12428,7 @@
         </is>
       </c>
       <c r="C6" s="29">
-        <f>COUNTIF(RCM!$Q$2:$Q$118,B6)</f>
+        <f>COUNTIF(RCM!$Q$2:$Q$119,B6)</f>
         <v/>
       </c>
     </row>
@@ -12352,7 +12439,7 @@
         </is>
       </c>
       <c r="C7" s="29">
-        <f>COUNTIF(RCM!$Q$2:$Q$118,B7)</f>
+        <f>COUNTIF(RCM!$Q$2:$Q$119,B7)</f>
         <v/>
       </c>
     </row>
@@ -12363,7 +12450,7 @@
         </is>
       </c>
       <c r="C8" s="32">
-        <f>COUNTA(RCM!$A$2:$A$118)</f>
+        <f>COUNTA(RCM!$A$2:$A$119)</f>
         <v/>
       </c>
     </row>
@@ -12381,7 +12468,7 @@
         </is>
       </c>
       <c r="C11" s="29">
-        <f>COUNTIF(RCM!$C$2:$C$118,B11)</f>
+        <f>COUNTIF(RCM!$C$2:$C$119,B11)</f>
         <v/>
       </c>
     </row>
@@ -12392,7 +12479,7 @@
         </is>
       </c>
       <c r="C12" s="29">
-        <f>COUNTIF(RCM!$C$2:$C$118,B12)</f>
+        <f>COUNTIF(RCM!$C$2:$C$119,B12)</f>
         <v/>
       </c>
     </row>
@@ -12403,7 +12490,7 @@
         </is>
       </c>
       <c r="C13" s="29">
-        <f>COUNTIF(RCM!$C$2:$C$118,B13)</f>
+        <f>COUNTIF(RCM!$C$2:$C$119,B13)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(gl): WS2.1 — hard period close + checklist (GL-15, GL-16)
- close_runs + close_run_steps tables (migration 0162) + RLS;
  'Locked' added to period_status enum
- CloseService: startClose (seeds 6-step checklist), completeStep
  (→ReadyToLock when required steps done), lockPeriod (STEPS_INCOMPLETE
  gate + SELF_LOCK maker-checker, sets fiscal_periods.status=Locked)
- postEntry: additive hard PERIOD_LOCKED gate (stronger than soft
  PERIOD_CLOSED); only source='CLOSE' year-end entry exempt
- Controller POST start/step/lock, GET status/list (perm gl_close)
- basics 170/170, worldclass 57/57 green
- GL-15/GL-16 RCM (120 controls); narrative §2.1 + user-manual + UAT

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/compliance/Oshinei_ERP_SOX_RCM_v1.xlsx
+++ b/compliance/Oshinei_ERP_SOX_RCM_v1.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'RCM'!$A$1:$Q$119</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'RCM'!$A$1:$Q$121</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Gap Remediation'!$A$2:$H$18</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -858,7 +858,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q119"/>
+  <dimension ref="A1:Q121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -9061,12 +9061,12 @@
     <row r="95">
       <c r="A95" s="15" t="inlineStr">
         <is>
-          <t>EXP-07</t>
+          <t>GL-15</t>
         </is>
       </c>
       <c r="B95" s="16" t="inlineStr">
         <is>
-          <t>Expenditure</t>
+          <t>General Ledger</t>
         </is>
       </c>
       <c r="C95" s="17" t="inlineStr">
@@ -9076,27 +9076,27 @@
       </c>
       <c r="D95" s="16" t="inlineStr">
         <is>
-          <t>Cash; Operating expense</t>
+          <t>All</t>
         </is>
       </c>
       <c r="E95" s="16" t="inlineStr">
         <is>
-          <t>Petty-cash / employee advance issued but never accounted for — cash leakage, expense unrecorded.</t>
+          <t>A period is 'closed' on paper but key close procedures (sub-ledger tie-out, bank rec, depreciation, recurring/prepaid, trial-balance review) were skipped, OR a closed period is silently re-opened and re-posted — the financial statements are produced on an incomplete/altered basis.</t>
         </is>
       </c>
       <c r="F95" s="16" t="inlineStr">
         <is>
-          <t>Existence/Completeness</t>
+          <t>Completeness/Accuracy/Cutoff</t>
         </is>
       </c>
       <c r="G95" s="16" t="inlineStr">
         <is>
-          <t>Employee cash advances: issuing an advance debits the 1180 Employee Advances control (Dr 1180 / Cr 1000); settlement clears it against actual spend + returned cash (Dr expense + Dr 1000 / Cr 1180), enforced to reconcile (settled_expense + returned_cash must equal the advance → SETTLE_MISMATCH). The 1180 balance is the outstanding float subject to review.</t>
+          <t>Hard period close + checklist: POST /api/ledger/close/start opens a close_runs record (status InProgress) per (tenant, period) and seeds a standard checklist of close_run_steps (subledger_tieout, bank_rec, depreciation, recurring, fx_reval[advisory], trial_balance_review). POST /api/ledger/close/step marks a step Done (records completedBy/At); when all REQUIRED steps are Done the run advances to ReadyToLock. POST /api/ledger/close/lock requires ReadyToLock (else STEPS_INCOMPLETE listing the pending required steps) before the period can be locked. Locking writes 'Locked' into fiscal_periods.status; LedgerService.postEntry then REJECTS every posting dated into a Locked period with PERIOD_LOCKED, regardless of the legacy allowClosedPeriod escape (the only exception is the system year-end closing entry, source='CLOSE'). Locked is strictly stronger than the soft 'Closed' status — it is the irreversible hard close.</t>
         </is>
       </c>
       <c r="H95" s="17" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I95" s="17" t="inlineStr">
@@ -9106,12 +9106,12 @@
       </c>
       <c r="J95" s="17" t="inlineStr">
         <is>
-          <t>Per advance</t>
+          <t>Monthly</t>
         </is>
       </c>
       <c r="K95" s="16" t="inlineStr">
         <is>
-          <t>AP / Controller</t>
+          <t>Financial Controller</t>
         </is>
       </c>
       <c r="L95" s="17" t="inlineStr">
@@ -9121,22 +9121,22 @@
       </c>
       <c r="M95" s="16" t="inlineStr">
         <is>
-          <t>finance.service.ts (issueAdvance, settleAdvance reconcile-or-reject, listAdvances outstanding); finance.controller.ts (creditors/exec); schema/finance.ts (employee_advances) + migration 0120; cutover/basics.ts (ToE)</t>
+          <t>close.service.ts (startClose seeds checklist, completeStep → ReadyToLock when required steps Done, lockPeriod STEPS_INCOMPLETE gate + fiscal_periods Locked write, status/list); close.controller.ts (gl_close start/step/lock, gl_close/gl_post/exec read); schema/close-runs.ts (close_runs + close_run_steps, uq on tenant/period and run/step_key); schema/ledger.ts (period_status enum + 'Locked'); ledger.service.ts (postEntry PERIOD_LOCKED hard gate, source='CLOSE' exemption); migration 0162 (tables + RLS + ALTER TYPE Locked); ledger.module.ts (service+controller wired); cutover/basics.ts (GL-15/GL-16 ToE)</t>
         </is>
       </c>
       <c r="N95" s="16" t="inlineStr">
         <is>
-          <t>Inspect issue/settle GL + settlement reconciliation guard.</t>
+          <t>Inspect the seeded checklist + ReadyToLock gating + STEPS_INCOMPLETE lock rejection + PERIOD_LOCKED hard gate in postEntry (incl. the CLOSE exemption).</t>
         </is>
       </c>
       <c r="O95" s="16" t="inlineStr">
         <is>
-          <t>Issue an advance (1180 up); settle 700+300 clears 1180; mismatched settle → SETTLE_MISMATCH (re-performed by the harness).</t>
+          <t>TC-GL-15-01: start close seeds ≥4 steps (InProgress); TC-GL-15-02: lock before steps done → STEPS_INCOMPLETE (400); TC-GL-15-03: post into locked period → PERIOD_LOCKED (400) (re-performed by the basics.ts harness).</t>
         </is>
       </c>
       <c r="P95" s="16" t="inlineStr">
         <is>
-          <t>Advance register; outstanding float</t>
+          <t>close_runs / close_run_steps with completion trail; fiscal_periods.status=Locked; monthly close sign-off</t>
         </is>
       </c>
       <c r="Q95" s="18" t="inlineStr">
@@ -9148,12 +9148,12 @@
     <row r="96">
       <c r="A96" s="11" t="inlineStr">
         <is>
-          <t>EXP-08</t>
+          <t>GL-16</t>
         </is>
       </c>
       <c r="B96" s="12" t="inlineStr">
         <is>
-          <t>Expenditure</t>
+          <t>General Ledger</t>
         </is>
       </c>
       <c r="C96" s="13" t="inlineStr">
@@ -9163,22 +9163,22 @@
       </c>
       <c r="D96" s="12" t="inlineStr">
         <is>
-          <t>Cash; Operating expense</t>
+          <t>All</t>
         </is>
       </c>
       <c r="E96" s="12" t="inlineStr">
         <is>
-          <t>Petty-cash disbursed beyond authority / without independent review, or drawn past the fund's limit — cash leakage, unauthorised or unrecorded expense, over-extended float.</t>
+          <t>One person both performs the close and locks the period, defeating segregation of duties — a preparer could conceal a misstatement by closing over their own work without independent review.</t>
         </is>
       </c>
       <c r="F96" s="12" t="inlineStr">
         <is>
-          <t>Authorization; Completeness</t>
+          <t>Authorization/Segregation of Duties</t>
         </is>
       </c>
       <c r="G96" s="12" t="inlineStr">
         <is>
-          <t>Petty-cash imprest float + maker-checker on disbursement (SoD): a fund holds cash capped at a credit limit/วงเงิน (1015 Petty Cash, a cash account); each direct EXPENSE or ADVANCE is a REQUEST that posts NOTHING and a DIFFERENT user must approve before the GL posts (expense Dr &lt;expense&gt; / Cr 1015; advance Dr 1180 / Cr 1015) and the fund balance is decremented. Self-approval → SOD_VIOLATION (binds even Admin). A draw beyond the fund balance → INSUFFICIENT_FLOAT; establishing/replenishing above the float limit → OVER_FLOAT. Advances settle (Dr expense + Dr 1015 returned / Cr 1180), returning unused cash to the fund. Every request carries a document reference + receipt key + a status trail (StatusLog) and surfaces in the GOV-01 pending-approvals monitor.</t>
+          <t>Segregated period lock (maker-checker): the close_runs.started_by (the user who started the close and ran the checklist steps) is recorded, and POST /api/ledger/close/lock REJECTS a lockedBy equal to startedBy with SELF_LOCK — the gl_close user who locks the period MUST differ from the user who started/ran the close. Both identities and the lock timestamp are retained on the close_runs row (started_by / locked_by / locked_at) as the SoD evidence trail. This complements the existing SoD rule that gl_close is segregated from gl_post (JE posting).</t>
         </is>
       </c>
       <c r="H96" s="13" t="inlineStr">
@@ -9193,12 +9193,12 @@
       </c>
       <c r="J96" s="13" t="inlineStr">
         <is>
-          <t>Per disbursement</t>
+          <t>Monthly</t>
         </is>
       </c>
       <c r="K96" s="12" t="inlineStr">
         <is>
-          <t>AP / Controller</t>
+          <t>Financial Controller</t>
         </is>
       </c>
       <c r="L96" s="13" t="inlineStr">
@@ -9208,22 +9208,22 @@
       </c>
       <c r="M96" s="12" t="inlineStr">
         <is>
-          <t>petty-cash.service.ts (establishFund/replenishFund float guards, createRequest INSUFFICIENT_FLOAT, approveRequest SoD+GL, rejectRequest, settleRequest); petty-cash.controller.ts (creditors/exec); schema/petty-cash.ts (petty_cash_funds, expense_requests) + migration 0139; finance.service.ts pendingApprovals (GOV-01 source 7); cutover/basics.ts + compliance.ts (ToE)</t>
+          <t>close.service.ts (lockPeriod SELF_LOCK maker-checker gate; started_by vs locked_by); close.controller.ts (gl_close lock, acting username from JWT); schema/close-runs.ts (started_by, locked_by, locked_at columns); permissions.ts (gl_post×gl_close SoD pair); cutover/basics.ts (GL-16 ToE)</t>
         </is>
       </c>
       <c r="N96" s="12" t="inlineStr">
         <is>
-          <t>Inspect the float ceiling + the request→approve flow + the approver≠requester check + that the request posts nothing until approval.</t>
+          <t>Inspect the SELF_LOCK gate (startedBy ≠ lockedBy) + the started_by/locked_by/locked_at evidence trail.</t>
         </is>
       </c>
       <c r="O96" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: establish a fund (Dr 1015), request an expense (no GL), self-approve → SOD_VIOLATION, approve as a different user → Dr expense/Cr 1015 + fund down; over-balance draw → INSUFFICIENT_FLOAT; advance approve→settle clears 1180; replenish past float → OVER_FLOAT (re-performed by the harnesses).</t>
+          <t>TC-GL-16-01: self-lock by the starter → SELF_LOCK (400); TC-GL-16-02: lock by a different gl_close user → Locked, locked_by recorded (re-performed by the basics.ts harness).</t>
         </is>
       </c>
       <c r="P96" s="12" t="inlineStr">
         <is>
-          <t>Fund register + disbursement approval log + SoD test</t>
+          <t>close_runs.started_by / locked_by / locked_at SoD trail; monthly close sign-off</t>
         </is>
       </c>
       <c r="Q96" s="18" t="inlineStr">
@@ -9235,12 +9235,12 @@
     <row r="97">
       <c r="A97" s="15" t="inlineStr">
         <is>
-          <t>FA-07</t>
+          <t>EXP-07</t>
         </is>
       </c>
       <c r="B97" s="16" t="inlineStr">
         <is>
-          <t>Fixed Assets</t>
+          <t>Expenditure</t>
         </is>
       </c>
       <c r="C97" s="17" t="inlineStr">
@@ -9250,22 +9250,22 @@
       </c>
       <c r="D97" s="16" t="inlineStr">
         <is>
-          <t>Property, Plant &amp; Equipment; Equity</t>
+          <t>Cash; Operating expense</t>
         </is>
       </c>
       <c r="E97" s="16" t="inlineStr">
         <is>
-          <t>Carrying amount not adjusted for revaluation/impairment — asset over/understated.</t>
+          <t>Petty-cash / employee advance issued but never accounted for — cash leakage, expense unrecorded.</t>
         </is>
       </c>
       <c r="F97" s="16" t="inlineStr">
         <is>
-          <t>Valuation</t>
+          <t>Existence/Completeness</t>
         </is>
       </c>
       <c r="G97" s="16" t="inlineStr">
         <is>
-          <t>Asset revaluation / impairment: an upward revaluation credits the revaluation surplus in equity (Dr 1500 / Cr 3200); a downward revaluation (impairment) debits impairment loss (Dr 5820 / Cr 1500). The gross 1500 moves by the delta so the register stays tied to the GL; a no-op revaluation is rejected (NO_CHANGE). Every event is logged for the audit trail.</t>
+          <t>Employee cash advances: issuing an advance debits the 1180 Employee Advances control (Dr 1180 / Cr 1000); settlement clears it against actual spend + returned cash (Dr expense + Dr 1000 / Cr 1180), enforced to reconcile (settled_expense + returned_cash must equal the advance → SETTLE_MISMATCH). The 1180 balance is the outstanding float subject to review.</t>
         </is>
       </c>
       <c r="H97" s="17" t="inlineStr">
@@ -9280,12 +9280,12 @@
       </c>
       <c r="J97" s="17" t="inlineStr">
         <is>
-          <t>Per event</t>
+          <t>Per advance</t>
         </is>
       </c>
       <c r="K97" s="16" t="inlineStr">
         <is>
-          <t>FaAccountant / Controller</t>
+          <t>AP / Controller</t>
         </is>
       </c>
       <c r="L97" s="17" t="inlineStr">
@@ -9295,22 +9295,22 @@
       </c>
       <c r="M97" s="16" t="inlineStr">
         <is>
-          <t>assets.service.ts (revalue up→3200 / down→5820, listRevaluations; dispose recycles surplus 3200→3100); assets.controller.ts (exec/creditors); schema/assets.ts (asset_revaluations) + migration 0120; cutover/basics.ts (ToE)</t>
+          <t>finance.service.ts (issueAdvance, settleAdvance reconcile-or-reject, listAdvances outstanding); finance.controller.ts (creditors/exec); schema/finance.ts (employee_advances) + migration 0120; cutover/basics.ts (ToE)</t>
         </is>
       </c>
       <c r="N97" s="16" t="inlineStr">
         <is>
-          <t>Inspect revaluation/impairment routing + audit log + disposal recycling.</t>
+          <t>Inspect issue/settle GL + settlement reconciliation guard.</t>
         </is>
       </c>
       <c r="O97" s="16" t="inlineStr">
         <is>
-          <t>Upward revaluation credits 3200; impairment debits 5820; no-change → NO_CHANGE; both events logged; on disposal the revaluation surplus is recycled to retained earnings (Dr 3200 / Cr 3100), not through P&amp;L (re-performed by the harness).</t>
+          <t>Issue an advance (1180 up); settle 700+300 clears 1180; mismatched settle → SETTLE_MISMATCH (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P97" s="16" t="inlineStr">
         <is>
-          <t>Revaluation log; disposal recycling JE</t>
+          <t>Advance register; outstanding float</t>
         </is>
       </c>
       <c r="Q97" s="18" t="inlineStr">
@@ -9322,12 +9322,12 @@
     <row r="98">
       <c r="A98" s="11" t="inlineStr">
         <is>
-          <t>FA-08</t>
+          <t>EXP-08</t>
         </is>
       </c>
       <c r="B98" s="12" t="inlineStr">
         <is>
-          <t>Fixed Assets</t>
+          <t>Expenditure</t>
         </is>
       </c>
       <c r="C98" s="13" t="inlineStr">
@@ -9337,22 +9337,22 @@
       </c>
       <c r="D98" s="12" t="inlineStr">
         <is>
-          <t>Property, Plant &amp; Equipment; Equity</t>
+          <t>Cash; Operating expense</t>
         </is>
       </c>
       <c r="E98" s="12" t="inlineStr">
         <is>
-          <t>Carrying amount changed by fair-value revaluation/impairment without independent review — the preparer revalues the asset and posts to equity/P&amp;L on their own (earnings/equity management).</t>
+          <t>Petty-cash disbursed beyond authority / without independent review, or drawn past the fund's limit — cash leakage, unauthorised or unrecorded expense, over-extended float.</t>
         </is>
       </c>
       <c r="F98" s="12" t="inlineStr">
         <is>
-          <t>Authorization</t>
+          <t>Authorization; Completeness</t>
         </is>
       </c>
       <c r="G98" s="12" t="inlineStr">
         <is>
-          <t>Asset-revaluation maker-checker (SoD): a revalue/impairment request posts its GL entry as a DRAFT (excluded from balances) and records status 'PendingApproval' WITHOUT moving the carrying value; a DIFFERENT user must approve before the JE is effective and the register is re-valued (approver ≠ preparer enforced regardless of permissions, reusing the GL-05 ledger approval). Reject voids the draft; only one revaluation may be pending per asset; the disposal surplus recycle counts only approved revaluations.</t>
+          <t>Petty-cash imprest float + maker-checker on disbursement (SoD): a fund holds cash capped at a credit limit/วงเงิน (1015 Petty Cash, a cash account); each direct EXPENSE or ADVANCE is a REQUEST that posts NOTHING and a DIFFERENT user must approve before the GL posts (expense Dr &lt;expense&gt; / Cr 1015; advance Dr 1180 / Cr 1015) and the fund balance is decremented. Self-approval → SOD_VIOLATION (binds even Admin). A draw beyond the fund balance → INSUFFICIENT_FLOAT; establishing/replenishing above the float limit → OVER_FLOAT. Advances settle (Dr expense + Dr 1015 returned / Cr 1180), returning unused cash to the fund. Every request carries a document reference + receipt key + a status trail (StatusLog) and surfaces in the GOV-01 pending-approvals monitor.</t>
         </is>
       </c>
       <c r="H98" s="13" t="inlineStr">
@@ -9367,12 +9367,12 @@
       </c>
       <c r="J98" s="13" t="inlineStr">
         <is>
-          <t>Per event</t>
+          <t>Per disbursement</t>
         </is>
       </c>
       <c r="K98" s="12" t="inlineStr">
         <is>
-          <t>FaAccountant / Controller</t>
+          <t>AP / Controller</t>
         </is>
       </c>
       <c r="L98" s="13" t="inlineStr">
@@ -9382,22 +9382,22 @@
       </c>
       <c r="M98" s="12" t="inlineStr">
         <is>
-          <t>assets.service.ts revalue(pendingApproval Draft)/approveRevaluation/rejectRevaluation; assets.controller.ts (:assetNo/revalue/approve|reject); schema/assets.ts asset_revaluations.status + migration 0134; cutover/basics.ts + compliance.ts (ToE)</t>
+          <t>petty-cash.service.ts (establishFund/replenishFund float guards, createRequest INSUFFICIENT_FLOAT, approveRequest SoD+GL, rejectRequest, settleRequest); petty-cash.controller.ts (creditors/exec); schema/petty-cash.ts (petty_cash_funds, expense_requests) + migration 0139; finance.service.ts pendingApprovals (GOV-01 source 7); cutover/basics.ts + compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N98" s="12" t="inlineStr">
         <is>
-          <t>Inspect Draft→approve flow + the approver≠preparer check + deferred carrying-value update.</t>
+          <t>Inspect the float ceiling + the request→approve flow + the approver≠requester check + that the request posts nothing until approval.</t>
         </is>
       </c>
       <c r="O98" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: request a revaluation (Draft JE excluded from 3200), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm the surplus/impairment + carrying value move only after approval (re-performed by the harnesses).</t>
+          <t>Re-perform: establish a fund (Dr 1015), request an expense (no GL), self-approve → SOD_VIOLATION, approve as a different user → Dr expense/Cr 1015 + fund down; over-balance draw → INSUFFICIENT_FLOAT; advance approve→settle clears 1180; replenish past float → OVER_FLOAT (re-performed by the harnesses).</t>
         </is>
       </c>
       <c r="P98" s="12" t="inlineStr">
         <is>
-          <t>Revaluation approval log + SoD test</t>
+          <t>Fund register + disbursement approval log + SoD test</t>
         </is>
       </c>
       <c r="Q98" s="18" t="inlineStr">
@@ -9409,12 +9409,12 @@
     <row r="99">
       <c r="A99" s="15" t="inlineStr">
         <is>
-          <t>LSE-01</t>
+          <t>FA-07</t>
         </is>
       </c>
       <c r="B99" s="16" t="inlineStr">
         <is>
-          <t>Leases</t>
+          <t>Fixed Assets</t>
         </is>
       </c>
       <c r="C99" s="17" t="inlineStr">
@@ -9424,22 +9424,22 @@
       </c>
       <c r="D99" s="16" t="inlineStr">
         <is>
-          <t>Right-of-use assets; Lease liabilities</t>
+          <t>Property, Plant &amp; Equipment; Equity</t>
         </is>
       </c>
       <c r="E99" s="16" t="inlineStr">
         <is>
-          <t>Lease not capitalised (IFRS 16 / TFRS 16) — ROU asset + lease liability omitted; interest/depreciation mis-stated.</t>
+          <t>Carrying amount not adjusted for revaluation/impairment — asset over/understated.</t>
         </is>
       </c>
       <c r="F99" s="16" t="inlineStr">
         <is>
-          <t>Completeness/Accuracy/Valuation</t>
+          <t>Valuation</t>
         </is>
       </c>
       <c r="G99" s="16" t="inlineStr">
         <is>
-          <t>Lease accounting: at commencement a right-of-use asset and lease liability are recognised at the present value of the lease payments (Dr 1600 / Cr 2600). The scheduled job lease_periodic_run posts each period — interest unwinding on the liability (Dr 5900), the cash payment reducing the liability (Dr 2600 / Cr 1000), and straight-line ROU depreciation (Dr 5210 / Cr 1690) — the last period clearing the liability + ROU exactly. Idempotent per (lease, period).</t>
+          <t>Asset revaluation / impairment: an upward revaluation credits the revaluation surplus in equity (Dr 1500 / Cr 3200); a downward revaluation (impairment) debits impairment loss (Dr 5820 / Cr 1500). The gross 1500 moves by the delta so the register stays tied to the GL; a no-op revaluation is rejected (NO_CHANGE). Every event is logged for the audit trail.</t>
         </is>
       </c>
       <c r="H99" s="17" t="inlineStr">
@@ -9454,12 +9454,12 @@
       </c>
       <c r="J99" s="17" t="inlineStr">
         <is>
-          <t>Per period / per lease</t>
+          <t>Per event</t>
         </is>
       </c>
       <c r="K99" s="16" t="inlineStr">
         <is>
-          <t>Controller</t>
+          <t>FaAccountant / Controller</t>
         </is>
       </c>
       <c r="L99" s="17" t="inlineStr">
@@ -9469,22 +9469,22 @@
       </c>
       <c r="M99" s="16" t="inlineStr">
         <is>
-          <t>leases.service.ts (createLease PV recognition, runDueLeases interest+payment+depreciation, modifyLease remeasurement); leases.controller.ts (gl_post); bi.service.ts (lease_periodic_run); schema/leases.ts (leases, rou_nbv) + migration 0120/0121; cutover/basics.ts (ToE)</t>
+          <t>assets.service.ts (revalue up→3200 / down→5820, listRevaluations; dispose recycles surplus 3200→3100); assets.controller.ts (exec/creditors); schema/assets.ts (asset_revaluations) + migration 0120; cutover/basics.ts (ToE)</t>
         </is>
       </c>
       <c r="N99" s="16" t="inlineStr">
         <is>
-          <t>Inspect PV recognition + periodic interest/payment/depreciation + final-period clearing + modification remeasurement.</t>
+          <t>Inspect revaluation/impairment routing + audit log + disposal recycling.</t>
         </is>
       </c>
       <c r="O99" s="16" t="inlineStr">
         <is>
-          <t>Commencement recognises ROU=liability=PV; periodic run posts interest+principal(=payment)+ROU depreciation; liability + ROU reduce; a modification remeasures the liability at the revised PV and adjusts the ROU by the same delta (Dr/Cr 1600↔2600), then depreciates over the remaining term (re-performed by the harness).</t>
+          <t>Upward revaluation credits 3200; impairment debits 5820; no-change → NO_CHANGE; both events logged; on disposal the revaluation surplus is recycled to retained earnings (Dr 3200 / Cr 3100), not through P&amp;L (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P99" s="16" t="inlineStr">
         <is>
-          <t>Lease register; periodic run log; modification remeasurement</t>
+          <t>Revaluation log; disposal recycling JE</t>
         </is>
       </c>
       <c r="Q99" s="18" t="inlineStr">
@@ -9496,12 +9496,12 @@
     <row r="100">
       <c r="A100" s="11" t="inlineStr">
         <is>
-          <t>REC-01</t>
+          <t>FA-08</t>
         </is>
       </c>
       <c r="B100" s="12" t="inlineStr">
         <is>
-          <t>Reconciliation</t>
+          <t>Fixed Assets</t>
         </is>
       </c>
       <c r="C100" s="13" t="inlineStr">
@@ -9511,67 +9511,67 @@
       </c>
       <c r="D100" s="12" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Property, Plant &amp; Equipment; Equity</t>
         </is>
       </c>
       <c r="E100" s="12" t="inlineStr">
         <is>
-          <t>Subledgers diverge from GL undetected.</t>
+          <t>Carrying amount changed by fair-value revaluation/impairment without independent review — the preparer revalues the asset and posts to equity/P&amp;L on their own (earnings/equity management).</t>
         </is>
       </c>
       <c r="F100" s="12" t="inlineStr">
         <is>
-          <t>Completeness/Accuracy</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="G100" s="12" t="inlineStr">
         <is>
-          <t>Subledger-to-GL reconciliation per period: import GL, auto-match, certify (sign-off via 'approvals').</t>
+          <t>Asset-revaluation maker-checker (SoD): a revalue/impairment request posts its GL entry as a DRAFT (excluded from balances) and records status 'PendingApproval' WITHOUT moving the carrying value; a DIFFERENT user must approve before the JE is effective and the register is re-valued (approver ≠ preparer enforced regardless of permissions, reusing the GL-05 ledger approval). Reject voids the draft; only one revaluation may be pending per asset; the disposal surplus recycle counts only approved revaluations.</t>
         </is>
       </c>
       <c r="H100" s="13" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I100" s="13" t="inlineStr">
         <is>
-          <t>Auto+Manual</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J100" s="13" t="inlineStr">
         <is>
-          <t>Monthly</t>
+          <t>Per event</t>
         </is>
       </c>
       <c r="K100" s="12" t="inlineStr">
         <is>
-          <t>Controller</t>
+          <t>FaAccountant / Controller</t>
         </is>
       </c>
       <c r="L100" s="13" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="M100" s="12" t="inlineStr">
         <is>
-          <t>reconciliation.service.ts (importGlItems/autoMatch/certify)</t>
+          <t>assets.service.ts revalue(pendingApproval Draft)/approveRevaluation/rejectRevaluation; assets.controller.ts (:assetNo/revalue/approve|reject); schema/assets.ts asset_revaluations.status + migration 0134; cutover/basics.ts + compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N100" s="12" t="inlineStr">
         <is>
-          <t>Inspect recon + certify gate.</t>
+          <t>Inspect Draft→approve flow + the approver≠preparer check + deferred carrying-value update.</t>
         </is>
       </c>
       <c r="O100" s="12" t="inlineStr">
         <is>
-          <t>Sample periods: reconciled, unmatched cleared, certified.</t>
+          <t>Re-perform: request a revaluation (Draft JE excluded from 3200), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm the surplus/impairment + carrying value move only after approval (re-performed by the harnesses).</t>
         </is>
       </c>
       <c r="P100" s="12" t="inlineStr">
         <is>
-          <t>Certified recon</t>
+          <t>Revaluation approval log + SoD test</t>
         </is>
       </c>
       <c r="Q100" s="18" t="inlineStr">
@@ -9583,12 +9583,12 @@
     <row r="101">
       <c r="A101" s="15" t="inlineStr">
         <is>
-          <t>REC-02</t>
+          <t>LSE-01</t>
         </is>
       </c>
       <c r="B101" s="16" t="inlineStr">
         <is>
-          <t>Reconciliation</t>
+          <t>Leases</t>
         </is>
       </c>
       <c r="C101" s="17" t="inlineStr">
@@ -9598,22 +9598,22 @@
       </c>
       <c r="D101" s="16" t="inlineStr">
         <is>
-          <t>Cash</t>
+          <t>Right-of-use assets; Lease liabilities</t>
         </is>
       </c>
       <c r="E101" s="16" t="inlineStr">
         <is>
-          <t>Bank balance not reconciled to GL.</t>
+          <t>Lease not capitalised (IFRS 16 / TFRS 16) — ROU asset + lease liability omitted; interest/depreciation mis-stated.</t>
         </is>
       </c>
       <c r="F101" s="16" t="inlineStr">
         <is>
-          <t>Existence/Completeness</t>
+          <t>Completeness/Accuracy/Valuation</t>
         </is>
       </c>
       <c r="G101" s="16" t="inlineStr">
         <is>
-          <t>Bank reconciliation against statements.</t>
+          <t>Lease accounting: at commencement a right-of-use asset and lease liability are recognised at the present value of the lease payments (Dr 1600 / Cr 2600). The scheduled job lease_periodic_run posts each period — interest unwinding on the liability (Dr 5900), the cash payment reducing the liability (Dr 2600 / Cr 1000), and straight-line ROU depreciation (Dr 5210 / Cr 1690) — the last period clearing the liability + ROU exactly. Idempotent per (lease, period).</t>
         </is>
       </c>
       <c r="H101" s="17" t="inlineStr">
@@ -9623,12 +9623,12 @@
       </c>
       <c r="I101" s="17" t="inlineStr">
         <is>
-          <t>Auto+Manual</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J101" s="17" t="inlineStr">
         <is>
-          <t>Monthly</t>
+          <t>Per period / per lease</t>
         </is>
       </c>
       <c r="K101" s="16" t="inlineStr">
@@ -9638,27 +9638,27 @@
       </c>
       <c r="L101" s="17" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="M101" s="16" t="inlineStr">
         <is>
-          <t>bank module; drizzle/0015_bank_reconciliation</t>
+          <t>leases.service.ts (createLease PV recognition, runDueLeases interest+payment+depreciation, modifyLease remeasurement); leases.controller.ts (gl_post); bi.service.ts (lease_periodic_run); schema/leases.ts (leases, rou_nbv) + migration 0120/0121; cutover/basics.ts (ToE)</t>
         </is>
       </c>
       <c r="N101" s="16" t="inlineStr">
         <is>
-          <t>Inspect bank-rec process.</t>
+          <t>Inspect PV recognition + periodic interest/payment/depreciation + final-period clearing + modification remeasurement.</t>
         </is>
       </c>
       <c r="O101" s="16" t="inlineStr">
         <is>
-          <t>Sample months reconciled &amp; reviewed.</t>
+          <t>Commencement recognises ROU=liability=PV; periodic run posts interest+principal(=payment)+ROU depreciation; liability + ROU reduce; a modification remeasures the liability at the revised PV and adjusts the ROU by the same delta (Dr/Cr 1600↔2600), then depreciates over the remaining term (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P101" s="16" t="inlineStr">
         <is>
-          <t>Bank rec</t>
+          <t>Lease register; periodic run log; modification remeasurement</t>
         </is>
       </c>
       <c r="Q101" s="18" t="inlineStr">
@@ -9670,12 +9670,12 @@
     <row r="102">
       <c r="A102" s="11" t="inlineStr">
         <is>
-          <t>BANK-02</t>
+          <t>REC-01</t>
         </is>
       </c>
       <c r="B102" s="12" t="inlineStr">
         <is>
-          <t>Cash &amp; Treasury</t>
+          <t>Reconciliation</t>
         </is>
       </c>
       <c r="C102" s="13" t="inlineStr">
@@ -9685,37 +9685,37 @@
       </c>
       <c r="D102" s="12" t="inlineStr">
         <is>
-          <t>Cash; Operating expense; Interest income</t>
+          <t>All</t>
         </is>
       </c>
       <c r="E102" s="12" t="inlineStr">
         <is>
-          <t>A bank fee/interest adjustment is posted straight to the GL by one person during reconciliation — a cash outflow mis-booked as interest income, or a fictitious fee posted, with no independent review (single-person posting to the cash account).</t>
+          <t>Subledgers diverge from GL undetected.</t>
         </is>
       </c>
       <c r="F102" s="12" t="inlineStr">
         <is>
-          <t>Authorization/Accuracy</t>
+          <t>Completeness/Accuracy</t>
         </is>
       </c>
       <c r="G102" s="12" t="inlineStr">
         <is>
-          <t>Bank adjustment maker-checker (SoD): a fee/interest adjustment on a statement line is a REQUEST that posts a DRAFT JE (no balance/GL effect; the line stays unreconciled) until a DIFFERENT user with approval authority approves (POST /api/bank/lines/:id/adjustment/approve). Self-approval → SOD_VIOLATION (binds even Admin); approval flips the line to reconciled and the JE to Posted; reject voids the Draft and frees the line. The Draft JE (source BANKADJ) is also surfaced, aged, by the pending-approvals monitor (GOV-01).</t>
+          <t>Subledger-to-GL reconciliation per period: import GL, auto-match, certify (sign-off via 'approvals').</t>
         </is>
       </c>
       <c r="H102" s="13" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I102" s="13" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="J102" s="13" t="inlineStr">
         <is>
-          <t>Per adjustment</t>
+          <t>Monthly</t>
         </is>
       </c>
       <c r="K102" s="12" t="inlineStr">
@@ -9725,27 +9725,27 @@
       </c>
       <c r="L102" s="13" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="M102" s="12" t="inlineStr">
         <is>
-          <t>bank.service.ts requestAdjustment/approveAdjustment/rejectAdjustment/listPendingAdjustments (reuses ledger.approveEntry SoD); bank.controller.ts (lines/:id/adjustment requests; adjustment/approve|reject gated approvals/gl_close); cutover/bankrec.ts (ToE)</t>
+          <t>reconciliation.service.ts (importGlItems/autoMatch/certify)</t>
         </is>
       </c>
       <c r="N102" s="12" t="inlineStr">
         <is>
-          <t>Inspect the request→approve flow + the approver≠requester check + that the Draft posts nothing until approval.</t>
+          <t>Inspect recon + certify gate.</t>
         </is>
       </c>
       <c r="O102" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: request a fee adjustment (line unreconciled, GL difference unchanged), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm the difference closes to 0 only after approval (re-performed by the bankrec harness).</t>
+          <t>Sample periods: reconciled, unmatched cleared, certified.</t>
         </is>
       </c>
       <c r="P102" s="12" t="inlineStr">
         <is>
-          <t>Bank adjustment queue + SoD test</t>
+          <t>Certified recon</t>
         </is>
       </c>
       <c r="Q102" s="18" t="inlineStr">
@@ -9757,7 +9757,7 @@
     <row r="103">
       <c r="A103" s="15" t="inlineStr">
         <is>
-          <t>REC-03</t>
+          <t>REC-02</t>
         </is>
       </c>
       <c r="B103" s="16" t="inlineStr">
@@ -9772,22 +9772,22 @@
       </c>
       <c r="D103" s="16" t="inlineStr">
         <is>
-          <t>Consolidation</t>
+          <t>Cash</t>
         </is>
       </c>
       <c r="E103" s="16" t="inlineStr">
         <is>
-          <t>Intercompany balances not eliminated/agreed.</t>
+          <t>Bank balance not reconciled to GL.</t>
         </is>
       </c>
       <c r="F103" s="16" t="inlineStr">
         <is>
-          <t>Accuracy</t>
+          <t>Existence/Completeness</t>
         </is>
       </c>
       <c r="G103" s="16" t="inlineStr">
         <is>
-          <t>Intercompany reconciliation &amp; elimination on consolidation.</t>
+          <t>Bank reconciliation against statements.</t>
         </is>
       </c>
       <c r="H103" s="17" t="inlineStr">
@@ -9802,12 +9802,12 @@
       </c>
       <c r="J103" s="17" t="inlineStr">
         <is>
-          <t>Period</t>
+          <t>Monthly</t>
         </is>
       </c>
       <c r="K103" s="16" t="inlineStr">
         <is>
-          <t>Group Controller</t>
+          <t>Controller</t>
         </is>
       </c>
       <c r="L103" s="17" t="inlineStr">
@@ -9817,39 +9817,39 @@
       </c>
       <c r="M103" s="16" t="inlineStr">
         <is>
-          <t>intercompany; consolidation</t>
+          <t>bank module; drizzle/0015_bank_reconciliation</t>
         </is>
       </c>
       <c r="N103" s="16" t="inlineStr">
         <is>
-          <t>Inspect IC matching + elimination.</t>
+          <t>Inspect bank-rec process.</t>
         </is>
       </c>
       <c r="O103" s="16" t="inlineStr">
         <is>
-          <t>Sample IC pairs agree &amp; eliminate.</t>
+          <t>Sample months reconciled &amp; reviewed.</t>
         </is>
       </c>
       <c r="P103" s="16" t="inlineStr">
         <is>
-          <t>IC recon</t>
-        </is>
-      </c>
-      <c r="Q103" s="19" t="inlineStr">
-        <is>
-          <t>Partial</t>
+          <t>Bank rec</t>
+        </is>
+      </c>
+      <c r="Q103" s="18" t="inlineStr">
+        <is>
+          <t>Implemented</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="11" t="inlineStr">
         <is>
-          <t>REC-04</t>
+          <t>BANK-02</t>
         </is>
       </c>
       <c r="B104" s="12" t="inlineStr">
         <is>
-          <t>Reconciliation</t>
+          <t>Cash &amp; Treasury</t>
         </is>
       </c>
       <c r="C104" s="13" t="inlineStr">
@@ -9859,27 +9859,27 @@
       </c>
       <c r="D104" s="12" t="inlineStr">
         <is>
-          <t>All control accounts</t>
+          <t>Cash; Operating expense; Interest income</t>
         </is>
       </c>
       <c r="E104" s="12" t="inlineStr">
         <is>
-          <t>A sub-ledger silently drifts from its GL control account at period-end and no single review catches it (incomplete/inaccurate balances reach the financial statements).</t>
+          <t>A bank fee/interest adjustment is posted straight to the GL by one person during reconciliation — a cash outflow mis-booked as interest income, or a fictitious fee posted, with no independent review (single-person posting to the cash account).</t>
         </is>
       </c>
       <c r="F104" s="12" t="inlineStr">
         <is>
-          <t>Completeness/Accuracy</t>
+          <t>Authorization/Accuracy</t>
         </is>
       </c>
       <c r="G104" s="12" t="inlineStr">
         <is>
-          <t>Period-end control-account reconciliation PACK: one read (GET /api/finance/reconciliation/controls) ties every major sub-ledger to its GL control account and FLAGS any out-of-balance — AR↔1100, AP↔2000, Inventory↔1200, Gift cards/Customer-deposits↔2200, Deferred revenue↔2400 — reporting per line {sub_ledger, gl_control, variance, reconciled} plus an overall all_reconciled flag and an exceptions count. Liability controls are sign-flipped before comparison. The controller's single 'are the books reconciled?' close view; an exception is a control finding to investigate before sign-off.</t>
+          <t>Bank adjustment maker-checker (SoD): a fee/interest adjustment on a statement line is a REQUEST that posts a DRAFT JE (no balance/GL effect; the line stays unreconciled) until a DIFFERENT user with approval authority approves (POST /api/bank/lines/:id/adjustment/approve). Self-approval → SOD_VIOLATION (binds even Admin); approval flips the line to reconciled and the JE to Posted; reject voids the Draft and frees the line. The Draft JE (source BANKADJ) is also surfaced, aged, by the pending-approvals monitor (GOV-01).</t>
         </is>
       </c>
       <c r="H104" s="13" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I104" s="13" t="inlineStr">
@@ -9889,37 +9889,37 @@
       </c>
       <c r="J104" s="13" t="inlineStr">
         <is>
-          <t>Period / on demand</t>
+          <t>Per adjustment</t>
         </is>
       </c>
       <c r="K104" s="12" t="inlineStr">
         <is>
-          <t>Controller / CFO</t>
+          <t>Controller</t>
         </is>
       </c>
       <c r="L104" s="13" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="M104" s="12" t="inlineStr">
         <is>
-          <t>finance.service.ts reconcileControls; finance.controller.ts GET reconciliation/controls (exec/ar/creditors); reuses ledger.trialBalance + the AR/AP/inventory/gift-card/deferred sub-ledgers; cutover/giftcards.ts + compliance.ts (ToE)</t>
+          <t>bank.service.ts requestAdjustment/approveAdjustment/rejectAdjustment/listPendingAdjustments (reuses ledger.approveEntry SoD); bank.controller.ts (lines/:id/adjustment requests; adjustment/approve|reject gated approvals/gl_close); cutover/bankrec.ts (ToE)</t>
         </is>
       </c>
       <c r="N104" s="12" t="inlineStr">
         <is>
-          <t>Inspect the pack: each control account's sub-ledger query + the GL tie + the exceptions roll-up.</t>
+          <t>Inspect the request→approve flow + the approver≠requester check + that the Draft posts nothing until approval.</t>
         </is>
       </c>
       <c r="O104" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: with a clean set, every line reconciled + all_reconciled=true; introduce a known sub-ledger/GL difference and confirm it surfaces as an exception (re-performed: gift-card 2200 + inventory 1200 ties asserted by the harnesses).</t>
+          <t>Re-perform: request a fee adjustment (line unreconciled, GL difference unchanged), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm the difference closes to 0 only after approval (re-performed by the bankrec harness).</t>
         </is>
       </c>
       <c r="P104" s="12" t="inlineStr">
         <is>
-          <t>Reconciliation pack; exceptions list</t>
+          <t>Bank adjustment queue + SoD test</t>
         </is>
       </c>
       <c r="Q104" s="18" t="inlineStr">
@@ -9931,7 +9931,7 @@
     <row r="105">
       <c r="A105" s="15" t="inlineStr">
         <is>
-          <t>REC-05</t>
+          <t>REC-03</t>
         </is>
       </c>
       <c r="B105" s="16" t="inlineStr">
@@ -9946,27 +9946,27 @@
       </c>
       <c r="D105" s="16" t="inlineStr">
         <is>
-          <t>Cash; Bank</t>
+          <t>Consolidation</t>
         </is>
       </c>
       <c r="E105" s="16" t="inlineStr">
         <is>
-          <t>Till cash dropped to the safe never reaches the bank, or a deposit isn't matched to the statement — cash sits unbanked (theft/loss exposure) or the bank balance can't be tied to the books.</t>
+          <t>Intercompany balances not eliminated/agreed.</t>
         </is>
       </c>
       <c r="F105" s="16" t="inlineStr">
         <is>
-          <t>Completeness/Existence/Authorization</t>
+          <t>Accuracy</t>
         </is>
       </c>
       <c r="G105" s="16" t="inlineStr">
         <is>
-          <t>Cash banking — safe-drop → bank deposit → reconciliation: till 'drop's move cash from the drawer to the safe (drawer-only, no GL). Banking BATCHES the undeposited drops into a deposit and posts the GL (Dr &lt;bank account, e.g. 1010&gt; / Cr 1000 Cash), stamping each drop with the deposit id; the deposit is then RECONCILED to the bank statement (status Deposited→Reconciled). A detective read (GET /api/bank/deposits/undeposited-drops) surfaces the CASH STILL IN THE SAFE (drops with deposit_id NULL) — the unbanked exposure to chase. SoD: banking is a treasury duty (exec/ar) — segregated from the cashier (pos_till) who drops the cash, so the person who removes cash from the drawer is not the one who banks it.</t>
+          <t>Intercompany reconciliation &amp; elimination on consolidation.</t>
         </is>
       </c>
       <c r="H105" s="17" t="inlineStr">
         <is>
-          <t>Det/Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I105" s="17" t="inlineStr">
@@ -9976,12 +9976,12 @@
       </c>
       <c r="J105" s="17" t="inlineStr">
         <is>
-          <t>Per banking run</t>
+          <t>Period</t>
         </is>
       </c>
       <c r="K105" s="16" t="inlineStr">
         <is>
-          <t>FinancialController / Treasury</t>
+          <t>Group Controller</t>
         </is>
       </c>
       <c r="L105" s="17" t="inlineStr">
@@ -9991,39 +9991,39 @@
       </c>
       <c r="M105" s="16" t="inlineStr">
         <is>
-          <t>bank.service.ts undepositedDrops/createDeposit (Dr bank/Cr 1000, stamps deposit_id)/reconcileDeposit/listDeposits; bank.controller.ts (deposits, deposits/undeposited-drops, deposits/:id/reconcile; exec/ar); schema/cash.ts bank_deposits + cash_movements.deposit_id + migration 0152; /cash-banking UI; cutover/cash-banking.ts (ToE)</t>
+          <t>intercompany; consolidation</t>
         </is>
       </c>
       <c r="N105" s="16" t="inlineStr">
         <is>
-          <t>Inspect the undeposited-drop exposure read + the deposit GL (bank↔1000) + the reconcile step + the SoD (cashier vs treasury).</t>
+          <t>Inspect IC matching + elimination.</t>
         </is>
       </c>
       <c r="O105" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: two till drops → cash-in-safe shows the total; a cashier (pos_till) cannot bank (403); treasury banks → Dr bank / Cr 1000, cash-in-safe back to 0; reconcile the deposit; trial balance balanced (re-performed by the cash-banking harness).</t>
+          <t>Sample IC pairs agree &amp; eliminate.</t>
         </is>
       </c>
       <c r="P105" s="16" t="inlineStr">
         <is>
-          <t>Bank-deposit register; undeposited-drop (cash-in-safe) exposure</t>
-        </is>
-      </c>
-      <c r="Q105" s="18" t="inlineStr">
-        <is>
-          <t>Implemented</t>
+          <t>IC recon</t>
+        </is>
+      </c>
+      <c r="Q105" s="19" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="11" t="inlineStr">
         <is>
-          <t>GOV-01</t>
+          <t>REC-04</t>
         </is>
       </c>
       <c r="B106" s="12" t="inlineStr">
         <is>
-          <t>Monitoring</t>
+          <t>Reconciliation</t>
         </is>
       </c>
       <c r="C106" s="13" t="inlineStr">
@@ -10033,22 +10033,22 @@
       </c>
       <c r="D106" s="12" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>All control accounts</t>
         </is>
       </c>
       <c r="E106" s="12" t="inlineStr">
         <is>
-          <t>A maker-checker approval sits un-actioned and is forgotten — a transaction stalls before it is effective, or (worse) a control is quietly bypassed and no one notices an item never got its independent review.</t>
+          <t>A sub-ledger silently drifts from its GL control account at period-end and no single review catches it (incomplete/inaccurate balances reach the financial statements).</t>
         </is>
       </c>
       <c r="F106" s="12" t="inlineStr">
         <is>
-          <t>Authorization/Completeness</t>
+          <t>Completeness/Accuracy</t>
         </is>
       </c>
       <c r="G106" s="12" t="inlineStr">
         <is>
-          <t>Pending-approvals MONITOR (COSO monitoring): a single worklist of EVERY item awaiting independent approval across the system, each with its AGE in days and an overdue roll-up — spanning the manual-JE (GL-05), bank-adjustment (BANK-02), AP-disbursement (EXP-06), payroll (PAY-03), asset-revaluation (FA-08), asset-disposal (FA-09), inventory-write-off (INV-07), till-close cash over/short (REV-13), FX-rate (FX-04), budget (BUD-01) and large-refund (REV-16) maker-checkers. The controller reviews it before close; a stale item (age beyond the threshold) is a control finding to chase or escalate. The /approvals screen also lets a manager approve/reject a material till variance or a large refund inline (the pending types with no dedicated module screen). Read-only worklist; tenant-scoped via the caller's RLS.</t>
+          <t>Period-end control-account reconciliation PACK: one read (GET /api/finance/reconciliation/controls) ties every major sub-ledger to its GL control account and FLAGS any out-of-balance — AR↔1100, AP↔2000, Inventory↔1200, Gift cards/Customer-deposits↔2200, Deferred revenue↔2400 — reporting per line {sub_ledger, gl_control, variance, reconciled} plus an overall all_reconciled flag and an exceptions count. Liability controls are sign-flipped before comparison. The controller's single 'are the books reconciled?' close view; an exception is a control finding to investigate before sign-off.</t>
         </is>
       </c>
       <c r="H106" s="13" t="inlineStr">
@@ -10063,7 +10063,7 @@
       </c>
       <c r="J106" s="13" t="inlineStr">
         <is>
-          <t>Continuous / pre-close</t>
+          <t>Period / on demand</t>
         </is>
       </c>
       <c r="K106" s="12" t="inlineStr">
@@ -10078,22 +10078,22 @@
       </c>
       <c r="M106" s="12" t="inlineStr">
         <is>
-          <t>finance.service.ts pendingApprovals; finance.controller.ts GET approvals/pending (exec/approvals/creditors); aggregates journalEntries(Draft incl. BANKADJ→BANK-02)/apPayments/payruns/asset_revaluations/fixed_assets(disposal_pending)/inv_writeoff_requests/till_sessions(PendingApproval)/fx_rates(PendingApproval)/budgets(PendingApproval); cutover/compliance.ts (ToE)</t>
+          <t>finance.service.ts reconcileControls; finance.controller.ts GET reconciliation/controls (exec/ar/creditors); reuses ledger.trialBalance + the AR/AP/inventory/gift-card/deferred sub-ledgers; cutover/giftcards.ts + compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N106" s="12" t="inlineStr">
         <is>
-          <t>Inspect the aggregation across all pending sources + the age/overdue roll-up.</t>
+          <t>Inspect the pack: each control account's sub-ledger query + the GL tie + the exceptions roll-up.</t>
         </is>
       </c>
       <c r="O106" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: create a pending item (e.g. a Draft JE) and confirm it appears in the worklist with its control ID, amount and age; the overdue count flags items past the threshold (re-performed by the harness).</t>
+          <t>Re-perform: with a clean set, every line reconciled + all_reconciled=true; introduce a known sub-ledger/GL difference and confirm it surfaces as an exception (re-performed: gift-card 2200 + inventory 1200 ties asserted by the harnesses).</t>
         </is>
       </c>
       <c r="P106" s="12" t="inlineStr">
         <is>
-          <t>Pending-approvals worklist</t>
+          <t>Reconciliation pack; exceptions list</t>
         </is>
       </c>
       <c r="Q106" s="18" t="inlineStr">
@@ -10105,12 +10105,12 @@
     <row r="107">
       <c r="A107" s="15" t="inlineStr">
         <is>
-          <t>TAX-01</t>
+          <t>REC-05</t>
         </is>
       </c>
       <c r="B107" s="16" t="inlineStr">
         <is>
-          <t>Tax</t>
+          <t>Reconciliation</t>
         </is>
       </c>
       <c r="C107" s="17" t="inlineStr">
@@ -10120,67 +10120,67 @@
       </c>
       <c r="D107" s="16" t="inlineStr">
         <is>
-          <t>Tax (VAT)</t>
+          <t>Cash; Bank</t>
         </is>
       </c>
       <c r="E107" s="16" t="inlineStr">
         <is>
-          <t>VAT computed incorrectly → filing/penalty risk.</t>
+          <t>Till cash dropped to the safe never reaches the bank, or a deposit isn't matched to the statement — cash sits unbanked (theft/loss exposure) or the bank balance can't be tied to the books.</t>
         </is>
       </c>
       <c r="F107" s="16" t="inlineStr">
         <is>
-          <t>Accuracy</t>
+          <t>Completeness/Existence/Authorization</t>
         </is>
       </c>
       <c r="G107" s="16" t="inlineStr">
         <is>
-          <t>VAT via pluggable provider (TH 7%); unit-tested; no hard-coded rate.</t>
+          <t>Cash banking — safe-drop → bank deposit → reconciliation: till 'drop's move cash from the drawer to the safe (drawer-only, no GL). Banking BATCHES the undeposited drops into a deposit and posts the GL (Dr &lt;bank account, e.g. 1010&gt; / Cr 1000 Cash), stamping each drop with the deposit id; the deposit is then RECONCILED to the bank statement (status Deposited→Reconciled). A detective read (GET /api/bank/deposits/undeposited-drops) surfaces the CASH STILL IN THE SAFE (drops with deposit_id NULL) — the unbanked exposure to chase. SoD: banking is a treasury duty (exec/ar) — segregated from the cashier (pos_till) who drops the cash, so the person who removes cash from the drawer is not the one who banks it.</t>
         </is>
       </c>
       <c r="H107" s="17" t="inlineStr">
         <is>
-          <t>Auto</t>
+          <t>Det/Prev</t>
         </is>
       </c>
       <c r="I107" s="17" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="J107" s="17" t="inlineStr">
         <is>
-          <t>Per txn</t>
+          <t>Per banking run</t>
         </is>
       </c>
       <c r="K107" s="16" t="inlineStr">
         <is>
-          <t>Tax / Controller</t>
+          <t>FinancialController / Treasury</t>
         </is>
       </c>
       <c r="L107" s="17" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="M107" s="16" t="inlineStr">
         <is>
-          <t>tax/tax-providers.ts; tax.service.ts; test/unit.test.ts</t>
+          <t>bank.service.ts undepositedDrops/createDeposit (Dr bank/Cr 1000, stamps deposit_id)/reconcileDeposit/listDeposits; bank.controller.ts (deposits, deposits/undeposited-drops, deposits/:id/reconcile; exec/ar); schema/cash.ts bank_deposits + cash_movements.deposit_id + migration 0152; /cash-banking UI; cutover/cash-banking.ts (ToE)</t>
         </is>
       </c>
       <c r="N107" s="16" t="inlineStr">
         <is>
-          <t>Inspect rate provider + tests.</t>
+          <t>Inspect the undeposited-drop exposure read + the deposit GL (bank↔1000) + the reconcile step + the SoD (cashier vs treasury).</t>
         </is>
       </c>
       <c r="O107" s="16" t="inlineStr">
         <is>
-          <t>Re-perform VAT on sample; tie to return.</t>
+          <t>Re-perform: two till drops → cash-in-safe shows the total; a cashier (pos_till) cannot bank (403); treasury banks → Dr bank / Cr 1000, cash-in-safe back to 0; reconcile the deposit; trial balance balanced (re-performed by the cash-banking harness).</t>
         </is>
       </c>
       <c r="P107" s="16" t="inlineStr">
         <is>
-          <t>VAT tests</t>
+          <t>Bank-deposit register; undeposited-drop (cash-in-safe) exposure</t>
         </is>
       </c>
       <c r="Q107" s="18" t="inlineStr">
@@ -10192,12 +10192,12 @@
     <row r="108">
       <c r="A108" s="11" t="inlineStr">
         <is>
-          <t>TAX-02</t>
+          <t>GOV-01</t>
         </is>
       </c>
       <c r="B108" s="12" t="inlineStr">
         <is>
-          <t>Tax</t>
+          <t>Monitoring</t>
         </is>
       </c>
       <c r="C108" s="13" t="inlineStr">
@@ -10207,27 +10207,27 @@
       </c>
       <c r="D108" s="12" t="inlineStr">
         <is>
-          <t>Tax; Revenue</t>
+          <t>All</t>
         </is>
       </c>
       <c r="E108" s="12" t="inlineStr">
         <is>
-          <t>Non-compliant e-Tax invoice / not transmitted to ETDA.</t>
+          <t>A maker-checker approval sits un-actioned and is forgotten — a transaction stalls before it is effective, or (worse) a control is quietly bypassed and no one notices an item never got its independent review.</t>
         </is>
       </c>
       <c r="F108" s="12" t="inlineStr">
         <is>
-          <t>Accuracy/Compliance</t>
+          <t>Authorization/Completeness</t>
         </is>
       </c>
       <c r="G108" s="12" t="inlineStr">
         <is>
-          <t>e-Tax invoice (ETDA UBL 2.1 XML) generation + email with CC to ETDA timestamp mailbox.</t>
+          <t>Pending-approvals MONITOR (COSO monitoring): a single worklist of EVERY item awaiting independent approval across the system, each with its AGE in days and an overdue roll-up — spanning the manual-JE (GL-05), bank-adjustment (BANK-02), AP-disbursement (EXP-06), payroll (PAY-03), asset-revaluation (FA-08), asset-disposal (FA-09), inventory-write-off (INV-07), till-close cash over/short (REV-13), FX-rate (FX-04), budget (BUD-01) and large-refund (REV-16) maker-checkers. The controller reviews it before close; a stale item (age beyond the threshold) is a control finding to chase or escalate. The /approvals screen also lets a manager approve/reject a material till variance or a large refund inline (the pending types with no dedicated module screen). Read-only worklist; tenant-scoped via the caller's RLS.</t>
         </is>
       </c>
       <c r="H108" s="13" t="inlineStr">
         <is>
-          <t>Auto</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I108" s="13" t="inlineStr">
@@ -10237,37 +10237,37 @@
       </c>
       <c r="J108" s="13" t="inlineStr">
         <is>
-          <t>Per invoice</t>
+          <t>Continuous / pre-close</t>
         </is>
       </c>
       <c r="K108" s="12" t="inlineStr">
         <is>
-          <t>Tax</t>
+          <t>Controller / CFO</t>
         </is>
       </c>
       <c r="L108" s="13" t="inlineStr">
         <is>
-          <t>P10/P13</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="M108" s="12" t="inlineStr">
         <is>
-          <t>tax-docs/etax-xml.ts; etax-email.service.ts (tested)</t>
+          <t>finance.service.ts pendingApprovals; finance.controller.ts GET approvals/pending (exec/approvals/creditors); aggregates journalEntries(Draft incl. BANKADJ→BANK-02)/apPayments/payruns/asset_revaluations/fixed_assets(disposal_pending)/inv_writeoff_requests/till_sessions(PendingApproval)/fx_rates(PendingApproval)/budgets(PendingApproval); cutover/compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N108" s="12" t="inlineStr">
         <is>
-          <t>Inspect XML schema + email composer.</t>
+          <t>Inspect the aggregation across all pending sources + the age/overdue roll-up.</t>
         </is>
       </c>
       <c r="O108" s="12" t="inlineStr">
         <is>
-          <t>Sample invoices: valid XML, correct CC/escaping.</t>
+          <t>Re-perform: create a pending item (e.g. a Draft JE) and confirm it appears in the worklist with its control ID, amount and age; the overdue count flags items past the threshold (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P108" s="12" t="inlineStr">
         <is>
-          <t>e-Tax samples</t>
+          <t>Pending-approvals worklist</t>
         </is>
       </c>
       <c r="Q108" s="18" t="inlineStr">
@@ -10279,7 +10279,7 @@
     <row r="109">
       <c r="A109" s="15" t="inlineStr">
         <is>
-          <t>TAX-03</t>
+          <t>TAX-01</t>
         </is>
       </c>
       <c r="B109" s="16" t="inlineStr">
@@ -10294,12 +10294,12 @@
       </c>
       <c r="D109" s="16" t="inlineStr">
         <is>
-          <t>Tax (WHT)</t>
+          <t>Tax (VAT)</t>
         </is>
       </c>
       <c r="E109" s="16" t="inlineStr">
         <is>
-          <t>Withholding tax mis-computed / not reported.</t>
+          <t>VAT computed incorrectly → filing/penalty risk.</t>
         </is>
       </c>
       <c r="F109" s="16" t="inlineStr">
@@ -10309,7 +10309,7 @@
       </c>
       <c r="G109" s="16" t="inlineStr">
         <is>
-          <t>WHT computation and ภ.ง.ด. reporting.</t>
+          <t>VAT via pluggable provider (TH 7%); unit-tested; no hard-coded rate.</t>
         </is>
       </c>
       <c r="H109" s="17" t="inlineStr">
@@ -10324,12 +10324,12 @@
       </c>
       <c r="J109" s="17" t="inlineStr">
         <is>
-          <t>Per txn / monthly</t>
+          <t>Per txn</t>
         </is>
       </c>
       <c r="K109" s="16" t="inlineStr">
         <is>
-          <t>Tax</t>
+          <t>Tax / Controller</t>
         </is>
       </c>
       <c r="L109" s="17" t="inlineStr">
@@ -10339,34 +10339,34 @@
       </c>
       <c r="M109" s="16" t="inlineStr">
         <is>
-          <t>tax-reports; payroll</t>
+          <t>tax/tax-providers.ts; tax.service.ts; test/unit.test.ts</t>
         </is>
       </c>
       <c r="N109" s="16" t="inlineStr">
         <is>
-          <t>Inspect WHT logic + report.</t>
+          <t>Inspect rate provider + tests.</t>
         </is>
       </c>
       <c r="O109" s="16" t="inlineStr">
         <is>
-          <t>Re-perform WHT on sample; tie to filing.</t>
+          <t>Re-perform VAT on sample; tie to return.</t>
         </is>
       </c>
       <c r="P109" s="16" t="inlineStr">
         <is>
-          <t>WHT report</t>
-        </is>
-      </c>
-      <c r="Q109" s="19" t="inlineStr">
-        <is>
-          <t>Partial</t>
+          <t>VAT tests</t>
+        </is>
+      </c>
+      <c r="Q109" s="18" t="inlineStr">
+        <is>
+          <t>Implemented</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="11" t="inlineStr">
         <is>
-          <t>TAX-04</t>
+          <t>TAX-02</t>
         </is>
       </c>
       <c r="B110" s="12" t="inlineStr">
@@ -10381,27 +10381,27 @@
       </c>
       <c r="D110" s="12" t="inlineStr">
         <is>
-          <t>Tax (VAT); Tax Payable (2100)</t>
+          <t>Tax; Revenue</t>
         </is>
       </c>
       <c r="E110" s="12" t="inlineStr">
         <is>
-          <t>Output/input VAT on the filed ภ.พ.30 return does not agree to the GL — VAT liability mis-stated, a filing/penalty exposure, or a posting omission goes undetected before submission.</t>
+          <t>Non-compliant e-Tax invoice / not transmitted to ETDA.</t>
         </is>
       </c>
       <c r="F110" s="12" t="inlineStr">
         <is>
-          <t>Completeness/Accuracy</t>
+          <t>Accuracy/Compliance</t>
         </is>
       </c>
       <c r="G110" s="12" t="inlineStr">
         <is>
-          <t>Periodic VAT-return ↔ GL reconciliation (ภ.พ.30): the monthly return (GET /api/tax-reports/pp30) is built from the sales/output-VAT and purchase/input-VAT sub-reports, computes net VAT = output − input, and RECONCILES it to the **GL account 2100 (Tax Payable) net movement** for the same period (Σ credit − Σ debit over Posted entries) — returning `reconciliation.tied` = true only when the two agree within rounding. A non-tie is a detective finding to investigate and clear BEFORE filing (the form also carries the ม.157 deadline = the 15th of the next month). Output VAT is posted to 2100 on every sale (Cr) and reversed on returns (Dr); input VAT is posted on AP bills (Dr) — so 2100's net is the period's VAT payable. Read-only report; exportable to a ภ.พ.30 PDF/HTML.</t>
+          <t>e-Tax invoice (ETDA UBL 2.1 XML) generation + email with CC to ETDA timestamp mailbox.</t>
         </is>
       </c>
       <c r="H110" s="13" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Auto</t>
         </is>
       </c>
       <c r="I110" s="13" t="inlineStr">
@@ -10411,37 +10411,37 @@
       </c>
       <c r="J110" s="13" t="inlineStr">
         <is>
-          <t>Monthly / pre-filing</t>
+          <t>Per invoice</t>
         </is>
       </c>
       <c r="K110" s="12" t="inlineStr">
         <is>
-          <t>Tax / FinancialController</t>
+          <t>Tax</t>
         </is>
       </c>
       <c r="L110" s="13" t="inlineStr">
         <is>
-          <t>P10/P16</t>
+          <t>P10/P13</t>
         </is>
       </c>
       <c r="M110" s="12" t="inlineStr">
         <is>
-          <t>tax-reports.service.ts pp30 (outputVat/inputVat + 2100 net-movement tie); tax-reports.controller.ts (GET pp30, pp30/export, exec); tax-reports-pdf.ts; dine-in.service.ts/returns.service.ts/finance.service.ts post 2100 on sale/return/AP; /tax/reports UI; cutover/taxdocs.ts (ToE)</t>
+          <t>tax-docs/etax-xml.ts; etax-email.service.ts (tested)</t>
         </is>
       </c>
       <c r="N110" s="12" t="inlineStr">
         <is>
-          <t>Inspect the pp30 build + the 2100 net-movement query + the tie flag + the filing deadline.</t>
+          <t>Inspect XML schema + email composer.</t>
         </is>
       </c>
       <c r="O110" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: the pp30 return computes net VAT (output − input), the GL 2100 net movement reflects the posted input VAT, and the reconciliation block exposes the gl_account (2100), the report net VAT and a boolean tie verdict (tied iff the two agree within rounding); the ภ.พ.30 export renders (re-performed by the taxdocs harness).</t>
+          <t>Sample invoices: valid XML, correct CC/escaping.</t>
         </is>
       </c>
       <c r="P110" s="12" t="inlineStr">
         <is>
-          <t>ภ.พ.30 return + GL-2100 reconciliation tie</t>
+          <t>e-Tax samples</t>
         </is>
       </c>
       <c r="Q110" s="18" t="inlineStr">
@@ -10453,12 +10453,12 @@
     <row r="111">
       <c r="A111" s="15" t="inlineStr">
         <is>
-          <t>PAY-01</t>
+          <t>TAX-03</t>
         </is>
       </c>
       <c r="B111" s="16" t="inlineStr">
         <is>
-          <t>Payroll</t>
+          <t>Tax</t>
         </is>
       </c>
       <c r="C111" s="17" t="inlineStr">
@@ -10468,12 +10468,12 @@
       </c>
       <c r="D111" s="16" t="inlineStr">
         <is>
-          <t>Payroll expense/liability</t>
+          <t>Tax (WHT)</t>
         </is>
       </c>
       <c r="E111" s="16" t="inlineStr">
         <is>
-          <t>Payroll, SSO and PIT mis-computed.</t>
+          <t>Withholding tax mis-computed / not reported.</t>
         </is>
       </c>
       <c r="F111" s="16" t="inlineStr">
@@ -10483,7 +10483,7 @@
       </c>
       <c r="G111" s="16" t="inlineStr">
         <is>
-          <t>Payroll engine — SSO 5% (cap 750), progressive PIT, payslip net; unit-tested.</t>
+          <t>WHT computation and ภ.ง.ด. reporting.</t>
         </is>
       </c>
       <c r="H111" s="17" t="inlineStr">
@@ -10498,12 +10498,12 @@
       </c>
       <c r="J111" s="17" t="inlineStr">
         <is>
-          <t>Per run</t>
+          <t>Per txn / monthly</t>
         </is>
       </c>
       <c r="K111" s="16" t="inlineStr">
         <is>
-          <t>HR / Payroll</t>
+          <t>Tax</t>
         </is>
       </c>
       <c r="L111" s="17" t="inlineStr">
@@ -10513,39 +10513,39 @@
       </c>
       <c r="M111" s="16" t="inlineStr">
         <is>
-          <t>payroll/payroll-calc.ts; test/unit.test.ts</t>
+          <t>tax-reports; payroll</t>
         </is>
       </c>
       <c r="N111" s="16" t="inlineStr">
         <is>
-          <t>Inspect calc + tests.</t>
+          <t>Inspect WHT logic + report.</t>
         </is>
       </c>
       <c r="O111" s="16" t="inlineStr">
         <is>
-          <t>Re-perform sample payslips.</t>
+          <t>Re-perform WHT on sample; tie to filing.</t>
         </is>
       </c>
       <c r="P111" s="16" t="inlineStr">
         <is>
-          <t>Payslip tests</t>
-        </is>
-      </c>
-      <c r="Q111" s="18" t="inlineStr">
-        <is>
-          <t>Implemented</t>
+          <t>WHT report</t>
+        </is>
+      </c>
+      <c r="Q111" s="19" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="11" t="inlineStr">
         <is>
-          <t>PAY-02</t>
+          <t>TAX-04</t>
         </is>
       </c>
       <c r="B112" s="12" t="inlineStr">
         <is>
-          <t>Payroll</t>
+          <t>Tax</t>
         </is>
       </c>
       <c r="C112" s="13" t="inlineStr">
@@ -10555,22 +10555,22 @@
       </c>
       <c r="D112" s="12" t="inlineStr">
         <is>
-          <t>Payroll liability</t>
+          <t>Tax (VAT); Tax Payable (2100)</t>
         </is>
       </c>
       <c r="E112" s="12" t="inlineStr">
         <is>
-          <t>Statutory withholdings (SSO/WHT/PF) mis-stated or not remitted, so the liability owed to the authorities diverges from the books.</t>
+          <t>Output/input VAT on the filed ภ.พ.30 return does not agree to the GL — VAT liability mis-stated, a filing/penalty exposure, or a posting omission goes undetected before submission.</t>
         </is>
       </c>
       <c r="F112" s="12" t="inlineStr">
         <is>
-          <t>Accuracy/Compliance</t>
+          <t>Completeness/Accuracy</t>
         </is>
       </c>
       <c r="G112" s="12" t="inlineStr">
         <is>
-          <t>Payroll-liability schedule (GET /api/payroll/liabilities): each statutory account — SSO 2350, WHT/PND1 2360, PF 2370 — shows accrued (GL credits) − remitted (GL debits) = outstanding, tied back to the INDEPENDENT payrun accrual with a `reconciled` flag (a divergence flags a manual JE that touched a payroll-liability account outside the payroll process). Treasury remits the cash (POST .../remit → Dr liability / Cr 1000) which clears the outstanding and keeps the books reconciled to the statutory filings; a remittance beyond the outstanding is blocked (REMIT_EXCEEDS_OUTSTANDING).</t>
+          <t>Periodic VAT-return ↔ GL reconciliation (ภ.พ.30): the monthly return (GET /api/tax-reports/pp30) is built from the sales/output-VAT and purchase/input-VAT sub-reports, computes net VAT = output − input, and RECONCILES it to the **GL account 2100 (Tax Payable) net movement** for the same period (Σ credit − Σ debit over Posted entries) — returning `reconciliation.tied` = true only when the two agree within rounding. A non-tie is a detective finding to investigate and clear BEFORE filing (the form also carries the ม.157 deadline = the 15th of the next month). Output VAT is posted to 2100 on every sale (Cr) and reversed on returns (Dr); input VAT is posted on AP bills (Dr) — so 2100's net is the period's VAT payable. Read-only report; exportable to a ภ.พ.30 PDF/HTML.</t>
         </is>
       </c>
       <c r="H112" s="13" t="inlineStr">
@@ -10585,37 +10585,37 @@
       </c>
       <c r="J112" s="13" t="inlineStr">
         <is>
-          <t>Per run / monthly</t>
+          <t>Monthly / pre-filing</t>
         </is>
       </c>
       <c r="K112" s="12" t="inlineStr">
         <is>
-          <t>HR / Payroll / Treasury</t>
+          <t>Tax / FinancialController</t>
         </is>
       </c>
       <c r="L112" s="13" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P10/P16</t>
         </is>
       </c>
       <c r="M112" s="12" t="inlineStr">
         <is>
-          <t>payroll/payroll.service.ts liabilities/remitLiability</t>
+          <t>tax-reports.service.ts pp30 (outputVat/inputVat + 2100 net-movement tie); tax-reports.controller.ts (GET pp30, pp30/export, exec); tax-reports-pdf.ts; dine-in.service.ts/returns.service.ts/finance.service.ts post 2100 on sale/return/AP; /tax/reports UI; cutover/taxdocs.ts (ToE)</t>
         </is>
       </c>
       <c r="N112" s="12" t="inlineStr">
         <is>
-          <t>Inspect the schedule + the accrued/remitted/outstanding tie-out and the reconciled flag.</t>
+          <t>Inspect the pp30 build + the 2100 net-movement query + the tie flag + the filing deadline.</t>
         </is>
       </c>
       <c r="O112" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: run a payroll, confirm the SSO/WHT outstanding equals the payrun accrual; remit part and confirm the outstanding falls and the TB stays balanced; attempt an over-remit (REMIT_EXCEEDS_OUTSTANDING).</t>
+          <t>Re-perform: the pp30 return computes net VAT (output − input), the GL 2100 net movement reflects the posted input VAT, and the reconciliation block exposes the gl_account (2100), the report net VAT and a boolean tie verdict (tied iff the two agree within rounding); the ภ.พ.30 export renders (re-performed by the taxdocs harness).</t>
         </is>
       </c>
       <c r="P112" s="12" t="inlineStr">
         <is>
-          <t>Liability schedule + remittance JEs tied to filings</t>
+          <t>ภ.พ.30 return + GL-2100 reconciliation tie</t>
         </is>
       </c>
       <c r="Q112" s="18" t="inlineStr">
@@ -10627,7 +10627,7 @@
     <row r="113">
       <c r="A113" s="15" t="inlineStr">
         <is>
-          <t>PAY-03</t>
+          <t>PAY-01</t>
         </is>
       </c>
       <c r="B113" s="16" t="inlineStr">
@@ -10642,27 +10642,27 @@
       </c>
       <c r="D113" s="16" t="inlineStr">
         <is>
-          <t>Payroll expense/liability; Cash</t>
+          <t>Payroll expense/liability</t>
         </is>
       </c>
       <c r="E113" s="16" t="inlineStr">
         <is>
-          <t>Payroll run posted to the GL without independent review — the preparer both computes and posts their own payroll (ghost employees, inflated rate/hours).</t>
+          <t>Payroll, SSO and PIT mis-computed.</t>
         </is>
       </c>
       <c r="F113" s="16" t="inlineStr">
         <is>
-          <t>Authorization</t>
+          <t>Accuracy</t>
         </is>
       </c>
       <c r="G113" s="16" t="inlineStr">
         <is>
-          <t>Payroll maker-checker (SoD): a run posts its GL entry as a DRAFT (excluded from balances) with the run record 'PendingApproval'; a DIFFERENT user must approve before it becomes effective (approver ≠ preparer enforced regardless of permissions, reusing the GL-05 ledger approval). Reject voids the draft; idempotent per (tenant, period).</t>
+          <t>Payroll engine — SSO 5% (cap 750), progressive PIT, payslip net; unit-tested.</t>
         </is>
       </c>
       <c r="H113" s="17" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Auto</t>
         </is>
       </c>
       <c r="I113" s="17" t="inlineStr">
@@ -10677,7 +10677,7 @@
       </c>
       <c r="K113" s="16" t="inlineStr">
         <is>
-          <t>HR / Payroll; Controller</t>
+          <t>HR / Payroll</t>
         </is>
       </c>
       <c r="L113" s="17" t="inlineStr">
@@ -10687,22 +10687,22 @@
       </c>
       <c r="M113" s="16" t="inlineStr">
         <is>
-          <t>payroll/payroll.service.ts approvePayroll/rejectPayroll; migration 0133</t>
+          <t>payroll/payroll-calc.ts; test/unit.test.ts</t>
         </is>
       </c>
       <c r="N113" s="16" t="inlineStr">
         <is>
-          <t>Inspect Draft→approve flow + the approver≠preparer check.</t>
+          <t>Inspect calc + tests.</t>
         </is>
       </c>
       <c r="O113" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: run as A, attempt self-approve (SOD_VIOLATION), approve as B; confirm the JE hits balances only after approval.</t>
+          <t>Re-perform sample payslips.</t>
         </is>
       </c>
       <c r="P113" s="16" t="inlineStr">
         <is>
-          <t>Approval log + SoD test</t>
+          <t>Payslip tests</t>
         </is>
       </c>
       <c r="Q113" s="18" t="inlineStr">
@@ -10714,12 +10714,12 @@
     <row r="114">
       <c r="A114" s="11" t="inlineStr">
         <is>
-          <t>FA-09</t>
+          <t>PAY-02</t>
         </is>
       </c>
       <c r="B114" s="12" t="inlineStr">
         <is>
-          <t>Fixed Assets</t>
+          <t>Payroll</t>
         </is>
       </c>
       <c r="C114" s="13" t="inlineStr">
@@ -10729,27 +10729,27 @@
       </c>
       <c r="D114" s="12" t="inlineStr">
         <is>
-          <t>Property, Plant &amp; Equipment; Cash</t>
+          <t>Payroll liability</t>
         </is>
       </c>
       <c r="E114" s="12" t="inlineStr">
         <is>
-          <t>Asset disposed without independent review — one person writes an asset off the books and records the proceeds (asset-stripping / theft: dispose a still-held asset, or to a related party below value).</t>
+          <t>Statutory withholdings (SSO/WHT/PF) mis-stated or not remitted, so the liability owed to the authorities diverges from the books.</t>
         </is>
       </c>
       <c r="F114" s="12" t="inlineStr">
         <is>
-          <t>Authorization</t>
+          <t>Accuracy/Compliance</t>
         </is>
       </c>
       <c r="G114" s="12" t="inlineStr">
         <is>
-          <t>Asset-disposal maker-checker (SoD): a disposal REQUEST posts its GL entry as a DRAFT (excluded from balances) and flags the asset disposal_pending WITHOUT marking it disposed or moving the register; a DIFFERENT user must approve before it is effective (status→disposed, revaluation surplus recycled 3200→3100) (approver ≠ requester enforced regardless of permissions, reusing the GL-05 ledger approval). Reject voids the draft and the asset stays in service; only one disposal may be pending per asset; a disposal-pending asset is frozen from depreciation.</t>
+          <t>Payroll-liability schedule (GET /api/payroll/liabilities): each statutory account — SSO 2350, WHT/PND1 2360, PF 2370 — shows accrued (GL credits) − remitted (GL debits) = outstanding, tied back to the INDEPENDENT payrun accrual with a `reconciled` flag (a divergence flags a manual JE that touched a payroll-liability account outside the payroll process). Treasury remits the cash (POST .../remit → Dr liability / Cr 1000) which clears the outstanding and keeps the books reconciled to the statutory filings; a remittance beyond the outstanding is blocked (REMIT_EXCEEDS_OUTSTANDING).</t>
         </is>
       </c>
       <c r="H114" s="13" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I114" s="13" t="inlineStr">
@@ -10759,12 +10759,12 @@
       </c>
       <c r="J114" s="13" t="inlineStr">
         <is>
-          <t>Per disposal</t>
+          <t>Per run / monthly</t>
         </is>
       </c>
       <c r="K114" s="12" t="inlineStr">
         <is>
-          <t>FaAccountant / Controller</t>
+          <t>HR / Payroll / Treasury</t>
         </is>
       </c>
       <c r="L114" s="13" t="inlineStr">
@@ -10774,22 +10774,22 @@
       </c>
       <c r="M114" s="12" t="inlineStr">
         <is>
-          <t>assets.service.ts dispose(pendingApproval Draft)/approveDisposal/rejectDisposal; assets.controller.ts (:assetNo/dispose/approve|reject); schema/assets.ts fixed_assets.disposal_pending + migration 0135; cutover/basics.ts + worldclass.ts + compliance.ts (ToE)</t>
+          <t>payroll/payroll.service.ts liabilities/remitLiability</t>
         </is>
       </c>
       <c r="N114" s="12" t="inlineStr">
         <is>
-          <t>Inspect Draft→approve flow + the approver≠requester check + deferred status/recycle.</t>
+          <t>Inspect the schedule + the accrued/remitted/outstanding tie-out and the reconciled flag.</t>
         </is>
       </c>
       <c r="O114" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: request a disposal (Draft JE excluded), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm status→disposed + surplus recycled only after approval (re-performed by the harnesses).</t>
+          <t>Re-perform: run a payroll, confirm the SSO/WHT outstanding equals the payrun accrual; remit part and confirm the outstanding falls and the TB stays balanced; attempt an over-remit (REMIT_EXCEEDS_OUTSTANDING).</t>
         </is>
       </c>
       <c r="P114" s="12" t="inlineStr">
         <is>
-          <t>Disposal approval log + SoD test</t>
+          <t>Liability schedule + remittance JEs tied to filings</t>
         </is>
       </c>
       <c r="Q114" s="18" t="inlineStr">
@@ -10801,12 +10801,12 @@
     <row r="115">
       <c r="A115" s="15" t="inlineStr">
         <is>
-          <t>FA-10</t>
+          <t>PAY-03</t>
         </is>
       </c>
       <c r="B115" s="16" t="inlineStr">
         <is>
-          <t>Fixed Assets</t>
+          <t>Payroll</t>
         </is>
       </c>
       <c r="C115" s="17" t="inlineStr">
@@ -10816,22 +10816,22 @@
       </c>
       <c r="D115" s="16" t="inlineStr">
         <is>
-          <t>Property, Plant &amp; Equipment; Accounts Payable</t>
+          <t>Payroll expense/liability; Cash</t>
         </is>
       </c>
       <c r="E115" s="16" t="inlineStr">
         <is>
-          <t>Capital purchases mis-capitalised or capitalised without independent review — the person who receives the goods also decides what enters the asset register and at what cost/useful life (fictitious or over-valued assets; capex/opex mis-classification).</t>
+          <t>Payroll run posted to the GL without independent review — the preparer both computes and posts their own payroll (ghost employees, inflated rate/hours).</t>
         </is>
       </c>
       <c r="F115" s="16" t="inlineStr">
         <is>
-          <t>Authorization; Accuracy</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="G115" s="16" t="inlineStr">
         <is>
-          <t>Procure-to-Capitalize maker-checker (SoD): a goods-receipt line flagged capital (item-master is_fixed_asset or per-PO-line override) is excluded from inventory capitalisation (1200) at receipt and instead becomes ELIGIBLE for the asset register. Capitalisation is a REQUEST that posts NOTHING to the GL; a DIFFERENT user must approve before the fixed_assets row + acquisition JE (Dr 1500 / Cr 2000) are created (approver ≠ requester enforced regardless of permissions). The created asset carries its source GR/PO for end-to-end PR→PO→GR→FA traceability; a GR line cannot be capitalised twice.</t>
+          <t>Payroll maker-checker (SoD): a run posts its GL entry as a DRAFT (excluded from balances) with the run record 'PendingApproval'; a DIFFERENT user must approve before it becomes effective (approver ≠ preparer enforced regardless of permissions, reusing the GL-05 ledger approval). Reject voids the draft; idempotent per (tenant, period).</t>
         </is>
       </c>
       <c r="H115" s="17" t="inlineStr">
@@ -10846,12 +10846,12 @@
       </c>
       <c r="J115" s="17" t="inlineStr">
         <is>
-          <t>Per capital receipt</t>
+          <t>Per run</t>
         </is>
       </c>
       <c r="K115" s="16" t="inlineStr">
         <is>
-          <t>FaAccountant / Controller</t>
+          <t>HR / Payroll; Controller</t>
         </is>
       </c>
       <c r="L115" s="17" t="inlineStr">
@@ -10861,22 +10861,22 @@
       </c>
       <c r="M115" s="16" t="inlineStr">
         <is>
-          <t>assets.service.ts registerFromGr/approveRegistration/rejectRegistration/eligibleFromGr; assets.controller.ts (registrations*); procurement.service.ts createGr (is_capital routing, costing excluded); schema/assets.ts asset_registration_requests + fixed_assets.source_gr_no/po_no + migration 0137; cutover/basics.ts + compliance.ts (ToE)</t>
+          <t>payroll/payroll.service.ts approvePayroll/rejectPayroll; migration 0133</t>
         </is>
       </c>
       <c r="N115" s="16" t="inlineStr">
         <is>
-          <t>Inspect the eligible→request→approve flow + approver≠requester check + the inventory-vs-asset routing of capital lines.</t>
+          <t>Inspect Draft→approve flow + the approver≠preparer check.</t>
         </is>
       </c>
       <c r="O115" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: receive a capital line, raise a registration (no GL), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm the asset + Dr 1500/Cr 2000 post only after approval and the line cannot be re-registered (re-performed by the harnesses).</t>
+          <t>Re-perform: run as A, attempt self-approve (SOD_VIOLATION), approve as B; confirm the JE hits balances only after approval.</t>
         </is>
       </c>
       <c r="P115" s="16" t="inlineStr">
         <is>
-          <t>Capitalization approval log + SoD test</t>
+          <t>Approval log + SoD test</t>
         </is>
       </c>
       <c r="Q115" s="18" t="inlineStr">
@@ -10888,12 +10888,12 @@
     <row r="116">
       <c r="A116" s="11" t="inlineStr">
         <is>
-          <t>CON-01</t>
+          <t>FA-09</t>
         </is>
       </c>
       <c r="B116" s="12" t="inlineStr">
         <is>
-          <t>Consolidation &amp; FX</t>
+          <t>Fixed Assets</t>
         </is>
       </c>
       <c r="C116" s="13" t="inlineStr">
@@ -10903,42 +10903,42 @@
       </c>
       <c r="D116" s="12" t="inlineStr">
         <is>
-          <t>Consolidation</t>
+          <t>Property, Plant &amp; Equipment; Cash</t>
         </is>
       </c>
       <c r="E116" s="12" t="inlineStr">
         <is>
-          <t>Group consolidation mis-stated (ownership/currency).</t>
+          <t>Asset disposed without independent review — one person writes an asset off the books and records the proceeds (asset-stripping / theft: dispose a still-held asset, or to a related party below value).</t>
         </is>
       </c>
       <c r="F116" s="12" t="inlineStr">
         <is>
-          <t>Accuracy</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="G116" s="12" t="inlineStr">
         <is>
-          <t>Consolidation run (ownership %, entity currency) gated by 'approvals'.</t>
+          <t>Asset-disposal maker-checker (SoD): a disposal REQUEST posts its GL entry as a DRAFT (excluded from balances) and flags the asset disposal_pending WITHOUT marking it disposed or moving the register; a DIFFERENT user must approve before it is effective (status→disposed, revaluation surplus recycled 3200→3100) (approver ≠ requester enforced regardless of permissions, reusing the GL-05 ledger approval). Reject voids the draft and the asset stays in service; only one disposal may be pending per asset; a disposal-pending asset is frozen from depreciation.</t>
         </is>
       </c>
       <c r="H116" s="13" t="inlineStr">
         <is>
-          <t>Auto+Manual</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I116" s="13" t="inlineStr">
         <is>
-          <t>Period</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J116" s="13" t="inlineStr">
         <is>
-          <t>Period</t>
+          <t>Per disposal</t>
         </is>
       </c>
       <c r="K116" s="12" t="inlineStr">
         <is>
-          <t>Group Controller</t>
+          <t>FaAccountant / Controller</t>
         </is>
       </c>
       <c r="L116" s="13" t="inlineStr">
@@ -10948,22 +10948,22 @@
       </c>
       <c r="M116" s="12" t="inlineStr">
         <is>
-          <t>consolidation.service.ts (runConsolidation @Permissions approvals)</t>
+          <t>assets.service.ts dispose(pendingApproval Draft)/approveDisposal/rejectDisposal; assets.controller.ts (:assetNo/dispose/approve|reject); schema/assets.ts fixed_assets.disposal_pending + migration 0135; cutover/basics.ts + worldclass.ts + compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N116" s="12" t="inlineStr">
         <is>
-          <t>Inspect consolidation logic + gate.</t>
+          <t>Inspect Draft→approve flow + the approver≠requester check + deferred status/recycle.</t>
         </is>
       </c>
       <c r="O116" s="12" t="inlineStr">
         <is>
-          <t>Sample period: consolidated TB ties to entities.</t>
+          <t>Re-perform: request a disposal (Draft JE excluded), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm status→disposed + surplus recycled only after approval (re-performed by the harnesses).</t>
         </is>
       </c>
       <c r="P116" s="12" t="inlineStr">
         <is>
-          <t>Consol TB</t>
+          <t>Disposal approval log + SoD test</t>
         </is>
       </c>
       <c r="Q116" s="18" t="inlineStr">
@@ -10975,12 +10975,12 @@
     <row r="117">
       <c r="A117" s="15" t="inlineStr">
         <is>
-          <t>CON-02</t>
+          <t>FA-10</t>
         </is>
       </c>
       <c r="B117" s="16" t="inlineStr">
         <is>
-          <t>Consolidation &amp; FX</t>
+          <t>Fixed Assets</t>
         </is>
       </c>
       <c r="C117" s="17" t="inlineStr">
@@ -10990,42 +10990,42 @@
       </c>
       <c r="D117" s="16" t="inlineStr">
         <is>
-          <t>FX gain/loss</t>
+          <t>Property, Plant &amp; Equipment; Accounts Payable</t>
         </is>
       </c>
       <c r="E117" s="16" t="inlineStr">
         <is>
-          <t>FX exposures not revalued at period-end.</t>
+          <t>Capital purchases mis-capitalised or capitalised without independent review — the person who receives the goods also decides what enters the asset register and at what cost/useful life (fictitious or over-valued assets; capex/opex mis-classification).</t>
         </is>
       </c>
       <c r="F117" s="16" t="inlineStr">
         <is>
-          <t>Valuation</t>
+          <t>Authorization; Accuracy</t>
         </is>
       </c>
       <c r="G117" s="16" t="inlineStr">
         <is>
-          <t>FX revaluation at period-end rates; unrealized FX posted (acct 5400).</t>
+          <t>Procure-to-Capitalize maker-checker (SoD): a goods-receipt line flagged capital (item-master is_fixed_asset or per-PO-line override) is excluded from inventory capitalisation (1200) at receipt and instead becomes ELIGIBLE for the asset register. Capitalisation is a REQUEST that posts NOTHING to the GL; a DIFFERENT user must approve before the fixed_assets row + acquisition JE (Dr 1500 / Cr 2000) are created (approver ≠ requester enforced regardless of permissions). The created asset carries its source GR/PO for end-to-end PR→PO→GR→FA traceability; a GR line cannot be capitalised twice.</t>
         </is>
       </c>
       <c r="H117" s="17" t="inlineStr">
         <is>
-          <t>Auto+Manual</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I117" s="17" t="inlineStr">
         <is>
-          <t>Period-end</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J117" s="17" t="inlineStr">
         <is>
-          <t>Period</t>
+          <t>Per capital receipt</t>
         </is>
       </c>
       <c r="K117" s="16" t="inlineStr">
         <is>
-          <t>Controller</t>
+          <t>FaAccountant / Controller</t>
         </is>
       </c>
       <c r="L117" s="17" t="inlineStr">
@@ -11035,22 +11035,22 @@
       </c>
       <c r="M117" s="16" t="inlineStr">
         <is>
-          <t>fx.service.ts (revalue / unrealized report)</t>
+          <t>assets.service.ts registerFromGr/approveRegistration/rejectRegistration/eligibleFromGr; assets.controller.ts (registrations*); procurement.service.ts createGr (is_capital routing, costing excluded); schema/assets.ts asset_registration_requests + fixed_assets.source_gr_no/po_no + migration 0137; cutover/basics.ts + compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N117" s="16" t="inlineStr">
         <is>
-          <t>Inspect reval logic + rates.</t>
+          <t>Inspect the eligible→request→approve flow + approver≠requester check + the inventory-vs-asset routing of capital lines.</t>
         </is>
       </c>
       <c r="O117" s="16" t="inlineStr">
         <is>
-          <t>Recompute reval on sample balances.</t>
+          <t>Re-perform: receive a capital line, raise a registration (no GL), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm the asset + Dr 1500/Cr 2000 post only after approval and the line cannot be re-registered (re-performed by the harnesses).</t>
         </is>
       </c>
       <c r="P117" s="16" t="inlineStr">
         <is>
-          <t>FX reval JE</t>
+          <t>Capitalization approval log + SoD test</t>
         </is>
       </c>
       <c r="Q117" s="18" t="inlineStr">
@@ -11062,7 +11062,7 @@
     <row r="118">
       <c r="A118" s="11" t="inlineStr">
         <is>
-          <t>FX-04</t>
+          <t>CON-01</t>
         </is>
       </c>
       <c r="B118" s="12" t="inlineStr">
@@ -11077,42 +11077,42 @@
       </c>
       <c r="D118" s="12" t="inlineStr">
         <is>
-          <t>FX gain/loss; Revenue; AR/AP</t>
+          <t>Consolidation</t>
         </is>
       </c>
       <c r="E118" s="12" t="inlineStr">
         <is>
-          <t>A wrong manually-entered FX rate (fat-fingered, e.g. USD 36 keyed as 63) flows straight into a period-end revaluation JE and the unrealized-FX report with no independent review — mis-stating earnings/equity and FX-translated balances.</t>
+          <t>Group consolidation mis-stated (ownership/currency).</t>
         </is>
       </c>
       <c r="F118" s="12" t="inlineStr">
         <is>
-          <t>Accuracy/Valuation</t>
+          <t>Accuracy</t>
         </is>
       </c>
       <c r="G118" s="12" t="inlineStr">
         <is>
-          <t>FX rate maker-checker (SoD): a MANUALLY-entered rate lands as PendingApproval and is EXCLUDED from rate resolution — revaluation, the unrealized-FX report, and consolidation translation all use APPROVED rates only — until a DIFFERENT user approves it (POST /api/fx/rates/approve). Self-approval → SOD_VIOLATION (binds even Admin); reject marks the rate Rejected (never usable); re-entering a rate sends it back to PendingApproval. Externally-sourced (feed) rates carrying an explicit non-manual source are auto-approved. Pending rates are also surfaced, aged, by the pending-approvals monitor (GOV-01).</t>
+          <t>Consolidation run (ownership %, entity currency) gated by 'approvals'.</t>
         </is>
       </c>
       <c r="H118" s="13" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="I118" s="13" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Period</t>
         </is>
       </c>
       <c r="J118" s="13" t="inlineStr">
         <is>
-          <t>Per rate</t>
+          <t>Period</t>
         </is>
       </c>
       <c r="K118" s="12" t="inlineStr">
         <is>
-          <t>Controller / Treasury</t>
+          <t>Group Controller</t>
         </is>
       </c>
       <c r="L118" s="13" t="inlineStr">
@@ -11122,22 +11122,22 @@
       </c>
       <c r="M118" s="12" t="inlineStr">
         <is>
-          <t>fx.service.ts setRate(manual→PendingApproval)/approveRate/rejectRate/rateAsOf(Approved only); fx.controller.ts (rates/approve|reject|pending gated approvals/gl_close); consolidation.service.ts (translation reads Approved rates); schema/fx.ts fx_rates.status + migration 0141; cutover/fxreval.ts (ToE)</t>
+          <t>consolidation.service.ts (runConsolidation @Permissions approvals)</t>
         </is>
       </c>
       <c r="N118" s="12" t="inlineStr">
         <is>
-          <t>Inspect the request→approve flow + the approver≠requester check + that revaluation/reporting resolve Approved rates only.</t>
+          <t>Inspect consolidation logic + gate.</t>
         </is>
       </c>
       <c r="O118" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: enter a manual rate (PendingApproval), confirm revalue is blocked NO_RATE while pending, attempt self-approve (SOD_VIOLATION), approve as a different user, then revalue succeeds (re-performed by the fxreval harness).</t>
+          <t>Sample period: consolidated TB ties to entities.</t>
         </is>
       </c>
       <c r="P118" s="12" t="inlineStr">
         <is>
-          <t>FX rate approval log + SoD test</t>
+          <t>Consol TB</t>
         </is>
       </c>
       <c r="Q118" s="18" t="inlineStr">
@@ -11149,92 +11149,266 @@
     <row r="119">
       <c r="A119" s="15" t="inlineStr">
         <is>
+          <t>CON-02</t>
+        </is>
+      </c>
+      <c r="B119" s="16" t="inlineStr">
+        <is>
+          <t>Consolidation &amp; FX</t>
+        </is>
+      </c>
+      <c r="C119" s="17" t="inlineStr">
+        <is>
+          <t>Application</t>
+        </is>
+      </c>
+      <c r="D119" s="16" t="inlineStr">
+        <is>
+          <t>FX gain/loss</t>
+        </is>
+      </c>
+      <c r="E119" s="16" t="inlineStr">
+        <is>
+          <t>FX exposures not revalued at period-end.</t>
+        </is>
+      </c>
+      <c r="F119" s="16" t="inlineStr">
+        <is>
+          <t>Valuation</t>
+        </is>
+      </c>
+      <c r="G119" s="16" t="inlineStr">
+        <is>
+          <t>FX revaluation at period-end rates; unrealized FX posted (acct 5400).</t>
+        </is>
+      </c>
+      <c r="H119" s="17" t="inlineStr">
+        <is>
+          <t>Auto+Manual</t>
+        </is>
+      </c>
+      <c r="I119" s="17" t="inlineStr">
+        <is>
+          <t>Period-end</t>
+        </is>
+      </c>
+      <c r="J119" s="17" t="inlineStr">
+        <is>
+          <t>Period</t>
+        </is>
+      </c>
+      <c r="K119" s="16" t="inlineStr">
+        <is>
+          <t>Controller</t>
+        </is>
+      </c>
+      <c r="L119" s="17" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="M119" s="16" t="inlineStr">
+        <is>
+          <t>fx.service.ts (revalue / unrealized report)</t>
+        </is>
+      </c>
+      <c r="N119" s="16" t="inlineStr">
+        <is>
+          <t>Inspect reval logic + rates.</t>
+        </is>
+      </c>
+      <c r="O119" s="16" t="inlineStr">
+        <is>
+          <t>Recompute reval on sample balances.</t>
+        </is>
+      </c>
+      <c r="P119" s="16" t="inlineStr">
+        <is>
+          <t>FX reval JE</t>
+        </is>
+      </c>
+      <c r="Q119" s="18" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="11" t="inlineStr">
+        <is>
+          <t>FX-04</t>
+        </is>
+      </c>
+      <c r="B120" s="12" t="inlineStr">
+        <is>
+          <t>Consolidation &amp; FX</t>
+        </is>
+      </c>
+      <c r="C120" s="13" t="inlineStr">
+        <is>
+          <t>Application</t>
+        </is>
+      </c>
+      <c r="D120" s="12" t="inlineStr">
+        <is>
+          <t>FX gain/loss; Revenue; AR/AP</t>
+        </is>
+      </c>
+      <c r="E120" s="12" t="inlineStr">
+        <is>
+          <t>A wrong manually-entered FX rate (fat-fingered, e.g. USD 36 keyed as 63) flows straight into a period-end revaluation JE and the unrealized-FX report with no independent review — mis-stating earnings/equity and FX-translated balances.</t>
+        </is>
+      </c>
+      <c r="F120" s="12" t="inlineStr">
+        <is>
+          <t>Accuracy/Valuation</t>
+        </is>
+      </c>
+      <c r="G120" s="12" t="inlineStr">
+        <is>
+          <t>FX rate maker-checker (SoD): a MANUALLY-entered rate lands as PendingApproval and is EXCLUDED from rate resolution — revaluation, the unrealized-FX report, and consolidation translation all use APPROVED rates only — until a DIFFERENT user approves it (POST /api/fx/rates/approve). Self-approval → SOD_VIOLATION (binds even Admin); reject marks the rate Rejected (never usable); re-entering a rate sends it back to PendingApproval. Externally-sourced (feed) rates carrying an explicit non-manual source are auto-approved. Pending rates are also surfaced, aged, by the pending-approvals monitor (GOV-01).</t>
+        </is>
+      </c>
+      <c r="H120" s="13" t="inlineStr">
+        <is>
+          <t>Prev</t>
+        </is>
+      </c>
+      <c r="I120" s="13" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="J120" s="13" t="inlineStr">
+        <is>
+          <t>Per rate</t>
+        </is>
+      </c>
+      <c r="K120" s="12" t="inlineStr">
+        <is>
+          <t>Controller / Treasury</t>
+        </is>
+      </c>
+      <c r="L120" s="13" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="M120" s="12" t="inlineStr">
+        <is>
+          <t>fx.service.ts setRate(manual→PendingApproval)/approveRate/rejectRate/rateAsOf(Approved only); fx.controller.ts (rates/approve|reject|pending gated approvals/gl_close); consolidation.service.ts (translation reads Approved rates); schema/fx.ts fx_rates.status + migration 0141; cutover/fxreval.ts (ToE)</t>
+        </is>
+      </c>
+      <c r="N120" s="12" t="inlineStr">
+        <is>
+          <t>Inspect the request→approve flow + the approver≠requester check + that revaluation/reporting resolve Approved rates only.</t>
+        </is>
+      </c>
+      <c r="O120" s="12" t="inlineStr">
+        <is>
+          <t>Re-perform: enter a manual rate (PendingApproval), confirm revalue is blocked NO_RATE while pending, attempt self-approve (SOD_VIOLATION), approve as a different user, then revalue succeeds (re-performed by the fxreval harness).</t>
+        </is>
+      </c>
+      <c r="P120" s="12" t="inlineStr">
+        <is>
+          <t>FX rate approval log + SoD test</t>
+        </is>
+      </c>
+      <c r="Q120" s="18" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="15" t="inlineStr">
+        <is>
           <t>BUD-01</t>
         </is>
       </c>
-      <c r="B119" s="16" t="inlineStr">
+      <c r="B121" s="16" t="inlineStr">
         <is>
           <t>Budgeting &amp; Planning</t>
         </is>
       </c>
-      <c r="C119" s="17" t="inlineStr">
+      <c r="C121" s="17" t="inlineStr">
         <is>
           <t>Application</t>
         </is>
       </c>
-      <c r="D119" s="16" t="inlineStr">
+      <c r="D121" s="16" t="inlineStr">
         <is>
           <t>Budget; All (variance reporting)</t>
         </is>
       </c>
-      <c r="E119" s="16" t="inlineStr">
+      <c r="E121" s="16" t="inlineStr">
         <is>
           <t>A budget figure is entered/changed by one person and immediately drives the budget-vs-actual variance report — the basis for spend authorization and performance review — with no independent approval; a wrong or self-serving budget makes overspending look 'on budget'.</t>
         </is>
       </c>
-      <c r="F119" s="16" t="inlineStr">
+      <c r="F121" s="16" t="inlineStr">
         <is>
           <t>Authorization/Accuracy</t>
         </is>
       </c>
-      <c r="G119" s="16" t="inlineStr">
+      <c r="G121" s="16" t="inlineStr">
         <is>
           <t>Budget maker-checker (SoD): an upserted budget (POST /api/ledger/budgets) lands as PendingApproval and is EXCLUDED from budget-vs-actual until a DIFFERENT user approves it (POST /api/ledger/budgets/approve for the fiscal_year/account/cost-centre[/period]). Self-approval → SOD_VIOLATION (binds even Admin); reject marks it Rejected (excluded). DEFAULT 'Approved' keeps existing rows + direct planning seeds usable. Pending budgets are also surfaced, aged, by the pending-approvals monitor (GOV-01).</t>
         </is>
       </c>
-      <c r="H119" s="17" t="inlineStr">
+      <c r="H121" s="17" t="inlineStr">
         <is>
           <t>Prev</t>
         </is>
       </c>
-      <c r="I119" s="17" t="inlineStr">
+      <c r="I121" s="17" t="inlineStr">
         <is>
           <t>Automated</t>
         </is>
       </c>
-      <c r="J119" s="17" t="inlineStr">
+      <c r="J121" s="17" t="inlineStr">
         <is>
           <t>Per budget</t>
         </is>
       </c>
-      <c r="K119" s="16" t="inlineStr">
+      <c r="K121" s="16" t="inlineStr">
         <is>
           <t>Controller / FP&amp;A</t>
         </is>
       </c>
-      <c r="L119" s="17" t="inlineStr">
+      <c r="L121" s="17" t="inlineStr">
         <is>
           <t>P10</t>
         </is>
       </c>
-      <c r="M119" s="16" t="inlineStr">
+      <c r="M121" s="16" t="inlineStr">
         <is>
           <t>budget.service.ts upsertBudget(→PendingApproval)/approveBudget/rejectBudget/budgetVsActual(Approved only); budget.controller.ts (budgets/approve|reject|pending gated approvals/gl_close); schema/budgets.ts budgets.status + migration 0142; cutover/budget.ts (ToE)</t>
         </is>
       </c>
-      <c r="N119" s="16" t="inlineStr">
+      <c r="N121" s="16" t="inlineStr">
         <is>
           <t>Inspect the request→approve flow + the approver≠requester check + that budget-vs-actual counts Approved budgets only.</t>
         </is>
       </c>
-      <c r="O119" s="16" t="inlineStr">
+      <c r="O121" s="16" t="inlineStr">
         <is>
           <t>Re-perform: upsert a budget (PendingApproval, excluded from variance), attempt self-approve (SOD_VIOLATION), approve as a different user, confirm it then appears in budget-vs-actual (re-performed by the budget harness).</t>
         </is>
       </c>
-      <c r="P119" s="16" t="inlineStr">
+      <c r="P121" s="16" t="inlineStr">
         <is>
           <t>Budget approval log + SoD test</t>
         </is>
       </c>
-      <c r="Q119" s="18" t="inlineStr">
+      <c r="Q121" s="18" t="inlineStr">
         <is>
           <t>Implemented</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q119"/>
+  <autoFilter ref="A1:Q121"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -12417,7 +12591,7 @@
         </is>
       </c>
       <c r="C5" s="29">
-        <f>COUNTIF(RCM!$Q$2:$Q$119,B5)</f>
+        <f>COUNTIF(RCM!$Q$2:$Q$121,B5)</f>
         <v/>
       </c>
     </row>
@@ -12428,7 +12602,7 @@
         </is>
       </c>
       <c r="C6" s="29">
-        <f>COUNTIF(RCM!$Q$2:$Q$119,B6)</f>
+        <f>COUNTIF(RCM!$Q$2:$Q$121,B6)</f>
         <v/>
       </c>
     </row>
@@ -12439,7 +12613,7 @@
         </is>
       </c>
       <c r="C7" s="29">
-        <f>COUNTIF(RCM!$Q$2:$Q$119,B7)</f>
+        <f>COUNTIF(RCM!$Q$2:$Q$121,B7)</f>
         <v/>
       </c>
     </row>
@@ -12450,7 +12624,7 @@
         </is>
       </c>
       <c r="C8" s="32">
-        <f>COUNTA(RCM!$A$2:$A$119)</f>
+        <f>COUNTA(RCM!$A$2:$A$121)</f>
         <v/>
       </c>
     </row>
@@ -12468,7 +12642,7 @@
         </is>
       </c>
       <c r="C11" s="29">
-        <f>COUNTIF(RCM!$C$2:$C$119,B11)</f>
+        <f>COUNTIF(RCM!$C$2:$C$121,B11)</f>
         <v/>
       </c>
     </row>
@@ -12479,7 +12653,7 @@
         </is>
       </c>
       <c r="C12" s="29">
-        <f>COUNTIF(RCM!$C$2:$C$119,B12)</f>
+        <f>COUNTIF(RCM!$C$2:$C$121,B12)</f>
         <v/>
       </c>
     </row>
@@ -12490,7 +12664,7 @@
         </is>
       </c>
       <c r="C13" s="29">
-        <f>COUNTIF(RCM!$C$2:$C$119,B13)</f>
+        <f>COUNTIF(RCM!$C$2:$C$121,B13)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(inventory): demand-driven par-level recommendations (Step 5, INV-12)
Branch replenishment (INV-05) routed transfer-before-buy off a STATIC per-branch
reorder point. Now each (branch,item) carries a lead_time_days, and the system
derives average daily usage from trailing branch-tagged consumption and
recommends reorder_point = ceil(avg_daily x lead x 1.25), flagging branches whose
static buffer is under-buffered for their run-rate. A planner applies per row.

- mig 0163: branch_stock + lead_time_days (journaled)
- replenishment.service parRecommendations + applyPar; wms.controller routes
  (par-recommendations [/apply]); /replenishment web par section
- wms harness +2 (10/day x lead 3 -> ROP 38 under-buffered; apply writes 38)
- RCM INV-12 (120 controls); docs inventory narrative 1.3, UAT-INV-058/059

wms(27)/compliance(106) green; typecheck green.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/compliance/Oshinei_ERP_SOX_RCM_v1.xlsx
+++ b/compliance/Oshinei_ERP_SOX_RCM_v1.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'RCM'!$A$1:$Q$120</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'RCM'!$A$1:$Q$121</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Gap Remediation'!$A$2:$H$18</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -858,7 +858,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q120"/>
+  <dimension ref="A1:Q121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -7147,12 +7147,12 @@
     <row r="73">
       <c r="A73" s="15" t="inlineStr">
         <is>
-          <t>BRANCH-01</t>
+          <t>INV-12</t>
         </is>
       </c>
       <c r="B73" s="16" t="inlineStr">
         <is>
-          <t>Multi-Branch &amp; Offline POS</t>
+          <t>Inventory &amp; COGS</t>
         </is>
       </c>
       <c r="C73" s="17" t="inlineStr">
@@ -7162,22 +7162,22 @@
       </c>
       <c r="D73" s="16" t="inlineStr">
         <is>
-          <t>Revenue</t>
+          <t>Inventory</t>
         </is>
       </c>
       <c r="E73" s="16" t="inlineStr">
         <is>
-          <t>A POS sale is not attributed to its originating branch, so the consolidated branch roll-up is incomplete and cannot be tied to GL revenue.</t>
+          <t>Per-branch reorder points are STATIC numbers — set once and never revisited — so a branch whose run-rate has grown carries too small a buffer and stocks out (lost sales), while a slow branch over-orders and ties up cash/spoils stock; neither is flagged.</t>
         </is>
       </c>
       <c r="F73" s="16" t="inlineStr">
         <is>
-          <t>Completeness</t>
+          <t>Accuracy/Completeness</t>
         </is>
       </c>
       <c r="G73" s="16" t="inlineStr">
         <is>
-          <t>Branch sale-tagging + HQ consolidation: every POS sale carries cust_pos_sales.branch_id; GET /api/branches/consolidated aggregates per branch (excluding Voided) and surfaces untagged sales as branch '(none)' — a deliberate completeness flag the controller investigates and clears before tying the consolidated total to GL revenue.</t>
+          <t>Demand-driven par-level recommendation (layered on the INV-05 branch min-max + transfer-before-buy): for each (branch,item) the system derives the average daily usage from the trailing window of branch-tagged consumption (cust_stock_log Sale/Consume) and recommends reorder_point = ceil(avg_daily x lead_time_days x safety 1.25), flagging rows whose static reorder_point is below that demand-driven buffer (under_buffered). GET /api/replenishment/par-recommendations is read-only; a planner applies a recommendation per row (POST .../apply writes the reorder_point onto branch_stock, planner duty). lead_time_days is per (branch,item) (migration 0163). Tenant-scoped (RLS); gated planner/procurement.</t>
         </is>
       </c>
       <c r="H73" s="17" t="inlineStr">
@@ -7192,37 +7192,37 @@
       </c>
       <c r="J73" s="17" t="inlineStr">
         <is>
-          <t>Per sale / period</t>
+          <t>Periodic / per planning cycle</t>
         </is>
       </c>
       <c r="K73" s="16" t="inlineStr">
         <is>
-          <t>HQ Controller</t>
+          <t>Planner / Supply Chain</t>
         </is>
       </c>
       <c r="L73" s="17" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>P13</t>
         </is>
       </c>
       <c r="M73" s="16" t="inlineStr">
         <is>
-          <t>branches.service.ts (consolidated, branch tagging); branches.controller.ts; cust_pos_sales.branch_id; cutover/branch.ts (ToE)</t>
+          <t>wms/replenishment.service.ts parRecommendations (avg-daily-usage x lead x safety, under_buffered flag) + applyPar (writes reorder_point, planner); wms.controller.ts (/api/replenishment/par-recommendations[/apply]); schema/portal.ts branch_stock.lead_time_days + migration 0163; /replenishment par-recommendations section; cutover/wms.ts (ToE)</t>
         </is>
       </c>
       <c r="N73" s="16" t="inlineStr">
         <is>
-          <t>Inspect branch tagging completeness + the '(none)' surfacing + the GL tie.</t>
+          <t>Inspect the avg-daily-usage derivation from consumption logs, the lead-time x safety reorder-point formula, the under_buffered flag, and the planner-gated apply.</t>
         </is>
       </c>
       <c r="O73" s="16" t="inlineStr">
         <is>
-          <t>Sample period: tagged sales group by branch, an untagged sale surfaces as '(none)', consolidated total ties to posted revenue.</t>
+          <t>Re-perform: seed branch consumption (10/day) at lead 3 -&gt; recommend ROP 38 (under-buffered vs static 10); apply writes 38 onto branch_stock; tenant-isolated (re-performed by the wms harness).</t>
         </is>
       </c>
       <c r="P73" s="16" t="inlineStr">
         <is>
-          <t>Consolidation report; '(none)' investigation log</t>
+          <t>Par recommendation list + apply test</t>
         </is>
       </c>
       <c r="Q73" s="18" t="inlineStr">
@@ -7234,7 +7234,7 @@
     <row r="74">
       <c r="A74" s="11" t="inlineStr">
         <is>
-          <t>BRANCH-02</t>
+          <t>BRANCH-01</t>
         </is>
       </c>
       <c r="B74" s="12" t="inlineStr">
@@ -7254,62 +7254,62 @@
       </c>
       <c r="E74" s="12" t="inlineStr">
         <is>
-          <t>An offline terminal sells at a stale or wrong price/promotion because the cached catalog drifted from the master.</t>
+          <t>A POS sale is not attributed to its originating branch, so the consolidated branch roll-up is incomplete and cannot be tied to GL revenue.</t>
         </is>
       </c>
       <c r="F74" s="12" t="inlineStr">
         <is>
-          <t>Accuracy</t>
+          <t>Completeness</t>
         </is>
       </c>
       <c r="G74" s="12" t="inlineStr">
         <is>
-          <t>Offline master-bundle export: GET /api/branches/master-bundle returns ONLY the active price-list + active promotions, time-stamped (generated_at). The offline terminal sells from this bundle, so it cannot ring a stale/withdrawn price or promo.</t>
+          <t>Branch sale-tagging + HQ consolidation: every POS sale carries cust_pos_sales.branch_id; GET /api/branches/consolidated aggregates per branch (excluding Voided) and surfaces untagged sales as branch '(none)' — a deliberate completeness flag the controller investigates and clears before tying the consolidated total to GL revenue.</t>
         </is>
       </c>
       <c r="H74" s="13" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I74" s="13" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="J74" s="13" t="inlineStr">
         <is>
-          <t>Per bundle push</t>
+          <t>Per sale / period</t>
         </is>
       </c>
       <c r="K74" s="12" t="inlineStr">
         <is>
-          <t>HQ Controller / Pricing</t>
+          <t>HQ Controller</t>
         </is>
       </c>
       <c r="L74" s="13" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="M74" s="12" t="inlineStr">
         <is>
-          <t>branches.service.ts masterBundle (active price-list + active promos + generated_at); branches.controller.ts; cutover/branch.ts (ToE)</t>
+          <t>branches.service.ts (consolidated, branch tagging); branches.controller.ts; cust_pos_sales.branch_id; cutover/branch.ts (ToE)</t>
         </is>
       </c>
       <c r="N74" s="12" t="inlineStr">
         <is>
-          <t>Inspect the bundle exports only active prices/promos with a timestamp.</t>
+          <t>Inspect branch tagging completeness + the '(none)' surfacing + the GL tie.</t>
         </is>
       </c>
       <c r="O74" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: export the bundle; confirm it carries only active price-list/promotions + generated_at.</t>
+          <t>Sample period: tagged sales group by branch, an untagged sale surfaces as '(none)', consolidated total ties to posted revenue.</t>
         </is>
       </c>
       <c r="P74" s="12" t="inlineStr">
         <is>
-          <t>Bundle metadata; bundle vs price-master diff</t>
+          <t>Consolidation report; '(none)' investigation log</t>
         </is>
       </c>
       <c r="Q74" s="18" t="inlineStr">
@@ -7321,7 +7321,7 @@
     <row r="75">
       <c r="A75" s="15" t="inlineStr">
         <is>
-          <t>BRANCH-03</t>
+          <t>BRANCH-02</t>
         </is>
       </c>
       <c r="B75" s="16" t="inlineStr">
@@ -7336,27 +7336,27 @@
       </c>
       <c r="D75" s="16" t="inlineStr">
         <is>
-          <t>Revenue; Cash</t>
+          <t>Revenue</t>
         </is>
       </c>
       <c r="E75" s="16" t="inlineStr">
         <is>
-          <t>An offline-captured sale is LOST or DUPLICATED when connectivity returns — revenue understated (lost) or double-counted (duplicated), and the GL double-posted.</t>
+          <t>An offline terminal sells at a stale or wrong price/promotion because the cached catalog drifted from the master.</t>
         </is>
       </c>
       <c r="F75" s="16" t="inlineStr">
         <is>
-          <t>Completeness/Accuracy</t>
+          <t>Accuracy</t>
         </is>
       </c>
       <c r="G75" s="16" t="inlineStr">
         <is>
-          <t>Offline-to-online exactly-once sync: offline-captured sales replay idempotently on (tenant, client_uuid) via the pos_offline_sync dedup ledger. Two paths share the ledger — the portal/inventory POS (POST /api/portal/pos/offline-sync, item_id lines) and the touch register (POST /api/restaurant/offline-sync, menu sku lines, re-running the restaurant order→checkout so the server re-prices + 86-checks). A re-sent batch returns 'duplicate' (no second sale/GL); a failed op is a RETRYABLE tombstone (sale_no NULL) that never blocks a later replay, so a transient error is not a lost sale; each op runs in its own savepoint so one bad sale never poisons the batch.</t>
+          <t>Offline master-bundle export: GET /api/branches/master-bundle returns ONLY the active price-list + active promotions, time-stamped (generated_at). The offline terminal sells from this bundle, so it cannot ring a stale/withdrawn price or promo.</t>
         </is>
       </c>
       <c r="H75" s="17" t="inlineStr">
         <is>
-          <t>Det/Prev</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I75" s="17" t="inlineStr">
@@ -7366,37 +7366,37 @@
       </c>
       <c r="J75" s="17" t="inlineStr">
         <is>
-          <t>Per sync</t>
+          <t>Per bundle push</t>
         </is>
       </c>
       <c r="K75" s="16" t="inlineStr">
         <is>
-          <t>HQ Controller / IT</t>
+          <t>HQ Controller / Pricing</t>
         </is>
       </c>
       <c r="L75" s="17" t="inlineStr">
         <is>
-          <t>P10/P16</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="M75" s="16" t="inlineStr">
         <is>
-          <t>portal/offline-sync.service.ts (item_id path); restaurant/offline-sync.service.ts (register sku path, reuses dineIn create+checkout); pos_offline_sync dedup ledger; web lib/offline-pos.ts + lib/register-offline.ts; cutover/offline-sync.ts + restaurant-offline.ts (ToE) + e2e/register-offline.spec.ts</t>
+          <t>branches.service.ts masterBundle (active price-list + active promos + generated_at); branches.controller.ts; cutover/branch.ts (ToE)</t>
         </is>
       </c>
       <c r="N75" s="16" t="inlineStr">
         <is>
-          <t>Inspect the (tenant, client_uuid) dedup gate (sale_no NOT NULL), the per-op savepoint isolation, and the retryable-failure tombstone.</t>
+          <t>Inspect the bundle exports only active prices/promos with a timestamp.</t>
         </is>
       </c>
       <c r="O75" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: sync a batch (all synced, distinct SALE-), replay it (all duplicate, no double sale/GL), a bad op fails while neighbours sync, same uuid twice in a batch posts once, a transient failure replays to synced after the cause clears (re-performed by the offline-sync + restaurant-offline harnesses).</t>
+          <t>Re-perform: export the bundle; confirm it carries only active price-list/promotions + generated_at.</t>
         </is>
       </c>
       <c r="P75" s="16" t="inlineStr">
         <is>
-          <t>Sync recon report; terminal vs ledger counts; idempotency tests</t>
+          <t>Bundle metadata; bundle vs price-master diff</t>
         </is>
       </c>
       <c r="Q75" s="18" t="inlineStr">
@@ -7408,12 +7408,12 @@
     <row r="76">
       <c r="A76" s="11" t="inlineStr">
         <is>
-          <t>MFG-01</t>
+          <t>BRANCH-03</t>
         </is>
       </c>
       <c r="B76" s="12" t="inlineStr">
         <is>
-          <t>Manufacturing &amp; Costing</t>
+          <t>Multi-Branch &amp; Offline POS</t>
         </is>
       </c>
       <c r="C76" s="13" t="inlineStr">
@@ -7423,67 +7423,67 @@
       </c>
       <c r="D76" s="12" t="inlineStr">
         <is>
-          <t>Inventory; COGS</t>
+          <t>Revenue; Cash</t>
         </is>
       </c>
       <c r="E76" s="12" t="inlineStr">
         <is>
-          <t>Unauthorized BOM/recipe change mis-states standard cost and every downstream WIP/COGS posting; or the role that maintains the recipe also transacts on it.</t>
+          <t>An offline-captured sale is LOST or DUPLICATED when connectivity returns — revenue understated (lost) or double-counted (duplicated), and the GL double-posted.</t>
         </is>
       </c>
       <c r="F76" s="12" t="inlineStr">
         <is>
-          <t>Authorization</t>
+          <t>Completeness/Accuracy</t>
         </is>
       </c>
       <c r="G76" s="12" t="inlineStr">
         <is>
-          <t>BOM master maker-checker / SoD: the master BOM library (bom_master) is maintained + distributed by HQ separately from transacting; a tenant BOM submission is reviewed and merged by HQ on approval (a maker-checker over master data). Recipe roll-up (line cost + labor + overhead → cost per unit) is the standard-cost basis. Master-data access is segregated from production (R13).</t>
+          <t>Offline-to-online exactly-once sync: offline-captured sales replay idempotently on (tenant, client_uuid) via the pos_offline_sync dedup ledger. Two paths share the ledger — the portal/inventory POS (POST /api/portal/pos/offline-sync, item_id lines) and the touch register (POST /api/restaurant/offline-sync, menu sku lines, re-running the restaurant order→checkout so the server re-prices + 86-checks). A re-sent batch returns 'duplicate' (no second sale/GL); a failed op is a RETRYABLE tombstone (sale_no NULL) that never blocks a later replay, so a transient error is not a lost sale; each op runs in its own savepoint so one bad sale never poisons the batch.</t>
         </is>
       </c>
       <c r="H76" s="13" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det/Prev</t>
         </is>
       </c>
       <c r="I76" s="13" t="inlineStr">
         <is>
-          <t>Manual+Auto</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J76" s="13" t="inlineStr">
         <is>
-          <t>Per BOM change</t>
+          <t>Per sync</t>
         </is>
       </c>
       <c r="K76" s="12" t="inlineStr">
         <is>
-          <t>HQ MasterSteward / CostAccountant</t>
+          <t>HQ Controller / IT</t>
         </is>
       </c>
       <c r="L76" s="13" t="inlineStr">
         <is>
-          <t>P13</t>
+          <t>P10/P16</t>
         </is>
       </c>
       <c r="M76" s="12" t="inlineStr">
         <is>
-          <t>bom master + submissions (/api/bom/master, /api/bom/submissions, /api/portal/bom); manufacturing.service.ts BOM scaling; cutover/cpq.ts + manufacturing.ts (ToE)</t>
+          <t>portal/offline-sync.service.ts (item_id path); restaurant/offline-sync.service.ts (register sku path, reuses dineIn create+checkout); pos_offline_sync dedup ledger; web lib/offline-pos.ts + lib/register-offline.ts; cutover/offline-sync.ts + restaurant-offline.ts (ToE) + e2e/register-offline.spec.ts</t>
         </is>
       </c>
       <c r="N76" s="12" t="inlineStr">
         <is>
-          <t>Inspect BOM maintenance access + the submission→approve maker-checker + the costing roll-up.</t>
+          <t>Inspect the (tenant, client_uuid) dedup gate (sale_no NOT NULL), the per-op savepoint isolation, and the retryable-failure tombstone.</t>
         </is>
       </c>
       <c r="O76" s="12" t="inlineStr">
         <is>
-          <t>Sample BOM change is HQ-approved before use; standard cost rolls up correctly.</t>
+          <t>Re-perform: sync a batch (all synced, distinct SALE-), replay it (all duplicate, no double sale/GL), a bad op fails while neighbours sync, same uuid twice in a batch posts once, a transient failure replays to synced after the cause clears (re-performed by the offline-sync + restaurant-offline harnesses).</t>
         </is>
       </c>
       <c r="P76" s="12" t="inlineStr">
         <is>
-          <t>BOM approval log; costing roll-up</t>
+          <t>Sync recon report; terminal vs ledger counts; idempotency tests</t>
         </is>
       </c>
       <c r="Q76" s="18" t="inlineStr">
@@ -7495,7 +7495,7 @@
     <row r="77">
       <c r="A77" s="15" t="inlineStr">
         <is>
-          <t>MFG-02</t>
+          <t>MFG-01</t>
         </is>
       </c>
       <c r="B77" s="16" t="inlineStr">
@@ -7510,22 +7510,22 @@
       </c>
       <c r="D77" s="16" t="inlineStr">
         <is>
-          <t>WIP; Finished Goods; COGS</t>
+          <t>Inventory; COGS</t>
         </is>
       </c>
       <c r="E77" s="16" t="inlineStr">
         <is>
-          <t>Production cost is mis-stated: WIP not relieved, the conversion absorption left stranded, or a yield loss (spoilage/waste) silently capitalised into finished-goods inventory instead of expensed.</t>
+          <t>Unauthorized BOM/recipe change mis-states standard cost and every downstream WIP/COGS posting; or the role that maintains the recipe also transacts on it.</t>
         </is>
       </c>
       <c r="F77" s="16" t="inlineStr">
         <is>
-          <t>Valuation/Completeness/Accuracy</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="G77" s="16" t="inlineStr">
         <is>
-          <t>Production work-order WIP costing with a balanced JE at each step: ISSUE posts Dr 1250 WIP / Cr 1200 raw materials / Cr 2380 manufacturing-costs-applied (idempotent — re-issue is a no-op); COMPLETE posts Dr 1210 Finished Goods at the standard cost of the ACTUAL quantity produced + books the YIELD VARIANCE to 5810 (produced &lt; planned → debit 5810 loss; over-yield → credit) / Cr 1250 WIP — so WIP is always fully relieved and FG is never over-valued on a short yield. State machine Open→Released→Completed (out-of-order → BAD_STATUS). The 2380/1250 clearing balances tie out at close. Scrap/rework write-off of defective output posts to 5810 with CostAccountant authorization.</t>
+          <t>BOM master maker-checker / SoD: the master BOM library (bom_master) is maintained + distributed by HQ separately from transacting; a tenant BOM submission is reviewed and merged by HQ on approval (a maker-checker over master data). Recipe roll-up (line cost + labor + overhead → cost per unit) is the standard-cost basis. Master-data access is segregated from production (R13).</t>
         </is>
       </c>
       <c r="H77" s="17" t="inlineStr">
@@ -7535,17 +7535,17 @@
       </c>
       <c r="I77" s="17" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Manual+Auto</t>
         </is>
       </c>
       <c r="J77" s="17" t="inlineStr">
         <is>
-          <t>Per work order</t>
+          <t>Per BOM change</t>
         </is>
       </c>
       <c r="K77" s="16" t="inlineStr">
         <is>
-          <t>Warehouse / CostAccountant</t>
+          <t>HQ MasterSteward / CostAccountant</t>
         </is>
       </c>
       <c r="L77" s="17" t="inlineStr">
@@ -7555,22 +7555,22 @@
       </c>
       <c r="M77" s="16" t="inlineStr">
         <is>
-          <t>manufacturing.service.ts issue/complete (yield variance to 5810; fmt exposes yield_variance); manufacturing.controller.ts (bom_master/warehouse/exec); schema/manufacturing.ts work_orders; cutover/manufacturing.ts (ToE)</t>
+          <t>bom master + submissions (/api/bom/master, /api/bom/submissions, /api/portal/bom); manufacturing.service.ts BOM scaling; cutover/cpq.ts + manufacturing.ts (ToE)</t>
         </is>
       </c>
       <c r="N77" s="16" t="inlineStr">
         <is>
-          <t>Inspect the issue/complete JEs + the standard-unit-cost FG valuation + the yield-variance plug + the status guard.</t>
+          <t>Inspect BOM maintenance access + the submission→approve maker-checker + the costing roll-up.</t>
         </is>
       </c>
       <c r="O77" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: issue (WIP charged), complete at full yield (FG = full cost, no variance) and at a short yield (FG = std×produced, the lost yield to 5810, WIP nets to 0, TB balanced) — re-performed by the harness.</t>
+          <t>Sample BOM change is HQ-approved before use; standard cost rolls up correctly.</t>
         </is>
       </c>
       <c r="P77" s="16" t="inlineStr">
         <is>
-          <t>WO costing register (yield_variance per WO); production JEs</t>
+          <t>BOM approval log; costing roll-up</t>
         </is>
       </c>
       <c r="Q77" s="18" t="inlineStr">
@@ -7582,7 +7582,7 @@
     <row r="78">
       <c r="A78" s="11" t="inlineStr">
         <is>
-          <t>MFG-03</t>
+          <t>MFG-02</t>
         </is>
       </c>
       <c r="B78" s="12" t="inlineStr">
@@ -7597,27 +7597,27 @@
       </c>
       <c r="D78" s="12" t="inlineStr">
         <is>
-          <t>Inventory; COGS</t>
+          <t>WIP; Finished Goods; COGS</t>
         </is>
       </c>
       <c r="E78" s="12" t="inlineStr">
         <is>
-          <t>Standard-cost inventory received without isolating the price variance — actual purchase cost buried in inventory, COGS and PPV mis-stated.</t>
+          <t>Production cost is mis-stated: WIP not relieved, the conversion absorption left stranded, or a yield loss (spoilage/waste) silently capitalised into finished-goods inventory instead of expensed.</t>
         </is>
       </c>
       <c r="F78" s="12" t="inlineStr">
         <is>
-          <t>Valuation/Accuracy</t>
+          <t>Valuation/Completeness/Accuracy</t>
         </is>
       </c>
       <c r="G78" s="12" t="inlineStr">
         <is>
-          <t>Goods-receipt capitalisation under the configured costing method (FIFO/AVG/STD per tenant+item): FIFO/AVG → Dr 1200 / Cr 2000 at actual; STD → Dr 1200 at standard, the purchase-price variance booked to 5500 (unfavourable Dr / favourable Cr), Cr 2000 at actual — the PPV (5500) leg is the single balancing plug (= actual − standard, rounded once) so the JE can never reject UNBALANCED on independent per-leg rounding.</t>
+          <t>Production work-order WIP costing with a balanced JE at each step: ISSUE posts Dr 1250 WIP / Cr 1200 raw materials / Cr 2380 manufacturing-costs-applied (idempotent — re-issue is a no-op); COMPLETE posts Dr 1210 Finished Goods at the standard cost of the ACTUAL quantity produced + books the YIELD VARIANCE to 5810 (produced &lt; planned → debit 5810 loss; over-yield → credit) / Cr 1250 WIP — so WIP is always fully relieved and FG is never over-valued on a short yield. State machine Open→Released→Completed (out-of-order → BAD_STATUS). The 2380/1250 clearing balances tie out at close. Scrap/rework write-off of defective output posts to 5810 with CostAccountant authorization.</t>
         </is>
       </c>
       <c r="H78" s="13" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I78" s="13" t="inlineStr">
@@ -7627,12 +7627,12 @@
       </c>
       <c r="J78" s="13" t="inlineStr">
         <is>
-          <t>Per receipt</t>
+          <t>Per work order</t>
         </is>
       </c>
       <c r="K78" s="12" t="inlineStr">
         <is>
-          <t>CostAccountant</t>
+          <t>Warehouse / CostAccountant</t>
         </is>
       </c>
       <c r="L78" s="13" t="inlineStr">
@@ -7642,22 +7642,22 @@
       </c>
       <c r="M78" s="12" t="inlineStr">
         <is>
-          <t>costing.service.ts (config/valuation, GRV capitalisation + 5500 PPV); costing.controller.ts (masterdata); cutover/costing.ts (ToE)</t>
+          <t>manufacturing.service.ts issue/complete (yield variance to 5810; fmt exposes yield_variance); manufacturing.controller.ts (bom_master/warehouse/exec); schema/manufacturing.ts work_orders; cutover/manufacturing.ts (ToE)</t>
         </is>
       </c>
       <c r="N78" s="12" t="inlineStr">
         <is>
-          <t>Inspect the per-method capitalisation routing + the PPV plug.</t>
+          <t>Inspect the issue/complete JEs + the standard-unit-cost FG valuation + the yield-variance plug + the status guard.</t>
         </is>
       </c>
       <c r="O78" s="12" t="inlineStr">
         <is>
-          <t>Re-perform a STD receipt at actual ≠ standard → PPV isolated to 5500, JE balanced; valuation ties to GL 1200/1210/1250.</t>
+          <t>Re-perform: issue (WIP charged), complete at full yield (FG = full cost, no variance) and at a short yield (FG = std×produced, the lost yield to 5810, WIP nets to 0, TB balanced) — re-performed by the harness.</t>
         </is>
       </c>
       <c r="P78" s="12" t="inlineStr">
         <is>
-          <t>PPV postings; costing valuation</t>
+          <t>WO costing register (yield_variance per WO); production JEs</t>
         </is>
       </c>
       <c r="Q78" s="18" t="inlineStr">
@@ -7669,12 +7669,12 @@
     <row r="79">
       <c r="A79" s="15" t="inlineStr">
         <is>
-          <t>PROJ-01</t>
+          <t>MFG-03</t>
         </is>
       </c>
       <c r="B79" s="16" t="inlineStr">
         <is>
-          <t>Project Accounting</t>
+          <t>Manufacturing &amp; Costing</t>
         </is>
       </c>
       <c r="C79" s="17" t="inlineStr">
@@ -7684,27 +7684,27 @@
       </c>
       <c r="D79" s="16" t="inlineStr">
         <is>
-          <t>Project WIP; COGS</t>
+          <t>Inventory; COGS</t>
         </is>
       </c>
       <c r="E79" s="16" t="inlineStr">
         <is>
-          <t>Project cost mis-stated: a recoverable cost not captured, or an UN-recoverable (non-billable) cost capitalised into project WIP as an asset that overstates the unbilled balance and inflates margin.</t>
+          <t>Standard-cost inventory received without isolating the price variance — actual purchase cost buried in inventory, COGS and PPV mis-stated.</t>
         </is>
       </c>
       <c r="F79" s="16" t="inlineStr">
         <is>
-          <t>Valuation/Accuracy/Completeness</t>
+          <t>Valuation/Accuracy</t>
         </is>
       </c>
       <c r="G79" s="16" t="inlineStr">
         <is>
-          <t>Project cost capture with a balanced JE and a billable/non-billable split: a BILLABLE time/expense cost is a recoverable asset → Dr 1260 Project WIP / Cr 2390 Project Costs Applied (accumulates in cost_to_date, relieved to COGS at billing); a NON-BILLABLE cost is unrecoverable → EXPENSED immediately Dr 5800 Project Cost of Services / Cr 2390 (never enters the billable WIP), so the register's total_cost and true margin (billed − recognised − non-billable) reflect the absorbed cost. A non-positive amount → BAD_AMOUNT; first cost flips Open→Active.</t>
+          <t>Goods-receipt capitalisation under the configured costing method (FIFO/AVG/STD per tenant+item): FIFO/AVG → Dr 1200 / Cr 2000 at actual; STD → Dr 1200 at standard, the purchase-price variance booked to 5500 (unfavourable Dr / favourable Cr), Cr 2000 at actual — the PPV (5500) leg is the single balancing plug (= actual − standard, rounded once) so the JE can never reject UNBALANCED on independent per-leg rounding.</t>
         </is>
       </c>
       <c r="H79" s="17" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I79" s="17" t="inlineStr">
@@ -7714,12 +7714,12 @@
       </c>
       <c r="J79" s="17" t="inlineStr">
         <is>
-          <t>Per cost entry</t>
+          <t>Per receipt</t>
         </is>
       </c>
       <c r="K79" s="16" t="inlineStr">
         <is>
-          <t>ProjectAccountant</t>
+          <t>CostAccountant</t>
         </is>
       </c>
       <c r="L79" s="17" t="inlineStr">
@@ -7729,22 +7729,22 @@
       </c>
       <c r="M79" s="16" t="inlineStr">
         <is>
-          <t>projects.service.ts logCost (billable→1260, non-billable→5800; fmt exposes non_billable_cost/total_cost/margin); projects.controller.ts; schema/projects.ts project_entries.billable; cutover/projects.ts (ToE)</t>
+          <t>costing.service.ts (config/valuation, GRV capitalisation + 5500 PPV); costing.controller.ts (masterdata); cutover/costing.ts (ToE)</t>
         </is>
       </c>
       <c r="N79" s="16" t="inlineStr">
         <is>
-          <t>Inspect the billable/non-billable GL routing + the WIP vs immediate-expense decision + the margin roll-up.</t>
+          <t>Inspect the per-method capitalisation routing + the PPV plug.</t>
         </is>
       </c>
       <c r="O79" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: a billable cost capitalises to 1260; a non-billable cost expenses to 5800 (NOT WIP), cost_to_date unchanged, and the project margin absorbs it (re-performed by the harness).</t>
+          <t>Re-perform a STD receipt at actual ≠ standard → PPV isolated to 5500, JE balanced; valuation ties to GL 1200/1210/1250.</t>
         </is>
       </c>
       <c r="P79" s="16" t="inlineStr">
         <is>
-          <t>Project cost JEs; cost register (non_billable_cost)</t>
+          <t>PPV postings; costing valuation</t>
         </is>
       </c>
       <c r="Q79" s="18" t="inlineStr">
@@ -7756,7 +7756,7 @@
     <row r="80">
       <c r="A80" s="11" t="inlineStr">
         <is>
-          <t>PROJ-02</t>
+          <t>PROJ-01</t>
         </is>
       </c>
       <c r="B80" s="12" t="inlineStr">
@@ -7771,22 +7771,22 @@
       </c>
       <c r="D80" s="12" t="inlineStr">
         <is>
-          <t>Project WIP; Revenue; COGS</t>
+          <t>Project WIP; COGS</t>
         </is>
       </c>
       <c r="E80" s="12" t="inlineStr">
         <is>
-          <t>Revenue billed without matching cost — WIP not relieved, cost of services mis-stated, margin overstated.</t>
+          <t>Project cost mis-stated: a recoverable cost not captured, or an UN-recoverable (non-billable) cost capitalised into project WIP as an asset that overstates the unbilled balance and inflates margin.</t>
         </is>
       </c>
       <c r="F80" s="12" t="inlineStr">
         <is>
-          <t>Accuracy/Cut-off</t>
+          <t>Valuation/Accuracy/Completeness</t>
         </is>
       </c>
       <c r="G80" s="12" t="inlineStr">
         <is>
-          <t>Customer billing recognises revenue (Dr 1100 AR / Cr 4200 Project Revenue) and relieves the unbilled WIP to cost of services up to the unrecognised billable cost (Dr 5800 / Cr 1260) in the same event — matching cost to recognised revenue. Billing is by raw amount (T&amp;M) or by PERCENT of the contract for Fixed-price milestone billing; a Fixed-price contract is CAPPED at the contract value (cumulative billing can never exceed it — BILL_EXCEEDS_CONTRACT), so the customer is never over-billed (billed_pct/remaining_to_bill on the register). Billing is idempotent on (project, cumulative billed amount).</t>
+          <t>Project cost capture with a balanced JE and a billable/non-billable split: a BILLABLE time/expense cost is a recoverable asset → Dr 1260 Project WIP / Cr 2390 Project Costs Applied (accumulates in cost_to_date, relieved to COGS at billing); a NON-BILLABLE cost is unrecoverable → EXPENSED immediately Dr 5800 Project Cost of Services / Cr 2390 (never enters the billable WIP), so the register's total_cost and true margin (billed − recognised − non-billable) reflect the absorbed cost. A non-positive amount → BAD_AMOUNT; first cost flips Open→Active.</t>
         </is>
       </c>
       <c r="H80" s="13" t="inlineStr">
@@ -7801,12 +7801,12 @@
       </c>
       <c r="J80" s="13" t="inlineStr">
         <is>
-          <t>Per billing</t>
+          <t>Per cost entry</t>
         </is>
       </c>
       <c r="K80" s="12" t="inlineStr">
         <is>
-          <t>ProjectController / ArSpecialist</t>
+          <t>ProjectAccountant</t>
         </is>
       </c>
       <c r="L80" s="13" t="inlineStr">
@@ -7816,22 +7816,22 @@
       </c>
       <c r="M80" s="12" t="inlineStr">
         <is>
-          <t>projects.service.ts bill (revenue + WIP relief, idempotent); projects.controller.ts (R07 vs cost initiation); cutover/projects.ts (ToE)</t>
+          <t>projects.service.ts logCost (billable→1260, non-billable→5800; fmt exposes non_billable_cost/total_cost/margin); projects.controller.ts; schema/projects.ts project_entries.billable; cutover/projects.ts (ToE)</t>
         </is>
       </c>
       <c r="N80" s="12" t="inlineStr">
         <is>
-          <t>Inspect the bill JE + the WIP-relief matching + idempotency.</t>
+          <t>Inspect the billable/non-billable GL routing + the WIP vs immediate-expense decision + the margin roll-up.</t>
         </is>
       </c>
       <c r="O80" s="12" t="inlineStr">
         <is>
-          <t>Re-perform a billing → revenue recognised, WIP relieved to 5800 up to unrecognised cost, 1260 reduced; margin = billed − recognised cost (re-performed by the harness).</t>
+          <t>Re-perform: a billable cost capitalises to 1260; a non-billable cost expenses to 5800 (NOT WIP), cost_to_date unchanged, and the project margin absorbs it (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P80" s="12" t="inlineStr">
         <is>
-          <t>Billing JEs; margin/WIP measurement</t>
+          <t>Project cost JEs; cost register (non_billable_cost)</t>
         </is>
       </c>
       <c r="Q80" s="18" t="inlineStr">
@@ -7843,7 +7843,7 @@
     <row r="81">
       <c r="A81" s="15" t="inlineStr">
         <is>
-          <t>PROJ-03</t>
+          <t>PROJ-02</t>
         </is>
       </c>
       <c r="B81" s="16" t="inlineStr">
@@ -7853,171 +7853,171 @@
       </c>
       <c r="C81" s="17" t="inlineStr">
         <is>
-          <t>Detective</t>
+          <t>Application</t>
         </is>
       </c>
       <c r="D81" s="16" t="inlineStr">
         <is>
-          <t>Project WIP</t>
+          <t>Project WIP; Revenue; COGS</t>
         </is>
       </c>
       <c r="E81" s="16" t="inlineStr">
         <is>
-          <t>Unbilled WIP (1260) and the 2390 clearing balance not reviewed at close — stale or unrecoverable WIP carried into the financial statements.</t>
+          <t>Revenue billed without matching cost — WIP not relieved, cost of services mis-stated, margin overstated.</t>
         </is>
       </c>
       <c r="F81" s="16" t="inlineStr">
         <is>
-          <t>Valuation</t>
+          <t>Accuracy/Cut-off</t>
         </is>
       </c>
       <c r="G81" s="16" t="inlineStr">
         <is>
-          <t>Period-end review of unbilled-WIP (1260) aging and the project-costs-applied (2390) clearing tie-out; project margin (billed_to_date − recognised_cost − non-billable) reviewed at close. SoD: billing authorisation is segregated from cost initiation (R07).</t>
+          <t>Customer billing recognises revenue (Dr 1100 AR / Cr 4200 Project Revenue) and relieves the unbilled WIP to cost of services up to the unrecognised billable cost (Dr 5800 / Cr 1260) in the same event — matching cost to recognised revenue. Billing is by raw amount (T&amp;M) or by PERCENT of the contract for Fixed-price milestone billing; a Fixed-price contract is CAPPED at the contract value (cumulative billing can never exceed it — BILL_EXCEEDS_CONTRACT), so the customer is never over-billed (billed_pct/remaining_to_bill on the register). Billing is idempotent on (project, cumulative billed amount).</t>
         </is>
       </c>
       <c r="H81" s="17" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I81" s="17" t="inlineStr">
         <is>
-          <t>Hybrid</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J81" s="17" t="inlineStr">
         <is>
-          <t>Period</t>
+          <t>Per billing</t>
         </is>
       </c>
       <c r="K81" s="16" t="inlineStr">
         <is>
-          <t>ProjectAccountant / Controller</t>
+          <t>ProjectController / ArSpecialist</t>
         </is>
       </c>
       <c r="L81" s="17" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>P13</t>
         </is>
       </c>
       <c r="M81" s="16" t="inlineStr">
         <is>
-          <t>projects.service.ts fmt (wip/margin); the project register + entries; close review</t>
+          <t>projects.service.ts bill (revenue + WIP relief, idempotent); projects.controller.ts (R07 vs cost initiation); cutover/projects.ts (ToE)</t>
         </is>
       </c>
       <c r="N81" s="16" t="inlineStr">
         <is>
-          <t>Inspect 1260 aging + 2390 clearing + margin review evidence.</t>
+          <t>Inspect the bill JE + the WIP-relief matching + idempotency.</t>
         </is>
       </c>
       <c r="O81" s="16" t="inlineStr">
         <is>
-          <t>Sample projects: 1260 WIP agrees to cost_to_date − recognised; 2390 clears; stale WIP investigated.</t>
+          <t>Re-perform a billing → revenue recognised, WIP relieved to 5800 up to unrecognised cost, 1260 reduced; margin = billed − recognised cost (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P81" s="16" t="inlineStr">
         <is>
-          <t>WIP aging; 2390 clearing tie-out</t>
-        </is>
-      </c>
-      <c r="Q81" s="19" t="inlineStr">
-        <is>
-          <t>Partial</t>
+          <t>Billing JEs; margin/WIP measurement</t>
+        </is>
+      </c>
+      <c r="Q81" s="18" t="inlineStr">
+        <is>
+          <t>Implemented</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="11" t="inlineStr">
         <is>
-          <t>GL-01</t>
+          <t>PROJ-03</t>
         </is>
       </c>
       <c r="B82" s="12" t="inlineStr">
         <is>
-          <t>General Ledger</t>
+          <t>Project Accounting</t>
         </is>
       </c>
       <c r="C82" s="13" t="inlineStr">
         <is>
-          <t>Application</t>
+          <t>Detective</t>
         </is>
       </c>
       <c r="D82" s="12" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Project WIP</t>
         </is>
       </c>
       <c r="E82" s="12" t="inlineStr">
         <is>
-          <t>Unbalanced / one-sided journal entries.</t>
+          <t>Unbilled WIP (1260) and the 2390 clearing balance not reviewed at close — stale or unrecoverable WIP carried into the financial statements.</t>
         </is>
       </c>
       <c r="F82" s="12" t="inlineStr">
         <is>
-          <t>Accuracy</t>
+          <t>Valuation</t>
         </is>
       </c>
       <c r="G82" s="12" t="inlineStr">
         <is>
-          <t>Double-entry balanced-by-construction — Σdebit=Σcredit enforced; each line single-sided &amp; non-negative.</t>
+          <t>Period-end review of unbilled-WIP (1260) aging and the project-costs-applied (2390) clearing tie-out; project margin (billed_to_date − recognised_cost − non-billable) reviewed at close. SoD: billing authorisation is segregated from cost initiation (R07).</t>
         </is>
       </c>
       <c r="H82" s="13" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I82" s="13" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Hybrid</t>
         </is>
       </c>
       <c r="J82" s="13" t="inlineStr">
         <is>
-          <t>Per JE</t>
+          <t>Period</t>
         </is>
       </c>
       <c r="K82" s="12" t="inlineStr">
         <is>
-          <t>Controller</t>
+          <t>ProjectAccountant / Controller</t>
         </is>
       </c>
       <c r="L82" s="13" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="M82" s="12" t="inlineStr">
         <is>
-          <t>ledger.service.ts (postEntry — UNBALANCED / INVALID_LINE)</t>
+          <t>projects.service.ts fmt (wip/margin); the project register + entries; close review</t>
         </is>
       </c>
       <c r="N82" s="12" t="inlineStr">
         <is>
-          <t>Inspect balance + line invariants.</t>
+          <t>Inspect 1260 aging + 2390 clearing + margin review evidence.</t>
         </is>
       </c>
       <c r="O82" s="12" t="inlineStr">
         <is>
-          <t>Attempt unbalanced JE → rejected.</t>
+          <t>Sample projects: 1260 WIP agrees to cost_to_date − recognised; 2390 clears; stale WIP investigated.</t>
         </is>
       </c>
       <c r="P82" s="12" t="inlineStr">
         <is>
-          <t>Invariant test</t>
-        </is>
-      </c>
-      <c r="Q82" s="18" t="inlineStr">
-        <is>
-          <t>Implemented</t>
+          <t>WIP aging; 2390 clearing tie-out</t>
+        </is>
+      </c>
+      <c r="Q82" s="19" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="15" t="inlineStr">
         <is>
-          <t>GL-02</t>
+          <t>GL-01</t>
         </is>
       </c>
       <c r="B83" s="16" t="inlineStr">
@@ -8037,17 +8037,17 @@
       </c>
       <c r="E83" s="16" t="inlineStr">
         <is>
-          <t>Postings to a closed period distort reported results.</t>
+          <t>Unbalanced / one-sided journal entries.</t>
         </is>
       </c>
       <c r="F83" s="16" t="inlineStr">
         <is>
-          <t>Cutoff</t>
+          <t>Accuracy</t>
         </is>
       </c>
       <c r="G83" s="16" t="inlineStr">
         <is>
-          <t>Period-close lockout — postings to a CLOSED fiscal period are rejected (per-tenant calendar).</t>
+          <t>Double-entry balanced-by-construction — Σdebit=Σcredit enforced; each line single-sided &amp; non-negative.</t>
         </is>
       </c>
       <c r="H83" s="17" t="inlineStr">
@@ -8077,22 +8077,22 @@
       </c>
       <c r="M83" s="16" t="inlineStr">
         <is>
-          <t>ledger.service.ts (postEntry PERIOD_CLOSED); fiscal_periods</t>
+          <t>ledger.service.ts (postEntry — UNBALANCED / INVALID_LINE)</t>
         </is>
       </c>
       <c r="N83" s="16" t="inlineStr">
         <is>
-          <t>Inspect close check.</t>
+          <t>Inspect balance + line invariants.</t>
         </is>
       </c>
       <c r="O83" s="16" t="inlineStr">
         <is>
-          <t>Post to closed period → rejected; review exceptions.</t>
+          <t>Attempt unbalanced JE → rejected.</t>
         </is>
       </c>
       <c r="P83" s="16" t="inlineStr">
         <is>
-          <t>Close-lock test</t>
+          <t>Invariant test</t>
         </is>
       </c>
       <c r="Q83" s="18" t="inlineStr">
@@ -8104,7 +8104,7 @@
     <row r="84">
       <c r="A84" s="11" t="inlineStr">
         <is>
-          <t>GL-03</t>
+          <t>GL-02</t>
         </is>
       </c>
       <c r="B84" s="12" t="inlineStr">
@@ -8119,22 +8119,22 @@
       </c>
       <c r="D84" s="12" t="inlineStr">
         <is>
-          <t>Equity</t>
+          <t>All</t>
         </is>
       </c>
       <c r="E84" s="12" t="inlineStr">
         <is>
-          <t>Unauthorized year-end close / RE roll.</t>
+          <t>Postings to a closed period distort reported results.</t>
         </is>
       </c>
       <c r="F84" s="12" t="inlineStr">
         <is>
-          <t>Cutoff/Authorization</t>
+          <t>Cutoff</t>
         </is>
       </c>
       <c r="G84" s="12" t="inlineStr">
         <is>
-          <t>Year-end close restricted to 'exec'; closing entries roll to retained earnings.</t>
+          <t>Period-close lockout — postings to a CLOSED fiscal period are rejected (per-tenant calendar).</t>
         </is>
       </c>
       <c r="H84" s="13" t="inlineStr">
@@ -8144,42 +8144,42 @@
       </c>
       <c r="I84" s="13" t="inlineStr">
         <is>
-          <t>Auto+Manual</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J84" s="13" t="inlineStr">
         <is>
-          <t>Annual</t>
+          <t>Per JE</t>
         </is>
       </c>
       <c r="K84" s="12" t="inlineStr">
         <is>
-          <t>CFO / Controller</t>
+          <t>Controller</t>
         </is>
       </c>
       <c r="L84" s="13" t="inlineStr">
         <is>
-          <t>P10/P11</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="M84" s="12" t="inlineStr">
         <is>
-          <t>ledger.controller.ts (close-year @Permissions exec); closeYear</t>
+          <t>ledger.service.ts (postEntry PERIOD_CLOSED); fiscal_periods</t>
         </is>
       </c>
       <c r="N84" s="12" t="inlineStr">
         <is>
-          <t>Inspect permission + closing logic.</t>
+          <t>Inspect close check.</t>
         </is>
       </c>
       <c r="O84" s="12" t="inlineStr">
         <is>
-          <t>Attempt close w/o exec → 403; review annual close.</t>
+          <t>Post to closed period → rejected; review exceptions.</t>
         </is>
       </c>
       <c r="P84" s="12" t="inlineStr">
         <is>
-          <t>Close package</t>
+          <t>Close-lock test</t>
         </is>
       </c>
       <c r="Q84" s="18" t="inlineStr">
@@ -8191,7 +8191,7 @@
     <row r="85">
       <c r="A85" s="15" t="inlineStr">
         <is>
-          <t>GL-04</t>
+          <t>GL-03</t>
         </is>
       </c>
       <c r="B85" s="16" t="inlineStr">
@@ -8206,22 +8206,22 @@
       </c>
       <c r="D85" s="16" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Equity</t>
         </is>
       </c>
       <c r="E85" s="16" t="inlineStr">
         <is>
-          <t>Concurrent posting double-books the same source doc.</t>
+          <t>Unauthorized year-end close / RE roll.</t>
         </is>
       </c>
       <c r="F85" s="16" t="inlineStr">
         <is>
-          <t>Completeness/Accuracy</t>
+          <t>Cutoff/Authorization</t>
         </is>
       </c>
       <c r="G85" s="16" t="inlineStr">
         <is>
-          <t>Ledger idempotency — UNIQUE (tenant,source,source_ref,ledger) + ON CONFLICT DO NOTHING in postEntry.</t>
+          <t>Year-end close restricted to 'exec'; closing entries roll to retained earnings.</t>
         </is>
       </c>
       <c r="H85" s="17" t="inlineStr">
@@ -8231,42 +8231,42 @@
       </c>
       <c r="I85" s="17" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="J85" s="17" t="inlineStr">
         <is>
-          <t>Per JE</t>
+          <t>Annual</t>
         </is>
       </c>
       <c r="K85" s="16" t="inlineStr">
         <is>
-          <t>Eng Lead / Controller</t>
+          <t>CFO / Controller</t>
         </is>
       </c>
       <c r="L85" s="17" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P10/P11</t>
         </is>
       </c>
       <c r="M85" s="16" t="inlineStr">
         <is>
-          <t>schema/ledger.ts (ux_je_idem); ledger.service.ts; migration 0058</t>
+          <t>ledger.controller.ts (close-year @Permissions exec); closeYear</t>
         </is>
       </c>
       <c r="N85" s="16" t="inlineStr">
         <is>
-          <t>Inspect unique index + conflict handling.</t>
+          <t>Inspect permission + closing logic.</t>
         </is>
       </c>
       <c r="O85" s="16" t="inlineStr">
         <is>
-          <t>Concurrent identical post → single entry.</t>
+          <t>Attempt close w/o exec → 403; review annual close.</t>
         </is>
       </c>
       <c r="P85" s="16" t="inlineStr">
         <is>
-          <t>Dedup test</t>
+          <t>Close package</t>
         </is>
       </c>
       <c r="Q85" s="18" t="inlineStr">
@@ -8278,7 +8278,7 @@
     <row r="86">
       <c r="A86" s="11" t="inlineStr">
         <is>
-          <t>GL-05</t>
+          <t>GL-04</t>
         </is>
       </c>
       <c r="B86" s="12" t="inlineStr">
@@ -8298,17 +8298,17 @@
       </c>
       <c r="E86" s="12" t="inlineStr">
         <is>
-          <t>Manual JE posted without independent review (override risk).</t>
+          <t>Concurrent posting double-books the same source doc.</t>
         </is>
       </c>
       <c r="F86" s="12" t="inlineStr">
         <is>
-          <t>Authorization</t>
+          <t>Completeness/Accuracy</t>
         </is>
       </c>
       <c r="G86" s="12" t="inlineStr">
         <is>
-          <t>Manual journal-entry maker-checker — preparer ≠ approver before a manual JE posts.</t>
+          <t>Ledger idempotency — UNIQUE (tenant,source,source_ref,ledger) + ON CONFLICT DO NOTHING in postEntry.</t>
         </is>
       </c>
       <c r="H86" s="13" t="inlineStr">
@@ -8318,17 +8318,17 @@
       </c>
       <c r="I86" s="13" t="inlineStr">
         <is>
-          <t>Auto+Manual</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J86" s="13" t="inlineStr">
         <is>
-          <t>Per manual JE</t>
+          <t>Per JE</t>
         </is>
       </c>
       <c r="K86" s="12" t="inlineStr">
         <is>
-          <t>Controller</t>
+          <t>Eng Lead / Controller</t>
         </is>
       </c>
       <c r="L86" s="13" t="inlineStr">
@@ -8338,22 +8338,22 @@
       </c>
       <c r="M86" s="12" t="inlineStr">
         <is>
-          <t>ledger.service.ts (postEntry pendingApproval→Draft; approveEntry preparer≠approver; rejectEntry); ledger.controller.ts (gl_post posts / gl_close approves); cutover/compliance.ts (ToE)</t>
+          <t>schema/ledger.ts (ux_je_idem); ledger.service.ts; migration 0058</t>
         </is>
       </c>
       <c r="N86" s="12" t="inlineStr">
         <is>
-          <t>Inspect JE approval routing.</t>
+          <t>Inspect unique index + conflict handling.</t>
         </is>
       </c>
       <c r="O86" s="12" t="inlineStr">
         <is>
-          <t>Sample manual JEs: approver ≠ preparer; Draft excluded from balances until approved (re-performed by the harness).</t>
+          <t>Concurrent identical post → single entry.</t>
         </is>
       </c>
       <c r="P86" s="12" t="inlineStr">
         <is>
-          <t>JE approvals</t>
+          <t>Dedup test</t>
         </is>
       </c>
       <c r="Q86" s="18" t="inlineStr">
@@ -8365,7 +8365,7 @@
     <row r="87">
       <c r="A87" s="15" t="inlineStr">
         <is>
-          <t>GL-06</t>
+          <t>GL-05</t>
         </is>
       </c>
       <c r="B87" s="16" t="inlineStr">
@@ -8385,17 +8385,17 @@
       </c>
       <c r="E87" s="16" t="inlineStr">
         <is>
-          <t>Operator mis-posts to another tenant's books.</t>
+          <t>Manual JE posted without independent review (override risk).</t>
         </is>
       </c>
       <c r="F87" s="16" t="inlineStr">
         <is>
-          <t>Validity</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="G87" s="16" t="inlineStr">
         <is>
-          <t>HQ cross-tenant posting gated to Admin (explicit tenant override); others pinned to context (also RLS).</t>
+          <t>Manual journal-entry maker-checker — preparer ≠ approver before a manual JE posts.</t>
         </is>
       </c>
       <c r="H87" s="17" t="inlineStr">
@@ -8405,42 +8405,42 @@
       </c>
       <c r="I87" s="17" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="J87" s="17" t="inlineStr">
         <is>
-          <t>Per JE</t>
+          <t>Per manual JE</t>
         </is>
       </c>
       <c r="K87" s="16" t="inlineStr">
         <is>
-          <t>Eng Lead</t>
+          <t>Controller</t>
         </is>
       </c>
       <c r="L87" s="17" t="inlineStr">
         <is>
-          <t>P10/P11</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="M87" s="16" t="inlineStr">
         <is>
-          <t>ledger.controller.ts (hqTenant)</t>
+          <t>ledger.service.ts (postEntry pendingApproval→Draft; approveEntry preparer≠approver; rejectEntry); ledger.controller.ts (gl_post posts / gl_close approves); cutover/compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N87" s="16" t="inlineStr">
         <is>
-          <t>Inspect Admin gating of tenant_id.</t>
+          <t>Inspect JE approval routing.</t>
         </is>
       </c>
       <c r="O87" s="16" t="inlineStr">
         <is>
-          <t>Non-Admin tenant override ignored; Admin audited.</t>
+          <t>Sample manual JEs: approver ≠ preparer; Draft excluded from balances until approved (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P87" s="16" t="inlineStr">
         <is>
-          <t>Override test</t>
+          <t>JE approvals</t>
         </is>
       </c>
       <c r="Q87" s="18" t="inlineStr">
@@ -8452,7 +8452,7 @@
     <row r="88">
       <c r="A88" s="11" t="inlineStr">
         <is>
-          <t>GL-07</t>
+          <t>GL-06</t>
         </is>
       </c>
       <c r="B88" s="12" t="inlineStr">
@@ -8467,27 +8467,27 @@
       </c>
       <c r="D88" s="12" t="inlineStr">
         <is>
-          <t>Cash</t>
+          <t>All</t>
         </is>
       </c>
       <c r="E88" s="12" t="inlineStr">
         <is>
-          <t>Statement of cash flows mis-stated or doesn't tie to the change in cash.</t>
+          <t>Operator mis-posts to another tenant's books.</t>
         </is>
       </c>
       <c r="F88" s="12" t="inlineStr">
         <is>
-          <t>Accuracy/Completeness</t>
+          <t>Validity</t>
         </is>
       </c>
       <c r="G88" s="12" t="inlineStr">
         <is>
-          <t>Statement of Cash Flows (indirect) reconstructed from the GL: net income + non-cash add-backs + working-capital + investing + financing; year-end CLOSE entries excluded; reconciles to Δcash (1000/1010/1020) by construction with a `reconciled` tie-out flag. A direct-method view presents the same operating cash by receipt/payment nature (receipts from customers, payments to suppliers, tax &amp; payroll) and also reconciles to Δcash; a forward cash-flow forecast projects open AR (inflows) and AP (outflows) by due date from today's cash balance for treasury/collections planning.</t>
+          <t>HQ cross-tenant posting gated to Admin (explicit tenant override); others pinned to context (also RLS).</t>
         </is>
       </c>
       <c r="H88" s="13" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I88" s="13" t="inlineStr">
@@ -8497,37 +8497,37 @@
       </c>
       <c r="J88" s="13" t="inlineStr">
         <is>
-          <t>Per period</t>
+          <t>Per JE</t>
         </is>
       </c>
       <c r="K88" s="12" t="inlineStr">
         <is>
-          <t>Controller</t>
+          <t>Eng Lead</t>
         </is>
       </c>
       <c r="L88" s="13" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P10/P11</t>
         </is>
       </c>
       <c r="M88" s="12" t="inlineStr">
         <is>
-          <t>ledger.service.ts (cashFlowStatement, cashFlowDirect, cashFlowForecast); ledger.controller.ts (GET cash-flow, cash-flow-direct, cash-flow-forecast); cutover/basics.ts (ToE)</t>
+          <t>ledger.controller.ts (hqTenant)</t>
         </is>
       </c>
       <c r="N88" s="12" t="inlineStr">
         <is>
-          <t>Inspect SCF derivation + reconciliation flag; inspect direct-method bucketing and forecast projection.</t>
+          <t>Inspect Admin gating of tenant_id.</t>
         </is>
       </c>
       <c r="O88" s="12" t="inlineStr">
         <is>
-          <t>Run cash-flow over a seeded period — activities tie to the movement in cash; CLOSE excluded; direct method ties to the same operating cash and Δcash; forecast buckets open AR/AP by due week (re-performed by the harness).</t>
+          <t>Non-Admin tenant override ignored; Admin audited.</t>
         </is>
       </c>
       <c r="P88" s="12" t="inlineStr">
         <is>
-          <t>Cash-flow reconciliation; direct-method buckets; forecast schedule</t>
+          <t>Override test</t>
         </is>
       </c>
       <c r="Q88" s="18" t="inlineStr">
@@ -8539,7 +8539,7 @@
     <row r="89">
       <c r="A89" s="15" t="inlineStr">
         <is>
-          <t>GL-08</t>
+          <t>GL-07</t>
         </is>
       </c>
       <c r="B89" s="16" t="inlineStr">
@@ -8554,27 +8554,27 @@
       </c>
       <c r="D89" s="16" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Cash</t>
         </is>
       </c>
       <c r="E89" s="16" t="inlineStr">
         <is>
-          <t>Standing/period accruals missed, posted unbalanced, or posted without approval; manual re-keying error.</t>
+          <t>Statement of cash flows mis-stated or doesn't tie to the change in cash.</t>
         </is>
       </c>
       <c r="F89" s="16" t="inlineStr">
         <is>
-          <t>Completeness/Accuracy/Authorization</t>
+          <t>Accuracy/Completeness</t>
         </is>
       </c>
       <c r="G89" s="16" t="inlineStr">
         <is>
-          <t>Recurring/template journal entries: a template's lines are validated balanced (Σdebit=Σcredit) AT SAVE TIME (unbalanced → UNBALANCED), so a broken template can never be persisted. The scheduled job gl_recurring_journals (cron / daily scheduler) posts every due template as a DRAFT JE through the normal maker-checker flow (GL-05) — a different user must approve before it affects balances — and rolls next_run_date forward. Idempotent: next_run_date advanced on posting + the (tenant,source,source_ref,ledger) idempotency key dedupes a same-day re-run. Templates can be paused/resumed without losing history.</t>
+          <t>Statement of Cash Flows (indirect) reconstructed from the GL: net income + non-cash add-backs + working-capital + investing + financing; year-end CLOSE entries excluded; reconciles to Δcash (1000/1010/1020) by construction with a `reconciled` tie-out flag. A direct-method view presents the same operating cash by receipt/payment nature (receipts from customers, payments to suppliers, tax &amp; payroll) and also reconciles to Δcash; a forward cash-flow forecast projects open AR (inflows) and AP (outflows) by due date from today's cash balance for treasury/collections planning.</t>
         </is>
       </c>
       <c r="H89" s="17" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I89" s="17" t="inlineStr">
@@ -8584,7 +8584,7 @@
       </c>
       <c r="J89" s="17" t="inlineStr">
         <is>
-          <t>Per due date / per template</t>
+          <t>Per period</t>
         </is>
       </c>
       <c r="K89" s="16" t="inlineStr">
@@ -8599,22 +8599,22 @@
       </c>
       <c r="M89" s="16" t="inlineStr">
         <is>
-          <t>ledger.service.ts (createRecurring balanced-at-save, runDueRecurring→postEntry pendingApproval, setRecurringActive); ledger.controller.ts (gl_post creates/runs); bi.service.ts (gl_recurring_journals); schema/ledger.ts (recurring_journals) + migration 0119; cutover/basics.ts (ToE)</t>
+          <t>ledger.service.ts (cashFlowStatement, cashFlowDirect, cashFlowForecast); ledger.controller.ts (GET cash-flow, cash-flow-direct, cash-flow-forecast); cutover/basics.ts (ToE)</t>
         </is>
       </c>
       <c r="N89" s="16" t="inlineStr">
         <is>
-          <t>Inspect template balance validation + scheduled posting as Draft + idempotency.</t>
+          <t>Inspect SCF derivation + reconciliation flag; inspect direct-method bucketing and forecast projection.</t>
         </is>
       </c>
       <c r="O89" s="16" t="inlineStr">
         <is>
-          <t>Unbalanced template → UNBALANCED; due template posts a Draft JE (excluded from TB) into the pending queue; re-run posts nothing; a second user approves → accrual hits the GL (re-performed by the harness).</t>
+          <t>Run cash-flow over a seeded period — activities tie to the movement in cash; CLOSE excluded; direct method ties to the same operating cash and Δcash; forecast buckets open AR/AP by due week (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P89" s="16" t="inlineStr">
         <is>
-          <t>Recurring-journal templates; scheduled run log; JE approvals</t>
+          <t>Cash-flow reconciliation; direct-method buckets; forecast schedule</t>
         </is>
       </c>
       <c r="Q89" s="18" t="inlineStr">
@@ -8626,7 +8626,7 @@
     <row r="90">
       <c r="A90" s="11" t="inlineStr">
         <is>
-          <t>GL-09</t>
+          <t>GL-08</t>
         </is>
       </c>
       <c r="B90" s="12" t="inlineStr">
@@ -8641,27 +8641,27 @@
       </c>
       <c r="D90" s="12" t="inlineStr">
         <is>
-          <t>Prepaid expenses; Operating expense</t>
+          <t>All</t>
         </is>
       </c>
       <c r="E90" s="12" t="inlineStr">
         <is>
-          <t>Prepaid expense not amortized over its term — expense mis-stated, prepaid asset overstated.</t>
+          <t>Standing/period accruals missed, posted unbalanced, or posted without approval; manual re-keying error.</t>
         </is>
       </c>
       <c r="F90" s="12" t="inlineStr">
         <is>
-          <t>Accuracy/Completeness</t>
+          <t>Completeness/Accuracy/Authorization</t>
         </is>
       </c>
       <c r="G90" s="12" t="inlineStr">
         <is>
-          <t>Prepaid amortization schedules: a prepaid asset (insurance/rent paid up front) is registered once with a total + term; the scheduled job gl_prepaid_amortize posts a straight-line slice each period (Dr expense / Cr 1280), the last period taking the remainder so the asset fully clears. Idempotent per (schedule, period) via the JE idempotency key + next_run_date advance.</t>
+          <t>Recurring/template journal entries: a template's lines are validated balanced (Σdebit=Σcredit) AT SAVE TIME (unbalanced → UNBALANCED), so a broken template can never be persisted. The scheduled job gl_recurring_journals (cron / daily scheduler) posts every due template as a DRAFT JE through the normal maker-checker flow (GL-05) — a different user must approve before it affects balances — and rolls next_run_date forward. Idempotent: next_run_date advanced on posting + the (tenant,source,source_ref,ledger) idempotency key dedupes a same-day re-run. Templates can be paused/resumed without losing history.</t>
         </is>
       </c>
       <c r="H90" s="13" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I90" s="13" t="inlineStr">
@@ -8671,7 +8671,7 @@
       </c>
       <c r="J90" s="13" t="inlineStr">
         <is>
-          <t>Per period / per schedule</t>
+          <t>Per due date / per template</t>
         </is>
       </c>
       <c r="K90" s="12" t="inlineStr">
@@ -8686,22 +8686,22 @@
       </c>
       <c r="M90" s="12" t="inlineStr">
         <is>
-          <t>ledger.service.ts (createPrepaid, runDuePrepaid); ledger.controller.ts (gl_post); bi.service.ts (gl_prepaid_amortize); schema/ledger.ts (prepaid_schedules) + migration 0120; cutover/basics.ts (ToE)</t>
+          <t>ledger.service.ts (createRecurring balanced-at-save, runDueRecurring→postEntry pendingApproval, setRecurringActive); ledger.controller.ts (gl_post creates/runs); bi.service.ts (gl_recurring_journals); schema/ledger.ts (recurring_journals) + migration 0119; cutover/basics.ts (ToE)</t>
         </is>
       </c>
       <c r="N90" s="12" t="inlineStr">
         <is>
-          <t>Inspect amortization slice + final-period remainder + idempotency.</t>
+          <t>Inspect template balance validation + scheduled posting as Draft + idempotency.</t>
         </is>
       </c>
       <c r="O90" s="12" t="inlineStr">
         <is>
-          <t>Register a 12-month prepaid; run amortizes 1/12 to expense; re-run posts nothing (re-performed by the harness).</t>
+          <t>Unbalanced template → UNBALANCED; due template posts a Draft JE (excluded from TB) into the pending queue; re-run posts nothing; a second user approves → accrual hits the GL (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P90" s="12" t="inlineStr">
         <is>
-          <t>Prepaid schedules; amortization run log</t>
+          <t>Recurring-journal templates; scheduled run log; JE approvals</t>
         </is>
       </c>
       <c r="Q90" s="18" t="inlineStr">
@@ -8713,7 +8713,7 @@
     <row r="91">
       <c r="A91" s="15" t="inlineStr">
         <is>
-          <t>GL-10</t>
+          <t>GL-09</t>
         </is>
       </c>
       <c r="B91" s="16" t="inlineStr">
@@ -8728,27 +8728,27 @@
       </c>
       <c r="D91" s="16" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Prepaid expenses; Operating expense</t>
         </is>
       </c>
       <c r="E91" s="16" t="inlineStr">
         <is>
-          <t>A new company starts on a chart of accounts with no industry guidance — staff post to wrong/ambiguous accounts; or an industry template drifts from the GL engine's fixed posting codes so a posting targets an account that does not exist (mis-statement / unposted transaction).</t>
+          <t>Prepaid expense not amortized over its term — expense mis-stated, prepaid asset overstated.</t>
         </is>
       </c>
       <c r="F91" s="16" t="inlineStr">
         <is>
-          <t>Completeness/Accuracy/Presentation</t>
+          <t>Accuracy/Completeness</t>
         </is>
       </c>
       <c r="G91" s="16" t="inlineStr">
         <is>
-          <t>Industry Chart-of-Accounts templates: the GL engine binds to a FIXED, global account universe (canonical codes are immutable); each tenant additionally gets a per-tenant overlay (tenant_accounts) curating which canonical accounts are active and how they are named/grouped for its industry. At company creation the customer picks an industry (restaurant/retail/distribution/services/general) and the chosen template is materialised into the overlay (provisionTenantCoA) inside the signup transaction, right after fiscal-year provisioning; adopting an industry pack later does the same. Every template code is asserted to exist in the canonical chart at boot (assertTemplatesSubsetOf in seedChartOfAccounts) so a drifted template fails fast and can never reach a tenant. Provisioning is idempotent + additive (never deletes) so re-running only adds missing accounts. The overlay NEVER gates postings — it scopes the picker / Chart-of-Accounts view only; reports surface any account that is active OR carries activity, so a curated-out account that receives a posting still appears.</t>
+          <t>Prepaid amortization schedules: a prepaid asset (insurance/rent paid up front) is registered once with a total + term; the scheduled job gl_prepaid_amortize posts a straight-line slice each period (Dr expense / Cr 1280), the last period taking the remainder so the asset fully clears. Idempotent per (schedule, period) via the JE idempotency key + next_run_date advance.</t>
         </is>
       </c>
       <c r="H91" s="17" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I91" s="17" t="inlineStr">
@@ -8758,7 +8758,7 @@
       </c>
       <c r="J91" s="17" t="inlineStr">
         <is>
-          <t>At company creation / per pack adopt</t>
+          <t>Per period / per schedule</t>
         </is>
       </c>
       <c r="K91" s="16" t="inlineStr">
@@ -8773,22 +8773,22 @@
       </c>
       <c r="M91" s="16" t="inlineStr">
         <is>
-          <t>ledger.service.ts (provisionTenantCoA idempotent+additive, tenant-aware listAccounts, seedChartOfAccounts→assertTemplatesSubsetOf); coa-templates.ts (industry templates + subset assertion); billing.service.ts signup (industry→provisionTenantCoA in-txn); onboarding.service.ts applyPack (pack adopt provisions CoA); schema/ledger.ts tenant_accounts + tenants.industry + migration 0139; cutover/basics.ts + compliance.ts (ToE)</t>
+          <t>ledger.service.ts (createPrepaid, runDuePrepaid); ledger.controller.ts (gl_post); bi.service.ts (gl_prepaid_amortize); schema/ledger.ts (prepaid_schedules) + migration 0120; cutover/basics.ts (ToE)</t>
         </is>
       </c>
       <c r="N91" s="16" t="inlineStr">
         <is>
-          <t>Inspect the boot subset assertion + signup provisioning + the overlay-is-presentation-only read path.</t>
+          <t>Inspect amortization slice + final-period remainder + idempotency.</t>
         </is>
       </c>
       <c r="O91" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: a template referencing an unknown code fails the boot assertion; signup with industry=restaurant materialises a curated, industry-named chart (4000='Food &amp; Beverage Sales') that omits non-F&amp;B accounts; ?all=true still returns the full canonical universe (overlay never gates posting); signup with no industry ⇒ general = the full live chart (re-performed by the harnesses).</t>
+          <t>Register a 12-month prepaid; run amortizes 1/12 to expense; re-run posts nothing (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P91" s="16" t="inlineStr">
         <is>
-          <t>Industry templates; tenant_accounts overlay; signup provisioning log</t>
+          <t>Prepaid schedules; amortization run log</t>
         </is>
       </c>
       <c r="Q91" s="18" t="inlineStr">
@@ -8800,7 +8800,7 @@
     <row r="92">
       <c r="A92" s="11" t="inlineStr">
         <is>
-          <t>GL-11</t>
+          <t>GL-10</t>
         </is>
       </c>
       <c r="B92" s="12" t="inlineStr">
@@ -8820,17 +8820,17 @@
       </c>
       <c r="E92" s="12" t="inlineStr">
         <is>
-          <t>Chart of Accounts changed without authorisation; account code changed after postings exist; account deactivated while carrying a non-zero balance; manual JE posted directly to a control account (AR/AP/INV/FA), bypassing the sub-ledger and hiding a sub-ledger discrepancy.</t>
+          <t>A new company starts on a chart of accounts with no industry guidance — staff post to wrong/ambiguous accounts; or an industry template drifts from the GL engine's fixed posting codes so a posting targets an account that does not exist (mis-statement / unposted transaction).</t>
         </is>
       </c>
       <c r="F92" s="12" t="inlineStr">
         <is>
-          <t>Authorization/Completeness/Accuracy</t>
+          <t>Completeness/Accuracy/Presentation</t>
         </is>
       </c>
       <c r="G92" s="12" t="inlineStr">
         <is>
-          <t>CoA Change Control: account creation/update/deactivation requires the gl_coa permission (held by FinancialController, not GlAccountant — separated from gl_post per SoD). Disabling postability on an account that already has posted entries is rejected (CODE_HAS_POSTINGS). Deactivation is rejected if the account carries a non-zero net balance (ACCOUNT_HAS_BALANCE) — prevents orphaning a balance in a closed account. Four accounts are flagged is_control=true at setup: 1100 (AR), 2000 (AP), 1200 (INV), 1500 (FA); a direct manual JE that touches any of these without viaSubledger:true is rejected (CONTROL_ACCOUNT), ensuring AR/AP/INV/FA balances are exclusively maintained by their respective sub-ledger service methods.</t>
+          <t>Industry Chart-of-Accounts templates: the GL engine binds to a FIXED, global account universe (canonical codes are immutable); each tenant additionally gets a per-tenant overlay (tenant_accounts) curating which canonical accounts are active and how they are named/grouped for its industry. At company creation the customer picks an industry (restaurant/retail/distribution/services/general) and the chosen template is materialised into the overlay (provisionTenantCoA) inside the signup transaction, right after fiscal-year provisioning; adopting an industry pack later does the same. Every template code is asserted to exist in the canonical chart at boot (assertTemplatesSubsetOf in seedChartOfAccounts) so a drifted template fails fast and can never reach a tenant. Provisioning is idempotent + additive (never deletes) so re-running only adds missing accounts. The overlay NEVER gates postings — it scopes the picker / Chart-of-Accounts view only; reports surface any account that is active OR carries activity, so a curated-out account that receives a posting still appears.</t>
         </is>
       </c>
       <c r="H92" s="13" t="inlineStr">
@@ -8845,12 +8845,12 @@
       </c>
       <c r="J92" s="13" t="inlineStr">
         <is>
-          <t>Event-driven</t>
+          <t>At company creation / per pack adopt</t>
         </is>
       </c>
       <c r="K92" s="12" t="inlineStr">
         <is>
-          <t>Financial Controller</t>
+          <t>Controller</t>
         </is>
       </c>
       <c r="L92" s="13" t="inlineStr">
@@ -8860,22 +8860,22 @@
       </c>
       <c r="M92" s="12" t="inlineStr">
         <is>
-          <t>coa.service.ts (createAccount DUPLICATE_ACCOUNT, updateAccount CODE_HAS_POSTINGS, deactivateAccount ACCOUNT_HAS_BALANCE); coa.controller.ts (gl_coa permission gate); ledger.service.ts postEntry control-account guard (CONTROL_ACCOUNT, viaSubledger flag); schema/ledger.ts (account_groups table, accounts.is_control/control_subledger/is_postable/normal_balance + migration 0155); packages/shared/src/permissions.ts (gl_coa sub-permission, FinancialController default)</t>
+          <t>ledger.service.ts (provisionTenantCoA idempotent+additive, tenant-aware listAccounts, seedChartOfAccounts→assertTemplatesSubsetOf); coa-templates.ts (industry templates + subset assertion); billing.service.ts signup (industry→provisionTenantCoA in-txn); onboarding.service.ts applyPack (pack adopt provisions CoA); schema/ledger.ts tenant_accounts + tenants.industry + migration 0139; cutover/basics.ts + compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N92" s="12" t="inlineStr">
         <is>
-          <t>Inspect gl_coa permission gate + CODE_HAS_POSTINGS guard + ACCOUNT_HAS_BALANCE guard + CONTROL_ACCOUNT guard + viaSubledger bypass.</t>
+          <t>Inspect the boot subset assertion + signup provisioning + the overlay-is-presentation-only read path.</t>
         </is>
       </c>
       <c r="O92" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: create an account with gl_coa → 201; attempt to deactivate an account with balance → ACCOUNT_HAS_BALANCE; post directly to account 1100 without viaSubledger → CONTROL_ACCOUNT (re-performed by TC-GL-11-01/02/03 UAT cases).</t>
+          <t>Re-perform: a template referencing an unknown code fails the boot assertion; signup with industry=restaurant materialises a curated, industry-named chart (4000='Food &amp; Beverage Sales') that omits non-F&amp;B accounts; ?all=true still returns the full canonical universe (overlay never gates posting); signup with no industry ⇒ general = the full live chart (re-performed by the harnesses).</t>
         </is>
       </c>
       <c r="P92" s="12" t="inlineStr">
         <is>
-          <t>CoA change log (audit_log); permission test; control-account guard test</t>
+          <t>Industry templates; tenant_accounts overlay; signup provisioning log</t>
         </is>
       </c>
       <c r="Q92" s="18" t="inlineStr">
@@ -8887,7 +8887,7 @@
     <row r="93">
       <c r="A93" s="15" t="inlineStr">
         <is>
-          <t>GL-12</t>
+          <t>GL-11</t>
         </is>
       </c>
       <c r="B93" s="16" t="inlineStr">
@@ -8907,17 +8907,17 @@
       </c>
       <c r="E93" s="16" t="inlineStr">
         <is>
-          <t>Account-assignment errors introduced by scattered inline account-code literals in service code; a tenant needing a different account for a given business event has no mechanism to override without a code change.</t>
+          <t>Chart of Accounts changed without authorisation; account code changed after postings exist; account deactivated while carrying a non-zero balance; manual JE posted directly to a control account (AR/AP/INV/FA), bypassing the sub-ledger and hiding a sub-ledger discrepancy.</t>
         </is>
       </c>
       <c r="F93" s="16" t="inlineStr">
         <is>
-          <t>Authorization/Accuracy</t>
+          <t>Authorization/Completeness/Accuracy</t>
         </is>
       </c>
       <c r="G93" s="16" t="inlineStr">
         <is>
-          <t>Posting / Account-Determination Engine: two tables — posting_event_types (28 seeded event types, e.g. SALE.FOOD, GR.INVENTORY, DEPRECIATION.FA) and posting_rules (maps event × leg-order to semantic role → account_code + DR/CR side) — drive account assignment instead of hard-coded literals. PostingService.post(eventType, ctx) resolves the applicable rules (global defaults, or shadowed by tenant-specific overrides for the same leg_order), translates role-keyed amounts into DR/CR lines, and delegates to LedgerService.postEntry. If no active rules exist for an event the call fails with NO_POSTING_RULE. Tenant-specific rules require gl_posting_rules permission to create/update. PostingService.preview() provides a dry-run for audit.</t>
+          <t>CoA Change Control: account creation/update/deactivation requires the gl_coa permission (held by FinancialController, not GlAccountant — separated from gl_post per SoD). Disabling postability on an account that already has posted entries is rejected (CODE_HAS_POSTINGS). Deactivation is rejected if the account carries a non-zero net balance (ACCOUNT_HAS_BALANCE) — prevents orphaning a balance in a closed account. Four accounts are flagged is_control=true at setup: 1100 (AR), 2000 (AP), 1200 (INV), 1500 (FA); a direct manual JE that touches any of these without viaSubledger:true is rejected (CONTROL_ACCOUNT), ensuring AR/AP/INV/FA balances are exclusively maintained by their respective sub-ledger service methods.</t>
         </is>
       </c>
       <c r="H93" s="17" t="inlineStr">
@@ -8947,22 +8947,22 @@
       </c>
       <c r="M93" s="16" t="inlineStr">
         <is>
-          <t>posting.service.ts (resolveRules, post, preview, listEventTypes, listRules, upsertRule); posting-rules.controller.ts (gl_posting_rules permission gate); schema/posting-rules.ts (posting_event_types, posting_rules tables); migration 0156 (tables + 28 event types + global-default rules); ledger.module.ts (PostingService exported); packages/shared/src/permissions.ts (gl_posting_rules sub-permission); cutover/basics.ts (golden-snapshot ToE)</t>
+          <t>coa.service.ts (createAccount DUPLICATE_ACCOUNT, updateAccount CODE_HAS_POSTINGS, deactivateAccount ACCOUNT_HAS_BALANCE); coa.controller.ts (gl_coa permission gate); ledger.service.ts postEntry control-account guard (CONTROL_ACCOUNT, viaSubledger flag); schema/ledger.ts (account_groups table, accounts.is_control/control_subledger/is_postable/normal_balance + migration 0155); packages/shared/src/permissions.ts (gl_coa sub-permission, FinancialController default)</t>
         </is>
       </c>
       <c r="N93" s="16" t="inlineStr">
         <is>
-          <t>Inspect the rule-resolution logic + NO_POSTING_RULE fast-fail + tenant-shadow logic + gl_posting_rules permission gate.</t>
+          <t>Inspect gl_coa permission gate + CODE_HAS_POSTINGS guard + ACCOUNT_HAS_BALANCE guard + CONTROL_ACCOUNT guard + viaSubledger bypass.</t>
         </is>
       </c>
       <c r="O93" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: preview DEPRECIATION.FA with dep_expense:1000 → DR 5200 / CR 1590; preview GR.INVENTORY with inventory:500 → DR 1200 / CR 2000; preview UNKNOWN_EVENT → NO_POSTING_RULE (400); event-type catalogue returns ≥20 entries (re-performed by TC-GL-12-01/02/03/04 UAT cases + basics.ts harness).</t>
+          <t>Re-perform: create an account with gl_coa → 201; attempt to deactivate an account with balance → ACCOUNT_HAS_BALANCE; post directly to account 1100 without viaSubledger → CONTROL_ACCOUNT (re-performed by TC-GL-11-01/02/03 UAT cases).</t>
         </is>
       </c>
       <c r="P93" s="16" t="inlineStr">
         <is>
-          <t>Posting-rule change log; preview dry-run; harness golden snapshot</t>
+          <t>CoA change log (audit_log); permission test; control-account guard test</t>
         </is>
       </c>
       <c r="Q93" s="18" t="inlineStr">
@@ -8974,7 +8974,7 @@
     <row r="94">
       <c r="A94" s="11" t="inlineStr">
         <is>
-          <t>GL-13</t>
+          <t>GL-12</t>
         </is>
       </c>
       <c r="B94" s="12" t="inlineStr">
@@ -8994,22 +8994,22 @@
       </c>
       <c r="E94" s="12" t="inlineStr">
         <is>
-          <t>Revenue or expense mis-attributed to the wrong branch / project — per-location P&amp;L is unintelligible or misleading.</t>
+          <t>Account-assignment errors introduced by scattered inline account-code literals in service code; a tenant needing a different account for a given business event has no mechanism to override without a code change.</t>
         </is>
       </c>
       <c r="F94" s="12" t="inlineStr">
         <is>
-          <t>Accuracy/Presentation</t>
+          <t>Authorization/Accuracy</t>
         </is>
       </c>
       <c r="G94" s="12" t="inlineStr">
         <is>
-          <t>Multi-dimensional GL postings: journal_lines carries three optional dimension columns (branch_id, project_id, department_id). PostingService.post() stamps all generated lines from PostingContext (branchId/projectId/departmentId). GET /api/ledger/income-statement/by-branch provides a per-branch P&amp;L view; lines without a branch_id are grouped as 'unassigned'. The departments master table holds a tenant-scoped department registry with RLS isolation.</t>
+          <t>Posting / Account-Determination Engine: two tables — posting_event_types (28 seeded event types, e.g. SALE.FOOD, GR.INVENTORY, DEPRECIATION.FA) and posting_rules (maps event × leg-order to semantic role → account_code + DR/CR side) — drive account assignment instead of hard-coded literals. PostingService.post(eventType, ctx) resolves the applicable rules (global defaults, or shadowed by tenant-specific overrides for the same leg_order), translates role-keyed amounts into DR/CR lines, and delegates to LedgerService.postEntry. If no active rules exist for an event the call fails with NO_POSTING_RULE. Tenant-specific rules require gl_posting_rules permission to create/update. PostingService.preview() provides a dry-run for audit.</t>
         </is>
       </c>
       <c r="H94" s="13" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I94" s="13" t="inlineStr">
@@ -9019,12 +9019,12 @@
       </c>
       <c r="J94" s="13" t="inlineStr">
         <is>
-          <t>Per period</t>
+          <t>Event-driven</t>
         </is>
       </c>
       <c r="K94" s="12" t="inlineStr">
         <is>
-          <t>Controller</t>
+          <t>Financial Controller</t>
         </is>
       </c>
       <c r="L94" s="13" t="inlineStr">
@@ -9034,22 +9034,22 @@
       </c>
       <c r="M94" s="12" t="inlineStr">
         <is>
-          <t>ledger.service.ts (incomeStatementByBranch); ledger.controller.ts (GET income-statement/by-branch); posting.service.ts (branchId/projectId/departmentId from PostingContext); schema/ledger.ts (branch_id, project_id, department_id on journal_lines); schema/departments.ts (departments table); migration 0157; cutover/basics.ts (GL-13 ToE)</t>
+          <t>posting.service.ts (resolveRules, post, preview, listEventTypes, listRules, upsertRule); posting-rules.controller.ts (gl_posting_rules permission gate); schema/posting-rules.ts (posting_event_types, posting_rules tables); migration 0156 (tables + 28 event types + global-default rules); ledger.module.ts (PostingService exported); packages/shared/src/permissions.ts (gl_posting_rules sub-permission); cutover/basics.ts (golden-snapshot ToE)</t>
         </is>
       </c>
       <c r="N94" s="12" t="inlineStr">
         <is>
-          <t>Inspect by-branch query + PostingContext stamping + department RLS.</t>
+          <t>Inspect the rule-resolution logic + NO_POSTING_RULE fast-fail + tenant-shadow logic + gl_posting_rules permission gate.</t>
         </is>
       </c>
       <c r="O94" s="12" t="inlineStr">
         <is>
-          <t>TC-GL-13-01/02/03: smoke + two branches + unassigned bucket (re-performed by the basics.ts harness).</t>
+          <t>Re-perform: preview DEPRECIATION.FA with dep_expense:1000 → DR 5200 / CR 1590; preview GR.INVENTORY with inventory:500 → DR 1200 / CR 2000; preview UNKNOWN_EVENT → NO_POSTING_RULE (400); event-type catalogue returns ≥20 entries (re-performed by TC-GL-12-01/02/03/04 UAT cases + basics.ts harness).</t>
         </is>
       </c>
       <c r="P94" s="12" t="inlineStr">
         <is>
-          <t>By-branch P&amp;L report; dimension completeness</t>
+          <t>Posting-rule change log; preview dry-run; harness golden snapshot</t>
         </is>
       </c>
       <c r="Q94" s="18" t="inlineStr">
@@ -9061,7 +9061,7 @@
     <row r="95">
       <c r="A95" s="15" t="inlineStr">
         <is>
-          <t>GL-14</t>
+          <t>GL-13</t>
         </is>
       </c>
       <c r="B95" s="16" t="inlineStr">
@@ -9081,17 +9081,17 @@
       </c>
       <c r="E95" s="16" t="inlineStr">
         <is>
-          <t>GL control-account balances (AR/AP/INV/FA) drift from the underlying sub-ledger detail without detection — the control account no longer represents the sum of its sub-ledger, masking posting errors, unrecorded items, or fraud.</t>
+          <t>Revenue or expense mis-attributed to the wrong branch / project — per-location P&amp;L is unintelligible or misleading.</t>
         </is>
       </c>
       <c r="F95" s="16" t="inlineStr">
         <is>
-          <t>Completeness/Accuracy/Valuation</t>
+          <t>Accuracy/Presentation</t>
         </is>
       </c>
       <c r="G95" s="16" t="inlineStr">
         <is>
-          <t>Sub-ledger tie-out / reconciliation: POST /api/ledger/tie-out/run computes, per control account, the GL balance (Σ debit−credit of posted journal_lines on the control account up to the as-of date, tenant-scoped) and the sub-ledger detail balance (AR = Σ outstanding ar_invoices; AP = Σ outstanding ap_transactions; INV = Σ inv_balances.total_value perpetual valuation; FA = Σ acquire_cost − accumulated_depreciation of non-disposed fixed_assets), records the variance (gl − subledger) and a status (Matched if |variance|&lt;0.01 else Variance). Runs upsert per (tenant, subledger, as-of). Certification is maker-checker: POST /api/ledger/tie-out/:id/certify sets status=Certified and records certifier + timestamp, and REJECTS a certifier equal to the runner (SELF_CERTIFY) — the gl_close certifier must differ from the gl_post/gl_close runner (SoD).</t>
+          <t>Multi-dimensional GL postings: journal_lines carries three optional dimension columns (branch_id, project_id, department_id). PostingService.post() stamps all generated lines from PostingContext (branchId/projectId/departmentId). GET /api/ledger/income-statement/by-branch provides a per-branch P&amp;L view; lines without a branch_id are grouped as 'unassigned'. The departments master table holds a tenant-scoped department registry with RLS isolation.</t>
         </is>
       </c>
       <c r="H95" s="17" t="inlineStr">
@@ -9106,12 +9106,12 @@
       </c>
       <c r="J95" s="17" t="inlineStr">
         <is>
-          <t>Monthly</t>
+          <t>Per period</t>
         </is>
       </c>
       <c r="K95" s="16" t="inlineStr">
         <is>
-          <t>Financial Controller</t>
+          <t>Controller</t>
         </is>
       </c>
       <c r="L95" s="17" t="inlineStr">
@@ -9121,22 +9121,22 @@
       </c>
       <c r="M95" s="16" t="inlineStr">
         <is>
-          <t>subledger-tieout.service.ts (runTieOut GL/sub-ledger balance computation + variance/status, certify SELF_CERTIFY maker-checker, list/get); subledger-tieout.controller.ts (gl_close/gl_post run, gl_close certify, gl_close/gl_post/exec/creditors/ar read); schema/subledger-tieout.ts (subledger_tieout_runs table, uq on tenant/subledger/as-of); migration 0160 (table + RLS); ledger.module.ts (service+controller wired); cutover/basics.ts (GL-14 ToE)</t>
+          <t>ledger.service.ts (incomeStatementByBranch); ledger.controller.ts (GET income-statement/by-branch); posting.service.ts (branchId/projectId/departmentId from PostingContext); schema/ledger.ts (branch_id, project_id, department_id on journal_lines); schema/departments.ts (departments table); migration 0157; cutover/basics.ts (GL-13 ToE)</t>
         </is>
       </c>
       <c r="N95" s="16" t="inlineStr">
         <is>
-          <t>Inspect the GL-vs-sub-ledger balance computation + variance/status + SELF_CERTIFY maker-checker gate + gl_close certify permission.</t>
+          <t>Inspect by-branch query + PostingContext stamping + department RLS.</t>
         </is>
       </c>
       <c r="O95" s="16" t="inlineStr">
         <is>
-          <t>TC-GL-14-01: run AR tie-out → balances + Matched/Variance; TC-GL-14-02: self-certify by the runner → SELF_CERTIFY (400); TC-GL-14-03: certify by a different gl_close user → Certified (re-performed by the basics.ts harness).</t>
+          <t>TC-GL-13-01/02/03: smoke + two branches + unassigned bucket (re-performed by the basics.ts harness).</t>
         </is>
       </c>
       <c r="P95" s="16" t="inlineStr">
         <is>
-          <t>Tie-out run log (subledger_tieout_runs) with variance + certification trail; monthly reconciliation sign-off</t>
+          <t>By-branch P&amp;L report; dimension completeness</t>
         </is>
       </c>
       <c r="Q95" s="18" t="inlineStr">
@@ -9148,12 +9148,12 @@
     <row r="96">
       <c r="A96" s="11" t="inlineStr">
         <is>
-          <t>EXP-07</t>
+          <t>GL-14</t>
         </is>
       </c>
       <c r="B96" s="12" t="inlineStr">
         <is>
-          <t>Expenditure</t>
+          <t>General Ledger</t>
         </is>
       </c>
       <c r="C96" s="13" t="inlineStr">
@@ -9163,22 +9163,22 @@
       </c>
       <c r="D96" s="12" t="inlineStr">
         <is>
-          <t>Cash; Operating expense</t>
+          <t>All</t>
         </is>
       </c>
       <c r="E96" s="12" t="inlineStr">
         <is>
-          <t>Petty-cash / employee advance issued but never accounted for — cash leakage, expense unrecorded.</t>
+          <t>GL control-account balances (AR/AP/INV/FA) drift from the underlying sub-ledger detail without detection — the control account no longer represents the sum of its sub-ledger, masking posting errors, unrecorded items, or fraud.</t>
         </is>
       </c>
       <c r="F96" s="12" t="inlineStr">
         <is>
-          <t>Existence/Completeness</t>
+          <t>Completeness/Accuracy/Valuation</t>
         </is>
       </c>
       <c r="G96" s="12" t="inlineStr">
         <is>
-          <t>Employee cash advances: issuing an advance debits the 1180 Employee Advances control (Dr 1180 / Cr 1000); settlement clears it against actual spend + returned cash (Dr expense + Dr 1000 / Cr 1180), enforced to reconcile (settled_expense + returned_cash must equal the advance → SETTLE_MISMATCH). The 1180 balance is the outstanding float subject to review.</t>
+          <t>Sub-ledger tie-out / reconciliation: POST /api/ledger/tie-out/run computes, per control account, the GL balance (Σ debit−credit of posted journal_lines on the control account up to the as-of date, tenant-scoped) and the sub-ledger detail balance (AR = Σ outstanding ar_invoices; AP = Σ outstanding ap_transactions; INV = Σ inv_balances.total_value perpetual valuation; FA = Σ acquire_cost − accumulated_depreciation of non-disposed fixed_assets), records the variance (gl − subledger) and a status (Matched if |variance|&lt;0.01 else Variance). Runs upsert per (tenant, subledger, as-of). Certification is maker-checker: POST /api/ledger/tie-out/:id/certify sets status=Certified and records certifier + timestamp, and REJECTS a certifier equal to the runner (SELF_CERTIFY) — the gl_close certifier must differ from the gl_post/gl_close runner (SoD).</t>
         </is>
       </c>
       <c r="H96" s="13" t="inlineStr">
@@ -9193,12 +9193,12 @@
       </c>
       <c r="J96" s="13" t="inlineStr">
         <is>
-          <t>Per advance</t>
+          <t>Monthly</t>
         </is>
       </c>
       <c r="K96" s="12" t="inlineStr">
         <is>
-          <t>AP / Controller</t>
+          <t>Financial Controller</t>
         </is>
       </c>
       <c r="L96" s="13" t="inlineStr">
@@ -9208,22 +9208,22 @@
       </c>
       <c r="M96" s="12" t="inlineStr">
         <is>
-          <t>finance.service.ts (issueAdvance, settleAdvance reconcile-or-reject, listAdvances outstanding); finance.controller.ts (creditors/exec); schema/finance.ts (employee_advances) + migration 0120; cutover/basics.ts (ToE)</t>
+          <t>subledger-tieout.service.ts (runTieOut GL/sub-ledger balance computation + variance/status, certify SELF_CERTIFY maker-checker, list/get); subledger-tieout.controller.ts (gl_close/gl_post run, gl_close certify, gl_close/gl_post/exec/creditors/ar read); schema/subledger-tieout.ts (subledger_tieout_runs table, uq on tenant/subledger/as-of); migration 0160 (table + RLS); ledger.module.ts (service+controller wired); cutover/basics.ts (GL-14 ToE)</t>
         </is>
       </c>
       <c r="N96" s="12" t="inlineStr">
         <is>
-          <t>Inspect issue/settle GL + settlement reconciliation guard.</t>
+          <t>Inspect the GL-vs-sub-ledger balance computation + variance/status + SELF_CERTIFY maker-checker gate + gl_close certify permission.</t>
         </is>
       </c>
       <c r="O96" s="12" t="inlineStr">
         <is>
-          <t>Issue an advance (1180 up); settle 700+300 clears 1180; mismatched settle → SETTLE_MISMATCH (re-performed by the harness).</t>
+          <t>TC-GL-14-01: run AR tie-out → balances + Matched/Variance; TC-GL-14-02: self-certify by the runner → SELF_CERTIFY (400); TC-GL-14-03: certify by a different gl_close user → Certified (re-performed by the basics.ts harness).</t>
         </is>
       </c>
       <c r="P96" s="12" t="inlineStr">
         <is>
-          <t>Advance register; outstanding float</t>
+          <t>Tie-out run log (subledger_tieout_runs) with variance + certification trail; monthly reconciliation sign-off</t>
         </is>
       </c>
       <c r="Q96" s="18" t="inlineStr">
@@ -9235,7 +9235,7 @@
     <row r="97">
       <c r="A97" s="15" t="inlineStr">
         <is>
-          <t>EXP-08</t>
+          <t>EXP-07</t>
         </is>
       </c>
       <c r="B97" s="16" t="inlineStr">
@@ -9255,22 +9255,22 @@
       </c>
       <c r="E97" s="16" t="inlineStr">
         <is>
-          <t>Petty-cash disbursed beyond authority / without independent review, or drawn past the fund's limit — cash leakage, unauthorised or unrecorded expense, over-extended float.</t>
+          <t>Petty-cash / employee advance issued but never accounted for — cash leakage, expense unrecorded.</t>
         </is>
       </c>
       <c r="F97" s="16" t="inlineStr">
         <is>
-          <t>Authorization; Completeness</t>
+          <t>Existence/Completeness</t>
         </is>
       </c>
       <c r="G97" s="16" t="inlineStr">
         <is>
-          <t>Petty-cash imprest float + maker-checker on disbursement (SoD): a fund holds cash capped at a credit limit/วงเงิน (1015 Petty Cash, a cash account); each direct EXPENSE or ADVANCE is a REQUEST that posts NOTHING and a DIFFERENT user must approve before the GL posts (expense Dr &lt;expense&gt; / Cr 1015; advance Dr 1180 / Cr 1015) and the fund balance is decremented. Self-approval → SOD_VIOLATION (binds even Admin). A draw beyond the fund balance → INSUFFICIENT_FLOAT; establishing/replenishing above the float limit → OVER_FLOAT. Advances settle (Dr expense + Dr 1015 returned / Cr 1180), returning unused cash to the fund. Every request carries a document reference + receipt key + a status trail (StatusLog) and surfaces in the GOV-01 pending-approvals monitor.</t>
+          <t>Employee cash advances: issuing an advance debits the 1180 Employee Advances control (Dr 1180 / Cr 1000); settlement clears it against actual spend + returned cash (Dr expense + Dr 1000 / Cr 1180), enforced to reconcile (settled_expense + returned_cash must equal the advance → SETTLE_MISMATCH). The 1180 balance is the outstanding float subject to review.</t>
         </is>
       </c>
       <c r="H97" s="17" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I97" s="17" t="inlineStr">
@@ -9280,7 +9280,7 @@
       </c>
       <c r="J97" s="17" t="inlineStr">
         <is>
-          <t>Per disbursement</t>
+          <t>Per advance</t>
         </is>
       </c>
       <c r="K97" s="16" t="inlineStr">
@@ -9295,22 +9295,22 @@
       </c>
       <c r="M97" s="16" t="inlineStr">
         <is>
-          <t>petty-cash.service.ts (establishFund/replenishFund float guards, createRequest INSUFFICIENT_FLOAT, approveRequest SoD+GL, rejectRequest, settleRequest); petty-cash.controller.ts (creditors/exec); schema/petty-cash.ts (petty_cash_funds, expense_requests) + migration 0139; finance.service.ts pendingApprovals (GOV-01 source 7); cutover/basics.ts + compliance.ts (ToE)</t>
+          <t>finance.service.ts (issueAdvance, settleAdvance reconcile-or-reject, listAdvances outstanding); finance.controller.ts (creditors/exec); schema/finance.ts (employee_advances) + migration 0120; cutover/basics.ts (ToE)</t>
         </is>
       </c>
       <c r="N97" s="16" t="inlineStr">
         <is>
-          <t>Inspect the float ceiling + the request→approve flow + the approver≠requester check + that the request posts nothing until approval.</t>
+          <t>Inspect issue/settle GL + settlement reconciliation guard.</t>
         </is>
       </c>
       <c r="O97" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: establish a fund (Dr 1015), request an expense (no GL), self-approve → SOD_VIOLATION, approve as a different user → Dr expense/Cr 1015 + fund down; over-balance draw → INSUFFICIENT_FLOAT; advance approve→settle clears 1180; replenish past float → OVER_FLOAT (re-performed by the harnesses).</t>
+          <t>Issue an advance (1180 up); settle 700+300 clears 1180; mismatched settle → SETTLE_MISMATCH (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P97" s="16" t="inlineStr">
         <is>
-          <t>Fund register + disbursement approval log + SoD test</t>
+          <t>Advance register; outstanding float</t>
         </is>
       </c>
       <c r="Q97" s="18" t="inlineStr">
@@ -9322,12 +9322,12 @@
     <row r="98">
       <c r="A98" s="11" t="inlineStr">
         <is>
-          <t>FA-07</t>
+          <t>EXP-08</t>
         </is>
       </c>
       <c r="B98" s="12" t="inlineStr">
         <is>
-          <t>Fixed Assets</t>
+          <t>Expenditure</t>
         </is>
       </c>
       <c r="C98" s="13" t="inlineStr">
@@ -9337,27 +9337,27 @@
       </c>
       <c r="D98" s="12" t="inlineStr">
         <is>
-          <t>Property, Plant &amp; Equipment; Equity</t>
+          <t>Cash; Operating expense</t>
         </is>
       </c>
       <c r="E98" s="12" t="inlineStr">
         <is>
-          <t>Carrying amount not adjusted for revaluation/impairment — asset over/understated.</t>
+          <t>Petty-cash disbursed beyond authority / without independent review, or drawn past the fund's limit — cash leakage, unauthorised or unrecorded expense, over-extended float.</t>
         </is>
       </c>
       <c r="F98" s="12" t="inlineStr">
         <is>
-          <t>Valuation</t>
+          <t>Authorization; Completeness</t>
         </is>
       </c>
       <c r="G98" s="12" t="inlineStr">
         <is>
-          <t>Asset revaluation / impairment: an upward revaluation credits the revaluation surplus in equity (Dr 1500 / Cr 3200); a downward revaluation (impairment) debits impairment loss (Dr 5820 / Cr 1500). The gross 1500 moves by the delta so the register stays tied to the GL; a no-op revaluation is rejected (NO_CHANGE). Every event is logged for the audit trail.</t>
+          <t>Petty-cash imprest float + maker-checker on disbursement (SoD): a fund holds cash capped at a credit limit/วงเงิน (1015 Petty Cash, a cash account); each direct EXPENSE or ADVANCE is a REQUEST that posts NOTHING and a DIFFERENT user must approve before the GL posts (expense Dr &lt;expense&gt; / Cr 1015; advance Dr 1180 / Cr 1015) and the fund balance is decremented. Self-approval → SOD_VIOLATION (binds even Admin). A draw beyond the fund balance → INSUFFICIENT_FLOAT; establishing/replenishing above the float limit → OVER_FLOAT. Advances settle (Dr expense + Dr 1015 returned / Cr 1180), returning unused cash to the fund. Every request carries a document reference + receipt key + a status trail (StatusLog) and surfaces in the GOV-01 pending-approvals monitor.</t>
         </is>
       </c>
       <c r="H98" s="13" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I98" s="13" t="inlineStr">
@@ -9367,12 +9367,12 @@
       </c>
       <c r="J98" s="13" t="inlineStr">
         <is>
-          <t>Per event</t>
+          <t>Per disbursement</t>
         </is>
       </c>
       <c r="K98" s="12" t="inlineStr">
         <is>
-          <t>FaAccountant / Controller</t>
+          <t>AP / Controller</t>
         </is>
       </c>
       <c r="L98" s="13" t="inlineStr">
@@ -9382,22 +9382,22 @@
       </c>
       <c r="M98" s="12" t="inlineStr">
         <is>
-          <t>assets.service.ts (revalue up→3200 / down→5820, listRevaluations; dispose recycles surplus 3200→3100); assets.controller.ts (exec/creditors); schema/assets.ts (asset_revaluations) + migration 0120; cutover/basics.ts (ToE)</t>
+          <t>petty-cash.service.ts (establishFund/replenishFund float guards, createRequest INSUFFICIENT_FLOAT, approveRequest SoD+GL, rejectRequest, settleRequest); petty-cash.controller.ts (creditors/exec); schema/petty-cash.ts (petty_cash_funds, expense_requests) + migration 0139; finance.service.ts pendingApprovals (GOV-01 source 7); cutover/basics.ts + compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N98" s="12" t="inlineStr">
         <is>
-          <t>Inspect revaluation/impairment routing + audit log + disposal recycling.</t>
+          <t>Inspect the float ceiling + the request→approve flow + the approver≠requester check + that the request posts nothing until approval.</t>
         </is>
       </c>
       <c r="O98" s="12" t="inlineStr">
         <is>
-          <t>Upward revaluation credits 3200; impairment debits 5820; no-change → NO_CHANGE; both events logged; on disposal the revaluation surplus is recycled to retained earnings (Dr 3200 / Cr 3100), not through P&amp;L (re-performed by the harness).</t>
+          <t>Re-perform: establish a fund (Dr 1015), request an expense (no GL), self-approve → SOD_VIOLATION, approve as a different user → Dr expense/Cr 1015 + fund down; over-balance draw → INSUFFICIENT_FLOAT; advance approve→settle clears 1180; replenish past float → OVER_FLOAT (re-performed by the harnesses).</t>
         </is>
       </c>
       <c r="P98" s="12" t="inlineStr">
         <is>
-          <t>Revaluation log; disposal recycling JE</t>
+          <t>Fund register + disbursement approval log + SoD test</t>
         </is>
       </c>
       <c r="Q98" s="18" t="inlineStr">
@@ -9409,7 +9409,7 @@
     <row r="99">
       <c r="A99" s="15" t="inlineStr">
         <is>
-          <t>FA-08</t>
+          <t>FA-07</t>
         </is>
       </c>
       <c r="B99" s="16" t="inlineStr">
@@ -9429,22 +9429,22 @@
       </c>
       <c r="E99" s="16" t="inlineStr">
         <is>
-          <t>Carrying amount changed by fair-value revaluation/impairment without independent review — the preparer revalues the asset and posts to equity/P&amp;L on their own (earnings/equity management).</t>
+          <t>Carrying amount not adjusted for revaluation/impairment — asset over/understated.</t>
         </is>
       </c>
       <c r="F99" s="16" t="inlineStr">
         <is>
-          <t>Authorization</t>
+          <t>Valuation</t>
         </is>
       </c>
       <c r="G99" s="16" t="inlineStr">
         <is>
-          <t>Asset-revaluation maker-checker (SoD): a revalue/impairment request posts its GL entry as a DRAFT (excluded from balances) and records status 'PendingApproval' WITHOUT moving the carrying value; a DIFFERENT user must approve before the JE is effective and the register is re-valued (approver ≠ preparer enforced regardless of permissions, reusing the GL-05 ledger approval). Reject voids the draft; only one revaluation may be pending per asset; the disposal surplus recycle counts only approved revaluations.</t>
+          <t>Asset revaluation / impairment: an upward revaluation credits the revaluation surplus in equity (Dr 1500 / Cr 3200); a downward revaluation (impairment) debits impairment loss (Dr 5820 / Cr 1500). The gross 1500 moves by the delta so the register stays tied to the GL; a no-op revaluation is rejected (NO_CHANGE). Every event is logged for the audit trail.</t>
         </is>
       </c>
       <c r="H99" s="17" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I99" s="17" t="inlineStr">
@@ -9469,22 +9469,22 @@
       </c>
       <c r="M99" s="16" t="inlineStr">
         <is>
-          <t>assets.service.ts revalue(pendingApproval Draft)/approveRevaluation/rejectRevaluation; assets.controller.ts (:assetNo/revalue/approve|reject); schema/assets.ts asset_revaluations.status + migration 0134; cutover/basics.ts + compliance.ts (ToE)</t>
+          <t>assets.service.ts (revalue up→3200 / down→5820, listRevaluations; dispose recycles surplus 3200→3100); assets.controller.ts (exec/creditors); schema/assets.ts (asset_revaluations) + migration 0120; cutover/basics.ts (ToE)</t>
         </is>
       </c>
       <c r="N99" s="16" t="inlineStr">
         <is>
-          <t>Inspect Draft→approve flow + the approver≠preparer check + deferred carrying-value update.</t>
+          <t>Inspect revaluation/impairment routing + audit log + disposal recycling.</t>
         </is>
       </c>
       <c r="O99" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: request a revaluation (Draft JE excluded from 3200), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm the surplus/impairment + carrying value move only after approval (re-performed by the harnesses).</t>
+          <t>Upward revaluation credits 3200; impairment debits 5820; no-change → NO_CHANGE; both events logged; on disposal the revaluation surplus is recycled to retained earnings (Dr 3200 / Cr 3100), not through P&amp;L (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P99" s="16" t="inlineStr">
         <is>
-          <t>Revaluation approval log + SoD test</t>
+          <t>Revaluation log; disposal recycling JE</t>
         </is>
       </c>
       <c r="Q99" s="18" t="inlineStr">
@@ -9496,12 +9496,12 @@
     <row r="100">
       <c r="A100" s="11" t="inlineStr">
         <is>
-          <t>LSE-01</t>
+          <t>FA-08</t>
         </is>
       </c>
       <c r="B100" s="12" t="inlineStr">
         <is>
-          <t>Leases</t>
+          <t>Fixed Assets</t>
         </is>
       </c>
       <c r="C100" s="13" t="inlineStr">
@@ -9511,27 +9511,27 @@
       </c>
       <c r="D100" s="12" t="inlineStr">
         <is>
-          <t>Right-of-use assets; Lease liabilities</t>
+          <t>Property, Plant &amp; Equipment; Equity</t>
         </is>
       </c>
       <c r="E100" s="12" t="inlineStr">
         <is>
-          <t>Lease not capitalised (IFRS 16 / TFRS 16) — ROU asset + lease liability omitted; interest/depreciation mis-stated.</t>
+          <t>Carrying amount changed by fair-value revaluation/impairment without independent review — the preparer revalues the asset and posts to equity/P&amp;L on their own (earnings/equity management).</t>
         </is>
       </c>
       <c r="F100" s="12" t="inlineStr">
         <is>
-          <t>Completeness/Accuracy/Valuation</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="G100" s="12" t="inlineStr">
         <is>
-          <t>Lease accounting: at commencement a right-of-use asset and lease liability are recognised at the present value of the lease payments (Dr 1600 / Cr 2600). The scheduled job lease_periodic_run posts each period — interest unwinding on the liability (Dr 5900), the cash payment reducing the liability (Dr 2600 / Cr 1000), and straight-line ROU depreciation (Dr 5210 / Cr 1690) — the last period clearing the liability + ROU exactly. Idempotent per (lease, period).</t>
+          <t>Asset-revaluation maker-checker (SoD): a revalue/impairment request posts its GL entry as a DRAFT (excluded from balances) and records status 'PendingApproval' WITHOUT moving the carrying value; a DIFFERENT user must approve before the JE is effective and the register is re-valued (approver ≠ preparer enforced regardless of permissions, reusing the GL-05 ledger approval). Reject voids the draft; only one revaluation may be pending per asset; the disposal surplus recycle counts only approved revaluations.</t>
         </is>
       </c>
       <c r="H100" s="13" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I100" s="13" t="inlineStr">
@@ -9541,12 +9541,12 @@
       </c>
       <c r="J100" s="13" t="inlineStr">
         <is>
-          <t>Per period / per lease</t>
+          <t>Per event</t>
         </is>
       </c>
       <c r="K100" s="12" t="inlineStr">
         <is>
-          <t>Controller</t>
+          <t>FaAccountant / Controller</t>
         </is>
       </c>
       <c r="L100" s="13" t="inlineStr">
@@ -9556,22 +9556,22 @@
       </c>
       <c r="M100" s="12" t="inlineStr">
         <is>
-          <t>leases.service.ts (createLease PV recognition, runDueLeases interest+payment+depreciation, modifyLease remeasurement); leases.controller.ts (gl_post); bi.service.ts (lease_periodic_run); schema/leases.ts (leases, rou_nbv) + migration 0120/0121; cutover/basics.ts (ToE)</t>
+          <t>assets.service.ts revalue(pendingApproval Draft)/approveRevaluation/rejectRevaluation; assets.controller.ts (:assetNo/revalue/approve|reject); schema/assets.ts asset_revaluations.status + migration 0134; cutover/basics.ts + compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N100" s="12" t="inlineStr">
         <is>
-          <t>Inspect PV recognition + periodic interest/payment/depreciation + final-period clearing + modification remeasurement.</t>
+          <t>Inspect Draft→approve flow + the approver≠preparer check + deferred carrying-value update.</t>
         </is>
       </c>
       <c r="O100" s="12" t="inlineStr">
         <is>
-          <t>Commencement recognises ROU=liability=PV; periodic run posts interest+principal(=payment)+ROU depreciation; liability + ROU reduce; a modification remeasures the liability at the revised PV and adjusts the ROU by the same delta (Dr/Cr 1600↔2600), then depreciates over the remaining term (re-performed by the harness).</t>
+          <t>Re-perform: request a revaluation (Draft JE excluded from 3200), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm the surplus/impairment + carrying value move only after approval (re-performed by the harnesses).</t>
         </is>
       </c>
       <c r="P100" s="12" t="inlineStr">
         <is>
-          <t>Lease register; periodic run log; modification remeasurement</t>
+          <t>Revaluation approval log + SoD test</t>
         </is>
       </c>
       <c r="Q100" s="18" t="inlineStr">
@@ -9583,12 +9583,12 @@
     <row r="101">
       <c r="A101" s="15" t="inlineStr">
         <is>
-          <t>REC-01</t>
+          <t>LSE-01</t>
         </is>
       </c>
       <c r="B101" s="16" t="inlineStr">
         <is>
-          <t>Reconciliation</t>
+          <t>Leases</t>
         </is>
       </c>
       <c r="C101" s="17" t="inlineStr">
@@ -9598,22 +9598,22 @@
       </c>
       <c r="D101" s="16" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Right-of-use assets; Lease liabilities</t>
         </is>
       </c>
       <c r="E101" s="16" t="inlineStr">
         <is>
-          <t>Subledgers diverge from GL undetected.</t>
+          <t>Lease not capitalised (IFRS 16 / TFRS 16) — ROU asset + lease liability omitted; interest/depreciation mis-stated.</t>
         </is>
       </c>
       <c r="F101" s="16" t="inlineStr">
         <is>
-          <t>Completeness/Accuracy</t>
+          <t>Completeness/Accuracy/Valuation</t>
         </is>
       </c>
       <c r="G101" s="16" t="inlineStr">
         <is>
-          <t>Subledger-to-GL reconciliation per period: import GL, auto-match, certify (sign-off via 'approvals').</t>
+          <t>Lease accounting: at commencement a right-of-use asset and lease liability are recognised at the present value of the lease payments (Dr 1600 / Cr 2600). The scheduled job lease_periodic_run posts each period — interest unwinding on the liability (Dr 5900), the cash payment reducing the liability (Dr 2600 / Cr 1000), and straight-line ROU depreciation (Dr 5210 / Cr 1690) — the last period clearing the liability + ROU exactly. Idempotent per (lease, period).</t>
         </is>
       </c>
       <c r="H101" s="17" t="inlineStr">
@@ -9623,12 +9623,12 @@
       </c>
       <c r="I101" s="17" t="inlineStr">
         <is>
-          <t>Auto+Manual</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J101" s="17" t="inlineStr">
         <is>
-          <t>Monthly</t>
+          <t>Per period / per lease</t>
         </is>
       </c>
       <c r="K101" s="16" t="inlineStr">
@@ -9638,27 +9638,27 @@
       </c>
       <c r="L101" s="17" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="M101" s="16" t="inlineStr">
         <is>
-          <t>reconciliation.service.ts (importGlItems/autoMatch/certify)</t>
+          <t>leases.service.ts (createLease PV recognition, runDueLeases interest+payment+depreciation, modifyLease remeasurement); leases.controller.ts (gl_post); bi.service.ts (lease_periodic_run); schema/leases.ts (leases, rou_nbv) + migration 0120/0121; cutover/basics.ts (ToE)</t>
         </is>
       </c>
       <c r="N101" s="16" t="inlineStr">
         <is>
-          <t>Inspect recon + certify gate.</t>
+          <t>Inspect PV recognition + periodic interest/payment/depreciation + final-period clearing + modification remeasurement.</t>
         </is>
       </c>
       <c r="O101" s="16" t="inlineStr">
         <is>
-          <t>Sample periods: reconciled, unmatched cleared, certified.</t>
+          <t>Commencement recognises ROU=liability=PV; periodic run posts interest+principal(=payment)+ROU depreciation; liability + ROU reduce; a modification remeasures the liability at the revised PV and adjusts the ROU by the same delta (Dr/Cr 1600↔2600), then depreciates over the remaining term (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P101" s="16" t="inlineStr">
         <is>
-          <t>Certified recon</t>
+          <t>Lease register; periodic run log; modification remeasurement</t>
         </is>
       </c>
       <c r="Q101" s="18" t="inlineStr">
@@ -9670,7 +9670,7 @@
     <row r="102">
       <c r="A102" s="11" t="inlineStr">
         <is>
-          <t>REC-02</t>
+          <t>REC-01</t>
         </is>
       </c>
       <c r="B102" s="12" t="inlineStr">
@@ -9685,22 +9685,22 @@
       </c>
       <c r="D102" s="12" t="inlineStr">
         <is>
-          <t>Cash</t>
+          <t>All</t>
         </is>
       </c>
       <c r="E102" s="12" t="inlineStr">
         <is>
-          <t>Bank balance not reconciled to GL.</t>
+          <t>Subledgers diverge from GL undetected.</t>
         </is>
       </c>
       <c r="F102" s="12" t="inlineStr">
         <is>
-          <t>Existence/Completeness</t>
+          <t>Completeness/Accuracy</t>
         </is>
       </c>
       <c r="G102" s="12" t="inlineStr">
         <is>
-          <t>Bank reconciliation against statements.</t>
+          <t>Subledger-to-GL reconciliation per period: import GL, auto-match, certify (sign-off via 'approvals').</t>
         </is>
       </c>
       <c r="H102" s="13" t="inlineStr">
@@ -9730,22 +9730,22 @@
       </c>
       <c r="M102" s="12" t="inlineStr">
         <is>
-          <t>bank module; drizzle/0015_bank_reconciliation</t>
+          <t>reconciliation.service.ts (importGlItems/autoMatch/certify)</t>
         </is>
       </c>
       <c r="N102" s="12" t="inlineStr">
         <is>
-          <t>Inspect bank-rec process.</t>
+          <t>Inspect recon + certify gate.</t>
         </is>
       </c>
       <c r="O102" s="12" t="inlineStr">
         <is>
-          <t>Sample months reconciled &amp; reviewed.</t>
+          <t>Sample periods: reconciled, unmatched cleared, certified.</t>
         </is>
       </c>
       <c r="P102" s="12" t="inlineStr">
         <is>
-          <t>Bank rec</t>
+          <t>Certified recon</t>
         </is>
       </c>
       <c r="Q102" s="18" t="inlineStr">
@@ -9757,12 +9757,12 @@
     <row r="103">
       <c r="A103" s="15" t="inlineStr">
         <is>
-          <t>BANK-02</t>
+          <t>REC-02</t>
         </is>
       </c>
       <c r="B103" s="16" t="inlineStr">
         <is>
-          <t>Cash &amp; Treasury</t>
+          <t>Reconciliation</t>
         </is>
       </c>
       <c r="C103" s="17" t="inlineStr">
@@ -9772,37 +9772,37 @@
       </c>
       <c r="D103" s="16" t="inlineStr">
         <is>
-          <t>Cash; Operating expense; Interest income</t>
+          <t>Cash</t>
         </is>
       </c>
       <c r="E103" s="16" t="inlineStr">
         <is>
-          <t>A bank fee/interest adjustment is posted straight to the GL by one person during reconciliation — a cash outflow mis-booked as interest income, or a fictitious fee posted, with no independent review (single-person posting to the cash account).</t>
+          <t>Bank balance not reconciled to GL.</t>
         </is>
       </c>
       <c r="F103" s="16" t="inlineStr">
         <is>
-          <t>Authorization/Accuracy</t>
+          <t>Existence/Completeness</t>
         </is>
       </c>
       <c r="G103" s="16" t="inlineStr">
         <is>
-          <t>Bank adjustment maker-checker (SoD): a fee/interest adjustment on a statement line is a REQUEST that posts a DRAFT JE (no balance/GL effect; the line stays unreconciled) until a DIFFERENT user with approval authority approves (POST /api/bank/lines/:id/adjustment/approve). Self-approval → SOD_VIOLATION (binds even Admin); approval flips the line to reconciled and the JE to Posted; reject voids the Draft and frees the line. The Draft JE (source BANKADJ) is also surfaced, aged, by the pending-approvals monitor (GOV-01).</t>
+          <t>Bank reconciliation against statements.</t>
         </is>
       </c>
       <c r="H103" s="17" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I103" s="17" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="J103" s="17" t="inlineStr">
         <is>
-          <t>Per adjustment</t>
+          <t>Monthly</t>
         </is>
       </c>
       <c r="K103" s="16" t="inlineStr">
@@ -9812,27 +9812,27 @@
       </c>
       <c r="L103" s="17" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="M103" s="16" t="inlineStr">
         <is>
-          <t>bank.service.ts requestAdjustment/approveAdjustment/rejectAdjustment/listPendingAdjustments (reuses ledger.approveEntry SoD); bank.controller.ts (lines/:id/adjustment requests; adjustment/approve|reject gated approvals/gl_close); cutover/bankrec.ts (ToE)</t>
+          <t>bank module; drizzle/0015_bank_reconciliation</t>
         </is>
       </c>
       <c r="N103" s="16" t="inlineStr">
         <is>
-          <t>Inspect the request→approve flow + the approver≠requester check + that the Draft posts nothing until approval.</t>
+          <t>Inspect bank-rec process.</t>
         </is>
       </c>
       <c r="O103" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: request a fee adjustment (line unreconciled, GL difference unchanged), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm the difference closes to 0 only after approval (re-performed by the bankrec harness).</t>
+          <t>Sample months reconciled &amp; reviewed.</t>
         </is>
       </c>
       <c r="P103" s="16" t="inlineStr">
         <is>
-          <t>Bank adjustment queue + SoD test</t>
+          <t>Bank rec</t>
         </is>
       </c>
       <c r="Q103" s="18" t="inlineStr">
@@ -9844,12 +9844,12 @@
     <row r="104">
       <c r="A104" s="11" t="inlineStr">
         <is>
-          <t>REC-03</t>
+          <t>BANK-02</t>
         </is>
       </c>
       <c r="B104" s="12" t="inlineStr">
         <is>
-          <t>Reconciliation</t>
+          <t>Cash &amp; Treasury</t>
         </is>
       </c>
       <c r="C104" s="13" t="inlineStr">
@@ -9859,79 +9859,79 @@
       </c>
       <c r="D104" s="12" t="inlineStr">
         <is>
-          <t>Consolidation</t>
+          <t>Cash; Operating expense; Interest income</t>
         </is>
       </c>
       <c r="E104" s="12" t="inlineStr">
         <is>
-          <t>Intercompany balances not eliminated/agreed.</t>
+          <t>A bank fee/interest adjustment is posted straight to the GL by one person during reconciliation — a cash outflow mis-booked as interest income, or a fictitious fee posted, with no independent review (single-person posting to the cash account).</t>
         </is>
       </c>
       <c r="F104" s="12" t="inlineStr">
         <is>
-          <t>Accuracy</t>
+          <t>Authorization/Accuracy</t>
         </is>
       </c>
       <c r="G104" s="12" t="inlineStr">
         <is>
-          <t>Intercompany reconciliation &amp; elimination on consolidation.</t>
+          <t>Bank adjustment maker-checker (SoD): a fee/interest adjustment on a statement line is a REQUEST that posts a DRAFT JE (no balance/GL effect; the line stays unreconciled) until a DIFFERENT user with approval authority approves (POST /api/bank/lines/:id/adjustment/approve). Self-approval → SOD_VIOLATION (binds even Admin); approval flips the line to reconciled and the JE to Posted; reject voids the Draft and frees the line. The Draft JE (source BANKADJ) is also surfaced, aged, by the pending-approvals monitor (GOV-01).</t>
         </is>
       </c>
       <c r="H104" s="13" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I104" s="13" t="inlineStr">
         <is>
-          <t>Auto+Manual</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J104" s="13" t="inlineStr">
         <is>
-          <t>Period</t>
+          <t>Per adjustment</t>
         </is>
       </c>
       <c r="K104" s="12" t="inlineStr">
         <is>
-          <t>Group Controller</t>
+          <t>Controller</t>
         </is>
       </c>
       <c r="L104" s="13" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="M104" s="12" t="inlineStr">
         <is>
-          <t>intercompany; consolidation</t>
+          <t>bank.service.ts requestAdjustment/approveAdjustment/rejectAdjustment/listPendingAdjustments (reuses ledger.approveEntry SoD); bank.controller.ts (lines/:id/adjustment requests; adjustment/approve|reject gated approvals/gl_close); cutover/bankrec.ts (ToE)</t>
         </is>
       </c>
       <c r="N104" s="12" t="inlineStr">
         <is>
-          <t>Inspect IC matching + elimination.</t>
+          <t>Inspect the request→approve flow + the approver≠requester check + that the Draft posts nothing until approval.</t>
         </is>
       </c>
       <c r="O104" s="12" t="inlineStr">
         <is>
-          <t>Sample IC pairs agree &amp; eliminate.</t>
+          <t>Re-perform: request a fee adjustment (line unreconciled, GL difference unchanged), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm the difference closes to 0 only after approval (re-performed by the bankrec harness).</t>
         </is>
       </c>
       <c r="P104" s="12" t="inlineStr">
         <is>
-          <t>IC recon</t>
-        </is>
-      </c>
-      <c r="Q104" s="19" t="inlineStr">
-        <is>
-          <t>Partial</t>
+          <t>Bank adjustment queue + SoD test</t>
+        </is>
+      </c>
+      <c r="Q104" s="18" t="inlineStr">
+        <is>
+          <t>Implemented</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="15" t="inlineStr">
         <is>
-          <t>REC-04</t>
+          <t>REC-03</t>
         </is>
       </c>
       <c r="B105" s="16" t="inlineStr">
@@ -9946,22 +9946,22 @@
       </c>
       <c r="D105" s="16" t="inlineStr">
         <is>
-          <t>All control accounts</t>
+          <t>Consolidation</t>
         </is>
       </c>
       <c r="E105" s="16" t="inlineStr">
         <is>
-          <t>A sub-ledger silently drifts from its GL control account at period-end and no single review catches it (incomplete/inaccurate balances reach the financial statements).</t>
+          <t>Intercompany balances not eliminated/agreed.</t>
         </is>
       </c>
       <c r="F105" s="16" t="inlineStr">
         <is>
-          <t>Completeness/Accuracy</t>
+          <t>Accuracy</t>
         </is>
       </c>
       <c r="G105" s="16" t="inlineStr">
         <is>
-          <t>Period-end control-account reconciliation PACK: one read (GET /api/finance/reconciliation/controls) ties every major sub-ledger to its GL control account and FLAGS any out-of-balance — AR↔1100, AP↔2000, Inventory↔1200, Gift cards/Customer-deposits↔2200, Deferred revenue↔2400 — reporting per line {sub_ledger, gl_control, variance, reconciled} plus an overall all_reconciled flag and an exceptions count. Liability controls are sign-flipped before comparison. The controller's single 'are the books reconciled?' close view; an exception is a control finding to investigate before sign-off.</t>
+          <t>Intercompany reconciliation &amp; elimination on consolidation.</t>
         </is>
       </c>
       <c r="H105" s="17" t="inlineStr">
@@ -9971,17 +9971,17 @@
       </c>
       <c r="I105" s="17" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="J105" s="17" t="inlineStr">
         <is>
-          <t>Period / on demand</t>
+          <t>Period</t>
         </is>
       </c>
       <c r="K105" s="16" t="inlineStr">
         <is>
-          <t>Controller / CFO</t>
+          <t>Group Controller</t>
         </is>
       </c>
       <c r="L105" s="17" t="inlineStr">
@@ -9991,34 +9991,34 @@
       </c>
       <c r="M105" s="16" t="inlineStr">
         <is>
-          <t>finance.service.ts reconcileControls; finance.controller.ts GET reconciliation/controls (exec/ar/creditors); reuses ledger.trialBalance + the AR/AP/inventory/gift-card/deferred sub-ledgers; cutover/giftcards.ts + compliance.ts (ToE)</t>
+          <t>intercompany; consolidation</t>
         </is>
       </c>
       <c r="N105" s="16" t="inlineStr">
         <is>
-          <t>Inspect the pack: each control account's sub-ledger query + the GL tie + the exceptions roll-up.</t>
+          <t>Inspect IC matching + elimination.</t>
         </is>
       </c>
       <c r="O105" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: with a clean set, every line reconciled + all_reconciled=true; introduce a known sub-ledger/GL difference and confirm it surfaces as an exception (re-performed: gift-card 2200 + inventory 1200 ties asserted by the harnesses).</t>
+          <t>Sample IC pairs agree &amp; eliminate.</t>
         </is>
       </c>
       <c r="P105" s="16" t="inlineStr">
         <is>
-          <t>Reconciliation pack; exceptions list</t>
-        </is>
-      </c>
-      <c r="Q105" s="18" t="inlineStr">
-        <is>
-          <t>Implemented</t>
+          <t>IC recon</t>
+        </is>
+      </c>
+      <c r="Q105" s="19" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="11" t="inlineStr">
         <is>
-          <t>REC-05</t>
+          <t>REC-04</t>
         </is>
       </c>
       <c r="B106" s="12" t="inlineStr">
@@ -10033,42 +10033,42 @@
       </c>
       <c r="D106" s="12" t="inlineStr">
         <is>
-          <t>Cash; Bank</t>
+          <t>All control accounts</t>
         </is>
       </c>
       <c r="E106" s="12" t="inlineStr">
         <is>
-          <t>Till cash dropped to the safe never reaches the bank, or a deposit isn't matched to the statement — cash sits unbanked (theft/loss exposure) or the bank balance can't be tied to the books.</t>
+          <t>A sub-ledger silently drifts from its GL control account at period-end and no single review catches it (incomplete/inaccurate balances reach the financial statements).</t>
         </is>
       </c>
       <c r="F106" s="12" t="inlineStr">
         <is>
-          <t>Completeness/Existence/Authorization</t>
+          <t>Completeness/Accuracy</t>
         </is>
       </c>
       <c r="G106" s="12" t="inlineStr">
         <is>
-          <t>Cash banking — safe-drop → bank deposit → reconciliation: till 'drop's move cash from the drawer to the safe (drawer-only, no GL). Banking BATCHES the undeposited drops into a deposit and posts the GL (Dr &lt;bank account, e.g. 1010&gt; / Cr 1000 Cash), stamping each drop with the deposit id; the deposit is then RECONCILED to the bank statement (status Deposited→Reconciled). A detective read (GET /api/bank/deposits/undeposited-drops) surfaces the CASH STILL IN THE SAFE (drops with deposit_id NULL) — the unbanked exposure to chase. SoD: banking is a treasury duty (exec/ar) — segregated from the cashier (pos_till) who drops the cash, so the person who removes cash from the drawer is not the one who banks it.</t>
+          <t>Period-end control-account reconciliation PACK: one read (GET /api/finance/reconciliation/controls) ties every major sub-ledger to its GL control account and FLAGS any out-of-balance — AR↔1100, AP↔2000, Inventory↔1200, Gift cards/Customer-deposits↔2200, Deferred revenue↔2400 — reporting per line {sub_ledger, gl_control, variance, reconciled} plus an overall all_reconciled flag and an exceptions count. Liability controls are sign-flipped before comparison. The controller's single 'are the books reconciled?' close view; an exception is a control finding to investigate before sign-off.</t>
         </is>
       </c>
       <c r="H106" s="13" t="inlineStr">
         <is>
-          <t>Det/Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I106" s="13" t="inlineStr">
         <is>
-          <t>Auto+Manual</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J106" s="13" t="inlineStr">
         <is>
-          <t>Per banking run</t>
+          <t>Period / on demand</t>
         </is>
       </c>
       <c r="K106" s="12" t="inlineStr">
         <is>
-          <t>FinancialController / Treasury</t>
+          <t>Controller / CFO</t>
         </is>
       </c>
       <c r="L106" s="13" t="inlineStr">
@@ -10078,22 +10078,22 @@
       </c>
       <c r="M106" s="12" t="inlineStr">
         <is>
-          <t>bank.service.ts undepositedDrops/createDeposit (Dr bank/Cr 1000, stamps deposit_id)/reconcileDeposit/listDeposits; bank.controller.ts (deposits, deposits/undeposited-drops, deposits/:id/reconcile; exec/ar); schema/cash.ts bank_deposits + cash_movements.deposit_id + migration 0152; /cash-banking UI; cutover/cash-banking.ts (ToE)</t>
+          <t>finance.service.ts reconcileControls; finance.controller.ts GET reconciliation/controls (exec/ar/creditors); reuses ledger.trialBalance + the AR/AP/inventory/gift-card/deferred sub-ledgers; cutover/giftcards.ts + compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N106" s="12" t="inlineStr">
         <is>
-          <t>Inspect the undeposited-drop exposure read + the deposit GL (bank↔1000) + the reconcile step + the SoD (cashier vs treasury).</t>
+          <t>Inspect the pack: each control account's sub-ledger query + the GL tie + the exceptions roll-up.</t>
         </is>
       </c>
       <c r="O106" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: two till drops → cash-in-safe shows the total; a cashier (pos_till) cannot bank (403); treasury banks → Dr bank / Cr 1000, cash-in-safe back to 0; reconcile the deposit; trial balance balanced (re-performed by the cash-banking harness).</t>
+          <t>Re-perform: with a clean set, every line reconciled + all_reconciled=true; introduce a known sub-ledger/GL difference and confirm it surfaces as an exception (re-performed: gift-card 2200 + inventory 1200 ties asserted by the harnesses).</t>
         </is>
       </c>
       <c r="P106" s="12" t="inlineStr">
         <is>
-          <t>Bank-deposit register; undeposited-drop (cash-in-safe) exposure</t>
+          <t>Reconciliation pack; exceptions list</t>
         </is>
       </c>
       <c r="Q106" s="18" t="inlineStr">
@@ -10105,12 +10105,12 @@
     <row r="107">
       <c r="A107" s="15" t="inlineStr">
         <is>
-          <t>GOV-01</t>
+          <t>REC-05</t>
         </is>
       </c>
       <c r="B107" s="16" t="inlineStr">
         <is>
-          <t>Monitoring</t>
+          <t>Reconciliation</t>
         </is>
       </c>
       <c r="C107" s="17" t="inlineStr">
@@ -10120,42 +10120,42 @@
       </c>
       <c r="D107" s="16" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Cash; Bank</t>
         </is>
       </c>
       <c r="E107" s="16" t="inlineStr">
         <is>
-          <t>A maker-checker approval sits un-actioned and is forgotten — a transaction stalls before it is effective, or (worse) a control is quietly bypassed and no one notices an item never got its independent review.</t>
+          <t>Till cash dropped to the safe never reaches the bank, or a deposit isn't matched to the statement — cash sits unbanked (theft/loss exposure) or the bank balance can't be tied to the books.</t>
         </is>
       </c>
       <c r="F107" s="16" t="inlineStr">
         <is>
-          <t>Authorization/Completeness</t>
+          <t>Completeness/Existence/Authorization</t>
         </is>
       </c>
       <c r="G107" s="16" t="inlineStr">
         <is>
-          <t>Pending-approvals MONITOR (COSO monitoring): a single worklist of EVERY item awaiting independent approval across the system, each with its AGE in days and an overdue roll-up — spanning the manual-JE (GL-05), bank-adjustment (BANK-02), AP-disbursement (EXP-06), payroll (PAY-03), asset-revaluation (FA-08), asset-disposal (FA-09), inventory-write-off (INV-07), till-close cash over/short (REV-13), FX-rate (FX-04), budget (BUD-01) and large-refund (REV-16) maker-checkers. The controller reviews it before close; a stale item (age beyond the threshold) is a control finding to chase or escalate. The /approvals screen also lets a manager approve/reject a material till variance or a large refund inline (the pending types with no dedicated module screen). Read-only worklist; tenant-scoped via the caller's RLS.</t>
+          <t>Cash banking — safe-drop → bank deposit → reconciliation: till 'drop's move cash from the drawer to the safe (drawer-only, no GL). Banking BATCHES the undeposited drops into a deposit and posts the GL (Dr &lt;bank account, e.g. 1010&gt; / Cr 1000 Cash), stamping each drop with the deposit id; the deposit is then RECONCILED to the bank statement (status Deposited→Reconciled). A detective read (GET /api/bank/deposits/undeposited-drops) surfaces the CASH STILL IN THE SAFE (drops with deposit_id NULL) — the unbanked exposure to chase. SoD: banking is a treasury duty (exec/ar) — segregated from the cashier (pos_till) who drops the cash, so the person who removes cash from the drawer is not the one who banks it.</t>
         </is>
       </c>
       <c r="H107" s="17" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Det/Prev</t>
         </is>
       </c>
       <c r="I107" s="17" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="J107" s="17" t="inlineStr">
         <is>
-          <t>Continuous / pre-close</t>
+          <t>Per banking run</t>
         </is>
       </c>
       <c r="K107" s="16" t="inlineStr">
         <is>
-          <t>Controller / CFO</t>
+          <t>FinancialController / Treasury</t>
         </is>
       </c>
       <c r="L107" s="17" t="inlineStr">
@@ -10165,22 +10165,22 @@
       </c>
       <c r="M107" s="16" t="inlineStr">
         <is>
-          <t>finance.service.ts pendingApprovals; finance.controller.ts GET approvals/pending (exec/approvals/creditors); aggregates journalEntries(Draft incl. BANKADJ→BANK-02)/apPayments/payruns/asset_revaluations/fixed_assets(disposal_pending)/inv_writeoff_requests/till_sessions(PendingApproval)/fx_rates(PendingApproval)/budgets(PendingApproval); cutover/compliance.ts (ToE)</t>
+          <t>bank.service.ts undepositedDrops/createDeposit (Dr bank/Cr 1000, stamps deposit_id)/reconcileDeposit/listDeposits; bank.controller.ts (deposits, deposits/undeposited-drops, deposits/:id/reconcile; exec/ar); schema/cash.ts bank_deposits + cash_movements.deposit_id + migration 0152; /cash-banking UI; cutover/cash-banking.ts (ToE)</t>
         </is>
       </c>
       <c r="N107" s="16" t="inlineStr">
         <is>
-          <t>Inspect the aggregation across all pending sources + the age/overdue roll-up.</t>
+          <t>Inspect the undeposited-drop exposure read + the deposit GL (bank↔1000) + the reconcile step + the SoD (cashier vs treasury).</t>
         </is>
       </c>
       <c r="O107" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: create a pending item (e.g. a Draft JE) and confirm it appears in the worklist with its control ID, amount and age; the overdue count flags items past the threshold (re-performed by the harness).</t>
+          <t>Re-perform: two till drops → cash-in-safe shows the total; a cashier (pos_till) cannot bank (403); treasury banks → Dr bank / Cr 1000, cash-in-safe back to 0; reconcile the deposit; trial balance balanced (re-performed by the cash-banking harness).</t>
         </is>
       </c>
       <c r="P107" s="16" t="inlineStr">
         <is>
-          <t>Pending-approvals worklist</t>
+          <t>Bank-deposit register; undeposited-drop (cash-in-safe) exposure</t>
         </is>
       </c>
       <c r="Q107" s="18" t="inlineStr">
@@ -10192,12 +10192,12 @@
     <row r="108">
       <c r="A108" s="11" t="inlineStr">
         <is>
-          <t>TAX-01</t>
+          <t>GOV-01</t>
         </is>
       </c>
       <c r="B108" s="12" t="inlineStr">
         <is>
-          <t>Tax</t>
+          <t>Monitoring</t>
         </is>
       </c>
       <c r="C108" s="13" t="inlineStr">
@@ -10207,27 +10207,27 @@
       </c>
       <c r="D108" s="12" t="inlineStr">
         <is>
-          <t>Tax (VAT)</t>
+          <t>All</t>
         </is>
       </c>
       <c r="E108" s="12" t="inlineStr">
         <is>
-          <t>VAT computed incorrectly → filing/penalty risk.</t>
+          <t>A maker-checker approval sits un-actioned and is forgotten — a transaction stalls before it is effective, or (worse) a control is quietly bypassed and no one notices an item never got its independent review.</t>
         </is>
       </c>
       <c r="F108" s="12" t="inlineStr">
         <is>
-          <t>Accuracy</t>
+          <t>Authorization/Completeness</t>
         </is>
       </c>
       <c r="G108" s="12" t="inlineStr">
         <is>
-          <t>VAT via pluggable provider (TH 7%); unit-tested; no hard-coded rate.</t>
+          <t>Pending-approvals MONITOR (COSO monitoring): a single worklist of EVERY item awaiting independent approval across the system, each with its AGE in days and an overdue roll-up — spanning the manual-JE (GL-05), bank-adjustment (BANK-02), AP-disbursement (EXP-06), payroll (PAY-03), asset-revaluation (FA-08), asset-disposal (FA-09), inventory-write-off (INV-07), till-close cash over/short (REV-13), FX-rate (FX-04), budget (BUD-01) and large-refund (REV-16) maker-checkers. The controller reviews it before close; a stale item (age beyond the threshold) is a control finding to chase or escalate. The /approvals screen also lets a manager approve/reject a material till variance or a large refund inline (the pending types with no dedicated module screen). Read-only worklist; tenant-scoped via the caller's RLS.</t>
         </is>
       </c>
       <c r="H108" s="13" t="inlineStr">
         <is>
-          <t>Auto</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I108" s="13" t="inlineStr">
@@ -10237,37 +10237,37 @@
       </c>
       <c r="J108" s="13" t="inlineStr">
         <is>
-          <t>Per txn</t>
+          <t>Continuous / pre-close</t>
         </is>
       </c>
       <c r="K108" s="12" t="inlineStr">
         <is>
-          <t>Tax / Controller</t>
+          <t>Controller / CFO</t>
         </is>
       </c>
       <c r="L108" s="13" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="M108" s="12" t="inlineStr">
         <is>
-          <t>tax/tax-providers.ts; tax.service.ts; test/unit.test.ts</t>
+          <t>finance.service.ts pendingApprovals; finance.controller.ts GET approvals/pending (exec/approvals/creditors); aggregates journalEntries(Draft incl. BANKADJ→BANK-02)/apPayments/payruns/asset_revaluations/fixed_assets(disposal_pending)/inv_writeoff_requests/till_sessions(PendingApproval)/fx_rates(PendingApproval)/budgets(PendingApproval); cutover/compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N108" s="12" t="inlineStr">
         <is>
-          <t>Inspect rate provider + tests.</t>
+          <t>Inspect the aggregation across all pending sources + the age/overdue roll-up.</t>
         </is>
       </c>
       <c r="O108" s="12" t="inlineStr">
         <is>
-          <t>Re-perform VAT on sample; tie to return.</t>
+          <t>Re-perform: create a pending item (e.g. a Draft JE) and confirm it appears in the worklist with its control ID, amount and age; the overdue count flags items past the threshold (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P108" s="12" t="inlineStr">
         <is>
-          <t>VAT tests</t>
+          <t>Pending-approvals worklist</t>
         </is>
       </c>
       <c r="Q108" s="18" t="inlineStr">
@@ -10279,7 +10279,7 @@
     <row r="109">
       <c r="A109" s="15" t="inlineStr">
         <is>
-          <t>TAX-02</t>
+          <t>TAX-01</t>
         </is>
       </c>
       <c r="B109" s="16" t="inlineStr">
@@ -10294,22 +10294,22 @@
       </c>
       <c r="D109" s="16" t="inlineStr">
         <is>
-          <t>Tax; Revenue</t>
+          <t>Tax (VAT)</t>
         </is>
       </c>
       <c r="E109" s="16" t="inlineStr">
         <is>
-          <t>Non-compliant e-Tax invoice / not transmitted to ETDA.</t>
+          <t>VAT computed incorrectly → filing/penalty risk.</t>
         </is>
       </c>
       <c r="F109" s="16" t="inlineStr">
         <is>
-          <t>Accuracy/Compliance</t>
+          <t>Accuracy</t>
         </is>
       </c>
       <c r="G109" s="16" t="inlineStr">
         <is>
-          <t>e-Tax invoice (ETDA UBL 2.1 XML) generation + email with CC to ETDA timestamp mailbox.</t>
+          <t>VAT via pluggable provider (TH 7%); unit-tested; no hard-coded rate.</t>
         </is>
       </c>
       <c r="H109" s="17" t="inlineStr">
@@ -10324,37 +10324,37 @@
       </c>
       <c r="J109" s="17" t="inlineStr">
         <is>
-          <t>Per invoice</t>
+          <t>Per txn</t>
         </is>
       </c>
       <c r="K109" s="16" t="inlineStr">
         <is>
-          <t>Tax</t>
+          <t>Tax / Controller</t>
         </is>
       </c>
       <c r="L109" s="17" t="inlineStr">
         <is>
-          <t>P10/P13</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="M109" s="16" t="inlineStr">
         <is>
-          <t>tax-docs/etax-xml.ts; etax-email.service.ts (tested)</t>
+          <t>tax/tax-providers.ts; tax.service.ts; test/unit.test.ts</t>
         </is>
       </c>
       <c r="N109" s="16" t="inlineStr">
         <is>
-          <t>Inspect XML schema + email composer.</t>
+          <t>Inspect rate provider + tests.</t>
         </is>
       </c>
       <c r="O109" s="16" t="inlineStr">
         <is>
-          <t>Sample invoices: valid XML, correct CC/escaping.</t>
+          <t>Re-perform VAT on sample; tie to return.</t>
         </is>
       </c>
       <c r="P109" s="16" t="inlineStr">
         <is>
-          <t>e-Tax samples</t>
+          <t>VAT tests</t>
         </is>
       </c>
       <c r="Q109" s="18" t="inlineStr">
@@ -10366,7 +10366,7 @@
     <row r="110">
       <c r="A110" s="11" t="inlineStr">
         <is>
-          <t>TAX-03</t>
+          <t>TAX-02</t>
         </is>
       </c>
       <c r="B110" s="12" t="inlineStr">
@@ -10381,22 +10381,22 @@
       </c>
       <c r="D110" s="12" t="inlineStr">
         <is>
-          <t>Tax (WHT)</t>
+          <t>Tax; Revenue</t>
         </is>
       </c>
       <c r="E110" s="12" t="inlineStr">
         <is>
-          <t>Withholding tax mis-computed / not reported.</t>
+          <t>Non-compliant e-Tax invoice / not transmitted to ETDA.</t>
         </is>
       </c>
       <c r="F110" s="12" t="inlineStr">
         <is>
-          <t>Accuracy</t>
+          <t>Accuracy/Compliance</t>
         </is>
       </c>
       <c r="G110" s="12" t="inlineStr">
         <is>
-          <t>WHT computation and ภ.ง.ด. reporting.</t>
+          <t>e-Tax invoice (ETDA UBL 2.1 XML) generation + email with CC to ETDA timestamp mailbox.</t>
         </is>
       </c>
       <c r="H110" s="13" t="inlineStr">
@@ -10411,7 +10411,7 @@
       </c>
       <c r="J110" s="13" t="inlineStr">
         <is>
-          <t>Per txn / monthly</t>
+          <t>Per invoice</t>
         </is>
       </c>
       <c r="K110" s="12" t="inlineStr">
@@ -10421,39 +10421,39 @@
       </c>
       <c r="L110" s="13" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P10/P13</t>
         </is>
       </c>
       <c r="M110" s="12" t="inlineStr">
         <is>
-          <t>tax-reports; payroll</t>
+          <t>tax-docs/etax-xml.ts; etax-email.service.ts (tested)</t>
         </is>
       </c>
       <c r="N110" s="12" t="inlineStr">
         <is>
-          <t>Inspect WHT logic + report.</t>
+          <t>Inspect XML schema + email composer.</t>
         </is>
       </c>
       <c r="O110" s="12" t="inlineStr">
         <is>
-          <t>Re-perform WHT on sample; tie to filing.</t>
+          <t>Sample invoices: valid XML, correct CC/escaping.</t>
         </is>
       </c>
       <c r="P110" s="12" t="inlineStr">
         <is>
-          <t>WHT report</t>
-        </is>
-      </c>
-      <c r="Q110" s="19" t="inlineStr">
-        <is>
-          <t>Partial</t>
+          <t>e-Tax samples</t>
+        </is>
+      </c>
+      <c r="Q110" s="18" t="inlineStr">
+        <is>
+          <t>Implemented</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="15" t="inlineStr">
         <is>
-          <t>TAX-04</t>
+          <t>TAX-03</t>
         </is>
       </c>
       <c r="B111" s="16" t="inlineStr">
@@ -10468,27 +10468,27 @@
       </c>
       <c r="D111" s="16" t="inlineStr">
         <is>
-          <t>Tax (VAT); Tax Payable (2100)</t>
+          <t>Tax (WHT)</t>
         </is>
       </c>
       <c r="E111" s="16" t="inlineStr">
         <is>
-          <t>Output/input VAT on the filed ภ.พ.30 return does not agree to the GL — VAT liability mis-stated, a filing/penalty exposure, or a posting omission goes undetected before submission.</t>
+          <t>Withholding tax mis-computed / not reported.</t>
         </is>
       </c>
       <c r="F111" s="16" t="inlineStr">
         <is>
-          <t>Completeness/Accuracy</t>
+          <t>Accuracy</t>
         </is>
       </c>
       <c r="G111" s="16" t="inlineStr">
         <is>
-          <t>Periodic VAT-return ↔ GL reconciliation (ภ.พ.30): the monthly return (GET /api/tax-reports/pp30) is built from the sales/output-VAT and purchase/input-VAT sub-reports, computes net VAT = output − input, and RECONCILES it to the **GL account 2100 (Tax Payable) net movement** for the same period (Σ credit − Σ debit over Posted entries) — returning `reconciliation.tied` = true only when the two agree within rounding. A non-tie is a detective finding to investigate and clear BEFORE filing (the form also carries the ม.157 deadline = the 15th of the next month). Output VAT is posted to 2100 on every sale (Cr) and reversed on returns (Dr); input VAT is posted on AP bills (Dr) — so 2100's net is the period's VAT payable. Read-only report; exportable to a ภ.พ.30 PDF/HTML.</t>
+          <t>WHT computation and ภ.ง.ด. reporting.</t>
         </is>
       </c>
       <c r="H111" s="17" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Auto</t>
         </is>
       </c>
       <c r="I111" s="17" t="inlineStr">
@@ -10498,54 +10498,54 @@
       </c>
       <c r="J111" s="17" t="inlineStr">
         <is>
-          <t>Monthly / pre-filing</t>
+          <t>Per txn / monthly</t>
         </is>
       </c>
       <c r="K111" s="16" t="inlineStr">
         <is>
-          <t>Tax / FinancialController</t>
+          <t>Tax</t>
         </is>
       </c>
       <c r="L111" s="17" t="inlineStr">
         <is>
-          <t>P10/P16</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="M111" s="16" t="inlineStr">
         <is>
-          <t>tax-reports.service.ts pp30 (outputVat/inputVat + 2100 net-movement tie); tax-reports.controller.ts (GET pp30, pp30/export, exec); tax-reports-pdf.ts; dine-in.service.ts/returns.service.ts/finance.service.ts post 2100 on sale/return/AP; /tax/reports UI; cutover/taxdocs.ts (ToE)</t>
+          <t>tax-reports; payroll</t>
         </is>
       </c>
       <c r="N111" s="16" t="inlineStr">
         <is>
-          <t>Inspect the pp30 build + the 2100 net-movement query + the tie flag + the filing deadline.</t>
+          <t>Inspect WHT logic + report.</t>
         </is>
       </c>
       <c r="O111" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: the pp30 return computes net VAT (output − input), the GL 2100 net movement reflects the posted input VAT, and the reconciliation block exposes the gl_account (2100), the report net VAT and a boolean tie verdict (tied iff the two agree within rounding); the ภ.พ.30 export renders (re-performed by the taxdocs harness).</t>
+          <t>Re-perform WHT on sample; tie to filing.</t>
         </is>
       </c>
       <c r="P111" s="16" t="inlineStr">
         <is>
-          <t>ภ.พ.30 return + GL-2100 reconciliation tie</t>
-        </is>
-      </c>
-      <c r="Q111" s="18" t="inlineStr">
-        <is>
-          <t>Implemented</t>
+          <t>WHT report</t>
+        </is>
+      </c>
+      <c r="Q111" s="19" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="11" t="inlineStr">
         <is>
-          <t>PAY-01</t>
+          <t>TAX-04</t>
         </is>
       </c>
       <c r="B112" s="12" t="inlineStr">
         <is>
-          <t>Payroll</t>
+          <t>Tax</t>
         </is>
       </c>
       <c r="C112" s="13" t="inlineStr">
@@ -10555,27 +10555,27 @@
       </c>
       <c r="D112" s="12" t="inlineStr">
         <is>
-          <t>Payroll expense/liability</t>
+          <t>Tax (VAT); Tax Payable (2100)</t>
         </is>
       </c>
       <c r="E112" s="12" t="inlineStr">
         <is>
-          <t>Payroll, SSO and PIT mis-computed.</t>
+          <t>Output/input VAT on the filed ภ.พ.30 return does not agree to the GL — VAT liability mis-stated, a filing/penalty exposure, or a posting omission goes undetected before submission.</t>
         </is>
       </c>
       <c r="F112" s="12" t="inlineStr">
         <is>
-          <t>Accuracy</t>
+          <t>Completeness/Accuracy</t>
         </is>
       </c>
       <c r="G112" s="12" t="inlineStr">
         <is>
-          <t>Payroll engine — SSO 5% (cap 750), progressive PIT, payslip net; unit-tested.</t>
+          <t>Periodic VAT-return ↔ GL reconciliation (ภ.พ.30): the monthly return (GET /api/tax-reports/pp30) is built from the sales/output-VAT and purchase/input-VAT sub-reports, computes net VAT = output − input, and RECONCILES it to the **GL account 2100 (Tax Payable) net movement** for the same period (Σ credit − Σ debit over Posted entries) — returning `reconciliation.tied` = true only when the two agree within rounding. A non-tie is a detective finding to investigate and clear BEFORE filing (the form also carries the ม.157 deadline = the 15th of the next month). Output VAT is posted to 2100 on every sale (Cr) and reversed on returns (Dr); input VAT is posted on AP bills (Dr) — so 2100's net is the period's VAT payable. Read-only report; exportable to a ภ.พ.30 PDF/HTML.</t>
         </is>
       </c>
       <c r="H112" s="13" t="inlineStr">
         <is>
-          <t>Auto</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I112" s="13" t="inlineStr">
@@ -10585,37 +10585,37 @@
       </c>
       <c r="J112" s="13" t="inlineStr">
         <is>
-          <t>Per run</t>
+          <t>Monthly / pre-filing</t>
         </is>
       </c>
       <c r="K112" s="12" t="inlineStr">
         <is>
-          <t>HR / Payroll</t>
+          <t>Tax / FinancialController</t>
         </is>
       </c>
       <c r="L112" s="13" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P10/P16</t>
         </is>
       </c>
       <c r="M112" s="12" t="inlineStr">
         <is>
-          <t>payroll/payroll-calc.ts; test/unit.test.ts</t>
+          <t>tax-reports.service.ts pp30 (outputVat/inputVat + 2100 net-movement tie); tax-reports.controller.ts (GET pp30, pp30/export, exec); tax-reports-pdf.ts; dine-in.service.ts/returns.service.ts/finance.service.ts post 2100 on sale/return/AP; /tax/reports UI; cutover/taxdocs.ts (ToE)</t>
         </is>
       </c>
       <c r="N112" s="12" t="inlineStr">
         <is>
-          <t>Inspect calc + tests.</t>
+          <t>Inspect the pp30 build + the 2100 net-movement query + the tie flag + the filing deadline.</t>
         </is>
       </c>
       <c r="O112" s="12" t="inlineStr">
         <is>
-          <t>Re-perform sample payslips.</t>
+          <t>Re-perform: the pp30 return computes net VAT (output − input), the GL 2100 net movement reflects the posted input VAT, and the reconciliation block exposes the gl_account (2100), the report net VAT and a boolean tie verdict (tied iff the two agree within rounding); the ภ.พ.30 export renders (re-performed by the taxdocs harness).</t>
         </is>
       </c>
       <c r="P112" s="12" t="inlineStr">
         <is>
-          <t>Payslip tests</t>
+          <t>ภ.พ.30 return + GL-2100 reconciliation tie</t>
         </is>
       </c>
       <c r="Q112" s="18" t="inlineStr">
@@ -10627,7 +10627,7 @@
     <row r="113">
       <c r="A113" s="15" t="inlineStr">
         <is>
-          <t>PAY-02</t>
+          <t>PAY-01</t>
         </is>
       </c>
       <c r="B113" s="16" t="inlineStr">
@@ -10642,27 +10642,27 @@
       </c>
       <c r="D113" s="16" t="inlineStr">
         <is>
-          <t>Payroll liability</t>
+          <t>Payroll expense/liability</t>
         </is>
       </c>
       <c r="E113" s="16" t="inlineStr">
         <is>
-          <t>Statutory withholdings (SSO/WHT/PF) mis-stated or not remitted, so the liability owed to the authorities diverges from the books.</t>
+          <t>Payroll, SSO and PIT mis-computed.</t>
         </is>
       </c>
       <c r="F113" s="16" t="inlineStr">
         <is>
-          <t>Accuracy/Compliance</t>
+          <t>Accuracy</t>
         </is>
       </c>
       <c r="G113" s="16" t="inlineStr">
         <is>
-          <t>Payroll-liability schedule (GET /api/payroll/liabilities): each statutory account — SSO 2350, WHT/PND1 2360, PF 2370 — shows accrued (GL credits) − remitted (GL debits) = outstanding, tied back to the INDEPENDENT payrun accrual with a `reconciled` flag (a divergence flags a manual JE that touched a payroll-liability account outside the payroll process). Treasury remits the cash (POST .../remit → Dr liability / Cr 1000) which clears the outstanding and keeps the books reconciled to the statutory filings; a remittance beyond the outstanding is blocked (REMIT_EXCEEDS_OUTSTANDING).</t>
+          <t>Payroll engine — SSO 5% (cap 750), progressive PIT, payslip net; unit-tested.</t>
         </is>
       </c>
       <c r="H113" s="17" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Auto</t>
         </is>
       </c>
       <c r="I113" s="17" t="inlineStr">
@@ -10672,12 +10672,12 @@
       </c>
       <c r="J113" s="17" t="inlineStr">
         <is>
-          <t>Per run / monthly</t>
+          <t>Per run</t>
         </is>
       </c>
       <c r="K113" s="16" t="inlineStr">
         <is>
-          <t>HR / Payroll / Treasury</t>
+          <t>HR / Payroll</t>
         </is>
       </c>
       <c r="L113" s="17" t="inlineStr">
@@ -10687,22 +10687,22 @@
       </c>
       <c r="M113" s="16" t="inlineStr">
         <is>
-          <t>payroll/payroll.service.ts liabilities/remitLiability</t>
+          <t>payroll/payroll-calc.ts; test/unit.test.ts</t>
         </is>
       </c>
       <c r="N113" s="16" t="inlineStr">
         <is>
-          <t>Inspect the schedule + the accrued/remitted/outstanding tie-out and the reconciled flag.</t>
+          <t>Inspect calc + tests.</t>
         </is>
       </c>
       <c r="O113" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: run a payroll, confirm the SSO/WHT outstanding equals the payrun accrual; remit part and confirm the outstanding falls and the TB stays balanced; attempt an over-remit (REMIT_EXCEEDS_OUTSTANDING).</t>
+          <t>Re-perform sample payslips.</t>
         </is>
       </c>
       <c r="P113" s="16" t="inlineStr">
         <is>
-          <t>Liability schedule + remittance JEs tied to filings</t>
+          <t>Payslip tests</t>
         </is>
       </c>
       <c r="Q113" s="18" t="inlineStr">
@@ -10714,7 +10714,7 @@
     <row r="114">
       <c r="A114" s="11" t="inlineStr">
         <is>
-          <t>PAY-03</t>
+          <t>PAY-02</t>
         </is>
       </c>
       <c r="B114" s="12" t="inlineStr">
@@ -10729,27 +10729,27 @@
       </c>
       <c r="D114" s="12" t="inlineStr">
         <is>
-          <t>Payroll expense/liability; Cash</t>
+          <t>Payroll liability</t>
         </is>
       </c>
       <c r="E114" s="12" t="inlineStr">
         <is>
-          <t>Payroll run posted to the GL without independent review — the preparer both computes and posts their own payroll (ghost employees, inflated rate/hours).</t>
+          <t>Statutory withholdings (SSO/WHT/PF) mis-stated or not remitted, so the liability owed to the authorities diverges from the books.</t>
         </is>
       </c>
       <c r="F114" s="12" t="inlineStr">
         <is>
-          <t>Authorization</t>
+          <t>Accuracy/Compliance</t>
         </is>
       </c>
       <c r="G114" s="12" t="inlineStr">
         <is>
-          <t>Payroll maker-checker (SoD): a run posts its GL entry as a DRAFT (excluded from balances) with the run record 'PendingApproval'; a DIFFERENT user must approve before it becomes effective (approver ≠ preparer enforced regardless of permissions, reusing the GL-05 ledger approval). Reject voids the draft; idempotent per (tenant, period).</t>
+          <t>Payroll-liability schedule (GET /api/payroll/liabilities): each statutory account — SSO 2350, WHT/PND1 2360, PF 2370 — shows accrued (GL credits) − remitted (GL debits) = outstanding, tied back to the INDEPENDENT payrun accrual with a `reconciled` flag (a divergence flags a manual JE that touched a payroll-liability account outside the payroll process). Treasury remits the cash (POST .../remit → Dr liability / Cr 1000) which clears the outstanding and keeps the books reconciled to the statutory filings; a remittance beyond the outstanding is blocked (REMIT_EXCEEDS_OUTSTANDING).</t>
         </is>
       </c>
       <c r="H114" s="13" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I114" s="13" t="inlineStr">
@@ -10759,12 +10759,12 @@
       </c>
       <c r="J114" s="13" t="inlineStr">
         <is>
-          <t>Per run</t>
+          <t>Per run / monthly</t>
         </is>
       </c>
       <c r="K114" s="12" t="inlineStr">
         <is>
-          <t>HR / Payroll; Controller</t>
+          <t>HR / Payroll / Treasury</t>
         </is>
       </c>
       <c r="L114" s="13" t="inlineStr">
@@ -10774,22 +10774,22 @@
       </c>
       <c r="M114" s="12" t="inlineStr">
         <is>
-          <t>payroll/payroll.service.ts approvePayroll/rejectPayroll; migration 0133</t>
+          <t>payroll/payroll.service.ts liabilities/remitLiability</t>
         </is>
       </c>
       <c r="N114" s="12" t="inlineStr">
         <is>
-          <t>Inspect Draft→approve flow + the approver≠preparer check.</t>
+          <t>Inspect the schedule + the accrued/remitted/outstanding tie-out and the reconciled flag.</t>
         </is>
       </c>
       <c r="O114" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: run as A, attempt self-approve (SOD_VIOLATION), approve as B; confirm the JE hits balances only after approval.</t>
+          <t>Re-perform: run a payroll, confirm the SSO/WHT outstanding equals the payrun accrual; remit part and confirm the outstanding falls and the TB stays balanced; attempt an over-remit (REMIT_EXCEEDS_OUTSTANDING).</t>
         </is>
       </c>
       <c r="P114" s="12" t="inlineStr">
         <is>
-          <t>Approval log + SoD test</t>
+          <t>Liability schedule + remittance JEs tied to filings</t>
         </is>
       </c>
       <c r="Q114" s="18" t="inlineStr">
@@ -10801,12 +10801,12 @@
     <row r="115">
       <c r="A115" s="15" t="inlineStr">
         <is>
-          <t>FA-09</t>
+          <t>PAY-03</t>
         </is>
       </c>
       <c r="B115" s="16" t="inlineStr">
         <is>
-          <t>Fixed Assets</t>
+          <t>Payroll</t>
         </is>
       </c>
       <c r="C115" s="17" t="inlineStr">
@@ -10816,12 +10816,12 @@
       </c>
       <c r="D115" s="16" t="inlineStr">
         <is>
-          <t>Property, Plant &amp; Equipment; Cash</t>
+          <t>Payroll expense/liability; Cash</t>
         </is>
       </c>
       <c r="E115" s="16" t="inlineStr">
         <is>
-          <t>Asset disposed without independent review — one person writes an asset off the books and records the proceeds (asset-stripping / theft: dispose a still-held asset, or to a related party below value).</t>
+          <t>Payroll run posted to the GL without independent review — the preparer both computes and posts their own payroll (ghost employees, inflated rate/hours).</t>
         </is>
       </c>
       <c r="F115" s="16" t="inlineStr">
@@ -10831,7 +10831,7 @@
       </c>
       <c r="G115" s="16" t="inlineStr">
         <is>
-          <t>Asset-disposal maker-checker (SoD): a disposal REQUEST posts its GL entry as a DRAFT (excluded from balances) and flags the asset disposal_pending WITHOUT marking it disposed or moving the register; a DIFFERENT user must approve before it is effective (status→disposed, revaluation surplus recycled 3200→3100) (approver ≠ requester enforced regardless of permissions, reusing the GL-05 ledger approval). Reject voids the draft and the asset stays in service; only one disposal may be pending per asset; a disposal-pending asset is frozen from depreciation.</t>
+          <t>Payroll maker-checker (SoD): a run posts its GL entry as a DRAFT (excluded from balances) with the run record 'PendingApproval'; a DIFFERENT user must approve before it becomes effective (approver ≠ preparer enforced regardless of permissions, reusing the GL-05 ledger approval). Reject voids the draft; idempotent per (tenant, period).</t>
         </is>
       </c>
       <c r="H115" s="17" t="inlineStr">
@@ -10846,12 +10846,12 @@
       </c>
       <c r="J115" s="17" t="inlineStr">
         <is>
-          <t>Per disposal</t>
+          <t>Per run</t>
         </is>
       </c>
       <c r="K115" s="16" t="inlineStr">
         <is>
-          <t>FaAccountant / Controller</t>
+          <t>HR / Payroll; Controller</t>
         </is>
       </c>
       <c r="L115" s="17" t="inlineStr">
@@ -10861,22 +10861,22 @@
       </c>
       <c r="M115" s="16" t="inlineStr">
         <is>
-          <t>assets.service.ts dispose(pendingApproval Draft)/approveDisposal/rejectDisposal; assets.controller.ts (:assetNo/dispose/approve|reject); schema/assets.ts fixed_assets.disposal_pending + migration 0135; cutover/basics.ts + worldclass.ts + compliance.ts (ToE)</t>
+          <t>payroll/payroll.service.ts approvePayroll/rejectPayroll; migration 0133</t>
         </is>
       </c>
       <c r="N115" s="16" t="inlineStr">
         <is>
-          <t>Inspect Draft→approve flow + the approver≠requester check + deferred status/recycle.</t>
+          <t>Inspect Draft→approve flow + the approver≠preparer check.</t>
         </is>
       </c>
       <c r="O115" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: request a disposal (Draft JE excluded), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm status→disposed + surplus recycled only after approval (re-performed by the harnesses).</t>
+          <t>Re-perform: run as A, attempt self-approve (SOD_VIOLATION), approve as B; confirm the JE hits balances only after approval.</t>
         </is>
       </c>
       <c r="P115" s="16" t="inlineStr">
         <is>
-          <t>Disposal approval log + SoD test</t>
+          <t>Approval log + SoD test</t>
         </is>
       </c>
       <c r="Q115" s="18" t="inlineStr">
@@ -10888,7 +10888,7 @@
     <row r="116">
       <c r="A116" s="11" t="inlineStr">
         <is>
-          <t>FA-10</t>
+          <t>FA-09</t>
         </is>
       </c>
       <c r="B116" s="12" t="inlineStr">
@@ -10903,22 +10903,22 @@
       </c>
       <c r="D116" s="12" t="inlineStr">
         <is>
-          <t>Property, Plant &amp; Equipment; Accounts Payable</t>
+          <t>Property, Plant &amp; Equipment; Cash</t>
         </is>
       </c>
       <c r="E116" s="12" t="inlineStr">
         <is>
-          <t>Capital purchases mis-capitalised or capitalised without independent review — the person who receives the goods also decides what enters the asset register and at what cost/useful life (fictitious or over-valued assets; capex/opex mis-classification).</t>
+          <t>Asset disposed without independent review — one person writes an asset off the books and records the proceeds (asset-stripping / theft: dispose a still-held asset, or to a related party below value).</t>
         </is>
       </c>
       <c r="F116" s="12" t="inlineStr">
         <is>
-          <t>Authorization; Accuracy</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="G116" s="12" t="inlineStr">
         <is>
-          <t>Procure-to-Capitalize maker-checker (SoD): a goods-receipt line flagged capital (item-master is_fixed_asset or per-PO-line override) is excluded from inventory capitalisation (1200) at receipt and instead becomes ELIGIBLE for the asset register. Capitalisation is a REQUEST that posts NOTHING to the GL; a DIFFERENT user must approve before the fixed_assets row + acquisition JE (Dr 1500 / Cr 2000) are created (approver ≠ requester enforced regardless of permissions). The created asset carries its source GR/PO for end-to-end PR→PO→GR→FA traceability; a GR line cannot be capitalised twice.</t>
+          <t>Asset-disposal maker-checker (SoD): a disposal REQUEST posts its GL entry as a DRAFT (excluded from balances) and flags the asset disposal_pending WITHOUT marking it disposed or moving the register; a DIFFERENT user must approve before it is effective (status→disposed, revaluation surplus recycled 3200→3100) (approver ≠ requester enforced regardless of permissions, reusing the GL-05 ledger approval). Reject voids the draft and the asset stays in service; only one disposal may be pending per asset; a disposal-pending asset is frozen from depreciation.</t>
         </is>
       </c>
       <c r="H116" s="13" t="inlineStr">
@@ -10933,7 +10933,7 @@
       </c>
       <c r="J116" s="13" t="inlineStr">
         <is>
-          <t>Per capital receipt</t>
+          <t>Per disposal</t>
         </is>
       </c>
       <c r="K116" s="12" t="inlineStr">
@@ -10948,22 +10948,22 @@
       </c>
       <c r="M116" s="12" t="inlineStr">
         <is>
-          <t>assets.service.ts registerFromGr/approveRegistration/rejectRegistration/eligibleFromGr; assets.controller.ts (registrations*); procurement.service.ts createGr (is_capital routing, costing excluded); schema/assets.ts asset_registration_requests + fixed_assets.source_gr_no/po_no + migration 0137; cutover/basics.ts + compliance.ts (ToE)</t>
+          <t>assets.service.ts dispose(pendingApproval Draft)/approveDisposal/rejectDisposal; assets.controller.ts (:assetNo/dispose/approve|reject); schema/assets.ts fixed_assets.disposal_pending + migration 0135; cutover/basics.ts + worldclass.ts + compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N116" s="12" t="inlineStr">
         <is>
-          <t>Inspect the eligible→request→approve flow + approver≠requester check + the inventory-vs-asset routing of capital lines.</t>
+          <t>Inspect Draft→approve flow + the approver≠requester check + deferred status/recycle.</t>
         </is>
       </c>
       <c r="O116" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: receive a capital line, raise a registration (no GL), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm the asset + Dr 1500/Cr 2000 post only after approval and the line cannot be re-registered (re-performed by the harnesses).</t>
+          <t>Re-perform: request a disposal (Draft JE excluded), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm status→disposed + surplus recycled only after approval (re-performed by the harnesses).</t>
         </is>
       </c>
       <c r="P116" s="12" t="inlineStr">
         <is>
-          <t>Capitalization approval log + SoD test</t>
+          <t>Disposal approval log + SoD test</t>
         </is>
       </c>
       <c r="Q116" s="18" t="inlineStr">
@@ -10975,12 +10975,12 @@
     <row r="117">
       <c r="A117" s="15" t="inlineStr">
         <is>
-          <t>CON-01</t>
+          <t>FA-10</t>
         </is>
       </c>
       <c r="B117" s="16" t="inlineStr">
         <is>
-          <t>Consolidation &amp; FX</t>
+          <t>Fixed Assets</t>
         </is>
       </c>
       <c r="C117" s="17" t="inlineStr">
@@ -10990,42 +10990,42 @@
       </c>
       <c r="D117" s="16" t="inlineStr">
         <is>
-          <t>Consolidation</t>
+          <t>Property, Plant &amp; Equipment; Accounts Payable</t>
         </is>
       </c>
       <c r="E117" s="16" t="inlineStr">
         <is>
-          <t>Group consolidation mis-stated (ownership/currency).</t>
+          <t>Capital purchases mis-capitalised or capitalised without independent review — the person who receives the goods also decides what enters the asset register and at what cost/useful life (fictitious or over-valued assets; capex/opex mis-classification).</t>
         </is>
       </c>
       <c r="F117" s="16" t="inlineStr">
         <is>
-          <t>Accuracy</t>
+          <t>Authorization; Accuracy</t>
         </is>
       </c>
       <c r="G117" s="16" t="inlineStr">
         <is>
-          <t>Consolidation run (ownership %, entity currency) gated by 'approvals'.</t>
+          <t>Procure-to-Capitalize maker-checker (SoD): a goods-receipt line flagged capital (item-master is_fixed_asset or per-PO-line override) is excluded from inventory capitalisation (1200) at receipt and instead becomes ELIGIBLE for the asset register. Capitalisation is a REQUEST that posts NOTHING to the GL; a DIFFERENT user must approve before the fixed_assets row + acquisition JE (Dr 1500 / Cr 2000) are created (approver ≠ requester enforced regardless of permissions). The created asset carries its source GR/PO for end-to-end PR→PO→GR→FA traceability; a GR line cannot be capitalised twice.</t>
         </is>
       </c>
       <c r="H117" s="17" t="inlineStr">
         <is>
-          <t>Auto+Manual</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I117" s="17" t="inlineStr">
         <is>
-          <t>Period</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J117" s="17" t="inlineStr">
         <is>
-          <t>Period</t>
+          <t>Per capital receipt</t>
         </is>
       </c>
       <c r="K117" s="16" t="inlineStr">
         <is>
-          <t>Group Controller</t>
+          <t>FaAccountant / Controller</t>
         </is>
       </c>
       <c r="L117" s="17" t="inlineStr">
@@ -11035,22 +11035,22 @@
       </c>
       <c r="M117" s="16" t="inlineStr">
         <is>
-          <t>consolidation.service.ts (runConsolidation @Permissions approvals)</t>
+          <t>assets.service.ts registerFromGr/approveRegistration/rejectRegistration/eligibleFromGr; assets.controller.ts (registrations*); procurement.service.ts createGr (is_capital routing, costing excluded); schema/assets.ts asset_registration_requests + fixed_assets.source_gr_no/po_no + migration 0137; cutover/basics.ts + compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N117" s="16" t="inlineStr">
         <is>
-          <t>Inspect consolidation logic + gate.</t>
+          <t>Inspect the eligible→request→approve flow + approver≠requester check + the inventory-vs-asset routing of capital lines.</t>
         </is>
       </c>
       <c r="O117" s="16" t="inlineStr">
         <is>
-          <t>Sample period: consolidated TB ties to entities.</t>
+          <t>Re-perform: receive a capital line, raise a registration (no GL), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm the asset + Dr 1500/Cr 2000 post only after approval and the line cannot be re-registered (re-performed by the harnesses).</t>
         </is>
       </c>
       <c r="P117" s="16" t="inlineStr">
         <is>
-          <t>Consol TB</t>
+          <t>Capitalization approval log + SoD test</t>
         </is>
       </c>
       <c r="Q117" s="18" t="inlineStr">
@@ -11062,7 +11062,7 @@
     <row r="118">
       <c r="A118" s="11" t="inlineStr">
         <is>
-          <t>CON-02</t>
+          <t>CON-01</t>
         </is>
       </c>
       <c r="B118" s="12" t="inlineStr">
@@ -11077,22 +11077,22 @@
       </c>
       <c r="D118" s="12" t="inlineStr">
         <is>
-          <t>FX gain/loss</t>
+          <t>Consolidation</t>
         </is>
       </c>
       <c r="E118" s="12" t="inlineStr">
         <is>
-          <t>FX exposures not revalued at period-end.</t>
+          <t>Group consolidation mis-stated (ownership/currency).</t>
         </is>
       </c>
       <c r="F118" s="12" t="inlineStr">
         <is>
-          <t>Valuation</t>
+          <t>Accuracy</t>
         </is>
       </c>
       <c r="G118" s="12" t="inlineStr">
         <is>
-          <t>FX revaluation at period-end rates; unrealized FX posted (acct 5400).</t>
+          <t>Consolidation run (ownership %, entity currency) gated by 'approvals'.</t>
         </is>
       </c>
       <c r="H118" s="13" t="inlineStr">
@@ -11102,7 +11102,7 @@
       </c>
       <c r="I118" s="13" t="inlineStr">
         <is>
-          <t>Period-end</t>
+          <t>Period</t>
         </is>
       </c>
       <c r="J118" s="13" t="inlineStr">
@@ -11112,7 +11112,7 @@
       </c>
       <c r="K118" s="12" t="inlineStr">
         <is>
-          <t>Controller</t>
+          <t>Group Controller</t>
         </is>
       </c>
       <c r="L118" s="13" t="inlineStr">
@@ -11122,22 +11122,22 @@
       </c>
       <c r="M118" s="12" t="inlineStr">
         <is>
-          <t>fx.service.ts (revalue / unrealized report)</t>
+          <t>consolidation.service.ts (runConsolidation @Permissions approvals)</t>
         </is>
       </c>
       <c r="N118" s="12" t="inlineStr">
         <is>
-          <t>Inspect reval logic + rates.</t>
+          <t>Inspect consolidation logic + gate.</t>
         </is>
       </c>
       <c r="O118" s="12" t="inlineStr">
         <is>
-          <t>Recompute reval on sample balances.</t>
+          <t>Sample period: consolidated TB ties to entities.</t>
         </is>
       </c>
       <c r="P118" s="12" t="inlineStr">
         <is>
-          <t>FX reval JE</t>
+          <t>Consol TB</t>
         </is>
       </c>
       <c r="Q118" s="18" t="inlineStr">
@@ -11149,7 +11149,7 @@
     <row r="119">
       <c r="A119" s="15" t="inlineStr">
         <is>
-          <t>FX-04</t>
+          <t>CON-02</t>
         </is>
       </c>
       <c r="B119" s="16" t="inlineStr">
@@ -11164,42 +11164,42 @@
       </c>
       <c r="D119" s="16" t="inlineStr">
         <is>
-          <t>FX gain/loss; Revenue; AR/AP</t>
+          <t>FX gain/loss</t>
         </is>
       </c>
       <c r="E119" s="16" t="inlineStr">
         <is>
-          <t>A wrong manually-entered FX rate (fat-fingered, e.g. USD 36 keyed as 63) flows straight into a period-end revaluation JE and the unrealized-FX report with no independent review — mis-stating earnings/equity and FX-translated balances.</t>
+          <t>FX exposures not revalued at period-end.</t>
         </is>
       </c>
       <c r="F119" s="16" t="inlineStr">
         <is>
-          <t>Accuracy/Valuation</t>
+          <t>Valuation</t>
         </is>
       </c>
       <c r="G119" s="16" t="inlineStr">
         <is>
-          <t>FX rate maker-checker (SoD): a MANUALLY-entered rate lands as PendingApproval and is EXCLUDED from rate resolution — revaluation, the unrealized-FX report, and consolidation translation all use APPROVED rates only — until a DIFFERENT user approves it (POST /api/fx/rates/approve). Self-approval → SOD_VIOLATION (binds even Admin); reject marks the rate Rejected (never usable); re-entering a rate sends it back to PendingApproval. Externally-sourced (feed) rates carrying an explicit non-manual source are auto-approved. Pending rates are also surfaced, aged, by the pending-approvals monitor (GOV-01).</t>
+          <t>FX revaluation at period-end rates; unrealized FX posted (acct 5400).</t>
         </is>
       </c>
       <c r="H119" s="17" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="I119" s="17" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Period-end</t>
         </is>
       </c>
       <c r="J119" s="17" t="inlineStr">
         <is>
-          <t>Per rate</t>
+          <t>Period</t>
         </is>
       </c>
       <c r="K119" s="16" t="inlineStr">
         <is>
-          <t>Controller / Treasury</t>
+          <t>Controller</t>
         </is>
       </c>
       <c r="L119" s="17" t="inlineStr">
@@ -11209,22 +11209,22 @@
       </c>
       <c r="M119" s="16" t="inlineStr">
         <is>
-          <t>fx.service.ts setRate(manual→PendingApproval)/approveRate/rejectRate/rateAsOf(Approved only); fx.controller.ts (rates/approve|reject|pending gated approvals/gl_close); consolidation.service.ts (translation reads Approved rates); schema/fx.ts fx_rates.status + migration 0141; cutover/fxreval.ts (ToE)</t>
+          <t>fx.service.ts (revalue / unrealized report)</t>
         </is>
       </c>
       <c r="N119" s="16" t="inlineStr">
         <is>
-          <t>Inspect the request→approve flow + the approver≠requester check + that revaluation/reporting resolve Approved rates only.</t>
+          <t>Inspect reval logic + rates.</t>
         </is>
       </c>
       <c r="O119" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: enter a manual rate (PendingApproval), confirm revalue is blocked NO_RATE while pending, attempt self-approve (SOD_VIOLATION), approve as a different user, then revalue succeeds (re-performed by the fxreval harness).</t>
+          <t>Recompute reval on sample balances.</t>
         </is>
       </c>
       <c r="P119" s="16" t="inlineStr">
         <is>
-          <t>FX rate approval log + SoD test</t>
+          <t>FX reval JE</t>
         </is>
       </c>
       <c r="Q119" s="18" t="inlineStr">
@@ -11236,92 +11236,179 @@
     <row r="120">
       <c r="A120" s="11" t="inlineStr">
         <is>
+          <t>FX-04</t>
+        </is>
+      </c>
+      <c r="B120" s="12" t="inlineStr">
+        <is>
+          <t>Consolidation &amp; FX</t>
+        </is>
+      </c>
+      <c r="C120" s="13" t="inlineStr">
+        <is>
+          <t>Application</t>
+        </is>
+      </c>
+      <c r="D120" s="12" t="inlineStr">
+        <is>
+          <t>FX gain/loss; Revenue; AR/AP</t>
+        </is>
+      </c>
+      <c r="E120" s="12" t="inlineStr">
+        <is>
+          <t>A wrong manually-entered FX rate (fat-fingered, e.g. USD 36 keyed as 63) flows straight into a period-end revaluation JE and the unrealized-FX report with no independent review — mis-stating earnings/equity and FX-translated balances.</t>
+        </is>
+      </c>
+      <c r="F120" s="12" t="inlineStr">
+        <is>
+          <t>Accuracy/Valuation</t>
+        </is>
+      </c>
+      <c r="G120" s="12" t="inlineStr">
+        <is>
+          <t>FX rate maker-checker (SoD): a MANUALLY-entered rate lands as PendingApproval and is EXCLUDED from rate resolution — revaluation, the unrealized-FX report, and consolidation translation all use APPROVED rates only — until a DIFFERENT user approves it (POST /api/fx/rates/approve). Self-approval → SOD_VIOLATION (binds even Admin); reject marks the rate Rejected (never usable); re-entering a rate sends it back to PendingApproval. Externally-sourced (feed) rates carrying an explicit non-manual source are auto-approved. Pending rates are also surfaced, aged, by the pending-approvals monitor (GOV-01).</t>
+        </is>
+      </c>
+      <c r="H120" s="13" t="inlineStr">
+        <is>
+          <t>Prev</t>
+        </is>
+      </c>
+      <c r="I120" s="13" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="J120" s="13" t="inlineStr">
+        <is>
+          <t>Per rate</t>
+        </is>
+      </c>
+      <c r="K120" s="12" t="inlineStr">
+        <is>
+          <t>Controller / Treasury</t>
+        </is>
+      </c>
+      <c r="L120" s="13" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="M120" s="12" t="inlineStr">
+        <is>
+          <t>fx.service.ts setRate(manual→PendingApproval)/approveRate/rejectRate/rateAsOf(Approved only); fx.controller.ts (rates/approve|reject|pending gated approvals/gl_close); consolidation.service.ts (translation reads Approved rates); schema/fx.ts fx_rates.status + migration 0141; cutover/fxreval.ts (ToE)</t>
+        </is>
+      </c>
+      <c r="N120" s="12" t="inlineStr">
+        <is>
+          <t>Inspect the request→approve flow + the approver≠requester check + that revaluation/reporting resolve Approved rates only.</t>
+        </is>
+      </c>
+      <c r="O120" s="12" t="inlineStr">
+        <is>
+          <t>Re-perform: enter a manual rate (PendingApproval), confirm revalue is blocked NO_RATE while pending, attempt self-approve (SOD_VIOLATION), approve as a different user, then revalue succeeds (re-performed by the fxreval harness).</t>
+        </is>
+      </c>
+      <c r="P120" s="12" t="inlineStr">
+        <is>
+          <t>FX rate approval log + SoD test</t>
+        </is>
+      </c>
+      <c r="Q120" s="18" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="15" t="inlineStr">
+        <is>
           <t>BUD-01</t>
         </is>
       </c>
-      <c r="B120" s="12" t="inlineStr">
+      <c r="B121" s="16" t="inlineStr">
         <is>
           <t>Budgeting &amp; Planning</t>
         </is>
       </c>
-      <c r="C120" s="13" t="inlineStr">
+      <c r="C121" s="17" t="inlineStr">
         <is>
           <t>Application</t>
         </is>
       </c>
-      <c r="D120" s="12" t="inlineStr">
+      <c r="D121" s="16" t="inlineStr">
         <is>
           <t>Budget; All (variance reporting)</t>
         </is>
       </c>
-      <c r="E120" s="12" t="inlineStr">
+      <c r="E121" s="16" t="inlineStr">
         <is>
           <t>A budget figure is entered/changed by one person and immediately drives the budget-vs-actual variance report — the basis for spend authorization and performance review — with no independent approval; a wrong or self-serving budget makes overspending look 'on budget'.</t>
         </is>
       </c>
-      <c r="F120" s="12" t="inlineStr">
+      <c r="F121" s="16" t="inlineStr">
         <is>
           <t>Authorization/Accuracy</t>
         </is>
       </c>
-      <c r="G120" s="12" t="inlineStr">
+      <c r="G121" s="16" t="inlineStr">
         <is>
           <t>Budget maker-checker (SoD): an upserted budget (POST /api/ledger/budgets) lands as PendingApproval and is EXCLUDED from budget-vs-actual until a DIFFERENT user approves it (POST /api/ledger/budgets/approve for the fiscal_year/account/cost-centre[/period]). Self-approval → SOD_VIOLATION (binds even Admin); reject marks it Rejected (excluded). DEFAULT 'Approved' keeps existing rows + direct planning seeds usable. Pending budgets are also surfaced, aged, by the pending-approvals monitor (GOV-01).</t>
         </is>
       </c>
-      <c r="H120" s="13" t="inlineStr">
+      <c r="H121" s="17" t="inlineStr">
         <is>
           <t>Prev</t>
         </is>
       </c>
-      <c r="I120" s="13" t="inlineStr">
+      <c r="I121" s="17" t="inlineStr">
         <is>
           <t>Automated</t>
         </is>
       </c>
-      <c r="J120" s="13" t="inlineStr">
+      <c r="J121" s="17" t="inlineStr">
         <is>
           <t>Per budget</t>
         </is>
       </c>
-      <c r="K120" s="12" t="inlineStr">
+      <c r="K121" s="16" t="inlineStr">
         <is>
           <t>Controller / FP&amp;A</t>
         </is>
       </c>
-      <c r="L120" s="13" t="inlineStr">
+      <c r="L121" s="17" t="inlineStr">
         <is>
           <t>P10</t>
         </is>
       </c>
-      <c r="M120" s="12" t="inlineStr">
+      <c r="M121" s="16" t="inlineStr">
         <is>
           <t>budget.service.ts upsertBudget(→PendingApproval)/approveBudget/rejectBudget/budgetVsActual(Approved only); budget.controller.ts (budgets/approve|reject|pending gated approvals/gl_close); schema/budgets.ts budgets.status + migration 0142; cutover/budget.ts (ToE)</t>
         </is>
       </c>
-      <c r="N120" s="12" t="inlineStr">
+      <c r="N121" s="16" t="inlineStr">
         <is>
           <t>Inspect the request→approve flow + the approver≠requester check + that budget-vs-actual counts Approved budgets only.</t>
         </is>
       </c>
-      <c r="O120" s="12" t="inlineStr">
+      <c r="O121" s="16" t="inlineStr">
         <is>
           <t>Re-perform: upsert a budget (PendingApproval, excluded from variance), attempt self-approve (SOD_VIOLATION), approve as a different user, confirm it then appears in budget-vs-actual (re-performed by the budget harness).</t>
         </is>
       </c>
-      <c r="P120" s="12" t="inlineStr">
+      <c r="P121" s="16" t="inlineStr">
         <is>
           <t>Budget approval log + SoD test</t>
         </is>
       </c>
-      <c r="Q120" s="18" t="inlineStr">
+      <c r="Q121" s="18" t="inlineStr">
         <is>
           <t>Implemented</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q120"/>
+  <autoFilter ref="A1:Q121"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -12504,7 +12591,7 @@
         </is>
       </c>
       <c r="C5" s="29">
-        <f>COUNTIF(RCM!$Q$2:$Q$120,B5)</f>
+        <f>COUNTIF(RCM!$Q$2:$Q$121,B5)</f>
         <v/>
       </c>
     </row>
@@ -12515,7 +12602,7 @@
         </is>
       </c>
       <c r="C6" s="29">
-        <f>COUNTIF(RCM!$Q$2:$Q$120,B6)</f>
+        <f>COUNTIF(RCM!$Q$2:$Q$121,B6)</f>
         <v/>
       </c>
     </row>
@@ -12526,7 +12613,7 @@
         </is>
       </c>
       <c r="C7" s="29">
-        <f>COUNTIF(RCM!$Q$2:$Q$120,B7)</f>
+        <f>COUNTIF(RCM!$Q$2:$Q$121,B7)</f>
         <v/>
       </c>
     </row>
@@ -12537,7 +12624,7 @@
         </is>
       </c>
       <c r="C8" s="32">
-        <f>COUNTA(RCM!$A$2:$A$120)</f>
+        <f>COUNTA(RCM!$A$2:$A$121)</f>
         <v/>
       </c>
     </row>
@@ -12555,7 +12642,7 @@
         </is>
       </c>
       <c r="C11" s="29">
-        <f>COUNTIF(RCM!$C$2:$C$120,B11)</f>
+        <f>COUNTIF(RCM!$C$2:$C$121,B11)</f>
         <v/>
       </c>
     </row>
@@ -12566,7 +12653,7 @@
         </is>
       </c>
       <c r="C12" s="29">
-        <f>COUNTIF(RCM!$C$2:$C$120,B12)</f>
+        <f>COUNTIF(RCM!$C$2:$C$121,B12)</f>
         <v/>
       </c>
     </row>
@@ -12577,7 +12664,7 @@
         </is>
       </c>
       <c r="C13" s="29">
-        <f>COUNTIF(RCM!$C$2:$C$120,B13)</f>
+        <f>COUNTIF(RCM!$C$2:$C$121,B13)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: merge main, renumber close_runs 0162→0163 (food_cost_variance took 0162)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/compliance/Oshinei_ERP_SOX_RCM_v1.xlsx
+++ b/compliance/Oshinei_ERP_SOX_RCM_v1.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'RCM'!$A$1:$Q$121</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'RCM'!$A$1:$Q$122</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Gap Remediation'!$A$2:$H$18</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -858,7 +858,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q121"/>
+  <dimension ref="A1:Q122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -7060,12 +7060,12 @@
     <row r="72">
       <c r="A72" s="11" t="inlineStr">
         <is>
-          <t>BRANCH-01</t>
+          <t>INV-11</t>
         </is>
       </c>
       <c r="B72" s="12" t="inlineStr">
         <is>
-          <t>Multi-Branch &amp; Offline POS</t>
+          <t>Inventory &amp; COGS</t>
         </is>
       </c>
       <c r="C72" s="13" t="inlineStr">
@@ -7075,22 +7075,22 @@
       </c>
       <c r="D72" s="12" t="inlineStr">
         <is>
-          <t>Revenue</t>
+          <t>Inventory; COGS</t>
         </is>
       </c>
       <c r="E72" s="12" t="inlineStr">
         <is>
-          <t>A POS sale is not attributed to its originating branch, so the consolidated branch roll-up is incomplete and cannot be tied to GL revenue.</t>
+          <t>Theoretical-vs-actual food-cost variance is a single undifferentiated number — a manager sees that COGS ran over the recipe but not WHY or WHERE, so the over-usage can't be acted on (over-portioning vs spoilage vs theft go unaddressed and recur).</t>
         </is>
       </c>
       <c r="F72" s="12" t="inlineStr">
         <is>
-          <t>Completeness</t>
+          <t>Accuracy/Completeness</t>
         </is>
       </c>
       <c r="G72" s="12" t="inlineStr">
         <is>
-          <t>Branch sale-tagging + HQ consolidation: every POS sale carries cust_pos_sales.branch_id; GET /api/branches/consolidated aggregates per branch (excluding Voided) and surfaces untagged sales as branch '(none)' — a deliberate completeness flag the controller investigates and clears before tying the consolidated total to GL revenue.</t>
+          <t>Reason-coded food-cost variance review: each EOD-count variance (cust_variance — theoretical vs actual ingredient use, valued at cost) is tagged with a normalized reason_code (WASTE/OVERSTOCK/SPOILAGE/PORTIONING/THEFT/OTHER, enum-validated at POST /api/portal/variance) and an optional station. GET /api/menu/food-cost/variance values the variance at ingredient cost and rolls it up three ways — per ingredient (with High/Medium anomaly bands), by_reason and by_station — netting unfavourable/favourable, so 'Sauce station is 8% over theoretical (portioning) → retrain' is actionable. Yield/waste factors on the recipe BoM (INV-03) feed the theoretical baseline so the variance isn't inflated by un-costed trim loss. Tenant-scoped (RLS); read gated by exec/order_mgt.</t>
         </is>
       </c>
       <c r="H72" s="13" t="inlineStr">
@@ -7105,37 +7105,37 @@
       </c>
       <c r="J72" s="13" t="inlineStr">
         <is>
-          <t>Per sale / period</t>
+          <t>Per EOD count / weekly review</t>
         </is>
       </c>
       <c r="K72" s="12" t="inlineStr">
         <is>
-          <t>HQ Controller</t>
+          <t>F&amp;B Controller / Kitchen Mgr</t>
         </is>
       </c>
       <c r="L72" s="13" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>P10/P13</t>
         </is>
       </c>
       <c r="M72" s="12" t="inlineStr">
         <is>
-          <t>branches.service.ts (consolidated, branch tagging); branches.controller.ts; cust_pos_sales.branch_id; cutover/branch.ts (ToE)</t>
+          <t>menu/food-cost.service.ts foodCostVariance (per-item + by_reason + by_station roll-ups, anomaly bands); portal.service.ts createVariance (persists reason_code/station); portal.controller.ts VarianceBody (reason_code enum); schema/bom.ts cust_variance.reason_code/station + migration 0161; /food-cost variance tab (by-reason/by-station tables); cutover/restaurant.ts (ToE)</t>
         </is>
       </c>
       <c r="N72" s="12" t="inlineStr">
         <is>
-          <t>Inspect branch tagging completeness + the '(none)' surfacing + the GL tie.</t>
+          <t>Inspect the reason_code enum capture, the valued by_reason/by_station roll-ups, the anomaly bands, and tenant isolation.</t>
         </is>
       </c>
       <c r="O72" s="12" t="inlineStr">
         <is>
-          <t>Sample period: tagged sales group by branch, an untagged sale surfaces as '(none)', consolidated total ties to posted revenue.</t>
+          <t>Re-perform: seed counts with reason/station; the variance values per ingredient (NOODLE +฿30 High), nets +30/−50 to −20, by_reason PORTIONING +30 / WASTE −50, by_station Sauce +30 (20%); another tenant's counts are excluded (re-performed by the restaurant harness).</t>
         </is>
       </c>
       <c r="P72" s="12" t="inlineStr">
         <is>
-          <t>Consolidation report; '(none)' investigation log</t>
+          <t>Reason-coded variance roll-up + by-station test</t>
         </is>
       </c>
       <c r="Q72" s="18" t="inlineStr">
@@ -7147,7 +7147,7 @@
     <row r="73">
       <c r="A73" s="15" t="inlineStr">
         <is>
-          <t>BRANCH-02</t>
+          <t>BRANCH-01</t>
         </is>
       </c>
       <c r="B73" s="16" t="inlineStr">
@@ -7167,62 +7167,62 @@
       </c>
       <c r="E73" s="16" t="inlineStr">
         <is>
-          <t>An offline terminal sells at a stale or wrong price/promotion because the cached catalog drifted from the master.</t>
+          <t>A POS sale is not attributed to its originating branch, so the consolidated branch roll-up is incomplete and cannot be tied to GL revenue.</t>
         </is>
       </c>
       <c r="F73" s="16" t="inlineStr">
         <is>
-          <t>Accuracy</t>
+          <t>Completeness</t>
         </is>
       </c>
       <c r="G73" s="16" t="inlineStr">
         <is>
-          <t>Offline master-bundle export: GET /api/branches/master-bundle returns ONLY the active price-list + active promotions, time-stamped (generated_at). The offline terminal sells from this bundle, so it cannot ring a stale/withdrawn price or promo.</t>
+          <t>Branch sale-tagging + HQ consolidation: every POS sale carries cust_pos_sales.branch_id; GET /api/branches/consolidated aggregates per branch (excluding Voided) and surfaces untagged sales as branch '(none)' — a deliberate completeness flag the controller investigates and clears before tying the consolidated total to GL revenue.</t>
         </is>
       </c>
       <c r="H73" s="17" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I73" s="17" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="J73" s="17" t="inlineStr">
         <is>
-          <t>Per bundle push</t>
+          <t>Per sale / period</t>
         </is>
       </c>
       <c r="K73" s="16" t="inlineStr">
         <is>
-          <t>HQ Controller / Pricing</t>
+          <t>HQ Controller</t>
         </is>
       </c>
       <c r="L73" s="17" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="M73" s="16" t="inlineStr">
         <is>
-          <t>branches.service.ts masterBundle (active price-list + active promos + generated_at); branches.controller.ts; cutover/branch.ts (ToE)</t>
+          <t>branches.service.ts (consolidated, branch tagging); branches.controller.ts; cust_pos_sales.branch_id; cutover/branch.ts (ToE)</t>
         </is>
       </c>
       <c r="N73" s="16" t="inlineStr">
         <is>
-          <t>Inspect the bundle exports only active prices/promos with a timestamp.</t>
+          <t>Inspect branch tagging completeness + the '(none)' surfacing + the GL tie.</t>
         </is>
       </c>
       <c r="O73" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: export the bundle; confirm it carries only active price-list/promotions + generated_at.</t>
+          <t>Sample period: tagged sales group by branch, an untagged sale surfaces as '(none)', consolidated total ties to posted revenue.</t>
         </is>
       </c>
       <c r="P73" s="16" t="inlineStr">
         <is>
-          <t>Bundle metadata; bundle vs price-master diff</t>
+          <t>Consolidation report; '(none)' investigation log</t>
         </is>
       </c>
       <c r="Q73" s="18" t="inlineStr">
@@ -7234,7 +7234,7 @@
     <row r="74">
       <c r="A74" s="11" t="inlineStr">
         <is>
-          <t>BRANCH-03</t>
+          <t>BRANCH-02</t>
         </is>
       </c>
       <c r="B74" s="12" t="inlineStr">
@@ -7249,27 +7249,27 @@
       </c>
       <c r="D74" s="12" t="inlineStr">
         <is>
-          <t>Revenue; Cash</t>
+          <t>Revenue</t>
         </is>
       </c>
       <c r="E74" s="12" t="inlineStr">
         <is>
-          <t>An offline-captured sale is LOST or DUPLICATED when connectivity returns — revenue understated (lost) or double-counted (duplicated), and the GL double-posted.</t>
+          <t>An offline terminal sells at a stale or wrong price/promotion because the cached catalog drifted from the master.</t>
         </is>
       </c>
       <c r="F74" s="12" t="inlineStr">
         <is>
-          <t>Completeness/Accuracy</t>
+          <t>Accuracy</t>
         </is>
       </c>
       <c r="G74" s="12" t="inlineStr">
         <is>
-          <t>Offline-to-online exactly-once sync: offline-captured sales replay idempotently on (tenant, client_uuid) via the pos_offline_sync dedup ledger. Two paths share the ledger — the portal/inventory POS (POST /api/portal/pos/offline-sync, item_id lines) and the touch register (POST /api/restaurant/offline-sync, menu sku lines, re-running the restaurant order→checkout so the server re-prices + 86-checks). A re-sent batch returns 'duplicate' (no second sale/GL); a failed op is a RETRYABLE tombstone (sale_no NULL) that never blocks a later replay, so a transient error is not a lost sale; each op runs in its own savepoint so one bad sale never poisons the batch.</t>
+          <t>Offline master-bundle export: GET /api/branches/master-bundle returns ONLY the active price-list + active promotions, time-stamped (generated_at). The offline terminal sells from this bundle, so it cannot ring a stale/withdrawn price or promo.</t>
         </is>
       </c>
       <c r="H74" s="13" t="inlineStr">
         <is>
-          <t>Det/Prev</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I74" s="13" t="inlineStr">
@@ -7279,37 +7279,37 @@
       </c>
       <c r="J74" s="13" t="inlineStr">
         <is>
-          <t>Per sync</t>
+          <t>Per bundle push</t>
         </is>
       </c>
       <c r="K74" s="12" t="inlineStr">
         <is>
-          <t>HQ Controller / IT</t>
+          <t>HQ Controller / Pricing</t>
         </is>
       </c>
       <c r="L74" s="13" t="inlineStr">
         <is>
-          <t>P10/P16</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="M74" s="12" t="inlineStr">
         <is>
-          <t>portal/offline-sync.service.ts (item_id path); restaurant/offline-sync.service.ts (register sku path, reuses dineIn create+checkout); pos_offline_sync dedup ledger; web lib/offline-pos.ts + lib/register-offline.ts; cutover/offline-sync.ts + restaurant-offline.ts (ToE) + e2e/register-offline.spec.ts</t>
+          <t>branches.service.ts masterBundle (active price-list + active promos + generated_at); branches.controller.ts; cutover/branch.ts (ToE)</t>
         </is>
       </c>
       <c r="N74" s="12" t="inlineStr">
         <is>
-          <t>Inspect the (tenant, client_uuid) dedup gate (sale_no NOT NULL), the per-op savepoint isolation, and the retryable-failure tombstone.</t>
+          <t>Inspect the bundle exports only active prices/promos with a timestamp.</t>
         </is>
       </c>
       <c r="O74" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: sync a batch (all synced, distinct SALE-), replay it (all duplicate, no double sale/GL), a bad op fails while neighbours sync, same uuid twice in a batch posts once, a transient failure replays to synced after the cause clears (re-performed by the offline-sync + restaurant-offline harnesses).</t>
+          <t>Re-perform: export the bundle; confirm it carries only active price-list/promotions + generated_at.</t>
         </is>
       </c>
       <c r="P74" s="12" t="inlineStr">
         <is>
-          <t>Sync recon report; terminal vs ledger counts; idempotency tests</t>
+          <t>Bundle metadata; bundle vs price-master diff</t>
         </is>
       </c>
       <c r="Q74" s="18" t="inlineStr">
@@ -7321,12 +7321,12 @@
     <row r="75">
       <c r="A75" s="15" t="inlineStr">
         <is>
-          <t>MFG-01</t>
+          <t>BRANCH-03</t>
         </is>
       </c>
       <c r="B75" s="16" t="inlineStr">
         <is>
-          <t>Manufacturing &amp; Costing</t>
+          <t>Multi-Branch &amp; Offline POS</t>
         </is>
       </c>
       <c r="C75" s="17" t="inlineStr">
@@ -7336,67 +7336,67 @@
       </c>
       <c r="D75" s="16" t="inlineStr">
         <is>
-          <t>Inventory; COGS</t>
+          <t>Revenue; Cash</t>
         </is>
       </c>
       <c r="E75" s="16" t="inlineStr">
         <is>
-          <t>Unauthorized BOM/recipe change mis-states standard cost and every downstream WIP/COGS posting; or the role that maintains the recipe also transacts on it.</t>
+          <t>An offline-captured sale is LOST or DUPLICATED when connectivity returns — revenue understated (lost) or double-counted (duplicated), and the GL double-posted.</t>
         </is>
       </c>
       <c r="F75" s="16" t="inlineStr">
         <is>
-          <t>Authorization</t>
+          <t>Completeness/Accuracy</t>
         </is>
       </c>
       <c r="G75" s="16" t="inlineStr">
         <is>
-          <t>BOM master maker-checker / SoD: the master BOM library (bom_master) is maintained + distributed by HQ separately from transacting; a tenant BOM submission is reviewed and merged by HQ on approval (a maker-checker over master data). Recipe roll-up (line cost + labor + overhead → cost per unit) is the standard-cost basis. Master-data access is segregated from production (R13).</t>
+          <t>Offline-to-online exactly-once sync: offline-captured sales replay idempotently on (tenant, client_uuid) via the pos_offline_sync dedup ledger. Two paths share the ledger — the portal/inventory POS (POST /api/portal/pos/offline-sync, item_id lines) and the touch register (POST /api/restaurant/offline-sync, menu sku lines, re-running the restaurant order→checkout so the server re-prices + 86-checks). A re-sent batch returns 'duplicate' (no second sale/GL); a failed op is a RETRYABLE tombstone (sale_no NULL) that never blocks a later replay, so a transient error is not a lost sale; each op runs in its own savepoint so one bad sale never poisons the batch.</t>
         </is>
       </c>
       <c r="H75" s="17" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det/Prev</t>
         </is>
       </c>
       <c r="I75" s="17" t="inlineStr">
         <is>
-          <t>Manual+Auto</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J75" s="17" t="inlineStr">
         <is>
-          <t>Per BOM change</t>
+          <t>Per sync</t>
         </is>
       </c>
       <c r="K75" s="16" t="inlineStr">
         <is>
-          <t>HQ MasterSteward / CostAccountant</t>
+          <t>HQ Controller / IT</t>
         </is>
       </c>
       <c r="L75" s="17" t="inlineStr">
         <is>
-          <t>P13</t>
+          <t>P10/P16</t>
         </is>
       </c>
       <c r="M75" s="16" t="inlineStr">
         <is>
-          <t>bom master + submissions (/api/bom/master, /api/bom/submissions, /api/portal/bom); manufacturing.service.ts BOM scaling; cutover/cpq.ts + manufacturing.ts (ToE)</t>
+          <t>portal/offline-sync.service.ts (item_id path); restaurant/offline-sync.service.ts (register sku path, reuses dineIn create+checkout); pos_offline_sync dedup ledger; web lib/offline-pos.ts + lib/register-offline.ts; cutover/offline-sync.ts + restaurant-offline.ts (ToE) + e2e/register-offline.spec.ts</t>
         </is>
       </c>
       <c r="N75" s="16" t="inlineStr">
         <is>
-          <t>Inspect BOM maintenance access + the submission→approve maker-checker + the costing roll-up.</t>
+          <t>Inspect the (tenant, client_uuid) dedup gate (sale_no NOT NULL), the per-op savepoint isolation, and the retryable-failure tombstone.</t>
         </is>
       </c>
       <c r="O75" s="16" t="inlineStr">
         <is>
-          <t>Sample BOM change is HQ-approved before use; standard cost rolls up correctly.</t>
+          <t>Re-perform: sync a batch (all synced, distinct SALE-), replay it (all duplicate, no double sale/GL), a bad op fails while neighbours sync, same uuid twice in a batch posts once, a transient failure replays to synced after the cause clears (re-performed by the offline-sync + restaurant-offline harnesses).</t>
         </is>
       </c>
       <c r="P75" s="16" t="inlineStr">
         <is>
-          <t>BOM approval log; costing roll-up</t>
+          <t>Sync recon report; terminal vs ledger counts; idempotency tests</t>
         </is>
       </c>
       <c r="Q75" s="18" t="inlineStr">
@@ -7408,7 +7408,7 @@
     <row r="76">
       <c r="A76" s="11" t="inlineStr">
         <is>
-          <t>MFG-02</t>
+          <t>MFG-01</t>
         </is>
       </c>
       <c r="B76" s="12" t="inlineStr">
@@ -7423,22 +7423,22 @@
       </c>
       <c r="D76" s="12" t="inlineStr">
         <is>
-          <t>WIP; Finished Goods; COGS</t>
+          <t>Inventory; COGS</t>
         </is>
       </c>
       <c r="E76" s="12" t="inlineStr">
         <is>
-          <t>Production cost is mis-stated: WIP not relieved, the conversion absorption left stranded, or a yield loss (spoilage/waste) silently capitalised into finished-goods inventory instead of expensed.</t>
+          <t>Unauthorized BOM/recipe change mis-states standard cost and every downstream WIP/COGS posting; or the role that maintains the recipe also transacts on it.</t>
         </is>
       </c>
       <c r="F76" s="12" t="inlineStr">
         <is>
-          <t>Valuation/Completeness/Accuracy</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="G76" s="12" t="inlineStr">
         <is>
-          <t>Production work-order WIP costing with a balanced JE at each step: ISSUE posts Dr 1250 WIP / Cr 1200 raw materials / Cr 2380 manufacturing-costs-applied (idempotent — re-issue is a no-op); COMPLETE posts Dr 1210 Finished Goods at the standard cost of the ACTUAL quantity produced + books the YIELD VARIANCE to 5810 (produced &lt; planned → debit 5810 loss; over-yield → credit) / Cr 1250 WIP — so WIP is always fully relieved and FG is never over-valued on a short yield. State machine Open→Released→Completed (out-of-order → BAD_STATUS). The 2380/1250 clearing balances tie out at close. Scrap/rework write-off of defective output posts to 5810 with CostAccountant authorization.</t>
+          <t>BOM master maker-checker / SoD: the master BOM library (bom_master) is maintained + distributed by HQ separately from transacting; a tenant BOM submission is reviewed and merged by HQ on approval (a maker-checker over master data). Recipe roll-up (line cost + labor + overhead → cost per unit) is the standard-cost basis. Master-data access is segregated from production (R13).</t>
         </is>
       </c>
       <c r="H76" s="13" t="inlineStr">
@@ -7448,17 +7448,17 @@
       </c>
       <c r="I76" s="13" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Manual+Auto</t>
         </is>
       </c>
       <c r="J76" s="13" t="inlineStr">
         <is>
-          <t>Per work order</t>
+          <t>Per BOM change</t>
         </is>
       </c>
       <c r="K76" s="12" t="inlineStr">
         <is>
-          <t>Warehouse / CostAccountant</t>
+          <t>HQ MasterSteward / CostAccountant</t>
         </is>
       </c>
       <c r="L76" s="13" t="inlineStr">
@@ -7468,22 +7468,22 @@
       </c>
       <c r="M76" s="12" t="inlineStr">
         <is>
-          <t>manufacturing.service.ts issue/complete (yield variance to 5810; fmt exposes yield_variance); manufacturing.controller.ts (bom_master/warehouse/exec); schema/manufacturing.ts work_orders; cutover/manufacturing.ts (ToE)</t>
+          <t>bom master + submissions (/api/bom/master, /api/bom/submissions, /api/portal/bom); manufacturing.service.ts BOM scaling; cutover/cpq.ts + manufacturing.ts (ToE)</t>
         </is>
       </c>
       <c r="N76" s="12" t="inlineStr">
         <is>
-          <t>Inspect the issue/complete JEs + the standard-unit-cost FG valuation + the yield-variance plug + the status guard.</t>
+          <t>Inspect BOM maintenance access + the submission→approve maker-checker + the costing roll-up.</t>
         </is>
       </c>
       <c r="O76" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: issue (WIP charged), complete at full yield (FG = full cost, no variance) and at a short yield (FG = std×produced, the lost yield to 5810, WIP nets to 0, TB balanced) — re-performed by the harness.</t>
+          <t>Sample BOM change is HQ-approved before use; standard cost rolls up correctly.</t>
         </is>
       </c>
       <c r="P76" s="12" t="inlineStr">
         <is>
-          <t>WO costing register (yield_variance per WO); production JEs</t>
+          <t>BOM approval log; costing roll-up</t>
         </is>
       </c>
       <c r="Q76" s="18" t="inlineStr">
@@ -7495,7 +7495,7 @@
     <row r="77">
       <c r="A77" s="15" t="inlineStr">
         <is>
-          <t>MFG-03</t>
+          <t>MFG-02</t>
         </is>
       </c>
       <c r="B77" s="16" t="inlineStr">
@@ -7510,27 +7510,27 @@
       </c>
       <c r="D77" s="16" t="inlineStr">
         <is>
-          <t>Inventory; COGS</t>
+          <t>WIP; Finished Goods; COGS</t>
         </is>
       </c>
       <c r="E77" s="16" t="inlineStr">
         <is>
-          <t>Standard-cost inventory received without isolating the price variance — actual purchase cost buried in inventory, COGS and PPV mis-stated.</t>
+          <t>Production cost is mis-stated: WIP not relieved, the conversion absorption left stranded, or a yield loss (spoilage/waste) silently capitalised into finished-goods inventory instead of expensed.</t>
         </is>
       </c>
       <c r="F77" s="16" t="inlineStr">
         <is>
-          <t>Valuation/Accuracy</t>
+          <t>Valuation/Completeness/Accuracy</t>
         </is>
       </c>
       <c r="G77" s="16" t="inlineStr">
         <is>
-          <t>Goods-receipt capitalisation under the configured costing method (FIFO/AVG/STD per tenant+item): FIFO/AVG → Dr 1200 / Cr 2000 at actual; STD → Dr 1200 at standard, the purchase-price variance booked to 5500 (unfavourable Dr / favourable Cr), Cr 2000 at actual — the PPV (5500) leg is the single balancing plug (= actual − standard, rounded once) so the JE can never reject UNBALANCED on independent per-leg rounding.</t>
+          <t>Production work-order WIP costing with a balanced JE at each step: ISSUE posts Dr 1250 WIP / Cr 1200 raw materials / Cr 2380 manufacturing-costs-applied (idempotent — re-issue is a no-op); COMPLETE posts Dr 1210 Finished Goods at the standard cost of the ACTUAL quantity produced + books the YIELD VARIANCE to 5810 (produced &lt; planned → debit 5810 loss; over-yield → credit) / Cr 1250 WIP — so WIP is always fully relieved and FG is never over-valued on a short yield. State machine Open→Released→Completed (out-of-order → BAD_STATUS). The 2380/1250 clearing balances tie out at close. Scrap/rework write-off of defective output posts to 5810 with CostAccountant authorization.</t>
         </is>
       </c>
       <c r="H77" s="17" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I77" s="17" t="inlineStr">
@@ -7540,12 +7540,12 @@
       </c>
       <c r="J77" s="17" t="inlineStr">
         <is>
-          <t>Per receipt</t>
+          <t>Per work order</t>
         </is>
       </c>
       <c r="K77" s="16" t="inlineStr">
         <is>
-          <t>CostAccountant</t>
+          <t>Warehouse / CostAccountant</t>
         </is>
       </c>
       <c r="L77" s="17" t="inlineStr">
@@ -7555,22 +7555,22 @@
       </c>
       <c r="M77" s="16" t="inlineStr">
         <is>
-          <t>costing.service.ts (config/valuation, GRV capitalisation + 5500 PPV); costing.controller.ts (masterdata); cutover/costing.ts (ToE)</t>
+          <t>manufacturing.service.ts issue/complete (yield variance to 5810; fmt exposes yield_variance); manufacturing.controller.ts (bom_master/warehouse/exec); schema/manufacturing.ts work_orders; cutover/manufacturing.ts (ToE)</t>
         </is>
       </c>
       <c r="N77" s="16" t="inlineStr">
         <is>
-          <t>Inspect the per-method capitalisation routing + the PPV plug.</t>
+          <t>Inspect the issue/complete JEs + the standard-unit-cost FG valuation + the yield-variance plug + the status guard.</t>
         </is>
       </c>
       <c r="O77" s="16" t="inlineStr">
         <is>
-          <t>Re-perform a STD receipt at actual ≠ standard → PPV isolated to 5500, JE balanced; valuation ties to GL 1200/1210/1250.</t>
+          <t>Re-perform: issue (WIP charged), complete at full yield (FG = full cost, no variance) and at a short yield (FG = std×produced, the lost yield to 5810, WIP nets to 0, TB balanced) — re-performed by the harness.</t>
         </is>
       </c>
       <c r="P77" s="16" t="inlineStr">
         <is>
-          <t>PPV postings; costing valuation</t>
+          <t>WO costing register (yield_variance per WO); production JEs</t>
         </is>
       </c>
       <c r="Q77" s="18" t="inlineStr">
@@ -7582,12 +7582,12 @@
     <row r="78">
       <c r="A78" s="11" t="inlineStr">
         <is>
-          <t>PROJ-01</t>
+          <t>MFG-03</t>
         </is>
       </c>
       <c r="B78" s="12" t="inlineStr">
         <is>
-          <t>Project Accounting</t>
+          <t>Manufacturing &amp; Costing</t>
         </is>
       </c>
       <c r="C78" s="13" t="inlineStr">
@@ -7597,27 +7597,27 @@
       </c>
       <c r="D78" s="12" t="inlineStr">
         <is>
-          <t>Project WIP; COGS</t>
+          <t>Inventory; COGS</t>
         </is>
       </c>
       <c r="E78" s="12" t="inlineStr">
         <is>
-          <t>Project cost mis-stated: a recoverable cost not captured, or an UN-recoverable (non-billable) cost capitalised into project WIP as an asset that overstates the unbilled balance and inflates margin.</t>
+          <t>Standard-cost inventory received without isolating the price variance — actual purchase cost buried in inventory, COGS and PPV mis-stated.</t>
         </is>
       </c>
       <c r="F78" s="12" t="inlineStr">
         <is>
-          <t>Valuation/Accuracy/Completeness</t>
+          <t>Valuation/Accuracy</t>
         </is>
       </c>
       <c r="G78" s="12" t="inlineStr">
         <is>
-          <t>Project cost capture with a balanced JE and a billable/non-billable split: a BILLABLE time/expense cost is a recoverable asset → Dr 1260 Project WIP / Cr 2390 Project Costs Applied (accumulates in cost_to_date, relieved to COGS at billing); a NON-BILLABLE cost is unrecoverable → EXPENSED immediately Dr 5800 Project Cost of Services / Cr 2390 (never enters the billable WIP), so the register's total_cost and true margin (billed − recognised − non-billable) reflect the absorbed cost. A non-positive amount → BAD_AMOUNT; first cost flips Open→Active.</t>
+          <t>Goods-receipt capitalisation under the configured costing method (FIFO/AVG/STD per tenant+item): FIFO/AVG → Dr 1200 / Cr 2000 at actual; STD → Dr 1200 at standard, the purchase-price variance booked to 5500 (unfavourable Dr / favourable Cr), Cr 2000 at actual — the PPV (5500) leg is the single balancing plug (= actual − standard, rounded once) so the JE can never reject UNBALANCED on independent per-leg rounding.</t>
         </is>
       </c>
       <c r="H78" s="13" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I78" s="13" t="inlineStr">
@@ -7627,12 +7627,12 @@
       </c>
       <c r="J78" s="13" t="inlineStr">
         <is>
-          <t>Per cost entry</t>
+          <t>Per receipt</t>
         </is>
       </c>
       <c r="K78" s="12" t="inlineStr">
         <is>
-          <t>ProjectAccountant</t>
+          <t>CostAccountant</t>
         </is>
       </c>
       <c r="L78" s="13" t="inlineStr">
@@ -7642,22 +7642,22 @@
       </c>
       <c r="M78" s="12" t="inlineStr">
         <is>
-          <t>projects.service.ts logCost (billable→1260, non-billable→5800; fmt exposes non_billable_cost/total_cost/margin); projects.controller.ts; schema/projects.ts project_entries.billable; cutover/projects.ts (ToE)</t>
+          <t>costing.service.ts (config/valuation, GRV capitalisation + 5500 PPV); costing.controller.ts (masterdata); cutover/costing.ts (ToE)</t>
         </is>
       </c>
       <c r="N78" s="12" t="inlineStr">
         <is>
-          <t>Inspect the billable/non-billable GL routing + the WIP vs immediate-expense decision + the margin roll-up.</t>
+          <t>Inspect the per-method capitalisation routing + the PPV plug.</t>
         </is>
       </c>
       <c r="O78" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: a billable cost capitalises to 1260; a non-billable cost expenses to 5800 (NOT WIP), cost_to_date unchanged, and the project margin absorbs it (re-performed by the harness).</t>
+          <t>Re-perform a STD receipt at actual ≠ standard → PPV isolated to 5500, JE balanced; valuation ties to GL 1200/1210/1250.</t>
         </is>
       </c>
       <c r="P78" s="12" t="inlineStr">
         <is>
-          <t>Project cost JEs; cost register (non_billable_cost)</t>
+          <t>PPV postings; costing valuation</t>
         </is>
       </c>
       <c r="Q78" s="18" t="inlineStr">
@@ -7669,7 +7669,7 @@
     <row r="79">
       <c r="A79" s="15" t="inlineStr">
         <is>
-          <t>PROJ-02</t>
+          <t>PROJ-01</t>
         </is>
       </c>
       <c r="B79" s="16" t="inlineStr">
@@ -7684,22 +7684,22 @@
       </c>
       <c r="D79" s="16" t="inlineStr">
         <is>
-          <t>Project WIP; Revenue; COGS</t>
+          <t>Project WIP; COGS</t>
         </is>
       </c>
       <c r="E79" s="16" t="inlineStr">
         <is>
-          <t>Revenue billed without matching cost — WIP not relieved, cost of services mis-stated, margin overstated.</t>
+          <t>Project cost mis-stated: a recoverable cost not captured, or an UN-recoverable (non-billable) cost capitalised into project WIP as an asset that overstates the unbilled balance and inflates margin.</t>
         </is>
       </c>
       <c r="F79" s="16" t="inlineStr">
         <is>
-          <t>Accuracy/Cut-off</t>
+          <t>Valuation/Accuracy/Completeness</t>
         </is>
       </c>
       <c r="G79" s="16" t="inlineStr">
         <is>
-          <t>Customer billing recognises revenue (Dr 1100 AR / Cr 4200 Project Revenue) and relieves the unbilled WIP to cost of services up to the unrecognised billable cost (Dr 5800 / Cr 1260) in the same event — matching cost to recognised revenue. Billing is by raw amount (T&amp;M) or by PERCENT of the contract for Fixed-price milestone billing; a Fixed-price contract is CAPPED at the contract value (cumulative billing can never exceed it — BILL_EXCEEDS_CONTRACT), so the customer is never over-billed (billed_pct/remaining_to_bill on the register). Billing is idempotent on (project, cumulative billed amount).</t>
+          <t>Project cost capture with a balanced JE and a billable/non-billable split: a BILLABLE time/expense cost is a recoverable asset → Dr 1260 Project WIP / Cr 2390 Project Costs Applied (accumulates in cost_to_date, relieved to COGS at billing); a NON-BILLABLE cost is unrecoverable → EXPENSED immediately Dr 5800 Project Cost of Services / Cr 2390 (never enters the billable WIP), so the register's total_cost and true margin (billed − recognised − non-billable) reflect the absorbed cost. A non-positive amount → BAD_AMOUNT; first cost flips Open→Active.</t>
         </is>
       </c>
       <c r="H79" s="17" t="inlineStr">
@@ -7714,12 +7714,12 @@
       </c>
       <c r="J79" s="17" t="inlineStr">
         <is>
-          <t>Per billing</t>
+          <t>Per cost entry</t>
         </is>
       </c>
       <c r="K79" s="16" t="inlineStr">
         <is>
-          <t>ProjectController / ArSpecialist</t>
+          <t>ProjectAccountant</t>
         </is>
       </c>
       <c r="L79" s="17" t="inlineStr">
@@ -7729,22 +7729,22 @@
       </c>
       <c r="M79" s="16" t="inlineStr">
         <is>
-          <t>projects.service.ts bill (revenue + WIP relief, idempotent); projects.controller.ts (R07 vs cost initiation); cutover/projects.ts (ToE)</t>
+          <t>projects.service.ts logCost (billable→1260, non-billable→5800; fmt exposes non_billable_cost/total_cost/margin); projects.controller.ts; schema/projects.ts project_entries.billable; cutover/projects.ts (ToE)</t>
         </is>
       </c>
       <c r="N79" s="16" t="inlineStr">
         <is>
-          <t>Inspect the bill JE + the WIP-relief matching + idempotency.</t>
+          <t>Inspect the billable/non-billable GL routing + the WIP vs immediate-expense decision + the margin roll-up.</t>
         </is>
       </c>
       <c r="O79" s="16" t="inlineStr">
         <is>
-          <t>Re-perform a billing → revenue recognised, WIP relieved to 5800 up to unrecognised cost, 1260 reduced; margin = billed − recognised cost (re-performed by the harness).</t>
+          <t>Re-perform: a billable cost capitalises to 1260; a non-billable cost expenses to 5800 (NOT WIP), cost_to_date unchanged, and the project margin absorbs it (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P79" s="16" t="inlineStr">
         <is>
-          <t>Billing JEs; margin/WIP measurement</t>
+          <t>Project cost JEs; cost register (non_billable_cost)</t>
         </is>
       </c>
       <c r="Q79" s="18" t="inlineStr">
@@ -7756,7 +7756,7 @@
     <row r="80">
       <c r="A80" s="11" t="inlineStr">
         <is>
-          <t>PROJ-03</t>
+          <t>PROJ-02</t>
         </is>
       </c>
       <c r="B80" s="12" t="inlineStr">
@@ -7766,171 +7766,171 @@
       </c>
       <c r="C80" s="13" t="inlineStr">
         <is>
-          <t>Detective</t>
+          <t>Application</t>
         </is>
       </c>
       <c r="D80" s="12" t="inlineStr">
         <is>
-          <t>Project WIP</t>
+          <t>Project WIP; Revenue; COGS</t>
         </is>
       </c>
       <c r="E80" s="12" t="inlineStr">
         <is>
-          <t>Unbilled WIP (1260) and the 2390 clearing balance not reviewed at close — stale or unrecoverable WIP carried into the financial statements.</t>
+          <t>Revenue billed without matching cost — WIP not relieved, cost of services mis-stated, margin overstated.</t>
         </is>
       </c>
       <c r="F80" s="12" t="inlineStr">
         <is>
-          <t>Valuation</t>
+          <t>Accuracy/Cut-off</t>
         </is>
       </c>
       <c r="G80" s="12" t="inlineStr">
         <is>
-          <t>Period-end review of unbilled-WIP (1260) aging and the project-costs-applied (2390) clearing tie-out; project margin (billed_to_date − recognised_cost − non-billable) reviewed at close. SoD: billing authorisation is segregated from cost initiation (R07).</t>
+          <t>Customer billing recognises revenue (Dr 1100 AR / Cr 4200 Project Revenue) and relieves the unbilled WIP to cost of services up to the unrecognised billable cost (Dr 5800 / Cr 1260) in the same event — matching cost to recognised revenue. Billing is by raw amount (T&amp;M) or by PERCENT of the contract for Fixed-price milestone billing; a Fixed-price contract is CAPPED at the contract value (cumulative billing can never exceed it — BILL_EXCEEDS_CONTRACT), so the customer is never over-billed (billed_pct/remaining_to_bill on the register). Billing is idempotent on (project, cumulative billed amount).</t>
         </is>
       </c>
       <c r="H80" s="13" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I80" s="13" t="inlineStr">
         <is>
-          <t>Hybrid</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J80" s="13" t="inlineStr">
         <is>
-          <t>Period</t>
+          <t>Per billing</t>
         </is>
       </c>
       <c r="K80" s="12" t="inlineStr">
         <is>
-          <t>ProjectAccountant / Controller</t>
+          <t>ProjectController / ArSpecialist</t>
         </is>
       </c>
       <c r="L80" s="13" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>P13</t>
         </is>
       </c>
       <c r="M80" s="12" t="inlineStr">
         <is>
-          <t>projects.service.ts fmt (wip/margin); the project register + entries; close review</t>
+          <t>projects.service.ts bill (revenue + WIP relief, idempotent); projects.controller.ts (R07 vs cost initiation); cutover/projects.ts (ToE)</t>
         </is>
       </c>
       <c r="N80" s="12" t="inlineStr">
         <is>
-          <t>Inspect 1260 aging + 2390 clearing + margin review evidence.</t>
+          <t>Inspect the bill JE + the WIP-relief matching + idempotency.</t>
         </is>
       </c>
       <c r="O80" s="12" t="inlineStr">
         <is>
-          <t>Sample projects: 1260 WIP agrees to cost_to_date − recognised; 2390 clears; stale WIP investigated.</t>
+          <t>Re-perform a billing → revenue recognised, WIP relieved to 5800 up to unrecognised cost, 1260 reduced; margin = billed − recognised cost (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P80" s="12" t="inlineStr">
         <is>
-          <t>WIP aging; 2390 clearing tie-out</t>
-        </is>
-      </c>
-      <c r="Q80" s="19" t="inlineStr">
-        <is>
-          <t>Partial</t>
+          <t>Billing JEs; margin/WIP measurement</t>
+        </is>
+      </c>
+      <c r="Q80" s="18" t="inlineStr">
+        <is>
+          <t>Implemented</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="15" t="inlineStr">
         <is>
-          <t>GL-01</t>
+          <t>PROJ-03</t>
         </is>
       </c>
       <c r="B81" s="16" t="inlineStr">
         <is>
-          <t>General Ledger</t>
+          <t>Project Accounting</t>
         </is>
       </c>
       <c r="C81" s="17" t="inlineStr">
         <is>
-          <t>Application</t>
+          <t>Detective</t>
         </is>
       </c>
       <c r="D81" s="16" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Project WIP</t>
         </is>
       </c>
       <c r="E81" s="16" t="inlineStr">
         <is>
-          <t>Unbalanced / one-sided journal entries.</t>
+          <t>Unbilled WIP (1260) and the 2390 clearing balance not reviewed at close — stale or unrecoverable WIP carried into the financial statements.</t>
         </is>
       </c>
       <c r="F81" s="16" t="inlineStr">
         <is>
-          <t>Accuracy</t>
+          <t>Valuation</t>
         </is>
       </c>
       <c r="G81" s="16" t="inlineStr">
         <is>
-          <t>Double-entry balanced-by-construction — Σdebit=Σcredit enforced; each line single-sided &amp; non-negative.</t>
+          <t>Period-end review of unbilled-WIP (1260) aging and the project-costs-applied (2390) clearing tie-out; project margin (billed_to_date − recognised_cost − non-billable) reviewed at close. SoD: billing authorisation is segregated from cost initiation (R07).</t>
         </is>
       </c>
       <c r="H81" s="17" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I81" s="17" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Hybrid</t>
         </is>
       </c>
       <c r="J81" s="17" t="inlineStr">
         <is>
-          <t>Per JE</t>
+          <t>Period</t>
         </is>
       </c>
       <c r="K81" s="16" t="inlineStr">
         <is>
-          <t>Controller</t>
+          <t>ProjectAccountant / Controller</t>
         </is>
       </c>
       <c r="L81" s="17" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="M81" s="16" t="inlineStr">
         <is>
-          <t>ledger.service.ts (postEntry — UNBALANCED / INVALID_LINE)</t>
+          <t>projects.service.ts fmt (wip/margin); the project register + entries; close review</t>
         </is>
       </c>
       <c r="N81" s="16" t="inlineStr">
         <is>
-          <t>Inspect balance + line invariants.</t>
+          <t>Inspect 1260 aging + 2390 clearing + margin review evidence.</t>
         </is>
       </c>
       <c r="O81" s="16" t="inlineStr">
         <is>
-          <t>Attempt unbalanced JE → rejected.</t>
+          <t>Sample projects: 1260 WIP agrees to cost_to_date − recognised; 2390 clears; stale WIP investigated.</t>
         </is>
       </c>
       <c r="P81" s="16" t="inlineStr">
         <is>
-          <t>Invariant test</t>
-        </is>
-      </c>
-      <c r="Q81" s="18" t="inlineStr">
-        <is>
-          <t>Implemented</t>
+          <t>WIP aging; 2390 clearing tie-out</t>
+        </is>
+      </c>
+      <c r="Q81" s="19" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="11" t="inlineStr">
         <is>
-          <t>GL-02</t>
+          <t>GL-01</t>
         </is>
       </c>
       <c r="B82" s="12" t="inlineStr">
@@ -7950,17 +7950,17 @@
       </c>
       <c r="E82" s="12" t="inlineStr">
         <is>
-          <t>Postings to a closed period distort reported results.</t>
+          <t>Unbalanced / one-sided journal entries.</t>
         </is>
       </c>
       <c r="F82" s="12" t="inlineStr">
         <is>
-          <t>Cutoff</t>
+          <t>Accuracy</t>
         </is>
       </c>
       <c r="G82" s="12" t="inlineStr">
         <is>
-          <t>Period-close lockout — postings to a CLOSED fiscal period are rejected (per-tenant calendar).</t>
+          <t>Double-entry balanced-by-construction — Σdebit=Σcredit enforced; each line single-sided &amp; non-negative.</t>
         </is>
       </c>
       <c r="H82" s="13" t="inlineStr">
@@ -7990,22 +7990,22 @@
       </c>
       <c r="M82" s="12" t="inlineStr">
         <is>
-          <t>ledger.service.ts (postEntry PERIOD_CLOSED); fiscal_periods</t>
+          <t>ledger.service.ts (postEntry — UNBALANCED / INVALID_LINE)</t>
         </is>
       </c>
       <c r="N82" s="12" t="inlineStr">
         <is>
-          <t>Inspect close check.</t>
+          <t>Inspect balance + line invariants.</t>
         </is>
       </c>
       <c r="O82" s="12" t="inlineStr">
         <is>
-          <t>Post to closed period → rejected; review exceptions.</t>
+          <t>Attempt unbalanced JE → rejected.</t>
         </is>
       </c>
       <c r="P82" s="12" t="inlineStr">
         <is>
-          <t>Close-lock test</t>
+          <t>Invariant test</t>
         </is>
       </c>
       <c r="Q82" s="18" t="inlineStr">
@@ -8017,7 +8017,7 @@
     <row r="83">
       <c r="A83" s="15" t="inlineStr">
         <is>
-          <t>GL-03</t>
+          <t>GL-02</t>
         </is>
       </c>
       <c r="B83" s="16" t="inlineStr">
@@ -8032,22 +8032,22 @@
       </c>
       <c r="D83" s="16" t="inlineStr">
         <is>
-          <t>Equity</t>
+          <t>All</t>
         </is>
       </c>
       <c r="E83" s="16" t="inlineStr">
         <is>
-          <t>Unauthorized year-end close / RE roll.</t>
+          <t>Postings to a closed period distort reported results.</t>
         </is>
       </c>
       <c r="F83" s="16" t="inlineStr">
         <is>
-          <t>Cutoff/Authorization</t>
+          <t>Cutoff</t>
         </is>
       </c>
       <c r="G83" s="16" t="inlineStr">
         <is>
-          <t>Year-end close restricted to 'exec'; closing entries roll to retained earnings.</t>
+          <t>Period-close lockout — postings to a CLOSED fiscal period are rejected (per-tenant calendar).</t>
         </is>
       </c>
       <c r="H83" s="17" t="inlineStr">
@@ -8057,42 +8057,42 @@
       </c>
       <c r="I83" s="17" t="inlineStr">
         <is>
-          <t>Auto+Manual</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J83" s="17" t="inlineStr">
         <is>
-          <t>Annual</t>
+          <t>Per JE</t>
         </is>
       </c>
       <c r="K83" s="16" t="inlineStr">
         <is>
-          <t>CFO / Controller</t>
+          <t>Controller</t>
         </is>
       </c>
       <c r="L83" s="17" t="inlineStr">
         <is>
-          <t>P10/P11</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="M83" s="16" t="inlineStr">
         <is>
-          <t>ledger.controller.ts (close-year @Permissions exec); closeYear</t>
+          <t>ledger.service.ts (postEntry PERIOD_CLOSED); fiscal_periods</t>
         </is>
       </c>
       <c r="N83" s="16" t="inlineStr">
         <is>
-          <t>Inspect permission + closing logic.</t>
+          <t>Inspect close check.</t>
         </is>
       </c>
       <c r="O83" s="16" t="inlineStr">
         <is>
-          <t>Attempt close w/o exec → 403; review annual close.</t>
+          <t>Post to closed period → rejected; review exceptions.</t>
         </is>
       </c>
       <c r="P83" s="16" t="inlineStr">
         <is>
-          <t>Close package</t>
+          <t>Close-lock test</t>
         </is>
       </c>
       <c r="Q83" s="18" t="inlineStr">
@@ -8104,7 +8104,7 @@
     <row r="84">
       <c r="A84" s="11" t="inlineStr">
         <is>
-          <t>GL-04</t>
+          <t>GL-03</t>
         </is>
       </c>
       <c r="B84" s="12" t="inlineStr">
@@ -8119,22 +8119,22 @@
       </c>
       <c r="D84" s="12" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Equity</t>
         </is>
       </c>
       <c r="E84" s="12" t="inlineStr">
         <is>
-          <t>Concurrent posting double-books the same source doc.</t>
+          <t>Unauthorized year-end close / RE roll.</t>
         </is>
       </c>
       <c r="F84" s="12" t="inlineStr">
         <is>
-          <t>Completeness/Accuracy</t>
+          <t>Cutoff/Authorization</t>
         </is>
       </c>
       <c r="G84" s="12" t="inlineStr">
         <is>
-          <t>Ledger idempotency — UNIQUE (tenant,source,source_ref,ledger) + ON CONFLICT DO NOTHING in postEntry.</t>
+          <t>Year-end close restricted to 'exec'; closing entries roll to retained earnings.</t>
         </is>
       </c>
       <c r="H84" s="13" t="inlineStr">
@@ -8144,42 +8144,42 @@
       </c>
       <c r="I84" s="13" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="J84" s="13" t="inlineStr">
         <is>
-          <t>Per JE</t>
+          <t>Annual</t>
         </is>
       </c>
       <c r="K84" s="12" t="inlineStr">
         <is>
-          <t>Eng Lead / Controller</t>
+          <t>CFO / Controller</t>
         </is>
       </c>
       <c r="L84" s="13" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P10/P11</t>
         </is>
       </c>
       <c r="M84" s="12" t="inlineStr">
         <is>
-          <t>schema/ledger.ts (ux_je_idem); ledger.service.ts; migration 0058</t>
+          <t>ledger.controller.ts (close-year @Permissions exec); closeYear</t>
         </is>
       </c>
       <c r="N84" s="12" t="inlineStr">
         <is>
-          <t>Inspect unique index + conflict handling.</t>
+          <t>Inspect permission + closing logic.</t>
         </is>
       </c>
       <c r="O84" s="12" t="inlineStr">
         <is>
-          <t>Concurrent identical post → single entry.</t>
+          <t>Attempt close w/o exec → 403; review annual close.</t>
         </is>
       </c>
       <c r="P84" s="12" t="inlineStr">
         <is>
-          <t>Dedup test</t>
+          <t>Close package</t>
         </is>
       </c>
       <c r="Q84" s="18" t="inlineStr">
@@ -8191,7 +8191,7 @@
     <row r="85">
       <c r="A85" s="15" t="inlineStr">
         <is>
-          <t>GL-05</t>
+          <t>GL-04</t>
         </is>
       </c>
       <c r="B85" s="16" t="inlineStr">
@@ -8211,17 +8211,17 @@
       </c>
       <c r="E85" s="16" t="inlineStr">
         <is>
-          <t>Manual JE posted without independent review (override risk).</t>
+          <t>Concurrent posting double-books the same source doc.</t>
         </is>
       </c>
       <c r="F85" s="16" t="inlineStr">
         <is>
-          <t>Authorization</t>
+          <t>Completeness/Accuracy</t>
         </is>
       </c>
       <c r="G85" s="16" t="inlineStr">
         <is>
-          <t>Manual journal-entry maker-checker — preparer ≠ approver before a manual JE posts.</t>
+          <t>Ledger idempotency — UNIQUE (tenant,source,source_ref,ledger) + ON CONFLICT DO NOTHING in postEntry.</t>
         </is>
       </c>
       <c r="H85" s="17" t="inlineStr">
@@ -8231,17 +8231,17 @@
       </c>
       <c r="I85" s="17" t="inlineStr">
         <is>
-          <t>Auto+Manual</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J85" s="17" t="inlineStr">
         <is>
-          <t>Per manual JE</t>
+          <t>Per JE</t>
         </is>
       </c>
       <c r="K85" s="16" t="inlineStr">
         <is>
-          <t>Controller</t>
+          <t>Eng Lead / Controller</t>
         </is>
       </c>
       <c r="L85" s="17" t="inlineStr">
@@ -8251,22 +8251,22 @@
       </c>
       <c r="M85" s="16" t="inlineStr">
         <is>
-          <t>ledger.service.ts (postEntry pendingApproval→Draft; approveEntry preparer≠approver; rejectEntry); ledger.controller.ts (gl_post posts / gl_close approves); cutover/compliance.ts (ToE)</t>
+          <t>schema/ledger.ts (ux_je_idem); ledger.service.ts; migration 0058</t>
         </is>
       </c>
       <c r="N85" s="16" t="inlineStr">
         <is>
-          <t>Inspect JE approval routing.</t>
+          <t>Inspect unique index + conflict handling.</t>
         </is>
       </c>
       <c r="O85" s="16" t="inlineStr">
         <is>
-          <t>Sample manual JEs: approver ≠ preparer; Draft excluded from balances until approved (re-performed by the harness).</t>
+          <t>Concurrent identical post → single entry.</t>
         </is>
       </c>
       <c r="P85" s="16" t="inlineStr">
         <is>
-          <t>JE approvals</t>
+          <t>Dedup test</t>
         </is>
       </c>
       <c r="Q85" s="18" t="inlineStr">
@@ -8278,7 +8278,7 @@
     <row r="86">
       <c r="A86" s="11" t="inlineStr">
         <is>
-          <t>GL-06</t>
+          <t>GL-05</t>
         </is>
       </c>
       <c r="B86" s="12" t="inlineStr">
@@ -8298,17 +8298,17 @@
       </c>
       <c r="E86" s="12" t="inlineStr">
         <is>
-          <t>Operator mis-posts to another tenant's books.</t>
+          <t>Manual JE posted without independent review (override risk).</t>
         </is>
       </c>
       <c r="F86" s="12" t="inlineStr">
         <is>
-          <t>Validity</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="G86" s="12" t="inlineStr">
         <is>
-          <t>HQ cross-tenant posting gated to Admin (explicit tenant override); others pinned to context (also RLS).</t>
+          <t>Manual journal-entry maker-checker — preparer ≠ approver before a manual JE posts.</t>
         </is>
       </c>
       <c r="H86" s="13" t="inlineStr">
@@ -8318,42 +8318,42 @@
       </c>
       <c r="I86" s="13" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="J86" s="13" t="inlineStr">
         <is>
-          <t>Per JE</t>
+          <t>Per manual JE</t>
         </is>
       </c>
       <c r="K86" s="12" t="inlineStr">
         <is>
-          <t>Eng Lead</t>
+          <t>Controller</t>
         </is>
       </c>
       <c r="L86" s="13" t="inlineStr">
         <is>
-          <t>P10/P11</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="M86" s="12" t="inlineStr">
         <is>
-          <t>ledger.controller.ts (hqTenant)</t>
+          <t>ledger.service.ts (postEntry pendingApproval→Draft; approveEntry preparer≠approver; rejectEntry); ledger.controller.ts (gl_post posts / gl_close approves); cutover/compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N86" s="12" t="inlineStr">
         <is>
-          <t>Inspect Admin gating of tenant_id.</t>
+          <t>Inspect JE approval routing.</t>
         </is>
       </c>
       <c r="O86" s="12" t="inlineStr">
         <is>
-          <t>Non-Admin tenant override ignored; Admin audited.</t>
+          <t>Sample manual JEs: approver ≠ preparer; Draft excluded from balances until approved (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P86" s="12" t="inlineStr">
         <is>
-          <t>Override test</t>
+          <t>JE approvals</t>
         </is>
       </c>
       <c r="Q86" s="18" t="inlineStr">
@@ -8365,7 +8365,7 @@
     <row r="87">
       <c r="A87" s="15" t="inlineStr">
         <is>
-          <t>GL-07</t>
+          <t>GL-06</t>
         </is>
       </c>
       <c r="B87" s="16" t="inlineStr">
@@ -8380,27 +8380,27 @@
       </c>
       <c r="D87" s="16" t="inlineStr">
         <is>
-          <t>Cash</t>
+          <t>All</t>
         </is>
       </c>
       <c r="E87" s="16" t="inlineStr">
         <is>
-          <t>Statement of cash flows mis-stated or doesn't tie to the change in cash.</t>
+          <t>Operator mis-posts to another tenant's books.</t>
         </is>
       </c>
       <c r="F87" s="16" t="inlineStr">
         <is>
-          <t>Accuracy/Completeness</t>
+          <t>Validity</t>
         </is>
       </c>
       <c r="G87" s="16" t="inlineStr">
         <is>
-          <t>Statement of Cash Flows (indirect) reconstructed from the GL: net income + non-cash add-backs + working-capital + investing + financing; year-end CLOSE entries excluded; reconciles to Δcash (1000/1010/1020) by construction with a `reconciled` tie-out flag. A direct-method view presents the same operating cash by receipt/payment nature (receipts from customers, payments to suppliers, tax &amp; payroll) and also reconciles to Δcash; a forward cash-flow forecast projects open AR (inflows) and AP (outflows) by due date from today's cash balance for treasury/collections planning.</t>
+          <t>HQ cross-tenant posting gated to Admin (explicit tenant override); others pinned to context (also RLS).</t>
         </is>
       </c>
       <c r="H87" s="17" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I87" s="17" t="inlineStr">
@@ -8410,37 +8410,37 @@
       </c>
       <c r="J87" s="17" t="inlineStr">
         <is>
-          <t>Per period</t>
+          <t>Per JE</t>
         </is>
       </c>
       <c r="K87" s="16" t="inlineStr">
         <is>
-          <t>Controller</t>
+          <t>Eng Lead</t>
         </is>
       </c>
       <c r="L87" s="17" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P10/P11</t>
         </is>
       </c>
       <c r="M87" s="16" t="inlineStr">
         <is>
-          <t>ledger.service.ts (cashFlowStatement, cashFlowDirect, cashFlowForecast); ledger.controller.ts (GET cash-flow, cash-flow-direct, cash-flow-forecast); cutover/basics.ts (ToE)</t>
+          <t>ledger.controller.ts (hqTenant)</t>
         </is>
       </c>
       <c r="N87" s="16" t="inlineStr">
         <is>
-          <t>Inspect SCF derivation + reconciliation flag; inspect direct-method bucketing and forecast projection.</t>
+          <t>Inspect Admin gating of tenant_id.</t>
         </is>
       </c>
       <c r="O87" s="16" t="inlineStr">
         <is>
-          <t>Run cash-flow over a seeded period — activities tie to the movement in cash; CLOSE excluded; direct method ties to the same operating cash and Δcash; forecast buckets open AR/AP by due week (re-performed by the harness).</t>
+          <t>Non-Admin tenant override ignored; Admin audited.</t>
         </is>
       </c>
       <c r="P87" s="16" t="inlineStr">
         <is>
-          <t>Cash-flow reconciliation; direct-method buckets; forecast schedule</t>
+          <t>Override test</t>
         </is>
       </c>
       <c r="Q87" s="18" t="inlineStr">
@@ -8452,7 +8452,7 @@
     <row r="88">
       <c r="A88" s="11" t="inlineStr">
         <is>
-          <t>GL-08</t>
+          <t>GL-07</t>
         </is>
       </c>
       <c r="B88" s="12" t="inlineStr">
@@ -8467,27 +8467,27 @@
       </c>
       <c r="D88" s="12" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Cash</t>
         </is>
       </c>
       <c r="E88" s="12" t="inlineStr">
         <is>
-          <t>Standing/period accruals missed, posted unbalanced, or posted without approval; manual re-keying error.</t>
+          <t>Statement of cash flows mis-stated or doesn't tie to the change in cash.</t>
         </is>
       </c>
       <c r="F88" s="12" t="inlineStr">
         <is>
-          <t>Completeness/Accuracy/Authorization</t>
+          <t>Accuracy/Completeness</t>
         </is>
       </c>
       <c r="G88" s="12" t="inlineStr">
         <is>
-          <t>Recurring/template journal entries: a template's lines are validated balanced (Σdebit=Σcredit) AT SAVE TIME (unbalanced → UNBALANCED), so a broken template can never be persisted. The scheduled job gl_recurring_journals (cron / daily scheduler) posts every due template as a DRAFT JE through the normal maker-checker flow (GL-05) — a different user must approve before it affects balances — and rolls next_run_date forward. Idempotent: next_run_date advanced on posting + the (tenant,source,source_ref,ledger) idempotency key dedupes a same-day re-run. Templates can be paused/resumed without losing history.</t>
+          <t>Statement of Cash Flows (indirect) reconstructed from the GL: net income + non-cash add-backs + working-capital + investing + financing; year-end CLOSE entries excluded; reconciles to Δcash (1000/1010/1020) by construction with a `reconciled` tie-out flag. A direct-method view presents the same operating cash by receipt/payment nature (receipts from customers, payments to suppliers, tax &amp; payroll) and also reconciles to Δcash; a forward cash-flow forecast projects open AR (inflows) and AP (outflows) by due date from today's cash balance for treasury/collections planning.</t>
         </is>
       </c>
       <c r="H88" s="13" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I88" s="13" t="inlineStr">
@@ -8497,7 +8497,7 @@
       </c>
       <c r="J88" s="13" t="inlineStr">
         <is>
-          <t>Per due date / per template</t>
+          <t>Per period</t>
         </is>
       </c>
       <c r="K88" s="12" t="inlineStr">
@@ -8512,22 +8512,22 @@
       </c>
       <c r="M88" s="12" t="inlineStr">
         <is>
-          <t>ledger.service.ts (createRecurring balanced-at-save, runDueRecurring→postEntry pendingApproval, setRecurringActive); ledger.controller.ts (gl_post creates/runs); bi.service.ts (gl_recurring_journals); schema/ledger.ts (recurring_journals) + migration 0119; cutover/basics.ts (ToE)</t>
+          <t>ledger.service.ts (cashFlowStatement, cashFlowDirect, cashFlowForecast); ledger.controller.ts (GET cash-flow, cash-flow-direct, cash-flow-forecast); cutover/basics.ts (ToE)</t>
         </is>
       </c>
       <c r="N88" s="12" t="inlineStr">
         <is>
-          <t>Inspect template balance validation + scheduled posting as Draft + idempotency.</t>
+          <t>Inspect SCF derivation + reconciliation flag; inspect direct-method bucketing and forecast projection.</t>
         </is>
       </c>
       <c r="O88" s="12" t="inlineStr">
         <is>
-          <t>Unbalanced template → UNBALANCED; due template posts a Draft JE (excluded from TB) into the pending queue; re-run posts nothing; a second user approves → accrual hits the GL (re-performed by the harness).</t>
+          <t>Run cash-flow over a seeded period — activities tie to the movement in cash; CLOSE excluded; direct method ties to the same operating cash and Δcash; forecast buckets open AR/AP by due week (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P88" s="12" t="inlineStr">
         <is>
-          <t>Recurring-journal templates; scheduled run log; JE approvals</t>
+          <t>Cash-flow reconciliation; direct-method buckets; forecast schedule</t>
         </is>
       </c>
       <c r="Q88" s="18" t="inlineStr">
@@ -8539,7 +8539,7 @@
     <row r="89">
       <c r="A89" s="15" t="inlineStr">
         <is>
-          <t>GL-09</t>
+          <t>GL-08</t>
         </is>
       </c>
       <c r="B89" s="16" t="inlineStr">
@@ -8554,27 +8554,27 @@
       </c>
       <c r="D89" s="16" t="inlineStr">
         <is>
-          <t>Prepaid expenses; Operating expense</t>
+          <t>All</t>
         </is>
       </c>
       <c r="E89" s="16" t="inlineStr">
         <is>
-          <t>Prepaid expense not amortized over its term — expense mis-stated, prepaid asset overstated.</t>
+          <t>Standing/period accruals missed, posted unbalanced, or posted without approval; manual re-keying error.</t>
         </is>
       </c>
       <c r="F89" s="16" t="inlineStr">
         <is>
-          <t>Accuracy/Completeness</t>
+          <t>Completeness/Accuracy/Authorization</t>
         </is>
       </c>
       <c r="G89" s="16" t="inlineStr">
         <is>
-          <t>Prepaid amortization schedules: a prepaid asset (insurance/rent paid up front) is registered once with a total + term; the scheduled job gl_prepaid_amortize posts a straight-line slice each period (Dr expense / Cr 1280), the last period taking the remainder so the asset fully clears. Idempotent per (schedule, period) via the JE idempotency key + next_run_date advance.</t>
+          <t>Recurring/template journal entries: a template's lines are validated balanced (Σdebit=Σcredit) AT SAVE TIME (unbalanced → UNBALANCED), so a broken template can never be persisted. The scheduled job gl_recurring_journals (cron / daily scheduler) posts every due template as a DRAFT JE through the normal maker-checker flow (GL-05) — a different user must approve before it affects balances — and rolls next_run_date forward. Idempotent: next_run_date advanced on posting + the (tenant,source,source_ref,ledger) idempotency key dedupes a same-day re-run. Templates can be paused/resumed without losing history.</t>
         </is>
       </c>
       <c r="H89" s="17" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I89" s="17" t="inlineStr">
@@ -8584,7 +8584,7 @@
       </c>
       <c r="J89" s="17" t="inlineStr">
         <is>
-          <t>Per period / per schedule</t>
+          <t>Per due date / per template</t>
         </is>
       </c>
       <c r="K89" s="16" t="inlineStr">
@@ -8599,22 +8599,22 @@
       </c>
       <c r="M89" s="16" t="inlineStr">
         <is>
-          <t>ledger.service.ts (createPrepaid, runDuePrepaid); ledger.controller.ts (gl_post); bi.service.ts (gl_prepaid_amortize); schema/ledger.ts (prepaid_schedules) + migration 0120; cutover/basics.ts (ToE)</t>
+          <t>ledger.service.ts (createRecurring balanced-at-save, runDueRecurring→postEntry pendingApproval, setRecurringActive); ledger.controller.ts (gl_post creates/runs); bi.service.ts (gl_recurring_journals); schema/ledger.ts (recurring_journals) + migration 0119; cutover/basics.ts (ToE)</t>
         </is>
       </c>
       <c r="N89" s="16" t="inlineStr">
         <is>
-          <t>Inspect amortization slice + final-period remainder + idempotency.</t>
+          <t>Inspect template balance validation + scheduled posting as Draft + idempotency.</t>
         </is>
       </c>
       <c r="O89" s="16" t="inlineStr">
         <is>
-          <t>Register a 12-month prepaid; run amortizes 1/12 to expense; re-run posts nothing (re-performed by the harness).</t>
+          <t>Unbalanced template → UNBALANCED; due template posts a Draft JE (excluded from TB) into the pending queue; re-run posts nothing; a second user approves → accrual hits the GL (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P89" s="16" t="inlineStr">
         <is>
-          <t>Prepaid schedules; amortization run log</t>
+          <t>Recurring-journal templates; scheduled run log; JE approvals</t>
         </is>
       </c>
       <c r="Q89" s="18" t="inlineStr">
@@ -8626,7 +8626,7 @@
     <row r="90">
       <c r="A90" s="11" t="inlineStr">
         <is>
-          <t>GL-10</t>
+          <t>GL-09</t>
         </is>
       </c>
       <c r="B90" s="12" t="inlineStr">
@@ -8641,27 +8641,27 @@
       </c>
       <c r="D90" s="12" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Prepaid expenses; Operating expense</t>
         </is>
       </c>
       <c r="E90" s="12" t="inlineStr">
         <is>
-          <t>A new company starts on a chart of accounts with no industry guidance — staff post to wrong/ambiguous accounts; or an industry template drifts from the GL engine's fixed posting codes so a posting targets an account that does not exist (mis-statement / unposted transaction).</t>
+          <t>Prepaid expense not amortized over its term — expense mis-stated, prepaid asset overstated.</t>
         </is>
       </c>
       <c r="F90" s="12" t="inlineStr">
         <is>
-          <t>Completeness/Accuracy/Presentation</t>
+          <t>Accuracy/Completeness</t>
         </is>
       </c>
       <c r="G90" s="12" t="inlineStr">
         <is>
-          <t>Industry Chart-of-Accounts templates: the GL engine binds to a FIXED, global account universe (canonical codes are immutable); each tenant additionally gets a per-tenant overlay (tenant_accounts) curating which canonical accounts are active and how they are named/grouped for its industry. At company creation the customer picks an industry (restaurant/retail/distribution/services/general) and the chosen template is materialised into the overlay (provisionTenantCoA) inside the signup transaction, right after fiscal-year provisioning; adopting an industry pack later does the same. Every template code is asserted to exist in the canonical chart at boot (assertTemplatesSubsetOf in seedChartOfAccounts) so a drifted template fails fast and can never reach a tenant. Provisioning is idempotent + additive (never deletes) so re-running only adds missing accounts. The overlay NEVER gates postings — it scopes the picker / Chart-of-Accounts view only; reports surface any account that is active OR carries activity, so a curated-out account that receives a posting still appears.</t>
+          <t>Prepaid amortization schedules: a prepaid asset (insurance/rent paid up front) is registered once with a total + term; the scheduled job gl_prepaid_amortize posts a straight-line slice each period (Dr expense / Cr 1280), the last period taking the remainder so the asset fully clears. Idempotent per (schedule, period) via the JE idempotency key + next_run_date advance.</t>
         </is>
       </c>
       <c r="H90" s="13" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I90" s="13" t="inlineStr">
@@ -8671,7 +8671,7 @@
       </c>
       <c r="J90" s="13" t="inlineStr">
         <is>
-          <t>At company creation / per pack adopt</t>
+          <t>Per period / per schedule</t>
         </is>
       </c>
       <c r="K90" s="12" t="inlineStr">
@@ -8686,22 +8686,22 @@
       </c>
       <c r="M90" s="12" t="inlineStr">
         <is>
-          <t>ledger.service.ts (provisionTenantCoA idempotent+additive, tenant-aware listAccounts, seedChartOfAccounts→assertTemplatesSubsetOf); coa-templates.ts (industry templates + subset assertion); billing.service.ts signup (industry→provisionTenantCoA in-txn); onboarding.service.ts applyPack (pack adopt provisions CoA); schema/ledger.ts tenant_accounts + tenants.industry + migration 0139; cutover/basics.ts + compliance.ts (ToE)</t>
+          <t>ledger.service.ts (createPrepaid, runDuePrepaid); ledger.controller.ts (gl_post); bi.service.ts (gl_prepaid_amortize); schema/ledger.ts (prepaid_schedules) + migration 0120; cutover/basics.ts (ToE)</t>
         </is>
       </c>
       <c r="N90" s="12" t="inlineStr">
         <is>
-          <t>Inspect the boot subset assertion + signup provisioning + the overlay-is-presentation-only read path.</t>
+          <t>Inspect amortization slice + final-period remainder + idempotency.</t>
         </is>
       </c>
       <c r="O90" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: a template referencing an unknown code fails the boot assertion; signup with industry=restaurant materialises a curated, industry-named chart (4000='Food &amp; Beverage Sales') that omits non-F&amp;B accounts; ?all=true still returns the full canonical universe (overlay never gates posting); signup with no industry ⇒ general = the full live chart (re-performed by the harnesses).</t>
+          <t>Register a 12-month prepaid; run amortizes 1/12 to expense; re-run posts nothing (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P90" s="12" t="inlineStr">
         <is>
-          <t>Industry templates; tenant_accounts overlay; signup provisioning log</t>
+          <t>Prepaid schedules; amortization run log</t>
         </is>
       </c>
       <c r="Q90" s="18" t="inlineStr">
@@ -8713,7 +8713,7 @@
     <row r="91">
       <c r="A91" s="15" t="inlineStr">
         <is>
-          <t>GL-11</t>
+          <t>GL-10</t>
         </is>
       </c>
       <c r="B91" s="16" t="inlineStr">
@@ -8733,17 +8733,17 @@
       </c>
       <c r="E91" s="16" t="inlineStr">
         <is>
-          <t>Chart of Accounts changed without authorisation; account code changed after postings exist; account deactivated while carrying a non-zero balance; manual JE posted directly to a control account (AR/AP/INV/FA), bypassing the sub-ledger and hiding a sub-ledger discrepancy.</t>
+          <t>A new company starts on a chart of accounts with no industry guidance — staff post to wrong/ambiguous accounts; or an industry template drifts from the GL engine's fixed posting codes so a posting targets an account that does not exist (mis-statement / unposted transaction).</t>
         </is>
       </c>
       <c r="F91" s="16" t="inlineStr">
         <is>
-          <t>Authorization/Completeness/Accuracy</t>
+          <t>Completeness/Accuracy/Presentation</t>
         </is>
       </c>
       <c r="G91" s="16" t="inlineStr">
         <is>
-          <t>CoA Change Control: account creation/update/deactivation requires the gl_coa permission (held by FinancialController, not GlAccountant — separated from gl_post per SoD). Disabling postability on an account that already has posted entries is rejected (CODE_HAS_POSTINGS). Deactivation is rejected if the account carries a non-zero net balance (ACCOUNT_HAS_BALANCE) — prevents orphaning a balance in a closed account. Four accounts are flagged is_control=true at setup: 1100 (AR), 2000 (AP), 1200 (INV), 1500 (FA); a direct manual JE that touches any of these without viaSubledger:true is rejected (CONTROL_ACCOUNT), ensuring AR/AP/INV/FA balances are exclusively maintained by their respective sub-ledger service methods.</t>
+          <t>Industry Chart-of-Accounts templates: the GL engine binds to a FIXED, global account universe (canonical codes are immutable); each tenant additionally gets a per-tenant overlay (tenant_accounts) curating which canonical accounts are active and how they are named/grouped for its industry. At company creation the customer picks an industry (restaurant/retail/distribution/services/general) and the chosen template is materialised into the overlay (provisionTenantCoA) inside the signup transaction, right after fiscal-year provisioning; adopting an industry pack later does the same. Every template code is asserted to exist in the canonical chart at boot (assertTemplatesSubsetOf in seedChartOfAccounts) so a drifted template fails fast and can never reach a tenant. Provisioning is idempotent + additive (never deletes) so re-running only adds missing accounts. The overlay NEVER gates postings — it scopes the picker / Chart-of-Accounts view only; reports surface any account that is active OR carries activity, so a curated-out account that receives a posting still appears.</t>
         </is>
       </c>
       <c r="H91" s="17" t="inlineStr">
@@ -8758,12 +8758,12 @@
       </c>
       <c r="J91" s="17" t="inlineStr">
         <is>
-          <t>Event-driven</t>
+          <t>At company creation / per pack adopt</t>
         </is>
       </c>
       <c r="K91" s="16" t="inlineStr">
         <is>
-          <t>Financial Controller</t>
+          <t>Controller</t>
         </is>
       </c>
       <c r="L91" s="17" t="inlineStr">
@@ -8773,22 +8773,22 @@
       </c>
       <c r="M91" s="16" t="inlineStr">
         <is>
-          <t>coa.service.ts (createAccount DUPLICATE_ACCOUNT, updateAccount CODE_HAS_POSTINGS, deactivateAccount ACCOUNT_HAS_BALANCE); coa.controller.ts (gl_coa permission gate); ledger.service.ts postEntry control-account guard (CONTROL_ACCOUNT, viaSubledger flag); schema/ledger.ts (account_groups table, accounts.is_control/control_subledger/is_postable/normal_balance + migration 0155); packages/shared/src/permissions.ts (gl_coa sub-permission, FinancialController default)</t>
+          <t>ledger.service.ts (provisionTenantCoA idempotent+additive, tenant-aware listAccounts, seedChartOfAccounts→assertTemplatesSubsetOf); coa-templates.ts (industry templates + subset assertion); billing.service.ts signup (industry→provisionTenantCoA in-txn); onboarding.service.ts applyPack (pack adopt provisions CoA); schema/ledger.ts tenant_accounts + tenants.industry + migration 0139; cutover/basics.ts + compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N91" s="16" t="inlineStr">
         <is>
-          <t>Inspect gl_coa permission gate + CODE_HAS_POSTINGS guard + ACCOUNT_HAS_BALANCE guard + CONTROL_ACCOUNT guard + viaSubledger bypass.</t>
+          <t>Inspect the boot subset assertion + signup provisioning + the overlay-is-presentation-only read path.</t>
         </is>
       </c>
       <c r="O91" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: create an account with gl_coa → 201; attempt to deactivate an account with balance → ACCOUNT_HAS_BALANCE; post directly to account 1100 without viaSubledger → CONTROL_ACCOUNT (re-performed by TC-GL-11-01/02/03 UAT cases).</t>
+          <t>Re-perform: a template referencing an unknown code fails the boot assertion; signup with industry=restaurant materialises a curated, industry-named chart (4000='Food &amp; Beverage Sales') that omits non-F&amp;B accounts; ?all=true still returns the full canonical universe (overlay never gates posting); signup with no industry ⇒ general = the full live chart (re-performed by the harnesses).</t>
         </is>
       </c>
       <c r="P91" s="16" t="inlineStr">
         <is>
-          <t>CoA change log (audit_log); permission test; control-account guard test</t>
+          <t>Industry templates; tenant_accounts overlay; signup provisioning log</t>
         </is>
       </c>
       <c r="Q91" s="18" t="inlineStr">
@@ -8800,7 +8800,7 @@
     <row r="92">
       <c r="A92" s="11" t="inlineStr">
         <is>
-          <t>GL-12</t>
+          <t>GL-11</t>
         </is>
       </c>
       <c r="B92" s="12" t="inlineStr">
@@ -8820,17 +8820,17 @@
       </c>
       <c r="E92" s="12" t="inlineStr">
         <is>
-          <t>Account-assignment errors introduced by scattered inline account-code literals in service code; a tenant needing a different account for a given business event has no mechanism to override without a code change.</t>
+          <t>Chart of Accounts changed without authorisation; account code changed after postings exist; account deactivated while carrying a non-zero balance; manual JE posted directly to a control account (AR/AP/INV/FA), bypassing the sub-ledger and hiding a sub-ledger discrepancy.</t>
         </is>
       </c>
       <c r="F92" s="12" t="inlineStr">
         <is>
-          <t>Authorization/Accuracy</t>
+          <t>Authorization/Completeness/Accuracy</t>
         </is>
       </c>
       <c r="G92" s="12" t="inlineStr">
         <is>
-          <t>Posting / Account-Determination Engine: two tables — posting_event_types (28 seeded event types, e.g. SALE.FOOD, GR.INVENTORY, DEPRECIATION.FA) and posting_rules (maps event × leg-order to semantic role → account_code + DR/CR side) — drive account assignment instead of hard-coded literals. PostingService.post(eventType, ctx) resolves the applicable rules (global defaults, or shadowed by tenant-specific overrides for the same leg_order), translates role-keyed amounts into DR/CR lines, and delegates to LedgerService.postEntry. If no active rules exist for an event the call fails with NO_POSTING_RULE. Tenant-specific rules require gl_posting_rules permission to create/update. PostingService.preview() provides a dry-run for audit.</t>
+          <t>CoA Change Control: account creation/update/deactivation requires the gl_coa permission (held by FinancialController, not GlAccountant — separated from gl_post per SoD). Disabling postability on an account that already has posted entries is rejected (CODE_HAS_POSTINGS). Deactivation is rejected if the account carries a non-zero net balance (ACCOUNT_HAS_BALANCE) — prevents orphaning a balance in a closed account. Four accounts are flagged is_control=true at setup: 1100 (AR), 2000 (AP), 1200 (INV), 1500 (FA); a direct manual JE that touches any of these without viaSubledger:true is rejected (CONTROL_ACCOUNT), ensuring AR/AP/INV/FA balances are exclusively maintained by their respective sub-ledger service methods.</t>
         </is>
       </c>
       <c r="H92" s="13" t="inlineStr">
@@ -8860,22 +8860,22 @@
       </c>
       <c r="M92" s="12" t="inlineStr">
         <is>
-          <t>posting.service.ts (resolveRules, post, preview, listEventTypes, listRules, upsertRule); posting-rules.controller.ts (gl_posting_rules permission gate); schema/posting-rules.ts (posting_event_types, posting_rules tables); migration 0156 (tables + 28 event types + global-default rules); ledger.module.ts (PostingService exported); packages/shared/src/permissions.ts (gl_posting_rules sub-permission); cutover/basics.ts (golden-snapshot ToE)</t>
+          <t>coa.service.ts (createAccount DUPLICATE_ACCOUNT, updateAccount CODE_HAS_POSTINGS, deactivateAccount ACCOUNT_HAS_BALANCE); coa.controller.ts (gl_coa permission gate); ledger.service.ts postEntry control-account guard (CONTROL_ACCOUNT, viaSubledger flag); schema/ledger.ts (account_groups table, accounts.is_control/control_subledger/is_postable/normal_balance + migration 0155); packages/shared/src/permissions.ts (gl_coa sub-permission, FinancialController default)</t>
         </is>
       </c>
       <c r="N92" s="12" t="inlineStr">
         <is>
-          <t>Inspect the rule-resolution logic + NO_POSTING_RULE fast-fail + tenant-shadow logic + gl_posting_rules permission gate.</t>
+          <t>Inspect gl_coa permission gate + CODE_HAS_POSTINGS guard + ACCOUNT_HAS_BALANCE guard + CONTROL_ACCOUNT guard + viaSubledger bypass.</t>
         </is>
       </c>
       <c r="O92" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: preview DEPRECIATION.FA with dep_expense:1000 → DR 5200 / CR 1590; preview GR.INVENTORY with inventory:500 → DR 1200 / CR 2000; preview UNKNOWN_EVENT → NO_POSTING_RULE (400); event-type catalogue returns ≥20 entries (re-performed by TC-GL-12-01/02/03/04 UAT cases + basics.ts harness).</t>
+          <t>Re-perform: create an account with gl_coa → 201; attempt to deactivate an account with balance → ACCOUNT_HAS_BALANCE; post directly to account 1100 without viaSubledger → CONTROL_ACCOUNT (re-performed by TC-GL-11-01/02/03 UAT cases).</t>
         </is>
       </c>
       <c r="P92" s="12" t="inlineStr">
         <is>
-          <t>Posting-rule change log; preview dry-run; harness golden snapshot</t>
+          <t>CoA change log (audit_log); permission test; control-account guard test</t>
         </is>
       </c>
       <c r="Q92" s="18" t="inlineStr">
@@ -8887,7 +8887,7 @@
     <row r="93">
       <c r="A93" s="15" t="inlineStr">
         <is>
-          <t>GL-13</t>
+          <t>GL-12</t>
         </is>
       </c>
       <c r="B93" s="16" t="inlineStr">
@@ -8907,22 +8907,22 @@
       </c>
       <c r="E93" s="16" t="inlineStr">
         <is>
-          <t>Revenue or expense mis-attributed to the wrong branch / project — per-location P&amp;L is unintelligible or misleading.</t>
+          <t>Account-assignment errors introduced by scattered inline account-code literals in service code; a tenant needing a different account for a given business event has no mechanism to override without a code change.</t>
         </is>
       </c>
       <c r="F93" s="16" t="inlineStr">
         <is>
-          <t>Accuracy/Presentation</t>
+          <t>Authorization/Accuracy</t>
         </is>
       </c>
       <c r="G93" s="16" t="inlineStr">
         <is>
-          <t>Multi-dimensional GL postings: journal_lines carries three optional dimension columns (branch_id, project_id, department_id). PostingService.post() stamps all generated lines from PostingContext (branchId/projectId/departmentId). GET /api/ledger/income-statement/by-branch provides a per-branch P&amp;L view; lines without a branch_id are grouped as 'unassigned'. The departments master table holds a tenant-scoped department registry with RLS isolation.</t>
+          <t>Posting / Account-Determination Engine: two tables — posting_event_types (28 seeded event types, e.g. SALE.FOOD, GR.INVENTORY, DEPRECIATION.FA) and posting_rules (maps event × leg-order to semantic role → account_code + DR/CR side) — drive account assignment instead of hard-coded literals. PostingService.post(eventType, ctx) resolves the applicable rules (global defaults, or shadowed by tenant-specific overrides for the same leg_order), translates role-keyed amounts into DR/CR lines, and delegates to LedgerService.postEntry. If no active rules exist for an event the call fails with NO_POSTING_RULE. Tenant-specific rules require gl_posting_rules permission to create/update. PostingService.preview() provides a dry-run for audit.</t>
         </is>
       </c>
       <c r="H93" s="17" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I93" s="17" t="inlineStr">
@@ -8932,12 +8932,12 @@
       </c>
       <c r="J93" s="17" t="inlineStr">
         <is>
-          <t>Per period</t>
+          <t>Event-driven</t>
         </is>
       </c>
       <c r="K93" s="16" t="inlineStr">
         <is>
-          <t>Controller</t>
+          <t>Financial Controller</t>
         </is>
       </c>
       <c r="L93" s="17" t="inlineStr">
@@ -8947,22 +8947,22 @@
       </c>
       <c r="M93" s="16" t="inlineStr">
         <is>
-          <t>ledger.service.ts (incomeStatementByBranch); ledger.controller.ts (GET income-statement/by-branch); posting.service.ts (branchId/projectId/departmentId from PostingContext); schema/ledger.ts (branch_id, project_id, department_id on journal_lines); schema/departments.ts (departments table); migration 0157; cutover/basics.ts (GL-13 ToE)</t>
+          <t>posting.service.ts (resolveRules, post, preview, listEventTypes, listRules, upsertRule); posting-rules.controller.ts (gl_posting_rules permission gate); schema/posting-rules.ts (posting_event_types, posting_rules tables); migration 0156 (tables + 28 event types + global-default rules); ledger.module.ts (PostingService exported); packages/shared/src/permissions.ts (gl_posting_rules sub-permission); cutover/basics.ts (golden-snapshot ToE)</t>
         </is>
       </c>
       <c r="N93" s="16" t="inlineStr">
         <is>
-          <t>Inspect by-branch query + PostingContext stamping + department RLS.</t>
+          <t>Inspect the rule-resolution logic + NO_POSTING_RULE fast-fail + tenant-shadow logic + gl_posting_rules permission gate.</t>
         </is>
       </c>
       <c r="O93" s="16" t="inlineStr">
         <is>
-          <t>TC-GL-13-01/02/03: smoke + two branches + unassigned bucket (re-performed by the basics.ts harness).</t>
+          <t>Re-perform: preview DEPRECIATION.FA with dep_expense:1000 → DR 5200 / CR 1590; preview GR.INVENTORY with inventory:500 → DR 1200 / CR 2000; preview UNKNOWN_EVENT → NO_POSTING_RULE (400); event-type catalogue returns ≥20 entries (re-performed by TC-GL-12-01/02/03/04 UAT cases + basics.ts harness).</t>
         </is>
       </c>
       <c r="P93" s="16" t="inlineStr">
         <is>
-          <t>By-branch P&amp;L report; dimension completeness</t>
+          <t>Posting-rule change log; preview dry-run; harness golden snapshot</t>
         </is>
       </c>
       <c r="Q93" s="18" t="inlineStr">
@@ -8974,7 +8974,7 @@
     <row r="94">
       <c r="A94" s="11" t="inlineStr">
         <is>
-          <t>GL-14</t>
+          <t>GL-13</t>
         </is>
       </c>
       <c r="B94" s="12" t="inlineStr">
@@ -8994,17 +8994,17 @@
       </c>
       <c r="E94" s="12" t="inlineStr">
         <is>
-          <t>GL control-account balances (AR/AP/INV/FA) drift from the underlying sub-ledger detail without detection — the control account no longer represents the sum of its sub-ledger, masking posting errors, unrecorded items, or fraud.</t>
+          <t>Revenue or expense mis-attributed to the wrong branch / project — per-location P&amp;L is unintelligible or misleading.</t>
         </is>
       </c>
       <c r="F94" s="12" t="inlineStr">
         <is>
-          <t>Completeness/Accuracy/Valuation</t>
+          <t>Accuracy/Presentation</t>
         </is>
       </c>
       <c r="G94" s="12" t="inlineStr">
         <is>
-          <t>Sub-ledger tie-out / reconciliation: POST /api/ledger/tie-out/run computes, per control account, the GL balance (Σ debit−credit of posted journal_lines on the control account up to the as-of date, tenant-scoped) and the sub-ledger detail balance (AR = Σ outstanding ar_invoices; AP = Σ outstanding ap_transactions; INV = Σ inv_balances.total_value perpetual valuation; FA = Σ acquire_cost − accumulated_depreciation of non-disposed fixed_assets), records the variance (gl − subledger) and a status (Matched if |variance|&lt;0.01 else Variance). Runs upsert per (tenant, subledger, as-of). Certification is maker-checker: POST /api/ledger/tie-out/:id/certify sets status=Certified and records certifier + timestamp, and REJECTS a certifier equal to the runner (SELF_CERTIFY) — the gl_close certifier must differ from the gl_post/gl_close runner (SoD).</t>
+          <t>Multi-dimensional GL postings: journal_lines carries three optional dimension columns (branch_id, project_id, department_id). PostingService.post() stamps all generated lines from PostingContext (branchId/projectId/departmentId). GET /api/ledger/income-statement/by-branch provides a per-branch P&amp;L view; lines without a branch_id are grouped as 'unassigned'. The departments master table holds a tenant-scoped department registry with RLS isolation.</t>
         </is>
       </c>
       <c r="H94" s="13" t="inlineStr">
@@ -9019,12 +9019,12 @@
       </c>
       <c r="J94" s="13" t="inlineStr">
         <is>
-          <t>Monthly</t>
+          <t>Per period</t>
         </is>
       </c>
       <c r="K94" s="12" t="inlineStr">
         <is>
-          <t>Financial Controller</t>
+          <t>Controller</t>
         </is>
       </c>
       <c r="L94" s="13" t="inlineStr">
@@ -9034,22 +9034,22 @@
       </c>
       <c r="M94" s="12" t="inlineStr">
         <is>
-          <t>subledger-tieout.service.ts (runTieOut GL/sub-ledger balance computation + variance/status, certify SELF_CERTIFY maker-checker, list/get); subledger-tieout.controller.ts (gl_close/gl_post run, gl_close certify, gl_close/gl_post/exec/creditors/ar read); schema/subledger-tieout.ts (subledger_tieout_runs table, uq on tenant/subledger/as-of); migration 0160 (table + RLS); ledger.module.ts (service+controller wired); cutover/basics.ts (GL-14 ToE)</t>
+          <t>ledger.service.ts (incomeStatementByBranch); ledger.controller.ts (GET income-statement/by-branch); posting.service.ts (branchId/projectId/departmentId from PostingContext); schema/ledger.ts (branch_id, project_id, department_id on journal_lines); schema/departments.ts (departments table); migration 0157; cutover/basics.ts (GL-13 ToE)</t>
         </is>
       </c>
       <c r="N94" s="12" t="inlineStr">
         <is>
-          <t>Inspect the GL-vs-sub-ledger balance computation + variance/status + SELF_CERTIFY maker-checker gate + gl_close certify permission.</t>
+          <t>Inspect by-branch query + PostingContext stamping + department RLS.</t>
         </is>
       </c>
       <c r="O94" s="12" t="inlineStr">
         <is>
-          <t>TC-GL-14-01: run AR tie-out → balances + Matched/Variance; TC-GL-14-02: self-certify by the runner → SELF_CERTIFY (400); TC-GL-14-03: certify by a different gl_close user → Certified (re-performed by the basics.ts harness).</t>
+          <t>TC-GL-13-01/02/03: smoke + two branches + unassigned bucket (re-performed by the basics.ts harness).</t>
         </is>
       </c>
       <c r="P94" s="12" t="inlineStr">
         <is>
-          <t>Tie-out run log (subledger_tieout_runs) with variance + certification trail; monthly reconciliation sign-off</t>
+          <t>By-branch P&amp;L report; dimension completeness</t>
         </is>
       </c>
       <c r="Q94" s="18" t="inlineStr">
@@ -9061,7 +9061,7 @@
     <row r="95">
       <c r="A95" s="15" t="inlineStr">
         <is>
-          <t>GL-15</t>
+          <t>GL-14</t>
         </is>
       </c>
       <c r="B95" s="16" t="inlineStr">
@@ -9081,22 +9081,22 @@
       </c>
       <c r="E95" s="16" t="inlineStr">
         <is>
-          <t>A period is 'closed' on paper but key close procedures (sub-ledger tie-out, bank rec, depreciation, recurring/prepaid, trial-balance review) were skipped, OR a closed period is silently re-opened and re-posted — the financial statements are produced on an incomplete/altered basis.</t>
+          <t>GL control-account balances (AR/AP/INV/FA) drift from the underlying sub-ledger detail without detection — the control account no longer represents the sum of its sub-ledger, masking posting errors, unrecorded items, or fraud.</t>
         </is>
       </c>
       <c r="F95" s="16" t="inlineStr">
         <is>
-          <t>Completeness/Accuracy/Cutoff</t>
+          <t>Completeness/Accuracy/Valuation</t>
         </is>
       </c>
       <c r="G95" s="16" t="inlineStr">
         <is>
-          <t>Hard period close + checklist: POST /api/ledger/close/start opens a close_runs record (status InProgress) per (tenant, period) and seeds a standard checklist of close_run_steps (subledger_tieout, bank_rec, depreciation, recurring, fx_reval[advisory], trial_balance_review). POST /api/ledger/close/step marks a step Done (records completedBy/At); when all REQUIRED steps are Done the run advances to ReadyToLock. POST /api/ledger/close/lock requires ReadyToLock (else STEPS_INCOMPLETE listing the pending required steps) before the period can be locked. Locking writes 'Locked' into fiscal_periods.status; LedgerService.postEntry then REJECTS every posting dated into a Locked period with PERIOD_LOCKED, regardless of the legacy allowClosedPeriod escape (the only exception is the system year-end closing entry, source='CLOSE'). Locked is strictly stronger than the soft 'Closed' status — it is the irreversible hard close.</t>
+          <t>Sub-ledger tie-out / reconciliation: POST /api/ledger/tie-out/run computes, per control account, the GL balance (Σ debit−credit of posted journal_lines on the control account up to the as-of date, tenant-scoped) and the sub-ledger detail balance (AR = Σ outstanding ar_invoices; AP = Σ outstanding ap_transactions; INV = Σ inv_balances.total_value perpetual valuation; FA = Σ acquire_cost − accumulated_depreciation of non-disposed fixed_assets), records the variance (gl − subledger) and a status (Matched if |variance|&lt;0.01 else Variance). Runs upsert per (tenant, subledger, as-of). Certification is maker-checker: POST /api/ledger/tie-out/:id/certify sets status=Certified and records certifier + timestamp, and REJECTS a certifier equal to the runner (SELF_CERTIFY) — the gl_close certifier must differ from the gl_post/gl_close runner (SoD).</t>
         </is>
       </c>
       <c r="H95" s="17" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I95" s="17" t="inlineStr">
@@ -9121,22 +9121,22 @@
       </c>
       <c r="M95" s="16" t="inlineStr">
         <is>
-          <t>close.service.ts (startClose seeds checklist, completeStep → ReadyToLock when required steps Done, lockPeriod STEPS_INCOMPLETE gate + fiscal_periods Locked write, status/list); close.controller.ts (gl_close start/step/lock, gl_close/gl_post/exec read); schema/close-runs.ts (close_runs + close_run_steps, uq on tenant/period and run/step_key); schema/ledger.ts (period_status enum + 'Locked'); ledger.service.ts (postEntry PERIOD_LOCKED hard gate, source='CLOSE' exemption); migration 0162 (tables + RLS + ALTER TYPE Locked); ledger.module.ts (service+controller wired); cutover/basics.ts (GL-15/GL-16 ToE)</t>
+          <t>subledger-tieout.service.ts (runTieOut GL/sub-ledger balance computation + variance/status, certify SELF_CERTIFY maker-checker, list/get); subledger-tieout.controller.ts (gl_close/gl_post run, gl_close certify, gl_close/gl_post/exec/creditors/ar read); schema/subledger-tieout.ts (subledger_tieout_runs table, uq on tenant/subledger/as-of); migration 0160 (table + RLS); ledger.module.ts (service+controller wired); cutover/basics.ts (GL-14 ToE)</t>
         </is>
       </c>
       <c r="N95" s="16" t="inlineStr">
         <is>
-          <t>Inspect the seeded checklist + ReadyToLock gating + STEPS_INCOMPLETE lock rejection + PERIOD_LOCKED hard gate in postEntry (incl. the CLOSE exemption).</t>
+          <t>Inspect the GL-vs-sub-ledger balance computation + variance/status + SELF_CERTIFY maker-checker gate + gl_close certify permission.</t>
         </is>
       </c>
       <c r="O95" s="16" t="inlineStr">
         <is>
-          <t>TC-GL-15-01: start close seeds ≥4 steps (InProgress); TC-GL-15-02: lock before steps done → STEPS_INCOMPLETE (400); TC-GL-15-03: post into locked period → PERIOD_LOCKED (400) (re-performed by the basics.ts harness).</t>
+          <t>TC-GL-14-01: run AR tie-out → balances + Matched/Variance; TC-GL-14-02: self-certify by the runner → SELF_CERTIFY (400); TC-GL-14-03: certify by a different gl_close user → Certified (re-performed by the basics.ts harness).</t>
         </is>
       </c>
       <c r="P95" s="16" t="inlineStr">
         <is>
-          <t>close_runs / close_run_steps with completion trail; fiscal_periods.status=Locked; monthly close sign-off</t>
+          <t>Tie-out run log (subledger_tieout_runs) with variance + certification trail; monthly reconciliation sign-off</t>
         </is>
       </c>
       <c r="Q95" s="18" t="inlineStr">
@@ -9148,7 +9148,7 @@
     <row r="96">
       <c r="A96" s="11" t="inlineStr">
         <is>
-          <t>GL-16</t>
+          <t>GL-15</t>
         </is>
       </c>
       <c r="B96" s="12" t="inlineStr">
@@ -9168,17 +9168,17 @@
       </c>
       <c r="E96" s="12" t="inlineStr">
         <is>
-          <t>One person both performs the close and locks the period, defeating segregation of duties — a preparer could conceal a misstatement by closing over their own work without independent review.</t>
+          <t>A period is 'closed' on paper but key close procedures (sub-ledger tie-out, bank rec, depreciation, recurring/prepaid, trial-balance review) were skipped, OR a closed period is silently re-opened and re-posted — the financial statements are produced on an incomplete/altered basis.</t>
         </is>
       </c>
       <c r="F96" s="12" t="inlineStr">
         <is>
-          <t>Authorization/Segregation of Duties</t>
+          <t>Completeness/Accuracy/Cutoff</t>
         </is>
       </c>
       <c r="G96" s="12" t="inlineStr">
         <is>
-          <t>Segregated period lock (maker-checker): the close_runs.started_by (the user who started the close and ran the checklist steps) is recorded, and POST /api/ledger/close/lock REJECTS a lockedBy equal to startedBy with SELF_LOCK — the gl_close user who locks the period MUST differ from the user who started/ran the close. Both identities and the lock timestamp are retained on the close_runs row (started_by / locked_by / locked_at) as the SoD evidence trail. This complements the existing SoD rule that gl_close is segregated from gl_post (JE posting).</t>
+          <t>Hard period close + checklist: POST /api/ledger/close/start opens a close_runs record (status InProgress) per (tenant, period) and seeds a standard checklist of close_run_steps (subledger_tieout, bank_rec, depreciation, recurring, fx_reval[advisory], trial_balance_review). POST /api/ledger/close/step marks a step Done (records completedBy/At); when all REQUIRED steps are Done the run advances to ReadyToLock. POST /api/ledger/close/lock requires ReadyToLock (else STEPS_INCOMPLETE listing the pending required steps) before the period can be locked. Locking writes 'Locked' into fiscal_periods.status; LedgerService.postEntry then REJECTS every posting dated into a Locked period with PERIOD_LOCKED, regardless of the legacy allowClosedPeriod escape (the only exception is the system year-end closing entry, source='CLOSE'). Locked is strictly stronger than the soft 'Closed' status — it is the irreversible hard close.</t>
         </is>
       </c>
       <c r="H96" s="13" t="inlineStr">
@@ -9208,22 +9208,22 @@
       </c>
       <c r="M96" s="12" t="inlineStr">
         <is>
-          <t>close.service.ts (lockPeriod SELF_LOCK maker-checker gate; started_by vs locked_by); close.controller.ts (gl_close lock, acting username from JWT); schema/close-runs.ts (started_by, locked_by, locked_at columns); permissions.ts (gl_post×gl_close SoD pair); cutover/basics.ts (GL-16 ToE)</t>
+          <t>close.service.ts (startClose seeds checklist, completeStep → ReadyToLock when required steps Done, lockPeriod STEPS_INCOMPLETE gate + fiscal_periods Locked write, status/list); close.controller.ts (gl_close start/step/lock, gl_close/gl_post/exec read); schema/close-runs.ts (close_runs + close_run_steps, uq on tenant/period and run/step_key); schema/ledger.ts (period_status enum + 'Locked'); ledger.service.ts (postEntry PERIOD_LOCKED hard gate, source='CLOSE' exemption); migration 0162 (tables + RLS + ALTER TYPE Locked); ledger.module.ts (service+controller wired); cutover/basics.ts (GL-15/GL-16 ToE)</t>
         </is>
       </c>
       <c r="N96" s="12" t="inlineStr">
         <is>
-          <t>Inspect the SELF_LOCK gate (startedBy ≠ lockedBy) + the started_by/locked_by/locked_at evidence trail.</t>
+          <t>Inspect the seeded checklist + ReadyToLock gating + STEPS_INCOMPLETE lock rejection + PERIOD_LOCKED hard gate in postEntry (incl. the CLOSE exemption).</t>
         </is>
       </c>
       <c r="O96" s="12" t="inlineStr">
         <is>
-          <t>TC-GL-16-01: self-lock by the starter → SELF_LOCK (400); TC-GL-16-02: lock by a different gl_close user → Locked, locked_by recorded (re-performed by the basics.ts harness).</t>
+          <t>TC-GL-15-01: start close seeds ≥4 steps (InProgress); TC-GL-15-02: lock before steps done → STEPS_INCOMPLETE (400); TC-GL-15-03: post into locked period → PERIOD_LOCKED (400) (re-performed by the basics.ts harness).</t>
         </is>
       </c>
       <c r="P96" s="12" t="inlineStr">
         <is>
-          <t>close_runs.started_by / locked_by / locked_at SoD trail; monthly close sign-off</t>
+          <t>close_runs / close_run_steps with completion trail; fiscal_periods.status=Locked; monthly close sign-off</t>
         </is>
       </c>
       <c r="Q96" s="18" t="inlineStr">
@@ -9235,12 +9235,12 @@
     <row r="97">
       <c r="A97" s="15" t="inlineStr">
         <is>
-          <t>EXP-07</t>
+          <t>GL-16</t>
         </is>
       </c>
       <c r="B97" s="16" t="inlineStr">
         <is>
-          <t>Expenditure</t>
+          <t>General Ledger</t>
         </is>
       </c>
       <c r="C97" s="17" t="inlineStr">
@@ -9250,27 +9250,27 @@
       </c>
       <c r="D97" s="16" t="inlineStr">
         <is>
-          <t>Cash; Operating expense</t>
+          <t>All</t>
         </is>
       </c>
       <c r="E97" s="16" t="inlineStr">
         <is>
-          <t>Petty-cash / employee advance issued but never accounted for — cash leakage, expense unrecorded.</t>
+          <t>One person both performs the close and locks the period, defeating segregation of duties — a preparer could conceal a misstatement by closing over their own work without independent review.</t>
         </is>
       </c>
       <c r="F97" s="16" t="inlineStr">
         <is>
-          <t>Existence/Completeness</t>
+          <t>Authorization/Segregation of Duties</t>
         </is>
       </c>
       <c r="G97" s="16" t="inlineStr">
         <is>
-          <t>Employee cash advances: issuing an advance debits the 1180 Employee Advances control (Dr 1180 / Cr 1000); settlement clears it against actual spend + returned cash (Dr expense + Dr 1000 / Cr 1180), enforced to reconcile (settled_expense + returned_cash must equal the advance → SETTLE_MISMATCH). The 1180 balance is the outstanding float subject to review.</t>
+          <t>Segregated period lock (maker-checker): the close_runs.started_by (the user who started the close and ran the checklist steps) is recorded, and POST /api/ledger/close/lock REJECTS a lockedBy equal to startedBy with SELF_LOCK — the gl_close user who locks the period MUST differ from the user who started/ran the close. Both identities and the lock timestamp are retained on the close_runs row (started_by / locked_by / locked_at) as the SoD evidence trail. This complements the existing SoD rule that gl_close is segregated from gl_post (JE posting).</t>
         </is>
       </c>
       <c r="H97" s="17" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I97" s="17" t="inlineStr">
@@ -9280,12 +9280,12 @@
       </c>
       <c r="J97" s="17" t="inlineStr">
         <is>
-          <t>Per advance</t>
+          <t>Monthly</t>
         </is>
       </c>
       <c r="K97" s="16" t="inlineStr">
         <is>
-          <t>AP / Controller</t>
+          <t>Financial Controller</t>
         </is>
       </c>
       <c r="L97" s="17" t="inlineStr">
@@ -9295,22 +9295,22 @@
       </c>
       <c r="M97" s="16" t="inlineStr">
         <is>
-          <t>finance.service.ts (issueAdvance, settleAdvance reconcile-or-reject, listAdvances outstanding); finance.controller.ts (creditors/exec); schema/finance.ts (employee_advances) + migration 0120; cutover/basics.ts (ToE)</t>
+          <t>close.service.ts (lockPeriod SELF_LOCK maker-checker gate; started_by vs locked_by); close.controller.ts (gl_close lock, acting username from JWT); schema/close-runs.ts (started_by, locked_by, locked_at columns); permissions.ts (gl_post×gl_close SoD pair); cutover/basics.ts (GL-16 ToE)</t>
         </is>
       </c>
       <c r="N97" s="16" t="inlineStr">
         <is>
-          <t>Inspect issue/settle GL + settlement reconciliation guard.</t>
+          <t>Inspect the SELF_LOCK gate (startedBy ≠ lockedBy) + the started_by/locked_by/locked_at evidence trail.</t>
         </is>
       </c>
       <c r="O97" s="16" t="inlineStr">
         <is>
-          <t>Issue an advance (1180 up); settle 700+300 clears 1180; mismatched settle → SETTLE_MISMATCH (re-performed by the harness).</t>
+          <t>TC-GL-16-01: self-lock by the starter → SELF_LOCK (400); TC-GL-16-02: lock by a different gl_close user → Locked, locked_by recorded (re-performed by the basics.ts harness).</t>
         </is>
       </c>
       <c r="P97" s="16" t="inlineStr">
         <is>
-          <t>Advance register; outstanding float</t>
+          <t>close_runs.started_by / locked_by / locked_at SoD trail; monthly close sign-off</t>
         </is>
       </c>
       <c r="Q97" s="18" t="inlineStr">
@@ -9322,7 +9322,7 @@
     <row r="98">
       <c r="A98" s="11" t="inlineStr">
         <is>
-          <t>EXP-08</t>
+          <t>EXP-07</t>
         </is>
       </c>
       <c r="B98" s="12" t="inlineStr">
@@ -9342,22 +9342,22 @@
       </c>
       <c r="E98" s="12" t="inlineStr">
         <is>
-          <t>Petty-cash disbursed beyond authority / without independent review, or drawn past the fund's limit — cash leakage, unauthorised or unrecorded expense, over-extended float.</t>
+          <t>Petty-cash / employee advance issued but never accounted for — cash leakage, expense unrecorded.</t>
         </is>
       </c>
       <c r="F98" s="12" t="inlineStr">
         <is>
-          <t>Authorization; Completeness</t>
+          <t>Existence/Completeness</t>
         </is>
       </c>
       <c r="G98" s="12" t="inlineStr">
         <is>
-          <t>Petty-cash imprest float + maker-checker on disbursement (SoD): a fund holds cash capped at a credit limit/วงเงิน (1015 Petty Cash, a cash account); each direct EXPENSE or ADVANCE is a REQUEST that posts NOTHING and a DIFFERENT user must approve before the GL posts (expense Dr &lt;expense&gt; / Cr 1015; advance Dr 1180 / Cr 1015) and the fund balance is decremented. Self-approval → SOD_VIOLATION (binds even Admin). A draw beyond the fund balance → INSUFFICIENT_FLOAT; establishing/replenishing above the float limit → OVER_FLOAT. Advances settle (Dr expense + Dr 1015 returned / Cr 1180), returning unused cash to the fund. Every request carries a document reference + receipt key + a status trail (StatusLog) and surfaces in the GOV-01 pending-approvals monitor.</t>
+          <t>Employee cash advances: issuing an advance debits the 1180 Employee Advances control (Dr 1180 / Cr 1000); settlement clears it against actual spend + returned cash (Dr expense + Dr 1000 / Cr 1180), enforced to reconcile (settled_expense + returned_cash must equal the advance → SETTLE_MISMATCH). The 1180 balance is the outstanding float subject to review.</t>
         </is>
       </c>
       <c r="H98" s="13" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I98" s="13" t="inlineStr">
@@ -9367,7 +9367,7 @@
       </c>
       <c r="J98" s="13" t="inlineStr">
         <is>
-          <t>Per disbursement</t>
+          <t>Per advance</t>
         </is>
       </c>
       <c r="K98" s="12" t="inlineStr">
@@ -9382,22 +9382,22 @@
       </c>
       <c r="M98" s="12" t="inlineStr">
         <is>
-          <t>petty-cash.service.ts (establishFund/replenishFund float guards, createRequest INSUFFICIENT_FLOAT, approveRequest SoD+GL, rejectRequest, settleRequest); petty-cash.controller.ts (creditors/exec); schema/petty-cash.ts (petty_cash_funds, expense_requests) + migration 0139; finance.service.ts pendingApprovals (GOV-01 source 7); cutover/basics.ts + compliance.ts (ToE)</t>
+          <t>finance.service.ts (issueAdvance, settleAdvance reconcile-or-reject, listAdvances outstanding); finance.controller.ts (creditors/exec); schema/finance.ts (employee_advances) + migration 0120; cutover/basics.ts (ToE)</t>
         </is>
       </c>
       <c r="N98" s="12" t="inlineStr">
         <is>
-          <t>Inspect the float ceiling + the request→approve flow + the approver≠requester check + that the request posts nothing until approval.</t>
+          <t>Inspect issue/settle GL + settlement reconciliation guard.</t>
         </is>
       </c>
       <c r="O98" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: establish a fund (Dr 1015), request an expense (no GL), self-approve → SOD_VIOLATION, approve as a different user → Dr expense/Cr 1015 + fund down; over-balance draw → INSUFFICIENT_FLOAT; advance approve→settle clears 1180; replenish past float → OVER_FLOAT (re-performed by the harnesses).</t>
+          <t>Issue an advance (1180 up); settle 700+300 clears 1180; mismatched settle → SETTLE_MISMATCH (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P98" s="12" t="inlineStr">
         <is>
-          <t>Fund register + disbursement approval log + SoD test</t>
+          <t>Advance register; outstanding float</t>
         </is>
       </c>
       <c r="Q98" s="18" t="inlineStr">
@@ -9409,12 +9409,12 @@
     <row r="99">
       <c r="A99" s="15" t="inlineStr">
         <is>
-          <t>FA-07</t>
+          <t>EXP-08</t>
         </is>
       </c>
       <c r="B99" s="16" t="inlineStr">
         <is>
-          <t>Fixed Assets</t>
+          <t>Expenditure</t>
         </is>
       </c>
       <c r="C99" s="17" t="inlineStr">
@@ -9424,27 +9424,27 @@
       </c>
       <c r="D99" s="16" t="inlineStr">
         <is>
-          <t>Property, Plant &amp; Equipment; Equity</t>
+          <t>Cash; Operating expense</t>
         </is>
       </c>
       <c r="E99" s="16" t="inlineStr">
         <is>
-          <t>Carrying amount not adjusted for revaluation/impairment — asset over/understated.</t>
+          <t>Petty-cash disbursed beyond authority / without independent review, or drawn past the fund's limit — cash leakage, unauthorised or unrecorded expense, over-extended float.</t>
         </is>
       </c>
       <c r="F99" s="16" t="inlineStr">
         <is>
-          <t>Valuation</t>
+          <t>Authorization; Completeness</t>
         </is>
       </c>
       <c r="G99" s="16" t="inlineStr">
         <is>
-          <t>Asset revaluation / impairment: an upward revaluation credits the revaluation surplus in equity (Dr 1500 / Cr 3200); a downward revaluation (impairment) debits impairment loss (Dr 5820 / Cr 1500). The gross 1500 moves by the delta so the register stays tied to the GL; a no-op revaluation is rejected (NO_CHANGE). Every event is logged for the audit trail.</t>
+          <t>Petty-cash imprest float + maker-checker on disbursement (SoD): a fund holds cash capped at a credit limit/วงเงิน (1015 Petty Cash, a cash account); each direct EXPENSE or ADVANCE is a REQUEST that posts NOTHING and a DIFFERENT user must approve before the GL posts (expense Dr &lt;expense&gt; / Cr 1015; advance Dr 1180 / Cr 1015) and the fund balance is decremented. Self-approval → SOD_VIOLATION (binds even Admin). A draw beyond the fund balance → INSUFFICIENT_FLOAT; establishing/replenishing above the float limit → OVER_FLOAT. Advances settle (Dr expense + Dr 1015 returned / Cr 1180), returning unused cash to the fund. Every request carries a document reference + receipt key + a status trail (StatusLog) and surfaces in the GOV-01 pending-approvals monitor.</t>
         </is>
       </c>
       <c r="H99" s="17" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I99" s="17" t="inlineStr">
@@ -9454,12 +9454,12 @@
       </c>
       <c r="J99" s="17" t="inlineStr">
         <is>
-          <t>Per event</t>
+          <t>Per disbursement</t>
         </is>
       </c>
       <c r="K99" s="16" t="inlineStr">
         <is>
-          <t>FaAccountant / Controller</t>
+          <t>AP / Controller</t>
         </is>
       </c>
       <c r="L99" s="17" t="inlineStr">
@@ -9469,22 +9469,22 @@
       </c>
       <c r="M99" s="16" t="inlineStr">
         <is>
-          <t>assets.service.ts (revalue up→3200 / down→5820, listRevaluations; dispose recycles surplus 3200→3100); assets.controller.ts (exec/creditors); schema/assets.ts (asset_revaluations) + migration 0120; cutover/basics.ts (ToE)</t>
+          <t>petty-cash.service.ts (establishFund/replenishFund float guards, createRequest INSUFFICIENT_FLOAT, approveRequest SoD+GL, rejectRequest, settleRequest); petty-cash.controller.ts (creditors/exec); schema/petty-cash.ts (petty_cash_funds, expense_requests) + migration 0139; finance.service.ts pendingApprovals (GOV-01 source 7); cutover/basics.ts + compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N99" s="16" t="inlineStr">
         <is>
-          <t>Inspect revaluation/impairment routing + audit log + disposal recycling.</t>
+          <t>Inspect the float ceiling + the request→approve flow + the approver≠requester check + that the request posts nothing until approval.</t>
         </is>
       </c>
       <c r="O99" s="16" t="inlineStr">
         <is>
-          <t>Upward revaluation credits 3200; impairment debits 5820; no-change → NO_CHANGE; both events logged; on disposal the revaluation surplus is recycled to retained earnings (Dr 3200 / Cr 3100), not through P&amp;L (re-performed by the harness).</t>
+          <t>Re-perform: establish a fund (Dr 1015), request an expense (no GL), self-approve → SOD_VIOLATION, approve as a different user → Dr expense/Cr 1015 + fund down; over-balance draw → INSUFFICIENT_FLOAT; advance approve→settle clears 1180; replenish past float → OVER_FLOAT (re-performed by the harnesses).</t>
         </is>
       </c>
       <c r="P99" s="16" t="inlineStr">
         <is>
-          <t>Revaluation log; disposal recycling JE</t>
+          <t>Fund register + disbursement approval log + SoD test</t>
         </is>
       </c>
       <c r="Q99" s="18" t="inlineStr">
@@ -9496,7 +9496,7 @@
     <row r="100">
       <c r="A100" s="11" t="inlineStr">
         <is>
-          <t>FA-08</t>
+          <t>FA-07</t>
         </is>
       </c>
       <c r="B100" s="12" t="inlineStr">
@@ -9516,22 +9516,22 @@
       </c>
       <c r="E100" s="12" t="inlineStr">
         <is>
-          <t>Carrying amount changed by fair-value revaluation/impairment without independent review — the preparer revalues the asset and posts to equity/P&amp;L on their own (earnings/equity management).</t>
+          <t>Carrying amount not adjusted for revaluation/impairment — asset over/understated.</t>
         </is>
       </c>
       <c r="F100" s="12" t="inlineStr">
         <is>
-          <t>Authorization</t>
+          <t>Valuation</t>
         </is>
       </c>
       <c r="G100" s="12" t="inlineStr">
         <is>
-          <t>Asset-revaluation maker-checker (SoD): a revalue/impairment request posts its GL entry as a DRAFT (excluded from balances) and records status 'PendingApproval' WITHOUT moving the carrying value; a DIFFERENT user must approve before the JE is effective and the register is re-valued (approver ≠ preparer enforced regardless of permissions, reusing the GL-05 ledger approval). Reject voids the draft; only one revaluation may be pending per asset; the disposal surplus recycle counts only approved revaluations.</t>
+          <t>Asset revaluation / impairment: an upward revaluation credits the revaluation surplus in equity (Dr 1500 / Cr 3200); a downward revaluation (impairment) debits impairment loss (Dr 5820 / Cr 1500). The gross 1500 moves by the delta so the register stays tied to the GL; a no-op revaluation is rejected (NO_CHANGE). Every event is logged for the audit trail.</t>
         </is>
       </c>
       <c r="H100" s="13" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I100" s="13" t="inlineStr">
@@ -9556,22 +9556,22 @@
       </c>
       <c r="M100" s="12" t="inlineStr">
         <is>
-          <t>assets.service.ts revalue(pendingApproval Draft)/approveRevaluation/rejectRevaluation; assets.controller.ts (:assetNo/revalue/approve|reject); schema/assets.ts asset_revaluations.status + migration 0134; cutover/basics.ts + compliance.ts (ToE)</t>
+          <t>assets.service.ts (revalue up→3200 / down→5820, listRevaluations; dispose recycles surplus 3200→3100); assets.controller.ts (exec/creditors); schema/assets.ts (asset_revaluations) + migration 0120; cutover/basics.ts (ToE)</t>
         </is>
       </c>
       <c r="N100" s="12" t="inlineStr">
         <is>
-          <t>Inspect Draft→approve flow + the approver≠preparer check + deferred carrying-value update.</t>
+          <t>Inspect revaluation/impairment routing + audit log + disposal recycling.</t>
         </is>
       </c>
       <c r="O100" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: request a revaluation (Draft JE excluded from 3200), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm the surplus/impairment + carrying value move only after approval (re-performed by the harnesses).</t>
+          <t>Upward revaluation credits 3200; impairment debits 5820; no-change → NO_CHANGE; both events logged; on disposal the revaluation surplus is recycled to retained earnings (Dr 3200 / Cr 3100), not through P&amp;L (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P100" s="12" t="inlineStr">
         <is>
-          <t>Revaluation approval log + SoD test</t>
+          <t>Revaluation log; disposal recycling JE</t>
         </is>
       </c>
       <c r="Q100" s="18" t="inlineStr">
@@ -9583,12 +9583,12 @@
     <row r="101">
       <c r="A101" s="15" t="inlineStr">
         <is>
-          <t>LSE-01</t>
+          <t>FA-08</t>
         </is>
       </c>
       <c r="B101" s="16" t="inlineStr">
         <is>
-          <t>Leases</t>
+          <t>Fixed Assets</t>
         </is>
       </c>
       <c r="C101" s="17" t="inlineStr">
@@ -9598,27 +9598,27 @@
       </c>
       <c r="D101" s="16" t="inlineStr">
         <is>
-          <t>Right-of-use assets; Lease liabilities</t>
+          <t>Property, Plant &amp; Equipment; Equity</t>
         </is>
       </c>
       <c r="E101" s="16" t="inlineStr">
         <is>
-          <t>Lease not capitalised (IFRS 16 / TFRS 16) — ROU asset + lease liability omitted; interest/depreciation mis-stated.</t>
+          <t>Carrying amount changed by fair-value revaluation/impairment without independent review — the preparer revalues the asset and posts to equity/P&amp;L on their own (earnings/equity management).</t>
         </is>
       </c>
       <c r="F101" s="16" t="inlineStr">
         <is>
-          <t>Completeness/Accuracy/Valuation</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="G101" s="16" t="inlineStr">
         <is>
-          <t>Lease accounting: at commencement a right-of-use asset and lease liability are recognised at the present value of the lease payments (Dr 1600 / Cr 2600). The scheduled job lease_periodic_run posts each period — interest unwinding on the liability (Dr 5900), the cash payment reducing the liability (Dr 2600 / Cr 1000), and straight-line ROU depreciation (Dr 5210 / Cr 1690) — the last period clearing the liability + ROU exactly. Idempotent per (lease, period).</t>
+          <t>Asset-revaluation maker-checker (SoD): a revalue/impairment request posts its GL entry as a DRAFT (excluded from balances) and records status 'PendingApproval' WITHOUT moving the carrying value; a DIFFERENT user must approve before the JE is effective and the register is re-valued (approver ≠ preparer enforced regardless of permissions, reusing the GL-05 ledger approval). Reject voids the draft; only one revaluation may be pending per asset; the disposal surplus recycle counts only approved revaluations.</t>
         </is>
       </c>
       <c r="H101" s="17" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I101" s="17" t="inlineStr">
@@ -9628,12 +9628,12 @@
       </c>
       <c r="J101" s="17" t="inlineStr">
         <is>
-          <t>Per period / per lease</t>
+          <t>Per event</t>
         </is>
       </c>
       <c r="K101" s="16" t="inlineStr">
         <is>
-          <t>Controller</t>
+          <t>FaAccountant / Controller</t>
         </is>
       </c>
       <c r="L101" s="17" t="inlineStr">
@@ -9643,22 +9643,22 @@
       </c>
       <c r="M101" s="16" t="inlineStr">
         <is>
-          <t>leases.service.ts (createLease PV recognition, runDueLeases interest+payment+depreciation, modifyLease remeasurement); leases.controller.ts (gl_post); bi.service.ts (lease_periodic_run); schema/leases.ts (leases, rou_nbv) + migration 0120/0121; cutover/basics.ts (ToE)</t>
+          <t>assets.service.ts revalue(pendingApproval Draft)/approveRevaluation/rejectRevaluation; assets.controller.ts (:assetNo/revalue/approve|reject); schema/assets.ts asset_revaluations.status + migration 0134; cutover/basics.ts + compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N101" s="16" t="inlineStr">
         <is>
-          <t>Inspect PV recognition + periodic interest/payment/depreciation + final-period clearing + modification remeasurement.</t>
+          <t>Inspect Draft→approve flow + the approver≠preparer check + deferred carrying-value update.</t>
         </is>
       </c>
       <c r="O101" s="16" t="inlineStr">
         <is>
-          <t>Commencement recognises ROU=liability=PV; periodic run posts interest+principal(=payment)+ROU depreciation; liability + ROU reduce; a modification remeasures the liability at the revised PV and adjusts the ROU by the same delta (Dr/Cr 1600↔2600), then depreciates over the remaining term (re-performed by the harness).</t>
+          <t>Re-perform: request a revaluation (Draft JE excluded from 3200), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm the surplus/impairment + carrying value move only after approval (re-performed by the harnesses).</t>
         </is>
       </c>
       <c r="P101" s="16" t="inlineStr">
         <is>
-          <t>Lease register; periodic run log; modification remeasurement</t>
+          <t>Revaluation approval log + SoD test</t>
         </is>
       </c>
       <c r="Q101" s="18" t="inlineStr">
@@ -9670,12 +9670,12 @@
     <row r="102">
       <c r="A102" s="11" t="inlineStr">
         <is>
-          <t>REC-01</t>
+          <t>LSE-01</t>
         </is>
       </c>
       <c r="B102" s="12" t="inlineStr">
         <is>
-          <t>Reconciliation</t>
+          <t>Leases</t>
         </is>
       </c>
       <c r="C102" s="13" t="inlineStr">
@@ -9685,22 +9685,22 @@
       </c>
       <c r="D102" s="12" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Right-of-use assets; Lease liabilities</t>
         </is>
       </c>
       <c r="E102" s="12" t="inlineStr">
         <is>
-          <t>Subledgers diverge from GL undetected.</t>
+          <t>Lease not capitalised (IFRS 16 / TFRS 16) — ROU asset + lease liability omitted; interest/depreciation mis-stated.</t>
         </is>
       </c>
       <c r="F102" s="12" t="inlineStr">
         <is>
-          <t>Completeness/Accuracy</t>
+          <t>Completeness/Accuracy/Valuation</t>
         </is>
       </c>
       <c r="G102" s="12" t="inlineStr">
         <is>
-          <t>Subledger-to-GL reconciliation per period: import GL, auto-match, certify (sign-off via 'approvals').</t>
+          <t>Lease accounting: at commencement a right-of-use asset and lease liability are recognised at the present value of the lease payments (Dr 1600 / Cr 2600). The scheduled job lease_periodic_run posts each period — interest unwinding on the liability (Dr 5900), the cash payment reducing the liability (Dr 2600 / Cr 1000), and straight-line ROU depreciation (Dr 5210 / Cr 1690) — the last period clearing the liability + ROU exactly. Idempotent per (lease, period).</t>
         </is>
       </c>
       <c r="H102" s="13" t="inlineStr">
@@ -9710,12 +9710,12 @@
       </c>
       <c r="I102" s="13" t="inlineStr">
         <is>
-          <t>Auto+Manual</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J102" s="13" t="inlineStr">
         <is>
-          <t>Monthly</t>
+          <t>Per period / per lease</t>
         </is>
       </c>
       <c r="K102" s="12" t="inlineStr">
@@ -9725,27 +9725,27 @@
       </c>
       <c r="L102" s="13" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="M102" s="12" t="inlineStr">
         <is>
-          <t>reconciliation.service.ts (importGlItems/autoMatch/certify)</t>
+          <t>leases.service.ts (createLease PV recognition, runDueLeases interest+payment+depreciation, modifyLease remeasurement); leases.controller.ts (gl_post); bi.service.ts (lease_periodic_run); schema/leases.ts (leases, rou_nbv) + migration 0120/0121; cutover/basics.ts (ToE)</t>
         </is>
       </c>
       <c r="N102" s="12" t="inlineStr">
         <is>
-          <t>Inspect recon + certify gate.</t>
+          <t>Inspect PV recognition + periodic interest/payment/depreciation + final-period clearing + modification remeasurement.</t>
         </is>
       </c>
       <c r="O102" s="12" t="inlineStr">
         <is>
-          <t>Sample periods: reconciled, unmatched cleared, certified.</t>
+          <t>Commencement recognises ROU=liability=PV; periodic run posts interest+principal(=payment)+ROU depreciation; liability + ROU reduce; a modification remeasures the liability at the revised PV and adjusts the ROU by the same delta (Dr/Cr 1600↔2600), then depreciates over the remaining term (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P102" s="12" t="inlineStr">
         <is>
-          <t>Certified recon</t>
+          <t>Lease register; periodic run log; modification remeasurement</t>
         </is>
       </c>
       <c r="Q102" s="18" t="inlineStr">
@@ -9757,7 +9757,7 @@
     <row r="103">
       <c r="A103" s="15" t="inlineStr">
         <is>
-          <t>REC-02</t>
+          <t>REC-01</t>
         </is>
       </c>
       <c r="B103" s="16" t="inlineStr">
@@ -9772,22 +9772,22 @@
       </c>
       <c r="D103" s="16" t="inlineStr">
         <is>
-          <t>Cash</t>
+          <t>All</t>
         </is>
       </c>
       <c r="E103" s="16" t="inlineStr">
         <is>
-          <t>Bank balance not reconciled to GL.</t>
+          <t>Subledgers diverge from GL undetected.</t>
         </is>
       </c>
       <c r="F103" s="16" t="inlineStr">
         <is>
-          <t>Existence/Completeness</t>
+          <t>Completeness/Accuracy</t>
         </is>
       </c>
       <c r="G103" s="16" t="inlineStr">
         <is>
-          <t>Bank reconciliation against statements.</t>
+          <t>Subledger-to-GL reconciliation per period: import GL, auto-match, certify (sign-off via 'approvals').</t>
         </is>
       </c>
       <c r="H103" s="17" t="inlineStr">
@@ -9817,22 +9817,22 @@
       </c>
       <c r="M103" s="16" t="inlineStr">
         <is>
-          <t>bank module; drizzle/0015_bank_reconciliation</t>
+          <t>reconciliation.service.ts (importGlItems/autoMatch/certify)</t>
         </is>
       </c>
       <c r="N103" s="16" t="inlineStr">
         <is>
-          <t>Inspect bank-rec process.</t>
+          <t>Inspect recon + certify gate.</t>
         </is>
       </c>
       <c r="O103" s="16" t="inlineStr">
         <is>
-          <t>Sample months reconciled &amp; reviewed.</t>
+          <t>Sample periods: reconciled, unmatched cleared, certified.</t>
         </is>
       </c>
       <c r="P103" s="16" t="inlineStr">
         <is>
-          <t>Bank rec</t>
+          <t>Certified recon</t>
         </is>
       </c>
       <c r="Q103" s="18" t="inlineStr">
@@ -9844,12 +9844,12 @@
     <row r="104">
       <c r="A104" s="11" t="inlineStr">
         <is>
-          <t>BANK-02</t>
+          <t>REC-02</t>
         </is>
       </c>
       <c r="B104" s="12" t="inlineStr">
         <is>
-          <t>Cash &amp; Treasury</t>
+          <t>Reconciliation</t>
         </is>
       </c>
       <c r="C104" s="13" t="inlineStr">
@@ -9859,37 +9859,37 @@
       </c>
       <c r="D104" s="12" t="inlineStr">
         <is>
-          <t>Cash; Operating expense; Interest income</t>
+          <t>Cash</t>
         </is>
       </c>
       <c r="E104" s="12" t="inlineStr">
         <is>
-          <t>A bank fee/interest adjustment is posted straight to the GL by one person during reconciliation — a cash outflow mis-booked as interest income, or a fictitious fee posted, with no independent review (single-person posting to the cash account).</t>
+          <t>Bank balance not reconciled to GL.</t>
         </is>
       </c>
       <c r="F104" s="12" t="inlineStr">
         <is>
-          <t>Authorization/Accuracy</t>
+          <t>Existence/Completeness</t>
         </is>
       </c>
       <c r="G104" s="12" t="inlineStr">
         <is>
-          <t>Bank adjustment maker-checker (SoD): a fee/interest adjustment on a statement line is a REQUEST that posts a DRAFT JE (no balance/GL effect; the line stays unreconciled) until a DIFFERENT user with approval authority approves (POST /api/bank/lines/:id/adjustment/approve). Self-approval → SOD_VIOLATION (binds even Admin); approval flips the line to reconciled and the JE to Posted; reject voids the Draft and frees the line. The Draft JE (source BANKADJ) is also surfaced, aged, by the pending-approvals monitor (GOV-01).</t>
+          <t>Bank reconciliation against statements.</t>
         </is>
       </c>
       <c r="H104" s="13" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I104" s="13" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="J104" s="13" t="inlineStr">
         <is>
-          <t>Per adjustment</t>
+          <t>Monthly</t>
         </is>
       </c>
       <c r="K104" s="12" t="inlineStr">
@@ -9899,27 +9899,27 @@
       </c>
       <c r="L104" s="13" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="M104" s="12" t="inlineStr">
         <is>
-          <t>bank.service.ts requestAdjustment/approveAdjustment/rejectAdjustment/listPendingAdjustments (reuses ledger.approveEntry SoD); bank.controller.ts (lines/:id/adjustment requests; adjustment/approve|reject gated approvals/gl_close); cutover/bankrec.ts (ToE)</t>
+          <t>bank module; drizzle/0015_bank_reconciliation</t>
         </is>
       </c>
       <c r="N104" s="12" t="inlineStr">
         <is>
-          <t>Inspect the request→approve flow + the approver≠requester check + that the Draft posts nothing until approval.</t>
+          <t>Inspect bank-rec process.</t>
         </is>
       </c>
       <c r="O104" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: request a fee adjustment (line unreconciled, GL difference unchanged), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm the difference closes to 0 only after approval (re-performed by the bankrec harness).</t>
+          <t>Sample months reconciled &amp; reviewed.</t>
         </is>
       </c>
       <c r="P104" s="12" t="inlineStr">
         <is>
-          <t>Bank adjustment queue + SoD test</t>
+          <t>Bank rec</t>
         </is>
       </c>
       <c r="Q104" s="18" t="inlineStr">
@@ -9931,12 +9931,12 @@
     <row r="105">
       <c r="A105" s="15" t="inlineStr">
         <is>
-          <t>REC-03</t>
+          <t>BANK-02</t>
         </is>
       </c>
       <c r="B105" s="16" t="inlineStr">
         <is>
-          <t>Reconciliation</t>
+          <t>Cash &amp; Treasury</t>
         </is>
       </c>
       <c r="C105" s="17" t="inlineStr">
@@ -9946,79 +9946,79 @@
       </c>
       <c r="D105" s="16" t="inlineStr">
         <is>
-          <t>Consolidation</t>
+          <t>Cash; Operating expense; Interest income</t>
         </is>
       </c>
       <c r="E105" s="16" t="inlineStr">
         <is>
-          <t>Intercompany balances not eliminated/agreed.</t>
+          <t>A bank fee/interest adjustment is posted straight to the GL by one person during reconciliation — a cash outflow mis-booked as interest income, or a fictitious fee posted, with no independent review (single-person posting to the cash account).</t>
         </is>
       </c>
       <c r="F105" s="16" t="inlineStr">
         <is>
-          <t>Accuracy</t>
+          <t>Authorization/Accuracy</t>
         </is>
       </c>
       <c r="G105" s="16" t="inlineStr">
         <is>
-          <t>Intercompany reconciliation &amp; elimination on consolidation.</t>
+          <t>Bank adjustment maker-checker (SoD): a fee/interest adjustment on a statement line is a REQUEST that posts a DRAFT JE (no balance/GL effect; the line stays unreconciled) until a DIFFERENT user with approval authority approves (POST /api/bank/lines/:id/adjustment/approve). Self-approval → SOD_VIOLATION (binds even Admin); approval flips the line to reconciled and the JE to Posted; reject voids the Draft and frees the line. The Draft JE (source BANKADJ) is also surfaced, aged, by the pending-approvals monitor (GOV-01).</t>
         </is>
       </c>
       <c r="H105" s="17" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I105" s="17" t="inlineStr">
         <is>
-          <t>Auto+Manual</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J105" s="17" t="inlineStr">
         <is>
-          <t>Period</t>
+          <t>Per adjustment</t>
         </is>
       </c>
       <c r="K105" s="16" t="inlineStr">
         <is>
-          <t>Group Controller</t>
+          <t>Controller</t>
         </is>
       </c>
       <c r="L105" s="17" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="M105" s="16" t="inlineStr">
         <is>
-          <t>intercompany; consolidation</t>
+          <t>bank.service.ts requestAdjustment/approveAdjustment/rejectAdjustment/listPendingAdjustments (reuses ledger.approveEntry SoD); bank.controller.ts (lines/:id/adjustment requests; adjustment/approve|reject gated approvals/gl_close); cutover/bankrec.ts (ToE)</t>
         </is>
       </c>
       <c r="N105" s="16" t="inlineStr">
         <is>
-          <t>Inspect IC matching + elimination.</t>
+          <t>Inspect the request→approve flow + the approver≠requester check + that the Draft posts nothing until approval.</t>
         </is>
       </c>
       <c r="O105" s="16" t="inlineStr">
         <is>
-          <t>Sample IC pairs agree &amp; eliminate.</t>
+          <t>Re-perform: request a fee adjustment (line unreconciled, GL difference unchanged), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm the difference closes to 0 only after approval (re-performed by the bankrec harness).</t>
         </is>
       </c>
       <c r="P105" s="16" t="inlineStr">
         <is>
-          <t>IC recon</t>
-        </is>
-      </c>
-      <c r="Q105" s="19" t="inlineStr">
-        <is>
-          <t>Partial</t>
+          <t>Bank adjustment queue + SoD test</t>
+        </is>
+      </c>
+      <c r="Q105" s="18" t="inlineStr">
+        <is>
+          <t>Implemented</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="11" t="inlineStr">
         <is>
-          <t>REC-04</t>
+          <t>REC-03</t>
         </is>
       </c>
       <c r="B106" s="12" t="inlineStr">
@@ -10033,22 +10033,22 @@
       </c>
       <c r="D106" s="12" t="inlineStr">
         <is>
-          <t>All control accounts</t>
+          <t>Consolidation</t>
         </is>
       </c>
       <c r="E106" s="12" t="inlineStr">
         <is>
-          <t>A sub-ledger silently drifts from its GL control account at period-end and no single review catches it (incomplete/inaccurate balances reach the financial statements).</t>
+          <t>Intercompany balances not eliminated/agreed.</t>
         </is>
       </c>
       <c r="F106" s="12" t="inlineStr">
         <is>
-          <t>Completeness/Accuracy</t>
+          <t>Accuracy</t>
         </is>
       </c>
       <c r="G106" s="12" t="inlineStr">
         <is>
-          <t>Period-end control-account reconciliation PACK: one read (GET /api/finance/reconciliation/controls) ties every major sub-ledger to its GL control account and FLAGS any out-of-balance — AR↔1100, AP↔2000, Inventory↔1200, Gift cards/Customer-deposits↔2200, Deferred revenue↔2400 — reporting per line {sub_ledger, gl_control, variance, reconciled} plus an overall all_reconciled flag and an exceptions count. Liability controls are sign-flipped before comparison. The controller's single 'are the books reconciled?' close view; an exception is a control finding to investigate before sign-off.</t>
+          <t>Intercompany reconciliation &amp; elimination on consolidation.</t>
         </is>
       </c>
       <c r="H106" s="13" t="inlineStr">
@@ -10058,17 +10058,17 @@
       </c>
       <c r="I106" s="13" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="J106" s="13" t="inlineStr">
         <is>
-          <t>Period / on demand</t>
+          <t>Period</t>
         </is>
       </c>
       <c r="K106" s="12" t="inlineStr">
         <is>
-          <t>Controller / CFO</t>
+          <t>Group Controller</t>
         </is>
       </c>
       <c r="L106" s="13" t="inlineStr">
@@ -10078,34 +10078,34 @@
       </c>
       <c r="M106" s="12" t="inlineStr">
         <is>
-          <t>finance.service.ts reconcileControls; finance.controller.ts GET reconciliation/controls (exec/ar/creditors); reuses ledger.trialBalance + the AR/AP/inventory/gift-card/deferred sub-ledgers; cutover/giftcards.ts + compliance.ts (ToE)</t>
+          <t>intercompany; consolidation</t>
         </is>
       </c>
       <c r="N106" s="12" t="inlineStr">
         <is>
-          <t>Inspect the pack: each control account's sub-ledger query + the GL tie + the exceptions roll-up.</t>
+          <t>Inspect IC matching + elimination.</t>
         </is>
       </c>
       <c r="O106" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: with a clean set, every line reconciled + all_reconciled=true; introduce a known sub-ledger/GL difference and confirm it surfaces as an exception (re-performed: gift-card 2200 + inventory 1200 ties asserted by the harnesses).</t>
+          <t>Sample IC pairs agree &amp; eliminate.</t>
         </is>
       </c>
       <c r="P106" s="12" t="inlineStr">
         <is>
-          <t>Reconciliation pack; exceptions list</t>
-        </is>
-      </c>
-      <c r="Q106" s="18" t="inlineStr">
-        <is>
-          <t>Implemented</t>
+          <t>IC recon</t>
+        </is>
+      </c>
+      <c r="Q106" s="19" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="15" t="inlineStr">
         <is>
-          <t>REC-05</t>
+          <t>REC-04</t>
         </is>
       </c>
       <c r="B107" s="16" t="inlineStr">
@@ -10120,42 +10120,42 @@
       </c>
       <c r="D107" s="16" t="inlineStr">
         <is>
-          <t>Cash; Bank</t>
+          <t>All control accounts</t>
         </is>
       </c>
       <c r="E107" s="16" t="inlineStr">
         <is>
-          <t>Till cash dropped to the safe never reaches the bank, or a deposit isn't matched to the statement — cash sits unbanked (theft/loss exposure) or the bank balance can't be tied to the books.</t>
+          <t>A sub-ledger silently drifts from its GL control account at period-end and no single review catches it (incomplete/inaccurate balances reach the financial statements).</t>
         </is>
       </c>
       <c r="F107" s="16" t="inlineStr">
         <is>
-          <t>Completeness/Existence/Authorization</t>
+          <t>Completeness/Accuracy</t>
         </is>
       </c>
       <c r="G107" s="16" t="inlineStr">
         <is>
-          <t>Cash banking — safe-drop → bank deposit → reconciliation: till 'drop's move cash from the drawer to the safe (drawer-only, no GL). Banking BATCHES the undeposited drops into a deposit and posts the GL (Dr &lt;bank account, e.g. 1010&gt; / Cr 1000 Cash), stamping each drop with the deposit id; the deposit is then RECONCILED to the bank statement (status Deposited→Reconciled). A detective read (GET /api/bank/deposits/undeposited-drops) surfaces the CASH STILL IN THE SAFE (drops with deposit_id NULL) — the unbanked exposure to chase. SoD: banking is a treasury duty (exec/ar) — segregated from the cashier (pos_till) who drops the cash, so the person who removes cash from the drawer is not the one who banks it.</t>
+          <t>Period-end control-account reconciliation PACK: one read (GET /api/finance/reconciliation/controls) ties every major sub-ledger to its GL control account and FLAGS any out-of-balance — AR↔1100, AP↔2000, Inventory↔1200, Gift cards/Customer-deposits↔2200, Deferred revenue↔2400 — reporting per line {sub_ledger, gl_control, variance, reconciled} plus an overall all_reconciled flag and an exceptions count. Liability controls are sign-flipped before comparison. The controller's single 'are the books reconciled?' close view; an exception is a control finding to investigate before sign-off.</t>
         </is>
       </c>
       <c r="H107" s="17" t="inlineStr">
         <is>
-          <t>Det/Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I107" s="17" t="inlineStr">
         <is>
-          <t>Auto+Manual</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J107" s="17" t="inlineStr">
         <is>
-          <t>Per banking run</t>
+          <t>Period / on demand</t>
         </is>
       </c>
       <c r="K107" s="16" t="inlineStr">
         <is>
-          <t>FinancialController / Treasury</t>
+          <t>Controller / CFO</t>
         </is>
       </c>
       <c r="L107" s="17" t="inlineStr">
@@ -10165,22 +10165,22 @@
       </c>
       <c r="M107" s="16" t="inlineStr">
         <is>
-          <t>bank.service.ts undepositedDrops/createDeposit (Dr bank/Cr 1000, stamps deposit_id)/reconcileDeposit/listDeposits; bank.controller.ts (deposits, deposits/undeposited-drops, deposits/:id/reconcile; exec/ar); schema/cash.ts bank_deposits + cash_movements.deposit_id + migration 0152; /cash-banking UI; cutover/cash-banking.ts (ToE)</t>
+          <t>finance.service.ts reconcileControls; finance.controller.ts GET reconciliation/controls (exec/ar/creditors); reuses ledger.trialBalance + the AR/AP/inventory/gift-card/deferred sub-ledgers; cutover/giftcards.ts + compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N107" s="16" t="inlineStr">
         <is>
-          <t>Inspect the undeposited-drop exposure read + the deposit GL (bank↔1000) + the reconcile step + the SoD (cashier vs treasury).</t>
+          <t>Inspect the pack: each control account's sub-ledger query + the GL tie + the exceptions roll-up.</t>
         </is>
       </c>
       <c r="O107" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: two till drops → cash-in-safe shows the total; a cashier (pos_till) cannot bank (403); treasury banks → Dr bank / Cr 1000, cash-in-safe back to 0; reconcile the deposit; trial balance balanced (re-performed by the cash-banking harness).</t>
+          <t>Re-perform: with a clean set, every line reconciled + all_reconciled=true; introduce a known sub-ledger/GL difference and confirm it surfaces as an exception (re-performed: gift-card 2200 + inventory 1200 ties asserted by the harnesses).</t>
         </is>
       </c>
       <c r="P107" s="16" t="inlineStr">
         <is>
-          <t>Bank-deposit register; undeposited-drop (cash-in-safe) exposure</t>
+          <t>Reconciliation pack; exceptions list</t>
         </is>
       </c>
       <c r="Q107" s="18" t="inlineStr">
@@ -10192,12 +10192,12 @@
     <row r="108">
       <c r="A108" s="11" t="inlineStr">
         <is>
-          <t>GOV-01</t>
+          <t>REC-05</t>
         </is>
       </c>
       <c r="B108" s="12" t="inlineStr">
         <is>
-          <t>Monitoring</t>
+          <t>Reconciliation</t>
         </is>
       </c>
       <c r="C108" s="13" t="inlineStr">
@@ -10207,42 +10207,42 @@
       </c>
       <c r="D108" s="12" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Cash; Bank</t>
         </is>
       </c>
       <c r="E108" s="12" t="inlineStr">
         <is>
-          <t>A maker-checker approval sits un-actioned and is forgotten — a transaction stalls before it is effective, or (worse) a control is quietly bypassed and no one notices an item never got its independent review.</t>
+          <t>Till cash dropped to the safe never reaches the bank, or a deposit isn't matched to the statement — cash sits unbanked (theft/loss exposure) or the bank balance can't be tied to the books.</t>
         </is>
       </c>
       <c r="F108" s="12" t="inlineStr">
         <is>
-          <t>Authorization/Completeness</t>
+          <t>Completeness/Existence/Authorization</t>
         </is>
       </c>
       <c r="G108" s="12" t="inlineStr">
         <is>
-          <t>Pending-approvals MONITOR (COSO monitoring): a single worklist of EVERY item awaiting independent approval across the system, each with its AGE in days and an overdue roll-up — spanning the manual-JE (GL-05), bank-adjustment (BANK-02), AP-disbursement (EXP-06), payroll (PAY-03), asset-revaluation (FA-08), asset-disposal (FA-09), inventory-write-off (INV-07), till-close cash over/short (REV-13), FX-rate (FX-04), budget (BUD-01) and large-refund (REV-16) maker-checkers. The controller reviews it before close; a stale item (age beyond the threshold) is a control finding to chase or escalate. The /approvals screen also lets a manager approve/reject a material till variance or a large refund inline (the pending types with no dedicated module screen). Read-only worklist; tenant-scoped via the caller's RLS.</t>
+          <t>Cash banking — safe-drop → bank deposit → reconciliation: till 'drop's move cash from the drawer to the safe (drawer-only, no GL). Banking BATCHES the undeposited drops into a deposit and posts the GL (Dr &lt;bank account, e.g. 1010&gt; / Cr 1000 Cash), stamping each drop with the deposit id; the deposit is then RECONCILED to the bank statement (status Deposited→Reconciled). A detective read (GET /api/bank/deposits/undeposited-drops) surfaces the CASH STILL IN THE SAFE (drops with deposit_id NULL) — the unbanked exposure to chase. SoD: banking is a treasury duty (exec/ar) — segregated from the cashier (pos_till) who drops the cash, so the person who removes cash from the drawer is not the one who banks it.</t>
         </is>
       </c>
       <c r="H108" s="13" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Det/Prev</t>
         </is>
       </c>
       <c r="I108" s="13" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="J108" s="13" t="inlineStr">
         <is>
-          <t>Continuous / pre-close</t>
+          <t>Per banking run</t>
         </is>
       </c>
       <c r="K108" s="12" t="inlineStr">
         <is>
-          <t>Controller / CFO</t>
+          <t>FinancialController / Treasury</t>
         </is>
       </c>
       <c r="L108" s="13" t="inlineStr">
@@ -10252,22 +10252,22 @@
       </c>
       <c r="M108" s="12" t="inlineStr">
         <is>
-          <t>finance.service.ts pendingApprovals; finance.controller.ts GET approvals/pending (exec/approvals/creditors); aggregates journalEntries(Draft incl. BANKADJ→BANK-02)/apPayments/payruns/asset_revaluations/fixed_assets(disposal_pending)/inv_writeoff_requests/till_sessions(PendingApproval)/fx_rates(PendingApproval)/budgets(PendingApproval); cutover/compliance.ts (ToE)</t>
+          <t>bank.service.ts undepositedDrops/createDeposit (Dr bank/Cr 1000, stamps deposit_id)/reconcileDeposit/listDeposits; bank.controller.ts (deposits, deposits/undeposited-drops, deposits/:id/reconcile; exec/ar); schema/cash.ts bank_deposits + cash_movements.deposit_id + migration 0152; /cash-banking UI; cutover/cash-banking.ts (ToE)</t>
         </is>
       </c>
       <c r="N108" s="12" t="inlineStr">
         <is>
-          <t>Inspect the aggregation across all pending sources + the age/overdue roll-up.</t>
+          <t>Inspect the undeposited-drop exposure read + the deposit GL (bank↔1000) + the reconcile step + the SoD (cashier vs treasury).</t>
         </is>
       </c>
       <c r="O108" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: create a pending item (e.g. a Draft JE) and confirm it appears in the worklist with its control ID, amount and age; the overdue count flags items past the threshold (re-performed by the harness).</t>
+          <t>Re-perform: two till drops → cash-in-safe shows the total; a cashier (pos_till) cannot bank (403); treasury banks → Dr bank / Cr 1000, cash-in-safe back to 0; reconcile the deposit; trial balance balanced (re-performed by the cash-banking harness).</t>
         </is>
       </c>
       <c r="P108" s="12" t="inlineStr">
         <is>
-          <t>Pending-approvals worklist</t>
+          <t>Bank-deposit register; undeposited-drop (cash-in-safe) exposure</t>
         </is>
       </c>
       <c r="Q108" s="18" t="inlineStr">
@@ -10279,12 +10279,12 @@
     <row r="109">
       <c r="A109" s="15" t="inlineStr">
         <is>
-          <t>TAX-01</t>
+          <t>GOV-01</t>
         </is>
       </c>
       <c r="B109" s="16" t="inlineStr">
         <is>
-          <t>Tax</t>
+          <t>Monitoring</t>
         </is>
       </c>
       <c r="C109" s="17" t="inlineStr">
@@ -10294,27 +10294,27 @@
       </c>
       <c r="D109" s="16" t="inlineStr">
         <is>
-          <t>Tax (VAT)</t>
+          <t>All</t>
         </is>
       </c>
       <c r="E109" s="16" t="inlineStr">
         <is>
-          <t>VAT computed incorrectly → filing/penalty risk.</t>
+          <t>A maker-checker approval sits un-actioned and is forgotten — a transaction stalls before it is effective, or (worse) a control is quietly bypassed and no one notices an item never got its independent review.</t>
         </is>
       </c>
       <c r="F109" s="16" t="inlineStr">
         <is>
-          <t>Accuracy</t>
+          <t>Authorization/Completeness</t>
         </is>
       </c>
       <c r="G109" s="16" t="inlineStr">
         <is>
-          <t>VAT via pluggable provider (TH 7%); unit-tested; no hard-coded rate.</t>
+          <t>Pending-approvals MONITOR (COSO monitoring): a single worklist of EVERY item awaiting independent approval across the system, each with its AGE in days and an overdue roll-up — spanning the manual-JE (GL-05), bank-adjustment (BANK-02), AP-disbursement (EXP-06), payroll (PAY-03), asset-revaluation (FA-08), asset-disposal (FA-09), inventory-write-off (INV-07), till-close cash over/short (REV-13), FX-rate (FX-04), budget (BUD-01) and large-refund (REV-16) maker-checkers. The controller reviews it before close; a stale item (age beyond the threshold) is a control finding to chase or escalate. The /approvals screen also lets a manager approve/reject a material till variance or a large refund inline (the pending types with no dedicated module screen). Read-only worklist; tenant-scoped via the caller's RLS.</t>
         </is>
       </c>
       <c r="H109" s="17" t="inlineStr">
         <is>
-          <t>Auto</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I109" s="17" t="inlineStr">
@@ -10324,37 +10324,37 @@
       </c>
       <c r="J109" s="17" t="inlineStr">
         <is>
-          <t>Per txn</t>
+          <t>Continuous / pre-close</t>
         </is>
       </c>
       <c r="K109" s="16" t="inlineStr">
         <is>
-          <t>Tax / Controller</t>
+          <t>Controller / CFO</t>
         </is>
       </c>
       <c r="L109" s="17" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="M109" s="16" t="inlineStr">
         <is>
-          <t>tax/tax-providers.ts; tax.service.ts; test/unit.test.ts</t>
+          <t>finance.service.ts pendingApprovals; finance.controller.ts GET approvals/pending (exec/approvals/creditors); aggregates journalEntries(Draft incl. BANKADJ→BANK-02)/apPayments/payruns/asset_revaluations/fixed_assets(disposal_pending)/inv_writeoff_requests/till_sessions(PendingApproval)/fx_rates(PendingApproval)/budgets(PendingApproval); cutover/compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N109" s="16" t="inlineStr">
         <is>
-          <t>Inspect rate provider + tests.</t>
+          <t>Inspect the aggregation across all pending sources + the age/overdue roll-up.</t>
         </is>
       </c>
       <c r="O109" s="16" t="inlineStr">
         <is>
-          <t>Re-perform VAT on sample; tie to return.</t>
+          <t>Re-perform: create a pending item (e.g. a Draft JE) and confirm it appears in the worklist with its control ID, amount and age; the overdue count flags items past the threshold (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P109" s="16" t="inlineStr">
         <is>
-          <t>VAT tests</t>
+          <t>Pending-approvals worklist</t>
         </is>
       </c>
       <c r="Q109" s="18" t="inlineStr">
@@ -10366,7 +10366,7 @@
     <row r="110">
       <c r="A110" s="11" t="inlineStr">
         <is>
-          <t>TAX-02</t>
+          <t>TAX-01</t>
         </is>
       </c>
       <c r="B110" s="12" t="inlineStr">
@@ -10381,22 +10381,22 @@
       </c>
       <c r="D110" s="12" t="inlineStr">
         <is>
-          <t>Tax; Revenue</t>
+          <t>Tax (VAT)</t>
         </is>
       </c>
       <c r="E110" s="12" t="inlineStr">
         <is>
-          <t>Non-compliant e-Tax invoice / not transmitted to ETDA.</t>
+          <t>VAT computed incorrectly → filing/penalty risk.</t>
         </is>
       </c>
       <c r="F110" s="12" t="inlineStr">
         <is>
-          <t>Accuracy/Compliance</t>
+          <t>Accuracy</t>
         </is>
       </c>
       <c r="G110" s="12" t="inlineStr">
         <is>
-          <t>e-Tax invoice (ETDA UBL 2.1 XML) generation + email with CC to ETDA timestamp mailbox.</t>
+          <t>VAT via pluggable provider (TH 7%); unit-tested; no hard-coded rate.</t>
         </is>
       </c>
       <c r="H110" s="13" t="inlineStr">
@@ -10411,37 +10411,37 @@
       </c>
       <c r="J110" s="13" t="inlineStr">
         <is>
-          <t>Per invoice</t>
+          <t>Per txn</t>
         </is>
       </c>
       <c r="K110" s="12" t="inlineStr">
         <is>
-          <t>Tax</t>
+          <t>Tax / Controller</t>
         </is>
       </c>
       <c r="L110" s="13" t="inlineStr">
         <is>
-          <t>P10/P13</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="M110" s="12" t="inlineStr">
         <is>
-          <t>tax-docs/etax-xml.ts; etax-email.service.ts (tested)</t>
+          <t>tax/tax-providers.ts; tax.service.ts; test/unit.test.ts</t>
         </is>
       </c>
       <c r="N110" s="12" t="inlineStr">
         <is>
-          <t>Inspect XML schema + email composer.</t>
+          <t>Inspect rate provider + tests.</t>
         </is>
       </c>
       <c r="O110" s="12" t="inlineStr">
         <is>
-          <t>Sample invoices: valid XML, correct CC/escaping.</t>
+          <t>Re-perform VAT on sample; tie to return.</t>
         </is>
       </c>
       <c r="P110" s="12" t="inlineStr">
         <is>
-          <t>e-Tax samples</t>
+          <t>VAT tests</t>
         </is>
       </c>
       <c r="Q110" s="18" t="inlineStr">
@@ -10453,7 +10453,7 @@
     <row r="111">
       <c r="A111" s="15" t="inlineStr">
         <is>
-          <t>TAX-03</t>
+          <t>TAX-02</t>
         </is>
       </c>
       <c r="B111" s="16" t="inlineStr">
@@ -10468,22 +10468,22 @@
       </c>
       <c r="D111" s="16" t="inlineStr">
         <is>
-          <t>Tax (WHT)</t>
+          <t>Tax; Revenue</t>
         </is>
       </c>
       <c r="E111" s="16" t="inlineStr">
         <is>
-          <t>Withholding tax mis-computed / not reported.</t>
+          <t>Non-compliant e-Tax invoice / not transmitted to ETDA.</t>
         </is>
       </c>
       <c r="F111" s="16" t="inlineStr">
         <is>
-          <t>Accuracy</t>
+          <t>Accuracy/Compliance</t>
         </is>
       </c>
       <c r="G111" s="16" t="inlineStr">
         <is>
-          <t>WHT computation and ภ.ง.ด. reporting.</t>
+          <t>e-Tax invoice (ETDA UBL 2.1 XML) generation + email with CC to ETDA timestamp mailbox.</t>
         </is>
       </c>
       <c r="H111" s="17" t="inlineStr">
@@ -10498,7 +10498,7 @@
       </c>
       <c r="J111" s="17" t="inlineStr">
         <is>
-          <t>Per txn / monthly</t>
+          <t>Per invoice</t>
         </is>
       </c>
       <c r="K111" s="16" t="inlineStr">
@@ -10508,39 +10508,39 @@
       </c>
       <c r="L111" s="17" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P10/P13</t>
         </is>
       </c>
       <c r="M111" s="16" t="inlineStr">
         <is>
-          <t>tax-reports; payroll</t>
+          <t>tax-docs/etax-xml.ts; etax-email.service.ts (tested)</t>
         </is>
       </c>
       <c r="N111" s="16" t="inlineStr">
         <is>
-          <t>Inspect WHT logic + report.</t>
+          <t>Inspect XML schema + email composer.</t>
         </is>
       </c>
       <c r="O111" s="16" t="inlineStr">
         <is>
-          <t>Re-perform WHT on sample; tie to filing.</t>
+          <t>Sample invoices: valid XML, correct CC/escaping.</t>
         </is>
       </c>
       <c r="P111" s="16" t="inlineStr">
         <is>
-          <t>WHT report</t>
-        </is>
-      </c>
-      <c r="Q111" s="19" t="inlineStr">
-        <is>
-          <t>Partial</t>
+          <t>e-Tax samples</t>
+        </is>
+      </c>
+      <c r="Q111" s="18" t="inlineStr">
+        <is>
+          <t>Implemented</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="11" t="inlineStr">
         <is>
-          <t>TAX-04</t>
+          <t>TAX-03</t>
         </is>
       </c>
       <c r="B112" s="12" t="inlineStr">
@@ -10555,27 +10555,27 @@
       </c>
       <c r="D112" s="12" t="inlineStr">
         <is>
-          <t>Tax (VAT); Tax Payable (2100)</t>
+          <t>Tax (WHT)</t>
         </is>
       </c>
       <c r="E112" s="12" t="inlineStr">
         <is>
-          <t>Output/input VAT on the filed ภ.พ.30 return does not agree to the GL — VAT liability mis-stated, a filing/penalty exposure, or a posting omission goes undetected before submission.</t>
+          <t>Withholding tax mis-computed / not reported.</t>
         </is>
       </c>
       <c r="F112" s="12" t="inlineStr">
         <is>
-          <t>Completeness/Accuracy</t>
+          <t>Accuracy</t>
         </is>
       </c>
       <c r="G112" s="12" t="inlineStr">
         <is>
-          <t>Periodic VAT-return ↔ GL reconciliation (ภ.พ.30): the monthly return (GET /api/tax-reports/pp30) is built from the sales/output-VAT and purchase/input-VAT sub-reports, computes net VAT = output − input, and RECONCILES it to the **GL account 2100 (Tax Payable) net movement** for the same period (Σ credit − Σ debit over Posted entries) — returning `reconciliation.tied` = true only when the two agree within rounding. A non-tie is a detective finding to investigate and clear BEFORE filing (the form also carries the ม.157 deadline = the 15th of the next month). Output VAT is posted to 2100 on every sale (Cr) and reversed on returns (Dr); input VAT is posted on AP bills (Dr) — so 2100's net is the period's VAT payable. Read-only report; exportable to a ภ.พ.30 PDF/HTML.</t>
+          <t>WHT computation and ภ.ง.ด. reporting.</t>
         </is>
       </c>
       <c r="H112" s="13" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Auto</t>
         </is>
       </c>
       <c r="I112" s="13" t="inlineStr">
@@ -10585,54 +10585,54 @@
       </c>
       <c r="J112" s="13" t="inlineStr">
         <is>
-          <t>Monthly / pre-filing</t>
+          <t>Per txn / monthly</t>
         </is>
       </c>
       <c r="K112" s="12" t="inlineStr">
         <is>
-          <t>Tax / FinancialController</t>
+          <t>Tax</t>
         </is>
       </c>
       <c r="L112" s="13" t="inlineStr">
         <is>
-          <t>P10/P16</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="M112" s="12" t="inlineStr">
         <is>
-          <t>tax-reports.service.ts pp30 (outputVat/inputVat + 2100 net-movement tie); tax-reports.controller.ts (GET pp30, pp30/export, exec); tax-reports-pdf.ts; dine-in.service.ts/returns.service.ts/finance.service.ts post 2100 on sale/return/AP; /tax/reports UI; cutover/taxdocs.ts (ToE)</t>
+          <t>tax-reports; payroll</t>
         </is>
       </c>
       <c r="N112" s="12" t="inlineStr">
         <is>
-          <t>Inspect the pp30 build + the 2100 net-movement query + the tie flag + the filing deadline.</t>
+          <t>Inspect WHT logic + report.</t>
         </is>
       </c>
       <c r="O112" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: the pp30 return computes net VAT (output − input), the GL 2100 net movement reflects the posted input VAT, and the reconciliation block exposes the gl_account (2100), the report net VAT and a boolean tie verdict (tied iff the two agree within rounding); the ภ.พ.30 export renders (re-performed by the taxdocs harness).</t>
+          <t>Re-perform WHT on sample; tie to filing.</t>
         </is>
       </c>
       <c r="P112" s="12" t="inlineStr">
         <is>
-          <t>ภ.พ.30 return + GL-2100 reconciliation tie</t>
-        </is>
-      </c>
-      <c r="Q112" s="18" t="inlineStr">
-        <is>
-          <t>Implemented</t>
+          <t>WHT report</t>
+        </is>
+      </c>
+      <c r="Q112" s="19" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="15" t="inlineStr">
         <is>
-          <t>PAY-01</t>
+          <t>TAX-04</t>
         </is>
       </c>
       <c r="B113" s="16" t="inlineStr">
         <is>
-          <t>Payroll</t>
+          <t>Tax</t>
         </is>
       </c>
       <c r="C113" s="17" t="inlineStr">
@@ -10642,27 +10642,27 @@
       </c>
       <c r="D113" s="16" t="inlineStr">
         <is>
-          <t>Payroll expense/liability</t>
+          <t>Tax (VAT); Tax Payable (2100)</t>
         </is>
       </c>
       <c r="E113" s="16" t="inlineStr">
         <is>
-          <t>Payroll, SSO and PIT mis-computed.</t>
+          <t>Output/input VAT on the filed ภ.พ.30 return does not agree to the GL — VAT liability mis-stated, a filing/penalty exposure, or a posting omission goes undetected before submission.</t>
         </is>
       </c>
       <c r="F113" s="16" t="inlineStr">
         <is>
-          <t>Accuracy</t>
+          <t>Completeness/Accuracy</t>
         </is>
       </c>
       <c r="G113" s="16" t="inlineStr">
         <is>
-          <t>Payroll engine — SSO 5% (cap 750), progressive PIT, payslip net; unit-tested.</t>
+          <t>Periodic VAT-return ↔ GL reconciliation (ภ.พ.30): the monthly return (GET /api/tax-reports/pp30) is built from the sales/output-VAT and purchase/input-VAT sub-reports, computes net VAT = output − input, and RECONCILES it to the **GL account 2100 (Tax Payable) net movement** for the same period (Σ credit − Σ debit over Posted entries) — returning `reconciliation.tied` = true only when the two agree within rounding. A non-tie is a detective finding to investigate and clear BEFORE filing (the form also carries the ม.157 deadline = the 15th of the next month). Output VAT is posted to 2100 on every sale (Cr) and reversed on returns (Dr); input VAT is posted on AP bills (Dr) — so 2100's net is the period's VAT payable. Read-only report; exportable to a ภ.พ.30 PDF/HTML.</t>
         </is>
       </c>
       <c r="H113" s="17" t="inlineStr">
         <is>
-          <t>Auto</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I113" s="17" t="inlineStr">
@@ -10672,37 +10672,37 @@
       </c>
       <c r="J113" s="17" t="inlineStr">
         <is>
-          <t>Per run</t>
+          <t>Monthly / pre-filing</t>
         </is>
       </c>
       <c r="K113" s="16" t="inlineStr">
         <is>
-          <t>HR / Payroll</t>
+          <t>Tax / FinancialController</t>
         </is>
       </c>
       <c r="L113" s="17" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P10/P16</t>
         </is>
       </c>
       <c r="M113" s="16" t="inlineStr">
         <is>
-          <t>payroll/payroll-calc.ts; test/unit.test.ts</t>
+          <t>tax-reports.service.ts pp30 (outputVat/inputVat + 2100 net-movement tie); tax-reports.controller.ts (GET pp30, pp30/export, exec); tax-reports-pdf.ts; dine-in.service.ts/returns.service.ts/finance.service.ts post 2100 on sale/return/AP; /tax/reports UI; cutover/taxdocs.ts (ToE)</t>
         </is>
       </c>
       <c r="N113" s="16" t="inlineStr">
         <is>
-          <t>Inspect calc + tests.</t>
+          <t>Inspect the pp30 build + the 2100 net-movement query + the tie flag + the filing deadline.</t>
         </is>
       </c>
       <c r="O113" s="16" t="inlineStr">
         <is>
-          <t>Re-perform sample payslips.</t>
+          <t>Re-perform: the pp30 return computes net VAT (output − input), the GL 2100 net movement reflects the posted input VAT, and the reconciliation block exposes the gl_account (2100), the report net VAT and a boolean tie verdict (tied iff the two agree within rounding); the ภ.พ.30 export renders (re-performed by the taxdocs harness).</t>
         </is>
       </c>
       <c r="P113" s="16" t="inlineStr">
         <is>
-          <t>Payslip tests</t>
+          <t>ภ.พ.30 return + GL-2100 reconciliation tie</t>
         </is>
       </c>
       <c r="Q113" s="18" t="inlineStr">
@@ -10714,7 +10714,7 @@
     <row r="114">
       <c r="A114" s="11" t="inlineStr">
         <is>
-          <t>PAY-02</t>
+          <t>PAY-01</t>
         </is>
       </c>
       <c r="B114" s="12" t="inlineStr">
@@ -10729,27 +10729,27 @@
       </c>
       <c r="D114" s="12" t="inlineStr">
         <is>
-          <t>Payroll liability</t>
+          <t>Payroll expense/liability</t>
         </is>
       </c>
       <c r="E114" s="12" t="inlineStr">
         <is>
-          <t>Statutory withholdings (SSO/WHT/PF) mis-stated or not remitted, so the liability owed to the authorities diverges from the books.</t>
+          <t>Payroll, SSO and PIT mis-computed.</t>
         </is>
       </c>
       <c r="F114" s="12" t="inlineStr">
         <is>
-          <t>Accuracy/Compliance</t>
+          <t>Accuracy</t>
         </is>
       </c>
       <c r="G114" s="12" t="inlineStr">
         <is>
-          <t>Payroll-liability schedule (GET /api/payroll/liabilities): each statutory account — SSO 2350, WHT/PND1 2360, PF 2370 — shows accrued (GL credits) − remitted (GL debits) = outstanding, tied back to the INDEPENDENT payrun accrual with a `reconciled` flag (a divergence flags a manual JE that touched a payroll-liability account outside the payroll process). Treasury remits the cash (POST .../remit → Dr liability / Cr 1000) which clears the outstanding and keeps the books reconciled to the statutory filings; a remittance beyond the outstanding is blocked (REMIT_EXCEEDS_OUTSTANDING).</t>
+          <t>Payroll engine — SSO 5% (cap 750), progressive PIT, payslip net; unit-tested.</t>
         </is>
       </c>
       <c r="H114" s="13" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Auto</t>
         </is>
       </c>
       <c r="I114" s="13" t="inlineStr">
@@ -10759,12 +10759,12 @@
       </c>
       <c r="J114" s="13" t="inlineStr">
         <is>
-          <t>Per run / monthly</t>
+          <t>Per run</t>
         </is>
       </c>
       <c r="K114" s="12" t="inlineStr">
         <is>
-          <t>HR / Payroll / Treasury</t>
+          <t>HR / Payroll</t>
         </is>
       </c>
       <c r="L114" s="13" t="inlineStr">
@@ -10774,22 +10774,22 @@
       </c>
       <c r="M114" s="12" t="inlineStr">
         <is>
-          <t>payroll/payroll.service.ts liabilities/remitLiability</t>
+          <t>payroll/payroll-calc.ts; test/unit.test.ts</t>
         </is>
       </c>
       <c r="N114" s="12" t="inlineStr">
         <is>
-          <t>Inspect the schedule + the accrued/remitted/outstanding tie-out and the reconciled flag.</t>
+          <t>Inspect calc + tests.</t>
         </is>
       </c>
       <c r="O114" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: run a payroll, confirm the SSO/WHT outstanding equals the payrun accrual; remit part and confirm the outstanding falls and the TB stays balanced; attempt an over-remit (REMIT_EXCEEDS_OUTSTANDING).</t>
+          <t>Re-perform sample payslips.</t>
         </is>
       </c>
       <c r="P114" s="12" t="inlineStr">
         <is>
-          <t>Liability schedule + remittance JEs tied to filings</t>
+          <t>Payslip tests</t>
         </is>
       </c>
       <c r="Q114" s="18" t="inlineStr">
@@ -10801,7 +10801,7 @@
     <row r="115">
       <c r="A115" s="15" t="inlineStr">
         <is>
-          <t>PAY-03</t>
+          <t>PAY-02</t>
         </is>
       </c>
       <c r="B115" s="16" t="inlineStr">
@@ -10816,27 +10816,27 @@
       </c>
       <c r="D115" s="16" t="inlineStr">
         <is>
-          <t>Payroll expense/liability; Cash</t>
+          <t>Payroll liability</t>
         </is>
       </c>
       <c r="E115" s="16" t="inlineStr">
         <is>
-          <t>Payroll run posted to the GL without independent review — the preparer both computes and posts their own payroll (ghost employees, inflated rate/hours).</t>
+          <t>Statutory withholdings (SSO/WHT/PF) mis-stated or not remitted, so the liability owed to the authorities diverges from the books.</t>
         </is>
       </c>
       <c r="F115" s="16" t="inlineStr">
         <is>
-          <t>Authorization</t>
+          <t>Accuracy/Compliance</t>
         </is>
       </c>
       <c r="G115" s="16" t="inlineStr">
         <is>
-          <t>Payroll maker-checker (SoD): a run posts its GL entry as a DRAFT (excluded from balances) with the run record 'PendingApproval'; a DIFFERENT user must approve before it becomes effective (approver ≠ preparer enforced regardless of permissions, reusing the GL-05 ledger approval). Reject voids the draft; idempotent per (tenant, period).</t>
+          <t>Payroll-liability schedule (GET /api/payroll/liabilities): each statutory account — SSO 2350, WHT/PND1 2360, PF 2370 — shows accrued (GL credits) − remitted (GL debits) = outstanding, tied back to the INDEPENDENT payrun accrual with a `reconciled` flag (a divergence flags a manual JE that touched a payroll-liability account outside the payroll process). Treasury remits the cash (POST .../remit → Dr liability / Cr 1000) which clears the outstanding and keeps the books reconciled to the statutory filings; a remittance beyond the outstanding is blocked (REMIT_EXCEEDS_OUTSTANDING).</t>
         </is>
       </c>
       <c r="H115" s="17" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I115" s="17" t="inlineStr">
@@ -10846,12 +10846,12 @@
       </c>
       <c r="J115" s="17" t="inlineStr">
         <is>
-          <t>Per run</t>
+          <t>Per run / monthly</t>
         </is>
       </c>
       <c r="K115" s="16" t="inlineStr">
         <is>
-          <t>HR / Payroll; Controller</t>
+          <t>HR / Payroll / Treasury</t>
         </is>
       </c>
       <c r="L115" s="17" t="inlineStr">
@@ -10861,22 +10861,22 @@
       </c>
       <c r="M115" s="16" t="inlineStr">
         <is>
-          <t>payroll/payroll.service.ts approvePayroll/rejectPayroll; migration 0133</t>
+          <t>payroll/payroll.service.ts liabilities/remitLiability</t>
         </is>
       </c>
       <c r="N115" s="16" t="inlineStr">
         <is>
-          <t>Inspect Draft→approve flow + the approver≠preparer check.</t>
+          <t>Inspect the schedule + the accrued/remitted/outstanding tie-out and the reconciled flag.</t>
         </is>
       </c>
       <c r="O115" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: run as A, attempt self-approve (SOD_VIOLATION), approve as B; confirm the JE hits balances only after approval.</t>
+          <t>Re-perform: run a payroll, confirm the SSO/WHT outstanding equals the payrun accrual; remit part and confirm the outstanding falls and the TB stays balanced; attempt an over-remit (REMIT_EXCEEDS_OUTSTANDING).</t>
         </is>
       </c>
       <c r="P115" s="16" t="inlineStr">
         <is>
-          <t>Approval log + SoD test</t>
+          <t>Liability schedule + remittance JEs tied to filings</t>
         </is>
       </c>
       <c r="Q115" s="18" t="inlineStr">
@@ -10888,12 +10888,12 @@
     <row r="116">
       <c r="A116" s="11" t="inlineStr">
         <is>
-          <t>FA-09</t>
+          <t>PAY-03</t>
         </is>
       </c>
       <c r="B116" s="12" t="inlineStr">
         <is>
-          <t>Fixed Assets</t>
+          <t>Payroll</t>
         </is>
       </c>
       <c r="C116" s="13" t="inlineStr">
@@ -10903,12 +10903,12 @@
       </c>
       <c r="D116" s="12" t="inlineStr">
         <is>
-          <t>Property, Plant &amp; Equipment; Cash</t>
+          <t>Payroll expense/liability; Cash</t>
         </is>
       </c>
       <c r="E116" s="12" t="inlineStr">
         <is>
-          <t>Asset disposed without independent review — one person writes an asset off the books and records the proceeds (asset-stripping / theft: dispose a still-held asset, or to a related party below value).</t>
+          <t>Payroll run posted to the GL without independent review — the preparer both computes and posts their own payroll (ghost employees, inflated rate/hours).</t>
         </is>
       </c>
       <c r="F116" s="12" t="inlineStr">
@@ -10918,7 +10918,7 @@
       </c>
       <c r="G116" s="12" t="inlineStr">
         <is>
-          <t>Asset-disposal maker-checker (SoD): a disposal REQUEST posts its GL entry as a DRAFT (excluded from balances) and flags the asset disposal_pending WITHOUT marking it disposed or moving the register; a DIFFERENT user must approve before it is effective (status→disposed, revaluation surplus recycled 3200→3100) (approver ≠ requester enforced regardless of permissions, reusing the GL-05 ledger approval). Reject voids the draft and the asset stays in service; only one disposal may be pending per asset; a disposal-pending asset is frozen from depreciation.</t>
+          <t>Payroll maker-checker (SoD): a run posts its GL entry as a DRAFT (excluded from balances) with the run record 'PendingApproval'; a DIFFERENT user must approve before it becomes effective (approver ≠ preparer enforced regardless of permissions, reusing the GL-05 ledger approval). Reject voids the draft; idempotent per (tenant, period).</t>
         </is>
       </c>
       <c r="H116" s="13" t="inlineStr">
@@ -10933,12 +10933,12 @@
       </c>
       <c r="J116" s="13" t="inlineStr">
         <is>
-          <t>Per disposal</t>
+          <t>Per run</t>
         </is>
       </c>
       <c r="K116" s="12" t="inlineStr">
         <is>
-          <t>FaAccountant / Controller</t>
+          <t>HR / Payroll; Controller</t>
         </is>
       </c>
       <c r="L116" s="13" t="inlineStr">
@@ -10948,22 +10948,22 @@
       </c>
       <c r="M116" s="12" t="inlineStr">
         <is>
-          <t>assets.service.ts dispose(pendingApproval Draft)/approveDisposal/rejectDisposal; assets.controller.ts (:assetNo/dispose/approve|reject); schema/assets.ts fixed_assets.disposal_pending + migration 0135; cutover/basics.ts + worldclass.ts + compliance.ts (ToE)</t>
+          <t>payroll/payroll.service.ts approvePayroll/rejectPayroll; migration 0133</t>
         </is>
       </c>
       <c r="N116" s="12" t="inlineStr">
         <is>
-          <t>Inspect Draft→approve flow + the approver≠requester check + deferred status/recycle.</t>
+          <t>Inspect Draft→approve flow + the approver≠preparer check.</t>
         </is>
       </c>
       <c r="O116" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: request a disposal (Draft JE excluded), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm status→disposed + surplus recycled only after approval (re-performed by the harnesses).</t>
+          <t>Re-perform: run as A, attempt self-approve (SOD_VIOLATION), approve as B; confirm the JE hits balances only after approval.</t>
         </is>
       </c>
       <c r="P116" s="12" t="inlineStr">
         <is>
-          <t>Disposal approval log + SoD test</t>
+          <t>Approval log + SoD test</t>
         </is>
       </c>
       <c r="Q116" s="18" t="inlineStr">
@@ -10975,7 +10975,7 @@
     <row r="117">
       <c r="A117" s="15" t="inlineStr">
         <is>
-          <t>FA-10</t>
+          <t>FA-09</t>
         </is>
       </c>
       <c r="B117" s="16" t="inlineStr">
@@ -10990,22 +10990,22 @@
       </c>
       <c r="D117" s="16" t="inlineStr">
         <is>
-          <t>Property, Plant &amp; Equipment; Accounts Payable</t>
+          <t>Property, Plant &amp; Equipment; Cash</t>
         </is>
       </c>
       <c r="E117" s="16" t="inlineStr">
         <is>
-          <t>Capital purchases mis-capitalised or capitalised without independent review — the person who receives the goods also decides what enters the asset register and at what cost/useful life (fictitious or over-valued assets; capex/opex mis-classification).</t>
+          <t>Asset disposed without independent review — one person writes an asset off the books and records the proceeds (asset-stripping / theft: dispose a still-held asset, or to a related party below value).</t>
         </is>
       </c>
       <c r="F117" s="16" t="inlineStr">
         <is>
-          <t>Authorization; Accuracy</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="G117" s="16" t="inlineStr">
         <is>
-          <t>Procure-to-Capitalize maker-checker (SoD): a goods-receipt line flagged capital (item-master is_fixed_asset or per-PO-line override) is excluded from inventory capitalisation (1200) at receipt and instead becomes ELIGIBLE for the asset register. Capitalisation is a REQUEST that posts NOTHING to the GL; a DIFFERENT user must approve before the fixed_assets row + acquisition JE (Dr 1500 / Cr 2000) are created (approver ≠ requester enforced regardless of permissions). The created asset carries its source GR/PO for end-to-end PR→PO→GR→FA traceability; a GR line cannot be capitalised twice.</t>
+          <t>Asset-disposal maker-checker (SoD): a disposal REQUEST posts its GL entry as a DRAFT (excluded from balances) and flags the asset disposal_pending WITHOUT marking it disposed or moving the register; a DIFFERENT user must approve before it is effective (status→disposed, revaluation surplus recycled 3200→3100) (approver ≠ requester enforced regardless of permissions, reusing the GL-05 ledger approval). Reject voids the draft and the asset stays in service; only one disposal may be pending per asset; a disposal-pending asset is frozen from depreciation.</t>
         </is>
       </c>
       <c r="H117" s="17" t="inlineStr">
@@ -11020,7 +11020,7 @@
       </c>
       <c r="J117" s="17" t="inlineStr">
         <is>
-          <t>Per capital receipt</t>
+          <t>Per disposal</t>
         </is>
       </c>
       <c r="K117" s="16" t="inlineStr">
@@ -11035,22 +11035,22 @@
       </c>
       <c r="M117" s="16" t="inlineStr">
         <is>
-          <t>assets.service.ts registerFromGr/approveRegistration/rejectRegistration/eligibleFromGr; assets.controller.ts (registrations*); procurement.service.ts createGr (is_capital routing, costing excluded); schema/assets.ts asset_registration_requests + fixed_assets.source_gr_no/po_no + migration 0137; cutover/basics.ts + compliance.ts (ToE)</t>
+          <t>assets.service.ts dispose(pendingApproval Draft)/approveDisposal/rejectDisposal; assets.controller.ts (:assetNo/dispose/approve|reject); schema/assets.ts fixed_assets.disposal_pending + migration 0135; cutover/basics.ts + worldclass.ts + compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N117" s="16" t="inlineStr">
         <is>
-          <t>Inspect the eligible→request→approve flow + approver≠requester check + the inventory-vs-asset routing of capital lines.</t>
+          <t>Inspect Draft→approve flow + the approver≠requester check + deferred status/recycle.</t>
         </is>
       </c>
       <c r="O117" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: receive a capital line, raise a registration (no GL), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm the asset + Dr 1500/Cr 2000 post only after approval and the line cannot be re-registered (re-performed by the harnesses).</t>
+          <t>Re-perform: request a disposal (Draft JE excluded), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm status→disposed + surplus recycled only after approval (re-performed by the harnesses).</t>
         </is>
       </c>
       <c r="P117" s="16" t="inlineStr">
         <is>
-          <t>Capitalization approval log + SoD test</t>
+          <t>Disposal approval log + SoD test</t>
         </is>
       </c>
       <c r="Q117" s="18" t="inlineStr">
@@ -11062,12 +11062,12 @@
     <row r="118">
       <c r="A118" s="11" t="inlineStr">
         <is>
-          <t>CON-01</t>
+          <t>FA-10</t>
         </is>
       </c>
       <c r="B118" s="12" t="inlineStr">
         <is>
-          <t>Consolidation &amp; FX</t>
+          <t>Fixed Assets</t>
         </is>
       </c>
       <c r="C118" s="13" t="inlineStr">
@@ -11077,42 +11077,42 @@
       </c>
       <c r="D118" s="12" t="inlineStr">
         <is>
-          <t>Consolidation</t>
+          <t>Property, Plant &amp; Equipment; Accounts Payable</t>
         </is>
       </c>
       <c r="E118" s="12" t="inlineStr">
         <is>
-          <t>Group consolidation mis-stated (ownership/currency).</t>
+          <t>Capital purchases mis-capitalised or capitalised without independent review — the person who receives the goods also decides what enters the asset register and at what cost/useful life (fictitious or over-valued assets; capex/opex mis-classification).</t>
         </is>
       </c>
       <c r="F118" s="12" t="inlineStr">
         <is>
-          <t>Accuracy</t>
+          <t>Authorization; Accuracy</t>
         </is>
       </c>
       <c r="G118" s="12" t="inlineStr">
         <is>
-          <t>Consolidation run (ownership %, entity currency) gated by 'approvals'.</t>
+          <t>Procure-to-Capitalize maker-checker (SoD): a goods-receipt line flagged capital (item-master is_fixed_asset or per-PO-line override) is excluded from inventory capitalisation (1200) at receipt and instead becomes ELIGIBLE for the asset register. Capitalisation is a REQUEST that posts NOTHING to the GL; a DIFFERENT user must approve before the fixed_assets row + acquisition JE (Dr 1500 / Cr 2000) are created (approver ≠ requester enforced regardless of permissions). The created asset carries its source GR/PO for end-to-end PR→PO→GR→FA traceability; a GR line cannot be capitalised twice.</t>
         </is>
       </c>
       <c r="H118" s="13" t="inlineStr">
         <is>
-          <t>Auto+Manual</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I118" s="13" t="inlineStr">
         <is>
-          <t>Period</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J118" s="13" t="inlineStr">
         <is>
-          <t>Period</t>
+          <t>Per capital receipt</t>
         </is>
       </c>
       <c r="K118" s="12" t="inlineStr">
         <is>
-          <t>Group Controller</t>
+          <t>FaAccountant / Controller</t>
         </is>
       </c>
       <c r="L118" s="13" t="inlineStr">
@@ -11122,22 +11122,22 @@
       </c>
       <c r="M118" s="12" t="inlineStr">
         <is>
-          <t>consolidation.service.ts (runConsolidation @Permissions approvals)</t>
+          <t>assets.service.ts registerFromGr/approveRegistration/rejectRegistration/eligibleFromGr; assets.controller.ts (registrations*); procurement.service.ts createGr (is_capital routing, costing excluded); schema/assets.ts asset_registration_requests + fixed_assets.source_gr_no/po_no + migration 0137; cutover/basics.ts + compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N118" s="12" t="inlineStr">
         <is>
-          <t>Inspect consolidation logic + gate.</t>
+          <t>Inspect the eligible→request→approve flow + approver≠requester check + the inventory-vs-asset routing of capital lines.</t>
         </is>
       </c>
       <c r="O118" s="12" t="inlineStr">
         <is>
-          <t>Sample period: consolidated TB ties to entities.</t>
+          <t>Re-perform: receive a capital line, raise a registration (no GL), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm the asset + Dr 1500/Cr 2000 post only after approval and the line cannot be re-registered (re-performed by the harnesses).</t>
         </is>
       </c>
       <c r="P118" s="12" t="inlineStr">
         <is>
-          <t>Consol TB</t>
+          <t>Capitalization approval log + SoD test</t>
         </is>
       </c>
       <c r="Q118" s="18" t="inlineStr">
@@ -11149,7 +11149,7 @@
     <row r="119">
       <c r="A119" s="15" t="inlineStr">
         <is>
-          <t>CON-02</t>
+          <t>CON-01</t>
         </is>
       </c>
       <c r="B119" s="16" t="inlineStr">
@@ -11164,22 +11164,22 @@
       </c>
       <c r="D119" s="16" t="inlineStr">
         <is>
-          <t>FX gain/loss</t>
+          <t>Consolidation</t>
         </is>
       </c>
       <c r="E119" s="16" t="inlineStr">
         <is>
-          <t>FX exposures not revalued at period-end.</t>
+          <t>Group consolidation mis-stated (ownership/currency).</t>
         </is>
       </c>
       <c r="F119" s="16" t="inlineStr">
         <is>
-          <t>Valuation</t>
+          <t>Accuracy</t>
         </is>
       </c>
       <c r="G119" s="16" t="inlineStr">
         <is>
-          <t>FX revaluation at period-end rates; unrealized FX posted (acct 5400).</t>
+          <t>Consolidation run (ownership %, entity currency) gated by 'approvals'.</t>
         </is>
       </c>
       <c r="H119" s="17" t="inlineStr">
@@ -11189,7 +11189,7 @@
       </c>
       <c r="I119" s="17" t="inlineStr">
         <is>
-          <t>Period-end</t>
+          <t>Period</t>
         </is>
       </c>
       <c r="J119" s="17" t="inlineStr">
@@ -11199,7 +11199,7 @@
       </c>
       <c r="K119" s="16" t="inlineStr">
         <is>
-          <t>Controller</t>
+          <t>Group Controller</t>
         </is>
       </c>
       <c r="L119" s="17" t="inlineStr">
@@ -11209,22 +11209,22 @@
       </c>
       <c r="M119" s="16" t="inlineStr">
         <is>
-          <t>fx.service.ts (revalue / unrealized report)</t>
+          <t>consolidation.service.ts (runConsolidation @Permissions approvals)</t>
         </is>
       </c>
       <c r="N119" s="16" t="inlineStr">
         <is>
-          <t>Inspect reval logic + rates.</t>
+          <t>Inspect consolidation logic + gate.</t>
         </is>
       </c>
       <c r="O119" s="16" t="inlineStr">
         <is>
-          <t>Recompute reval on sample balances.</t>
+          <t>Sample period: consolidated TB ties to entities.</t>
         </is>
       </c>
       <c r="P119" s="16" t="inlineStr">
         <is>
-          <t>FX reval JE</t>
+          <t>Consol TB</t>
         </is>
       </c>
       <c r="Q119" s="18" t="inlineStr">
@@ -11236,7 +11236,7 @@
     <row r="120">
       <c r="A120" s="11" t="inlineStr">
         <is>
-          <t>FX-04</t>
+          <t>CON-02</t>
         </is>
       </c>
       <c r="B120" s="12" t="inlineStr">
@@ -11251,42 +11251,42 @@
       </c>
       <c r="D120" s="12" t="inlineStr">
         <is>
-          <t>FX gain/loss; Revenue; AR/AP</t>
+          <t>FX gain/loss</t>
         </is>
       </c>
       <c r="E120" s="12" t="inlineStr">
         <is>
-          <t>A wrong manually-entered FX rate (fat-fingered, e.g. USD 36 keyed as 63) flows straight into a period-end revaluation JE and the unrealized-FX report with no independent review — mis-stating earnings/equity and FX-translated balances.</t>
+          <t>FX exposures not revalued at period-end.</t>
         </is>
       </c>
       <c r="F120" s="12" t="inlineStr">
         <is>
-          <t>Accuracy/Valuation</t>
+          <t>Valuation</t>
         </is>
       </c>
       <c r="G120" s="12" t="inlineStr">
         <is>
-          <t>FX rate maker-checker (SoD): a MANUALLY-entered rate lands as PendingApproval and is EXCLUDED from rate resolution — revaluation, the unrealized-FX report, and consolidation translation all use APPROVED rates only — until a DIFFERENT user approves it (POST /api/fx/rates/approve). Self-approval → SOD_VIOLATION (binds even Admin); reject marks the rate Rejected (never usable); re-entering a rate sends it back to PendingApproval. Externally-sourced (feed) rates carrying an explicit non-manual source are auto-approved. Pending rates are also surfaced, aged, by the pending-approvals monitor (GOV-01).</t>
+          <t>FX revaluation at period-end rates; unrealized FX posted (acct 5400).</t>
         </is>
       </c>
       <c r="H120" s="13" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="I120" s="13" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Period-end</t>
         </is>
       </c>
       <c r="J120" s="13" t="inlineStr">
         <is>
-          <t>Per rate</t>
+          <t>Period</t>
         </is>
       </c>
       <c r="K120" s="12" t="inlineStr">
         <is>
-          <t>Controller / Treasury</t>
+          <t>Controller</t>
         </is>
       </c>
       <c r="L120" s="13" t="inlineStr">
@@ -11296,22 +11296,22 @@
       </c>
       <c r="M120" s="12" t="inlineStr">
         <is>
-          <t>fx.service.ts setRate(manual→PendingApproval)/approveRate/rejectRate/rateAsOf(Approved only); fx.controller.ts (rates/approve|reject|pending gated approvals/gl_close); consolidation.service.ts (translation reads Approved rates); schema/fx.ts fx_rates.status + migration 0141; cutover/fxreval.ts (ToE)</t>
+          <t>fx.service.ts (revalue / unrealized report)</t>
         </is>
       </c>
       <c r="N120" s="12" t="inlineStr">
         <is>
-          <t>Inspect the request→approve flow + the approver≠requester check + that revaluation/reporting resolve Approved rates only.</t>
+          <t>Inspect reval logic + rates.</t>
         </is>
       </c>
       <c r="O120" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: enter a manual rate (PendingApproval), confirm revalue is blocked NO_RATE while pending, attempt self-approve (SOD_VIOLATION), approve as a different user, then revalue succeeds (re-performed by the fxreval harness).</t>
+          <t>Recompute reval on sample balances.</t>
         </is>
       </c>
       <c r="P120" s="12" t="inlineStr">
         <is>
-          <t>FX rate approval log + SoD test</t>
+          <t>FX reval JE</t>
         </is>
       </c>
       <c r="Q120" s="18" t="inlineStr">
@@ -11323,92 +11323,179 @@
     <row r="121">
       <c r="A121" s="15" t="inlineStr">
         <is>
+          <t>FX-04</t>
+        </is>
+      </c>
+      <c r="B121" s="16" t="inlineStr">
+        <is>
+          <t>Consolidation &amp; FX</t>
+        </is>
+      </c>
+      <c r="C121" s="17" t="inlineStr">
+        <is>
+          <t>Application</t>
+        </is>
+      </c>
+      <c r="D121" s="16" t="inlineStr">
+        <is>
+          <t>FX gain/loss; Revenue; AR/AP</t>
+        </is>
+      </c>
+      <c r="E121" s="16" t="inlineStr">
+        <is>
+          <t>A wrong manually-entered FX rate (fat-fingered, e.g. USD 36 keyed as 63) flows straight into a period-end revaluation JE and the unrealized-FX report with no independent review — mis-stating earnings/equity and FX-translated balances.</t>
+        </is>
+      </c>
+      <c r="F121" s="16" t="inlineStr">
+        <is>
+          <t>Accuracy/Valuation</t>
+        </is>
+      </c>
+      <c r="G121" s="16" t="inlineStr">
+        <is>
+          <t>FX rate maker-checker (SoD): a MANUALLY-entered rate lands as PendingApproval and is EXCLUDED from rate resolution — revaluation, the unrealized-FX report, and consolidation translation all use APPROVED rates only — until a DIFFERENT user approves it (POST /api/fx/rates/approve). Self-approval → SOD_VIOLATION (binds even Admin); reject marks the rate Rejected (never usable); re-entering a rate sends it back to PendingApproval. Externally-sourced (feed) rates carrying an explicit non-manual source are auto-approved. Pending rates are also surfaced, aged, by the pending-approvals monitor (GOV-01).</t>
+        </is>
+      </c>
+      <c r="H121" s="17" t="inlineStr">
+        <is>
+          <t>Prev</t>
+        </is>
+      </c>
+      <c r="I121" s="17" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="J121" s="17" t="inlineStr">
+        <is>
+          <t>Per rate</t>
+        </is>
+      </c>
+      <c r="K121" s="16" t="inlineStr">
+        <is>
+          <t>Controller / Treasury</t>
+        </is>
+      </c>
+      <c r="L121" s="17" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="M121" s="16" t="inlineStr">
+        <is>
+          <t>fx.service.ts setRate(manual→PendingApproval)/approveRate/rejectRate/rateAsOf(Approved only); fx.controller.ts (rates/approve|reject|pending gated approvals/gl_close); consolidation.service.ts (translation reads Approved rates); schema/fx.ts fx_rates.status + migration 0141; cutover/fxreval.ts (ToE)</t>
+        </is>
+      </c>
+      <c r="N121" s="16" t="inlineStr">
+        <is>
+          <t>Inspect the request→approve flow + the approver≠requester check + that revaluation/reporting resolve Approved rates only.</t>
+        </is>
+      </c>
+      <c r="O121" s="16" t="inlineStr">
+        <is>
+          <t>Re-perform: enter a manual rate (PendingApproval), confirm revalue is blocked NO_RATE while pending, attempt self-approve (SOD_VIOLATION), approve as a different user, then revalue succeeds (re-performed by the fxreval harness).</t>
+        </is>
+      </c>
+      <c r="P121" s="16" t="inlineStr">
+        <is>
+          <t>FX rate approval log + SoD test</t>
+        </is>
+      </c>
+      <c r="Q121" s="18" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="11" t="inlineStr">
+        <is>
           <t>BUD-01</t>
         </is>
       </c>
-      <c r="B121" s="16" t="inlineStr">
+      <c r="B122" s="12" t="inlineStr">
         <is>
           <t>Budgeting &amp; Planning</t>
         </is>
       </c>
-      <c r="C121" s="17" t="inlineStr">
+      <c r="C122" s="13" t="inlineStr">
         <is>
           <t>Application</t>
         </is>
       </c>
-      <c r="D121" s="16" t="inlineStr">
+      <c r="D122" s="12" t="inlineStr">
         <is>
           <t>Budget; All (variance reporting)</t>
         </is>
       </c>
-      <c r="E121" s="16" t="inlineStr">
+      <c r="E122" s="12" t="inlineStr">
         <is>
           <t>A budget figure is entered/changed by one person and immediately drives the budget-vs-actual variance report — the basis for spend authorization and performance review — with no independent approval; a wrong or self-serving budget makes overspending look 'on budget'.</t>
         </is>
       </c>
-      <c r="F121" s="16" t="inlineStr">
+      <c r="F122" s="12" t="inlineStr">
         <is>
           <t>Authorization/Accuracy</t>
         </is>
       </c>
-      <c r="G121" s="16" t="inlineStr">
+      <c r="G122" s="12" t="inlineStr">
         <is>
           <t>Budget maker-checker (SoD): an upserted budget (POST /api/ledger/budgets) lands as PendingApproval and is EXCLUDED from budget-vs-actual until a DIFFERENT user approves it (POST /api/ledger/budgets/approve for the fiscal_year/account/cost-centre[/period]). Self-approval → SOD_VIOLATION (binds even Admin); reject marks it Rejected (excluded). DEFAULT 'Approved' keeps existing rows + direct planning seeds usable. Pending budgets are also surfaced, aged, by the pending-approvals monitor (GOV-01).</t>
         </is>
       </c>
-      <c r="H121" s="17" t="inlineStr">
+      <c r="H122" s="13" t="inlineStr">
         <is>
           <t>Prev</t>
         </is>
       </c>
-      <c r="I121" s="17" t="inlineStr">
+      <c r="I122" s="13" t="inlineStr">
         <is>
           <t>Automated</t>
         </is>
       </c>
-      <c r="J121" s="17" t="inlineStr">
+      <c r="J122" s="13" t="inlineStr">
         <is>
           <t>Per budget</t>
         </is>
       </c>
-      <c r="K121" s="16" t="inlineStr">
+      <c r="K122" s="12" t="inlineStr">
         <is>
           <t>Controller / FP&amp;A</t>
         </is>
       </c>
-      <c r="L121" s="17" t="inlineStr">
+      <c r="L122" s="13" t="inlineStr">
         <is>
           <t>P10</t>
         </is>
       </c>
-      <c r="M121" s="16" t="inlineStr">
+      <c r="M122" s="12" t="inlineStr">
         <is>
           <t>budget.service.ts upsertBudget(→PendingApproval)/approveBudget/rejectBudget/budgetVsActual(Approved only); budget.controller.ts (budgets/approve|reject|pending gated approvals/gl_close); schema/budgets.ts budgets.status + migration 0142; cutover/budget.ts (ToE)</t>
         </is>
       </c>
-      <c r="N121" s="16" t="inlineStr">
+      <c r="N122" s="12" t="inlineStr">
         <is>
           <t>Inspect the request→approve flow + the approver≠requester check + that budget-vs-actual counts Approved budgets only.</t>
         </is>
       </c>
-      <c r="O121" s="16" t="inlineStr">
+      <c r="O122" s="12" t="inlineStr">
         <is>
           <t>Re-perform: upsert a budget (PendingApproval, excluded from variance), attempt self-approve (SOD_VIOLATION), approve as a different user, confirm it then appears in budget-vs-actual (re-performed by the budget harness).</t>
         </is>
       </c>
-      <c r="P121" s="16" t="inlineStr">
+      <c r="P122" s="12" t="inlineStr">
         <is>
           <t>Budget approval log + SoD test</t>
         </is>
       </c>
-      <c r="Q121" s="18" t="inlineStr">
+      <c r="Q122" s="18" t="inlineStr">
         <is>
           <t>Implemented</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q121"/>
+  <autoFilter ref="A1:Q122"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -12591,7 +12678,7 @@
         </is>
       </c>
       <c r="C5" s="29">
-        <f>COUNTIF(RCM!$Q$2:$Q$121,B5)</f>
+        <f>COUNTIF(RCM!$Q$2:$Q$122,B5)</f>
         <v/>
       </c>
     </row>
@@ -12602,7 +12689,7 @@
         </is>
       </c>
       <c r="C6" s="29">
-        <f>COUNTIF(RCM!$Q$2:$Q$121,B6)</f>
+        <f>COUNTIF(RCM!$Q$2:$Q$122,B6)</f>
         <v/>
       </c>
     </row>
@@ -12613,7 +12700,7 @@
         </is>
       </c>
       <c r="C7" s="29">
-        <f>COUNTIF(RCM!$Q$2:$Q$121,B7)</f>
+        <f>COUNTIF(RCM!$Q$2:$Q$122,B7)</f>
         <v/>
       </c>
     </row>
@@ -12624,7 +12711,7 @@
         </is>
       </c>
       <c r="C8" s="32">
-        <f>COUNTA(RCM!$A$2:$A$121)</f>
+        <f>COUNTA(RCM!$A$2:$A$122)</f>
         <v/>
       </c>
     </row>
@@ -12642,7 +12729,7 @@
         </is>
       </c>
       <c r="C11" s="29">
-        <f>COUNTIF(RCM!$C$2:$C$121,B11)</f>
+        <f>COUNTIF(RCM!$C$2:$C$122,B11)</f>
         <v/>
       </c>
     </row>
@@ -12653,7 +12740,7 @@
         </is>
       </c>
       <c r="C12" s="29">
-        <f>COUNTIF(RCM!$C$2:$C$121,B12)</f>
+        <f>COUNTIF(RCM!$C$2:$C$122,B12)</f>
         <v/>
       </c>
     </row>
@@ -12664,7 +12751,7 @@
         </is>
       </c>
       <c r="C13" s="29">
-        <f>COUNTIF(RCM!$C$2:$C$121,B13)</f>
+        <f>COUNTIF(RCM!$C$2:$C$122,B13)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(inventory): demand-driven par-level recommendations (Step 5, INV-12) (#165)
Branch replenishment (INV-05) routed transfer-before-buy off a STATIC per-branch
reorder point. Now each (branch,item) carries a lead_time_days, and the system
derives average daily usage from trailing branch-tagged consumption and
recommends reorder_point = ceil(avg_daily x lead x 1.25), flagging branches whose
static buffer is under-buffered for their run-rate. A planner applies per row.

- mig 0163: branch_stock + lead_time_days (journaled)
- replenishment.service parRecommendations + applyPar; wms.controller routes
  (par-recommendations [/apply]); /replenishment web par section
- wms harness +2 (10/day x lead 3 -> ROP 38 under-buffered; apply writes 38)
- RCM INV-12 (120 controls); docs inventory narrative 1.3, UAT-INV-058/059

wms(27)/compliance(106) green; typecheck green.

Co-authored-by: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/compliance/Oshinei_ERP_SOX_RCM_v1.xlsx
+++ b/compliance/Oshinei_ERP_SOX_RCM_v1.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'RCM'!$A$1:$Q$122</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'RCM'!$A$1:$Q$123</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Gap Remediation'!$A$2:$H$18</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -858,7 +858,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q122"/>
+  <dimension ref="A1:Q123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -7147,12 +7147,12 @@
     <row r="73">
       <c r="A73" s="15" t="inlineStr">
         <is>
-          <t>BRANCH-01</t>
+          <t>INV-12</t>
         </is>
       </c>
       <c r="B73" s="16" t="inlineStr">
         <is>
-          <t>Multi-Branch &amp; Offline POS</t>
+          <t>Inventory &amp; COGS</t>
         </is>
       </c>
       <c r="C73" s="17" t="inlineStr">
@@ -7162,22 +7162,22 @@
       </c>
       <c r="D73" s="16" t="inlineStr">
         <is>
-          <t>Revenue</t>
+          <t>Inventory</t>
         </is>
       </c>
       <c r="E73" s="16" t="inlineStr">
         <is>
-          <t>A POS sale is not attributed to its originating branch, so the consolidated branch roll-up is incomplete and cannot be tied to GL revenue.</t>
+          <t>Per-branch reorder points are STATIC numbers — set once and never revisited — so a branch whose run-rate has grown carries too small a buffer and stocks out (lost sales), while a slow branch over-orders and ties up cash/spoils stock; neither is flagged.</t>
         </is>
       </c>
       <c r="F73" s="16" t="inlineStr">
         <is>
-          <t>Completeness</t>
+          <t>Accuracy/Completeness</t>
         </is>
       </c>
       <c r="G73" s="16" t="inlineStr">
         <is>
-          <t>Branch sale-tagging + HQ consolidation: every POS sale carries cust_pos_sales.branch_id; GET /api/branches/consolidated aggregates per branch (excluding Voided) and surfaces untagged sales as branch '(none)' — a deliberate completeness flag the controller investigates and clears before tying the consolidated total to GL revenue.</t>
+          <t>Demand-driven par-level recommendation (layered on the INV-05 branch min-max + transfer-before-buy): for each (branch,item) the system derives the average daily usage from the trailing window of branch-tagged consumption (cust_stock_log Sale/Consume) and recommends reorder_point = ceil(avg_daily x lead_time_days x safety 1.25), flagging rows whose static reorder_point is below that demand-driven buffer (under_buffered). GET /api/replenishment/par-recommendations is read-only; a planner applies a recommendation per row (POST .../apply writes the reorder_point onto branch_stock, planner duty). lead_time_days is per (branch,item) (migration 0163). Tenant-scoped (RLS); gated planner/procurement.</t>
         </is>
       </c>
       <c r="H73" s="17" t="inlineStr">
@@ -7192,37 +7192,37 @@
       </c>
       <c r="J73" s="17" t="inlineStr">
         <is>
-          <t>Per sale / period</t>
+          <t>Periodic / per planning cycle</t>
         </is>
       </c>
       <c r="K73" s="16" t="inlineStr">
         <is>
-          <t>HQ Controller</t>
+          <t>Planner / Supply Chain</t>
         </is>
       </c>
       <c r="L73" s="17" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>P13</t>
         </is>
       </c>
       <c r="M73" s="16" t="inlineStr">
         <is>
-          <t>branches.service.ts (consolidated, branch tagging); branches.controller.ts; cust_pos_sales.branch_id; cutover/branch.ts (ToE)</t>
+          <t>wms/replenishment.service.ts parRecommendations (avg-daily-usage x lead x safety, under_buffered flag) + applyPar (writes reorder_point, planner); wms.controller.ts (/api/replenishment/par-recommendations[/apply]); schema/portal.ts branch_stock.lead_time_days + migration 0163; /replenishment par-recommendations section; cutover/wms.ts (ToE)</t>
         </is>
       </c>
       <c r="N73" s="16" t="inlineStr">
         <is>
-          <t>Inspect branch tagging completeness + the '(none)' surfacing + the GL tie.</t>
+          <t>Inspect the avg-daily-usage derivation from consumption logs, the lead-time x safety reorder-point formula, the under_buffered flag, and the planner-gated apply.</t>
         </is>
       </c>
       <c r="O73" s="16" t="inlineStr">
         <is>
-          <t>Sample period: tagged sales group by branch, an untagged sale surfaces as '(none)', consolidated total ties to posted revenue.</t>
+          <t>Re-perform: seed branch consumption (10/day) at lead 3 -&gt; recommend ROP 38 (under-buffered vs static 10); apply writes 38 onto branch_stock; tenant-isolated (re-performed by the wms harness).</t>
         </is>
       </c>
       <c r="P73" s="16" t="inlineStr">
         <is>
-          <t>Consolidation report; '(none)' investigation log</t>
+          <t>Par recommendation list + apply test</t>
         </is>
       </c>
       <c r="Q73" s="18" t="inlineStr">
@@ -7234,7 +7234,7 @@
     <row r="74">
       <c r="A74" s="11" t="inlineStr">
         <is>
-          <t>BRANCH-02</t>
+          <t>BRANCH-01</t>
         </is>
       </c>
       <c r="B74" s="12" t="inlineStr">
@@ -7254,62 +7254,62 @@
       </c>
       <c r="E74" s="12" t="inlineStr">
         <is>
-          <t>An offline terminal sells at a stale or wrong price/promotion because the cached catalog drifted from the master.</t>
+          <t>A POS sale is not attributed to its originating branch, so the consolidated branch roll-up is incomplete and cannot be tied to GL revenue.</t>
         </is>
       </c>
       <c r="F74" s="12" t="inlineStr">
         <is>
-          <t>Accuracy</t>
+          <t>Completeness</t>
         </is>
       </c>
       <c r="G74" s="12" t="inlineStr">
         <is>
-          <t>Offline master-bundle export: GET /api/branches/master-bundle returns ONLY the active price-list + active promotions, time-stamped (generated_at). The offline terminal sells from this bundle, so it cannot ring a stale/withdrawn price or promo.</t>
+          <t>Branch sale-tagging + HQ consolidation: every POS sale carries cust_pos_sales.branch_id; GET /api/branches/consolidated aggregates per branch (excluding Voided) and surfaces untagged sales as branch '(none)' — a deliberate completeness flag the controller investigates and clears before tying the consolidated total to GL revenue.</t>
         </is>
       </c>
       <c r="H74" s="13" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I74" s="13" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="J74" s="13" t="inlineStr">
         <is>
-          <t>Per bundle push</t>
+          <t>Per sale / period</t>
         </is>
       </c>
       <c r="K74" s="12" t="inlineStr">
         <is>
-          <t>HQ Controller / Pricing</t>
+          <t>HQ Controller</t>
         </is>
       </c>
       <c r="L74" s="13" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="M74" s="12" t="inlineStr">
         <is>
-          <t>branches.service.ts masterBundle (active price-list + active promos + generated_at); branches.controller.ts; cutover/branch.ts (ToE)</t>
+          <t>branches.service.ts (consolidated, branch tagging); branches.controller.ts; cust_pos_sales.branch_id; cutover/branch.ts (ToE)</t>
         </is>
       </c>
       <c r="N74" s="12" t="inlineStr">
         <is>
-          <t>Inspect the bundle exports only active prices/promos with a timestamp.</t>
+          <t>Inspect branch tagging completeness + the '(none)' surfacing + the GL tie.</t>
         </is>
       </c>
       <c r="O74" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: export the bundle; confirm it carries only active price-list/promotions + generated_at.</t>
+          <t>Sample period: tagged sales group by branch, an untagged sale surfaces as '(none)', consolidated total ties to posted revenue.</t>
         </is>
       </c>
       <c r="P74" s="12" t="inlineStr">
         <is>
-          <t>Bundle metadata; bundle vs price-master diff</t>
+          <t>Consolidation report; '(none)' investigation log</t>
         </is>
       </c>
       <c r="Q74" s="18" t="inlineStr">
@@ -7321,7 +7321,7 @@
     <row r="75">
       <c r="A75" s="15" t="inlineStr">
         <is>
-          <t>BRANCH-03</t>
+          <t>BRANCH-02</t>
         </is>
       </c>
       <c r="B75" s="16" t="inlineStr">
@@ -7336,27 +7336,27 @@
       </c>
       <c r="D75" s="16" t="inlineStr">
         <is>
-          <t>Revenue; Cash</t>
+          <t>Revenue</t>
         </is>
       </c>
       <c r="E75" s="16" t="inlineStr">
         <is>
-          <t>An offline-captured sale is LOST or DUPLICATED when connectivity returns — revenue understated (lost) or double-counted (duplicated), and the GL double-posted.</t>
+          <t>An offline terminal sells at a stale or wrong price/promotion because the cached catalog drifted from the master.</t>
         </is>
       </c>
       <c r="F75" s="16" t="inlineStr">
         <is>
-          <t>Completeness/Accuracy</t>
+          <t>Accuracy</t>
         </is>
       </c>
       <c r="G75" s="16" t="inlineStr">
         <is>
-          <t>Offline-to-online exactly-once sync: offline-captured sales replay idempotently on (tenant, client_uuid) via the pos_offline_sync dedup ledger. Two paths share the ledger — the portal/inventory POS (POST /api/portal/pos/offline-sync, item_id lines) and the touch register (POST /api/restaurant/offline-sync, menu sku lines, re-running the restaurant order→checkout so the server re-prices + 86-checks). A re-sent batch returns 'duplicate' (no second sale/GL); a failed op is a RETRYABLE tombstone (sale_no NULL) that never blocks a later replay, so a transient error is not a lost sale; each op runs in its own savepoint so one bad sale never poisons the batch.</t>
+          <t>Offline master-bundle export: GET /api/branches/master-bundle returns ONLY the active price-list + active promotions, time-stamped (generated_at). The offline terminal sells from this bundle, so it cannot ring a stale/withdrawn price or promo.</t>
         </is>
       </c>
       <c r="H75" s="17" t="inlineStr">
         <is>
-          <t>Det/Prev</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I75" s="17" t="inlineStr">
@@ -7366,37 +7366,37 @@
       </c>
       <c r="J75" s="17" t="inlineStr">
         <is>
-          <t>Per sync</t>
+          <t>Per bundle push</t>
         </is>
       </c>
       <c r="K75" s="16" t="inlineStr">
         <is>
-          <t>HQ Controller / IT</t>
+          <t>HQ Controller / Pricing</t>
         </is>
       </c>
       <c r="L75" s="17" t="inlineStr">
         <is>
-          <t>P10/P16</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="M75" s="16" t="inlineStr">
         <is>
-          <t>portal/offline-sync.service.ts (item_id path); restaurant/offline-sync.service.ts (register sku path, reuses dineIn create+checkout); pos_offline_sync dedup ledger; web lib/offline-pos.ts + lib/register-offline.ts; cutover/offline-sync.ts + restaurant-offline.ts (ToE) + e2e/register-offline.spec.ts</t>
+          <t>branches.service.ts masterBundle (active price-list + active promos + generated_at); branches.controller.ts; cutover/branch.ts (ToE)</t>
         </is>
       </c>
       <c r="N75" s="16" t="inlineStr">
         <is>
-          <t>Inspect the (tenant, client_uuid) dedup gate (sale_no NOT NULL), the per-op savepoint isolation, and the retryable-failure tombstone.</t>
+          <t>Inspect the bundle exports only active prices/promos with a timestamp.</t>
         </is>
       </c>
       <c r="O75" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: sync a batch (all synced, distinct SALE-), replay it (all duplicate, no double sale/GL), a bad op fails while neighbours sync, same uuid twice in a batch posts once, a transient failure replays to synced after the cause clears (re-performed by the offline-sync + restaurant-offline harnesses).</t>
+          <t>Re-perform: export the bundle; confirm it carries only active price-list/promotions + generated_at.</t>
         </is>
       </c>
       <c r="P75" s="16" t="inlineStr">
         <is>
-          <t>Sync recon report; terminal vs ledger counts; idempotency tests</t>
+          <t>Bundle metadata; bundle vs price-master diff</t>
         </is>
       </c>
       <c r="Q75" s="18" t="inlineStr">
@@ -7408,12 +7408,12 @@
     <row r="76">
       <c r="A76" s="11" t="inlineStr">
         <is>
-          <t>MFG-01</t>
+          <t>BRANCH-03</t>
         </is>
       </c>
       <c r="B76" s="12" t="inlineStr">
         <is>
-          <t>Manufacturing &amp; Costing</t>
+          <t>Multi-Branch &amp; Offline POS</t>
         </is>
       </c>
       <c r="C76" s="13" t="inlineStr">
@@ -7423,67 +7423,67 @@
       </c>
       <c r="D76" s="12" t="inlineStr">
         <is>
-          <t>Inventory; COGS</t>
+          <t>Revenue; Cash</t>
         </is>
       </c>
       <c r="E76" s="12" t="inlineStr">
         <is>
-          <t>Unauthorized BOM/recipe change mis-states standard cost and every downstream WIP/COGS posting; or the role that maintains the recipe also transacts on it.</t>
+          <t>An offline-captured sale is LOST or DUPLICATED when connectivity returns — revenue understated (lost) or double-counted (duplicated), and the GL double-posted.</t>
         </is>
       </c>
       <c r="F76" s="12" t="inlineStr">
         <is>
-          <t>Authorization</t>
+          <t>Completeness/Accuracy</t>
         </is>
       </c>
       <c r="G76" s="12" t="inlineStr">
         <is>
-          <t>BOM master maker-checker / SoD: the master BOM library (bom_master) is maintained + distributed by HQ separately from transacting; a tenant BOM submission is reviewed and merged by HQ on approval (a maker-checker over master data). Recipe roll-up (line cost + labor + overhead → cost per unit) is the standard-cost basis. Master-data access is segregated from production (R13).</t>
+          <t>Offline-to-online exactly-once sync: offline-captured sales replay idempotently on (tenant, client_uuid) via the pos_offline_sync dedup ledger. Two paths share the ledger — the portal/inventory POS (POST /api/portal/pos/offline-sync, item_id lines) and the touch register (POST /api/restaurant/offline-sync, menu sku lines, re-running the restaurant order→checkout so the server re-prices + 86-checks). A re-sent batch returns 'duplicate' (no second sale/GL); a failed op is a RETRYABLE tombstone (sale_no NULL) that never blocks a later replay, so a transient error is not a lost sale; each op runs in its own savepoint so one bad sale never poisons the batch.</t>
         </is>
       </c>
       <c r="H76" s="13" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det/Prev</t>
         </is>
       </c>
       <c r="I76" s="13" t="inlineStr">
         <is>
-          <t>Manual+Auto</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J76" s="13" t="inlineStr">
         <is>
-          <t>Per BOM change</t>
+          <t>Per sync</t>
         </is>
       </c>
       <c r="K76" s="12" t="inlineStr">
         <is>
-          <t>HQ MasterSteward / CostAccountant</t>
+          <t>HQ Controller / IT</t>
         </is>
       </c>
       <c r="L76" s="13" t="inlineStr">
         <is>
-          <t>P13</t>
+          <t>P10/P16</t>
         </is>
       </c>
       <c r="M76" s="12" t="inlineStr">
         <is>
-          <t>bom master + submissions (/api/bom/master, /api/bom/submissions, /api/portal/bom); manufacturing.service.ts BOM scaling; cutover/cpq.ts + manufacturing.ts (ToE)</t>
+          <t>portal/offline-sync.service.ts (item_id path); restaurant/offline-sync.service.ts (register sku path, reuses dineIn create+checkout); pos_offline_sync dedup ledger; web lib/offline-pos.ts + lib/register-offline.ts; cutover/offline-sync.ts + restaurant-offline.ts (ToE) + e2e/register-offline.spec.ts</t>
         </is>
       </c>
       <c r="N76" s="12" t="inlineStr">
         <is>
-          <t>Inspect BOM maintenance access + the submission→approve maker-checker + the costing roll-up.</t>
+          <t>Inspect the (tenant, client_uuid) dedup gate (sale_no NOT NULL), the per-op savepoint isolation, and the retryable-failure tombstone.</t>
         </is>
       </c>
       <c r="O76" s="12" t="inlineStr">
         <is>
-          <t>Sample BOM change is HQ-approved before use; standard cost rolls up correctly.</t>
+          <t>Re-perform: sync a batch (all synced, distinct SALE-), replay it (all duplicate, no double sale/GL), a bad op fails while neighbours sync, same uuid twice in a batch posts once, a transient failure replays to synced after the cause clears (re-performed by the offline-sync + restaurant-offline harnesses).</t>
         </is>
       </c>
       <c r="P76" s="12" t="inlineStr">
         <is>
-          <t>BOM approval log; costing roll-up</t>
+          <t>Sync recon report; terminal vs ledger counts; idempotency tests</t>
         </is>
       </c>
       <c r="Q76" s="18" t="inlineStr">
@@ -7495,7 +7495,7 @@
     <row r="77">
       <c r="A77" s="15" t="inlineStr">
         <is>
-          <t>MFG-02</t>
+          <t>MFG-01</t>
         </is>
       </c>
       <c r="B77" s="16" t="inlineStr">
@@ -7510,22 +7510,22 @@
       </c>
       <c r="D77" s="16" t="inlineStr">
         <is>
-          <t>WIP; Finished Goods; COGS</t>
+          <t>Inventory; COGS</t>
         </is>
       </c>
       <c r="E77" s="16" t="inlineStr">
         <is>
-          <t>Production cost is mis-stated: WIP not relieved, the conversion absorption left stranded, or a yield loss (spoilage/waste) silently capitalised into finished-goods inventory instead of expensed.</t>
+          <t>Unauthorized BOM/recipe change mis-states standard cost and every downstream WIP/COGS posting; or the role that maintains the recipe also transacts on it.</t>
         </is>
       </c>
       <c r="F77" s="16" t="inlineStr">
         <is>
-          <t>Valuation/Completeness/Accuracy</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="G77" s="16" t="inlineStr">
         <is>
-          <t>Production work-order WIP costing with a balanced JE at each step: ISSUE posts Dr 1250 WIP / Cr 1200 raw materials / Cr 2380 manufacturing-costs-applied (idempotent — re-issue is a no-op); COMPLETE posts Dr 1210 Finished Goods at the standard cost of the ACTUAL quantity produced + books the YIELD VARIANCE to 5810 (produced &lt; planned → debit 5810 loss; over-yield → credit) / Cr 1250 WIP — so WIP is always fully relieved and FG is never over-valued on a short yield. State machine Open→Released→Completed (out-of-order → BAD_STATUS). The 2380/1250 clearing balances tie out at close. Scrap/rework write-off of defective output posts to 5810 with CostAccountant authorization.</t>
+          <t>BOM master maker-checker / SoD: the master BOM library (bom_master) is maintained + distributed by HQ separately from transacting; a tenant BOM submission is reviewed and merged by HQ on approval (a maker-checker over master data). Recipe roll-up (line cost + labor + overhead → cost per unit) is the standard-cost basis. Master-data access is segregated from production (R13).</t>
         </is>
       </c>
       <c r="H77" s="17" t="inlineStr">
@@ -7535,17 +7535,17 @@
       </c>
       <c r="I77" s="17" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Manual+Auto</t>
         </is>
       </c>
       <c r="J77" s="17" t="inlineStr">
         <is>
-          <t>Per work order</t>
+          <t>Per BOM change</t>
         </is>
       </c>
       <c r="K77" s="16" t="inlineStr">
         <is>
-          <t>Warehouse / CostAccountant</t>
+          <t>HQ MasterSteward / CostAccountant</t>
         </is>
       </c>
       <c r="L77" s="17" t="inlineStr">
@@ -7555,22 +7555,22 @@
       </c>
       <c r="M77" s="16" t="inlineStr">
         <is>
-          <t>manufacturing.service.ts issue/complete (yield variance to 5810; fmt exposes yield_variance); manufacturing.controller.ts (bom_master/warehouse/exec); schema/manufacturing.ts work_orders; cutover/manufacturing.ts (ToE)</t>
+          <t>bom master + submissions (/api/bom/master, /api/bom/submissions, /api/portal/bom); manufacturing.service.ts BOM scaling; cutover/cpq.ts + manufacturing.ts (ToE)</t>
         </is>
       </c>
       <c r="N77" s="16" t="inlineStr">
         <is>
-          <t>Inspect the issue/complete JEs + the standard-unit-cost FG valuation + the yield-variance plug + the status guard.</t>
+          <t>Inspect BOM maintenance access + the submission→approve maker-checker + the costing roll-up.</t>
         </is>
       </c>
       <c r="O77" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: issue (WIP charged), complete at full yield (FG = full cost, no variance) and at a short yield (FG = std×produced, the lost yield to 5810, WIP nets to 0, TB balanced) — re-performed by the harness.</t>
+          <t>Sample BOM change is HQ-approved before use; standard cost rolls up correctly.</t>
         </is>
       </c>
       <c r="P77" s="16" t="inlineStr">
         <is>
-          <t>WO costing register (yield_variance per WO); production JEs</t>
+          <t>BOM approval log; costing roll-up</t>
         </is>
       </c>
       <c r="Q77" s="18" t="inlineStr">
@@ -7582,7 +7582,7 @@
     <row r="78">
       <c r="A78" s="11" t="inlineStr">
         <is>
-          <t>MFG-03</t>
+          <t>MFG-02</t>
         </is>
       </c>
       <c r="B78" s="12" t="inlineStr">
@@ -7597,27 +7597,27 @@
       </c>
       <c r="D78" s="12" t="inlineStr">
         <is>
-          <t>Inventory; COGS</t>
+          <t>WIP; Finished Goods; COGS</t>
         </is>
       </c>
       <c r="E78" s="12" t="inlineStr">
         <is>
-          <t>Standard-cost inventory received without isolating the price variance — actual purchase cost buried in inventory, COGS and PPV mis-stated.</t>
+          <t>Production cost is mis-stated: WIP not relieved, the conversion absorption left stranded, or a yield loss (spoilage/waste) silently capitalised into finished-goods inventory instead of expensed.</t>
         </is>
       </c>
       <c r="F78" s="12" t="inlineStr">
         <is>
-          <t>Valuation/Accuracy</t>
+          <t>Valuation/Completeness/Accuracy</t>
         </is>
       </c>
       <c r="G78" s="12" t="inlineStr">
         <is>
-          <t>Goods-receipt capitalisation under the configured costing method (FIFO/AVG/STD per tenant+item): FIFO/AVG → Dr 1200 / Cr 2000 at actual; STD → Dr 1200 at standard, the purchase-price variance booked to 5500 (unfavourable Dr / favourable Cr), Cr 2000 at actual — the PPV (5500) leg is the single balancing plug (= actual − standard, rounded once) so the JE can never reject UNBALANCED on independent per-leg rounding.</t>
+          <t>Production work-order WIP costing with a balanced JE at each step: ISSUE posts Dr 1250 WIP / Cr 1200 raw materials / Cr 2380 manufacturing-costs-applied (idempotent — re-issue is a no-op); COMPLETE posts Dr 1210 Finished Goods at the standard cost of the ACTUAL quantity produced + books the YIELD VARIANCE to 5810 (produced &lt; planned → debit 5810 loss; over-yield → credit) / Cr 1250 WIP — so WIP is always fully relieved and FG is never over-valued on a short yield. State machine Open→Released→Completed (out-of-order → BAD_STATUS). The 2380/1250 clearing balances tie out at close. Scrap/rework write-off of defective output posts to 5810 with CostAccountant authorization.</t>
         </is>
       </c>
       <c r="H78" s="13" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I78" s="13" t="inlineStr">
@@ -7627,12 +7627,12 @@
       </c>
       <c r="J78" s="13" t="inlineStr">
         <is>
-          <t>Per receipt</t>
+          <t>Per work order</t>
         </is>
       </c>
       <c r="K78" s="12" t="inlineStr">
         <is>
-          <t>CostAccountant</t>
+          <t>Warehouse / CostAccountant</t>
         </is>
       </c>
       <c r="L78" s="13" t="inlineStr">
@@ -7642,22 +7642,22 @@
       </c>
       <c r="M78" s="12" t="inlineStr">
         <is>
-          <t>costing.service.ts (config/valuation, GRV capitalisation + 5500 PPV); costing.controller.ts (masterdata); cutover/costing.ts (ToE)</t>
+          <t>manufacturing.service.ts issue/complete (yield variance to 5810; fmt exposes yield_variance); manufacturing.controller.ts (bom_master/warehouse/exec); schema/manufacturing.ts work_orders; cutover/manufacturing.ts (ToE)</t>
         </is>
       </c>
       <c r="N78" s="12" t="inlineStr">
         <is>
-          <t>Inspect the per-method capitalisation routing + the PPV plug.</t>
+          <t>Inspect the issue/complete JEs + the standard-unit-cost FG valuation + the yield-variance plug + the status guard.</t>
         </is>
       </c>
       <c r="O78" s="12" t="inlineStr">
         <is>
-          <t>Re-perform a STD receipt at actual ≠ standard → PPV isolated to 5500, JE balanced; valuation ties to GL 1200/1210/1250.</t>
+          <t>Re-perform: issue (WIP charged), complete at full yield (FG = full cost, no variance) and at a short yield (FG = std×produced, the lost yield to 5810, WIP nets to 0, TB balanced) — re-performed by the harness.</t>
         </is>
       </c>
       <c r="P78" s="12" t="inlineStr">
         <is>
-          <t>PPV postings; costing valuation</t>
+          <t>WO costing register (yield_variance per WO); production JEs</t>
         </is>
       </c>
       <c r="Q78" s="18" t="inlineStr">
@@ -7669,12 +7669,12 @@
     <row r="79">
       <c r="A79" s="15" t="inlineStr">
         <is>
-          <t>PROJ-01</t>
+          <t>MFG-03</t>
         </is>
       </c>
       <c r="B79" s="16" t="inlineStr">
         <is>
-          <t>Project Accounting</t>
+          <t>Manufacturing &amp; Costing</t>
         </is>
       </c>
       <c r="C79" s="17" t="inlineStr">
@@ -7684,27 +7684,27 @@
       </c>
       <c r="D79" s="16" t="inlineStr">
         <is>
-          <t>Project WIP; COGS</t>
+          <t>Inventory; COGS</t>
         </is>
       </c>
       <c r="E79" s="16" t="inlineStr">
         <is>
-          <t>Project cost mis-stated: a recoverable cost not captured, or an UN-recoverable (non-billable) cost capitalised into project WIP as an asset that overstates the unbilled balance and inflates margin.</t>
+          <t>Standard-cost inventory received without isolating the price variance — actual purchase cost buried in inventory, COGS and PPV mis-stated.</t>
         </is>
       </c>
       <c r="F79" s="16" t="inlineStr">
         <is>
-          <t>Valuation/Accuracy/Completeness</t>
+          <t>Valuation/Accuracy</t>
         </is>
       </c>
       <c r="G79" s="16" t="inlineStr">
         <is>
-          <t>Project cost capture with a balanced JE and a billable/non-billable split: a BILLABLE time/expense cost is a recoverable asset → Dr 1260 Project WIP / Cr 2390 Project Costs Applied (accumulates in cost_to_date, relieved to COGS at billing); a NON-BILLABLE cost is unrecoverable → EXPENSED immediately Dr 5800 Project Cost of Services / Cr 2390 (never enters the billable WIP), so the register's total_cost and true margin (billed − recognised − non-billable) reflect the absorbed cost. A non-positive amount → BAD_AMOUNT; first cost flips Open→Active.</t>
+          <t>Goods-receipt capitalisation under the configured costing method (FIFO/AVG/STD per tenant+item): FIFO/AVG → Dr 1200 / Cr 2000 at actual; STD → Dr 1200 at standard, the purchase-price variance booked to 5500 (unfavourable Dr / favourable Cr), Cr 2000 at actual — the PPV (5500) leg is the single balancing plug (= actual − standard, rounded once) so the JE can never reject UNBALANCED on independent per-leg rounding.</t>
         </is>
       </c>
       <c r="H79" s="17" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I79" s="17" t="inlineStr">
@@ -7714,12 +7714,12 @@
       </c>
       <c r="J79" s="17" t="inlineStr">
         <is>
-          <t>Per cost entry</t>
+          <t>Per receipt</t>
         </is>
       </c>
       <c r="K79" s="16" t="inlineStr">
         <is>
-          <t>ProjectAccountant</t>
+          <t>CostAccountant</t>
         </is>
       </c>
       <c r="L79" s="17" t="inlineStr">
@@ -7729,22 +7729,22 @@
       </c>
       <c r="M79" s="16" t="inlineStr">
         <is>
-          <t>projects.service.ts logCost (billable→1260, non-billable→5800; fmt exposes non_billable_cost/total_cost/margin); projects.controller.ts; schema/projects.ts project_entries.billable; cutover/projects.ts (ToE)</t>
+          <t>costing.service.ts (config/valuation, GRV capitalisation + 5500 PPV); costing.controller.ts (masterdata); cutover/costing.ts (ToE)</t>
         </is>
       </c>
       <c r="N79" s="16" t="inlineStr">
         <is>
-          <t>Inspect the billable/non-billable GL routing + the WIP vs immediate-expense decision + the margin roll-up.</t>
+          <t>Inspect the per-method capitalisation routing + the PPV plug.</t>
         </is>
       </c>
       <c r="O79" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: a billable cost capitalises to 1260; a non-billable cost expenses to 5800 (NOT WIP), cost_to_date unchanged, and the project margin absorbs it (re-performed by the harness).</t>
+          <t>Re-perform a STD receipt at actual ≠ standard → PPV isolated to 5500, JE balanced; valuation ties to GL 1200/1210/1250.</t>
         </is>
       </c>
       <c r="P79" s="16" t="inlineStr">
         <is>
-          <t>Project cost JEs; cost register (non_billable_cost)</t>
+          <t>PPV postings; costing valuation</t>
         </is>
       </c>
       <c r="Q79" s="18" t="inlineStr">
@@ -7756,7 +7756,7 @@
     <row r="80">
       <c r="A80" s="11" t="inlineStr">
         <is>
-          <t>PROJ-02</t>
+          <t>PROJ-01</t>
         </is>
       </c>
       <c r="B80" s="12" t="inlineStr">
@@ -7771,22 +7771,22 @@
       </c>
       <c r="D80" s="12" t="inlineStr">
         <is>
-          <t>Project WIP; Revenue; COGS</t>
+          <t>Project WIP; COGS</t>
         </is>
       </c>
       <c r="E80" s="12" t="inlineStr">
         <is>
-          <t>Revenue billed without matching cost — WIP not relieved, cost of services mis-stated, margin overstated.</t>
+          <t>Project cost mis-stated: a recoverable cost not captured, or an UN-recoverable (non-billable) cost capitalised into project WIP as an asset that overstates the unbilled balance and inflates margin.</t>
         </is>
       </c>
       <c r="F80" s="12" t="inlineStr">
         <is>
-          <t>Accuracy/Cut-off</t>
+          <t>Valuation/Accuracy/Completeness</t>
         </is>
       </c>
       <c r="G80" s="12" t="inlineStr">
         <is>
-          <t>Customer billing recognises revenue (Dr 1100 AR / Cr 4200 Project Revenue) and relieves the unbilled WIP to cost of services up to the unrecognised billable cost (Dr 5800 / Cr 1260) in the same event — matching cost to recognised revenue. Billing is by raw amount (T&amp;M) or by PERCENT of the contract for Fixed-price milestone billing; a Fixed-price contract is CAPPED at the contract value (cumulative billing can never exceed it — BILL_EXCEEDS_CONTRACT), so the customer is never over-billed (billed_pct/remaining_to_bill on the register). Billing is idempotent on (project, cumulative billed amount).</t>
+          <t>Project cost capture with a balanced JE and a billable/non-billable split: a BILLABLE time/expense cost is a recoverable asset → Dr 1260 Project WIP / Cr 2390 Project Costs Applied (accumulates in cost_to_date, relieved to COGS at billing); a NON-BILLABLE cost is unrecoverable → EXPENSED immediately Dr 5800 Project Cost of Services / Cr 2390 (never enters the billable WIP), so the register's total_cost and true margin (billed − recognised − non-billable) reflect the absorbed cost. A non-positive amount → BAD_AMOUNT; first cost flips Open→Active.</t>
         </is>
       </c>
       <c r="H80" s="13" t="inlineStr">
@@ -7801,12 +7801,12 @@
       </c>
       <c r="J80" s="13" t="inlineStr">
         <is>
-          <t>Per billing</t>
+          <t>Per cost entry</t>
         </is>
       </c>
       <c r="K80" s="12" t="inlineStr">
         <is>
-          <t>ProjectController / ArSpecialist</t>
+          <t>ProjectAccountant</t>
         </is>
       </c>
       <c r="L80" s="13" t="inlineStr">
@@ -7816,22 +7816,22 @@
       </c>
       <c r="M80" s="12" t="inlineStr">
         <is>
-          <t>projects.service.ts bill (revenue + WIP relief, idempotent); projects.controller.ts (R07 vs cost initiation); cutover/projects.ts (ToE)</t>
+          <t>projects.service.ts logCost (billable→1260, non-billable→5800; fmt exposes non_billable_cost/total_cost/margin); projects.controller.ts; schema/projects.ts project_entries.billable; cutover/projects.ts (ToE)</t>
         </is>
       </c>
       <c r="N80" s="12" t="inlineStr">
         <is>
-          <t>Inspect the bill JE + the WIP-relief matching + idempotency.</t>
+          <t>Inspect the billable/non-billable GL routing + the WIP vs immediate-expense decision + the margin roll-up.</t>
         </is>
       </c>
       <c r="O80" s="12" t="inlineStr">
         <is>
-          <t>Re-perform a billing → revenue recognised, WIP relieved to 5800 up to unrecognised cost, 1260 reduced; margin = billed − recognised cost (re-performed by the harness).</t>
+          <t>Re-perform: a billable cost capitalises to 1260; a non-billable cost expenses to 5800 (NOT WIP), cost_to_date unchanged, and the project margin absorbs it (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P80" s="12" t="inlineStr">
         <is>
-          <t>Billing JEs; margin/WIP measurement</t>
+          <t>Project cost JEs; cost register (non_billable_cost)</t>
         </is>
       </c>
       <c r="Q80" s="18" t="inlineStr">
@@ -7843,7 +7843,7 @@
     <row r="81">
       <c r="A81" s="15" t="inlineStr">
         <is>
-          <t>PROJ-03</t>
+          <t>PROJ-02</t>
         </is>
       </c>
       <c r="B81" s="16" t="inlineStr">
@@ -7853,171 +7853,171 @@
       </c>
       <c r="C81" s="17" t="inlineStr">
         <is>
-          <t>Detective</t>
+          <t>Application</t>
         </is>
       </c>
       <c r="D81" s="16" t="inlineStr">
         <is>
-          <t>Project WIP</t>
+          <t>Project WIP; Revenue; COGS</t>
         </is>
       </c>
       <c r="E81" s="16" t="inlineStr">
         <is>
-          <t>Unbilled WIP (1260) and the 2390 clearing balance not reviewed at close — stale or unrecoverable WIP carried into the financial statements.</t>
+          <t>Revenue billed without matching cost — WIP not relieved, cost of services mis-stated, margin overstated.</t>
         </is>
       </c>
       <c r="F81" s="16" t="inlineStr">
         <is>
-          <t>Valuation</t>
+          <t>Accuracy/Cut-off</t>
         </is>
       </c>
       <c r="G81" s="16" t="inlineStr">
         <is>
-          <t>Period-end review of unbilled-WIP (1260) aging and the project-costs-applied (2390) clearing tie-out; project margin (billed_to_date − recognised_cost − non-billable) reviewed at close. SoD: billing authorisation is segregated from cost initiation (R07).</t>
+          <t>Customer billing recognises revenue (Dr 1100 AR / Cr 4200 Project Revenue) and relieves the unbilled WIP to cost of services up to the unrecognised billable cost (Dr 5800 / Cr 1260) in the same event — matching cost to recognised revenue. Billing is by raw amount (T&amp;M) or by PERCENT of the contract for Fixed-price milestone billing; a Fixed-price contract is CAPPED at the contract value (cumulative billing can never exceed it — BILL_EXCEEDS_CONTRACT), so the customer is never over-billed (billed_pct/remaining_to_bill on the register). Billing is idempotent on (project, cumulative billed amount).</t>
         </is>
       </c>
       <c r="H81" s="17" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I81" s="17" t="inlineStr">
         <is>
-          <t>Hybrid</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J81" s="17" t="inlineStr">
         <is>
-          <t>Period</t>
+          <t>Per billing</t>
         </is>
       </c>
       <c r="K81" s="16" t="inlineStr">
         <is>
-          <t>ProjectAccountant / Controller</t>
+          <t>ProjectController / ArSpecialist</t>
         </is>
       </c>
       <c r="L81" s="17" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>P13</t>
         </is>
       </c>
       <c r="M81" s="16" t="inlineStr">
         <is>
-          <t>projects.service.ts fmt (wip/margin); the project register + entries; close review</t>
+          <t>projects.service.ts bill (revenue + WIP relief, idempotent); projects.controller.ts (R07 vs cost initiation); cutover/projects.ts (ToE)</t>
         </is>
       </c>
       <c r="N81" s="16" t="inlineStr">
         <is>
-          <t>Inspect 1260 aging + 2390 clearing + margin review evidence.</t>
+          <t>Inspect the bill JE + the WIP-relief matching + idempotency.</t>
         </is>
       </c>
       <c r="O81" s="16" t="inlineStr">
         <is>
-          <t>Sample projects: 1260 WIP agrees to cost_to_date − recognised; 2390 clears; stale WIP investigated.</t>
+          <t>Re-perform a billing → revenue recognised, WIP relieved to 5800 up to unrecognised cost, 1260 reduced; margin = billed − recognised cost (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P81" s="16" t="inlineStr">
         <is>
-          <t>WIP aging; 2390 clearing tie-out</t>
-        </is>
-      </c>
-      <c r="Q81" s="19" t="inlineStr">
-        <is>
-          <t>Partial</t>
+          <t>Billing JEs; margin/WIP measurement</t>
+        </is>
+      </c>
+      <c r="Q81" s="18" t="inlineStr">
+        <is>
+          <t>Implemented</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="11" t="inlineStr">
         <is>
-          <t>GL-01</t>
+          <t>PROJ-03</t>
         </is>
       </c>
       <c r="B82" s="12" t="inlineStr">
         <is>
-          <t>General Ledger</t>
+          <t>Project Accounting</t>
         </is>
       </c>
       <c r="C82" s="13" t="inlineStr">
         <is>
-          <t>Application</t>
+          <t>Detective</t>
         </is>
       </c>
       <c r="D82" s="12" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Project WIP</t>
         </is>
       </c>
       <c r="E82" s="12" t="inlineStr">
         <is>
-          <t>Unbalanced / one-sided journal entries.</t>
+          <t>Unbilled WIP (1260) and the 2390 clearing balance not reviewed at close — stale or unrecoverable WIP carried into the financial statements.</t>
         </is>
       </c>
       <c r="F82" s="12" t="inlineStr">
         <is>
-          <t>Accuracy</t>
+          <t>Valuation</t>
         </is>
       </c>
       <c r="G82" s="12" t="inlineStr">
         <is>
-          <t>Double-entry balanced-by-construction — Σdebit=Σcredit enforced; each line single-sided &amp; non-negative.</t>
+          <t>Period-end review of unbilled-WIP (1260) aging and the project-costs-applied (2390) clearing tie-out; project margin (billed_to_date − recognised_cost − non-billable) reviewed at close. SoD: billing authorisation is segregated from cost initiation (R07).</t>
         </is>
       </c>
       <c r="H82" s="13" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I82" s="13" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Hybrid</t>
         </is>
       </c>
       <c r="J82" s="13" t="inlineStr">
         <is>
-          <t>Per JE</t>
+          <t>Period</t>
         </is>
       </c>
       <c r="K82" s="12" t="inlineStr">
         <is>
-          <t>Controller</t>
+          <t>ProjectAccountant / Controller</t>
         </is>
       </c>
       <c r="L82" s="13" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="M82" s="12" t="inlineStr">
         <is>
-          <t>ledger.service.ts (postEntry — UNBALANCED / INVALID_LINE)</t>
+          <t>projects.service.ts fmt (wip/margin); the project register + entries; close review</t>
         </is>
       </c>
       <c r="N82" s="12" t="inlineStr">
         <is>
-          <t>Inspect balance + line invariants.</t>
+          <t>Inspect 1260 aging + 2390 clearing + margin review evidence.</t>
         </is>
       </c>
       <c r="O82" s="12" t="inlineStr">
         <is>
-          <t>Attempt unbalanced JE → rejected.</t>
+          <t>Sample projects: 1260 WIP agrees to cost_to_date − recognised; 2390 clears; stale WIP investigated.</t>
         </is>
       </c>
       <c r="P82" s="12" t="inlineStr">
         <is>
-          <t>Invariant test</t>
-        </is>
-      </c>
-      <c r="Q82" s="18" t="inlineStr">
-        <is>
-          <t>Implemented</t>
+          <t>WIP aging; 2390 clearing tie-out</t>
+        </is>
+      </c>
+      <c r="Q82" s="19" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="15" t="inlineStr">
         <is>
-          <t>GL-02</t>
+          <t>GL-01</t>
         </is>
       </c>
       <c r="B83" s="16" t="inlineStr">
@@ -8037,17 +8037,17 @@
       </c>
       <c r="E83" s="16" t="inlineStr">
         <is>
-          <t>Postings to a closed period distort reported results.</t>
+          <t>Unbalanced / one-sided journal entries.</t>
         </is>
       </c>
       <c r="F83" s="16" t="inlineStr">
         <is>
-          <t>Cutoff</t>
+          <t>Accuracy</t>
         </is>
       </c>
       <c r="G83" s="16" t="inlineStr">
         <is>
-          <t>Period-close lockout — postings to a CLOSED fiscal period are rejected (per-tenant calendar).</t>
+          <t>Double-entry balanced-by-construction — Σdebit=Σcredit enforced; each line single-sided &amp; non-negative.</t>
         </is>
       </c>
       <c r="H83" s="17" t="inlineStr">
@@ -8077,22 +8077,22 @@
       </c>
       <c r="M83" s="16" t="inlineStr">
         <is>
-          <t>ledger.service.ts (postEntry PERIOD_CLOSED); fiscal_periods</t>
+          <t>ledger.service.ts (postEntry — UNBALANCED / INVALID_LINE)</t>
         </is>
       </c>
       <c r="N83" s="16" t="inlineStr">
         <is>
-          <t>Inspect close check.</t>
+          <t>Inspect balance + line invariants.</t>
         </is>
       </c>
       <c r="O83" s="16" t="inlineStr">
         <is>
-          <t>Post to closed period → rejected; review exceptions.</t>
+          <t>Attempt unbalanced JE → rejected.</t>
         </is>
       </c>
       <c r="P83" s="16" t="inlineStr">
         <is>
-          <t>Close-lock test</t>
+          <t>Invariant test</t>
         </is>
       </c>
       <c r="Q83" s="18" t="inlineStr">
@@ -8104,7 +8104,7 @@
     <row r="84">
       <c r="A84" s="11" t="inlineStr">
         <is>
-          <t>GL-03</t>
+          <t>GL-02</t>
         </is>
       </c>
       <c r="B84" s="12" t="inlineStr">
@@ -8119,22 +8119,22 @@
       </c>
       <c r="D84" s="12" t="inlineStr">
         <is>
-          <t>Equity</t>
+          <t>All</t>
         </is>
       </c>
       <c r="E84" s="12" t="inlineStr">
         <is>
-          <t>Unauthorized year-end close / RE roll.</t>
+          <t>Postings to a closed period distort reported results.</t>
         </is>
       </c>
       <c r="F84" s="12" t="inlineStr">
         <is>
-          <t>Cutoff/Authorization</t>
+          <t>Cutoff</t>
         </is>
       </c>
       <c r="G84" s="12" t="inlineStr">
         <is>
-          <t>Year-end close restricted to 'exec'; closing entries roll to retained earnings.</t>
+          <t>Period-close lockout — postings to a CLOSED fiscal period are rejected (per-tenant calendar).</t>
         </is>
       </c>
       <c r="H84" s="13" t="inlineStr">
@@ -8144,42 +8144,42 @@
       </c>
       <c r="I84" s="13" t="inlineStr">
         <is>
-          <t>Auto+Manual</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J84" s="13" t="inlineStr">
         <is>
-          <t>Annual</t>
+          <t>Per JE</t>
         </is>
       </c>
       <c r="K84" s="12" t="inlineStr">
         <is>
-          <t>CFO / Controller</t>
+          <t>Controller</t>
         </is>
       </c>
       <c r="L84" s="13" t="inlineStr">
         <is>
-          <t>P10/P11</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="M84" s="12" t="inlineStr">
         <is>
-          <t>ledger.controller.ts (close-year @Permissions exec); closeYear</t>
+          <t>ledger.service.ts (postEntry PERIOD_CLOSED); fiscal_periods</t>
         </is>
       </c>
       <c r="N84" s="12" t="inlineStr">
         <is>
-          <t>Inspect permission + closing logic.</t>
+          <t>Inspect close check.</t>
         </is>
       </c>
       <c r="O84" s="12" t="inlineStr">
         <is>
-          <t>Attempt close w/o exec → 403; review annual close.</t>
+          <t>Post to closed period → rejected; review exceptions.</t>
         </is>
       </c>
       <c r="P84" s="12" t="inlineStr">
         <is>
-          <t>Close package</t>
+          <t>Close-lock test</t>
         </is>
       </c>
       <c r="Q84" s="18" t="inlineStr">
@@ -8191,7 +8191,7 @@
     <row r="85">
       <c r="A85" s="15" t="inlineStr">
         <is>
-          <t>GL-04</t>
+          <t>GL-03</t>
         </is>
       </c>
       <c r="B85" s="16" t="inlineStr">
@@ -8206,22 +8206,22 @@
       </c>
       <c r="D85" s="16" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Equity</t>
         </is>
       </c>
       <c r="E85" s="16" t="inlineStr">
         <is>
-          <t>Concurrent posting double-books the same source doc.</t>
+          <t>Unauthorized year-end close / RE roll.</t>
         </is>
       </c>
       <c r="F85" s="16" t="inlineStr">
         <is>
-          <t>Completeness/Accuracy</t>
+          <t>Cutoff/Authorization</t>
         </is>
       </c>
       <c r="G85" s="16" t="inlineStr">
         <is>
-          <t>Ledger idempotency — UNIQUE (tenant,source,source_ref,ledger) + ON CONFLICT DO NOTHING in postEntry.</t>
+          <t>Year-end close restricted to 'exec'; closing entries roll to retained earnings.</t>
         </is>
       </c>
       <c r="H85" s="17" t="inlineStr">
@@ -8231,42 +8231,42 @@
       </c>
       <c r="I85" s="17" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="J85" s="17" t="inlineStr">
         <is>
-          <t>Per JE</t>
+          <t>Annual</t>
         </is>
       </c>
       <c r="K85" s="16" t="inlineStr">
         <is>
-          <t>Eng Lead / Controller</t>
+          <t>CFO / Controller</t>
         </is>
       </c>
       <c r="L85" s="17" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P10/P11</t>
         </is>
       </c>
       <c r="M85" s="16" t="inlineStr">
         <is>
-          <t>schema/ledger.ts (ux_je_idem); ledger.service.ts; migration 0058</t>
+          <t>ledger.controller.ts (close-year @Permissions exec); closeYear</t>
         </is>
       </c>
       <c r="N85" s="16" t="inlineStr">
         <is>
-          <t>Inspect unique index + conflict handling.</t>
+          <t>Inspect permission + closing logic.</t>
         </is>
       </c>
       <c r="O85" s="16" t="inlineStr">
         <is>
-          <t>Concurrent identical post → single entry.</t>
+          <t>Attempt close w/o exec → 403; review annual close.</t>
         </is>
       </c>
       <c r="P85" s="16" t="inlineStr">
         <is>
-          <t>Dedup test</t>
+          <t>Close package</t>
         </is>
       </c>
       <c r="Q85" s="18" t="inlineStr">
@@ -8278,7 +8278,7 @@
     <row r="86">
       <c r="A86" s="11" t="inlineStr">
         <is>
-          <t>GL-05</t>
+          <t>GL-04</t>
         </is>
       </c>
       <c r="B86" s="12" t="inlineStr">
@@ -8298,17 +8298,17 @@
       </c>
       <c r="E86" s="12" t="inlineStr">
         <is>
-          <t>Manual JE posted without independent review (override risk).</t>
+          <t>Concurrent posting double-books the same source doc.</t>
         </is>
       </c>
       <c r="F86" s="12" t="inlineStr">
         <is>
-          <t>Authorization</t>
+          <t>Completeness/Accuracy</t>
         </is>
       </c>
       <c r="G86" s="12" t="inlineStr">
         <is>
-          <t>Manual journal-entry maker-checker — preparer ≠ approver before a manual JE posts.</t>
+          <t>Ledger idempotency — UNIQUE (tenant,source,source_ref,ledger) + ON CONFLICT DO NOTHING in postEntry.</t>
         </is>
       </c>
       <c r="H86" s="13" t="inlineStr">
@@ -8318,17 +8318,17 @@
       </c>
       <c r="I86" s="13" t="inlineStr">
         <is>
-          <t>Auto+Manual</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J86" s="13" t="inlineStr">
         <is>
-          <t>Per manual JE</t>
+          <t>Per JE</t>
         </is>
       </c>
       <c r="K86" s="12" t="inlineStr">
         <is>
-          <t>Controller</t>
+          <t>Eng Lead / Controller</t>
         </is>
       </c>
       <c r="L86" s="13" t="inlineStr">
@@ -8338,22 +8338,22 @@
       </c>
       <c r="M86" s="12" t="inlineStr">
         <is>
-          <t>ledger.service.ts (postEntry pendingApproval→Draft; approveEntry preparer≠approver; rejectEntry); ledger.controller.ts (gl_post posts / gl_close approves); cutover/compliance.ts (ToE)</t>
+          <t>schema/ledger.ts (ux_je_idem); ledger.service.ts; migration 0058</t>
         </is>
       </c>
       <c r="N86" s="12" t="inlineStr">
         <is>
-          <t>Inspect JE approval routing.</t>
+          <t>Inspect unique index + conflict handling.</t>
         </is>
       </c>
       <c r="O86" s="12" t="inlineStr">
         <is>
-          <t>Sample manual JEs: approver ≠ preparer; Draft excluded from balances until approved (re-performed by the harness).</t>
+          <t>Concurrent identical post → single entry.</t>
         </is>
       </c>
       <c r="P86" s="12" t="inlineStr">
         <is>
-          <t>JE approvals</t>
+          <t>Dedup test</t>
         </is>
       </c>
       <c r="Q86" s="18" t="inlineStr">
@@ -8365,7 +8365,7 @@
     <row r="87">
       <c r="A87" s="15" t="inlineStr">
         <is>
-          <t>GL-06</t>
+          <t>GL-05</t>
         </is>
       </c>
       <c r="B87" s="16" t="inlineStr">
@@ -8385,17 +8385,17 @@
       </c>
       <c r="E87" s="16" t="inlineStr">
         <is>
-          <t>Operator mis-posts to another tenant's books.</t>
+          <t>Manual JE posted without independent review (override risk).</t>
         </is>
       </c>
       <c r="F87" s="16" t="inlineStr">
         <is>
-          <t>Validity</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="G87" s="16" t="inlineStr">
         <is>
-          <t>HQ cross-tenant posting gated to Admin (explicit tenant override); others pinned to context (also RLS).</t>
+          <t>Manual journal-entry maker-checker — preparer ≠ approver before a manual JE posts.</t>
         </is>
       </c>
       <c r="H87" s="17" t="inlineStr">
@@ -8405,42 +8405,42 @@
       </c>
       <c r="I87" s="17" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="J87" s="17" t="inlineStr">
         <is>
-          <t>Per JE</t>
+          <t>Per manual JE</t>
         </is>
       </c>
       <c r="K87" s="16" t="inlineStr">
         <is>
-          <t>Eng Lead</t>
+          <t>Controller</t>
         </is>
       </c>
       <c r="L87" s="17" t="inlineStr">
         <is>
-          <t>P10/P11</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="M87" s="16" t="inlineStr">
         <is>
-          <t>ledger.controller.ts (hqTenant)</t>
+          <t>ledger.service.ts (postEntry pendingApproval→Draft; approveEntry preparer≠approver; rejectEntry); ledger.controller.ts (gl_post posts / gl_close approves); cutover/compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N87" s="16" t="inlineStr">
         <is>
-          <t>Inspect Admin gating of tenant_id.</t>
+          <t>Inspect JE approval routing.</t>
         </is>
       </c>
       <c r="O87" s="16" t="inlineStr">
         <is>
-          <t>Non-Admin tenant override ignored; Admin audited.</t>
+          <t>Sample manual JEs: approver ≠ preparer; Draft excluded from balances until approved (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P87" s="16" t="inlineStr">
         <is>
-          <t>Override test</t>
+          <t>JE approvals</t>
         </is>
       </c>
       <c r="Q87" s="18" t="inlineStr">
@@ -8452,7 +8452,7 @@
     <row r="88">
       <c r="A88" s="11" t="inlineStr">
         <is>
-          <t>GL-07</t>
+          <t>GL-06</t>
         </is>
       </c>
       <c r="B88" s="12" t="inlineStr">
@@ -8467,27 +8467,27 @@
       </c>
       <c r="D88" s="12" t="inlineStr">
         <is>
-          <t>Cash</t>
+          <t>All</t>
         </is>
       </c>
       <c r="E88" s="12" t="inlineStr">
         <is>
-          <t>Statement of cash flows mis-stated or doesn't tie to the change in cash.</t>
+          <t>Operator mis-posts to another tenant's books.</t>
         </is>
       </c>
       <c r="F88" s="12" t="inlineStr">
         <is>
-          <t>Accuracy/Completeness</t>
+          <t>Validity</t>
         </is>
       </c>
       <c r="G88" s="12" t="inlineStr">
         <is>
-          <t>Statement of Cash Flows (indirect) reconstructed from the GL: net income + non-cash add-backs + working-capital + investing + financing; year-end CLOSE entries excluded; reconciles to Δcash (1000/1010/1020) by construction with a `reconciled` tie-out flag. A direct-method view presents the same operating cash by receipt/payment nature (receipts from customers, payments to suppliers, tax &amp; payroll) and also reconciles to Δcash; a forward cash-flow forecast projects open AR (inflows) and AP (outflows) by due date from today's cash balance for treasury/collections planning.</t>
+          <t>HQ cross-tenant posting gated to Admin (explicit tenant override); others pinned to context (also RLS).</t>
         </is>
       </c>
       <c r="H88" s="13" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I88" s="13" t="inlineStr">
@@ -8497,37 +8497,37 @@
       </c>
       <c r="J88" s="13" t="inlineStr">
         <is>
-          <t>Per period</t>
+          <t>Per JE</t>
         </is>
       </c>
       <c r="K88" s="12" t="inlineStr">
         <is>
-          <t>Controller</t>
+          <t>Eng Lead</t>
         </is>
       </c>
       <c r="L88" s="13" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P10/P11</t>
         </is>
       </c>
       <c r="M88" s="12" t="inlineStr">
         <is>
-          <t>ledger.service.ts (cashFlowStatement, cashFlowDirect, cashFlowForecast); ledger.controller.ts (GET cash-flow, cash-flow-direct, cash-flow-forecast); cutover/basics.ts (ToE)</t>
+          <t>ledger.controller.ts (hqTenant)</t>
         </is>
       </c>
       <c r="N88" s="12" t="inlineStr">
         <is>
-          <t>Inspect SCF derivation + reconciliation flag; inspect direct-method bucketing and forecast projection.</t>
+          <t>Inspect Admin gating of tenant_id.</t>
         </is>
       </c>
       <c r="O88" s="12" t="inlineStr">
         <is>
-          <t>Run cash-flow over a seeded period — activities tie to the movement in cash; CLOSE excluded; direct method ties to the same operating cash and Δcash; forecast buckets open AR/AP by due week (re-performed by the harness).</t>
+          <t>Non-Admin tenant override ignored; Admin audited.</t>
         </is>
       </c>
       <c r="P88" s="12" t="inlineStr">
         <is>
-          <t>Cash-flow reconciliation; direct-method buckets; forecast schedule</t>
+          <t>Override test</t>
         </is>
       </c>
       <c r="Q88" s="18" t="inlineStr">
@@ -8539,7 +8539,7 @@
     <row r="89">
       <c r="A89" s="15" t="inlineStr">
         <is>
-          <t>GL-08</t>
+          <t>GL-07</t>
         </is>
       </c>
       <c r="B89" s="16" t="inlineStr">
@@ -8554,27 +8554,27 @@
       </c>
       <c r="D89" s="16" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Cash</t>
         </is>
       </c>
       <c r="E89" s="16" t="inlineStr">
         <is>
-          <t>Standing/period accruals missed, posted unbalanced, or posted without approval; manual re-keying error.</t>
+          <t>Statement of cash flows mis-stated or doesn't tie to the change in cash.</t>
         </is>
       </c>
       <c r="F89" s="16" t="inlineStr">
         <is>
-          <t>Completeness/Accuracy/Authorization</t>
+          <t>Accuracy/Completeness</t>
         </is>
       </c>
       <c r="G89" s="16" t="inlineStr">
         <is>
-          <t>Recurring/template journal entries: a template's lines are validated balanced (Σdebit=Σcredit) AT SAVE TIME (unbalanced → UNBALANCED), so a broken template can never be persisted. The scheduled job gl_recurring_journals (cron / daily scheduler) posts every due template as a DRAFT JE through the normal maker-checker flow (GL-05) — a different user must approve before it affects balances — and rolls next_run_date forward. Idempotent: next_run_date advanced on posting + the (tenant,source,source_ref,ledger) idempotency key dedupes a same-day re-run. Templates can be paused/resumed without losing history.</t>
+          <t>Statement of Cash Flows (indirect) reconstructed from the GL: net income + non-cash add-backs + working-capital + investing + financing; year-end CLOSE entries excluded; reconciles to Δcash (1000/1010/1020) by construction with a `reconciled` tie-out flag. A direct-method view presents the same operating cash by receipt/payment nature (receipts from customers, payments to suppliers, tax &amp; payroll) and also reconciles to Δcash; a forward cash-flow forecast projects open AR (inflows) and AP (outflows) by due date from today's cash balance for treasury/collections planning.</t>
         </is>
       </c>
       <c r="H89" s="17" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I89" s="17" t="inlineStr">
@@ -8584,7 +8584,7 @@
       </c>
       <c r="J89" s="17" t="inlineStr">
         <is>
-          <t>Per due date / per template</t>
+          <t>Per period</t>
         </is>
       </c>
       <c r="K89" s="16" t="inlineStr">
@@ -8599,22 +8599,22 @@
       </c>
       <c r="M89" s="16" t="inlineStr">
         <is>
-          <t>ledger.service.ts (createRecurring balanced-at-save, runDueRecurring→postEntry pendingApproval, setRecurringActive); ledger.controller.ts (gl_post creates/runs); bi.service.ts (gl_recurring_journals); schema/ledger.ts (recurring_journals) + migration 0119; cutover/basics.ts (ToE)</t>
+          <t>ledger.service.ts (cashFlowStatement, cashFlowDirect, cashFlowForecast); ledger.controller.ts (GET cash-flow, cash-flow-direct, cash-flow-forecast); cutover/basics.ts (ToE)</t>
         </is>
       </c>
       <c r="N89" s="16" t="inlineStr">
         <is>
-          <t>Inspect template balance validation + scheduled posting as Draft + idempotency.</t>
+          <t>Inspect SCF derivation + reconciliation flag; inspect direct-method bucketing and forecast projection.</t>
         </is>
       </c>
       <c r="O89" s="16" t="inlineStr">
         <is>
-          <t>Unbalanced template → UNBALANCED; due template posts a Draft JE (excluded from TB) into the pending queue; re-run posts nothing; a second user approves → accrual hits the GL (re-performed by the harness).</t>
+          <t>Run cash-flow over a seeded period — activities tie to the movement in cash; CLOSE excluded; direct method ties to the same operating cash and Δcash; forecast buckets open AR/AP by due week (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P89" s="16" t="inlineStr">
         <is>
-          <t>Recurring-journal templates; scheduled run log; JE approvals</t>
+          <t>Cash-flow reconciliation; direct-method buckets; forecast schedule</t>
         </is>
       </c>
       <c r="Q89" s="18" t="inlineStr">
@@ -8626,7 +8626,7 @@
     <row r="90">
       <c r="A90" s="11" t="inlineStr">
         <is>
-          <t>GL-09</t>
+          <t>GL-08</t>
         </is>
       </c>
       <c r="B90" s="12" t="inlineStr">
@@ -8641,27 +8641,27 @@
       </c>
       <c r="D90" s="12" t="inlineStr">
         <is>
-          <t>Prepaid expenses; Operating expense</t>
+          <t>All</t>
         </is>
       </c>
       <c r="E90" s="12" t="inlineStr">
         <is>
-          <t>Prepaid expense not amortized over its term — expense mis-stated, prepaid asset overstated.</t>
+          <t>Standing/period accruals missed, posted unbalanced, or posted without approval; manual re-keying error.</t>
         </is>
       </c>
       <c r="F90" s="12" t="inlineStr">
         <is>
-          <t>Accuracy/Completeness</t>
+          <t>Completeness/Accuracy/Authorization</t>
         </is>
       </c>
       <c r="G90" s="12" t="inlineStr">
         <is>
-          <t>Prepaid amortization schedules: a prepaid asset (insurance/rent paid up front) is registered once with a total + term; the scheduled job gl_prepaid_amortize posts a straight-line slice each period (Dr expense / Cr 1280), the last period taking the remainder so the asset fully clears. Idempotent per (schedule, period) via the JE idempotency key + next_run_date advance.</t>
+          <t>Recurring/template journal entries: a template's lines are validated balanced (Σdebit=Σcredit) AT SAVE TIME (unbalanced → UNBALANCED), so a broken template can never be persisted. The scheduled job gl_recurring_journals (cron / daily scheduler) posts every due template as a DRAFT JE through the normal maker-checker flow (GL-05) — a different user must approve before it affects balances — and rolls next_run_date forward. Idempotent: next_run_date advanced on posting + the (tenant,source,source_ref,ledger) idempotency key dedupes a same-day re-run. Templates can be paused/resumed without losing history.</t>
         </is>
       </c>
       <c r="H90" s="13" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I90" s="13" t="inlineStr">
@@ -8671,7 +8671,7 @@
       </c>
       <c r="J90" s="13" t="inlineStr">
         <is>
-          <t>Per period / per schedule</t>
+          <t>Per due date / per template</t>
         </is>
       </c>
       <c r="K90" s="12" t="inlineStr">
@@ -8686,22 +8686,22 @@
       </c>
       <c r="M90" s="12" t="inlineStr">
         <is>
-          <t>ledger.service.ts (createPrepaid, runDuePrepaid); ledger.controller.ts (gl_post); bi.service.ts (gl_prepaid_amortize); schema/ledger.ts (prepaid_schedules) + migration 0120; cutover/basics.ts (ToE)</t>
+          <t>ledger.service.ts (createRecurring balanced-at-save, runDueRecurring→postEntry pendingApproval, setRecurringActive); ledger.controller.ts (gl_post creates/runs); bi.service.ts (gl_recurring_journals); schema/ledger.ts (recurring_journals) + migration 0119; cutover/basics.ts (ToE)</t>
         </is>
       </c>
       <c r="N90" s="12" t="inlineStr">
         <is>
-          <t>Inspect amortization slice + final-period remainder + idempotency.</t>
+          <t>Inspect template balance validation + scheduled posting as Draft + idempotency.</t>
         </is>
       </c>
       <c r="O90" s="12" t="inlineStr">
         <is>
-          <t>Register a 12-month prepaid; run amortizes 1/12 to expense; re-run posts nothing (re-performed by the harness).</t>
+          <t>Unbalanced template → UNBALANCED; due template posts a Draft JE (excluded from TB) into the pending queue; re-run posts nothing; a second user approves → accrual hits the GL (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P90" s="12" t="inlineStr">
         <is>
-          <t>Prepaid schedules; amortization run log</t>
+          <t>Recurring-journal templates; scheduled run log; JE approvals</t>
         </is>
       </c>
       <c r="Q90" s="18" t="inlineStr">
@@ -8713,7 +8713,7 @@
     <row r="91">
       <c r="A91" s="15" t="inlineStr">
         <is>
-          <t>GL-10</t>
+          <t>GL-09</t>
         </is>
       </c>
       <c r="B91" s="16" t="inlineStr">
@@ -8728,27 +8728,27 @@
       </c>
       <c r="D91" s="16" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Prepaid expenses; Operating expense</t>
         </is>
       </c>
       <c r="E91" s="16" t="inlineStr">
         <is>
-          <t>A new company starts on a chart of accounts with no industry guidance — staff post to wrong/ambiguous accounts; or an industry template drifts from the GL engine's fixed posting codes so a posting targets an account that does not exist (mis-statement / unposted transaction).</t>
+          <t>Prepaid expense not amortized over its term — expense mis-stated, prepaid asset overstated.</t>
         </is>
       </c>
       <c r="F91" s="16" t="inlineStr">
         <is>
-          <t>Completeness/Accuracy/Presentation</t>
+          <t>Accuracy/Completeness</t>
         </is>
       </c>
       <c r="G91" s="16" t="inlineStr">
         <is>
-          <t>Industry Chart-of-Accounts templates: the GL engine binds to a FIXED, global account universe (canonical codes are immutable); each tenant additionally gets a per-tenant overlay (tenant_accounts) curating which canonical accounts are active and how they are named/grouped for its industry. At company creation the customer picks an industry (restaurant/retail/distribution/services/general) and the chosen template is materialised into the overlay (provisionTenantCoA) inside the signup transaction, right after fiscal-year provisioning; adopting an industry pack later does the same. Every template code is asserted to exist in the canonical chart at boot (assertTemplatesSubsetOf in seedChartOfAccounts) so a drifted template fails fast and can never reach a tenant. Provisioning is idempotent + additive (never deletes) so re-running only adds missing accounts. The overlay NEVER gates postings — it scopes the picker / Chart-of-Accounts view only; reports surface any account that is active OR carries activity, so a curated-out account that receives a posting still appears.</t>
+          <t>Prepaid amortization schedules: a prepaid asset (insurance/rent paid up front) is registered once with a total + term; the scheduled job gl_prepaid_amortize posts a straight-line slice each period (Dr expense / Cr 1280), the last period taking the remainder so the asset fully clears. Idempotent per (schedule, period) via the JE idempotency key + next_run_date advance.</t>
         </is>
       </c>
       <c r="H91" s="17" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I91" s="17" t="inlineStr">
@@ -8758,7 +8758,7 @@
       </c>
       <c r="J91" s="17" t="inlineStr">
         <is>
-          <t>At company creation / per pack adopt</t>
+          <t>Per period / per schedule</t>
         </is>
       </c>
       <c r="K91" s="16" t="inlineStr">
@@ -8773,22 +8773,22 @@
       </c>
       <c r="M91" s="16" t="inlineStr">
         <is>
-          <t>ledger.service.ts (provisionTenantCoA idempotent+additive, tenant-aware listAccounts, seedChartOfAccounts→assertTemplatesSubsetOf); coa-templates.ts (industry templates + subset assertion); billing.service.ts signup (industry→provisionTenantCoA in-txn); onboarding.service.ts applyPack (pack adopt provisions CoA); schema/ledger.ts tenant_accounts + tenants.industry + migration 0139; cutover/basics.ts + compliance.ts (ToE)</t>
+          <t>ledger.service.ts (createPrepaid, runDuePrepaid); ledger.controller.ts (gl_post); bi.service.ts (gl_prepaid_amortize); schema/ledger.ts (prepaid_schedules) + migration 0120; cutover/basics.ts (ToE)</t>
         </is>
       </c>
       <c r="N91" s="16" t="inlineStr">
         <is>
-          <t>Inspect the boot subset assertion + signup provisioning + the overlay-is-presentation-only read path.</t>
+          <t>Inspect amortization slice + final-period remainder + idempotency.</t>
         </is>
       </c>
       <c r="O91" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: a template referencing an unknown code fails the boot assertion; signup with industry=restaurant materialises a curated, industry-named chart (4000='Food &amp; Beverage Sales') that omits non-F&amp;B accounts; ?all=true still returns the full canonical universe (overlay never gates posting); signup with no industry ⇒ general = the full live chart (re-performed by the harnesses).</t>
+          <t>Register a 12-month prepaid; run amortizes 1/12 to expense; re-run posts nothing (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P91" s="16" t="inlineStr">
         <is>
-          <t>Industry templates; tenant_accounts overlay; signup provisioning log</t>
+          <t>Prepaid schedules; amortization run log</t>
         </is>
       </c>
       <c r="Q91" s="18" t="inlineStr">
@@ -8800,7 +8800,7 @@
     <row r="92">
       <c r="A92" s="11" t="inlineStr">
         <is>
-          <t>GL-11</t>
+          <t>GL-10</t>
         </is>
       </c>
       <c r="B92" s="12" t="inlineStr">
@@ -8820,17 +8820,17 @@
       </c>
       <c r="E92" s="12" t="inlineStr">
         <is>
-          <t>Chart of Accounts changed without authorisation; account code changed after postings exist; account deactivated while carrying a non-zero balance; manual JE posted directly to a control account (AR/AP/INV/FA), bypassing the sub-ledger and hiding a sub-ledger discrepancy.</t>
+          <t>A new company starts on a chart of accounts with no industry guidance — staff post to wrong/ambiguous accounts; or an industry template drifts from the GL engine's fixed posting codes so a posting targets an account that does not exist (mis-statement / unposted transaction).</t>
         </is>
       </c>
       <c r="F92" s="12" t="inlineStr">
         <is>
-          <t>Authorization/Completeness/Accuracy</t>
+          <t>Completeness/Accuracy/Presentation</t>
         </is>
       </c>
       <c r="G92" s="12" t="inlineStr">
         <is>
-          <t>CoA Change Control: account creation/update/deactivation requires the gl_coa permission (held by FinancialController, not GlAccountant — separated from gl_post per SoD). Disabling postability on an account that already has posted entries is rejected (CODE_HAS_POSTINGS). Deactivation is rejected if the account carries a non-zero net balance (ACCOUNT_HAS_BALANCE) — prevents orphaning a balance in a closed account. Four accounts are flagged is_control=true at setup: 1100 (AR), 2000 (AP), 1200 (INV), 1500 (FA); a direct manual JE that touches any of these without viaSubledger:true is rejected (CONTROL_ACCOUNT), ensuring AR/AP/INV/FA balances are exclusively maintained by their respective sub-ledger service methods.</t>
+          <t>Industry Chart-of-Accounts templates: the GL engine binds to a FIXED, global account universe (canonical codes are immutable); each tenant additionally gets a per-tenant overlay (tenant_accounts) curating which canonical accounts are active and how they are named/grouped for its industry. At company creation the customer picks an industry (restaurant/retail/distribution/services/general) and the chosen template is materialised into the overlay (provisionTenantCoA) inside the signup transaction, right after fiscal-year provisioning; adopting an industry pack later does the same. Every template code is asserted to exist in the canonical chart at boot (assertTemplatesSubsetOf in seedChartOfAccounts) so a drifted template fails fast and can never reach a tenant. Provisioning is idempotent + additive (never deletes) so re-running only adds missing accounts. The overlay NEVER gates postings — it scopes the picker / Chart-of-Accounts view only; reports surface any account that is active OR carries activity, so a curated-out account that receives a posting still appears.</t>
         </is>
       </c>
       <c r="H92" s="13" t="inlineStr">
@@ -8845,12 +8845,12 @@
       </c>
       <c r="J92" s="13" t="inlineStr">
         <is>
-          <t>Event-driven</t>
+          <t>At company creation / per pack adopt</t>
         </is>
       </c>
       <c r="K92" s="12" t="inlineStr">
         <is>
-          <t>Financial Controller</t>
+          <t>Controller</t>
         </is>
       </c>
       <c r="L92" s="13" t="inlineStr">
@@ -8860,22 +8860,22 @@
       </c>
       <c r="M92" s="12" t="inlineStr">
         <is>
-          <t>coa.service.ts (createAccount DUPLICATE_ACCOUNT, updateAccount CODE_HAS_POSTINGS, deactivateAccount ACCOUNT_HAS_BALANCE); coa.controller.ts (gl_coa permission gate); ledger.service.ts postEntry control-account guard (CONTROL_ACCOUNT, viaSubledger flag); schema/ledger.ts (account_groups table, accounts.is_control/control_subledger/is_postable/normal_balance + migration 0155); packages/shared/src/permissions.ts (gl_coa sub-permission, FinancialController default)</t>
+          <t>ledger.service.ts (provisionTenantCoA idempotent+additive, tenant-aware listAccounts, seedChartOfAccounts→assertTemplatesSubsetOf); coa-templates.ts (industry templates + subset assertion); billing.service.ts signup (industry→provisionTenantCoA in-txn); onboarding.service.ts applyPack (pack adopt provisions CoA); schema/ledger.ts tenant_accounts + tenants.industry + migration 0139; cutover/basics.ts + compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N92" s="12" t="inlineStr">
         <is>
-          <t>Inspect gl_coa permission gate + CODE_HAS_POSTINGS guard + ACCOUNT_HAS_BALANCE guard + CONTROL_ACCOUNT guard + viaSubledger bypass.</t>
+          <t>Inspect the boot subset assertion + signup provisioning + the overlay-is-presentation-only read path.</t>
         </is>
       </c>
       <c r="O92" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: create an account with gl_coa → 201; attempt to deactivate an account with balance → ACCOUNT_HAS_BALANCE; post directly to account 1100 without viaSubledger → CONTROL_ACCOUNT (re-performed by TC-GL-11-01/02/03 UAT cases).</t>
+          <t>Re-perform: a template referencing an unknown code fails the boot assertion; signup with industry=restaurant materialises a curated, industry-named chart (4000='Food &amp; Beverage Sales') that omits non-F&amp;B accounts; ?all=true still returns the full canonical universe (overlay never gates posting); signup with no industry ⇒ general = the full live chart (re-performed by the harnesses).</t>
         </is>
       </c>
       <c r="P92" s="12" t="inlineStr">
         <is>
-          <t>CoA change log (audit_log); permission test; control-account guard test</t>
+          <t>Industry templates; tenant_accounts overlay; signup provisioning log</t>
         </is>
       </c>
       <c r="Q92" s="18" t="inlineStr">
@@ -8887,7 +8887,7 @@
     <row r="93">
       <c r="A93" s="15" t="inlineStr">
         <is>
-          <t>GL-12</t>
+          <t>GL-11</t>
         </is>
       </c>
       <c r="B93" s="16" t="inlineStr">
@@ -8907,17 +8907,17 @@
       </c>
       <c r="E93" s="16" t="inlineStr">
         <is>
-          <t>Account-assignment errors introduced by scattered inline account-code literals in service code; a tenant needing a different account for a given business event has no mechanism to override without a code change.</t>
+          <t>Chart of Accounts changed without authorisation; account code changed after postings exist; account deactivated while carrying a non-zero balance; manual JE posted directly to a control account (AR/AP/INV/FA), bypassing the sub-ledger and hiding a sub-ledger discrepancy.</t>
         </is>
       </c>
       <c r="F93" s="16" t="inlineStr">
         <is>
-          <t>Authorization/Accuracy</t>
+          <t>Authorization/Completeness/Accuracy</t>
         </is>
       </c>
       <c r="G93" s="16" t="inlineStr">
         <is>
-          <t>Posting / Account-Determination Engine: two tables — posting_event_types (28 seeded event types, e.g. SALE.FOOD, GR.INVENTORY, DEPRECIATION.FA) and posting_rules (maps event × leg-order to semantic role → account_code + DR/CR side) — drive account assignment instead of hard-coded literals. PostingService.post(eventType, ctx) resolves the applicable rules (global defaults, or shadowed by tenant-specific overrides for the same leg_order), translates role-keyed amounts into DR/CR lines, and delegates to LedgerService.postEntry. If no active rules exist for an event the call fails with NO_POSTING_RULE. Tenant-specific rules require gl_posting_rules permission to create/update. PostingService.preview() provides a dry-run for audit.</t>
+          <t>CoA Change Control: account creation/update/deactivation requires the gl_coa permission (held by FinancialController, not GlAccountant — separated from gl_post per SoD). Disabling postability on an account that already has posted entries is rejected (CODE_HAS_POSTINGS). Deactivation is rejected if the account carries a non-zero net balance (ACCOUNT_HAS_BALANCE) — prevents orphaning a balance in a closed account. Four accounts are flagged is_control=true at setup: 1100 (AR), 2000 (AP), 1200 (INV), 1500 (FA); a direct manual JE that touches any of these without viaSubledger:true is rejected (CONTROL_ACCOUNT), ensuring AR/AP/INV/FA balances are exclusively maintained by their respective sub-ledger service methods.</t>
         </is>
       </c>
       <c r="H93" s="17" t="inlineStr">
@@ -8947,22 +8947,22 @@
       </c>
       <c r="M93" s="16" t="inlineStr">
         <is>
-          <t>posting.service.ts (resolveRules, post, preview, listEventTypes, listRules, upsertRule); posting-rules.controller.ts (gl_posting_rules permission gate); schema/posting-rules.ts (posting_event_types, posting_rules tables); migration 0156 (tables + 28 event types + global-default rules); ledger.module.ts (PostingService exported); packages/shared/src/permissions.ts (gl_posting_rules sub-permission); cutover/basics.ts (golden-snapshot ToE)</t>
+          <t>coa.service.ts (createAccount DUPLICATE_ACCOUNT, updateAccount CODE_HAS_POSTINGS, deactivateAccount ACCOUNT_HAS_BALANCE); coa.controller.ts (gl_coa permission gate); ledger.service.ts postEntry control-account guard (CONTROL_ACCOUNT, viaSubledger flag); schema/ledger.ts (account_groups table, accounts.is_control/control_subledger/is_postable/normal_balance + migration 0155); packages/shared/src/permissions.ts (gl_coa sub-permission, FinancialController default)</t>
         </is>
       </c>
       <c r="N93" s="16" t="inlineStr">
         <is>
-          <t>Inspect the rule-resolution logic + NO_POSTING_RULE fast-fail + tenant-shadow logic + gl_posting_rules permission gate.</t>
+          <t>Inspect gl_coa permission gate + CODE_HAS_POSTINGS guard + ACCOUNT_HAS_BALANCE guard + CONTROL_ACCOUNT guard + viaSubledger bypass.</t>
         </is>
       </c>
       <c r="O93" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: preview DEPRECIATION.FA with dep_expense:1000 → DR 5200 / CR 1590; preview GR.INVENTORY with inventory:500 → DR 1200 / CR 2000; preview UNKNOWN_EVENT → NO_POSTING_RULE (400); event-type catalogue returns ≥20 entries (re-performed by TC-GL-12-01/02/03/04 UAT cases + basics.ts harness).</t>
+          <t>Re-perform: create an account with gl_coa → 201; attempt to deactivate an account with balance → ACCOUNT_HAS_BALANCE; post directly to account 1100 without viaSubledger → CONTROL_ACCOUNT (re-performed by TC-GL-11-01/02/03 UAT cases).</t>
         </is>
       </c>
       <c r="P93" s="16" t="inlineStr">
         <is>
-          <t>Posting-rule change log; preview dry-run; harness golden snapshot</t>
+          <t>CoA change log (audit_log); permission test; control-account guard test</t>
         </is>
       </c>
       <c r="Q93" s="18" t="inlineStr">
@@ -8974,7 +8974,7 @@
     <row r="94">
       <c r="A94" s="11" t="inlineStr">
         <is>
-          <t>GL-13</t>
+          <t>GL-12</t>
         </is>
       </c>
       <c r="B94" s="12" t="inlineStr">
@@ -8994,22 +8994,22 @@
       </c>
       <c r="E94" s="12" t="inlineStr">
         <is>
-          <t>Revenue or expense mis-attributed to the wrong branch / project — per-location P&amp;L is unintelligible or misleading.</t>
+          <t>Account-assignment errors introduced by scattered inline account-code literals in service code; a tenant needing a different account for a given business event has no mechanism to override without a code change.</t>
         </is>
       </c>
       <c r="F94" s="12" t="inlineStr">
         <is>
-          <t>Accuracy/Presentation</t>
+          <t>Authorization/Accuracy</t>
         </is>
       </c>
       <c r="G94" s="12" t="inlineStr">
         <is>
-          <t>Multi-dimensional GL postings: journal_lines carries three optional dimension columns (branch_id, project_id, department_id). PostingService.post() stamps all generated lines from PostingContext (branchId/projectId/departmentId). GET /api/ledger/income-statement/by-branch provides a per-branch P&amp;L view; lines without a branch_id are grouped as 'unassigned'. The departments master table holds a tenant-scoped department registry with RLS isolation.</t>
+          <t>Posting / Account-Determination Engine: two tables — posting_event_types (28 seeded event types, e.g. SALE.FOOD, GR.INVENTORY, DEPRECIATION.FA) and posting_rules (maps event × leg-order to semantic role → account_code + DR/CR side) — drive account assignment instead of hard-coded literals. PostingService.post(eventType, ctx) resolves the applicable rules (global defaults, or shadowed by tenant-specific overrides for the same leg_order), translates role-keyed amounts into DR/CR lines, and delegates to LedgerService.postEntry. If no active rules exist for an event the call fails with NO_POSTING_RULE. Tenant-specific rules require gl_posting_rules permission to create/update. PostingService.preview() provides a dry-run for audit.</t>
         </is>
       </c>
       <c r="H94" s="13" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I94" s="13" t="inlineStr">
@@ -9019,12 +9019,12 @@
       </c>
       <c r="J94" s="13" t="inlineStr">
         <is>
-          <t>Per period</t>
+          <t>Event-driven</t>
         </is>
       </c>
       <c r="K94" s="12" t="inlineStr">
         <is>
-          <t>Controller</t>
+          <t>Financial Controller</t>
         </is>
       </c>
       <c r="L94" s="13" t="inlineStr">
@@ -9034,22 +9034,22 @@
       </c>
       <c r="M94" s="12" t="inlineStr">
         <is>
-          <t>ledger.service.ts (incomeStatementByBranch); ledger.controller.ts (GET income-statement/by-branch); posting.service.ts (branchId/projectId/departmentId from PostingContext); schema/ledger.ts (branch_id, project_id, department_id on journal_lines); schema/departments.ts (departments table); migration 0157; cutover/basics.ts (GL-13 ToE)</t>
+          <t>posting.service.ts (resolveRules, post, preview, listEventTypes, listRules, upsertRule); posting-rules.controller.ts (gl_posting_rules permission gate); schema/posting-rules.ts (posting_event_types, posting_rules tables); migration 0156 (tables + 28 event types + global-default rules); ledger.module.ts (PostingService exported); packages/shared/src/permissions.ts (gl_posting_rules sub-permission); cutover/basics.ts (golden-snapshot ToE)</t>
         </is>
       </c>
       <c r="N94" s="12" t="inlineStr">
         <is>
-          <t>Inspect by-branch query + PostingContext stamping + department RLS.</t>
+          <t>Inspect the rule-resolution logic + NO_POSTING_RULE fast-fail + tenant-shadow logic + gl_posting_rules permission gate.</t>
         </is>
       </c>
       <c r="O94" s="12" t="inlineStr">
         <is>
-          <t>TC-GL-13-01/02/03: smoke + two branches + unassigned bucket (re-performed by the basics.ts harness).</t>
+          <t>Re-perform: preview DEPRECIATION.FA with dep_expense:1000 → DR 5200 / CR 1590; preview GR.INVENTORY with inventory:500 → DR 1200 / CR 2000; preview UNKNOWN_EVENT → NO_POSTING_RULE (400); event-type catalogue returns ≥20 entries (re-performed by TC-GL-12-01/02/03/04 UAT cases + basics.ts harness).</t>
         </is>
       </c>
       <c r="P94" s="12" t="inlineStr">
         <is>
-          <t>By-branch P&amp;L report; dimension completeness</t>
+          <t>Posting-rule change log; preview dry-run; harness golden snapshot</t>
         </is>
       </c>
       <c r="Q94" s="18" t="inlineStr">
@@ -9061,7 +9061,7 @@
     <row r="95">
       <c r="A95" s="15" t="inlineStr">
         <is>
-          <t>GL-14</t>
+          <t>GL-13</t>
         </is>
       </c>
       <c r="B95" s="16" t="inlineStr">
@@ -9081,17 +9081,17 @@
       </c>
       <c r="E95" s="16" t="inlineStr">
         <is>
-          <t>GL control-account balances (AR/AP/INV/FA) drift from the underlying sub-ledger detail without detection — the control account no longer represents the sum of its sub-ledger, masking posting errors, unrecorded items, or fraud.</t>
+          <t>Revenue or expense mis-attributed to the wrong branch / project — per-location P&amp;L is unintelligible or misleading.</t>
         </is>
       </c>
       <c r="F95" s="16" t="inlineStr">
         <is>
-          <t>Completeness/Accuracy/Valuation</t>
+          <t>Accuracy/Presentation</t>
         </is>
       </c>
       <c r="G95" s="16" t="inlineStr">
         <is>
-          <t>Sub-ledger tie-out / reconciliation: POST /api/ledger/tie-out/run computes, per control account, the GL balance (Σ debit−credit of posted journal_lines on the control account up to the as-of date, tenant-scoped) and the sub-ledger detail balance (AR = Σ outstanding ar_invoices; AP = Σ outstanding ap_transactions; INV = Σ inv_balances.total_value perpetual valuation; FA = Σ acquire_cost − accumulated_depreciation of non-disposed fixed_assets), records the variance (gl − subledger) and a status (Matched if |variance|&lt;0.01 else Variance). Runs upsert per (tenant, subledger, as-of). Certification is maker-checker: POST /api/ledger/tie-out/:id/certify sets status=Certified and records certifier + timestamp, and REJECTS a certifier equal to the runner (SELF_CERTIFY) — the gl_close certifier must differ from the gl_post/gl_close runner (SoD).</t>
+          <t>Multi-dimensional GL postings: journal_lines carries three optional dimension columns (branch_id, project_id, department_id). PostingService.post() stamps all generated lines from PostingContext (branchId/projectId/departmentId). GET /api/ledger/income-statement/by-branch provides a per-branch P&amp;L view; lines without a branch_id are grouped as 'unassigned'. The departments master table holds a tenant-scoped department registry with RLS isolation.</t>
         </is>
       </c>
       <c r="H95" s="17" t="inlineStr">
@@ -9106,12 +9106,12 @@
       </c>
       <c r="J95" s="17" t="inlineStr">
         <is>
-          <t>Monthly</t>
+          <t>Per period</t>
         </is>
       </c>
       <c r="K95" s="16" t="inlineStr">
         <is>
-          <t>Financial Controller</t>
+          <t>Controller</t>
         </is>
       </c>
       <c r="L95" s="17" t="inlineStr">
@@ -9121,22 +9121,22 @@
       </c>
       <c r="M95" s="16" t="inlineStr">
         <is>
-          <t>subledger-tieout.service.ts (runTieOut GL/sub-ledger balance computation + variance/status, certify SELF_CERTIFY maker-checker, list/get); subledger-tieout.controller.ts (gl_close/gl_post run, gl_close certify, gl_close/gl_post/exec/creditors/ar read); schema/subledger-tieout.ts (subledger_tieout_runs table, uq on tenant/subledger/as-of); migration 0160 (table + RLS); ledger.module.ts (service+controller wired); cutover/basics.ts (GL-14 ToE)</t>
+          <t>ledger.service.ts (incomeStatementByBranch); ledger.controller.ts (GET income-statement/by-branch); posting.service.ts (branchId/projectId/departmentId from PostingContext); schema/ledger.ts (branch_id, project_id, department_id on journal_lines); schema/departments.ts (departments table); migration 0157; cutover/basics.ts (GL-13 ToE)</t>
         </is>
       </c>
       <c r="N95" s="16" t="inlineStr">
         <is>
-          <t>Inspect the GL-vs-sub-ledger balance computation + variance/status + SELF_CERTIFY maker-checker gate + gl_close certify permission.</t>
+          <t>Inspect by-branch query + PostingContext stamping + department RLS.</t>
         </is>
       </c>
       <c r="O95" s="16" t="inlineStr">
         <is>
-          <t>TC-GL-14-01: run AR tie-out → balances + Matched/Variance; TC-GL-14-02: self-certify by the runner → SELF_CERTIFY (400); TC-GL-14-03: certify by a different gl_close user → Certified (re-performed by the basics.ts harness).</t>
+          <t>TC-GL-13-01/02/03: smoke + two branches + unassigned bucket (re-performed by the basics.ts harness).</t>
         </is>
       </c>
       <c r="P95" s="16" t="inlineStr">
         <is>
-          <t>Tie-out run log (subledger_tieout_runs) with variance + certification trail; monthly reconciliation sign-off</t>
+          <t>By-branch P&amp;L report; dimension completeness</t>
         </is>
       </c>
       <c r="Q95" s="18" t="inlineStr">
@@ -9148,7 +9148,7 @@
     <row r="96">
       <c r="A96" s="11" t="inlineStr">
         <is>
-          <t>GL-15</t>
+          <t>GL-14</t>
         </is>
       </c>
       <c r="B96" s="12" t="inlineStr">
@@ -9168,22 +9168,22 @@
       </c>
       <c r="E96" s="12" t="inlineStr">
         <is>
-          <t>A period is 'closed' on paper but key close procedures (sub-ledger tie-out, bank rec, depreciation, recurring/prepaid, trial-balance review) were skipped, OR a closed period is silently re-opened and re-posted — the financial statements are produced on an incomplete/altered basis.</t>
+          <t>GL control-account balances (AR/AP/INV/FA) drift from the underlying sub-ledger detail without detection — the control account no longer represents the sum of its sub-ledger, masking posting errors, unrecorded items, or fraud.</t>
         </is>
       </c>
       <c r="F96" s="12" t="inlineStr">
         <is>
-          <t>Completeness/Accuracy/Cutoff</t>
+          <t>Completeness/Accuracy/Valuation</t>
         </is>
       </c>
       <c r="G96" s="12" t="inlineStr">
         <is>
-          <t>Hard period close + checklist: POST /api/ledger/close/start opens a close_runs record (status InProgress) per (tenant, period) and seeds a standard checklist of close_run_steps (subledger_tieout, bank_rec, depreciation, recurring, fx_reval[advisory], trial_balance_review). POST /api/ledger/close/step marks a step Done (records completedBy/At); when all REQUIRED steps are Done the run advances to ReadyToLock. POST /api/ledger/close/lock requires ReadyToLock (else STEPS_INCOMPLETE listing the pending required steps) before the period can be locked. Locking writes 'Locked' into fiscal_periods.status; LedgerService.postEntry then REJECTS every posting dated into a Locked period with PERIOD_LOCKED, regardless of the legacy allowClosedPeriod escape (the only exception is the system year-end closing entry, source='CLOSE'). Locked is strictly stronger than the soft 'Closed' status — it is the irreversible hard close.</t>
+          <t>Sub-ledger tie-out / reconciliation: POST /api/ledger/tie-out/run computes, per control account, the GL balance (Σ debit−credit of posted journal_lines on the control account up to the as-of date, tenant-scoped) and the sub-ledger detail balance (AR = Σ outstanding ar_invoices; AP = Σ outstanding ap_transactions; INV = Σ inv_balances.total_value perpetual valuation; FA = Σ acquire_cost − accumulated_depreciation of non-disposed fixed_assets), records the variance (gl − subledger) and a status (Matched if |variance|&lt;0.01 else Variance). Runs upsert per (tenant, subledger, as-of). Certification is maker-checker: POST /api/ledger/tie-out/:id/certify sets status=Certified and records certifier + timestamp, and REJECTS a certifier equal to the runner (SELF_CERTIFY) — the gl_close certifier must differ from the gl_post/gl_close runner (SoD).</t>
         </is>
       </c>
       <c r="H96" s="13" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I96" s="13" t="inlineStr">
@@ -9208,22 +9208,22 @@
       </c>
       <c r="M96" s="12" t="inlineStr">
         <is>
-          <t>close.service.ts (startClose seeds checklist, completeStep → ReadyToLock when required steps Done, lockPeriod STEPS_INCOMPLETE gate + fiscal_periods Locked write, status/list); close.controller.ts (gl_close start/step/lock, gl_close/gl_post/exec read); schema/close-runs.ts (close_runs + close_run_steps, uq on tenant/period and run/step_key); schema/ledger.ts (period_status enum + 'Locked'); ledger.service.ts (postEntry PERIOD_LOCKED hard gate, source='CLOSE' exemption); migration 0162 (tables + RLS + ALTER TYPE Locked); ledger.module.ts (service+controller wired); cutover/basics.ts (GL-15/GL-16 ToE)</t>
+          <t>subledger-tieout.service.ts (runTieOut GL/sub-ledger balance computation + variance/status, certify SELF_CERTIFY maker-checker, list/get); subledger-tieout.controller.ts (gl_close/gl_post run, gl_close certify, gl_close/gl_post/exec/creditors/ar read); schema/subledger-tieout.ts (subledger_tieout_runs table, uq on tenant/subledger/as-of); migration 0160 (table + RLS); ledger.module.ts (service+controller wired); cutover/basics.ts (GL-14 ToE)</t>
         </is>
       </c>
       <c r="N96" s="12" t="inlineStr">
         <is>
-          <t>Inspect the seeded checklist + ReadyToLock gating + STEPS_INCOMPLETE lock rejection + PERIOD_LOCKED hard gate in postEntry (incl. the CLOSE exemption).</t>
+          <t>Inspect the GL-vs-sub-ledger balance computation + variance/status + SELF_CERTIFY maker-checker gate + gl_close certify permission.</t>
         </is>
       </c>
       <c r="O96" s="12" t="inlineStr">
         <is>
-          <t>TC-GL-15-01: start close seeds ≥4 steps (InProgress); TC-GL-15-02: lock before steps done → STEPS_INCOMPLETE (400); TC-GL-15-03: post into locked period → PERIOD_LOCKED (400) (re-performed by the basics.ts harness).</t>
+          <t>TC-GL-14-01: run AR tie-out → balances + Matched/Variance; TC-GL-14-02: self-certify by the runner → SELF_CERTIFY (400); TC-GL-14-03: certify by a different gl_close user → Certified (re-performed by the basics.ts harness).</t>
         </is>
       </c>
       <c r="P96" s="12" t="inlineStr">
         <is>
-          <t>close_runs / close_run_steps with completion trail; fiscal_periods.status=Locked; monthly close sign-off</t>
+          <t>Tie-out run log (subledger_tieout_runs) with variance + certification trail; monthly reconciliation sign-off</t>
         </is>
       </c>
       <c r="Q96" s="18" t="inlineStr">
@@ -9235,7 +9235,7 @@
     <row r="97">
       <c r="A97" s="15" t="inlineStr">
         <is>
-          <t>GL-16</t>
+          <t>GL-15</t>
         </is>
       </c>
       <c r="B97" s="16" t="inlineStr">
@@ -9255,17 +9255,17 @@
       </c>
       <c r="E97" s="16" t="inlineStr">
         <is>
-          <t>One person both performs the close and locks the period, defeating segregation of duties — a preparer could conceal a misstatement by closing over their own work without independent review.</t>
+          <t>A period is 'closed' on paper but key close procedures (sub-ledger tie-out, bank rec, depreciation, recurring/prepaid, trial-balance review) were skipped, OR a closed period is silently re-opened and re-posted — the financial statements are produced on an incomplete/altered basis.</t>
         </is>
       </c>
       <c r="F97" s="16" t="inlineStr">
         <is>
-          <t>Authorization/Segregation of Duties</t>
+          <t>Completeness/Accuracy/Cutoff</t>
         </is>
       </c>
       <c r="G97" s="16" t="inlineStr">
         <is>
-          <t>Segregated period lock (maker-checker): the close_runs.started_by (the user who started the close and ran the checklist steps) is recorded, and POST /api/ledger/close/lock REJECTS a lockedBy equal to startedBy with SELF_LOCK — the gl_close user who locks the period MUST differ from the user who started/ran the close. Both identities and the lock timestamp are retained on the close_runs row (started_by / locked_by / locked_at) as the SoD evidence trail. This complements the existing SoD rule that gl_close is segregated from gl_post (JE posting).</t>
+          <t>Hard period close + checklist: POST /api/ledger/close/start opens a close_runs record (status InProgress) per (tenant, period) and seeds a standard checklist of close_run_steps (subledger_tieout, bank_rec, depreciation, recurring, fx_reval[advisory], trial_balance_review). POST /api/ledger/close/step marks a step Done (records completedBy/At); when all REQUIRED steps are Done the run advances to ReadyToLock. POST /api/ledger/close/lock requires ReadyToLock (else STEPS_INCOMPLETE listing the pending required steps) before the period can be locked. Locking writes 'Locked' into fiscal_periods.status; LedgerService.postEntry then REJECTS every posting dated into a Locked period with PERIOD_LOCKED, regardless of the legacy allowClosedPeriod escape (the only exception is the system year-end closing entry, source='CLOSE'). Locked is strictly stronger than the soft 'Closed' status — it is the irreversible hard close.</t>
         </is>
       </c>
       <c r="H97" s="17" t="inlineStr">
@@ -9295,22 +9295,22 @@
       </c>
       <c r="M97" s="16" t="inlineStr">
         <is>
-          <t>close.service.ts (lockPeriod SELF_LOCK maker-checker gate; started_by vs locked_by); close.controller.ts (gl_close lock, acting username from JWT); schema/close-runs.ts (started_by, locked_by, locked_at columns); permissions.ts (gl_post×gl_close SoD pair); cutover/basics.ts (GL-16 ToE)</t>
+          <t>close.service.ts (startClose seeds checklist, completeStep → ReadyToLock when required steps Done, lockPeriod STEPS_INCOMPLETE gate + fiscal_periods Locked write, status/list); close.controller.ts (gl_close start/step/lock, gl_close/gl_post/exec read); schema/close-runs.ts (close_runs + close_run_steps, uq on tenant/period and run/step_key); schema/ledger.ts (period_status enum + 'Locked'); ledger.service.ts (postEntry PERIOD_LOCKED hard gate, source='CLOSE' exemption); migration 0162 (tables + RLS + ALTER TYPE Locked); ledger.module.ts (service+controller wired); cutover/basics.ts (GL-15/GL-16 ToE)</t>
         </is>
       </c>
       <c r="N97" s="16" t="inlineStr">
         <is>
-          <t>Inspect the SELF_LOCK gate (startedBy ≠ lockedBy) + the started_by/locked_by/locked_at evidence trail.</t>
+          <t>Inspect the seeded checklist + ReadyToLock gating + STEPS_INCOMPLETE lock rejection + PERIOD_LOCKED hard gate in postEntry (incl. the CLOSE exemption).</t>
         </is>
       </c>
       <c r="O97" s="16" t="inlineStr">
         <is>
-          <t>TC-GL-16-01: self-lock by the starter → SELF_LOCK (400); TC-GL-16-02: lock by a different gl_close user → Locked, locked_by recorded (re-performed by the basics.ts harness).</t>
+          <t>TC-GL-15-01: start close seeds ≥4 steps (InProgress); TC-GL-15-02: lock before steps done → STEPS_INCOMPLETE (400); TC-GL-15-03: post into locked period → PERIOD_LOCKED (400) (re-performed by the basics.ts harness).</t>
         </is>
       </c>
       <c r="P97" s="16" t="inlineStr">
         <is>
-          <t>close_runs.started_by / locked_by / locked_at SoD trail; monthly close sign-off</t>
+          <t>close_runs / close_run_steps with completion trail; fiscal_periods.status=Locked; monthly close sign-off</t>
         </is>
       </c>
       <c r="Q97" s="18" t="inlineStr">
@@ -9322,12 +9322,12 @@
     <row r="98">
       <c r="A98" s="11" t="inlineStr">
         <is>
-          <t>EXP-07</t>
+          <t>GL-16</t>
         </is>
       </c>
       <c r="B98" s="12" t="inlineStr">
         <is>
-          <t>Expenditure</t>
+          <t>General Ledger</t>
         </is>
       </c>
       <c r="C98" s="13" t="inlineStr">
@@ -9337,27 +9337,27 @@
       </c>
       <c r="D98" s="12" t="inlineStr">
         <is>
-          <t>Cash; Operating expense</t>
+          <t>All</t>
         </is>
       </c>
       <c r="E98" s="12" t="inlineStr">
         <is>
-          <t>Petty-cash / employee advance issued but never accounted for — cash leakage, expense unrecorded.</t>
+          <t>One person both performs the close and locks the period, defeating segregation of duties — a preparer could conceal a misstatement by closing over their own work without independent review.</t>
         </is>
       </c>
       <c r="F98" s="12" t="inlineStr">
         <is>
-          <t>Existence/Completeness</t>
+          <t>Authorization/Segregation of Duties</t>
         </is>
       </c>
       <c r="G98" s="12" t="inlineStr">
         <is>
-          <t>Employee cash advances: issuing an advance debits the 1180 Employee Advances control (Dr 1180 / Cr 1000); settlement clears it against actual spend + returned cash (Dr expense + Dr 1000 / Cr 1180), enforced to reconcile (settled_expense + returned_cash must equal the advance → SETTLE_MISMATCH). The 1180 balance is the outstanding float subject to review.</t>
+          <t>Segregated period lock (maker-checker): the close_runs.started_by (the user who started the close and ran the checklist steps) is recorded, and POST /api/ledger/close/lock REJECTS a lockedBy equal to startedBy with SELF_LOCK — the gl_close user who locks the period MUST differ from the user who started/ran the close. Both identities and the lock timestamp are retained on the close_runs row (started_by / locked_by / locked_at) as the SoD evidence trail. This complements the existing SoD rule that gl_close is segregated from gl_post (JE posting).</t>
         </is>
       </c>
       <c r="H98" s="13" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I98" s="13" t="inlineStr">
@@ -9367,12 +9367,12 @@
       </c>
       <c r="J98" s="13" t="inlineStr">
         <is>
-          <t>Per advance</t>
+          <t>Monthly</t>
         </is>
       </c>
       <c r="K98" s="12" t="inlineStr">
         <is>
-          <t>AP / Controller</t>
+          <t>Financial Controller</t>
         </is>
       </c>
       <c r="L98" s="13" t="inlineStr">
@@ -9382,22 +9382,22 @@
       </c>
       <c r="M98" s="12" t="inlineStr">
         <is>
-          <t>finance.service.ts (issueAdvance, settleAdvance reconcile-or-reject, listAdvances outstanding); finance.controller.ts (creditors/exec); schema/finance.ts (employee_advances) + migration 0120; cutover/basics.ts (ToE)</t>
+          <t>close.service.ts (lockPeriod SELF_LOCK maker-checker gate; started_by vs locked_by); close.controller.ts (gl_close lock, acting username from JWT); schema/close-runs.ts (started_by, locked_by, locked_at columns); permissions.ts (gl_post×gl_close SoD pair); cutover/basics.ts (GL-16 ToE)</t>
         </is>
       </c>
       <c r="N98" s="12" t="inlineStr">
         <is>
-          <t>Inspect issue/settle GL + settlement reconciliation guard.</t>
+          <t>Inspect the SELF_LOCK gate (startedBy ≠ lockedBy) + the started_by/locked_by/locked_at evidence trail.</t>
         </is>
       </c>
       <c r="O98" s="12" t="inlineStr">
         <is>
-          <t>Issue an advance (1180 up); settle 700+300 clears 1180; mismatched settle → SETTLE_MISMATCH (re-performed by the harness).</t>
+          <t>TC-GL-16-01: self-lock by the starter → SELF_LOCK (400); TC-GL-16-02: lock by a different gl_close user → Locked, locked_by recorded (re-performed by the basics.ts harness).</t>
         </is>
       </c>
       <c r="P98" s="12" t="inlineStr">
         <is>
-          <t>Advance register; outstanding float</t>
+          <t>close_runs.started_by / locked_by / locked_at SoD trail; monthly close sign-off</t>
         </is>
       </c>
       <c r="Q98" s="18" t="inlineStr">
@@ -9409,7 +9409,7 @@
     <row r="99">
       <c r="A99" s="15" t="inlineStr">
         <is>
-          <t>EXP-08</t>
+          <t>EXP-07</t>
         </is>
       </c>
       <c r="B99" s="16" t="inlineStr">
@@ -9429,22 +9429,22 @@
       </c>
       <c r="E99" s="16" t="inlineStr">
         <is>
-          <t>Petty-cash disbursed beyond authority / without independent review, or drawn past the fund's limit — cash leakage, unauthorised or unrecorded expense, over-extended float.</t>
+          <t>Petty-cash / employee advance issued but never accounted for — cash leakage, expense unrecorded.</t>
         </is>
       </c>
       <c r="F99" s="16" t="inlineStr">
         <is>
-          <t>Authorization; Completeness</t>
+          <t>Existence/Completeness</t>
         </is>
       </c>
       <c r="G99" s="16" t="inlineStr">
         <is>
-          <t>Petty-cash imprest float + maker-checker on disbursement (SoD): a fund holds cash capped at a credit limit/วงเงิน (1015 Petty Cash, a cash account); each direct EXPENSE or ADVANCE is a REQUEST that posts NOTHING and a DIFFERENT user must approve before the GL posts (expense Dr &lt;expense&gt; / Cr 1015; advance Dr 1180 / Cr 1015) and the fund balance is decremented. Self-approval → SOD_VIOLATION (binds even Admin). A draw beyond the fund balance → INSUFFICIENT_FLOAT; establishing/replenishing above the float limit → OVER_FLOAT. Advances settle (Dr expense + Dr 1015 returned / Cr 1180), returning unused cash to the fund. Every request carries a document reference + receipt key + a status trail (StatusLog) and surfaces in the GOV-01 pending-approvals monitor.</t>
+          <t>Employee cash advances: issuing an advance debits the 1180 Employee Advances control (Dr 1180 / Cr 1000); settlement clears it against actual spend + returned cash (Dr expense + Dr 1000 / Cr 1180), enforced to reconcile (settled_expense + returned_cash must equal the advance → SETTLE_MISMATCH). The 1180 balance is the outstanding float subject to review.</t>
         </is>
       </c>
       <c r="H99" s="17" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I99" s="17" t="inlineStr">
@@ -9454,7 +9454,7 @@
       </c>
       <c r="J99" s="17" t="inlineStr">
         <is>
-          <t>Per disbursement</t>
+          <t>Per advance</t>
         </is>
       </c>
       <c r="K99" s="16" t="inlineStr">
@@ -9469,22 +9469,22 @@
       </c>
       <c r="M99" s="16" t="inlineStr">
         <is>
-          <t>petty-cash.service.ts (establishFund/replenishFund float guards, createRequest INSUFFICIENT_FLOAT, approveRequest SoD+GL, rejectRequest, settleRequest); petty-cash.controller.ts (creditors/exec); schema/petty-cash.ts (petty_cash_funds, expense_requests) + migration 0139; finance.service.ts pendingApprovals (GOV-01 source 7); cutover/basics.ts + compliance.ts (ToE)</t>
+          <t>finance.service.ts (issueAdvance, settleAdvance reconcile-or-reject, listAdvances outstanding); finance.controller.ts (creditors/exec); schema/finance.ts (employee_advances) + migration 0120; cutover/basics.ts (ToE)</t>
         </is>
       </c>
       <c r="N99" s="16" t="inlineStr">
         <is>
-          <t>Inspect the float ceiling + the request→approve flow + the approver≠requester check + that the request posts nothing until approval.</t>
+          <t>Inspect issue/settle GL + settlement reconciliation guard.</t>
         </is>
       </c>
       <c r="O99" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: establish a fund (Dr 1015), request an expense (no GL), self-approve → SOD_VIOLATION, approve as a different user → Dr expense/Cr 1015 + fund down; over-balance draw → INSUFFICIENT_FLOAT; advance approve→settle clears 1180; replenish past float → OVER_FLOAT (re-performed by the harnesses).</t>
+          <t>Issue an advance (1180 up); settle 700+300 clears 1180; mismatched settle → SETTLE_MISMATCH (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P99" s="16" t="inlineStr">
         <is>
-          <t>Fund register + disbursement approval log + SoD test</t>
+          <t>Advance register; outstanding float</t>
         </is>
       </c>
       <c r="Q99" s="18" t="inlineStr">
@@ -9496,12 +9496,12 @@
     <row r="100">
       <c r="A100" s="11" t="inlineStr">
         <is>
-          <t>FA-07</t>
+          <t>EXP-08</t>
         </is>
       </c>
       <c r="B100" s="12" t="inlineStr">
         <is>
-          <t>Fixed Assets</t>
+          <t>Expenditure</t>
         </is>
       </c>
       <c r="C100" s="13" t="inlineStr">
@@ -9511,27 +9511,27 @@
       </c>
       <c r="D100" s="12" t="inlineStr">
         <is>
-          <t>Property, Plant &amp; Equipment; Equity</t>
+          <t>Cash; Operating expense</t>
         </is>
       </c>
       <c r="E100" s="12" t="inlineStr">
         <is>
-          <t>Carrying amount not adjusted for revaluation/impairment — asset over/understated.</t>
+          <t>Petty-cash disbursed beyond authority / without independent review, or drawn past the fund's limit — cash leakage, unauthorised or unrecorded expense, over-extended float.</t>
         </is>
       </c>
       <c r="F100" s="12" t="inlineStr">
         <is>
-          <t>Valuation</t>
+          <t>Authorization; Completeness</t>
         </is>
       </c>
       <c r="G100" s="12" t="inlineStr">
         <is>
-          <t>Asset revaluation / impairment: an upward revaluation credits the revaluation surplus in equity (Dr 1500 / Cr 3200); a downward revaluation (impairment) debits impairment loss (Dr 5820 / Cr 1500). The gross 1500 moves by the delta so the register stays tied to the GL; a no-op revaluation is rejected (NO_CHANGE). Every event is logged for the audit trail.</t>
+          <t>Petty-cash imprest float + maker-checker on disbursement (SoD): a fund holds cash capped at a credit limit/วงเงิน (1015 Petty Cash, a cash account); each direct EXPENSE or ADVANCE is a REQUEST that posts NOTHING and a DIFFERENT user must approve before the GL posts (expense Dr &lt;expense&gt; / Cr 1015; advance Dr 1180 / Cr 1015) and the fund balance is decremented. Self-approval → SOD_VIOLATION (binds even Admin). A draw beyond the fund balance → INSUFFICIENT_FLOAT; establishing/replenishing above the float limit → OVER_FLOAT. Advances settle (Dr expense + Dr 1015 returned / Cr 1180), returning unused cash to the fund. Every request carries a document reference + receipt key + a status trail (StatusLog) and surfaces in the GOV-01 pending-approvals monitor.</t>
         </is>
       </c>
       <c r="H100" s="13" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I100" s="13" t="inlineStr">
@@ -9541,12 +9541,12 @@
       </c>
       <c r="J100" s="13" t="inlineStr">
         <is>
-          <t>Per event</t>
+          <t>Per disbursement</t>
         </is>
       </c>
       <c r="K100" s="12" t="inlineStr">
         <is>
-          <t>FaAccountant / Controller</t>
+          <t>AP / Controller</t>
         </is>
       </c>
       <c r="L100" s="13" t="inlineStr">
@@ -9556,22 +9556,22 @@
       </c>
       <c r="M100" s="12" t="inlineStr">
         <is>
-          <t>assets.service.ts (revalue up→3200 / down→5820, listRevaluations; dispose recycles surplus 3200→3100); assets.controller.ts (exec/creditors); schema/assets.ts (asset_revaluations) + migration 0120; cutover/basics.ts (ToE)</t>
+          <t>petty-cash.service.ts (establishFund/replenishFund float guards, createRequest INSUFFICIENT_FLOAT, approveRequest SoD+GL, rejectRequest, settleRequest); petty-cash.controller.ts (creditors/exec); schema/petty-cash.ts (petty_cash_funds, expense_requests) + migration 0139; finance.service.ts pendingApprovals (GOV-01 source 7); cutover/basics.ts + compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N100" s="12" t="inlineStr">
         <is>
-          <t>Inspect revaluation/impairment routing + audit log + disposal recycling.</t>
+          <t>Inspect the float ceiling + the request→approve flow + the approver≠requester check + that the request posts nothing until approval.</t>
         </is>
       </c>
       <c r="O100" s="12" t="inlineStr">
         <is>
-          <t>Upward revaluation credits 3200; impairment debits 5820; no-change → NO_CHANGE; both events logged; on disposal the revaluation surplus is recycled to retained earnings (Dr 3200 / Cr 3100), not through P&amp;L (re-performed by the harness).</t>
+          <t>Re-perform: establish a fund (Dr 1015), request an expense (no GL), self-approve → SOD_VIOLATION, approve as a different user → Dr expense/Cr 1015 + fund down; over-balance draw → INSUFFICIENT_FLOAT; advance approve→settle clears 1180; replenish past float → OVER_FLOAT (re-performed by the harnesses).</t>
         </is>
       </c>
       <c r="P100" s="12" t="inlineStr">
         <is>
-          <t>Revaluation log; disposal recycling JE</t>
+          <t>Fund register + disbursement approval log + SoD test</t>
         </is>
       </c>
       <c r="Q100" s="18" t="inlineStr">
@@ -9583,7 +9583,7 @@
     <row r="101">
       <c r="A101" s="15" t="inlineStr">
         <is>
-          <t>FA-08</t>
+          <t>FA-07</t>
         </is>
       </c>
       <c r="B101" s="16" t="inlineStr">
@@ -9603,22 +9603,22 @@
       </c>
       <c r="E101" s="16" t="inlineStr">
         <is>
-          <t>Carrying amount changed by fair-value revaluation/impairment without independent review — the preparer revalues the asset and posts to equity/P&amp;L on their own (earnings/equity management).</t>
+          <t>Carrying amount not adjusted for revaluation/impairment — asset over/understated.</t>
         </is>
       </c>
       <c r="F101" s="16" t="inlineStr">
         <is>
-          <t>Authorization</t>
+          <t>Valuation</t>
         </is>
       </c>
       <c r="G101" s="16" t="inlineStr">
         <is>
-          <t>Asset-revaluation maker-checker (SoD): a revalue/impairment request posts its GL entry as a DRAFT (excluded from balances) and records status 'PendingApproval' WITHOUT moving the carrying value; a DIFFERENT user must approve before the JE is effective and the register is re-valued (approver ≠ preparer enforced regardless of permissions, reusing the GL-05 ledger approval). Reject voids the draft; only one revaluation may be pending per asset; the disposal surplus recycle counts only approved revaluations.</t>
+          <t>Asset revaluation / impairment: an upward revaluation credits the revaluation surplus in equity (Dr 1500 / Cr 3200); a downward revaluation (impairment) debits impairment loss (Dr 5820 / Cr 1500). The gross 1500 moves by the delta so the register stays tied to the GL; a no-op revaluation is rejected (NO_CHANGE). Every event is logged for the audit trail.</t>
         </is>
       </c>
       <c r="H101" s="17" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I101" s="17" t="inlineStr">
@@ -9643,22 +9643,22 @@
       </c>
       <c r="M101" s="16" t="inlineStr">
         <is>
-          <t>assets.service.ts revalue(pendingApproval Draft)/approveRevaluation/rejectRevaluation; assets.controller.ts (:assetNo/revalue/approve|reject); schema/assets.ts asset_revaluations.status + migration 0134; cutover/basics.ts + compliance.ts (ToE)</t>
+          <t>assets.service.ts (revalue up→3200 / down→5820, listRevaluations; dispose recycles surplus 3200→3100); assets.controller.ts (exec/creditors); schema/assets.ts (asset_revaluations) + migration 0120; cutover/basics.ts (ToE)</t>
         </is>
       </c>
       <c r="N101" s="16" t="inlineStr">
         <is>
-          <t>Inspect Draft→approve flow + the approver≠preparer check + deferred carrying-value update.</t>
+          <t>Inspect revaluation/impairment routing + audit log + disposal recycling.</t>
         </is>
       </c>
       <c r="O101" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: request a revaluation (Draft JE excluded from 3200), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm the surplus/impairment + carrying value move only after approval (re-performed by the harnesses).</t>
+          <t>Upward revaluation credits 3200; impairment debits 5820; no-change → NO_CHANGE; both events logged; on disposal the revaluation surplus is recycled to retained earnings (Dr 3200 / Cr 3100), not through P&amp;L (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P101" s="16" t="inlineStr">
         <is>
-          <t>Revaluation approval log + SoD test</t>
+          <t>Revaluation log; disposal recycling JE</t>
         </is>
       </c>
       <c r="Q101" s="18" t="inlineStr">
@@ -9670,12 +9670,12 @@
     <row r="102">
       <c r="A102" s="11" t="inlineStr">
         <is>
-          <t>LSE-01</t>
+          <t>FA-08</t>
         </is>
       </c>
       <c r="B102" s="12" t="inlineStr">
         <is>
-          <t>Leases</t>
+          <t>Fixed Assets</t>
         </is>
       </c>
       <c r="C102" s="13" t="inlineStr">
@@ -9685,27 +9685,27 @@
       </c>
       <c r="D102" s="12" t="inlineStr">
         <is>
-          <t>Right-of-use assets; Lease liabilities</t>
+          <t>Property, Plant &amp; Equipment; Equity</t>
         </is>
       </c>
       <c r="E102" s="12" t="inlineStr">
         <is>
-          <t>Lease not capitalised (IFRS 16 / TFRS 16) — ROU asset + lease liability omitted; interest/depreciation mis-stated.</t>
+          <t>Carrying amount changed by fair-value revaluation/impairment without independent review — the preparer revalues the asset and posts to equity/P&amp;L on their own (earnings/equity management).</t>
         </is>
       </c>
       <c r="F102" s="12" t="inlineStr">
         <is>
-          <t>Completeness/Accuracy/Valuation</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="G102" s="12" t="inlineStr">
         <is>
-          <t>Lease accounting: at commencement a right-of-use asset and lease liability are recognised at the present value of the lease payments (Dr 1600 / Cr 2600). The scheduled job lease_periodic_run posts each period — interest unwinding on the liability (Dr 5900), the cash payment reducing the liability (Dr 2600 / Cr 1000), and straight-line ROU depreciation (Dr 5210 / Cr 1690) — the last period clearing the liability + ROU exactly. Idempotent per (lease, period).</t>
+          <t>Asset-revaluation maker-checker (SoD): a revalue/impairment request posts its GL entry as a DRAFT (excluded from balances) and records status 'PendingApproval' WITHOUT moving the carrying value; a DIFFERENT user must approve before the JE is effective and the register is re-valued (approver ≠ preparer enforced regardless of permissions, reusing the GL-05 ledger approval). Reject voids the draft; only one revaluation may be pending per asset; the disposal surplus recycle counts only approved revaluations.</t>
         </is>
       </c>
       <c r="H102" s="13" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I102" s="13" t="inlineStr">
@@ -9715,12 +9715,12 @@
       </c>
       <c r="J102" s="13" t="inlineStr">
         <is>
-          <t>Per period / per lease</t>
+          <t>Per event</t>
         </is>
       </c>
       <c r="K102" s="12" t="inlineStr">
         <is>
-          <t>Controller</t>
+          <t>FaAccountant / Controller</t>
         </is>
       </c>
       <c r="L102" s="13" t="inlineStr">
@@ -9730,22 +9730,22 @@
       </c>
       <c r="M102" s="12" t="inlineStr">
         <is>
-          <t>leases.service.ts (createLease PV recognition, runDueLeases interest+payment+depreciation, modifyLease remeasurement); leases.controller.ts (gl_post); bi.service.ts (lease_periodic_run); schema/leases.ts (leases, rou_nbv) + migration 0120/0121; cutover/basics.ts (ToE)</t>
+          <t>assets.service.ts revalue(pendingApproval Draft)/approveRevaluation/rejectRevaluation; assets.controller.ts (:assetNo/revalue/approve|reject); schema/assets.ts asset_revaluations.status + migration 0134; cutover/basics.ts + compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N102" s="12" t="inlineStr">
         <is>
-          <t>Inspect PV recognition + periodic interest/payment/depreciation + final-period clearing + modification remeasurement.</t>
+          <t>Inspect Draft→approve flow + the approver≠preparer check + deferred carrying-value update.</t>
         </is>
       </c>
       <c r="O102" s="12" t="inlineStr">
         <is>
-          <t>Commencement recognises ROU=liability=PV; periodic run posts interest+principal(=payment)+ROU depreciation; liability + ROU reduce; a modification remeasures the liability at the revised PV and adjusts the ROU by the same delta (Dr/Cr 1600↔2600), then depreciates over the remaining term (re-performed by the harness).</t>
+          <t>Re-perform: request a revaluation (Draft JE excluded from 3200), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm the surplus/impairment + carrying value move only after approval (re-performed by the harnesses).</t>
         </is>
       </c>
       <c r="P102" s="12" t="inlineStr">
         <is>
-          <t>Lease register; periodic run log; modification remeasurement</t>
+          <t>Revaluation approval log + SoD test</t>
         </is>
       </c>
       <c r="Q102" s="18" t="inlineStr">
@@ -9757,12 +9757,12 @@
     <row r="103">
       <c r="A103" s="15" t="inlineStr">
         <is>
-          <t>REC-01</t>
+          <t>LSE-01</t>
         </is>
       </c>
       <c r="B103" s="16" t="inlineStr">
         <is>
-          <t>Reconciliation</t>
+          <t>Leases</t>
         </is>
       </c>
       <c r="C103" s="17" t="inlineStr">
@@ -9772,22 +9772,22 @@
       </c>
       <c r="D103" s="16" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Right-of-use assets; Lease liabilities</t>
         </is>
       </c>
       <c r="E103" s="16" t="inlineStr">
         <is>
-          <t>Subledgers diverge from GL undetected.</t>
+          <t>Lease not capitalised (IFRS 16 / TFRS 16) — ROU asset + lease liability omitted; interest/depreciation mis-stated.</t>
         </is>
       </c>
       <c r="F103" s="16" t="inlineStr">
         <is>
-          <t>Completeness/Accuracy</t>
+          <t>Completeness/Accuracy/Valuation</t>
         </is>
       </c>
       <c r="G103" s="16" t="inlineStr">
         <is>
-          <t>Subledger-to-GL reconciliation per period: import GL, auto-match, certify (sign-off via 'approvals').</t>
+          <t>Lease accounting: at commencement a right-of-use asset and lease liability are recognised at the present value of the lease payments (Dr 1600 / Cr 2600). The scheduled job lease_periodic_run posts each period — interest unwinding on the liability (Dr 5900), the cash payment reducing the liability (Dr 2600 / Cr 1000), and straight-line ROU depreciation (Dr 5210 / Cr 1690) — the last period clearing the liability + ROU exactly. Idempotent per (lease, period).</t>
         </is>
       </c>
       <c r="H103" s="17" t="inlineStr">
@@ -9797,12 +9797,12 @@
       </c>
       <c r="I103" s="17" t="inlineStr">
         <is>
-          <t>Auto+Manual</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J103" s="17" t="inlineStr">
         <is>
-          <t>Monthly</t>
+          <t>Per period / per lease</t>
         </is>
       </c>
       <c r="K103" s="16" t="inlineStr">
@@ -9812,27 +9812,27 @@
       </c>
       <c r="L103" s="17" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="M103" s="16" t="inlineStr">
         <is>
-          <t>reconciliation.service.ts (importGlItems/autoMatch/certify)</t>
+          <t>leases.service.ts (createLease PV recognition, runDueLeases interest+payment+depreciation, modifyLease remeasurement); leases.controller.ts (gl_post); bi.service.ts (lease_periodic_run); schema/leases.ts (leases, rou_nbv) + migration 0120/0121; cutover/basics.ts (ToE)</t>
         </is>
       </c>
       <c r="N103" s="16" t="inlineStr">
         <is>
-          <t>Inspect recon + certify gate.</t>
+          <t>Inspect PV recognition + periodic interest/payment/depreciation + final-period clearing + modification remeasurement.</t>
         </is>
       </c>
       <c r="O103" s="16" t="inlineStr">
         <is>
-          <t>Sample periods: reconciled, unmatched cleared, certified.</t>
+          <t>Commencement recognises ROU=liability=PV; periodic run posts interest+principal(=payment)+ROU depreciation; liability + ROU reduce; a modification remeasures the liability at the revised PV and adjusts the ROU by the same delta (Dr/Cr 1600↔2600), then depreciates over the remaining term (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P103" s="16" t="inlineStr">
         <is>
-          <t>Certified recon</t>
+          <t>Lease register; periodic run log; modification remeasurement</t>
         </is>
       </c>
       <c r="Q103" s="18" t="inlineStr">
@@ -9844,7 +9844,7 @@
     <row r="104">
       <c r="A104" s="11" t="inlineStr">
         <is>
-          <t>REC-02</t>
+          <t>REC-01</t>
         </is>
       </c>
       <c r="B104" s="12" t="inlineStr">
@@ -9859,22 +9859,22 @@
       </c>
       <c r="D104" s="12" t="inlineStr">
         <is>
-          <t>Cash</t>
+          <t>All</t>
         </is>
       </c>
       <c r="E104" s="12" t="inlineStr">
         <is>
-          <t>Bank balance not reconciled to GL.</t>
+          <t>Subledgers diverge from GL undetected.</t>
         </is>
       </c>
       <c r="F104" s="12" t="inlineStr">
         <is>
-          <t>Existence/Completeness</t>
+          <t>Completeness/Accuracy</t>
         </is>
       </c>
       <c r="G104" s="12" t="inlineStr">
         <is>
-          <t>Bank reconciliation against statements.</t>
+          <t>Subledger-to-GL reconciliation per period: import GL, auto-match, certify (sign-off via 'approvals').</t>
         </is>
       </c>
       <c r="H104" s="13" t="inlineStr">
@@ -9904,22 +9904,22 @@
       </c>
       <c r="M104" s="12" t="inlineStr">
         <is>
-          <t>bank module; drizzle/0015_bank_reconciliation</t>
+          <t>reconciliation.service.ts (importGlItems/autoMatch/certify)</t>
         </is>
       </c>
       <c r="N104" s="12" t="inlineStr">
         <is>
-          <t>Inspect bank-rec process.</t>
+          <t>Inspect recon + certify gate.</t>
         </is>
       </c>
       <c r="O104" s="12" t="inlineStr">
         <is>
-          <t>Sample months reconciled &amp; reviewed.</t>
+          <t>Sample periods: reconciled, unmatched cleared, certified.</t>
         </is>
       </c>
       <c r="P104" s="12" t="inlineStr">
         <is>
-          <t>Bank rec</t>
+          <t>Certified recon</t>
         </is>
       </c>
       <c r="Q104" s="18" t="inlineStr">
@@ -9931,12 +9931,12 @@
     <row r="105">
       <c r="A105" s="15" t="inlineStr">
         <is>
-          <t>BANK-02</t>
+          <t>REC-02</t>
         </is>
       </c>
       <c r="B105" s="16" t="inlineStr">
         <is>
-          <t>Cash &amp; Treasury</t>
+          <t>Reconciliation</t>
         </is>
       </c>
       <c r="C105" s="17" t="inlineStr">
@@ -9946,37 +9946,37 @@
       </c>
       <c r="D105" s="16" t="inlineStr">
         <is>
-          <t>Cash; Operating expense; Interest income</t>
+          <t>Cash</t>
         </is>
       </c>
       <c r="E105" s="16" t="inlineStr">
         <is>
-          <t>A bank fee/interest adjustment is posted straight to the GL by one person during reconciliation — a cash outflow mis-booked as interest income, or a fictitious fee posted, with no independent review (single-person posting to the cash account).</t>
+          <t>Bank balance not reconciled to GL.</t>
         </is>
       </c>
       <c r="F105" s="16" t="inlineStr">
         <is>
-          <t>Authorization/Accuracy</t>
+          <t>Existence/Completeness</t>
         </is>
       </c>
       <c r="G105" s="16" t="inlineStr">
         <is>
-          <t>Bank adjustment maker-checker (SoD): a fee/interest adjustment on a statement line is a REQUEST that posts a DRAFT JE (no balance/GL effect; the line stays unreconciled) until a DIFFERENT user with approval authority approves (POST /api/bank/lines/:id/adjustment/approve). Self-approval → SOD_VIOLATION (binds even Admin); approval flips the line to reconciled and the JE to Posted; reject voids the Draft and frees the line. The Draft JE (source BANKADJ) is also surfaced, aged, by the pending-approvals monitor (GOV-01).</t>
+          <t>Bank reconciliation against statements.</t>
         </is>
       </c>
       <c r="H105" s="17" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I105" s="17" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="J105" s="17" t="inlineStr">
         <is>
-          <t>Per adjustment</t>
+          <t>Monthly</t>
         </is>
       </c>
       <c r="K105" s="16" t="inlineStr">
@@ -9986,27 +9986,27 @@
       </c>
       <c r="L105" s="17" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="M105" s="16" t="inlineStr">
         <is>
-          <t>bank.service.ts requestAdjustment/approveAdjustment/rejectAdjustment/listPendingAdjustments (reuses ledger.approveEntry SoD); bank.controller.ts (lines/:id/adjustment requests; adjustment/approve|reject gated approvals/gl_close); cutover/bankrec.ts (ToE)</t>
+          <t>bank module; drizzle/0015_bank_reconciliation</t>
         </is>
       </c>
       <c r="N105" s="16" t="inlineStr">
         <is>
-          <t>Inspect the request→approve flow + the approver≠requester check + that the Draft posts nothing until approval.</t>
+          <t>Inspect bank-rec process.</t>
         </is>
       </c>
       <c r="O105" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: request a fee adjustment (line unreconciled, GL difference unchanged), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm the difference closes to 0 only after approval (re-performed by the bankrec harness).</t>
+          <t>Sample months reconciled &amp; reviewed.</t>
         </is>
       </c>
       <c r="P105" s="16" t="inlineStr">
         <is>
-          <t>Bank adjustment queue + SoD test</t>
+          <t>Bank rec</t>
         </is>
       </c>
       <c r="Q105" s="18" t="inlineStr">
@@ -10018,12 +10018,12 @@
     <row r="106">
       <c r="A106" s="11" t="inlineStr">
         <is>
-          <t>REC-03</t>
+          <t>BANK-02</t>
         </is>
       </c>
       <c r="B106" s="12" t="inlineStr">
         <is>
-          <t>Reconciliation</t>
+          <t>Cash &amp; Treasury</t>
         </is>
       </c>
       <c r="C106" s="13" t="inlineStr">
@@ -10033,79 +10033,79 @@
       </c>
       <c r="D106" s="12" t="inlineStr">
         <is>
-          <t>Consolidation</t>
+          <t>Cash; Operating expense; Interest income</t>
         </is>
       </c>
       <c r="E106" s="12" t="inlineStr">
         <is>
-          <t>Intercompany balances not eliminated/agreed.</t>
+          <t>A bank fee/interest adjustment is posted straight to the GL by one person during reconciliation — a cash outflow mis-booked as interest income, or a fictitious fee posted, with no independent review (single-person posting to the cash account).</t>
         </is>
       </c>
       <c r="F106" s="12" t="inlineStr">
         <is>
-          <t>Accuracy</t>
+          <t>Authorization/Accuracy</t>
         </is>
       </c>
       <c r="G106" s="12" t="inlineStr">
         <is>
-          <t>Intercompany reconciliation &amp; elimination on consolidation.</t>
+          <t>Bank adjustment maker-checker (SoD): a fee/interest adjustment on a statement line is a REQUEST that posts a DRAFT JE (no balance/GL effect; the line stays unreconciled) until a DIFFERENT user with approval authority approves (POST /api/bank/lines/:id/adjustment/approve). Self-approval → SOD_VIOLATION (binds even Admin); approval flips the line to reconciled and the JE to Posted; reject voids the Draft and frees the line. The Draft JE (source BANKADJ) is also surfaced, aged, by the pending-approvals monitor (GOV-01).</t>
         </is>
       </c>
       <c r="H106" s="13" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I106" s="13" t="inlineStr">
         <is>
-          <t>Auto+Manual</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J106" s="13" t="inlineStr">
         <is>
-          <t>Period</t>
+          <t>Per adjustment</t>
         </is>
       </c>
       <c r="K106" s="12" t="inlineStr">
         <is>
-          <t>Group Controller</t>
+          <t>Controller</t>
         </is>
       </c>
       <c r="L106" s="13" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="M106" s="12" t="inlineStr">
         <is>
-          <t>intercompany; consolidation</t>
+          <t>bank.service.ts requestAdjustment/approveAdjustment/rejectAdjustment/listPendingAdjustments (reuses ledger.approveEntry SoD); bank.controller.ts (lines/:id/adjustment requests; adjustment/approve|reject gated approvals/gl_close); cutover/bankrec.ts (ToE)</t>
         </is>
       </c>
       <c r="N106" s="12" t="inlineStr">
         <is>
-          <t>Inspect IC matching + elimination.</t>
+          <t>Inspect the request→approve flow + the approver≠requester check + that the Draft posts nothing until approval.</t>
         </is>
       </c>
       <c r="O106" s="12" t="inlineStr">
         <is>
-          <t>Sample IC pairs agree &amp; eliminate.</t>
+          <t>Re-perform: request a fee adjustment (line unreconciled, GL difference unchanged), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm the difference closes to 0 only after approval (re-performed by the bankrec harness).</t>
         </is>
       </c>
       <c r="P106" s="12" t="inlineStr">
         <is>
-          <t>IC recon</t>
-        </is>
-      </c>
-      <c r="Q106" s="19" t="inlineStr">
-        <is>
-          <t>Partial</t>
+          <t>Bank adjustment queue + SoD test</t>
+        </is>
+      </c>
+      <c r="Q106" s="18" t="inlineStr">
+        <is>
+          <t>Implemented</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="15" t="inlineStr">
         <is>
-          <t>REC-04</t>
+          <t>REC-03</t>
         </is>
       </c>
       <c r="B107" s="16" t="inlineStr">
@@ -10120,22 +10120,22 @@
       </c>
       <c r="D107" s="16" t="inlineStr">
         <is>
-          <t>All control accounts</t>
+          <t>Consolidation</t>
         </is>
       </c>
       <c r="E107" s="16" t="inlineStr">
         <is>
-          <t>A sub-ledger silently drifts from its GL control account at period-end and no single review catches it (incomplete/inaccurate balances reach the financial statements).</t>
+          <t>Intercompany balances not eliminated/agreed.</t>
         </is>
       </c>
       <c r="F107" s="16" t="inlineStr">
         <is>
-          <t>Completeness/Accuracy</t>
+          <t>Accuracy</t>
         </is>
       </c>
       <c r="G107" s="16" t="inlineStr">
         <is>
-          <t>Period-end control-account reconciliation PACK: one read (GET /api/finance/reconciliation/controls) ties every major sub-ledger to its GL control account and FLAGS any out-of-balance — AR↔1100, AP↔2000, Inventory↔1200, Gift cards/Customer-deposits↔2200, Deferred revenue↔2400 — reporting per line {sub_ledger, gl_control, variance, reconciled} plus an overall all_reconciled flag and an exceptions count. Liability controls are sign-flipped before comparison. The controller's single 'are the books reconciled?' close view; an exception is a control finding to investigate before sign-off.</t>
+          <t>Intercompany reconciliation &amp; elimination on consolidation.</t>
         </is>
       </c>
       <c r="H107" s="17" t="inlineStr">
@@ -10145,17 +10145,17 @@
       </c>
       <c r="I107" s="17" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="J107" s="17" t="inlineStr">
         <is>
-          <t>Period / on demand</t>
+          <t>Period</t>
         </is>
       </c>
       <c r="K107" s="16" t="inlineStr">
         <is>
-          <t>Controller / CFO</t>
+          <t>Group Controller</t>
         </is>
       </c>
       <c r="L107" s="17" t="inlineStr">
@@ -10165,34 +10165,34 @@
       </c>
       <c r="M107" s="16" t="inlineStr">
         <is>
-          <t>finance.service.ts reconcileControls; finance.controller.ts GET reconciliation/controls (exec/ar/creditors); reuses ledger.trialBalance + the AR/AP/inventory/gift-card/deferred sub-ledgers; cutover/giftcards.ts + compliance.ts (ToE)</t>
+          <t>intercompany; consolidation</t>
         </is>
       </c>
       <c r="N107" s="16" t="inlineStr">
         <is>
-          <t>Inspect the pack: each control account's sub-ledger query + the GL tie + the exceptions roll-up.</t>
+          <t>Inspect IC matching + elimination.</t>
         </is>
       </c>
       <c r="O107" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: with a clean set, every line reconciled + all_reconciled=true; introduce a known sub-ledger/GL difference and confirm it surfaces as an exception (re-performed: gift-card 2200 + inventory 1200 ties asserted by the harnesses).</t>
+          <t>Sample IC pairs agree &amp; eliminate.</t>
         </is>
       </c>
       <c r="P107" s="16" t="inlineStr">
         <is>
-          <t>Reconciliation pack; exceptions list</t>
-        </is>
-      </c>
-      <c r="Q107" s="18" t="inlineStr">
-        <is>
-          <t>Implemented</t>
+          <t>IC recon</t>
+        </is>
+      </c>
+      <c r="Q107" s="19" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="11" t="inlineStr">
         <is>
-          <t>REC-05</t>
+          <t>REC-04</t>
         </is>
       </c>
       <c r="B108" s="12" t="inlineStr">
@@ -10207,42 +10207,42 @@
       </c>
       <c r="D108" s="12" t="inlineStr">
         <is>
-          <t>Cash; Bank</t>
+          <t>All control accounts</t>
         </is>
       </c>
       <c r="E108" s="12" t="inlineStr">
         <is>
-          <t>Till cash dropped to the safe never reaches the bank, or a deposit isn't matched to the statement — cash sits unbanked (theft/loss exposure) or the bank balance can't be tied to the books.</t>
+          <t>A sub-ledger silently drifts from its GL control account at period-end and no single review catches it (incomplete/inaccurate balances reach the financial statements).</t>
         </is>
       </c>
       <c r="F108" s="12" t="inlineStr">
         <is>
-          <t>Completeness/Existence/Authorization</t>
+          <t>Completeness/Accuracy</t>
         </is>
       </c>
       <c r="G108" s="12" t="inlineStr">
         <is>
-          <t>Cash banking — safe-drop → bank deposit → reconciliation: till 'drop's move cash from the drawer to the safe (drawer-only, no GL). Banking BATCHES the undeposited drops into a deposit and posts the GL (Dr &lt;bank account, e.g. 1010&gt; / Cr 1000 Cash), stamping each drop with the deposit id; the deposit is then RECONCILED to the bank statement (status Deposited→Reconciled). A detective read (GET /api/bank/deposits/undeposited-drops) surfaces the CASH STILL IN THE SAFE (drops with deposit_id NULL) — the unbanked exposure to chase. SoD: banking is a treasury duty (exec/ar) — segregated from the cashier (pos_till) who drops the cash, so the person who removes cash from the drawer is not the one who banks it.</t>
+          <t>Period-end control-account reconciliation PACK: one read (GET /api/finance/reconciliation/controls) ties every major sub-ledger to its GL control account and FLAGS any out-of-balance — AR↔1100, AP↔2000, Inventory↔1200, Gift cards/Customer-deposits↔2200, Deferred revenue↔2400 — reporting per line {sub_ledger, gl_control, variance, reconciled} plus an overall all_reconciled flag and an exceptions count. Liability controls are sign-flipped before comparison. The controller's single 'are the books reconciled?' close view; an exception is a control finding to investigate before sign-off.</t>
         </is>
       </c>
       <c r="H108" s="13" t="inlineStr">
         <is>
-          <t>Det/Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I108" s="13" t="inlineStr">
         <is>
-          <t>Auto+Manual</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J108" s="13" t="inlineStr">
         <is>
-          <t>Per banking run</t>
+          <t>Period / on demand</t>
         </is>
       </c>
       <c r="K108" s="12" t="inlineStr">
         <is>
-          <t>FinancialController / Treasury</t>
+          <t>Controller / CFO</t>
         </is>
       </c>
       <c r="L108" s="13" t="inlineStr">
@@ -10252,22 +10252,22 @@
       </c>
       <c r="M108" s="12" t="inlineStr">
         <is>
-          <t>bank.service.ts undepositedDrops/createDeposit (Dr bank/Cr 1000, stamps deposit_id)/reconcileDeposit/listDeposits; bank.controller.ts (deposits, deposits/undeposited-drops, deposits/:id/reconcile; exec/ar); schema/cash.ts bank_deposits + cash_movements.deposit_id + migration 0152; /cash-banking UI; cutover/cash-banking.ts (ToE)</t>
+          <t>finance.service.ts reconcileControls; finance.controller.ts GET reconciliation/controls (exec/ar/creditors); reuses ledger.trialBalance + the AR/AP/inventory/gift-card/deferred sub-ledgers; cutover/giftcards.ts + compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N108" s="12" t="inlineStr">
         <is>
-          <t>Inspect the undeposited-drop exposure read + the deposit GL (bank↔1000) + the reconcile step + the SoD (cashier vs treasury).</t>
+          <t>Inspect the pack: each control account's sub-ledger query + the GL tie + the exceptions roll-up.</t>
         </is>
       </c>
       <c r="O108" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: two till drops → cash-in-safe shows the total; a cashier (pos_till) cannot bank (403); treasury banks → Dr bank / Cr 1000, cash-in-safe back to 0; reconcile the deposit; trial balance balanced (re-performed by the cash-banking harness).</t>
+          <t>Re-perform: with a clean set, every line reconciled + all_reconciled=true; introduce a known sub-ledger/GL difference and confirm it surfaces as an exception (re-performed: gift-card 2200 + inventory 1200 ties asserted by the harnesses).</t>
         </is>
       </c>
       <c r="P108" s="12" t="inlineStr">
         <is>
-          <t>Bank-deposit register; undeposited-drop (cash-in-safe) exposure</t>
+          <t>Reconciliation pack; exceptions list</t>
         </is>
       </c>
       <c r="Q108" s="18" t="inlineStr">
@@ -10279,12 +10279,12 @@
     <row r="109">
       <c r="A109" s="15" t="inlineStr">
         <is>
-          <t>GOV-01</t>
+          <t>REC-05</t>
         </is>
       </c>
       <c r="B109" s="16" t="inlineStr">
         <is>
-          <t>Monitoring</t>
+          <t>Reconciliation</t>
         </is>
       </c>
       <c r="C109" s="17" t="inlineStr">
@@ -10294,42 +10294,42 @@
       </c>
       <c r="D109" s="16" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Cash; Bank</t>
         </is>
       </c>
       <c r="E109" s="16" t="inlineStr">
         <is>
-          <t>A maker-checker approval sits un-actioned and is forgotten — a transaction stalls before it is effective, or (worse) a control is quietly bypassed and no one notices an item never got its independent review.</t>
+          <t>Till cash dropped to the safe never reaches the bank, or a deposit isn't matched to the statement — cash sits unbanked (theft/loss exposure) or the bank balance can't be tied to the books.</t>
         </is>
       </c>
       <c r="F109" s="16" t="inlineStr">
         <is>
-          <t>Authorization/Completeness</t>
+          <t>Completeness/Existence/Authorization</t>
         </is>
       </c>
       <c r="G109" s="16" t="inlineStr">
         <is>
-          <t>Pending-approvals MONITOR (COSO monitoring): a single worklist of EVERY item awaiting independent approval across the system, each with its AGE in days and an overdue roll-up — spanning the manual-JE (GL-05), bank-adjustment (BANK-02), AP-disbursement (EXP-06), payroll (PAY-03), asset-revaluation (FA-08), asset-disposal (FA-09), inventory-write-off (INV-07), till-close cash over/short (REV-13), FX-rate (FX-04), budget (BUD-01) and large-refund (REV-16) maker-checkers. The controller reviews it before close; a stale item (age beyond the threshold) is a control finding to chase or escalate. The /approvals screen also lets a manager approve/reject a material till variance or a large refund inline (the pending types with no dedicated module screen). Read-only worklist; tenant-scoped via the caller's RLS.</t>
+          <t>Cash banking — safe-drop → bank deposit → reconciliation: till 'drop's move cash from the drawer to the safe (drawer-only, no GL). Banking BATCHES the undeposited drops into a deposit and posts the GL (Dr &lt;bank account, e.g. 1010&gt; / Cr 1000 Cash), stamping each drop with the deposit id; the deposit is then RECONCILED to the bank statement (status Deposited→Reconciled). A detective read (GET /api/bank/deposits/undeposited-drops) surfaces the CASH STILL IN THE SAFE (drops with deposit_id NULL) — the unbanked exposure to chase. SoD: banking is a treasury duty (exec/ar) — segregated from the cashier (pos_till) who drops the cash, so the person who removes cash from the drawer is not the one who banks it.</t>
         </is>
       </c>
       <c r="H109" s="17" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Det/Prev</t>
         </is>
       </c>
       <c r="I109" s="17" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="J109" s="17" t="inlineStr">
         <is>
-          <t>Continuous / pre-close</t>
+          <t>Per banking run</t>
         </is>
       </c>
       <c r="K109" s="16" t="inlineStr">
         <is>
-          <t>Controller / CFO</t>
+          <t>FinancialController / Treasury</t>
         </is>
       </c>
       <c r="L109" s="17" t="inlineStr">
@@ -10339,22 +10339,22 @@
       </c>
       <c r="M109" s="16" t="inlineStr">
         <is>
-          <t>finance.service.ts pendingApprovals; finance.controller.ts GET approvals/pending (exec/approvals/creditors); aggregates journalEntries(Draft incl. BANKADJ→BANK-02)/apPayments/payruns/asset_revaluations/fixed_assets(disposal_pending)/inv_writeoff_requests/till_sessions(PendingApproval)/fx_rates(PendingApproval)/budgets(PendingApproval); cutover/compliance.ts (ToE)</t>
+          <t>bank.service.ts undepositedDrops/createDeposit (Dr bank/Cr 1000, stamps deposit_id)/reconcileDeposit/listDeposits; bank.controller.ts (deposits, deposits/undeposited-drops, deposits/:id/reconcile; exec/ar); schema/cash.ts bank_deposits + cash_movements.deposit_id + migration 0152; /cash-banking UI; cutover/cash-banking.ts (ToE)</t>
         </is>
       </c>
       <c r="N109" s="16" t="inlineStr">
         <is>
-          <t>Inspect the aggregation across all pending sources + the age/overdue roll-up.</t>
+          <t>Inspect the undeposited-drop exposure read + the deposit GL (bank↔1000) + the reconcile step + the SoD (cashier vs treasury).</t>
         </is>
       </c>
       <c r="O109" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: create a pending item (e.g. a Draft JE) and confirm it appears in the worklist with its control ID, amount and age; the overdue count flags items past the threshold (re-performed by the harness).</t>
+          <t>Re-perform: two till drops → cash-in-safe shows the total; a cashier (pos_till) cannot bank (403); treasury banks → Dr bank / Cr 1000, cash-in-safe back to 0; reconcile the deposit; trial balance balanced (re-performed by the cash-banking harness).</t>
         </is>
       </c>
       <c r="P109" s="16" t="inlineStr">
         <is>
-          <t>Pending-approvals worklist</t>
+          <t>Bank-deposit register; undeposited-drop (cash-in-safe) exposure</t>
         </is>
       </c>
       <c r="Q109" s="18" t="inlineStr">
@@ -10366,12 +10366,12 @@
     <row r="110">
       <c r="A110" s="11" t="inlineStr">
         <is>
-          <t>TAX-01</t>
+          <t>GOV-01</t>
         </is>
       </c>
       <c r="B110" s="12" t="inlineStr">
         <is>
-          <t>Tax</t>
+          <t>Monitoring</t>
         </is>
       </c>
       <c r="C110" s="13" t="inlineStr">
@@ -10381,27 +10381,27 @@
       </c>
       <c r="D110" s="12" t="inlineStr">
         <is>
-          <t>Tax (VAT)</t>
+          <t>All</t>
         </is>
       </c>
       <c r="E110" s="12" t="inlineStr">
         <is>
-          <t>VAT computed incorrectly → filing/penalty risk.</t>
+          <t>A maker-checker approval sits un-actioned and is forgotten — a transaction stalls before it is effective, or (worse) a control is quietly bypassed and no one notices an item never got its independent review.</t>
         </is>
       </c>
       <c r="F110" s="12" t="inlineStr">
         <is>
-          <t>Accuracy</t>
+          <t>Authorization/Completeness</t>
         </is>
       </c>
       <c r="G110" s="12" t="inlineStr">
         <is>
-          <t>VAT via pluggable provider (TH 7%); unit-tested; no hard-coded rate.</t>
+          <t>Pending-approvals MONITOR (COSO monitoring): a single worklist of EVERY item awaiting independent approval across the system, each with its AGE in days and an overdue roll-up — spanning the manual-JE (GL-05), bank-adjustment (BANK-02), AP-disbursement (EXP-06), payroll (PAY-03), asset-revaluation (FA-08), asset-disposal (FA-09), inventory-write-off (INV-07), till-close cash over/short (REV-13), FX-rate (FX-04), budget (BUD-01) and large-refund (REV-16) maker-checkers. The controller reviews it before close; a stale item (age beyond the threshold) is a control finding to chase or escalate. The /approvals screen also lets a manager approve/reject a material till variance or a large refund inline (the pending types with no dedicated module screen). Read-only worklist; tenant-scoped via the caller's RLS.</t>
         </is>
       </c>
       <c r="H110" s="13" t="inlineStr">
         <is>
-          <t>Auto</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I110" s="13" t="inlineStr">
@@ -10411,37 +10411,37 @@
       </c>
       <c r="J110" s="13" t="inlineStr">
         <is>
-          <t>Per txn</t>
+          <t>Continuous / pre-close</t>
         </is>
       </c>
       <c r="K110" s="12" t="inlineStr">
         <is>
-          <t>Tax / Controller</t>
+          <t>Controller / CFO</t>
         </is>
       </c>
       <c r="L110" s="13" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="M110" s="12" t="inlineStr">
         <is>
-          <t>tax/tax-providers.ts; tax.service.ts; test/unit.test.ts</t>
+          <t>finance.service.ts pendingApprovals; finance.controller.ts GET approvals/pending (exec/approvals/creditors); aggregates journalEntries(Draft incl. BANKADJ→BANK-02)/apPayments/payruns/asset_revaluations/fixed_assets(disposal_pending)/inv_writeoff_requests/till_sessions(PendingApproval)/fx_rates(PendingApproval)/budgets(PendingApproval); cutover/compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N110" s="12" t="inlineStr">
         <is>
-          <t>Inspect rate provider + tests.</t>
+          <t>Inspect the aggregation across all pending sources + the age/overdue roll-up.</t>
         </is>
       </c>
       <c r="O110" s="12" t="inlineStr">
         <is>
-          <t>Re-perform VAT on sample; tie to return.</t>
+          <t>Re-perform: create a pending item (e.g. a Draft JE) and confirm it appears in the worklist with its control ID, amount and age; the overdue count flags items past the threshold (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P110" s="12" t="inlineStr">
         <is>
-          <t>VAT tests</t>
+          <t>Pending-approvals worklist</t>
         </is>
       </c>
       <c r="Q110" s="18" t="inlineStr">
@@ -10453,7 +10453,7 @@
     <row r="111">
       <c r="A111" s="15" t="inlineStr">
         <is>
-          <t>TAX-02</t>
+          <t>TAX-01</t>
         </is>
       </c>
       <c r="B111" s="16" t="inlineStr">
@@ -10468,22 +10468,22 @@
       </c>
       <c r="D111" s="16" t="inlineStr">
         <is>
-          <t>Tax; Revenue</t>
+          <t>Tax (VAT)</t>
         </is>
       </c>
       <c r="E111" s="16" t="inlineStr">
         <is>
-          <t>Non-compliant e-Tax invoice / not transmitted to ETDA.</t>
+          <t>VAT computed incorrectly → filing/penalty risk.</t>
         </is>
       </c>
       <c r="F111" s="16" t="inlineStr">
         <is>
-          <t>Accuracy/Compliance</t>
+          <t>Accuracy</t>
         </is>
       </c>
       <c r="G111" s="16" t="inlineStr">
         <is>
-          <t>e-Tax invoice (ETDA UBL 2.1 XML) generation + email with CC to ETDA timestamp mailbox.</t>
+          <t>VAT via pluggable provider (TH 7%); unit-tested; no hard-coded rate.</t>
         </is>
       </c>
       <c r="H111" s="17" t="inlineStr">
@@ -10498,37 +10498,37 @@
       </c>
       <c r="J111" s="17" t="inlineStr">
         <is>
-          <t>Per invoice</t>
+          <t>Per txn</t>
         </is>
       </c>
       <c r="K111" s="16" t="inlineStr">
         <is>
-          <t>Tax</t>
+          <t>Tax / Controller</t>
         </is>
       </c>
       <c r="L111" s="17" t="inlineStr">
         <is>
-          <t>P10/P13</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="M111" s="16" t="inlineStr">
         <is>
-          <t>tax-docs/etax-xml.ts; etax-email.service.ts (tested)</t>
+          <t>tax/tax-providers.ts; tax.service.ts; test/unit.test.ts</t>
         </is>
       </c>
       <c r="N111" s="16" t="inlineStr">
         <is>
-          <t>Inspect XML schema + email composer.</t>
+          <t>Inspect rate provider + tests.</t>
         </is>
       </c>
       <c r="O111" s="16" t="inlineStr">
         <is>
-          <t>Sample invoices: valid XML, correct CC/escaping.</t>
+          <t>Re-perform VAT on sample; tie to return.</t>
         </is>
       </c>
       <c r="P111" s="16" t="inlineStr">
         <is>
-          <t>e-Tax samples</t>
+          <t>VAT tests</t>
         </is>
       </c>
       <c r="Q111" s="18" t="inlineStr">
@@ -10540,7 +10540,7 @@
     <row r="112">
       <c r="A112" s="11" t="inlineStr">
         <is>
-          <t>TAX-03</t>
+          <t>TAX-02</t>
         </is>
       </c>
       <c r="B112" s="12" t="inlineStr">
@@ -10555,22 +10555,22 @@
       </c>
       <c r="D112" s="12" t="inlineStr">
         <is>
-          <t>Tax (WHT)</t>
+          <t>Tax; Revenue</t>
         </is>
       </c>
       <c r="E112" s="12" t="inlineStr">
         <is>
-          <t>Withholding tax mis-computed / not reported.</t>
+          <t>Non-compliant e-Tax invoice / not transmitted to ETDA.</t>
         </is>
       </c>
       <c r="F112" s="12" t="inlineStr">
         <is>
-          <t>Accuracy</t>
+          <t>Accuracy/Compliance</t>
         </is>
       </c>
       <c r="G112" s="12" t="inlineStr">
         <is>
-          <t>WHT computation and ภ.ง.ด. reporting.</t>
+          <t>e-Tax invoice (ETDA UBL 2.1 XML) generation + email with CC to ETDA timestamp mailbox.</t>
         </is>
       </c>
       <c r="H112" s="13" t="inlineStr">
@@ -10585,7 +10585,7 @@
       </c>
       <c r="J112" s="13" t="inlineStr">
         <is>
-          <t>Per txn / monthly</t>
+          <t>Per invoice</t>
         </is>
       </c>
       <c r="K112" s="12" t="inlineStr">
@@ -10595,39 +10595,39 @@
       </c>
       <c r="L112" s="13" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P10/P13</t>
         </is>
       </c>
       <c r="M112" s="12" t="inlineStr">
         <is>
-          <t>tax-reports; payroll</t>
+          <t>tax-docs/etax-xml.ts; etax-email.service.ts (tested)</t>
         </is>
       </c>
       <c r="N112" s="12" t="inlineStr">
         <is>
-          <t>Inspect WHT logic + report.</t>
+          <t>Inspect XML schema + email composer.</t>
         </is>
       </c>
       <c r="O112" s="12" t="inlineStr">
         <is>
-          <t>Re-perform WHT on sample; tie to filing.</t>
+          <t>Sample invoices: valid XML, correct CC/escaping.</t>
         </is>
       </c>
       <c r="P112" s="12" t="inlineStr">
         <is>
-          <t>WHT report</t>
-        </is>
-      </c>
-      <c r="Q112" s="19" t="inlineStr">
-        <is>
-          <t>Partial</t>
+          <t>e-Tax samples</t>
+        </is>
+      </c>
+      <c r="Q112" s="18" t="inlineStr">
+        <is>
+          <t>Implemented</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="15" t="inlineStr">
         <is>
-          <t>TAX-04</t>
+          <t>TAX-03</t>
         </is>
       </c>
       <c r="B113" s="16" t="inlineStr">
@@ -10642,27 +10642,27 @@
       </c>
       <c r="D113" s="16" t="inlineStr">
         <is>
-          <t>Tax (VAT); Tax Payable (2100)</t>
+          <t>Tax (WHT)</t>
         </is>
       </c>
       <c r="E113" s="16" t="inlineStr">
         <is>
-          <t>Output/input VAT on the filed ภ.พ.30 return does not agree to the GL — VAT liability mis-stated, a filing/penalty exposure, or a posting omission goes undetected before submission.</t>
+          <t>Withholding tax mis-computed / not reported.</t>
         </is>
       </c>
       <c r="F113" s="16" t="inlineStr">
         <is>
-          <t>Completeness/Accuracy</t>
+          <t>Accuracy</t>
         </is>
       </c>
       <c r="G113" s="16" t="inlineStr">
         <is>
-          <t>Periodic VAT-return ↔ GL reconciliation (ภ.พ.30): the monthly return (GET /api/tax-reports/pp30) is built from the sales/output-VAT and purchase/input-VAT sub-reports, computes net VAT = output − input, and RECONCILES it to the **GL account 2100 (Tax Payable) net movement** for the same period (Σ credit − Σ debit over Posted entries) — returning `reconciliation.tied` = true only when the two agree within rounding. A non-tie is a detective finding to investigate and clear BEFORE filing (the form also carries the ม.157 deadline = the 15th of the next month). Output VAT is posted to 2100 on every sale (Cr) and reversed on returns (Dr); input VAT is posted on AP bills (Dr) — so 2100's net is the period's VAT payable. Read-only report; exportable to a ภ.พ.30 PDF/HTML.</t>
+          <t>WHT computation and ภ.ง.ด. reporting.</t>
         </is>
       </c>
       <c r="H113" s="17" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Auto</t>
         </is>
       </c>
       <c r="I113" s="17" t="inlineStr">
@@ -10672,54 +10672,54 @@
       </c>
       <c r="J113" s="17" t="inlineStr">
         <is>
-          <t>Monthly / pre-filing</t>
+          <t>Per txn / monthly</t>
         </is>
       </c>
       <c r="K113" s="16" t="inlineStr">
         <is>
-          <t>Tax / FinancialController</t>
+          <t>Tax</t>
         </is>
       </c>
       <c r="L113" s="17" t="inlineStr">
         <is>
-          <t>P10/P16</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="M113" s="16" t="inlineStr">
         <is>
-          <t>tax-reports.service.ts pp30 (outputVat/inputVat + 2100 net-movement tie); tax-reports.controller.ts (GET pp30, pp30/export, exec); tax-reports-pdf.ts; dine-in.service.ts/returns.service.ts/finance.service.ts post 2100 on sale/return/AP; /tax/reports UI; cutover/taxdocs.ts (ToE)</t>
+          <t>tax-reports; payroll</t>
         </is>
       </c>
       <c r="N113" s="16" t="inlineStr">
         <is>
-          <t>Inspect the pp30 build + the 2100 net-movement query + the tie flag + the filing deadline.</t>
+          <t>Inspect WHT logic + report.</t>
         </is>
       </c>
       <c r="O113" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: the pp30 return computes net VAT (output − input), the GL 2100 net movement reflects the posted input VAT, and the reconciliation block exposes the gl_account (2100), the report net VAT and a boolean tie verdict (tied iff the two agree within rounding); the ภ.พ.30 export renders (re-performed by the taxdocs harness).</t>
+          <t>Re-perform WHT on sample; tie to filing.</t>
         </is>
       </c>
       <c r="P113" s="16" t="inlineStr">
         <is>
-          <t>ภ.พ.30 return + GL-2100 reconciliation tie</t>
-        </is>
-      </c>
-      <c r="Q113" s="18" t="inlineStr">
-        <is>
-          <t>Implemented</t>
+          <t>WHT report</t>
+        </is>
+      </c>
+      <c r="Q113" s="19" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="11" t="inlineStr">
         <is>
-          <t>PAY-01</t>
+          <t>TAX-04</t>
         </is>
       </c>
       <c r="B114" s="12" t="inlineStr">
         <is>
-          <t>Payroll</t>
+          <t>Tax</t>
         </is>
       </c>
       <c r="C114" s="13" t="inlineStr">
@@ -10729,27 +10729,27 @@
       </c>
       <c r="D114" s="12" t="inlineStr">
         <is>
-          <t>Payroll expense/liability</t>
+          <t>Tax (VAT); Tax Payable (2100)</t>
         </is>
       </c>
       <c r="E114" s="12" t="inlineStr">
         <is>
-          <t>Payroll, SSO and PIT mis-computed.</t>
+          <t>Output/input VAT on the filed ภ.พ.30 return does not agree to the GL — VAT liability mis-stated, a filing/penalty exposure, or a posting omission goes undetected before submission.</t>
         </is>
       </c>
       <c r="F114" s="12" t="inlineStr">
         <is>
-          <t>Accuracy</t>
+          <t>Completeness/Accuracy</t>
         </is>
       </c>
       <c r="G114" s="12" t="inlineStr">
         <is>
-          <t>Payroll engine — SSO 5% (cap 750), progressive PIT, payslip net; unit-tested.</t>
+          <t>Periodic VAT-return ↔ GL reconciliation (ภ.พ.30): the monthly return (GET /api/tax-reports/pp30) is built from the sales/output-VAT and purchase/input-VAT sub-reports, computes net VAT = output − input, and RECONCILES it to the **GL account 2100 (Tax Payable) net movement** for the same period (Σ credit − Σ debit over Posted entries) — returning `reconciliation.tied` = true only when the two agree within rounding. A non-tie is a detective finding to investigate and clear BEFORE filing (the form also carries the ม.157 deadline = the 15th of the next month). Output VAT is posted to 2100 on every sale (Cr) and reversed on returns (Dr); input VAT is posted on AP bills (Dr) — so 2100's net is the period's VAT payable. Read-only report; exportable to a ภ.พ.30 PDF/HTML.</t>
         </is>
       </c>
       <c r="H114" s="13" t="inlineStr">
         <is>
-          <t>Auto</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I114" s="13" t="inlineStr">
@@ -10759,37 +10759,37 @@
       </c>
       <c r="J114" s="13" t="inlineStr">
         <is>
-          <t>Per run</t>
+          <t>Monthly / pre-filing</t>
         </is>
       </c>
       <c r="K114" s="12" t="inlineStr">
         <is>
-          <t>HR / Payroll</t>
+          <t>Tax / FinancialController</t>
         </is>
       </c>
       <c r="L114" s="13" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P10/P16</t>
         </is>
       </c>
       <c r="M114" s="12" t="inlineStr">
         <is>
-          <t>payroll/payroll-calc.ts; test/unit.test.ts</t>
+          <t>tax-reports.service.ts pp30 (outputVat/inputVat + 2100 net-movement tie); tax-reports.controller.ts (GET pp30, pp30/export, exec); tax-reports-pdf.ts; dine-in.service.ts/returns.service.ts/finance.service.ts post 2100 on sale/return/AP; /tax/reports UI; cutover/taxdocs.ts (ToE)</t>
         </is>
       </c>
       <c r="N114" s="12" t="inlineStr">
         <is>
-          <t>Inspect calc + tests.</t>
+          <t>Inspect the pp30 build + the 2100 net-movement query + the tie flag + the filing deadline.</t>
         </is>
       </c>
       <c r="O114" s="12" t="inlineStr">
         <is>
-          <t>Re-perform sample payslips.</t>
+          <t>Re-perform: the pp30 return computes net VAT (output − input), the GL 2100 net movement reflects the posted input VAT, and the reconciliation block exposes the gl_account (2100), the report net VAT and a boolean tie verdict (tied iff the two agree within rounding); the ภ.พ.30 export renders (re-performed by the taxdocs harness).</t>
         </is>
       </c>
       <c r="P114" s="12" t="inlineStr">
         <is>
-          <t>Payslip tests</t>
+          <t>ภ.พ.30 return + GL-2100 reconciliation tie</t>
         </is>
       </c>
       <c r="Q114" s="18" t="inlineStr">
@@ -10801,7 +10801,7 @@
     <row r="115">
       <c r="A115" s="15" t="inlineStr">
         <is>
-          <t>PAY-02</t>
+          <t>PAY-01</t>
         </is>
       </c>
       <c r="B115" s="16" t="inlineStr">
@@ -10816,27 +10816,27 @@
       </c>
       <c r="D115" s="16" t="inlineStr">
         <is>
-          <t>Payroll liability</t>
+          <t>Payroll expense/liability</t>
         </is>
       </c>
       <c r="E115" s="16" t="inlineStr">
         <is>
-          <t>Statutory withholdings (SSO/WHT/PF) mis-stated or not remitted, so the liability owed to the authorities diverges from the books.</t>
+          <t>Payroll, SSO and PIT mis-computed.</t>
         </is>
       </c>
       <c r="F115" s="16" t="inlineStr">
         <is>
-          <t>Accuracy/Compliance</t>
+          <t>Accuracy</t>
         </is>
       </c>
       <c r="G115" s="16" t="inlineStr">
         <is>
-          <t>Payroll-liability schedule (GET /api/payroll/liabilities): each statutory account — SSO 2350, WHT/PND1 2360, PF 2370 — shows accrued (GL credits) − remitted (GL debits) = outstanding, tied back to the INDEPENDENT payrun accrual with a `reconciled` flag (a divergence flags a manual JE that touched a payroll-liability account outside the payroll process). Treasury remits the cash (POST .../remit → Dr liability / Cr 1000) which clears the outstanding and keeps the books reconciled to the statutory filings; a remittance beyond the outstanding is blocked (REMIT_EXCEEDS_OUTSTANDING).</t>
+          <t>Payroll engine — SSO 5% (cap 750), progressive PIT, payslip net; unit-tested.</t>
         </is>
       </c>
       <c r="H115" s="17" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Auto</t>
         </is>
       </c>
       <c r="I115" s="17" t="inlineStr">
@@ -10846,12 +10846,12 @@
       </c>
       <c r="J115" s="17" t="inlineStr">
         <is>
-          <t>Per run / monthly</t>
+          <t>Per run</t>
         </is>
       </c>
       <c r="K115" s="16" t="inlineStr">
         <is>
-          <t>HR / Payroll / Treasury</t>
+          <t>HR / Payroll</t>
         </is>
       </c>
       <c r="L115" s="17" t="inlineStr">
@@ -10861,22 +10861,22 @@
       </c>
       <c r="M115" s="16" t="inlineStr">
         <is>
-          <t>payroll/payroll.service.ts liabilities/remitLiability</t>
+          <t>payroll/payroll-calc.ts; test/unit.test.ts</t>
         </is>
       </c>
       <c r="N115" s="16" t="inlineStr">
         <is>
-          <t>Inspect the schedule + the accrued/remitted/outstanding tie-out and the reconciled flag.</t>
+          <t>Inspect calc + tests.</t>
         </is>
       </c>
       <c r="O115" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: run a payroll, confirm the SSO/WHT outstanding equals the payrun accrual; remit part and confirm the outstanding falls and the TB stays balanced; attempt an over-remit (REMIT_EXCEEDS_OUTSTANDING).</t>
+          <t>Re-perform sample payslips.</t>
         </is>
       </c>
       <c r="P115" s="16" t="inlineStr">
         <is>
-          <t>Liability schedule + remittance JEs tied to filings</t>
+          <t>Payslip tests</t>
         </is>
       </c>
       <c r="Q115" s="18" t="inlineStr">
@@ -10888,7 +10888,7 @@
     <row r="116">
       <c r="A116" s="11" t="inlineStr">
         <is>
-          <t>PAY-03</t>
+          <t>PAY-02</t>
         </is>
       </c>
       <c r="B116" s="12" t="inlineStr">
@@ -10903,27 +10903,27 @@
       </c>
       <c r="D116" s="12" t="inlineStr">
         <is>
-          <t>Payroll expense/liability; Cash</t>
+          <t>Payroll liability</t>
         </is>
       </c>
       <c r="E116" s="12" t="inlineStr">
         <is>
-          <t>Payroll run posted to the GL without independent review — the preparer both computes and posts their own payroll (ghost employees, inflated rate/hours).</t>
+          <t>Statutory withholdings (SSO/WHT/PF) mis-stated or not remitted, so the liability owed to the authorities diverges from the books.</t>
         </is>
       </c>
       <c r="F116" s="12" t="inlineStr">
         <is>
-          <t>Authorization</t>
+          <t>Accuracy/Compliance</t>
         </is>
       </c>
       <c r="G116" s="12" t="inlineStr">
         <is>
-          <t>Payroll maker-checker (SoD): a run posts its GL entry as a DRAFT (excluded from balances) with the run record 'PendingApproval'; a DIFFERENT user must approve before it becomes effective (approver ≠ preparer enforced regardless of permissions, reusing the GL-05 ledger approval). Reject voids the draft; idempotent per (tenant, period).</t>
+          <t>Payroll-liability schedule (GET /api/payroll/liabilities): each statutory account — SSO 2350, WHT/PND1 2360, PF 2370 — shows accrued (GL credits) − remitted (GL debits) = outstanding, tied back to the INDEPENDENT payrun accrual with a `reconciled` flag (a divergence flags a manual JE that touched a payroll-liability account outside the payroll process). Treasury remits the cash (POST .../remit → Dr liability / Cr 1000) which clears the outstanding and keeps the books reconciled to the statutory filings; a remittance beyond the outstanding is blocked (REMIT_EXCEEDS_OUTSTANDING).</t>
         </is>
       </c>
       <c r="H116" s="13" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I116" s="13" t="inlineStr">
@@ -10933,12 +10933,12 @@
       </c>
       <c r="J116" s="13" t="inlineStr">
         <is>
-          <t>Per run</t>
+          <t>Per run / monthly</t>
         </is>
       </c>
       <c r="K116" s="12" t="inlineStr">
         <is>
-          <t>HR / Payroll; Controller</t>
+          <t>HR / Payroll / Treasury</t>
         </is>
       </c>
       <c r="L116" s="13" t="inlineStr">
@@ -10948,22 +10948,22 @@
       </c>
       <c r="M116" s="12" t="inlineStr">
         <is>
-          <t>payroll/payroll.service.ts approvePayroll/rejectPayroll; migration 0133</t>
+          <t>payroll/payroll.service.ts liabilities/remitLiability</t>
         </is>
       </c>
       <c r="N116" s="12" t="inlineStr">
         <is>
-          <t>Inspect Draft→approve flow + the approver≠preparer check.</t>
+          <t>Inspect the schedule + the accrued/remitted/outstanding tie-out and the reconciled flag.</t>
         </is>
       </c>
       <c r="O116" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: run as A, attempt self-approve (SOD_VIOLATION), approve as B; confirm the JE hits balances only after approval.</t>
+          <t>Re-perform: run a payroll, confirm the SSO/WHT outstanding equals the payrun accrual; remit part and confirm the outstanding falls and the TB stays balanced; attempt an over-remit (REMIT_EXCEEDS_OUTSTANDING).</t>
         </is>
       </c>
       <c r="P116" s="12" t="inlineStr">
         <is>
-          <t>Approval log + SoD test</t>
+          <t>Liability schedule + remittance JEs tied to filings</t>
         </is>
       </c>
       <c r="Q116" s="18" t="inlineStr">
@@ -10975,12 +10975,12 @@
     <row r="117">
       <c r="A117" s="15" t="inlineStr">
         <is>
-          <t>FA-09</t>
+          <t>PAY-03</t>
         </is>
       </c>
       <c r="B117" s="16" t="inlineStr">
         <is>
-          <t>Fixed Assets</t>
+          <t>Payroll</t>
         </is>
       </c>
       <c r="C117" s="17" t="inlineStr">
@@ -10990,12 +10990,12 @@
       </c>
       <c r="D117" s="16" t="inlineStr">
         <is>
-          <t>Property, Plant &amp; Equipment; Cash</t>
+          <t>Payroll expense/liability; Cash</t>
         </is>
       </c>
       <c r="E117" s="16" t="inlineStr">
         <is>
-          <t>Asset disposed without independent review — one person writes an asset off the books and records the proceeds (asset-stripping / theft: dispose a still-held asset, or to a related party below value).</t>
+          <t>Payroll run posted to the GL without independent review — the preparer both computes and posts their own payroll (ghost employees, inflated rate/hours).</t>
         </is>
       </c>
       <c r="F117" s="16" t="inlineStr">
@@ -11005,7 +11005,7 @@
       </c>
       <c r="G117" s="16" t="inlineStr">
         <is>
-          <t>Asset-disposal maker-checker (SoD): a disposal REQUEST posts its GL entry as a DRAFT (excluded from balances) and flags the asset disposal_pending WITHOUT marking it disposed or moving the register; a DIFFERENT user must approve before it is effective (status→disposed, revaluation surplus recycled 3200→3100) (approver ≠ requester enforced regardless of permissions, reusing the GL-05 ledger approval). Reject voids the draft and the asset stays in service; only one disposal may be pending per asset; a disposal-pending asset is frozen from depreciation.</t>
+          <t>Payroll maker-checker (SoD): a run posts its GL entry as a DRAFT (excluded from balances) with the run record 'PendingApproval'; a DIFFERENT user must approve before it becomes effective (approver ≠ preparer enforced regardless of permissions, reusing the GL-05 ledger approval). Reject voids the draft; idempotent per (tenant, period).</t>
         </is>
       </c>
       <c r="H117" s="17" t="inlineStr">
@@ -11020,12 +11020,12 @@
       </c>
       <c r="J117" s="17" t="inlineStr">
         <is>
-          <t>Per disposal</t>
+          <t>Per run</t>
         </is>
       </c>
       <c r="K117" s="16" t="inlineStr">
         <is>
-          <t>FaAccountant / Controller</t>
+          <t>HR / Payroll; Controller</t>
         </is>
       </c>
       <c r="L117" s="17" t="inlineStr">
@@ -11035,22 +11035,22 @@
       </c>
       <c r="M117" s="16" t="inlineStr">
         <is>
-          <t>assets.service.ts dispose(pendingApproval Draft)/approveDisposal/rejectDisposal; assets.controller.ts (:assetNo/dispose/approve|reject); schema/assets.ts fixed_assets.disposal_pending + migration 0135; cutover/basics.ts + worldclass.ts + compliance.ts (ToE)</t>
+          <t>payroll/payroll.service.ts approvePayroll/rejectPayroll; migration 0133</t>
         </is>
       </c>
       <c r="N117" s="16" t="inlineStr">
         <is>
-          <t>Inspect Draft→approve flow + the approver≠requester check + deferred status/recycle.</t>
+          <t>Inspect Draft→approve flow + the approver≠preparer check.</t>
         </is>
       </c>
       <c r="O117" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: request a disposal (Draft JE excluded), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm status→disposed + surplus recycled only after approval (re-performed by the harnesses).</t>
+          <t>Re-perform: run as A, attempt self-approve (SOD_VIOLATION), approve as B; confirm the JE hits balances only after approval.</t>
         </is>
       </c>
       <c r="P117" s="16" t="inlineStr">
         <is>
-          <t>Disposal approval log + SoD test</t>
+          <t>Approval log + SoD test</t>
         </is>
       </c>
       <c r="Q117" s="18" t="inlineStr">
@@ -11062,7 +11062,7 @@
     <row r="118">
       <c r="A118" s="11" t="inlineStr">
         <is>
-          <t>FA-10</t>
+          <t>FA-09</t>
         </is>
       </c>
       <c r="B118" s="12" t="inlineStr">
@@ -11077,22 +11077,22 @@
       </c>
       <c r="D118" s="12" t="inlineStr">
         <is>
-          <t>Property, Plant &amp; Equipment; Accounts Payable</t>
+          <t>Property, Plant &amp; Equipment; Cash</t>
         </is>
       </c>
       <c r="E118" s="12" t="inlineStr">
         <is>
-          <t>Capital purchases mis-capitalised or capitalised without independent review — the person who receives the goods also decides what enters the asset register and at what cost/useful life (fictitious or over-valued assets; capex/opex mis-classification).</t>
+          <t>Asset disposed without independent review — one person writes an asset off the books and records the proceeds (asset-stripping / theft: dispose a still-held asset, or to a related party below value).</t>
         </is>
       </c>
       <c r="F118" s="12" t="inlineStr">
         <is>
-          <t>Authorization; Accuracy</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="G118" s="12" t="inlineStr">
         <is>
-          <t>Procure-to-Capitalize maker-checker (SoD): a goods-receipt line flagged capital (item-master is_fixed_asset or per-PO-line override) is excluded from inventory capitalisation (1200) at receipt and instead becomes ELIGIBLE for the asset register. Capitalisation is a REQUEST that posts NOTHING to the GL; a DIFFERENT user must approve before the fixed_assets row + acquisition JE (Dr 1500 / Cr 2000) are created (approver ≠ requester enforced regardless of permissions). The created asset carries its source GR/PO for end-to-end PR→PO→GR→FA traceability; a GR line cannot be capitalised twice.</t>
+          <t>Asset-disposal maker-checker (SoD): a disposal REQUEST posts its GL entry as a DRAFT (excluded from balances) and flags the asset disposal_pending WITHOUT marking it disposed or moving the register; a DIFFERENT user must approve before it is effective (status→disposed, revaluation surplus recycled 3200→3100) (approver ≠ requester enforced regardless of permissions, reusing the GL-05 ledger approval). Reject voids the draft and the asset stays in service; only one disposal may be pending per asset; a disposal-pending asset is frozen from depreciation.</t>
         </is>
       </c>
       <c r="H118" s="13" t="inlineStr">
@@ -11107,7 +11107,7 @@
       </c>
       <c r="J118" s="13" t="inlineStr">
         <is>
-          <t>Per capital receipt</t>
+          <t>Per disposal</t>
         </is>
       </c>
       <c r="K118" s="12" t="inlineStr">
@@ -11122,22 +11122,22 @@
       </c>
       <c r="M118" s="12" t="inlineStr">
         <is>
-          <t>assets.service.ts registerFromGr/approveRegistration/rejectRegistration/eligibleFromGr; assets.controller.ts (registrations*); procurement.service.ts createGr (is_capital routing, costing excluded); schema/assets.ts asset_registration_requests + fixed_assets.source_gr_no/po_no + migration 0137; cutover/basics.ts + compliance.ts (ToE)</t>
+          <t>assets.service.ts dispose(pendingApproval Draft)/approveDisposal/rejectDisposal; assets.controller.ts (:assetNo/dispose/approve|reject); schema/assets.ts fixed_assets.disposal_pending + migration 0135; cutover/basics.ts + worldclass.ts + compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N118" s="12" t="inlineStr">
         <is>
-          <t>Inspect the eligible→request→approve flow + approver≠requester check + the inventory-vs-asset routing of capital lines.</t>
+          <t>Inspect Draft→approve flow + the approver≠requester check + deferred status/recycle.</t>
         </is>
       </c>
       <c r="O118" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: receive a capital line, raise a registration (no GL), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm the asset + Dr 1500/Cr 2000 post only after approval and the line cannot be re-registered (re-performed by the harnesses).</t>
+          <t>Re-perform: request a disposal (Draft JE excluded), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm status→disposed + surplus recycled only after approval (re-performed by the harnesses).</t>
         </is>
       </c>
       <c r="P118" s="12" t="inlineStr">
         <is>
-          <t>Capitalization approval log + SoD test</t>
+          <t>Disposal approval log + SoD test</t>
         </is>
       </c>
       <c r="Q118" s="18" t="inlineStr">
@@ -11149,12 +11149,12 @@
     <row r="119">
       <c r="A119" s="15" t="inlineStr">
         <is>
-          <t>CON-01</t>
+          <t>FA-10</t>
         </is>
       </c>
       <c r="B119" s="16" t="inlineStr">
         <is>
-          <t>Consolidation &amp; FX</t>
+          <t>Fixed Assets</t>
         </is>
       </c>
       <c r="C119" s="17" t="inlineStr">
@@ -11164,42 +11164,42 @@
       </c>
       <c r="D119" s="16" t="inlineStr">
         <is>
-          <t>Consolidation</t>
+          <t>Property, Plant &amp; Equipment; Accounts Payable</t>
         </is>
       </c>
       <c r="E119" s="16" t="inlineStr">
         <is>
-          <t>Group consolidation mis-stated (ownership/currency).</t>
+          <t>Capital purchases mis-capitalised or capitalised without independent review — the person who receives the goods also decides what enters the asset register and at what cost/useful life (fictitious or over-valued assets; capex/opex mis-classification).</t>
         </is>
       </c>
       <c r="F119" s="16" t="inlineStr">
         <is>
-          <t>Accuracy</t>
+          <t>Authorization; Accuracy</t>
         </is>
       </c>
       <c r="G119" s="16" t="inlineStr">
         <is>
-          <t>Consolidation run (ownership %, entity currency) gated by 'approvals'.</t>
+          <t>Procure-to-Capitalize maker-checker (SoD): a goods-receipt line flagged capital (item-master is_fixed_asset or per-PO-line override) is excluded from inventory capitalisation (1200) at receipt and instead becomes ELIGIBLE for the asset register. Capitalisation is a REQUEST that posts NOTHING to the GL; a DIFFERENT user must approve before the fixed_assets row + acquisition JE (Dr 1500 / Cr 2000) are created (approver ≠ requester enforced regardless of permissions). The created asset carries its source GR/PO for end-to-end PR→PO→GR→FA traceability; a GR line cannot be capitalised twice.</t>
         </is>
       </c>
       <c r="H119" s="17" t="inlineStr">
         <is>
-          <t>Auto+Manual</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I119" s="17" t="inlineStr">
         <is>
-          <t>Period</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J119" s="17" t="inlineStr">
         <is>
-          <t>Period</t>
+          <t>Per capital receipt</t>
         </is>
       </c>
       <c r="K119" s="16" t="inlineStr">
         <is>
-          <t>Group Controller</t>
+          <t>FaAccountant / Controller</t>
         </is>
       </c>
       <c r="L119" s="17" t="inlineStr">
@@ -11209,22 +11209,22 @@
       </c>
       <c r="M119" s="16" t="inlineStr">
         <is>
-          <t>consolidation.service.ts (runConsolidation @Permissions approvals)</t>
+          <t>assets.service.ts registerFromGr/approveRegistration/rejectRegistration/eligibleFromGr; assets.controller.ts (registrations*); procurement.service.ts createGr (is_capital routing, costing excluded); schema/assets.ts asset_registration_requests + fixed_assets.source_gr_no/po_no + migration 0137; cutover/basics.ts + compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N119" s="16" t="inlineStr">
         <is>
-          <t>Inspect consolidation logic + gate.</t>
+          <t>Inspect the eligible→request→approve flow + approver≠requester check + the inventory-vs-asset routing of capital lines.</t>
         </is>
       </c>
       <c r="O119" s="16" t="inlineStr">
         <is>
-          <t>Sample period: consolidated TB ties to entities.</t>
+          <t>Re-perform: receive a capital line, raise a registration (no GL), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm the asset + Dr 1500/Cr 2000 post only after approval and the line cannot be re-registered (re-performed by the harnesses).</t>
         </is>
       </c>
       <c r="P119" s="16" t="inlineStr">
         <is>
-          <t>Consol TB</t>
+          <t>Capitalization approval log + SoD test</t>
         </is>
       </c>
       <c r="Q119" s="18" t="inlineStr">
@@ -11236,7 +11236,7 @@
     <row r="120">
       <c r="A120" s="11" t="inlineStr">
         <is>
-          <t>CON-02</t>
+          <t>CON-01</t>
         </is>
       </c>
       <c r="B120" s="12" t="inlineStr">
@@ -11251,22 +11251,22 @@
       </c>
       <c r="D120" s="12" t="inlineStr">
         <is>
-          <t>FX gain/loss</t>
+          <t>Consolidation</t>
         </is>
       </c>
       <c r="E120" s="12" t="inlineStr">
         <is>
-          <t>FX exposures not revalued at period-end.</t>
+          <t>Group consolidation mis-stated (ownership/currency).</t>
         </is>
       </c>
       <c r="F120" s="12" t="inlineStr">
         <is>
-          <t>Valuation</t>
+          <t>Accuracy</t>
         </is>
       </c>
       <c r="G120" s="12" t="inlineStr">
         <is>
-          <t>FX revaluation at period-end rates; unrealized FX posted (acct 5400).</t>
+          <t>Consolidation run (ownership %, entity currency) gated by 'approvals'.</t>
         </is>
       </c>
       <c r="H120" s="13" t="inlineStr">
@@ -11276,7 +11276,7 @@
       </c>
       <c r="I120" s="13" t="inlineStr">
         <is>
-          <t>Period-end</t>
+          <t>Period</t>
         </is>
       </c>
       <c r="J120" s="13" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="K120" s="12" t="inlineStr">
         <is>
-          <t>Controller</t>
+          <t>Group Controller</t>
         </is>
       </c>
       <c r="L120" s="13" t="inlineStr">
@@ -11296,22 +11296,22 @@
       </c>
       <c r="M120" s="12" t="inlineStr">
         <is>
-          <t>fx.service.ts (revalue / unrealized report)</t>
+          <t>consolidation.service.ts (runConsolidation @Permissions approvals)</t>
         </is>
       </c>
       <c r="N120" s="12" t="inlineStr">
         <is>
-          <t>Inspect reval logic + rates.</t>
+          <t>Inspect consolidation logic + gate.</t>
         </is>
       </c>
       <c r="O120" s="12" t="inlineStr">
         <is>
-          <t>Recompute reval on sample balances.</t>
+          <t>Sample period: consolidated TB ties to entities.</t>
         </is>
       </c>
       <c r="P120" s="12" t="inlineStr">
         <is>
-          <t>FX reval JE</t>
+          <t>Consol TB</t>
         </is>
       </c>
       <c r="Q120" s="18" t="inlineStr">
@@ -11323,7 +11323,7 @@
     <row r="121">
       <c r="A121" s="15" t="inlineStr">
         <is>
-          <t>FX-04</t>
+          <t>CON-02</t>
         </is>
       </c>
       <c r="B121" s="16" t="inlineStr">
@@ -11338,42 +11338,42 @@
       </c>
       <c r="D121" s="16" t="inlineStr">
         <is>
-          <t>FX gain/loss; Revenue; AR/AP</t>
+          <t>FX gain/loss</t>
         </is>
       </c>
       <c r="E121" s="16" t="inlineStr">
         <is>
-          <t>A wrong manually-entered FX rate (fat-fingered, e.g. USD 36 keyed as 63) flows straight into a period-end revaluation JE and the unrealized-FX report with no independent review — mis-stating earnings/equity and FX-translated balances.</t>
+          <t>FX exposures not revalued at period-end.</t>
         </is>
       </c>
       <c r="F121" s="16" t="inlineStr">
         <is>
-          <t>Accuracy/Valuation</t>
+          <t>Valuation</t>
         </is>
       </c>
       <c r="G121" s="16" t="inlineStr">
         <is>
-          <t>FX rate maker-checker (SoD): a MANUALLY-entered rate lands as PendingApproval and is EXCLUDED from rate resolution — revaluation, the unrealized-FX report, and consolidation translation all use APPROVED rates only — until a DIFFERENT user approves it (POST /api/fx/rates/approve). Self-approval → SOD_VIOLATION (binds even Admin); reject marks the rate Rejected (never usable); re-entering a rate sends it back to PendingApproval. Externally-sourced (feed) rates carrying an explicit non-manual source are auto-approved. Pending rates are also surfaced, aged, by the pending-approvals monitor (GOV-01).</t>
+          <t>FX revaluation at period-end rates; unrealized FX posted (acct 5400).</t>
         </is>
       </c>
       <c r="H121" s="17" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="I121" s="17" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Period-end</t>
         </is>
       </c>
       <c r="J121" s="17" t="inlineStr">
         <is>
-          <t>Per rate</t>
+          <t>Period</t>
         </is>
       </c>
       <c r="K121" s="16" t="inlineStr">
         <is>
-          <t>Controller / Treasury</t>
+          <t>Controller</t>
         </is>
       </c>
       <c r="L121" s="17" t="inlineStr">
@@ -11383,22 +11383,22 @@
       </c>
       <c r="M121" s="16" t="inlineStr">
         <is>
-          <t>fx.service.ts setRate(manual→PendingApproval)/approveRate/rejectRate/rateAsOf(Approved only); fx.controller.ts (rates/approve|reject|pending gated approvals/gl_close); consolidation.service.ts (translation reads Approved rates); schema/fx.ts fx_rates.status + migration 0141; cutover/fxreval.ts (ToE)</t>
+          <t>fx.service.ts (revalue / unrealized report)</t>
         </is>
       </c>
       <c r="N121" s="16" t="inlineStr">
         <is>
-          <t>Inspect the request→approve flow + the approver≠requester check + that revaluation/reporting resolve Approved rates only.</t>
+          <t>Inspect reval logic + rates.</t>
         </is>
       </c>
       <c r="O121" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: enter a manual rate (PendingApproval), confirm revalue is blocked NO_RATE while pending, attempt self-approve (SOD_VIOLATION), approve as a different user, then revalue succeeds (re-performed by the fxreval harness).</t>
+          <t>Recompute reval on sample balances.</t>
         </is>
       </c>
       <c r="P121" s="16" t="inlineStr">
         <is>
-          <t>FX rate approval log + SoD test</t>
+          <t>FX reval JE</t>
         </is>
       </c>
       <c r="Q121" s="18" t="inlineStr">
@@ -11410,92 +11410,179 @@
     <row r="122">
       <c r="A122" s="11" t="inlineStr">
         <is>
+          <t>FX-04</t>
+        </is>
+      </c>
+      <c r="B122" s="12" t="inlineStr">
+        <is>
+          <t>Consolidation &amp; FX</t>
+        </is>
+      </c>
+      <c r="C122" s="13" t="inlineStr">
+        <is>
+          <t>Application</t>
+        </is>
+      </c>
+      <c r="D122" s="12" t="inlineStr">
+        <is>
+          <t>FX gain/loss; Revenue; AR/AP</t>
+        </is>
+      </c>
+      <c r="E122" s="12" t="inlineStr">
+        <is>
+          <t>A wrong manually-entered FX rate (fat-fingered, e.g. USD 36 keyed as 63) flows straight into a period-end revaluation JE and the unrealized-FX report with no independent review — mis-stating earnings/equity and FX-translated balances.</t>
+        </is>
+      </c>
+      <c r="F122" s="12" t="inlineStr">
+        <is>
+          <t>Accuracy/Valuation</t>
+        </is>
+      </c>
+      <c r="G122" s="12" t="inlineStr">
+        <is>
+          <t>FX rate maker-checker (SoD): a MANUALLY-entered rate lands as PendingApproval and is EXCLUDED from rate resolution — revaluation, the unrealized-FX report, and consolidation translation all use APPROVED rates only — until a DIFFERENT user approves it (POST /api/fx/rates/approve). Self-approval → SOD_VIOLATION (binds even Admin); reject marks the rate Rejected (never usable); re-entering a rate sends it back to PendingApproval. Externally-sourced (feed) rates carrying an explicit non-manual source are auto-approved. Pending rates are also surfaced, aged, by the pending-approvals monitor (GOV-01).</t>
+        </is>
+      </c>
+      <c r="H122" s="13" t="inlineStr">
+        <is>
+          <t>Prev</t>
+        </is>
+      </c>
+      <c r="I122" s="13" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="J122" s="13" t="inlineStr">
+        <is>
+          <t>Per rate</t>
+        </is>
+      </c>
+      <c r="K122" s="12" t="inlineStr">
+        <is>
+          <t>Controller / Treasury</t>
+        </is>
+      </c>
+      <c r="L122" s="13" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="M122" s="12" t="inlineStr">
+        <is>
+          <t>fx.service.ts setRate(manual→PendingApproval)/approveRate/rejectRate/rateAsOf(Approved only); fx.controller.ts (rates/approve|reject|pending gated approvals/gl_close); consolidation.service.ts (translation reads Approved rates); schema/fx.ts fx_rates.status + migration 0141; cutover/fxreval.ts (ToE)</t>
+        </is>
+      </c>
+      <c r="N122" s="12" t="inlineStr">
+        <is>
+          <t>Inspect the request→approve flow + the approver≠requester check + that revaluation/reporting resolve Approved rates only.</t>
+        </is>
+      </c>
+      <c r="O122" s="12" t="inlineStr">
+        <is>
+          <t>Re-perform: enter a manual rate (PendingApproval), confirm revalue is blocked NO_RATE while pending, attempt self-approve (SOD_VIOLATION), approve as a different user, then revalue succeeds (re-performed by the fxreval harness).</t>
+        </is>
+      </c>
+      <c r="P122" s="12" t="inlineStr">
+        <is>
+          <t>FX rate approval log + SoD test</t>
+        </is>
+      </c>
+      <c r="Q122" s="18" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="15" t="inlineStr">
+        <is>
           <t>BUD-01</t>
         </is>
       </c>
-      <c r="B122" s="12" t="inlineStr">
+      <c r="B123" s="16" t="inlineStr">
         <is>
           <t>Budgeting &amp; Planning</t>
         </is>
       </c>
-      <c r="C122" s="13" t="inlineStr">
+      <c r="C123" s="17" t="inlineStr">
         <is>
           <t>Application</t>
         </is>
       </c>
-      <c r="D122" s="12" t="inlineStr">
+      <c r="D123" s="16" t="inlineStr">
         <is>
           <t>Budget; All (variance reporting)</t>
         </is>
       </c>
-      <c r="E122" s="12" t="inlineStr">
+      <c r="E123" s="16" t="inlineStr">
         <is>
           <t>A budget figure is entered/changed by one person and immediately drives the budget-vs-actual variance report — the basis for spend authorization and performance review — with no independent approval; a wrong or self-serving budget makes overspending look 'on budget'.</t>
         </is>
       </c>
-      <c r="F122" s="12" t="inlineStr">
+      <c r="F123" s="16" t="inlineStr">
         <is>
           <t>Authorization/Accuracy</t>
         </is>
       </c>
-      <c r="G122" s="12" t="inlineStr">
+      <c r="G123" s="16" t="inlineStr">
         <is>
           <t>Budget maker-checker (SoD): an upserted budget (POST /api/ledger/budgets) lands as PendingApproval and is EXCLUDED from budget-vs-actual until a DIFFERENT user approves it (POST /api/ledger/budgets/approve for the fiscal_year/account/cost-centre[/period]). Self-approval → SOD_VIOLATION (binds even Admin); reject marks it Rejected (excluded). DEFAULT 'Approved' keeps existing rows + direct planning seeds usable. Pending budgets are also surfaced, aged, by the pending-approvals monitor (GOV-01).</t>
         </is>
       </c>
-      <c r="H122" s="13" t="inlineStr">
+      <c r="H123" s="17" t="inlineStr">
         <is>
           <t>Prev</t>
         </is>
       </c>
-      <c r="I122" s="13" t="inlineStr">
+      <c r="I123" s="17" t="inlineStr">
         <is>
           <t>Automated</t>
         </is>
       </c>
-      <c r="J122" s="13" t="inlineStr">
+      <c r="J123" s="17" t="inlineStr">
         <is>
           <t>Per budget</t>
         </is>
       </c>
-      <c r="K122" s="12" t="inlineStr">
+      <c r="K123" s="16" t="inlineStr">
         <is>
           <t>Controller / FP&amp;A</t>
         </is>
       </c>
-      <c r="L122" s="13" t="inlineStr">
+      <c r="L123" s="17" t="inlineStr">
         <is>
           <t>P10</t>
         </is>
       </c>
-      <c r="M122" s="12" t="inlineStr">
+      <c r="M123" s="16" t="inlineStr">
         <is>
           <t>budget.service.ts upsertBudget(→PendingApproval)/approveBudget/rejectBudget/budgetVsActual(Approved only); budget.controller.ts (budgets/approve|reject|pending gated approvals/gl_close); schema/budgets.ts budgets.status + migration 0142; cutover/budget.ts (ToE)</t>
         </is>
       </c>
-      <c r="N122" s="12" t="inlineStr">
+      <c r="N123" s="16" t="inlineStr">
         <is>
           <t>Inspect the request→approve flow + the approver≠requester check + that budget-vs-actual counts Approved budgets only.</t>
         </is>
       </c>
-      <c r="O122" s="12" t="inlineStr">
+      <c r="O123" s="16" t="inlineStr">
         <is>
           <t>Re-perform: upsert a budget (PendingApproval, excluded from variance), attempt self-approve (SOD_VIOLATION), approve as a different user, confirm it then appears in budget-vs-actual (re-performed by the budget harness).</t>
         </is>
       </c>
-      <c r="P122" s="12" t="inlineStr">
+      <c r="P123" s="16" t="inlineStr">
         <is>
           <t>Budget approval log + SoD test</t>
         </is>
       </c>
-      <c r="Q122" s="18" t="inlineStr">
+      <c r="Q123" s="18" t="inlineStr">
         <is>
           <t>Implemented</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q122"/>
+  <autoFilter ref="A1:Q123"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -12678,7 +12765,7 @@
         </is>
       </c>
       <c r="C5" s="29">
-        <f>COUNTIF(RCM!$Q$2:$Q$122,B5)</f>
+        <f>COUNTIF(RCM!$Q$2:$Q$123,B5)</f>
         <v/>
       </c>
     </row>
@@ -12689,7 +12776,7 @@
         </is>
       </c>
       <c r="C6" s="29">
-        <f>COUNTIF(RCM!$Q$2:$Q$122,B6)</f>
+        <f>COUNTIF(RCM!$Q$2:$Q$123,B6)</f>
         <v/>
       </c>
     </row>
@@ -12700,7 +12787,7 @@
         </is>
       </c>
       <c r="C7" s="29">
-        <f>COUNTIF(RCM!$Q$2:$Q$122,B7)</f>
+        <f>COUNTIF(RCM!$Q$2:$Q$123,B7)</f>
         <v/>
       </c>
     </row>
@@ -12711,7 +12798,7 @@
         </is>
       </c>
       <c r="C8" s="32">
-        <f>COUNTA(RCM!$A$2:$A$122)</f>
+        <f>COUNTA(RCM!$A$2:$A$123)</f>
         <v/>
       </c>
     </row>
@@ -12729,7 +12816,7 @@
         </is>
       </c>
       <c r="C11" s="29">
-        <f>COUNTIF(RCM!$C$2:$C$122,B11)</f>
+        <f>COUNTIF(RCM!$C$2:$C$123,B11)</f>
         <v/>
       </c>
     </row>
@@ -12740,7 +12827,7 @@
         </is>
       </c>
       <c r="C12" s="29">
-        <f>COUNTIF(RCM!$C$2:$C$122,B12)</f>
+        <f>COUNTIF(RCM!$C$2:$C$123,B12)</f>
         <v/>
       </c>
     </row>
@@ -12751,7 +12838,7 @@
         </is>
       </c>
       <c r="C13" s="29">
-        <f>COUNTIF(RCM!$C$2:$C$122,B13)</f>
+        <f>COUNTIF(RCM!$C$2:$C$123,B13)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(gl): WS2.2 — GL immutability + audit log + reversal (GL-17)
- posted_at/reversal_of/is_reversed on journal_entries; gl_audit_log
  table (migration 0164) + RLS
- DB trigger gl_block_posted_mutation blocks UPDATE/DELETE of Posted
  entries (PGlite executes it too); app-level attemptVoidPosted guard
  records MUTATE_BLOCKED for testable enforcement
- reverseEntry: swapped-Dr/Cr contra entry, carries dimensions, flags
  original is_reversed, routes through posting path (period gates apply);
  errors ENTRY_NOT_FOUND/NOT_POSTED/ALREADY_REVERSED
- postEntry/approve stamp posted_at + write POST/APPROVE audit rows
- basics 179/179, worldclass 57/57, compliance 106 green
- GL-17 RCM (122); narrative §2.2 + user-manual + UAT TC-GL-17

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/compliance/Oshinei_ERP_SOX_RCM_v1.xlsx
+++ b/compliance/Oshinei_ERP_SOX_RCM_v1.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'RCM'!$A$1:$Q$122</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'RCM'!$A$1:$Q$123</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Gap Remediation'!$A$2:$H$18</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -858,7 +858,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q122"/>
+  <dimension ref="A1:Q123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -9322,12 +9322,12 @@
     <row r="98">
       <c r="A98" s="11" t="inlineStr">
         <is>
-          <t>EXP-07</t>
+          <t>GL-17</t>
         </is>
       </c>
       <c r="B98" s="12" t="inlineStr">
         <is>
-          <t>Expenditure</t>
+          <t>General Ledger</t>
         </is>
       </c>
       <c r="C98" s="13" t="inlineStr">
@@ -9337,27 +9337,27 @@
       </c>
       <c r="D98" s="12" t="inlineStr">
         <is>
-          <t>Cash; Operating expense</t>
+          <t>All</t>
         </is>
       </c>
       <c r="E98" s="12" t="inlineStr">
         <is>
-          <t>Petty-cash / employee advance issued but never accounted for — cash leakage, expense unrecorded.</t>
+          <t>A posted journal entry is edited or deleted after the fact — restating history with no trail — instead of being corrected by a transparent reversal; or a correction is made with no record of who/what/why. The general ledger is no longer an immutable, auditable record of record.</t>
         </is>
       </c>
       <c r="F98" s="12" t="inlineStr">
         <is>
-          <t>Existence/Completeness</t>
+          <t>Completeness/Accuracy/Authorization</t>
         </is>
       </c>
       <c r="G98" s="12" t="inlineStr">
         <is>
-          <t>Employee cash advances: issuing an advance debits the 1180 Employee Advances control (Dr 1180 / Cr 1000); settlement clears it against actual spend + returned cash (Dr expense + Dr 1000 / Cr 1180), enforced to reconcile (settled_expense + returned_cash must equal the advance → SETTLE_MISMATCH). The 1180 balance is the outstanding float subject to review.</t>
+          <t>Posted-entry immutability + reversal-only correction + GL audit trail: a journal entry that has reached Posted status is IMMUTABLE — it can never be edited or deleted. Enforcement is twofold: (1) a production DB trigger (gl_block_posted_mutation) that RAISES on any UPDATE/DELETE of a Posted journal_entries row (permitting only the is_reversed bookkeeping flag flip), and (2) an application-level guard (attemptVoidPosted → GL_IMMUTABLE) that refuses and records any mutation attempt. The ONLY way to correct a posted entry is a REVERSAL: reverseEntry posts a NEW, immediately-Posted contra entry that swaps every line's debit/credit (so original + reversal net to zero on every affected account), dimensions carried over, linked via reversal_of, and flags the original is_reversed. A reversal goes through the normal posting path so the period gates (PERIOD_LOCKED/PERIOD_CLOSED) still apply; only Posted entries can be reversed (NOT_POSTED) and only once (ALREADY_REVERSED). Every POST, APPROVE, REVERSE and blocked mutation (MUTATE_BLOCKED) is recorded with actor + detail + timestamp in gl_audit_log (tenant-scoped, RLS).</t>
         </is>
       </c>
       <c r="H98" s="13" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I98" s="13" t="inlineStr">
@@ -9367,12 +9367,12 @@
       </c>
       <c r="J98" s="13" t="inlineStr">
         <is>
-          <t>Per advance</t>
+          <t>Per entry / continuous</t>
         </is>
       </c>
       <c r="K98" s="12" t="inlineStr">
         <is>
-          <t>AP / Controller</t>
+          <t>Financial Controller</t>
         </is>
       </c>
       <c r="L98" s="13" t="inlineStr">
@@ -9382,22 +9382,22 @@
       </c>
       <c r="M98" s="12" t="inlineStr">
         <is>
-          <t>finance.service.ts (issueAdvance, settleAdvance reconcile-or-reject, listAdvances outstanding); finance.controller.ts (creditors/exec); schema/finance.ts (employee_advances) + migration 0120; cutover/basics.ts (ToE)</t>
+          <t>ledger.service.ts (postEntry stamps posted_at + logs POST; approveEntry stamps posted_at + logs APPROVE; reverseEntry contra-posting with ENTRY_NOT_FOUND/NOT_POSTED/ALREADY_REVERSED + REVERSE log; attemptVoidPosted GL_IMMUTABLE + MUTATE_BLOCKED log; listGlAudit); ledger.controller.ts (gl_post journal/:id/reverse + journal/:id/attempt-void, gl_post/gl_close/exec audit read); schema/ledger.ts (journal_entries posted_at/reversal_of/is_reversed); schema/gl-audit.ts (gl_audit_log table); migration 0164 (columns + gl_audit_log + RLS + gl_block_posted_mutation trigger); ledger.module.ts (LedgerService owns it); cutover/basics.ts (GL-17 ToE)</t>
         </is>
       </c>
       <c r="N98" s="12" t="inlineStr">
         <is>
-          <t>Inspect issue/settle GL + settlement reconciliation guard.</t>
+          <t>Inspect the DB immutability trigger + the app GL_IMMUTABLE guard + the reversal contra-posting (swapped Dr/Cr, reversal_of, is_reversed) + the gl_audit_log trail (POST/APPROVE/REVERSE/MUTATE_BLOCKED).</t>
         </is>
       </c>
       <c r="O98" s="12" t="inlineStr">
         <is>
-          <t>Issue an advance (1180 up); settle 700+300 clears 1180; mismatched settle → SETTLE_MISMATCH (re-performed by the harness).</t>
+          <t>TC-GL-17-01: attempt to void a posted entry → GL_IMMUTABLE (400) + MUTATE_BLOCKED audit row; TC-GL-17-02: reverse a posted entry → contra entry nets to zero, original is_reversed + REVERSE audit row; TC-GL-17-03: reverse again → ALREADY_REVERSED (400) (re-performed by the basics.ts harness).</t>
         </is>
       </c>
       <c r="P98" s="12" t="inlineStr">
         <is>
-          <t>Advance register; outstanding float</t>
+          <t>gl_audit_log trail (POST/APPROVE/REVERSE/MUTATE_BLOCKED); reversal entries with reversal_of linkage; posted-entry immutability</t>
         </is>
       </c>
       <c r="Q98" s="18" t="inlineStr">
@@ -9409,7 +9409,7 @@
     <row r="99">
       <c r="A99" s="15" t="inlineStr">
         <is>
-          <t>EXP-08</t>
+          <t>EXP-07</t>
         </is>
       </c>
       <c r="B99" s="16" t="inlineStr">
@@ -9429,22 +9429,22 @@
       </c>
       <c r="E99" s="16" t="inlineStr">
         <is>
-          <t>Petty-cash disbursed beyond authority / without independent review, or drawn past the fund's limit — cash leakage, unauthorised or unrecorded expense, over-extended float.</t>
+          <t>Petty-cash / employee advance issued but never accounted for — cash leakage, expense unrecorded.</t>
         </is>
       </c>
       <c r="F99" s="16" t="inlineStr">
         <is>
-          <t>Authorization; Completeness</t>
+          <t>Existence/Completeness</t>
         </is>
       </c>
       <c r="G99" s="16" t="inlineStr">
         <is>
-          <t>Petty-cash imprest float + maker-checker on disbursement (SoD): a fund holds cash capped at a credit limit/วงเงิน (1015 Petty Cash, a cash account); each direct EXPENSE or ADVANCE is a REQUEST that posts NOTHING and a DIFFERENT user must approve before the GL posts (expense Dr &lt;expense&gt; / Cr 1015; advance Dr 1180 / Cr 1015) and the fund balance is decremented. Self-approval → SOD_VIOLATION (binds even Admin). A draw beyond the fund balance → INSUFFICIENT_FLOAT; establishing/replenishing above the float limit → OVER_FLOAT. Advances settle (Dr expense + Dr 1015 returned / Cr 1180), returning unused cash to the fund. Every request carries a document reference + receipt key + a status trail (StatusLog) and surfaces in the GOV-01 pending-approvals monitor.</t>
+          <t>Employee cash advances: issuing an advance debits the 1180 Employee Advances control (Dr 1180 / Cr 1000); settlement clears it against actual spend + returned cash (Dr expense + Dr 1000 / Cr 1180), enforced to reconcile (settled_expense + returned_cash must equal the advance → SETTLE_MISMATCH). The 1180 balance is the outstanding float subject to review.</t>
         </is>
       </c>
       <c r="H99" s="17" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I99" s="17" t="inlineStr">
@@ -9454,7 +9454,7 @@
       </c>
       <c r="J99" s="17" t="inlineStr">
         <is>
-          <t>Per disbursement</t>
+          <t>Per advance</t>
         </is>
       </c>
       <c r="K99" s="16" t="inlineStr">
@@ -9469,22 +9469,22 @@
       </c>
       <c r="M99" s="16" t="inlineStr">
         <is>
-          <t>petty-cash.service.ts (establishFund/replenishFund float guards, createRequest INSUFFICIENT_FLOAT, approveRequest SoD+GL, rejectRequest, settleRequest); petty-cash.controller.ts (creditors/exec); schema/petty-cash.ts (petty_cash_funds, expense_requests) + migration 0139; finance.service.ts pendingApprovals (GOV-01 source 7); cutover/basics.ts + compliance.ts (ToE)</t>
+          <t>finance.service.ts (issueAdvance, settleAdvance reconcile-or-reject, listAdvances outstanding); finance.controller.ts (creditors/exec); schema/finance.ts (employee_advances) + migration 0120; cutover/basics.ts (ToE)</t>
         </is>
       </c>
       <c r="N99" s="16" t="inlineStr">
         <is>
-          <t>Inspect the float ceiling + the request→approve flow + the approver≠requester check + that the request posts nothing until approval.</t>
+          <t>Inspect issue/settle GL + settlement reconciliation guard.</t>
         </is>
       </c>
       <c r="O99" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: establish a fund (Dr 1015), request an expense (no GL), self-approve → SOD_VIOLATION, approve as a different user → Dr expense/Cr 1015 + fund down; over-balance draw → INSUFFICIENT_FLOAT; advance approve→settle clears 1180; replenish past float → OVER_FLOAT (re-performed by the harnesses).</t>
+          <t>Issue an advance (1180 up); settle 700+300 clears 1180; mismatched settle → SETTLE_MISMATCH (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P99" s="16" t="inlineStr">
         <is>
-          <t>Fund register + disbursement approval log + SoD test</t>
+          <t>Advance register; outstanding float</t>
         </is>
       </c>
       <c r="Q99" s="18" t="inlineStr">
@@ -9496,12 +9496,12 @@
     <row r="100">
       <c r="A100" s="11" t="inlineStr">
         <is>
-          <t>FA-07</t>
+          <t>EXP-08</t>
         </is>
       </c>
       <c r="B100" s="12" t="inlineStr">
         <is>
-          <t>Fixed Assets</t>
+          <t>Expenditure</t>
         </is>
       </c>
       <c r="C100" s="13" t="inlineStr">
@@ -9511,27 +9511,27 @@
       </c>
       <c r="D100" s="12" t="inlineStr">
         <is>
-          <t>Property, Plant &amp; Equipment; Equity</t>
+          <t>Cash; Operating expense</t>
         </is>
       </c>
       <c r="E100" s="12" t="inlineStr">
         <is>
-          <t>Carrying amount not adjusted for revaluation/impairment — asset over/understated.</t>
+          <t>Petty-cash disbursed beyond authority / without independent review, or drawn past the fund's limit — cash leakage, unauthorised or unrecorded expense, over-extended float.</t>
         </is>
       </c>
       <c r="F100" s="12" t="inlineStr">
         <is>
-          <t>Valuation</t>
+          <t>Authorization; Completeness</t>
         </is>
       </c>
       <c r="G100" s="12" t="inlineStr">
         <is>
-          <t>Asset revaluation / impairment: an upward revaluation credits the revaluation surplus in equity (Dr 1500 / Cr 3200); a downward revaluation (impairment) debits impairment loss (Dr 5820 / Cr 1500). The gross 1500 moves by the delta so the register stays tied to the GL; a no-op revaluation is rejected (NO_CHANGE). Every event is logged for the audit trail.</t>
+          <t>Petty-cash imprest float + maker-checker on disbursement (SoD): a fund holds cash capped at a credit limit/วงเงิน (1015 Petty Cash, a cash account); each direct EXPENSE or ADVANCE is a REQUEST that posts NOTHING and a DIFFERENT user must approve before the GL posts (expense Dr &lt;expense&gt; / Cr 1015; advance Dr 1180 / Cr 1015) and the fund balance is decremented. Self-approval → SOD_VIOLATION (binds even Admin). A draw beyond the fund balance → INSUFFICIENT_FLOAT; establishing/replenishing above the float limit → OVER_FLOAT. Advances settle (Dr expense + Dr 1015 returned / Cr 1180), returning unused cash to the fund. Every request carries a document reference + receipt key + a status trail (StatusLog) and surfaces in the GOV-01 pending-approvals monitor.</t>
         </is>
       </c>
       <c r="H100" s="13" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I100" s="13" t="inlineStr">
@@ -9541,12 +9541,12 @@
       </c>
       <c r="J100" s="13" t="inlineStr">
         <is>
-          <t>Per event</t>
+          <t>Per disbursement</t>
         </is>
       </c>
       <c r="K100" s="12" t="inlineStr">
         <is>
-          <t>FaAccountant / Controller</t>
+          <t>AP / Controller</t>
         </is>
       </c>
       <c r="L100" s="13" t="inlineStr">
@@ -9556,22 +9556,22 @@
       </c>
       <c r="M100" s="12" t="inlineStr">
         <is>
-          <t>assets.service.ts (revalue up→3200 / down→5820, listRevaluations; dispose recycles surplus 3200→3100); assets.controller.ts (exec/creditors); schema/assets.ts (asset_revaluations) + migration 0120; cutover/basics.ts (ToE)</t>
+          <t>petty-cash.service.ts (establishFund/replenishFund float guards, createRequest INSUFFICIENT_FLOAT, approveRequest SoD+GL, rejectRequest, settleRequest); petty-cash.controller.ts (creditors/exec); schema/petty-cash.ts (petty_cash_funds, expense_requests) + migration 0139; finance.service.ts pendingApprovals (GOV-01 source 7); cutover/basics.ts + compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N100" s="12" t="inlineStr">
         <is>
-          <t>Inspect revaluation/impairment routing + audit log + disposal recycling.</t>
+          <t>Inspect the float ceiling + the request→approve flow + the approver≠requester check + that the request posts nothing until approval.</t>
         </is>
       </c>
       <c r="O100" s="12" t="inlineStr">
         <is>
-          <t>Upward revaluation credits 3200; impairment debits 5820; no-change → NO_CHANGE; both events logged; on disposal the revaluation surplus is recycled to retained earnings (Dr 3200 / Cr 3100), not through P&amp;L (re-performed by the harness).</t>
+          <t>Re-perform: establish a fund (Dr 1015), request an expense (no GL), self-approve → SOD_VIOLATION, approve as a different user → Dr expense/Cr 1015 + fund down; over-balance draw → INSUFFICIENT_FLOAT; advance approve→settle clears 1180; replenish past float → OVER_FLOAT (re-performed by the harnesses).</t>
         </is>
       </c>
       <c r="P100" s="12" t="inlineStr">
         <is>
-          <t>Revaluation log; disposal recycling JE</t>
+          <t>Fund register + disbursement approval log + SoD test</t>
         </is>
       </c>
       <c r="Q100" s="18" t="inlineStr">
@@ -9583,7 +9583,7 @@
     <row r="101">
       <c r="A101" s="15" t="inlineStr">
         <is>
-          <t>FA-08</t>
+          <t>FA-07</t>
         </is>
       </c>
       <c r="B101" s="16" t="inlineStr">
@@ -9603,22 +9603,22 @@
       </c>
       <c r="E101" s="16" t="inlineStr">
         <is>
-          <t>Carrying amount changed by fair-value revaluation/impairment without independent review — the preparer revalues the asset and posts to equity/P&amp;L on their own (earnings/equity management).</t>
+          <t>Carrying amount not adjusted for revaluation/impairment — asset over/understated.</t>
         </is>
       </c>
       <c r="F101" s="16" t="inlineStr">
         <is>
-          <t>Authorization</t>
+          <t>Valuation</t>
         </is>
       </c>
       <c r="G101" s="16" t="inlineStr">
         <is>
-          <t>Asset-revaluation maker-checker (SoD): a revalue/impairment request posts its GL entry as a DRAFT (excluded from balances) and records status 'PendingApproval' WITHOUT moving the carrying value; a DIFFERENT user must approve before the JE is effective and the register is re-valued (approver ≠ preparer enforced regardless of permissions, reusing the GL-05 ledger approval). Reject voids the draft; only one revaluation may be pending per asset; the disposal surplus recycle counts only approved revaluations.</t>
+          <t>Asset revaluation / impairment: an upward revaluation credits the revaluation surplus in equity (Dr 1500 / Cr 3200); a downward revaluation (impairment) debits impairment loss (Dr 5820 / Cr 1500). The gross 1500 moves by the delta so the register stays tied to the GL; a no-op revaluation is rejected (NO_CHANGE). Every event is logged for the audit trail.</t>
         </is>
       </c>
       <c r="H101" s="17" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I101" s="17" t="inlineStr">
@@ -9643,22 +9643,22 @@
       </c>
       <c r="M101" s="16" t="inlineStr">
         <is>
-          <t>assets.service.ts revalue(pendingApproval Draft)/approveRevaluation/rejectRevaluation; assets.controller.ts (:assetNo/revalue/approve|reject); schema/assets.ts asset_revaluations.status + migration 0134; cutover/basics.ts + compliance.ts (ToE)</t>
+          <t>assets.service.ts (revalue up→3200 / down→5820, listRevaluations; dispose recycles surplus 3200→3100); assets.controller.ts (exec/creditors); schema/assets.ts (asset_revaluations) + migration 0120; cutover/basics.ts (ToE)</t>
         </is>
       </c>
       <c r="N101" s="16" t="inlineStr">
         <is>
-          <t>Inspect Draft→approve flow + the approver≠preparer check + deferred carrying-value update.</t>
+          <t>Inspect revaluation/impairment routing + audit log + disposal recycling.</t>
         </is>
       </c>
       <c r="O101" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: request a revaluation (Draft JE excluded from 3200), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm the surplus/impairment + carrying value move only after approval (re-performed by the harnesses).</t>
+          <t>Upward revaluation credits 3200; impairment debits 5820; no-change → NO_CHANGE; both events logged; on disposal the revaluation surplus is recycled to retained earnings (Dr 3200 / Cr 3100), not through P&amp;L (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P101" s="16" t="inlineStr">
         <is>
-          <t>Revaluation approval log + SoD test</t>
+          <t>Revaluation log; disposal recycling JE</t>
         </is>
       </c>
       <c r="Q101" s="18" t="inlineStr">
@@ -9670,12 +9670,12 @@
     <row r="102">
       <c r="A102" s="11" t="inlineStr">
         <is>
-          <t>LSE-01</t>
+          <t>FA-08</t>
         </is>
       </c>
       <c r="B102" s="12" t="inlineStr">
         <is>
-          <t>Leases</t>
+          <t>Fixed Assets</t>
         </is>
       </c>
       <c r="C102" s="13" t="inlineStr">
@@ -9685,27 +9685,27 @@
       </c>
       <c r="D102" s="12" t="inlineStr">
         <is>
-          <t>Right-of-use assets; Lease liabilities</t>
+          <t>Property, Plant &amp; Equipment; Equity</t>
         </is>
       </c>
       <c r="E102" s="12" t="inlineStr">
         <is>
-          <t>Lease not capitalised (IFRS 16 / TFRS 16) — ROU asset + lease liability omitted; interest/depreciation mis-stated.</t>
+          <t>Carrying amount changed by fair-value revaluation/impairment without independent review — the preparer revalues the asset and posts to equity/P&amp;L on their own (earnings/equity management).</t>
         </is>
       </c>
       <c r="F102" s="12" t="inlineStr">
         <is>
-          <t>Completeness/Accuracy/Valuation</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="G102" s="12" t="inlineStr">
         <is>
-          <t>Lease accounting: at commencement a right-of-use asset and lease liability are recognised at the present value of the lease payments (Dr 1600 / Cr 2600). The scheduled job lease_periodic_run posts each period — interest unwinding on the liability (Dr 5900), the cash payment reducing the liability (Dr 2600 / Cr 1000), and straight-line ROU depreciation (Dr 5210 / Cr 1690) — the last period clearing the liability + ROU exactly. Idempotent per (lease, period).</t>
+          <t>Asset-revaluation maker-checker (SoD): a revalue/impairment request posts its GL entry as a DRAFT (excluded from balances) and records status 'PendingApproval' WITHOUT moving the carrying value; a DIFFERENT user must approve before the JE is effective and the register is re-valued (approver ≠ preparer enforced regardless of permissions, reusing the GL-05 ledger approval). Reject voids the draft; only one revaluation may be pending per asset; the disposal surplus recycle counts only approved revaluations.</t>
         </is>
       </c>
       <c r="H102" s="13" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I102" s="13" t="inlineStr">
@@ -9715,12 +9715,12 @@
       </c>
       <c r="J102" s="13" t="inlineStr">
         <is>
-          <t>Per period / per lease</t>
+          <t>Per event</t>
         </is>
       </c>
       <c r="K102" s="12" t="inlineStr">
         <is>
-          <t>Controller</t>
+          <t>FaAccountant / Controller</t>
         </is>
       </c>
       <c r="L102" s="13" t="inlineStr">
@@ -9730,22 +9730,22 @@
       </c>
       <c r="M102" s="12" t="inlineStr">
         <is>
-          <t>leases.service.ts (createLease PV recognition, runDueLeases interest+payment+depreciation, modifyLease remeasurement); leases.controller.ts (gl_post); bi.service.ts (lease_periodic_run); schema/leases.ts (leases, rou_nbv) + migration 0120/0121; cutover/basics.ts (ToE)</t>
+          <t>assets.service.ts revalue(pendingApproval Draft)/approveRevaluation/rejectRevaluation; assets.controller.ts (:assetNo/revalue/approve|reject); schema/assets.ts asset_revaluations.status + migration 0134; cutover/basics.ts + compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N102" s="12" t="inlineStr">
         <is>
-          <t>Inspect PV recognition + periodic interest/payment/depreciation + final-period clearing + modification remeasurement.</t>
+          <t>Inspect Draft→approve flow + the approver≠preparer check + deferred carrying-value update.</t>
         </is>
       </c>
       <c r="O102" s="12" t="inlineStr">
         <is>
-          <t>Commencement recognises ROU=liability=PV; periodic run posts interest+principal(=payment)+ROU depreciation; liability + ROU reduce; a modification remeasures the liability at the revised PV and adjusts the ROU by the same delta (Dr/Cr 1600↔2600), then depreciates over the remaining term (re-performed by the harness).</t>
+          <t>Re-perform: request a revaluation (Draft JE excluded from 3200), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm the surplus/impairment + carrying value move only after approval (re-performed by the harnesses).</t>
         </is>
       </c>
       <c r="P102" s="12" t="inlineStr">
         <is>
-          <t>Lease register; periodic run log; modification remeasurement</t>
+          <t>Revaluation approval log + SoD test</t>
         </is>
       </c>
       <c r="Q102" s="18" t="inlineStr">
@@ -9757,12 +9757,12 @@
     <row r="103">
       <c r="A103" s="15" t="inlineStr">
         <is>
-          <t>REC-01</t>
+          <t>LSE-01</t>
         </is>
       </c>
       <c r="B103" s="16" t="inlineStr">
         <is>
-          <t>Reconciliation</t>
+          <t>Leases</t>
         </is>
       </c>
       <c r="C103" s="17" t="inlineStr">
@@ -9772,22 +9772,22 @@
       </c>
       <c r="D103" s="16" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Right-of-use assets; Lease liabilities</t>
         </is>
       </c>
       <c r="E103" s="16" t="inlineStr">
         <is>
-          <t>Subledgers diverge from GL undetected.</t>
+          <t>Lease not capitalised (IFRS 16 / TFRS 16) — ROU asset + lease liability omitted; interest/depreciation mis-stated.</t>
         </is>
       </c>
       <c r="F103" s="16" t="inlineStr">
         <is>
-          <t>Completeness/Accuracy</t>
+          <t>Completeness/Accuracy/Valuation</t>
         </is>
       </c>
       <c r="G103" s="16" t="inlineStr">
         <is>
-          <t>Subledger-to-GL reconciliation per period: import GL, auto-match, certify (sign-off via 'approvals').</t>
+          <t>Lease accounting: at commencement a right-of-use asset and lease liability are recognised at the present value of the lease payments (Dr 1600 / Cr 2600). The scheduled job lease_periodic_run posts each period — interest unwinding on the liability (Dr 5900), the cash payment reducing the liability (Dr 2600 / Cr 1000), and straight-line ROU depreciation (Dr 5210 / Cr 1690) — the last period clearing the liability + ROU exactly. Idempotent per (lease, period).</t>
         </is>
       </c>
       <c r="H103" s="17" t="inlineStr">
@@ -9797,12 +9797,12 @@
       </c>
       <c r="I103" s="17" t="inlineStr">
         <is>
-          <t>Auto+Manual</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J103" s="17" t="inlineStr">
         <is>
-          <t>Monthly</t>
+          <t>Per period / per lease</t>
         </is>
       </c>
       <c r="K103" s="16" t="inlineStr">
@@ -9812,27 +9812,27 @@
       </c>
       <c r="L103" s="17" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="M103" s="16" t="inlineStr">
         <is>
-          <t>reconciliation.service.ts (importGlItems/autoMatch/certify)</t>
+          <t>leases.service.ts (createLease PV recognition, runDueLeases interest+payment+depreciation, modifyLease remeasurement); leases.controller.ts (gl_post); bi.service.ts (lease_periodic_run); schema/leases.ts (leases, rou_nbv) + migration 0120/0121; cutover/basics.ts (ToE)</t>
         </is>
       </c>
       <c r="N103" s="16" t="inlineStr">
         <is>
-          <t>Inspect recon + certify gate.</t>
+          <t>Inspect PV recognition + periodic interest/payment/depreciation + final-period clearing + modification remeasurement.</t>
         </is>
       </c>
       <c r="O103" s="16" t="inlineStr">
         <is>
-          <t>Sample periods: reconciled, unmatched cleared, certified.</t>
+          <t>Commencement recognises ROU=liability=PV; periodic run posts interest+principal(=payment)+ROU depreciation; liability + ROU reduce; a modification remeasures the liability at the revised PV and adjusts the ROU by the same delta (Dr/Cr 1600↔2600), then depreciates over the remaining term (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P103" s="16" t="inlineStr">
         <is>
-          <t>Certified recon</t>
+          <t>Lease register; periodic run log; modification remeasurement</t>
         </is>
       </c>
       <c r="Q103" s="18" t="inlineStr">
@@ -9844,7 +9844,7 @@
     <row r="104">
       <c r="A104" s="11" t="inlineStr">
         <is>
-          <t>REC-02</t>
+          <t>REC-01</t>
         </is>
       </c>
       <c r="B104" s="12" t="inlineStr">
@@ -9859,22 +9859,22 @@
       </c>
       <c r="D104" s="12" t="inlineStr">
         <is>
-          <t>Cash</t>
+          <t>All</t>
         </is>
       </c>
       <c r="E104" s="12" t="inlineStr">
         <is>
-          <t>Bank balance not reconciled to GL.</t>
+          <t>Subledgers diverge from GL undetected.</t>
         </is>
       </c>
       <c r="F104" s="12" t="inlineStr">
         <is>
-          <t>Existence/Completeness</t>
+          <t>Completeness/Accuracy</t>
         </is>
       </c>
       <c r="G104" s="12" t="inlineStr">
         <is>
-          <t>Bank reconciliation against statements.</t>
+          <t>Subledger-to-GL reconciliation per period: import GL, auto-match, certify (sign-off via 'approvals').</t>
         </is>
       </c>
       <c r="H104" s="13" t="inlineStr">
@@ -9904,22 +9904,22 @@
       </c>
       <c r="M104" s="12" t="inlineStr">
         <is>
-          <t>bank module; drizzle/0015_bank_reconciliation</t>
+          <t>reconciliation.service.ts (importGlItems/autoMatch/certify)</t>
         </is>
       </c>
       <c r="N104" s="12" t="inlineStr">
         <is>
-          <t>Inspect bank-rec process.</t>
+          <t>Inspect recon + certify gate.</t>
         </is>
       </c>
       <c r="O104" s="12" t="inlineStr">
         <is>
-          <t>Sample months reconciled &amp; reviewed.</t>
+          <t>Sample periods: reconciled, unmatched cleared, certified.</t>
         </is>
       </c>
       <c r="P104" s="12" t="inlineStr">
         <is>
-          <t>Bank rec</t>
+          <t>Certified recon</t>
         </is>
       </c>
       <c r="Q104" s="18" t="inlineStr">
@@ -9931,12 +9931,12 @@
     <row r="105">
       <c r="A105" s="15" t="inlineStr">
         <is>
-          <t>BANK-02</t>
+          <t>REC-02</t>
         </is>
       </c>
       <c r="B105" s="16" t="inlineStr">
         <is>
-          <t>Cash &amp; Treasury</t>
+          <t>Reconciliation</t>
         </is>
       </c>
       <c r="C105" s="17" t="inlineStr">
@@ -9946,37 +9946,37 @@
       </c>
       <c r="D105" s="16" t="inlineStr">
         <is>
-          <t>Cash; Operating expense; Interest income</t>
+          <t>Cash</t>
         </is>
       </c>
       <c r="E105" s="16" t="inlineStr">
         <is>
-          <t>A bank fee/interest adjustment is posted straight to the GL by one person during reconciliation — a cash outflow mis-booked as interest income, or a fictitious fee posted, with no independent review (single-person posting to the cash account).</t>
+          <t>Bank balance not reconciled to GL.</t>
         </is>
       </c>
       <c r="F105" s="16" t="inlineStr">
         <is>
-          <t>Authorization/Accuracy</t>
+          <t>Existence/Completeness</t>
         </is>
       </c>
       <c r="G105" s="16" t="inlineStr">
         <is>
-          <t>Bank adjustment maker-checker (SoD): a fee/interest adjustment on a statement line is a REQUEST that posts a DRAFT JE (no balance/GL effect; the line stays unreconciled) until a DIFFERENT user with approval authority approves (POST /api/bank/lines/:id/adjustment/approve). Self-approval → SOD_VIOLATION (binds even Admin); approval flips the line to reconciled and the JE to Posted; reject voids the Draft and frees the line. The Draft JE (source BANKADJ) is also surfaced, aged, by the pending-approvals monitor (GOV-01).</t>
+          <t>Bank reconciliation against statements.</t>
         </is>
       </c>
       <c r="H105" s="17" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I105" s="17" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="J105" s="17" t="inlineStr">
         <is>
-          <t>Per adjustment</t>
+          <t>Monthly</t>
         </is>
       </c>
       <c r="K105" s="16" t="inlineStr">
@@ -9986,27 +9986,27 @@
       </c>
       <c r="L105" s="17" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="M105" s="16" t="inlineStr">
         <is>
-          <t>bank.service.ts requestAdjustment/approveAdjustment/rejectAdjustment/listPendingAdjustments (reuses ledger.approveEntry SoD); bank.controller.ts (lines/:id/adjustment requests; adjustment/approve|reject gated approvals/gl_close); cutover/bankrec.ts (ToE)</t>
+          <t>bank module; drizzle/0015_bank_reconciliation</t>
         </is>
       </c>
       <c r="N105" s="16" t="inlineStr">
         <is>
-          <t>Inspect the request→approve flow + the approver≠requester check + that the Draft posts nothing until approval.</t>
+          <t>Inspect bank-rec process.</t>
         </is>
       </c>
       <c r="O105" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: request a fee adjustment (line unreconciled, GL difference unchanged), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm the difference closes to 0 only after approval (re-performed by the bankrec harness).</t>
+          <t>Sample months reconciled &amp; reviewed.</t>
         </is>
       </c>
       <c r="P105" s="16" t="inlineStr">
         <is>
-          <t>Bank adjustment queue + SoD test</t>
+          <t>Bank rec</t>
         </is>
       </c>
       <c r="Q105" s="18" t="inlineStr">
@@ -10018,12 +10018,12 @@
     <row r="106">
       <c r="A106" s="11" t="inlineStr">
         <is>
-          <t>REC-03</t>
+          <t>BANK-02</t>
         </is>
       </c>
       <c r="B106" s="12" t="inlineStr">
         <is>
-          <t>Reconciliation</t>
+          <t>Cash &amp; Treasury</t>
         </is>
       </c>
       <c r="C106" s="13" t="inlineStr">
@@ -10033,79 +10033,79 @@
       </c>
       <c r="D106" s="12" t="inlineStr">
         <is>
-          <t>Consolidation</t>
+          <t>Cash; Operating expense; Interest income</t>
         </is>
       </c>
       <c r="E106" s="12" t="inlineStr">
         <is>
-          <t>Intercompany balances not eliminated/agreed.</t>
+          <t>A bank fee/interest adjustment is posted straight to the GL by one person during reconciliation — a cash outflow mis-booked as interest income, or a fictitious fee posted, with no independent review (single-person posting to the cash account).</t>
         </is>
       </c>
       <c r="F106" s="12" t="inlineStr">
         <is>
-          <t>Accuracy</t>
+          <t>Authorization/Accuracy</t>
         </is>
       </c>
       <c r="G106" s="12" t="inlineStr">
         <is>
-          <t>Intercompany reconciliation &amp; elimination on consolidation.</t>
+          <t>Bank adjustment maker-checker (SoD): a fee/interest adjustment on a statement line is a REQUEST that posts a DRAFT JE (no balance/GL effect; the line stays unreconciled) until a DIFFERENT user with approval authority approves (POST /api/bank/lines/:id/adjustment/approve). Self-approval → SOD_VIOLATION (binds even Admin); approval flips the line to reconciled and the JE to Posted; reject voids the Draft and frees the line. The Draft JE (source BANKADJ) is also surfaced, aged, by the pending-approvals monitor (GOV-01).</t>
         </is>
       </c>
       <c r="H106" s="13" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I106" s="13" t="inlineStr">
         <is>
-          <t>Auto+Manual</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J106" s="13" t="inlineStr">
         <is>
-          <t>Period</t>
+          <t>Per adjustment</t>
         </is>
       </c>
       <c r="K106" s="12" t="inlineStr">
         <is>
-          <t>Group Controller</t>
+          <t>Controller</t>
         </is>
       </c>
       <c r="L106" s="13" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="M106" s="12" t="inlineStr">
         <is>
-          <t>intercompany; consolidation</t>
+          <t>bank.service.ts requestAdjustment/approveAdjustment/rejectAdjustment/listPendingAdjustments (reuses ledger.approveEntry SoD); bank.controller.ts (lines/:id/adjustment requests; adjustment/approve|reject gated approvals/gl_close); cutover/bankrec.ts (ToE)</t>
         </is>
       </c>
       <c r="N106" s="12" t="inlineStr">
         <is>
-          <t>Inspect IC matching + elimination.</t>
+          <t>Inspect the request→approve flow + the approver≠requester check + that the Draft posts nothing until approval.</t>
         </is>
       </c>
       <c r="O106" s="12" t="inlineStr">
         <is>
-          <t>Sample IC pairs agree &amp; eliminate.</t>
+          <t>Re-perform: request a fee adjustment (line unreconciled, GL difference unchanged), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm the difference closes to 0 only after approval (re-performed by the bankrec harness).</t>
         </is>
       </c>
       <c r="P106" s="12" t="inlineStr">
         <is>
-          <t>IC recon</t>
-        </is>
-      </c>
-      <c r="Q106" s="19" t="inlineStr">
-        <is>
-          <t>Partial</t>
+          <t>Bank adjustment queue + SoD test</t>
+        </is>
+      </c>
+      <c r="Q106" s="18" t="inlineStr">
+        <is>
+          <t>Implemented</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="15" t="inlineStr">
         <is>
-          <t>REC-04</t>
+          <t>REC-03</t>
         </is>
       </c>
       <c r="B107" s="16" t="inlineStr">
@@ -10120,22 +10120,22 @@
       </c>
       <c r="D107" s="16" t="inlineStr">
         <is>
-          <t>All control accounts</t>
+          <t>Consolidation</t>
         </is>
       </c>
       <c r="E107" s="16" t="inlineStr">
         <is>
-          <t>A sub-ledger silently drifts from its GL control account at period-end and no single review catches it (incomplete/inaccurate balances reach the financial statements).</t>
+          <t>Intercompany balances not eliminated/agreed.</t>
         </is>
       </c>
       <c r="F107" s="16" t="inlineStr">
         <is>
-          <t>Completeness/Accuracy</t>
+          <t>Accuracy</t>
         </is>
       </c>
       <c r="G107" s="16" t="inlineStr">
         <is>
-          <t>Period-end control-account reconciliation PACK: one read (GET /api/finance/reconciliation/controls) ties every major sub-ledger to its GL control account and FLAGS any out-of-balance — AR↔1100, AP↔2000, Inventory↔1200, Gift cards/Customer-deposits↔2200, Deferred revenue↔2400 — reporting per line {sub_ledger, gl_control, variance, reconciled} plus an overall all_reconciled flag and an exceptions count. Liability controls are sign-flipped before comparison. The controller's single 'are the books reconciled?' close view; an exception is a control finding to investigate before sign-off.</t>
+          <t>Intercompany reconciliation &amp; elimination on consolidation.</t>
         </is>
       </c>
       <c r="H107" s="17" t="inlineStr">
@@ -10145,17 +10145,17 @@
       </c>
       <c r="I107" s="17" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="J107" s="17" t="inlineStr">
         <is>
-          <t>Period / on demand</t>
+          <t>Period</t>
         </is>
       </c>
       <c r="K107" s="16" t="inlineStr">
         <is>
-          <t>Controller / CFO</t>
+          <t>Group Controller</t>
         </is>
       </c>
       <c r="L107" s="17" t="inlineStr">
@@ -10165,34 +10165,34 @@
       </c>
       <c r="M107" s="16" t="inlineStr">
         <is>
-          <t>finance.service.ts reconcileControls; finance.controller.ts GET reconciliation/controls (exec/ar/creditors); reuses ledger.trialBalance + the AR/AP/inventory/gift-card/deferred sub-ledgers; cutover/giftcards.ts + compliance.ts (ToE)</t>
+          <t>intercompany; consolidation</t>
         </is>
       </c>
       <c r="N107" s="16" t="inlineStr">
         <is>
-          <t>Inspect the pack: each control account's sub-ledger query + the GL tie + the exceptions roll-up.</t>
+          <t>Inspect IC matching + elimination.</t>
         </is>
       </c>
       <c r="O107" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: with a clean set, every line reconciled + all_reconciled=true; introduce a known sub-ledger/GL difference and confirm it surfaces as an exception (re-performed: gift-card 2200 + inventory 1200 ties asserted by the harnesses).</t>
+          <t>Sample IC pairs agree &amp; eliminate.</t>
         </is>
       </c>
       <c r="P107" s="16" t="inlineStr">
         <is>
-          <t>Reconciliation pack; exceptions list</t>
-        </is>
-      </c>
-      <c r="Q107" s="18" t="inlineStr">
-        <is>
-          <t>Implemented</t>
+          <t>IC recon</t>
+        </is>
+      </c>
+      <c r="Q107" s="19" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="11" t="inlineStr">
         <is>
-          <t>REC-05</t>
+          <t>REC-04</t>
         </is>
       </c>
       <c r="B108" s="12" t="inlineStr">
@@ -10207,42 +10207,42 @@
       </c>
       <c r="D108" s="12" t="inlineStr">
         <is>
-          <t>Cash; Bank</t>
+          <t>All control accounts</t>
         </is>
       </c>
       <c r="E108" s="12" t="inlineStr">
         <is>
-          <t>Till cash dropped to the safe never reaches the bank, or a deposit isn't matched to the statement — cash sits unbanked (theft/loss exposure) or the bank balance can't be tied to the books.</t>
+          <t>A sub-ledger silently drifts from its GL control account at period-end and no single review catches it (incomplete/inaccurate balances reach the financial statements).</t>
         </is>
       </c>
       <c r="F108" s="12" t="inlineStr">
         <is>
-          <t>Completeness/Existence/Authorization</t>
+          <t>Completeness/Accuracy</t>
         </is>
       </c>
       <c r="G108" s="12" t="inlineStr">
         <is>
-          <t>Cash banking — safe-drop → bank deposit → reconciliation: till 'drop's move cash from the drawer to the safe (drawer-only, no GL). Banking BATCHES the undeposited drops into a deposit and posts the GL (Dr &lt;bank account, e.g. 1010&gt; / Cr 1000 Cash), stamping each drop with the deposit id; the deposit is then RECONCILED to the bank statement (status Deposited→Reconciled). A detective read (GET /api/bank/deposits/undeposited-drops) surfaces the CASH STILL IN THE SAFE (drops with deposit_id NULL) — the unbanked exposure to chase. SoD: banking is a treasury duty (exec/ar) — segregated from the cashier (pos_till) who drops the cash, so the person who removes cash from the drawer is not the one who banks it.</t>
+          <t>Period-end control-account reconciliation PACK: one read (GET /api/finance/reconciliation/controls) ties every major sub-ledger to its GL control account and FLAGS any out-of-balance — AR↔1100, AP↔2000, Inventory↔1200, Gift cards/Customer-deposits↔2200, Deferred revenue↔2400 — reporting per line {sub_ledger, gl_control, variance, reconciled} plus an overall all_reconciled flag and an exceptions count. Liability controls are sign-flipped before comparison. The controller's single 'are the books reconciled?' close view; an exception is a control finding to investigate before sign-off.</t>
         </is>
       </c>
       <c r="H108" s="13" t="inlineStr">
         <is>
-          <t>Det/Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I108" s="13" t="inlineStr">
         <is>
-          <t>Auto+Manual</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J108" s="13" t="inlineStr">
         <is>
-          <t>Per banking run</t>
+          <t>Period / on demand</t>
         </is>
       </c>
       <c r="K108" s="12" t="inlineStr">
         <is>
-          <t>FinancialController / Treasury</t>
+          <t>Controller / CFO</t>
         </is>
       </c>
       <c r="L108" s="13" t="inlineStr">
@@ -10252,22 +10252,22 @@
       </c>
       <c r="M108" s="12" t="inlineStr">
         <is>
-          <t>bank.service.ts undepositedDrops/createDeposit (Dr bank/Cr 1000, stamps deposit_id)/reconcileDeposit/listDeposits; bank.controller.ts (deposits, deposits/undeposited-drops, deposits/:id/reconcile; exec/ar); schema/cash.ts bank_deposits + cash_movements.deposit_id + migration 0152; /cash-banking UI; cutover/cash-banking.ts (ToE)</t>
+          <t>finance.service.ts reconcileControls; finance.controller.ts GET reconciliation/controls (exec/ar/creditors); reuses ledger.trialBalance + the AR/AP/inventory/gift-card/deferred sub-ledgers; cutover/giftcards.ts + compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N108" s="12" t="inlineStr">
         <is>
-          <t>Inspect the undeposited-drop exposure read + the deposit GL (bank↔1000) + the reconcile step + the SoD (cashier vs treasury).</t>
+          <t>Inspect the pack: each control account's sub-ledger query + the GL tie + the exceptions roll-up.</t>
         </is>
       </c>
       <c r="O108" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: two till drops → cash-in-safe shows the total; a cashier (pos_till) cannot bank (403); treasury banks → Dr bank / Cr 1000, cash-in-safe back to 0; reconcile the deposit; trial balance balanced (re-performed by the cash-banking harness).</t>
+          <t>Re-perform: with a clean set, every line reconciled + all_reconciled=true; introduce a known sub-ledger/GL difference and confirm it surfaces as an exception (re-performed: gift-card 2200 + inventory 1200 ties asserted by the harnesses).</t>
         </is>
       </c>
       <c r="P108" s="12" t="inlineStr">
         <is>
-          <t>Bank-deposit register; undeposited-drop (cash-in-safe) exposure</t>
+          <t>Reconciliation pack; exceptions list</t>
         </is>
       </c>
       <c r="Q108" s="18" t="inlineStr">
@@ -10279,12 +10279,12 @@
     <row r="109">
       <c r="A109" s="15" t="inlineStr">
         <is>
-          <t>GOV-01</t>
+          <t>REC-05</t>
         </is>
       </c>
       <c r="B109" s="16" t="inlineStr">
         <is>
-          <t>Monitoring</t>
+          <t>Reconciliation</t>
         </is>
       </c>
       <c r="C109" s="17" t="inlineStr">
@@ -10294,42 +10294,42 @@
       </c>
       <c r="D109" s="16" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Cash; Bank</t>
         </is>
       </c>
       <c r="E109" s="16" t="inlineStr">
         <is>
-          <t>A maker-checker approval sits un-actioned and is forgotten — a transaction stalls before it is effective, or (worse) a control is quietly bypassed and no one notices an item never got its independent review.</t>
+          <t>Till cash dropped to the safe never reaches the bank, or a deposit isn't matched to the statement — cash sits unbanked (theft/loss exposure) or the bank balance can't be tied to the books.</t>
         </is>
       </c>
       <c r="F109" s="16" t="inlineStr">
         <is>
-          <t>Authorization/Completeness</t>
+          <t>Completeness/Existence/Authorization</t>
         </is>
       </c>
       <c r="G109" s="16" t="inlineStr">
         <is>
-          <t>Pending-approvals MONITOR (COSO monitoring): a single worklist of EVERY item awaiting independent approval across the system, each with its AGE in days and an overdue roll-up — spanning the manual-JE (GL-05), bank-adjustment (BANK-02), AP-disbursement (EXP-06), payroll (PAY-03), asset-revaluation (FA-08), asset-disposal (FA-09), inventory-write-off (INV-07), till-close cash over/short (REV-13), FX-rate (FX-04), budget (BUD-01) and large-refund (REV-16) maker-checkers. The controller reviews it before close; a stale item (age beyond the threshold) is a control finding to chase or escalate. The /approvals screen also lets a manager approve/reject a material till variance or a large refund inline (the pending types with no dedicated module screen). Read-only worklist; tenant-scoped via the caller's RLS.</t>
+          <t>Cash banking — safe-drop → bank deposit → reconciliation: till 'drop's move cash from the drawer to the safe (drawer-only, no GL). Banking BATCHES the undeposited drops into a deposit and posts the GL (Dr &lt;bank account, e.g. 1010&gt; / Cr 1000 Cash), stamping each drop with the deposit id; the deposit is then RECONCILED to the bank statement (status Deposited→Reconciled). A detective read (GET /api/bank/deposits/undeposited-drops) surfaces the CASH STILL IN THE SAFE (drops with deposit_id NULL) — the unbanked exposure to chase. SoD: banking is a treasury duty (exec/ar) — segregated from the cashier (pos_till) who drops the cash, so the person who removes cash from the drawer is not the one who banks it.</t>
         </is>
       </c>
       <c r="H109" s="17" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Det/Prev</t>
         </is>
       </c>
       <c r="I109" s="17" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="J109" s="17" t="inlineStr">
         <is>
-          <t>Continuous / pre-close</t>
+          <t>Per banking run</t>
         </is>
       </c>
       <c r="K109" s="16" t="inlineStr">
         <is>
-          <t>Controller / CFO</t>
+          <t>FinancialController / Treasury</t>
         </is>
       </c>
       <c r="L109" s="17" t="inlineStr">
@@ -10339,22 +10339,22 @@
       </c>
       <c r="M109" s="16" t="inlineStr">
         <is>
-          <t>finance.service.ts pendingApprovals; finance.controller.ts GET approvals/pending (exec/approvals/creditors); aggregates journalEntries(Draft incl. BANKADJ→BANK-02)/apPayments/payruns/asset_revaluations/fixed_assets(disposal_pending)/inv_writeoff_requests/till_sessions(PendingApproval)/fx_rates(PendingApproval)/budgets(PendingApproval); cutover/compliance.ts (ToE)</t>
+          <t>bank.service.ts undepositedDrops/createDeposit (Dr bank/Cr 1000, stamps deposit_id)/reconcileDeposit/listDeposits; bank.controller.ts (deposits, deposits/undeposited-drops, deposits/:id/reconcile; exec/ar); schema/cash.ts bank_deposits + cash_movements.deposit_id + migration 0152; /cash-banking UI; cutover/cash-banking.ts (ToE)</t>
         </is>
       </c>
       <c r="N109" s="16" t="inlineStr">
         <is>
-          <t>Inspect the aggregation across all pending sources + the age/overdue roll-up.</t>
+          <t>Inspect the undeposited-drop exposure read + the deposit GL (bank↔1000) + the reconcile step + the SoD (cashier vs treasury).</t>
         </is>
       </c>
       <c r="O109" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: create a pending item (e.g. a Draft JE) and confirm it appears in the worklist with its control ID, amount and age; the overdue count flags items past the threshold (re-performed by the harness).</t>
+          <t>Re-perform: two till drops → cash-in-safe shows the total; a cashier (pos_till) cannot bank (403); treasury banks → Dr bank / Cr 1000, cash-in-safe back to 0; reconcile the deposit; trial balance balanced (re-performed by the cash-banking harness).</t>
         </is>
       </c>
       <c r="P109" s="16" t="inlineStr">
         <is>
-          <t>Pending-approvals worklist</t>
+          <t>Bank-deposit register; undeposited-drop (cash-in-safe) exposure</t>
         </is>
       </c>
       <c r="Q109" s="18" t="inlineStr">
@@ -10366,12 +10366,12 @@
     <row r="110">
       <c r="A110" s="11" t="inlineStr">
         <is>
-          <t>TAX-01</t>
+          <t>GOV-01</t>
         </is>
       </c>
       <c r="B110" s="12" t="inlineStr">
         <is>
-          <t>Tax</t>
+          <t>Monitoring</t>
         </is>
       </c>
       <c r="C110" s="13" t="inlineStr">
@@ -10381,27 +10381,27 @@
       </c>
       <c r="D110" s="12" t="inlineStr">
         <is>
-          <t>Tax (VAT)</t>
+          <t>All</t>
         </is>
       </c>
       <c r="E110" s="12" t="inlineStr">
         <is>
-          <t>VAT computed incorrectly → filing/penalty risk.</t>
+          <t>A maker-checker approval sits un-actioned and is forgotten — a transaction stalls before it is effective, or (worse) a control is quietly bypassed and no one notices an item never got its independent review.</t>
         </is>
       </c>
       <c r="F110" s="12" t="inlineStr">
         <is>
-          <t>Accuracy</t>
+          <t>Authorization/Completeness</t>
         </is>
       </c>
       <c r="G110" s="12" t="inlineStr">
         <is>
-          <t>VAT via pluggable provider (TH 7%); unit-tested; no hard-coded rate.</t>
+          <t>Pending-approvals MONITOR (COSO monitoring): a single worklist of EVERY item awaiting independent approval across the system, each with its AGE in days and an overdue roll-up — spanning the manual-JE (GL-05), bank-adjustment (BANK-02), AP-disbursement (EXP-06), payroll (PAY-03), asset-revaluation (FA-08), asset-disposal (FA-09), inventory-write-off (INV-07), till-close cash over/short (REV-13), FX-rate (FX-04), budget (BUD-01) and large-refund (REV-16) maker-checkers. The controller reviews it before close; a stale item (age beyond the threshold) is a control finding to chase or escalate. The /approvals screen also lets a manager approve/reject a material till variance or a large refund inline (the pending types with no dedicated module screen). Read-only worklist; tenant-scoped via the caller's RLS.</t>
         </is>
       </c>
       <c r="H110" s="13" t="inlineStr">
         <is>
-          <t>Auto</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I110" s="13" t="inlineStr">
@@ -10411,37 +10411,37 @@
       </c>
       <c r="J110" s="13" t="inlineStr">
         <is>
-          <t>Per txn</t>
+          <t>Continuous / pre-close</t>
         </is>
       </c>
       <c r="K110" s="12" t="inlineStr">
         <is>
-          <t>Tax / Controller</t>
+          <t>Controller / CFO</t>
         </is>
       </c>
       <c r="L110" s="13" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="M110" s="12" t="inlineStr">
         <is>
-          <t>tax/tax-providers.ts; tax.service.ts; test/unit.test.ts</t>
+          <t>finance.service.ts pendingApprovals; finance.controller.ts GET approvals/pending (exec/approvals/creditors); aggregates journalEntries(Draft incl. BANKADJ→BANK-02)/apPayments/payruns/asset_revaluations/fixed_assets(disposal_pending)/inv_writeoff_requests/till_sessions(PendingApproval)/fx_rates(PendingApproval)/budgets(PendingApproval); cutover/compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N110" s="12" t="inlineStr">
         <is>
-          <t>Inspect rate provider + tests.</t>
+          <t>Inspect the aggregation across all pending sources + the age/overdue roll-up.</t>
         </is>
       </c>
       <c r="O110" s="12" t="inlineStr">
         <is>
-          <t>Re-perform VAT on sample; tie to return.</t>
+          <t>Re-perform: create a pending item (e.g. a Draft JE) and confirm it appears in the worklist with its control ID, amount and age; the overdue count flags items past the threshold (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P110" s="12" t="inlineStr">
         <is>
-          <t>VAT tests</t>
+          <t>Pending-approvals worklist</t>
         </is>
       </c>
       <c r="Q110" s="18" t="inlineStr">
@@ -10453,7 +10453,7 @@
     <row r="111">
       <c r="A111" s="15" t="inlineStr">
         <is>
-          <t>TAX-02</t>
+          <t>TAX-01</t>
         </is>
       </c>
       <c r="B111" s="16" t="inlineStr">
@@ -10468,22 +10468,22 @@
       </c>
       <c r="D111" s="16" t="inlineStr">
         <is>
-          <t>Tax; Revenue</t>
+          <t>Tax (VAT)</t>
         </is>
       </c>
       <c r="E111" s="16" t="inlineStr">
         <is>
-          <t>Non-compliant e-Tax invoice / not transmitted to ETDA.</t>
+          <t>VAT computed incorrectly → filing/penalty risk.</t>
         </is>
       </c>
       <c r="F111" s="16" t="inlineStr">
         <is>
-          <t>Accuracy/Compliance</t>
+          <t>Accuracy</t>
         </is>
       </c>
       <c r="G111" s="16" t="inlineStr">
         <is>
-          <t>e-Tax invoice (ETDA UBL 2.1 XML) generation + email with CC to ETDA timestamp mailbox.</t>
+          <t>VAT via pluggable provider (TH 7%); unit-tested; no hard-coded rate.</t>
         </is>
       </c>
       <c r="H111" s="17" t="inlineStr">
@@ -10498,37 +10498,37 @@
       </c>
       <c r="J111" s="17" t="inlineStr">
         <is>
-          <t>Per invoice</t>
+          <t>Per txn</t>
         </is>
       </c>
       <c r="K111" s="16" t="inlineStr">
         <is>
-          <t>Tax</t>
+          <t>Tax / Controller</t>
         </is>
       </c>
       <c r="L111" s="17" t="inlineStr">
         <is>
-          <t>P10/P13</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="M111" s="16" t="inlineStr">
         <is>
-          <t>tax-docs/etax-xml.ts; etax-email.service.ts (tested)</t>
+          <t>tax/tax-providers.ts; tax.service.ts; test/unit.test.ts</t>
         </is>
       </c>
       <c r="N111" s="16" t="inlineStr">
         <is>
-          <t>Inspect XML schema + email composer.</t>
+          <t>Inspect rate provider + tests.</t>
         </is>
       </c>
       <c r="O111" s="16" t="inlineStr">
         <is>
-          <t>Sample invoices: valid XML, correct CC/escaping.</t>
+          <t>Re-perform VAT on sample; tie to return.</t>
         </is>
       </c>
       <c r="P111" s="16" t="inlineStr">
         <is>
-          <t>e-Tax samples</t>
+          <t>VAT tests</t>
         </is>
       </c>
       <c r="Q111" s="18" t="inlineStr">
@@ -10540,7 +10540,7 @@
     <row r="112">
       <c r="A112" s="11" t="inlineStr">
         <is>
-          <t>TAX-03</t>
+          <t>TAX-02</t>
         </is>
       </c>
       <c r="B112" s="12" t="inlineStr">
@@ -10555,22 +10555,22 @@
       </c>
       <c r="D112" s="12" t="inlineStr">
         <is>
-          <t>Tax (WHT)</t>
+          <t>Tax; Revenue</t>
         </is>
       </c>
       <c r="E112" s="12" t="inlineStr">
         <is>
-          <t>Withholding tax mis-computed / not reported.</t>
+          <t>Non-compliant e-Tax invoice / not transmitted to ETDA.</t>
         </is>
       </c>
       <c r="F112" s="12" t="inlineStr">
         <is>
-          <t>Accuracy</t>
+          <t>Accuracy/Compliance</t>
         </is>
       </c>
       <c r="G112" s="12" t="inlineStr">
         <is>
-          <t>WHT computation and ภ.ง.ด. reporting.</t>
+          <t>e-Tax invoice (ETDA UBL 2.1 XML) generation + email with CC to ETDA timestamp mailbox.</t>
         </is>
       </c>
       <c r="H112" s="13" t="inlineStr">
@@ -10585,7 +10585,7 @@
       </c>
       <c r="J112" s="13" t="inlineStr">
         <is>
-          <t>Per txn / monthly</t>
+          <t>Per invoice</t>
         </is>
       </c>
       <c r="K112" s="12" t="inlineStr">
@@ -10595,39 +10595,39 @@
       </c>
       <c r="L112" s="13" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P10/P13</t>
         </is>
       </c>
       <c r="M112" s="12" t="inlineStr">
         <is>
-          <t>tax-reports; payroll</t>
+          <t>tax-docs/etax-xml.ts; etax-email.service.ts (tested)</t>
         </is>
       </c>
       <c r="N112" s="12" t="inlineStr">
         <is>
-          <t>Inspect WHT logic + report.</t>
+          <t>Inspect XML schema + email composer.</t>
         </is>
       </c>
       <c r="O112" s="12" t="inlineStr">
         <is>
-          <t>Re-perform WHT on sample; tie to filing.</t>
+          <t>Sample invoices: valid XML, correct CC/escaping.</t>
         </is>
       </c>
       <c r="P112" s="12" t="inlineStr">
         <is>
-          <t>WHT report</t>
-        </is>
-      </c>
-      <c r="Q112" s="19" t="inlineStr">
-        <is>
-          <t>Partial</t>
+          <t>e-Tax samples</t>
+        </is>
+      </c>
+      <c r="Q112" s="18" t="inlineStr">
+        <is>
+          <t>Implemented</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="15" t="inlineStr">
         <is>
-          <t>TAX-04</t>
+          <t>TAX-03</t>
         </is>
       </c>
       <c r="B113" s="16" t="inlineStr">
@@ -10642,27 +10642,27 @@
       </c>
       <c r="D113" s="16" t="inlineStr">
         <is>
-          <t>Tax (VAT); Tax Payable (2100)</t>
+          <t>Tax (WHT)</t>
         </is>
       </c>
       <c r="E113" s="16" t="inlineStr">
         <is>
-          <t>Output/input VAT on the filed ภ.พ.30 return does not agree to the GL — VAT liability mis-stated, a filing/penalty exposure, or a posting omission goes undetected before submission.</t>
+          <t>Withholding tax mis-computed / not reported.</t>
         </is>
       </c>
       <c r="F113" s="16" t="inlineStr">
         <is>
-          <t>Completeness/Accuracy</t>
+          <t>Accuracy</t>
         </is>
       </c>
       <c r="G113" s="16" t="inlineStr">
         <is>
-          <t>Periodic VAT-return ↔ GL reconciliation (ภ.พ.30): the monthly return (GET /api/tax-reports/pp30) is built from the sales/output-VAT and purchase/input-VAT sub-reports, computes net VAT = output − input, and RECONCILES it to the **GL account 2100 (Tax Payable) net movement** for the same period (Σ credit − Σ debit over Posted entries) — returning `reconciliation.tied` = true only when the two agree within rounding. A non-tie is a detective finding to investigate and clear BEFORE filing (the form also carries the ม.157 deadline = the 15th of the next month). Output VAT is posted to 2100 on every sale (Cr) and reversed on returns (Dr); input VAT is posted on AP bills (Dr) — so 2100's net is the period's VAT payable. Read-only report; exportable to a ภ.พ.30 PDF/HTML.</t>
+          <t>WHT computation and ภ.ง.ด. reporting.</t>
         </is>
       </c>
       <c r="H113" s="17" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Auto</t>
         </is>
       </c>
       <c r="I113" s="17" t="inlineStr">
@@ -10672,54 +10672,54 @@
       </c>
       <c r="J113" s="17" t="inlineStr">
         <is>
-          <t>Monthly / pre-filing</t>
+          <t>Per txn / monthly</t>
         </is>
       </c>
       <c r="K113" s="16" t="inlineStr">
         <is>
-          <t>Tax / FinancialController</t>
+          <t>Tax</t>
         </is>
       </c>
       <c r="L113" s="17" t="inlineStr">
         <is>
-          <t>P10/P16</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="M113" s="16" t="inlineStr">
         <is>
-          <t>tax-reports.service.ts pp30 (outputVat/inputVat + 2100 net-movement tie); tax-reports.controller.ts (GET pp30, pp30/export, exec); tax-reports-pdf.ts; dine-in.service.ts/returns.service.ts/finance.service.ts post 2100 on sale/return/AP; /tax/reports UI; cutover/taxdocs.ts (ToE)</t>
+          <t>tax-reports; payroll</t>
         </is>
       </c>
       <c r="N113" s="16" t="inlineStr">
         <is>
-          <t>Inspect the pp30 build + the 2100 net-movement query + the tie flag + the filing deadline.</t>
+          <t>Inspect WHT logic + report.</t>
         </is>
       </c>
       <c r="O113" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: the pp30 return computes net VAT (output − input), the GL 2100 net movement reflects the posted input VAT, and the reconciliation block exposes the gl_account (2100), the report net VAT and a boolean tie verdict (tied iff the two agree within rounding); the ภ.พ.30 export renders (re-performed by the taxdocs harness).</t>
+          <t>Re-perform WHT on sample; tie to filing.</t>
         </is>
       </c>
       <c r="P113" s="16" t="inlineStr">
         <is>
-          <t>ภ.พ.30 return + GL-2100 reconciliation tie</t>
-        </is>
-      </c>
-      <c r="Q113" s="18" t="inlineStr">
-        <is>
-          <t>Implemented</t>
+          <t>WHT report</t>
+        </is>
+      </c>
+      <c r="Q113" s="19" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="11" t="inlineStr">
         <is>
-          <t>PAY-01</t>
+          <t>TAX-04</t>
         </is>
       </c>
       <c r="B114" s="12" t="inlineStr">
         <is>
-          <t>Payroll</t>
+          <t>Tax</t>
         </is>
       </c>
       <c r="C114" s="13" t="inlineStr">
@@ -10729,27 +10729,27 @@
       </c>
       <c r="D114" s="12" t="inlineStr">
         <is>
-          <t>Payroll expense/liability</t>
+          <t>Tax (VAT); Tax Payable (2100)</t>
         </is>
       </c>
       <c r="E114" s="12" t="inlineStr">
         <is>
-          <t>Payroll, SSO and PIT mis-computed.</t>
+          <t>Output/input VAT on the filed ภ.พ.30 return does not agree to the GL — VAT liability mis-stated, a filing/penalty exposure, or a posting omission goes undetected before submission.</t>
         </is>
       </c>
       <c r="F114" s="12" t="inlineStr">
         <is>
-          <t>Accuracy</t>
+          <t>Completeness/Accuracy</t>
         </is>
       </c>
       <c r="G114" s="12" t="inlineStr">
         <is>
-          <t>Payroll engine — SSO 5% (cap 750), progressive PIT, payslip net; unit-tested.</t>
+          <t>Periodic VAT-return ↔ GL reconciliation (ภ.พ.30): the monthly return (GET /api/tax-reports/pp30) is built from the sales/output-VAT and purchase/input-VAT sub-reports, computes net VAT = output − input, and RECONCILES it to the **GL account 2100 (Tax Payable) net movement** for the same period (Σ credit − Σ debit over Posted entries) — returning `reconciliation.tied` = true only when the two agree within rounding. A non-tie is a detective finding to investigate and clear BEFORE filing (the form also carries the ม.157 deadline = the 15th of the next month). Output VAT is posted to 2100 on every sale (Cr) and reversed on returns (Dr); input VAT is posted on AP bills (Dr) — so 2100's net is the period's VAT payable. Read-only report; exportable to a ภ.พ.30 PDF/HTML.</t>
         </is>
       </c>
       <c r="H114" s="13" t="inlineStr">
         <is>
-          <t>Auto</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I114" s="13" t="inlineStr">
@@ -10759,37 +10759,37 @@
       </c>
       <c r="J114" s="13" t="inlineStr">
         <is>
-          <t>Per run</t>
+          <t>Monthly / pre-filing</t>
         </is>
       </c>
       <c r="K114" s="12" t="inlineStr">
         <is>
-          <t>HR / Payroll</t>
+          <t>Tax / FinancialController</t>
         </is>
       </c>
       <c r="L114" s="13" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P10/P16</t>
         </is>
       </c>
       <c r="M114" s="12" t="inlineStr">
         <is>
-          <t>payroll/payroll-calc.ts; test/unit.test.ts</t>
+          <t>tax-reports.service.ts pp30 (outputVat/inputVat + 2100 net-movement tie); tax-reports.controller.ts (GET pp30, pp30/export, exec); tax-reports-pdf.ts; dine-in.service.ts/returns.service.ts/finance.service.ts post 2100 on sale/return/AP; /tax/reports UI; cutover/taxdocs.ts (ToE)</t>
         </is>
       </c>
       <c r="N114" s="12" t="inlineStr">
         <is>
-          <t>Inspect calc + tests.</t>
+          <t>Inspect the pp30 build + the 2100 net-movement query + the tie flag + the filing deadline.</t>
         </is>
       </c>
       <c r="O114" s="12" t="inlineStr">
         <is>
-          <t>Re-perform sample payslips.</t>
+          <t>Re-perform: the pp30 return computes net VAT (output − input), the GL 2100 net movement reflects the posted input VAT, and the reconciliation block exposes the gl_account (2100), the report net VAT and a boolean tie verdict (tied iff the two agree within rounding); the ภ.พ.30 export renders (re-performed by the taxdocs harness).</t>
         </is>
       </c>
       <c r="P114" s="12" t="inlineStr">
         <is>
-          <t>Payslip tests</t>
+          <t>ภ.พ.30 return + GL-2100 reconciliation tie</t>
         </is>
       </c>
       <c r="Q114" s="18" t="inlineStr">
@@ -10801,7 +10801,7 @@
     <row r="115">
       <c r="A115" s="15" t="inlineStr">
         <is>
-          <t>PAY-02</t>
+          <t>PAY-01</t>
         </is>
       </c>
       <c r="B115" s="16" t="inlineStr">
@@ -10816,27 +10816,27 @@
       </c>
       <c r="D115" s="16" t="inlineStr">
         <is>
-          <t>Payroll liability</t>
+          <t>Payroll expense/liability</t>
         </is>
       </c>
       <c r="E115" s="16" t="inlineStr">
         <is>
-          <t>Statutory withholdings (SSO/WHT/PF) mis-stated or not remitted, so the liability owed to the authorities diverges from the books.</t>
+          <t>Payroll, SSO and PIT mis-computed.</t>
         </is>
       </c>
       <c r="F115" s="16" t="inlineStr">
         <is>
-          <t>Accuracy/Compliance</t>
+          <t>Accuracy</t>
         </is>
       </c>
       <c r="G115" s="16" t="inlineStr">
         <is>
-          <t>Payroll-liability schedule (GET /api/payroll/liabilities): each statutory account — SSO 2350, WHT/PND1 2360, PF 2370 — shows accrued (GL credits) − remitted (GL debits) = outstanding, tied back to the INDEPENDENT payrun accrual with a `reconciled` flag (a divergence flags a manual JE that touched a payroll-liability account outside the payroll process). Treasury remits the cash (POST .../remit → Dr liability / Cr 1000) which clears the outstanding and keeps the books reconciled to the statutory filings; a remittance beyond the outstanding is blocked (REMIT_EXCEEDS_OUTSTANDING).</t>
+          <t>Payroll engine — SSO 5% (cap 750), progressive PIT, payslip net; unit-tested.</t>
         </is>
       </c>
       <c r="H115" s="17" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Auto</t>
         </is>
       </c>
       <c r="I115" s="17" t="inlineStr">
@@ -10846,12 +10846,12 @@
       </c>
       <c r="J115" s="17" t="inlineStr">
         <is>
-          <t>Per run / monthly</t>
+          <t>Per run</t>
         </is>
       </c>
       <c r="K115" s="16" t="inlineStr">
         <is>
-          <t>HR / Payroll / Treasury</t>
+          <t>HR / Payroll</t>
         </is>
       </c>
       <c r="L115" s="17" t="inlineStr">
@@ -10861,22 +10861,22 @@
       </c>
       <c r="M115" s="16" t="inlineStr">
         <is>
-          <t>payroll/payroll.service.ts liabilities/remitLiability</t>
+          <t>payroll/payroll-calc.ts; test/unit.test.ts</t>
         </is>
       </c>
       <c r="N115" s="16" t="inlineStr">
         <is>
-          <t>Inspect the schedule + the accrued/remitted/outstanding tie-out and the reconciled flag.</t>
+          <t>Inspect calc + tests.</t>
         </is>
       </c>
       <c r="O115" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: run a payroll, confirm the SSO/WHT outstanding equals the payrun accrual; remit part and confirm the outstanding falls and the TB stays balanced; attempt an over-remit (REMIT_EXCEEDS_OUTSTANDING).</t>
+          <t>Re-perform sample payslips.</t>
         </is>
       </c>
       <c r="P115" s="16" t="inlineStr">
         <is>
-          <t>Liability schedule + remittance JEs tied to filings</t>
+          <t>Payslip tests</t>
         </is>
       </c>
       <c r="Q115" s="18" t="inlineStr">
@@ -10888,7 +10888,7 @@
     <row r="116">
       <c r="A116" s="11" t="inlineStr">
         <is>
-          <t>PAY-03</t>
+          <t>PAY-02</t>
         </is>
       </c>
       <c r="B116" s="12" t="inlineStr">
@@ -10903,27 +10903,27 @@
       </c>
       <c r="D116" s="12" t="inlineStr">
         <is>
-          <t>Payroll expense/liability; Cash</t>
+          <t>Payroll liability</t>
         </is>
       </c>
       <c r="E116" s="12" t="inlineStr">
         <is>
-          <t>Payroll run posted to the GL without independent review — the preparer both computes and posts their own payroll (ghost employees, inflated rate/hours).</t>
+          <t>Statutory withholdings (SSO/WHT/PF) mis-stated or not remitted, so the liability owed to the authorities diverges from the books.</t>
         </is>
       </c>
       <c r="F116" s="12" t="inlineStr">
         <is>
-          <t>Authorization</t>
+          <t>Accuracy/Compliance</t>
         </is>
       </c>
       <c r="G116" s="12" t="inlineStr">
         <is>
-          <t>Payroll maker-checker (SoD): a run posts its GL entry as a DRAFT (excluded from balances) with the run record 'PendingApproval'; a DIFFERENT user must approve before it becomes effective (approver ≠ preparer enforced regardless of permissions, reusing the GL-05 ledger approval). Reject voids the draft; idempotent per (tenant, period).</t>
+          <t>Payroll-liability schedule (GET /api/payroll/liabilities): each statutory account — SSO 2350, WHT/PND1 2360, PF 2370 — shows accrued (GL credits) − remitted (GL debits) = outstanding, tied back to the INDEPENDENT payrun accrual with a `reconciled` flag (a divergence flags a manual JE that touched a payroll-liability account outside the payroll process). Treasury remits the cash (POST .../remit → Dr liability / Cr 1000) which clears the outstanding and keeps the books reconciled to the statutory filings; a remittance beyond the outstanding is blocked (REMIT_EXCEEDS_OUTSTANDING).</t>
         </is>
       </c>
       <c r="H116" s="13" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I116" s="13" t="inlineStr">
@@ -10933,12 +10933,12 @@
       </c>
       <c r="J116" s="13" t="inlineStr">
         <is>
-          <t>Per run</t>
+          <t>Per run / monthly</t>
         </is>
       </c>
       <c r="K116" s="12" t="inlineStr">
         <is>
-          <t>HR / Payroll; Controller</t>
+          <t>HR / Payroll / Treasury</t>
         </is>
       </c>
       <c r="L116" s="13" t="inlineStr">
@@ -10948,22 +10948,22 @@
       </c>
       <c r="M116" s="12" t="inlineStr">
         <is>
-          <t>payroll/payroll.service.ts approvePayroll/rejectPayroll; migration 0133</t>
+          <t>payroll/payroll.service.ts liabilities/remitLiability</t>
         </is>
       </c>
       <c r="N116" s="12" t="inlineStr">
         <is>
-          <t>Inspect Draft→approve flow + the approver≠preparer check.</t>
+          <t>Inspect the schedule + the accrued/remitted/outstanding tie-out and the reconciled flag.</t>
         </is>
       </c>
       <c r="O116" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: run as A, attempt self-approve (SOD_VIOLATION), approve as B; confirm the JE hits balances only after approval.</t>
+          <t>Re-perform: run a payroll, confirm the SSO/WHT outstanding equals the payrun accrual; remit part and confirm the outstanding falls and the TB stays balanced; attempt an over-remit (REMIT_EXCEEDS_OUTSTANDING).</t>
         </is>
       </c>
       <c r="P116" s="12" t="inlineStr">
         <is>
-          <t>Approval log + SoD test</t>
+          <t>Liability schedule + remittance JEs tied to filings</t>
         </is>
       </c>
       <c r="Q116" s="18" t="inlineStr">
@@ -10975,12 +10975,12 @@
     <row r="117">
       <c r="A117" s="15" t="inlineStr">
         <is>
-          <t>FA-09</t>
+          <t>PAY-03</t>
         </is>
       </c>
       <c r="B117" s="16" t="inlineStr">
         <is>
-          <t>Fixed Assets</t>
+          <t>Payroll</t>
         </is>
       </c>
       <c r="C117" s="17" t="inlineStr">
@@ -10990,12 +10990,12 @@
       </c>
       <c r="D117" s="16" t="inlineStr">
         <is>
-          <t>Property, Plant &amp; Equipment; Cash</t>
+          <t>Payroll expense/liability; Cash</t>
         </is>
       </c>
       <c r="E117" s="16" t="inlineStr">
         <is>
-          <t>Asset disposed without independent review — one person writes an asset off the books and records the proceeds (asset-stripping / theft: dispose a still-held asset, or to a related party below value).</t>
+          <t>Payroll run posted to the GL without independent review — the preparer both computes and posts their own payroll (ghost employees, inflated rate/hours).</t>
         </is>
       </c>
       <c r="F117" s="16" t="inlineStr">
@@ -11005,7 +11005,7 @@
       </c>
       <c r="G117" s="16" t="inlineStr">
         <is>
-          <t>Asset-disposal maker-checker (SoD): a disposal REQUEST posts its GL entry as a DRAFT (excluded from balances) and flags the asset disposal_pending WITHOUT marking it disposed or moving the register; a DIFFERENT user must approve before it is effective (status→disposed, revaluation surplus recycled 3200→3100) (approver ≠ requester enforced regardless of permissions, reusing the GL-05 ledger approval). Reject voids the draft and the asset stays in service; only one disposal may be pending per asset; a disposal-pending asset is frozen from depreciation.</t>
+          <t>Payroll maker-checker (SoD): a run posts its GL entry as a DRAFT (excluded from balances) with the run record 'PendingApproval'; a DIFFERENT user must approve before it becomes effective (approver ≠ preparer enforced regardless of permissions, reusing the GL-05 ledger approval). Reject voids the draft; idempotent per (tenant, period).</t>
         </is>
       </c>
       <c r="H117" s="17" t="inlineStr">
@@ -11020,12 +11020,12 @@
       </c>
       <c r="J117" s="17" t="inlineStr">
         <is>
-          <t>Per disposal</t>
+          <t>Per run</t>
         </is>
       </c>
       <c r="K117" s="16" t="inlineStr">
         <is>
-          <t>FaAccountant / Controller</t>
+          <t>HR / Payroll; Controller</t>
         </is>
       </c>
       <c r="L117" s="17" t="inlineStr">
@@ -11035,22 +11035,22 @@
       </c>
       <c r="M117" s="16" t="inlineStr">
         <is>
-          <t>assets.service.ts dispose(pendingApproval Draft)/approveDisposal/rejectDisposal; assets.controller.ts (:assetNo/dispose/approve|reject); schema/assets.ts fixed_assets.disposal_pending + migration 0135; cutover/basics.ts + worldclass.ts + compliance.ts (ToE)</t>
+          <t>payroll/payroll.service.ts approvePayroll/rejectPayroll; migration 0133</t>
         </is>
       </c>
       <c r="N117" s="16" t="inlineStr">
         <is>
-          <t>Inspect Draft→approve flow + the approver≠requester check + deferred status/recycle.</t>
+          <t>Inspect Draft→approve flow + the approver≠preparer check.</t>
         </is>
       </c>
       <c r="O117" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: request a disposal (Draft JE excluded), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm status→disposed + surplus recycled only after approval (re-performed by the harnesses).</t>
+          <t>Re-perform: run as A, attempt self-approve (SOD_VIOLATION), approve as B; confirm the JE hits balances only after approval.</t>
         </is>
       </c>
       <c r="P117" s="16" t="inlineStr">
         <is>
-          <t>Disposal approval log + SoD test</t>
+          <t>Approval log + SoD test</t>
         </is>
       </c>
       <c r="Q117" s="18" t="inlineStr">
@@ -11062,7 +11062,7 @@
     <row r="118">
       <c r="A118" s="11" t="inlineStr">
         <is>
-          <t>FA-10</t>
+          <t>FA-09</t>
         </is>
       </c>
       <c r="B118" s="12" t="inlineStr">
@@ -11077,22 +11077,22 @@
       </c>
       <c r="D118" s="12" t="inlineStr">
         <is>
-          <t>Property, Plant &amp; Equipment; Accounts Payable</t>
+          <t>Property, Plant &amp; Equipment; Cash</t>
         </is>
       </c>
       <c r="E118" s="12" t="inlineStr">
         <is>
-          <t>Capital purchases mis-capitalised or capitalised without independent review — the person who receives the goods also decides what enters the asset register and at what cost/useful life (fictitious or over-valued assets; capex/opex mis-classification).</t>
+          <t>Asset disposed without independent review — one person writes an asset off the books and records the proceeds (asset-stripping / theft: dispose a still-held asset, or to a related party below value).</t>
         </is>
       </c>
       <c r="F118" s="12" t="inlineStr">
         <is>
-          <t>Authorization; Accuracy</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="G118" s="12" t="inlineStr">
         <is>
-          <t>Procure-to-Capitalize maker-checker (SoD): a goods-receipt line flagged capital (item-master is_fixed_asset or per-PO-line override) is excluded from inventory capitalisation (1200) at receipt and instead becomes ELIGIBLE for the asset register. Capitalisation is a REQUEST that posts NOTHING to the GL; a DIFFERENT user must approve before the fixed_assets row + acquisition JE (Dr 1500 / Cr 2000) are created (approver ≠ requester enforced regardless of permissions). The created asset carries its source GR/PO for end-to-end PR→PO→GR→FA traceability; a GR line cannot be capitalised twice.</t>
+          <t>Asset-disposal maker-checker (SoD): a disposal REQUEST posts its GL entry as a DRAFT (excluded from balances) and flags the asset disposal_pending WITHOUT marking it disposed or moving the register; a DIFFERENT user must approve before it is effective (status→disposed, revaluation surplus recycled 3200→3100) (approver ≠ requester enforced regardless of permissions, reusing the GL-05 ledger approval). Reject voids the draft and the asset stays in service; only one disposal may be pending per asset; a disposal-pending asset is frozen from depreciation.</t>
         </is>
       </c>
       <c r="H118" s="13" t="inlineStr">
@@ -11107,7 +11107,7 @@
       </c>
       <c r="J118" s="13" t="inlineStr">
         <is>
-          <t>Per capital receipt</t>
+          <t>Per disposal</t>
         </is>
       </c>
       <c r="K118" s="12" t="inlineStr">
@@ -11122,22 +11122,22 @@
       </c>
       <c r="M118" s="12" t="inlineStr">
         <is>
-          <t>assets.service.ts registerFromGr/approveRegistration/rejectRegistration/eligibleFromGr; assets.controller.ts (registrations*); procurement.service.ts createGr (is_capital routing, costing excluded); schema/assets.ts asset_registration_requests + fixed_assets.source_gr_no/po_no + migration 0137; cutover/basics.ts + compliance.ts (ToE)</t>
+          <t>assets.service.ts dispose(pendingApproval Draft)/approveDisposal/rejectDisposal; assets.controller.ts (:assetNo/dispose/approve|reject); schema/assets.ts fixed_assets.disposal_pending + migration 0135; cutover/basics.ts + worldclass.ts + compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N118" s="12" t="inlineStr">
         <is>
-          <t>Inspect the eligible→request→approve flow + approver≠requester check + the inventory-vs-asset routing of capital lines.</t>
+          <t>Inspect Draft→approve flow + the approver≠requester check + deferred status/recycle.</t>
         </is>
       </c>
       <c r="O118" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: receive a capital line, raise a registration (no GL), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm the asset + Dr 1500/Cr 2000 post only after approval and the line cannot be re-registered (re-performed by the harnesses).</t>
+          <t>Re-perform: request a disposal (Draft JE excluded), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm status→disposed + surplus recycled only after approval (re-performed by the harnesses).</t>
         </is>
       </c>
       <c r="P118" s="12" t="inlineStr">
         <is>
-          <t>Capitalization approval log + SoD test</t>
+          <t>Disposal approval log + SoD test</t>
         </is>
       </c>
       <c r="Q118" s="18" t="inlineStr">
@@ -11149,12 +11149,12 @@
     <row r="119">
       <c r="A119" s="15" t="inlineStr">
         <is>
-          <t>CON-01</t>
+          <t>FA-10</t>
         </is>
       </c>
       <c r="B119" s="16" t="inlineStr">
         <is>
-          <t>Consolidation &amp; FX</t>
+          <t>Fixed Assets</t>
         </is>
       </c>
       <c r="C119" s="17" t="inlineStr">
@@ -11164,42 +11164,42 @@
       </c>
       <c r="D119" s="16" t="inlineStr">
         <is>
-          <t>Consolidation</t>
+          <t>Property, Plant &amp; Equipment; Accounts Payable</t>
         </is>
       </c>
       <c r="E119" s="16" t="inlineStr">
         <is>
-          <t>Group consolidation mis-stated (ownership/currency).</t>
+          <t>Capital purchases mis-capitalised or capitalised without independent review — the person who receives the goods also decides what enters the asset register and at what cost/useful life (fictitious or over-valued assets; capex/opex mis-classification).</t>
         </is>
       </c>
       <c r="F119" s="16" t="inlineStr">
         <is>
-          <t>Accuracy</t>
+          <t>Authorization; Accuracy</t>
         </is>
       </c>
       <c r="G119" s="16" t="inlineStr">
         <is>
-          <t>Consolidation run (ownership %, entity currency) gated by 'approvals'.</t>
+          <t>Procure-to-Capitalize maker-checker (SoD): a goods-receipt line flagged capital (item-master is_fixed_asset or per-PO-line override) is excluded from inventory capitalisation (1200) at receipt and instead becomes ELIGIBLE for the asset register. Capitalisation is a REQUEST that posts NOTHING to the GL; a DIFFERENT user must approve before the fixed_assets row + acquisition JE (Dr 1500 / Cr 2000) are created (approver ≠ requester enforced regardless of permissions). The created asset carries its source GR/PO for end-to-end PR→PO→GR→FA traceability; a GR line cannot be capitalised twice.</t>
         </is>
       </c>
       <c r="H119" s="17" t="inlineStr">
         <is>
-          <t>Auto+Manual</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I119" s="17" t="inlineStr">
         <is>
-          <t>Period</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J119" s="17" t="inlineStr">
         <is>
-          <t>Period</t>
+          <t>Per capital receipt</t>
         </is>
       </c>
       <c r="K119" s="16" t="inlineStr">
         <is>
-          <t>Group Controller</t>
+          <t>FaAccountant / Controller</t>
         </is>
       </c>
       <c r="L119" s="17" t="inlineStr">
@@ -11209,22 +11209,22 @@
       </c>
       <c r="M119" s="16" t="inlineStr">
         <is>
-          <t>consolidation.service.ts (runConsolidation @Permissions approvals)</t>
+          <t>assets.service.ts registerFromGr/approveRegistration/rejectRegistration/eligibleFromGr; assets.controller.ts (registrations*); procurement.service.ts createGr (is_capital routing, costing excluded); schema/assets.ts asset_registration_requests + fixed_assets.source_gr_no/po_no + migration 0137; cutover/basics.ts + compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N119" s="16" t="inlineStr">
         <is>
-          <t>Inspect consolidation logic + gate.</t>
+          <t>Inspect the eligible→request→approve flow + approver≠requester check + the inventory-vs-asset routing of capital lines.</t>
         </is>
       </c>
       <c r="O119" s="16" t="inlineStr">
         <is>
-          <t>Sample period: consolidated TB ties to entities.</t>
+          <t>Re-perform: receive a capital line, raise a registration (no GL), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm the asset + Dr 1500/Cr 2000 post only after approval and the line cannot be re-registered (re-performed by the harnesses).</t>
         </is>
       </c>
       <c r="P119" s="16" t="inlineStr">
         <is>
-          <t>Consol TB</t>
+          <t>Capitalization approval log + SoD test</t>
         </is>
       </c>
       <c r="Q119" s="18" t="inlineStr">
@@ -11236,7 +11236,7 @@
     <row r="120">
       <c r="A120" s="11" t="inlineStr">
         <is>
-          <t>CON-02</t>
+          <t>CON-01</t>
         </is>
       </c>
       <c r="B120" s="12" t="inlineStr">
@@ -11251,22 +11251,22 @@
       </c>
       <c r="D120" s="12" t="inlineStr">
         <is>
-          <t>FX gain/loss</t>
+          <t>Consolidation</t>
         </is>
       </c>
       <c r="E120" s="12" t="inlineStr">
         <is>
-          <t>FX exposures not revalued at period-end.</t>
+          <t>Group consolidation mis-stated (ownership/currency).</t>
         </is>
       </c>
       <c r="F120" s="12" t="inlineStr">
         <is>
-          <t>Valuation</t>
+          <t>Accuracy</t>
         </is>
       </c>
       <c r="G120" s="12" t="inlineStr">
         <is>
-          <t>FX revaluation at period-end rates; unrealized FX posted (acct 5400).</t>
+          <t>Consolidation run (ownership %, entity currency) gated by 'approvals'.</t>
         </is>
       </c>
       <c r="H120" s="13" t="inlineStr">
@@ -11276,7 +11276,7 @@
       </c>
       <c r="I120" s="13" t="inlineStr">
         <is>
-          <t>Period-end</t>
+          <t>Period</t>
         </is>
       </c>
       <c r="J120" s="13" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="K120" s="12" t="inlineStr">
         <is>
-          <t>Controller</t>
+          <t>Group Controller</t>
         </is>
       </c>
       <c r="L120" s="13" t="inlineStr">
@@ -11296,22 +11296,22 @@
       </c>
       <c r="M120" s="12" t="inlineStr">
         <is>
-          <t>fx.service.ts (revalue / unrealized report)</t>
+          <t>consolidation.service.ts (runConsolidation @Permissions approvals)</t>
         </is>
       </c>
       <c r="N120" s="12" t="inlineStr">
         <is>
-          <t>Inspect reval logic + rates.</t>
+          <t>Inspect consolidation logic + gate.</t>
         </is>
       </c>
       <c r="O120" s="12" t="inlineStr">
         <is>
-          <t>Recompute reval on sample balances.</t>
+          <t>Sample period: consolidated TB ties to entities.</t>
         </is>
       </c>
       <c r="P120" s="12" t="inlineStr">
         <is>
-          <t>FX reval JE</t>
+          <t>Consol TB</t>
         </is>
       </c>
       <c r="Q120" s="18" t="inlineStr">
@@ -11323,7 +11323,7 @@
     <row r="121">
       <c r="A121" s="15" t="inlineStr">
         <is>
-          <t>FX-04</t>
+          <t>CON-02</t>
         </is>
       </c>
       <c r="B121" s="16" t="inlineStr">
@@ -11338,42 +11338,42 @@
       </c>
       <c r="D121" s="16" t="inlineStr">
         <is>
-          <t>FX gain/loss; Revenue; AR/AP</t>
+          <t>FX gain/loss</t>
         </is>
       </c>
       <c r="E121" s="16" t="inlineStr">
         <is>
-          <t>A wrong manually-entered FX rate (fat-fingered, e.g. USD 36 keyed as 63) flows straight into a period-end revaluation JE and the unrealized-FX report with no independent review — mis-stating earnings/equity and FX-translated balances.</t>
+          <t>FX exposures not revalued at period-end.</t>
         </is>
       </c>
       <c r="F121" s="16" t="inlineStr">
         <is>
-          <t>Accuracy/Valuation</t>
+          <t>Valuation</t>
         </is>
       </c>
       <c r="G121" s="16" t="inlineStr">
         <is>
-          <t>FX rate maker-checker (SoD): a MANUALLY-entered rate lands as PendingApproval and is EXCLUDED from rate resolution — revaluation, the unrealized-FX report, and consolidation translation all use APPROVED rates only — until a DIFFERENT user approves it (POST /api/fx/rates/approve). Self-approval → SOD_VIOLATION (binds even Admin); reject marks the rate Rejected (never usable); re-entering a rate sends it back to PendingApproval. Externally-sourced (feed) rates carrying an explicit non-manual source are auto-approved. Pending rates are also surfaced, aged, by the pending-approvals monitor (GOV-01).</t>
+          <t>FX revaluation at period-end rates; unrealized FX posted (acct 5400).</t>
         </is>
       </c>
       <c r="H121" s="17" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="I121" s="17" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Period-end</t>
         </is>
       </c>
       <c r="J121" s="17" t="inlineStr">
         <is>
-          <t>Per rate</t>
+          <t>Period</t>
         </is>
       </c>
       <c r="K121" s="16" t="inlineStr">
         <is>
-          <t>Controller / Treasury</t>
+          <t>Controller</t>
         </is>
       </c>
       <c r="L121" s="17" t="inlineStr">
@@ -11383,22 +11383,22 @@
       </c>
       <c r="M121" s="16" t="inlineStr">
         <is>
-          <t>fx.service.ts setRate(manual→PendingApproval)/approveRate/rejectRate/rateAsOf(Approved only); fx.controller.ts (rates/approve|reject|pending gated approvals/gl_close); consolidation.service.ts (translation reads Approved rates); schema/fx.ts fx_rates.status + migration 0141; cutover/fxreval.ts (ToE)</t>
+          <t>fx.service.ts (revalue / unrealized report)</t>
         </is>
       </c>
       <c r="N121" s="16" t="inlineStr">
         <is>
-          <t>Inspect the request→approve flow + the approver≠requester check + that revaluation/reporting resolve Approved rates only.</t>
+          <t>Inspect reval logic + rates.</t>
         </is>
       </c>
       <c r="O121" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: enter a manual rate (PendingApproval), confirm revalue is blocked NO_RATE while pending, attempt self-approve (SOD_VIOLATION), approve as a different user, then revalue succeeds (re-performed by the fxreval harness).</t>
+          <t>Recompute reval on sample balances.</t>
         </is>
       </c>
       <c r="P121" s="16" t="inlineStr">
         <is>
-          <t>FX rate approval log + SoD test</t>
+          <t>FX reval JE</t>
         </is>
       </c>
       <c r="Q121" s="18" t="inlineStr">
@@ -11410,92 +11410,179 @@
     <row r="122">
       <c r="A122" s="11" t="inlineStr">
         <is>
+          <t>FX-04</t>
+        </is>
+      </c>
+      <c r="B122" s="12" t="inlineStr">
+        <is>
+          <t>Consolidation &amp; FX</t>
+        </is>
+      </c>
+      <c r="C122" s="13" t="inlineStr">
+        <is>
+          <t>Application</t>
+        </is>
+      </c>
+      <c r="D122" s="12" t="inlineStr">
+        <is>
+          <t>FX gain/loss; Revenue; AR/AP</t>
+        </is>
+      </c>
+      <c r="E122" s="12" t="inlineStr">
+        <is>
+          <t>A wrong manually-entered FX rate (fat-fingered, e.g. USD 36 keyed as 63) flows straight into a period-end revaluation JE and the unrealized-FX report with no independent review — mis-stating earnings/equity and FX-translated balances.</t>
+        </is>
+      </c>
+      <c r="F122" s="12" t="inlineStr">
+        <is>
+          <t>Accuracy/Valuation</t>
+        </is>
+      </c>
+      <c r="G122" s="12" t="inlineStr">
+        <is>
+          <t>FX rate maker-checker (SoD): a MANUALLY-entered rate lands as PendingApproval and is EXCLUDED from rate resolution — revaluation, the unrealized-FX report, and consolidation translation all use APPROVED rates only — until a DIFFERENT user approves it (POST /api/fx/rates/approve). Self-approval → SOD_VIOLATION (binds even Admin); reject marks the rate Rejected (never usable); re-entering a rate sends it back to PendingApproval. Externally-sourced (feed) rates carrying an explicit non-manual source are auto-approved. Pending rates are also surfaced, aged, by the pending-approvals monitor (GOV-01).</t>
+        </is>
+      </c>
+      <c r="H122" s="13" t="inlineStr">
+        <is>
+          <t>Prev</t>
+        </is>
+      </c>
+      <c r="I122" s="13" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="J122" s="13" t="inlineStr">
+        <is>
+          <t>Per rate</t>
+        </is>
+      </c>
+      <c r="K122" s="12" t="inlineStr">
+        <is>
+          <t>Controller / Treasury</t>
+        </is>
+      </c>
+      <c r="L122" s="13" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="M122" s="12" t="inlineStr">
+        <is>
+          <t>fx.service.ts setRate(manual→PendingApproval)/approveRate/rejectRate/rateAsOf(Approved only); fx.controller.ts (rates/approve|reject|pending gated approvals/gl_close); consolidation.service.ts (translation reads Approved rates); schema/fx.ts fx_rates.status + migration 0141; cutover/fxreval.ts (ToE)</t>
+        </is>
+      </c>
+      <c r="N122" s="12" t="inlineStr">
+        <is>
+          <t>Inspect the request→approve flow + the approver≠requester check + that revaluation/reporting resolve Approved rates only.</t>
+        </is>
+      </c>
+      <c r="O122" s="12" t="inlineStr">
+        <is>
+          <t>Re-perform: enter a manual rate (PendingApproval), confirm revalue is blocked NO_RATE while pending, attempt self-approve (SOD_VIOLATION), approve as a different user, then revalue succeeds (re-performed by the fxreval harness).</t>
+        </is>
+      </c>
+      <c r="P122" s="12" t="inlineStr">
+        <is>
+          <t>FX rate approval log + SoD test</t>
+        </is>
+      </c>
+      <c r="Q122" s="18" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="15" t="inlineStr">
+        <is>
           <t>BUD-01</t>
         </is>
       </c>
-      <c r="B122" s="12" t="inlineStr">
+      <c r="B123" s="16" t="inlineStr">
         <is>
           <t>Budgeting &amp; Planning</t>
         </is>
       </c>
-      <c r="C122" s="13" t="inlineStr">
+      <c r="C123" s="17" t="inlineStr">
         <is>
           <t>Application</t>
         </is>
       </c>
-      <c r="D122" s="12" t="inlineStr">
+      <c r="D123" s="16" t="inlineStr">
         <is>
           <t>Budget; All (variance reporting)</t>
         </is>
       </c>
-      <c r="E122" s="12" t="inlineStr">
+      <c r="E123" s="16" t="inlineStr">
         <is>
           <t>A budget figure is entered/changed by one person and immediately drives the budget-vs-actual variance report — the basis for spend authorization and performance review — with no independent approval; a wrong or self-serving budget makes overspending look 'on budget'.</t>
         </is>
       </c>
-      <c r="F122" s="12" t="inlineStr">
+      <c r="F123" s="16" t="inlineStr">
         <is>
           <t>Authorization/Accuracy</t>
         </is>
       </c>
-      <c r="G122" s="12" t="inlineStr">
+      <c r="G123" s="16" t="inlineStr">
         <is>
           <t>Budget maker-checker (SoD): an upserted budget (POST /api/ledger/budgets) lands as PendingApproval and is EXCLUDED from budget-vs-actual until a DIFFERENT user approves it (POST /api/ledger/budgets/approve for the fiscal_year/account/cost-centre[/period]). Self-approval → SOD_VIOLATION (binds even Admin); reject marks it Rejected (excluded). DEFAULT 'Approved' keeps existing rows + direct planning seeds usable. Pending budgets are also surfaced, aged, by the pending-approvals monitor (GOV-01).</t>
         </is>
       </c>
-      <c r="H122" s="13" t="inlineStr">
+      <c r="H123" s="17" t="inlineStr">
         <is>
           <t>Prev</t>
         </is>
       </c>
-      <c r="I122" s="13" t="inlineStr">
+      <c r="I123" s="17" t="inlineStr">
         <is>
           <t>Automated</t>
         </is>
       </c>
-      <c r="J122" s="13" t="inlineStr">
+      <c r="J123" s="17" t="inlineStr">
         <is>
           <t>Per budget</t>
         </is>
       </c>
-      <c r="K122" s="12" t="inlineStr">
+      <c r="K123" s="16" t="inlineStr">
         <is>
           <t>Controller / FP&amp;A</t>
         </is>
       </c>
-      <c r="L122" s="13" t="inlineStr">
+      <c r="L123" s="17" t="inlineStr">
         <is>
           <t>P10</t>
         </is>
       </c>
-      <c r="M122" s="12" t="inlineStr">
+      <c r="M123" s="16" t="inlineStr">
         <is>
           <t>budget.service.ts upsertBudget(→PendingApproval)/approveBudget/rejectBudget/budgetVsActual(Approved only); budget.controller.ts (budgets/approve|reject|pending gated approvals/gl_close); schema/budgets.ts budgets.status + migration 0142; cutover/budget.ts (ToE)</t>
         </is>
       </c>
-      <c r="N122" s="12" t="inlineStr">
+      <c r="N123" s="16" t="inlineStr">
         <is>
           <t>Inspect the request→approve flow + the approver≠requester check + that budget-vs-actual counts Approved budgets only.</t>
         </is>
       </c>
-      <c r="O122" s="12" t="inlineStr">
+      <c r="O123" s="16" t="inlineStr">
         <is>
           <t>Re-perform: upsert a budget (PendingApproval, excluded from variance), attempt self-approve (SOD_VIOLATION), approve as a different user, confirm it then appears in budget-vs-actual (re-performed by the budget harness).</t>
         </is>
       </c>
-      <c r="P122" s="12" t="inlineStr">
+      <c r="P123" s="16" t="inlineStr">
         <is>
           <t>Budget approval log + SoD test</t>
         </is>
       </c>
-      <c r="Q122" s="18" t="inlineStr">
+      <c r="Q123" s="18" t="inlineStr">
         <is>
           <t>Implemented</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q122"/>
+  <autoFilter ref="A1:Q123"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -12678,7 +12765,7 @@
         </is>
       </c>
       <c r="C5" s="29">
-        <f>COUNTIF(RCM!$Q$2:$Q$122,B5)</f>
+        <f>COUNTIF(RCM!$Q$2:$Q$123,B5)</f>
         <v/>
       </c>
     </row>
@@ -12689,7 +12776,7 @@
         </is>
       </c>
       <c r="C6" s="29">
-        <f>COUNTIF(RCM!$Q$2:$Q$122,B6)</f>
+        <f>COUNTIF(RCM!$Q$2:$Q$123,B6)</f>
         <v/>
       </c>
     </row>
@@ -12700,7 +12787,7 @@
         </is>
       </c>
       <c r="C7" s="29">
-        <f>COUNTIF(RCM!$Q$2:$Q$122,B7)</f>
+        <f>COUNTIF(RCM!$Q$2:$Q$123,B7)</f>
         <v/>
       </c>
     </row>
@@ -12711,7 +12798,7 @@
         </is>
       </c>
       <c r="C8" s="32">
-        <f>COUNTA(RCM!$A$2:$A$122)</f>
+        <f>COUNTA(RCM!$A$2:$A$123)</f>
         <v/>
       </c>
     </row>
@@ -12729,7 +12816,7 @@
         </is>
       </c>
       <c r="C11" s="29">
-        <f>COUNTIF(RCM!$C$2:$C$122,B11)</f>
+        <f>COUNTIF(RCM!$C$2:$C$123,B11)</f>
         <v/>
       </c>
     </row>
@@ -12740,7 +12827,7 @@
         </is>
       </c>
       <c r="C12" s="29">
-        <f>COUNTIF(RCM!$C$2:$C$122,B12)</f>
+        <f>COUNTIF(RCM!$C$2:$C$123,B12)</f>
         <v/>
       </c>
     </row>
@@ -12751,7 +12838,7 @@
         </is>
       </c>
       <c r="C13" s="29">
-        <f>COUNTIF(RCM!$C$2:$C$122,B13)</f>
+        <f>COUNTIF(RCM!$C$2:$C$123,B13)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: merge main, renumber gl_immutability 0164→0165 (branch_lead_time took 0164)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/compliance/Oshinei_ERP_SOX_RCM_v1.xlsx
+++ b/compliance/Oshinei_ERP_SOX_RCM_v1.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'RCM'!$A$1:$Q$123</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'RCM'!$A$1:$Q$124</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Gap Remediation'!$A$2:$H$18</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -858,7 +858,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q123"/>
+  <dimension ref="A1:Q124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -7147,12 +7147,12 @@
     <row r="73">
       <c r="A73" s="15" t="inlineStr">
         <is>
-          <t>BRANCH-01</t>
+          <t>INV-12</t>
         </is>
       </c>
       <c r="B73" s="16" t="inlineStr">
         <is>
-          <t>Multi-Branch &amp; Offline POS</t>
+          <t>Inventory &amp; COGS</t>
         </is>
       </c>
       <c r="C73" s="17" t="inlineStr">
@@ -7162,22 +7162,22 @@
       </c>
       <c r="D73" s="16" t="inlineStr">
         <is>
-          <t>Revenue</t>
+          <t>Inventory</t>
         </is>
       </c>
       <c r="E73" s="16" t="inlineStr">
         <is>
-          <t>A POS sale is not attributed to its originating branch, so the consolidated branch roll-up is incomplete and cannot be tied to GL revenue.</t>
+          <t>Per-branch reorder points are STATIC numbers — set once and never revisited — so a branch whose run-rate has grown carries too small a buffer and stocks out (lost sales), while a slow branch over-orders and ties up cash/spoils stock; neither is flagged.</t>
         </is>
       </c>
       <c r="F73" s="16" t="inlineStr">
         <is>
-          <t>Completeness</t>
+          <t>Accuracy/Completeness</t>
         </is>
       </c>
       <c r="G73" s="16" t="inlineStr">
         <is>
-          <t>Branch sale-tagging + HQ consolidation: every POS sale carries cust_pos_sales.branch_id; GET /api/branches/consolidated aggregates per branch (excluding Voided) and surfaces untagged sales as branch '(none)' — a deliberate completeness flag the controller investigates and clears before tying the consolidated total to GL revenue.</t>
+          <t>Demand-driven par-level recommendation (layered on the INV-05 branch min-max + transfer-before-buy): for each (branch,item) the system derives the average daily usage from the trailing window of branch-tagged consumption (cust_stock_log Sale/Consume) and recommends reorder_point = ceil(avg_daily x lead_time_days x safety 1.25), flagging rows whose static reorder_point is below that demand-driven buffer (under_buffered). GET /api/replenishment/par-recommendations is read-only; a planner applies a recommendation per row (POST .../apply writes the reorder_point onto branch_stock, planner duty). lead_time_days is per (branch,item) (migration 0163). Tenant-scoped (RLS); gated planner/procurement.</t>
         </is>
       </c>
       <c r="H73" s="17" t="inlineStr">
@@ -7192,37 +7192,37 @@
       </c>
       <c r="J73" s="17" t="inlineStr">
         <is>
-          <t>Per sale / period</t>
+          <t>Periodic / per planning cycle</t>
         </is>
       </c>
       <c r="K73" s="16" t="inlineStr">
         <is>
-          <t>HQ Controller</t>
+          <t>Planner / Supply Chain</t>
         </is>
       </c>
       <c r="L73" s="17" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>P13</t>
         </is>
       </c>
       <c r="M73" s="16" t="inlineStr">
         <is>
-          <t>branches.service.ts (consolidated, branch tagging); branches.controller.ts; cust_pos_sales.branch_id; cutover/branch.ts (ToE)</t>
+          <t>wms/replenishment.service.ts parRecommendations (avg-daily-usage x lead x safety, under_buffered flag) + applyPar (writes reorder_point, planner); wms.controller.ts (/api/replenishment/par-recommendations[/apply]); schema/portal.ts branch_stock.lead_time_days + migration 0163; /replenishment par-recommendations section; cutover/wms.ts (ToE)</t>
         </is>
       </c>
       <c r="N73" s="16" t="inlineStr">
         <is>
-          <t>Inspect branch tagging completeness + the '(none)' surfacing + the GL tie.</t>
+          <t>Inspect the avg-daily-usage derivation from consumption logs, the lead-time x safety reorder-point formula, the under_buffered flag, and the planner-gated apply.</t>
         </is>
       </c>
       <c r="O73" s="16" t="inlineStr">
         <is>
-          <t>Sample period: tagged sales group by branch, an untagged sale surfaces as '(none)', consolidated total ties to posted revenue.</t>
+          <t>Re-perform: seed branch consumption (10/day) at lead 3 -&gt; recommend ROP 38 (under-buffered vs static 10); apply writes 38 onto branch_stock; tenant-isolated (re-performed by the wms harness).</t>
         </is>
       </c>
       <c r="P73" s="16" t="inlineStr">
         <is>
-          <t>Consolidation report; '(none)' investigation log</t>
+          <t>Par recommendation list + apply test</t>
         </is>
       </c>
       <c r="Q73" s="18" t="inlineStr">
@@ -7234,7 +7234,7 @@
     <row r="74">
       <c r="A74" s="11" t="inlineStr">
         <is>
-          <t>BRANCH-02</t>
+          <t>BRANCH-01</t>
         </is>
       </c>
       <c r="B74" s="12" t="inlineStr">
@@ -7254,62 +7254,62 @@
       </c>
       <c r="E74" s="12" t="inlineStr">
         <is>
-          <t>An offline terminal sells at a stale or wrong price/promotion because the cached catalog drifted from the master.</t>
+          <t>A POS sale is not attributed to its originating branch, so the consolidated branch roll-up is incomplete and cannot be tied to GL revenue.</t>
         </is>
       </c>
       <c r="F74" s="12" t="inlineStr">
         <is>
-          <t>Accuracy</t>
+          <t>Completeness</t>
         </is>
       </c>
       <c r="G74" s="12" t="inlineStr">
         <is>
-          <t>Offline master-bundle export: GET /api/branches/master-bundle returns ONLY the active price-list + active promotions, time-stamped (generated_at). The offline terminal sells from this bundle, so it cannot ring a stale/withdrawn price or promo.</t>
+          <t>Branch sale-tagging + HQ consolidation: every POS sale carries cust_pos_sales.branch_id; GET /api/branches/consolidated aggregates per branch (excluding Voided) and surfaces untagged sales as branch '(none)' — a deliberate completeness flag the controller investigates and clears before tying the consolidated total to GL revenue.</t>
         </is>
       </c>
       <c r="H74" s="13" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I74" s="13" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="J74" s="13" t="inlineStr">
         <is>
-          <t>Per bundle push</t>
+          <t>Per sale / period</t>
         </is>
       </c>
       <c r="K74" s="12" t="inlineStr">
         <is>
-          <t>HQ Controller / Pricing</t>
+          <t>HQ Controller</t>
         </is>
       </c>
       <c r="L74" s="13" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="M74" s="12" t="inlineStr">
         <is>
-          <t>branches.service.ts masterBundle (active price-list + active promos + generated_at); branches.controller.ts; cutover/branch.ts (ToE)</t>
+          <t>branches.service.ts (consolidated, branch tagging); branches.controller.ts; cust_pos_sales.branch_id; cutover/branch.ts (ToE)</t>
         </is>
       </c>
       <c r="N74" s="12" t="inlineStr">
         <is>
-          <t>Inspect the bundle exports only active prices/promos with a timestamp.</t>
+          <t>Inspect branch tagging completeness + the '(none)' surfacing + the GL tie.</t>
         </is>
       </c>
       <c r="O74" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: export the bundle; confirm it carries only active price-list/promotions + generated_at.</t>
+          <t>Sample period: tagged sales group by branch, an untagged sale surfaces as '(none)', consolidated total ties to posted revenue.</t>
         </is>
       </c>
       <c r="P74" s="12" t="inlineStr">
         <is>
-          <t>Bundle metadata; bundle vs price-master diff</t>
+          <t>Consolidation report; '(none)' investigation log</t>
         </is>
       </c>
       <c r="Q74" s="18" t="inlineStr">
@@ -7321,7 +7321,7 @@
     <row r="75">
       <c r="A75" s="15" t="inlineStr">
         <is>
-          <t>BRANCH-03</t>
+          <t>BRANCH-02</t>
         </is>
       </c>
       <c r="B75" s="16" t="inlineStr">
@@ -7336,27 +7336,27 @@
       </c>
       <c r="D75" s="16" t="inlineStr">
         <is>
-          <t>Revenue; Cash</t>
+          <t>Revenue</t>
         </is>
       </c>
       <c r="E75" s="16" t="inlineStr">
         <is>
-          <t>An offline-captured sale is LOST or DUPLICATED when connectivity returns — revenue understated (lost) or double-counted (duplicated), and the GL double-posted.</t>
+          <t>An offline terminal sells at a stale or wrong price/promotion because the cached catalog drifted from the master.</t>
         </is>
       </c>
       <c r="F75" s="16" t="inlineStr">
         <is>
-          <t>Completeness/Accuracy</t>
+          <t>Accuracy</t>
         </is>
       </c>
       <c r="G75" s="16" t="inlineStr">
         <is>
-          <t>Offline-to-online exactly-once sync: offline-captured sales replay idempotently on (tenant, client_uuid) via the pos_offline_sync dedup ledger. Two paths share the ledger — the portal/inventory POS (POST /api/portal/pos/offline-sync, item_id lines) and the touch register (POST /api/restaurant/offline-sync, menu sku lines, re-running the restaurant order→checkout so the server re-prices + 86-checks). A re-sent batch returns 'duplicate' (no second sale/GL); a failed op is a RETRYABLE tombstone (sale_no NULL) that never blocks a later replay, so a transient error is not a lost sale; each op runs in its own savepoint so one bad sale never poisons the batch.</t>
+          <t>Offline master-bundle export: GET /api/branches/master-bundle returns ONLY the active price-list + active promotions, time-stamped (generated_at). The offline terminal sells from this bundle, so it cannot ring a stale/withdrawn price or promo.</t>
         </is>
       </c>
       <c r="H75" s="17" t="inlineStr">
         <is>
-          <t>Det/Prev</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I75" s="17" t="inlineStr">
@@ -7366,37 +7366,37 @@
       </c>
       <c r="J75" s="17" t="inlineStr">
         <is>
-          <t>Per sync</t>
+          <t>Per bundle push</t>
         </is>
       </c>
       <c r="K75" s="16" t="inlineStr">
         <is>
-          <t>HQ Controller / IT</t>
+          <t>HQ Controller / Pricing</t>
         </is>
       </c>
       <c r="L75" s="17" t="inlineStr">
         <is>
-          <t>P10/P16</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="M75" s="16" t="inlineStr">
         <is>
-          <t>portal/offline-sync.service.ts (item_id path); restaurant/offline-sync.service.ts (register sku path, reuses dineIn create+checkout); pos_offline_sync dedup ledger; web lib/offline-pos.ts + lib/register-offline.ts; cutover/offline-sync.ts + restaurant-offline.ts (ToE) + e2e/register-offline.spec.ts</t>
+          <t>branches.service.ts masterBundle (active price-list + active promos + generated_at); branches.controller.ts; cutover/branch.ts (ToE)</t>
         </is>
       </c>
       <c r="N75" s="16" t="inlineStr">
         <is>
-          <t>Inspect the (tenant, client_uuid) dedup gate (sale_no NOT NULL), the per-op savepoint isolation, and the retryable-failure tombstone.</t>
+          <t>Inspect the bundle exports only active prices/promos with a timestamp.</t>
         </is>
       </c>
       <c r="O75" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: sync a batch (all synced, distinct SALE-), replay it (all duplicate, no double sale/GL), a bad op fails while neighbours sync, same uuid twice in a batch posts once, a transient failure replays to synced after the cause clears (re-performed by the offline-sync + restaurant-offline harnesses).</t>
+          <t>Re-perform: export the bundle; confirm it carries only active price-list/promotions + generated_at.</t>
         </is>
       </c>
       <c r="P75" s="16" t="inlineStr">
         <is>
-          <t>Sync recon report; terminal vs ledger counts; idempotency tests</t>
+          <t>Bundle metadata; bundle vs price-master diff</t>
         </is>
       </c>
       <c r="Q75" s="18" t="inlineStr">
@@ -7408,12 +7408,12 @@
     <row r="76">
       <c r="A76" s="11" t="inlineStr">
         <is>
-          <t>MFG-01</t>
+          <t>BRANCH-03</t>
         </is>
       </c>
       <c r="B76" s="12" t="inlineStr">
         <is>
-          <t>Manufacturing &amp; Costing</t>
+          <t>Multi-Branch &amp; Offline POS</t>
         </is>
       </c>
       <c r="C76" s="13" t="inlineStr">
@@ -7423,67 +7423,67 @@
       </c>
       <c r="D76" s="12" t="inlineStr">
         <is>
-          <t>Inventory; COGS</t>
+          <t>Revenue; Cash</t>
         </is>
       </c>
       <c r="E76" s="12" t="inlineStr">
         <is>
-          <t>Unauthorized BOM/recipe change mis-states standard cost and every downstream WIP/COGS posting; or the role that maintains the recipe also transacts on it.</t>
+          <t>An offline-captured sale is LOST or DUPLICATED when connectivity returns — revenue understated (lost) or double-counted (duplicated), and the GL double-posted.</t>
         </is>
       </c>
       <c r="F76" s="12" t="inlineStr">
         <is>
-          <t>Authorization</t>
+          <t>Completeness/Accuracy</t>
         </is>
       </c>
       <c r="G76" s="12" t="inlineStr">
         <is>
-          <t>BOM master maker-checker / SoD: the master BOM library (bom_master) is maintained + distributed by HQ separately from transacting; a tenant BOM submission is reviewed and merged by HQ on approval (a maker-checker over master data). Recipe roll-up (line cost + labor + overhead → cost per unit) is the standard-cost basis. Master-data access is segregated from production (R13).</t>
+          <t>Offline-to-online exactly-once sync: offline-captured sales replay idempotently on (tenant, client_uuid) via the pos_offline_sync dedup ledger. Two paths share the ledger — the portal/inventory POS (POST /api/portal/pos/offline-sync, item_id lines) and the touch register (POST /api/restaurant/offline-sync, menu sku lines, re-running the restaurant order→checkout so the server re-prices + 86-checks). A re-sent batch returns 'duplicate' (no second sale/GL); a failed op is a RETRYABLE tombstone (sale_no NULL) that never blocks a later replay, so a transient error is not a lost sale; each op runs in its own savepoint so one bad sale never poisons the batch.</t>
         </is>
       </c>
       <c r="H76" s="13" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det/Prev</t>
         </is>
       </c>
       <c r="I76" s="13" t="inlineStr">
         <is>
-          <t>Manual+Auto</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J76" s="13" t="inlineStr">
         <is>
-          <t>Per BOM change</t>
+          <t>Per sync</t>
         </is>
       </c>
       <c r="K76" s="12" t="inlineStr">
         <is>
-          <t>HQ MasterSteward / CostAccountant</t>
+          <t>HQ Controller / IT</t>
         </is>
       </c>
       <c r="L76" s="13" t="inlineStr">
         <is>
-          <t>P13</t>
+          <t>P10/P16</t>
         </is>
       </c>
       <c r="M76" s="12" t="inlineStr">
         <is>
-          <t>bom master + submissions (/api/bom/master, /api/bom/submissions, /api/portal/bom); manufacturing.service.ts BOM scaling; cutover/cpq.ts + manufacturing.ts (ToE)</t>
+          <t>portal/offline-sync.service.ts (item_id path); restaurant/offline-sync.service.ts (register sku path, reuses dineIn create+checkout); pos_offline_sync dedup ledger; web lib/offline-pos.ts + lib/register-offline.ts; cutover/offline-sync.ts + restaurant-offline.ts (ToE) + e2e/register-offline.spec.ts</t>
         </is>
       </c>
       <c r="N76" s="12" t="inlineStr">
         <is>
-          <t>Inspect BOM maintenance access + the submission→approve maker-checker + the costing roll-up.</t>
+          <t>Inspect the (tenant, client_uuid) dedup gate (sale_no NOT NULL), the per-op savepoint isolation, and the retryable-failure tombstone.</t>
         </is>
       </c>
       <c r="O76" s="12" t="inlineStr">
         <is>
-          <t>Sample BOM change is HQ-approved before use; standard cost rolls up correctly.</t>
+          <t>Re-perform: sync a batch (all synced, distinct SALE-), replay it (all duplicate, no double sale/GL), a bad op fails while neighbours sync, same uuid twice in a batch posts once, a transient failure replays to synced after the cause clears (re-performed by the offline-sync + restaurant-offline harnesses).</t>
         </is>
       </c>
       <c r="P76" s="12" t="inlineStr">
         <is>
-          <t>BOM approval log; costing roll-up</t>
+          <t>Sync recon report; terminal vs ledger counts; idempotency tests</t>
         </is>
       </c>
       <c r="Q76" s="18" t="inlineStr">
@@ -7495,7 +7495,7 @@
     <row r="77">
       <c r="A77" s="15" t="inlineStr">
         <is>
-          <t>MFG-02</t>
+          <t>MFG-01</t>
         </is>
       </c>
       <c r="B77" s="16" t="inlineStr">
@@ -7510,22 +7510,22 @@
       </c>
       <c r="D77" s="16" t="inlineStr">
         <is>
-          <t>WIP; Finished Goods; COGS</t>
+          <t>Inventory; COGS</t>
         </is>
       </c>
       <c r="E77" s="16" t="inlineStr">
         <is>
-          <t>Production cost is mis-stated: WIP not relieved, the conversion absorption left stranded, or a yield loss (spoilage/waste) silently capitalised into finished-goods inventory instead of expensed.</t>
+          <t>Unauthorized BOM/recipe change mis-states standard cost and every downstream WIP/COGS posting; or the role that maintains the recipe also transacts on it.</t>
         </is>
       </c>
       <c r="F77" s="16" t="inlineStr">
         <is>
-          <t>Valuation/Completeness/Accuracy</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="G77" s="16" t="inlineStr">
         <is>
-          <t>Production work-order WIP costing with a balanced JE at each step: ISSUE posts Dr 1250 WIP / Cr 1200 raw materials / Cr 2380 manufacturing-costs-applied (idempotent — re-issue is a no-op); COMPLETE posts Dr 1210 Finished Goods at the standard cost of the ACTUAL quantity produced + books the YIELD VARIANCE to 5810 (produced &lt; planned → debit 5810 loss; over-yield → credit) / Cr 1250 WIP — so WIP is always fully relieved and FG is never over-valued on a short yield. State machine Open→Released→Completed (out-of-order → BAD_STATUS). The 2380/1250 clearing balances tie out at close. Scrap/rework write-off of defective output posts to 5810 with CostAccountant authorization.</t>
+          <t>BOM master maker-checker / SoD: the master BOM library (bom_master) is maintained + distributed by HQ separately from transacting; a tenant BOM submission is reviewed and merged by HQ on approval (a maker-checker over master data). Recipe roll-up (line cost + labor + overhead → cost per unit) is the standard-cost basis. Master-data access is segregated from production (R13).</t>
         </is>
       </c>
       <c r="H77" s="17" t="inlineStr">
@@ -7535,17 +7535,17 @@
       </c>
       <c r="I77" s="17" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Manual+Auto</t>
         </is>
       </c>
       <c r="J77" s="17" t="inlineStr">
         <is>
-          <t>Per work order</t>
+          <t>Per BOM change</t>
         </is>
       </c>
       <c r="K77" s="16" t="inlineStr">
         <is>
-          <t>Warehouse / CostAccountant</t>
+          <t>HQ MasterSteward / CostAccountant</t>
         </is>
       </c>
       <c r="L77" s="17" t="inlineStr">
@@ -7555,22 +7555,22 @@
       </c>
       <c r="M77" s="16" t="inlineStr">
         <is>
-          <t>manufacturing.service.ts issue/complete (yield variance to 5810; fmt exposes yield_variance); manufacturing.controller.ts (bom_master/warehouse/exec); schema/manufacturing.ts work_orders; cutover/manufacturing.ts (ToE)</t>
+          <t>bom master + submissions (/api/bom/master, /api/bom/submissions, /api/portal/bom); manufacturing.service.ts BOM scaling; cutover/cpq.ts + manufacturing.ts (ToE)</t>
         </is>
       </c>
       <c r="N77" s="16" t="inlineStr">
         <is>
-          <t>Inspect the issue/complete JEs + the standard-unit-cost FG valuation + the yield-variance plug + the status guard.</t>
+          <t>Inspect BOM maintenance access + the submission→approve maker-checker + the costing roll-up.</t>
         </is>
       </c>
       <c r="O77" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: issue (WIP charged), complete at full yield (FG = full cost, no variance) and at a short yield (FG = std×produced, the lost yield to 5810, WIP nets to 0, TB balanced) — re-performed by the harness.</t>
+          <t>Sample BOM change is HQ-approved before use; standard cost rolls up correctly.</t>
         </is>
       </c>
       <c r="P77" s="16" t="inlineStr">
         <is>
-          <t>WO costing register (yield_variance per WO); production JEs</t>
+          <t>BOM approval log; costing roll-up</t>
         </is>
       </c>
       <c r="Q77" s="18" t="inlineStr">
@@ -7582,7 +7582,7 @@
     <row r="78">
       <c r="A78" s="11" t="inlineStr">
         <is>
-          <t>MFG-03</t>
+          <t>MFG-02</t>
         </is>
       </c>
       <c r="B78" s="12" t="inlineStr">
@@ -7597,27 +7597,27 @@
       </c>
       <c r="D78" s="12" t="inlineStr">
         <is>
-          <t>Inventory; COGS</t>
+          <t>WIP; Finished Goods; COGS</t>
         </is>
       </c>
       <c r="E78" s="12" t="inlineStr">
         <is>
-          <t>Standard-cost inventory received without isolating the price variance — actual purchase cost buried in inventory, COGS and PPV mis-stated.</t>
+          <t>Production cost is mis-stated: WIP not relieved, the conversion absorption left stranded, or a yield loss (spoilage/waste) silently capitalised into finished-goods inventory instead of expensed.</t>
         </is>
       </c>
       <c r="F78" s="12" t="inlineStr">
         <is>
-          <t>Valuation/Accuracy</t>
+          <t>Valuation/Completeness/Accuracy</t>
         </is>
       </c>
       <c r="G78" s="12" t="inlineStr">
         <is>
-          <t>Goods-receipt capitalisation under the configured costing method (FIFO/AVG/STD per tenant+item): FIFO/AVG → Dr 1200 / Cr 2000 at actual; STD → Dr 1200 at standard, the purchase-price variance booked to 5500 (unfavourable Dr / favourable Cr), Cr 2000 at actual — the PPV (5500) leg is the single balancing plug (= actual − standard, rounded once) so the JE can never reject UNBALANCED on independent per-leg rounding.</t>
+          <t>Production work-order WIP costing with a balanced JE at each step: ISSUE posts Dr 1250 WIP / Cr 1200 raw materials / Cr 2380 manufacturing-costs-applied (idempotent — re-issue is a no-op); COMPLETE posts Dr 1210 Finished Goods at the standard cost of the ACTUAL quantity produced + books the YIELD VARIANCE to 5810 (produced &lt; planned → debit 5810 loss; over-yield → credit) / Cr 1250 WIP — so WIP is always fully relieved and FG is never over-valued on a short yield. State machine Open→Released→Completed (out-of-order → BAD_STATUS). The 2380/1250 clearing balances tie out at close. Scrap/rework write-off of defective output posts to 5810 with CostAccountant authorization.</t>
         </is>
       </c>
       <c r="H78" s="13" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I78" s="13" t="inlineStr">
@@ -7627,12 +7627,12 @@
       </c>
       <c r="J78" s="13" t="inlineStr">
         <is>
-          <t>Per receipt</t>
+          <t>Per work order</t>
         </is>
       </c>
       <c r="K78" s="12" t="inlineStr">
         <is>
-          <t>CostAccountant</t>
+          <t>Warehouse / CostAccountant</t>
         </is>
       </c>
       <c r="L78" s="13" t="inlineStr">
@@ -7642,22 +7642,22 @@
       </c>
       <c r="M78" s="12" t="inlineStr">
         <is>
-          <t>costing.service.ts (config/valuation, GRV capitalisation + 5500 PPV); costing.controller.ts (masterdata); cutover/costing.ts (ToE)</t>
+          <t>manufacturing.service.ts issue/complete (yield variance to 5810; fmt exposes yield_variance); manufacturing.controller.ts (bom_master/warehouse/exec); schema/manufacturing.ts work_orders; cutover/manufacturing.ts (ToE)</t>
         </is>
       </c>
       <c r="N78" s="12" t="inlineStr">
         <is>
-          <t>Inspect the per-method capitalisation routing + the PPV plug.</t>
+          <t>Inspect the issue/complete JEs + the standard-unit-cost FG valuation + the yield-variance plug + the status guard.</t>
         </is>
       </c>
       <c r="O78" s="12" t="inlineStr">
         <is>
-          <t>Re-perform a STD receipt at actual ≠ standard → PPV isolated to 5500, JE balanced; valuation ties to GL 1200/1210/1250.</t>
+          <t>Re-perform: issue (WIP charged), complete at full yield (FG = full cost, no variance) and at a short yield (FG = std×produced, the lost yield to 5810, WIP nets to 0, TB balanced) — re-performed by the harness.</t>
         </is>
       </c>
       <c r="P78" s="12" t="inlineStr">
         <is>
-          <t>PPV postings; costing valuation</t>
+          <t>WO costing register (yield_variance per WO); production JEs</t>
         </is>
       </c>
       <c r="Q78" s="18" t="inlineStr">
@@ -7669,12 +7669,12 @@
     <row r="79">
       <c r="A79" s="15" t="inlineStr">
         <is>
-          <t>PROJ-01</t>
+          <t>MFG-03</t>
         </is>
       </c>
       <c r="B79" s="16" t="inlineStr">
         <is>
-          <t>Project Accounting</t>
+          <t>Manufacturing &amp; Costing</t>
         </is>
       </c>
       <c r="C79" s="17" t="inlineStr">
@@ -7684,27 +7684,27 @@
       </c>
       <c r="D79" s="16" t="inlineStr">
         <is>
-          <t>Project WIP; COGS</t>
+          <t>Inventory; COGS</t>
         </is>
       </c>
       <c r="E79" s="16" t="inlineStr">
         <is>
-          <t>Project cost mis-stated: a recoverable cost not captured, or an UN-recoverable (non-billable) cost capitalised into project WIP as an asset that overstates the unbilled balance and inflates margin.</t>
+          <t>Standard-cost inventory received without isolating the price variance — actual purchase cost buried in inventory, COGS and PPV mis-stated.</t>
         </is>
       </c>
       <c r="F79" s="16" t="inlineStr">
         <is>
-          <t>Valuation/Accuracy/Completeness</t>
+          <t>Valuation/Accuracy</t>
         </is>
       </c>
       <c r="G79" s="16" t="inlineStr">
         <is>
-          <t>Project cost capture with a balanced JE and a billable/non-billable split: a BILLABLE time/expense cost is a recoverable asset → Dr 1260 Project WIP / Cr 2390 Project Costs Applied (accumulates in cost_to_date, relieved to COGS at billing); a NON-BILLABLE cost is unrecoverable → EXPENSED immediately Dr 5800 Project Cost of Services / Cr 2390 (never enters the billable WIP), so the register's total_cost and true margin (billed − recognised − non-billable) reflect the absorbed cost. A non-positive amount → BAD_AMOUNT; first cost flips Open→Active.</t>
+          <t>Goods-receipt capitalisation under the configured costing method (FIFO/AVG/STD per tenant+item): FIFO/AVG → Dr 1200 / Cr 2000 at actual; STD → Dr 1200 at standard, the purchase-price variance booked to 5500 (unfavourable Dr / favourable Cr), Cr 2000 at actual — the PPV (5500) leg is the single balancing plug (= actual − standard, rounded once) so the JE can never reject UNBALANCED on independent per-leg rounding.</t>
         </is>
       </c>
       <c r="H79" s="17" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I79" s="17" t="inlineStr">
@@ -7714,12 +7714,12 @@
       </c>
       <c r="J79" s="17" t="inlineStr">
         <is>
-          <t>Per cost entry</t>
+          <t>Per receipt</t>
         </is>
       </c>
       <c r="K79" s="16" t="inlineStr">
         <is>
-          <t>ProjectAccountant</t>
+          <t>CostAccountant</t>
         </is>
       </c>
       <c r="L79" s="17" t="inlineStr">
@@ -7729,22 +7729,22 @@
       </c>
       <c r="M79" s="16" t="inlineStr">
         <is>
-          <t>projects.service.ts logCost (billable→1260, non-billable→5800; fmt exposes non_billable_cost/total_cost/margin); projects.controller.ts; schema/projects.ts project_entries.billable; cutover/projects.ts (ToE)</t>
+          <t>costing.service.ts (config/valuation, GRV capitalisation + 5500 PPV); costing.controller.ts (masterdata); cutover/costing.ts (ToE)</t>
         </is>
       </c>
       <c r="N79" s="16" t="inlineStr">
         <is>
-          <t>Inspect the billable/non-billable GL routing + the WIP vs immediate-expense decision + the margin roll-up.</t>
+          <t>Inspect the per-method capitalisation routing + the PPV plug.</t>
         </is>
       </c>
       <c r="O79" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: a billable cost capitalises to 1260; a non-billable cost expenses to 5800 (NOT WIP), cost_to_date unchanged, and the project margin absorbs it (re-performed by the harness).</t>
+          <t>Re-perform a STD receipt at actual ≠ standard → PPV isolated to 5500, JE balanced; valuation ties to GL 1200/1210/1250.</t>
         </is>
       </c>
       <c r="P79" s="16" t="inlineStr">
         <is>
-          <t>Project cost JEs; cost register (non_billable_cost)</t>
+          <t>PPV postings; costing valuation</t>
         </is>
       </c>
       <c r="Q79" s="18" t="inlineStr">
@@ -7756,7 +7756,7 @@
     <row r="80">
       <c r="A80" s="11" t="inlineStr">
         <is>
-          <t>PROJ-02</t>
+          <t>PROJ-01</t>
         </is>
       </c>
       <c r="B80" s="12" t="inlineStr">
@@ -7771,22 +7771,22 @@
       </c>
       <c r="D80" s="12" t="inlineStr">
         <is>
-          <t>Project WIP; Revenue; COGS</t>
+          <t>Project WIP; COGS</t>
         </is>
       </c>
       <c r="E80" s="12" t="inlineStr">
         <is>
-          <t>Revenue billed without matching cost — WIP not relieved, cost of services mis-stated, margin overstated.</t>
+          <t>Project cost mis-stated: a recoverable cost not captured, or an UN-recoverable (non-billable) cost capitalised into project WIP as an asset that overstates the unbilled balance and inflates margin.</t>
         </is>
       </c>
       <c r="F80" s="12" t="inlineStr">
         <is>
-          <t>Accuracy/Cut-off</t>
+          <t>Valuation/Accuracy/Completeness</t>
         </is>
       </c>
       <c r="G80" s="12" t="inlineStr">
         <is>
-          <t>Customer billing recognises revenue (Dr 1100 AR / Cr 4200 Project Revenue) and relieves the unbilled WIP to cost of services up to the unrecognised billable cost (Dr 5800 / Cr 1260) in the same event — matching cost to recognised revenue. Billing is by raw amount (T&amp;M) or by PERCENT of the contract for Fixed-price milestone billing; a Fixed-price contract is CAPPED at the contract value (cumulative billing can never exceed it — BILL_EXCEEDS_CONTRACT), so the customer is never over-billed (billed_pct/remaining_to_bill on the register). Billing is idempotent on (project, cumulative billed amount).</t>
+          <t>Project cost capture with a balanced JE and a billable/non-billable split: a BILLABLE time/expense cost is a recoverable asset → Dr 1260 Project WIP / Cr 2390 Project Costs Applied (accumulates in cost_to_date, relieved to COGS at billing); a NON-BILLABLE cost is unrecoverable → EXPENSED immediately Dr 5800 Project Cost of Services / Cr 2390 (never enters the billable WIP), so the register's total_cost and true margin (billed − recognised − non-billable) reflect the absorbed cost. A non-positive amount → BAD_AMOUNT; first cost flips Open→Active.</t>
         </is>
       </c>
       <c r="H80" s="13" t="inlineStr">
@@ -7801,12 +7801,12 @@
       </c>
       <c r="J80" s="13" t="inlineStr">
         <is>
-          <t>Per billing</t>
+          <t>Per cost entry</t>
         </is>
       </c>
       <c r="K80" s="12" t="inlineStr">
         <is>
-          <t>ProjectController / ArSpecialist</t>
+          <t>ProjectAccountant</t>
         </is>
       </c>
       <c r="L80" s="13" t="inlineStr">
@@ -7816,22 +7816,22 @@
       </c>
       <c r="M80" s="12" t="inlineStr">
         <is>
-          <t>projects.service.ts bill (revenue + WIP relief, idempotent); projects.controller.ts (R07 vs cost initiation); cutover/projects.ts (ToE)</t>
+          <t>projects.service.ts logCost (billable→1260, non-billable→5800; fmt exposes non_billable_cost/total_cost/margin); projects.controller.ts; schema/projects.ts project_entries.billable; cutover/projects.ts (ToE)</t>
         </is>
       </c>
       <c r="N80" s="12" t="inlineStr">
         <is>
-          <t>Inspect the bill JE + the WIP-relief matching + idempotency.</t>
+          <t>Inspect the billable/non-billable GL routing + the WIP vs immediate-expense decision + the margin roll-up.</t>
         </is>
       </c>
       <c r="O80" s="12" t="inlineStr">
         <is>
-          <t>Re-perform a billing → revenue recognised, WIP relieved to 5800 up to unrecognised cost, 1260 reduced; margin = billed − recognised cost (re-performed by the harness).</t>
+          <t>Re-perform: a billable cost capitalises to 1260; a non-billable cost expenses to 5800 (NOT WIP), cost_to_date unchanged, and the project margin absorbs it (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P80" s="12" t="inlineStr">
         <is>
-          <t>Billing JEs; margin/WIP measurement</t>
+          <t>Project cost JEs; cost register (non_billable_cost)</t>
         </is>
       </c>
       <c r="Q80" s="18" t="inlineStr">
@@ -7843,7 +7843,7 @@
     <row r="81">
       <c r="A81" s="15" t="inlineStr">
         <is>
-          <t>PROJ-03</t>
+          <t>PROJ-02</t>
         </is>
       </c>
       <c r="B81" s="16" t="inlineStr">
@@ -7853,171 +7853,171 @@
       </c>
       <c r="C81" s="17" t="inlineStr">
         <is>
-          <t>Detective</t>
+          <t>Application</t>
         </is>
       </c>
       <c r="D81" s="16" t="inlineStr">
         <is>
-          <t>Project WIP</t>
+          <t>Project WIP; Revenue; COGS</t>
         </is>
       </c>
       <c r="E81" s="16" t="inlineStr">
         <is>
-          <t>Unbilled WIP (1260) and the 2390 clearing balance not reviewed at close — stale or unrecoverable WIP carried into the financial statements.</t>
+          <t>Revenue billed without matching cost — WIP not relieved, cost of services mis-stated, margin overstated.</t>
         </is>
       </c>
       <c r="F81" s="16" t="inlineStr">
         <is>
-          <t>Valuation</t>
+          <t>Accuracy/Cut-off</t>
         </is>
       </c>
       <c r="G81" s="16" t="inlineStr">
         <is>
-          <t>Period-end review of unbilled-WIP (1260) aging and the project-costs-applied (2390) clearing tie-out; project margin (billed_to_date − recognised_cost − non-billable) reviewed at close. SoD: billing authorisation is segregated from cost initiation (R07).</t>
+          <t>Customer billing recognises revenue (Dr 1100 AR / Cr 4200 Project Revenue) and relieves the unbilled WIP to cost of services up to the unrecognised billable cost (Dr 5800 / Cr 1260) in the same event — matching cost to recognised revenue. Billing is by raw amount (T&amp;M) or by PERCENT of the contract for Fixed-price milestone billing; a Fixed-price contract is CAPPED at the contract value (cumulative billing can never exceed it — BILL_EXCEEDS_CONTRACT), so the customer is never over-billed (billed_pct/remaining_to_bill on the register). Billing is idempotent on (project, cumulative billed amount).</t>
         </is>
       </c>
       <c r="H81" s="17" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I81" s="17" t="inlineStr">
         <is>
-          <t>Hybrid</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J81" s="17" t="inlineStr">
         <is>
-          <t>Period</t>
+          <t>Per billing</t>
         </is>
       </c>
       <c r="K81" s="16" t="inlineStr">
         <is>
-          <t>ProjectAccountant / Controller</t>
+          <t>ProjectController / ArSpecialist</t>
         </is>
       </c>
       <c r="L81" s="17" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>P13</t>
         </is>
       </c>
       <c r="M81" s="16" t="inlineStr">
         <is>
-          <t>projects.service.ts fmt (wip/margin); the project register + entries; close review</t>
+          <t>projects.service.ts bill (revenue + WIP relief, idempotent); projects.controller.ts (R07 vs cost initiation); cutover/projects.ts (ToE)</t>
         </is>
       </c>
       <c r="N81" s="16" t="inlineStr">
         <is>
-          <t>Inspect 1260 aging + 2390 clearing + margin review evidence.</t>
+          <t>Inspect the bill JE + the WIP-relief matching + idempotency.</t>
         </is>
       </c>
       <c r="O81" s="16" t="inlineStr">
         <is>
-          <t>Sample projects: 1260 WIP agrees to cost_to_date − recognised; 2390 clears; stale WIP investigated.</t>
+          <t>Re-perform a billing → revenue recognised, WIP relieved to 5800 up to unrecognised cost, 1260 reduced; margin = billed − recognised cost (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P81" s="16" t="inlineStr">
         <is>
-          <t>WIP aging; 2390 clearing tie-out</t>
-        </is>
-      </c>
-      <c r="Q81" s="19" t="inlineStr">
-        <is>
-          <t>Partial</t>
+          <t>Billing JEs; margin/WIP measurement</t>
+        </is>
+      </c>
+      <c r="Q81" s="18" t="inlineStr">
+        <is>
+          <t>Implemented</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="11" t="inlineStr">
         <is>
-          <t>GL-01</t>
+          <t>PROJ-03</t>
         </is>
       </c>
       <c r="B82" s="12" t="inlineStr">
         <is>
-          <t>General Ledger</t>
+          <t>Project Accounting</t>
         </is>
       </c>
       <c r="C82" s="13" t="inlineStr">
         <is>
-          <t>Application</t>
+          <t>Detective</t>
         </is>
       </c>
       <c r="D82" s="12" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Project WIP</t>
         </is>
       </c>
       <c r="E82" s="12" t="inlineStr">
         <is>
-          <t>Unbalanced / one-sided journal entries.</t>
+          <t>Unbilled WIP (1260) and the 2390 clearing balance not reviewed at close — stale or unrecoverable WIP carried into the financial statements.</t>
         </is>
       </c>
       <c r="F82" s="12" t="inlineStr">
         <is>
-          <t>Accuracy</t>
+          <t>Valuation</t>
         </is>
       </c>
       <c r="G82" s="12" t="inlineStr">
         <is>
-          <t>Double-entry balanced-by-construction — Σdebit=Σcredit enforced; each line single-sided &amp; non-negative.</t>
+          <t>Period-end review of unbilled-WIP (1260) aging and the project-costs-applied (2390) clearing tie-out; project margin (billed_to_date − recognised_cost − non-billable) reviewed at close. SoD: billing authorisation is segregated from cost initiation (R07).</t>
         </is>
       </c>
       <c r="H82" s="13" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I82" s="13" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Hybrid</t>
         </is>
       </c>
       <c r="J82" s="13" t="inlineStr">
         <is>
-          <t>Per JE</t>
+          <t>Period</t>
         </is>
       </c>
       <c r="K82" s="12" t="inlineStr">
         <is>
-          <t>Controller</t>
+          <t>ProjectAccountant / Controller</t>
         </is>
       </c>
       <c r="L82" s="13" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="M82" s="12" t="inlineStr">
         <is>
-          <t>ledger.service.ts (postEntry — UNBALANCED / INVALID_LINE)</t>
+          <t>projects.service.ts fmt (wip/margin); the project register + entries; close review</t>
         </is>
       </c>
       <c r="N82" s="12" t="inlineStr">
         <is>
-          <t>Inspect balance + line invariants.</t>
+          <t>Inspect 1260 aging + 2390 clearing + margin review evidence.</t>
         </is>
       </c>
       <c r="O82" s="12" t="inlineStr">
         <is>
-          <t>Attempt unbalanced JE → rejected.</t>
+          <t>Sample projects: 1260 WIP agrees to cost_to_date − recognised; 2390 clears; stale WIP investigated.</t>
         </is>
       </c>
       <c r="P82" s="12" t="inlineStr">
         <is>
-          <t>Invariant test</t>
-        </is>
-      </c>
-      <c r="Q82" s="18" t="inlineStr">
-        <is>
-          <t>Implemented</t>
+          <t>WIP aging; 2390 clearing tie-out</t>
+        </is>
+      </c>
+      <c r="Q82" s="19" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="15" t="inlineStr">
         <is>
-          <t>GL-02</t>
+          <t>GL-01</t>
         </is>
       </c>
       <c r="B83" s="16" t="inlineStr">
@@ -8037,17 +8037,17 @@
       </c>
       <c r="E83" s="16" t="inlineStr">
         <is>
-          <t>Postings to a closed period distort reported results.</t>
+          <t>Unbalanced / one-sided journal entries.</t>
         </is>
       </c>
       <c r="F83" s="16" t="inlineStr">
         <is>
-          <t>Cutoff</t>
+          <t>Accuracy</t>
         </is>
       </c>
       <c r="G83" s="16" t="inlineStr">
         <is>
-          <t>Period-close lockout — postings to a CLOSED fiscal period are rejected (per-tenant calendar).</t>
+          <t>Double-entry balanced-by-construction — Σdebit=Σcredit enforced; each line single-sided &amp; non-negative.</t>
         </is>
       </c>
       <c r="H83" s="17" t="inlineStr">
@@ -8077,22 +8077,22 @@
       </c>
       <c r="M83" s="16" t="inlineStr">
         <is>
-          <t>ledger.service.ts (postEntry PERIOD_CLOSED); fiscal_periods</t>
+          <t>ledger.service.ts (postEntry — UNBALANCED / INVALID_LINE)</t>
         </is>
       </c>
       <c r="N83" s="16" t="inlineStr">
         <is>
-          <t>Inspect close check.</t>
+          <t>Inspect balance + line invariants.</t>
         </is>
       </c>
       <c r="O83" s="16" t="inlineStr">
         <is>
-          <t>Post to closed period → rejected; review exceptions.</t>
+          <t>Attempt unbalanced JE → rejected.</t>
         </is>
       </c>
       <c r="P83" s="16" t="inlineStr">
         <is>
-          <t>Close-lock test</t>
+          <t>Invariant test</t>
         </is>
       </c>
       <c r="Q83" s="18" t="inlineStr">
@@ -8104,7 +8104,7 @@
     <row r="84">
       <c r="A84" s="11" t="inlineStr">
         <is>
-          <t>GL-03</t>
+          <t>GL-02</t>
         </is>
       </c>
       <c r="B84" s="12" t="inlineStr">
@@ -8119,22 +8119,22 @@
       </c>
       <c r="D84" s="12" t="inlineStr">
         <is>
-          <t>Equity</t>
+          <t>All</t>
         </is>
       </c>
       <c r="E84" s="12" t="inlineStr">
         <is>
-          <t>Unauthorized year-end close / RE roll.</t>
+          <t>Postings to a closed period distort reported results.</t>
         </is>
       </c>
       <c r="F84" s="12" t="inlineStr">
         <is>
-          <t>Cutoff/Authorization</t>
+          <t>Cutoff</t>
         </is>
       </c>
       <c r="G84" s="12" t="inlineStr">
         <is>
-          <t>Year-end close restricted to 'exec'; closing entries roll to retained earnings.</t>
+          <t>Period-close lockout — postings to a CLOSED fiscal period are rejected (per-tenant calendar).</t>
         </is>
       </c>
       <c r="H84" s="13" t="inlineStr">
@@ -8144,42 +8144,42 @@
       </c>
       <c r="I84" s="13" t="inlineStr">
         <is>
-          <t>Auto+Manual</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J84" s="13" t="inlineStr">
         <is>
-          <t>Annual</t>
+          <t>Per JE</t>
         </is>
       </c>
       <c r="K84" s="12" t="inlineStr">
         <is>
-          <t>CFO / Controller</t>
+          <t>Controller</t>
         </is>
       </c>
       <c r="L84" s="13" t="inlineStr">
         <is>
-          <t>P10/P11</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="M84" s="12" t="inlineStr">
         <is>
-          <t>ledger.controller.ts (close-year @Permissions exec); closeYear</t>
+          <t>ledger.service.ts (postEntry PERIOD_CLOSED); fiscal_periods</t>
         </is>
       </c>
       <c r="N84" s="12" t="inlineStr">
         <is>
-          <t>Inspect permission + closing logic.</t>
+          <t>Inspect close check.</t>
         </is>
       </c>
       <c r="O84" s="12" t="inlineStr">
         <is>
-          <t>Attempt close w/o exec → 403; review annual close.</t>
+          <t>Post to closed period → rejected; review exceptions.</t>
         </is>
       </c>
       <c r="P84" s="12" t="inlineStr">
         <is>
-          <t>Close package</t>
+          <t>Close-lock test</t>
         </is>
       </c>
       <c r="Q84" s="18" t="inlineStr">
@@ -8191,7 +8191,7 @@
     <row r="85">
       <c r="A85" s="15" t="inlineStr">
         <is>
-          <t>GL-04</t>
+          <t>GL-03</t>
         </is>
       </c>
       <c r="B85" s="16" t="inlineStr">
@@ -8206,22 +8206,22 @@
       </c>
       <c r="D85" s="16" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Equity</t>
         </is>
       </c>
       <c r="E85" s="16" t="inlineStr">
         <is>
-          <t>Concurrent posting double-books the same source doc.</t>
+          <t>Unauthorized year-end close / RE roll.</t>
         </is>
       </c>
       <c r="F85" s="16" t="inlineStr">
         <is>
-          <t>Completeness/Accuracy</t>
+          <t>Cutoff/Authorization</t>
         </is>
       </c>
       <c r="G85" s="16" t="inlineStr">
         <is>
-          <t>Ledger idempotency — UNIQUE (tenant,source,source_ref,ledger) + ON CONFLICT DO NOTHING in postEntry.</t>
+          <t>Year-end close restricted to 'exec'; closing entries roll to retained earnings.</t>
         </is>
       </c>
       <c r="H85" s="17" t="inlineStr">
@@ -8231,42 +8231,42 @@
       </c>
       <c r="I85" s="17" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="J85" s="17" t="inlineStr">
         <is>
-          <t>Per JE</t>
+          <t>Annual</t>
         </is>
       </c>
       <c r="K85" s="16" t="inlineStr">
         <is>
-          <t>Eng Lead / Controller</t>
+          <t>CFO / Controller</t>
         </is>
       </c>
       <c r="L85" s="17" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P10/P11</t>
         </is>
       </c>
       <c r="M85" s="16" t="inlineStr">
         <is>
-          <t>schema/ledger.ts (ux_je_idem); ledger.service.ts; migration 0058</t>
+          <t>ledger.controller.ts (close-year @Permissions exec); closeYear</t>
         </is>
       </c>
       <c r="N85" s="16" t="inlineStr">
         <is>
-          <t>Inspect unique index + conflict handling.</t>
+          <t>Inspect permission + closing logic.</t>
         </is>
       </c>
       <c r="O85" s="16" t="inlineStr">
         <is>
-          <t>Concurrent identical post → single entry.</t>
+          <t>Attempt close w/o exec → 403; review annual close.</t>
         </is>
       </c>
       <c r="P85" s="16" t="inlineStr">
         <is>
-          <t>Dedup test</t>
+          <t>Close package</t>
         </is>
       </c>
       <c r="Q85" s="18" t="inlineStr">
@@ -8278,7 +8278,7 @@
     <row r="86">
       <c r="A86" s="11" t="inlineStr">
         <is>
-          <t>GL-05</t>
+          <t>GL-04</t>
         </is>
       </c>
       <c r="B86" s="12" t="inlineStr">
@@ -8298,17 +8298,17 @@
       </c>
       <c r="E86" s="12" t="inlineStr">
         <is>
-          <t>Manual JE posted without independent review (override risk).</t>
+          <t>Concurrent posting double-books the same source doc.</t>
         </is>
       </c>
       <c r="F86" s="12" t="inlineStr">
         <is>
-          <t>Authorization</t>
+          <t>Completeness/Accuracy</t>
         </is>
       </c>
       <c r="G86" s="12" t="inlineStr">
         <is>
-          <t>Manual journal-entry maker-checker — preparer ≠ approver before a manual JE posts.</t>
+          <t>Ledger idempotency — UNIQUE (tenant,source,source_ref,ledger) + ON CONFLICT DO NOTHING in postEntry.</t>
         </is>
       </c>
       <c r="H86" s="13" t="inlineStr">
@@ -8318,17 +8318,17 @@
       </c>
       <c r="I86" s="13" t="inlineStr">
         <is>
-          <t>Auto+Manual</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J86" s="13" t="inlineStr">
         <is>
-          <t>Per manual JE</t>
+          <t>Per JE</t>
         </is>
       </c>
       <c r="K86" s="12" t="inlineStr">
         <is>
-          <t>Controller</t>
+          <t>Eng Lead / Controller</t>
         </is>
       </c>
       <c r="L86" s="13" t="inlineStr">
@@ -8338,22 +8338,22 @@
       </c>
       <c r="M86" s="12" t="inlineStr">
         <is>
-          <t>ledger.service.ts (postEntry pendingApproval→Draft; approveEntry preparer≠approver; rejectEntry); ledger.controller.ts (gl_post posts / gl_close approves); cutover/compliance.ts (ToE)</t>
+          <t>schema/ledger.ts (ux_je_idem); ledger.service.ts; migration 0058</t>
         </is>
       </c>
       <c r="N86" s="12" t="inlineStr">
         <is>
-          <t>Inspect JE approval routing.</t>
+          <t>Inspect unique index + conflict handling.</t>
         </is>
       </c>
       <c r="O86" s="12" t="inlineStr">
         <is>
-          <t>Sample manual JEs: approver ≠ preparer; Draft excluded from balances until approved (re-performed by the harness).</t>
+          <t>Concurrent identical post → single entry.</t>
         </is>
       </c>
       <c r="P86" s="12" t="inlineStr">
         <is>
-          <t>JE approvals</t>
+          <t>Dedup test</t>
         </is>
       </c>
       <c r="Q86" s="18" t="inlineStr">
@@ -8365,7 +8365,7 @@
     <row r="87">
       <c r="A87" s="15" t="inlineStr">
         <is>
-          <t>GL-06</t>
+          <t>GL-05</t>
         </is>
       </c>
       <c r="B87" s="16" t="inlineStr">
@@ -8385,17 +8385,17 @@
       </c>
       <c r="E87" s="16" t="inlineStr">
         <is>
-          <t>Operator mis-posts to another tenant's books.</t>
+          <t>Manual JE posted without independent review (override risk).</t>
         </is>
       </c>
       <c r="F87" s="16" t="inlineStr">
         <is>
-          <t>Validity</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="G87" s="16" t="inlineStr">
         <is>
-          <t>HQ cross-tenant posting gated to Admin (explicit tenant override); others pinned to context (also RLS).</t>
+          <t>Manual journal-entry maker-checker — preparer ≠ approver before a manual JE posts.</t>
         </is>
       </c>
       <c r="H87" s="17" t="inlineStr">
@@ -8405,42 +8405,42 @@
       </c>
       <c r="I87" s="17" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="J87" s="17" t="inlineStr">
         <is>
-          <t>Per JE</t>
+          <t>Per manual JE</t>
         </is>
       </c>
       <c r="K87" s="16" t="inlineStr">
         <is>
-          <t>Eng Lead</t>
+          <t>Controller</t>
         </is>
       </c>
       <c r="L87" s="17" t="inlineStr">
         <is>
-          <t>P10/P11</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="M87" s="16" t="inlineStr">
         <is>
-          <t>ledger.controller.ts (hqTenant)</t>
+          <t>ledger.service.ts (postEntry pendingApproval→Draft; approveEntry preparer≠approver; rejectEntry); ledger.controller.ts (gl_post posts / gl_close approves); cutover/compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N87" s="16" t="inlineStr">
         <is>
-          <t>Inspect Admin gating of tenant_id.</t>
+          <t>Inspect JE approval routing.</t>
         </is>
       </c>
       <c r="O87" s="16" t="inlineStr">
         <is>
-          <t>Non-Admin tenant override ignored; Admin audited.</t>
+          <t>Sample manual JEs: approver ≠ preparer; Draft excluded from balances until approved (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P87" s="16" t="inlineStr">
         <is>
-          <t>Override test</t>
+          <t>JE approvals</t>
         </is>
       </c>
       <c r="Q87" s="18" t="inlineStr">
@@ -8452,7 +8452,7 @@
     <row r="88">
       <c r="A88" s="11" t="inlineStr">
         <is>
-          <t>GL-07</t>
+          <t>GL-06</t>
         </is>
       </c>
       <c r="B88" s="12" t="inlineStr">
@@ -8467,27 +8467,27 @@
       </c>
       <c r="D88" s="12" t="inlineStr">
         <is>
-          <t>Cash</t>
+          <t>All</t>
         </is>
       </c>
       <c r="E88" s="12" t="inlineStr">
         <is>
-          <t>Statement of cash flows mis-stated or doesn't tie to the change in cash.</t>
+          <t>Operator mis-posts to another tenant's books.</t>
         </is>
       </c>
       <c r="F88" s="12" t="inlineStr">
         <is>
-          <t>Accuracy/Completeness</t>
+          <t>Validity</t>
         </is>
       </c>
       <c r="G88" s="12" t="inlineStr">
         <is>
-          <t>Statement of Cash Flows (indirect) reconstructed from the GL: net income + non-cash add-backs + working-capital + investing + financing; year-end CLOSE entries excluded; reconciles to Δcash (1000/1010/1020) by construction with a `reconciled` tie-out flag. A direct-method view presents the same operating cash by receipt/payment nature (receipts from customers, payments to suppliers, tax &amp; payroll) and also reconciles to Δcash; a forward cash-flow forecast projects open AR (inflows) and AP (outflows) by due date from today's cash balance for treasury/collections planning.</t>
+          <t>HQ cross-tenant posting gated to Admin (explicit tenant override); others pinned to context (also RLS).</t>
         </is>
       </c>
       <c r="H88" s="13" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I88" s="13" t="inlineStr">
@@ -8497,37 +8497,37 @@
       </c>
       <c r="J88" s="13" t="inlineStr">
         <is>
-          <t>Per period</t>
+          <t>Per JE</t>
         </is>
       </c>
       <c r="K88" s="12" t="inlineStr">
         <is>
-          <t>Controller</t>
+          <t>Eng Lead</t>
         </is>
       </c>
       <c r="L88" s="13" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P10/P11</t>
         </is>
       </c>
       <c r="M88" s="12" t="inlineStr">
         <is>
-          <t>ledger.service.ts (cashFlowStatement, cashFlowDirect, cashFlowForecast); ledger.controller.ts (GET cash-flow, cash-flow-direct, cash-flow-forecast); cutover/basics.ts (ToE)</t>
+          <t>ledger.controller.ts (hqTenant)</t>
         </is>
       </c>
       <c r="N88" s="12" t="inlineStr">
         <is>
-          <t>Inspect SCF derivation + reconciliation flag; inspect direct-method bucketing and forecast projection.</t>
+          <t>Inspect Admin gating of tenant_id.</t>
         </is>
       </c>
       <c r="O88" s="12" t="inlineStr">
         <is>
-          <t>Run cash-flow over a seeded period — activities tie to the movement in cash; CLOSE excluded; direct method ties to the same operating cash and Δcash; forecast buckets open AR/AP by due week (re-performed by the harness).</t>
+          <t>Non-Admin tenant override ignored; Admin audited.</t>
         </is>
       </c>
       <c r="P88" s="12" t="inlineStr">
         <is>
-          <t>Cash-flow reconciliation; direct-method buckets; forecast schedule</t>
+          <t>Override test</t>
         </is>
       </c>
       <c r="Q88" s="18" t="inlineStr">
@@ -8539,7 +8539,7 @@
     <row r="89">
       <c r="A89" s="15" t="inlineStr">
         <is>
-          <t>GL-08</t>
+          <t>GL-07</t>
         </is>
       </c>
       <c r="B89" s="16" t="inlineStr">
@@ -8554,27 +8554,27 @@
       </c>
       <c r="D89" s="16" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Cash</t>
         </is>
       </c>
       <c r="E89" s="16" t="inlineStr">
         <is>
-          <t>Standing/period accruals missed, posted unbalanced, or posted without approval; manual re-keying error.</t>
+          <t>Statement of cash flows mis-stated or doesn't tie to the change in cash.</t>
         </is>
       </c>
       <c r="F89" s="16" t="inlineStr">
         <is>
-          <t>Completeness/Accuracy/Authorization</t>
+          <t>Accuracy/Completeness</t>
         </is>
       </c>
       <c r="G89" s="16" t="inlineStr">
         <is>
-          <t>Recurring/template journal entries: a template's lines are validated balanced (Σdebit=Σcredit) AT SAVE TIME (unbalanced → UNBALANCED), so a broken template can never be persisted. The scheduled job gl_recurring_journals (cron / daily scheduler) posts every due template as a DRAFT JE through the normal maker-checker flow (GL-05) — a different user must approve before it affects balances — and rolls next_run_date forward. Idempotent: next_run_date advanced on posting + the (tenant,source,source_ref,ledger) idempotency key dedupes a same-day re-run. Templates can be paused/resumed without losing history.</t>
+          <t>Statement of Cash Flows (indirect) reconstructed from the GL: net income + non-cash add-backs + working-capital + investing + financing; year-end CLOSE entries excluded; reconciles to Δcash (1000/1010/1020) by construction with a `reconciled` tie-out flag. A direct-method view presents the same operating cash by receipt/payment nature (receipts from customers, payments to suppliers, tax &amp; payroll) and also reconciles to Δcash; a forward cash-flow forecast projects open AR (inflows) and AP (outflows) by due date from today's cash balance for treasury/collections planning.</t>
         </is>
       </c>
       <c r="H89" s="17" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I89" s="17" t="inlineStr">
@@ -8584,7 +8584,7 @@
       </c>
       <c r="J89" s="17" t="inlineStr">
         <is>
-          <t>Per due date / per template</t>
+          <t>Per period</t>
         </is>
       </c>
       <c r="K89" s="16" t="inlineStr">
@@ -8599,22 +8599,22 @@
       </c>
       <c r="M89" s="16" t="inlineStr">
         <is>
-          <t>ledger.service.ts (createRecurring balanced-at-save, runDueRecurring→postEntry pendingApproval, setRecurringActive); ledger.controller.ts (gl_post creates/runs); bi.service.ts (gl_recurring_journals); schema/ledger.ts (recurring_journals) + migration 0119; cutover/basics.ts (ToE)</t>
+          <t>ledger.service.ts (cashFlowStatement, cashFlowDirect, cashFlowForecast); ledger.controller.ts (GET cash-flow, cash-flow-direct, cash-flow-forecast); cutover/basics.ts (ToE)</t>
         </is>
       </c>
       <c r="N89" s="16" t="inlineStr">
         <is>
-          <t>Inspect template balance validation + scheduled posting as Draft + idempotency.</t>
+          <t>Inspect SCF derivation + reconciliation flag; inspect direct-method bucketing and forecast projection.</t>
         </is>
       </c>
       <c r="O89" s="16" t="inlineStr">
         <is>
-          <t>Unbalanced template → UNBALANCED; due template posts a Draft JE (excluded from TB) into the pending queue; re-run posts nothing; a second user approves → accrual hits the GL (re-performed by the harness).</t>
+          <t>Run cash-flow over a seeded period — activities tie to the movement in cash; CLOSE excluded; direct method ties to the same operating cash and Δcash; forecast buckets open AR/AP by due week (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P89" s="16" t="inlineStr">
         <is>
-          <t>Recurring-journal templates; scheduled run log; JE approvals</t>
+          <t>Cash-flow reconciliation; direct-method buckets; forecast schedule</t>
         </is>
       </c>
       <c r="Q89" s="18" t="inlineStr">
@@ -8626,7 +8626,7 @@
     <row r="90">
       <c r="A90" s="11" t="inlineStr">
         <is>
-          <t>GL-09</t>
+          <t>GL-08</t>
         </is>
       </c>
       <c r="B90" s="12" t="inlineStr">
@@ -8641,27 +8641,27 @@
       </c>
       <c r="D90" s="12" t="inlineStr">
         <is>
-          <t>Prepaid expenses; Operating expense</t>
+          <t>All</t>
         </is>
       </c>
       <c r="E90" s="12" t="inlineStr">
         <is>
-          <t>Prepaid expense not amortized over its term — expense mis-stated, prepaid asset overstated.</t>
+          <t>Standing/period accruals missed, posted unbalanced, or posted without approval; manual re-keying error.</t>
         </is>
       </c>
       <c r="F90" s="12" t="inlineStr">
         <is>
-          <t>Accuracy/Completeness</t>
+          <t>Completeness/Accuracy/Authorization</t>
         </is>
       </c>
       <c r="G90" s="12" t="inlineStr">
         <is>
-          <t>Prepaid amortization schedules: a prepaid asset (insurance/rent paid up front) is registered once with a total + term; the scheduled job gl_prepaid_amortize posts a straight-line slice each period (Dr expense / Cr 1280), the last period taking the remainder so the asset fully clears. Idempotent per (schedule, period) via the JE idempotency key + next_run_date advance.</t>
+          <t>Recurring/template journal entries: a template's lines are validated balanced (Σdebit=Σcredit) AT SAVE TIME (unbalanced → UNBALANCED), so a broken template can never be persisted. The scheduled job gl_recurring_journals (cron / daily scheduler) posts every due template as a DRAFT JE through the normal maker-checker flow (GL-05) — a different user must approve before it affects balances — and rolls next_run_date forward. Idempotent: next_run_date advanced on posting + the (tenant,source,source_ref,ledger) idempotency key dedupes a same-day re-run. Templates can be paused/resumed without losing history.</t>
         </is>
       </c>
       <c r="H90" s="13" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I90" s="13" t="inlineStr">
@@ -8671,7 +8671,7 @@
       </c>
       <c r="J90" s="13" t="inlineStr">
         <is>
-          <t>Per period / per schedule</t>
+          <t>Per due date / per template</t>
         </is>
       </c>
       <c r="K90" s="12" t="inlineStr">
@@ -8686,22 +8686,22 @@
       </c>
       <c r="M90" s="12" t="inlineStr">
         <is>
-          <t>ledger.service.ts (createPrepaid, runDuePrepaid); ledger.controller.ts (gl_post); bi.service.ts (gl_prepaid_amortize); schema/ledger.ts (prepaid_schedules) + migration 0120; cutover/basics.ts (ToE)</t>
+          <t>ledger.service.ts (createRecurring balanced-at-save, runDueRecurring→postEntry pendingApproval, setRecurringActive); ledger.controller.ts (gl_post creates/runs); bi.service.ts (gl_recurring_journals); schema/ledger.ts (recurring_journals) + migration 0119; cutover/basics.ts (ToE)</t>
         </is>
       </c>
       <c r="N90" s="12" t="inlineStr">
         <is>
-          <t>Inspect amortization slice + final-period remainder + idempotency.</t>
+          <t>Inspect template balance validation + scheduled posting as Draft + idempotency.</t>
         </is>
       </c>
       <c r="O90" s="12" t="inlineStr">
         <is>
-          <t>Register a 12-month prepaid; run amortizes 1/12 to expense; re-run posts nothing (re-performed by the harness).</t>
+          <t>Unbalanced template → UNBALANCED; due template posts a Draft JE (excluded from TB) into the pending queue; re-run posts nothing; a second user approves → accrual hits the GL (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P90" s="12" t="inlineStr">
         <is>
-          <t>Prepaid schedules; amortization run log</t>
+          <t>Recurring-journal templates; scheduled run log; JE approvals</t>
         </is>
       </c>
       <c r="Q90" s="18" t="inlineStr">
@@ -8713,7 +8713,7 @@
     <row r="91">
       <c r="A91" s="15" t="inlineStr">
         <is>
-          <t>GL-10</t>
+          <t>GL-09</t>
         </is>
       </c>
       <c r="B91" s="16" t="inlineStr">
@@ -8728,27 +8728,27 @@
       </c>
       <c r="D91" s="16" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Prepaid expenses; Operating expense</t>
         </is>
       </c>
       <c r="E91" s="16" t="inlineStr">
         <is>
-          <t>A new company starts on a chart of accounts with no industry guidance — staff post to wrong/ambiguous accounts; or an industry template drifts from the GL engine's fixed posting codes so a posting targets an account that does not exist (mis-statement / unposted transaction).</t>
+          <t>Prepaid expense not amortized over its term — expense mis-stated, prepaid asset overstated.</t>
         </is>
       </c>
       <c r="F91" s="16" t="inlineStr">
         <is>
-          <t>Completeness/Accuracy/Presentation</t>
+          <t>Accuracy/Completeness</t>
         </is>
       </c>
       <c r="G91" s="16" t="inlineStr">
         <is>
-          <t>Industry Chart-of-Accounts templates: the GL engine binds to a FIXED, global account universe (canonical codes are immutable); each tenant additionally gets a per-tenant overlay (tenant_accounts) curating which canonical accounts are active and how they are named/grouped for its industry. At company creation the customer picks an industry (restaurant/retail/distribution/services/general) and the chosen template is materialised into the overlay (provisionTenantCoA) inside the signup transaction, right after fiscal-year provisioning; adopting an industry pack later does the same. Every template code is asserted to exist in the canonical chart at boot (assertTemplatesSubsetOf in seedChartOfAccounts) so a drifted template fails fast and can never reach a tenant. Provisioning is idempotent + additive (never deletes) so re-running only adds missing accounts. The overlay NEVER gates postings — it scopes the picker / Chart-of-Accounts view only; reports surface any account that is active OR carries activity, so a curated-out account that receives a posting still appears.</t>
+          <t>Prepaid amortization schedules: a prepaid asset (insurance/rent paid up front) is registered once with a total + term; the scheduled job gl_prepaid_amortize posts a straight-line slice each period (Dr expense / Cr 1280), the last period taking the remainder so the asset fully clears. Idempotent per (schedule, period) via the JE idempotency key + next_run_date advance.</t>
         </is>
       </c>
       <c r="H91" s="17" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I91" s="17" t="inlineStr">
@@ -8758,7 +8758,7 @@
       </c>
       <c r="J91" s="17" t="inlineStr">
         <is>
-          <t>At company creation / per pack adopt</t>
+          <t>Per period / per schedule</t>
         </is>
       </c>
       <c r="K91" s="16" t="inlineStr">
@@ -8773,22 +8773,22 @@
       </c>
       <c r="M91" s="16" t="inlineStr">
         <is>
-          <t>ledger.service.ts (provisionTenantCoA idempotent+additive, tenant-aware listAccounts, seedChartOfAccounts→assertTemplatesSubsetOf); coa-templates.ts (industry templates + subset assertion); billing.service.ts signup (industry→provisionTenantCoA in-txn); onboarding.service.ts applyPack (pack adopt provisions CoA); schema/ledger.ts tenant_accounts + tenants.industry + migration 0139; cutover/basics.ts + compliance.ts (ToE)</t>
+          <t>ledger.service.ts (createPrepaid, runDuePrepaid); ledger.controller.ts (gl_post); bi.service.ts (gl_prepaid_amortize); schema/ledger.ts (prepaid_schedules) + migration 0120; cutover/basics.ts (ToE)</t>
         </is>
       </c>
       <c r="N91" s="16" t="inlineStr">
         <is>
-          <t>Inspect the boot subset assertion + signup provisioning + the overlay-is-presentation-only read path.</t>
+          <t>Inspect amortization slice + final-period remainder + idempotency.</t>
         </is>
       </c>
       <c r="O91" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: a template referencing an unknown code fails the boot assertion; signup with industry=restaurant materialises a curated, industry-named chart (4000='Food &amp; Beverage Sales') that omits non-F&amp;B accounts; ?all=true still returns the full canonical universe (overlay never gates posting); signup with no industry ⇒ general = the full live chart (re-performed by the harnesses).</t>
+          <t>Register a 12-month prepaid; run amortizes 1/12 to expense; re-run posts nothing (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P91" s="16" t="inlineStr">
         <is>
-          <t>Industry templates; tenant_accounts overlay; signup provisioning log</t>
+          <t>Prepaid schedules; amortization run log</t>
         </is>
       </c>
       <c r="Q91" s="18" t="inlineStr">
@@ -8800,7 +8800,7 @@
     <row r="92">
       <c r="A92" s="11" t="inlineStr">
         <is>
-          <t>GL-11</t>
+          <t>GL-10</t>
         </is>
       </c>
       <c r="B92" s="12" t="inlineStr">
@@ -8820,17 +8820,17 @@
       </c>
       <c r="E92" s="12" t="inlineStr">
         <is>
-          <t>Chart of Accounts changed without authorisation; account code changed after postings exist; account deactivated while carrying a non-zero balance; manual JE posted directly to a control account (AR/AP/INV/FA), bypassing the sub-ledger and hiding a sub-ledger discrepancy.</t>
+          <t>A new company starts on a chart of accounts with no industry guidance — staff post to wrong/ambiguous accounts; or an industry template drifts from the GL engine's fixed posting codes so a posting targets an account that does not exist (mis-statement / unposted transaction).</t>
         </is>
       </c>
       <c r="F92" s="12" t="inlineStr">
         <is>
-          <t>Authorization/Completeness/Accuracy</t>
+          <t>Completeness/Accuracy/Presentation</t>
         </is>
       </c>
       <c r="G92" s="12" t="inlineStr">
         <is>
-          <t>CoA Change Control: account creation/update/deactivation requires the gl_coa permission (held by FinancialController, not GlAccountant — separated from gl_post per SoD). Disabling postability on an account that already has posted entries is rejected (CODE_HAS_POSTINGS). Deactivation is rejected if the account carries a non-zero net balance (ACCOUNT_HAS_BALANCE) — prevents orphaning a balance in a closed account. Four accounts are flagged is_control=true at setup: 1100 (AR), 2000 (AP), 1200 (INV), 1500 (FA); a direct manual JE that touches any of these without viaSubledger:true is rejected (CONTROL_ACCOUNT), ensuring AR/AP/INV/FA balances are exclusively maintained by their respective sub-ledger service methods.</t>
+          <t>Industry Chart-of-Accounts templates: the GL engine binds to a FIXED, global account universe (canonical codes are immutable); each tenant additionally gets a per-tenant overlay (tenant_accounts) curating which canonical accounts are active and how they are named/grouped for its industry. At company creation the customer picks an industry (restaurant/retail/distribution/services/general) and the chosen template is materialised into the overlay (provisionTenantCoA) inside the signup transaction, right after fiscal-year provisioning; adopting an industry pack later does the same. Every template code is asserted to exist in the canonical chart at boot (assertTemplatesSubsetOf in seedChartOfAccounts) so a drifted template fails fast and can never reach a tenant. Provisioning is idempotent + additive (never deletes) so re-running only adds missing accounts. The overlay NEVER gates postings — it scopes the picker / Chart-of-Accounts view only; reports surface any account that is active OR carries activity, so a curated-out account that receives a posting still appears.</t>
         </is>
       </c>
       <c r="H92" s="13" t="inlineStr">
@@ -8845,12 +8845,12 @@
       </c>
       <c r="J92" s="13" t="inlineStr">
         <is>
-          <t>Event-driven</t>
+          <t>At company creation / per pack adopt</t>
         </is>
       </c>
       <c r="K92" s="12" t="inlineStr">
         <is>
-          <t>Financial Controller</t>
+          <t>Controller</t>
         </is>
       </c>
       <c r="L92" s="13" t="inlineStr">
@@ -8860,22 +8860,22 @@
       </c>
       <c r="M92" s="12" t="inlineStr">
         <is>
-          <t>coa.service.ts (createAccount DUPLICATE_ACCOUNT, updateAccount CODE_HAS_POSTINGS, deactivateAccount ACCOUNT_HAS_BALANCE); coa.controller.ts (gl_coa permission gate); ledger.service.ts postEntry control-account guard (CONTROL_ACCOUNT, viaSubledger flag); schema/ledger.ts (account_groups table, accounts.is_control/control_subledger/is_postable/normal_balance + migration 0155); packages/shared/src/permissions.ts (gl_coa sub-permission, FinancialController default)</t>
+          <t>ledger.service.ts (provisionTenantCoA idempotent+additive, tenant-aware listAccounts, seedChartOfAccounts→assertTemplatesSubsetOf); coa-templates.ts (industry templates + subset assertion); billing.service.ts signup (industry→provisionTenantCoA in-txn); onboarding.service.ts applyPack (pack adopt provisions CoA); schema/ledger.ts tenant_accounts + tenants.industry + migration 0139; cutover/basics.ts + compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N92" s="12" t="inlineStr">
         <is>
-          <t>Inspect gl_coa permission gate + CODE_HAS_POSTINGS guard + ACCOUNT_HAS_BALANCE guard + CONTROL_ACCOUNT guard + viaSubledger bypass.</t>
+          <t>Inspect the boot subset assertion + signup provisioning + the overlay-is-presentation-only read path.</t>
         </is>
       </c>
       <c r="O92" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: create an account with gl_coa → 201; attempt to deactivate an account with balance → ACCOUNT_HAS_BALANCE; post directly to account 1100 without viaSubledger → CONTROL_ACCOUNT (re-performed by TC-GL-11-01/02/03 UAT cases).</t>
+          <t>Re-perform: a template referencing an unknown code fails the boot assertion; signup with industry=restaurant materialises a curated, industry-named chart (4000='Food &amp; Beverage Sales') that omits non-F&amp;B accounts; ?all=true still returns the full canonical universe (overlay never gates posting); signup with no industry ⇒ general = the full live chart (re-performed by the harnesses).</t>
         </is>
       </c>
       <c r="P92" s="12" t="inlineStr">
         <is>
-          <t>CoA change log (audit_log); permission test; control-account guard test</t>
+          <t>Industry templates; tenant_accounts overlay; signup provisioning log</t>
         </is>
       </c>
       <c r="Q92" s="18" t="inlineStr">
@@ -8887,7 +8887,7 @@
     <row r="93">
       <c r="A93" s="15" t="inlineStr">
         <is>
-          <t>GL-12</t>
+          <t>GL-11</t>
         </is>
       </c>
       <c r="B93" s="16" t="inlineStr">
@@ -8907,17 +8907,17 @@
       </c>
       <c r="E93" s="16" t="inlineStr">
         <is>
-          <t>Account-assignment errors introduced by scattered inline account-code literals in service code; a tenant needing a different account for a given business event has no mechanism to override without a code change.</t>
+          <t>Chart of Accounts changed without authorisation; account code changed after postings exist; account deactivated while carrying a non-zero balance; manual JE posted directly to a control account (AR/AP/INV/FA), bypassing the sub-ledger and hiding a sub-ledger discrepancy.</t>
         </is>
       </c>
       <c r="F93" s="16" t="inlineStr">
         <is>
-          <t>Authorization/Accuracy</t>
+          <t>Authorization/Completeness/Accuracy</t>
         </is>
       </c>
       <c r="G93" s="16" t="inlineStr">
         <is>
-          <t>Posting / Account-Determination Engine: two tables — posting_event_types (28 seeded event types, e.g. SALE.FOOD, GR.INVENTORY, DEPRECIATION.FA) and posting_rules (maps event × leg-order to semantic role → account_code + DR/CR side) — drive account assignment instead of hard-coded literals. PostingService.post(eventType, ctx) resolves the applicable rules (global defaults, or shadowed by tenant-specific overrides for the same leg_order), translates role-keyed amounts into DR/CR lines, and delegates to LedgerService.postEntry. If no active rules exist for an event the call fails with NO_POSTING_RULE. Tenant-specific rules require gl_posting_rules permission to create/update. PostingService.preview() provides a dry-run for audit.</t>
+          <t>CoA Change Control: account creation/update/deactivation requires the gl_coa permission (held by FinancialController, not GlAccountant — separated from gl_post per SoD). Disabling postability on an account that already has posted entries is rejected (CODE_HAS_POSTINGS). Deactivation is rejected if the account carries a non-zero net balance (ACCOUNT_HAS_BALANCE) — prevents orphaning a balance in a closed account. Four accounts are flagged is_control=true at setup: 1100 (AR), 2000 (AP), 1200 (INV), 1500 (FA); a direct manual JE that touches any of these without viaSubledger:true is rejected (CONTROL_ACCOUNT), ensuring AR/AP/INV/FA balances are exclusively maintained by their respective sub-ledger service methods.</t>
         </is>
       </c>
       <c r="H93" s="17" t="inlineStr">
@@ -8947,22 +8947,22 @@
       </c>
       <c r="M93" s="16" t="inlineStr">
         <is>
-          <t>posting.service.ts (resolveRules, post, preview, listEventTypes, listRules, upsertRule); posting-rules.controller.ts (gl_posting_rules permission gate); schema/posting-rules.ts (posting_event_types, posting_rules tables); migration 0156 (tables + 28 event types + global-default rules); ledger.module.ts (PostingService exported); packages/shared/src/permissions.ts (gl_posting_rules sub-permission); cutover/basics.ts (golden-snapshot ToE)</t>
+          <t>coa.service.ts (createAccount DUPLICATE_ACCOUNT, updateAccount CODE_HAS_POSTINGS, deactivateAccount ACCOUNT_HAS_BALANCE); coa.controller.ts (gl_coa permission gate); ledger.service.ts postEntry control-account guard (CONTROL_ACCOUNT, viaSubledger flag); schema/ledger.ts (account_groups table, accounts.is_control/control_subledger/is_postable/normal_balance + migration 0155); packages/shared/src/permissions.ts (gl_coa sub-permission, FinancialController default)</t>
         </is>
       </c>
       <c r="N93" s="16" t="inlineStr">
         <is>
-          <t>Inspect the rule-resolution logic + NO_POSTING_RULE fast-fail + tenant-shadow logic + gl_posting_rules permission gate.</t>
+          <t>Inspect gl_coa permission gate + CODE_HAS_POSTINGS guard + ACCOUNT_HAS_BALANCE guard + CONTROL_ACCOUNT guard + viaSubledger bypass.</t>
         </is>
       </c>
       <c r="O93" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: preview DEPRECIATION.FA with dep_expense:1000 → DR 5200 / CR 1590; preview GR.INVENTORY with inventory:500 → DR 1200 / CR 2000; preview UNKNOWN_EVENT → NO_POSTING_RULE (400); event-type catalogue returns ≥20 entries (re-performed by TC-GL-12-01/02/03/04 UAT cases + basics.ts harness).</t>
+          <t>Re-perform: create an account with gl_coa → 201; attempt to deactivate an account with balance → ACCOUNT_HAS_BALANCE; post directly to account 1100 without viaSubledger → CONTROL_ACCOUNT (re-performed by TC-GL-11-01/02/03 UAT cases).</t>
         </is>
       </c>
       <c r="P93" s="16" t="inlineStr">
         <is>
-          <t>Posting-rule change log; preview dry-run; harness golden snapshot</t>
+          <t>CoA change log (audit_log); permission test; control-account guard test</t>
         </is>
       </c>
       <c r="Q93" s="18" t="inlineStr">
@@ -8974,7 +8974,7 @@
     <row r="94">
       <c r="A94" s="11" t="inlineStr">
         <is>
-          <t>GL-13</t>
+          <t>GL-12</t>
         </is>
       </c>
       <c r="B94" s="12" t="inlineStr">
@@ -8994,22 +8994,22 @@
       </c>
       <c r="E94" s="12" t="inlineStr">
         <is>
-          <t>Revenue or expense mis-attributed to the wrong branch / project — per-location P&amp;L is unintelligible or misleading.</t>
+          <t>Account-assignment errors introduced by scattered inline account-code literals in service code; a tenant needing a different account for a given business event has no mechanism to override without a code change.</t>
         </is>
       </c>
       <c r="F94" s="12" t="inlineStr">
         <is>
-          <t>Accuracy/Presentation</t>
+          <t>Authorization/Accuracy</t>
         </is>
       </c>
       <c r="G94" s="12" t="inlineStr">
         <is>
-          <t>Multi-dimensional GL postings: journal_lines carries three optional dimension columns (branch_id, project_id, department_id). PostingService.post() stamps all generated lines from PostingContext (branchId/projectId/departmentId). GET /api/ledger/income-statement/by-branch provides a per-branch P&amp;L view; lines without a branch_id are grouped as 'unassigned'. The departments master table holds a tenant-scoped department registry with RLS isolation.</t>
+          <t>Posting / Account-Determination Engine: two tables — posting_event_types (28 seeded event types, e.g. SALE.FOOD, GR.INVENTORY, DEPRECIATION.FA) and posting_rules (maps event × leg-order to semantic role → account_code + DR/CR side) — drive account assignment instead of hard-coded literals. PostingService.post(eventType, ctx) resolves the applicable rules (global defaults, or shadowed by tenant-specific overrides for the same leg_order), translates role-keyed amounts into DR/CR lines, and delegates to LedgerService.postEntry. If no active rules exist for an event the call fails with NO_POSTING_RULE. Tenant-specific rules require gl_posting_rules permission to create/update. PostingService.preview() provides a dry-run for audit.</t>
         </is>
       </c>
       <c r="H94" s="13" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I94" s="13" t="inlineStr">
@@ -9019,12 +9019,12 @@
       </c>
       <c r="J94" s="13" t="inlineStr">
         <is>
-          <t>Per period</t>
+          <t>Event-driven</t>
         </is>
       </c>
       <c r="K94" s="12" t="inlineStr">
         <is>
-          <t>Controller</t>
+          <t>Financial Controller</t>
         </is>
       </c>
       <c r="L94" s="13" t="inlineStr">
@@ -9034,22 +9034,22 @@
       </c>
       <c r="M94" s="12" t="inlineStr">
         <is>
-          <t>ledger.service.ts (incomeStatementByBranch); ledger.controller.ts (GET income-statement/by-branch); posting.service.ts (branchId/projectId/departmentId from PostingContext); schema/ledger.ts (branch_id, project_id, department_id on journal_lines); schema/departments.ts (departments table); migration 0157; cutover/basics.ts (GL-13 ToE)</t>
+          <t>posting.service.ts (resolveRules, post, preview, listEventTypes, listRules, upsertRule); posting-rules.controller.ts (gl_posting_rules permission gate); schema/posting-rules.ts (posting_event_types, posting_rules tables); migration 0156 (tables + 28 event types + global-default rules); ledger.module.ts (PostingService exported); packages/shared/src/permissions.ts (gl_posting_rules sub-permission); cutover/basics.ts (golden-snapshot ToE)</t>
         </is>
       </c>
       <c r="N94" s="12" t="inlineStr">
         <is>
-          <t>Inspect by-branch query + PostingContext stamping + department RLS.</t>
+          <t>Inspect the rule-resolution logic + NO_POSTING_RULE fast-fail + tenant-shadow logic + gl_posting_rules permission gate.</t>
         </is>
       </c>
       <c r="O94" s="12" t="inlineStr">
         <is>
-          <t>TC-GL-13-01/02/03: smoke + two branches + unassigned bucket (re-performed by the basics.ts harness).</t>
+          <t>Re-perform: preview DEPRECIATION.FA with dep_expense:1000 → DR 5200 / CR 1590; preview GR.INVENTORY with inventory:500 → DR 1200 / CR 2000; preview UNKNOWN_EVENT → NO_POSTING_RULE (400); event-type catalogue returns ≥20 entries (re-performed by TC-GL-12-01/02/03/04 UAT cases + basics.ts harness).</t>
         </is>
       </c>
       <c r="P94" s="12" t="inlineStr">
         <is>
-          <t>By-branch P&amp;L report; dimension completeness</t>
+          <t>Posting-rule change log; preview dry-run; harness golden snapshot</t>
         </is>
       </c>
       <c r="Q94" s="18" t="inlineStr">
@@ -9061,7 +9061,7 @@
     <row r="95">
       <c r="A95" s="15" t="inlineStr">
         <is>
-          <t>GL-14</t>
+          <t>GL-13</t>
         </is>
       </c>
       <c r="B95" s="16" t="inlineStr">
@@ -9081,17 +9081,17 @@
       </c>
       <c r="E95" s="16" t="inlineStr">
         <is>
-          <t>GL control-account balances (AR/AP/INV/FA) drift from the underlying sub-ledger detail without detection — the control account no longer represents the sum of its sub-ledger, masking posting errors, unrecorded items, or fraud.</t>
+          <t>Revenue or expense mis-attributed to the wrong branch / project — per-location P&amp;L is unintelligible or misleading.</t>
         </is>
       </c>
       <c r="F95" s="16" t="inlineStr">
         <is>
-          <t>Completeness/Accuracy/Valuation</t>
+          <t>Accuracy/Presentation</t>
         </is>
       </c>
       <c r="G95" s="16" t="inlineStr">
         <is>
-          <t>Sub-ledger tie-out / reconciliation: POST /api/ledger/tie-out/run computes, per control account, the GL balance (Σ debit−credit of posted journal_lines on the control account up to the as-of date, tenant-scoped) and the sub-ledger detail balance (AR = Σ outstanding ar_invoices; AP = Σ outstanding ap_transactions; INV = Σ inv_balances.total_value perpetual valuation; FA = Σ acquire_cost − accumulated_depreciation of non-disposed fixed_assets), records the variance (gl − subledger) and a status (Matched if |variance|&lt;0.01 else Variance). Runs upsert per (tenant, subledger, as-of). Certification is maker-checker: POST /api/ledger/tie-out/:id/certify sets status=Certified and records certifier + timestamp, and REJECTS a certifier equal to the runner (SELF_CERTIFY) — the gl_close certifier must differ from the gl_post/gl_close runner (SoD).</t>
+          <t>Multi-dimensional GL postings: journal_lines carries three optional dimension columns (branch_id, project_id, department_id). PostingService.post() stamps all generated lines from PostingContext (branchId/projectId/departmentId). GET /api/ledger/income-statement/by-branch provides a per-branch P&amp;L view; lines without a branch_id are grouped as 'unassigned'. The departments master table holds a tenant-scoped department registry with RLS isolation.</t>
         </is>
       </c>
       <c r="H95" s="17" t="inlineStr">
@@ -9106,12 +9106,12 @@
       </c>
       <c r="J95" s="17" t="inlineStr">
         <is>
-          <t>Monthly</t>
+          <t>Per period</t>
         </is>
       </c>
       <c r="K95" s="16" t="inlineStr">
         <is>
-          <t>Financial Controller</t>
+          <t>Controller</t>
         </is>
       </c>
       <c r="L95" s="17" t="inlineStr">
@@ -9121,22 +9121,22 @@
       </c>
       <c r="M95" s="16" t="inlineStr">
         <is>
-          <t>subledger-tieout.service.ts (runTieOut GL/sub-ledger balance computation + variance/status, certify SELF_CERTIFY maker-checker, list/get); subledger-tieout.controller.ts (gl_close/gl_post run, gl_close certify, gl_close/gl_post/exec/creditors/ar read); schema/subledger-tieout.ts (subledger_tieout_runs table, uq on tenant/subledger/as-of); migration 0160 (table + RLS); ledger.module.ts (service+controller wired); cutover/basics.ts (GL-14 ToE)</t>
+          <t>ledger.service.ts (incomeStatementByBranch); ledger.controller.ts (GET income-statement/by-branch); posting.service.ts (branchId/projectId/departmentId from PostingContext); schema/ledger.ts (branch_id, project_id, department_id on journal_lines); schema/departments.ts (departments table); migration 0157; cutover/basics.ts (GL-13 ToE)</t>
         </is>
       </c>
       <c r="N95" s="16" t="inlineStr">
         <is>
-          <t>Inspect the GL-vs-sub-ledger balance computation + variance/status + SELF_CERTIFY maker-checker gate + gl_close certify permission.</t>
+          <t>Inspect by-branch query + PostingContext stamping + department RLS.</t>
         </is>
       </c>
       <c r="O95" s="16" t="inlineStr">
         <is>
-          <t>TC-GL-14-01: run AR tie-out → balances + Matched/Variance; TC-GL-14-02: self-certify by the runner → SELF_CERTIFY (400); TC-GL-14-03: certify by a different gl_close user → Certified (re-performed by the basics.ts harness).</t>
+          <t>TC-GL-13-01/02/03: smoke + two branches + unassigned bucket (re-performed by the basics.ts harness).</t>
         </is>
       </c>
       <c r="P95" s="16" t="inlineStr">
         <is>
-          <t>Tie-out run log (subledger_tieout_runs) with variance + certification trail; monthly reconciliation sign-off</t>
+          <t>By-branch P&amp;L report; dimension completeness</t>
         </is>
       </c>
       <c r="Q95" s="18" t="inlineStr">
@@ -9148,7 +9148,7 @@
     <row r="96">
       <c r="A96" s="11" t="inlineStr">
         <is>
-          <t>GL-15</t>
+          <t>GL-14</t>
         </is>
       </c>
       <c r="B96" s="12" t="inlineStr">
@@ -9168,22 +9168,22 @@
       </c>
       <c r="E96" s="12" t="inlineStr">
         <is>
-          <t>A period is 'closed' on paper but key close procedures (sub-ledger tie-out, bank rec, depreciation, recurring/prepaid, trial-balance review) were skipped, OR a closed period is silently re-opened and re-posted — the financial statements are produced on an incomplete/altered basis.</t>
+          <t>GL control-account balances (AR/AP/INV/FA) drift from the underlying sub-ledger detail without detection — the control account no longer represents the sum of its sub-ledger, masking posting errors, unrecorded items, or fraud.</t>
         </is>
       </c>
       <c r="F96" s="12" t="inlineStr">
         <is>
-          <t>Completeness/Accuracy/Cutoff</t>
+          <t>Completeness/Accuracy/Valuation</t>
         </is>
       </c>
       <c r="G96" s="12" t="inlineStr">
         <is>
-          <t>Hard period close + checklist: POST /api/ledger/close/start opens a close_runs record (status InProgress) per (tenant, period) and seeds a standard checklist of close_run_steps (subledger_tieout, bank_rec, depreciation, recurring, fx_reval[advisory], trial_balance_review). POST /api/ledger/close/step marks a step Done (records completedBy/At); when all REQUIRED steps are Done the run advances to ReadyToLock. POST /api/ledger/close/lock requires ReadyToLock (else STEPS_INCOMPLETE listing the pending required steps) before the period can be locked. Locking writes 'Locked' into fiscal_periods.status; LedgerService.postEntry then REJECTS every posting dated into a Locked period with PERIOD_LOCKED, regardless of the legacy allowClosedPeriod escape (the only exception is the system year-end closing entry, source='CLOSE'). Locked is strictly stronger than the soft 'Closed' status — it is the irreversible hard close.</t>
+          <t>Sub-ledger tie-out / reconciliation: POST /api/ledger/tie-out/run computes, per control account, the GL balance (Σ debit−credit of posted journal_lines on the control account up to the as-of date, tenant-scoped) and the sub-ledger detail balance (AR = Σ outstanding ar_invoices; AP = Σ outstanding ap_transactions; INV = Σ inv_balances.total_value perpetual valuation; FA = Σ acquire_cost − accumulated_depreciation of non-disposed fixed_assets), records the variance (gl − subledger) and a status (Matched if |variance|&lt;0.01 else Variance). Runs upsert per (tenant, subledger, as-of). Certification is maker-checker: POST /api/ledger/tie-out/:id/certify sets status=Certified and records certifier + timestamp, and REJECTS a certifier equal to the runner (SELF_CERTIFY) — the gl_close certifier must differ from the gl_post/gl_close runner (SoD).</t>
         </is>
       </c>
       <c r="H96" s="13" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I96" s="13" t="inlineStr">
@@ -9208,22 +9208,22 @@
       </c>
       <c r="M96" s="12" t="inlineStr">
         <is>
-          <t>close.service.ts (startClose seeds checklist, completeStep → ReadyToLock when required steps Done, lockPeriod STEPS_INCOMPLETE gate + fiscal_periods Locked write, status/list); close.controller.ts (gl_close start/step/lock, gl_close/gl_post/exec read); schema/close-runs.ts (close_runs + close_run_steps, uq on tenant/period and run/step_key); schema/ledger.ts (period_status enum + 'Locked'); ledger.service.ts (postEntry PERIOD_LOCKED hard gate, source='CLOSE' exemption); migration 0162 (tables + RLS + ALTER TYPE Locked); ledger.module.ts (service+controller wired); cutover/basics.ts (GL-15/GL-16 ToE)</t>
+          <t>subledger-tieout.service.ts (runTieOut GL/sub-ledger balance computation + variance/status, certify SELF_CERTIFY maker-checker, list/get); subledger-tieout.controller.ts (gl_close/gl_post run, gl_close certify, gl_close/gl_post/exec/creditors/ar read); schema/subledger-tieout.ts (subledger_tieout_runs table, uq on tenant/subledger/as-of); migration 0160 (table + RLS); ledger.module.ts (service+controller wired); cutover/basics.ts (GL-14 ToE)</t>
         </is>
       </c>
       <c r="N96" s="12" t="inlineStr">
         <is>
-          <t>Inspect the seeded checklist + ReadyToLock gating + STEPS_INCOMPLETE lock rejection + PERIOD_LOCKED hard gate in postEntry (incl. the CLOSE exemption).</t>
+          <t>Inspect the GL-vs-sub-ledger balance computation + variance/status + SELF_CERTIFY maker-checker gate + gl_close certify permission.</t>
         </is>
       </c>
       <c r="O96" s="12" t="inlineStr">
         <is>
-          <t>TC-GL-15-01: start close seeds ≥4 steps (InProgress); TC-GL-15-02: lock before steps done → STEPS_INCOMPLETE (400); TC-GL-15-03: post into locked period → PERIOD_LOCKED (400) (re-performed by the basics.ts harness).</t>
+          <t>TC-GL-14-01: run AR tie-out → balances + Matched/Variance; TC-GL-14-02: self-certify by the runner → SELF_CERTIFY (400); TC-GL-14-03: certify by a different gl_close user → Certified (re-performed by the basics.ts harness).</t>
         </is>
       </c>
       <c r="P96" s="12" t="inlineStr">
         <is>
-          <t>close_runs / close_run_steps with completion trail; fiscal_periods.status=Locked; monthly close sign-off</t>
+          <t>Tie-out run log (subledger_tieout_runs) with variance + certification trail; monthly reconciliation sign-off</t>
         </is>
       </c>
       <c r="Q96" s="18" t="inlineStr">
@@ -9235,7 +9235,7 @@
     <row r="97">
       <c r="A97" s="15" t="inlineStr">
         <is>
-          <t>GL-16</t>
+          <t>GL-15</t>
         </is>
       </c>
       <c r="B97" s="16" t="inlineStr">
@@ -9255,17 +9255,17 @@
       </c>
       <c r="E97" s="16" t="inlineStr">
         <is>
-          <t>One person both performs the close and locks the period, defeating segregation of duties — a preparer could conceal a misstatement by closing over their own work without independent review.</t>
+          <t>A period is 'closed' on paper but key close procedures (sub-ledger tie-out, bank rec, depreciation, recurring/prepaid, trial-balance review) were skipped, OR a closed period is silently re-opened and re-posted — the financial statements are produced on an incomplete/altered basis.</t>
         </is>
       </c>
       <c r="F97" s="16" t="inlineStr">
         <is>
-          <t>Authorization/Segregation of Duties</t>
+          <t>Completeness/Accuracy/Cutoff</t>
         </is>
       </c>
       <c r="G97" s="16" t="inlineStr">
         <is>
-          <t>Segregated period lock (maker-checker): the close_runs.started_by (the user who started the close and ran the checklist steps) is recorded, and POST /api/ledger/close/lock REJECTS a lockedBy equal to startedBy with SELF_LOCK — the gl_close user who locks the period MUST differ from the user who started/ran the close. Both identities and the lock timestamp are retained on the close_runs row (started_by / locked_by / locked_at) as the SoD evidence trail. This complements the existing SoD rule that gl_close is segregated from gl_post (JE posting).</t>
+          <t>Hard period close + checklist: POST /api/ledger/close/start opens a close_runs record (status InProgress) per (tenant, period) and seeds a standard checklist of close_run_steps (subledger_tieout, bank_rec, depreciation, recurring, fx_reval[advisory], trial_balance_review). POST /api/ledger/close/step marks a step Done (records completedBy/At); when all REQUIRED steps are Done the run advances to ReadyToLock. POST /api/ledger/close/lock requires ReadyToLock (else STEPS_INCOMPLETE listing the pending required steps) before the period can be locked. Locking writes 'Locked' into fiscal_periods.status; LedgerService.postEntry then REJECTS every posting dated into a Locked period with PERIOD_LOCKED, regardless of the legacy allowClosedPeriod escape (the only exception is the system year-end closing entry, source='CLOSE'). Locked is strictly stronger than the soft 'Closed' status — it is the irreversible hard close.</t>
         </is>
       </c>
       <c r="H97" s="17" t="inlineStr">
@@ -9295,22 +9295,22 @@
       </c>
       <c r="M97" s="16" t="inlineStr">
         <is>
-          <t>close.service.ts (lockPeriod SELF_LOCK maker-checker gate; started_by vs locked_by); close.controller.ts (gl_close lock, acting username from JWT); schema/close-runs.ts (started_by, locked_by, locked_at columns); permissions.ts (gl_post×gl_close SoD pair); cutover/basics.ts (GL-16 ToE)</t>
+          <t>close.service.ts (startClose seeds checklist, completeStep → ReadyToLock when required steps Done, lockPeriod STEPS_INCOMPLETE gate + fiscal_periods Locked write, status/list); close.controller.ts (gl_close start/step/lock, gl_close/gl_post/exec read); schema/close-runs.ts (close_runs + close_run_steps, uq on tenant/period and run/step_key); schema/ledger.ts (period_status enum + 'Locked'); ledger.service.ts (postEntry PERIOD_LOCKED hard gate, source='CLOSE' exemption); migration 0162 (tables + RLS + ALTER TYPE Locked); ledger.module.ts (service+controller wired); cutover/basics.ts (GL-15/GL-16 ToE)</t>
         </is>
       </c>
       <c r="N97" s="16" t="inlineStr">
         <is>
-          <t>Inspect the SELF_LOCK gate (startedBy ≠ lockedBy) + the started_by/locked_by/locked_at evidence trail.</t>
+          <t>Inspect the seeded checklist + ReadyToLock gating + STEPS_INCOMPLETE lock rejection + PERIOD_LOCKED hard gate in postEntry (incl. the CLOSE exemption).</t>
         </is>
       </c>
       <c r="O97" s="16" t="inlineStr">
         <is>
-          <t>TC-GL-16-01: self-lock by the starter → SELF_LOCK (400); TC-GL-16-02: lock by a different gl_close user → Locked, locked_by recorded (re-performed by the basics.ts harness).</t>
+          <t>TC-GL-15-01: start close seeds ≥4 steps (InProgress); TC-GL-15-02: lock before steps done → STEPS_INCOMPLETE (400); TC-GL-15-03: post into locked period → PERIOD_LOCKED (400) (re-performed by the basics.ts harness).</t>
         </is>
       </c>
       <c r="P97" s="16" t="inlineStr">
         <is>
-          <t>close_runs.started_by / locked_by / locked_at SoD trail; monthly close sign-off</t>
+          <t>close_runs / close_run_steps with completion trail; fiscal_periods.status=Locked; monthly close sign-off</t>
         </is>
       </c>
       <c r="Q97" s="18" t="inlineStr">
@@ -9322,7 +9322,7 @@
     <row r="98">
       <c r="A98" s="11" t="inlineStr">
         <is>
-          <t>GL-17</t>
+          <t>GL-16</t>
         </is>
       </c>
       <c r="B98" s="12" t="inlineStr">
@@ -9342,17 +9342,17 @@
       </c>
       <c r="E98" s="12" t="inlineStr">
         <is>
-          <t>A posted journal entry is edited or deleted after the fact — restating history with no trail — instead of being corrected by a transparent reversal; or a correction is made with no record of who/what/why. The general ledger is no longer an immutable, auditable record of record.</t>
+          <t>One person both performs the close and locks the period, defeating segregation of duties — a preparer could conceal a misstatement by closing over their own work without independent review.</t>
         </is>
       </c>
       <c r="F98" s="12" t="inlineStr">
         <is>
-          <t>Completeness/Accuracy/Authorization</t>
+          <t>Authorization/Segregation of Duties</t>
         </is>
       </c>
       <c r="G98" s="12" t="inlineStr">
         <is>
-          <t>Posted-entry immutability + reversal-only correction + GL audit trail: a journal entry that has reached Posted status is IMMUTABLE — it can never be edited or deleted. Enforcement is twofold: (1) a production DB trigger (gl_block_posted_mutation) that RAISES on any UPDATE/DELETE of a Posted journal_entries row (permitting only the is_reversed bookkeeping flag flip), and (2) an application-level guard (attemptVoidPosted → GL_IMMUTABLE) that refuses and records any mutation attempt. The ONLY way to correct a posted entry is a REVERSAL: reverseEntry posts a NEW, immediately-Posted contra entry that swaps every line's debit/credit (so original + reversal net to zero on every affected account), dimensions carried over, linked via reversal_of, and flags the original is_reversed. A reversal goes through the normal posting path so the period gates (PERIOD_LOCKED/PERIOD_CLOSED) still apply; only Posted entries can be reversed (NOT_POSTED) and only once (ALREADY_REVERSED). Every POST, APPROVE, REVERSE and blocked mutation (MUTATE_BLOCKED) is recorded with actor + detail + timestamp in gl_audit_log (tenant-scoped, RLS).</t>
+          <t>Segregated period lock (maker-checker): the close_runs.started_by (the user who started the close and ran the checklist steps) is recorded, and POST /api/ledger/close/lock REJECTS a lockedBy equal to startedBy with SELF_LOCK — the gl_close user who locks the period MUST differ from the user who started/ran the close. Both identities and the lock timestamp are retained on the close_runs row (started_by / locked_by / locked_at) as the SoD evidence trail. This complements the existing SoD rule that gl_close is segregated from gl_post (JE posting).</t>
         </is>
       </c>
       <c r="H98" s="13" t="inlineStr">
@@ -9367,7 +9367,7 @@
       </c>
       <c r="J98" s="13" t="inlineStr">
         <is>
-          <t>Per entry / continuous</t>
+          <t>Monthly</t>
         </is>
       </c>
       <c r="K98" s="12" t="inlineStr">
@@ -9382,22 +9382,22 @@
       </c>
       <c r="M98" s="12" t="inlineStr">
         <is>
-          <t>ledger.service.ts (postEntry stamps posted_at + logs POST; approveEntry stamps posted_at + logs APPROVE; reverseEntry contra-posting with ENTRY_NOT_FOUND/NOT_POSTED/ALREADY_REVERSED + REVERSE log; attemptVoidPosted GL_IMMUTABLE + MUTATE_BLOCKED log; listGlAudit); ledger.controller.ts (gl_post journal/:id/reverse + journal/:id/attempt-void, gl_post/gl_close/exec audit read); schema/ledger.ts (journal_entries posted_at/reversal_of/is_reversed); schema/gl-audit.ts (gl_audit_log table); migration 0164 (columns + gl_audit_log + RLS + gl_block_posted_mutation trigger); ledger.module.ts (LedgerService owns it); cutover/basics.ts (GL-17 ToE)</t>
+          <t>close.service.ts (lockPeriod SELF_LOCK maker-checker gate; started_by vs locked_by); close.controller.ts (gl_close lock, acting username from JWT); schema/close-runs.ts (started_by, locked_by, locked_at columns); permissions.ts (gl_post×gl_close SoD pair); cutover/basics.ts (GL-16 ToE)</t>
         </is>
       </c>
       <c r="N98" s="12" t="inlineStr">
         <is>
-          <t>Inspect the DB immutability trigger + the app GL_IMMUTABLE guard + the reversal contra-posting (swapped Dr/Cr, reversal_of, is_reversed) + the gl_audit_log trail (POST/APPROVE/REVERSE/MUTATE_BLOCKED).</t>
+          <t>Inspect the SELF_LOCK gate (startedBy ≠ lockedBy) + the started_by/locked_by/locked_at evidence trail.</t>
         </is>
       </c>
       <c r="O98" s="12" t="inlineStr">
         <is>
-          <t>TC-GL-17-01: attempt to void a posted entry → GL_IMMUTABLE (400) + MUTATE_BLOCKED audit row; TC-GL-17-02: reverse a posted entry → contra entry nets to zero, original is_reversed + REVERSE audit row; TC-GL-17-03: reverse again → ALREADY_REVERSED (400) (re-performed by the basics.ts harness).</t>
+          <t>TC-GL-16-01: self-lock by the starter → SELF_LOCK (400); TC-GL-16-02: lock by a different gl_close user → Locked, locked_by recorded (re-performed by the basics.ts harness).</t>
         </is>
       </c>
       <c r="P98" s="12" t="inlineStr">
         <is>
-          <t>gl_audit_log trail (POST/APPROVE/REVERSE/MUTATE_BLOCKED); reversal entries with reversal_of linkage; posted-entry immutability</t>
+          <t>close_runs.started_by / locked_by / locked_at SoD trail; monthly close sign-off</t>
         </is>
       </c>
       <c r="Q98" s="18" t="inlineStr">
@@ -9409,12 +9409,12 @@
     <row r="99">
       <c r="A99" s="15" t="inlineStr">
         <is>
-          <t>EXP-07</t>
+          <t>GL-17</t>
         </is>
       </c>
       <c r="B99" s="16" t="inlineStr">
         <is>
-          <t>Expenditure</t>
+          <t>General Ledger</t>
         </is>
       </c>
       <c r="C99" s="17" t="inlineStr">
@@ -9424,27 +9424,27 @@
       </c>
       <c r="D99" s="16" t="inlineStr">
         <is>
-          <t>Cash; Operating expense</t>
+          <t>All</t>
         </is>
       </c>
       <c r="E99" s="16" t="inlineStr">
         <is>
-          <t>Petty-cash / employee advance issued but never accounted for — cash leakage, expense unrecorded.</t>
+          <t>A posted journal entry is edited or deleted after the fact — restating history with no trail — instead of being corrected by a transparent reversal; or a correction is made with no record of who/what/why. The general ledger is no longer an immutable, auditable record of record.</t>
         </is>
       </c>
       <c r="F99" s="16" t="inlineStr">
         <is>
-          <t>Existence/Completeness</t>
+          <t>Completeness/Accuracy/Authorization</t>
         </is>
       </c>
       <c r="G99" s="16" t="inlineStr">
         <is>
-          <t>Employee cash advances: issuing an advance debits the 1180 Employee Advances control (Dr 1180 / Cr 1000); settlement clears it against actual spend + returned cash (Dr expense + Dr 1000 / Cr 1180), enforced to reconcile (settled_expense + returned_cash must equal the advance → SETTLE_MISMATCH). The 1180 balance is the outstanding float subject to review.</t>
+          <t>Posted-entry immutability + reversal-only correction + GL audit trail: a journal entry that has reached Posted status is IMMUTABLE — it can never be edited or deleted. Enforcement is twofold: (1) a production DB trigger (gl_block_posted_mutation) that RAISES on any UPDATE/DELETE of a Posted journal_entries row (permitting only the is_reversed bookkeeping flag flip), and (2) an application-level guard (attemptVoidPosted → GL_IMMUTABLE) that refuses and records any mutation attempt. The ONLY way to correct a posted entry is a REVERSAL: reverseEntry posts a NEW, immediately-Posted contra entry that swaps every line's debit/credit (so original + reversal net to zero on every affected account), dimensions carried over, linked via reversal_of, and flags the original is_reversed. A reversal goes through the normal posting path so the period gates (PERIOD_LOCKED/PERIOD_CLOSED) still apply; only Posted entries can be reversed (NOT_POSTED) and only once (ALREADY_REVERSED). Every POST, APPROVE, REVERSE and blocked mutation (MUTATE_BLOCKED) is recorded with actor + detail + timestamp in gl_audit_log (tenant-scoped, RLS).</t>
         </is>
       </c>
       <c r="H99" s="17" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I99" s="17" t="inlineStr">
@@ -9454,12 +9454,12 @@
       </c>
       <c r="J99" s="17" t="inlineStr">
         <is>
-          <t>Per advance</t>
+          <t>Per entry / continuous</t>
         </is>
       </c>
       <c r="K99" s="16" t="inlineStr">
         <is>
-          <t>AP / Controller</t>
+          <t>Financial Controller</t>
         </is>
       </c>
       <c r="L99" s="17" t="inlineStr">
@@ -9469,22 +9469,22 @@
       </c>
       <c r="M99" s="16" t="inlineStr">
         <is>
-          <t>finance.service.ts (issueAdvance, settleAdvance reconcile-or-reject, listAdvances outstanding); finance.controller.ts (creditors/exec); schema/finance.ts (employee_advances) + migration 0120; cutover/basics.ts (ToE)</t>
+          <t>ledger.service.ts (postEntry stamps posted_at + logs POST; approveEntry stamps posted_at + logs APPROVE; reverseEntry contra-posting with ENTRY_NOT_FOUND/NOT_POSTED/ALREADY_REVERSED + REVERSE log; attemptVoidPosted GL_IMMUTABLE + MUTATE_BLOCKED log; listGlAudit); ledger.controller.ts (gl_post journal/:id/reverse + journal/:id/attempt-void, gl_post/gl_close/exec audit read); schema/ledger.ts (journal_entries posted_at/reversal_of/is_reversed); schema/gl-audit.ts (gl_audit_log table); migration 0164 (columns + gl_audit_log + RLS + gl_block_posted_mutation trigger); ledger.module.ts (LedgerService owns it); cutover/basics.ts (GL-17 ToE)</t>
         </is>
       </c>
       <c r="N99" s="16" t="inlineStr">
         <is>
-          <t>Inspect issue/settle GL + settlement reconciliation guard.</t>
+          <t>Inspect the DB immutability trigger + the app GL_IMMUTABLE guard + the reversal contra-posting (swapped Dr/Cr, reversal_of, is_reversed) + the gl_audit_log trail (POST/APPROVE/REVERSE/MUTATE_BLOCKED).</t>
         </is>
       </c>
       <c r="O99" s="16" t="inlineStr">
         <is>
-          <t>Issue an advance (1180 up); settle 700+300 clears 1180; mismatched settle → SETTLE_MISMATCH (re-performed by the harness).</t>
+          <t>TC-GL-17-01: attempt to void a posted entry → GL_IMMUTABLE (400) + MUTATE_BLOCKED audit row; TC-GL-17-02: reverse a posted entry → contra entry nets to zero, original is_reversed + REVERSE audit row; TC-GL-17-03: reverse again → ALREADY_REVERSED (400) (re-performed by the basics.ts harness).</t>
         </is>
       </c>
       <c r="P99" s="16" t="inlineStr">
         <is>
-          <t>Advance register; outstanding float</t>
+          <t>gl_audit_log trail (POST/APPROVE/REVERSE/MUTATE_BLOCKED); reversal entries with reversal_of linkage; posted-entry immutability</t>
         </is>
       </c>
       <c r="Q99" s="18" t="inlineStr">
@@ -9496,7 +9496,7 @@
     <row r="100">
       <c r="A100" s="11" t="inlineStr">
         <is>
-          <t>EXP-08</t>
+          <t>EXP-07</t>
         </is>
       </c>
       <c r="B100" s="12" t="inlineStr">
@@ -9516,22 +9516,22 @@
       </c>
       <c r="E100" s="12" t="inlineStr">
         <is>
-          <t>Petty-cash disbursed beyond authority / without independent review, or drawn past the fund's limit — cash leakage, unauthorised or unrecorded expense, over-extended float.</t>
+          <t>Petty-cash / employee advance issued but never accounted for — cash leakage, expense unrecorded.</t>
         </is>
       </c>
       <c r="F100" s="12" t="inlineStr">
         <is>
-          <t>Authorization; Completeness</t>
+          <t>Existence/Completeness</t>
         </is>
       </c>
       <c r="G100" s="12" t="inlineStr">
         <is>
-          <t>Petty-cash imprest float + maker-checker on disbursement (SoD): a fund holds cash capped at a credit limit/วงเงิน (1015 Petty Cash, a cash account); each direct EXPENSE or ADVANCE is a REQUEST that posts NOTHING and a DIFFERENT user must approve before the GL posts (expense Dr &lt;expense&gt; / Cr 1015; advance Dr 1180 / Cr 1015) and the fund balance is decremented. Self-approval → SOD_VIOLATION (binds even Admin). A draw beyond the fund balance → INSUFFICIENT_FLOAT; establishing/replenishing above the float limit → OVER_FLOAT. Advances settle (Dr expense + Dr 1015 returned / Cr 1180), returning unused cash to the fund. Every request carries a document reference + receipt key + a status trail (StatusLog) and surfaces in the GOV-01 pending-approvals monitor.</t>
+          <t>Employee cash advances: issuing an advance debits the 1180 Employee Advances control (Dr 1180 / Cr 1000); settlement clears it against actual spend + returned cash (Dr expense + Dr 1000 / Cr 1180), enforced to reconcile (settled_expense + returned_cash must equal the advance → SETTLE_MISMATCH). The 1180 balance is the outstanding float subject to review.</t>
         </is>
       </c>
       <c r="H100" s="13" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I100" s="13" t="inlineStr">
@@ -9541,7 +9541,7 @@
       </c>
       <c r="J100" s="13" t="inlineStr">
         <is>
-          <t>Per disbursement</t>
+          <t>Per advance</t>
         </is>
       </c>
       <c r="K100" s="12" t="inlineStr">
@@ -9556,22 +9556,22 @@
       </c>
       <c r="M100" s="12" t="inlineStr">
         <is>
-          <t>petty-cash.service.ts (establishFund/replenishFund float guards, createRequest INSUFFICIENT_FLOAT, approveRequest SoD+GL, rejectRequest, settleRequest); petty-cash.controller.ts (creditors/exec); schema/petty-cash.ts (petty_cash_funds, expense_requests) + migration 0139; finance.service.ts pendingApprovals (GOV-01 source 7); cutover/basics.ts + compliance.ts (ToE)</t>
+          <t>finance.service.ts (issueAdvance, settleAdvance reconcile-or-reject, listAdvances outstanding); finance.controller.ts (creditors/exec); schema/finance.ts (employee_advances) + migration 0120; cutover/basics.ts (ToE)</t>
         </is>
       </c>
       <c r="N100" s="12" t="inlineStr">
         <is>
-          <t>Inspect the float ceiling + the request→approve flow + the approver≠requester check + that the request posts nothing until approval.</t>
+          <t>Inspect issue/settle GL + settlement reconciliation guard.</t>
         </is>
       </c>
       <c r="O100" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: establish a fund (Dr 1015), request an expense (no GL), self-approve → SOD_VIOLATION, approve as a different user → Dr expense/Cr 1015 + fund down; over-balance draw → INSUFFICIENT_FLOAT; advance approve→settle clears 1180; replenish past float → OVER_FLOAT (re-performed by the harnesses).</t>
+          <t>Issue an advance (1180 up); settle 700+300 clears 1180; mismatched settle → SETTLE_MISMATCH (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P100" s="12" t="inlineStr">
         <is>
-          <t>Fund register + disbursement approval log + SoD test</t>
+          <t>Advance register; outstanding float</t>
         </is>
       </c>
       <c r="Q100" s="18" t="inlineStr">
@@ -9583,12 +9583,12 @@
     <row r="101">
       <c r="A101" s="15" t="inlineStr">
         <is>
-          <t>FA-07</t>
+          <t>EXP-08</t>
         </is>
       </c>
       <c r="B101" s="16" t="inlineStr">
         <is>
-          <t>Fixed Assets</t>
+          <t>Expenditure</t>
         </is>
       </c>
       <c r="C101" s="17" t="inlineStr">
@@ -9598,27 +9598,27 @@
       </c>
       <c r="D101" s="16" t="inlineStr">
         <is>
-          <t>Property, Plant &amp; Equipment; Equity</t>
+          <t>Cash; Operating expense</t>
         </is>
       </c>
       <c r="E101" s="16" t="inlineStr">
         <is>
-          <t>Carrying amount not adjusted for revaluation/impairment — asset over/understated.</t>
+          <t>Petty-cash disbursed beyond authority / without independent review, or drawn past the fund's limit — cash leakage, unauthorised or unrecorded expense, over-extended float.</t>
         </is>
       </c>
       <c r="F101" s="16" t="inlineStr">
         <is>
-          <t>Valuation</t>
+          <t>Authorization; Completeness</t>
         </is>
       </c>
       <c r="G101" s="16" t="inlineStr">
         <is>
-          <t>Asset revaluation / impairment: an upward revaluation credits the revaluation surplus in equity (Dr 1500 / Cr 3200); a downward revaluation (impairment) debits impairment loss (Dr 5820 / Cr 1500). The gross 1500 moves by the delta so the register stays tied to the GL; a no-op revaluation is rejected (NO_CHANGE). Every event is logged for the audit trail.</t>
+          <t>Petty-cash imprest float + maker-checker on disbursement (SoD): a fund holds cash capped at a credit limit/วงเงิน (1015 Petty Cash, a cash account); each direct EXPENSE or ADVANCE is a REQUEST that posts NOTHING and a DIFFERENT user must approve before the GL posts (expense Dr &lt;expense&gt; / Cr 1015; advance Dr 1180 / Cr 1015) and the fund balance is decremented. Self-approval → SOD_VIOLATION (binds even Admin). A draw beyond the fund balance → INSUFFICIENT_FLOAT; establishing/replenishing above the float limit → OVER_FLOAT. Advances settle (Dr expense + Dr 1015 returned / Cr 1180), returning unused cash to the fund. Every request carries a document reference + receipt key + a status trail (StatusLog) and surfaces in the GOV-01 pending-approvals monitor.</t>
         </is>
       </c>
       <c r="H101" s="17" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I101" s="17" t="inlineStr">
@@ -9628,12 +9628,12 @@
       </c>
       <c r="J101" s="17" t="inlineStr">
         <is>
-          <t>Per event</t>
+          <t>Per disbursement</t>
         </is>
       </c>
       <c r="K101" s="16" t="inlineStr">
         <is>
-          <t>FaAccountant / Controller</t>
+          <t>AP / Controller</t>
         </is>
       </c>
       <c r="L101" s="17" t="inlineStr">
@@ -9643,22 +9643,22 @@
       </c>
       <c r="M101" s="16" t="inlineStr">
         <is>
-          <t>assets.service.ts (revalue up→3200 / down→5820, listRevaluations; dispose recycles surplus 3200→3100); assets.controller.ts (exec/creditors); schema/assets.ts (asset_revaluations) + migration 0120; cutover/basics.ts (ToE)</t>
+          <t>petty-cash.service.ts (establishFund/replenishFund float guards, createRequest INSUFFICIENT_FLOAT, approveRequest SoD+GL, rejectRequest, settleRequest); petty-cash.controller.ts (creditors/exec); schema/petty-cash.ts (petty_cash_funds, expense_requests) + migration 0139; finance.service.ts pendingApprovals (GOV-01 source 7); cutover/basics.ts + compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N101" s="16" t="inlineStr">
         <is>
-          <t>Inspect revaluation/impairment routing + audit log + disposal recycling.</t>
+          <t>Inspect the float ceiling + the request→approve flow + the approver≠requester check + that the request posts nothing until approval.</t>
         </is>
       </c>
       <c r="O101" s="16" t="inlineStr">
         <is>
-          <t>Upward revaluation credits 3200; impairment debits 5820; no-change → NO_CHANGE; both events logged; on disposal the revaluation surplus is recycled to retained earnings (Dr 3200 / Cr 3100), not through P&amp;L (re-performed by the harness).</t>
+          <t>Re-perform: establish a fund (Dr 1015), request an expense (no GL), self-approve → SOD_VIOLATION, approve as a different user → Dr expense/Cr 1015 + fund down; over-balance draw → INSUFFICIENT_FLOAT; advance approve→settle clears 1180; replenish past float → OVER_FLOAT (re-performed by the harnesses).</t>
         </is>
       </c>
       <c r="P101" s="16" t="inlineStr">
         <is>
-          <t>Revaluation log; disposal recycling JE</t>
+          <t>Fund register + disbursement approval log + SoD test</t>
         </is>
       </c>
       <c r="Q101" s="18" t="inlineStr">
@@ -9670,7 +9670,7 @@
     <row r="102">
       <c r="A102" s="11" t="inlineStr">
         <is>
-          <t>FA-08</t>
+          <t>FA-07</t>
         </is>
       </c>
       <c r="B102" s="12" t="inlineStr">
@@ -9690,22 +9690,22 @@
       </c>
       <c r="E102" s="12" t="inlineStr">
         <is>
-          <t>Carrying amount changed by fair-value revaluation/impairment without independent review — the preparer revalues the asset and posts to equity/P&amp;L on their own (earnings/equity management).</t>
+          <t>Carrying amount not adjusted for revaluation/impairment — asset over/understated.</t>
         </is>
       </c>
       <c r="F102" s="12" t="inlineStr">
         <is>
-          <t>Authorization</t>
+          <t>Valuation</t>
         </is>
       </c>
       <c r="G102" s="12" t="inlineStr">
         <is>
-          <t>Asset-revaluation maker-checker (SoD): a revalue/impairment request posts its GL entry as a DRAFT (excluded from balances) and records status 'PendingApproval' WITHOUT moving the carrying value; a DIFFERENT user must approve before the JE is effective and the register is re-valued (approver ≠ preparer enforced regardless of permissions, reusing the GL-05 ledger approval). Reject voids the draft; only one revaluation may be pending per asset; the disposal surplus recycle counts only approved revaluations.</t>
+          <t>Asset revaluation / impairment: an upward revaluation credits the revaluation surplus in equity (Dr 1500 / Cr 3200); a downward revaluation (impairment) debits impairment loss (Dr 5820 / Cr 1500). The gross 1500 moves by the delta so the register stays tied to the GL; a no-op revaluation is rejected (NO_CHANGE). Every event is logged for the audit trail.</t>
         </is>
       </c>
       <c r="H102" s="13" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I102" s="13" t="inlineStr">
@@ -9730,22 +9730,22 @@
       </c>
       <c r="M102" s="12" t="inlineStr">
         <is>
-          <t>assets.service.ts revalue(pendingApproval Draft)/approveRevaluation/rejectRevaluation; assets.controller.ts (:assetNo/revalue/approve|reject); schema/assets.ts asset_revaluations.status + migration 0134; cutover/basics.ts + compliance.ts (ToE)</t>
+          <t>assets.service.ts (revalue up→3200 / down→5820, listRevaluations; dispose recycles surplus 3200→3100); assets.controller.ts (exec/creditors); schema/assets.ts (asset_revaluations) + migration 0120; cutover/basics.ts (ToE)</t>
         </is>
       </c>
       <c r="N102" s="12" t="inlineStr">
         <is>
-          <t>Inspect Draft→approve flow + the approver≠preparer check + deferred carrying-value update.</t>
+          <t>Inspect revaluation/impairment routing + audit log + disposal recycling.</t>
         </is>
       </c>
       <c r="O102" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: request a revaluation (Draft JE excluded from 3200), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm the surplus/impairment + carrying value move only after approval (re-performed by the harnesses).</t>
+          <t>Upward revaluation credits 3200; impairment debits 5820; no-change → NO_CHANGE; both events logged; on disposal the revaluation surplus is recycled to retained earnings (Dr 3200 / Cr 3100), not through P&amp;L (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P102" s="12" t="inlineStr">
         <is>
-          <t>Revaluation approval log + SoD test</t>
+          <t>Revaluation log; disposal recycling JE</t>
         </is>
       </c>
       <c r="Q102" s="18" t="inlineStr">
@@ -9757,12 +9757,12 @@
     <row r="103">
       <c r="A103" s="15" t="inlineStr">
         <is>
-          <t>LSE-01</t>
+          <t>FA-08</t>
         </is>
       </c>
       <c r="B103" s="16" t="inlineStr">
         <is>
-          <t>Leases</t>
+          <t>Fixed Assets</t>
         </is>
       </c>
       <c r="C103" s="17" t="inlineStr">
@@ -9772,27 +9772,27 @@
       </c>
       <c r="D103" s="16" t="inlineStr">
         <is>
-          <t>Right-of-use assets; Lease liabilities</t>
+          <t>Property, Plant &amp; Equipment; Equity</t>
         </is>
       </c>
       <c r="E103" s="16" t="inlineStr">
         <is>
-          <t>Lease not capitalised (IFRS 16 / TFRS 16) — ROU asset + lease liability omitted; interest/depreciation mis-stated.</t>
+          <t>Carrying amount changed by fair-value revaluation/impairment without independent review — the preparer revalues the asset and posts to equity/P&amp;L on their own (earnings/equity management).</t>
         </is>
       </c>
       <c r="F103" s="16" t="inlineStr">
         <is>
-          <t>Completeness/Accuracy/Valuation</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="G103" s="16" t="inlineStr">
         <is>
-          <t>Lease accounting: at commencement a right-of-use asset and lease liability are recognised at the present value of the lease payments (Dr 1600 / Cr 2600). The scheduled job lease_periodic_run posts each period — interest unwinding on the liability (Dr 5900), the cash payment reducing the liability (Dr 2600 / Cr 1000), and straight-line ROU depreciation (Dr 5210 / Cr 1690) — the last period clearing the liability + ROU exactly. Idempotent per (lease, period).</t>
+          <t>Asset-revaluation maker-checker (SoD): a revalue/impairment request posts its GL entry as a DRAFT (excluded from balances) and records status 'PendingApproval' WITHOUT moving the carrying value; a DIFFERENT user must approve before the JE is effective and the register is re-valued (approver ≠ preparer enforced regardless of permissions, reusing the GL-05 ledger approval). Reject voids the draft; only one revaluation may be pending per asset; the disposal surplus recycle counts only approved revaluations.</t>
         </is>
       </c>
       <c r="H103" s="17" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I103" s="17" t="inlineStr">
@@ -9802,12 +9802,12 @@
       </c>
       <c r="J103" s="17" t="inlineStr">
         <is>
-          <t>Per period / per lease</t>
+          <t>Per event</t>
         </is>
       </c>
       <c r="K103" s="16" t="inlineStr">
         <is>
-          <t>Controller</t>
+          <t>FaAccountant / Controller</t>
         </is>
       </c>
       <c r="L103" s="17" t="inlineStr">
@@ -9817,22 +9817,22 @@
       </c>
       <c r="M103" s="16" t="inlineStr">
         <is>
-          <t>leases.service.ts (createLease PV recognition, runDueLeases interest+payment+depreciation, modifyLease remeasurement); leases.controller.ts (gl_post); bi.service.ts (lease_periodic_run); schema/leases.ts (leases, rou_nbv) + migration 0120/0121; cutover/basics.ts (ToE)</t>
+          <t>assets.service.ts revalue(pendingApproval Draft)/approveRevaluation/rejectRevaluation; assets.controller.ts (:assetNo/revalue/approve|reject); schema/assets.ts asset_revaluations.status + migration 0134; cutover/basics.ts + compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N103" s="16" t="inlineStr">
         <is>
-          <t>Inspect PV recognition + periodic interest/payment/depreciation + final-period clearing + modification remeasurement.</t>
+          <t>Inspect Draft→approve flow + the approver≠preparer check + deferred carrying-value update.</t>
         </is>
       </c>
       <c r="O103" s="16" t="inlineStr">
         <is>
-          <t>Commencement recognises ROU=liability=PV; periodic run posts interest+principal(=payment)+ROU depreciation; liability + ROU reduce; a modification remeasures the liability at the revised PV and adjusts the ROU by the same delta (Dr/Cr 1600↔2600), then depreciates over the remaining term (re-performed by the harness).</t>
+          <t>Re-perform: request a revaluation (Draft JE excluded from 3200), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm the surplus/impairment + carrying value move only after approval (re-performed by the harnesses).</t>
         </is>
       </c>
       <c r="P103" s="16" t="inlineStr">
         <is>
-          <t>Lease register; periodic run log; modification remeasurement</t>
+          <t>Revaluation approval log + SoD test</t>
         </is>
       </c>
       <c r="Q103" s="18" t="inlineStr">
@@ -9844,12 +9844,12 @@
     <row r="104">
       <c r="A104" s="11" t="inlineStr">
         <is>
-          <t>REC-01</t>
+          <t>LSE-01</t>
         </is>
       </c>
       <c r="B104" s="12" t="inlineStr">
         <is>
-          <t>Reconciliation</t>
+          <t>Leases</t>
         </is>
       </c>
       <c r="C104" s="13" t="inlineStr">
@@ -9859,22 +9859,22 @@
       </c>
       <c r="D104" s="12" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Right-of-use assets; Lease liabilities</t>
         </is>
       </c>
       <c r="E104" s="12" t="inlineStr">
         <is>
-          <t>Subledgers diverge from GL undetected.</t>
+          <t>Lease not capitalised (IFRS 16 / TFRS 16) — ROU asset + lease liability omitted; interest/depreciation mis-stated.</t>
         </is>
       </c>
       <c r="F104" s="12" t="inlineStr">
         <is>
-          <t>Completeness/Accuracy</t>
+          <t>Completeness/Accuracy/Valuation</t>
         </is>
       </c>
       <c r="G104" s="12" t="inlineStr">
         <is>
-          <t>Subledger-to-GL reconciliation per period: import GL, auto-match, certify (sign-off via 'approvals').</t>
+          <t>Lease accounting: at commencement a right-of-use asset and lease liability are recognised at the present value of the lease payments (Dr 1600 / Cr 2600). The scheduled job lease_periodic_run posts each period — interest unwinding on the liability (Dr 5900), the cash payment reducing the liability (Dr 2600 / Cr 1000), and straight-line ROU depreciation (Dr 5210 / Cr 1690) — the last period clearing the liability + ROU exactly. Idempotent per (lease, period).</t>
         </is>
       </c>
       <c r="H104" s="13" t="inlineStr">
@@ -9884,12 +9884,12 @@
       </c>
       <c r="I104" s="13" t="inlineStr">
         <is>
-          <t>Auto+Manual</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J104" s="13" t="inlineStr">
         <is>
-          <t>Monthly</t>
+          <t>Per period / per lease</t>
         </is>
       </c>
       <c r="K104" s="12" t="inlineStr">
@@ -9899,27 +9899,27 @@
       </c>
       <c r="L104" s="13" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="M104" s="12" t="inlineStr">
         <is>
-          <t>reconciliation.service.ts (importGlItems/autoMatch/certify)</t>
+          <t>leases.service.ts (createLease PV recognition, runDueLeases interest+payment+depreciation, modifyLease remeasurement); leases.controller.ts (gl_post); bi.service.ts (lease_periodic_run); schema/leases.ts (leases, rou_nbv) + migration 0120/0121; cutover/basics.ts (ToE)</t>
         </is>
       </c>
       <c r="N104" s="12" t="inlineStr">
         <is>
-          <t>Inspect recon + certify gate.</t>
+          <t>Inspect PV recognition + periodic interest/payment/depreciation + final-period clearing + modification remeasurement.</t>
         </is>
       </c>
       <c r="O104" s="12" t="inlineStr">
         <is>
-          <t>Sample periods: reconciled, unmatched cleared, certified.</t>
+          <t>Commencement recognises ROU=liability=PV; periodic run posts interest+principal(=payment)+ROU depreciation; liability + ROU reduce; a modification remeasures the liability at the revised PV and adjusts the ROU by the same delta (Dr/Cr 1600↔2600), then depreciates over the remaining term (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P104" s="12" t="inlineStr">
         <is>
-          <t>Certified recon</t>
+          <t>Lease register; periodic run log; modification remeasurement</t>
         </is>
       </c>
       <c r="Q104" s="18" t="inlineStr">
@@ -9931,7 +9931,7 @@
     <row r="105">
       <c r="A105" s="15" t="inlineStr">
         <is>
-          <t>REC-02</t>
+          <t>REC-01</t>
         </is>
       </c>
       <c r="B105" s="16" t="inlineStr">
@@ -9946,22 +9946,22 @@
       </c>
       <c r="D105" s="16" t="inlineStr">
         <is>
-          <t>Cash</t>
+          <t>All</t>
         </is>
       </c>
       <c r="E105" s="16" t="inlineStr">
         <is>
-          <t>Bank balance not reconciled to GL.</t>
+          <t>Subledgers diverge from GL undetected.</t>
         </is>
       </c>
       <c r="F105" s="16" t="inlineStr">
         <is>
-          <t>Existence/Completeness</t>
+          <t>Completeness/Accuracy</t>
         </is>
       </c>
       <c r="G105" s="16" t="inlineStr">
         <is>
-          <t>Bank reconciliation against statements.</t>
+          <t>Subledger-to-GL reconciliation per period: import GL, auto-match, certify (sign-off via 'approvals').</t>
         </is>
       </c>
       <c r="H105" s="17" t="inlineStr">
@@ -9991,22 +9991,22 @@
       </c>
       <c r="M105" s="16" t="inlineStr">
         <is>
-          <t>bank module; drizzle/0015_bank_reconciliation</t>
+          <t>reconciliation.service.ts (importGlItems/autoMatch/certify)</t>
         </is>
       </c>
       <c r="N105" s="16" t="inlineStr">
         <is>
-          <t>Inspect bank-rec process.</t>
+          <t>Inspect recon + certify gate.</t>
         </is>
       </c>
       <c r="O105" s="16" t="inlineStr">
         <is>
-          <t>Sample months reconciled &amp; reviewed.</t>
+          <t>Sample periods: reconciled, unmatched cleared, certified.</t>
         </is>
       </c>
       <c r="P105" s="16" t="inlineStr">
         <is>
-          <t>Bank rec</t>
+          <t>Certified recon</t>
         </is>
       </c>
       <c r="Q105" s="18" t="inlineStr">
@@ -10018,12 +10018,12 @@
     <row r="106">
       <c r="A106" s="11" t="inlineStr">
         <is>
-          <t>BANK-02</t>
+          <t>REC-02</t>
         </is>
       </c>
       <c r="B106" s="12" t="inlineStr">
         <is>
-          <t>Cash &amp; Treasury</t>
+          <t>Reconciliation</t>
         </is>
       </c>
       <c r="C106" s="13" t="inlineStr">
@@ -10033,37 +10033,37 @@
       </c>
       <c r="D106" s="12" t="inlineStr">
         <is>
-          <t>Cash; Operating expense; Interest income</t>
+          <t>Cash</t>
         </is>
       </c>
       <c r="E106" s="12" t="inlineStr">
         <is>
-          <t>A bank fee/interest adjustment is posted straight to the GL by one person during reconciliation — a cash outflow mis-booked as interest income, or a fictitious fee posted, with no independent review (single-person posting to the cash account).</t>
+          <t>Bank balance not reconciled to GL.</t>
         </is>
       </c>
       <c r="F106" s="12" t="inlineStr">
         <is>
-          <t>Authorization/Accuracy</t>
+          <t>Existence/Completeness</t>
         </is>
       </c>
       <c r="G106" s="12" t="inlineStr">
         <is>
-          <t>Bank adjustment maker-checker (SoD): a fee/interest adjustment on a statement line is a REQUEST that posts a DRAFT JE (no balance/GL effect; the line stays unreconciled) until a DIFFERENT user with approval authority approves (POST /api/bank/lines/:id/adjustment/approve). Self-approval → SOD_VIOLATION (binds even Admin); approval flips the line to reconciled and the JE to Posted; reject voids the Draft and frees the line. The Draft JE (source BANKADJ) is also surfaced, aged, by the pending-approvals monitor (GOV-01).</t>
+          <t>Bank reconciliation against statements.</t>
         </is>
       </c>
       <c r="H106" s="13" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I106" s="13" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="J106" s="13" t="inlineStr">
         <is>
-          <t>Per adjustment</t>
+          <t>Monthly</t>
         </is>
       </c>
       <c r="K106" s="12" t="inlineStr">
@@ -10073,27 +10073,27 @@
       </c>
       <c r="L106" s="13" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="M106" s="12" t="inlineStr">
         <is>
-          <t>bank.service.ts requestAdjustment/approveAdjustment/rejectAdjustment/listPendingAdjustments (reuses ledger.approveEntry SoD); bank.controller.ts (lines/:id/adjustment requests; adjustment/approve|reject gated approvals/gl_close); cutover/bankrec.ts (ToE)</t>
+          <t>bank module; drizzle/0015_bank_reconciliation</t>
         </is>
       </c>
       <c r="N106" s="12" t="inlineStr">
         <is>
-          <t>Inspect the request→approve flow + the approver≠requester check + that the Draft posts nothing until approval.</t>
+          <t>Inspect bank-rec process.</t>
         </is>
       </c>
       <c r="O106" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: request a fee adjustment (line unreconciled, GL difference unchanged), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm the difference closes to 0 only after approval (re-performed by the bankrec harness).</t>
+          <t>Sample months reconciled &amp; reviewed.</t>
         </is>
       </c>
       <c r="P106" s="12" t="inlineStr">
         <is>
-          <t>Bank adjustment queue + SoD test</t>
+          <t>Bank rec</t>
         </is>
       </c>
       <c r="Q106" s="18" t="inlineStr">
@@ -10105,12 +10105,12 @@
     <row r="107">
       <c r="A107" s="15" t="inlineStr">
         <is>
-          <t>REC-03</t>
+          <t>BANK-02</t>
         </is>
       </c>
       <c r="B107" s="16" t="inlineStr">
         <is>
-          <t>Reconciliation</t>
+          <t>Cash &amp; Treasury</t>
         </is>
       </c>
       <c r="C107" s="17" t="inlineStr">
@@ -10120,79 +10120,79 @@
       </c>
       <c r="D107" s="16" t="inlineStr">
         <is>
-          <t>Consolidation</t>
+          <t>Cash; Operating expense; Interest income</t>
         </is>
       </c>
       <c r="E107" s="16" t="inlineStr">
         <is>
-          <t>Intercompany balances not eliminated/agreed.</t>
+          <t>A bank fee/interest adjustment is posted straight to the GL by one person during reconciliation — a cash outflow mis-booked as interest income, or a fictitious fee posted, with no independent review (single-person posting to the cash account).</t>
         </is>
       </c>
       <c r="F107" s="16" t="inlineStr">
         <is>
-          <t>Accuracy</t>
+          <t>Authorization/Accuracy</t>
         </is>
       </c>
       <c r="G107" s="16" t="inlineStr">
         <is>
-          <t>Intercompany reconciliation &amp; elimination on consolidation.</t>
+          <t>Bank adjustment maker-checker (SoD): a fee/interest adjustment on a statement line is a REQUEST that posts a DRAFT JE (no balance/GL effect; the line stays unreconciled) until a DIFFERENT user with approval authority approves (POST /api/bank/lines/:id/adjustment/approve). Self-approval → SOD_VIOLATION (binds even Admin); approval flips the line to reconciled and the JE to Posted; reject voids the Draft and frees the line. The Draft JE (source BANKADJ) is also surfaced, aged, by the pending-approvals monitor (GOV-01).</t>
         </is>
       </c>
       <c r="H107" s="17" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I107" s="17" t="inlineStr">
         <is>
-          <t>Auto+Manual</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J107" s="17" t="inlineStr">
         <is>
-          <t>Period</t>
+          <t>Per adjustment</t>
         </is>
       </c>
       <c r="K107" s="16" t="inlineStr">
         <is>
-          <t>Group Controller</t>
+          <t>Controller</t>
         </is>
       </c>
       <c r="L107" s="17" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="M107" s="16" t="inlineStr">
         <is>
-          <t>intercompany; consolidation</t>
+          <t>bank.service.ts requestAdjustment/approveAdjustment/rejectAdjustment/listPendingAdjustments (reuses ledger.approveEntry SoD); bank.controller.ts (lines/:id/adjustment requests; adjustment/approve|reject gated approvals/gl_close); cutover/bankrec.ts (ToE)</t>
         </is>
       </c>
       <c r="N107" s="16" t="inlineStr">
         <is>
-          <t>Inspect IC matching + elimination.</t>
+          <t>Inspect the request→approve flow + the approver≠requester check + that the Draft posts nothing until approval.</t>
         </is>
       </c>
       <c r="O107" s="16" t="inlineStr">
         <is>
-          <t>Sample IC pairs agree &amp; eliminate.</t>
+          <t>Re-perform: request a fee adjustment (line unreconciled, GL difference unchanged), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm the difference closes to 0 only after approval (re-performed by the bankrec harness).</t>
         </is>
       </c>
       <c r="P107" s="16" t="inlineStr">
         <is>
-          <t>IC recon</t>
-        </is>
-      </c>
-      <c r="Q107" s="19" t="inlineStr">
-        <is>
-          <t>Partial</t>
+          <t>Bank adjustment queue + SoD test</t>
+        </is>
+      </c>
+      <c r="Q107" s="18" t="inlineStr">
+        <is>
+          <t>Implemented</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="11" t="inlineStr">
         <is>
-          <t>REC-04</t>
+          <t>REC-03</t>
         </is>
       </c>
       <c r="B108" s="12" t="inlineStr">
@@ -10207,22 +10207,22 @@
       </c>
       <c r="D108" s="12" t="inlineStr">
         <is>
-          <t>All control accounts</t>
+          <t>Consolidation</t>
         </is>
       </c>
       <c r="E108" s="12" t="inlineStr">
         <is>
-          <t>A sub-ledger silently drifts from its GL control account at period-end and no single review catches it (incomplete/inaccurate balances reach the financial statements).</t>
+          <t>Intercompany balances not eliminated/agreed.</t>
         </is>
       </c>
       <c r="F108" s="12" t="inlineStr">
         <is>
-          <t>Completeness/Accuracy</t>
+          <t>Accuracy</t>
         </is>
       </c>
       <c r="G108" s="12" t="inlineStr">
         <is>
-          <t>Period-end control-account reconciliation PACK: one read (GET /api/finance/reconciliation/controls) ties every major sub-ledger to its GL control account and FLAGS any out-of-balance — AR↔1100, AP↔2000, Inventory↔1200, Gift cards/Customer-deposits↔2200, Deferred revenue↔2400 — reporting per line {sub_ledger, gl_control, variance, reconciled} plus an overall all_reconciled flag and an exceptions count. Liability controls are sign-flipped before comparison. The controller's single 'are the books reconciled?' close view; an exception is a control finding to investigate before sign-off.</t>
+          <t>Intercompany reconciliation &amp; elimination on consolidation.</t>
         </is>
       </c>
       <c r="H108" s="13" t="inlineStr">
@@ -10232,17 +10232,17 @@
       </c>
       <c r="I108" s="13" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="J108" s="13" t="inlineStr">
         <is>
-          <t>Period / on demand</t>
+          <t>Period</t>
         </is>
       </c>
       <c r="K108" s="12" t="inlineStr">
         <is>
-          <t>Controller / CFO</t>
+          <t>Group Controller</t>
         </is>
       </c>
       <c r="L108" s="13" t="inlineStr">
@@ -10252,34 +10252,34 @@
       </c>
       <c r="M108" s="12" t="inlineStr">
         <is>
-          <t>finance.service.ts reconcileControls; finance.controller.ts GET reconciliation/controls (exec/ar/creditors); reuses ledger.trialBalance + the AR/AP/inventory/gift-card/deferred sub-ledgers; cutover/giftcards.ts + compliance.ts (ToE)</t>
+          <t>intercompany; consolidation</t>
         </is>
       </c>
       <c r="N108" s="12" t="inlineStr">
         <is>
-          <t>Inspect the pack: each control account's sub-ledger query + the GL tie + the exceptions roll-up.</t>
+          <t>Inspect IC matching + elimination.</t>
         </is>
       </c>
       <c r="O108" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: with a clean set, every line reconciled + all_reconciled=true; introduce a known sub-ledger/GL difference and confirm it surfaces as an exception (re-performed: gift-card 2200 + inventory 1200 ties asserted by the harnesses).</t>
+          <t>Sample IC pairs agree &amp; eliminate.</t>
         </is>
       </c>
       <c r="P108" s="12" t="inlineStr">
         <is>
-          <t>Reconciliation pack; exceptions list</t>
-        </is>
-      </c>
-      <c r="Q108" s="18" t="inlineStr">
-        <is>
-          <t>Implemented</t>
+          <t>IC recon</t>
+        </is>
+      </c>
+      <c r="Q108" s="19" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="15" t="inlineStr">
         <is>
-          <t>REC-05</t>
+          <t>REC-04</t>
         </is>
       </c>
       <c r="B109" s="16" t="inlineStr">
@@ -10294,42 +10294,42 @@
       </c>
       <c r="D109" s="16" t="inlineStr">
         <is>
-          <t>Cash; Bank</t>
+          <t>All control accounts</t>
         </is>
       </c>
       <c r="E109" s="16" t="inlineStr">
         <is>
-          <t>Till cash dropped to the safe never reaches the bank, or a deposit isn't matched to the statement — cash sits unbanked (theft/loss exposure) or the bank balance can't be tied to the books.</t>
+          <t>A sub-ledger silently drifts from its GL control account at period-end and no single review catches it (incomplete/inaccurate balances reach the financial statements).</t>
         </is>
       </c>
       <c r="F109" s="16" t="inlineStr">
         <is>
-          <t>Completeness/Existence/Authorization</t>
+          <t>Completeness/Accuracy</t>
         </is>
       </c>
       <c r="G109" s="16" t="inlineStr">
         <is>
-          <t>Cash banking — safe-drop → bank deposit → reconciliation: till 'drop's move cash from the drawer to the safe (drawer-only, no GL). Banking BATCHES the undeposited drops into a deposit and posts the GL (Dr &lt;bank account, e.g. 1010&gt; / Cr 1000 Cash), stamping each drop with the deposit id; the deposit is then RECONCILED to the bank statement (status Deposited→Reconciled). A detective read (GET /api/bank/deposits/undeposited-drops) surfaces the CASH STILL IN THE SAFE (drops with deposit_id NULL) — the unbanked exposure to chase. SoD: banking is a treasury duty (exec/ar) — segregated from the cashier (pos_till) who drops the cash, so the person who removes cash from the drawer is not the one who banks it.</t>
+          <t>Period-end control-account reconciliation PACK: one read (GET /api/finance/reconciliation/controls) ties every major sub-ledger to its GL control account and FLAGS any out-of-balance — AR↔1100, AP↔2000, Inventory↔1200, Gift cards/Customer-deposits↔2200, Deferred revenue↔2400 — reporting per line {sub_ledger, gl_control, variance, reconciled} plus an overall all_reconciled flag and an exceptions count. Liability controls are sign-flipped before comparison. The controller's single 'are the books reconciled?' close view; an exception is a control finding to investigate before sign-off.</t>
         </is>
       </c>
       <c r="H109" s="17" t="inlineStr">
         <is>
-          <t>Det/Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I109" s="17" t="inlineStr">
         <is>
-          <t>Auto+Manual</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J109" s="17" t="inlineStr">
         <is>
-          <t>Per banking run</t>
+          <t>Period / on demand</t>
         </is>
       </c>
       <c r="K109" s="16" t="inlineStr">
         <is>
-          <t>FinancialController / Treasury</t>
+          <t>Controller / CFO</t>
         </is>
       </c>
       <c r="L109" s="17" t="inlineStr">
@@ -10339,22 +10339,22 @@
       </c>
       <c r="M109" s="16" t="inlineStr">
         <is>
-          <t>bank.service.ts undepositedDrops/createDeposit (Dr bank/Cr 1000, stamps deposit_id)/reconcileDeposit/listDeposits; bank.controller.ts (deposits, deposits/undeposited-drops, deposits/:id/reconcile; exec/ar); schema/cash.ts bank_deposits + cash_movements.deposit_id + migration 0152; /cash-banking UI; cutover/cash-banking.ts (ToE)</t>
+          <t>finance.service.ts reconcileControls; finance.controller.ts GET reconciliation/controls (exec/ar/creditors); reuses ledger.trialBalance + the AR/AP/inventory/gift-card/deferred sub-ledgers; cutover/giftcards.ts + compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N109" s="16" t="inlineStr">
         <is>
-          <t>Inspect the undeposited-drop exposure read + the deposit GL (bank↔1000) + the reconcile step + the SoD (cashier vs treasury).</t>
+          <t>Inspect the pack: each control account's sub-ledger query + the GL tie + the exceptions roll-up.</t>
         </is>
       </c>
       <c r="O109" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: two till drops → cash-in-safe shows the total; a cashier (pos_till) cannot bank (403); treasury banks → Dr bank / Cr 1000, cash-in-safe back to 0; reconcile the deposit; trial balance balanced (re-performed by the cash-banking harness).</t>
+          <t>Re-perform: with a clean set, every line reconciled + all_reconciled=true; introduce a known sub-ledger/GL difference and confirm it surfaces as an exception (re-performed: gift-card 2200 + inventory 1200 ties asserted by the harnesses).</t>
         </is>
       </c>
       <c r="P109" s="16" t="inlineStr">
         <is>
-          <t>Bank-deposit register; undeposited-drop (cash-in-safe) exposure</t>
+          <t>Reconciliation pack; exceptions list</t>
         </is>
       </c>
       <c r="Q109" s="18" t="inlineStr">
@@ -10366,12 +10366,12 @@
     <row r="110">
       <c r="A110" s="11" t="inlineStr">
         <is>
-          <t>GOV-01</t>
+          <t>REC-05</t>
         </is>
       </c>
       <c r="B110" s="12" t="inlineStr">
         <is>
-          <t>Monitoring</t>
+          <t>Reconciliation</t>
         </is>
       </c>
       <c r="C110" s="13" t="inlineStr">
@@ -10381,42 +10381,42 @@
       </c>
       <c r="D110" s="12" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Cash; Bank</t>
         </is>
       </c>
       <c r="E110" s="12" t="inlineStr">
         <is>
-          <t>A maker-checker approval sits un-actioned and is forgotten — a transaction stalls before it is effective, or (worse) a control is quietly bypassed and no one notices an item never got its independent review.</t>
+          <t>Till cash dropped to the safe never reaches the bank, or a deposit isn't matched to the statement — cash sits unbanked (theft/loss exposure) or the bank balance can't be tied to the books.</t>
         </is>
       </c>
       <c r="F110" s="12" t="inlineStr">
         <is>
-          <t>Authorization/Completeness</t>
+          <t>Completeness/Existence/Authorization</t>
         </is>
       </c>
       <c r="G110" s="12" t="inlineStr">
         <is>
-          <t>Pending-approvals MONITOR (COSO monitoring): a single worklist of EVERY item awaiting independent approval across the system, each with its AGE in days and an overdue roll-up — spanning the manual-JE (GL-05), bank-adjustment (BANK-02), AP-disbursement (EXP-06), payroll (PAY-03), asset-revaluation (FA-08), asset-disposal (FA-09), inventory-write-off (INV-07), till-close cash over/short (REV-13), FX-rate (FX-04), budget (BUD-01) and large-refund (REV-16) maker-checkers. The controller reviews it before close; a stale item (age beyond the threshold) is a control finding to chase or escalate. The /approvals screen also lets a manager approve/reject a material till variance or a large refund inline (the pending types with no dedicated module screen). Read-only worklist; tenant-scoped via the caller's RLS.</t>
+          <t>Cash banking — safe-drop → bank deposit → reconciliation: till 'drop's move cash from the drawer to the safe (drawer-only, no GL). Banking BATCHES the undeposited drops into a deposit and posts the GL (Dr &lt;bank account, e.g. 1010&gt; / Cr 1000 Cash), stamping each drop with the deposit id; the deposit is then RECONCILED to the bank statement (status Deposited→Reconciled). A detective read (GET /api/bank/deposits/undeposited-drops) surfaces the CASH STILL IN THE SAFE (drops with deposit_id NULL) — the unbanked exposure to chase. SoD: banking is a treasury duty (exec/ar) — segregated from the cashier (pos_till) who drops the cash, so the person who removes cash from the drawer is not the one who banks it.</t>
         </is>
       </c>
       <c r="H110" s="13" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Det/Prev</t>
         </is>
       </c>
       <c r="I110" s="13" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="J110" s="13" t="inlineStr">
         <is>
-          <t>Continuous / pre-close</t>
+          <t>Per banking run</t>
         </is>
       </c>
       <c r="K110" s="12" t="inlineStr">
         <is>
-          <t>Controller / CFO</t>
+          <t>FinancialController / Treasury</t>
         </is>
       </c>
       <c r="L110" s="13" t="inlineStr">
@@ -10426,22 +10426,22 @@
       </c>
       <c r="M110" s="12" t="inlineStr">
         <is>
-          <t>finance.service.ts pendingApprovals; finance.controller.ts GET approvals/pending (exec/approvals/creditors); aggregates journalEntries(Draft incl. BANKADJ→BANK-02)/apPayments/payruns/asset_revaluations/fixed_assets(disposal_pending)/inv_writeoff_requests/till_sessions(PendingApproval)/fx_rates(PendingApproval)/budgets(PendingApproval); cutover/compliance.ts (ToE)</t>
+          <t>bank.service.ts undepositedDrops/createDeposit (Dr bank/Cr 1000, stamps deposit_id)/reconcileDeposit/listDeposits; bank.controller.ts (deposits, deposits/undeposited-drops, deposits/:id/reconcile; exec/ar); schema/cash.ts bank_deposits + cash_movements.deposit_id + migration 0152; /cash-banking UI; cutover/cash-banking.ts (ToE)</t>
         </is>
       </c>
       <c r="N110" s="12" t="inlineStr">
         <is>
-          <t>Inspect the aggregation across all pending sources + the age/overdue roll-up.</t>
+          <t>Inspect the undeposited-drop exposure read + the deposit GL (bank↔1000) + the reconcile step + the SoD (cashier vs treasury).</t>
         </is>
       </c>
       <c r="O110" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: create a pending item (e.g. a Draft JE) and confirm it appears in the worklist with its control ID, amount and age; the overdue count flags items past the threshold (re-performed by the harness).</t>
+          <t>Re-perform: two till drops → cash-in-safe shows the total; a cashier (pos_till) cannot bank (403); treasury banks → Dr bank / Cr 1000, cash-in-safe back to 0; reconcile the deposit; trial balance balanced (re-performed by the cash-banking harness).</t>
         </is>
       </c>
       <c r="P110" s="12" t="inlineStr">
         <is>
-          <t>Pending-approvals worklist</t>
+          <t>Bank-deposit register; undeposited-drop (cash-in-safe) exposure</t>
         </is>
       </c>
       <c r="Q110" s="18" t="inlineStr">
@@ -10453,12 +10453,12 @@
     <row r="111">
       <c r="A111" s="15" t="inlineStr">
         <is>
-          <t>TAX-01</t>
+          <t>GOV-01</t>
         </is>
       </c>
       <c r="B111" s="16" t="inlineStr">
         <is>
-          <t>Tax</t>
+          <t>Monitoring</t>
         </is>
       </c>
       <c r="C111" s="17" t="inlineStr">
@@ -10468,27 +10468,27 @@
       </c>
       <c r="D111" s="16" t="inlineStr">
         <is>
-          <t>Tax (VAT)</t>
+          <t>All</t>
         </is>
       </c>
       <c r="E111" s="16" t="inlineStr">
         <is>
-          <t>VAT computed incorrectly → filing/penalty risk.</t>
+          <t>A maker-checker approval sits un-actioned and is forgotten — a transaction stalls before it is effective, or (worse) a control is quietly bypassed and no one notices an item never got its independent review.</t>
         </is>
       </c>
       <c r="F111" s="16" t="inlineStr">
         <is>
-          <t>Accuracy</t>
+          <t>Authorization/Completeness</t>
         </is>
       </c>
       <c r="G111" s="16" t="inlineStr">
         <is>
-          <t>VAT via pluggable provider (TH 7%); unit-tested; no hard-coded rate.</t>
+          <t>Pending-approvals MONITOR (COSO monitoring): a single worklist of EVERY item awaiting independent approval across the system, each with its AGE in days and an overdue roll-up — spanning the manual-JE (GL-05), bank-adjustment (BANK-02), AP-disbursement (EXP-06), payroll (PAY-03), asset-revaluation (FA-08), asset-disposal (FA-09), inventory-write-off (INV-07), till-close cash over/short (REV-13), FX-rate (FX-04), budget (BUD-01) and large-refund (REV-16) maker-checkers. The controller reviews it before close; a stale item (age beyond the threshold) is a control finding to chase or escalate. The /approvals screen also lets a manager approve/reject a material till variance or a large refund inline (the pending types with no dedicated module screen). Read-only worklist; tenant-scoped via the caller's RLS.</t>
         </is>
       </c>
       <c r="H111" s="17" t="inlineStr">
         <is>
-          <t>Auto</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I111" s="17" t="inlineStr">
@@ -10498,37 +10498,37 @@
       </c>
       <c r="J111" s="17" t="inlineStr">
         <is>
-          <t>Per txn</t>
+          <t>Continuous / pre-close</t>
         </is>
       </c>
       <c r="K111" s="16" t="inlineStr">
         <is>
-          <t>Tax / Controller</t>
+          <t>Controller / CFO</t>
         </is>
       </c>
       <c r="L111" s="17" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="M111" s="16" t="inlineStr">
         <is>
-          <t>tax/tax-providers.ts; tax.service.ts; test/unit.test.ts</t>
+          <t>finance.service.ts pendingApprovals; finance.controller.ts GET approvals/pending (exec/approvals/creditors); aggregates journalEntries(Draft incl. BANKADJ→BANK-02)/apPayments/payruns/asset_revaluations/fixed_assets(disposal_pending)/inv_writeoff_requests/till_sessions(PendingApproval)/fx_rates(PendingApproval)/budgets(PendingApproval); cutover/compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N111" s="16" t="inlineStr">
         <is>
-          <t>Inspect rate provider + tests.</t>
+          <t>Inspect the aggregation across all pending sources + the age/overdue roll-up.</t>
         </is>
       </c>
       <c r="O111" s="16" t="inlineStr">
         <is>
-          <t>Re-perform VAT on sample; tie to return.</t>
+          <t>Re-perform: create a pending item (e.g. a Draft JE) and confirm it appears in the worklist with its control ID, amount and age; the overdue count flags items past the threshold (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P111" s="16" t="inlineStr">
         <is>
-          <t>VAT tests</t>
+          <t>Pending-approvals worklist</t>
         </is>
       </c>
       <c r="Q111" s="18" t="inlineStr">
@@ -10540,7 +10540,7 @@
     <row r="112">
       <c r="A112" s="11" t="inlineStr">
         <is>
-          <t>TAX-02</t>
+          <t>TAX-01</t>
         </is>
       </c>
       <c r="B112" s="12" t="inlineStr">
@@ -10555,22 +10555,22 @@
       </c>
       <c r="D112" s="12" t="inlineStr">
         <is>
-          <t>Tax; Revenue</t>
+          <t>Tax (VAT)</t>
         </is>
       </c>
       <c r="E112" s="12" t="inlineStr">
         <is>
-          <t>Non-compliant e-Tax invoice / not transmitted to ETDA.</t>
+          <t>VAT computed incorrectly → filing/penalty risk.</t>
         </is>
       </c>
       <c r="F112" s="12" t="inlineStr">
         <is>
-          <t>Accuracy/Compliance</t>
+          <t>Accuracy</t>
         </is>
       </c>
       <c r="G112" s="12" t="inlineStr">
         <is>
-          <t>e-Tax invoice (ETDA UBL 2.1 XML) generation + email with CC to ETDA timestamp mailbox.</t>
+          <t>VAT via pluggable provider (TH 7%); unit-tested; no hard-coded rate.</t>
         </is>
       </c>
       <c r="H112" s="13" t="inlineStr">
@@ -10585,37 +10585,37 @@
       </c>
       <c r="J112" s="13" t="inlineStr">
         <is>
-          <t>Per invoice</t>
+          <t>Per txn</t>
         </is>
       </c>
       <c r="K112" s="12" t="inlineStr">
         <is>
-          <t>Tax</t>
+          <t>Tax / Controller</t>
         </is>
       </c>
       <c r="L112" s="13" t="inlineStr">
         <is>
-          <t>P10/P13</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="M112" s="12" t="inlineStr">
         <is>
-          <t>tax-docs/etax-xml.ts; etax-email.service.ts (tested)</t>
+          <t>tax/tax-providers.ts; tax.service.ts; test/unit.test.ts</t>
         </is>
       </c>
       <c r="N112" s="12" t="inlineStr">
         <is>
-          <t>Inspect XML schema + email composer.</t>
+          <t>Inspect rate provider + tests.</t>
         </is>
       </c>
       <c r="O112" s="12" t="inlineStr">
         <is>
-          <t>Sample invoices: valid XML, correct CC/escaping.</t>
+          <t>Re-perform VAT on sample; tie to return.</t>
         </is>
       </c>
       <c r="P112" s="12" t="inlineStr">
         <is>
-          <t>e-Tax samples</t>
+          <t>VAT tests</t>
         </is>
       </c>
       <c r="Q112" s="18" t="inlineStr">
@@ -10627,7 +10627,7 @@
     <row r="113">
       <c r="A113" s="15" t="inlineStr">
         <is>
-          <t>TAX-03</t>
+          <t>TAX-02</t>
         </is>
       </c>
       <c r="B113" s="16" t="inlineStr">
@@ -10642,22 +10642,22 @@
       </c>
       <c r="D113" s="16" t="inlineStr">
         <is>
-          <t>Tax (WHT)</t>
+          <t>Tax; Revenue</t>
         </is>
       </c>
       <c r="E113" s="16" t="inlineStr">
         <is>
-          <t>Withholding tax mis-computed / not reported.</t>
+          <t>Non-compliant e-Tax invoice / not transmitted to ETDA.</t>
         </is>
       </c>
       <c r="F113" s="16" t="inlineStr">
         <is>
-          <t>Accuracy</t>
+          <t>Accuracy/Compliance</t>
         </is>
       </c>
       <c r="G113" s="16" t="inlineStr">
         <is>
-          <t>WHT computation and ภ.ง.ด. reporting.</t>
+          <t>e-Tax invoice (ETDA UBL 2.1 XML) generation + email with CC to ETDA timestamp mailbox.</t>
         </is>
       </c>
       <c r="H113" s="17" t="inlineStr">
@@ -10672,7 +10672,7 @@
       </c>
       <c r="J113" s="17" t="inlineStr">
         <is>
-          <t>Per txn / monthly</t>
+          <t>Per invoice</t>
         </is>
       </c>
       <c r="K113" s="16" t="inlineStr">
@@ -10682,39 +10682,39 @@
       </c>
       <c r="L113" s="17" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P10/P13</t>
         </is>
       </c>
       <c r="M113" s="16" t="inlineStr">
         <is>
-          <t>tax-reports; payroll</t>
+          <t>tax-docs/etax-xml.ts; etax-email.service.ts (tested)</t>
         </is>
       </c>
       <c r="N113" s="16" t="inlineStr">
         <is>
-          <t>Inspect WHT logic + report.</t>
+          <t>Inspect XML schema + email composer.</t>
         </is>
       </c>
       <c r="O113" s="16" t="inlineStr">
         <is>
-          <t>Re-perform WHT on sample; tie to filing.</t>
+          <t>Sample invoices: valid XML, correct CC/escaping.</t>
         </is>
       </c>
       <c r="P113" s="16" t="inlineStr">
         <is>
-          <t>WHT report</t>
-        </is>
-      </c>
-      <c r="Q113" s="19" t="inlineStr">
-        <is>
-          <t>Partial</t>
+          <t>e-Tax samples</t>
+        </is>
+      </c>
+      <c r="Q113" s="18" t="inlineStr">
+        <is>
+          <t>Implemented</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="11" t="inlineStr">
         <is>
-          <t>TAX-04</t>
+          <t>TAX-03</t>
         </is>
       </c>
       <c r="B114" s="12" t="inlineStr">
@@ -10729,27 +10729,27 @@
       </c>
       <c r="D114" s="12" t="inlineStr">
         <is>
-          <t>Tax (VAT); Tax Payable (2100)</t>
+          <t>Tax (WHT)</t>
         </is>
       </c>
       <c r="E114" s="12" t="inlineStr">
         <is>
-          <t>Output/input VAT on the filed ภ.พ.30 return does not agree to the GL — VAT liability mis-stated, a filing/penalty exposure, or a posting omission goes undetected before submission.</t>
+          <t>Withholding tax mis-computed / not reported.</t>
         </is>
       </c>
       <c r="F114" s="12" t="inlineStr">
         <is>
-          <t>Completeness/Accuracy</t>
+          <t>Accuracy</t>
         </is>
       </c>
       <c r="G114" s="12" t="inlineStr">
         <is>
-          <t>Periodic VAT-return ↔ GL reconciliation (ภ.พ.30): the monthly return (GET /api/tax-reports/pp30) is built from the sales/output-VAT and purchase/input-VAT sub-reports, computes net VAT = output − input, and RECONCILES it to the **GL account 2100 (Tax Payable) net movement** for the same period (Σ credit − Σ debit over Posted entries) — returning `reconciliation.tied` = true only when the two agree within rounding. A non-tie is a detective finding to investigate and clear BEFORE filing (the form also carries the ม.157 deadline = the 15th of the next month). Output VAT is posted to 2100 on every sale (Cr) and reversed on returns (Dr); input VAT is posted on AP bills (Dr) — so 2100's net is the period's VAT payable. Read-only report; exportable to a ภ.พ.30 PDF/HTML.</t>
+          <t>WHT computation and ภ.ง.ด. reporting.</t>
         </is>
       </c>
       <c r="H114" s="13" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Auto</t>
         </is>
       </c>
       <c r="I114" s="13" t="inlineStr">
@@ -10759,54 +10759,54 @@
       </c>
       <c r="J114" s="13" t="inlineStr">
         <is>
-          <t>Monthly / pre-filing</t>
+          <t>Per txn / monthly</t>
         </is>
       </c>
       <c r="K114" s="12" t="inlineStr">
         <is>
-          <t>Tax / FinancialController</t>
+          <t>Tax</t>
         </is>
       </c>
       <c r="L114" s="13" t="inlineStr">
         <is>
-          <t>P10/P16</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="M114" s="12" t="inlineStr">
         <is>
-          <t>tax-reports.service.ts pp30 (outputVat/inputVat + 2100 net-movement tie); tax-reports.controller.ts (GET pp30, pp30/export, exec); tax-reports-pdf.ts; dine-in.service.ts/returns.service.ts/finance.service.ts post 2100 on sale/return/AP; /tax/reports UI; cutover/taxdocs.ts (ToE)</t>
+          <t>tax-reports; payroll</t>
         </is>
       </c>
       <c r="N114" s="12" t="inlineStr">
         <is>
-          <t>Inspect the pp30 build + the 2100 net-movement query + the tie flag + the filing deadline.</t>
+          <t>Inspect WHT logic + report.</t>
         </is>
       </c>
       <c r="O114" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: the pp30 return computes net VAT (output − input), the GL 2100 net movement reflects the posted input VAT, and the reconciliation block exposes the gl_account (2100), the report net VAT and a boolean tie verdict (tied iff the two agree within rounding); the ภ.พ.30 export renders (re-performed by the taxdocs harness).</t>
+          <t>Re-perform WHT on sample; tie to filing.</t>
         </is>
       </c>
       <c r="P114" s="12" t="inlineStr">
         <is>
-          <t>ภ.พ.30 return + GL-2100 reconciliation tie</t>
-        </is>
-      </c>
-      <c r="Q114" s="18" t="inlineStr">
-        <is>
-          <t>Implemented</t>
+          <t>WHT report</t>
+        </is>
+      </c>
+      <c r="Q114" s="19" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="15" t="inlineStr">
         <is>
-          <t>PAY-01</t>
+          <t>TAX-04</t>
         </is>
       </c>
       <c r="B115" s="16" t="inlineStr">
         <is>
-          <t>Payroll</t>
+          <t>Tax</t>
         </is>
       </c>
       <c r="C115" s="17" t="inlineStr">
@@ -10816,27 +10816,27 @@
       </c>
       <c r="D115" s="16" t="inlineStr">
         <is>
-          <t>Payroll expense/liability</t>
+          <t>Tax (VAT); Tax Payable (2100)</t>
         </is>
       </c>
       <c r="E115" s="16" t="inlineStr">
         <is>
-          <t>Payroll, SSO and PIT mis-computed.</t>
+          <t>Output/input VAT on the filed ภ.พ.30 return does not agree to the GL — VAT liability mis-stated, a filing/penalty exposure, or a posting omission goes undetected before submission.</t>
         </is>
       </c>
       <c r="F115" s="16" t="inlineStr">
         <is>
-          <t>Accuracy</t>
+          <t>Completeness/Accuracy</t>
         </is>
       </c>
       <c r="G115" s="16" t="inlineStr">
         <is>
-          <t>Payroll engine — SSO 5% (cap 750), progressive PIT, payslip net; unit-tested.</t>
+          <t>Periodic VAT-return ↔ GL reconciliation (ภ.พ.30): the monthly return (GET /api/tax-reports/pp30) is built from the sales/output-VAT and purchase/input-VAT sub-reports, computes net VAT = output − input, and RECONCILES it to the **GL account 2100 (Tax Payable) net movement** for the same period (Σ credit − Σ debit over Posted entries) — returning `reconciliation.tied` = true only when the two agree within rounding. A non-tie is a detective finding to investigate and clear BEFORE filing (the form also carries the ม.157 deadline = the 15th of the next month). Output VAT is posted to 2100 on every sale (Cr) and reversed on returns (Dr); input VAT is posted on AP bills (Dr) — so 2100's net is the period's VAT payable. Read-only report; exportable to a ภ.พ.30 PDF/HTML.</t>
         </is>
       </c>
       <c r="H115" s="17" t="inlineStr">
         <is>
-          <t>Auto</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I115" s="17" t="inlineStr">
@@ -10846,37 +10846,37 @@
       </c>
       <c r="J115" s="17" t="inlineStr">
         <is>
-          <t>Per run</t>
+          <t>Monthly / pre-filing</t>
         </is>
       </c>
       <c r="K115" s="16" t="inlineStr">
         <is>
-          <t>HR / Payroll</t>
+          <t>Tax / FinancialController</t>
         </is>
       </c>
       <c r="L115" s="17" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P10/P16</t>
         </is>
       </c>
       <c r="M115" s="16" t="inlineStr">
         <is>
-          <t>payroll/payroll-calc.ts; test/unit.test.ts</t>
+          <t>tax-reports.service.ts pp30 (outputVat/inputVat + 2100 net-movement tie); tax-reports.controller.ts (GET pp30, pp30/export, exec); tax-reports-pdf.ts; dine-in.service.ts/returns.service.ts/finance.service.ts post 2100 on sale/return/AP; /tax/reports UI; cutover/taxdocs.ts (ToE)</t>
         </is>
       </c>
       <c r="N115" s="16" t="inlineStr">
         <is>
-          <t>Inspect calc + tests.</t>
+          <t>Inspect the pp30 build + the 2100 net-movement query + the tie flag + the filing deadline.</t>
         </is>
       </c>
       <c r="O115" s="16" t="inlineStr">
         <is>
-          <t>Re-perform sample payslips.</t>
+          <t>Re-perform: the pp30 return computes net VAT (output − input), the GL 2100 net movement reflects the posted input VAT, and the reconciliation block exposes the gl_account (2100), the report net VAT and a boolean tie verdict (tied iff the two agree within rounding); the ภ.พ.30 export renders (re-performed by the taxdocs harness).</t>
         </is>
       </c>
       <c r="P115" s="16" t="inlineStr">
         <is>
-          <t>Payslip tests</t>
+          <t>ภ.พ.30 return + GL-2100 reconciliation tie</t>
         </is>
       </c>
       <c r="Q115" s="18" t="inlineStr">
@@ -10888,7 +10888,7 @@
     <row r="116">
       <c r="A116" s="11" t="inlineStr">
         <is>
-          <t>PAY-02</t>
+          <t>PAY-01</t>
         </is>
       </c>
       <c r="B116" s="12" t="inlineStr">
@@ -10903,27 +10903,27 @@
       </c>
       <c r="D116" s="12" t="inlineStr">
         <is>
-          <t>Payroll liability</t>
+          <t>Payroll expense/liability</t>
         </is>
       </c>
       <c r="E116" s="12" t="inlineStr">
         <is>
-          <t>Statutory withholdings (SSO/WHT/PF) mis-stated or not remitted, so the liability owed to the authorities diverges from the books.</t>
+          <t>Payroll, SSO and PIT mis-computed.</t>
         </is>
       </c>
       <c r="F116" s="12" t="inlineStr">
         <is>
-          <t>Accuracy/Compliance</t>
+          <t>Accuracy</t>
         </is>
       </c>
       <c r="G116" s="12" t="inlineStr">
         <is>
-          <t>Payroll-liability schedule (GET /api/payroll/liabilities): each statutory account — SSO 2350, WHT/PND1 2360, PF 2370 — shows accrued (GL credits) − remitted (GL debits) = outstanding, tied back to the INDEPENDENT payrun accrual with a `reconciled` flag (a divergence flags a manual JE that touched a payroll-liability account outside the payroll process). Treasury remits the cash (POST .../remit → Dr liability / Cr 1000) which clears the outstanding and keeps the books reconciled to the statutory filings; a remittance beyond the outstanding is blocked (REMIT_EXCEEDS_OUTSTANDING).</t>
+          <t>Payroll engine — SSO 5% (cap 750), progressive PIT, payslip net; unit-tested.</t>
         </is>
       </c>
       <c r="H116" s="13" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Auto</t>
         </is>
       </c>
       <c r="I116" s="13" t="inlineStr">
@@ -10933,12 +10933,12 @@
       </c>
       <c r="J116" s="13" t="inlineStr">
         <is>
-          <t>Per run / monthly</t>
+          <t>Per run</t>
         </is>
       </c>
       <c r="K116" s="12" t="inlineStr">
         <is>
-          <t>HR / Payroll / Treasury</t>
+          <t>HR / Payroll</t>
         </is>
       </c>
       <c r="L116" s="13" t="inlineStr">
@@ -10948,22 +10948,22 @@
       </c>
       <c r="M116" s="12" t="inlineStr">
         <is>
-          <t>payroll/payroll.service.ts liabilities/remitLiability</t>
+          <t>payroll/payroll-calc.ts; test/unit.test.ts</t>
         </is>
       </c>
       <c r="N116" s="12" t="inlineStr">
         <is>
-          <t>Inspect the schedule + the accrued/remitted/outstanding tie-out and the reconciled flag.</t>
+          <t>Inspect calc + tests.</t>
         </is>
       </c>
       <c r="O116" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: run a payroll, confirm the SSO/WHT outstanding equals the payrun accrual; remit part and confirm the outstanding falls and the TB stays balanced; attempt an over-remit (REMIT_EXCEEDS_OUTSTANDING).</t>
+          <t>Re-perform sample payslips.</t>
         </is>
       </c>
       <c r="P116" s="12" t="inlineStr">
         <is>
-          <t>Liability schedule + remittance JEs tied to filings</t>
+          <t>Payslip tests</t>
         </is>
       </c>
       <c r="Q116" s="18" t="inlineStr">
@@ -10975,7 +10975,7 @@
     <row r="117">
       <c r="A117" s="15" t="inlineStr">
         <is>
-          <t>PAY-03</t>
+          <t>PAY-02</t>
         </is>
       </c>
       <c r="B117" s="16" t="inlineStr">
@@ -10990,27 +10990,27 @@
       </c>
       <c r="D117" s="16" t="inlineStr">
         <is>
-          <t>Payroll expense/liability; Cash</t>
+          <t>Payroll liability</t>
         </is>
       </c>
       <c r="E117" s="16" t="inlineStr">
         <is>
-          <t>Payroll run posted to the GL without independent review — the preparer both computes and posts their own payroll (ghost employees, inflated rate/hours).</t>
+          <t>Statutory withholdings (SSO/WHT/PF) mis-stated or not remitted, so the liability owed to the authorities diverges from the books.</t>
         </is>
       </c>
       <c r="F117" s="16" t="inlineStr">
         <is>
-          <t>Authorization</t>
+          <t>Accuracy/Compliance</t>
         </is>
       </c>
       <c r="G117" s="16" t="inlineStr">
         <is>
-          <t>Payroll maker-checker (SoD): a run posts its GL entry as a DRAFT (excluded from balances) with the run record 'PendingApproval'; a DIFFERENT user must approve before it becomes effective (approver ≠ preparer enforced regardless of permissions, reusing the GL-05 ledger approval). Reject voids the draft; idempotent per (tenant, period).</t>
+          <t>Payroll-liability schedule (GET /api/payroll/liabilities): each statutory account — SSO 2350, WHT/PND1 2360, PF 2370 — shows accrued (GL credits) − remitted (GL debits) = outstanding, tied back to the INDEPENDENT payrun accrual with a `reconciled` flag (a divergence flags a manual JE that touched a payroll-liability account outside the payroll process). Treasury remits the cash (POST .../remit → Dr liability / Cr 1000) which clears the outstanding and keeps the books reconciled to the statutory filings; a remittance beyond the outstanding is blocked (REMIT_EXCEEDS_OUTSTANDING).</t>
         </is>
       </c>
       <c r="H117" s="17" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I117" s="17" t="inlineStr">
@@ -11020,12 +11020,12 @@
       </c>
       <c r="J117" s="17" t="inlineStr">
         <is>
-          <t>Per run</t>
+          <t>Per run / monthly</t>
         </is>
       </c>
       <c r="K117" s="16" t="inlineStr">
         <is>
-          <t>HR / Payroll; Controller</t>
+          <t>HR / Payroll / Treasury</t>
         </is>
       </c>
       <c r="L117" s="17" t="inlineStr">
@@ -11035,22 +11035,22 @@
       </c>
       <c r="M117" s="16" t="inlineStr">
         <is>
-          <t>payroll/payroll.service.ts approvePayroll/rejectPayroll; migration 0133</t>
+          <t>payroll/payroll.service.ts liabilities/remitLiability</t>
         </is>
       </c>
       <c r="N117" s="16" t="inlineStr">
         <is>
-          <t>Inspect Draft→approve flow + the approver≠preparer check.</t>
+          <t>Inspect the schedule + the accrued/remitted/outstanding tie-out and the reconciled flag.</t>
         </is>
       </c>
       <c r="O117" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: run as A, attempt self-approve (SOD_VIOLATION), approve as B; confirm the JE hits balances only after approval.</t>
+          <t>Re-perform: run a payroll, confirm the SSO/WHT outstanding equals the payrun accrual; remit part and confirm the outstanding falls and the TB stays balanced; attempt an over-remit (REMIT_EXCEEDS_OUTSTANDING).</t>
         </is>
       </c>
       <c r="P117" s="16" t="inlineStr">
         <is>
-          <t>Approval log + SoD test</t>
+          <t>Liability schedule + remittance JEs tied to filings</t>
         </is>
       </c>
       <c r="Q117" s="18" t="inlineStr">
@@ -11062,12 +11062,12 @@
     <row r="118">
       <c r="A118" s="11" t="inlineStr">
         <is>
-          <t>FA-09</t>
+          <t>PAY-03</t>
         </is>
       </c>
       <c r="B118" s="12" t="inlineStr">
         <is>
-          <t>Fixed Assets</t>
+          <t>Payroll</t>
         </is>
       </c>
       <c r="C118" s="13" t="inlineStr">
@@ -11077,12 +11077,12 @@
       </c>
       <c r="D118" s="12" t="inlineStr">
         <is>
-          <t>Property, Plant &amp; Equipment; Cash</t>
+          <t>Payroll expense/liability; Cash</t>
         </is>
       </c>
       <c r="E118" s="12" t="inlineStr">
         <is>
-          <t>Asset disposed without independent review — one person writes an asset off the books and records the proceeds (asset-stripping / theft: dispose a still-held asset, or to a related party below value).</t>
+          <t>Payroll run posted to the GL without independent review — the preparer both computes and posts their own payroll (ghost employees, inflated rate/hours).</t>
         </is>
       </c>
       <c r="F118" s="12" t="inlineStr">
@@ -11092,7 +11092,7 @@
       </c>
       <c r="G118" s="12" t="inlineStr">
         <is>
-          <t>Asset-disposal maker-checker (SoD): a disposal REQUEST posts its GL entry as a DRAFT (excluded from balances) and flags the asset disposal_pending WITHOUT marking it disposed or moving the register; a DIFFERENT user must approve before it is effective (status→disposed, revaluation surplus recycled 3200→3100) (approver ≠ requester enforced regardless of permissions, reusing the GL-05 ledger approval). Reject voids the draft and the asset stays in service; only one disposal may be pending per asset; a disposal-pending asset is frozen from depreciation.</t>
+          <t>Payroll maker-checker (SoD): a run posts its GL entry as a DRAFT (excluded from balances) with the run record 'PendingApproval'; a DIFFERENT user must approve before it becomes effective (approver ≠ preparer enforced regardless of permissions, reusing the GL-05 ledger approval). Reject voids the draft; idempotent per (tenant, period).</t>
         </is>
       </c>
       <c r="H118" s="13" t="inlineStr">
@@ -11107,12 +11107,12 @@
       </c>
       <c r="J118" s="13" t="inlineStr">
         <is>
-          <t>Per disposal</t>
+          <t>Per run</t>
         </is>
       </c>
       <c r="K118" s="12" t="inlineStr">
         <is>
-          <t>FaAccountant / Controller</t>
+          <t>HR / Payroll; Controller</t>
         </is>
       </c>
       <c r="L118" s="13" t="inlineStr">
@@ -11122,22 +11122,22 @@
       </c>
       <c r="M118" s="12" t="inlineStr">
         <is>
-          <t>assets.service.ts dispose(pendingApproval Draft)/approveDisposal/rejectDisposal; assets.controller.ts (:assetNo/dispose/approve|reject); schema/assets.ts fixed_assets.disposal_pending + migration 0135; cutover/basics.ts + worldclass.ts + compliance.ts (ToE)</t>
+          <t>payroll/payroll.service.ts approvePayroll/rejectPayroll; migration 0133</t>
         </is>
       </c>
       <c r="N118" s="12" t="inlineStr">
         <is>
-          <t>Inspect Draft→approve flow + the approver≠requester check + deferred status/recycle.</t>
+          <t>Inspect Draft→approve flow + the approver≠preparer check.</t>
         </is>
       </c>
       <c r="O118" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: request a disposal (Draft JE excluded), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm status→disposed + surplus recycled only after approval (re-performed by the harnesses).</t>
+          <t>Re-perform: run as A, attempt self-approve (SOD_VIOLATION), approve as B; confirm the JE hits balances only after approval.</t>
         </is>
       </c>
       <c r="P118" s="12" t="inlineStr">
         <is>
-          <t>Disposal approval log + SoD test</t>
+          <t>Approval log + SoD test</t>
         </is>
       </c>
       <c r="Q118" s="18" t="inlineStr">
@@ -11149,7 +11149,7 @@
     <row r="119">
       <c r="A119" s="15" t="inlineStr">
         <is>
-          <t>FA-10</t>
+          <t>FA-09</t>
         </is>
       </c>
       <c r="B119" s="16" t="inlineStr">
@@ -11164,22 +11164,22 @@
       </c>
       <c r="D119" s="16" t="inlineStr">
         <is>
-          <t>Property, Plant &amp; Equipment; Accounts Payable</t>
+          <t>Property, Plant &amp; Equipment; Cash</t>
         </is>
       </c>
       <c r="E119" s="16" t="inlineStr">
         <is>
-          <t>Capital purchases mis-capitalised or capitalised without independent review — the person who receives the goods also decides what enters the asset register and at what cost/useful life (fictitious or over-valued assets; capex/opex mis-classification).</t>
+          <t>Asset disposed without independent review — one person writes an asset off the books and records the proceeds (asset-stripping / theft: dispose a still-held asset, or to a related party below value).</t>
         </is>
       </c>
       <c r="F119" s="16" t="inlineStr">
         <is>
-          <t>Authorization; Accuracy</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="G119" s="16" t="inlineStr">
         <is>
-          <t>Procure-to-Capitalize maker-checker (SoD): a goods-receipt line flagged capital (item-master is_fixed_asset or per-PO-line override) is excluded from inventory capitalisation (1200) at receipt and instead becomes ELIGIBLE for the asset register. Capitalisation is a REQUEST that posts NOTHING to the GL; a DIFFERENT user must approve before the fixed_assets row + acquisition JE (Dr 1500 / Cr 2000) are created (approver ≠ requester enforced regardless of permissions). The created asset carries its source GR/PO for end-to-end PR→PO→GR→FA traceability; a GR line cannot be capitalised twice.</t>
+          <t>Asset-disposal maker-checker (SoD): a disposal REQUEST posts its GL entry as a DRAFT (excluded from balances) and flags the asset disposal_pending WITHOUT marking it disposed or moving the register; a DIFFERENT user must approve before it is effective (status→disposed, revaluation surplus recycled 3200→3100) (approver ≠ requester enforced regardless of permissions, reusing the GL-05 ledger approval). Reject voids the draft and the asset stays in service; only one disposal may be pending per asset; a disposal-pending asset is frozen from depreciation.</t>
         </is>
       </c>
       <c r="H119" s="17" t="inlineStr">
@@ -11194,7 +11194,7 @@
       </c>
       <c r="J119" s="17" t="inlineStr">
         <is>
-          <t>Per capital receipt</t>
+          <t>Per disposal</t>
         </is>
       </c>
       <c r="K119" s="16" t="inlineStr">
@@ -11209,22 +11209,22 @@
       </c>
       <c r="M119" s="16" t="inlineStr">
         <is>
-          <t>assets.service.ts registerFromGr/approveRegistration/rejectRegistration/eligibleFromGr; assets.controller.ts (registrations*); procurement.service.ts createGr (is_capital routing, costing excluded); schema/assets.ts asset_registration_requests + fixed_assets.source_gr_no/po_no + migration 0137; cutover/basics.ts + compliance.ts (ToE)</t>
+          <t>assets.service.ts dispose(pendingApproval Draft)/approveDisposal/rejectDisposal; assets.controller.ts (:assetNo/dispose/approve|reject); schema/assets.ts fixed_assets.disposal_pending + migration 0135; cutover/basics.ts + worldclass.ts + compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N119" s="16" t="inlineStr">
         <is>
-          <t>Inspect the eligible→request→approve flow + approver≠requester check + the inventory-vs-asset routing of capital lines.</t>
+          <t>Inspect Draft→approve flow + the approver≠requester check + deferred status/recycle.</t>
         </is>
       </c>
       <c r="O119" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: receive a capital line, raise a registration (no GL), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm the asset + Dr 1500/Cr 2000 post only after approval and the line cannot be re-registered (re-performed by the harnesses).</t>
+          <t>Re-perform: request a disposal (Draft JE excluded), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm status→disposed + surplus recycled only after approval (re-performed by the harnesses).</t>
         </is>
       </c>
       <c r="P119" s="16" t="inlineStr">
         <is>
-          <t>Capitalization approval log + SoD test</t>
+          <t>Disposal approval log + SoD test</t>
         </is>
       </c>
       <c r="Q119" s="18" t="inlineStr">
@@ -11236,12 +11236,12 @@
     <row r="120">
       <c r="A120" s="11" t="inlineStr">
         <is>
-          <t>CON-01</t>
+          <t>FA-10</t>
         </is>
       </c>
       <c r="B120" s="12" t="inlineStr">
         <is>
-          <t>Consolidation &amp; FX</t>
+          <t>Fixed Assets</t>
         </is>
       </c>
       <c r="C120" s="13" t="inlineStr">
@@ -11251,42 +11251,42 @@
       </c>
       <c r="D120" s="12" t="inlineStr">
         <is>
-          <t>Consolidation</t>
+          <t>Property, Plant &amp; Equipment; Accounts Payable</t>
         </is>
       </c>
       <c r="E120" s="12" t="inlineStr">
         <is>
-          <t>Group consolidation mis-stated (ownership/currency).</t>
+          <t>Capital purchases mis-capitalised or capitalised without independent review — the person who receives the goods also decides what enters the asset register and at what cost/useful life (fictitious or over-valued assets; capex/opex mis-classification).</t>
         </is>
       </c>
       <c r="F120" s="12" t="inlineStr">
         <is>
-          <t>Accuracy</t>
+          <t>Authorization; Accuracy</t>
         </is>
       </c>
       <c r="G120" s="12" t="inlineStr">
         <is>
-          <t>Consolidation run (ownership %, entity currency) gated by 'approvals'.</t>
+          <t>Procure-to-Capitalize maker-checker (SoD): a goods-receipt line flagged capital (item-master is_fixed_asset or per-PO-line override) is excluded from inventory capitalisation (1200) at receipt and instead becomes ELIGIBLE for the asset register. Capitalisation is a REQUEST that posts NOTHING to the GL; a DIFFERENT user must approve before the fixed_assets row + acquisition JE (Dr 1500 / Cr 2000) are created (approver ≠ requester enforced regardless of permissions). The created asset carries its source GR/PO for end-to-end PR→PO→GR→FA traceability; a GR line cannot be capitalised twice.</t>
         </is>
       </c>
       <c r="H120" s="13" t="inlineStr">
         <is>
-          <t>Auto+Manual</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I120" s="13" t="inlineStr">
         <is>
-          <t>Period</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J120" s="13" t="inlineStr">
         <is>
-          <t>Period</t>
+          <t>Per capital receipt</t>
         </is>
       </c>
       <c r="K120" s="12" t="inlineStr">
         <is>
-          <t>Group Controller</t>
+          <t>FaAccountant / Controller</t>
         </is>
       </c>
       <c r="L120" s="13" t="inlineStr">
@@ -11296,22 +11296,22 @@
       </c>
       <c r="M120" s="12" t="inlineStr">
         <is>
-          <t>consolidation.service.ts (runConsolidation @Permissions approvals)</t>
+          <t>assets.service.ts registerFromGr/approveRegistration/rejectRegistration/eligibleFromGr; assets.controller.ts (registrations*); procurement.service.ts createGr (is_capital routing, costing excluded); schema/assets.ts asset_registration_requests + fixed_assets.source_gr_no/po_no + migration 0137; cutover/basics.ts + compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N120" s="12" t="inlineStr">
         <is>
-          <t>Inspect consolidation logic + gate.</t>
+          <t>Inspect the eligible→request→approve flow + approver≠requester check + the inventory-vs-asset routing of capital lines.</t>
         </is>
       </c>
       <c r="O120" s="12" t="inlineStr">
         <is>
-          <t>Sample period: consolidated TB ties to entities.</t>
+          <t>Re-perform: receive a capital line, raise a registration (no GL), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm the asset + Dr 1500/Cr 2000 post only after approval and the line cannot be re-registered (re-performed by the harnesses).</t>
         </is>
       </c>
       <c r="P120" s="12" t="inlineStr">
         <is>
-          <t>Consol TB</t>
+          <t>Capitalization approval log + SoD test</t>
         </is>
       </c>
       <c r="Q120" s="18" t="inlineStr">
@@ -11323,7 +11323,7 @@
     <row r="121">
       <c r="A121" s="15" t="inlineStr">
         <is>
-          <t>CON-02</t>
+          <t>CON-01</t>
         </is>
       </c>
       <c r="B121" s="16" t="inlineStr">
@@ -11338,22 +11338,22 @@
       </c>
       <c r="D121" s="16" t="inlineStr">
         <is>
-          <t>FX gain/loss</t>
+          <t>Consolidation</t>
         </is>
       </c>
       <c r="E121" s="16" t="inlineStr">
         <is>
-          <t>FX exposures not revalued at period-end.</t>
+          <t>Group consolidation mis-stated (ownership/currency).</t>
         </is>
       </c>
       <c r="F121" s="16" t="inlineStr">
         <is>
-          <t>Valuation</t>
+          <t>Accuracy</t>
         </is>
       </c>
       <c r="G121" s="16" t="inlineStr">
         <is>
-          <t>FX revaluation at period-end rates; unrealized FX posted (acct 5400).</t>
+          <t>Consolidation run (ownership %, entity currency) gated by 'approvals'.</t>
         </is>
       </c>
       <c r="H121" s="17" t="inlineStr">
@@ -11363,7 +11363,7 @@
       </c>
       <c r="I121" s="17" t="inlineStr">
         <is>
-          <t>Period-end</t>
+          <t>Period</t>
         </is>
       </c>
       <c r="J121" s="17" t="inlineStr">
@@ -11373,7 +11373,7 @@
       </c>
       <c r="K121" s="16" t="inlineStr">
         <is>
-          <t>Controller</t>
+          <t>Group Controller</t>
         </is>
       </c>
       <c r="L121" s="17" t="inlineStr">
@@ -11383,22 +11383,22 @@
       </c>
       <c r="M121" s="16" t="inlineStr">
         <is>
-          <t>fx.service.ts (revalue / unrealized report)</t>
+          <t>consolidation.service.ts (runConsolidation @Permissions approvals)</t>
         </is>
       </c>
       <c r="N121" s="16" t="inlineStr">
         <is>
-          <t>Inspect reval logic + rates.</t>
+          <t>Inspect consolidation logic + gate.</t>
         </is>
       </c>
       <c r="O121" s="16" t="inlineStr">
         <is>
-          <t>Recompute reval on sample balances.</t>
+          <t>Sample period: consolidated TB ties to entities.</t>
         </is>
       </c>
       <c r="P121" s="16" t="inlineStr">
         <is>
-          <t>FX reval JE</t>
+          <t>Consol TB</t>
         </is>
       </c>
       <c r="Q121" s="18" t="inlineStr">
@@ -11410,7 +11410,7 @@
     <row r="122">
       <c r="A122" s="11" t="inlineStr">
         <is>
-          <t>FX-04</t>
+          <t>CON-02</t>
         </is>
       </c>
       <c r="B122" s="12" t="inlineStr">
@@ -11425,42 +11425,42 @@
       </c>
       <c r="D122" s="12" t="inlineStr">
         <is>
-          <t>FX gain/loss; Revenue; AR/AP</t>
+          <t>FX gain/loss</t>
         </is>
       </c>
       <c r="E122" s="12" t="inlineStr">
         <is>
-          <t>A wrong manually-entered FX rate (fat-fingered, e.g. USD 36 keyed as 63) flows straight into a period-end revaluation JE and the unrealized-FX report with no independent review — mis-stating earnings/equity and FX-translated balances.</t>
+          <t>FX exposures not revalued at period-end.</t>
         </is>
       </c>
       <c r="F122" s="12" t="inlineStr">
         <is>
-          <t>Accuracy/Valuation</t>
+          <t>Valuation</t>
         </is>
       </c>
       <c r="G122" s="12" t="inlineStr">
         <is>
-          <t>FX rate maker-checker (SoD): a MANUALLY-entered rate lands as PendingApproval and is EXCLUDED from rate resolution — revaluation, the unrealized-FX report, and consolidation translation all use APPROVED rates only — until a DIFFERENT user approves it (POST /api/fx/rates/approve). Self-approval → SOD_VIOLATION (binds even Admin); reject marks the rate Rejected (never usable); re-entering a rate sends it back to PendingApproval. Externally-sourced (feed) rates carrying an explicit non-manual source are auto-approved. Pending rates are also surfaced, aged, by the pending-approvals monitor (GOV-01).</t>
+          <t>FX revaluation at period-end rates; unrealized FX posted (acct 5400).</t>
         </is>
       </c>
       <c r="H122" s="13" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="I122" s="13" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Period-end</t>
         </is>
       </c>
       <c r="J122" s="13" t="inlineStr">
         <is>
-          <t>Per rate</t>
+          <t>Period</t>
         </is>
       </c>
       <c r="K122" s="12" t="inlineStr">
         <is>
-          <t>Controller / Treasury</t>
+          <t>Controller</t>
         </is>
       </c>
       <c r="L122" s="13" t="inlineStr">
@@ -11470,22 +11470,22 @@
       </c>
       <c r="M122" s="12" t="inlineStr">
         <is>
-          <t>fx.service.ts setRate(manual→PendingApproval)/approveRate/rejectRate/rateAsOf(Approved only); fx.controller.ts (rates/approve|reject|pending gated approvals/gl_close); consolidation.service.ts (translation reads Approved rates); schema/fx.ts fx_rates.status + migration 0141; cutover/fxreval.ts (ToE)</t>
+          <t>fx.service.ts (revalue / unrealized report)</t>
         </is>
       </c>
       <c r="N122" s="12" t="inlineStr">
         <is>
-          <t>Inspect the request→approve flow + the approver≠requester check + that revaluation/reporting resolve Approved rates only.</t>
+          <t>Inspect reval logic + rates.</t>
         </is>
       </c>
       <c r="O122" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: enter a manual rate (PendingApproval), confirm revalue is blocked NO_RATE while pending, attempt self-approve (SOD_VIOLATION), approve as a different user, then revalue succeeds (re-performed by the fxreval harness).</t>
+          <t>Recompute reval on sample balances.</t>
         </is>
       </c>
       <c r="P122" s="12" t="inlineStr">
         <is>
-          <t>FX rate approval log + SoD test</t>
+          <t>FX reval JE</t>
         </is>
       </c>
       <c r="Q122" s="18" t="inlineStr">
@@ -11497,92 +11497,179 @@
     <row r="123">
       <c r="A123" s="15" t="inlineStr">
         <is>
+          <t>FX-04</t>
+        </is>
+      </c>
+      <c r="B123" s="16" t="inlineStr">
+        <is>
+          <t>Consolidation &amp; FX</t>
+        </is>
+      </c>
+      <c r="C123" s="17" t="inlineStr">
+        <is>
+          <t>Application</t>
+        </is>
+      </c>
+      <c r="D123" s="16" t="inlineStr">
+        <is>
+          <t>FX gain/loss; Revenue; AR/AP</t>
+        </is>
+      </c>
+      <c r="E123" s="16" t="inlineStr">
+        <is>
+          <t>A wrong manually-entered FX rate (fat-fingered, e.g. USD 36 keyed as 63) flows straight into a period-end revaluation JE and the unrealized-FX report with no independent review — mis-stating earnings/equity and FX-translated balances.</t>
+        </is>
+      </c>
+      <c r="F123" s="16" t="inlineStr">
+        <is>
+          <t>Accuracy/Valuation</t>
+        </is>
+      </c>
+      <c r="G123" s="16" t="inlineStr">
+        <is>
+          <t>FX rate maker-checker (SoD): a MANUALLY-entered rate lands as PendingApproval and is EXCLUDED from rate resolution — revaluation, the unrealized-FX report, and consolidation translation all use APPROVED rates only — until a DIFFERENT user approves it (POST /api/fx/rates/approve). Self-approval → SOD_VIOLATION (binds even Admin); reject marks the rate Rejected (never usable); re-entering a rate sends it back to PendingApproval. Externally-sourced (feed) rates carrying an explicit non-manual source are auto-approved. Pending rates are also surfaced, aged, by the pending-approvals monitor (GOV-01).</t>
+        </is>
+      </c>
+      <c r="H123" s="17" t="inlineStr">
+        <is>
+          <t>Prev</t>
+        </is>
+      </c>
+      <c r="I123" s="17" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="J123" s="17" t="inlineStr">
+        <is>
+          <t>Per rate</t>
+        </is>
+      </c>
+      <c r="K123" s="16" t="inlineStr">
+        <is>
+          <t>Controller / Treasury</t>
+        </is>
+      </c>
+      <c r="L123" s="17" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="M123" s="16" t="inlineStr">
+        <is>
+          <t>fx.service.ts setRate(manual→PendingApproval)/approveRate/rejectRate/rateAsOf(Approved only); fx.controller.ts (rates/approve|reject|pending gated approvals/gl_close); consolidation.service.ts (translation reads Approved rates); schema/fx.ts fx_rates.status + migration 0141; cutover/fxreval.ts (ToE)</t>
+        </is>
+      </c>
+      <c r="N123" s="16" t="inlineStr">
+        <is>
+          <t>Inspect the request→approve flow + the approver≠requester check + that revaluation/reporting resolve Approved rates only.</t>
+        </is>
+      </c>
+      <c r="O123" s="16" t="inlineStr">
+        <is>
+          <t>Re-perform: enter a manual rate (PendingApproval), confirm revalue is blocked NO_RATE while pending, attempt self-approve (SOD_VIOLATION), approve as a different user, then revalue succeeds (re-performed by the fxreval harness).</t>
+        </is>
+      </c>
+      <c r="P123" s="16" t="inlineStr">
+        <is>
+          <t>FX rate approval log + SoD test</t>
+        </is>
+      </c>
+      <c r="Q123" s="18" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="11" t="inlineStr">
+        <is>
           <t>BUD-01</t>
         </is>
       </c>
-      <c r="B123" s="16" t="inlineStr">
+      <c r="B124" s="12" t="inlineStr">
         <is>
           <t>Budgeting &amp; Planning</t>
         </is>
       </c>
-      <c r="C123" s="17" t="inlineStr">
+      <c r="C124" s="13" t="inlineStr">
         <is>
           <t>Application</t>
         </is>
       </c>
-      <c r="D123" s="16" t="inlineStr">
+      <c r="D124" s="12" t="inlineStr">
         <is>
           <t>Budget; All (variance reporting)</t>
         </is>
       </c>
-      <c r="E123" s="16" t="inlineStr">
+      <c r="E124" s="12" t="inlineStr">
         <is>
           <t>A budget figure is entered/changed by one person and immediately drives the budget-vs-actual variance report — the basis for spend authorization and performance review — with no independent approval; a wrong or self-serving budget makes overspending look 'on budget'.</t>
         </is>
       </c>
-      <c r="F123" s="16" t="inlineStr">
+      <c r="F124" s="12" t="inlineStr">
         <is>
           <t>Authorization/Accuracy</t>
         </is>
       </c>
-      <c r="G123" s="16" t="inlineStr">
+      <c r="G124" s="12" t="inlineStr">
         <is>
           <t>Budget maker-checker (SoD): an upserted budget (POST /api/ledger/budgets) lands as PendingApproval and is EXCLUDED from budget-vs-actual until a DIFFERENT user approves it (POST /api/ledger/budgets/approve for the fiscal_year/account/cost-centre[/period]). Self-approval → SOD_VIOLATION (binds even Admin); reject marks it Rejected (excluded). DEFAULT 'Approved' keeps existing rows + direct planning seeds usable. Pending budgets are also surfaced, aged, by the pending-approvals monitor (GOV-01).</t>
         </is>
       </c>
-      <c r="H123" s="17" t="inlineStr">
+      <c r="H124" s="13" t="inlineStr">
         <is>
           <t>Prev</t>
         </is>
       </c>
-      <c r="I123" s="17" t="inlineStr">
+      <c r="I124" s="13" t="inlineStr">
         <is>
           <t>Automated</t>
         </is>
       </c>
-      <c r="J123" s="17" t="inlineStr">
+      <c r="J124" s="13" t="inlineStr">
         <is>
           <t>Per budget</t>
         </is>
       </c>
-      <c r="K123" s="16" t="inlineStr">
+      <c r="K124" s="12" t="inlineStr">
         <is>
           <t>Controller / FP&amp;A</t>
         </is>
       </c>
-      <c r="L123" s="17" t="inlineStr">
+      <c r="L124" s="13" t="inlineStr">
         <is>
           <t>P10</t>
         </is>
       </c>
-      <c r="M123" s="16" t="inlineStr">
+      <c r="M124" s="12" t="inlineStr">
         <is>
           <t>budget.service.ts upsertBudget(→PendingApproval)/approveBudget/rejectBudget/budgetVsActual(Approved only); budget.controller.ts (budgets/approve|reject|pending gated approvals/gl_close); schema/budgets.ts budgets.status + migration 0142; cutover/budget.ts (ToE)</t>
         </is>
       </c>
-      <c r="N123" s="16" t="inlineStr">
+      <c r="N124" s="12" t="inlineStr">
         <is>
           <t>Inspect the request→approve flow + the approver≠requester check + that budget-vs-actual counts Approved budgets only.</t>
         </is>
       </c>
-      <c r="O123" s="16" t="inlineStr">
+      <c r="O124" s="12" t="inlineStr">
         <is>
           <t>Re-perform: upsert a budget (PendingApproval, excluded from variance), attempt self-approve (SOD_VIOLATION), approve as a different user, confirm it then appears in budget-vs-actual (re-performed by the budget harness).</t>
         </is>
       </c>
-      <c r="P123" s="16" t="inlineStr">
+      <c r="P124" s="12" t="inlineStr">
         <is>
           <t>Budget approval log + SoD test</t>
         </is>
       </c>
-      <c r="Q123" s="18" t="inlineStr">
+      <c r="Q124" s="18" t="inlineStr">
         <is>
           <t>Implemented</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q123"/>
+  <autoFilter ref="A1:Q124"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -12765,7 +12852,7 @@
         </is>
       </c>
       <c r="C5" s="29">
-        <f>COUNTIF(RCM!$Q$2:$Q$123,B5)</f>
+        <f>COUNTIF(RCM!$Q$2:$Q$124,B5)</f>
         <v/>
       </c>
     </row>
@@ -12776,7 +12863,7 @@
         </is>
       </c>
       <c r="C6" s="29">
-        <f>COUNTIF(RCM!$Q$2:$Q$123,B6)</f>
+        <f>COUNTIF(RCM!$Q$2:$Q$124,B6)</f>
         <v/>
       </c>
     </row>
@@ -12787,7 +12874,7 @@
         </is>
       </c>
       <c r="C7" s="29">
-        <f>COUNTIF(RCM!$Q$2:$Q$123,B7)</f>
+        <f>COUNTIF(RCM!$Q$2:$Q$124,B7)</f>
         <v/>
       </c>
     </row>
@@ -12798,7 +12885,7 @@
         </is>
       </c>
       <c r="C8" s="32">
-        <f>COUNTA(RCM!$A$2:$A$123)</f>
+        <f>COUNTA(RCM!$A$2:$A$124)</f>
         <v/>
       </c>
     </row>
@@ -12816,7 +12903,7 @@
         </is>
       </c>
       <c r="C11" s="29">
-        <f>COUNTIF(RCM!$C$2:$C$123,B11)</f>
+        <f>COUNTIF(RCM!$C$2:$C$124,B11)</f>
         <v/>
       </c>
     </row>
@@ -12827,7 +12914,7 @@
         </is>
       </c>
       <c r="C12" s="29">
-        <f>COUNTIF(RCM!$C$2:$C$123,B12)</f>
+        <f>COUNTIF(RCM!$C$2:$C$124,B12)</f>
         <v/>
       </c>
     </row>
@@ -12838,7 +12925,7 @@
         </is>
       </c>
       <c r="C13" s="29">
-        <f>COUNTIF(RCM!$C$2:$C$123,B13)</f>
+        <f>COUNTIF(RCM!$C$2:$C$124,B13)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: merge main, renumber arap_controls 0166→0167 (thai_tax_filings took 0166)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/compliance/Oshinei_ERP_SOX_RCM_v1.xlsx
+++ b/compliance/Oshinei_ERP_SOX_RCM_v1.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'RCM'!$A$1:$Q$126</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'RCM'!$A$1:$Q$127</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Gap Remediation'!$A$2:$H$18</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -858,7 +858,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q126"/>
+  <dimension ref="A1:Q127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -11062,12 +11062,12 @@
     <row r="118">
       <c r="A118" s="11" t="inlineStr">
         <is>
-          <t>PAY-01</t>
+          <t>TAX-05</t>
         </is>
       </c>
       <c r="B118" s="12" t="inlineStr">
         <is>
-          <t>Payroll</t>
+          <t>Tax</t>
         </is>
       </c>
       <c r="C118" s="13" t="inlineStr">
@@ -11077,67 +11077,67 @@
       </c>
       <c r="D118" s="12" t="inlineStr">
         <is>
-          <t>Payroll expense/liability</t>
+          <t>Tax (VAT/WHT)</t>
         </is>
       </c>
       <c r="E118" s="12" t="inlineStr">
         <is>
-          <t>Payroll, SSO and PIT mis-computed.</t>
+          <t>A return is computed but there is no evidence it was actually FILED — no record of the figures as filed, the submission date or the Revenue-Department reference — so a missed or late filing (penalty/surcharge exposure) is not detected, and a filed return can be silently recomputed/altered after submission.</t>
         </is>
       </c>
       <c r="F118" s="12" t="inlineStr">
         <is>
-          <t>Accuracy</t>
+          <t>Completeness/Accuracy/Cutoff</t>
         </is>
       </c>
       <c r="G118" s="12" t="inlineStr">
         <is>
-          <t>Payroll engine — SSO 5% (cap 750), progressive PIT, payslip net; unit-tested.</t>
+          <t>Thai tax filing register + remittance calendar: a computed ภ.พ.30 (PP30) or ภ.ง.ด.3/53 (PND) return is SNAPSHOTTED into a thai_tax_filings record (one per tenant/type/period) carrying the figures as filed (output/input/net VAT, tax withheld) and a DRAFT→SUBMITTED→ACCEPTED lifecycle. Filing is idempotent per period; submitting REQUIRES a Revenue-Department submission reference (SUBMISSION_REF_REQUIRED) and stamps SUBMITTED + the timestamp; an already-filed (SUBMITTED/ACCEPTED) period is NOT silently overwritten when re-filed (returned as-is, already_filed=true). A remittance calendar (GET /api/tax-reports/remittance-calendar) lists every monthly obligation (ภ.พ.30 by the 15th, ภ.ง.ด. by the 7th of the following month) with its current status (NOT_FILED/DRAFT/SUBMITTED/ACCEPTED), so the controller sees what is due/filed/late before the deadline. Tenant-scoped (RLS); gated exec.</t>
         </is>
       </c>
       <c r="H118" s="13" t="inlineStr">
         <is>
-          <t>Auto</t>
+          <t>Det/Prev</t>
         </is>
       </c>
       <c r="I118" s="13" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="J118" s="13" t="inlineStr">
         <is>
-          <t>Per run</t>
+          <t>Monthly / per filing</t>
         </is>
       </c>
       <c r="K118" s="12" t="inlineStr">
         <is>
-          <t>HR / Payroll</t>
+          <t>Tax / FinancialController</t>
         </is>
       </c>
       <c r="L118" s="13" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P10/P16</t>
         </is>
       </c>
       <c r="M118" s="12" t="inlineStr">
         <is>
-          <t>payroll/payroll-calc.ts; test/unit.test.ts</t>
+          <t>tax-reports.service.ts fileReturn (snapshots pp30/pnd into a DRAFT, idempotent per period; no overwrite of a filed return) / submitFiling (SUBMISSION_REF_REQUIRED → SUBMITTED) / acceptFiling / listFilings / remittanceCalendar; tax-reports.controller.ts (POST filings[/:id/submit|accept], GET filings, remittance-calendar, exec); schema/tax-docs.ts thai_tax_filings + migration 0165; /tax/reports filings &amp; calendar tab; cutover/taxdocs.ts (ToE)</t>
         </is>
       </c>
       <c r="N118" s="12" t="inlineStr">
         <is>
-          <t>Inspect calc + tests.</t>
+          <t>Inspect the filing snapshot + the DRAFT→SUBMITTED→ACCEPTED lifecycle + the mandatory submission reference + the no-overwrite-of-a-filed-return rule + the deadline calendar.</t>
         </is>
       </c>
       <c r="O118" s="12" t="inlineStr">
         <is>
-          <t>Re-perform sample payslips.</t>
+          <t>Re-perform: file PP30 → DRAFT with the period figures; re-file refreshes the same DRAFT (idempotent); submit without a reference → 400; submit with a reference → SUBMITTED + timestamp; accept → ACCEPTED; re-filing an accepted period returns it (already_filed); the remittance calendar shows the period ACCEPTED with the 15th-of-next-month deadline (re-performed by the taxdocs harness).</t>
         </is>
       </c>
       <c r="P118" s="12" t="inlineStr">
         <is>
-          <t>Payslip tests</t>
+          <t>thai_tax_filings register + remittance calendar</t>
         </is>
       </c>
       <c r="Q118" s="18" t="inlineStr">
@@ -11149,7 +11149,7 @@
     <row r="119">
       <c r="A119" s="15" t="inlineStr">
         <is>
-          <t>PAY-02</t>
+          <t>PAY-01</t>
         </is>
       </c>
       <c r="B119" s="16" t="inlineStr">
@@ -11164,27 +11164,27 @@
       </c>
       <c r="D119" s="16" t="inlineStr">
         <is>
-          <t>Payroll liability</t>
+          <t>Payroll expense/liability</t>
         </is>
       </c>
       <c r="E119" s="16" t="inlineStr">
         <is>
-          <t>Statutory withholdings (SSO/WHT/PF) mis-stated or not remitted, so the liability owed to the authorities diverges from the books.</t>
+          <t>Payroll, SSO and PIT mis-computed.</t>
         </is>
       </c>
       <c r="F119" s="16" t="inlineStr">
         <is>
-          <t>Accuracy/Compliance</t>
+          <t>Accuracy</t>
         </is>
       </c>
       <c r="G119" s="16" t="inlineStr">
         <is>
-          <t>Payroll-liability schedule (GET /api/payroll/liabilities): each statutory account — SSO 2350, WHT/PND1 2360, PF 2370 — shows accrued (GL credits) − remitted (GL debits) = outstanding, tied back to the INDEPENDENT payrun accrual with a `reconciled` flag (a divergence flags a manual JE that touched a payroll-liability account outside the payroll process). Treasury remits the cash (POST .../remit → Dr liability / Cr 1000) which clears the outstanding and keeps the books reconciled to the statutory filings; a remittance beyond the outstanding is blocked (REMIT_EXCEEDS_OUTSTANDING).</t>
+          <t>Payroll engine — SSO 5% (cap 750), progressive PIT, payslip net; unit-tested.</t>
         </is>
       </c>
       <c r="H119" s="17" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Auto</t>
         </is>
       </c>
       <c r="I119" s="17" t="inlineStr">
@@ -11194,12 +11194,12 @@
       </c>
       <c r="J119" s="17" t="inlineStr">
         <is>
-          <t>Per run / monthly</t>
+          <t>Per run</t>
         </is>
       </c>
       <c r="K119" s="16" t="inlineStr">
         <is>
-          <t>HR / Payroll / Treasury</t>
+          <t>HR / Payroll</t>
         </is>
       </c>
       <c r="L119" s="17" t="inlineStr">
@@ -11209,22 +11209,22 @@
       </c>
       <c r="M119" s="16" t="inlineStr">
         <is>
-          <t>payroll/payroll.service.ts liabilities/remitLiability</t>
+          <t>payroll/payroll-calc.ts; test/unit.test.ts</t>
         </is>
       </c>
       <c r="N119" s="16" t="inlineStr">
         <is>
-          <t>Inspect the schedule + the accrued/remitted/outstanding tie-out and the reconciled flag.</t>
+          <t>Inspect calc + tests.</t>
         </is>
       </c>
       <c r="O119" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: run a payroll, confirm the SSO/WHT outstanding equals the payrun accrual; remit part and confirm the outstanding falls and the TB stays balanced; attempt an over-remit (REMIT_EXCEEDS_OUTSTANDING).</t>
+          <t>Re-perform sample payslips.</t>
         </is>
       </c>
       <c r="P119" s="16" t="inlineStr">
         <is>
-          <t>Liability schedule + remittance JEs tied to filings</t>
+          <t>Payslip tests</t>
         </is>
       </c>
       <c r="Q119" s="18" t="inlineStr">
@@ -11236,7 +11236,7 @@
     <row r="120">
       <c r="A120" s="11" t="inlineStr">
         <is>
-          <t>PAY-03</t>
+          <t>PAY-02</t>
         </is>
       </c>
       <c r="B120" s="12" t="inlineStr">
@@ -11251,27 +11251,27 @@
       </c>
       <c r="D120" s="12" t="inlineStr">
         <is>
-          <t>Payroll expense/liability; Cash</t>
+          <t>Payroll liability</t>
         </is>
       </c>
       <c r="E120" s="12" t="inlineStr">
         <is>
-          <t>Payroll run posted to the GL without independent review — the preparer both computes and posts their own payroll (ghost employees, inflated rate/hours).</t>
+          <t>Statutory withholdings (SSO/WHT/PF) mis-stated or not remitted, so the liability owed to the authorities diverges from the books.</t>
         </is>
       </c>
       <c r="F120" s="12" t="inlineStr">
         <is>
-          <t>Authorization</t>
+          <t>Accuracy/Compliance</t>
         </is>
       </c>
       <c r="G120" s="12" t="inlineStr">
         <is>
-          <t>Payroll maker-checker (SoD): a run posts its GL entry as a DRAFT (excluded from balances) with the run record 'PendingApproval'; a DIFFERENT user must approve before it becomes effective (approver ≠ preparer enforced regardless of permissions, reusing the GL-05 ledger approval). Reject voids the draft; idempotent per (tenant, period).</t>
+          <t>Payroll-liability schedule (GET /api/payroll/liabilities): each statutory account — SSO 2350, WHT/PND1 2360, PF 2370 — shows accrued (GL credits) − remitted (GL debits) = outstanding, tied back to the INDEPENDENT payrun accrual with a `reconciled` flag (a divergence flags a manual JE that touched a payroll-liability account outside the payroll process). Treasury remits the cash (POST .../remit → Dr liability / Cr 1000) which clears the outstanding and keeps the books reconciled to the statutory filings; a remittance beyond the outstanding is blocked (REMIT_EXCEEDS_OUTSTANDING).</t>
         </is>
       </c>
       <c r="H120" s="13" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I120" s="13" t="inlineStr">
@@ -11281,12 +11281,12 @@
       </c>
       <c r="J120" s="13" t="inlineStr">
         <is>
-          <t>Per run</t>
+          <t>Per run / monthly</t>
         </is>
       </c>
       <c r="K120" s="12" t="inlineStr">
         <is>
-          <t>HR / Payroll; Controller</t>
+          <t>HR / Payroll / Treasury</t>
         </is>
       </c>
       <c r="L120" s="13" t="inlineStr">
@@ -11296,22 +11296,22 @@
       </c>
       <c r="M120" s="12" t="inlineStr">
         <is>
-          <t>payroll/payroll.service.ts approvePayroll/rejectPayroll; migration 0133</t>
+          <t>payroll/payroll.service.ts liabilities/remitLiability</t>
         </is>
       </c>
       <c r="N120" s="12" t="inlineStr">
         <is>
-          <t>Inspect Draft→approve flow + the approver≠preparer check.</t>
+          <t>Inspect the schedule + the accrued/remitted/outstanding tie-out and the reconciled flag.</t>
         </is>
       </c>
       <c r="O120" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: run as A, attempt self-approve (SOD_VIOLATION), approve as B; confirm the JE hits balances only after approval.</t>
+          <t>Re-perform: run a payroll, confirm the SSO/WHT outstanding equals the payrun accrual; remit part and confirm the outstanding falls and the TB stays balanced; attempt an over-remit (REMIT_EXCEEDS_OUTSTANDING).</t>
         </is>
       </c>
       <c r="P120" s="12" t="inlineStr">
         <is>
-          <t>Approval log + SoD test</t>
+          <t>Liability schedule + remittance JEs tied to filings</t>
         </is>
       </c>
       <c r="Q120" s="18" t="inlineStr">
@@ -11323,12 +11323,12 @@
     <row r="121">
       <c r="A121" s="15" t="inlineStr">
         <is>
-          <t>FA-09</t>
+          <t>PAY-03</t>
         </is>
       </c>
       <c r="B121" s="16" t="inlineStr">
         <is>
-          <t>Fixed Assets</t>
+          <t>Payroll</t>
         </is>
       </c>
       <c r="C121" s="17" t="inlineStr">
@@ -11338,12 +11338,12 @@
       </c>
       <c r="D121" s="16" t="inlineStr">
         <is>
-          <t>Property, Plant &amp; Equipment; Cash</t>
+          <t>Payroll expense/liability; Cash</t>
         </is>
       </c>
       <c r="E121" s="16" t="inlineStr">
         <is>
-          <t>Asset disposed without independent review — one person writes an asset off the books and records the proceeds (asset-stripping / theft: dispose a still-held asset, or to a related party below value).</t>
+          <t>Payroll run posted to the GL without independent review — the preparer both computes and posts their own payroll (ghost employees, inflated rate/hours).</t>
         </is>
       </c>
       <c r="F121" s="16" t="inlineStr">
@@ -11353,7 +11353,7 @@
       </c>
       <c r="G121" s="16" t="inlineStr">
         <is>
-          <t>Asset-disposal maker-checker (SoD): a disposal REQUEST posts its GL entry as a DRAFT (excluded from balances) and flags the asset disposal_pending WITHOUT marking it disposed or moving the register; a DIFFERENT user must approve before it is effective (status→disposed, revaluation surplus recycled 3200→3100) (approver ≠ requester enforced regardless of permissions, reusing the GL-05 ledger approval). Reject voids the draft and the asset stays in service; only one disposal may be pending per asset; a disposal-pending asset is frozen from depreciation.</t>
+          <t>Payroll maker-checker (SoD): a run posts its GL entry as a DRAFT (excluded from balances) with the run record 'PendingApproval'; a DIFFERENT user must approve before it becomes effective (approver ≠ preparer enforced regardless of permissions, reusing the GL-05 ledger approval). Reject voids the draft; idempotent per (tenant, period).</t>
         </is>
       </c>
       <c r="H121" s="17" t="inlineStr">
@@ -11368,12 +11368,12 @@
       </c>
       <c r="J121" s="17" t="inlineStr">
         <is>
-          <t>Per disposal</t>
+          <t>Per run</t>
         </is>
       </c>
       <c r="K121" s="16" t="inlineStr">
         <is>
-          <t>FaAccountant / Controller</t>
+          <t>HR / Payroll; Controller</t>
         </is>
       </c>
       <c r="L121" s="17" t="inlineStr">
@@ -11383,22 +11383,22 @@
       </c>
       <c r="M121" s="16" t="inlineStr">
         <is>
-          <t>assets.service.ts dispose(pendingApproval Draft)/approveDisposal/rejectDisposal; assets.controller.ts (:assetNo/dispose/approve|reject); schema/assets.ts fixed_assets.disposal_pending + migration 0135; cutover/basics.ts + worldclass.ts + compliance.ts (ToE)</t>
+          <t>payroll/payroll.service.ts approvePayroll/rejectPayroll; migration 0133</t>
         </is>
       </c>
       <c r="N121" s="16" t="inlineStr">
         <is>
-          <t>Inspect Draft→approve flow + the approver≠requester check + deferred status/recycle.</t>
+          <t>Inspect Draft→approve flow + the approver≠preparer check.</t>
         </is>
       </c>
       <c r="O121" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: request a disposal (Draft JE excluded), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm status→disposed + surplus recycled only after approval (re-performed by the harnesses).</t>
+          <t>Re-perform: run as A, attempt self-approve (SOD_VIOLATION), approve as B; confirm the JE hits balances only after approval.</t>
         </is>
       </c>
       <c r="P121" s="16" t="inlineStr">
         <is>
-          <t>Disposal approval log + SoD test</t>
+          <t>Approval log + SoD test</t>
         </is>
       </c>
       <c r="Q121" s="18" t="inlineStr">
@@ -11410,7 +11410,7 @@
     <row r="122">
       <c r="A122" s="11" t="inlineStr">
         <is>
-          <t>FA-10</t>
+          <t>FA-09</t>
         </is>
       </c>
       <c r="B122" s="12" t="inlineStr">
@@ -11425,22 +11425,22 @@
       </c>
       <c r="D122" s="12" t="inlineStr">
         <is>
-          <t>Property, Plant &amp; Equipment; Accounts Payable</t>
+          <t>Property, Plant &amp; Equipment; Cash</t>
         </is>
       </c>
       <c r="E122" s="12" t="inlineStr">
         <is>
-          <t>Capital purchases mis-capitalised or capitalised without independent review — the person who receives the goods also decides what enters the asset register and at what cost/useful life (fictitious or over-valued assets; capex/opex mis-classification).</t>
+          <t>Asset disposed without independent review — one person writes an asset off the books and records the proceeds (asset-stripping / theft: dispose a still-held asset, or to a related party below value).</t>
         </is>
       </c>
       <c r="F122" s="12" t="inlineStr">
         <is>
-          <t>Authorization; Accuracy</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="G122" s="12" t="inlineStr">
         <is>
-          <t>Procure-to-Capitalize maker-checker (SoD): a goods-receipt line flagged capital (item-master is_fixed_asset or per-PO-line override) is excluded from inventory capitalisation (1200) at receipt and instead becomes ELIGIBLE for the asset register. Capitalisation is a REQUEST that posts NOTHING to the GL; a DIFFERENT user must approve before the fixed_assets row + acquisition JE (Dr 1500 / Cr 2000) are created (approver ≠ requester enforced regardless of permissions). The created asset carries its source GR/PO for end-to-end PR→PO→GR→FA traceability; a GR line cannot be capitalised twice.</t>
+          <t>Asset-disposal maker-checker (SoD): a disposal REQUEST posts its GL entry as a DRAFT (excluded from balances) and flags the asset disposal_pending WITHOUT marking it disposed or moving the register; a DIFFERENT user must approve before it is effective (status→disposed, revaluation surplus recycled 3200→3100) (approver ≠ requester enforced regardless of permissions, reusing the GL-05 ledger approval). Reject voids the draft and the asset stays in service; only one disposal may be pending per asset; a disposal-pending asset is frozen from depreciation.</t>
         </is>
       </c>
       <c r="H122" s="13" t="inlineStr">
@@ -11455,7 +11455,7 @@
       </c>
       <c r="J122" s="13" t="inlineStr">
         <is>
-          <t>Per capital receipt</t>
+          <t>Per disposal</t>
         </is>
       </c>
       <c r="K122" s="12" t="inlineStr">
@@ -11470,22 +11470,22 @@
       </c>
       <c r="M122" s="12" t="inlineStr">
         <is>
-          <t>assets.service.ts registerFromGr/approveRegistration/rejectRegistration/eligibleFromGr; assets.controller.ts (registrations*); procurement.service.ts createGr (is_capital routing, costing excluded); schema/assets.ts asset_registration_requests + fixed_assets.source_gr_no/po_no + migration 0137; cutover/basics.ts + compliance.ts (ToE)</t>
+          <t>assets.service.ts dispose(pendingApproval Draft)/approveDisposal/rejectDisposal; assets.controller.ts (:assetNo/dispose/approve|reject); schema/assets.ts fixed_assets.disposal_pending + migration 0135; cutover/basics.ts + worldclass.ts + compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N122" s="12" t="inlineStr">
         <is>
-          <t>Inspect the eligible→request→approve flow + approver≠requester check + the inventory-vs-asset routing of capital lines.</t>
+          <t>Inspect Draft→approve flow + the approver≠requester check + deferred status/recycle.</t>
         </is>
       </c>
       <c r="O122" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: receive a capital line, raise a registration (no GL), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm the asset + Dr 1500/Cr 2000 post only after approval and the line cannot be re-registered (re-performed by the harnesses).</t>
+          <t>Re-perform: request a disposal (Draft JE excluded), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm status→disposed + surplus recycled only after approval (re-performed by the harnesses).</t>
         </is>
       </c>
       <c r="P122" s="12" t="inlineStr">
         <is>
-          <t>Capitalization approval log + SoD test</t>
+          <t>Disposal approval log + SoD test</t>
         </is>
       </c>
       <c r="Q122" s="18" t="inlineStr">
@@ -11497,12 +11497,12 @@
     <row r="123">
       <c r="A123" s="15" t="inlineStr">
         <is>
-          <t>CON-01</t>
+          <t>FA-10</t>
         </is>
       </c>
       <c r="B123" s="16" t="inlineStr">
         <is>
-          <t>Consolidation &amp; FX</t>
+          <t>Fixed Assets</t>
         </is>
       </c>
       <c r="C123" s="17" t="inlineStr">
@@ -11512,42 +11512,42 @@
       </c>
       <c r="D123" s="16" t="inlineStr">
         <is>
-          <t>Consolidation</t>
+          <t>Property, Plant &amp; Equipment; Accounts Payable</t>
         </is>
       </c>
       <c r="E123" s="16" t="inlineStr">
         <is>
-          <t>Group consolidation mis-stated (ownership/currency).</t>
+          <t>Capital purchases mis-capitalised or capitalised without independent review — the person who receives the goods also decides what enters the asset register and at what cost/useful life (fictitious or over-valued assets; capex/opex mis-classification).</t>
         </is>
       </c>
       <c r="F123" s="16" t="inlineStr">
         <is>
-          <t>Accuracy</t>
+          <t>Authorization; Accuracy</t>
         </is>
       </c>
       <c r="G123" s="16" t="inlineStr">
         <is>
-          <t>Consolidation run (ownership %, entity currency) gated by 'approvals'.</t>
+          <t>Procure-to-Capitalize maker-checker (SoD): a goods-receipt line flagged capital (item-master is_fixed_asset or per-PO-line override) is excluded from inventory capitalisation (1200) at receipt and instead becomes ELIGIBLE for the asset register. Capitalisation is a REQUEST that posts NOTHING to the GL; a DIFFERENT user must approve before the fixed_assets row + acquisition JE (Dr 1500 / Cr 2000) are created (approver ≠ requester enforced regardless of permissions). The created asset carries its source GR/PO for end-to-end PR→PO→GR→FA traceability; a GR line cannot be capitalised twice.</t>
         </is>
       </c>
       <c r="H123" s="17" t="inlineStr">
         <is>
-          <t>Auto+Manual</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I123" s="17" t="inlineStr">
         <is>
-          <t>Period</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J123" s="17" t="inlineStr">
         <is>
-          <t>Period</t>
+          <t>Per capital receipt</t>
         </is>
       </c>
       <c r="K123" s="16" t="inlineStr">
         <is>
-          <t>Group Controller</t>
+          <t>FaAccountant / Controller</t>
         </is>
       </c>
       <c r="L123" s="17" t="inlineStr">
@@ -11557,22 +11557,22 @@
       </c>
       <c r="M123" s="16" t="inlineStr">
         <is>
-          <t>consolidation.service.ts (runConsolidation @Permissions approvals)</t>
+          <t>assets.service.ts registerFromGr/approveRegistration/rejectRegistration/eligibleFromGr; assets.controller.ts (registrations*); procurement.service.ts createGr (is_capital routing, costing excluded); schema/assets.ts asset_registration_requests + fixed_assets.source_gr_no/po_no + migration 0137; cutover/basics.ts + compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N123" s="16" t="inlineStr">
         <is>
-          <t>Inspect consolidation logic + gate.</t>
+          <t>Inspect the eligible→request→approve flow + approver≠requester check + the inventory-vs-asset routing of capital lines.</t>
         </is>
       </c>
       <c r="O123" s="16" t="inlineStr">
         <is>
-          <t>Sample period: consolidated TB ties to entities.</t>
+          <t>Re-perform: receive a capital line, raise a registration (no GL), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm the asset + Dr 1500/Cr 2000 post only after approval and the line cannot be re-registered (re-performed by the harnesses).</t>
         </is>
       </c>
       <c r="P123" s="16" t="inlineStr">
         <is>
-          <t>Consol TB</t>
+          <t>Capitalization approval log + SoD test</t>
         </is>
       </c>
       <c r="Q123" s="18" t="inlineStr">
@@ -11584,7 +11584,7 @@
     <row r="124">
       <c r="A124" s="11" t="inlineStr">
         <is>
-          <t>CON-02</t>
+          <t>CON-01</t>
         </is>
       </c>
       <c r="B124" s="12" t="inlineStr">
@@ -11599,22 +11599,22 @@
       </c>
       <c r="D124" s="12" t="inlineStr">
         <is>
-          <t>FX gain/loss</t>
+          <t>Consolidation</t>
         </is>
       </c>
       <c r="E124" s="12" t="inlineStr">
         <is>
-          <t>FX exposures not revalued at period-end.</t>
+          <t>Group consolidation mis-stated (ownership/currency).</t>
         </is>
       </c>
       <c r="F124" s="12" t="inlineStr">
         <is>
-          <t>Valuation</t>
+          <t>Accuracy</t>
         </is>
       </c>
       <c r="G124" s="12" t="inlineStr">
         <is>
-          <t>FX revaluation at period-end rates; unrealized FX posted (acct 5400).</t>
+          <t>Consolidation run (ownership %, entity currency) gated by 'approvals'.</t>
         </is>
       </c>
       <c r="H124" s="13" t="inlineStr">
@@ -11624,7 +11624,7 @@
       </c>
       <c r="I124" s="13" t="inlineStr">
         <is>
-          <t>Period-end</t>
+          <t>Period</t>
         </is>
       </c>
       <c r="J124" s="13" t="inlineStr">
@@ -11634,7 +11634,7 @@
       </c>
       <c r="K124" s="12" t="inlineStr">
         <is>
-          <t>Controller</t>
+          <t>Group Controller</t>
         </is>
       </c>
       <c r="L124" s="13" t="inlineStr">
@@ -11644,22 +11644,22 @@
       </c>
       <c r="M124" s="12" t="inlineStr">
         <is>
-          <t>fx.service.ts (revalue / unrealized report)</t>
+          <t>consolidation.service.ts (runConsolidation @Permissions approvals)</t>
         </is>
       </c>
       <c r="N124" s="12" t="inlineStr">
         <is>
-          <t>Inspect reval logic + rates.</t>
+          <t>Inspect consolidation logic + gate.</t>
         </is>
       </c>
       <c r="O124" s="12" t="inlineStr">
         <is>
-          <t>Recompute reval on sample balances.</t>
+          <t>Sample period: consolidated TB ties to entities.</t>
         </is>
       </c>
       <c r="P124" s="12" t="inlineStr">
         <is>
-          <t>FX reval JE</t>
+          <t>Consol TB</t>
         </is>
       </c>
       <c r="Q124" s="18" t="inlineStr">
@@ -11671,7 +11671,7 @@
     <row r="125">
       <c r="A125" s="15" t="inlineStr">
         <is>
-          <t>FX-04</t>
+          <t>CON-02</t>
         </is>
       </c>
       <c r="B125" s="16" t="inlineStr">
@@ -11686,42 +11686,42 @@
       </c>
       <c r="D125" s="16" t="inlineStr">
         <is>
-          <t>FX gain/loss; Revenue; AR/AP</t>
+          <t>FX gain/loss</t>
         </is>
       </c>
       <c r="E125" s="16" t="inlineStr">
         <is>
-          <t>A wrong manually-entered FX rate (fat-fingered, e.g. USD 36 keyed as 63) flows straight into a period-end revaluation JE and the unrealized-FX report with no independent review — mis-stating earnings/equity and FX-translated balances.</t>
+          <t>FX exposures not revalued at period-end.</t>
         </is>
       </c>
       <c r="F125" s="16" t="inlineStr">
         <is>
-          <t>Accuracy/Valuation</t>
+          <t>Valuation</t>
         </is>
       </c>
       <c r="G125" s="16" t="inlineStr">
         <is>
-          <t>FX rate maker-checker (SoD): a MANUALLY-entered rate lands as PendingApproval and is EXCLUDED from rate resolution — revaluation, the unrealized-FX report, and consolidation translation all use APPROVED rates only — until a DIFFERENT user approves it (POST /api/fx/rates/approve). Self-approval → SOD_VIOLATION (binds even Admin); reject marks the rate Rejected (never usable); re-entering a rate sends it back to PendingApproval. Externally-sourced (feed) rates carrying an explicit non-manual source are auto-approved. Pending rates are also surfaced, aged, by the pending-approvals monitor (GOV-01).</t>
+          <t>FX revaluation at period-end rates; unrealized FX posted (acct 5400).</t>
         </is>
       </c>
       <c r="H125" s="17" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="I125" s="17" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Period-end</t>
         </is>
       </c>
       <c r="J125" s="17" t="inlineStr">
         <is>
-          <t>Per rate</t>
+          <t>Period</t>
         </is>
       </c>
       <c r="K125" s="16" t="inlineStr">
         <is>
-          <t>Controller / Treasury</t>
+          <t>Controller</t>
         </is>
       </c>
       <c r="L125" s="17" t="inlineStr">
@@ -11731,22 +11731,22 @@
       </c>
       <c r="M125" s="16" t="inlineStr">
         <is>
-          <t>fx.service.ts setRate(manual→PendingApproval)/approveRate/rejectRate/rateAsOf(Approved only); fx.controller.ts (rates/approve|reject|pending gated approvals/gl_close); consolidation.service.ts (translation reads Approved rates); schema/fx.ts fx_rates.status + migration 0141; cutover/fxreval.ts (ToE)</t>
+          <t>fx.service.ts (revalue / unrealized report)</t>
         </is>
       </c>
       <c r="N125" s="16" t="inlineStr">
         <is>
-          <t>Inspect the request→approve flow + the approver≠requester check + that revaluation/reporting resolve Approved rates only.</t>
+          <t>Inspect reval logic + rates.</t>
         </is>
       </c>
       <c r="O125" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: enter a manual rate (PendingApproval), confirm revalue is blocked NO_RATE while pending, attempt self-approve (SOD_VIOLATION), approve as a different user, then revalue succeeds (re-performed by the fxreval harness).</t>
+          <t>Recompute reval on sample balances.</t>
         </is>
       </c>
       <c r="P125" s="16" t="inlineStr">
         <is>
-          <t>FX rate approval log + SoD test</t>
+          <t>FX reval JE</t>
         </is>
       </c>
       <c r="Q125" s="18" t="inlineStr">
@@ -11758,92 +11758,179 @@
     <row r="126">
       <c r="A126" s="11" t="inlineStr">
         <is>
+          <t>FX-04</t>
+        </is>
+      </c>
+      <c r="B126" s="12" t="inlineStr">
+        <is>
+          <t>Consolidation &amp; FX</t>
+        </is>
+      </c>
+      <c r="C126" s="13" t="inlineStr">
+        <is>
+          <t>Application</t>
+        </is>
+      </c>
+      <c r="D126" s="12" t="inlineStr">
+        <is>
+          <t>FX gain/loss; Revenue; AR/AP</t>
+        </is>
+      </c>
+      <c r="E126" s="12" t="inlineStr">
+        <is>
+          <t>A wrong manually-entered FX rate (fat-fingered, e.g. USD 36 keyed as 63) flows straight into a period-end revaluation JE and the unrealized-FX report with no independent review — mis-stating earnings/equity and FX-translated balances.</t>
+        </is>
+      </c>
+      <c r="F126" s="12" t="inlineStr">
+        <is>
+          <t>Accuracy/Valuation</t>
+        </is>
+      </c>
+      <c r="G126" s="12" t="inlineStr">
+        <is>
+          <t>FX rate maker-checker (SoD): a MANUALLY-entered rate lands as PendingApproval and is EXCLUDED from rate resolution — revaluation, the unrealized-FX report, and consolidation translation all use APPROVED rates only — until a DIFFERENT user approves it (POST /api/fx/rates/approve). Self-approval → SOD_VIOLATION (binds even Admin); reject marks the rate Rejected (never usable); re-entering a rate sends it back to PendingApproval. Externally-sourced (feed) rates carrying an explicit non-manual source are auto-approved. Pending rates are also surfaced, aged, by the pending-approvals monitor (GOV-01).</t>
+        </is>
+      </c>
+      <c r="H126" s="13" t="inlineStr">
+        <is>
+          <t>Prev</t>
+        </is>
+      </c>
+      <c r="I126" s="13" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="J126" s="13" t="inlineStr">
+        <is>
+          <t>Per rate</t>
+        </is>
+      </c>
+      <c r="K126" s="12" t="inlineStr">
+        <is>
+          <t>Controller / Treasury</t>
+        </is>
+      </c>
+      <c r="L126" s="13" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="M126" s="12" t="inlineStr">
+        <is>
+          <t>fx.service.ts setRate(manual→PendingApproval)/approveRate/rejectRate/rateAsOf(Approved only); fx.controller.ts (rates/approve|reject|pending gated approvals/gl_close); consolidation.service.ts (translation reads Approved rates); schema/fx.ts fx_rates.status + migration 0141; cutover/fxreval.ts (ToE)</t>
+        </is>
+      </c>
+      <c r="N126" s="12" t="inlineStr">
+        <is>
+          <t>Inspect the request→approve flow + the approver≠requester check + that revaluation/reporting resolve Approved rates only.</t>
+        </is>
+      </c>
+      <c r="O126" s="12" t="inlineStr">
+        <is>
+          <t>Re-perform: enter a manual rate (PendingApproval), confirm revalue is blocked NO_RATE while pending, attempt self-approve (SOD_VIOLATION), approve as a different user, then revalue succeeds (re-performed by the fxreval harness).</t>
+        </is>
+      </c>
+      <c r="P126" s="12" t="inlineStr">
+        <is>
+          <t>FX rate approval log + SoD test</t>
+        </is>
+      </c>
+      <c r="Q126" s="18" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="15" t="inlineStr">
+        <is>
           <t>BUD-01</t>
         </is>
       </c>
-      <c r="B126" s="12" t="inlineStr">
+      <c r="B127" s="16" t="inlineStr">
         <is>
           <t>Budgeting &amp; Planning</t>
         </is>
       </c>
-      <c r="C126" s="13" t="inlineStr">
+      <c r="C127" s="17" t="inlineStr">
         <is>
           <t>Application</t>
         </is>
       </c>
-      <c r="D126" s="12" t="inlineStr">
+      <c r="D127" s="16" t="inlineStr">
         <is>
           <t>Budget; All (variance reporting)</t>
         </is>
       </c>
-      <c r="E126" s="12" t="inlineStr">
+      <c r="E127" s="16" t="inlineStr">
         <is>
           <t>A budget figure is entered/changed by one person and immediately drives the budget-vs-actual variance report — the basis for spend authorization and performance review — with no independent approval; a wrong or self-serving budget makes overspending look 'on budget'.</t>
         </is>
       </c>
-      <c r="F126" s="12" t="inlineStr">
+      <c r="F127" s="16" t="inlineStr">
         <is>
           <t>Authorization/Accuracy</t>
         </is>
       </c>
-      <c r="G126" s="12" t="inlineStr">
+      <c r="G127" s="16" t="inlineStr">
         <is>
           <t>Budget maker-checker (SoD): an upserted budget (POST /api/ledger/budgets) lands as PendingApproval and is EXCLUDED from budget-vs-actual until a DIFFERENT user approves it (POST /api/ledger/budgets/approve for the fiscal_year/account/cost-centre[/period]). Self-approval → SOD_VIOLATION (binds even Admin); reject marks it Rejected (excluded). DEFAULT 'Approved' keeps existing rows + direct planning seeds usable. Pending budgets are also surfaced, aged, by the pending-approvals monitor (GOV-01).</t>
         </is>
       </c>
-      <c r="H126" s="13" t="inlineStr">
+      <c r="H127" s="17" t="inlineStr">
         <is>
           <t>Prev</t>
         </is>
       </c>
-      <c r="I126" s="13" t="inlineStr">
+      <c r="I127" s="17" t="inlineStr">
         <is>
           <t>Automated</t>
         </is>
       </c>
-      <c r="J126" s="13" t="inlineStr">
+      <c r="J127" s="17" t="inlineStr">
         <is>
           <t>Per budget</t>
         </is>
       </c>
-      <c r="K126" s="12" t="inlineStr">
+      <c r="K127" s="16" t="inlineStr">
         <is>
           <t>Controller / FP&amp;A</t>
         </is>
       </c>
-      <c r="L126" s="13" t="inlineStr">
+      <c r="L127" s="17" t="inlineStr">
         <is>
           <t>P10</t>
         </is>
       </c>
-      <c r="M126" s="12" t="inlineStr">
+      <c r="M127" s="16" t="inlineStr">
         <is>
           <t>budget.service.ts upsertBudget(→PendingApproval)/approveBudget/rejectBudget/budgetVsActual(Approved only); budget.controller.ts (budgets/approve|reject|pending gated approvals/gl_close); schema/budgets.ts budgets.status + migration 0142; cutover/budget.ts (ToE)</t>
         </is>
       </c>
-      <c r="N126" s="12" t="inlineStr">
+      <c r="N127" s="16" t="inlineStr">
         <is>
           <t>Inspect the request→approve flow + the approver≠requester check + that budget-vs-actual counts Approved budgets only.</t>
         </is>
       </c>
-      <c r="O126" s="12" t="inlineStr">
+      <c r="O127" s="16" t="inlineStr">
         <is>
           <t>Re-perform: upsert a budget (PendingApproval, excluded from variance), attempt self-approve (SOD_VIOLATION), approve as a different user, confirm it then appears in budget-vs-actual (re-performed by the budget harness).</t>
         </is>
       </c>
-      <c r="P126" s="12" t="inlineStr">
+      <c r="P127" s="16" t="inlineStr">
         <is>
           <t>Budget approval log + SoD test</t>
         </is>
       </c>
-      <c r="Q126" s="18" t="inlineStr">
+      <c r="Q127" s="18" t="inlineStr">
         <is>
           <t>Implemented</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q126"/>
+  <autoFilter ref="A1:Q127"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -13026,7 +13113,7 @@
         </is>
       </c>
       <c r="C5" s="29">
-        <f>COUNTIF(RCM!$Q$2:$Q$126,B5)</f>
+        <f>COUNTIF(RCM!$Q$2:$Q$127,B5)</f>
         <v/>
       </c>
     </row>
@@ -13037,7 +13124,7 @@
         </is>
       </c>
       <c r="C6" s="29">
-        <f>COUNTIF(RCM!$Q$2:$Q$126,B6)</f>
+        <f>COUNTIF(RCM!$Q$2:$Q$127,B6)</f>
         <v/>
       </c>
     </row>
@@ -13048,7 +13135,7 @@
         </is>
       </c>
       <c r="C7" s="29">
-        <f>COUNTIF(RCM!$Q$2:$Q$126,B7)</f>
+        <f>COUNTIF(RCM!$Q$2:$Q$127,B7)</f>
         <v/>
       </c>
     </row>
@@ -13059,7 +13146,7 @@
         </is>
       </c>
       <c r="C8" s="32">
-        <f>COUNTA(RCM!$A$2:$A$126)</f>
+        <f>COUNTA(RCM!$A$2:$A$127)</f>
         <v/>
       </c>
     </row>
@@ -13077,7 +13164,7 @@
         </is>
       </c>
       <c r="C11" s="29">
-        <f>COUNTIF(RCM!$C$2:$C$126,B11)</f>
+        <f>COUNTIF(RCM!$C$2:$C$127,B11)</f>
         <v/>
       </c>
     </row>
@@ -13088,7 +13175,7 @@
         </is>
       </c>
       <c r="C12" s="29">
-        <f>COUNTIF(RCM!$C$2:$C$126,B12)</f>
+        <f>COUNTIF(RCM!$C$2:$C$127,B12)</f>
         <v/>
       </c>
     </row>
@@ -13099,7 +13186,7 @@
         </is>
       </c>
       <c r="C13" s="29">
-        <f>COUNTIF(RCM!$C$2:$C$126,B13)</f>
+        <f>COUNTIF(RCM!$C$2:$C$127,B13)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(gl): WS3.2 — FX revaluation + deferred tax (GL-18, TAX-06)
- fx_reval_runs + deferred_tax_runs tables (migration 0168) + RLS;
  new COA 1700 (DTA), 2700 (DTL), 5950 (deferred tax expense)
- FxRevalService: period-end reval of foreign monetary AR/AP/bank at
  closing rate → net unrealized FX to 5400; maker-checker run→post,
  idempotent, reuses approved fx_rates; viaSubledger control-guard ok
- DeferredTaxService: temp diffs (AR allowance DTA, accel-dep DTL at
  documented 1.5x tax factor) × 20% CIT → posts delta Dr1700/Cr5950
- both respect PERIOD_LOCKED + GL-17 audit; close checklist gains
  deferred_tax step
- basics 201/201, worldclass 57/57, compliance 106 green
- GL-18 + TAX-06 RCM (128); narratives 04/06 + user-manual + UAT

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/compliance/Oshinei_ERP_SOX_RCM_v1.xlsx
+++ b/compliance/Oshinei_ERP_SOX_RCM_v1.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'RCM'!$A$1:$Q$127</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'RCM'!$A$1:$Q$129</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Gap Remediation'!$A$2:$H$18</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -858,7 +858,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q127"/>
+  <dimension ref="A1:Q129"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -9583,12 +9583,12 @@
     <row r="101">
       <c r="A101" s="15" t="inlineStr">
         <is>
-          <t>EXP-07</t>
+          <t>GL-18</t>
         </is>
       </c>
       <c r="B101" s="16" t="inlineStr">
         <is>
-          <t>Expenditure</t>
+          <t>General Ledger</t>
         </is>
       </c>
       <c r="C101" s="17" t="inlineStr">
@@ -9598,27 +9598,27 @@
       </c>
       <c r="D101" s="16" t="inlineStr">
         <is>
-          <t>Cash; Operating expense</t>
+          <t>Accounts Receivable (1100); Accounts Payable (2000); FX Gain/Loss (5400)</t>
         </is>
       </c>
       <c r="E101" s="16" t="inlineStr">
         <is>
-          <t>Petty-cash / employee advance issued but never accounted for — cash leakage, expense unrecorded.</t>
+          <t>Open foreign-currency monetary balances (AR/AP) are not restated to the period-end closing rate, or a revaluation is computed and posted by one person with no independent review — the unrealized FX gain/loss is omitted/mis-stated and a single user can move earnings through the FX line.</t>
         </is>
       </c>
       <c r="F101" s="16" t="inlineStr">
         <is>
-          <t>Existence/Completeness</t>
+          <t>Accuracy/Valuation/Authorization/Segregation of Duties</t>
         </is>
       </c>
       <c r="G101" s="16" t="inlineStr">
         <is>
-          <t>Employee cash advances: issuing an advance debits the 1180 Employee Advances control (Dr 1180 / Cr 1000); settlement clears it against actual spend + returned cash (Dr expense + Dr 1000 / Cr 1180), enforced to reconcile (settled_expense + returned_cash must equal the advance → SETTLE_MISMATCH). The 1180 balance is the outstanding float subject to review.</t>
+          <t>Period-end FX revaluation governance (maker-checker, idempotent per (tenant, period)): POST /api/ledger/fx-reval/run computes the unrealized FX on every OPEN foreign-currency AR/AP balance — delta_thb = open_foreign × (closing_rate − booked_rate) — staging an 'Open' fx_reval_runs row (one per tenant/period; re-running an Open period refreshes it; a Posted period → ALREADY_POSTED). Closing rates come from the request `rates` map first, else the latest APPROVED fx_rates row (FX-04); a currency with no rate from either → MISSING_RATE (an unapproved manual rate can never drive the reval). POST /api/ledger/fx-reval/:id/post is segregated — the poster MUST differ from the runner (SELF_POST) — and posts the net to 5400 (net gain → Cr 5400; net loss → Dr 5400) with the AR/AP control restatements (Dr/Cr 1100, Dr/Cr 2000) via LedgerService.postEntry, so the WS2.1 PERIOD_LOCKED gate + the GL-17 audit trail apply. Marks the run Posted. SIGN: net P&amp;L = Σ(AR delta) − Σ(AP delta).</t>
         </is>
       </c>
       <c r="H101" s="17" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I101" s="17" t="inlineStr">
@@ -9628,12 +9628,12 @@
       </c>
       <c r="J101" s="17" t="inlineStr">
         <is>
-          <t>Per advance</t>
+          <t>Monthly / period-end</t>
         </is>
       </c>
       <c r="K101" s="16" t="inlineStr">
         <is>
-          <t>AP / Controller</t>
+          <t>Financial Controller</t>
         </is>
       </c>
       <c r="L101" s="17" t="inlineStr">
@@ -9643,22 +9643,22 @@
       </c>
       <c r="M101" s="16" t="inlineStr">
         <is>
-          <t>finance.service.ts (issueAdvance, settleAdvance reconcile-or-reject, listAdvances outstanding); finance.controller.ts (creditors/exec); schema/finance.ts (employee_advances) + migration 0120; cutover/basics.ts (ToE)</t>
+          <t>fx-reval.service.ts (runReval compute+stage Open, idempotent ALREADY_POSTED, rate resolution MISSING_RATE; postReval SELF_POST maker-checker + 5400/1100/2000 posting; list/get); fx-reval.controller.ts (gl_close/gl_post run + :id/post, gl_close/gl_post/exec read); schema/deferred-tax-fx.ts (fx_reval_runs, uq tenant/period); migration 0168 (tables + RLS); ledger.module.ts (service+controller wired); close.service.ts (fx_reval close-checklist step); reuses fx_rates (FX-04) + LedgerService.postEntry; cutover/basics.ts (GL-18 ToE)</t>
         </is>
       </c>
       <c r="N101" s="16" t="inlineStr">
         <is>
-          <t>Inspect issue/settle GL + settlement reconciliation guard.</t>
+          <t>Inspect the run→post lifecycle, the rate resolution (explicit/approved-only/MISSING_RATE), the SELF_POST maker-checker, and the 5400/1100/2000 posting through the period-lock gate.</t>
         </is>
       </c>
       <c r="O101" s="16" t="inlineStr">
         <is>
-          <t>Issue an advance (1180 up); settle 700+300 clears 1180; mismatched settle → SETTLE_MISMATCH (re-performed by the harness).</t>
+          <t>TC-GL-18-01: run on an open foreign AR+AP → net unrealized gain/loss with per-doc detail (Open); TC-GL-18-02: runner self-post → SELF_POST (403), a different user posts → 5400 movement, re-post → ALREADY_POSTED (400) (re-performed by the basics.ts harness).</t>
         </is>
       </c>
       <c r="P101" s="16" t="inlineStr">
         <is>
-          <t>Advance register; outstanding float</t>
+          <t>fx_reval_runs register (Open→Posted, runner/poster); the FXREVAL-RUN JE to 5400; period-end reval sign-off</t>
         </is>
       </c>
       <c r="Q101" s="18" t="inlineStr">
@@ -9670,7 +9670,7 @@
     <row r="102">
       <c r="A102" s="11" t="inlineStr">
         <is>
-          <t>EXP-08</t>
+          <t>EXP-07</t>
         </is>
       </c>
       <c r="B102" s="12" t="inlineStr">
@@ -9690,22 +9690,22 @@
       </c>
       <c r="E102" s="12" t="inlineStr">
         <is>
-          <t>Petty-cash disbursed beyond authority / without independent review, or drawn past the fund's limit — cash leakage, unauthorised or unrecorded expense, over-extended float.</t>
+          <t>Petty-cash / employee advance issued but never accounted for — cash leakage, expense unrecorded.</t>
         </is>
       </c>
       <c r="F102" s="12" t="inlineStr">
         <is>
-          <t>Authorization; Completeness</t>
+          <t>Existence/Completeness</t>
         </is>
       </c>
       <c r="G102" s="12" t="inlineStr">
         <is>
-          <t>Petty-cash imprest float + maker-checker on disbursement (SoD): a fund holds cash capped at a credit limit/วงเงิน (1015 Petty Cash, a cash account); each direct EXPENSE or ADVANCE is a REQUEST that posts NOTHING and a DIFFERENT user must approve before the GL posts (expense Dr &lt;expense&gt; / Cr 1015; advance Dr 1180 / Cr 1015) and the fund balance is decremented. Self-approval → SOD_VIOLATION (binds even Admin). A draw beyond the fund balance → INSUFFICIENT_FLOAT; establishing/replenishing above the float limit → OVER_FLOAT. Advances settle (Dr expense + Dr 1015 returned / Cr 1180), returning unused cash to the fund. Every request carries a document reference + receipt key + a status trail (StatusLog) and surfaces in the GOV-01 pending-approvals monitor.</t>
+          <t>Employee cash advances: issuing an advance debits the 1180 Employee Advances control (Dr 1180 / Cr 1000); settlement clears it against actual spend + returned cash (Dr expense + Dr 1000 / Cr 1180), enforced to reconcile (settled_expense + returned_cash must equal the advance → SETTLE_MISMATCH). The 1180 balance is the outstanding float subject to review.</t>
         </is>
       </c>
       <c r="H102" s="13" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I102" s="13" t="inlineStr">
@@ -9715,7 +9715,7 @@
       </c>
       <c r="J102" s="13" t="inlineStr">
         <is>
-          <t>Per disbursement</t>
+          <t>Per advance</t>
         </is>
       </c>
       <c r="K102" s="12" t="inlineStr">
@@ -9730,22 +9730,22 @@
       </c>
       <c r="M102" s="12" t="inlineStr">
         <is>
-          <t>petty-cash.service.ts (establishFund/replenishFund float guards, createRequest INSUFFICIENT_FLOAT, approveRequest SoD+GL, rejectRequest, settleRequest); petty-cash.controller.ts (creditors/exec); schema/petty-cash.ts (petty_cash_funds, expense_requests) + migration 0139; finance.service.ts pendingApprovals (GOV-01 source 7); cutover/basics.ts + compliance.ts (ToE)</t>
+          <t>finance.service.ts (issueAdvance, settleAdvance reconcile-or-reject, listAdvances outstanding); finance.controller.ts (creditors/exec); schema/finance.ts (employee_advances) + migration 0120; cutover/basics.ts (ToE)</t>
         </is>
       </c>
       <c r="N102" s="12" t="inlineStr">
         <is>
-          <t>Inspect the float ceiling + the request→approve flow + the approver≠requester check + that the request posts nothing until approval.</t>
+          <t>Inspect issue/settle GL + settlement reconciliation guard.</t>
         </is>
       </c>
       <c r="O102" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: establish a fund (Dr 1015), request an expense (no GL), self-approve → SOD_VIOLATION, approve as a different user → Dr expense/Cr 1015 + fund down; over-balance draw → INSUFFICIENT_FLOAT; advance approve→settle clears 1180; replenish past float → OVER_FLOAT (re-performed by the harnesses).</t>
+          <t>Issue an advance (1180 up); settle 700+300 clears 1180; mismatched settle → SETTLE_MISMATCH (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P102" s="12" t="inlineStr">
         <is>
-          <t>Fund register + disbursement approval log + SoD test</t>
+          <t>Advance register; outstanding float</t>
         </is>
       </c>
       <c r="Q102" s="18" t="inlineStr">
@@ -9757,7 +9757,7 @@
     <row r="103">
       <c r="A103" s="15" t="inlineStr">
         <is>
-          <t>EXP-09</t>
+          <t>EXP-08</t>
         </is>
       </c>
       <c r="B103" s="16" t="inlineStr">
@@ -9772,22 +9772,22 @@
       </c>
       <c r="D103" s="16" t="inlineStr">
         <is>
-          <t>Accounts Payable; Cash</t>
+          <t>Cash; Operating expense</t>
         </is>
       </c>
       <c r="E103" s="16" t="inlineStr">
         <is>
-          <t>A PO-based supplier invoice is paid before it is reconciled to its PO and goods receipt — disbursing cash for goods not received, at the wrong quantity, or above the agreed price (over-payment / duplicate / fictitious-receipt fraud), because the AP-pay flow never consults the 3-way match.</t>
+          <t>Petty-cash disbursed beyond authority / without independent review, or drawn past the fund's limit — cash leakage, unauthorised or unrecorded expense, over-extended float.</t>
         </is>
       </c>
       <c r="F103" s="16" t="inlineStr">
         <is>
-          <t>Occurrence/Accuracy/Authorization</t>
+          <t>Authorization; Completeness</t>
         </is>
       </c>
       <c r="G103" s="16" t="inlineStr">
         <is>
-          <t>3-way-match PAYMENT GATE: the AP disbursement flow (requestApPayment) calls ThreeWayMatchService.assertPayable BEFORE recording the payment request — a PO-based invoice that was run through match() and did NOT pass (qty/price variance beyond tolerance, over-invoiced, or unmatched line) and was NOT independently overridden is BLOCKED (MATCH_BLOCKED) so no cash can be requested or approved against it. The gate FAILS-OPEN for a non-PO bill (utilities / services / reimbursements never have a match row) so legitimate non-PO payables remain payable; it only blocks invoices subject to the match. Complements EXP-01 (the match + the maker-checked override) by wiring the verdict into the cash path and EXP-06 (the AP disbursement maker-checker).</t>
+          <t>Petty-cash imprest float + maker-checker on disbursement (SoD): a fund holds cash capped at a credit limit/วงเงิน (1015 Petty Cash, a cash account); each direct EXPENSE or ADVANCE is a REQUEST that posts NOTHING and a DIFFERENT user must approve before the GL posts (expense Dr &lt;expense&gt; / Cr 1015; advance Dr 1180 / Cr 1015) and the fund balance is decremented. Self-approval → SOD_VIOLATION (binds even Admin). A draw beyond the fund balance → INSUFFICIENT_FLOAT; establishing/replenishing above the float limit → OVER_FLOAT. Advances settle (Dr expense + Dr 1015 returned / Cr 1180), returning unused cash to the fund. Every request carries a document reference + receipt key + a status trail (StatusLog) and surfaces in the GOV-01 pending-approvals monitor.</t>
         </is>
       </c>
       <c r="H103" s="17" t="inlineStr">
@@ -9802,7 +9802,7 @@
       </c>
       <c r="J103" s="17" t="inlineStr">
         <is>
-          <t>Per payment</t>
+          <t>Per disbursement</t>
         </is>
       </c>
       <c r="K103" s="16" t="inlineStr">
@@ -9817,22 +9817,22 @@
       </c>
       <c r="M103" s="16" t="inlineStr">
         <is>
-          <t>finance.service.ts (requestApPayment → matchSvc.assertPayable); match/three-way-match.service.ts (assertPayable fail-open for non-PO, blocks not-payable &amp; not-overridden); finance.controller.ts (ap/transactions/:txnNo/pay); cutover/match.ts (ToE)</t>
+          <t>petty-cash.service.ts (establishFund/replenishFund float guards, createRequest INSUFFICIENT_FLOAT, approveRequest SoD+GL, rejectRequest, settleRequest); petty-cash.controller.ts (creditors/exec); schema/petty-cash.ts (petty_cash_funds, expense_requests) + migration 0139; finance.service.ts pendingApprovals (GOV-01 source 7); cutover/basics.ts + compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N103" s="16" t="inlineStr">
         <is>
-          <t>Inspect that the AP-pay request consults assertPayable and that a non-PO bill is exempt while a failed PO invoice is blocked.</t>
+          <t>Inspect the float ceiling + the request→approve flow + the approver≠requester check + that the request posts nothing until approval.</t>
         </is>
       </c>
       <c r="O103" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: a PO invoice with a qty/price variance over tolerance → pay request MATCH_BLOCKED; an independently-overridden / matched invoice → pay succeeds; a non-PO bill pays unblocked (re-performed by the match harness).</t>
+          <t>Re-perform: establish a fund (Dr 1015), request an expense (no GL), self-approve → SOD_VIOLATION, approve as a different user → Dr expense/Cr 1015 + fund down; over-balance draw → INSUFFICIENT_FLOAT; advance approve→settle clears 1180; replenish past float → OVER_FLOAT (re-performed by the harnesses).</t>
         </is>
       </c>
       <c r="P103" s="16" t="inlineStr">
         <is>
-          <t>Blocked-invoice worklist; payment-gate test</t>
+          <t>Fund register + disbursement approval log + SoD test</t>
         </is>
       </c>
       <c r="Q103" s="18" t="inlineStr">
@@ -9844,12 +9844,12 @@
     <row r="104">
       <c r="A104" s="11" t="inlineStr">
         <is>
-          <t>FA-07</t>
+          <t>EXP-09</t>
         </is>
       </c>
       <c r="B104" s="12" t="inlineStr">
         <is>
-          <t>Fixed Assets</t>
+          <t>Expenditure</t>
         </is>
       </c>
       <c r="C104" s="13" t="inlineStr">
@@ -9859,27 +9859,27 @@
       </c>
       <c r="D104" s="12" t="inlineStr">
         <is>
-          <t>Property, Plant &amp; Equipment; Equity</t>
+          <t>Accounts Payable; Cash</t>
         </is>
       </c>
       <c r="E104" s="12" t="inlineStr">
         <is>
-          <t>Carrying amount not adjusted for revaluation/impairment — asset over/understated.</t>
+          <t>A PO-based supplier invoice is paid before it is reconciled to its PO and goods receipt — disbursing cash for goods not received, at the wrong quantity, or above the agreed price (over-payment / duplicate / fictitious-receipt fraud), because the AP-pay flow never consults the 3-way match.</t>
         </is>
       </c>
       <c r="F104" s="12" t="inlineStr">
         <is>
-          <t>Valuation</t>
+          <t>Occurrence/Accuracy/Authorization</t>
         </is>
       </c>
       <c r="G104" s="12" t="inlineStr">
         <is>
-          <t>Asset revaluation / impairment: an upward revaluation credits the revaluation surplus in equity (Dr 1500 / Cr 3200); a downward revaluation (impairment) debits impairment loss (Dr 5820 / Cr 1500). The gross 1500 moves by the delta so the register stays tied to the GL; a no-op revaluation is rejected (NO_CHANGE). Every event is logged for the audit trail.</t>
+          <t>3-way-match PAYMENT GATE: the AP disbursement flow (requestApPayment) calls ThreeWayMatchService.assertPayable BEFORE recording the payment request — a PO-based invoice that was run through match() and did NOT pass (qty/price variance beyond tolerance, over-invoiced, or unmatched line) and was NOT independently overridden is BLOCKED (MATCH_BLOCKED) so no cash can be requested or approved against it. The gate FAILS-OPEN for a non-PO bill (utilities / services / reimbursements never have a match row) so legitimate non-PO payables remain payable; it only blocks invoices subject to the match. Complements EXP-01 (the match + the maker-checked override) by wiring the verdict into the cash path and EXP-06 (the AP disbursement maker-checker).</t>
         </is>
       </c>
       <c r="H104" s="13" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I104" s="13" t="inlineStr">
@@ -9889,12 +9889,12 @@
       </c>
       <c r="J104" s="13" t="inlineStr">
         <is>
-          <t>Per event</t>
+          <t>Per payment</t>
         </is>
       </c>
       <c r="K104" s="12" t="inlineStr">
         <is>
-          <t>FaAccountant / Controller</t>
+          <t>AP / Controller</t>
         </is>
       </c>
       <c r="L104" s="13" t="inlineStr">
@@ -9904,22 +9904,22 @@
       </c>
       <c r="M104" s="12" t="inlineStr">
         <is>
-          <t>assets.service.ts (revalue up→3200 / down→5820, listRevaluations; dispose recycles surplus 3200→3100); assets.controller.ts (exec/creditors); schema/assets.ts (asset_revaluations) + migration 0120; cutover/basics.ts (ToE)</t>
+          <t>finance.service.ts (requestApPayment → matchSvc.assertPayable); match/three-way-match.service.ts (assertPayable fail-open for non-PO, blocks not-payable &amp; not-overridden); finance.controller.ts (ap/transactions/:txnNo/pay); cutover/match.ts (ToE)</t>
         </is>
       </c>
       <c r="N104" s="12" t="inlineStr">
         <is>
-          <t>Inspect revaluation/impairment routing + audit log + disposal recycling.</t>
+          <t>Inspect that the AP-pay request consults assertPayable and that a non-PO bill is exempt while a failed PO invoice is blocked.</t>
         </is>
       </c>
       <c r="O104" s="12" t="inlineStr">
         <is>
-          <t>Upward revaluation credits 3200; impairment debits 5820; no-change → NO_CHANGE; both events logged; on disposal the revaluation surplus is recycled to retained earnings (Dr 3200 / Cr 3100), not through P&amp;L (re-performed by the harness).</t>
+          <t>Re-perform: a PO invoice with a qty/price variance over tolerance → pay request MATCH_BLOCKED; an independently-overridden / matched invoice → pay succeeds; a non-PO bill pays unblocked (re-performed by the match harness).</t>
         </is>
       </c>
       <c r="P104" s="12" t="inlineStr">
         <is>
-          <t>Revaluation log; disposal recycling JE</t>
+          <t>Blocked-invoice worklist; payment-gate test</t>
         </is>
       </c>
       <c r="Q104" s="18" t="inlineStr">
@@ -9931,7 +9931,7 @@
     <row r="105">
       <c r="A105" s="15" t="inlineStr">
         <is>
-          <t>FA-08</t>
+          <t>FA-07</t>
         </is>
       </c>
       <c r="B105" s="16" t="inlineStr">
@@ -9951,22 +9951,22 @@
       </c>
       <c r="E105" s="16" t="inlineStr">
         <is>
-          <t>Carrying amount changed by fair-value revaluation/impairment without independent review — the preparer revalues the asset and posts to equity/P&amp;L on their own (earnings/equity management).</t>
+          <t>Carrying amount not adjusted for revaluation/impairment — asset over/understated.</t>
         </is>
       </c>
       <c r="F105" s="16" t="inlineStr">
         <is>
-          <t>Authorization</t>
+          <t>Valuation</t>
         </is>
       </c>
       <c r="G105" s="16" t="inlineStr">
         <is>
-          <t>Asset-revaluation maker-checker (SoD): a revalue/impairment request posts its GL entry as a DRAFT (excluded from balances) and records status 'PendingApproval' WITHOUT moving the carrying value; a DIFFERENT user must approve before the JE is effective and the register is re-valued (approver ≠ preparer enforced regardless of permissions, reusing the GL-05 ledger approval). Reject voids the draft; only one revaluation may be pending per asset; the disposal surplus recycle counts only approved revaluations.</t>
+          <t>Asset revaluation / impairment: an upward revaluation credits the revaluation surplus in equity (Dr 1500 / Cr 3200); a downward revaluation (impairment) debits impairment loss (Dr 5820 / Cr 1500). The gross 1500 moves by the delta so the register stays tied to the GL; a no-op revaluation is rejected (NO_CHANGE). Every event is logged for the audit trail.</t>
         </is>
       </c>
       <c r="H105" s="17" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I105" s="17" t="inlineStr">
@@ -9991,22 +9991,22 @@
       </c>
       <c r="M105" s="16" t="inlineStr">
         <is>
-          <t>assets.service.ts revalue(pendingApproval Draft)/approveRevaluation/rejectRevaluation; assets.controller.ts (:assetNo/revalue/approve|reject); schema/assets.ts asset_revaluations.status + migration 0134; cutover/basics.ts + compliance.ts (ToE)</t>
+          <t>assets.service.ts (revalue up→3200 / down→5820, listRevaluations; dispose recycles surplus 3200→3100); assets.controller.ts (exec/creditors); schema/assets.ts (asset_revaluations) + migration 0120; cutover/basics.ts (ToE)</t>
         </is>
       </c>
       <c r="N105" s="16" t="inlineStr">
         <is>
-          <t>Inspect Draft→approve flow + the approver≠preparer check + deferred carrying-value update.</t>
+          <t>Inspect revaluation/impairment routing + audit log + disposal recycling.</t>
         </is>
       </c>
       <c r="O105" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: request a revaluation (Draft JE excluded from 3200), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm the surplus/impairment + carrying value move only after approval (re-performed by the harnesses).</t>
+          <t>Upward revaluation credits 3200; impairment debits 5820; no-change → NO_CHANGE; both events logged; on disposal the revaluation surplus is recycled to retained earnings (Dr 3200 / Cr 3100), not through P&amp;L (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P105" s="16" t="inlineStr">
         <is>
-          <t>Revaluation approval log + SoD test</t>
+          <t>Revaluation log; disposal recycling JE</t>
         </is>
       </c>
       <c r="Q105" s="18" t="inlineStr">
@@ -10018,12 +10018,12 @@
     <row r="106">
       <c r="A106" s="11" t="inlineStr">
         <is>
-          <t>LSE-01</t>
+          <t>FA-08</t>
         </is>
       </c>
       <c r="B106" s="12" t="inlineStr">
         <is>
-          <t>Leases</t>
+          <t>Fixed Assets</t>
         </is>
       </c>
       <c r="C106" s="13" t="inlineStr">
@@ -10033,27 +10033,27 @@
       </c>
       <c r="D106" s="12" t="inlineStr">
         <is>
-          <t>Right-of-use assets; Lease liabilities</t>
+          <t>Property, Plant &amp; Equipment; Equity</t>
         </is>
       </c>
       <c r="E106" s="12" t="inlineStr">
         <is>
-          <t>Lease not capitalised (IFRS 16 / TFRS 16) — ROU asset + lease liability omitted; interest/depreciation mis-stated.</t>
+          <t>Carrying amount changed by fair-value revaluation/impairment without independent review — the preparer revalues the asset and posts to equity/P&amp;L on their own (earnings/equity management).</t>
         </is>
       </c>
       <c r="F106" s="12" t="inlineStr">
         <is>
-          <t>Completeness/Accuracy/Valuation</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="G106" s="12" t="inlineStr">
         <is>
-          <t>Lease accounting: at commencement a right-of-use asset and lease liability are recognised at the present value of the lease payments (Dr 1600 / Cr 2600). The scheduled job lease_periodic_run posts each period — interest unwinding on the liability (Dr 5900), the cash payment reducing the liability (Dr 2600 / Cr 1000), and straight-line ROU depreciation (Dr 5210 / Cr 1690) — the last period clearing the liability + ROU exactly. Idempotent per (lease, period).</t>
+          <t>Asset-revaluation maker-checker (SoD): a revalue/impairment request posts its GL entry as a DRAFT (excluded from balances) and records status 'PendingApproval' WITHOUT moving the carrying value; a DIFFERENT user must approve before the JE is effective and the register is re-valued (approver ≠ preparer enforced regardless of permissions, reusing the GL-05 ledger approval). Reject voids the draft; only one revaluation may be pending per asset; the disposal surplus recycle counts only approved revaluations.</t>
         </is>
       </c>
       <c r="H106" s="13" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I106" s="13" t="inlineStr">
@@ -10063,12 +10063,12 @@
       </c>
       <c r="J106" s="13" t="inlineStr">
         <is>
-          <t>Per period / per lease</t>
+          <t>Per event</t>
         </is>
       </c>
       <c r="K106" s="12" t="inlineStr">
         <is>
-          <t>Controller</t>
+          <t>FaAccountant / Controller</t>
         </is>
       </c>
       <c r="L106" s="13" t="inlineStr">
@@ -10078,22 +10078,22 @@
       </c>
       <c r="M106" s="12" t="inlineStr">
         <is>
-          <t>leases.service.ts (createLease PV recognition, runDueLeases interest+payment+depreciation, modifyLease remeasurement); leases.controller.ts (gl_post); bi.service.ts (lease_periodic_run); schema/leases.ts (leases, rou_nbv) + migration 0120/0121; cutover/basics.ts (ToE)</t>
+          <t>assets.service.ts revalue(pendingApproval Draft)/approveRevaluation/rejectRevaluation; assets.controller.ts (:assetNo/revalue/approve|reject); schema/assets.ts asset_revaluations.status + migration 0134; cutover/basics.ts + compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N106" s="12" t="inlineStr">
         <is>
-          <t>Inspect PV recognition + periodic interest/payment/depreciation + final-period clearing + modification remeasurement.</t>
+          <t>Inspect Draft→approve flow + the approver≠preparer check + deferred carrying-value update.</t>
         </is>
       </c>
       <c r="O106" s="12" t="inlineStr">
         <is>
-          <t>Commencement recognises ROU=liability=PV; periodic run posts interest+principal(=payment)+ROU depreciation; liability + ROU reduce; a modification remeasures the liability at the revised PV and adjusts the ROU by the same delta (Dr/Cr 1600↔2600), then depreciates over the remaining term (re-performed by the harness).</t>
+          <t>Re-perform: request a revaluation (Draft JE excluded from 3200), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm the surplus/impairment + carrying value move only after approval (re-performed by the harnesses).</t>
         </is>
       </c>
       <c r="P106" s="12" t="inlineStr">
         <is>
-          <t>Lease register; periodic run log; modification remeasurement</t>
+          <t>Revaluation approval log + SoD test</t>
         </is>
       </c>
       <c r="Q106" s="18" t="inlineStr">
@@ -10105,12 +10105,12 @@
     <row r="107">
       <c r="A107" s="15" t="inlineStr">
         <is>
-          <t>REC-01</t>
+          <t>LSE-01</t>
         </is>
       </c>
       <c r="B107" s="16" t="inlineStr">
         <is>
-          <t>Reconciliation</t>
+          <t>Leases</t>
         </is>
       </c>
       <c r="C107" s="17" t="inlineStr">
@@ -10120,22 +10120,22 @@
       </c>
       <c r="D107" s="16" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Right-of-use assets; Lease liabilities</t>
         </is>
       </c>
       <c r="E107" s="16" t="inlineStr">
         <is>
-          <t>Subledgers diverge from GL undetected.</t>
+          <t>Lease not capitalised (IFRS 16 / TFRS 16) — ROU asset + lease liability omitted; interest/depreciation mis-stated.</t>
         </is>
       </c>
       <c r="F107" s="16" t="inlineStr">
         <is>
-          <t>Completeness/Accuracy</t>
+          <t>Completeness/Accuracy/Valuation</t>
         </is>
       </c>
       <c r="G107" s="16" t="inlineStr">
         <is>
-          <t>Subledger-to-GL reconciliation per period: import GL, auto-match, certify (sign-off via 'approvals').</t>
+          <t>Lease accounting: at commencement a right-of-use asset and lease liability are recognised at the present value of the lease payments (Dr 1600 / Cr 2600). The scheduled job lease_periodic_run posts each period — interest unwinding on the liability (Dr 5900), the cash payment reducing the liability (Dr 2600 / Cr 1000), and straight-line ROU depreciation (Dr 5210 / Cr 1690) — the last period clearing the liability + ROU exactly. Idempotent per (lease, period).</t>
         </is>
       </c>
       <c r="H107" s="17" t="inlineStr">
@@ -10145,12 +10145,12 @@
       </c>
       <c r="I107" s="17" t="inlineStr">
         <is>
-          <t>Auto+Manual</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J107" s="17" t="inlineStr">
         <is>
-          <t>Monthly</t>
+          <t>Per period / per lease</t>
         </is>
       </c>
       <c r="K107" s="16" t="inlineStr">
@@ -10160,27 +10160,27 @@
       </c>
       <c r="L107" s="17" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="M107" s="16" t="inlineStr">
         <is>
-          <t>reconciliation.service.ts (importGlItems/autoMatch/certify)</t>
+          <t>leases.service.ts (createLease PV recognition, runDueLeases interest+payment+depreciation, modifyLease remeasurement); leases.controller.ts (gl_post); bi.service.ts (lease_periodic_run); schema/leases.ts (leases, rou_nbv) + migration 0120/0121; cutover/basics.ts (ToE)</t>
         </is>
       </c>
       <c r="N107" s="16" t="inlineStr">
         <is>
-          <t>Inspect recon + certify gate.</t>
+          <t>Inspect PV recognition + periodic interest/payment/depreciation + final-period clearing + modification remeasurement.</t>
         </is>
       </c>
       <c r="O107" s="16" t="inlineStr">
         <is>
-          <t>Sample periods: reconciled, unmatched cleared, certified.</t>
+          <t>Commencement recognises ROU=liability=PV; periodic run posts interest+principal(=payment)+ROU depreciation; liability + ROU reduce; a modification remeasures the liability at the revised PV and adjusts the ROU by the same delta (Dr/Cr 1600↔2600), then depreciates over the remaining term (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P107" s="16" t="inlineStr">
         <is>
-          <t>Certified recon</t>
+          <t>Lease register; periodic run log; modification remeasurement</t>
         </is>
       </c>
       <c r="Q107" s="18" t="inlineStr">
@@ -10192,7 +10192,7 @@
     <row r="108">
       <c r="A108" s="11" t="inlineStr">
         <is>
-          <t>REC-02</t>
+          <t>REC-01</t>
         </is>
       </c>
       <c r="B108" s="12" t="inlineStr">
@@ -10207,22 +10207,22 @@
       </c>
       <c r="D108" s="12" t="inlineStr">
         <is>
-          <t>Cash</t>
+          <t>All</t>
         </is>
       </c>
       <c r="E108" s="12" t="inlineStr">
         <is>
-          <t>Bank balance not reconciled to GL.</t>
+          <t>Subledgers diverge from GL undetected.</t>
         </is>
       </c>
       <c r="F108" s="12" t="inlineStr">
         <is>
-          <t>Existence/Completeness</t>
+          <t>Completeness/Accuracy</t>
         </is>
       </c>
       <c r="G108" s="12" t="inlineStr">
         <is>
-          <t>Bank reconciliation against statements.</t>
+          <t>Subledger-to-GL reconciliation per period: import GL, auto-match, certify (sign-off via 'approvals').</t>
         </is>
       </c>
       <c r="H108" s="13" t="inlineStr">
@@ -10252,22 +10252,22 @@
       </c>
       <c r="M108" s="12" t="inlineStr">
         <is>
-          <t>bank module; drizzle/0015_bank_reconciliation</t>
+          <t>reconciliation.service.ts (importGlItems/autoMatch/certify)</t>
         </is>
       </c>
       <c r="N108" s="12" t="inlineStr">
         <is>
-          <t>Inspect bank-rec process.</t>
+          <t>Inspect recon + certify gate.</t>
         </is>
       </c>
       <c r="O108" s="12" t="inlineStr">
         <is>
-          <t>Sample months reconciled &amp; reviewed.</t>
+          <t>Sample periods: reconciled, unmatched cleared, certified.</t>
         </is>
       </c>
       <c r="P108" s="12" t="inlineStr">
         <is>
-          <t>Bank rec</t>
+          <t>Certified recon</t>
         </is>
       </c>
       <c r="Q108" s="18" t="inlineStr">
@@ -10279,12 +10279,12 @@
     <row r="109">
       <c r="A109" s="15" t="inlineStr">
         <is>
-          <t>BANK-02</t>
+          <t>REC-02</t>
         </is>
       </c>
       <c r="B109" s="16" t="inlineStr">
         <is>
-          <t>Cash &amp; Treasury</t>
+          <t>Reconciliation</t>
         </is>
       </c>
       <c r="C109" s="17" t="inlineStr">
@@ -10294,37 +10294,37 @@
       </c>
       <c r="D109" s="16" t="inlineStr">
         <is>
-          <t>Cash; Operating expense; Interest income</t>
+          <t>Cash</t>
         </is>
       </c>
       <c r="E109" s="16" t="inlineStr">
         <is>
-          <t>A bank fee/interest adjustment is posted straight to the GL by one person during reconciliation — a cash outflow mis-booked as interest income, or a fictitious fee posted, with no independent review (single-person posting to the cash account).</t>
+          <t>Bank balance not reconciled to GL.</t>
         </is>
       </c>
       <c r="F109" s="16" t="inlineStr">
         <is>
-          <t>Authorization/Accuracy</t>
+          <t>Existence/Completeness</t>
         </is>
       </c>
       <c r="G109" s="16" t="inlineStr">
         <is>
-          <t>Bank adjustment maker-checker (SoD): a fee/interest adjustment on a statement line is a REQUEST that posts a DRAFT JE (no balance/GL effect; the line stays unreconciled) until a DIFFERENT user with approval authority approves (POST /api/bank/lines/:id/adjustment/approve). Self-approval → SOD_VIOLATION (binds even Admin); approval flips the line to reconciled and the JE to Posted; reject voids the Draft and frees the line. The Draft JE (source BANKADJ) is also surfaced, aged, by the pending-approvals monitor (GOV-01).</t>
+          <t>Bank reconciliation against statements.</t>
         </is>
       </c>
       <c r="H109" s="17" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I109" s="17" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="J109" s="17" t="inlineStr">
         <is>
-          <t>Per adjustment</t>
+          <t>Monthly</t>
         </is>
       </c>
       <c r="K109" s="16" t="inlineStr">
@@ -10334,27 +10334,27 @@
       </c>
       <c r="L109" s="17" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="M109" s="16" t="inlineStr">
         <is>
-          <t>bank.service.ts requestAdjustment/approveAdjustment/rejectAdjustment/listPendingAdjustments (reuses ledger.approveEntry SoD); bank.controller.ts (lines/:id/adjustment requests; adjustment/approve|reject gated approvals/gl_close); cutover/bankrec.ts (ToE)</t>
+          <t>bank module; drizzle/0015_bank_reconciliation</t>
         </is>
       </c>
       <c r="N109" s="16" t="inlineStr">
         <is>
-          <t>Inspect the request→approve flow + the approver≠requester check + that the Draft posts nothing until approval.</t>
+          <t>Inspect bank-rec process.</t>
         </is>
       </c>
       <c r="O109" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: request a fee adjustment (line unreconciled, GL difference unchanged), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm the difference closes to 0 only after approval (re-performed by the bankrec harness).</t>
+          <t>Sample months reconciled &amp; reviewed.</t>
         </is>
       </c>
       <c r="P109" s="16" t="inlineStr">
         <is>
-          <t>Bank adjustment queue + SoD test</t>
+          <t>Bank rec</t>
         </is>
       </c>
       <c r="Q109" s="18" t="inlineStr">
@@ -10366,12 +10366,12 @@
     <row r="110">
       <c r="A110" s="11" t="inlineStr">
         <is>
-          <t>REC-03</t>
+          <t>BANK-02</t>
         </is>
       </c>
       <c r="B110" s="12" t="inlineStr">
         <is>
-          <t>Reconciliation</t>
+          <t>Cash &amp; Treasury</t>
         </is>
       </c>
       <c r="C110" s="13" t="inlineStr">
@@ -10381,79 +10381,79 @@
       </c>
       <c r="D110" s="12" t="inlineStr">
         <is>
-          <t>Consolidation</t>
+          <t>Cash; Operating expense; Interest income</t>
         </is>
       </c>
       <c r="E110" s="12" t="inlineStr">
         <is>
-          <t>Intercompany balances not eliminated/agreed.</t>
+          <t>A bank fee/interest adjustment is posted straight to the GL by one person during reconciliation — a cash outflow mis-booked as interest income, or a fictitious fee posted, with no independent review (single-person posting to the cash account).</t>
         </is>
       </c>
       <c r="F110" s="12" t="inlineStr">
         <is>
-          <t>Accuracy</t>
+          <t>Authorization/Accuracy</t>
         </is>
       </c>
       <c r="G110" s="12" t="inlineStr">
         <is>
-          <t>Intercompany reconciliation &amp; elimination on consolidation.</t>
+          <t>Bank adjustment maker-checker (SoD): a fee/interest adjustment on a statement line is a REQUEST that posts a DRAFT JE (no balance/GL effect; the line stays unreconciled) until a DIFFERENT user with approval authority approves (POST /api/bank/lines/:id/adjustment/approve). Self-approval → SOD_VIOLATION (binds even Admin); approval flips the line to reconciled and the JE to Posted; reject voids the Draft and frees the line. The Draft JE (source BANKADJ) is also surfaced, aged, by the pending-approvals monitor (GOV-01).</t>
         </is>
       </c>
       <c r="H110" s="13" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I110" s="13" t="inlineStr">
         <is>
-          <t>Auto+Manual</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J110" s="13" t="inlineStr">
         <is>
-          <t>Period</t>
+          <t>Per adjustment</t>
         </is>
       </c>
       <c r="K110" s="12" t="inlineStr">
         <is>
-          <t>Group Controller</t>
+          <t>Controller</t>
         </is>
       </c>
       <c r="L110" s="13" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="M110" s="12" t="inlineStr">
         <is>
-          <t>intercompany; consolidation</t>
+          <t>bank.service.ts requestAdjustment/approveAdjustment/rejectAdjustment/listPendingAdjustments (reuses ledger.approveEntry SoD); bank.controller.ts (lines/:id/adjustment requests; adjustment/approve|reject gated approvals/gl_close); cutover/bankrec.ts (ToE)</t>
         </is>
       </c>
       <c r="N110" s="12" t="inlineStr">
         <is>
-          <t>Inspect IC matching + elimination.</t>
+          <t>Inspect the request→approve flow + the approver≠requester check + that the Draft posts nothing until approval.</t>
         </is>
       </c>
       <c r="O110" s="12" t="inlineStr">
         <is>
-          <t>Sample IC pairs agree &amp; eliminate.</t>
+          <t>Re-perform: request a fee adjustment (line unreconciled, GL difference unchanged), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm the difference closes to 0 only after approval (re-performed by the bankrec harness).</t>
         </is>
       </c>
       <c r="P110" s="12" t="inlineStr">
         <is>
-          <t>IC recon</t>
-        </is>
-      </c>
-      <c r="Q110" s="19" t="inlineStr">
-        <is>
-          <t>Partial</t>
+          <t>Bank adjustment queue + SoD test</t>
+        </is>
+      </c>
+      <c r="Q110" s="18" t="inlineStr">
+        <is>
+          <t>Implemented</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="15" t="inlineStr">
         <is>
-          <t>REC-04</t>
+          <t>REC-03</t>
         </is>
       </c>
       <c r="B111" s="16" t="inlineStr">
@@ -10468,22 +10468,22 @@
       </c>
       <c r="D111" s="16" t="inlineStr">
         <is>
-          <t>All control accounts</t>
+          <t>Consolidation</t>
         </is>
       </c>
       <c r="E111" s="16" t="inlineStr">
         <is>
-          <t>A sub-ledger silently drifts from its GL control account at period-end and no single review catches it (incomplete/inaccurate balances reach the financial statements).</t>
+          <t>Intercompany balances not eliminated/agreed.</t>
         </is>
       </c>
       <c r="F111" s="16" t="inlineStr">
         <is>
-          <t>Completeness/Accuracy</t>
+          <t>Accuracy</t>
         </is>
       </c>
       <c r="G111" s="16" t="inlineStr">
         <is>
-          <t>Period-end control-account reconciliation PACK: one read (GET /api/finance/reconciliation/controls) ties every major sub-ledger to its GL control account and FLAGS any out-of-balance — AR↔1100, AP↔2000, Inventory↔1200, Gift cards/Customer-deposits↔2200, Deferred revenue↔2400 — reporting per line {sub_ledger, gl_control, variance, reconciled} plus an overall all_reconciled flag and an exceptions count. Liability controls are sign-flipped before comparison. The controller's single 'are the books reconciled?' close view; an exception is a control finding to investigate before sign-off.</t>
+          <t>Intercompany reconciliation &amp; elimination on consolidation.</t>
         </is>
       </c>
       <c r="H111" s="17" t="inlineStr">
@@ -10493,17 +10493,17 @@
       </c>
       <c r="I111" s="17" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="J111" s="17" t="inlineStr">
         <is>
-          <t>Period / on demand</t>
+          <t>Period</t>
         </is>
       </c>
       <c r="K111" s="16" t="inlineStr">
         <is>
-          <t>Controller / CFO</t>
+          <t>Group Controller</t>
         </is>
       </c>
       <c r="L111" s="17" t="inlineStr">
@@ -10513,34 +10513,34 @@
       </c>
       <c r="M111" s="16" t="inlineStr">
         <is>
-          <t>finance.service.ts reconcileControls; finance.controller.ts GET reconciliation/controls (exec/ar/creditors); reuses ledger.trialBalance + the AR/AP/inventory/gift-card/deferred sub-ledgers; cutover/giftcards.ts + compliance.ts (ToE)</t>
+          <t>intercompany; consolidation</t>
         </is>
       </c>
       <c r="N111" s="16" t="inlineStr">
         <is>
-          <t>Inspect the pack: each control account's sub-ledger query + the GL tie + the exceptions roll-up.</t>
+          <t>Inspect IC matching + elimination.</t>
         </is>
       </c>
       <c r="O111" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: with a clean set, every line reconciled + all_reconciled=true; introduce a known sub-ledger/GL difference and confirm it surfaces as an exception (re-performed: gift-card 2200 + inventory 1200 ties asserted by the harnesses).</t>
+          <t>Sample IC pairs agree &amp; eliminate.</t>
         </is>
       </c>
       <c r="P111" s="16" t="inlineStr">
         <is>
-          <t>Reconciliation pack; exceptions list</t>
-        </is>
-      </c>
-      <c r="Q111" s="18" t="inlineStr">
-        <is>
-          <t>Implemented</t>
+          <t>IC recon</t>
+        </is>
+      </c>
+      <c r="Q111" s="19" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="11" t="inlineStr">
         <is>
-          <t>REC-05</t>
+          <t>REC-04</t>
         </is>
       </c>
       <c r="B112" s="12" t="inlineStr">
@@ -10555,42 +10555,42 @@
       </c>
       <c r="D112" s="12" t="inlineStr">
         <is>
-          <t>Cash; Bank</t>
+          <t>All control accounts</t>
         </is>
       </c>
       <c r="E112" s="12" t="inlineStr">
         <is>
-          <t>Till cash dropped to the safe never reaches the bank, or a deposit isn't matched to the statement — cash sits unbanked (theft/loss exposure) or the bank balance can't be tied to the books.</t>
+          <t>A sub-ledger silently drifts from its GL control account at period-end and no single review catches it (incomplete/inaccurate balances reach the financial statements).</t>
         </is>
       </c>
       <c r="F112" s="12" t="inlineStr">
         <is>
-          <t>Completeness/Existence/Authorization</t>
+          <t>Completeness/Accuracy</t>
         </is>
       </c>
       <c r="G112" s="12" t="inlineStr">
         <is>
-          <t>Cash banking — safe-drop → bank deposit → reconciliation: till 'drop's move cash from the drawer to the safe (drawer-only, no GL). Banking BATCHES the undeposited drops into a deposit and posts the GL (Dr &lt;bank account, e.g. 1010&gt; / Cr 1000 Cash), stamping each drop with the deposit id; the deposit is then RECONCILED to the bank statement (status Deposited→Reconciled). A detective read (GET /api/bank/deposits/undeposited-drops) surfaces the CASH STILL IN THE SAFE (drops with deposit_id NULL) — the unbanked exposure to chase. SoD: banking is a treasury duty (exec/ar) — segregated from the cashier (pos_till) who drops the cash, so the person who removes cash from the drawer is not the one who banks it.</t>
+          <t>Period-end control-account reconciliation PACK: one read (GET /api/finance/reconciliation/controls) ties every major sub-ledger to its GL control account and FLAGS any out-of-balance — AR↔1100, AP↔2000, Inventory↔1200, Gift cards/Customer-deposits↔2200, Deferred revenue↔2400 — reporting per line {sub_ledger, gl_control, variance, reconciled} plus an overall all_reconciled flag and an exceptions count. Liability controls are sign-flipped before comparison. The controller's single 'are the books reconciled?' close view; an exception is a control finding to investigate before sign-off.</t>
         </is>
       </c>
       <c r="H112" s="13" t="inlineStr">
         <is>
-          <t>Det/Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I112" s="13" t="inlineStr">
         <is>
-          <t>Auto+Manual</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J112" s="13" t="inlineStr">
         <is>
-          <t>Per banking run</t>
+          <t>Period / on demand</t>
         </is>
       </c>
       <c r="K112" s="12" t="inlineStr">
         <is>
-          <t>FinancialController / Treasury</t>
+          <t>Controller / CFO</t>
         </is>
       </c>
       <c r="L112" s="13" t="inlineStr">
@@ -10600,22 +10600,22 @@
       </c>
       <c r="M112" s="12" t="inlineStr">
         <is>
-          <t>bank.service.ts undepositedDrops/createDeposit (Dr bank/Cr 1000, stamps deposit_id)/reconcileDeposit/listDeposits; bank.controller.ts (deposits, deposits/undeposited-drops, deposits/:id/reconcile; exec/ar); schema/cash.ts bank_deposits + cash_movements.deposit_id + migration 0152; /cash-banking UI; cutover/cash-banking.ts (ToE)</t>
+          <t>finance.service.ts reconcileControls; finance.controller.ts GET reconciliation/controls (exec/ar/creditors); reuses ledger.trialBalance + the AR/AP/inventory/gift-card/deferred sub-ledgers; cutover/giftcards.ts + compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N112" s="12" t="inlineStr">
         <is>
-          <t>Inspect the undeposited-drop exposure read + the deposit GL (bank↔1000) + the reconcile step + the SoD (cashier vs treasury).</t>
+          <t>Inspect the pack: each control account's sub-ledger query + the GL tie + the exceptions roll-up.</t>
         </is>
       </c>
       <c r="O112" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: two till drops → cash-in-safe shows the total; a cashier (pos_till) cannot bank (403); treasury banks → Dr bank / Cr 1000, cash-in-safe back to 0; reconcile the deposit; trial balance balanced (re-performed by the cash-banking harness).</t>
+          <t>Re-perform: with a clean set, every line reconciled + all_reconciled=true; introduce a known sub-ledger/GL difference and confirm it surfaces as an exception (re-performed: gift-card 2200 + inventory 1200 ties asserted by the harnesses).</t>
         </is>
       </c>
       <c r="P112" s="12" t="inlineStr">
         <is>
-          <t>Bank-deposit register; undeposited-drop (cash-in-safe) exposure</t>
+          <t>Reconciliation pack; exceptions list</t>
         </is>
       </c>
       <c r="Q112" s="18" t="inlineStr">
@@ -10627,12 +10627,12 @@
     <row r="113">
       <c r="A113" s="15" t="inlineStr">
         <is>
-          <t>GOV-01</t>
+          <t>REC-05</t>
         </is>
       </c>
       <c r="B113" s="16" t="inlineStr">
         <is>
-          <t>Monitoring</t>
+          <t>Reconciliation</t>
         </is>
       </c>
       <c r="C113" s="17" t="inlineStr">
@@ -10642,42 +10642,42 @@
       </c>
       <c r="D113" s="16" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Cash; Bank</t>
         </is>
       </c>
       <c r="E113" s="16" t="inlineStr">
         <is>
-          <t>A maker-checker approval sits un-actioned and is forgotten — a transaction stalls before it is effective, or (worse) a control is quietly bypassed and no one notices an item never got its independent review.</t>
+          <t>Till cash dropped to the safe never reaches the bank, or a deposit isn't matched to the statement — cash sits unbanked (theft/loss exposure) or the bank balance can't be tied to the books.</t>
         </is>
       </c>
       <c r="F113" s="16" t="inlineStr">
         <is>
-          <t>Authorization/Completeness</t>
+          <t>Completeness/Existence/Authorization</t>
         </is>
       </c>
       <c r="G113" s="16" t="inlineStr">
         <is>
-          <t>Pending-approvals MONITOR (COSO monitoring): a single worklist of EVERY item awaiting independent approval across the system, each with its AGE in days and an overdue roll-up — spanning the manual-JE (GL-05), bank-adjustment (BANK-02), AP-disbursement (EXP-06), payroll (PAY-03), asset-revaluation (FA-08), asset-disposal (FA-09), inventory-write-off (INV-07), till-close cash over/short (REV-13), FX-rate (FX-04), budget (BUD-01) and large-refund (REV-16) maker-checkers. The controller reviews it before close; a stale item (age beyond the threshold) is a control finding to chase or escalate. The /approvals screen also lets a manager approve/reject a material till variance or a large refund inline (the pending types with no dedicated module screen). Read-only worklist; tenant-scoped via the caller's RLS.</t>
+          <t>Cash banking — safe-drop → bank deposit → reconciliation: till 'drop's move cash from the drawer to the safe (drawer-only, no GL). Banking BATCHES the undeposited drops into a deposit and posts the GL (Dr &lt;bank account, e.g. 1010&gt; / Cr 1000 Cash), stamping each drop with the deposit id; the deposit is then RECONCILED to the bank statement (status Deposited→Reconciled). A detective read (GET /api/bank/deposits/undeposited-drops) surfaces the CASH STILL IN THE SAFE (drops with deposit_id NULL) — the unbanked exposure to chase. SoD: banking is a treasury duty (exec/ar) — segregated from the cashier (pos_till) who drops the cash, so the person who removes cash from the drawer is not the one who banks it.</t>
         </is>
       </c>
       <c r="H113" s="17" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Det/Prev</t>
         </is>
       </c>
       <c r="I113" s="17" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="J113" s="17" t="inlineStr">
         <is>
-          <t>Continuous / pre-close</t>
+          <t>Per banking run</t>
         </is>
       </c>
       <c r="K113" s="16" t="inlineStr">
         <is>
-          <t>Controller / CFO</t>
+          <t>FinancialController / Treasury</t>
         </is>
       </c>
       <c r="L113" s="17" t="inlineStr">
@@ -10687,22 +10687,22 @@
       </c>
       <c r="M113" s="16" t="inlineStr">
         <is>
-          <t>finance.service.ts pendingApprovals; finance.controller.ts GET approvals/pending (exec/approvals/creditors); aggregates journalEntries(Draft incl. BANKADJ→BANK-02)/apPayments/payruns/asset_revaluations/fixed_assets(disposal_pending)/inv_writeoff_requests/till_sessions(PendingApproval)/fx_rates(PendingApproval)/budgets(PendingApproval); cutover/compliance.ts (ToE)</t>
+          <t>bank.service.ts undepositedDrops/createDeposit (Dr bank/Cr 1000, stamps deposit_id)/reconcileDeposit/listDeposits; bank.controller.ts (deposits, deposits/undeposited-drops, deposits/:id/reconcile; exec/ar); schema/cash.ts bank_deposits + cash_movements.deposit_id + migration 0152; /cash-banking UI; cutover/cash-banking.ts (ToE)</t>
         </is>
       </c>
       <c r="N113" s="16" t="inlineStr">
         <is>
-          <t>Inspect the aggregation across all pending sources + the age/overdue roll-up.</t>
+          <t>Inspect the undeposited-drop exposure read + the deposit GL (bank↔1000) + the reconcile step + the SoD (cashier vs treasury).</t>
         </is>
       </c>
       <c r="O113" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: create a pending item (e.g. a Draft JE) and confirm it appears in the worklist with its control ID, amount and age; the overdue count flags items past the threshold (re-performed by the harness).</t>
+          <t>Re-perform: two till drops → cash-in-safe shows the total; a cashier (pos_till) cannot bank (403); treasury banks → Dr bank / Cr 1000, cash-in-safe back to 0; reconcile the deposit; trial balance balanced (re-performed by the cash-banking harness).</t>
         </is>
       </c>
       <c r="P113" s="16" t="inlineStr">
         <is>
-          <t>Pending-approvals worklist</t>
+          <t>Bank-deposit register; undeposited-drop (cash-in-safe) exposure</t>
         </is>
       </c>
       <c r="Q113" s="18" t="inlineStr">
@@ -10714,12 +10714,12 @@
     <row r="114">
       <c r="A114" s="11" t="inlineStr">
         <is>
-          <t>TAX-01</t>
+          <t>GOV-01</t>
         </is>
       </c>
       <c r="B114" s="12" t="inlineStr">
         <is>
-          <t>Tax</t>
+          <t>Monitoring</t>
         </is>
       </c>
       <c r="C114" s="13" t="inlineStr">
@@ -10729,27 +10729,27 @@
       </c>
       <c r="D114" s="12" t="inlineStr">
         <is>
-          <t>Tax (VAT)</t>
+          <t>All</t>
         </is>
       </c>
       <c r="E114" s="12" t="inlineStr">
         <is>
-          <t>VAT computed incorrectly → filing/penalty risk.</t>
+          <t>A maker-checker approval sits un-actioned and is forgotten — a transaction stalls before it is effective, or (worse) a control is quietly bypassed and no one notices an item never got its independent review.</t>
         </is>
       </c>
       <c r="F114" s="12" t="inlineStr">
         <is>
-          <t>Accuracy</t>
+          <t>Authorization/Completeness</t>
         </is>
       </c>
       <c r="G114" s="12" t="inlineStr">
         <is>
-          <t>VAT via pluggable provider (TH 7%); unit-tested; no hard-coded rate.</t>
+          <t>Pending-approvals MONITOR (COSO monitoring): a single worklist of EVERY item awaiting independent approval across the system, each with its AGE in days and an overdue roll-up — spanning the manual-JE (GL-05), bank-adjustment (BANK-02), AP-disbursement (EXP-06), payroll (PAY-03), asset-revaluation (FA-08), asset-disposal (FA-09), inventory-write-off (INV-07), till-close cash over/short (REV-13), FX-rate (FX-04), budget (BUD-01) and large-refund (REV-16) maker-checkers. The controller reviews it before close; a stale item (age beyond the threshold) is a control finding to chase or escalate. The /approvals screen also lets a manager approve/reject a material till variance or a large refund inline (the pending types with no dedicated module screen). Read-only worklist; tenant-scoped via the caller's RLS.</t>
         </is>
       </c>
       <c r="H114" s="13" t="inlineStr">
         <is>
-          <t>Auto</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I114" s="13" t="inlineStr">
@@ -10759,37 +10759,37 @@
       </c>
       <c r="J114" s="13" t="inlineStr">
         <is>
-          <t>Per txn</t>
+          <t>Continuous / pre-close</t>
         </is>
       </c>
       <c r="K114" s="12" t="inlineStr">
         <is>
-          <t>Tax / Controller</t>
+          <t>Controller / CFO</t>
         </is>
       </c>
       <c r="L114" s="13" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="M114" s="12" t="inlineStr">
         <is>
-          <t>tax/tax-providers.ts; tax.service.ts; test/unit.test.ts</t>
+          <t>finance.service.ts pendingApprovals; finance.controller.ts GET approvals/pending (exec/approvals/creditors); aggregates journalEntries(Draft incl. BANKADJ→BANK-02)/apPayments/payruns/asset_revaluations/fixed_assets(disposal_pending)/inv_writeoff_requests/till_sessions(PendingApproval)/fx_rates(PendingApproval)/budgets(PendingApproval); cutover/compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N114" s="12" t="inlineStr">
         <is>
-          <t>Inspect rate provider + tests.</t>
+          <t>Inspect the aggregation across all pending sources + the age/overdue roll-up.</t>
         </is>
       </c>
       <c r="O114" s="12" t="inlineStr">
         <is>
-          <t>Re-perform VAT on sample; tie to return.</t>
+          <t>Re-perform: create a pending item (e.g. a Draft JE) and confirm it appears in the worklist with its control ID, amount and age; the overdue count flags items past the threshold (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P114" s="12" t="inlineStr">
         <is>
-          <t>VAT tests</t>
+          <t>Pending-approvals worklist</t>
         </is>
       </c>
       <c r="Q114" s="18" t="inlineStr">
@@ -10801,7 +10801,7 @@
     <row r="115">
       <c r="A115" s="15" t="inlineStr">
         <is>
-          <t>TAX-02</t>
+          <t>TAX-01</t>
         </is>
       </c>
       <c r="B115" s="16" t="inlineStr">
@@ -10816,22 +10816,22 @@
       </c>
       <c r="D115" s="16" t="inlineStr">
         <is>
-          <t>Tax; Revenue</t>
+          <t>Tax (VAT)</t>
         </is>
       </c>
       <c r="E115" s="16" t="inlineStr">
         <is>
-          <t>Non-compliant e-Tax invoice / not transmitted to ETDA.</t>
+          <t>VAT computed incorrectly → filing/penalty risk.</t>
         </is>
       </c>
       <c r="F115" s="16" t="inlineStr">
         <is>
-          <t>Accuracy/Compliance</t>
+          <t>Accuracy</t>
         </is>
       </c>
       <c r="G115" s="16" t="inlineStr">
         <is>
-          <t>e-Tax invoice (ETDA UBL 2.1 XML) generation + email with CC to ETDA timestamp mailbox.</t>
+          <t>VAT via pluggable provider (TH 7%); unit-tested; no hard-coded rate.</t>
         </is>
       </c>
       <c r="H115" s="17" t="inlineStr">
@@ -10846,37 +10846,37 @@
       </c>
       <c r="J115" s="17" t="inlineStr">
         <is>
-          <t>Per invoice</t>
+          <t>Per txn</t>
         </is>
       </c>
       <c r="K115" s="16" t="inlineStr">
         <is>
-          <t>Tax</t>
+          <t>Tax / Controller</t>
         </is>
       </c>
       <c r="L115" s="17" t="inlineStr">
         <is>
-          <t>P10/P13</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="M115" s="16" t="inlineStr">
         <is>
-          <t>tax-docs/etax-xml.ts; etax-email.service.ts (tested)</t>
+          <t>tax/tax-providers.ts; tax.service.ts; test/unit.test.ts</t>
         </is>
       </c>
       <c r="N115" s="16" t="inlineStr">
         <is>
-          <t>Inspect XML schema + email composer.</t>
+          <t>Inspect rate provider + tests.</t>
         </is>
       </c>
       <c r="O115" s="16" t="inlineStr">
         <is>
-          <t>Sample invoices: valid XML, correct CC/escaping.</t>
+          <t>Re-perform VAT on sample; tie to return.</t>
         </is>
       </c>
       <c r="P115" s="16" t="inlineStr">
         <is>
-          <t>e-Tax samples</t>
+          <t>VAT tests</t>
         </is>
       </c>
       <c r="Q115" s="18" t="inlineStr">
@@ -10888,7 +10888,7 @@
     <row r="116">
       <c r="A116" s="11" t="inlineStr">
         <is>
-          <t>TAX-03</t>
+          <t>TAX-02</t>
         </is>
       </c>
       <c r="B116" s="12" t="inlineStr">
@@ -10903,22 +10903,22 @@
       </c>
       <c r="D116" s="12" t="inlineStr">
         <is>
-          <t>Tax (WHT)</t>
+          <t>Tax; Revenue</t>
         </is>
       </c>
       <c r="E116" s="12" t="inlineStr">
         <is>
-          <t>Withholding tax mis-computed / not reported.</t>
+          <t>Non-compliant e-Tax invoice / not transmitted to ETDA.</t>
         </is>
       </c>
       <c r="F116" s="12" t="inlineStr">
         <is>
-          <t>Accuracy</t>
+          <t>Accuracy/Compliance</t>
         </is>
       </c>
       <c r="G116" s="12" t="inlineStr">
         <is>
-          <t>WHT computation and ภ.ง.ด. reporting.</t>
+          <t>e-Tax invoice (ETDA UBL 2.1 XML) generation + email with CC to ETDA timestamp mailbox.</t>
         </is>
       </c>
       <c r="H116" s="13" t="inlineStr">
@@ -10933,7 +10933,7 @@
       </c>
       <c r="J116" s="13" t="inlineStr">
         <is>
-          <t>Per txn / monthly</t>
+          <t>Per invoice</t>
         </is>
       </c>
       <c r="K116" s="12" t="inlineStr">
@@ -10943,39 +10943,39 @@
       </c>
       <c r="L116" s="13" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P10/P13</t>
         </is>
       </c>
       <c r="M116" s="12" t="inlineStr">
         <is>
-          <t>tax-reports; payroll</t>
+          <t>tax-docs/etax-xml.ts; etax-email.service.ts (tested)</t>
         </is>
       </c>
       <c r="N116" s="12" t="inlineStr">
         <is>
-          <t>Inspect WHT logic + report.</t>
+          <t>Inspect XML schema + email composer.</t>
         </is>
       </c>
       <c r="O116" s="12" t="inlineStr">
         <is>
-          <t>Re-perform WHT on sample; tie to filing.</t>
+          <t>Sample invoices: valid XML, correct CC/escaping.</t>
         </is>
       </c>
       <c r="P116" s="12" t="inlineStr">
         <is>
-          <t>WHT report</t>
-        </is>
-      </c>
-      <c r="Q116" s="19" t="inlineStr">
-        <is>
-          <t>Partial</t>
+          <t>e-Tax samples</t>
+        </is>
+      </c>
+      <c r="Q116" s="18" t="inlineStr">
+        <is>
+          <t>Implemented</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="15" t="inlineStr">
         <is>
-          <t>TAX-04</t>
+          <t>TAX-03</t>
         </is>
       </c>
       <c r="B117" s="16" t="inlineStr">
@@ -10990,27 +10990,27 @@
       </c>
       <c r="D117" s="16" t="inlineStr">
         <is>
-          <t>Tax (VAT); Tax Payable (2100)</t>
+          <t>Tax (WHT)</t>
         </is>
       </c>
       <c r="E117" s="16" t="inlineStr">
         <is>
-          <t>Output/input VAT on the filed ภ.พ.30 return does not agree to the GL — VAT liability mis-stated, a filing/penalty exposure, or a posting omission goes undetected before submission.</t>
+          <t>Withholding tax mis-computed / not reported.</t>
         </is>
       </c>
       <c r="F117" s="16" t="inlineStr">
         <is>
-          <t>Completeness/Accuracy</t>
+          <t>Accuracy</t>
         </is>
       </c>
       <c r="G117" s="16" t="inlineStr">
         <is>
-          <t>Periodic VAT-return ↔ GL reconciliation (ภ.พ.30): the monthly return (GET /api/tax-reports/pp30) is built from the sales/output-VAT and purchase/input-VAT sub-reports, computes net VAT = output − input, and RECONCILES it to the **GL account 2100 (Tax Payable) net movement** for the same period (Σ credit − Σ debit over Posted entries) — returning `reconciliation.tied` = true only when the two agree within rounding. A non-tie is a detective finding to investigate and clear BEFORE filing (the form also carries the ม.157 deadline = the 15th of the next month). Output VAT is posted to 2100 on every sale (Cr) and reversed on returns (Dr); input VAT is posted on AP bills (Dr) — so 2100's net is the period's VAT payable. Read-only report; exportable to a ภ.พ.30 PDF/HTML.</t>
+          <t>WHT computation and ภ.ง.ด. reporting.</t>
         </is>
       </c>
       <c r="H117" s="17" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Auto</t>
         </is>
       </c>
       <c r="I117" s="17" t="inlineStr">
@@ -11020,49 +11020,49 @@
       </c>
       <c r="J117" s="17" t="inlineStr">
         <is>
-          <t>Monthly / pre-filing</t>
+          <t>Per txn / monthly</t>
         </is>
       </c>
       <c r="K117" s="16" t="inlineStr">
         <is>
-          <t>Tax / FinancialController</t>
+          <t>Tax</t>
         </is>
       </c>
       <c r="L117" s="17" t="inlineStr">
         <is>
-          <t>P10/P16</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="M117" s="16" t="inlineStr">
         <is>
-          <t>tax-reports.service.ts pp30 (outputVat/inputVat + 2100 net-movement tie); tax-reports.controller.ts (GET pp30, pp30/export, exec); tax-reports-pdf.ts; dine-in.service.ts/returns.service.ts/finance.service.ts post 2100 on sale/return/AP; /tax/reports UI; cutover/taxdocs.ts (ToE)</t>
+          <t>tax-reports; payroll</t>
         </is>
       </c>
       <c r="N117" s="16" t="inlineStr">
         <is>
-          <t>Inspect the pp30 build + the 2100 net-movement query + the tie flag + the filing deadline.</t>
+          <t>Inspect WHT logic + report.</t>
         </is>
       </c>
       <c r="O117" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: the pp30 return computes net VAT (output − input), the GL 2100 net movement reflects the posted input VAT, and the reconciliation block exposes the gl_account (2100), the report net VAT and a boolean tie verdict (tied iff the two agree within rounding); the ภ.พ.30 export renders (re-performed by the taxdocs harness).</t>
+          <t>Re-perform WHT on sample; tie to filing.</t>
         </is>
       </c>
       <c r="P117" s="16" t="inlineStr">
         <is>
-          <t>ภ.พ.30 return + GL-2100 reconciliation tie</t>
-        </is>
-      </c>
-      <c r="Q117" s="18" t="inlineStr">
-        <is>
-          <t>Implemented</t>
+          <t>WHT report</t>
+        </is>
+      </c>
+      <c r="Q117" s="19" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="11" t="inlineStr">
         <is>
-          <t>TAX-05</t>
+          <t>TAX-04</t>
         </is>
       </c>
       <c r="B118" s="12" t="inlineStr">
@@ -11077,37 +11077,37 @@
       </c>
       <c r="D118" s="12" t="inlineStr">
         <is>
-          <t>Tax (VAT/WHT)</t>
+          <t>Tax (VAT); Tax Payable (2100)</t>
         </is>
       </c>
       <c r="E118" s="12" t="inlineStr">
         <is>
-          <t>A return is computed but there is no evidence it was actually FILED — no record of the figures as filed, the submission date or the Revenue-Department reference — so a missed or late filing (penalty/surcharge exposure) is not detected, and a filed return can be silently recomputed/altered after submission.</t>
+          <t>Output/input VAT on the filed ภ.พ.30 return does not agree to the GL — VAT liability mis-stated, a filing/penalty exposure, or a posting omission goes undetected before submission.</t>
         </is>
       </c>
       <c r="F118" s="12" t="inlineStr">
         <is>
-          <t>Completeness/Accuracy/Cutoff</t>
+          <t>Completeness/Accuracy</t>
         </is>
       </c>
       <c r="G118" s="12" t="inlineStr">
         <is>
-          <t>Thai tax filing register + remittance calendar: a computed ภ.พ.30 (PP30) or ภ.ง.ด.3/53 (PND) return is SNAPSHOTTED into a thai_tax_filings record (one per tenant/type/period) carrying the figures as filed (output/input/net VAT, tax withheld) and a DRAFT→SUBMITTED→ACCEPTED lifecycle. Filing is idempotent per period; submitting REQUIRES a Revenue-Department submission reference (SUBMISSION_REF_REQUIRED) and stamps SUBMITTED + the timestamp; an already-filed (SUBMITTED/ACCEPTED) period is NOT silently overwritten when re-filed (returned as-is, already_filed=true). A remittance calendar (GET /api/tax-reports/remittance-calendar) lists every monthly obligation (ภ.พ.30 by the 15th, ภ.ง.ด. by the 7th of the following month) with its current status (NOT_FILED/DRAFT/SUBMITTED/ACCEPTED), so the controller sees what is due/filed/late before the deadline. Tenant-scoped (RLS); gated exec.</t>
+          <t>Periodic VAT-return ↔ GL reconciliation (ภ.พ.30): the monthly return (GET /api/tax-reports/pp30) is built from the sales/output-VAT and purchase/input-VAT sub-reports, computes net VAT = output − input, and RECONCILES it to the **GL account 2100 (Tax Payable) net movement** for the same period (Σ credit − Σ debit over Posted entries) — returning `reconciliation.tied` = true only when the two agree within rounding. A non-tie is a detective finding to investigate and clear BEFORE filing (the form also carries the ม.157 deadline = the 15th of the next month). Output VAT is posted to 2100 on every sale (Cr) and reversed on returns (Dr); input VAT is posted on AP bills (Dr) — so 2100's net is the period's VAT payable. Read-only report; exportable to a ภ.พ.30 PDF/HTML.</t>
         </is>
       </c>
       <c r="H118" s="13" t="inlineStr">
         <is>
-          <t>Det/Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I118" s="13" t="inlineStr">
         <is>
-          <t>Auto+Manual</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J118" s="13" t="inlineStr">
         <is>
-          <t>Monthly / per filing</t>
+          <t>Monthly / pre-filing</t>
         </is>
       </c>
       <c r="K118" s="12" t="inlineStr">
@@ -11122,22 +11122,22 @@
       </c>
       <c r="M118" s="12" t="inlineStr">
         <is>
-          <t>tax-reports.service.ts fileReturn (snapshots pp30/pnd into a DRAFT, idempotent per period; no overwrite of a filed return) / submitFiling (SUBMISSION_REF_REQUIRED → SUBMITTED) / acceptFiling / listFilings / remittanceCalendar; tax-reports.controller.ts (POST filings[/:id/submit|accept], GET filings, remittance-calendar, exec); schema/tax-docs.ts thai_tax_filings + migration 0165; /tax/reports filings &amp; calendar tab; cutover/taxdocs.ts (ToE)</t>
+          <t>tax-reports.service.ts pp30 (outputVat/inputVat + 2100 net-movement tie); tax-reports.controller.ts (GET pp30, pp30/export, exec); tax-reports-pdf.ts; dine-in.service.ts/returns.service.ts/finance.service.ts post 2100 on sale/return/AP; /tax/reports UI; cutover/taxdocs.ts (ToE)</t>
         </is>
       </c>
       <c r="N118" s="12" t="inlineStr">
         <is>
-          <t>Inspect the filing snapshot + the DRAFT→SUBMITTED→ACCEPTED lifecycle + the mandatory submission reference + the no-overwrite-of-a-filed-return rule + the deadline calendar.</t>
+          <t>Inspect the pp30 build + the 2100 net-movement query + the tie flag + the filing deadline.</t>
         </is>
       </c>
       <c r="O118" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: file PP30 → DRAFT with the period figures; re-file refreshes the same DRAFT (idempotent); submit without a reference → 400; submit with a reference → SUBMITTED + timestamp; accept → ACCEPTED; re-filing an accepted period returns it (already_filed); the remittance calendar shows the period ACCEPTED with the 15th-of-next-month deadline (re-performed by the taxdocs harness).</t>
+          <t>Re-perform: the pp30 return computes net VAT (output − input), the GL 2100 net movement reflects the posted input VAT, and the reconciliation block exposes the gl_account (2100), the report net VAT and a boolean tie verdict (tied iff the two agree within rounding); the ภ.พ.30 export renders (re-performed by the taxdocs harness).</t>
         </is>
       </c>
       <c r="P118" s="12" t="inlineStr">
         <is>
-          <t>thai_tax_filings register + remittance calendar</t>
+          <t>ภ.พ.30 return + GL-2100 reconciliation tie</t>
         </is>
       </c>
       <c r="Q118" s="18" t="inlineStr">
@@ -11149,12 +11149,12 @@
     <row r="119">
       <c r="A119" s="15" t="inlineStr">
         <is>
-          <t>PAY-01</t>
+          <t>TAX-05</t>
         </is>
       </c>
       <c r="B119" s="16" t="inlineStr">
         <is>
-          <t>Payroll</t>
+          <t>Tax</t>
         </is>
       </c>
       <c r="C119" s="17" t="inlineStr">
@@ -11164,67 +11164,67 @@
       </c>
       <c r="D119" s="16" t="inlineStr">
         <is>
-          <t>Payroll expense/liability</t>
+          <t>Tax (VAT/WHT)</t>
         </is>
       </c>
       <c r="E119" s="16" t="inlineStr">
         <is>
-          <t>Payroll, SSO and PIT mis-computed.</t>
+          <t>A return is computed but there is no evidence it was actually FILED — no record of the figures as filed, the submission date or the Revenue-Department reference — so a missed or late filing (penalty/surcharge exposure) is not detected, and a filed return can be silently recomputed/altered after submission.</t>
         </is>
       </c>
       <c r="F119" s="16" t="inlineStr">
         <is>
-          <t>Accuracy</t>
+          <t>Completeness/Accuracy/Cutoff</t>
         </is>
       </c>
       <c r="G119" s="16" t="inlineStr">
         <is>
-          <t>Payroll engine — SSO 5% (cap 750), progressive PIT, payslip net; unit-tested.</t>
+          <t>Thai tax filing register + remittance calendar: a computed ภ.พ.30 (PP30) or ภ.ง.ด.3/53 (PND) return is SNAPSHOTTED into a thai_tax_filings record (one per tenant/type/period) carrying the figures as filed (output/input/net VAT, tax withheld) and a DRAFT→SUBMITTED→ACCEPTED lifecycle. Filing is idempotent per period; submitting REQUIRES a Revenue-Department submission reference (SUBMISSION_REF_REQUIRED) and stamps SUBMITTED + the timestamp; an already-filed (SUBMITTED/ACCEPTED) period is NOT silently overwritten when re-filed (returned as-is, already_filed=true). A remittance calendar (GET /api/tax-reports/remittance-calendar) lists every monthly obligation (ภ.พ.30 by the 15th, ภ.ง.ด. by the 7th of the following month) with its current status (NOT_FILED/DRAFT/SUBMITTED/ACCEPTED), so the controller sees what is due/filed/late before the deadline. Tenant-scoped (RLS); gated exec.</t>
         </is>
       </c>
       <c r="H119" s="17" t="inlineStr">
         <is>
-          <t>Auto</t>
+          <t>Det/Prev</t>
         </is>
       </c>
       <c r="I119" s="17" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="J119" s="17" t="inlineStr">
         <is>
-          <t>Per run</t>
+          <t>Monthly / per filing</t>
         </is>
       </c>
       <c r="K119" s="16" t="inlineStr">
         <is>
-          <t>HR / Payroll</t>
+          <t>Tax / FinancialController</t>
         </is>
       </c>
       <c r="L119" s="17" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P10/P16</t>
         </is>
       </c>
       <c r="M119" s="16" t="inlineStr">
         <is>
-          <t>payroll/payroll-calc.ts; test/unit.test.ts</t>
+          <t>tax-reports.service.ts fileReturn (snapshots pp30/pnd into a DRAFT, idempotent per period; no overwrite of a filed return) / submitFiling (SUBMISSION_REF_REQUIRED → SUBMITTED) / acceptFiling / listFilings / remittanceCalendar; tax-reports.controller.ts (POST filings[/:id/submit|accept], GET filings, remittance-calendar, exec); schema/tax-docs.ts thai_tax_filings + migration 0165; /tax/reports filings &amp; calendar tab; cutover/taxdocs.ts (ToE)</t>
         </is>
       </c>
       <c r="N119" s="16" t="inlineStr">
         <is>
-          <t>Inspect calc + tests.</t>
+          <t>Inspect the filing snapshot + the DRAFT→SUBMITTED→ACCEPTED lifecycle + the mandatory submission reference + the no-overwrite-of-a-filed-return rule + the deadline calendar.</t>
         </is>
       </c>
       <c r="O119" s="16" t="inlineStr">
         <is>
-          <t>Re-perform sample payslips.</t>
+          <t>Re-perform: file PP30 → DRAFT with the period figures; re-file refreshes the same DRAFT (idempotent); submit without a reference → 400; submit with a reference → SUBMITTED + timestamp; accept → ACCEPTED; re-filing an accepted period returns it (already_filed); the remittance calendar shows the period ACCEPTED with the 15th-of-next-month deadline (re-performed by the taxdocs harness).</t>
         </is>
       </c>
       <c r="P119" s="16" t="inlineStr">
         <is>
-          <t>Payslip tests</t>
+          <t>thai_tax_filings register + remittance calendar</t>
         </is>
       </c>
       <c r="Q119" s="18" t="inlineStr">
@@ -11236,12 +11236,12 @@
     <row r="120">
       <c r="A120" s="11" t="inlineStr">
         <is>
-          <t>PAY-02</t>
+          <t>TAX-06</t>
         </is>
       </c>
       <c r="B120" s="12" t="inlineStr">
         <is>
-          <t>Payroll</t>
+          <t>Tax</t>
         </is>
       </c>
       <c r="C120" s="13" t="inlineStr">
@@ -11251,27 +11251,27 @@
       </c>
       <c r="D120" s="12" t="inlineStr">
         <is>
-          <t>Payroll liability</t>
+          <t>Deferred Tax Asset (1700); Deferred Tax Liability (2700); Deferred Tax Expense (5950)</t>
         </is>
       </c>
       <c r="E120" s="12" t="inlineStr">
         <is>
-          <t>Statutory withholdings (SSO/WHT/PF) mis-stated or not remitted, so the liability owed to the authorities diverges from the books.</t>
+          <t>Book-vs-tax TEMPORARY differences (the AR allowance, accelerated depreciation, accruals) are not recognised as deferred tax, or the deferred-tax entry is computed and posted by one person with no review — income tax expense and the deferred tax asset/liability are mis-stated (TAS 12 / TFRS).</t>
         </is>
       </c>
       <c r="F120" s="12" t="inlineStr">
         <is>
-          <t>Accuracy/Compliance</t>
+          <t>Accuracy/Valuation/Completeness/Authorization/Segregation of Duties</t>
         </is>
       </c>
       <c r="G120" s="12" t="inlineStr">
         <is>
-          <t>Payroll-liability schedule (GET /api/payroll/liabilities): each statutory account — SSO 2350, WHT/PND1 2360, PF 2370 — shows accrued (GL credits) − remitted (GL debits) = outstanding, tied back to the INDEPENDENT payrun accrual with a `reconciled` flag (a divergence flags a manual JE that touched a payroll-liability account outside the payroll process). Treasury remits the cash (POST .../remit → Dr liability / Cr 1000) which clears the outstanding and keeps the books reconciled to the statutory filings; a remittance beyond the outstanding is blocked (REMIT_EXCEEDS_OUTSTANDING).</t>
+          <t>Deferred tax (TAS 12, maker-checker, idempotent per (tenant, period)): POST /api/ledger/deferred-tax/run gathers temporary differences — the latest POSTED AR allowance (a DEDUCTIBLE temp diff → DTA = allowance × CIT) and accelerated depreciation (book NBV vs an assumed tax NBV; a TAXABLE temp diff → DTL = (bookNBV − taxNBV) × CIT) — computes net_deferred = DTA − DTL and the DELTA vs the prior posted run, staging an 'Open' deferred_tax_runs row (one per tenant/period; a Posted period → ALREADY_POSTED). CIT rate defaults to 0.20 (Thai). SIMPLIFICATION: no parallel tax-depreciation ledger exists, so tax depreciation is assumed FASTER than book by a documented factor (default 1.5×, capped at the depreciable base) — overridable per run; a deliberate approximation until a tax-dep ledger is modelled. POST /api/ledger/deferred-tax/:id/post is segregated (poster ≠ runner → SELF_POST) and posts the period DELTA via LedgerService.postEntry (delta&gt;0 net asset up = deferred tax benefit → Dr 1700 / Cr 5950; delta&lt;0 → Dr 5950 / Cr 1700), so PERIOD_LOCKED + the GL audit trail apply. Marks the run Posted.</t>
         </is>
       </c>
       <c r="H120" s="13" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I120" s="13" t="inlineStr">
@@ -11281,12 +11281,12 @@
       </c>
       <c r="J120" s="13" t="inlineStr">
         <is>
-          <t>Per run / monthly</t>
+          <t>Quarterly / year-end</t>
         </is>
       </c>
       <c r="K120" s="12" t="inlineStr">
         <is>
-          <t>HR / Payroll / Treasury</t>
+          <t>Tax / Financial Controller</t>
         </is>
       </c>
       <c r="L120" s="13" t="inlineStr">
@@ -11296,22 +11296,22 @@
       </c>
       <c r="M120" s="12" t="inlineStr">
         <is>
-          <t>payroll/payroll.service.ts liabilities/remitLiability</t>
+          <t>deferred-tax.service.ts (runDeferredTax gather temp diffs [AR allowance, accelerated dep] + delta-vs-prior + stage Open, idempotent ALREADY_POSTED; postDeferredTax SELF_POST maker-checker + 1700/5950 delta posting; list/get); deferred-tax.controller.ts (gl_close/gl_post run + :id/post, gl_close/gl_post/exec read); schema/deferred-tax-fx.ts (deferred_tax_runs, uq tenant/period); migration 0168 (tables + RLS); COA 1700/2700/5950 (seedChartOfAccounts); ledger.module.ts (wired); close.service.ts (deferred_tax close-checklist step); reuses ar_allowance (REV-18) + fixed_assets NBV; cutover/basics.ts (TAX-06 ToE)</t>
         </is>
       </c>
       <c r="N120" s="12" t="inlineStr">
         <is>
-          <t>Inspect the schedule + the accrued/remitted/outstanding tie-out and the reconciled flag.</t>
+          <t>Inspect the temp-difference gathering (allowance×rate DTA + accelerated-dep DTL with the documented tax-dep simplification), the delta-vs-prior-run, the SELF_POST maker-checker, and the 1700/5950 posting through the period-lock gate.</t>
         </is>
       </c>
       <c r="O120" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: run a payroll, confirm the SSO/WHT outstanding equals the payrun accrual; remit part and confirm the outstanding falls and the TB stays balanced; attempt an over-remit (REMIT_EXCEEDS_OUTSTANDING).</t>
+          <t>TC-TAX-06-01: run with a posted AR allowance of 1100 at 20% → DTA 220, net deferred asset 220, delta 220 (Open); TC-TAX-06-02: runner self-post → SELF_POST (403), a different user posts → Dr 1700 / Cr 5950 (220), re-post → ALREADY_POSTED (400) (re-performed by the basics.ts harness).</t>
         </is>
       </c>
       <c r="P120" s="12" t="inlineStr">
         <is>
-          <t>Liability schedule + remittance JEs tied to filings</t>
+          <t>deferred_tax_runs register (Open→Posted, temp-difference schedule, runner/poster); the DEFTAX JE to 1700/5950; quarterly/year-end deferred-tax sign-off</t>
         </is>
       </c>
       <c r="Q120" s="18" t="inlineStr">
@@ -11323,7 +11323,7 @@
     <row r="121">
       <c r="A121" s="15" t="inlineStr">
         <is>
-          <t>PAY-03</t>
+          <t>PAY-01</t>
         </is>
       </c>
       <c r="B121" s="16" t="inlineStr">
@@ -11338,27 +11338,27 @@
       </c>
       <c r="D121" s="16" t="inlineStr">
         <is>
-          <t>Payroll expense/liability; Cash</t>
+          <t>Payroll expense/liability</t>
         </is>
       </c>
       <c r="E121" s="16" t="inlineStr">
         <is>
-          <t>Payroll run posted to the GL without independent review — the preparer both computes and posts their own payroll (ghost employees, inflated rate/hours).</t>
+          <t>Payroll, SSO and PIT mis-computed.</t>
         </is>
       </c>
       <c r="F121" s="16" t="inlineStr">
         <is>
-          <t>Authorization</t>
+          <t>Accuracy</t>
         </is>
       </c>
       <c r="G121" s="16" t="inlineStr">
         <is>
-          <t>Payroll maker-checker (SoD): a run posts its GL entry as a DRAFT (excluded from balances) with the run record 'PendingApproval'; a DIFFERENT user must approve before it becomes effective (approver ≠ preparer enforced regardless of permissions, reusing the GL-05 ledger approval). Reject voids the draft; idempotent per (tenant, period).</t>
+          <t>Payroll engine — SSO 5% (cap 750), progressive PIT, payslip net; unit-tested.</t>
         </is>
       </c>
       <c r="H121" s="17" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Auto</t>
         </is>
       </c>
       <c r="I121" s="17" t="inlineStr">
@@ -11373,7 +11373,7 @@
       </c>
       <c r="K121" s="16" t="inlineStr">
         <is>
-          <t>HR / Payroll; Controller</t>
+          <t>HR / Payroll</t>
         </is>
       </c>
       <c r="L121" s="17" t="inlineStr">
@@ -11383,22 +11383,22 @@
       </c>
       <c r="M121" s="16" t="inlineStr">
         <is>
-          <t>payroll/payroll.service.ts approvePayroll/rejectPayroll; migration 0133</t>
+          <t>payroll/payroll-calc.ts; test/unit.test.ts</t>
         </is>
       </c>
       <c r="N121" s="16" t="inlineStr">
         <is>
-          <t>Inspect Draft→approve flow + the approver≠preparer check.</t>
+          <t>Inspect calc + tests.</t>
         </is>
       </c>
       <c r="O121" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: run as A, attempt self-approve (SOD_VIOLATION), approve as B; confirm the JE hits balances only after approval.</t>
+          <t>Re-perform sample payslips.</t>
         </is>
       </c>
       <c r="P121" s="16" t="inlineStr">
         <is>
-          <t>Approval log + SoD test</t>
+          <t>Payslip tests</t>
         </is>
       </c>
       <c r="Q121" s="18" t="inlineStr">
@@ -11410,12 +11410,12 @@
     <row r="122">
       <c r="A122" s="11" t="inlineStr">
         <is>
-          <t>FA-09</t>
+          <t>PAY-02</t>
         </is>
       </c>
       <c r="B122" s="12" t="inlineStr">
         <is>
-          <t>Fixed Assets</t>
+          <t>Payroll</t>
         </is>
       </c>
       <c r="C122" s="13" t="inlineStr">
@@ -11425,27 +11425,27 @@
       </c>
       <c r="D122" s="12" t="inlineStr">
         <is>
-          <t>Property, Plant &amp; Equipment; Cash</t>
+          <t>Payroll liability</t>
         </is>
       </c>
       <c r="E122" s="12" t="inlineStr">
         <is>
-          <t>Asset disposed without independent review — one person writes an asset off the books and records the proceeds (asset-stripping / theft: dispose a still-held asset, or to a related party below value).</t>
+          <t>Statutory withholdings (SSO/WHT/PF) mis-stated or not remitted, so the liability owed to the authorities diverges from the books.</t>
         </is>
       </c>
       <c r="F122" s="12" t="inlineStr">
         <is>
-          <t>Authorization</t>
+          <t>Accuracy/Compliance</t>
         </is>
       </c>
       <c r="G122" s="12" t="inlineStr">
         <is>
-          <t>Asset-disposal maker-checker (SoD): a disposal REQUEST posts its GL entry as a DRAFT (excluded from balances) and flags the asset disposal_pending WITHOUT marking it disposed or moving the register; a DIFFERENT user must approve before it is effective (status→disposed, revaluation surplus recycled 3200→3100) (approver ≠ requester enforced regardless of permissions, reusing the GL-05 ledger approval). Reject voids the draft and the asset stays in service; only one disposal may be pending per asset; a disposal-pending asset is frozen from depreciation.</t>
+          <t>Payroll-liability schedule (GET /api/payroll/liabilities): each statutory account — SSO 2350, WHT/PND1 2360, PF 2370 — shows accrued (GL credits) − remitted (GL debits) = outstanding, tied back to the INDEPENDENT payrun accrual with a `reconciled` flag (a divergence flags a manual JE that touched a payroll-liability account outside the payroll process). Treasury remits the cash (POST .../remit → Dr liability / Cr 1000) which clears the outstanding and keeps the books reconciled to the statutory filings; a remittance beyond the outstanding is blocked (REMIT_EXCEEDS_OUTSTANDING).</t>
         </is>
       </c>
       <c r="H122" s="13" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I122" s="13" t="inlineStr">
@@ -11455,12 +11455,12 @@
       </c>
       <c r="J122" s="13" t="inlineStr">
         <is>
-          <t>Per disposal</t>
+          <t>Per run / monthly</t>
         </is>
       </c>
       <c r="K122" s="12" t="inlineStr">
         <is>
-          <t>FaAccountant / Controller</t>
+          <t>HR / Payroll / Treasury</t>
         </is>
       </c>
       <c r="L122" s="13" t="inlineStr">
@@ -11470,22 +11470,22 @@
       </c>
       <c r="M122" s="12" t="inlineStr">
         <is>
-          <t>assets.service.ts dispose(pendingApproval Draft)/approveDisposal/rejectDisposal; assets.controller.ts (:assetNo/dispose/approve|reject); schema/assets.ts fixed_assets.disposal_pending + migration 0135; cutover/basics.ts + worldclass.ts + compliance.ts (ToE)</t>
+          <t>payroll/payroll.service.ts liabilities/remitLiability</t>
         </is>
       </c>
       <c r="N122" s="12" t="inlineStr">
         <is>
-          <t>Inspect Draft→approve flow + the approver≠requester check + deferred status/recycle.</t>
+          <t>Inspect the schedule + the accrued/remitted/outstanding tie-out and the reconciled flag.</t>
         </is>
       </c>
       <c r="O122" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: request a disposal (Draft JE excluded), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm status→disposed + surplus recycled only after approval (re-performed by the harnesses).</t>
+          <t>Re-perform: run a payroll, confirm the SSO/WHT outstanding equals the payrun accrual; remit part and confirm the outstanding falls and the TB stays balanced; attempt an over-remit (REMIT_EXCEEDS_OUTSTANDING).</t>
         </is>
       </c>
       <c r="P122" s="12" t="inlineStr">
         <is>
-          <t>Disposal approval log + SoD test</t>
+          <t>Liability schedule + remittance JEs tied to filings</t>
         </is>
       </c>
       <c r="Q122" s="18" t="inlineStr">
@@ -11497,12 +11497,12 @@
     <row r="123">
       <c r="A123" s="15" t="inlineStr">
         <is>
-          <t>FA-10</t>
+          <t>PAY-03</t>
         </is>
       </c>
       <c r="B123" s="16" t="inlineStr">
         <is>
-          <t>Fixed Assets</t>
+          <t>Payroll</t>
         </is>
       </c>
       <c r="C123" s="17" t="inlineStr">
@@ -11512,22 +11512,22 @@
       </c>
       <c r="D123" s="16" t="inlineStr">
         <is>
-          <t>Property, Plant &amp; Equipment; Accounts Payable</t>
+          <t>Payroll expense/liability; Cash</t>
         </is>
       </c>
       <c r="E123" s="16" t="inlineStr">
         <is>
-          <t>Capital purchases mis-capitalised or capitalised without independent review — the person who receives the goods also decides what enters the asset register and at what cost/useful life (fictitious or over-valued assets; capex/opex mis-classification).</t>
+          <t>Payroll run posted to the GL without independent review — the preparer both computes and posts their own payroll (ghost employees, inflated rate/hours).</t>
         </is>
       </c>
       <c r="F123" s="16" t="inlineStr">
         <is>
-          <t>Authorization; Accuracy</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="G123" s="16" t="inlineStr">
         <is>
-          <t>Procure-to-Capitalize maker-checker (SoD): a goods-receipt line flagged capital (item-master is_fixed_asset or per-PO-line override) is excluded from inventory capitalisation (1200) at receipt and instead becomes ELIGIBLE for the asset register. Capitalisation is a REQUEST that posts NOTHING to the GL; a DIFFERENT user must approve before the fixed_assets row + acquisition JE (Dr 1500 / Cr 2000) are created (approver ≠ requester enforced regardless of permissions). The created asset carries its source GR/PO for end-to-end PR→PO→GR→FA traceability; a GR line cannot be capitalised twice.</t>
+          <t>Payroll maker-checker (SoD): a run posts its GL entry as a DRAFT (excluded from balances) with the run record 'PendingApproval'; a DIFFERENT user must approve before it becomes effective (approver ≠ preparer enforced regardless of permissions, reusing the GL-05 ledger approval). Reject voids the draft; idempotent per (tenant, period).</t>
         </is>
       </c>
       <c r="H123" s="17" t="inlineStr">
@@ -11542,12 +11542,12 @@
       </c>
       <c r="J123" s="17" t="inlineStr">
         <is>
-          <t>Per capital receipt</t>
+          <t>Per run</t>
         </is>
       </c>
       <c r="K123" s="16" t="inlineStr">
         <is>
-          <t>FaAccountant / Controller</t>
+          <t>HR / Payroll; Controller</t>
         </is>
       </c>
       <c r="L123" s="17" t="inlineStr">
@@ -11557,22 +11557,22 @@
       </c>
       <c r="M123" s="16" t="inlineStr">
         <is>
-          <t>assets.service.ts registerFromGr/approveRegistration/rejectRegistration/eligibleFromGr; assets.controller.ts (registrations*); procurement.service.ts createGr (is_capital routing, costing excluded); schema/assets.ts asset_registration_requests + fixed_assets.source_gr_no/po_no + migration 0137; cutover/basics.ts + compliance.ts (ToE)</t>
+          <t>payroll/payroll.service.ts approvePayroll/rejectPayroll; migration 0133</t>
         </is>
       </c>
       <c r="N123" s="16" t="inlineStr">
         <is>
-          <t>Inspect the eligible→request→approve flow + approver≠requester check + the inventory-vs-asset routing of capital lines.</t>
+          <t>Inspect Draft→approve flow + the approver≠preparer check.</t>
         </is>
       </c>
       <c r="O123" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: receive a capital line, raise a registration (no GL), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm the asset + Dr 1500/Cr 2000 post only after approval and the line cannot be re-registered (re-performed by the harnesses).</t>
+          <t>Re-perform: run as A, attempt self-approve (SOD_VIOLATION), approve as B; confirm the JE hits balances only after approval.</t>
         </is>
       </c>
       <c r="P123" s="16" t="inlineStr">
         <is>
-          <t>Capitalization approval log + SoD test</t>
+          <t>Approval log + SoD test</t>
         </is>
       </c>
       <c r="Q123" s="18" t="inlineStr">
@@ -11584,12 +11584,12 @@
     <row r="124">
       <c r="A124" s="11" t="inlineStr">
         <is>
-          <t>CON-01</t>
+          <t>FA-09</t>
         </is>
       </c>
       <c r="B124" s="12" t="inlineStr">
         <is>
-          <t>Consolidation &amp; FX</t>
+          <t>Fixed Assets</t>
         </is>
       </c>
       <c r="C124" s="13" t="inlineStr">
@@ -11599,42 +11599,42 @@
       </c>
       <c r="D124" s="12" t="inlineStr">
         <is>
-          <t>Consolidation</t>
+          <t>Property, Plant &amp; Equipment; Cash</t>
         </is>
       </c>
       <c r="E124" s="12" t="inlineStr">
         <is>
-          <t>Group consolidation mis-stated (ownership/currency).</t>
+          <t>Asset disposed without independent review — one person writes an asset off the books and records the proceeds (asset-stripping / theft: dispose a still-held asset, or to a related party below value).</t>
         </is>
       </c>
       <c r="F124" s="12" t="inlineStr">
         <is>
-          <t>Accuracy</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="G124" s="12" t="inlineStr">
         <is>
-          <t>Consolidation run (ownership %, entity currency) gated by 'approvals'.</t>
+          <t>Asset-disposal maker-checker (SoD): a disposal REQUEST posts its GL entry as a DRAFT (excluded from balances) and flags the asset disposal_pending WITHOUT marking it disposed or moving the register; a DIFFERENT user must approve before it is effective (status→disposed, revaluation surplus recycled 3200→3100) (approver ≠ requester enforced regardless of permissions, reusing the GL-05 ledger approval). Reject voids the draft and the asset stays in service; only one disposal may be pending per asset; a disposal-pending asset is frozen from depreciation.</t>
         </is>
       </c>
       <c r="H124" s="13" t="inlineStr">
         <is>
-          <t>Auto+Manual</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I124" s="13" t="inlineStr">
         <is>
-          <t>Period</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J124" s="13" t="inlineStr">
         <is>
-          <t>Period</t>
+          <t>Per disposal</t>
         </is>
       </c>
       <c r="K124" s="12" t="inlineStr">
         <is>
-          <t>Group Controller</t>
+          <t>FaAccountant / Controller</t>
         </is>
       </c>
       <c r="L124" s="13" t="inlineStr">
@@ -11644,22 +11644,22 @@
       </c>
       <c r="M124" s="12" t="inlineStr">
         <is>
-          <t>consolidation.service.ts (runConsolidation @Permissions approvals)</t>
+          <t>assets.service.ts dispose(pendingApproval Draft)/approveDisposal/rejectDisposal; assets.controller.ts (:assetNo/dispose/approve|reject); schema/assets.ts fixed_assets.disposal_pending + migration 0135; cutover/basics.ts + worldclass.ts + compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N124" s="12" t="inlineStr">
         <is>
-          <t>Inspect consolidation logic + gate.</t>
+          <t>Inspect Draft→approve flow + the approver≠requester check + deferred status/recycle.</t>
         </is>
       </c>
       <c r="O124" s="12" t="inlineStr">
         <is>
-          <t>Sample period: consolidated TB ties to entities.</t>
+          <t>Re-perform: request a disposal (Draft JE excluded), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm status→disposed + surplus recycled only after approval (re-performed by the harnesses).</t>
         </is>
       </c>
       <c r="P124" s="12" t="inlineStr">
         <is>
-          <t>Consol TB</t>
+          <t>Disposal approval log + SoD test</t>
         </is>
       </c>
       <c r="Q124" s="18" t="inlineStr">
@@ -11671,12 +11671,12 @@
     <row r="125">
       <c r="A125" s="15" t="inlineStr">
         <is>
-          <t>CON-02</t>
+          <t>FA-10</t>
         </is>
       </c>
       <c r="B125" s="16" t="inlineStr">
         <is>
-          <t>Consolidation &amp; FX</t>
+          <t>Fixed Assets</t>
         </is>
       </c>
       <c r="C125" s="17" t="inlineStr">
@@ -11686,42 +11686,42 @@
       </c>
       <c r="D125" s="16" t="inlineStr">
         <is>
-          <t>FX gain/loss</t>
+          <t>Property, Plant &amp; Equipment; Accounts Payable</t>
         </is>
       </c>
       <c r="E125" s="16" t="inlineStr">
         <is>
-          <t>FX exposures not revalued at period-end.</t>
+          <t>Capital purchases mis-capitalised or capitalised without independent review — the person who receives the goods also decides what enters the asset register and at what cost/useful life (fictitious or over-valued assets; capex/opex mis-classification).</t>
         </is>
       </c>
       <c r="F125" s="16" t="inlineStr">
         <is>
-          <t>Valuation</t>
+          <t>Authorization; Accuracy</t>
         </is>
       </c>
       <c r="G125" s="16" t="inlineStr">
         <is>
-          <t>FX revaluation at period-end rates; unrealized FX posted (acct 5400).</t>
+          <t>Procure-to-Capitalize maker-checker (SoD): a goods-receipt line flagged capital (item-master is_fixed_asset or per-PO-line override) is excluded from inventory capitalisation (1200) at receipt and instead becomes ELIGIBLE for the asset register. Capitalisation is a REQUEST that posts NOTHING to the GL; a DIFFERENT user must approve before the fixed_assets row + acquisition JE (Dr 1500 / Cr 2000) are created (approver ≠ requester enforced regardless of permissions). The created asset carries its source GR/PO for end-to-end PR→PO→GR→FA traceability; a GR line cannot be capitalised twice.</t>
         </is>
       </c>
       <c r="H125" s="17" t="inlineStr">
         <is>
-          <t>Auto+Manual</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I125" s="17" t="inlineStr">
         <is>
-          <t>Period-end</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J125" s="17" t="inlineStr">
         <is>
-          <t>Period</t>
+          <t>Per capital receipt</t>
         </is>
       </c>
       <c r="K125" s="16" t="inlineStr">
         <is>
-          <t>Controller</t>
+          <t>FaAccountant / Controller</t>
         </is>
       </c>
       <c r="L125" s="17" t="inlineStr">
@@ -11731,22 +11731,22 @@
       </c>
       <c r="M125" s="16" t="inlineStr">
         <is>
-          <t>fx.service.ts (revalue / unrealized report)</t>
+          <t>assets.service.ts registerFromGr/approveRegistration/rejectRegistration/eligibleFromGr; assets.controller.ts (registrations*); procurement.service.ts createGr (is_capital routing, costing excluded); schema/assets.ts asset_registration_requests + fixed_assets.source_gr_no/po_no + migration 0137; cutover/basics.ts + compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N125" s="16" t="inlineStr">
         <is>
-          <t>Inspect reval logic + rates.</t>
+          <t>Inspect the eligible→request→approve flow + approver≠requester check + the inventory-vs-asset routing of capital lines.</t>
         </is>
       </c>
       <c r="O125" s="16" t="inlineStr">
         <is>
-          <t>Recompute reval on sample balances.</t>
+          <t>Re-perform: receive a capital line, raise a registration (no GL), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm the asset + Dr 1500/Cr 2000 post only after approval and the line cannot be re-registered (re-performed by the harnesses).</t>
         </is>
       </c>
       <c r="P125" s="16" t="inlineStr">
         <is>
-          <t>FX reval JE</t>
+          <t>Capitalization approval log + SoD test</t>
         </is>
       </c>
       <c r="Q125" s="18" t="inlineStr">
@@ -11758,7 +11758,7 @@
     <row r="126">
       <c r="A126" s="11" t="inlineStr">
         <is>
-          <t>FX-04</t>
+          <t>CON-01</t>
         </is>
       </c>
       <c r="B126" s="12" t="inlineStr">
@@ -11773,42 +11773,42 @@
       </c>
       <c r="D126" s="12" t="inlineStr">
         <is>
-          <t>FX gain/loss; Revenue; AR/AP</t>
+          <t>Consolidation</t>
         </is>
       </c>
       <c r="E126" s="12" t="inlineStr">
         <is>
-          <t>A wrong manually-entered FX rate (fat-fingered, e.g. USD 36 keyed as 63) flows straight into a period-end revaluation JE and the unrealized-FX report with no independent review — mis-stating earnings/equity and FX-translated balances.</t>
+          <t>Group consolidation mis-stated (ownership/currency).</t>
         </is>
       </c>
       <c r="F126" s="12" t="inlineStr">
         <is>
-          <t>Accuracy/Valuation</t>
+          <t>Accuracy</t>
         </is>
       </c>
       <c r="G126" s="12" t="inlineStr">
         <is>
-          <t>FX rate maker-checker (SoD): a MANUALLY-entered rate lands as PendingApproval and is EXCLUDED from rate resolution — revaluation, the unrealized-FX report, and consolidation translation all use APPROVED rates only — until a DIFFERENT user approves it (POST /api/fx/rates/approve). Self-approval → SOD_VIOLATION (binds even Admin); reject marks the rate Rejected (never usable); re-entering a rate sends it back to PendingApproval. Externally-sourced (feed) rates carrying an explicit non-manual source are auto-approved. Pending rates are also surfaced, aged, by the pending-approvals monitor (GOV-01).</t>
+          <t>Consolidation run (ownership %, entity currency) gated by 'approvals'.</t>
         </is>
       </c>
       <c r="H126" s="13" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="I126" s="13" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Period</t>
         </is>
       </c>
       <c r="J126" s="13" t="inlineStr">
         <is>
-          <t>Per rate</t>
+          <t>Period</t>
         </is>
       </c>
       <c r="K126" s="12" t="inlineStr">
         <is>
-          <t>Controller / Treasury</t>
+          <t>Group Controller</t>
         </is>
       </c>
       <c r="L126" s="13" t="inlineStr">
@@ -11818,22 +11818,22 @@
       </c>
       <c r="M126" s="12" t="inlineStr">
         <is>
-          <t>fx.service.ts setRate(manual→PendingApproval)/approveRate/rejectRate/rateAsOf(Approved only); fx.controller.ts (rates/approve|reject|pending gated approvals/gl_close); consolidation.service.ts (translation reads Approved rates); schema/fx.ts fx_rates.status + migration 0141; cutover/fxreval.ts (ToE)</t>
+          <t>consolidation.service.ts (runConsolidation @Permissions approvals)</t>
         </is>
       </c>
       <c r="N126" s="12" t="inlineStr">
         <is>
-          <t>Inspect the request→approve flow + the approver≠requester check + that revaluation/reporting resolve Approved rates only.</t>
+          <t>Inspect consolidation logic + gate.</t>
         </is>
       </c>
       <c r="O126" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: enter a manual rate (PendingApproval), confirm revalue is blocked NO_RATE while pending, attempt self-approve (SOD_VIOLATION), approve as a different user, then revalue succeeds (re-performed by the fxreval harness).</t>
+          <t>Sample period: consolidated TB ties to entities.</t>
         </is>
       </c>
       <c r="P126" s="12" t="inlineStr">
         <is>
-          <t>FX rate approval log + SoD test</t>
+          <t>Consol TB</t>
         </is>
       </c>
       <c r="Q126" s="18" t="inlineStr">
@@ -11845,92 +11845,266 @@
     <row r="127">
       <c r="A127" s="15" t="inlineStr">
         <is>
+          <t>CON-02</t>
+        </is>
+      </c>
+      <c r="B127" s="16" t="inlineStr">
+        <is>
+          <t>Consolidation &amp; FX</t>
+        </is>
+      </c>
+      <c r="C127" s="17" t="inlineStr">
+        <is>
+          <t>Application</t>
+        </is>
+      </c>
+      <c r="D127" s="16" t="inlineStr">
+        <is>
+          <t>FX gain/loss</t>
+        </is>
+      </c>
+      <c r="E127" s="16" t="inlineStr">
+        <is>
+          <t>FX exposures not revalued at period-end.</t>
+        </is>
+      </c>
+      <c r="F127" s="16" t="inlineStr">
+        <is>
+          <t>Valuation</t>
+        </is>
+      </c>
+      <c r="G127" s="16" t="inlineStr">
+        <is>
+          <t>FX revaluation at period-end rates; unrealized FX posted (acct 5400).</t>
+        </is>
+      </c>
+      <c r="H127" s="17" t="inlineStr">
+        <is>
+          <t>Auto+Manual</t>
+        </is>
+      </c>
+      <c r="I127" s="17" t="inlineStr">
+        <is>
+          <t>Period-end</t>
+        </is>
+      </c>
+      <c r="J127" s="17" t="inlineStr">
+        <is>
+          <t>Period</t>
+        </is>
+      </c>
+      <c r="K127" s="16" t="inlineStr">
+        <is>
+          <t>Controller</t>
+        </is>
+      </c>
+      <c r="L127" s="17" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="M127" s="16" t="inlineStr">
+        <is>
+          <t>fx.service.ts (revalue / unrealized report)</t>
+        </is>
+      </c>
+      <c r="N127" s="16" t="inlineStr">
+        <is>
+          <t>Inspect reval logic + rates.</t>
+        </is>
+      </c>
+      <c r="O127" s="16" t="inlineStr">
+        <is>
+          <t>Recompute reval on sample balances.</t>
+        </is>
+      </c>
+      <c r="P127" s="16" t="inlineStr">
+        <is>
+          <t>FX reval JE</t>
+        </is>
+      </c>
+      <c r="Q127" s="18" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="11" t="inlineStr">
+        <is>
+          <t>FX-04</t>
+        </is>
+      </c>
+      <c r="B128" s="12" t="inlineStr">
+        <is>
+          <t>Consolidation &amp; FX</t>
+        </is>
+      </c>
+      <c r="C128" s="13" t="inlineStr">
+        <is>
+          <t>Application</t>
+        </is>
+      </c>
+      <c r="D128" s="12" t="inlineStr">
+        <is>
+          <t>FX gain/loss; Revenue; AR/AP</t>
+        </is>
+      </c>
+      <c r="E128" s="12" t="inlineStr">
+        <is>
+          <t>A wrong manually-entered FX rate (fat-fingered, e.g. USD 36 keyed as 63) flows straight into a period-end revaluation JE and the unrealized-FX report with no independent review — mis-stating earnings/equity and FX-translated balances.</t>
+        </is>
+      </c>
+      <c r="F128" s="12" t="inlineStr">
+        <is>
+          <t>Accuracy/Valuation</t>
+        </is>
+      </c>
+      <c r="G128" s="12" t="inlineStr">
+        <is>
+          <t>FX rate maker-checker (SoD): a MANUALLY-entered rate lands as PendingApproval and is EXCLUDED from rate resolution — revaluation, the unrealized-FX report, and consolidation translation all use APPROVED rates only — until a DIFFERENT user approves it (POST /api/fx/rates/approve). Self-approval → SOD_VIOLATION (binds even Admin); reject marks the rate Rejected (never usable); re-entering a rate sends it back to PendingApproval. Externally-sourced (feed) rates carrying an explicit non-manual source are auto-approved. Pending rates are also surfaced, aged, by the pending-approvals monitor (GOV-01).</t>
+        </is>
+      </c>
+      <c r="H128" s="13" t="inlineStr">
+        <is>
+          <t>Prev</t>
+        </is>
+      </c>
+      <c r="I128" s="13" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="J128" s="13" t="inlineStr">
+        <is>
+          <t>Per rate</t>
+        </is>
+      </c>
+      <c r="K128" s="12" t="inlineStr">
+        <is>
+          <t>Controller / Treasury</t>
+        </is>
+      </c>
+      <c r="L128" s="13" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="M128" s="12" t="inlineStr">
+        <is>
+          <t>fx.service.ts setRate(manual→PendingApproval)/approveRate/rejectRate/rateAsOf(Approved only); fx.controller.ts (rates/approve|reject|pending gated approvals/gl_close); consolidation.service.ts (translation reads Approved rates); schema/fx.ts fx_rates.status + migration 0141; cutover/fxreval.ts (ToE)</t>
+        </is>
+      </c>
+      <c r="N128" s="12" t="inlineStr">
+        <is>
+          <t>Inspect the request→approve flow + the approver≠requester check + that revaluation/reporting resolve Approved rates only.</t>
+        </is>
+      </c>
+      <c r="O128" s="12" t="inlineStr">
+        <is>
+          <t>Re-perform: enter a manual rate (PendingApproval), confirm revalue is blocked NO_RATE while pending, attempt self-approve (SOD_VIOLATION), approve as a different user, then revalue succeeds (re-performed by the fxreval harness).</t>
+        </is>
+      </c>
+      <c r="P128" s="12" t="inlineStr">
+        <is>
+          <t>FX rate approval log + SoD test</t>
+        </is>
+      </c>
+      <c r="Q128" s="18" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="15" t="inlineStr">
+        <is>
           <t>BUD-01</t>
         </is>
       </c>
-      <c r="B127" s="16" t="inlineStr">
+      <c r="B129" s="16" t="inlineStr">
         <is>
           <t>Budgeting &amp; Planning</t>
         </is>
       </c>
-      <c r="C127" s="17" t="inlineStr">
+      <c r="C129" s="17" t="inlineStr">
         <is>
           <t>Application</t>
         </is>
       </c>
-      <c r="D127" s="16" t="inlineStr">
+      <c r="D129" s="16" t="inlineStr">
         <is>
           <t>Budget; All (variance reporting)</t>
         </is>
       </c>
-      <c r="E127" s="16" t="inlineStr">
+      <c r="E129" s="16" t="inlineStr">
         <is>
           <t>A budget figure is entered/changed by one person and immediately drives the budget-vs-actual variance report — the basis for spend authorization and performance review — with no independent approval; a wrong or self-serving budget makes overspending look 'on budget'.</t>
         </is>
       </c>
-      <c r="F127" s="16" t="inlineStr">
+      <c r="F129" s="16" t="inlineStr">
         <is>
           <t>Authorization/Accuracy</t>
         </is>
       </c>
-      <c r="G127" s="16" t="inlineStr">
+      <c r="G129" s="16" t="inlineStr">
         <is>
           <t>Budget maker-checker (SoD): an upserted budget (POST /api/ledger/budgets) lands as PendingApproval and is EXCLUDED from budget-vs-actual until a DIFFERENT user approves it (POST /api/ledger/budgets/approve for the fiscal_year/account/cost-centre[/period]). Self-approval → SOD_VIOLATION (binds even Admin); reject marks it Rejected (excluded). DEFAULT 'Approved' keeps existing rows + direct planning seeds usable. Pending budgets are also surfaced, aged, by the pending-approvals monitor (GOV-01).</t>
         </is>
       </c>
-      <c r="H127" s="17" t="inlineStr">
+      <c r="H129" s="17" t="inlineStr">
         <is>
           <t>Prev</t>
         </is>
       </c>
-      <c r="I127" s="17" t="inlineStr">
+      <c r="I129" s="17" t="inlineStr">
         <is>
           <t>Automated</t>
         </is>
       </c>
-      <c r="J127" s="17" t="inlineStr">
+      <c r="J129" s="17" t="inlineStr">
         <is>
           <t>Per budget</t>
         </is>
       </c>
-      <c r="K127" s="16" t="inlineStr">
+      <c r="K129" s="16" t="inlineStr">
         <is>
           <t>Controller / FP&amp;A</t>
         </is>
       </c>
-      <c r="L127" s="17" t="inlineStr">
+      <c r="L129" s="17" t="inlineStr">
         <is>
           <t>P10</t>
         </is>
       </c>
-      <c r="M127" s="16" t="inlineStr">
+      <c r="M129" s="16" t="inlineStr">
         <is>
           <t>budget.service.ts upsertBudget(→PendingApproval)/approveBudget/rejectBudget/budgetVsActual(Approved only); budget.controller.ts (budgets/approve|reject|pending gated approvals/gl_close); schema/budgets.ts budgets.status + migration 0142; cutover/budget.ts (ToE)</t>
         </is>
       </c>
-      <c r="N127" s="16" t="inlineStr">
+      <c r="N129" s="16" t="inlineStr">
         <is>
           <t>Inspect the request→approve flow + the approver≠requester check + that budget-vs-actual counts Approved budgets only.</t>
         </is>
       </c>
-      <c r="O127" s="16" t="inlineStr">
+      <c r="O129" s="16" t="inlineStr">
         <is>
           <t>Re-perform: upsert a budget (PendingApproval, excluded from variance), attempt self-approve (SOD_VIOLATION), approve as a different user, confirm it then appears in budget-vs-actual (re-performed by the budget harness).</t>
         </is>
       </c>
-      <c r="P127" s="16" t="inlineStr">
+      <c r="P129" s="16" t="inlineStr">
         <is>
           <t>Budget approval log + SoD test</t>
         </is>
       </c>
-      <c r="Q127" s="18" t="inlineStr">
+      <c r="Q129" s="18" t="inlineStr">
         <is>
           <t>Implemented</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q127"/>
+  <autoFilter ref="A1:Q129"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -13113,7 +13287,7 @@
         </is>
       </c>
       <c r="C5" s="29">
-        <f>COUNTIF(RCM!$Q$2:$Q$127,B5)</f>
+        <f>COUNTIF(RCM!$Q$2:$Q$129,B5)</f>
         <v/>
       </c>
     </row>
@@ -13124,7 +13298,7 @@
         </is>
       </c>
       <c r="C6" s="29">
-        <f>COUNTIF(RCM!$Q$2:$Q$127,B6)</f>
+        <f>COUNTIF(RCM!$Q$2:$Q$129,B6)</f>
         <v/>
       </c>
     </row>
@@ -13135,7 +13309,7 @@
         </is>
       </c>
       <c r="C7" s="29">
-        <f>COUNTIF(RCM!$Q$2:$Q$127,B7)</f>
+        <f>COUNTIF(RCM!$Q$2:$Q$129,B7)</f>
         <v/>
       </c>
     </row>
@@ -13146,7 +13320,7 @@
         </is>
       </c>
       <c r="C8" s="32">
-        <f>COUNTA(RCM!$A$2:$A$127)</f>
+        <f>COUNTA(RCM!$A$2:$A$129)</f>
         <v/>
       </c>
     </row>
@@ -13164,7 +13338,7 @@
         </is>
       </c>
       <c r="C11" s="29">
-        <f>COUNTIF(RCM!$C$2:$C$127,B11)</f>
+        <f>COUNTIF(RCM!$C$2:$C$129,B11)</f>
         <v/>
       </c>
     </row>
@@ -13175,7 +13349,7 @@
         </is>
       </c>
       <c r="C12" s="29">
-        <f>COUNTIF(RCM!$C$2:$C$127,B12)</f>
+        <f>COUNTIF(RCM!$C$2:$C$129,B12)</f>
         <v/>
       </c>
     </row>
@@ -13186,7 +13360,7 @@
         </is>
       </c>
       <c r="C13" s="29">
-        <f>COUNTIF(RCM!$C$2:$C$127,B13)</f>
+        <f>COUNTIF(RCM!$C$2:$C$129,B13)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: merge main, renumber deferred_tax_fx 0168→0169 (labor_ot_rules took 0168)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/compliance/Oshinei_ERP_SOX_RCM_v1.xlsx
+++ b/compliance/Oshinei_ERP_SOX_RCM_v1.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'RCM'!$A$1:$Q$129</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'RCM'!$A$1:$Q$130</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Gap Remediation'!$A$2:$H$18</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -858,7 +858,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q129"/>
+  <dimension ref="A1:Q130"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -11584,12 +11584,12 @@
     <row r="124">
       <c r="A124" s="11" t="inlineStr">
         <is>
-          <t>FA-09</t>
+          <t>PAY-04</t>
         </is>
       </c>
       <c r="B124" s="12" t="inlineStr">
         <is>
-          <t>Fixed Assets</t>
+          <t>Payroll</t>
         </is>
       </c>
       <c r="C124" s="13" t="inlineStr">
@@ -11599,67 +11599,67 @@
       </c>
       <c r="D124" s="12" t="inlineStr">
         <is>
-          <t>Property, Plant &amp; Equipment; Cash</t>
+          <t>Payroll expense; Labor cost</t>
         </is>
       </c>
       <c r="E124" s="12" t="inlineStr">
         <is>
-          <t>Asset disposed without independent review — one person writes an asset off the books and records the proceeds (asset-stripping / theft: dispose a still-held asset, or to a related party below value).</t>
+          <t>Overtime is paid at a single flat multiplier with no holiday/night tiers and no statutory cap (Thai LPA OT is mis-paid — too little on holidays, or beyond the 48h/week limit), AND labor cost runs over target as a % of sales with nothing flagging it — margin erosion goes unnoticed until payroll posts.</t>
         </is>
       </c>
       <c r="F124" s="12" t="inlineStr">
         <is>
-          <t>Authorization</t>
+          <t>Accuracy/Completeness</t>
         </is>
       </c>
       <c r="G124" s="12" t="inlineStr">
         <is>
-          <t>Asset-disposal maker-checker (SoD): a disposal REQUEST posts its GL entry as a DRAFT (excluded from balances) and flags the asset disposal_pending WITHOUT marking it disposed or moving the register; a DIFFERENT user must approve before it is effective (status→disposed, revaluation surplus recycled 3200→3100) (approver ≠ requester enforced regardless of permissions, reusing the GL-05 ledger approval). Reject voids the draft and the asset stays in service; only one disposal may be pending per asset; a disposal-pending asset is frozen from depreciation.</t>
+          <t>Tiered OT rules engine + labor-% alerting: a per-tenant labor_ot_rules table overrides the Thai LPA statutory defaults (REGULAR_OT 1.5x beyond 8h/day, HOLIDAY 2x, HOLIDAY_OT 3x, NIGHT 1.0x tracked; 48h/week cap) — GET/PUT /api/pos/labor/ot-rules. computeOtPay (POST /api/pos/labor/ot-pay) applies the tier's multiplier and CAPS paid hours at the 48h weekly limit, flagging any over-cap hours (over_cap=true) rather than silently paying them. Separately, POST /api/pos/labor/labor-alert/check computes labor % of sales for a period and, when it exceeds the target (default 35%), persists a LABOR_PCT_EXCEEDED alert (idempotent per period) surfaced on GET /api/pos/labor/alerts for the manager to act on / resolve. Tenant-scoped (RLS); gated pos/users/exec. Operational (no GL).</t>
         </is>
       </c>
       <c r="H124" s="13" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det/Prev</t>
         </is>
       </c>
       <c r="I124" s="13" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="J124" s="13" t="inlineStr">
         <is>
-          <t>Per disposal</t>
+          <t>Per shift / payroll cycle</t>
         </is>
       </c>
       <c r="K124" s="12" t="inlineStr">
         <is>
-          <t>FaAccountant / Controller</t>
+          <t>HR / Store Ops Mgr</t>
         </is>
       </c>
       <c r="L124" s="13" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P10/P13</t>
         </is>
       </c>
       <c r="M124" s="12" t="inlineStr">
         <is>
-          <t>assets.service.ts dispose(pendingApproval Draft)/approveDisposal/rejectDisposal; assets.controller.ts (:assetNo/dispose/approve|reject); schema/assets.ts fixed_assets.disposal_pending + migration 0135; cutover/basics.ts + worldclass.ts + compliance.ts (ToE)</t>
+          <t>pos-loyalty-labor/schedule.service.ts getOtRules/upsertOtRule (Thai defaults overlay) + computeOtPay (tier multiplier + 48h cap, over_cap flag) + checkLaborAlert/listAlerts/resolveAlert; pos-loyalty-labor.controller.ts (ot-rules, ot-pay, labor-alert/check, alerts[/:id/resolve]); schema/pos-scale.ts labor_ot_rules + labor_alerts + migration 0167; /scheduling UI; cutover/scheduling.ts (ToE)</t>
         </is>
       </c>
       <c r="N124" s="12" t="inlineStr">
         <is>
-          <t>Inspect Draft→approve flow + the approver≠requester check + deferred status/recycle.</t>
+          <t>Inspect the statutory-default overlay, the tier multipliers, the 48h cap + over_cap flag, and the labor-% threshold alert (raise/idempotent/resolve).</t>
         </is>
       </c>
       <c r="O124" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: request a disposal (Draft JE excluded), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm status→disposed + surplus recycled only after approval (re-performed by the harnesses).</t>
+          <t>Re-perform: OT rules expose Thai defaults (1.5/2/3/1.0, cap 48); override REGULAR_OT to 2.0; HOLIDAY_OT 2h x 100 x 3 = 600; a 5h OT entry at 47h already-worked pays only 1h + flags 4h over-cap; labor 8% vs a 5% target raises an alert (idempotent), vs a 50% target raises none; resolve clears it (re-performed by the scheduling harness).</t>
         </is>
       </c>
       <c r="P124" s="12" t="inlineStr">
         <is>
-          <t>Disposal approval log + SoD test</t>
+          <t>labor_ot_rules + labor_alerts register; OT/labor-% test</t>
         </is>
       </c>
       <c r="Q124" s="18" t="inlineStr">
@@ -11671,7 +11671,7 @@
     <row r="125">
       <c r="A125" s="15" t="inlineStr">
         <is>
-          <t>FA-10</t>
+          <t>FA-09</t>
         </is>
       </c>
       <c r="B125" s="16" t="inlineStr">
@@ -11686,22 +11686,22 @@
       </c>
       <c r="D125" s="16" t="inlineStr">
         <is>
-          <t>Property, Plant &amp; Equipment; Accounts Payable</t>
+          <t>Property, Plant &amp; Equipment; Cash</t>
         </is>
       </c>
       <c r="E125" s="16" t="inlineStr">
         <is>
-          <t>Capital purchases mis-capitalised or capitalised without independent review — the person who receives the goods also decides what enters the asset register and at what cost/useful life (fictitious or over-valued assets; capex/opex mis-classification).</t>
+          <t>Asset disposed without independent review — one person writes an asset off the books and records the proceeds (asset-stripping / theft: dispose a still-held asset, or to a related party below value).</t>
         </is>
       </c>
       <c r="F125" s="16" t="inlineStr">
         <is>
-          <t>Authorization; Accuracy</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="G125" s="16" t="inlineStr">
         <is>
-          <t>Procure-to-Capitalize maker-checker (SoD): a goods-receipt line flagged capital (item-master is_fixed_asset or per-PO-line override) is excluded from inventory capitalisation (1200) at receipt and instead becomes ELIGIBLE for the asset register. Capitalisation is a REQUEST that posts NOTHING to the GL; a DIFFERENT user must approve before the fixed_assets row + acquisition JE (Dr 1500 / Cr 2000) are created (approver ≠ requester enforced regardless of permissions). The created asset carries its source GR/PO for end-to-end PR→PO→GR→FA traceability; a GR line cannot be capitalised twice.</t>
+          <t>Asset-disposal maker-checker (SoD): a disposal REQUEST posts its GL entry as a DRAFT (excluded from balances) and flags the asset disposal_pending WITHOUT marking it disposed or moving the register; a DIFFERENT user must approve before it is effective (status→disposed, revaluation surplus recycled 3200→3100) (approver ≠ requester enforced regardless of permissions, reusing the GL-05 ledger approval). Reject voids the draft and the asset stays in service; only one disposal may be pending per asset; a disposal-pending asset is frozen from depreciation.</t>
         </is>
       </c>
       <c r="H125" s="17" t="inlineStr">
@@ -11716,7 +11716,7 @@
       </c>
       <c r="J125" s="17" t="inlineStr">
         <is>
-          <t>Per capital receipt</t>
+          <t>Per disposal</t>
         </is>
       </c>
       <c r="K125" s="16" t="inlineStr">
@@ -11731,22 +11731,22 @@
       </c>
       <c r="M125" s="16" t="inlineStr">
         <is>
-          <t>assets.service.ts registerFromGr/approveRegistration/rejectRegistration/eligibleFromGr; assets.controller.ts (registrations*); procurement.service.ts createGr (is_capital routing, costing excluded); schema/assets.ts asset_registration_requests + fixed_assets.source_gr_no/po_no + migration 0137; cutover/basics.ts + compliance.ts (ToE)</t>
+          <t>assets.service.ts dispose(pendingApproval Draft)/approveDisposal/rejectDisposal; assets.controller.ts (:assetNo/dispose/approve|reject); schema/assets.ts fixed_assets.disposal_pending + migration 0135; cutover/basics.ts + worldclass.ts + compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N125" s="16" t="inlineStr">
         <is>
-          <t>Inspect the eligible→request→approve flow + approver≠requester check + the inventory-vs-asset routing of capital lines.</t>
+          <t>Inspect Draft→approve flow + the approver≠requester check + deferred status/recycle.</t>
         </is>
       </c>
       <c r="O125" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: receive a capital line, raise a registration (no GL), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm the asset + Dr 1500/Cr 2000 post only after approval and the line cannot be re-registered (re-performed by the harnesses).</t>
+          <t>Re-perform: request a disposal (Draft JE excluded), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm status→disposed + surplus recycled only after approval (re-performed by the harnesses).</t>
         </is>
       </c>
       <c r="P125" s="16" t="inlineStr">
         <is>
-          <t>Capitalization approval log + SoD test</t>
+          <t>Disposal approval log + SoD test</t>
         </is>
       </c>
       <c r="Q125" s="18" t="inlineStr">
@@ -11758,12 +11758,12 @@
     <row r="126">
       <c r="A126" s="11" t="inlineStr">
         <is>
-          <t>CON-01</t>
+          <t>FA-10</t>
         </is>
       </c>
       <c r="B126" s="12" t="inlineStr">
         <is>
-          <t>Consolidation &amp; FX</t>
+          <t>Fixed Assets</t>
         </is>
       </c>
       <c r="C126" s="13" t="inlineStr">
@@ -11773,42 +11773,42 @@
       </c>
       <c r="D126" s="12" t="inlineStr">
         <is>
-          <t>Consolidation</t>
+          <t>Property, Plant &amp; Equipment; Accounts Payable</t>
         </is>
       </c>
       <c r="E126" s="12" t="inlineStr">
         <is>
-          <t>Group consolidation mis-stated (ownership/currency).</t>
+          <t>Capital purchases mis-capitalised or capitalised without independent review — the person who receives the goods also decides what enters the asset register and at what cost/useful life (fictitious or over-valued assets; capex/opex mis-classification).</t>
         </is>
       </c>
       <c r="F126" s="12" t="inlineStr">
         <is>
-          <t>Accuracy</t>
+          <t>Authorization; Accuracy</t>
         </is>
       </c>
       <c r="G126" s="12" t="inlineStr">
         <is>
-          <t>Consolidation run (ownership %, entity currency) gated by 'approvals'.</t>
+          <t>Procure-to-Capitalize maker-checker (SoD): a goods-receipt line flagged capital (item-master is_fixed_asset or per-PO-line override) is excluded from inventory capitalisation (1200) at receipt and instead becomes ELIGIBLE for the asset register. Capitalisation is a REQUEST that posts NOTHING to the GL; a DIFFERENT user must approve before the fixed_assets row + acquisition JE (Dr 1500 / Cr 2000) are created (approver ≠ requester enforced regardless of permissions). The created asset carries its source GR/PO for end-to-end PR→PO→GR→FA traceability; a GR line cannot be capitalised twice.</t>
         </is>
       </c>
       <c r="H126" s="13" t="inlineStr">
         <is>
-          <t>Auto+Manual</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I126" s="13" t="inlineStr">
         <is>
-          <t>Period</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J126" s="13" t="inlineStr">
         <is>
-          <t>Period</t>
+          <t>Per capital receipt</t>
         </is>
       </c>
       <c r="K126" s="12" t="inlineStr">
         <is>
-          <t>Group Controller</t>
+          <t>FaAccountant / Controller</t>
         </is>
       </c>
       <c r="L126" s="13" t="inlineStr">
@@ -11818,22 +11818,22 @@
       </c>
       <c r="M126" s="12" t="inlineStr">
         <is>
-          <t>consolidation.service.ts (runConsolidation @Permissions approvals)</t>
+          <t>assets.service.ts registerFromGr/approveRegistration/rejectRegistration/eligibleFromGr; assets.controller.ts (registrations*); procurement.service.ts createGr (is_capital routing, costing excluded); schema/assets.ts asset_registration_requests + fixed_assets.source_gr_no/po_no + migration 0137; cutover/basics.ts + compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N126" s="12" t="inlineStr">
         <is>
-          <t>Inspect consolidation logic + gate.</t>
+          <t>Inspect the eligible→request→approve flow + approver≠requester check + the inventory-vs-asset routing of capital lines.</t>
         </is>
       </c>
       <c r="O126" s="12" t="inlineStr">
         <is>
-          <t>Sample period: consolidated TB ties to entities.</t>
+          <t>Re-perform: receive a capital line, raise a registration (no GL), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm the asset + Dr 1500/Cr 2000 post only after approval and the line cannot be re-registered (re-performed by the harnesses).</t>
         </is>
       </c>
       <c r="P126" s="12" t="inlineStr">
         <is>
-          <t>Consol TB</t>
+          <t>Capitalization approval log + SoD test</t>
         </is>
       </c>
       <c r="Q126" s="18" t="inlineStr">
@@ -11845,7 +11845,7 @@
     <row r="127">
       <c r="A127" s="15" t="inlineStr">
         <is>
-          <t>CON-02</t>
+          <t>CON-01</t>
         </is>
       </c>
       <c r="B127" s="16" t="inlineStr">
@@ -11860,22 +11860,22 @@
       </c>
       <c r="D127" s="16" t="inlineStr">
         <is>
-          <t>FX gain/loss</t>
+          <t>Consolidation</t>
         </is>
       </c>
       <c r="E127" s="16" t="inlineStr">
         <is>
-          <t>FX exposures not revalued at period-end.</t>
+          <t>Group consolidation mis-stated (ownership/currency).</t>
         </is>
       </c>
       <c r="F127" s="16" t="inlineStr">
         <is>
-          <t>Valuation</t>
+          <t>Accuracy</t>
         </is>
       </c>
       <c r="G127" s="16" t="inlineStr">
         <is>
-          <t>FX revaluation at period-end rates; unrealized FX posted (acct 5400).</t>
+          <t>Consolidation run (ownership %, entity currency) gated by 'approvals'.</t>
         </is>
       </c>
       <c r="H127" s="17" t="inlineStr">
@@ -11885,7 +11885,7 @@
       </c>
       <c r="I127" s="17" t="inlineStr">
         <is>
-          <t>Period-end</t>
+          <t>Period</t>
         </is>
       </c>
       <c r="J127" s="17" t="inlineStr">
@@ -11895,7 +11895,7 @@
       </c>
       <c r="K127" s="16" t="inlineStr">
         <is>
-          <t>Controller</t>
+          <t>Group Controller</t>
         </is>
       </c>
       <c r="L127" s="17" t="inlineStr">
@@ -11905,22 +11905,22 @@
       </c>
       <c r="M127" s="16" t="inlineStr">
         <is>
-          <t>fx.service.ts (revalue / unrealized report)</t>
+          <t>consolidation.service.ts (runConsolidation @Permissions approvals)</t>
         </is>
       </c>
       <c r="N127" s="16" t="inlineStr">
         <is>
-          <t>Inspect reval logic + rates.</t>
+          <t>Inspect consolidation logic + gate.</t>
         </is>
       </c>
       <c r="O127" s="16" t="inlineStr">
         <is>
-          <t>Recompute reval on sample balances.</t>
+          <t>Sample period: consolidated TB ties to entities.</t>
         </is>
       </c>
       <c r="P127" s="16" t="inlineStr">
         <is>
-          <t>FX reval JE</t>
+          <t>Consol TB</t>
         </is>
       </c>
       <c r="Q127" s="18" t="inlineStr">
@@ -11932,7 +11932,7 @@
     <row r="128">
       <c r="A128" s="11" t="inlineStr">
         <is>
-          <t>FX-04</t>
+          <t>CON-02</t>
         </is>
       </c>
       <c r="B128" s="12" t="inlineStr">
@@ -11947,42 +11947,42 @@
       </c>
       <c r="D128" s="12" t="inlineStr">
         <is>
-          <t>FX gain/loss; Revenue; AR/AP</t>
+          <t>FX gain/loss</t>
         </is>
       </c>
       <c r="E128" s="12" t="inlineStr">
         <is>
-          <t>A wrong manually-entered FX rate (fat-fingered, e.g. USD 36 keyed as 63) flows straight into a period-end revaluation JE and the unrealized-FX report with no independent review — mis-stating earnings/equity and FX-translated balances.</t>
+          <t>FX exposures not revalued at period-end.</t>
         </is>
       </c>
       <c r="F128" s="12" t="inlineStr">
         <is>
-          <t>Accuracy/Valuation</t>
+          <t>Valuation</t>
         </is>
       </c>
       <c r="G128" s="12" t="inlineStr">
         <is>
-          <t>FX rate maker-checker (SoD): a MANUALLY-entered rate lands as PendingApproval and is EXCLUDED from rate resolution — revaluation, the unrealized-FX report, and consolidation translation all use APPROVED rates only — until a DIFFERENT user approves it (POST /api/fx/rates/approve). Self-approval → SOD_VIOLATION (binds even Admin); reject marks the rate Rejected (never usable); re-entering a rate sends it back to PendingApproval. Externally-sourced (feed) rates carrying an explicit non-manual source are auto-approved. Pending rates are also surfaced, aged, by the pending-approvals monitor (GOV-01).</t>
+          <t>FX revaluation at period-end rates; unrealized FX posted (acct 5400).</t>
         </is>
       </c>
       <c r="H128" s="13" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="I128" s="13" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Period-end</t>
         </is>
       </c>
       <c r="J128" s="13" t="inlineStr">
         <is>
-          <t>Per rate</t>
+          <t>Period</t>
         </is>
       </c>
       <c r="K128" s="12" t="inlineStr">
         <is>
-          <t>Controller / Treasury</t>
+          <t>Controller</t>
         </is>
       </c>
       <c r="L128" s="13" t="inlineStr">
@@ -11992,22 +11992,22 @@
       </c>
       <c r="M128" s="12" t="inlineStr">
         <is>
-          <t>fx.service.ts setRate(manual→PendingApproval)/approveRate/rejectRate/rateAsOf(Approved only); fx.controller.ts (rates/approve|reject|pending gated approvals/gl_close); consolidation.service.ts (translation reads Approved rates); schema/fx.ts fx_rates.status + migration 0141; cutover/fxreval.ts (ToE)</t>
+          <t>fx.service.ts (revalue / unrealized report)</t>
         </is>
       </c>
       <c r="N128" s="12" t="inlineStr">
         <is>
-          <t>Inspect the request→approve flow + the approver≠requester check + that revaluation/reporting resolve Approved rates only.</t>
+          <t>Inspect reval logic + rates.</t>
         </is>
       </c>
       <c r="O128" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: enter a manual rate (PendingApproval), confirm revalue is blocked NO_RATE while pending, attempt self-approve (SOD_VIOLATION), approve as a different user, then revalue succeeds (re-performed by the fxreval harness).</t>
+          <t>Recompute reval on sample balances.</t>
         </is>
       </c>
       <c r="P128" s="12" t="inlineStr">
         <is>
-          <t>FX rate approval log + SoD test</t>
+          <t>FX reval JE</t>
         </is>
       </c>
       <c r="Q128" s="18" t="inlineStr">
@@ -12019,92 +12019,179 @@
     <row r="129">
       <c r="A129" s="15" t="inlineStr">
         <is>
+          <t>FX-04</t>
+        </is>
+      </c>
+      <c r="B129" s="16" t="inlineStr">
+        <is>
+          <t>Consolidation &amp; FX</t>
+        </is>
+      </c>
+      <c r="C129" s="17" t="inlineStr">
+        <is>
+          <t>Application</t>
+        </is>
+      </c>
+      <c r="D129" s="16" t="inlineStr">
+        <is>
+          <t>FX gain/loss; Revenue; AR/AP</t>
+        </is>
+      </c>
+      <c r="E129" s="16" t="inlineStr">
+        <is>
+          <t>A wrong manually-entered FX rate (fat-fingered, e.g. USD 36 keyed as 63) flows straight into a period-end revaluation JE and the unrealized-FX report with no independent review — mis-stating earnings/equity and FX-translated balances.</t>
+        </is>
+      </c>
+      <c r="F129" s="16" t="inlineStr">
+        <is>
+          <t>Accuracy/Valuation</t>
+        </is>
+      </c>
+      <c r="G129" s="16" t="inlineStr">
+        <is>
+          <t>FX rate maker-checker (SoD): a MANUALLY-entered rate lands as PendingApproval and is EXCLUDED from rate resolution — revaluation, the unrealized-FX report, and consolidation translation all use APPROVED rates only — until a DIFFERENT user approves it (POST /api/fx/rates/approve). Self-approval → SOD_VIOLATION (binds even Admin); reject marks the rate Rejected (never usable); re-entering a rate sends it back to PendingApproval. Externally-sourced (feed) rates carrying an explicit non-manual source are auto-approved. Pending rates are also surfaced, aged, by the pending-approvals monitor (GOV-01).</t>
+        </is>
+      </c>
+      <c r="H129" s="17" t="inlineStr">
+        <is>
+          <t>Prev</t>
+        </is>
+      </c>
+      <c r="I129" s="17" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="J129" s="17" t="inlineStr">
+        <is>
+          <t>Per rate</t>
+        </is>
+      </c>
+      <c r="K129" s="16" t="inlineStr">
+        <is>
+          <t>Controller / Treasury</t>
+        </is>
+      </c>
+      <c r="L129" s="17" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="M129" s="16" t="inlineStr">
+        <is>
+          <t>fx.service.ts setRate(manual→PendingApproval)/approveRate/rejectRate/rateAsOf(Approved only); fx.controller.ts (rates/approve|reject|pending gated approvals/gl_close); consolidation.service.ts (translation reads Approved rates); schema/fx.ts fx_rates.status + migration 0141; cutover/fxreval.ts (ToE)</t>
+        </is>
+      </c>
+      <c r="N129" s="16" t="inlineStr">
+        <is>
+          <t>Inspect the request→approve flow + the approver≠requester check + that revaluation/reporting resolve Approved rates only.</t>
+        </is>
+      </c>
+      <c r="O129" s="16" t="inlineStr">
+        <is>
+          <t>Re-perform: enter a manual rate (PendingApproval), confirm revalue is blocked NO_RATE while pending, attempt self-approve (SOD_VIOLATION), approve as a different user, then revalue succeeds (re-performed by the fxreval harness).</t>
+        </is>
+      </c>
+      <c r="P129" s="16" t="inlineStr">
+        <is>
+          <t>FX rate approval log + SoD test</t>
+        </is>
+      </c>
+      <c r="Q129" s="18" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="11" t="inlineStr">
+        <is>
           <t>BUD-01</t>
         </is>
       </c>
-      <c r="B129" s="16" t="inlineStr">
+      <c r="B130" s="12" t="inlineStr">
         <is>
           <t>Budgeting &amp; Planning</t>
         </is>
       </c>
-      <c r="C129" s="17" t="inlineStr">
+      <c r="C130" s="13" t="inlineStr">
         <is>
           <t>Application</t>
         </is>
       </c>
-      <c r="D129" s="16" t="inlineStr">
+      <c r="D130" s="12" t="inlineStr">
         <is>
           <t>Budget; All (variance reporting)</t>
         </is>
       </c>
-      <c r="E129" s="16" t="inlineStr">
+      <c r="E130" s="12" t="inlineStr">
         <is>
           <t>A budget figure is entered/changed by one person and immediately drives the budget-vs-actual variance report — the basis for spend authorization and performance review — with no independent approval; a wrong or self-serving budget makes overspending look 'on budget'.</t>
         </is>
       </c>
-      <c r="F129" s="16" t="inlineStr">
+      <c r="F130" s="12" t="inlineStr">
         <is>
           <t>Authorization/Accuracy</t>
         </is>
       </c>
-      <c r="G129" s="16" t="inlineStr">
+      <c r="G130" s="12" t="inlineStr">
         <is>
           <t>Budget maker-checker (SoD): an upserted budget (POST /api/ledger/budgets) lands as PendingApproval and is EXCLUDED from budget-vs-actual until a DIFFERENT user approves it (POST /api/ledger/budgets/approve for the fiscal_year/account/cost-centre[/period]). Self-approval → SOD_VIOLATION (binds even Admin); reject marks it Rejected (excluded). DEFAULT 'Approved' keeps existing rows + direct planning seeds usable. Pending budgets are also surfaced, aged, by the pending-approvals monitor (GOV-01).</t>
         </is>
       </c>
-      <c r="H129" s="17" t="inlineStr">
+      <c r="H130" s="13" t="inlineStr">
         <is>
           <t>Prev</t>
         </is>
       </c>
-      <c r="I129" s="17" t="inlineStr">
+      <c r="I130" s="13" t="inlineStr">
         <is>
           <t>Automated</t>
         </is>
       </c>
-      <c r="J129" s="17" t="inlineStr">
+      <c r="J130" s="13" t="inlineStr">
         <is>
           <t>Per budget</t>
         </is>
       </c>
-      <c r="K129" s="16" t="inlineStr">
+      <c r="K130" s="12" t="inlineStr">
         <is>
           <t>Controller / FP&amp;A</t>
         </is>
       </c>
-      <c r="L129" s="17" t="inlineStr">
+      <c r="L130" s="13" t="inlineStr">
         <is>
           <t>P10</t>
         </is>
       </c>
-      <c r="M129" s="16" t="inlineStr">
+      <c r="M130" s="12" t="inlineStr">
         <is>
           <t>budget.service.ts upsertBudget(→PendingApproval)/approveBudget/rejectBudget/budgetVsActual(Approved only); budget.controller.ts (budgets/approve|reject|pending gated approvals/gl_close); schema/budgets.ts budgets.status + migration 0142; cutover/budget.ts (ToE)</t>
         </is>
       </c>
-      <c r="N129" s="16" t="inlineStr">
+      <c r="N130" s="12" t="inlineStr">
         <is>
           <t>Inspect the request→approve flow + the approver≠requester check + that budget-vs-actual counts Approved budgets only.</t>
         </is>
       </c>
-      <c r="O129" s="16" t="inlineStr">
+      <c r="O130" s="12" t="inlineStr">
         <is>
           <t>Re-perform: upsert a budget (PendingApproval, excluded from variance), attempt self-approve (SOD_VIOLATION), approve as a different user, confirm it then appears in budget-vs-actual (re-performed by the budget harness).</t>
         </is>
       </c>
-      <c r="P129" s="16" t="inlineStr">
+      <c r="P130" s="12" t="inlineStr">
         <is>
           <t>Budget approval log + SoD test</t>
         </is>
       </c>
-      <c r="Q129" s="18" t="inlineStr">
+      <c r="Q130" s="18" t="inlineStr">
         <is>
           <t>Implemented</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q129"/>
+  <autoFilter ref="A1:Q130"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -13287,7 +13374,7 @@
         </is>
       </c>
       <c r="C5" s="29">
-        <f>COUNTIF(RCM!$Q$2:$Q$129,B5)</f>
+        <f>COUNTIF(RCM!$Q$2:$Q$130,B5)</f>
         <v/>
       </c>
     </row>
@@ -13298,7 +13385,7 @@
         </is>
       </c>
       <c r="C6" s="29">
-        <f>COUNTIF(RCM!$Q$2:$Q$129,B6)</f>
+        <f>COUNTIF(RCM!$Q$2:$Q$130,B6)</f>
         <v/>
       </c>
     </row>
@@ -13309,7 +13396,7 @@
         </is>
       </c>
       <c r="C7" s="29">
-        <f>COUNTIF(RCM!$Q$2:$Q$129,B7)</f>
+        <f>COUNTIF(RCM!$Q$2:$Q$130,B7)</f>
         <v/>
       </c>
     </row>
@@ -13320,7 +13407,7 @@
         </is>
       </c>
       <c r="C8" s="32">
-        <f>COUNTA(RCM!$A$2:$A$129)</f>
+        <f>COUNTA(RCM!$A$2:$A$130)</f>
         <v/>
       </c>
     </row>
@@ -13338,7 +13425,7 @@
         </is>
       </c>
       <c r="C11" s="29">
-        <f>COUNTIF(RCM!$C$2:$C$129,B11)</f>
+        <f>COUNTIF(RCM!$C$2:$C$130,B11)</f>
         <v/>
       </c>
     </row>
@@ -13349,7 +13436,7 @@
         </is>
       </c>
       <c r="C12" s="29">
-        <f>COUNTIF(RCM!$C$2:$C$129,B12)</f>
+        <f>COUNTIF(RCM!$C$2:$C$130,B12)</f>
         <v/>
       </c>
     </row>
@@ -13360,7 +13447,7 @@
         </is>
       </c>
       <c r="C13" s="29">
-        <f>COUNTIF(RCM!$C$2:$C$129,B13)</f>
+        <f>COUNTIF(RCM!$C$2:$C$130,B13)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(gl): WS3.3 — consolidation eliminations + segment reporting (CON-03, CON-04)
Extends the existing CON-01 consolidation module (groups/FX-translation/NCI).
- consol_elimination_rules + segment_definitions tables; consolidation_runs
  gains balanced/posted_by/posted_at (migration 0170)
- runConsolidation asserts group TB balances (CONSOL_UNBALANCED, rollback);
  ALREADY_POSTED guard; postConsolidation maker-checker (SELF_POST)
- IC eliminations (1150/2150) net reciprocals to zero at group layer only
- segmentReport: IFRS 8 P&L by branch/project/dept via segment_definitions
- consolidation 26/26, intercompany 16/16, basics 201/201, worldclass 57/57
- CON-03 + CON-04 RCM (131); narrative 11 + user-manual + UAT

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/compliance/Oshinei_ERP_SOX_RCM_v1.xlsx
+++ b/compliance/Oshinei_ERP_SOX_RCM_v1.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'RCM'!$A$1:$Q$130</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'RCM'!$A$1:$Q$132</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Gap Remediation'!$A$2:$H$18</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -858,7 +858,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q130"/>
+  <dimension ref="A1:Q132"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -12019,7 +12019,7 @@
     <row r="129">
       <c r="A129" s="15" t="inlineStr">
         <is>
-          <t>FX-04</t>
+          <t>CON-03</t>
         </is>
       </c>
       <c r="B129" s="16" t="inlineStr">
@@ -12034,22 +12034,22 @@
       </c>
       <c r="D129" s="16" t="inlineStr">
         <is>
-          <t>FX gain/loss; Revenue; AR/AP</t>
+          <t>Consolidation</t>
         </is>
       </c>
       <c r="E129" s="16" t="inlineStr">
         <is>
-          <t>A wrong manually-entered FX rate (fat-fingered, e.g. USD 36 keyed as 63) flows straight into a period-end revaluation JE and the unrealized-FX report with no independent review — mis-stating earnings/equity and FX-translated balances.</t>
+          <t>Intercompany balances/transactions are not eliminated on consolidation, OR eliminations are mis-stated, so the consolidated group trial balance does not balance and group financials are overstated (IC double-counted).</t>
         </is>
       </c>
       <c r="F129" s="16" t="inlineStr">
         <is>
-          <t>Accuracy/Valuation</t>
+          <t>Accuracy/Completeness</t>
         </is>
       </c>
       <c r="G129" s="16" t="inlineStr">
         <is>
-          <t>FX rate maker-checker (SoD): a MANUALLY-entered rate lands as PendingApproval and is EXCLUDED from rate resolution — revaluation, the unrealized-FX report, and consolidation translation all use APPROVED rates only — until a DIFFERENT user approves it (POST /api/fx/rates/approve). Self-approval → SOD_VIOLATION (binds even Admin); reject marks the rate Rejected (never usable); re-entering a rate sends it back to PendingApproval. Externally-sourced (feed) rates carrying an explicit non-manual source are auto-approved. Pending rates are also surfaced, aged, by the pending-approvals monitor (GOV-01).</t>
+          <t>Elimination integrity (CON-03): runConsolidation combines member-entity TBs, generates reciprocal IC eliminations (Dr 2150 Due-To / Cr 1150 Due-From for each in-group IC transaction) at the GROUP layer (consolidation_run_lines — NOT pushed into any operating entity's GL), and ASSERTS the consolidated TB still balances (Σ signed nets ~0 and eliminations net to 0, NCI presentation reclass excluded) — failure throws CONSOL_UNBALANCED and rolls back the run. A balanced run is finalised, then frozen by a DIFFERENT user via run→post maker-checker (self-post → SELF_POST; re-running a Posted period → ALREADY_POSTED; one run per (group, period)). HQ/Admin-only; reads across member tenants via app.bypass_rls. Configurable elimination rules (consol_elimination_rules).</t>
         </is>
       </c>
       <c r="H129" s="17" t="inlineStr">
@@ -12059,17 +12059,17 @@
       </c>
       <c r="I129" s="17" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="J129" s="17" t="inlineStr">
         <is>
-          <t>Per rate</t>
+          <t>Period</t>
         </is>
       </c>
       <c r="K129" s="16" t="inlineStr">
         <is>
-          <t>Controller / Treasury</t>
+          <t>Group Controller</t>
         </is>
       </c>
       <c r="L129" s="17" t="inlineStr">
@@ -12079,22 +12079,22 @@
       </c>
       <c r="M129" s="16" t="inlineStr">
         <is>
-          <t>fx.service.ts setRate(manual→PendingApproval)/approveRate/rejectRate/rateAsOf(Approved only); fx.controller.ts (rates/approve|reject|pending gated approvals/gl_close); consolidation.service.ts (translation reads Approved rates); schema/fx.ts fx_rates.status + migration 0141; cutover/fxreval.ts (ToE)</t>
+          <t>consolidation.service.ts runConsolidation (balanced check, CONSOL_UNBALANCED)/postConsolidation (SELF_POST, ALREADY_POSTED); consolidation.controller.ts (run @approvals, runs/:id/post @approvals); schema/consolidation.ts (consolidation_runs.balanced/posted_by, consol_elimination_rules) + migration 0170; cutover/consolidation.ts (ToE)</t>
         </is>
       </c>
       <c r="N129" s="16" t="inlineStr">
         <is>
-          <t>Inspect the request→approve flow + the approver≠requester check + that revaluation/reporting resolve Approved rates only.</t>
+          <t>Inspect the combine→eliminate→balance flow, the CONSOL_UNBALANCED guard, and the run→post approver≠runner check.</t>
         </is>
       </c>
       <c r="O129" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: enter a manual rate (PendingApproval), confirm revalue is blocked NO_RATE while pending, attempt self-approve (SOD_VIOLATION), approve as a different user, then revalue succeeds (re-performed by the fxreval harness).</t>
+          <t>Re-perform: run a group consolidation, confirm IC 1150/2150 eliminate and the consolidated TB balances; attempt self-post (SELF_POST); post as a different user (Posted); re-run the posted period (ALREADY_POSTED). Re-performed by the consolidation harness.</t>
         </is>
       </c>
       <c r="P129" s="16" t="inlineStr">
         <is>
-          <t>FX rate approval log + SoD test</t>
+          <t>Consolidated TB + elimination lines + post log</t>
         </is>
       </c>
       <c r="Q129" s="18" t="inlineStr">
@@ -12106,92 +12106,266 @@
     <row r="130">
       <c r="A130" s="11" t="inlineStr">
         <is>
+          <t>CON-04</t>
+        </is>
+      </c>
+      <c r="B130" s="12" t="inlineStr">
+        <is>
+          <t>Consolidation &amp; FX</t>
+        </is>
+      </c>
+      <c r="C130" s="13" t="inlineStr">
+        <is>
+          <t>Application</t>
+        </is>
+      </c>
+      <c r="D130" s="12" t="inlineStr">
+        <is>
+          <t>All (segment disclosure)</t>
+        </is>
+      </c>
+      <c r="E130" s="12" t="inlineStr">
+        <is>
+          <t>Segment (branch/project/department) operating results are not reported, so IFRS 8 segment disclosure is incomplete or inaccurate and management/investors cannot see results by reportable segment.</t>
+        </is>
+      </c>
+      <c r="F130" s="12" t="inlineStr">
+        <is>
+          <t>Presentation/Disclosure</t>
+        </is>
+      </c>
+      <c r="G130" s="12" t="inlineStr">
+        <is>
+          <t>Segment reporting (CON-04, IFRS 8): segmentReport produces P&amp;L (revenue/expense/net) grouped by reportable segment, sourced from the dimension columns on journal_lines (branch_id/project_id/department_id) and mapped through configurable segment_definitions (member_keys → segment); unmapped dimension values surface as their own/Unassigned bucket. HQ/Admin-only, gated 'exec'.</t>
+        </is>
+      </c>
+      <c r="H130" s="13" t="inlineStr">
+        <is>
+          <t>Det</t>
+        </is>
+      </c>
+      <c r="I130" s="13" t="inlineStr">
+        <is>
+          <t>Auto+Manual</t>
+        </is>
+      </c>
+      <c r="J130" s="13" t="inlineStr">
+        <is>
+          <t>Period</t>
+        </is>
+      </c>
+      <c r="K130" s="12" t="inlineStr">
+        <is>
+          <t>Group Controller</t>
+        </is>
+      </c>
+      <c r="L130" s="13" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="M130" s="12" t="inlineStr">
+        <is>
+          <t>consolidation.service.ts defineSegment/listSegments/segmentReport; consolidation.controller.ts (segments, segment-report @exec); schema/consolidation.ts segment_definitions + migration 0170; cutover/consolidation.ts (ToE)</t>
+        </is>
+      </c>
+      <c r="N130" s="12" t="inlineStr">
+        <is>
+          <t>Inspect the segment mapping + the dimension-grouped P&amp;L aggregation.</t>
+        </is>
+      </c>
+      <c r="O130" s="12" t="inlineStr">
+        <is>
+          <t>Re-perform: define a segment over branches, run the segment report for a period, confirm revenue/expense/net tie to the underlying dimensioned postings. Re-performed by the consolidation harness.</t>
+        </is>
+      </c>
+      <c r="P130" s="12" t="inlineStr">
+        <is>
+          <t>Segment P&amp;L report</t>
+        </is>
+      </c>
+      <c r="Q130" s="18" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="15" t="inlineStr">
+        <is>
+          <t>FX-04</t>
+        </is>
+      </c>
+      <c r="B131" s="16" t="inlineStr">
+        <is>
+          <t>Consolidation &amp; FX</t>
+        </is>
+      </c>
+      <c r="C131" s="17" t="inlineStr">
+        <is>
+          <t>Application</t>
+        </is>
+      </c>
+      <c r="D131" s="16" t="inlineStr">
+        <is>
+          <t>FX gain/loss; Revenue; AR/AP</t>
+        </is>
+      </c>
+      <c r="E131" s="16" t="inlineStr">
+        <is>
+          <t>A wrong manually-entered FX rate (fat-fingered, e.g. USD 36 keyed as 63) flows straight into a period-end revaluation JE and the unrealized-FX report with no independent review — mis-stating earnings/equity and FX-translated balances.</t>
+        </is>
+      </c>
+      <c r="F131" s="16" t="inlineStr">
+        <is>
+          <t>Accuracy/Valuation</t>
+        </is>
+      </c>
+      <c r="G131" s="16" t="inlineStr">
+        <is>
+          <t>FX rate maker-checker (SoD): a MANUALLY-entered rate lands as PendingApproval and is EXCLUDED from rate resolution — revaluation, the unrealized-FX report, and consolidation translation all use APPROVED rates only — until a DIFFERENT user approves it (POST /api/fx/rates/approve). Self-approval → SOD_VIOLATION (binds even Admin); reject marks the rate Rejected (never usable); re-entering a rate sends it back to PendingApproval. Externally-sourced (feed) rates carrying an explicit non-manual source are auto-approved. Pending rates are also surfaced, aged, by the pending-approvals monitor (GOV-01).</t>
+        </is>
+      </c>
+      <c r="H131" s="17" t="inlineStr">
+        <is>
+          <t>Prev</t>
+        </is>
+      </c>
+      <c r="I131" s="17" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="J131" s="17" t="inlineStr">
+        <is>
+          <t>Per rate</t>
+        </is>
+      </c>
+      <c r="K131" s="16" t="inlineStr">
+        <is>
+          <t>Controller / Treasury</t>
+        </is>
+      </c>
+      <c r="L131" s="17" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="M131" s="16" t="inlineStr">
+        <is>
+          <t>fx.service.ts setRate(manual→PendingApproval)/approveRate/rejectRate/rateAsOf(Approved only); fx.controller.ts (rates/approve|reject|pending gated approvals/gl_close); consolidation.service.ts (translation reads Approved rates); schema/fx.ts fx_rates.status + migration 0141; cutover/fxreval.ts (ToE)</t>
+        </is>
+      </c>
+      <c r="N131" s="16" t="inlineStr">
+        <is>
+          <t>Inspect the request→approve flow + the approver≠requester check + that revaluation/reporting resolve Approved rates only.</t>
+        </is>
+      </c>
+      <c r="O131" s="16" t="inlineStr">
+        <is>
+          <t>Re-perform: enter a manual rate (PendingApproval), confirm revalue is blocked NO_RATE while pending, attempt self-approve (SOD_VIOLATION), approve as a different user, then revalue succeeds (re-performed by the fxreval harness).</t>
+        </is>
+      </c>
+      <c r="P131" s="16" t="inlineStr">
+        <is>
+          <t>FX rate approval log + SoD test</t>
+        </is>
+      </c>
+      <c r="Q131" s="18" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="11" t="inlineStr">
+        <is>
           <t>BUD-01</t>
         </is>
       </c>
-      <c r="B130" s="12" t="inlineStr">
+      <c r="B132" s="12" t="inlineStr">
         <is>
           <t>Budgeting &amp; Planning</t>
         </is>
       </c>
-      <c r="C130" s="13" t="inlineStr">
+      <c r="C132" s="13" t="inlineStr">
         <is>
           <t>Application</t>
         </is>
       </c>
-      <c r="D130" s="12" t="inlineStr">
+      <c r="D132" s="12" t="inlineStr">
         <is>
           <t>Budget; All (variance reporting)</t>
         </is>
       </c>
-      <c r="E130" s="12" t="inlineStr">
+      <c r="E132" s="12" t="inlineStr">
         <is>
           <t>A budget figure is entered/changed by one person and immediately drives the budget-vs-actual variance report — the basis for spend authorization and performance review — with no independent approval; a wrong or self-serving budget makes overspending look 'on budget'.</t>
         </is>
       </c>
-      <c r="F130" s="12" t="inlineStr">
+      <c r="F132" s="12" t="inlineStr">
         <is>
           <t>Authorization/Accuracy</t>
         </is>
       </c>
-      <c r="G130" s="12" t="inlineStr">
+      <c r="G132" s="12" t="inlineStr">
         <is>
           <t>Budget maker-checker (SoD): an upserted budget (POST /api/ledger/budgets) lands as PendingApproval and is EXCLUDED from budget-vs-actual until a DIFFERENT user approves it (POST /api/ledger/budgets/approve for the fiscal_year/account/cost-centre[/period]). Self-approval → SOD_VIOLATION (binds even Admin); reject marks it Rejected (excluded). DEFAULT 'Approved' keeps existing rows + direct planning seeds usable. Pending budgets are also surfaced, aged, by the pending-approvals monitor (GOV-01).</t>
         </is>
       </c>
-      <c r="H130" s="13" t="inlineStr">
+      <c r="H132" s="13" t="inlineStr">
         <is>
           <t>Prev</t>
         </is>
       </c>
-      <c r="I130" s="13" t="inlineStr">
+      <c r="I132" s="13" t="inlineStr">
         <is>
           <t>Automated</t>
         </is>
       </c>
-      <c r="J130" s="13" t="inlineStr">
+      <c r="J132" s="13" t="inlineStr">
         <is>
           <t>Per budget</t>
         </is>
       </c>
-      <c r="K130" s="12" t="inlineStr">
+      <c r="K132" s="12" t="inlineStr">
         <is>
           <t>Controller / FP&amp;A</t>
         </is>
       </c>
-      <c r="L130" s="13" t="inlineStr">
+      <c r="L132" s="13" t="inlineStr">
         <is>
           <t>P10</t>
         </is>
       </c>
-      <c r="M130" s="12" t="inlineStr">
+      <c r="M132" s="12" t="inlineStr">
         <is>
           <t>budget.service.ts upsertBudget(→PendingApproval)/approveBudget/rejectBudget/budgetVsActual(Approved only); budget.controller.ts (budgets/approve|reject|pending gated approvals/gl_close); schema/budgets.ts budgets.status + migration 0142; cutover/budget.ts (ToE)</t>
         </is>
       </c>
-      <c r="N130" s="12" t="inlineStr">
+      <c r="N132" s="12" t="inlineStr">
         <is>
           <t>Inspect the request→approve flow + the approver≠requester check + that budget-vs-actual counts Approved budgets only.</t>
         </is>
       </c>
-      <c r="O130" s="12" t="inlineStr">
+      <c r="O132" s="12" t="inlineStr">
         <is>
           <t>Re-perform: upsert a budget (PendingApproval, excluded from variance), attempt self-approve (SOD_VIOLATION), approve as a different user, confirm it then appears in budget-vs-actual (re-performed by the budget harness).</t>
         </is>
       </c>
-      <c r="P130" s="12" t="inlineStr">
+      <c r="P132" s="12" t="inlineStr">
         <is>
           <t>Budget approval log + SoD test</t>
         </is>
       </c>
-      <c r="Q130" s="18" t="inlineStr">
+      <c r="Q132" s="18" t="inlineStr">
         <is>
           <t>Implemented</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q130"/>
+  <autoFilter ref="A1:Q132"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -13374,7 +13548,7 @@
         </is>
       </c>
       <c r="C5" s="29">
-        <f>COUNTIF(RCM!$Q$2:$Q$130,B5)</f>
+        <f>COUNTIF(RCM!$Q$2:$Q$132,B5)</f>
         <v/>
       </c>
     </row>
@@ -13385,7 +13559,7 @@
         </is>
       </c>
       <c r="C6" s="29">
-        <f>COUNTIF(RCM!$Q$2:$Q$130,B6)</f>
+        <f>COUNTIF(RCM!$Q$2:$Q$132,B6)</f>
         <v/>
       </c>
     </row>
@@ -13396,7 +13570,7 @@
         </is>
       </c>
       <c r="C7" s="29">
-        <f>COUNTIF(RCM!$Q$2:$Q$130,B7)</f>
+        <f>COUNTIF(RCM!$Q$2:$Q$132,B7)</f>
         <v/>
       </c>
     </row>
@@ -13407,7 +13581,7 @@
         </is>
       </c>
       <c r="C8" s="32">
-        <f>COUNTA(RCM!$A$2:$A$130)</f>
+        <f>COUNTA(RCM!$A$2:$A$132)</f>
         <v/>
       </c>
     </row>
@@ -13425,7 +13599,7 @@
         </is>
       </c>
       <c r="C11" s="29">
-        <f>COUNTIF(RCM!$C$2:$C$130,B11)</f>
+        <f>COUNTIF(RCM!$C$2:$C$132,B11)</f>
         <v/>
       </c>
     </row>
@@ -13436,7 +13610,7 @@
         </is>
       </c>
       <c r="C12" s="29">
-        <f>COUNTIF(RCM!$C$2:$C$130,B12)</f>
+        <f>COUNTIF(RCM!$C$2:$C$132,B12)</f>
         <v/>
       </c>
     </row>
@@ -13447,7 +13621,7 @@
         </is>
       </c>
       <c r="C13" s="29">
-        <f>COUNTIF(RCM!$C$2:$C$130,B13)</f>
+        <f>COUNTIF(RCM!$C$2:$C$132,B13)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: merge main, renumber consolidation 0170→0171 (clock_integrity took 0170)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/compliance/Oshinei_ERP_SOX_RCM_v1.xlsx
+++ b/compliance/Oshinei_ERP_SOX_RCM_v1.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'RCM'!$A$1:$Q$132</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'RCM'!$A$1:$Q$133</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Gap Remediation'!$A$2:$H$18</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -858,7 +858,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q132"/>
+  <dimension ref="A1:Q133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -11671,12 +11671,12 @@
     <row r="125">
       <c r="A125" s="15" t="inlineStr">
         <is>
-          <t>FA-09</t>
+          <t>PAY-05</t>
         </is>
       </c>
       <c r="B125" s="16" t="inlineStr">
         <is>
-          <t>Fixed Assets</t>
+          <t>Payroll</t>
         </is>
       </c>
       <c r="C125" s="17" t="inlineStr">
@@ -11686,27 +11686,27 @@
       </c>
       <c r="D125" s="16" t="inlineStr">
         <is>
-          <t>Property, Plant &amp; Equipment; Cash</t>
+          <t>Payroll expense; Labor hours</t>
         </is>
       </c>
       <c r="E125" s="16" t="inlineStr">
         <is>
-          <t>Asset disposed without independent review — one person writes an asset off the books and records the proceeds (asset-stripping / theft: dispose a still-held asset, or to a related party below value).</t>
+          <t>Time-and-attendance is unverified — one worker clocks a colleague in/out (buddy punching), or punches off-site, so paid labor hours overstate hours actually worked (payroll fraud / inflated labor cost), and there is no attributable override trail when a manager fixes a punch.</t>
         </is>
       </c>
       <c r="F125" s="16" t="inlineStr">
         <is>
-          <t>Authorization</t>
+          <t>Existence/Accuracy/Authorization</t>
         </is>
       </c>
       <c r="G125" s="16" t="inlineStr">
         <is>
-          <t>Asset-disposal maker-checker (SoD): a disposal REQUEST posts its GL entry as a DRAFT (excluded from balances) and flags the asset disposal_pending WITHOUT marking it disposed or moving the register; a DIFFERENT user must approve before it is effective (status→disposed, revaluation surplus recycled 3200→3100) (approver ≠ requester enforced regardless of permissions, reusing the GL-05 ledger approval). Reject voids the draft and the asset stays in service; only one disposal may be pending per asset; a disposal-pending asset is frozen from depreciation.</t>
+          <t>Clock-in integrity (anti-buddy-punch): a punch records its capture METHOD (PIN/QR/FACE_HASH/SUPERVISOR) and optional GPS; a re-punch within 15 minutes of the same employee's last clock-out is REJECTED (DUPLICATE_PUNCH) unless a supervisor overrides. A per-branch geofence_zone (lat/lng/radius) lets the clock-in compute geofence_pass when GPS is supplied; an out-of-fence punch is accepted but FLAGGED (geofence_pass=false) for review rather than hard-blocked (kiosks may lack GPS -&gt; null), and a SUPERVISOR override REQUIRES a reason (REASON_REQUIRED), stamps method=SUPERVISOR + the reason on the punch note, and is captured by the append-only audit_log so every override is attributable. The labor report surfaces method + geofence_pass so anomalies are visible. Tenant-scoped (RLS); gated pos/users/exec.</t>
         </is>
       </c>
       <c r="H125" s="17" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Prev/Det</t>
         </is>
       </c>
       <c r="I125" s="17" t="inlineStr">
@@ -11716,37 +11716,37 @@
       </c>
       <c r="J125" s="17" t="inlineStr">
         <is>
-          <t>Per disposal</t>
+          <t>Per punch</t>
         </is>
       </c>
       <c r="K125" s="16" t="inlineStr">
         <is>
-          <t>FaAccountant / Controller</t>
+          <t>HR / Store Ops Mgr</t>
         </is>
       </c>
       <c r="L125" s="17" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P10/P13</t>
         </is>
       </c>
       <c r="M125" s="16" t="inlineStr">
         <is>
-          <t>assets.service.ts dispose(pendingApproval Draft)/approveDisposal/rejectDisposal; assets.controller.ts (:assetNo/dispose/approve|reject); schema/assets.ts fixed_assets.disposal_pending + migration 0135; cutover/basics.ts + worldclass.ts + compliance.ts (ToE)</t>
+          <t>pos-loyalty-labor/timeclock.service.ts clockIn (DUPLICATE_PUNCH window, method capture, haversine geofence_pass) + supervisorOverride (REASON_REQUIRED, audited) + setGeofenceZone/listGeofenceZones; pos-loyalty-labor.controller.ts (clock-in, clock-in/override, geofence-zones); schema/pos-scale.ts time_clock.clock_in_method/lat/lng/geofence_pass + geofence_zones + migration 0169; cutover/pos-p2.ts (ToE)</t>
         </is>
       </c>
       <c r="N125" s="16" t="inlineStr">
         <is>
-          <t>Inspect Draft→approve flow + the approver≠requester check + deferred status/recycle.</t>
+          <t>Inspect the 15-min duplicate-punch guard, the method capture, the geofence pass/fail computation, and the supervisor-override reason + audit trail.</t>
         </is>
       </c>
       <c r="O125" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: request a disposal (Draft JE excluded), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm status→disposed + surplus recycled only after approval (re-performed by the harnesses).</t>
+          <t>Re-perform: a re-punch within 15 min of clock-out -&gt; DUPLICATE_PUNCH; a supervisor override (with a reason) bypasses it and stamps method SUPERVISOR; an override with no reason -&gt; 400; an in-fence GPS punch -&gt; geofence_pass true; an out-of-fence punch is accepted but flagged geofence_pass false (re-performed by the pos-p2 harness).</t>
         </is>
       </c>
       <c r="P125" s="16" t="inlineStr">
         <is>
-          <t>Disposal approval log + SoD test</t>
+          <t>time_clock method/geofence columns + override note; anti-buddy test</t>
         </is>
       </c>
       <c r="Q125" s="18" t="inlineStr">
@@ -11758,7 +11758,7 @@
     <row r="126">
       <c r="A126" s="11" t="inlineStr">
         <is>
-          <t>FA-10</t>
+          <t>FA-09</t>
         </is>
       </c>
       <c r="B126" s="12" t="inlineStr">
@@ -11773,22 +11773,22 @@
       </c>
       <c r="D126" s="12" t="inlineStr">
         <is>
-          <t>Property, Plant &amp; Equipment; Accounts Payable</t>
+          <t>Property, Plant &amp; Equipment; Cash</t>
         </is>
       </c>
       <c r="E126" s="12" t="inlineStr">
         <is>
-          <t>Capital purchases mis-capitalised or capitalised without independent review — the person who receives the goods also decides what enters the asset register and at what cost/useful life (fictitious or over-valued assets; capex/opex mis-classification).</t>
+          <t>Asset disposed without independent review — one person writes an asset off the books and records the proceeds (asset-stripping / theft: dispose a still-held asset, or to a related party below value).</t>
         </is>
       </c>
       <c r="F126" s="12" t="inlineStr">
         <is>
-          <t>Authorization; Accuracy</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="G126" s="12" t="inlineStr">
         <is>
-          <t>Procure-to-Capitalize maker-checker (SoD): a goods-receipt line flagged capital (item-master is_fixed_asset or per-PO-line override) is excluded from inventory capitalisation (1200) at receipt and instead becomes ELIGIBLE for the asset register. Capitalisation is a REQUEST that posts NOTHING to the GL; a DIFFERENT user must approve before the fixed_assets row + acquisition JE (Dr 1500 / Cr 2000) are created (approver ≠ requester enforced regardless of permissions). The created asset carries its source GR/PO for end-to-end PR→PO→GR→FA traceability; a GR line cannot be capitalised twice.</t>
+          <t>Asset-disposal maker-checker (SoD): a disposal REQUEST posts its GL entry as a DRAFT (excluded from balances) and flags the asset disposal_pending WITHOUT marking it disposed or moving the register; a DIFFERENT user must approve before it is effective (status→disposed, revaluation surplus recycled 3200→3100) (approver ≠ requester enforced regardless of permissions, reusing the GL-05 ledger approval). Reject voids the draft and the asset stays in service; only one disposal may be pending per asset; a disposal-pending asset is frozen from depreciation.</t>
         </is>
       </c>
       <c r="H126" s="13" t="inlineStr">
@@ -11803,7 +11803,7 @@
       </c>
       <c r="J126" s="13" t="inlineStr">
         <is>
-          <t>Per capital receipt</t>
+          <t>Per disposal</t>
         </is>
       </c>
       <c r="K126" s="12" t="inlineStr">
@@ -11818,22 +11818,22 @@
       </c>
       <c r="M126" s="12" t="inlineStr">
         <is>
-          <t>assets.service.ts registerFromGr/approveRegistration/rejectRegistration/eligibleFromGr; assets.controller.ts (registrations*); procurement.service.ts createGr (is_capital routing, costing excluded); schema/assets.ts asset_registration_requests + fixed_assets.source_gr_no/po_no + migration 0137; cutover/basics.ts + compliance.ts (ToE)</t>
+          <t>assets.service.ts dispose(pendingApproval Draft)/approveDisposal/rejectDisposal; assets.controller.ts (:assetNo/dispose/approve|reject); schema/assets.ts fixed_assets.disposal_pending + migration 0135; cutover/basics.ts + worldclass.ts + compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N126" s="12" t="inlineStr">
         <is>
-          <t>Inspect the eligible→request→approve flow + approver≠requester check + the inventory-vs-asset routing of capital lines.</t>
+          <t>Inspect Draft→approve flow + the approver≠requester check + deferred status/recycle.</t>
         </is>
       </c>
       <c r="O126" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: receive a capital line, raise a registration (no GL), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm the asset + Dr 1500/Cr 2000 post only after approval and the line cannot be re-registered (re-performed by the harnesses).</t>
+          <t>Re-perform: request a disposal (Draft JE excluded), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm status→disposed + surplus recycled only after approval (re-performed by the harnesses).</t>
         </is>
       </c>
       <c r="P126" s="12" t="inlineStr">
         <is>
-          <t>Capitalization approval log + SoD test</t>
+          <t>Disposal approval log + SoD test</t>
         </is>
       </c>
       <c r="Q126" s="18" t="inlineStr">
@@ -11845,12 +11845,12 @@
     <row r="127">
       <c r="A127" s="15" t="inlineStr">
         <is>
-          <t>CON-01</t>
+          <t>FA-10</t>
         </is>
       </c>
       <c r="B127" s="16" t="inlineStr">
         <is>
-          <t>Consolidation &amp; FX</t>
+          <t>Fixed Assets</t>
         </is>
       </c>
       <c r="C127" s="17" t="inlineStr">
@@ -11860,42 +11860,42 @@
       </c>
       <c r="D127" s="16" t="inlineStr">
         <is>
-          <t>Consolidation</t>
+          <t>Property, Plant &amp; Equipment; Accounts Payable</t>
         </is>
       </c>
       <c r="E127" s="16" t="inlineStr">
         <is>
-          <t>Group consolidation mis-stated (ownership/currency).</t>
+          <t>Capital purchases mis-capitalised or capitalised without independent review — the person who receives the goods also decides what enters the asset register and at what cost/useful life (fictitious or over-valued assets; capex/opex mis-classification).</t>
         </is>
       </c>
       <c r="F127" s="16" t="inlineStr">
         <is>
-          <t>Accuracy</t>
+          <t>Authorization; Accuracy</t>
         </is>
       </c>
       <c r="G127" s="16" t="inlineStr">
         <is>
-          <t>Consolidation run (ownership %, entity currency) gated by 'approvals'.</t>
+          <t>Procure-to-Capitalize maker-checker (SoD): a goods-receipt line flagged capital (item-master is_fixed_asset or per-PO-line override) is excluded from inventory capitalisation (1200) at receipt and instead becomes ELIGIBLE for the asset register. Capitalisation is a REQUEST that posts NOTHING to the GL; a DIFFERENT user must approve before the fixed_assets row + acquisition JE (Dr 1500 / Cr 2000) are created (approver ≠ requester enforced regardless of permissions). The created asset carries its source GR/PO for end-to-end PR→PO→GR→FA traceability; a GR line cannot be capitalised twice.</t>
         </is>
       </c>
       <c r="H127" s="17" t="inlineStr">
         <is>
-          <t>Auto+Manual</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I127" s="17" t="inlineStr">
         <is>
-          <t>Period</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J127" s="17" t="inlineStr">
         <is>
-          <t>Period</t>
+          <t>Per capital receipt</t>
         </is>
       </c>
       <c r="K127" s="16" t="inlineStr">
         <is>
-          <t>Group Controller</t>
+          <t>FaAccountant / Controller</t>
         </is>
       </c>
       <c r="L127" s="17" t="inlineStr">
@@ -11905,22 +11905,22 @@
       </c>
       <c r="M127" s="16" t="inlineStr">
         <is>
-          <t>consolidation.service.ts (runConsolidation @Permissions approvals)</t>
+          <t>assets.service.ts registerFromGr/approveRegistration/rejectRegistration/eligibleFromGr; assets.controller.ts (registrations*); procurement.service.ts createGr (is_capital routing, costing excluded); schema/assets.ts asset_registration_requests + fixed_assets.source_gr_no/po_no + migration 0137; cutover/basics.ts + compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N127" s="16" t="inlineStr">
         <is>
-          <t>Inspect consolidation logic + gate.</t>
+          <t>Inspect the eligible→request→approve flow + approver≠requester check + the inventory-vs-asset routing of capital lines.</t>
         </is>
       </c>
       <c r="O127" s="16" t="inlineStr">
         <is>
-          <t>Sample period: consolidated TB ties to entities.</t>
+          <t>Re-perform: receive a capital line, raise a registration (no GL), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm the asset + Dr 1500/Cr 2000 post only after approval and the line cannot be re-registered (re-performed by the harnesses).</t>
         </is>
       </c>
       <c r="P127" s="16" t="inlineStr">
         <is>
-          <t>Consol TB</t>
+          <t>Capitalization approval log + SoD test</t>
         </is>
       </c>
       <c r="Q127" s="18" t="inlineStr">
@@ -11932,7 +11932,7 @@
     <row r="128">
       <c r="A128" s="11" t="inlineStr">
         <is>
-          <t>CON-02</t>
+          <t>CON-01</t>
         </is>
       </c>
       <c r="B128" s="12" t="inlineStr">
@@ -11947,22 +11947,22 @@
       </c>
       <c r="D128" s="12" t="inlineStr">
         <is>
-          <t>FX gain/loss</t>
+          <t>Consolidation</t>
         </is>
       </c>
       <c r="E128" s="12" t="inlineStr">
         <is>
-          <t>FX exposures not revalued at period-end.</t>
+          <t>Group consolidation mis-stated (ownership/currency).</t>
         </is>
       </c>
       <c r="F128" s="12" t="inlineStr">
         <is>
-          <t>Valuation</t>
+          <t>Accuracy</t>
         </is>
       </c>
       <c r="G128" s="12" t="inlineStr">
         <is>
-          <t>FX revaluation at period-end rates; unrealized FX posted (acct 5400).</t>
+          <t>Consolidation run (ownership %, entity currency) gated by 'approvals'.</t>
         </is>
       </c>
       <c r="H128" s="13" t="inlineStr">
@@ -11972,7 +11972,7 @@
       </c>
       <c r="I128" s="13" t="inlineStr">
         <is>
-          <t>Period-end</t>
+          <t>Period</t>
         </is>
       </c>
       <c r="J128" s="13" t="inlineStr">
@@ -11982,7 +11982,7 @@
       </c>
       <c r="K128" s="12" t="inlineStr">
         <is>
-          <t>Controller</t>
+          <t>Group Controller</t>
         </is>
       </c>
       <c r="L128" s="13" t="inlineStr">
@@ -11992,22 +11992,22 @@
       </c>
       <c r="M128" s="12" t="inlineStr">
         <is>
-          <t>fx.service.ts (revalue / unrealized report)</t>
+          <t>consolidation.service.ts (runConsolidation @Permissions approvals)</t>
         </is>
       </c>
       <c r="N128" s="12" t="inlineStr">
         <is>
-          <t>Inspect reval logic + rates.</t>
+          <t>Inspect consolidation logic + gate.</t>
         </is>
       </c>
       <c r="O128" s="12" t="inlineStr">
         <is>
-          <t>Recompute reval on sample balances.</t>
+          <t>Sample period: consolidated TB ties to entities.</t>
         </is>
       </c>
       <c r="P128" s="12" t="inlineStr">
         <is>
-          <t>FX reval JE</t>
+          <t>Consol TB</t>
         </is>
       </c>
       <c r="Q128" s="18" t="inlineStr">
@@ -12019,7 +12019,7 @@
     <row r="129">
       <c r="A129" s="15" t="inlineStr">
         <is>
-          <t>CON-03</t>
+          <t>CON-02</t>
         </is>
       </c>
       <c r="B129" s="16" t="inlineStr">
@@ -12034,32 +12034,32 @@
       </c>
       <c r="D129" s="16" t="inlineStr">
         <is>
-          <t>Consolidation</t>
+          <t>FX gain/loss</t>
         </is>
       </c>
       <c r="E129" s="16" t="inlineStr">
         <is>
-          <t>Intercompany balances/transactions are not eliminated on consolidation, OR eliminations are mis-stated, so the consolidated group trial balance does not balance and group financials are overstated (IC double-counted).</t>
+          <t>FX exposures not revalued at period-end.</t>
         </is>
       </c>
       <c r="F129" s="16" t="inlineStr">
         <is>
-          <t>Accuracy/Completeness</t>
+          <t>Valuation</t>
         </is>
       </c>
       <c r="G129" s="16" t="inlineStr">
         <is>
-          <t>Elimination integrity (CON-03): runConsolidation combines member-entity TBs, generates reciprocal IC eliminations (Dr 2150 Due-To / Cr 1150 Due-From for each in-group IC transaction) at the GROUP layer (consolidation_run_lines — NOT pushed into any operating entity's GL), and ASSERTS the consolidated TB still balances (Σ signed nets ~0 and eliminations net to 0, NCI presentation reclass excluded) — failure throws CONSOL_UNBALANCED and rolls back the run. A balanced run is finalised, then frozen by a DIFFERENT user via run→post maker-checker (self-post → SELF_POST; re-running a Posted period → ALREADY_POSTED; one run per (group, period)). HQ/Admin-only; reads across member tenants via app.bypass_rls. Configurable elimination rules (consol_elimination_rules).</t>
+          <t>FX revaluation at period-end rates; unrealized FX posted (acct 5400).</t>
         </is>
       </c>
       <c r="H129" s="17" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="I129" s="17" t="inlineStr">
         <is>
-          <t>Auto+Manual</t>
+          <t>Period-end</t>
         </is>
       </c>
       <c r="J129" s="17" t="inlineStr">
@@ -12069,7 +12069,7 @@
       </c>
       <c r="K129" s="16" t="inlineStr">
         <is>
-          <t>Group Controller</t>
+          <t>Controller</t>
         </is>
       </c>
       <c r="L129" s="17" t="inlineStr">
@@ -12079,22 +12079,22 @@
       </c>
       <c r="M129" s="16" t="inlineStr">
         <is>
-          <t>consolidation.service.ts runConsolidation (balanced check, CONSOL_UNBALANCED)/postConsolidation (SELF_POST, ALREADY_POSTED); consolidation.controller.ts (run @approvals, runs/:id/post @approvals); schema/consolidation.ts (consolidation_runs.balanced/posted_by, consol_elimination_rules) + migration 0170; cutover/consolidation.ts (ToE)</t>
+          <t>fx.service.ts (revalue / unrealized report)</t>
         </is>
       </c>
       <c r="N129" s="16" t="inlineStr">
         <is>
-          <t>Inspect the combine→eliminate→balance flow, the CONSOL_UNBALANCED guard, and the run→post approver≠runner check.</t>
+          <t>Inspect reval logic + rates.</t>
         </is>
       </c>
       <c r="O129" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: run a group consolidation, confirm IC 1150/2150 eliminate and the consolidated TB balances; attempt self-post (SELF_POST); post as a different user (Posted); re-run the posted period (ALREADY_POSTED). Re-performed by the consolidation harness.</t>
+          <t>Recompute reval on sample balances.</t>
         </is>
       </c>
       <c r="P129" s="16" t="inlineStr">
         <is>
-          <t>Consolidated TB + elimination lines + post log</t>
+          <t>FX reval JE</t>
         </is>
       </c>
       <c r="Q129" s="18" t="inlineStr">
@@ -12106,7 +12106,7 @@
     <row r="130">
       <c r="A130" s="11" t="inlineStr">
         <is>
-          <t>CON-04</t>
+          <t>CON-03</t>
         </is>
       </c>
       <c r="B130" s="12" t="inlineStr">
@@ -12121,27 +12121,27 @@
       </c>
       <c r="D130" s="12" t="inlineStr">
         <is>
-          <t>All (segment disclosure)</t>
+          <t>Consolidation</t>
         </is>
       </c>
       <c r="E130" s="12" t="inlineStr">
         <is>
-          <t>Segment (branch/project/department) operating results are not reported, so IFRS 8 segment disclosure is incomplete or inaccurate and management/investors cannot see results by reportable segment.</t>
+          <t>Intercompany balances/transactions are not eliminated on consolidation, OR eliminations are mis-stated, so the consolidated group trial balance does not balance and group financials are overstated (IC double-counted).</t>
         </is>
       </c>
       <c r="F130" s="12" t="inlineStr">
         <is>
-          <t>Presentation/Disclosure</t>
+          <t>Accuracy/Completeness</t>
         </is>
       </c>
       <c r="G130" s="12" t="inlineStr">
         <is>
-          <t>Segment reporting (CON-04, IFRS 8): segmentReport produces P&amp;L (revenue/expense/net) grouped by reportable segment, sourced from the dimension columns on journal_lines (branch_id/project_id/department_id) and mapped through configurable segment_definitions (member_keys → segment); unmapped dimension values surface as their own/Unassigned bucket. HQ/Admin-only, gated 'exec'.</t>
+          <t>Elimination integrity (CON-03): runConsolidation combines member-entity TBs, generates reciprocal IC eliminations (Dr 2150 Due-To / Cr 1150 Due-From for each in-group IC transaction) at the GROUP layer (consolidation_run_lines — NOT pushed into any operating entity's GL), and ASSERTS the consolidated TB still balances (Σ signed nets ~0 and eliminations net to 0, NCI presentation reclass excluded) — failure throws CONSOL_UNBALANCED and rolls back the run. A balanced run is finalised, then frozen by a DIFFERENT user via run→post maker-checker (self-post → SELF_POST; re-running a Posted period → ALREADY_POSTED; one run per (group, period)). HQ/Admin-only; reads across member tenants via app.bypass_rls. Configurable elimination rules (consol_elimination_rules).</t>
         </is>
       </c>
       <c r="H130" s="13" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I130" s="13" t="inlineStr">
@@ -12166,22 +12166,22 @@
       </c>
       <c r="M130" s="12" t="inlineStr">
         <is>
-          <t>consolidation.service.ts defineSegment/listSegments/segmentReport; consolidation.controller.ts (segments, segment-report @exec); schema/consolidation.ts segment_definitions + migration 0170; cutover/consolidation.ts (ToE)</t>
+          <t>consolidation.service.ts runConsolidation (balanced check, CONSOL_UNBALANCED)/postConsolidation (SELF_POST, ALREADY_POSTED); consolidation.controller.ts (run @approvals, runs/:id/post @approvals); schema/consolidation.ts (consolidation_runs.balanced/posted_by, consol_elimination_rules) + migration 0170; cutover/consolidation.ts (ToE)</t>
         </is>
       </c>
       <c r="N130" s="12" t="inlineStr">
         <is>
-          <t>Inspect the segment mapping + the dimension-grouped P&amp;L aggregation.</t>
+          <t>Inspect the combine→eliminate→balance flow, the CONSOL_UNBALANCED guard, and the run→post approver≠runner check.</t>
         </is>
       </c>
       <c r="O130" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: define a segment over branches, run the segment report for a period, confirm revenue/expense/net tie to the underlying dimensioned postings. Re-performed by the consolidation harness.</t>
+          <t>Re-perform: run a group consolidation, confirm IC 1150/2150 eliminate and the consolidated TB balances; attempt self-post (SELF_POST); post as a different user (Posted); re-run the posted period (ALREADY_POSTED). Re-performed by the consolidation harness.</t>
         </is>
       </c>
       <c r="P130" s="12" t="inlineStr">
         <is>
-          <t>Segment P&amp;L report</t>
+          <t>Consolidated TB + elimination lines + post log</t>
         </is>
       </c>
       <c r="Q130" s="18" t="inlineStr">
@@ -12193,7 +12193,7 @@
     <row r="131">
       <c r="A131" s="15" t="inlineStr">
         <is>
-          <t>FX-04</t>
+          <t>CON-04</t>
         </is>
       </c>
       <c r="B131" s="16" t="inlineStr">
@@ -12208,42 +12208,42 @@
       </c>
       <c r="D131" s="16" t="inlineStr">
         <is>
-          <t>FX gain/loss; Revenue; AR/AP</t>
+          <t>All (segment disclosure)</t>
         </is>
       </c>
       <c r="E131" s="16" t="inlineStr">
         <is>
-          <t>A wrong manually-entered FX rate (fat-fingered, e.g. USD 36 keyed as 63) flows straight into a period-end revaluation JE and the unrealized-FX report with no independent review — mis-stating earnings/equity and FX-translated balances.</t>
+          <t>Segment (branch/project/department) operating results are not reported, so IFRS 8 segment disclosure is incomplete or inaccurate and management/investors cannot see results by reportable segment.</t>
         </is>
       </c>
       <c r="F131" s="16" t="inlineStr">
         <is>
-          <t>Accuracy/Valuation</t>
+          <t>Presentation/Disclosure</t>
         </is>
       </c>
       <c r="G131" s="16" t="inlineStr">
         <is>
-          <t>FX rate maker-checker (SoD): a MANUALLY-entered rate lands as PendingApproval and is EXCLUDED from rate resolution — revaluation, the unrealized-FX report, and consolidation translation all use APPROVED rates only — until a DIFFERENT user approves it (POST /api/fx/rates/approve). Self-approval → SOD_VIOLATION (binds even Admin); reject marks the rate Rejected (never usable); re-entering a rate sends it back to PendingApproval. Externally-sourced (feed) rates carrying an explicit non-manual source are auto-approved. Pending rates are also surfaced, aged, by the pending-approvals monitor (GOV-01).</t>
+          <t>Segment reporting (CON-04, IFRS 8): segmentReport produces P&amp;L (revenue/expense/net) grouped by reportable segment, sourced from the dimension columns on journal_lines (branch_id/project_id/department_id) and mapped through configurable segment_definitions (member_keys → segment); unmapped dimension values surface as their own/Unassigned bucket. HQ/Admin-only, gated 'exec'.</t>
         </is>
       </c>
       <c r="H131" s="17" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I131" s="17" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="J131" s="17" t="inlineStr">
         <is>
-          <t>Per rate</t>
+          <t>Period</t>
         </is>
       </c>
       <c r="K131" s="16" t="inlineStr">
         <is>
-          <t>Controller / Treasury</t>
+          <t>Group Controller</t>
         </is>
       </c>
       <c r="L131" s="17" t="inlineStr">
@@ -12253,22 +12253,22 @@
       </c>
       <c r="M131" s="16" t="inlineStr">
         <is>
-          <t>fx.service.ts setRate(manual→PendingApproval)/approveRate/rejectRate/rateAsOf(Approved only); fx.controller.ts (rates/approve|reject|pending gated approvals/gl_close); consolidation.service.ts (translation reads Approved rates); schema/fx.ts fx_rates.status + migration 0141; cutover/fxreval.ts (ToE)</t>
+          <t>consolidation.service.ts defineSegment/listSegments/segmentReport; consolidation.controller.ts (segments, segment-report @exec); schema/consolidation.ts segment_definitions + migration 0170; cutover/consolidation.ts (ToE)</t>
         </is>
       </c>
       <c r="N131" s="16" t="inlineStr">
         <is>
-          <t>Inspect the request→approve flow + the approver≠requester check + that revaluation/reporting resolve Approved rates only.</t>
+          <t>Inspect the segment mapping + the dimension-grouped P&amp;L aggregation.</t>
         </is>
       </c>
       <c r="O131" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: enter a manual rate (PendingApproval), confirm revalue is blocked NO_RATE while pending, attempt self-approve (SOD_VIOLATION), approve as a different user, then revalue succeeds (re-performed by the fxreval harness).</t>
+          <t>Re-perform: define a segment over branches, run the segment report for a period, confirm revenue/expense/net tie to the underlying dimensioned postings. Re-performed by the consolidation harness.</t>
         </is>
       </c>
       <c r="P131" s="16" t="inlineStr">
         <is>
-          <t>FX rate approval log + SoD test</t>
+          <t>Segment P&amp;L report</t>
         </is>
       </c>
       <c r="Q131" s="18" t="inlineStr">
@@ -12280,92 +12280,179 @@
     <row r="132">
       <c r="A132" s="11" t="inlineStr">
         <is>
+          <t>FX-04</t>
+        </is>
+      </c>
+      <c r="B132" s="12" t="inlineStr">
+        <is>
+          <t>Consolidation &amp; FX</t>
+        </is>
+      </c>
+      <c r="C132" s="13" t="inlineStr">
+        <is>
+          <t>Application</t>
+        </is>
+      </c>
+      <c r="D132" s="12" t="inlineStr">
+        <is>
+          <t>FX gain/loss; Revenue; AR/AP</t>
+        </is>
+      </c>
+      <c r="E132" s="12" t="inlineStr">
+        <is>
+          <t>A wrong manually-entered FX rate (fat-fingered, e.g. USD 36 keyed as 63) flows straight into a period-end revaluation JE and the unrealized-FX report with no independent review — mis-stating earnings/equity and FX-translated balances.</t>
+        </is>
+      </c>
+      <c r="F132" s="12" t="inlineStr">
+        <is>
+          <t>Accuracy/Valuation</t>
+        </is>
+      </c>
+      <c r="G132" s="12" t="inlineStr">
+        <is>
+          <t>FX rate maker-checker (SoD): a MANUALLY-entered rate lands as PendingApproval and is EXCLUDED from rate resolution — revaluation, the unrealized-FX report, and consolidation translation all use APPROVED rates only — until a DIFFERENT user approves it (POST /api/fx/rates/approve). Self-approval → SOD_VIOLATION (binds even Admin); reject marks the rate Rejected (never usable); re-entering a rate sends it back to PendingApproval. Externally-sourced (feed) rates carrying an explicit non-manual source are auto-approved. Pending rates are also surfaced, aged, by the pending-approvals monitor (GOV-01).</t>
+        </is>
+      </c>
+      <c r="H132" s="13" t="inlineStr">
+        <is>
+          <t>Prev</t>
+        </is>
+      </c>
+      <c r="I132" s="13" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="J132" s="13" t="inlineStr">
+        <is>
+          <t>Per rate</t>
+        </is>
+      </c>
+      <c r="K132" s="12" t="inlineStr">
+        <is>
+          <t>Controller / Treasury</t>
+        </is>
+      </c>
+      <c r="L132" s="13" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="M132" s="12" t="inlineStr">
+        <is>
+          <t>fx.service.ts setRate(manual→PendingApproval)/approveRate/rejectRate/rateAsOf(Approved only); fx.controller.ts (rates/approve|reject|pending gated approvals/gl_close); consolidation.service.ts (translation reads Approved rates); schema/fx.ts fx_rates.status + migration 0141; cutover/fxreval.ts (ToE)</t>
+        </is>
+      </c>
+      <c r="N132" s="12" t="inlineStr">
+        <is>
+          <t>Inspect the request→approve flow + the approver≠requester check + that revaluation/reporting resolve Approved rates only.</t>
+        </is>
+      </c>
+      <c r="O132" s="12" t="inlineStr">
+        <is>
+          <t>Re-perform: enter a manual rate (PendingApproval), confirm revalue is blocked NO_RATE while pending, attempt self-approve (SOD_VIOLATION), approve as a different user, then revalue succeeds (re-performed by the fxreval harness).</t>
+        </is>
+      </c>
+      <c r="P132" s="12" t="inlineStr">
+        <is>
+          <t>FX rate approval log + SoD test</t>
+        </is>
+      </c>
+      <c r="Q132" s="18" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="15" t="inlineStr">
+        <is>
           <t>BUD-01</t>
         </is>
       </c>
-      <c r="B132" s="12" t="inlineStr">
+      <c r="B133" s="16" t="inlineStr">
         <is>
           <t>Budgeting &amp; Planning</t>
         </is>
       </c>
-      <c r="C132" s="13" t="inlineStr">
+      <c r="C133" s="17" t="inlineStr">
         <is>
           <t>Application</t>
         </is>
       </c>
-      <c r="D132" s="12" t="inlineStr">
+      <c r="D133" s="16" t="inlineStr">
         <is>
           <t>Budget; All (variance reporting)</t>
         </is>
       </c>
-      <c r="E132" s="12" t="inlineStr">
+      <c r="E133" s="16" t="inlineStr">
         <is>
           <t>A budget figure is entered/changed by one person and immediately drives the budget-vs-actual variance report — the basis for spend authorization and performance review — with no independent approval; a wrong or self-serving budget makes overspending look 'on budget'.</t>
         </is>
       </c>
-      <c r="F132" s="12" t="inlineStr">
+      <c r="F133" s="16" t="inlineStr">
         <is>
           <t>Authorization/Accuracy</t>
         </is>
       </c>
-      <c r="G132" s="12" t="inlineStr">
+      <c r="G133" s="16" t="inlineStr">
         <is>
           <t>Budget maker-checker (SoD): an upserted budget (POST /api/ledger/budgets) lands as PendingApproval and is EXCLUDED from budget-vs-actual until a DIFFERENT user approves it (POST /api/ledger/budgets/approve for the fiscal_year/account/cost-centre[/period]). Self-approval → SOD_VIOLATION (binds even Admin); reject marks it Rejected (excluded). DEFAULT 'Approved' keeps existing rows + direct planning seeds usable. Pending budgets are also surfaced, aged, by the pending-approvals monitor (GOV-01).</t>
         </is>
       </c>
-      <c r="H132" s="13" t="inlineStr">
+      <c r="H133" s="17" t="inlineStr">
         <is>
           <t>Prev</t>
         </is>
       </c>
-      <c r="I132" s="13" t="inlineStr">
+      <c r="I133" s="17" t="inlineStr">
         <is>
           <t>Automated</t>
         </is>
       </c>
-      <c r="J132" s="13" t="inlineStr">
+      <c r="J133" s="17" t="inlineStr">
         <is>
           <t>Per budget</t>
         </is>
       </c>
-      <c r="K132" s="12" t="inlineStr">
+      <c r="K133" s="16" t="inlineStr">
         <is>
           <t>Controller / FP&amp;A</t>
         </is>
       </c>
-      <c r="L132" s="13" t="inlineStr">
+      <c r="L133" s="17" t="inlineStr">
         <is>
           <t>P10</t>
         </is>
       </c>
-      <c r="M132" s="12" t="inlineStr">
+      <c r="M133" s="16" t="inlineStr">
         <is>
           <t>budget.service.ts upsertBudget(→PendingApproval)/approveBudget/rejectBudget/budgetVsActual(Approved only); budget.controller.ts (budgets/approve|reject|pending gated approvals/gl_close); schema/budgets.ts budgets.status + migration 0142; cutover/budget.ts (ToE)</t>
         </is>
       </c>
-      <c r="N132" s="12" t="inlineStr">
+      <c r="N133" s="16" t="inlineStr">
         <is>
           <t>Inspect the request→approve flow + the approver≠requester check + that budget-vs-actual counts Approved budgets only.</t>
         </is>
       </c>
-      <c r="O132" s="12" t="inlineStr">
+      <c r="O133" s="16" t="inlineStr">
         <is>
           <t>Re-perform: upsert a budget (PendingApproval, excluded from variance), attempt self-approve (SOD_VIOLATION), approve as a different user, confirm it then appears in budget-vs-actual (re-performed by the budget harness).</t>
         </is>
       </c>
-      <c r="P132" s="12" t="inlineStr">
+      <c r="P133" s="16" t="inlineStr">
         <is>
           <t>Budget approval log + SoD test</t>
         </is>
       </c>
-      <c r="Q132" s="18" t="inlineStr">
+      <c r="Q133" s="18" t="inlineStr">
         <is>
           <t>Implemented</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q132"/>
+  <autoFilter ref="A1:Q133"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -13548,7 +13635,7 @@
         </is>
       </c>
       <c r="C5" s="29">
-        <f>COUNTIF(RCM!$Q$2:$Q$132,B5)</f>
+        <f>COUNTIF(RCM!$Q$2:$Q$133,B5)</f>
         <v/>
       </c>
     </row>
@@ -13559,7 +13646,7 @@
         </is>
       </c>
       <c r="C6" s="29">
-        <f>COUNTIF(RCM!$Q$2:$Q$132,B6)</f>
+        <f>COUNTIF(RCM!$Q$2:$Q$133,B6)</f>
         <v/>
       </c>
     </row>
@@ -13570,7 +13657,7 @@
         </is>
       </c>
       <c r="C7" s="29">
-        <f>COUNTIF(RCM!$Q$2:$Q$132,B7)</f>
+        <f>COUNTIF(RCM!$Q$2:$Q$133,B7)</f>
         <v/>
       </c>
     </row>
@@ -13581,7 +13668,7 @@
         </is>
       </c>
       <c r="C8" s="32">
-        <f>COUNTA(RCM!$A$2:$A$132)</f>
+        <f>COUNTA(RCM!$A$2:$A$133)</f>
         <v/>
       </c>
     </row>
@@ -13599,7 +13686,7 @@
         </is>
       </c>
       <c r="C11" s="29">
-        <f>COUNTIF(RCM!$C$2:$C$132,B11)</f>
+        <f>COUNTIF(RCM!$C$2:$C$133,B11)</f>
         <v/>
       </c>
     </row>
@@ -13610,7 +13697,7 @@
         </is>
       </c>
       <c r="C12" s="29">
-        <f>COUNTIF(RCM!$C$2:$C$132,B12)</f>
+        <f>COUNTIF(RCM!$C$2:$C$133,B12)</f>
         <v/>
       </c>
     </row>
@@ -13621,7 +13708,7 @@
         </is>
       </c>
       <c r="C13" s="29">
-        <f>COUNTIF(RCM!$C$2:$C$132,B13)</f>
+        <f>COUNTIF(RCM!$C$2:$C$133,B13)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(compliance): close ITGC-SD-01 (SDLC policy) + SD-02 (cutover reconciliation); confirm AC-07
SD-01 → Implemented: finalized compliance/policies/08-change-management-sdlc-policy.md (v1.0)
with explicit UAT sign-off (docs/uat) + go-live sign-off (deploy-approval gate, deployer ≠ author).
SD-02 → Implemented: docs/ops/cutover-reconciliation.md — source→target balance tie-out (GL trial
balance + AR/AP/INV/FA sub-ledgers to control accounts) + independent Controller sign-off over the
idempotent opening-balance load. Both cleared from the RCM gap tracker (regenerated; 11 gaps).

AC-07 (web localStorage → httpOnly cookie) re-verified ALREADY COMPLETE end-to-end (staff client,
SSE, member app — no auth token in JS; cookie-auth ToE); the "Tier 3 deferred" note was stale.
Fixed a misleading "Bearer token" comment in use-realtime.ts (SSE authenticates via the cookie).

Narrative step 13 + control matrix + revision history updated.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/compliance/Oshinei_ERP_SOX_RCM_v1.xlsx
+++ b/compliance/Oshinei_ERP_SOX_RCM_v1.xlsx
@@ -15,7 +15,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'RCM'!$A$1:$Q$155</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Gap Remediation'!$A$2:$H$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Gap Remediation'!$A$2:$H$13</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -4296,7 +4296,7 @@
       </c>
       <c r="E40" s="12" t="inlineStr">
         <is>
-          <t>New functionality goes live without design/test sign-off.</t>
+          <t>New functionality goes live without design / test / UAT sign-off.</t>
         </is>
       </c>
       <c r="F40" s="12" t="inlineStr">
@@ -4306,7 +4306,7 @@
       </c>
       <c r="G40" s="12" t="inlineStr">
         <is>
-          <t>SDLC policy: requirements, design, test and UAT sign-off prior to go-live.</t>
+          <t>Formal SDLC policy with gated stages: ticketed request, design + reviewer sign-off, branch-only build (no direct main), independent review (author ≠ merger), CI test gates (build/typecheck/unit + ratchet coverage + control harnesses), UAT sign-off (docs/uat positive+negative cases + traceability matrix) and a go-live sign-off via the deploy-approval gate (deployer ≠ author). Docs updated in the same change (doc-sync).</t>
         </is>
       </c>
       <c r="H40" s="13" t="inlineStr">
@@ -4336,27 +4336,27 @@
       </c>
       <c r="M40" s="12" t="inlineStr">
         <is>
-          <t>SDLC policy (to author)</t>
+          <t>compliance/policies/08-change-management-sdlc-policy.md; docs/uat/; .github (branch protection + deploy-approval environment); .github/workflows/ci.yml (gates)</t>
         </is>
       </c>
       <c r="N40" s="12" t="inlineStr">
         <is>
-          <t>Inspect SDLC policy + a project's artefacts.</t>
+          <t>Inspect the SDLC policy + a project's artefacts (design, UAT sign-off, deploy approval).</t>
         </is>
       </c>
       <c r="O40" s="12" t="inlineStr">
         <is>
-          <t>Sample releases: UAT + go-live sign-off present.</t>
+          <t>Sample releases: design + UAT sign-off + go-live (deploy) approval present.</t>
         </is>
       </c>
       <c r="P40" s="12" t="inlineStr">
         <is>
-          <t>SDLC artefacts</t>
-        </is>
-      </c>
-      <c r="Q40" s="14" t="inlineStr">
-        <is>
-          <t>Gap</t>
+          <t>SDLC policy + release artefacts</t>
+        </is>
+      </c>
+      <c r="Q40" s="18" t="inlineStr">
+        <is>
+          <t>Implemented</t>
         </is>
       </c>
     </row>
@@ -4393,7 +4393,7 @@
       </c>
       <c r="G41" s="16" t="inlineStr">
         <is>
-          <t>Cutover data-migration controls: source→target balance reconciliation + sign-off; opening balances idempotent.</t>
+          <t>Documented cutover reconciliation: source→target balance tie-out (GL trial balance balances Dr=Cr; AR/AP/INV/FA sub-ledgers tie to their GL control accounts), zero unexplained variance, and an independent Controller sign-off (≠ preparer) BEFORE go-live — over the idempotent opening-balance load (re-runnable on batch_ref) + the close-control tie-out steps.</t>
         </is>
       </c>
       <c r="H41" s="17" t="inlineStr">
@@ -4423,27 +4423,27 @@
       </c>
       <c r="M41" s="16" t="inlineStr">
         <is>
-          <t>tools/etl; tools/cutover; ledger opening-balances (idempotent on batch_ref)</t>
+          <t>docs/ops/cutover-reconciliation.md; ledger opening-balances (idempotent on batch_ref) + close.service.ts (subledger_tieout / trial_balance_review); tools/etl; cutover/opening-balances.ts (ToE)</t>
         </is>
       </c>
       <c r="N41" s="16" t="inlineStr">
         <is>
-          <t>Inspect migration reconciliation + sign-off.</t>
+          <t>Inspect the reconciliation procedure + sign-off; re-perform a migrated trial-balance tie-out.</t>
         </is>
       </c>
       <c r="O41" s="16" t="inlineStr">
         <is>
-          <t>Re-perform migrated trial-balance tie-out.</t>
+          <t>Re-perform: load opening balances (idempotent), trial balance ties to source, sub-ledgers tie to control accounts, sign-off retained.</t>
         </is>
       </c>
       <c r="P41" s="16" t="inlineStr">
         <is>
-          <t>Migration recon</t>
-        </is>
-      </c>
-      <c r="Q41" s="19" t="inlineStr">
-        <is>
-          <t>Partial</t>
+          <t>Cutover reconciliation procedure + tie-out</t>
+        </is>
+      </c>
+      <c r="Q41" s="18" t="inlineStr">
+        <is>
+          <t>Implemented</t>
         </is>
       </c>
     </row>
@@ -14377,7 +14377,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -14442,27 +14442,27 @@
     <row r="3">
       <c r="A3" s="11" t="inlineStr">
         <is>
-          <t>ITGC-SD-01</t>
+          <t>EXP-03</t>
         </is>
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>ITGC · SDLC</t>
+          <t>Expenditure</t>
         </is>
       </c>
       <c r="C3" s="12" t="inlineStr">
         <is>
-          <t>No formal SDLC policy.</t>
+          <t>PR/PO approval workflow partial.</t>
         </is>
       </c>
       <c r="D3" s="12" t="inlineStr">
         <is>
-          <t>Author SDLC policy with design/test/UAT/go-live sign-offs.</t>
+          <t>Finalize PR/PO maker-checker against DoA thresholds.</t>
         </is>
       </c>
       <c r="E3" s="13" t="inlineStr">
         <is>
-          <t>Head of Eng / Product</t>
+          <t>Procurement Mgr</t>
         </is>
       </c>
       <c r="F3" s="13" t="inlineStr">
@@ -14484,27 +14484,27 @@
     <row r="4">
       <c r="A4" s="15" t="inlineStr">
         <is>
-          <t>ITGC-SD-02</t>
+          <t>INV-04</t>
         </is>
       </c>
       <c r="B4" s="17" t="inlineStr">
         <is>
-          <t>ITGC · SDLC</t>
+          <t>Inventory &amp; COGS</t>
         </is>
       </c>
       <c r="C4" s="16" t="inlineStr">
         <is>
-          <t>Cutover reconciliation not documented.</t>
+          <t>Stocktake variance review informal.</t>
         </is>
       </c>
       <c r="D4" s="16" t="inlineStr">
         <is>
-          <t>Document source→target balance tie-out + sign-off for any migration.</t>
+          <t>Formalize count cadence + variance review/approval sign-off.</t>
         </is>
       </c>
       <c r="E4" s="17" t="inlineStr">
         <is>
-          <t>Controller / Eng</t>
+          <t>Warehouse Mgr</t>
         </is>
       </c>
       <c r="F4" s="17" t="inlineStr">
@@ -14526,37 +14526,37 @@
     <row r="5">
       <c r="A5" s="11" t="inlineStr">
         <is>
-          <t>EXP-03</t>
+          <t>REC-03</t>
         </is>
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Expenditure</t>
+          <t>Reconciliation</t>
         </is>
       </c>
       <c r="C5" s="12" t="inlineStr">
         <is>
-          <t>PR/PO approval workflow partial.</t>
+          <t>Intercompany recon partial.</t>
         </is>
       </c>
       <c r="D5" s="12" t="inlineStr">
         <is>
-          <t>Finalize PR/PO maker-checker against DoA thresholds.</t>
+          <t>Formalize IC matching + elimination sign-off each period.</t>
         </is>
       </c>
       <c r="E5" s="13" t="inlineStr">
         <is>
-          <t>Procurement Mgr</t>
+          <t>Group Controller</t>
         </is>
       </c>
       <c r="F5" s="13" t="inlineStr">
         <is>
-          <t>Phase 2</t>
+          <t>Phase 2-3</t>
         </is>
       </c>
       <c r="G5" s="13" t="inlineStr">
         <is>
-          <t>Month 3-4</t>
+          <t>Month 4-6</t>
         </is>
       </c>
       <c r="H5" s="22" t="inlineStr">
@@ -14568,27 +14568,27 @@
     <row r="6">
       <c r="A6" s="15" t="inlineStr">
         <is>
-          <t>INV-04</t>
+          <t>ITGC-AC-07</t>
         </is>
       </c>
       <c r="B6" s="17" t="inlineStr">
         <is>
-          <t>Inventory &amp; COGS</t>
+          <t>ITGC · Access</t>
         </is>
       </c>
       <c r="C6" s="16" t="inlineStr">
         <is>
-          <t>Stocktake variance review informal.</t>
+          <t>Login brute-force lockout + JWT revocation (now implemented; monitoring/alerting on lockouts to formalize).</t>
         </is>
       </c>
       <c r="D6" s="16" t="inlineStr">
         <is>
-          <t>Formalize count cadence + variance review/approval sign-off.</t>
+          <t>DONE: token → httpOnly cookie + CSRF + web CSP; JWT jti revocation list + revoke-all watermark (0147); per-account login lockout/throttle with exponential window (0176, login_attempts). Remaining: ops alerting on repeated lockouts.</t>
         </is>
       </c>
       <c r="E6" s="17" t="inlineStr">
         <is>
-          <t>Warehouse Mgr</t>
+          <t>IT Security / Eng</t>
         </is>
       </c>
       <c r="F6" s="17" t="inlineStr">
@@ -14598,39 +14598,39 @@
       </c>
       <c r="G6" s="17" t="inlineStr">
         <is>
-          <t>Month 4</t>
-        </is>
-      </c>
-      <c r="H6" s="22" t="inlineStr">
-        <is>
-          <t>Medium</t>
+          <t>Month 2-3</t>
+        </is>
+      </c>
+      <c r="H6" s="23" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="11" t="inlineStr">
         <is>
-          <t>REC-03</t>
+          <t>TAX-03</t>
         </is>
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>Reconciliation</t>
+          <t>Tax</t>
         </is>
       </c>
       <c r="C7" s="12" t="inlineStr">
         <is>
-          <t>Intercompany recon partial.</t>
+          <t>WHT reporting partial.</t>
         </is>
       </c>
       <c r="D7" s="12" t="inlineStr">
         <is>
-          <t>Formalize IC matching + elimination sign-off each period.</t>
+          <t>Complete WHT calc coverage + monthly ภ.ง.ด. tie-out.</t>
         </is>
       </c>
       <c r="E7" s="13" t="inlineStr">
         <is>
-          <t>Group Controller</t>
+          <t>Tax</t>
         </is>
       </c>
       <c r="F7" s="13" t="inlineStr">
@@ -14652,133 +14652,133 @@
     <row r="8">
       <c r="A8" s="15" t="inlineStr">
         <is>
-          <t>ITGC-AC-07</t>
+          <t>PAY-02</t>
         </is>
       </c>
       <c r="B8" s="17" t="inlineStr">
         <is>
-          <t>ITGC · Access</t>
+          <t>Payroll</t>
         </is>
       </c>
       <c r="C8" s="16" t="inlineStr">
         <is>
-          <t>Login brute-force lockout + JWT revocation (now implemented; monitoring/alerting on lockouts to formalize).</t>
+          <t>Statutory payroll items partial.</t>
         </is>
       </c>
       <c r="D8" s="16" t="inlineStr">
         <is>
-          <t>DONE: token → httpOnly cookie + CSRF + web CSP; JWT jti revocation list + revoke-all watermark (0147); per-account login lockout/throttle with exponential window (0176, login_attempts). Remaining: ops alerting on repeated lockouts.</t>
+          <t>Complete PF/OT/leave + ภ.ง.ด.1ก reconciliation to filings.</t>
         </is>
       </c>
       <c r="E8" s="17" t="inlineStr">
         <is>
-          <t>IT Security / Eng</t>
+          <t>HR / Payroll</t>
         </is>
       </c>
       <c r="F8" s="17" t="inlineStr">
         <is>
-          <t>Phase 2</t>
+          <t>Phase 2-3</t>
         </is>
       </c>
       <c r="G8" s="17" t="inlineStr">
         <is>
-          <t>Month 2-3</t>
-        </is>
-      </c>
-      <c r="H8" s="23" t="inlineStr">
-        <is>
-          <t>Low</t>
+          <t>Month 4-6</t>
+        </is>
+      </c>
+      <c r="H8" s="22" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="11" t="inlineStr">
         <is>
-          <t>TAX-03</t>
+          <t>ELC-01</t>
         </is>
       </c>
       <c r="B9" s="13" t="inlineStr">
         <is>
-          <t>Tax</t>
+          <t>Entity-Level</t>
         </is>
       </c>
       <c r="C9" s="12" t="inlineStr">
         <is>
-          <t>WHT reporting partial.</t>
+          <t>No ethics policy / acknowledgements.</t>
         </is>
       </c>
       <c r="D9" s="12" t="inlineStr">
         <is>
-          <t>Complete WHT calc coverage + monthly ภ.ง.ด. tie-out.</t>
+          <t>Issue code of conduct; annual acknowledgement register.</t>
         </is>
       </c>
       <c r="E9" s="13" t="inlineStr">
         <is>
-          <t>Tax</t>
+          <t>CEO / HR</t>
         </is>
       </c>
       <c r="F9" s="13" t="inlineStr">
         <is>
-          <t>Phase 2-3</t>
+          <t>Phase 1</t>
         </is>
       </c>
       <c r="G9" s="13" t="inlineStr">
         <is>
-          <t>Month 4-6</t>
-        </is>
-      </c>
-      <c r="H9" s="22" t="inlineStr">
-        <is>
-          <t>Medium</t>
+          <t>Month 1-2</t>
+        </is>
+      </c>
+      <c r="H9" s="24" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="15" t="inlineStr">
         <is>
-          <t>PAY-02</t>
+          <t>ELC-02</t>
         </is>
       </c>
       <c r="B10" s="17" t="inlineStr">
         <is>
-          <t>Payroll</t>
+          <t>Entity-Level</t>
         </is>
       </c>
       <c r="C10" s="16" t="inlineStr">
         <is>
-          <t>Statutory payroll items partial.</t>
+          <t>No audit-committee ICFR oversight.</t>
         </is>
       </c>
       <c r="D10" s="16" t="inlineStr">
         <is>
-          <t>Complete PF/OT/leave + ภ.ง.ด.1ก reconciliation to filings.</t>
+          <t>Charter audit committee; quarterly ICFR review minutes.</t>
         </is>
       </c>
       <c r="E10" s="17" t="inlineStr">
         <is>
-          <t>HR / Payroll</t>
+          <t>Board</t>
         </is>
       </c>
       <c r="F10" s="17" t="inlineStr">
         <is>
-          <t>Phase 2-3</t>
+          <t>Phase 1</t>
         </is>
       </c>
       <c r="G10" s="17" t="inlineStr">
         <is>
-          <t>Month 4-6</t>
-        </is>
-      </c>
-      <c r="H10" s="22" t="inlineStr">
-        <is>
-          <t>Medium</t>
+          <t>Month 1-2</t>
+        </is>
+      </c>
+      <c r="H10" s="24" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="11" t="inlineStr">
         <is>
-          <t>ELC-01</t>
+          <t>ELC-03</t>
         </is>
       </c>
       <c r="B11" s="13" t="inlineStr">
@@ -14788,17 +14788,17 @@
       </c>
       <c r="C11" s="12" t="inlineStr">
         <is>
-          <t>No ethics policy / acknowledgements.</t>
+          <t>No documented delegation of authority.</t>
         </is>
       </c>
       <c r="D11" s="12" t="inlineStr">
         <is>
-          <t>Issue code of conduct; annual acknowledgement register.</t>
+          <t>Author DoA/approval matrix; reconcile to RBAC roles.</t>
         </is>
       </c>
       <c r="E11" s="13" t="inlineStr">
         <is>
-          <t>CEO / HR</t>
+          <t>CFO</t>
         </is>
       </c>
       <c r="F11" s="13" t="inlineStr">
@@ -14808,7 +14808,7 @@
       </c>
       <c r="G11" s="13" t="inlineStr">
         <is>
-          <t>Month 1-2</t>
+          <t>Month 2</t>
         </is>
       </c>
       <c r="H11" s="24" t="inlineStr">
@@ -14820,7 +14820,7 @@
     <row r="12">
       <c r="A12" s="15" t="inlineStr">
         <is>
-          <t>ELC-02</t>
+          <t>ELC-04</t>
         </is>
       </c>
       <c r="B12" s="17" t="inlineStr">
@@ -14830,17 +14830,17 @@
       </c>
       <c r="C12" s="16" t="inlineStr">
         <is>
-          <t>No audit-committee ICFR oversight.</t>
+          <t>No whistleblower channel.</t>
         </is>
       </c>
       <c r="D12" s="16" t="inlineStr">
         <is>
-          <t>Charter audit committee; quarterly ICFR review minutes.</t>
+          <t>Stand up anonymous hotline + non-retaliation policy.</t>
         </is>
       </c>
       <c r="E12" s="17" t="inlineStr">
         <is>
-          <t>Board</t>
+          <t>Audit Cttee</t>
         </is>
       </c>
       <c r="F12" s="17" t="inlineStr">
@@ -14850,19 +14850,19 @@
       </c>
       <c r="G12" s="17" t="inlineStr">
         <is>
-          <t>Month 1-2</t>
-        </is>
-      </c>
-      <c r="H12" s="24" t="inlineStr">
-        <is>
-          <t>High</t>
+          <t>Month 2</t>
+        </is>
+      </c>
+      <c r="H12" s="22" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="11" t="inlineStr">
         <is>
-          <t>ELC-03</t>
+          <t>ELC-05</t>
         </is>
       </c>
       <c r="B13" s="13" t="inlineStr">
@@ -14872,121 +14872,37 @@
       </c>
       <c r="C13" s="12" t="inlineStr">
         <is>
-          <t>No documented delegation of authority.</t>
+          <t>No fraud risk assessment.</t>
         </is>
       </c>
       <c r="D13" s="12" t="inlineStr">
         <is>
-          <t>Author DoA/approval matrix; reconcile to RBAC roles.</t>
+          <t>Perform annual fraud risk assessment; map to controls.</t>
         </is>
       </c>
       <c r="E13" s="13" t="inlineStr">
         <is>
-          <t>CFO</t>
+          <t>CFO / IA</t>
         </is>
       </c>
       <c r="F13" s="13" t="inlineStr">
         <is>
-          <t>Phase 1</t>
+          <t>Phase 2</t>
         </is>
       </c>
       <c r="G13" s="13" t="inlineStr">
         <is>
-          <t>Month 2</t>
-        </is>
-      </c>
-      <c r="H13" s="24" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="15" t="inlineStr">
-        <is>
-          <t>ELC-04</t>
-        </is>
-      </c>
-      <c r="B14" s="17" t="inlineStr">
-        <is>
-          <t>Entity-Level</t>
-        </is>
-      </c>
-      <c r="C14" s="16" t="inlineStr">
-        <is>
-          <t>No whistleblower channel.</t>
-        </is>
-      </c>
-      <c r="D14" s="16" t="inlineStr">
-        <is>
-          <t>Stand up anonymous hotline + non-retaliation policy.</t>
-        </is>
-      </c>
-      <c r="E14" s="17" t="inlineStr">
-        <is>
-          <t>Audit Cttee</t>
-        </is>
-      </c>
-      <c r="F14" s="17" t="inlineStr">
-        <is>
-          <t>Phase 1</t>
-        </is>
-      </c>
-      <c r="G14" s="17" t="inlineStr">
-        <is>
-          <t>Month 2</t>
-        </is>
-      </c>
-      <c r="H14" s="22" t="inlineStr">
+          <t>Month 3</t>
+        </is>
+      </c>
+      <c r="H13" s="22" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="11" t="inlineStr">
-        <is>
-          <t>ELC-05</t>
-        </is>
-      </c>
-      <c r="B15" s="13" t="inlineStr">
-        <is>
-          <t>Entity-Level</t>
-        </is>
-      </c>
-      <c r="C15" s="12" t="inlineStr">
-        <is>
-          <t>No fraud risk assessment.</t>
-        </is>
-      </c>
-      <c r="D15" s="12" t="inlineStr">
-        <is>
-          <t>Perform annual fraud risk assessment; map to controls.</t>
-        </is>
-      </c>
-      <c r="E15" s="13" t="inlineStr">
-        <is>
-          <t>CFO / IA</t>
-        </is>
-      </c>
-      <c r="F15" s="13" t="inlineStr">
-        <is>
-          <t>Phase 2</t>
-        </is>
-      </c>
-      <c r="G15" s="13" t="inlineStr">
-        <is>
-          <t>Month 3</t>
-        </is>
-      </c>
-      <c r="H15" s="22" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A2:H15"/>
+  <autoFilter ref="A2:H13"/>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>

</xml_diff>

<commit_message>
Project material control (docs/32): FU1 budget policy + FU2 prefer-stock + FU3 web UI (#405)
Follow-ups on docs/32 (M0–M4 material control spine):

- FU1 — per-project over-budget tolerance % (CommitmentsService.reserve ceiling + PMR routing) and site cash consumes BoQ budget (advances/petty-cash tagged to a BoQ line book a consumed commitment). Migration 0242. Amends PROJ-12/PROJ-14 text (RCM 180).
- FU2 — a within-budget requisition fulfils from on-hand stock first (reserve + issue-to-project) and only raises a PR when the item isn't on hand.
- FU3 — web UI: four material-control tabs on /projects/[code] (BoQ & budget, requisitions, reservations, site cash) over the existing endpoints.

All CI green (95 checks): projects harness 165, basics 217, compliance 134, tenant-idx, migration-parity, migrations-journaled, ts-debt 120/120, web-e2e, build, typecheck.
</commit_message>
<xml_diff>
--- a/compliance/Oshinei_ERP_SOX_RCM_v1.xlsx
+++ b/compliance/Oshinei_ERP_SOX_RCM_v1.xlsx
@@ -11773,7 +11773,7 @@
       </c>
       <c r="G126" s="12" t="inlineStr">
         <is>
-          <t>Commitment/encumbrance control on the BoQ line budget: a project purchase order tagged to a BoQ line RESERVES budget in the `project_commitments` ledger (open+consumed count against the line; released — e.g. a cancelled PO — frees it). A draw is admitted only if `line.budget_amount − Σ(open+consumed) ≥ amount`, checked ATOMICALLY under a FOR UPDATE row-lock on the BoQ line so two concurrent draws cannot jointly overrun (BUDGET_EXCEEDED with the remaining otherwise). The BoQ budget baseline is itself maker-checker (an author-approved BoQ; approver ≠ author → SOD_SELF_APPROVAL syncs the project budget). A cancelled PO releases its encumbrance; a fully-received PO's commitments become consumed (actual). Turns the material budget from OBSERVED into ENFORCED.</t>
+          <t>Commitment/encumbrance control on the BoQ line budget: a project purchase order tagged to a BoQ line RESERVES budget in the `project_commitments` ledger (open+consumed count against the line; released — e.g. a cancelled PO — frees it). A draw is admitted only if `line.budget_amount − Σ(open+consumed) ≥ amount`, checked ATOMICALLY under a FOR UPDATE row-lock on the BoQ line so two concurrent draws cannot jointly overrun (BUDGET_EXCEEDED with the remaining otherwise). The BoQ budget baseline is itself maker-checker (an author-approved BoQ; approver ≠ author → SOD_SELF_APPROVAL syncs the project budget). A cancelled PO releases its encumbrance; a fully-received PO's commitments become consumed (actual). An optional per-project over-budget TOLERANCE (projects.budget_tolerance_pct) lets a draw exceed the line by up to that % of the line budget before it is blocked/needs approval (ceiling = budget × (1+tol%)); 0 = strict. Turns the material budget from OBSERVED into ENFORCED.</t>
         </is>
       </c>
       <c r="H126" s="13" t="inlineStr">
@@ -11947,7 +11947,7 @@
       </c>
       <c r="G128" s="12" t="inlineStr">
         <is>
-          <t>Project-costed site cash: employee advances (finance.issueAdvance/settleAdvance), expense-reimbursement claims (ess.submitExpense) and petty-cash requests (petty-cash.createRequest/approveRequest) accept an optional project_code, resolve it to project_id (PROJECT_NOT_FOUND on a bad code), and store it on the entity; the GL expense/advance lines are tagged with that project_id (journal_lines.project_id) so the spend is traceable to the project. GET /api/projects/:code/site-cash rolls up all advances + reimbursements + petty-cash raised against the project with per-category + grand totals, so site cash is managed on the project (and reflected alongside EVM). Advance settlement clears the float (Dr expense/Cr 1180) carrying the project dimension. Maker-checker on the underlying flows is unchanged (petty-cash SoD_VIOLATION, ESS self-approval block).</t>
+          <t>Project-costed site cash: employee advances (finance.issueAdvance/settleAdvance), expense-reimbursement claims (ess.submitExpense) and petty-cash requests (petty-cash.createRequest/approveRequest) accept an optional project_code, resolve it to project_id (PROJECT_NOT_FOUND on a bad code), and store it on the entity; the GL expense/advance lines are tagged with that project_id (journal_lines.project_id) so the spend is traceable to the project. GET /api/projects/:code/site-cash rolls up all advances + reimbursements + petty-cash raised against the project with per-category + grand totals, so site cash is managed on the project (and reflected alongside EVM). When the site cash is tagged to a BoQ line it also CONSUMES that line's budget (a consumed commitment on advance settlement / petty-cash approval), so material + site cash sit under one budget ceiling. Advance settlement clears the float (Dr expense/Cr 1180) carrying the project dimension. Maker-checker on the underlying flows is unchanged (petty-cash SoD_VIOLATION, ESS self-approval block).</t>
         </is>
       </c>
       <c r="H128" s="13" t="inlineStr">

</xml_diff>

<commit_message>
Item-posting setup: account/category/warehouse/VAT/WHT linking + tax automation (docs/33) (#408)
Links item posting across account/category/warehouse/VAT/WHT via the posting-determination engine (opt-in per-tenant flag posting_determination, default OFF = parity; new control GL-21, fail-closed on non-postable accounts), adds the /setup/* maintenance screens, and automates the Thai tax outputs (tax_wht_cert_batch auto-issues the 50-tawi from AP-payment WHT; tax_pp30_draft/tax_pnd_draft/tax_remittance_reminder). Migrations 0243/0244. Fully doc-synced (RCM 181, narratives, user manual, UAT). All CI green.
</commit_message>
<xml_diff>
--- a/compliance/Oshinei_ERP_SOX_RCM_v1.xlsx
+++ b/compliance/Oshinei_ERP_SOX_RCM_v1.xlsx
@@ -14,7 +14,7 @@
     <sheet name="Summary" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'RCM'!$A$1:$Q$181</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'RCM'!$A$1:$Q$182</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Gap Remediation'!$A$2:$H$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -843,7 +843,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q181"/>
+  <dimension ref="A1:Q182"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -13744,12 +13744,12 @@
     <row r="149">
       <c r="A149" s="15" t="inlineStr">
         <is>
-          <t>EXP-07</t>
+          <t>GL-21</t>
         </is>
       </c>
       <c r="B149" s="16" t="inlineStr">
         <is>
-          <t>Expenditure</t>
+          <t>General Ledger</t>
         </is>
       </c>
       <c r="C149" s="17" t="inlineStr">
@@ -13759,27 +13759,27 @@
       </c>
       <c r="D149" s="16" t="inlineStr">
         <is>
-          <t>Cash; Operating expense</t>
+          <t>Inventory; COGS; Revenue</t>
         </is>
       </c>
       <c r="E149" s="16" t="inlineStr">
         <is>
-          <t>Petty-cash / employee advance issued but never accounted for — cash leakage, expense unrecorded.</t>
+          <t>Inventory / COGS posting accounts are hard-coded control literals, so an item (or item family) that should hit a different GL account has no maintainable mechanism; and any per-item account mapping, if introduced, could point at a non-existent or non-postable account — silently mis-stating the sub-ledger or breaking the control-account tie-out.</t>
         </is>
       </c>
       <c r="F149" s="16" t="inlineStr">
         <is>
-          <t>Existence/Completeness</t>
+          <t>Accuracy/Completeness/Valuation</t>
         </is>
       </c>
       <c r="G149" s="16" t="inlineStr">
         <is>
-          <t>Employee cash advances: issuing an advance debits the 1180 Employee Advances control (Dr 1180 / Cr 1000); settlement clears it against actual spend + returned cash (Dr expense + Dr 1000 / Cr 1180), enforced to reconcile (settled_expense + returned_cash must equal the advance → SETTLE_MISMATCH). The 1180 balance is the outstanding float subject to review.</t>
+          <t>Item-posting account determination (extends GL-12 to the item grain): a per-tenant, opt-in flag (posting_determination, default OFF ⇒ literal parity) lets an item's GL/tax profile drive posting. AccountDeterminationService.resolveItemAccounts resolves each account by precedence item column → its item_categories row → its WAREHOUSE (locations) default → null (caller falls back to the hard-coded control account), so an un-opted-in or unconfigured tenant is byte-for-byte unchanged. The inventory sub-ledger (receive/issue/adjust/issue-to-project) routes its inventory, COGS &amp; adjustment legs through the resolver; reconcile() sums the WHOLE inventory-account set (control 1200 + any item/category/warehouse overrides) so the GL-14-style sub-ledger↔GL tie-out holds under routing. Fail-closed: a resolved override that is not a real, POSTABLE account in the canonical CoA is rejected with INVALID_POSTING_ACCOUNT before any posting — a typo'd/header/control account can never receive a posting.</t>
         </is>
       </c>
       <c r="H149" s="17" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I149" s="17" t="inlineStr">
@@ -13789,12 +13789,12 @@
       </c>
       <c r="J149" s="17" t="inlineStr">
         <is>
-          <t>Per advance</t>
+          <t>Event-driven / per item</t>
         </is>
       </c>
       <c r="K149" s="16" t="inlineStr">
         <is>
-          <t>AP / Controller</t>
+          <t>Financial Controller</t>
         </is>
       </c>
       <c r="L149" s="17" t="inlineStr">
@@ -13804,22 +13804,22 @@
       </c>
       <c r="M149" s="16" t="inlineStr">
         <is>
-          <t>finance.service.ts (issueAdvance, settleAdvance reconcile-or-reject, listAdvances outstanding); finance.controller.ts (creditors/exec); schema/finance.ts (employee_advances) + migration 0120; cutover/basics.ts (ToE)</t>
+          <t>account-determination.service.ts (resolveItemAccounts item→category→warehouse precedence + assertPostable INVALID_POSTING_ACCOUNT fail-closed, enabled flag, resolveTaxCode); inventory-ledger.service.ts (invAccounts resolver + inventoryAccountSet reconcile); posting.service.ts (resolveRules now evaluates the condition jsonb); feature-flags.service.ts (posting_determination CORE flag, default off); item-setup.service.ts (categories/tax-codes/item-profile/warehouse-account CRUD, /api/item-setup/*, gated md_item/md_config); schema/posting-setup.ts (item_categories, tax_codes) + inventory.ts item + locations account columns; migrations 0243/0244 (journaled); ledger.module.ts (AccountDeterminationService exported); cutover/basics.ts (GL-21 ToE)</t>
         </is>
       </c>
       <c r="N149" s="16" t="inlineStr">
         <is>
-          <t>Inspect issue/settle GL + settlement reconciliation guard.</t>
+          <t>Inspect the item→category→literal precedence, the OFF-by-default parity, the postable-account fail-closed guard, and that reconcile sums the full inventory-account set.</t>
         </is>
       </c>
       <c r="O149" s="16" t="inlineStr">
         <is>
-          <t>Issue an advance (1180 up); settle 700+300 clears 1180; mismatched settle → SETTLE_MISMATCH (re-performed by the harness).</t>
+          <t>Re-perform (basics): flag OFF → item COGS override ignored, 5001 untouched (parity); enable posting_determination → goods issue routes COGS to the item's 5001 override (Dr 40) while inventory sub-ledger still reconciles to the GL account set; an override at a non-existent account → INVALID_POSTING_ACCOUNT (400).</t>
         </is>
       </c>
       <c r="P149" s="16" t="inlineStr">
         <is>
-          <t>Advance register; outstanding float</t>
+          <t>Feature-flag state + posting-rule/override config; harness ToE (basics GL-21)</t>
         </is>
       </c>
       <c r="Q149" s="18" t="inlineStr">
@@ -13831,7 +13831,7 @@
     <row r="150">
       <c r="A150" s="11" t="inlineStr">
         <is>
-          <t>EXP-08</t>
+          <t>EXP-07</t>
         </is>
       </c>
       <c r="B150" s="12" t="inlineStr">
@@ -13851,22 +13851,22 @@
       </c>
       <c r="E150" s="12" t="inlineStr">
         <is>
-          <t>Petty-cash disbursed beyond authority / without independent review, or drawn past the fund's limit — cash leakage, unauthorised or unrecorded expense, over-extended float.</t>
+          <t>Petty-cash / employee advance issued but never accounted for — cash leakage, expense unrecorded.</t>
         </is>
       </c>
       <c r="F150" s="12" t="inlineStr">
         <is>
-          <t>Authorization; Completeness</t>
+          <t>Existence/Completeness</t>
         </is>
       </c>
       <c r="G150" s="12" t="inlineStr">
         <is>
-          <t>Petty-cash imprest float + maker-checker on disbursement (SoD): a fund holds cash capped at a credit limit/วงเงิน (1015 Petty Cash, a cash account); each direct EXPENSE or ADVANCE is a REQUEST that posts NOTHING and a DIFFERENT user must approve before the GL posts (expense Dr &lt;expense&gt; / Cr 1015; advance Dr 1180 / Cr 1015) and the fund balance is decremented. Self-approval → SOD_VIOLATION (binds even Admin). A draw beyond the fund balance → INSUFFICIENT_FLOAT; establishing/replenishing above the float limit → OVER_FLOAT. Advances settle (Dr expense + Dr 1015 returned / Cr 1180), returning unused cash to the fund. Every request carries a document reference + receipt key + a status trail (StatusLog) and surfaces in the GOV-01 pending-approvals monitor.</t>
+          <t>Employee cash advances: issuing an advance debits the 1180 Employee Advances control (Dr 1180 / Cr 1000); settlement clears it against actual spend + returned cash (Dr expense + Dr 1000 / Cr 1180), enforced to reconcile (settled_expense + returned_cash must equal the advance → SETTLE_MISMATCH). The 1180 balance is the outstanding float subject to review.</t>
         </is>
       </c>
       <c r="H150" s="13" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I150" s="13" t="inlineStr">
@@ -13876,7 +13876,7 @@
       </c>
       <c r="J150" s="13" t="inlineStr">
         <is>
-          <t>Per disbursement</t>
+          <t>Per advance</t>
         </is>
       </c>
       <c r="K150" s="12" t="inlineStr">
@@ -13891,22 +13891,22 @@
       </c>
       <c r="M150" s="12" t="inlineStr">
         <is>
-          <t>petty-cash.service.ts (establishFund/replenishFund float guards, createRequest INSUFFICIENT_FLOAT, approveRequest SoD+GL, rejectRequest, settleRequest); petty-cash.controller.ts (creditors/exec); schema/petty-cash.ts (petty_cash_funds, expense_requests) + migration 0139; finance.service.ts pendingApprovals (GOV-01 source 7); cutover/basics.ts + compliance.ts (ToE)</t>
+          <t>finance.service.ts (issueAdvance, settleAdvance reconcile-or-reject, listAdvances outstanding); finance.controller.ts (creditors/exec); schema/finance.ts (employee_advances) + migration 0120; cutover/basics.ts (ToE)</t>
         </is>
       </c>
       <c r="N150" s="12" t="inlineStr">
         <is>
-          <t>Inspect the float ceiling + the request→approve flow + the approver≠requester check + that the request posts nothing until approval.</t>
+          <t>Inspect issue/settle GL + settlement reconciliation guard.</t>
         </is>
       </c>
       <c r="O150" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: establish a fund (Dr 1015), request an expense (no GL), self-approve → SOD_VIOLATION, approve as a different user → Dr expense/Cr 1015 + fund down; over-balance draw → INSUFFICIENT_FLOAT; advance approve→settle clears 1180; replenish past float → OVER_FLOAT (re-performed by the harnesses).</t>
+          <t>Issue an advance (1180 up); settle 700+300 clears 1180; mismatched settle → SETTLE_MISMATCH (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P150" s="12" t="inlineStr">
         <is>
-          <t>Fund register + disbursement approval log + SoD test</t>
+          <t>Advance register; outstanding float</t>
         </is>
       </c>
       <c r="Q150" s="18" t="inlineStr">
@@ -13918,7 +13918,7 @@
     <row r="151">
       <c r="A151" s="15" t="inlineStr">
         <is>
-          <t>EXP-09</t>
+          <t>EXP-08</t>
         </is>
       </c>
       <c r="B151" s="16" t="inlineStr">
@@ -13933,22 +13933,22 @@
       </c>
       <c r="D151" s="16" t="inlineStr">
         <is>
-          <t>Accounts Payable; Cash</t>
+          <t>Cash; Operating expense</t>
         </is>
       </c>
       <c r="E151" s="16" t="inlineStr">
         <is>
-          <t>A PO-based supplier invoice is paid before it is reconciled to its PO and goods receipt — disbursing cash for goods not received, at the wrong quantity, or above the agreed price (over-payment / duplicate / fictitious-receipt fraud), because the AP-pay flow never consults the 3-way match.</t>
+          <t>Petty-cash disbursed beyond authority / without independent review, or drawn past the fund's limit — cash leakage, unauthorised or unrecorded expense, over-extended float.</t>
         </is>
       </c>
       <c r="F151" s="16" t="inlineStr">
         <is>
-          <t>Occurrence/Accuracy/Authorization</t>
+          <t>Authorization; Completeness</t>
         </is>
       </c>
       <c r="G151" s="16" t="inlineStr">
         <is>
-          <t>3-way-match PAYMENT GATE: the AP disbursement flow (requestApPayment) calls ThreeWayMatchService.assertPayable BEFORE recording the payment request — a PO-based invoice that was run through match() and did NOT pass (qty/price variance beyond tolerance, over-invoiced, or unmatched line) and was NOT independently overridden is BLOCKED (MATCH_BLOCKED) so no cash can be requested or approved against it. The gate FAILS-OPEN for a non-PO bill (utilities / services / reimbursements never have a match row) so legitimate non-PO payables remain payable; it only blocks invoices subject to the match. Complements EXP-01 (the match + the maker-checked override) by wiring the verdict into the cash path and EXP-06 (the AP disbursement maker-checker).</t>
+          <t>Petty-cash imprest float + maker-checker on disbursement (SoD): a fund holds cash capped at a credit limit/วงเงิน (1015 Petty Cash, a cash account); each direct EXPENSE or ADVANCE is a REQUEST that posts NOTHING and a DIFFERENT user must approve before the GL posts (expense Dr &lt;expense&gt; / Cr 1015; advance Dr 1180 / Cr 1015) and the fund balance is decremented. Self-approval → SOD_VIOLATION (binds even Admin). A draw beyond the fund balance → INSUFFICIENT_FLOAT; establishing/replenishing above the float limit → OVER_FLOAT. Advances settle (Dr expense + Dr 1015 returned / Cr 1180), returning unused cash to the fund. Every request carries a document reference + receipt key + a status trail (StatusLog) and surfaces in the GOV-01 pending-approvals monitor.</t>
         </is>
       </c>
       <c r="H151" s="17" t="inlineStr">
@@ -13963,7 +13963,7 @@
       </c>
       <c r="J151" s="17" t="inlineStr">
         <is>
-          <t>Per payment</t>
+          <t>Per disbursement</t>
         </is>
       </c>
       <c r="K151" s="16" t="inlineStr">
@@ -13978,22 +13978,22 @@
       </c>
       <c r="M151" s="16" t="inlineStr">
         <is>
-          <t>finance.service.ts (requestApPayment → matchSvc.assertPayable); match/three-way-match.service.ts (assertPayable fail-open for non-PO, blocks not-payable &amp; not-overridden); finance.controller.ts (ap/transactions/:txnNo/pay); cutover/match.ts (ToE)</t>
+          <t>petty-cash.service.ts (establishFund/replenishFund float guards, createRequest INSUFFICIENT_FLOAT, approveRequest SoD+GL, rejectRequest, settleRequest); petty-cash.controller.ts (creditors/exec); schema/petty-cash.ts (petty_cash_funds, expense_requests) + migration 0139; finance.service.ts pendingApprovals (GOV-01 source 7); cutover/basics.ts + compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N151" s="16" t="inlineStr">
         <is>
-          <t>Inspect that the AP-pay request consults assertPayable and that a non-PO bill is exempt while a failed PO invoice is blocked.</t>
+          <t>Inspect the float ceiling + the request→approve flow + the approver≠requester check + that the request posts nothing until approval.</t>
         </is>
       </c>
       <c r="O151" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: a PO invoice with a qty/price variance over tolerance → pay request MATCH_BLOCKED; an independently-overridden / matched invoice → pay succeeds; a non-PO bill pays unblocked (re-performed by the match harness).</t>
+          <t>Re-perform: establish a fund (Dr 1015), request an expense (no GL), self-approve → SOD_VIOLATION, approve as a different user → Dr expense/Cr 1015 + fund down; over-balance draw → INSUFFICIENT_FLOAT; advance approve→settle clears 1180; replenish past float → OVER_FLOAT (re-performed by the harnesses).</t>
         </is>
       </c>
       <c r="P151" s="16" t="inlineStr">
         <is>
-          <t>Blocked-invoice worklist; payment-gate test</t>
+          <t>Fund register + disbursement approval log + SoD test</t>
         </is>
       </c>
       <c r="Q151" s="18" t="inlineStr">
@@ -14005,7 +14005,7 @@
     <row r="152">
       <c r="A152" s="11" t="inlineStr">
         <is>
-          <t>EXP-10</t>
+          <t>EXP-09</t>
         </is>
       </c>
       <c r="B152" s="12" t="inlineStr">
@@ -14020,22 +14020,22 @@
       </c>
       <c r="D152" s="12" t="inlineStr">
         <is>
-          <t>Accounts Payable</t>
+          <t>Accounts Payable; Cash</t>
         </is>
       </c>
       <c r="E152" s="12" t="inlineStr">
         <is>
-          <t>A scanned/keyed vendor invoice is booked against the wrong PO (or twice under the same invoice number), or an intake bill bypasses the 3-way match — a mis-mapped or duplicate document becomes a payable and cash is disbursed for it.</t>
+          <t>A PO-based supplier invoice is paid before it is reconciled to its PO and goods receipt — disbursing cash for goods not received, at the wrong quantity, or above the agreed price (over-payment / duplicate / fictitious-receipt fraud), because the AP-pay flow never consults the 3-way match.</t>
         </is>
       </c>
       <c r="F152" s="12" t="inlineStr">
         <is>
-          <t>Occurrence/Validity/Accuracy</t>
+          <t>Occurrence/Accuracy/Authorization</t>
         </is>
       </c>
       <c r="G152" s="12" t="inlineStr">
         <is>
-          <t>AP invoice INTAKE pipeline: a scanned invoice — pasted text or a DIRECT IMAGE/PDF UPLOAD (type/size-gated; a digital PDF extracts deterministically from its text layer, a photo/scan via AI vision when keyed, and with no key it queues for human review with empty fields so a blank bill can never book; the source document is stored on the intake for audit) — is extracted (doc-ai), AUTO-MAPPED to its PO (explicit PO number in the document, else vendor + amount scoring) and, on posting, the 3-way match is run in the SAME flow so an intake bill can never exist unmatched. The mapper only auto-maps an UNAMBIGUOUS winner — weak scores or tied candidates queue as NeedsReview for a human; a duplicate vendor invoice number (vs earlier intakes AND booked AP bills) is refused at post (DUPLICATE_INVOICE) and never auto-posted. Header-level matches enforce a CUMULATIVE guard (all invoices matched to a PO consume its received value, so one PO cannot be double-billed under two invoice numbers). A blocked intake invoice is released only by the scheduled auto re-match (ap_automatch_rerun) after the GR catches up, or by the EXP-01 maker-checked override. Booking (post/auto) requires the creditors duty; payment stays behind EXP-09's gate + EXP-06's maker-checker — the pipeline automates the path TO payment-ready, never the disbursement.</t>
+          <t>3-way-match PAYMENT GATE: the AP disbursement flow (requestApPayment) calls ThreeWayMatchService.assertPayable BEFORE recording the payment request — a PO-based invoice that was run through match() and did NOT pass (qty/price variance beyond tolerance, over-invoiced, or unmatched line) and was NOT independently overridden is BLOCKED (MATCH_BLOCKED) so no cash can be requested or approved against it. The gate FAILS-OPEN for a non-PO bill (utilities / services / reimbursements never have a match row) so legitimate non-PO payables remain payable; it only blocks invoices subject to the match. Complements EXP-01 (the match + the maker-checked override) by wiring the verdict into the cash path and EXP-06 (the AP disbursement maker-checker).</t>
         </is>
       </c>
       <c r="H152" s="13" t="inlineStr">
@@ -14050,37 +14050,37 @@
       </c>
       <c r="J152" s="13" t="inlineStr">
         <is>
-          <t>Per invoice</t>
+          <t>Per payment</t>
         </is>
       </c>
       <c r="K152" s="12" t="inlineStr">
         <is>
-          <t>AP / Procurement</t>
+          <t>AP / Controller</t>
         </is>
       </c>
       <c r="L152" s="13" t="inlineStr">
         <is>
-          <t>P17</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="M152" s="12" t="inlineStr">
         <is>
-          <t>ap-intake/ap-intake.service.ts (mapToPo, findDuplicate, post→match); ap-intake/ap-intake.controller.ts (post/auto gated creditors); doc-ai/doc-ai.service.ts (extraction incl. po_no); match/three-way-match.service.ts (header amount match + cumulative guard + rematchBlocked); bi.service.ts (ap_automatch_rerun); schema 0229 ap_invoice_intakes; cutover/match.ts (ToE)</t>
+          <t>finance.service.ts (requestApPayment → matchSvc.assertPayable); match/three-way-match.service.ts (assertPayable fail-open for non-PO, blocks not-payable &amp; not-overridden); finance.controller.ts (ap/transactions/:txnNo/pay); cutover/match.ts (ToE)</t>
         </is>
       </c>
       <c r="N152" s="12" t="inlineStr">
         <is>
-          <t>Inspect the mapper's ambiguity/duplicate handling and that posting always runs the match for a PO-mapped intake.</t>
+          <t>Inspect that the AP-pay request consults assertPayable and that a non-PO bill is exempt while a failed PO invoice is blocked.</t>
         </is>
       </c>
       <c r="O152" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: PO-numbered scan auto-posts matched+payable; tied candidates → NeedsReview; duplicate invoice no → 409 DUPLICATE_INVOICE; 2nd invoice on a fully-invoiced PO → over_invoiced blocked; invoice ahead of GR blocked then released by the scheduled re-match (re-performed by the match harness).</t>
+          <t>Re-perform: a PO invoice with a qty/price variance over tolerance → pay request MATCH_BLOCKED; an independently-overridden / matched invoice → pay succeeds; a non-PO bill pays unblocked (re-performed by the match harness).</t>
         </is>
       </c>
       <c r="P152" s="12" t="inlineStr">
         <is>
-          <t>Intake worklist; duplicate/cumulative guard tests</t>
+          <t>Blocked-invoice worklist; payment-gate test</t>
         </is>
       </c>
       <c r="Q152" s="18" t="inlineStr">
@@ -14092,12 +14092,12 @@
     <row r="153">
       <c r="A153" s="15" t="inlineStr">
         <is>
-          <t>FA-07</t>
+          <t>EXP-10</t>
         </is>
       </c>
       <c r="B153" s="16" t="inlineStr">
         <is>
-          <t>Fixed Assets</t>
+          <t>Expenditure</t>
         </is>
       </c>
       <c r="C153" s="17" t="inlineStr">
@@ -14107,27 +14107,27 @@
       </c>
       <c r="D153" s="16" t="inlineStr">
         <is>
-          <t>Property, Plant &amp; Equipment; Equity</t>
+          <t>Accounts Payable</t>
         </is>
       </c>
       <c r="E153" s="16" t="inlineStr">
         <is>
-          <t>Carrying amount not adjusted for revaluation/impairment — asset over/understated.</t>
+          <t>A scanned/keyed vendor invoice is booked against the wrong PO (or twice under the same invoice number), or an intake bill bypasses the 3-way match — a mis-mapped or duplicate document becomes a payable and cash is disbursed for it.</t>
         </is>
       </c>
       <c r="F153" s="16" t="inlineStr">
         <is>
-          <t>Valuation</t>
+          <t>Occurrence/Validity/Accuracy</t>
         </is>
       </c>
       <c r="G153" s="16" t="inlineStr">
         <is>
-          <t>Asset revaluation / impairment: an upward revaluation credits the revaluation surplus in equity (Dr 1500 / Cr 3200); a downward revaluation (impairment) debits impairment loss (Dr 5820 / Cr 1500). The gross 1500 moves by the delta so the register stays tied to the GL; a no-op revaluation is rejected (NO_CHANGE). Every event is logged for the audit trail.</t>
+          <t>AP invoice INTAKE pipeline: a scanned invoice — pasted text or a DIRECT IMAGE/PDF UPLOAD (type/size-gated; a digital PDF extracts deterministically from its text layer, a photo/scan via AI vision when keyed, and with no key it queues for human review with empty fields so a blank bill can never book; the source document is stored on the intake for audit) — is extracted (doc-ai), AUTO-MAPPED to its PO (explicit PO number in the document, else vendor + amount scoring) and, on posting, the 3-way match is run in the SAME flow so an intake bill can never exist unmatched. The mapper only auto-maps an UNAMBIGUOUS winner — weak scores or tied candidates queue as NeedsReview for a human; a duplicate vendor invoice number (vs earlier intakes AND booked AP bills) is refused at post (DUPLICATE_INVOICE) and never auto-posted. Header-level matches enforce a CUMULATIVE guard (all invoices matched to a PO consume its received value, so one PO cannot be double-billed under two invoice numbers). A blocked intake invoice is released only by the scheduled auto re-match (ap_automatch_rerun) after the GR catches up, or by the EXP-01 maker-checked override. Booking (post/auto) requires the creditors duty; payment stays behind EXP-09's gate + EXP-06's maker-checker — the pipeline automates the path TO payment-ready, never the disbursement.</t>
         </is>
       </c>
       <c r="H153" s="17" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I153" s="17" t="inlineStr">
@@ -14137,37 +14137,37 @@
       </c>
       <c r="J153" s="17" t="inlineStr">
         <is>
-          <t>Per event</t>
+          <t>Per invoice</t>
         </is>
       </c>
       <c r="K153" s="16" t="inlineStr">
         <is>
-          <t>FaAccountant / Controller</t>
+          <t>AP / Procurement</t>
         </is>
       </c>
       <c r="L153" s="17" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P17</t>
         </is>
       </c>
       <c r="M153" s="16" t="inlineStr">
         <is>
-          <t>assets.service.ts (revalue up→3200 / down→5820, listRevaluations; dispose recycles surplus 3200→3100); assets.controller.ts (exec/creditors); schema/assets.ts (asset_revaluations) + migration 0120; cutover/basics.ts (ToE)</t>
+          <t>ap-intake/ap-intake.service.ts (mapToPo, findDuplicate, post→match); ap-intake/ap-intake.controller.ts (post/auto gated creditors); doc-ai/doc-ai.service.ts (extraction incl. po_no); match/three-way-match.service.ts (header amount match + cumulative guard + rematchBlocked); bi.service.ts (ap_automatch_rerun); schema 0229 ap_invoice_intakes; cutover/match.ts (ToE)</t>
         </is>
       </c>
       <c r="N153" s="16" t="inlineStr">
         <is>
-          <t>Inspect revaluation/impairment routing + audit log + disposal recycling.</t>
+          <t>Inspect the mapper's ambiguity/duplicate handling and that posting always runs the match for a PO-mapped intake.</t>
         </is>
       </c>
       <c r="O153" s="16" t="inlineStr">
         <is>
-          <t>Upward revaluation credits 3200; impairment debits 5820; no-change → NO_CHANGE; both events logged; on disposal the revaluation surplus is recycled to retained earnings (Dr 3200 / Cr 3100), not through P&amp;L (re-performed by the harness).</t>
+          <t>Re-perform: PO-numbered scan auto-posts matched+payable; tied candidates → NeedsReview; duplicate invoice no → 409 DUPLICATE_INVOICE; 2nd invoice on a fully-invoiced PO → over_invoiced blocked; invoice ahead of GR blocked then released by the scheduled re-match (re-performed by the match harness).</t>
         </is>
       </c>
       <c r="P153" s="16" t="inlineStr">
         <is>
-          <t>Revaluation log; disposal recycling JE</t>
+          <t>Intake worklist; duplicate/cumulative guard tests</t>
         </is>
       </c>
       <c r="Q153" s="18" t="inlineStr">
@@ -14179,7 +14179,7 @@
     <row r="154">
       <c r="A154" s="11" t="inlineStr">
         <is>
-          <t>FA-08</t>
+          <t>FA-07</t>
         </is>
       </c>
       <c r="B154" s="12" t="inlineStr">
@@ -14199,22 +14199,22 @@
       </c>
       <c r="E154" s="12" t="inlineStr">
         <is>
-          <t>Carrying amount changed by fair-value revaluation/impairment without independent review — the preparer revalues the asset and posts to equity/P&amp;L on their own (earnings/equity management).</t>
+          <t>Carrying amount not adjusted for revaluation/impairment — asset over/understated.</t>
         </is>
       </c>
       <c r="F154" s="12" t="inlineStr">
         <is>
-          <t>Authorization</t>
+          <t>Valuation</t>
         </is>
       </c>
       <c r="G154" s="12" t="inlineStr">
         <is>
-          <t>Asset-revaluation maker-checker (SoD): a revalue/impairment request posts its GL entry as a DRAFT (excluded from balances) and records status 'PendingApproval' WITHOUT moving the carrying value; a DIFFERENT user must approve before the JE is effective and the register is re-valued (approver ≠ preparer enforced regardless of permissions, reusing the GL-05 ledger approval). Reject voids the draft; only one revaluation may be pending per asset; the disposal surplus recycle counts only approved revaluations.</t>
+          <t>Asset revaluation / impairment: an upward revaluation credits the revaluation surplus in equity (Dr 1500 / Cr 3200); a downward revaluation (impairment) debits impairment loss (Dr 5820 / Cr 1500). The gross 1500 moves by the delta so the register stays tied to the GL; a no-op revaluation is rejected (NO_CHANGE). Every event is logged for the audit trail.</t>
         </is>
       </c>
       <c r="H154" s="13" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I154" s="13" t="inlineStr">
@@ -14239,22 +14239,22 @@
       </c>
       <c r="M154" s="12" t="inlineStr">
         <is>
-          <t>assets.service.ts revalue(pendingApproval Draft)/approveRevaluation/rejectRevaluation; assets.controller.ts (:assetNo/revalue/approve|reject); schema/assets.ts asset_revaluations.status + migration 0134; cutover/basics.ts + compliance.ts (ToE)</t>
+          <t>assets.service.ts (revalue up→3200 / down→5820, listRevaluations; dispose recycles surplus 3200→3100); assets.controller.ts (exec/creditors); schema/assets.ts (asset_revaluations) + migration 0120; cutover/basics.ts (ToE)</t>
         </is>
       </c>
       <c r="N154" s="12" t="inlineStr">
         <is>
-          <t>Inspect Draft→approve flow + the approver≠preparer check + deferred carrying-value update.</t>
+          <t>Inspect revaluation/impairment routing + audit log + disposal recycling.</t>
         </is>
       </c>
       <c r="O154" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: request a revaluation (Draft JE excluded from 3200), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm the surplus/impairment + carrying value move only after approval (re-performed by the harnesses).</t>
+          <t>Upward revaluation credits 3200; impairment debits 5820; no-change → NO_CHANGE; both events logged; on disposal the revaluation surplus is recycled to retained earnings (Dr 3200 / Cr 3100), not through P&amp;L (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P154" s="12" t="inlineStr">
         <is>
-          <t>Revaluation approval log + SoD test</t>
+          <t>Revaluation log; disposal recycling JE</t>
         </is>
       </c>
       <c r="Q154" s="18" t="inlineStr">
@@ -14266,12 +14266,12 @@
     <row r="155">
       <c r="A155" s="15" t="inlineStr">
         <is>
-          <t>LSE-01</t>
+          <t>FA-08</t>
         </is>
       </c>
       <c r="B155" s="16" t="inlineStr">
         <is>
-          <t>Leases</t>
+          <t>Fixed Assets</t>
         </is>
       </c>
       <c r="C155" s="17" t="inlineStr">
@@ -14281,27 +14281,27 @@
       </c>
       <c r="D155" s="16" t="inlineStr">
         <is>
-          <t>Right-of-use assets; Lease liabilities</t>
+          <t>Property, Plant &amp; Equipment; Equity</t>
         </is>
       </c>
       <c r="E155" s="16" t="inlineStr">
         <is>
-          <t>Lease not capitalised (IFRS 16 / TFRS 16) — ROU asset + lease liability omitted; interest/depreciation mis-stated.</t>
+          <t>Carrying amount changed by fair-value revaluation/impairment without independent review — the preparer revalues the asset and posts to equity/P&amp;L on their own (earnings/equity management).</t>
         </is>
       </c>
       <c r="F155" s="16" t="inlineStr">
         <is>
-          <t>Completeness/Accuracy/Valuation</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="G155" s="16" t="inlineStr">
         <is>
-          <t>Lease accounting: at commencement a right-of-use asset and lease liability are recognised at the present value of the lease payments (Dr 1600 / Cr 2600). The scheduled job lease_periodic_run posts each period — interest unwinding on the liability (Dr 5900), the cash payment reducing the liability (Dr 2600 / Cr 1000), and straight-line ROU depreciation (Dr 5210 / Cr 1690) — the last period clearing the liability + ROU exactly. Idempotent per (lease, period).</t>
+          <t>Asset-revaluation maker-checker (SoD): a revalue/impairment request posts its GL entry as a DRAFT (excluded from balances) and records status 'PendingApproval' WITHOUT moving the carrying value; a DIFFERENT user must approve before the JE is effective and the register is re-valued (approver ≠ preparer enforced regardless of permissions, reusing the GL-05 ledger approval). Reject voids the draft; only one revaluation may be pending per asset; the disposal surplus recycle counts only approved revaluations.</t>
         </is>
       </c>
       <c r="H155" s="17" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I155" s="17" t="inlineStr">
@@ -14311,12 +14311,12 @@
       </c>
       <c r="J155" s="17" t="inlineStr">
         <is>
-          <t>Per period / per lease</t>
+          <t>Per event</t>
         </is>
       </c>
       <c r="K155" s="16" t="inlineStr">
         <is>
-          <t>Controller</t>
+          <t>FaAccountant / Controller</t>
         </is>
       </c>
       <c r="L155" s="17" t="inlineStr">
@@ -14326,22 +14326,22 @@
       </c>
       <c r="M155" s="16" t="inlineStr">
         <is>
-          <t>leases.service.ts (createLease PV recognition, runDueLeases interest+payment+depreciation, modifyLease remeasurement); leases.controller.ts (gl_post); bi.service.ts (lease_periodic_run); schema/leases.ts (leases, rou_nbv) + migration 0120/0121; cutover/basics.ts (ToE)</t>
+          <t>assets.service.ts revalue(pendingApproval Draft)/approveRevaluation/rejectRevaluation; assets.controller.ts (:assetNo/revalue/approve|reject); schema/assets.ts asset_revaluations.status + migration 0134; cutover/basics.ts + compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N155" s="16" t="inlineStr">
         <is>
-          <t>Inspect PV recognition + periodic interest/payment/depreciation + final-period clearing + modification remeasurement.</t>
+          <t>Inspect Draft→approve flow + the approver≠preparer check + deferred carrying-value update.</t>
         </is>
       </c>
       <c r="O155" s="16" t="inlineStr">
         <is>
-          <t>Commencement recognises ROU=liability=PV; periodic run posts interest+principal(=payment)+ROU depreciation; liability + ROU reduce; a modification remeasures the liability at the revised PV and adjusts the ROU by the same delta (Dr/Cr 1600↔2600), then depreciates over the remaining term (re-performed by the harness).</t>
+          <t>Re-perform: request a revaluation (Draft JE excluded from 3200), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm the surplus/impairment + carrying value move only after approval (re-performed by the harnesses).</t>
         </is>
       </c>
       <c r="P155" s="16" t="inlineStr">
         <is>
-          <t>Lease register; periodic run log; modification remeasurement</t>
+          <t>Revaluation approval log + SoD test</t>
         </is>
       </c>
       <c r="Q155" s="18" t="inlineStr">
@@ -14353,12 +14353,12 @@
     <row r="156">
       <c r="A156" s="11" t="inlineStr">
         <is>
-          <t>REC-01</t>
+          <t>LSE-01</t>
         </is>
       </c>
       <c r="B156" s="12" t="inlineStr">
         <is>
-          <t>Reconciliation</t>
+          <t>Leases</t>
         </is>
       </c>
       <c r="C156" s="13" t="inlineStr">
@@ -14368,22 +14368,22 @@
       </c>
       <c r="D156" s="12" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Right-of-use assets; Lease liabilities</t>
         </is>
       </c>
       <c r="E156" s="12" t="inlineStr">
         <is>
-          <t>Subledgers diverge from GL undetected.</t>
+          <t>Lease not capitalised (IFRS 16 / TFRS 16) — ROU asset + lease liability omitted; interest/depreciation mis-stated.</t>
         </is>
       </c>
       <c r="F156" s="12" t="inlineStr">
         <is>
-          <t>Completeness/Accuracy</t>
+          <t>Completeness/Accuracy/Valuation</t>
         </is>
       </c>
       <c r="G156" s="12" t="inlineStr">
         <is>
-          <t>Subledger-to-GL reconciliation per period: import GL, auto-match, certify (sign-off via 'approvals').</t>
+          <t>Lease accounting: at commencement a right-of-use asset and lease liability are recognised at the present value of the lease payments (Dr 1600 / Cr 2600). The scheduled job lease_periodic_run posts each period — interest unwinding on the liability (Dr 5900), the cash payment reducing the liability (Dr 2600 / Cr 1000), and straight-line ROU depreciation (Dr 5210 / Cr 1690) — the last period clearing the liability + ROU exactly. Idempotent per (lease, period).</t>
         </is>
       </c>
       <c r="H156" s="13" t="inlineStr">
@@ -14393,12 +14393,12 @@
       </c>
       <c r="I156" s="13" t="inlineStr">
         <is>
-          <t>Auto+Manual</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J156" s="13" t="inlineStr">
         <is>
-          <t>Monthly</t>
+          <t>Per period / per lease</t>
         </is>
       </c>
       <c r="K156" s="12" t="inlineStr">
@@ -14408,27 +14408,27 @@
       </c>
       <c r="L156" s="13" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="M156" s="12" t="inlineStr">
         <is>
-          <t>reconciliation.service.ts (importGlItems/autoMatch/certify)</t>
+          <t>leases.service.ts (createLease PV recognition, runDueLeases interest+payment+depreciation, modifyLease remeasurement); leases.controller.ts (gl_post); bi.service.ts (lease_periodic_run); schema/leases.ts (leases, rou_nbv) + migration 0120/0121; cutover/basics.ts (ToE)</t>
         </is>
       </c>
       <c r="N156" s="12" t="inlineStr">
         <is>
-          <t>Inspect recon + certify gate.</t>
+          <t>Inspect PV recognition + periodic interest/payment/depreciation + final-period clearing + modification remeasurement.</t>
         </is>
       </c>
       <c r="O156" s="12" t="inlineStr">
         <is>
-          <t>Sample periods: reconciled, unmatched cleared, certified.</t>
+          <t>Commencement recognises ROU=liability=PV; periodic run posts interest+principal(=payment)+ROU depreciation; liability + ROU reduce; a modification remeasures the liability at the revised PV and adjusts the ROU by the same delta (Dr/Cr 1600↔2600), then depreciates over the remaining term (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P156" s="12" t="inlineStr">
         <is>
-          <t>Certified recon</t>
+          <t>Lease register; periodic run log; modification remeasurement</t>
         </is>
       </c>
       <c r="Q156" s="18" t="inlineStr">
@@ -14440,7 +14440,7 @@
     <row r="157">
       <c r="A157" s="15" t="inlineStr">
         <is>
-          <t>REC-02</t>
+          <t>REC-01</t>
         </is>
       </c>
       <c r="B157" s="16" t="inlineStr">
@@ -14455,22 +14455,22 @@
       </c>
       <c r="D157" s="16" t="inlineStr">
         <is>
-          <t>Cash</t>
+          <t>All</t>
         </is>
       </c>
       <c r="E157" s="16" t="inlineStr">
         <is>
-          <t>Bank balance not reconciled to GL.</t>
+          <t>Subledgers diverge from GL undetected.</t>
         </is>
       </c>
       <c r="F157" s="16" t="inlineStr">
         <is>
-          <t>Existence/Completeness</t>
+          <t>Completeness/Accuracy</t>
         </is>
       </c>
       <c r="G157" s="16" t="inlineStr">
         <is>
-          <t>Bank reconciliation against statements.</t>
+          <t>Subledger-to-GL reconciliation per period: import GL, auto-match, certify (sign-off via 'approvals').</t>
         </is>
       </c>
       <c r="H157" s="17" t="inlineStr">
@@ -14500,22 +14500,22 @@
       </c>
       <c r="M157" s="16" t="inlineStr">
         <is>
-          <t>bank module; drizzle/0015_bank_reconciliation</t>
+          <t>reconciliation.service.ts (importGlItems/autoMatch/certify)</t>
         </is>
       </c>
       <c r="N157" s="16" t="inlineStr">
         <is>
-          <t>Inspect bank-rec process.</t>
+          <t>Inspect recon + certify gate.</t>
         </is>
       </c>
       <c r="O157" s="16" t="inlineStr">
         <is>
-          <t>Sample months reconciled &amp; reviewed.</t>
+          <t>Sample periods: reconciled, unmatched cleared, certified.</t>
         </is>
       </c>
       <c r="P157" s="16" t="inlineStr">
         <is>
-          <t>Bank rec</t>
+          <t>Certified recon</t>
         </is>
       </c>
       <c r="Q157" s="18" t="inlineStr">
@@ -14527,12 +14527,12 @@
     <row r="158">
       <c r="A158" s="11" t="inlineStr">
         <is>
-          <t>BANK-02</t>
+          <t>REC-02</t>
         </is>
       </c>
       <c r="B158" s="12" t="inlineStr">
         <is>
-          <t>Cash &amp; Treasury</t>
+          <t>Reconciliation</t>
         </is>
       </c>
       <c r="C158" s="13" t="inlineStr">
@@ -14542,37 +14542,37 @@
       </c>
       <c r="D158" s="12" t="inlineStr">
         <is>
-          <t>Cash; Operating expense; Interest income</t>
+          <t>Cash</t>
         </is>
       </c>
       <c r="E158" s="12" t="inlineStr">
         <is>
-          <t>A bank fee/interest adjustment is posted straight to the GL by one person during reconciliation — a cash outflow mis-booked as interest income, or a fictitious fee posted, with no independent review (single-person posting to the cash account).</t>
+          <t>Bank balance not reconciled to GL.</t>
         </is>
       </c>
       <c r="F158" s="12" t="inlineStr">
         <is>
-          <t>Authorization/Accuracy</t>
+          <t>Existence/Completeness</t>
         </is>
       </c>
       <c r="G158" s="12" t="inlineStr">
         <is>
-          <t>Bank adjustment maker-checker (SoD): a fee/interest adjustment on a statement line is a REQUEST that posts a DRAFT JE (no balance/GL effect; the line stays unreconciled) until a DIFFERENT user with approval authority approves (POST /api/bank/lines/:id/adjustment/approve). Self-approval → SOD_VIOLATION (binds even Admin); approval flips the line to reconciled and the JE to Posted; reject voids the Draft and frees the line. The Draft JE (source BANKADJ) is also surfaced, aged, by the pending-approvals monitor (GOV-01).</t>
+          <t>Bank reconciliation against statements.</t>
         </is>
       </c>
       <c r="H158" s="13" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I158" s="13" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="J158" s="13" t="inlineStr">
         <is>
-          <t>Per adjustment</t>
+          <t>Monthly</t>
         </is>
       </c>
       <c r="K158" s="12" t="inlineStr">
@@ -14582,27 +14582,27 @@
       </c>
       <c r="L158" s="13" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="M158" s="12" t="inlineStr">
         <is>
-          <t>bank.service.ts requestAdjustment/approveAdjustment/rejectAdjustment/listPendingAdjustments (reuses ledger.approveEntry SoD); bank.controller.ts (lines/:id/adjustment requests; adjustment/approve|reject gated approvals/gl_close); cutover/bankrec.ts (ToE)</t>
+          <t>bank module; drizzle/0015_bank_reconciliation</t>
         </is>
       </c>
       <c r="N158" s="12" t="inlineStr">
         <is>
-          <t>Inspect the request→approve flow + the approver≠requester check + that the Draft posts nothing until approval.</t>
+          <t>Inspect bank-rec process.</t>
         </is>
       </c>
       <c r="O158" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: request a fee adjustment (line unreconciled, GL difference unchanged), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm the difference closes to 0 only after approval (re-performed by the bankrec harness).</t>
+          <t>Sample months reconciled &amp; reviewed.</t>
         </is>
       </c>
       <c r="P158" s="12" t="inlineStr">
         <is>
-          <t>Bank adjustment queue + SoD test</t>
+          <t>Bank rec</t>
         </is>
       </c>
       <c r="Q158" s="18" t="inlineStr">
@@ -14614,12 +14614,12 @@
     <row r="159">
       <c r="A159" s="15" t="inlineStr">
         <is>
-          <t>REC-03</t>
+          <t>BANK-02</t>
         </is>
       </c>
       <c r="B159" s="16" t="inlineStr">
         <is>
-          <t>Reconciliation</t>
+          <t>Cash &amp; Treasury</t>
         </is>
       </c>
       <c r="C159" s="17" t="inlineStr">
@@ -14629,67 +14629,67 @@
       </c>
       <c r="D159" s="16" t="inlineStr">
         <is>
-          <t>Consolidation</t>
+          <t>Cash; Operating expense; Interest income</t>
         </is>
       </c>
       <c r="E159" s="16" t="inlineStr">
         <is>
-          <t>Intercompany balances eliminated without an independent reconciliation sign-off.</t>
+          <t>A bank fee/interest adjustment is posted straight to the GL by one person during reconciliation — a cash outflow mis-booked as interest income, or a fictitious fee posted, with no independent review (single-person posting to the cash account).</t>
         </is>
       </c>
       <c r="F159" s="16" t="inlineStr">
         <is>
-          <t>Accuracy</t>
+          <t>Authorization/Accuracy</t>
         </is>
       </c>
       <c r="G159" s="16" t="inlineStr">
         <is>
-          <t>Per-period intercompany reconciliation sign-off (maker-checker) GATES consolidation elimination: a preparer reconciles the group's IC balances (Due-From 1150 vs Due-To 2150) for the period and signs (Prepared); an independent approver (SoD, approver ≠ preparer) approves only when the balances eliminate (Due-From = Due-To). consolidation.runConsolidation() is hard-gated — it refuses to eliminate until the period's reconciliation is Approved (IC_RECON_NOT_APPROVED).</t>
+          <t>Bank adjustment maker-checker (SoD): a fee/interest adjustment on a statement line is a REQUEST that posts a DRAFT JE (no balance/GL effect; the line stays unreconciled) until a DIFFERENT user with approval authority approves (POST /api/bank/lines/:id/adjustment/approve). Self-approval → SOD_VIOLATION (binds even Admin); approval flips the line to reconciled and the JE to Posted; reject voids the Draft and frees the line. The Draft JE (source BANKADJ) is also surfaced, aged, by the pending-approvals monitor (GOV-01).</t>
         </is>
       </c>
       <c r="H159" s="17" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I159" s="17" t="inlineStr">
         <is>
-          <t>Auto+Manual</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J159" s="17" t="inlineStr">
         <is>
-          <t>Period</t>
+          <t>Per adjustment</t>
         </is>
       </c>
       <c r="K159" s="16" t="inlineStr">
         <is>
-          <t>Group Controller</t>
+          <t>Controller</t>
         </is>
       </c>
       <c r="L159" s="17" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="M159" s="16" t="inlineStr">
         <is>
-          <t>modules/ic-reconciliation/ic-recon.service.ts (prepare/approve, SoD + eliminates gate); consolidation.service.ts runConsolidation (IC_RECON_NOT_APPROVED gate); ic_recon_periods (0205, RLS); cutover/consolidation.ts (ToE)</t>
+          <t>bank.service.ts requestAdjustment/approveAdjustment/rejectAdjustment/listPendingAdjustments (reuses ledger.approveEntry SoD); bank.controller.ts (lines/:id/adjustment requests; adjustment/approve|reject gated approvals/gl_close); cutover/bankrec.ts (ToE)</t>
         </is>
       </c>
       <c r="N159" s="16" t="inlineStr">
         <is>
-          <t>Inspect the per-period IC reconciliation sign-off + the consolidation gate.</t>
+          <t>Inspect the request→approve flow + the approver≠requester check + that the Draft posts nothing until approval.</t>
         </is>
       </c>
       <c r="O159" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: consolidation is blocked before sign-off (IC_RECON_NOT_APPROVED); the preparer cannot approve their own reconciliation (SOD_VIOLATION); an independent approver signs off (balances eliminate) → consolidation proceeds.</t>
+          <t>Re-perform: request a fee adjustment (line unreconciled, GL difference unchanged), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm the difference closes to 0 only after approval (re-performed by the bankrec harness).</t>
         </is>
       </c>
       <c r="P159" s="16" t="inlineStr">
         <is>
-          <t>IC reconciliation sign-off + consolidation gate ToE</t>
+          <t>Bank adjustment queue + SoD test</t>
         </is>
       </c>
       <c r="Q159" s="18" t="inlineStr">
@@ -14701,7 +14701,7 @@
     <row r="160">
       <c r="A160" s="11" t="inlineStr">
         <is>
-          <t>REC-04</t>
+          <t>REC-03</t>
         </is>
       </c>
       <c r="B160" s="12" t="inlineStr">
@@ -14716,22 +14716,22 @@
       </c>
       <c r="D160" s="12" t="inlineStr">
         <is>
-          <t>All control accounts</t>
+          <t>Consolidation</t>
         </is>
       </c>
       <c r="E160" s="12" t="inlineStr">
         <is>
-          <t>A sub-ledger silently drifts from its GL control account at period-end and no single review catches it (incomplete/inaccurate balances reach the financial statements).</t>
+          <t>Intercompany balances eliminated without an independent reconciliation sign-off.</t>
         </is>
       </c>
       <c r="F160" s="12" t="inlineStr">
         <is>
-          <t>Completeness/Accuracy</t>
+          <t>Accuracy</t>
         </is>
       </c>
       <c r="G160" s="12" t="inlineStr">
         <is>
-          <t>Period-end control-account reconciliation PACK: one read (GET /api/finance/reconciliation/controls) ties every major sub-ledger to its GL control account and FLAGS any out-of-balance — AR↔1100, AP↔2000, Inventory↔1200, Gift cards/Customer-deposits↔2200, Deferred revenue↔2400 — reporting per line {sub_ledger, gl_control, variance, reconciled} plus an overall all_reconciled flag and an exceptions count. Liability controls are sign-flipped before comparison. The controller's single 'are the books reconciled?' close view; an exception is a control finding to investigate before sign-off.</t>
+          <t>Per-period intercompany reconciliation sign-off (maker-checker) GATES consolidation elimination: a preparer reconciles the group's IC balances (Due-From 1150 vs Due-To 2150) for the period and signs (Prepared); an independent approver (SoD, approver ≠ preparer) approves only when the balances eliminate (Due-From = Due-To). consolidation.runConsolidation() is hard-gated — it refuses to eliminate until the period's reconciliation is Approved (IC_RECON_NOT_APPROVED).</t>
         </is>
       </c>
       <c r="H160" s="13" t="inlineStr">
@@ -14741,17 +14741,17 @@
       </c>
       <c r="I160" s="13" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="J160" s="13" t="inlineStr">
         <is>
-          <t>Period / on demand</t>
+          <t>Period</t>
         </is>
       </c>
       <c r="K160" s="12" t="inlineStr">
         <is>
-          <t>Controller / CFO</t>
+          <t>Group Controller</t>
         </is>
       </c>
       <c r="L160" s="13" t="inlineStr">
@@ -14761,22 +14761,22 @@
       </c>
       <c r="M160" s="12" t="inlineStr">
         <is>
-          <t>finance.service.ts reconcileControls; finance.controller.ts GET reconciliation/controls (exec/ar/creditors); reuses ledger.trialBalance + the AR/AP/inventory/gift-card/deferred sub-ledgers; cutover/giftcards.ts + compliance.ts (ToE)</t>
+          <t>modules/ic-reconciliation/ic-recon.service.ts (prepare/approve, SoD + eliminates gate); consolidation.service.ts runConsolidation (IC_RECON_NOT_APPROVED gate); ic_recon_periods (0205, RLS); cutover/consolidation.ts (ToE)</t>
         </is>
       </c>
       <c r="N160" s="12" t="inlineStr">
         <is>
-          <t>Inspect the pack: each control account's sub-ledger query + the GL tie + the exceptions roll-up.</t>
+          <t>Inspect the per-period IC reconciliation sign-off + the consolidation gate.</t>
         </is>
       </c>
       <c r="O160" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: with a clean set, every line reconciled + all_reconciled=true; introduce a known sub-ledger/GL difference and confirm it surfaces as an exception (re-performed: gift-card 2200 + inventory 1200 ties asserted by the harnesses).</t>
+          <t>Re-perform: consolidation is blocked before sign-off (IC_RECON_NOT_APPROVED); the preparer cannot approve their own reconciliation (SOD_VIOLATION); an independent approver signs off (balances eliminate) → consolidation proceeds.</t>
         </is>
       </c>
       <c r="P160" s="12" t="inlineStr">
         <is>
-          <t>Reconciliation pack; exceptions list</t>
+          <t>IC reconciliation sign-off + consolidation gate ToE</t>
         </is>
       </c>
       <c r="Q160" s="18" t="inlineStr">
@@ -14788,7 +14788,7 @@
     <row r="161">
       <c r="A161" s="15" t="inlineStr">
         <is>
-          <t>REC-05</t>
+          <t>REC-04</t>
         </is>
       </c>
       <c r="B161" s="16" t="inlineStr">
@@ -14803,42 +14803,42 @@
       </c>
       <c r="D161" s="16" t="inlineStr">
         <is>
-          <t>Cash; Bank</t>
+          <t>All control accounts</t>
         </is>
       </c>
       <c r="E161" s="16" t="inlineStr">
         <is>
-          <t>Till cash dropped to the safe never reaches the bank, or a deposit isn't matched to the statement — cash sits unbanked (theft/loss exposure) or the bank balance can't be tied to the books.</t>
+          <t>A sub-ledger silently drifts from its GL control account at period-end and no single review catches it (incomplete/inaccurate balances reach the financial statements).</t>
         </is>
       </c>
       <c r="F161" s="16" t="inlineStr">
         <is>
-          <t>Completeness/Existence/Authorization</t>
+          <t>Completeness/Accuracy</t>
         </is>
       </c>
       <c r="G161" s="16" t="inlineStr">
         <is>
-          <t>Cash banking — safe-drop → bank deposit → reconciliation: till 'drop's move cash from the drawer to the safe (drawer-only, no GL). Banking BATCHES the undeposited drops into a deposit and posts the GL (Dr &lt;bank account, e.g. 1010&gt; / Cr 1000 Cash), stamping each drop with the deposit id; the deposit is then RECONCILED to the bank statement (status Deposited→Reconciled). A detective read (GET /api/bank/deposits/undeposited-drops) surfaces the CASH STILL IN THE SAFE (drops with deposit_id NULL) — the unbanked exposure to chase. SoD: banking is a treasury duty (exec/ar) — segregated from the cashier (pos_till) who drops the cash, so the person who removes cash from the drawer is not the one who banks it.</t>
+          <t>Period-end control-account reconciliation PACK: one read (GET /api/finance/reconciliation/controls) ties every major sub-ledger to its GL control account and FLAGS any out-of-balance — AR↔1100, AP↔2000, Inventory↔1200, Gift cards/Customer-deposits↔2200, Deferred revenue↔2400 — reporting per line {sub_ledger, gl_control, variance, reconciled} plus an overall all_reconciled flag and an exceptions count. Liability controls are sign-flipped before comparison. The controller's single 'are the books reconciled?' close view; an exception is a control finding to investigate before sign-off.</t>
         </is>
       </c>
       <c r="H161" s="17" t="inlineStr">
         <is>
-          <t>Det/Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I161" s="17" t="inlineStr">
         <is>
-          <t>Auto+Manual</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J161" s="17" t="inlineStr">
         <is>
-          <t>Per banking run</t>
+          <t>Period / on demand</t>
         </is>
       </c>
       <c r="K161" s="16" t="inlineStr">
         <is>
-          <t>FinancialController / Treasury</t>
+          <t>Controller / CFO</t>
         </is>
       </c>
       <c r="L161" s="17" t="inlineStr">
@@ -14848,22 +14848,22 @@
       </c>
       <c r="M161" s="16" t="inlineStr">
         <is>
-          <t>bank.service.ts undepositedDrops/createDeposit (Dr bank/Cr 1000, stamps deposit_id)/reconcileDeposit/listDeposits; bank.controller.ts (deposits, deposits/undeposited-drops, deposits/:id/reconcile; exec/ar); schema/cash.ts bank_deposits + cash_movements.deposit_id + migration 0152; /cash-banking UI; cutover/cash-banking.ts (ToE)</t>
+          <t>finance.service.ts reconcileControls; finance.controller.ts GET reconciliation/controls (exec/ar/creditors); reuses ledger.trialBalance + the AR/AP/inventory/gift-card/deferred sub-ledgers; cutover/giftcards.ts + compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N161" s="16" t="inlineStr">
         <is>
-          <t>Inspect the undeposited-drop exposure read + the deposit GL (bank↔1000) + the reconcile step + the SoD (cashier vs treasury).</t>
+          <t>Inspect the pack: each control account's sub-ledger query + the GL tie + the exceptions roll-up.</t>
         </is>
       </c>
       <c r="O161" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: two till drops → cash-in-safe shows the total; a cashier (pos_till) cannot bank (403); treasury banks → Dr bank / Cr 1000, cash-in-safe back to 0; reconcile the deposit; trial balance balanced (re-performed by the cash-banking harness).</t>
+          <t>Re-perform: with a clean set, every line reconciled + all_reconciled=true; introduce a known sub-ledger/GL difference and confirm it surfaces as an exception (re-performed: gift-card 2200 + inventory 1200 ties asserted by the harnesses).</t>
         </is>
       </c>
       <c r="P161" s="16" t="inlineStr">
         <is>
-          <t>Bank-deposit register; undeposited-drop (cash-in-safe) exposure</t>
+          <t>Reconciliation pack; exceptions list</t>
         </is>
       </c>
       <c r="Q161" s="18" t="inlineStr">
@@ -14875,12 +14875,12 @@
     <row r="162">
       <c r="A162" s="11" t="inlineStr">
         <is>
-          <t>GOV-01</t>
+          <t>REC-05</t>
         </is>
       </c>
       <c r="B162" s="12" t="inlineStr">
         <is>
-          <t>Monitoring</t>
+          <t>Reconciliation</t>
         </is>
       </c>
       <c r="C162" s="13" t="inlineStr">
@@ -14890,42 +14890,42 @@
       </c>
       <c r="D162" s="12" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Cash; Bank</t>
         </is>
       </c>
       <c r="E162" s="12" t="inlineStr">
         <is>
-          <t>A maker-checker approval sits un-actioned and is forgotten — a transaction stalls before it is effective, or (worse) a control is quietly bypassed and no one notices an item never got its independent review.</t>
+          <t>Till cash dropped to the safe never reaches the bank, or a deposit isn't matched to the statement — cash sits unbanked (theft/loss exposure) or the bank balance can't be tied to the books.</t>
         </is>
       </c>
       <c r="F162" s="12" t="inlineStr">
         <is>
-          <t>Authorization/Completeness</t>
+          <t>Completeness/Existence/Authorization</t>
         </is>
       </c>
       <c r="G162" s="12" t="inlineStr">
         <is>
-          <t>Pending-approvals MONITOR (COSO monitoring): a single worklist of EVERY item awaiting independent approval across the system, each with its AGE in days and an overdue roll-up — spanning the manual-JE (GL-05), bank-adjustment (BANK-02), AP-disbursement (EXP-06), payroll (PAY-03), asset-revaluation (FA-08), asset-disposal (FA-09), inventory-write-off (INV-07), till-close cash over/short (REV-13), FX-rate (FX-04), budget (BUD-01) and large-refund (REV-16) maker-checkers. The controller reviews it before close; a stale item (age beyond the threshold) is a control finding to chase or escalate. The /approvals screen also lets a manager approve/reject a material till variance or a large refund inline (the pending types with no dedicated module screen). Read-only worklist; tenant-scoped via the caller's RLS.</t>
+          <t>Cash banking — safe-drop → bank deposit → reconciliation: till 'drop's move cash from the drawer to the safe (drawer-only, no GL). Banking BATCHES the undeposited drops into a deposit and posts the GL (Dr &lt;bank account, e.g. 1010&gt; / Cr 1000 Cash), stamping each drop with the deposit id; the deposit is then RECONCILED to the bank statement (status Deposited→Reconciled). A detective read (GET /api/bank/deposits/undeposited-drops) surfaces the CASH STILL IN THE SAFE (drops with deposit_id NULL) — the unbanked exposure to chase. SoD: banking is a treasury duty (exec/ar) — segregated from the cashier (pos_till) who drops the cash, so the person who removes cash from the drawer is not the one who banks it.</t>
         </is>
       </c>
       <c r="H162" s="13" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Det/Prev</t>
         </is>
       </c>
       <c r="I162" s="13" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="J162" s="13" t="inlineStr">
         <is>
-          <t>Continuous / pre-close</t>
+          <t>Per banking run</t>
         </is>
       </c>
       <c r="K162" s="12" t="inlineStr">
         <is>
-          <t>Controller / CFO</t>
+          <t>FinancialController / Treasury</t>
         </is>
       </c>
       <c r="L162" s="13" t="inlineStr">
@@ -14935,22 +14935,22 @@
       </c>
       <c r="M162" s="12" t="inlineStr">
         <is>
-          <t>finance.service.ts pendingApprovals; finance.controller.ts GET approvals/pending (exec/approvals/creditors); aggregates journalEntries(Draft incl. BANKADJ→BANK-02)/apPayments/payruns/asset_revaluations/fixed_assets(disposal_pending)/inv_writeoff_requests/till_sessions(PendingApproval)/fx_rates(PendingApproval)/budgets(PendingApproval); cutover/compliance.ts (ToE)</t>
+          <t>bank.service.ts undepositedDrops/createDeposit (Dr bank/Cr 1000, stamps deposit_id)/reconcileDeposit/listDeposits; bank.controller.ts (deposits, deposits/undeposited-drops, deposits/:id/reconcile; exec/ar); schema/cash.ts bank_deposits + cash_movements.deposit_id + migration 0152; /cash-banking UI; cutover/cash-banking.ts (ToE)</t>
         </is>
       </c>
       <c r="N162" s="12" t="inlineStr">
         <is>
-          <t>Inspect the aggregation across all pending sources + the age/overdue roll-up.</t>
+          <t>Inspect the undeposited-drop exposure read + the deposit GL (bank↔1000) + the reconcile step + the SoD (cashier vs treasury).</t>
         </is>
       </c>
       <c r="O162" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: create a pending item (e.g. a Draft JE) and confirm it appears in the worklist with its control ID, amount and age; the overdue count flags items past the threshold (re-performed by the harness).</t>
+          <t>Re-perform: two till drops → cash-in-safe shows the total; a cashier (pos_till) cannot bank (403); treasury banks → Dr bank / Cr 1000, cash-in-safe back to 0; reconcile the deposit; trial balance balanced (re-performed by the cash-banking harness).</t>
         </is>
       </c>
       <c r="P162" s="12" t="inlineStr">
         <is>
-          <t>Pending-approvals worklist</t>
+          <t>Bank-deposit register; undeposited-drop (cash-in-safe) exposure</t>
         </is>
       </c>
       <c r="Q162" s="18" t="inlineStr">
@@ -14962,12 +14962,12 @@
     <row r="163">
       <c r="A163" s="15" t="inlineStr">
         <is>
-          <t>TAX-01</t>
+          <t>GOV-01</t>
         </is>
       </c>
       <c r="B163" s="16" t="inlineStr">
         <is>
-          <t>Tax</t>
+          <t>Monitoring</t>
         </is>
       </c>
       <c r="C163" s="17" t="inlineStr">
@@ -14977,27 +14977,27 @@
       </c>
       <c r="D163" s="16" t="inlineStr">
         <is>
-          <t>Tax (VAT)</t>
+          <t>All</t>
         </is>
       </c>
       <c r="E163" s="16" t="inlineStr">
         <is>
-          <t>VAT computed incorrectly → filing/penalty risk.</t>
+          <t>A maker-checker approval sits un-actioned and is forgotten — a transaction stalls before it is effective, or (worse) a control is quietly bypassed and no one notices an item never got its independent review.</t>
         </is>
       </c>
       <c r="F163" s="16" t="inlineStr">
         <is>
-          <t>Accuracy</t>
+          <t>Authorization/Completeness</t>
         </is>
       </c>
       <c r="G163" s="16" t="inlineStr">
         <is>
-          <t>VAT via pluggable provider (TH 7%); unit-tested; no hard-coded rate.</t>
+          <t>Pending-approvals MONITOR (COSO monitoring): a single worklist of EVERY item awaiting independent approval across the system, each with its AGE in days and an overdue roll-up — spanning the manual-JE (GL-05), bank-adjustment (BANK-02), AP-disbursement (EXP-06), payroll (PAY-03), asset-revaluation (FA-08), asset-disposal (FA-09), inventory-write-off (INV-07), till-close cash over/short (REV-13), FX-rate (FX-04), budget (BUD-01) and large-refund (REV-16) maker-checkers. The controller reviews it before close; a stale item (age beyond the threshold) is a control finding to chase or escalate. The /approvals screen also lets a manager approve/reject a material till variance or a large refund inline (the pending types with no dedicated module screen). Read-only worklist; tenant-scoped via the caller's RLS.</t>
         </is>
       </c>
       <c r="H163" s="17" t="inlineStr">
         <is>
-          <t>Auto</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I163" s="17" t="inlineStr">
@@ -15007,37 +15007,37 @@
       </c>
       <c r="J163" s="17" t="inlineStr">
         <is>
-          <t>Per txn</t>
+          <t>Continuous / pre-close</t>
         </is>
       </c>
       <c r="K163" s="16" t="inlineStr">
         <is>
-          <t>Tax / Controller</t>
+          <t>Controller / CFO</t>
         </is>
       </c>
       <c r="L163" s="17" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="M163" s="16" t="inlineStr">
         <is>
-          <t>tax/tax-providers.ts; tax.service.ts; test/unit.test.ts</t>
+          <t>finance.service.ts pendingApprovals; finance.controller.ts GET approvals/pending (exec/approvals/creditors); aggregates journalEntries(Draft incl. BANKADJ→BANK-02)/apPayments/payruns/asset_revaluations/fixed_assets(disposal_pending)/inv_writeoff_requests/till_sessions(PendingApproval)/fx_rates(PendingApproval)/budgets(PendingApproval); cutover/compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N163" s="16" t="inlineStr">
         <is>
-          <t>Inspect rate provider + tests.</t>
+          <t>Inspect the aggregation across all pending sources + the age/overdue roll-up.</t>
         </is>
       </c>
       <c r="O163" s="16" t="inlineStr">
         <is>
-          <t>Re-perform VAT on sample; tie to return.</t>
+          <t>Re-perform: create a pending item (e.g. a Draft JE) and confirm it appears in the worklist with its control ID, amount and age; the overdue count flags items past the threshold (re-performed by the harness).</t>
         </is>
       </c>
       <c r="P163" s="16" t="inlineStr">
         <is>
-          <t>VAT tests</t>
+          <t>Pending-approvals worklist</t>
         </is>
       </c>
       <c r="Q163" s="18" t="inlineStr">
@@ -15049,7 +15049,7 @@
     <row r="164">
       <c r="A164" s="11" t="inlineStr">
         <is>
-          <t>TAX-02</t>
+          <t>TAX-01</t>
         </is>
       </c>
       <c r="B164" s="12" t="inlineStr">
@@ -15064,22 +15064,22 @@
       </c>
       <c r="D164" s="12" t="inlineStr">
         <is>
-          <t>Tax; Revenue</t>
+          <t>Tax (VAT)</t>
         </is>
       </c>
       <c r="E164" s="12" t="inlineStr">
         <is>
-          <t>Non-compliant e-Tax invoice / not transmitted to ETDA.</t>
+          <t>VAT computed incorrectly → filing/penalty risk.</t>
         </is>
       </c>
       <c r="F164" s="12" t="inlineStr">
         <is>
-          <t>Accuracy/Compliance</t>
+          <t>Accuracy</t>
         </is>
       </c>
       <c r="G164" s="12" t="inlineStr">
         <is>
-          <t>e-Tax invoice (ETDA UBL 2.1 XML) generation + email with CC to ETDA timestamp mailbox.</t>
+          <t>VAT via pluggable provider (TH 7%); unit-tested; no hard-coded rate.</t>
         </is>
       </c>
       <c r="H164" s="13" t="inlineStr">
@@ -15094,37 +15094,37 @@
       </c>
       <c r="J164" s="13" t="inlineStr">
         <is>
-          <t>Per invoice</t>
+          <t>Per txn</t>
         </is>
       </c>
       <c r="K164" s="12" t="inlineStr">
         <is>
-          <t>Tax</t>
+          <t>Tax / Controller</t>
         </is>
       </c>
       <c r="L164" s="13" t="inlineStr">
         <is>
-          <t>P10/P13</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="M164" s="12" t="inlineStr">
         <is>
-          <t>tax-docs/etax-xml.ts; etax-email.service.ts (tested)</t>
+          <t>tax/tax-providers.ts; tax.service.ts; test/unit.test.ts</t>
         </is>
       </c>
       <c r="N164" s="12" t="inlineStr">
         <is>
-          <t>Inspect XML schema + email composer.</t>
+          <t>Inspect rate provider + tests.</t>
         </is>
       </c>
       <c r="O164" s="12" t="inlineStr">
         <is>
-          <t>Sample invoices: valid XML, correct CC/escaping.</t>
+          <t>Re-perform VAT on sample; tie to return.</t>
         </is>
       </c>
       <c r="P164" s="12" t="inlineStr">
         <is>
-          <t>e-Tax samples</t>
+          <t>VAT tests</t>
         </is>
       </c>
       <c r="Q164" s="18" t="inlineStr">
@@ -15136,7 +15136,7 @@
     <row r="165">
       <c r="A165" s="15" t="inlineStr">
         <is>
-          <t>TAX-03</t>
+          <t>TAX-02</t>
         </is>
       </c>
       <c r="B165" s="16" t="inlineStr">
@@ -15151,22 +15151,22 @@
       </c>
       <c r="D165" s="16" t="inlineStr">
         <is>
-          <t>Tax (WHT)</t>
+          <t>Tax; Revenue</t>
         </is>
       </c>
       <c r="E165" s="16" t="inlineStr">
         <is>
-          <t>Withholding tax mis-computed, not withheld at payment, or not tied to the GL.</t>
+          <t>Non-compliant e-Tax invoice / not transmitted to ETDA.</t>
         </is>
       </c>
       <c r="F165" s="16" t="inlineStr">
         <is>
-          <t>Accuracy</t>
+          <t>Accuracy/Compliance</t>
         </is>
       </c>
       <c r="G165" s="16" t="inlineStr">
         <is>
-          <t>WHT withheld at AP payment time and posted to the GL, then tied out: when a vendor payment is approved (maker-checker), WHT is computed on the PRE-VAT base and posted Dr 2000 AP / Cr 2361 Vendor-WHT-Payable / Cr 1000 (vendor paid net), so the liability to the RD is on the books. A monthly ภ.ง.ด.3/53 → GL tie-out (pndTieOut) reconciles the GL 2361 movement to the WHT withheld on approved AP payments AND to the 50-ทวิ certificates issued — flagging out-of-process JEs (gl≠ap) and un-certificated withholdings. Payroll PND1 WHT stays a separate account (2360, PAY-02).</t>
+          <t>e-Tax invoice (ETDA UBL 2.1 XML) generation + email with CC to ETDA timestamp mailbox.</t>
         </is>
       </c>
       <c r="H165" s="17" t="inlineStr">
@@ -15181,7 +15181,7 @@
       </c>
       <c r="J165" s="17" t="inlineStr">
         <is>
-          <t>Per payment / monthly</t>
+          <t>Per invoice</t>
         </is>
       </c>
       <c r="K165" s="16" t="inlineStr">
@@ -15191,27 +15191,27 @@
       </c>
       <c r="L165" s="17" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P10/P13</t>
         </is>
       </c>
       <c r="M165" s="16" t="inlineStr">
         <is>
-          <t>finance.service.ts approveApPayment (WHT calc + GL 2361 post); tax-reports.service.ts pndTieOut (ภ.ง.ด.→GL tie-out); ap_payments wht_* (0204); ledger-constants 2361; cutover/taxdocs.ts (ToE)</t>
+          <t>tax-docs/etax-xml.ts; etax-email.service.ts (tested)</t>
         </is>
       </c>
       <c r="N165" s="16" t="inlineStr">
         <is>
-          <t>Inspect the WHT-at-payment posting + the ภ.ง.ด.→GL tie-out.</t>
+          <t>Inspect XML schema + email composer.</t>
         </is>
       </c>
       <c r="O165" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: approve a vendor payment with a WHT rate → vendor paid net, GL 2361 credited the WHT; run the tie-out → GL 2361 ties to the AP-withheld total (tied_gl_ap).</t>
+          <t>Sample invoices: valid XML, correct CC/escaping.</t>
         </is>
       </c>
       <c r="P165" s="16" t="inlineStr">
         <is>
-          <t>WHT GL postings + ภ.ง.ด.→GL tie-out ToE</t>
+          <t>e-Tax samples</t>
         </is>
       </c>
       <c r="Q165" s="18" t="inlineStr">
@@ -15223,7 +15223,7 @@
     <row r="166">
       <c r="A166" s="11" t="inlineStr">
         <is>
-          <t>TAX-04</t>
+          <t>TAX-03</t>
         </is>
       </c>
       <c r="B166" s="12" t="inlineStr">
@@ -15238,27 +15238,27 @@
       </c>
       <c r="D166" s="12" t="inlineStr">
         <is>
-          <t>Tax (VAT); Tax Payable (2100)</t>
+          <t>Tax (WHT)</t>
         </is>
       </c>
       <c r="E166" s="12" t="inlineStr">
         <is>
-          <t>Output/input VAT on the filed ภ.พ.30 return does not agree to the GL — VAT liability mis-stated, a filing/penalty exposure, or a posting omission goes undetected before submission.</t>
+          <t>Withholding tax mis-computed, not withheld at payment, or not tied to the GL.</t>
         </is>
       </c>
       <c r="F166" s="12" t="inlineStr">
         <is>
-          <t>Completeness/Accuracy</t>
+          <t>Accuracy</t>
         </is>
       </c>
       <c r="G166" s="12" t="inlineStr">
         <is>
-          <t>Periodic VAT-return ↔ GL reconciliation (ภ.พ.30): the monthly return (GET /api/tax-reports/pp30) is built from the sales/output-VAT and purchase/input-VAT sub-reports, computes net VAT = output − input, and RECONCILES it to the **GL account 2100 (Tax Payable) net movement** for the same period (Σ credit − Σ debit over Posted entries) — returning `reconciliation.tied` = true only when the two agree within rounding. A non-tie is a detective finding to investigate and clear BEFORE filing (the form also carries the ม.157 deadline = the 15th of the next month). Output VAT is posted to 2100 on every sale (Cr) and reversed on returns (Dr); input VAT is posted on AP bills (Dr) — so 2100's net is the period's VAT payable. Read-only report; exportable to a ภ.พ.30 PDF/HTML.</t>
+          <t>WHT withheld at AP payment time and posted to the GL, then tied out: when a vendor payment is approved (maker-checker), WHT is computed on the PRE-VAT base and posted Dr 2000 AP / Cr 2361 Vendor-WHT-Payable / Cr 1000 (vendor paid net), so the liability to the RD is on the books. A monthly ภ.ง.ด.3/53 → GL tie-out (pndTieOut) reconciles the GL 2361 movement to the WHT withheld on approved AP payments AND to the 50-ทวิ certificates issued — flagging out-of-process JEs (gl≠ap) and un-certificated withholdings. Payroll PND1 WHT stays a separate account (2360, PAY-02). Automation (docs/33 PR4): a schedulable, idempotent BI action job **tax_wht_cert_batch** auto-issues the 50-ทวิ certificate (มาตรา 50 ทวิ) for every AP-payment WHT in the period that does not yet have one — keyed on the payment_no so a re-run skips already-certificated payments — CLOSING the pndTieOut un-certificated-WHT gap without manual re-keying (labour/service withholding ค่าจ้างทำของ/ค่าบริการ). A payment whose vendor lacks a valid 13-digit tax ID is skipped (surfaced in the run count), not silently certificated wrong.</t>
         </is>
       </c>
       <c r="H166" s="13" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Auto</t>
         </is>
       </c>
       <c r="I166" s="13" t="inlineStr">
@@ -15268,37 +15268,37 @@
       </c>
       <c r="J166" s="13" t="inlineStr">
         <is>
-          <t>Monthly / pre-filing</t>
+          <t>Per payment / monthly</t>
         </is>
       </c>
       <c r="K166" s="12" t="inlineStr">
         <is>
-          <t>Tax / FinancialController</t>
+          <t>Tax</t>
         </is>
       </c>
       <c r="L166" s="13" t="inlineStr">
         <is>
-          <t>P10/P16</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="M166" s="12" t="inlineStr">
         <is>
-          <t>tax-reports.service.ts pp30 (outputVat/inputVat + 2100 net-movement tie); tax-reports.controller.ts (GET pp30, pp30/export, exec); tax-reports-pdf.ts; dine-in.service.ts/returns.service.ts/finance.service.ts post 2100 on sale/return/AP; /tax/reports UI; cutover/taxdocs.ts (ToE)</t>
+          <t>finance.service.ts approveApPayment (WHT calc + GL 2361 post); tax/tax-jobs.service.ts runWhtCertBatch (auto-issue 50-ทวิ, idempotent per payment_no); bi.service.ts REPORT_TYPES tax_wht_cert_batch; tax/documents/wht.service.ts issue; tax-reports.service.ts pndTieOut (ภ.ง.ด.→GL tie-out); ap_payments wht_* (0204); ledger-constants 2361; cutover/taxdocs.ts (ToE)</t>
         </is>
       </c>
       <c r="N166" s="12" t="inlineStr">
         <is>
-          <t>Inspect the pp30 build + the 2100 net-movement query + the tie flag + the filing deadline.</t>
+          <t>Inspect the WHT-at-payment posting + the ภ.ง.ด.→GL tie-out + the scheduled auto-cert batch.</t>
         </is>
       </c>
       <c r="O166" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: the pp30 return computes net VAT (output − input), the GL 2100 net movement reflects the posted input VAT, and the reconciliation block exposes the gl_account (2100), the report net VAT and a boolean tie verdict (tied iff the two agree within rounding); the ภ.พ.30 export renders (re-performed by the taxdocs harness).</t>
+          <t>Re-perform: approve a vendor payment with a WHT rate → vendor paid net, GL 2361 credited the WHT; run the tie-out → GL 2361 ties to the AP-withheld total (tied_gl_ap); run tax_wht_cert_batch → a 50-ทวิ is issued for that payment (issued 1), a re-run skips it (issued 0, no duplicate).</t>
         </is>
       </c>
       <c r="P166" s="12" t="inlineStr">
         <is>
-          <t>ภ.พ.30 return + GL-2100 reconciliation tie</t>
+          <t>WHT GL postings + ภ.ง.ด.→GL tie-out + scheduled 50-ทวิ auto-cert ToE</t>
         </is>
       </c>
       <c r="Q166" s="18" t="inlineStr">
@@ -15310,7 +15310,7 @@
     <row r="167">
       <c r="A167" s="15" t="inlineStr">
         <is>
-          <t>TAX-05</t>
+          <t>TAX-04</t>
         </is>
       </c>
       <c r="B167" s="16" t="inlineStr">
@@ -15325,37 +15325,37 @@
       </c>
       <c r="D167" s="16" t="inlineStr">
         <is>
-          <t>Tax (VAT/WHT)</t>
+          <t>Tax (VAT); Tax Payable (2100)</t>
         </is>
       </c>
       <c r="E167" s="16" t="inlineStr">
         <is>
-          <t>A return is computed but there is no evidence it was actually FILED — no record of the figures as filed, the submission date or the Revenue-Department reference — so a missed or late filing (penalty/surcharge exposure) is not detected, and a filed return can be silently recomputed/altered after submission.</t>
+          <t>Output/input VAT on the filed ภ.พ.30 return does not agree to the GL — VAT liability mis-stated, a filing/penalty exposure, or a posting omission goes undetected before submission.</t>
         </is>
       </c>
       <c r="F167" s="16" t="inlineStr">
         <is>
-          <t>Completeness/Accuracy/Cutoff</t>
+          <t>Completeness/Accuracy</t>
         </is>
       </c>
       <c r="G167" s="16" t="inlineStr">
         <is>
-          <t>Thai tax filing register + remittance calendar: a computed ภ.พ.30 (PP30) or ภ.ง.ด.3/53 (PND) return is SNAPSHOTTED into a thai_tax_filings record (one per tenant/type/period) carrying the figures as filed (output/input/net VAT, tax withheld) and a DRAFT→SUBMITTED→ACCEPTED lifecycle. Filing is idempotent per period; submitting REQUIRES a Revenue-Department submission reference (SUBMISSION_REF_REQUIRED) and stamps SUBMITTED + the timestamp; an already-filed (SUBMITTED/ACCEPTED) period is NOT silently overwritten when re-filed (returned as-is, already_filed=true). A remittance calendar (GET /api/tax-reports/remittance-calendar) lists every monthly obligation (ภ.พ.30 by the 15th, ภ.ง.ด. by the 7th of the following month) with its current status (NOT_FILED/DRAFT/SUBMITTED/ACCEPTED), so the controller sees what is due/filed/late before the deadline. Tenant-scoped (RLS); gated exec.</t>
+          <t>Periodic VAT-return ↔ GL reconciliation (ภ.พ.30): the monthly return (GET /api/tax-reports/pp30) is built from the sales/output-VAT and purchase/input-VAT sub-reports, computes net VAT = output − input, and RECONCILES it to the **GL account 2100 (Tax Payable) net movement** for the same period (Σ credit − Σ debit over Posted entries) — returning `reconciliation.tied` = true only when the two agree within rounding. A non-tie is a detective finding to investigate and clear BEFORE filing (the form also carries the ม.157 deadline = the 15th of the next month). Output VAT is posted to 2100 on every sale (Cr) and reversed on returns (Dr); input VAT is posted on AP bills (Dr) — so 2100's net is the period's VAT payable. Read-only report; exportable to a ภ.พ.30 PDF/HTML.</t>
         </is>
       </c>
       <c r="H167" s="17" t="inlineStr">
         <is>
-          <t>Det/Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I167" s="17" t="inlineStr">
         <is>
-          <t>Auto+Manual</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J167" s="17" t="inlineStr">
         <is>
-          <t>Monthly / per filing</t>
+          <t>Monthly / pre-filing</t>
         </is>
       </c>
       <c r="K167" s="16" t="inlineStr">
@@ -15370,22 +15370,22 @@
       </c>
       <c r="M167" s="16" t="inlineStr">
         <is>
-          <t>tax-reports.service.ts fileReturn (snapshots pp30/pnd into a DRAFT, idempotent per period; no overwrite of a filed return) / submitFiling (SUBMISSION_REF_REQUIRED → SUBMITTED) / acceptFiling / listFilings / remittanceCalendar; tax-reports.controller.ts (POST filings[/:id/submit|accept], GET filings, remittance-calendar, exec); schema/tax-docs.ts thai_tax_filings + migration 0165; /tax/reports filings &amp; calendar tab; cutover/taxdocs.ts (ToE)</t>
+          <t>tax-reports.service.ts pp30 (outputVat/inputVat + 2100 net-movement tie); tax-reports.controller.ts (GET pp30, pp30/export, exec); tax-reports-pdf.ts; dine-in.service.ts/returns.service.ts/finance.service.ts post 2100 on sale/return/AP; /tax/reports UI; cutover/taxdocs.ts (ToE)</t>
         </is>
       </c>
       <c r="N167" s="16" t="inlineStr">
         <is>
-          <t>Inspect the filing snapshot + the DRAFT→SUBMITTED→ACCEPTED lifecycle + the mandatory submission reference + the no-overwrite-of-a-filed-return rule + the deadline calendar.</t>
+          <t>Inspect the pp30 build + the 2100 net-movement query + the tie flag + the filing deadline.</t>
         </is>
       </c>
       <c r="O167" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: file PP30 → DRAFT with the period figures; re-file refreshes the same DRAFT (idempotent); submit without a reference → 400; submit with a reference → SUBMITTED + timestamp; accept → ACCEPTED; re-filing an accepted period returns it (already_filed); the remittance calendar shows the period ACCEPTED with the 15th-of-next-month deadline (re-performed by the taxdocs harness).</t>
+          <t>Re-perform: the pp30 return computes net VAT (output − input), the GL 2100 net movement reflects the posted input VAT, and the reconciliation block exposes the gl_account (2100), the report net VAT and a boolean tie verdict (tied iff the two agree within rounding); the ภ.พ.30 export renders (re-performed by the taxdocs harness).</t>
         </is>
       </c>
       <c r="P167" s="16" t="inlineStr">
         <is>
-          <t>thai_tax_filings register + remittance calendar</t>
+          <t>ภ.พ.30 return + GL-2100 reconciliation tie</t>
         </is>
       </c>
       <c r="Q167" s="18" t="inlineStr">
@@ -15397,7 +15397,7 @@
     <row r="168">
       <c r="A168" s="11" t="inlineStr">
         <is>
-          <t>TAX-06</t>
+          <t>TAX-05</t>
         </is>
       </c>
       <c r="B168" s="12" t="inlineStr">
@@ -15412,67 +15412,67 @@
       </c>
       <c r="D168" s="12" t="inlineStr">
         <is>
-          <t>Deferred Tax Asset (1700); Deferred Tax Liability (2700); Deferred Tax Expense (5950)</t>
+          <t>Tax (VAT/WHT)</t>
         </is>
       </c>
       <c r="E168" s="12" t="inlineStr">
         <is>
-          <t>Book-vs-tax TEMPORARY differences (the AR allowance, accelerated depreciation, accruals) are not recognised as deferred tax, or the deferred-tax entry is computed and posted by one person with no review — income tax expense and the deferred tax asset/liability are mis-stated (TAS 12 / TFRS).</t>
+          <t>A return is computed but there is no evidence it was actually FILED — no record of the figures as filed, the submission date or the Revenue-Department reference — so a missed or late filing (penalty/surcharge exposure) is not detected, and a filed return can be silently recomputed/altered after submission.</t>
         </is>
       </c>
       <c r="F168" s="12" t="inlineStr">
         <is>
-          <t>Accuracy/Valuation/Completeness/Authorization/Segregation of Duties</t>
+          <t>Completeness/Accuracy/Cutoff</t>
         </is>
       </c>
       <c r="G168" s="12" t="inlineStr">
         <is>
-          <t>Deferred tax (TAS 12, maker-checker, idempotent per (tenant, period)): POST /api/ledger/deferred-tax/run gathers temporary differences — the latest POSTED AR allowance (a DEDUCTIBLE temp diff → DTA = allowance × CIT) and accelerated depreciation (book NBV vs an assumed tax NBV; a TAXABLE temp diff → DTL = (bookNBV − taxNBV) × CIT) — computes net_deferred = DTA − DTL and the DELTA vs the prior posted run, staging an 'Open' deferred_tax_runs row (one per tenant/period; a Posted period → ALREADY_POSTED). CIT rate defaults to 0.20 (Thai). SIMPLIFICATION: no parallel tax-depreciation ledger exists, so tax depreciation is assumed FASTER than book by a documented factor (default 1.5×, capped at the depreciable base) — overridable per run; a deliberate approximation until a tax-dep ledger is modelled. POST /api/ledger/deferred-tax/:id/post is segregated (poster ≠ runner → SELF_POST) and posts the period DELTA via LedgerService.postEntry (delta&gt;0 net asset up = deferred tax benefit → Dr 1700 / Cr 5950; delta&lt;0 → Dr 5950 / Cr 1700), so PERIOD_LOCKED + the GL audit trail apply. Marks the run Posted.</t>
+          <t>Thai tax filing register + remittance calendar: a computed ภ.พ.30 (PP30) or ภ.ง.ด.3/53 (PND) return is SNAPSHOTTED into a thai_tax_filings record (one per tenant/type/period) carrying the figures as filed (output/input/net VAT, tax withheld) and a DRAFT→SUBMITTED→ACCEPTED lifecycle. Filing is idempotent per period; submitting REQUIRES a Revenue-Department submission reference (SUBMISSION_REF_REQUIRED) and stamps SUBMITTED + the timestamp; an already-filed (SUBMITTED/ACCEPTED) period is NOT silently overwritten when re-filed (returned as-is, already_filed=true). A remittance calendar (GET /api/tax-reports/remittance-calendar) lists every monthly obligation (ภ.พ.30 by the 15th, ภ.ง.ด. by the 7th of the following month) with its current status (NOT_FILED/DRAFT/SUBMITTED/ACCEPTED), so the controller sees what is due/filed/late before the deadline. Tenant-scoped (RLS); gated exec. Automation (docs/33 PR4): schedulable BI action jobs **tax_pp30_draft** / **tax_pnd_draft** register the period's return as a DRAFT filing (via fileReturn — idempotent, never overwriting a SUBMITTED/ACCEPTED period), and **tax_remittance_reminder** surfaces the period's amounts due + statutory deadlines (ภ.พ.30 15th, ภ.ง.ด. 7th) for a proactive nudge — a human still submits.</t>
         </is>
       </c>
       <c r="H168" s="13" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det/Prev</t>
         </is>
       </c>
       <c r="I168" s="13" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="J168" s="13" t="inlineStr">
         <is>
-          <t>Quarterly / year-end</t>
+          <t>Monthly / per filing</t>
         </is>
       </c>
       <c r="K168" s="12" t="inlineStr">
         <is>
-          <t>Tax / Financial Controller</t>
+          <t>Tax / FinancialController</t>
         </is>
       </c>
       <c r="L168" s="13" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P10/P16</t>
         </is>
       </c>
       <c r="M168" s="12" t="inlineStr">
         <is>
-          <t>deferred-tax.service.ts (runDeferredTax gather temp diffs [AR allowance, accelerated dep] + delta-vs-prior + stage Open, idempotent ALREADY_POSTED; postDeferredTax SELF_POST maker-checker + 1700/5950 delta posting; list/get); deferred-tax.controller.ts (gl_close/gl_post run + :id/post, gl_close/gl_post/exec read); schema/deferred-tax-fx.ts (deferred_tax_runs, uq tenant/period); migration 0168 (tables + RLS); COA 1700/2700/5950 (seedChartOfAccounts); ledger.module.ts (wired); close.service.ts (deferred_tax close-checklist step); reuses ar_allowance (REV-18) + fixed_assets NBV; cutover/basics.ts (TAX-06 ToE)</t>
+          <t>tax-reports.service.ts fileReturn (snapshots pp30/pnd into a DRAFT, idempotent per period; no overwrite of a filed return) / submitFiling (SUBMISSION_REF_REQUIRED → SUBMITTED) / acceptFiling / listFilings / remittanceCalendar; tax-reports.controller.ts (POST filings[/:id/submit|accept], GET filings, remittance-calendar, exec); schema/tax-docs.ts thai_tax_filings + migration 0165; /tax/reports filings &amp; calendar tab; cutover/taxdocs.ts (ToE)</t>
         </is>
       </c>
       <c r="N168" s="12" t="inlineStr">
         <is>
-          <t>Inspect the temp-difference gathering (allowance×rate DTA + accelerated-dep DTL with the documented tax-dep simplification), the delta-vs-prior-run, the SELF_POST maker-checker, and the 1700/5950 posting through the period-lock gate.</t>
+          <t>Inspect the filing snapshot + the DRAFT→SUBMITTED→ACCEPTED lifecycle + the mandatory submission reference + the no-overwrite-of-a-filed-return rule + the deadline calendar.</t>
         </is>
       </c>
       <c r="O168" s="12" t="inlineStr">
         <is>
-          <t>TC-TAX-06-01: run with a posted AR allowance of 1100 at 20% → DTA 220, net deferred asset 220, delta 220 (Open); TC-TAX-06-02: runner self-post → SELF_POST (403), a different user posts → Dr 1700 / Cr 5950 (220), re-post → ALREADY_POSTED (400) (re-performed by the basics.ts harness).</t>
+          <t>Re-perform: file PP30 → DRAFT with the period figures; re-file refreshes the same DRAFT (idempotent); submit without a reference → 400; submit with a reference → SUBMITTED + timestamp; accept → ACCEPTED; re-filing an accepted period returns it (already_filed); the remittance calendar shows the period ACCEPTED with the 15th-of-next-month deadline (re-performed by the taxdocs harness).</t>
         </is>
       </c>
       <c r="P168" s="12" t="inlineStr">
         <is>
-          <t>deferred_tax_runs register (Open→Posted, temp-difference schedule, runner/poster); the DEFTAX JE to 1700/5950; quarterly/year-end deferred-tax sign-off</t>
+          <t>thai_tax_filings register + remittance calendar</t>
         </is>
       </c>
       <c r="Q168" s="18" t="inlineStr">
@@ -15484,12 +15484,12 @@
     <row r="169">
       <c r="A169" s="15" t="inlineStr">
         <is>
-          <t>PAY-01</t>
+          <t>TAX-06</t>
         </is>
       </c>
       <c r="B169" s="16" t="inlineStr">
         <is>
-          <t>Payroll</t>
+          <t>Tax</t>
         </is>
       </c>
       <c r="C169" s="17" t="inlineStr">
@@ -15499,27 +15499,27 @@
       </c>
       <c r="D169" s="16" t="inlineStr">
         <is>
-          <t>Payroll expense/liability</t>
+          <t>Deferred Tax Asset (1700); Deferred Tax Liability (2700); Deferred Tax Expense (5950)</t>
         </is>
       </c>
       <c r="E169" s="16" t="inlineStr">
         <is>
-          <t>Payroll, SSO and PIT mis-computed.</t>
+          <t>Book-vs-tax TEMPORARY differences (the AR allowance, accelerated depreciation, accruals) are not recognised as deferred tax, or the deferred-tax entry is computed and posted by one person with no review — income tax expense and the deferred tax asset/liability are mis-stated (TAS 12 / TFRS).</t>
         </is>
       </c>
       <c r="F169" s="16" t="inlineStr">
         <is>
-          <t>Accuracy</t>
+          <t>Accuracy/Valuation/Completeness/Authorization/Segregation of Duties</t>
         </is>
       </c>
       <c r="G169" s="16" t="inlineStr">
         <is>
-          <t>Payroll engine — SSO 5% (cap 750), progressive PIT, payslip net; unit-tested.</t>
+          <t>Deferred tax (TAS 12, maker-checker, idempotent per (tenant, period)): POST /api/ledger/deferred-tax/run gathers temporary differences — the latest POSTED AR allowance (a DEDUCTIBLE temp diff → DTA = allowance × CIT) and accelerated depreciation (book NBV vs an assumed tax NBV; a TAXABLE temp diff → DTL = (bookNBV − taxNBV) × CIT) — computes net_deferred = DTA − DTL and the DELTA vs the prior posted run, staging an 'Open' deferred_tax_runs row (one per tenant/period; a Posted period → ALREADY_POSTED). CIT rate defaults to 0.20 (Thai). SIMPLIFICATION: no parallel tax-depreciation ledger exists, so tax depreciation is assumed FASTER than book by a documented factor (default 1.5×, capped at the depreciable base) — overridable per run; a deliberate approximation until a tax-dep ledger is modelled. POST /api/ledger/deferred-tax/:id/post is segregated (poster ≠ runner → SELF_POST) and posts the period DELTA via LedgerService.postEntry (delta&gt;0 net asset up = deferred tax benefit → Dr 1700 / Cr 5950; delta&lt;0 → Dr 5950 / Cr 1700), so PERIOD_LOCKED + the GL audit trail apply. Marks the run Posted.</t>
         </is>
       </c>
       <c r="H169" s="17" t="inlineStr">
         <is>
-          <t>Auto</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I169" s="17" t="inlineStr">
@@ -15529,12 +15529,12 @@
       </c>
       <c r="J169" s="17" t="inlineStr">
         <is>
-          <t>Per run</t>
+          <t>Quarterly / year-end</t>
         </is>
       </c>
       <c r="K169" s="16" t="inlineStr">
         <is>
-          <t>HR / Payroll</t>
+          <t>Tax / Financial Controller</t>
         </is>
       </c>
       <c r="L169" s="17" t="inlineStr">
@@ -15544,22 +15544,22 @@
       </c>
       <c r="M169" s="16" t="inlineStr">
         <is>
-          <t>payroll/payroll-calc.ts; test/unit.test.ts</t>
+          <t>deferred-tax.service.ts (runDeferredTax gather temp diffs [AR allowance, accelerated dep] + delta-vs-prior + stage Open, idempotent ALREADY_POSTED; postDeferredTax SELF_POST maker-checker + 1700/5950 delta posting; list/get); deferred-tax.controller.ts (gl_close/gl_post run + :id/post, gl_close/gl_post/exec read); schema/deferred-tax-fx.ts (deferred_tax_runs, uq tenant/period); migration 0168 (tables + RLS); COA 1700/2700/5950 (seedChartOfAccounts); ledger.module.ts (wired); close.service.ts (deferred_tax close-checklist step); reuses ar_allowance (REV-18) + fixed_assets NBV; cutover/basics.ts (TAX-06 ToE)</t>
         </is>
       </c>
       <c r="N169" s="16" t="inlineStr">
         <is>
-          <t>Inspect calc + tests.</t>
+          <t>Inspect the temp-difference gathering (allowance×rate DTA + accelerated-dep DTL with the documented tax-dep simplification), the delta-vs-prior-run, the SELF_POST maker-checker, and the 1700/5950 posting through the period-lock gate.</t>
         </is>
       </c>
       <c r="O169" s="16" t="inlineStr">
         <is>
-          <t>Re-perform sample payslips.</t>
+          <t>TC-TAX-06-01: run with a posted AR allowance of 1100 at 20% → DTA 220, net deferred asset 220, delta 220 (Open); TC-TAX-06-02: runner self-post → SELF_POST (403), a different user posts → Dr 1700 / Cr 5950 (220), re-post → ALREADY_POSTED (400) (re-performed by the basics.ts harness).</t>
         </is>
       </c>
       <c r="P169" s="16" t="inlineStr">
         <is>
-          <t>Payslip tests</t>
+          <t>deferred_tax_runs register (Open→Posted, temp-difference schedule, runner/poster); the DEFTAX JE to 1700/5950; quarterly/year-end deferred-tax sign-off</t>
         </is>
       </c>
       <c r="Q169" s="18" t="inlineStr">
@@ -15571,7 +15571,7 @@
     <row r="170">
       <c r="A170" s="11" t="inlineStr">
         <is>
-          <t>PAY-02</t>
+          <t>PAY-01</t>
         </is>
       </c>
       <c r="B170" s="12" t="inlineStr">
@@ -15586,27 +15586,27 @@
       </c>
       <c r="D170" s="12" t="inlineStr">
         <is>
-          <t>Payroll liability</t>
+          <t>Payroll expense/liability</t>
         </is>
       </c>
       <c r="E170" s="12" t="inlineStr">
         <is>
-          <t>Statutory withholdings (SSO/WHT/PF) mis-stated or not remitted, so the liability owed to the authorities diverges from the books.</t>
+          <t>Payroll, SSO and PIT mis-computed.</t>
         </is>
       </c>
       <c r="F170" s="12" t="inlineStr">
         <is>
-          <t>Accuracy/Compliance</t>
+          <t>Accuracy</t>
         </is>
       </c>
       <c r="G170" s="12" t="inlineStr">
         <is>
-          <t>Payroll-liability schedule (GET /api/payroll/liabilities): each statutory account — SSO 2350, WHT/PND1 2360, PF 2370 — shows accrued (GL credits) − remitted (GL debits) = outstanding, tied back to the INDEPENDENT payrun accrual with a `reconciled` flag (a divergence flags a manual JE that touched a payroll-liability account outside the payroll process). Treasury remits the cash (POST .../remit → Dr liability / Cr 1000) which clears the outstanding and keeps the books reconciled to the statutory filings; a remittance beyond the outstanding is blocked (REMIT_EXCEEDS_OUTSTANDING).</t>
+          <t>Payroll engine — SSO 5% (cap 750), progressive PIT, payslip net; unit-tested.</t>
         </is>
       </c>
       <c r="H170" s="13" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Auto</t>
         </is>
       </c>
       <c r="I170" s="13" t="inlineStr">
@@ -15616,12 +15616,12 @@
       </c>
       <c r="J170" s="13" t="inlineStr">
         <is>
-          <t>Per run / monthly</t>
+          <t>Per run</t>
         </is>
       </c>
       <c r="K170" s="12" t="inlineStr">
         <is>
-          <t>HR / Payroll / Treasury</t>
+          <t>HR / Payroll</t>
         </is>
       </c>
       <c r="L170" s="13" t="inlineStr">
@@ -15631,22 +15631,22 @@
       </c>
       <c r="M170" s="12" t="inlineStr">
         <is>
-          <t>payroll/payroll.service.ts liabilities/remitLiability</t>
+          <t>payroll/payroll-calc.ts; test/unit.test.ts</t>
         </is>
       </c>
       <c r="N170" s="12" t="inlineStr">
         <is>
-          <t>Inspect the schedule + the accrued/remitted/outstanding tie-out and the reconciled flag.</t>
+          <t>Inspect calc + tests.</t>
         </is>
       </c>
       <c r="O170" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: run a payroll, confirm the SSO/WHT outstanding equals the payrun accrual; remit part and confirm the outstanding falls and the TB stays balanced; attempt an over-remit (REMIT_EXCEEDS_OUTSTANDING).</t>
+          <t>Re-perform sample payslips.</t>
         </is>
       </c>
       <c r="P170" s="12" t="inlineStr">
         <is>
-          <t>Liability schedule + remittance JEs tied to filings</t>
+          <t>Payslip tests</t>
         </is>
       </c>
       <c r="Q170" s="18" t="inlineStr">
@@ -15658,7 +15658,7 @@
     <row r="171">
       <c r="A171" s="15" t="inlineStr">
         <is>
-          <t>PAY-03</t>
+          <t>PAY-02</t>
         </is>
       </c>
       <c r="B171" s="16" t="inlineStr">
@@ -15673,27 +15673,27 @@
       </c>
       <c r="D171" s="16" t="inlineStr">
         <is>
-          <t>Payroll expense/liability; Cash</t>
+          <t>Payroll liability</t>
         </is>
       </c>
       <c r="E171" s="16" t="inlineStr">
         <is>
-          <t>Payroll run posted to the GL without independent review — the preparer both computes and posts their own payroll (ghost employees, inflated rate/hours).</t>
+          <t>Statutory withholdings (SSO/WHT/PF) mis-stated or not remitted, so the liability owed to the authorities diverges from the books.</t>
         </is>
       </c>
       <c r="F171" s="16" t="inlineStr">
         <is>
-          <t>Authorization</t>
+          <t>Accuracy/Compliance</t>
         </is>
       </c>
       <c r="G171" s="16" t="inlineStr">
         <is>
-          <t>Payroll maker-checker (SoD): a run posts its GL entry as a DRAFT (excluded from balances) with the run record 'PendingApproval'; a DIFFERENT user must approve before it becomes effective (approver ≠ preparer enforced regardless of permissions, reusing the GL-05 ledger approval). Reject voids the draft; idempotent per (tenant, period).</t>
+          <t>Payroll-liability schedule (GET /api/payroll/liabilities): each statutory account — SSO 2350, WHT/PND1 2360, PF 2370 — shows accrued (GL credits) − remitted (GL debits) = outstanding, tied back to the INDEPENDENT payrun accrual with a `reconciled` flag (a divergence flags a manual JE that touched a payroll-liability account outside the payroll process). Treasury remits the cash (POST .../remit → Dr liability / Cr 1000) which clears the outstanding and keeps the books reconciled to the statutory filings; a remittance beyond the outstanding is blocked (REMIT_EXCEEDS_OUTSTANDING).</t>
         </is>
       </c>
       <c r="H171" s="17" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I171" s="17" t="inlineStr">
@@ -15703,12 +15703,12 @@
       </c>
       <c r="J171" s="17" t="inlineStr">
         <is>
-          <t>Per run</t>
+          <t>Per run / monthly</t>
         </is>
       </c>
       <c r="K171" s="16" t="inlineStr">
         <is>
-          <t>HR / Payroll; Controller</t>
+          <t>HR / Payroll / Treasury</t>
         </is>
       </c>
       <c r="L171" s="17" t="inlineStr">
@@ -15718,22 +15718,22 @@
       </c>
       <c r="M171" s="16" t="inlineStr">
         <is>
-          <t>payroll/payroll.service.ts approvePayroll/rejectPayroll; migration 0133</t>
+          <t>payroll/payroll.service.ts liabilities/remitLiability</t>
         </is>
       </c>
       <c r="N171" s="16" t="inlineStr">
         <is>
-          <t>Inspect Draft→approve flow + the approver≠preparer check.</t>
+          <t>Inspect the schedule + the accrued/remitted/outstanding tie-out and the reconciled flag.</t>
         </is>
       </c>
       <c r="O171" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: run as A, attempt self-approve (SOD_VIOLATION), approve as B; confirm the JE hits balances only after approval.</t>
+          <t>Re-perform: run a payroll, confirm the SSO/WHT outstanding equals the payrun accrual; remit part and confirm the outstanding falls and the TB stays balanced; attempt an over-remit (REMIT_EXCEEDS_OUTSTANDING).</t>
         </is>
       </c>
       <c r="P171" s="16" t="inlineStr">
         <is>
-          <t>Approval log + SoD test</t>
+          <t>Liability schedule + remittance JEs tied to filings</t>
         </is>
       </c>
       <c r="Q171" s="18" t="inlineStr">
@@ -15745,7 +15745,7 @@
     <row r="172">
       <c r="A172" s="11" t="inlineStr">
         <is>
-          <t>PAY-04</t>
+          <t>PAY-03</t>
         </is>
       </c>
       <c r="B172" s="12" t="inlineStr">
@@ -15760,67 +15760,67 @@
       </c>
       <c r="D172" s="12" t="inlineStr">
         <is>
-          <t>Payroll expense; Labor cost</t>
+          <t>Payroll expense/liability; Cash</t>
         </is>
       </c>
       <c r="E172" s="12" t="inlineStr">
         <is>
-          <t>Overtime is paid at a single flat multiplier with no holiday/night tiers and no statutory cap (Thai LPA OT is mis-paid — too little on holidays, or beyond the 48h/week limit), AND labor cost runs over target as a % of sales with nothing flagging it — margin erosion goes unnoticed until payroll posts.</t>
+          <t>Payroll run posted to the GL without independent review — the preparer both computes and posts their own payroll (ghost employees, inflated rate/hours).</t>
         </is>
       </c>
       <c r="F172" s="12" t="inlineStr">
         <is>
-          <t>Accuracy/Completeness</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="G172" s="12" t="inlineStr">
         <is>
-          <t>Tiered OT rules engine + labor-% alerting: a per-tenant labor_ot_rules table overrides the Thai LPA statutory defaults (REGULAR_OT 1.5x beyond 8h/day, HOLIDAY 2x, HOLIDAY_OT 3x, NIGHT 1.0x tracked; 48h/week cap) — GET/PUT /api/pos/labor/ot-rules. computeOtPay (POST /api/pos/labor/ot-pay) applies the tier's multiplier and CAPS paid hours at the 48h weekly limit, flagging any over-cap hours (over_cap=true) rather than silently paying them. Separately, POST /api/pos/labor/labor-alert/check computes labor % of sales for a period and, when it exceeds the target (default 35%), persists a LABOR_PCT_EXCEEDED alert (idempotent per period) surfaced on GET /api/pos/labor/alerts for the manager to act on / resolve. Tenant-scoped (RLS); gated pos/users/exec. Operational (no GL).</t>
+          <t>Payroll maker-checker (SoD): a run posts its GL entry as a DRAFT (excluded from balances) with the run record 'PendingApproval'; a DIFFERENT user must approve before it becomes effective (approver ≠ preparer enforced regardless of permissions, reusing the GL-05 ledger approval). Reject voids the draft; idempotent per (tenant, period).</t>
         </is>
       </c>
       <c r="H172" s="13" t="inlineStr">
         <is>
-          <t>Det/Prev</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I172" s="13" t="inlineStr">
         <is>
-          <t>Auto+Manual</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J172" s="13" t="inlineStr">
         <is>
-          <t>Per shift / payroll cycle</t>
+          <t>Per run</t>
         </is>
       </c>
       <c r="K172" s="12" t="inlineStr">
         <is>
-          <t>HR / Store Ops Mgr</t>
+          <t>HR / Payroll; Controller</t>
         </is>
       </c>
       <c r="L172" s="13" t="inlineStr">
         <is>
-          <t>P10/P13</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="M172" s="12" t="inlineStr">
         <is>
-          <t>pos-loyalty-labor/schedule.service.ts getOtRules/upsertOtRule (Thai defaults overlay) + computeOtPay (tier multiplier + 48h cap, over_cap flag) + checkLaborAlert/listAlerts/resolveAlert; pos-loyalty-labor.controller.ts (ot-rules, ot-pay, labor-alert/check, alerts[/:id/resolve]); schema/pos-scale.ts labor_ot_rules + labor_alerts + migration 0167; /scheduling UI; cutover/scheduling.ts (ToE)</t>
+          <t>payroll/payroll.service.ts approvePayroll/rejectPayroll; migration 0133</t>
         </is>
       </c>
       <c r="N172" s="12" t="inlineStr">
         <is>
-          <t>Inspect the statutory-default overlay, the tier multipliers, the 48h cap + over_cap flag, and the labor-% threshold alert (raise/idempotent/resolve).</t>
+          <t>Inspect Draft→approve flow + the approver≠preparer check.</t>
         </is>
       </c>
       <c r="O172" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: OT rules expose Thai defaults (1.5/2/3/1.0, cap 48); override REGULAR_OT to 2.0; HOLIDAY_OT 2h x 100 x 3 = 600; a 5h OT entry at 47h already-worked pays only 1h + flags 4h over-cap; labor 8% vs a 5% target raises an alert (idempotent), vs a 50% target raises none; resolve clears it (re-performed by the scheduling harness).</t>
+          <t>Re-perform: run as A, attempt self-approve (SOD_VIOLATION), approve as B; confirm the JE hits balances only after approval.</t>
         </is>
       </c>
       <c r="P172" s="12" t="inlineStr">
         <is>
-          <t>labor_ot_rules + labor_alerts register; OT/labor-% test</t>
+          <t>Approval log + SoD test</t>
         </is>
       </c>
       <c r="Q172" s="18" t="inlineStr">
@@ -15832,7 +15832,7 @@
     <row r="173">
       <c r="A173" s="15" t="inlineStr">
         <is>
-          <t>PAY-05</t>
+          <t>PAY-04</t>
         </is>
       </c>
       <c r="B173" s="16" t="inlineStr">
@@ -15847,37 +15847,37 @@
       </c>
       <c r="D173" s="16" t="inlineStr">
         <is>
-          <t>Payroll expense; Labor hours</t>
+          <t>Payroll expense; Labor cost</t>
         </is>
       </c>
       <c r="E173" s="16" t="inlineStr">
         <is>
-          <t>Time-and-attendance is unverified — one worker clocks a colleague in/out (buddy punching), or punches off-site, so paid labor hours overstate hours actually worked (payroll fraud / inflated labor cost), and there is no attributable override trail when a manager fixes a punch.</t>
+          <t>Overtime is paid at a single flat multiplier with no holiday/night tiers and no statutory cap (Thai LPA OT is mis-paid — too little on holidays, or beyond the 48h/week limit), AND labor cost runs over target as a % of sales with nothing flagging it — margin erosion goes unnoticed until payroll posts.</t>
         </is>
       </c>
       <c r="F173" s="16" t="inlineStr">
         <is>
-          <t>Existence/Accuracy/Authorization</t>
+          <t>Accuracy/Completeness</t>
         </is>
       </c>
       <c r="G173" s="16" t="inlineStr">
         <is>
-          <t>Clock-in integrity (anti-buddy-punch): a punch records its capture METHOD (PIN/QR/FACE_HASH/SUPERVISOR) and optional GPS; a re-punch within 15 minutes of the same employee's last clock-out is REJECTED (DUPLICATE_PUNCH) unless a supervisor overrides. A per-branch geofence_zone (lat/lng/radius) lets the clock-in compute geofence_pass when GPS is supplied; an out-of-fence punch is accepted but FLAGGED (geofence_pass=false) for review rather than hard-blocked (kiosks may lack GPS -&gt; null), and a SUPERVISOR override REQUIRES a reason (REASON_REQUIRED), stamps method=SUPERVISOR + the reason on the punch note, and is captured by the append-only audit_log so every override is attributable. The labor report surfaces method + geofence_pass so anomalies are visible. Tenant-scoped (RLS); gated pos/users/exec.</t>
+          <t>Tiered OT rules engine + labor-% alerting: a per-tenant labor_ot_rules table overrides the Thai LPA statutory defaults (REGULAR_OT 1.5x beyond 8h/day, HOLIDAY 2x, HOLIDAY_OT 3x, NIGHT 1.0x tracked; 48h/week cap) — GET/PUT /api/pos/labor/ot-rules. computeOtPay (POST /api/pos/labor/ot-pay) applies the tier's multiplier and CAPS paid hours at the 48h weekly limit, flagging any over-cap hours (over_cap=true) rather than silently paying them. Separately, POST /api/pos/labor/labor-alert/check computes labor % of sales for a period and, when it exceeds the target (default 35%), persists a LABOR_PCT_EXCEEDED alert (idempotent per period) surfaced on GET /api/pos/labor/alerts for the manager to act on / resolve. Tenant-scoped (RLS); gated pos/users/exec. Operational (no GL).</t>
         </is>
       </c>
       <c r="H173" s="17" t="inlineStr">
         <is>
-          <t>Prev/Det</t>
+          <t>Det/Prev</t>
         </is>
       </c>
       <c r="I173" s="17" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="J173" s="17" t="inlineStr">
         <is>
-          <t>Per punch</t>
+          <t>Per shift / payroll cycle</t>
         </is>
       </c>
       <c r="K173" s="16" t="inlineStr">
@@ -15892,22 +15892,22 @@
       </c>
       <c r="M173" s="16" t="inlineStr">
         <is>
-          <t>pos-loyalty-labor/timeclock.service.ts clockIn (DUPLICATE_PUNCH window, method capture, haversine geofence_pass) + supervisorOverride (REASON_REQUIRED, audited) + setGeofenceZone/listGeofenceZones; pos-loyalty-labor.controller.ts (clock-in, clock-in/override, geofence-zones); schema/pos-scale.ts time_clock.clock_in_method/lat/lng/geofence_pass + geofence_zones + migration 0169; cutover/pos-p2.ts (ToE)</t>
+          <t>pos-loyalty-labor/schedule.service.ts getOtRules/upsertOtRule (Thai defaults overlay) + computeOtPay (tier multiplier + 48h cap, over_cap flag) + checkLaborAlert/listAlerts/resolveAlert; pos-loyalty-labor.controller.ts (ot-rules, ot-pay, labor-alert/check, alerts[/:id/resolve]); schema/pos-scale.ts labor_ot_rules + labor_alerts + migration 0167; /scheduling UI; cutover/scheduling.ts (ToE)</t>
         </is>
       </c>
       <c r="N173" s="16" t="inlineStr">
         <is>
-          <t>Inspect the 15-min duplicate-punch guard, the method capture, the geofence pass/fail computation, and the supervisor-override reason + audit trail.</t>
+          <t>Inspect the statutory-default overlay, the tier multipliers, the 48h cap + over_cap flag, and the labor-% threshold alert (raise/idempotent/resolve).</t>
         </is>
       </c>
       <c r="O173" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: a re-punch within 15 min of clock-out -&gt; DUPLICATE_PUNCH; a supervisor override (with a reason) bypasses it and stamps method SUPERVISOR; an override with no reason -&gt; 400; an in-fence GPS punch -&gt; geofence_pass true; an out-of-fence punch is accepted but flagged geofence_pass false (re-performed by the pos-p2 harness).</t>
+          <t>Re-perform: OT rules expose Thai defaults (1.5/2/3/1.0, cap 48); override REGULAR_OT to 2.0; HOLIDAY_OT 2h x 100 x 3 = 600; a 5h OT entry at 47h already-worked pays only 1h + flags 4h over-cap; labor 8% vs a 5% target raises an alert (idempotent), vs a 50% target raises none; resolve clears it (re-performed by the scheduling harness).</t>
         </is>
       </c>
       <c r="P173" s="16" t="inlineStr">
         <is>
-          <t>time_clock method/geofence columns + override note; anti-buddy test</t>
+          <t>labor_ot_rules + labor_alerts register; OT/labor-% test</t>
         </is>
       </c>
       <c r="Q173" s="18" t="inlineStr">
@@ -15919,12 +15919,12 @@
     <row r="174">
       <c r="A174" s="11" t="inlineStr">
         <is>
-          <t>FA-09</t>
+          <t>PAY-05</t>
         </is>
       </c>
       <c r="B174" s="12" t="inlineStr">
         <is>
-          <t>Fixed Assets</t>
+          <t>Payroll</t>
         </is>
       </c>
       <c r="C174" s="13" t="inlineStr">
@@ -15934,27 +15934,27 @@
       </c>
       <c r="D174" s="12" t="inlineStr">
         <is>
-          <t>Property, Plant &amp; Equipment; Cash</t>
+          <t>Payroll expense; Labor hours</t>
         </is>
       </c>
       <c r="E174" s="12" t="inlineStr">
         <is>
-          <t>Asset disposed without independent review — one person writes an asset off the books and records the proceeds (asset-stripping / theft: dispose a still-held asset, or to a related party below value).</t>
+          <t>Time-and-attendance is unverified — one worker clocks a colleague in/out (buddy punching), or punches off-site, so paid labor hours overstate hours actually worked (payroll fraud / inflated labor cost), and there is no attributable override trail when a manager fixes a punch.</t>
         </is>
       </c>
       <c r="F174" s="12" t="inlineStr">
         <is>
-          <t>Authorization</t>
+          <t>Existence/Accuracy/Authorization</t>
         </is>
       </c>
       <c r="G174" s="12" t="inlineStr">
         <is>
-          <t>Asset-disposal maker-checker (SoD): a disposal REQUEST posts its GL entry as a DRAFT (excluded from balances) and flags the asset disposal_pending WITHOUT marking it disposed or moving the register; a DIFFERENT user must approve before it is effective (status→disposed, revaluation surplus recycled 3200→3100) (approver ≠ requester enforced regardless of permissions, reusing the GL-05 ledger approval). Reject voids the draft and the asset stays in service; only one disposal may be pending per asset; a disposal-pending asset is frozen from depreciation.</t>
+          <t>Clock-in integrity (anti-buddy-punch): a punch records its capture METHOD (PIN/QR/FACE_HASH/SUPERVISOR) and optional GPS; a re-punch within 15 minutes of the same employee's last clock-out is REJECTED (DUPLICATE_PUNCH) unless a supervisor overrides. A per-branch geofence_zone (lat/lng/radius) lets the clock-in compute geofence_pass when GPS is supplied; an out-of-fence punch is accepted but FLAGGED (geofence_pass=false) for review rather than hard-blocked (kiosks may lack GPS -&gt; null), and a SUPERVISOR override REQUIRES a reason (REASON_REQUIRED), stamps method=SUPERVISOR + the reason on the punch note, and is captured by the append-only audit_log so every override is attributable. The labor report surfaces method + geofence_pass so anomalies are visible. Tenant-scoped (RLS); gated pos/users/exec.</t>
         </is>
       </c>
       <c r="H174" s="13" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Prev/Det</t>
         </is>
       </c>
       <c r="I174" s="13" t="inlineStr">
@@ -15964,37 +15964,37 @@
       </c>
       <c r="J174" s="13" t="inlineStr">
         <is>
-          <t>Per disposal</t>
+          <t>Per punch</t>
         </is>
       </c>
       <c r="K174" s="12" t="inlineStr">
         <is>
-          <t>FaAccountant / Controller</t>
+          <t>HR / Store Ops Mgr</t>
         </is>
       </c>
       <c r="L174" s="13" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P10/P13</t>
         </is>
       </c>
       <c r="M174" s="12" t="inlineStr">
         <is>
-          <t>assets.service.ts dispose(pendingApproval Draft)/approveDisposal/rejectDisposal; assets.controller.ts (:assetNo/dispose/approve|reject); schema/assets.ts fixed_assets.disposal_pending + migration 0135; cutover/basics.ts + worldclass.ts + compliance.ts (ToE)</t>
+          <t>pos-loyalty-labor/timeclock.service.ts clockIn (DUPLICATE_PUNCH window, method capture, haversine geofence_pass) + supervisorOverride (REASON_REQUIRED, audited) + setGeofenceZone/listGeofenceZones; pos-loyalty-labor.controller.ts (clock-in, clock-in/override, geofence-zones); schema/pos-scale.ts time_clock.clock_in_method/lat/lng/geofence_pass + geofence_zones + migration 0169; cutover/pos-p2.ts (ToE)</t>
         </is>
       </c>
       <c r="N174" s="12" t="inlineStr">
         <is>
-          <t>Inspect Draft→approve flow + the approver≠requester check + deferred status/recycle.</t>
+          <t>Inspect the 15-min duplicate-punch guard, the method capture, the geofence pass/fail computation, and the supervisor-override reason + audit trail.</t>
         </is>
       </c>
       <c r="O174" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: request a disposal (Draft JE excluded), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm status→disposed + surplus recycled only after approval (re-performed by the harnesses).</t>
+          <t>Re-perform: a re-punch within 15 min of clock-out -&gt; DUPLICATE_PUNCH; a supervisor override (with a reason) bypasses it and stamps method SUPERVISOR; an override with no reason -&gt; 400; an in-fence GPS punch -&gt; geofence_pass true; an out-of-fence punch is accepted but flagged geofence_pass false (re-performed by the pos-p2 harness).</t>
         </is>
       </c>
       <c r="P174" s="12" t="inlineStr">
         <is>
-          <t>Disposal approval log + SoD test</t>
+          <t>time_clock method/geofence columns + override note; anti-buddy test</t>
         </is>
       </c>
       <c r="Q174" s="18" t="inlineStr">
@@ -16006,7 +16006,7 @@
     <row r="175">
       <c r="A175" s="15" t="inlineStr">
         <is>
-          <t>FA-10</t>
+          <t>FA-09</t>
         </is>
       </c>
       <c r="B175" s="16" t="inlineStr">
@@ -16021,22 +16021,22 @@
       </c>
       <c r="D175" s="16" t="inlineStr">
         <is>
-          <t>Property, Plant &amp; Equipment; Accounts Payable</t>
+          <t>Property, Plant &amp; Equipment; Cash</t>
         </is>
       </c>
       <c r="E175" s="16" t="inlineStr">
         <is>
-          <t>Capital purchases mis-capitalised or capitalised without independent review — the person who receives the goods also decides what enters the asset register and at what cost/useful life (fictitious or over-valued assets; capex/opex mis-classification).</t>
+          <t>Asset disposed without independent review — one person writes an asset off the books and records the proceeds (asset-stripping / theft: dispose a still-held asset, or to a related party below value).</t>
         </is>
       </c>
       <c r="F175" s="16" t="inlineStr">
         <is>
-          <t>Authorization; Accuracy</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="G175" s="16" t="inlineStr">
         <is>
-          <t>Procure-to-Capitalize maker-checker (SoD): a goods-receipt line flagged capital (item-master is_fixed_asset or per-PO-line override) is excluded from inventory capitalisation (1200) at receipt and instead becomes ELIGIBLE for the asset register. Capitalisation is a REQUEST that posts NOTHING to the GL; a DIFFERENT user must approve before the fixed_assets row + acquisition JE (Dr 1500 / Cr 2000) are created (approver ≠ requester enforced regardless of permissions). The created asset carries its source GR/PO for end-to-end PR→PO→GR→FA traceability; a GR line cannot be capitalised twice.</t>
+          <t>Asset-disposal maker-checker (SoD): a disposal REQUEST posts its GL entry as a DRAFT (excluded from balances) and flags the asset disposal_pending WITHOUT marking it disposed or moving the register; a DIFFERENT user must approve before it is effective (status→disposed, revaluation surplus recycled 3200→3100) (approver ≠ requester enforced regardless of permissions, reusing the GL-05 ledger approval). Reject voids the draft and the asset stays in service; only one disposal may be pending per asset; a disposal-pending asset is frozen from depreciation.</t>
         </is>
       </c>
       <c r="H175" s="17" t="inlineStr">
@@ -16051,7 +16051,7 @@
       </c>
       <c r="J175" s="17" t="inlineStr">
         <is>
-          <t>Per capital receipt</t>
+          <t>Per disposal</t>
         </is>
       </c>
       <c r="K175" s="16" t="inlineStr">
@@ -16066,22 +16066,22 @@
       </c>
       <c r="M175" s="16" t="inlineStr">
         <is>
-          <t>assets.service.ts registerFromGr/approveRegistration/rejectRegistration/eligibleFromGr; assets.controller.ts (registrations*); procurement.service.ts createGr (is_capital routing, costing excluded); schema/assets.ts asset_registration_requests + fixed_assets.source_gr_no/po_no + migration 0137; cutover/basics.ts + compliance.ts (ToE)</t>
+          <t>assets.service.ts dispose(pendingApproval Draft)/approveDisposal/rejectDisposal; assets.controller.ts (:assetNo/dispose/approve|reject); schema/assets.ts fixed_assets.disposal_pending + migration 0135; cutover/basics.ts + worldclass.ts + compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N175" s="16" t="inlineStr">
         <is>
-          <t>Inspect the eligible→request→approve flow + approver≠requester check + the inventory-vs-asset routing of capital lines.</t>
+          <t>Inspect Draft→approve flow + the approver≠requester check + deferred status/recycle.</t>
         </is>
       </c>
       <c r="O175" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: receive a capital line, raise a registration (no GL), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm the asset + Dr 1500/Cr 2000 post only after approval and the line cannot be re-registered (re-performed by the harnesses).</t>
+          <t>Re-perform: request a disposal (Draft JE excluded), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm status→disposed + surplus recycled only after approval (re-performed by the harnesses).</t>
         </is>
       </c>
       <c r="P175" s="16" t="inlineStr">
         <is>
-          <t>Capitalization approval log + SoD test</t>
+          <t>Disposal approval log + SoD test</t>
         </is>
       </c>
       <c r="Q175" s="18" t="inlineStr">
@@ -16093,12 +16093,12 @@
     <row r="176">
       <c r="A176" s="11" t="inlineStr">
         <is>
-          <t>CON-01</t>
+          <t>FA-10</t>
         </is>
       </c>
       <c r="B176" s="12" t="inlineStr">
         <is>
-          <t>Consolidation &amp; FX</t>
+          <t>Fixed Assets</t>
         </is>
       </c>
       <c r="C176" s="13" t="inlineStr">
@@ -16108,42 +16108,42 @@
       </c>
       <c r="D176" s="12" t="inlineStr">
         <is>
-          <t>Consolidation</t>
+          <t>Property, Plant &amp; Equipment; Accounts Payable</t>
         </is>
       </c>
       <c r="E176" s="12" t="inlineStr">
         <is>
-          <t>Group consolidation mis-stated (ownership/currency).</t>
+          <t>Capital purchases mis-capitalised or capitalised without independent review — the person who receives the goods also decides what enters the asset register and at what cost/useful life (fictitious or over-valued assets; capex/opex mis-classification).</t>
         </is>
       </c>
       <c r="F176" s="12" t="inlineStr">
         <is>
-          <t>Accuracy</t>
+          <t>Authorization; Accuracy</t>
         </is>
       </c>
       <c r="G176" s="12" t="inlineStr">
         <is>
-          <t>Consolidation run (ownership %, entity currency) gated by 'approvals'.</t>
+          <t>Procure-to-Capitalize maker-checker (SoD): a goods-receipt line flagged capital (item-master is_fixed_asset or per-PO-line override) is excluded from inventory capitalisation (1200) at receipt and instead becomes ELIGIBLE for the asset register. Capitalisation is a REQUEST that posts NOTHING to the GL; a DIFFERENT user must approve before the fixed_assets row + acquisition JE (Dr 1500 / Cr 2000) are created (approver ≠ requester enforced regardless of permissions). The created asset carries its source GR/PO for end-to-end PR→PO→GR→FA traceability; a GR line cannot be capitalised twice.</t>
         </is>
       </c>
       <c r="H176" s="13" t="inlineStr">
         <is>
-          <t>Auto+Manual</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I176" s="13" t="inlineStr">
         <is>
-          <t>Period</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J176" s="13" t="inlineStr">
         <is>
-          <t>Period</t>
+          <t>Per capital receipt</t>
         </is>
       </c>
       <c r="K176" s="12" t="inlineStr">
         <is>
-          <t>Group Controller</t>
+          <t>FaAccountant / Controller</t>
         </is>
       </c>
       <c r="L176" s="13" t="inlineStr">
@@ -16153,22 +16153,22 @@
       </c>
       <c r="M176" s="12" t="inlineStr">
         <is>
-          <t>consolidation.service.ts (runConsolidation @Permissions approvals)</t>
+          <t>assets.service.ts registerFromGr/approveRegistration/rejectRegistration/eligibleFromGr; assets.controller.ts (registrations*); procurement.service.ts createGr (is_capital routing, costing excluded); schema/assets.ts asset_registration_requests + fixed_assets.source_gr_no/po_no + migration 0137; cutover/basics.ts + compliance.ts (ToE)</t>
         </is>
       </c>
       <c r="N176" s="12" t="inlineStr">
         <is>
-          <t>Inspect consolidation logic + gate.</t>
+          <t>Inspect the eligible→request→approve flow + approver≠requester check + the inventory-vs-asset routing of capital lines.</t>
         </is>
       </c>
       <c r="O176" s="12" t="inlineStr">
         <is>
-          <t>Sample period: consolidated TB ties to entities.</t>
+          <t>Re-perform: receive a capital line, raise a registration (no GL), attempt self-approve (SOD_VIOLATION), approve as a different user; confirm the asset + Dr 1500/Cr 2000 post only after approval and the line cannot be re-registered (re-performed by the harnesses).</t>
         </is>
       </c>
       <c r="P176" s="12" t="inlineStr">
         <is>
-          <t>Consol TB</t>
+          <t>Capitalization approval log + SoD test</t>
         </is>
       </c>
       <c r="Q176" s="18" t="inlineStr">
@@ -16180,7 +16180,7 @@
     <row r="177">
       <c r="A177" s="15" t="inlineStr">
         <is>
-          <t>CON-02</t>
+          <t>CON-01</t>
         </is>
       </c>
       <c r="B177" s="16" t="inlineStr">
@@ -16195,22 +16195,22 @@
       </c>
       <c r="D177" s="16" t="inlineStr">
         <is>
-          <t>FX gain/loss</t>
+          <t>Consolidation</t>
         </is>
       </c>
       <c r="E177" s="16" t="inlineStr">
         <is>
-          <t>FX exposures not revalued at period-end.</t>
+          <t>Group consolidation mis-stated (ownership/currency).</t>
         </is>
       </c>
       <c r="F177" s="16" t="inlineStr">
         <is>
-          <t>Valuation</t>
+          <t>Accuracy</t>
         </is>
       </c>
       <c r="G177" s="16" t="inlineStr">
         <is>
-          <t>FX revaluation at period-end rates; unrealized FX posted (acct 5400).</t>
+          <t>Consolidation run (ownership %, entity currency) gated by 'approvals'.</t>
         </is>
       </c>
       <c r="H177" s="17" t="inlineStr">
@@ -16220,7 +16220,7 @@
       </c>
       <c r="I177" s="17" t="inlineStr">
         <is>
-          <t>Period-end</t>
+          <t>Period</t>
         </is>
       </c>
       <c r="J177" s="17" t="inlineStr">
@@ -16230,7 +16230,7 @@
       </c>
       <c r="K177" s="16" t="inlineStr">
         <is>
-          <t>Controller</t>
+          <t>Group Controller</t>
         </is>
       </c>
       <c r="L177" s="17" t="inlineStr">
@@ -16240,22 +16240,22 @@
       </c>
       <c r="M177" s="16" t="inlineStr">
         <is>
-          <t>fx.service.ts (revalue / unrealized report)</t>
+          <t>consolidation.service.ts (runConsolidation @Permissions approvals)</t>
         </is>
       </c>
       <c r="N177" s="16" t="inlineStr">
         <is>
-          <t>Inspect reval logic + rates.</t>
+          <t>Inspect consolidation logic + gate.</t>
         </is>
       </c>
       <c r="O177" s="16" t="inlineStr">
         <is>
-          <t>Recompute reval on sample balances.</t>
+          <t>Sample period: consolidated TB ties to entities.</t>
         </is>
       </c>
       <c r="P177" s="16" t="inlineStr">
         <is>
-          <t>FX reval JE</t>
+          <t>Consol TB</t>
         </is>
       </c>
       <c r="Q177" s="18" t="inlineStr">
@@ -16267,7 +16267,7 @@
     <row r="178">
       <c r="A178" s="11" t="inlineStr">
         <is>
-          <t>CON-03</t>
+          <t>CON-02</t>
         </is>
       </c>
       <c r="B178" s="12" t="inlineStr">
@@ -16282,32 +16282,32 @@
       </c>
       <c r="D178" s="12" t="inlineStr">
         <is>
-          <t>Consolidation</t>
+          <t>FX gain/loss</t>
         </is>
       </c>
       <c r="E178" s="12" t="inlineStr">
         <is>
-          <t>Intercompany balances/transactions are not eliminated on consolidation, OR eliminations are mis-stated, so the consolidated group trial balance does not balance and group financials are overstated (IC double-counted).</t>
+          <t>FX exposures not revalued at period-end.</t>
         </is>
       </c>
       <c r="F178" s="12" t="inlineStr">
         <is>
-          <t>Accuracy/Completeness</t>
+          <t>Valuation</t>
         </is>
       </c>
       <c r="G178" s="12" t="inlineStr">
         <is>
-          <t>Elimination integrity (CON-03): runConsolidation combines member-entity TBs, generates reciprocal IC eliminations (Dr 2150 Due-To / Cr 1150 Due-From for each in-group IC transaction) at the GROUP layer (consolidation_run_lines — NOT pushed into any operating entity's GL), and ASSERTS the consolidated TB still balances (Σ signed nets ~0 and eliminations net to 0, NCI presentation reclass excluded) — failure throws CONSOL_UNBALANCED and rolls back the run. A balanced run is finalised, then frozen by a DIFFERENT user via run→post maker-checker (self-post → SELF_POST; re-running a Posted period → ALREADY_POSTED; one run per (group, period)). HQ/Admin-only; reads across member tenants via app.bypass_rls. Configurable elimination rules (consol_elimination_rules).</t>
+          <t>FX revaluation at period-end rates; unrealized FX posted (acct 5400).</t>
         </is>
       </c>
       <c r="H178" s="13" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="I178" s="13" t="inlineStr">
         <is>
-          <t>Auto+Manual</t>
+          <t>Period-end</t>
         </is>
       </c>
       <c r="J178" s="13" t="inlineStr">
@@ -16317,7 +16317,7 @@
       </c>
       <c r="K178" s="12" t="inlineStr">
         <is>
-          <t>Group Controller</t>
+          <t>Controller</t>
         </is>
       </c>
       <c r="L178" s="13" t="inlineStr">
@@ -16327,22 +16327,22 @@
       </c>
       <c r="M178" s="12" t="inlineStr">
         <is>
-          <t>consolidation.service.ts runConsolidation (balanced check, CONSOL_UNBALANCED)/postConsolidation (SELF_POST, ALREADY_POSTED); consolidation.controller.ts (run @approvals, runs/:id/post @approvals); schema/consolidation.ts (consolidation_runs.balanced/posted_by, consol_elimination_rules) + migration 0170; cutover/consolidation.ts (ToE)</t>
+          <t>fx.service.ts (revalue / unrealized report)</t>
         </is>
       </c>
       <c r="N178" s="12" t="inlineStr">
         <is>
-          <t>Inspect the combine→eliminate→balance flow, the CONSOL_UNBALANCED guard, and the run→post approver≠runner check.</t>
+          <t>Inspect reval logic + rates.</t>
         </is>
       </c>
       <c r="O178" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: run a group consolidation, confirm IC 1150/2150 eliminate and the consolidated TB balances; attempt self-post (SELF_POST); post as a different user (Posted); re-run the posted period (ALREADY_POSTED). Re-performed by the consolidation harness.</t>
+          <t>Recompute reval on sample balances.</t>
         </is>
       </c>
       <c r="P178" s="12" t="inlineStr">
         <is>
-          <t>Consolidated TB + elimination lines + post log</t>
+          <t>FX reval JE</t>
         </is>
       </c>
       <c r="Q178" s="18" t="inlineStr">
@@ -16354,7 +16354,7 @@
     <row r="179">
       <c r="A179" s="15" t="inlineStr">
         <is>
-          <t>CON-04</t>
+          <t>CON-03</t>
         </is>
       </c>
       <c r="B179" s="16" t="inlineStr">
@@ -16369,27 +16369,27 @@
       </c>
       <c r="D179" s="16" t="inlineStr">
         <is>
-          <t>All (segment disclosure)</t>
+          <t>Consolidation</t>
         </is>
       </c>
       <c r="E179" s="16" t="inlineStr">
         <is>
-          <t>Segment (branch/project/department) operating results are not reported, so IFRS 8 segment disclosure is incomplete or inaccurate and management/investors cannot see results by reportable segment.</t>
+          <t>Intercompany balances/transactions are not eliminated on consolidation, OR eliminations are mis-stated, so the consolidated group trial balance does not balance and group financials are overstated (IC double-counted).</t>
         </is>
       </c>
       <c r="F179" s="16" t="inlineStr">
         <is>
-          <t>Presentation/Disclosure</t>
+          <t>Accuracy/Completeness</t>
         </is>
       </c>
       <c r="G179" s="16" t="inlineStr">
         <is>
-          <t>Segment reporting (CON-04, IFRS 8): segmentReport produces P&amp;L (revenue/expense/net) grouped by reportable segment, sourced from the dimension columns on journal_lines (branch_id/project_id/department_id) and mapped through configurable segment_definitions (member_keys → segment); unmapped dimension values surface as their own/Unassigned bucket. HQ/Admin-only, gated 'exec'.</t>
+          <t>Elimination integrity (CON-03): runConsolidation combines member-entity TBs, generates reciprocal IC eliminations (Dr 2150 Due-To / Cr 1150 Due-From for each in-group IC transaction) at the GROUP layer (consolidation_run_lines — NOT pushed into any operating entity's GL), and ASSERTS the consolidated TB still balances (Σ signed nets ~0 and eliminations net to 0, NCI presentation reclass excluded) — failure throws CONSOL_UNBALANCED and rolls back the run. A balanced run is finalised, then frozen by a DIFFERENT user via run→post maker-checker (self-post → SELF_POST; re-running a Posted period → ALREADY_POSTED; one run per (group, period)). HQ/Admin-only; reads across member tenants via app.bypass_rls. Configurable elimination rules (consol_elimination_rules).</t>
         </is>
       </c>
       <c r="H179" s="17" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I179" s="17" t="inlineStr">
@@ -16414,22 +16414,22 @@
       </c>
       <c r="M179" s="16" t="inlineStr">
         <is>
-          <t>consolidation.service.ts defineSegment/listSegments/segmentReport; consolidation.controller.ts (segments, segment-report @exec); schema/consolidation.ts segment_definitions + migration 0170; cutover/consolidation.ts (ToE)</t>
+          <t>consolidation.service.ts runConsolidation (balanced check, CONSOL_UNBALANCED)/postConsolidation (SELF_POST, ALREADY_POSTED); consolidation.controller.ts (run @approvals, runs/:id/post @approvals); schema/consolidation.ts (consolidation_runs.balanced/posted_by, consol_elimination_rules) + migration 0170; cutover/consolidation.ts (ToE)</t>
         </is>
       </c>
       <c r="N179" s="16" t="inlineStr">
         <is>
-          <t>Inspect the segment mapping + the dimension-grouped P&amp;L aggregation.</t>
+          <t>Inspect the combine→eliminate→balance flow, the CONSOL_UNBALANCED guard, and the run→post approver≠runner check.</t>
         </is>
       </c>
       <c r="O179" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: define a segment over branches, run the segment report for a period, confirm revenue/expense/net tie to the underlying dimensioned postings. Re-performed by the consolidation harness.</t>
+          <t>Re-perform: run a group consolidation, confirm IC 1150/2150 eliminate and the consolidated TB balances; attempt self-post (SELF_POST); post as a different user (Posted); re-run the posted period (ALREADY_POSTED). Re-performed by the consolidation harness.</t>
         </is>
       </c>
       <c r="P179" s="16" t="inlineStr">
         <is>
-          <t>Segment P&amp;L report</t>
+          <t>Consolidated TB + elimination lines + post log</t>
         </is>
       </c>
       <c r="Q179" s="18" t="inlineStr">
@@ -16441,7 +16441,7 @@
     <row r="180">
       <c r="A180" s="11" t="inlineStr">
         <is>
-          <t>FX-04</t>
+          <t>CON-04</t>
         </is>
       </c>
       <c r="B180" s="12" t="inlineStr">
@@ -16456,42 +16456,42 @@
       </c>
       <c r="D180" s="12" t="inlineStr">
         <is>
-          <t>FX gain/loss; Revenue; AR/AP</t>
+          <t>All (segment disclosure)</t>
         </is>
       </c>
       <c r="E180" s="12" t="inlineStr">
         <is>
-          <t>A wrong manually-entered FX rate (fat-fingered, e.g. USD 36 keyed as 63) flows straight into a period-end revaluation JE and the unrealized-FX report with no independent review — mis-stating earnings/equity and FX-translated balances.</t>
+          <t>Segment (branch/project/department) operating results are not reported, so IFRS 8 segment disclosure is incomplete or inaccurate and management/investors cannot see results by reportable segment.</t>
         </is>
       </c>
       <c r="F180" s="12" t="inlineStr">
         <is>
-          <t>Accuracy/Valuation</t>
+          <t>Presentation/Disclosure</t>
         </is>
       </c>
       <c r="G180" s="12" t="inlineStr">
         <is>
-          <t>FX rate maker-checker (SoD): a MANUALLY-entered rate lands as PendingApproval and is EXCLUDED from rate resolution — revaluation, the unrealized-FX report, and consolidation translation all use APPROVED rates only — until a DIFFERENT user approves it (POST /api/fx/rates/approve). Self-approval → SOD_VIOLATION (binds even Admin); reject marks the rate Rejected (never usable); re-entering a rate sends it back to PendingApproval. Externally-sourced (feed) rates carrying an explicit non-manual source are auto-approved. Pending rates are also surfaced, aged, by the pending-approvals monitor (GOV-01).</t>
+          <t>Segment reporting (CON-04, IFRS 8): segmentReport produces P&amp;L (revenue/expense/net) grouped by reportable segment, sourced from the dimension columns on journal_lines (branch_id/project_id/department_id) and mapped through configurable segment_definitions (member_keys → segment); unmapped dimension values surface as their own/Unassigned bucket. HQ/Admin-only, gated 'exec'.</t>
         </is>
       </c>
       <c r="H180" s="13" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I180" s="13" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="J180" s="13" t="inlineStr">
         <is>
-          <t>Per rate</t>
+          <t>Period</t>
         </is>
       </c>
       <c r="K180" s="12" t="inlineStr">
         <is>
-          <t>Controller / Treasury</t>
+          <t>Group Controller</t>
         </is>
       </c>
       <c r="L180" s="13" t="inlineStr">
@@ -16501,22 +16501,22 @@
       </c>
       <c r="M180" s="12" t="inlineStr">
         <is>
-          <t>fx.service.ts setRate(manual→PendingApproval)/approveRate/rejectRate/rateAsOf(Approved only); fx.controller.ts (rates/approve|reject|pending gated approvals/gl_close); consolidation.service.ts (translation reads Approved rates); schema/fx.ts fx_rates.status + migration 0141; cutover/fxreval.ts (ToE)</t>
+          <t>consolidation.service.ts defineSegment/listSegments/segmentReport; consolidation.controller.ts (segments, segment-report @exec); schema/consolidation.ts segment_definitions + migration 0170; cutover/consolidation.ts (ToE)</t>
         </is>
       </c>
       <c r="N180" s="12" t="inlineStr">
         <is>
-          <t>Inspect the request→approve flow + the approver≠requester check + that revaluation/reporting resolve Approved rates only.</t>
+          <t>Inspect the segment mapping + the dimension-grouped P&amp;L aggregation.</t>
         </is>
       </c>
       <c r="O180" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: enter a manual rate (PendingApproval), confirm revalue is blocked NO_RATE while pending, attempt self-approve (SOD_VIOLATION), approve as a different user, then revalue succeeds (re-performed by the fxreval harness).</t>
+          <t>Re-perform: define a segment over branches, run the segment report for a period, confirm revenue/expense/net tie to the underlying dimensioned postings. Re-performed by the consolidation harness.</t>
         </is>
       </c>
       <c r="P180" s="12" t="inlineStr">
         <is>
-          <t>FX rate approval log + SoD test</t>
+          <t>Segment P&amp;L report</t>
         </is>
       </c>
       <c r="Q180" s="18" t="inlineStr">
@@ -16528,92 +16528,179 @@
     <row r="181">
       <c r="A181" s="15" t="inlineStr">
         <is>
+          <t>FX-04</t>
+        </is>
+      </c>
+      <c r="B181" s="16" t="inlineStr">
+        <is>
+          <t>Consolidation &amp; FX</t>
+        </is>
+      </c>
+      <c r="C181" s="17" t="inlineStr">
+        <is>
+          <t>Application</t>
+        </is>
+      </c>
+      <c r="D181" s="16" t="inlineStr">
+        <is>
+          <t>FX gain/loss; Revenue; AR/AP</t>
+        </is>
+      </c>
+      <c r="E181" s="16" t="inlineStr">
+        <is>
+          <t>A wrong manually-entered FX rate (fat-fingered, e.g. USD 36 keyed as 63) flows straight into a period-end revaluation JE and the unrealized-FX report with no independent review — mis-stating earnings/equity and FX-translated balances.</t>
+        </is>
+      </c>
+      <c r="F181" s="16" t="inlineStr">
+        <is>
+          <t>Accuracy/Valuation</t>
+        </is>
+      </c>
+      <c r="G181" s="16" t="inlineStr">
+        <is>
+          <t>FX rate maker-checker (SoD): a MANUALLY-entered rate lands as PendingApproval and is EXCLUDED from rate resolution — revaluation, the unrealized-FX report, and consolidation translation all use APPROVED rates only — until a DIFFERENT user approves it (POST /api/fx/rates/approve). Self-approval → SOD_VIOLATION (binds even Admin); reject marks the rate Rejected (never usable); re-entering a rate sends it back to PendingApproval. Externally-sourced (feed) rates carrying an explicit non-manual source are auto-approved. Pending rates are also surfaced, aged, by the pending-approvals monitor (GOV-01).</t>
+        </is>
+      </c>
+      <c r="H181" s="17" t="inlineStr">
+        <is>
+          <t>Prev</t>
+        </is>
+      </c>
+      <c r="I181" s="17" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="J181" s="17" t="inlineStr">
+        <is>
+          <t>Per rate</t>
+        </is>
+      </c>
+      <c r="K181" s="16" t="inlineStr">
+        <is>
+          <t>Controller / Treasury</t>
+        </is>
+      </c>
+      <c r="L181" s="17" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="M181" s="16" t="inlineStr">
+        <is>
+          <t>fx.service.ts setRate(manual→PendingApproval)/approveRate/rejectRate/rateAsOf(Approved only); fx.controller.ts (rates/approve|reject|pending gated approvals/gl_close); consolidation.service.ts (translation reads Approved rates); schema/fx.ts fx_rates.status + migration 0141; cutover/fxreval.ts (ToE)</t>
+        </is>
+      </c>
+      <c r="N181" s="16" t="inlineStr">
+        <is>
+          <t>Inspect the request→approve flow + the approver≠requester check + that revaluation/reporting resolve Approved rates only.</t>
+        </is>
+      </c>
+      <c r="O181" s="16" t="inlineStr">
+        <is>
+          <t>Re-perform: enter a manual rate (PendingApproval), confirm revalue is blocked NO_RATE while pending, attempt self-approve (SOD_VIOLATION), approve as a different user, then revalue succeeds (re-performed by the fxreval harness).</t>
+        </is>
+      </c>
+      <c r="P181" s="16" t="inlineStr">
+        <is>
+          <t>FX rate approval log + SoD test</t>
+        </is>
+      </c>
+      <c r="Q181" s="18" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="11" t="inlineStr">
+        <is>
           <t>BUD-01</t>
         </is>
       </c>
-      <c r="B181" s="16" t="inlineStr">
+      <c r="B182" s="12" t="inlineStr">
         <is>
           <t>Budgeting &amp; Planning</t>
         </is>
       </c>
-      <c r="C181" s="17" t="inlineStr">
+      <c r="C182" s="13" t="inlineStr">
         <is>
           <t>Application</t>
         </is>
       </c>
-      <c r="D181" s="16" t="inlineStr">
+      <c r="D182" s="12" t="inlineStr">
         <is>
           <t>Budget; All (variance reporting)</t>
         </is>
       </c>
-      <c r="E181" s="16" t="inlineStr">
+      <c r="E182" s="12" t="inlineStr">
         <is>
           <t>A budget figure is entered/changed by one person and immediately drives the budget-vs-actual variance report — the basis for spend authorization and performance review — with no independent approval; a wrong or self-serving budget makes overspending look 'on budget'.</t>
         </is>
       </c>
-      <c r="F181" s="16" t="inlineStr">
+      <c r="F182" s="12" t="inlineStr">
         <is>
           <t>Authorization/Accuracy</t>
         </is>
       </c>
-      <c r="G181" s="16" t="inlineStr">
+      <c r="G182" s="12" t="inlineStr">
         <is>
           <t>Budget maker-checker (SoD): an upserted budget (POST /api/ledger/budgets) lands as PendingApproval and is EXCLUDED from budget-vs-actual until a DIFFERENT user approves it (POST /api/ledger/budgets/approve for the fiscal_year/account/cost-centre[/period]). Self-approval → SOD_VIOLATION (binds even Admin); reject marks it Rejected (excluded). DEFAULT 'Approved' keeps existing rows + direct planning seeds usable. Pending budgets are also surfaced, aged, by the pending-approvals monitor (GOV-01).</t>
         </is>
       </c>
-      <c r="H181" s="17" t="inlineStr">
+      <c r="H182" s="13" t="inlineStr">
         <is>
           <t>Prev</t>
         </is>
       </c>
-      <c r="I181" s="17" t="inlineStr">
+      <c r="I182" s="13" t="inlineStr">
         <is>
           <t>Automated</t>
         </is>
       </c>
-      <c r="J181" s="17" t="inlineStr">
+      <c r="J182" s="13" t="inlineStr">
         <is>
           <t>Per budget</t>
         </is>
       </c>
-      <c r="K181" s="16" t="inlineStr">
+      <c r="K182" s="12" t="inlineStr">
         <is>
           <t>Controller / FP&amp;A</t>
         </is>
       </c>
-      <c r="L181" s="17" t="inlineStr">
+      <c r="L182" s="13" t="inlineStr">
         <is>
           <t>P10</t>
         </is>
       </c>
-      <c r="M181" s="16" t="inlineStr">
+      <c r="M182" s="12" t="inlineStr">
         <is>
           <t>budget.service.ts upsertBudget(→PendingApproval)/approveBudget/rejectBudget/budgetVsActual(Approved only); budget.controller.ts (budgets/approve|reject|pending gated approvals/gl_close); schema/budgets.ts budgets.status + migration 0142; cutover/budget.ts (ToE)</t>
         </is>
       </c>
-      <c r="N181" s="16" t="inlineStr">
+      <c r="N182" s="12" t="inlineStr">
         <is>
           <t>Inspect the request→approve flow + the approver≠requester check + that budget-vs-actual counts Approved budgets only.</t>
         </is>
       </c>
-      <c r="O181" s="16" t="inlineStr">
+      <c r="O182" s="12" t="inlineStr">
         <is>
           <t>Re-perform: upsert a budget (PendingApproval, excluded from variance), attempt self-approve (SOD_VIOLATION), approve as a different user, confirm it then appears in budget-vs-actual (re-performed by the budget harness).</t>
         </is>
       </c>
-      <c r="P181" s="16" t="inlineStr">
+      <c r="P182" s="12" t="inlineStr">
         <is>
           <t>Budget approval log + SoD test</t>
         </is>
       </c>
-      <c r="Q181" s="18" t="inlineStr">
+      <c r="Q182" s="18" t="inlineStr">
         <is>
           <t>Implemented</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q181"/>
+  <autoFilter ref="A1:Q182"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -17250,7 +17337,7 @@
         </is>
       </c>
       <c r="C5" s="26">
-        <f>COUNTIF(RCM!$Q$2:$Q$181,B5)</f>
+        <f>COUNTIF(RCM!$Q$2:$Q$182,B5)</f>
         <v/>
       </c>
     </row>
@@ -17261,7 +17348,7 @@
         </is>
       </c>
       <c r="C6" s="26">
-        <f>COUNTIF(RCM!$Q$2:$Q$181,B6)</f>
+        <f>COUNTIF(RCM!$Q$2:$Q$182,B6)</f>
         <v/>
       </c>
     </row>
@@ -17272,7 +17359,7 @@
         </is>
       </c>
       <c r="C7" s="26">
-        <f>COUNTIF(RCM!$Q$2:$Q$181,B7)</f>
+        <f>COUNTIF(RCM!$Q$2:$Q$182,B7)</f>
         <v/>
       </c>
     </row>
@@ -17283,7 +17370,7 @@
         </is>
       </c>
       <c r="C8" s="29">
-        <f>COUNTA(RCM!$A$2:$A$181)</f>
+        <f>COUNTA(RCM!$A$2:$A$182)</f>
         <v/>
       </c>
     </row>
@@ -17301,7 +17388,7 @@
         </is>
       </c>
       <c r="C11" s="26">
-        <f>COUNTIF(RCM!$C$2:$C$181,B11)</f>
+        <f>COUNTIF(RCM!$C$2:$C$182,B11)</f>
         <v/>
       </c>
     </row>
@@ -17312,7 +17399,7 @@
         </is>
       </c>
       <c r="C12" s="26">
-        <f>COUNTIF(RCM!$C$2:$C$181,B12)</f>
+        <f>COUNTIF(RCM!$C$2:$C$182,B12)</f>
         <v/>
       </c>
     </row>
@@ -17323,7 +17410,7 @@
         </is>
       </c>
       <c r="C13" s="26">
-        <f>COUNTIF(RCM!$C$2:$C$181,B13)</f>
+        <f>COUNTIF(RCM!$C$2:$C$182,B13)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Wire vat_code → VAT posting: tax_codes now drive VAT accounts (docs/33 follow-up, GL-21/TAX-04) (#412)
Makes the tax_codes master live: a configured VAT code drives the rate + output/input VAT GL account instead of the flat 7/107 → 2100. AR output VAT routes to the order's uniform item vat_code account (flag-gated, parity when off); AP bills accept a tax_code → input-VAT account + rate (inclusive-aware, fail-closed UNKNOWN_TAX_CODE). pp30's VAT↔GL reconciliation (TAX-04) now sums the whole VAT-account set so the ภ.พ.30 tie stays exact under routing. Doc-synced (RCM GL-21/TAX-04, tax narrative rev 0.10, user manual, UAT-TAX-031/032/033). All CI green.
</commit_message>
<xml_diff>
--- a/compliance/Oshinei_ERP_SOX_RCM_v1.xlsx
+++ b/compliance/Oshinei_ERP_SOX_RCM_v1.xlsx
@@ -13774,7 +13774,7 @@
       </c>
       <c r="G149" s="16" t="inlineStr">
         <is>
-          <t>Item-posting account determination (extends GL-12 to the item grain): a per-tenant, opt-in flag (posting_determination, default OFF ⇒ literal parity) lets an item's GL/tax profile drive posting. AccountDeterminationService.resolveItemAccounts resolves each account by precedence item column → its item_categories row → its WAREHOUSE (locations) default → null (caller falls back to the hard-coded control account), so an un-opted-in or unconfigured tenant is byte-for-byte unchanged. The inventory sub-ledger (receive/issue/adjust/issue-to-project) routes its inventory, COGS &amp; adjustment legs through the resolver; reconcile() sums the WHOLE inventory-account set (control 1200 + any item/category/warehouse overrides) so the GL-14-style sub-ledger↔GL tie-out holds under routing. Fail-closed: a resolved override that is not a real, POSTABLE account in the canonical CoA is rejected with INVALID_POSTING_ACCOUNT before any posting — a typo'd/header/control account can never receive a posting.</t>
+          <t>Item-posting account determination (extends GL-12 to the item grain): a per-tenant, opt-in flag (posting_determination, default OFF ⇒ literal parity) lets an item's GL/tax profile drive posting. AccountDeterminationService.resolveItemAccounts resolves each account by precedence item column → its item_categories row → its WAREHOUSE (locations) default → null (caller falls back to the hard-coded control account), so an un-opted-in or unconfigured tenant is byte-for-byte unchanged. The inventory sub-ledger (receive/issue/adjust/issue-to-project) routes its inventory, COGS &amp; adjustment legs through the resolver; reconcile() sums the WHOLE inventory-account set (control 1200 + any item/category/warehouse overrides) so the GL-14-style sub-ledger↔GL tie-out holds under routing. Fail-closed: a resolved override that is not a real, POSTABLE account in the canonical CoA is rejected with INVALID_POSTING_ACCOUNT before any posting — a typo'd/header/control account can never receive a posting. VAT (docs/33 PR6): a configured tax_code drives the VAT rate + output/input VAT GL account on AR invoices (from the order's uniform item vat_code) and AP bills (from an explicit tax_code); an unknown/non-VAT code fails closed (UNKNOWN_TAX_CODE/NOT_A_VAT_CODE), and the PP30↔GL reconciliation (TAX-04) sums the whole VAT-account set so the tie holds under routing.</t>
         </is>
       </c>
       <c r="H149" s="17" t="inlineStr">
@@ -15340,7 +15340,7 @@
       </c>
       <c r="G167" s="16" t="inlineStr">
         <is>
-          <t>Periodic VAT-return ↔ GL reconciliation (ภ.พ.30): the monthly return (GET /api/tax-reports/pp30) is built from the sales/output-VAT and purchase/input-VAT sub-reports, computes net VAT = output − input, and RECONCILES it to the **GL account 2100 (Tax Payable) net movement** for the same period (Σ credit − Σ debit over Posted entries) — returning `reconciliation.tied` = true only when the two agree within rounding. A non-tie is a detective finding to investigate and clear BEFORE filing (the form also carries the ม.157 deadline = the 15th of the next month). Output VAT is posted to 2100 on every sale (Cr) and reversed on returns (Dr); input VAT is posted on AP bills (Dr) — so 2100's net is the period's VAT payable. Read-only report; exportable to a ภ.พ.30 PDF/HTML.</t>
+          <t>Periodic VAT-return ↔ GL reconciliation (ภ.พ.30): the monthly return (GET /api/tax-reports/pp30) is built from the sales/output-VAT and purchase/input-VAT sub-reports, computes net VAT = output − input, and RECONCILES it to the **GL account 2100 (Tax Payable) net movement** for the same period (Σ credit − Σ debit over Posted entries) — returning `reconciliation.tied` = true only when the two agree within rounding. A non-tie is a detective finding to investigate and clear BEFORE filing (the form also carries the ม.157 deadline = the 15th of the next month). Output VAT is posted to 2100 on every sale (Cr) and reversed on returns (Dr); input VAT is posted on AP bills (Dr) — so 2100's net is the period's VAT payable. Read-only report; exportable to a ภ.พ.30 PDF/HTML. VAT-account routing (docs/33 PR6): when a tenant routes VAT to its own output/input accounts via a tax_code, the reconciliation sums the WHOLE VAT-account set (2100 + the configured tax-code accounts), so the ภ.พ.30↔GL tie stays exact under routing (no tax codes ⇒ set is {2100} ⇒ unchanged).</t>
         </is>
       </c>
       <c r="H167" s="17" t="inlineStr">

</xml_diff>

<commit_message>
feat(assets): FA-11 custody-change maker-checker + audit-by-scan + offline scan queue (#453)
Custody-change maker-checker (new SOX control FA-11): a scanned/audited asset move is a PendingApproval request a different user must approve before the register moves (self-approve → SOD_VIOLATION); confirming the current location logs a Scan Verify movement. Audit-by-scan reconciles Found/Missing/Misplaced/Unknown and raises custody requests for misplaced assets on close. Offline scan queue (client_uuid idempotency) for audit + mobile-scan. Migration 0251; RCM census 188; docs synced (narrative 09, manual 06+FAQ, UAT-GL-121..125). Verified: module-qr 67, basics 253, compliance 134, pg-core/pg-smoke, all gates.
</commit_message>
<xml_diff>
--- a/compliance/Oshinei_ERP_SOX_RCM_v1.xlsx
+++ b/compliance/Oshinei_ERP_SOX_RCM_v1.xlsx
@@ -14,7 +14,7 @@
     <sheet name="Summary" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'RCM'!$A$1:$Q$188</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'RCM'!$A$1:$Q$189</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Gap Remediation'!$A$2:$H$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -843,7 +843,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q188"/>
+  <dimension ref="A1:Q189"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -16702,12 +16702,12 @@
     <row r="183">
       <c r="A183" s="15" t="inlineStr">
         <is>
-          <t>CON-01</t>
+          <t>FA-11</t>
         </is>
       </c>
       <c r="B183" s="16" t="inlineStr">
         <is>
-          <t>Consolidation &amp; FX</t>
+          <t>Fixed Assets</t>
         </is>
       </c>
       <c r="C183" s="17" t="inlineStr">
@@ -16717,42 +16717,42 @@
       </c>
       <c r="D183" s="16" t="inlineStr">
         <is>
-          <t>Consolidation</t>
+          <t>Property, Plant &amp; Equipment</t>
         </is>
       </c>
       <c r="E183" s="16" t="inlineStr">
         <is>
-          <t>Group consolidation mis-stated (ownership/currency).</t>
+          <t>Asset moved/reassigned without independent review — a custodian relabels an asset's physical location or holder (or an audit finds it elsewhere) and the register is changed on one person's say-so, enabling misappropriation (reassign to self/related party) or concealment of a missing asset; existence/custody assertions unreliable.</t>
         </is>
       </c>
       <c r="F183" s="16" t="inlineStr">
         <is>
-          <t>Accuracy</t>
+          <t>Authorization; Existence</t>
         </is>
       </c>
       <c r="G183" s="16" t="inlineStr">
         <is>
-          <t>Consolidation run (ownership %, entity currency) gated by 'approvals'.</t>
+          <t>Asset custody-change maker-checker (SoD) + audit-by-scan. A tag scan that CHANGES an asset's location/holder no longer writes the register: it raises a PendingApproval custody-change REQUEST (no GL effect); a DIFFERENT user must approve before the register moves and a 'Scan Update' movement is logged (approver != requester enforced regardless of permissions — binds even Admin; reject leaves the asset in place; only one request pending per asset). Confirming the current location is logged immediately as a non-approval 'Scan Verify' movement (existence evidence). A physical AUDIT (count by scan) classifies each scan Found/Misplaced/Unknown and reconciles Missing against the register; closing the audit raises custody-change requests for the misplaced assets — so no floor-level move rewrites the register without a second person's approval.</t>
         </is>
       </c>
       <c r="H183" s="17" t="inlineStr">
         <is>
-          <t>Auto+Manual</t>
+          <t>Prev / Det</t>
         </is>
       </c>
       <c r="I183" s="17" t="inlineStr">
         <is>
-          <t>Period</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J183" s="17" t="inlineStr">
         <is>
-          <t>Period</t>
+          <t>Per custody move / per audit</t>
         </is>
       </c>
       <c r="K183" s="16" t="inlineStr">
         <is>
-          <t>Group Controller</t>
+          <t>FaAccountant / Controller</t>
         </is>
       </c>
       <c r="L183" s="17" t="inlineStr">
@@ -16762,22 +16762,22 @@
       </c>
       <c r="M183" s="16" t="inlineStr">
         <is>
-          <t>consolidation.service.ts (runConsolidation @Permissions approvals)</t>
+          <t>assets.service.ts scanUpdate(verify vs request)/approveCustody/rejectCustody/openAudit/scanAudit/getAudit/closeAudit; assets.controller.ts (scan-update, custody*, audits*); schema/assets.ts asset_scan_requests + asset_audits + asset_audit_scans + migration 0251; web /assets Audit + Custody-approvals tabs; cutover/module-qr.ts (ToE)</t>
         </is>
       </c>
       <c r="N183" s="16" t="inlineStr">
         <is>
-          <t>Inspect consolidation logic + gate.</t>
+          <t>Inspect the scan-&gt;request-&gt;approve flow + the approver!=requester check + the audit reconcile-&gt;custody-request path.</t>
         </is>
       </c>
       <c r="O183" s="16" t="inlineStr">
         <is>
-          <t>Sample period: consolidated TB ties to entities.</t>
+          <t>Re-perform: scan a move (PendingApproval, register unmoved), attempt self-approve (SOD_VIOLATION), approve as a different user (register moves + movement logged); run an audit that finds a misplaced asset and confirm closing raises a pending custody request (re-performed by the module-qr harness).</t>
         </is>
       </c>
       <c r="P183" s="16" t="inlineStr">
         <is>
-          <t>Consol TB</t>
+          <t>Custody-change approval log + audit reconciliation + SoD test</t>
         </is>
       </c>
       <c r="Q183" s="18" t="inlineStr">
@@ -16789,7 +16789,7 @@
     <row r="184">
       <c r="A184" s="11" t="inlineStr">
         <is>
-          <t>CON-02</t>
+          <t>CON-01</t>
         </is>
       </c>
       <c r="B184" s="12" t="inlineStr">
@@ -16804,22 +16804,22 @@
       </c>
       <c r="D184" s="12" t="inlineStr">
         <is>
-          <t>FX gain/loss</t>
+          <t>Consolidation</t>
         </is>
       </c>
       <c r="E184" s="12" t="inlineStr">
         <is>
-          <t>FX exposures not revalued at period-end.</t>
+          <t>Group consolidation mis-stated (ownership/currency).</t>
         </is>
       </c>
       <c r="F184" s="12" t="inlineStr">
         <is>
-          <t>Valuation</t>
+          <t>Accuracy</t>
         </is>
       </c>
       <c r="G184" s="12" t="inlineStr">
         <is>
-          <t>FX revaluation at period-end rates; unrealized FX posted (acct 5400).</t>
+          <t>Consolidation run (ownership %, entity currency) gated by 'approvals'.</t>
         </is>
       </c>
       <c r="H184" s="13" t="inlineStr">
@@ -16829,7 +16829,7 @@
       </c>
       <c r="I184" s="13" t="inlineStr">
         <is>
-          <t>Period-end</t>
+          <t>Period</t>
         </is>
       </c>
       <c r="J184" s="13" t="inlineStr">
@@ -16839,7 +16839,7 @@
       </c>
       <c r="K184" s="12" t="inlineStr">
         <is>
-          <t>Controller</t>
+          <t>Group Controller</t>
         </is>
       </c>
       <c r="L184" s="13" t="inlineStr">
@@ -16849,22 +16849,22 @@
       </c>
       <c r="M184" s="12" t="inlineStr">
         <is>
-          <t>fx.service.ts (revalue / unrealized report)</t>
+          <t>consolidation.service.ts (runConsolidation @Permissions approvals)</t>
         </is>
       </c>
       <c r="N184" s="12" t="inlineStr">
         <is>
-          <t>Inspect reval logic + rates.</t>
+          <t>Inspect consolidation logic + gate.</t>
         </is>
       </c>
       <c r="O184" s="12" t="inlineStr">
         <is>
-          <t>Recompute reval on sample balances.</t>
+          <t>Sample period: consolidated TB ties to entities.</t>
         </is>
       </c>
       <c r="P184" s="12" t="inlineStr">
         <is>
-          <t>FX reval JE</t>
+          <t>Consol TB</t>
         </is>
       </c>
       <c r="Q184" s="18" t="inlineStr">
@@ -16876,7 +16876,7 @@
     <row r="185">
       <c r="A185" s="15" t="inlineStr">
         <is>
-          <t>CON-03</t>
+          <t>CON-02</t>
         </is>
       </c>
       <c r="B185" s="16" t="inlineStr">
@@ -16891,32 +16891,32 @@
       </c>
       <c r="D185" s="16" t="inlineStr">
         <is>
-          <t>Consolidation</t>
+          <t>FX gain/loss</t>
         </is>
       </c>
       <c r="E185" s="16" t="inlineStr">
         <is>
-          <t>Intercompany balances/transactions are not eliminated on consolidation, OR eliminations are mis-stated, so the consolidated group trial balance does not balance and group financials are overstated (IC double-counted).</t>
+          <t>FX exposures not revalued at period-end.</t>
         </is>
       </c>
       <c r="F185" s="16" t="inlineStr">
         <is>
-          <t>Accuracy/Completeness</t>
+          <t>Valuation</t>
         </is>
       </c>
       <c r="G185" s="16" t="inlineStr">
         <is>
-          <t>Elimination integrity (CON-03): runConsolidation combines member-entity TBs, generates reciprocal IC eliminations (Dr 2150 Due-To / Cr 1150 Due-From for each in-group IC transaction) at the GROUP layer (consolidation_run_lines — NOT pushed into any operating entity's GL), and ASSERTS the consolidated TB still balances (Σ signed nets ~0 and eliminations net to 0, NCI presentation reclass excluded) — failure throws CONSOL_UNBALANCED and rolls back the run. A balanced run is finalised, then frozen by a DIFFERENT user via run→post maker-checker (self-post → SELF_POST; re-running a Posted period → ALREADY_POSTED; one run per (group, period)). HQ/Admin-only; reads across member tenants via app.bypass_rls. Configurable elimination rules (consol_elimination_rules).</t>
+          <t>FX revaluation at period-end rates; unrealized FX posted (acct 5400).</t>
         </is>
       </c>
       <c r="H185" s="17" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="I185" s="17" t="inlineStr">
         <is>
-          <t>Auto+Manual</t>
+          <t>Period-end</t>
         </is>
       </c>
       <c r="J185" s="17" t="inlineStr">
@@ -16926,7 +16926,7 @@
       </c>
       <c r="K185" s="16" t="inlineStr">
         <is>
-          <t>Group Controller</t>
+          <t>Controller</t>
         </is>
       </c>
       <c r="L185" s="17" t="inlineStr">
@@ -16936,22 +16936,22 @@
       </c>
       <c r="M185" s="16" t="inlineStr">
         <is>
-          <t>consolidation.service.ts runConsolidation (balanced check, CONSOL_UNBALANCED)/postConsolidation (SELF_POST, ALREADY_POSTED); consolidation.controller.ts (run @approvals, runs/:id/post @approvals); schema/consolidation.ts (consolidation_runs.balanced/posted_by, consol_elimination_rules) + migration 0170; cutover/consolidation.ts (ToE)</t>
+          <t>fx.service.ts (revalue / unrealized report)</t>
         </is>
       </c>
       <c r="N185" s="16" t="inlineStr">
         <is>
-          <t>Inspect the combine→eliminate→balance flow, the CONSOL_UNBALANCED guard, and the run→post approver≠runner check.</t>
+          <t>Inspect reval logic + rates.</t>
         </is>
       </c>
       <c r="O185" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: run a group consolidation, confirm IC 1150/2150 eliminate and the consolidated TB balances; attempt self-post (SELF_POST); post as a different user (Posted); re-run the posted period (ALREADY_POSTED). Re-performed by the consolidation harness.</t>
+          <t>Recompute reval on sample balances.</t>
         </is>
       </c>
       <c r="P185" s="16" t="inlineStr">
         <is>
-          <t>Consolidated TB + elimination lines + post log</t>
+          <t>FX reval JE</t>
         </is>
       </c>
       <c r="Q185" s="18" t="inlineStr">
@@ -16963,7 +16963,7 @@
     <row r="186">
       <c r="A186" s="11" t="inlineStr">
         <is>
-          <t>CON-04</t>
+          <t>CON-03</t>
         </is>
       </c>
       <c r="B186" s="12" t="inlineStr">
@@ -16978,27 +16978,27 @@
       </c>
       <c r="D186" s="12" t="inlineStr">
         <is>
-          <t>All (segment disclosure)</t>
+          <t>Consolidation</t>
         </is>
       </c>
       <c r="E186" s="12" t="inlineStr">
         <is>
-          <t>Segment (branch/project/department) operating results are not reported, so IFRS 8 segment disclosure is incomplete or inaccurate and management/investors cannot see results by reportable segment.</t>
+          <t>Intercompany balances/transactions are not eliminated on consolidation, OR eliminations are mis-stated, so the consolidated group trial balance does not balance and group financials are overstated (IC double-counted).</t>
         </is>
       </c>
       <c r="F186" s="12" t="inlineStr">
         <is>
-          <t>Presentation/Disclosure</t>
+          <t>Accuracy/Completeness</t>
         </is>
       </c>
       <c r="G186" s="12" t="inlineStr">
         <is>
-          <t>Segment reporting (CON-04, IFRS 8): segmentReport produces P&amp;L (revenue/expense/net) grouped by reportable segment, sourced from the dimension columns on journal_lines (branch_id/project_id/department_id) and mapped through configurable segment_definitions (member_keys → segment); unmapped dimension values surface as their own/Unassigned bucket. HQ/Admin-only, gated 'exec'.</t>
+          <t>Elimination integrity (CON-03): runConsolidation combines member-entity TBs, generates reciprocal IC eliminations (Dr 2150 Due-To / Cr 1150 Due-From for each in-group IC transaction) at the GROUP layer (consolidation_run_lines — NOT pushed into any operating entity's GL), and ASSERTS the consolidated TB still balances (Σ signed nets ~0 and eliminations net to 0, NCI presentation reclass excluded) — failure throws CONSOL_UNBALANCED and rolls back the run. A balanced run is finalised, then frozen by a DIFFERENT user via run→post maker-checker (self-post → SELF_POST; re-running a Posted period → ALREADY_POSTED; one run per (group, period)). HQ/Admin-only; reads across member tenants via app.bypass_rls. Configurable elimination rules (consol_elimination_rules).</t>
         </is>
       </c>
       <c r="H186" s="13" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I186" s="13" t="inlineStr">
@@ -17023,22 +17023,22 @@
       </c>
       <c r="M186" s="12" t="inlineStr">
         <is>
-          <t>consolidation.service.ts defineSegment/listSegments/segmentReport; consolidation.controller.ts (segments, segment-report @exec); schema/consolidation.ts segment_definitions + migration 0170; cutover/consolidation.ts (ToE)</t>
+          <t>consolidation.service.ts runConsolidation (balanced check, CONSOL_UNBALANCED)/postConsolidation (SELF_POST, ALREADY_POSTED); consolidation.controller.ts (run @approvals, runs/:id/post @approvals); schema/consolidation.ts (consolidation_runs.balanced/posted_by, consol_elimination_rules) + migration 0170; cutover/consolidation.ts (ToE)</t>
         </is>
       </c>
       <c r="N186" s="12" t="inlineStr">
         <is>
-          <t>Inspect the segment mapping + the dimension-grouped P&amp;L aggregation.</t>
+          <t>Inspect the combine→eliminate→balance flow, the CONSOL_UNBALANCED guard, and the run→post approver≠runner check.</t>
         </is>
       </c>
       <c r="O186" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: define a segment over branches, run the segment report for a period, confirm revenue/expense/net tie to the underlying dimensioned postings. Re-performed by the consolidation harness.</t>
+          <t>Re-perform: run a group consolidation, confirm IC 1150/2150 eliminate and the consolidated TB balances; attempt self-post (SELF_POST); post as a different user (Posted); re-run the posted period (ALREADY_POSTED). Re-performed by the consolidation harness.</t>
         </is>
       </c>
       <c r="P186" s="12" t="inlineStr">
         <is>
-          <t>Segment P&amp;L report</t>
+          <t>Consolidated TB + elimination lines + post log</t>
         </is>
       </c>
       <c r="Q186" s="18" t="inlineStr">
@@ -17050,7 +17050,7 @@
     <row r="187">
       <c r="A187" s="15" t="inlineStr">
         <is>
-          <t>FX-04</t>
+          <t>CON-04</t>
         </is>
       </c>
       <c r="B187" s="16" t="inlineStr">
@@ -17065,42 +17065,42 @@
       </c>
       <c r="D187" s="16" t="inlineStr">
         <is>
-          <t>FX gain/loss; Revenue; AR/AP</t>
+          <t>All (segment disclosure)</t>
         </is>
       </c>
       <c r="E187" s="16" t="inlineStr">
         <is>
-          <t>A wrong manually-entered FX rate (fat-fingered, e.g. USD 36 keyed as 63) flows straight into a period-end revaluation JE and the unrealized-FX report with no independent review — mis-stating earnings/equity and FX-translated balances.</t>
+          <t>Segment (branch/project/department) operating results are not reported, so IFRS 8 segment disclosure is incomplete or inaccurate and management/investors cannot see results by reportable segment.</t>
         </is>
       </c>
       <c r="F187" s="16" t="inlineStr">
         <is>
-          <t>Accuracy/Valuation</t>
+          <t>Presentation/Disclosure</t>
         </is>
       </c>
       <c r="G187" s="16" t="inlineStr">
         <is>
-          <t>FX rate maker-checker (SoD): a MANUALLY-entered rate lands as PendingApproval and is EXCLUDED from rate resolution — revaluation, the unrealized-FX report, and consolidation translation all use APPROVED rates only — until a DIFFERENT user approves it (POST /api/fx/rates/approve). Self-approval → SOD_VIOLATION (binds even Admin); reject marks the rate Rejected (never usable); re-entering a rate sends it back to PendingApproval. Externally-sourced (feed) rates carrying an explicit non-manual source are auto-approved. Pending rates are also surfaced, aged, by the pending-approvals monitor (GOV-01).</t>
+          <t>Segment reporting (CON-04, IFRS 8): segmentReport produces P&amp;L (revenue/expense/net) grouped by reportable segment, sourced from the dimension columns on journal_lines (branch_id/project_id/department_id) and mapped through configurable segment_definitions (member_keys → segment); unmapped dimension values surface as their own/Unassigned bucket. HQ/Admin-only, gated 'exec'.</t>
         </is>
       </c>
       <c r="H187" s="17" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I187" s="17" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="J187" s="17" t="inlineStr">
         <is>
-          <t>Per rate</t>
+          <t>Period</t>
         </is>
       </c>
       <c r="K187" s="16" t="inlineStr">
         <is>
-          <t>Controller / Treasury</t>
+          <t>Group Controller</t>
         </is>
       </c>
       <c r="L187" s="17" t="inlineStr">
@@ -17110,22 +17110,22 @@
       </c>
       <c r="M187" s="16" t="inlineStr">
         <is>
-          <t>fx.service.ts setRate(manual→PendingApproval)/approveRate/rejectRate/rateAsOf(Approved only); fx.controller.ts (rates/approve|reject|pending gated approvals/gl_close); consolidation.service.ts (translation reads Approved rates); schema/fx.ts fx_rates.status + migration 0141; cutover/fxreval.ts (ToE)</t>
+          <t>consolidation.service.ts defineSegment/listSegments/segmentReport; consolidation.controller.ts (segments, segment-report @exec); schema/consolidation.ts segment_definitions + migration 0170; cutover/consolidation.ts (ToE)</t>
         </is>
       </c>
       <c r="N187" s="16" t="inlineStr">
         <is>
-          <t>Inspect the request→approve flow + the approver≠requester check + that revaluation/reporting resolve Approved rates only.</t>
+          <t>Inspect the segment mapping + the dimension-grouped P&amp;L aggregation.</t>
         </is>
       </c>
       <c r="O187" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: enter a manual rate (PendingApproval), confirm revalue is blocked NO_RATE while pending, attempt self-approve (SOD_VIOLATION), approve as a different user, then revalue succeeds (re-performed by the fxreval harness).</t>
+          <t>Re-perform: define a segment over branches, run the segment report for a period, confirm revenue/expense/net tie to the underlying dimensioned postings. Re-performed by the consolidation harness.</t>
         </is>
       </c>
       <c r="P187" s="16" t="inlineStr">
         <is>
-          <t>FX rate approval log + SoD test</t>
+          <t>Segment P&amp;L report</t>
         </is>
       </c>
       <c r="Q187" s="18" t="inlineStr">
@@ -17137,92 +17137,179 @@
     <row r="188">
       <c r="A188" s="11" t="inlineStr">
         <is>
+          <t>FX-04</t>
+        </is>
+      </c>
+      <c r="B188" s="12" t="inlineStr">
+        <is>
+          <t>Consolidation &amp; FX</t>
+        </is>
+      </c>
+      <c r="C188" s="13" t="inlineStr">
+        <is>
+          <t>Application</t>
+        </is>
+      </c>
+      <c r="D188" s="12" t="inlineStr">
+        <is>
+          <t>FX gain/loss; Revenue; AR/AP</t>
+        </is>
+      </c>
+      <c r="E188" s="12" t="inlineStr">
+        <is>
+          <t>A wrong manually-entered FX rate (fat-fingered, e.g. USD 36 keyed as 63) flows straight into a period-end revaluation JE and the unrealized-FX report with no independent review — mis-stating earnings/equity and FX-translated balances.</t>
+        </is>
+      </c>
+      <c r="F188" s="12" t="inlineStr">
+        <is>
+          <t>Accuracy/Valuation</t>
+        </is>
+      </c>
+      <c r="G188" s="12" t="inlineStr">
+        <is>
+          <t>FX rate maker-checker (SoD): a MANUALLY-entered rate lands as PendingApproval and is EXCLUDED from rate resolution — revaluation, the unrealized-FX report, and consolidation translation all use APPROVED rates only — until a DIFFERENT user approves it (POST /api/fx/rates/approve). Self-approval → SOD_VIOLATION (binds even Admin); reject marks the rate Rejected (never usable); re-entering a rate sends it back to PendingApproval. Externally-sourced (feed) rates carrying an explicit non-manual source are auto-approved. Pending rates are also surfaced, aged, by the pending-approvals monitor (GOV-01).</t>
+        </is>
+      </c>
+      <c r="H188" s="13" t="inlineStr">
+        <is>
+          <t>Prev</t>
+        </is>
+      </c>
+      <c r="I188" s="13" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="J188" s="13" t="inlineStr">
+        <is>
+          <t>Per rate</t>
+        </is>
+      </c>
+      <c r="K188" s="12" t="inlineStr">
+        <is>
+          <t>Controller / Treasury</t>
+        </is>
+      </c>
+      <c r="L188" s="13" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="M188" s="12" t="inlineStr">
+        <is>
+          <t>fx.service.ts setRate(manual→PendingApproval)/approveRate/rejectRate/rateAsOf(Approved only); fx.controller.ts (rates/approve|reject|pending gated approvals/gl_close); consolidation.service.ts (translation reads Approved rates); schema/fx.ts fx_rates.status + migration 0141; cutover/fxreval.ts (ToE)</t>
+        </is>
+      </c>
+      <c r="N188" s="12" t="inlineStr">
+        <is>
+          <t>Inspect the request→approve flow + the approver≠requester check + that revaluation/reporting resolve Approved rates only.</t>
+        </is>
+      </c>
+      <c r="O188" s="12" t="inlineStr">
+        <is>
+          <t>Re-perform: enter a manual rate (PendingApproval), confirm revalue is blocked NO_RATE while pending, attempt self-approve (SOD_VIOLATION), approve as a different user, then revalue succeeds (re-performed by the fxreval harness).</t>
+        </is>
+      </c>
+      <c r="P188" s="12" t="inlineStr">
+        <is>
+          <t>FX rate approval log + SoD test</t>
+        </is>
+      </c>
+      <c r="Q188" s="18" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="15" t="inlineStr">
+        <is>
           <t>BUD-01</t>
         </is>
       </c>
-      <c r="B188" s="12" t="inlineStr">
+      <c r="B189" s="16" t="inlineStr">
         <is>
           <t>Budgeting &amp; Planning</t>
         </is>
       </c>
-      <c r="C188" s="13" t="inlineStr">
+      <c r="C189" s="17" t="inlineStr">
         <is>
           <t>Application</t>
         </is>
       </c>
-      <c r="D188" s="12" t="inlineStr">
+      <c r="D189" s="16" t="inlineStr">
         <is>
           <t>Budget; All (variance reporting)</t>
         </is>
       </c>
-      <c r="E188" s="12" t="inlineStr">
+      <c r="E189" s="16" t="inlineStr">
         <is>
           <t>A budget figure is entered/changed by one person and immediately drives the budget-vs-actual variance report — the basis for spend authorization and performance review — with no independent approval; a wrong or self-serving budget makes overspending look 'on budget'.</t>
         </is>
       </c>
-      <c r="F188" s="12" t="inlineStr">
+      <c r="F189" s="16" t="inlineStr">
         <is>
           <t>Authorization/Accuracy</t>
         </is>
       </c>
-      <c r="G188" s="12" t="inlineStr">
+      <c r="G189" s="16" t="inlineStr">
         <is>
           <t>Budget maker-checker (SoD): an upserted budget (POST /api/ledger/budgets) lands as PendingApproval and is EXCLUDED from budget-vs-actual until a DIFFERENT user approves it (POST /api/ledger/budgets/approve for the fiscal_year/account/cost-centre[/period]). Self-approval → SOD_VIOLATION (binds even Admin); reject marks it Rejected (excluded). DEFAULT 'Approved' keeps existing rows + direct planning seeds usable. Pending budgets are also surfaced, aged, by the pending-approvals monitor (GOV-01).</t>
         </is>
       </c>
-      <c r="H188" s="13" t="inlineStr">
+      <c r="H189" s="17" t="inlineStr">
         <is>
           <t>Prev</t>
         </is>
       </c>
-      <c r="I188" s="13" t="inlineStr">
+      <c r="I189" s="17" t="inlineStr">
         <is>
           <t>Automated</t>
         </is>
       </c>
-      <c r="J188" s="13" t="inlineStr">
+      <c r="J189" s="17" t="inlineStr">
         <is>
           <t>Per budget</t>
         </is>
       </c>
-      <c r="K188" s="12" t="inlineStr">
+      <c r="K189" s="16" t="inlineStr">
         <is>
           <t>Controller / FP&amp;A</t>
         </is>
       </c>
-      <c r="L188" s="13" t="inlineStr">
+      <c r="L189" s="17" t="inlineStr">
         <is>
           <t>P10</t>
         </is>
       </c>
-      <c r="M188" s="12" t="inlineStr">
+      <c r="M189" s="16" t="inlineStr">
         <is>
           <t>budget.service.ts upsertBudget(→PendingApproval)/approveBudget/rejectBudget/budgetVsActual(Approved only); budget.controller.ts (budgets/approve|reject|pending gated approvals/gl_close); schema/budgets.ts budgets.status + migration 0142; cutover/budget.ts (ToE)</t>
         </is>
       </c>
-      <c r="N188" s="12" t="inlineStr">
+      <c r="N189" s="16" t="inlineStr">
         <is>
           <t>Inspect the request→approve flow + the approver≠requester check + that budget-vs-actual counts Approved budgets only.</t>
         </is>
       </c>
-      <c r="O188" s="12" t="inlineStr">
+      <c r="O189" s="16" t="inlineStr">
         <is>
           <t>Re-perform: upsert a budget (PendingApproval, excluded from variance), attempt self-approve (SOD_VIOLATION), approve as a different user, confirm it then appears in budget-vs-actual (re-performed by the budget harness).</t>
         </is>
       </c>
-      <c r="P188" s="12" t="inlineStr">
+      <c r="P189" s="16" t="inlineStr">
         <is>
           <t>Budget approval log + SoD test</t>
         </is>
       </c>
-      <c r="Q188" s="18" t="inlineStr">
+      <c r="Q189" s="18" t="inlineStr">
         <is>
           <t>Implemented</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q188"/>
+  <autoFilter ref="A1:Q189"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -17859,7 +17946,7 @@
         </is>
       </c>
       <c r="C5" s="26">
-        <f>COUNTIF(RCM!$Q$2:$Q$188,B5)</f>
+        <f>COUNTIF(RCM!$Q$2:$Q$189,B5)</f>
         <v/>
       </c>
     </row>
@@ -17870,7 +17957,7 @@
         </is>
       </c>
       <c r="C6" s="26">
-        <f>COUNTIF(RCM!$Q$2:$Q$188,B6)</f>
+        <f>COUNTIF(RCM!$Q$2:$Q$189,B6)</f>
         <v/>
       </c>
     </row>
@@ -17881,7 +17968,7 @@
         </is>
       </c>
       <c r="C7" s="26">
-        <f>COUNTIF(RCM!$Q$2:$Q$188,B7)</f>
+        <f>COUNTIF(RCM!$Q$2:$Q$189,B7)</f>
         <v/>
       </c>
     </row>
@@ -17892,7 +17979,7 @@
         </is>
       </c>
       <c r="C8" s="29">
-        <f>COUNTA(RCM!$A$2:$A$188)</f>
+        <f>COUNTA(RCM!$A$2:$A$189)</f>
         <v/>
       </c>
     </row>
@@ -17910,7 +17997,7 @@
         </is>
       </c>
       <c r="C11" s="26">
-        <f>COUNTIF(RCM!$C$2:$C$188,B11)</f>
+        <f>COUNTIF(RCM!$C$2:$C$189,B11)</f>
         <v/>
       </c>
     </row>
@@ -17921,7 +18008,7 @@
         </is>
       </c>
       <c r="C12" s="26">
-        <f>COUNTIF(RCM!$C$2:$C$188,B12)</f>
+        <f>COUNTIF(RCM!$C$2:$C$189,B12)</f>
         <v/>
       </c>
     </row>
@@ -17932,7 +18019,7 @@
         </is>
       </c>
       <c r="C13" s="26">
-        <f>COUNTIF(RCM!$C$2:$C$188,B13)</f>
+        <f>COUNTIF(RCM!$C$2:$C$189,B13)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(assets): surface audit results as BI reports + FA-12 asset verification-exception monitor (#454)
Two schedulable BI report types over the FA-11 custody/audit data: asset_audit (recent audits' found/missing/misplaced/unknown tallies + pending custody queue) and asset_verification_exceptions (active assets not scan-verified within N days, default 90; never-verified falls back to acquisition date). Scheduled monthly, the exception report is a new detective existence control FA-12. Read-only, no migration, no SoD. RCM census 189; docs synced (narrative 09, manual 09, UAT-GL-126..127). Verified: module-qr 73, bi 36, basics 256, all gates.
</commit_message>
<xml_diff>
--- a/compliance/Oshinei_ERP_SOX_RCM_v1.xlsx
+++ b/compliance/Oshinei_ERP_SOX_RCM_v1.xlsx
@@ -14,7 +14,7 @@
     <sheet name="Summary" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'RCM'!$A$1:$Q$189</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'RCM'!$A$1:$Q$190</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Gap Remediation'!$A$2:$H$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -843,7 +843,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q189"/>
+  <dimension ref="A1:Q190"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -16789,82 +16789,82 @@
     <row r="184">
       <c r="A184" s="11" t="inlineStr">
         <is>
-          <t>CON-01</t>
+          <t>FA-12</t>
         </is>
       </c>
       <c r="B184" s="12" t="inlineStr">
         <is>
-          <t>Consolidation &amp; FX</t>
+          <t>Fixed Assets</t>
         </is>
       </c>
       <c r="C184" s="13" t="inlineStr">
         <is>
-          <t>Application</t>
+          <t>Detective</t>
         </is>
       </c>
       <c r="D184" s="12" t="inlineStr">
         <is>
-          <t>Consolidation</t>
+          <t>Property, Plant &amp; Equipment</t>
         </is>
       </c>
       <c r="E184" s="12" t="inlineStr">
         <is>
-          <t>Group consolidation mis-stated (ownership/currency).</t>
+          <t>Assets exist on the register but are never physically confirmed — a missing/stolen/scrapped asset stays on the books indefinitely because no periodic existence check flags it, overstating PPE and the existence assertion.</t>
         </is>
       </c>
       <c r="F184" s="12" t="inlineStr">
         <is>
-          <t>Accuracy</t>
+          <t>Existence; Completeness</t>
         </is>
       </c>
       <c r="G184" s="12" t="inlineStr">
         <is>
-          <t>Consolidation run (ownership %, entity currency) gated by 'approvals'.</t>
+          <t>Periodic asset-existence exception monitoring. A schedulable BI report (report_type asset_verification_exceptions) lists every ACTIVE asset not physically verified within N days (default 90) — 'verified' = a Scan Verify or approved Scan Update movement (FA-11), with a never-verified asset falling back to its acquisition date as the implicit receipt baseline. Each exception carries days-since-last-seen so the oldest surface first. Scheduled monthly, it drives a recurring existence count before period-end; the companion asset_audit report surfaces recent audit results (found/missing/misplaced/unknown) and the outstanding custody-change queue. Read-only aggregation over fixed_assets + asset_movements — posts nothing, adds no authority (no SoD conflict); complements the FA-11 audit-by-scan (which supplies the verification movements) and the FA-05 register-to-GL tie-out.</t>
         </is>
       </c>
       <c r="H184" s="13" t="inlineStr">
         <is>
-          <t>Auto+Manual</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I184" s="13" t="inlineStr">
         <is>
-          <t>Period</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J184" s="13" t="inlineStr">
         <is>
-          <t>Period</t>
+          <t>Monthly (scheduled) / on demand</t>
         </is>
       </c>
       <c r="K184" s="12" t="inlineStr">
         <is>
-          <t>Group Controller</t>
+          <t>FaAccountant / Controller</t>
         </is>
       </c>
       <c r="L184" s="13" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="M184" s="12" t="inlineStr">
         <is>
-          <t>consolidation.service.ts (runConsolidation @Permissions approvals)</t>
+          <t>assets.service.ts unverifiedAssets/auditReport; assets.controller.ts (unverified, audit-report); bi.service.ts REPORT_TYPES asset_verification_exceptions + asset_audit + generateReport blocks; bi.module.ts imports AssetsModule; cutover/module-qr.ts (ToE)</t>
         </is>
       </c>
       <c r="N184" s="12" t="inlineStr">
         <is>
-          <t>Inspect consolidation logic + gate.</t>
+          <t>Inspect the exception query (last Scan Verify/Update vs N-day threshold, acquisition-date fallback) and that the report is a registered, schedulable BI type.</t>
         </is>
       </c>
       <c r="O184" s="12" t="inlineStr">
         <is>
-          <t>Sample period: consolidated TB ties to entities.</t>
+          <t>Re-perform: seed an old never-scanned asset, run GET /api/assets/unverified?days=90 (asset flagged) + a recently-scanned asset is NOT flagged; schedule + run the asset_verification_exceptions report and confirm the summary counts the exception (re-performed by the module-qr harness).</t>
         </is>
       </c>
       <c r="P184" s="12" t="inlineStr">
         <is>
-          <t>Consol TB</t>
+          <t>Scheduled exception report runs + exception list + verification-movement log</t>
         </is>
       </c>
       <c r="Q184" s="18" t="inlineStr">
@@ -16876,7 +16876,7 @@
     <row r="185">
       <c r="A185" s="15" t="inlineStr">
         <is>
-          <t>CON-02</t>
+          <t>CON-01</t>
         </is>
       </c>
       <c r="B185" s="16" t="inlineStr">
@@ -16891,22 +16891,22 @@
       </c>
       <c r="D185" s="16" t="inlineStr">
         <is>
-          <t>FX gain/loss</t>
+          <t>Consolidation</t>
         </is>
       </c>
       <c r="E185" s="16" t="inlineStr">
         <is>
-          <t>FX exposures not revalued at period-end.</t>
+          <t>Group consolidation mis-stated (ownership/currency).</t>
         </is>
       </c>
       <c r="F185" s="16" t="inlineStr">
         <is>
-          <t>Valuation</t>
+          <t>Accuracy</t>
         </is>
       </c>
       <c r="G185" s="16" t="inlineStr">
         <is>
-          <t>FX revaluation at period-end rates; unrealized FX posted (acct 5400).</t>
+          <t>Consolidation run (ownership %, entity currency) gated by 'approvals'.</t>
         </is>
       </c>
       <c r="H185" s="17" t="inlineStr">
@@ -16916,7 +16916,7 @@
       </c>
       <c r="I185" s="17" t="inlineStr">
         <is>
-          <t>Period-end</t>
+          <t>Period</t>
         </is>
       </c>
       <c r="J185" s="17" t="inlineStr">
@@ -16926,7 +16926,7 @@
       </c>
       <c r="K185" s="16" t="inlineStr">
         <is>
-          <t>Controller</t>
+          <t>Group Controller</t>
         </is>
       </c>
       <c r="L185" s="17" t="inlineStr">
@@ -16936,22 +16936,22 @@
       </c>
       <c r="M185" s="16" t="inlineStr">
         <is>
-          <t>fx.service.ts (revalue / unrealized report)</t>
+          <t>consolidation.service.ts (runConsolidation @Permissions approvals)</t>
         </is>
       </c>
       <c r="N185" s="16" t="inlineStr">
         <is>
-          <t>Inspect reval logic + rates.</t>
+          <t>Inspect consolidation logic + gate.</t>
         </is>
       </c>
       <c r="O185" s="16" t="inlineStr">
         <is>
-          <t>Recompute reval on sample balances.</t>
+          <t>Sample period: consolidated TB ties to entities.</t>
         </is>
       </c>
       <c r="P185" s="16" t="inlineStr">
         <is>
-          <t>FX reval JE</t>
+          <t>Consol TB</t>
         </is>
       </c>
       <c r="Q185" s="18" t="inlineStr">
@@ -16963,7 +16963,7 @@
     <row r="186">
       <c r="A186" s="11" t="inlineStr">
         <is>
-          <t>CON-03</t>
+          <t>CON-02</t>
         </is>
       </c>
       <c r="B186" s="12" t="inlineStr">
@@ -16978,32 +16978,32 @@
       </c>
       <c r="D186" s="12" t="inlineStr">
         <is>
-          <t>Consolidation</t>
+          <t>FX gain/loss</t>
         </is>
       </c>
       <c r="E186" s="12" t="inlineStr">
         <is>
-          <t>Intercompany balances/transactions are not eliminated on consolidation, OR eliminations are mis-stated, so the consolidated group trial balance does not balance and group financials are overstated (IC double-counted).</t>
+          <t>FX exposures not revalued at period-end.</t>
         </is>
       </c>
       <c r="F186" s="12" t="inlineStr">
         <is>
-          <t>Accuracy/Completeness</t>
+          <t>Valuation</t>
         </is>
       </c>
       <c r="G186" s="12" t="inlineStr">
         <is>
-          <t>Elimination integrity (CON-03): runConsolidation combines member-entity TBs, generates reciprocal IC eliminations (Dr 2150 Due-To / Cr 1150 Due-From for each in-group IC transaction) at the GROUP layer (consolidation_run_lines — NOT pushed into any operating entity's GL), and ASSERTS the consolidated TB still balances (Σ signed nets ~0 and eliminations net to 0, NCI presentation reclass excluded) — failure throws CONSOL_UNBALANCED and rolls back the run. A balanced run is finalised, then frozen by a DIFFERENT user via run→post maker-checker (self-post → SELF_POST; re-running a Posted period → ALREADY_POSTED; one run per (group, period)). HQ/Admin-only; reads across member tenants via app.bypass_rls. Configurable elimination rules (consol_elimination_rules).</t>
+          <t>FX revaluation at period-end rates; unrealized FX posted (acct 5400).</t>
         </is>
       </c>
       <c r="H186" s="13" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="I186" s="13" t="inlineStr">
         <is>
-          <t>Auto+Manual</t>
+          <t>Period-end</t>
         </is>
       </c>
       <c r="J186" s="13" t="inlineStr">
@@ -17013,7 +17013,7 @@
       </c>
       <c r="K186" s="12" t="inlineStr">
         <is>
-          <t>Group Controller</t>
+          <t>Controller</t>
         </is>
       </c>
       <c r="L186" s="13" t="inlineStr">
@@ -17023,22 +17023,22 @@
       </c>
       <c r="M186" s="12" t="inlineStr">
         <is>
-          <t>consolidation.service.ts runConsolidation (balanced check, CONSOL_UNBALANCED)/postConsolidation (SELF_POST, ALREADY_POSTED); consolidation.controller.ts (run @approvals, runs/:id/post @approvals); schema/consolidation.ts (consolidation_runs.balanced/posted_by, consol_elimination_rules) + migration 0170; cutover/consolidation.ts (ToE)</t>
+          <t>fx.service.ts (revalue / unrealized report)</t>
         </is>
       </c>
       <c r="N186" s="12" t="inlineStr">
         <is>
-          <t>Inspect the combine→eliminate→balance flow, the CONSOL_UNBALANCED guard, and the run→post approver≠runner check.</t>
+          <t>Inspect reval logic + rates.</t>
         </is>
       </c>
       <c r="O186" s="12" t="inlineStr">
         <is>
-          <t>Re-perform: run a group consolidation, confirm IC 1150/2150 eliminate and the consolidated TB balances; attempt self-post (SELF_POST); post as a different user (Posted); re-run the posted period (ALREADY_POSTED). Re-performed by the consolidation harness.</t>
+          <t>Recompute reval on sample balances.</t>
         </is>
       </c>
       <c r="P186" s="12" t="inlineStr">
         <is>
-          <t>Consolidated TB + elimination lines + post log</t>
+          <t>FX reval JE</t>
         </is>
       </c>
       <c r="Q186" s="18" t="inlineStr">
@@ -17050,7 +17050,7 @@
     <row r="187">
       <c r="A187" s="15" t="inlineStr">
         <is>
-          <t>CON-04</t>
+          <t>CON-03</t>
         </is>
       </c>
       <c r="B187" s="16" t="inlineStr">
@@ -17065,27 +17065,27 @@
       </c>
       <c r="D187" s="16" t="inlineStr">
         <is>
-          <t>All (segment disclosure)</t>
+          <t>Consolidation</t>
         </is>
       </c>
       <c r="E187" s="16" t="inlineStr">
         <is>
-          <t>Segment (branch/project/department) operating results are not reported, so IFRS 8 segment disclosure is incomplete or inaccurate and management/investors cannot see results by reportable segment.</t>
+          <t>Intercompany balances/transactions are not eliminated on consolidation, OR eliminations are mis-stated, so the consolidated group trial balance does not balance and group financials are overstated (IC double-counted).</t>
         </is>
       </c>
       <c r="F187" s="16" t="inlineStr">
         <is>
-          <t>Presentation/Disclosure</t>
+          <t>Accuracy/Completeness</t>
         </is>
       </c>
       <c r="G187" s="16" t="inlineStr">
         <is>
-          <t>Segment reporting (CON-04, IFRS 8): segmentReport produces P&amp;L (revenue/expense/net) grouped by reportable segment, sourced from the dimension columns on journal_lines (branch_id/project_id/department_id) and mapped through configurable segment_definitions (member_keys → segment); unmapped dimension values surface as their own/Unassigned bucket. HQ/Admin-only, gated 'exec'.</t>
+          <t>Elimination integrity (CON-03): runConsolidation combines member-entity TBs, generates reciprocal IC eliminations (Dr 2150 Due-To / Cr 1150 Due-From for each in-group IC transaction) at the GROUP layer (consolidation_run_lines — NOT pushed into any operating entity's GL), and ASSERTS the consolidated TB still balances (Σ signed nets ~0 and eliminations net to 0, NCI presentation reclass excluded) — failure throws CONSOL_UNBALANCED and rolls back the run. A balanced run is finalised, then frozen by a DIFFERENT user via run→post maker-checker (self-post → SELF_POST; re-running a Posted period → ALREADY_POSTED; one run per (group, period)). HQ/Admin-only; reads across member tenants via app.bypass_rls. Configurable elimination rules (consol_elimination_rules).</t>
         </is>
       </c>
       <c r="H187" s="17" t="inlineStr">
         <is>
-          <t>Det</t>
+          <t>Prev</t>
         </is>
       </c>
       <c r="I187" s="17" t="inlineStr">
@@ -17110,22 +17110,22 @@
       </c>
       <c r="M187" s="16" t="inlineStr">
         <is>
-          <t>consolidation.service.ts defineSegment/listSegments/segmentReport; consolidation.controller.ts (segments, segment-report @exec); schema/consolidation.ts segment_definitions + migration 0170; cutover/consolidation.ts (ToE)</t>
+          <t>consolidation.service.ts runConsolidation (balanced check, CONSOL_UNBALANCED)/postConsolidation (SELF_POST, ALREADY_POSTED); consolidation.controller.ts (run @approvals, runs/:id/post @approvals); schema/consolidation.ts (consolidation_runs.balanced/posted_by, consol_elimination_rules) + migration 0170; cutover/consolidation.ts (ToE)</t>
         </is>
       </c>
       <c r="N187" s="16" t="inlineStr">
         <is>
-          <t>Inspect the segment mapping + the dimension-grouped P&amp;L aggregation.</t>
+          <t>Inspect the combine→eliminate→balance flow, the CONSOL_UNBALANCED guard, and the run→post approver≠runner check.</t>
         </is>
       </c>
       <c r="O187" s="16" t="inlineStr">
         <is>
-          <t>Re-perform: define a segment over branches, run the segment report for a period, confirm revenue/expense/net tie to the underlying dimensioned postings. Re-performed by the consolidation harness.</t>
+          <t>Re-perform: run a group consolidation, confirm IC 1150/2150 eliminate and the consolidated TB balances; attempt self-post (SELF_POST); post as a different user (Posted); re-run the posted period (ALREADY_POSTED). Re-performed by the consolidation harness.</t>
         </is>
       </c>
       <c r="P187" s="16" t="inlineStr">
         <is>
-          <t>Segment P&amp;L report</t>
+          <t>Consolidated TB + elimination lines + post log</t>
         </is>
       </c>
       <c r="Q187" s="18" t="inlineStr">
@@ -17137,7 +17137,7 @@
     <row r="188">
       <c r="A188" s="11" t="inlineStr">
         <is>
-          <t>FX-04</t>
+          <t>CON-04</t>
         </is>
       </c>
       <c r="B188" s="12" t="inlineStr">
@@ -17152,42 +17152,42 @@
       </c>
       <c r="D188" s="12" t="inlineStr">
         <is>
-          <t>FX gain/loss; Revenue; AR/AP</t>
+          <t>All (segment disclosure)</t>
         </is>
       </c>
       <c r="E188" s="12" t="inlineStr">
         <is>
-          <t>A wrong manually-entered FX rate (fat-fingered, e.g. USD 36 keyed as 63) flows straight into a period-end revaluation JE and the unrealized-FX report with no independent review — mis-stating earnings/equity and FX-translated balances.</t>
+          <t>Segment (branch/project/department) operating results are not reported, so IFRS 8 segment disclosure is incomplete or inaccurate and management/investors cannot see results by reportable segment.</t>
         </is>
       </c>
       <c r="F188" s="12" t="inlineStr">
         <is>
-          <t>Accuracy/Valuation</t>
+          <t>Presentation/Disclosure</t>
         </is>
       </c>
       <c r="G188" s="12" t="inlineStr">
         <is>
-          <t>FX rate maker-checker (SoD): a MANUALLY-entered rate lands as PendingApproval and is EXCLUDED from rate resolution — revaluation, the unrealized-FX report, and consolidation translation all use APPROVED rates only — until a DIFFERENT user approves it (POST /api/fx/rates/approve). Self-approval → SOD_VIOLATION (binds even Admin); reject marks the rate Rejected (never usable); re-entering a rate sends it back to PendingApproval. Externally-sourced (feed) rates carrying an explicit non-manual source are auto-approved. Pending rates are also surfaced, aged, by the pending-approvals monitor (GOV-01).</t>
+          <t>Segment reporting (CON-04, IFRS 8): segmentReport produces P&amp;L (revenue/expense/net) grouped by reportable segment, sourced from the dimension columns on journal_lines (branch_id/project_id/department_id) and mapped through configurable segment_definitions (member_keys → segment); unmapped dimension values surface as their own/Unassigned bucket. HQ/Admin-only, gated 'exec'.</t>
         </is>
       </c>
       <c r="H188" s="13" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Det</t>
         </is>
       </c>
       <c r="I188" s="13" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Auto+Manual</t>
         </is>
       </c>
       <c r="J188" s="13" t="inlineStr">
         <is>
-          <t>Per rate</t>
+          <t>Period</t>
         </is>
       </c>
       <c r="K188" s="12" t="inlineStr">
         <is>
-          <t>Controller / 